<commit_message>
Extend Excel roster to stage20 and tune first planet and galaxy budgets; preserve save identities
</commit_message>
<xml_diff>
--- a/space-battleship/config_excel/level.xlsx
+++ b/space-battleship/config_excel/level.xlsx
@@ -1407,10 +1407,10 @@
         </ns0:is>
       </ns0:c>
       <ns0:c r="D9" s="1" t="n">
-        <ns0:v>38.33759992447472</ns0:v>
+        <ns0:v>15.40702157458636</ns0:v>
       </ns0:c>
       <ns0:c r="E9" s="1" t="n">
-        <ns0:v>38.33759992447472</ns0:v>
+        <ns0:v>15.40702157458636</ns0:v>
       </ns0:c>
       <ns0:c r="F9" s="1" t="n">
         <ns0:v>12</ns0:v>
@@ -1543,26 +1543,23 @@
       </ns0:c>
       <ns0:c r="C14" s="1" t="inlineStr">
         <ns0:is>
-          <ns0:t>{2|0.1,2|0.2,5|0.3,2|0.4,9|0.5,2|0.6,5|0.7,2|0.8,13|0.9}</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="D14" s="1">
-        <ns0:f>ROUND(($D$23-$D$13)^((A14-$A$13)/10)+$D$13,0)</ns0:f>
-        <ns0:v>56358.0</ns0:v>
-      </ns0:c>
-      <ns0:c r="E14" s="1">
-        <ns0:f>D14</ns0:f>
-        <ns0:v>56358.0</ns0:v>
-      </ns0:c>
-      <ns0:c r="F14" s="1">
-        <ns0:f>ROUND(($F$23-$F$13)^((A14-$A$13)/10)+$F$13,0)</ns0:f>
-        <ns0:v>17641.0</ns0:v>
+          <ns0:t>{30111|0.100000,30112|0.200000,30113|0.300000,30114|0.400000,30115|0.500000,30116|0.600000,30117|0.700000,30118|0.800000,30119|0.900000}</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D14" s="1" t="n">
+        <ns0:v>602880.1175788565</ns0:v>
+      </ns0:c>
+      <ns0:c r="E14" s="1" t="n">
+        <ns0:v>602880.1175788565</ns0:v>
+      </ns0:c>
+      <ns0:c r="F14" s="1" t="n">
+        <ns0:v>18870.66854784442</ns0:v>
       </ns0:c>
       <ns0:c r="G14" s="1" t="n">
         <ns0:v>3</ns0:v>
       </ns0:c>
       <ns0:c r="H14" s="1" t="n">
-        <ns0:v>1</ns0:v>
+        <ns0:v>0</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="15">
@@ -1574,26 +1571,23 @@
       </ns0:c>
       <ns0:c r="C15" s="1" t="inlineStr">
         <ns0:is>
-          <ns0:t>{1|0.1,1|0.2,4|0.3,1|0.4,10|0.5,1|0.6,4|0.7,1|0.8,14|0.9}</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="D15" s="1">
-        <ns0:f>ROUND(($D$23-$D$13)^((A15-$A$13)/10)+$D$13,0)</ns0:f>
-        <ns0:v>56448.0</ns0:v>
-      </ns0:c>
-      <ns0:c r="E15" s="1">
-        <ns0:f>D15</ns0:f>
-        <ns0:v>56448.0</ns0:v>
-      </ns0:c>
-      <ns0:c r="F15" s="1">
-        <ns0:f>ROUND(($F$23-$F$13)^((A15-$A$13)/10)+$F$13,0)</ns0:f>
-        <ns0:v>17651.0</ns0:v>
+          <ns0:t>{30121|0.100000,30122|0.200000,30123|0.300000,30124|0.400000,30125|0.500000,30126|0.600000,30127|0.700000,30128|0.800000,30129|0.900000}</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D15" s="1" t="n">
+        <ns0:v>6450407.623907364</ns0:v>
+      </ns0:c>
+      <ns0:c r="E15" s="1" t="n">
+        <ns0:v>6450407.623907364</ns0:v>
+      </ns0:c>
+      <ns0:c r="F15" s="1" t="n">
+        <ns0:v>201903.3315579912</ns0:v>
       </ns0:c>
       <ns0:c r="G15" s="1" t="n">
         <ns0:v>3.2</ns0:v>
       </ns0:c>
       <ns0:c r="H15" s="1" t="n">
-        <ns0:v>1</ns0:v>
+        <ns0:v>0</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="16">
@@ -1605,26 +1599,23 @@
       </ns0:c>
       <ns0:c r="C16" s="1" t="inlineStr">
         <ns0:is>
-          <ns0:t>{5|0.1,5|0.2,12|0.3,5|0.4,9|0.5,5|0.6,12|0.7,5|0.8,13|0.9}</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="D16" s="1">
-        <ns0:f>ROUND(($D$23-$D$13)^((A16-$A$13)/10)+$D$13,0)</ns0:f>
-        <ns0:v>57348.0</ns0:v>
-      </ns0:c>
-      <ns0:c r="E16" s="1">
-        <ns0:f>D16</ns0:f>
-        <ns0:v>57348.0</ns0:v>
-      </ns0:c>
-      <ns0:c r="F16" s="1">
-        <ns0:f>ROUND(($F$23-$F$13)^((A16-$A$13)/10)+$F$13,0)</ns0:f>
-        <ns0:v>17688.0</ns0:v>
+          <ns0:t>{30131|0.100000,30132|0.200000,30133|0.300000,30134|0.400000,30135|0.500000,30136|0.600000,30137|0.700000,30138|0.800000,30139|0.900000}</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D16" s="1" t="n">
+        <ns0:v>69014978.76834521</ns0:v>
+      </ns0:c>
+      <ns0:c r="E16" s="1" t="n">
+        <ns0:v>69014978.76834521</ns0:v>
+      </ns0:c>
+      <ns0:c r="F16" s="1" t="n">
+        <ns0:v>2160228.462010301</ns0:v>
       </ns0:c>
       <ns0:c r="G16" s="1" t="n">
         <ns0:v>3.4</ns0:v>
       </ns0:c>
       <ns0:c r="H16" s="1" t="n">
-        <ns0:v>1</ns0:v>
+        <ns0:v>0</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="17">
@@ -1636,26 +1627,23 @@
       </ns0:c>
       <ns0:c r="C17" s="1" t="inlineStr">
         <ns0:is>
-          <ns0:t>{4|0.1,4|0.2,11|0.3,4|0.4,10|0.5,4|0.6,11|0.7,4|0.8,14|0.9}</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="D17" s="1">
-        <ns0:f>ROUND(($D$23-$D$13)^((A17-$A$13)/10)+$D$13,0)</ns0:f>
-        <ns0:v>66347.0</ns0:v>
-      </ns0:c>
-      <ns0:c r="E17" s="1">
-        <ns0:f>D17</ns0:f>
-        <ns0:v>66347.0</ns0:v>
-      </ns0:c>
-      <ns0:c r="F17" s="1">
-        <ns0:f>ROUND(($F$23-$F$13)^((A17-$A$13)/10)+$F$13,0)</ns0:f>
-        <ns0:v>17825.0</ns0:v>
+          <ns0:t>{30141|0.100000,30142|0.200000,30143|0.300000,30144|0.400000,30145|0.500000,30146|0.600000,30147|0.700000,30148|0.800000,30149|0.900000}</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D17" s="1" t="n">
+        <ns0:v>738413379.7593849</ns0:v>
+      </ns0:c>
+      <ns0:c r="E17" s="1" t="n">
+        <ns0:v>738413379.7593849</ns0:v>
+      </ns0:c>
+      <ns0:c r="F17" s="1" t="n">
+        <ns0:v>23112976.75015848</ns0:v>
       </ns0:c>
       <ns0:c r="G17" s="1" t="n">
         <ns0:v>3.6</ns0:v>
       </ns0:c>
       <ns0:c r="H17" s="1" t="n">
-        <ns0:v>1</ns0:v>
+        <ns0:v>0</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="18">
@@ -1667,26 +1655,23 @@
       </ns0:c>
       <ns0:c r="C18" s="1" t="inlineStr">
         <ns0:is>
-          <ns0:t>{3|0.1,3|0.2,6|0.3,7|0.4,8|0.5,13|0.6,14|0.7,8|0.8,15|0.9}</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="D18" s="1">
-        <ns0:f>ROUND(($D$23-$D$13)^((A18-$A$13)/10)+$D$13,0)</ns0:f>
-        <ns0:v>156347.0</ns0:v>
-      </ns0:c>
-      <ns0:c r="E18" s="1">
-        <ns0:f>D18</ns0:f>
-        <ns0:v>156347.0</ns0:v>
-      </ns0:c>
-      <ns0:c r="F18" s="1">
-        <ns0:f>ROUND(($F$23-$F$13)^((A18-$A$13)/10)+$F$13,0)</ns0:f>
-        <ns0:v>18332.0</ns0:v>
+          <ns0:t>{30151|0.100000,30152|0.200000,30153|0.300000,30154|0.400000,30155|0.500000,30156|0.600000,30157|0.700000,30158|0.800000,30159|0.900000}</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D18" s="1" t="n">
+        <ns0:v>7900521439.525051</ns0:v>
+      </ns0:c>
+      <ns0:c r="E18" s="1" t="n">
+        <ns0:v>7900521439.525051</ns0:v>
+      </ns0:c>
+      <ns0:c r="F18" s="1" t="n">
+        <ns0:v>247293146.8351421</ns0:v>
       </ns0:c>
       <ns0:c r="G18" s="1" t="n">
         <ns0:v>3.8</ns0:v>
       </ns0:c>
       <ns0:c r="H18" s="1" t="n">
-        <ns0:v>1</ns0:v>
+        <ns0:v>0</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="19">
@@ -1698,26 +1683,23 @@
       </ns0:c>
       <ns0:c r="C19" s="1" t="inlineStr">
         <ns0:is>
-          <ns0:t>{2|0.1,2|0.2,5|0.3,2|0.4,9|0.5,2|0.6,5|0.7,2|0.8,13|0.9}</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="D19" s="1">
-        <ns0:f>ROUND(($D$23-$D$13)^((A19-$A$13)/10)+$D$13,0)</ns0:f>
-        <ns0:v>1056344.0</ns0:v>
-      </ns0:c>
-      <ns0:c r="E19" s="1">
-        <ns0:f>D19</ns0:f>
-        <ns0:v>1056344.0</ns0:v>
-      </ns0:c>
-      <ns0:c r="F19" s="1">
-        <ns0:f>ROUND(($F$23-$F$13)^((A19-$A$13)/10)+$F$13,0)</ns0:f>
-        <ns0:v>20208.0</ns0:v>
+          <ns0:t>{30161|0.100000,30162|0.200000,30163|0.300000,30164|0.400000,30165|0.500000,30166|0.600000,30167|0.700000,30168|0.800000,30169|0.900000}</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D19" s="1" t="n">
+        <ns0:v>84530211298.0865</ns0:v>
+      </ns0:c>
+      <ns0:c r="E19" s="1" t="n">
+        <ns0:v>84530211298.0865</ns0:v>
+      </ns0:c>
+      <ns0:c r="F19" s="1" t="n">
+        <ns0:v>2645868644.816936</ns0:v>
       </ns0:c>
       <ns0:c r="G19" s="1" t="n">
         <ns0:v>4</ns0:v>
       </ns0:c>
       <ns0:c r="H19" s="1" t="n">
-        <ns0:v>1</ns0:v>
+        <ns0:v>0</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="20">
@@ -1729,26 +1711,23 @@
       </ns0:c>
       <ns0:c r="C20" s="1" t="inlineStr">
         <ns0:is>
-          <ns0:t>{1|0.1,1|0.2,4|0.3,1|0.4,10|0.5,1|0.6,4|0.7,1|0.8,14|0.9}</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="D20" s="1">
-        <ns0:f>ROUND(($D$23-$D$13)^((A20-$A$13)/10)+$D$13,0)</ns0:f>
-        <ns0:v>10056308.0</ns0:v>
-      </ns0:c>
-      <ns0:c r="E20" s="1">
-        <ns0:f>D20</ns0:f>
-        <ns0:v>10056308.0</ns0:v>
-      </ns0:c>
-      <ns0:c r="F20" s="1">
-        <ns0:f>ROUND(($F$23-$F$13)^((A20-$A$13)/10)+$F$13,0)</ns0:f>
-        <ns0:v>27151.0</ns0:v>
+          <ns0:t>{30171|0.100000,30172|0.200000,30173|0.300000,30174|0.400000,30175|0.500000,30176|0.600000,30177|0.700000,30178|0.800000,30179|0.900000}</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D20" s="1" t="n">
+        <ns0:v>904415825815.2517</ns0:v>
+      </ns0:c>
+      <ns0:c r="E20" s="1" t="n">
+        <ns0:v>904415825815.2517</ns0:v>
+      </ns0:c>
+      <ns0:c r="F20" s="1" t="n">
+        <ns0:v>28308996732.09452</ns0:v>
       </ns0:c>
       <ns0:c r="G20" s="1" t="n">
         <ns0:v>4.2</ns0:v>
       </ns0:c>
       <ns0:c r="H20" s="1" t="n">
-        <ns0:v>1</ns0:v>
+        <ns0:v>0</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="21">
@@ -1760,26 +1739,23 @@
       </ns0:c>
       <ns0:c r="C21" s="1" t="inlineStr">
         <ns0:is>
-          <ns0:t>{5|0.1,5|0.2,12|0.3,5|0.4,9|0.5,5|0.6,12|0.7,5|0.8,13|0.9}</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="D21" s="1">
-        <ns0:f>ROUND(($D$23-$D$13)^((A21-$A$13)/10)+$D$13,0)</ns0:f>
-        <ns0:v>100055897.0</ns0:v>
-      </ns0:c>
-      <ns0:c r="E21" s="1">
-        <ns0:f>D21</ns0:f>
-        <ns0:v>100055897.0</ns0:v>
-      </ns0:c>
-      <ns0:c r="F21" s="1">
-        <ns0:f>ROUND(($F$23-$F$13)^((A21-$A$13)/10)+$F$13,0)</ns0:f>
-        <ns0:v>52850.0</ns0:v>
+          <ns0:t>{30181|0.100000,30182|0.200000,30183|0.300000,30184|0.400000,30185|0.500000,30186|0.600000,30187|0.700000,30188|0.800000,30189|0.900000}</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D21" s="1" t="n">
+        <ns0:v>9676634819953.418</ns0:v>
+      </ns0:c>
+      <ns0:c r="E21" s="1" t="n">
+        <ns0:v>9676634819953.418</ns0:v>
+      </ns0:c>
+      <ns0:c r="F21" s="1" t="n">
+        <ns0:v>302887030143.2465</ns0:v>
       </ns0:c>
       <ns0:c r="G21" s="1" t="n">
         <ns0:v>4.4</ns0:v>
       </ns0:c>
       <ns0:c r="H21" s="1" t="n">
-        <ns0:v>1</ns0:v>
+        <ns0:v>0</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="22">
@@ -1791,26 +1767,23 @@
       </ns0:c>
       <ns0:c r="C22" s="1" t="inlineStr">
         <ns0:is>
-          <ns0:t>{4|0.1,4|0.2,11|0.3,4|0.4,10|0.5,4|0.6,11|0.7,4|0.8,14|0.9}</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="D22" s="1">
-        <ns0:f>ROUND(($D$23-$D$13)^((A22-$A$13)/10)+$D$13,0)</ns0:f>
-        <ns0:v>1000051276.0</ns0:v>
-      </ns0:c>
-      <ns0:c r="E22" s="1">
-        <ns0:f>D22</ns0:f>
-        <ns0:v>1000051276.0</ns0:v>
-      </ns0:c>
-      <ns0:c r="F22" s="1">
-        <ns0:f>ROUND(($F$23-$F$13)^((A22-$A$13)/10)+$F$13,0)</ns0:f>
-        <ns0:v>147965.0</ns0:v>
+          <ns0:t>{30191|0.100000,30192|0.200000,30193|0.300000,30194|0.400000,30195|0.500000,30196|0.600000,30197|0.700000,30198|0.800000,30199|0.900000}</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D22" s="1" t="n">
+        <ns0:v>103533417666955.5</ns0:v>
+      </ns0:c>
+      <ns0:c r="E22" s="1" t="n">
+        <ns0:v>103533417666955.5</ns0:v>
+      </ns0:c>
+      <ns0:c r="F22" s="1" t="n">
+        <ns0:v>3240685422277.354</ns0:v>
       </ns0:c>
       <ns0:c r="G22" s="1" t="n">
         <ns0:v>4.6</ns0:v>
       </ns0:c>
       <ns0:c r="H22" s="1" t="n">
-        <ns0:v>1</ns0:v>
+        <ns0:v>0</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="23">
@@ -1822,23 +1795,23 @@
       </ns0:c>
       <ns0:c r="C23" s="1" t="inlineStr">
         <ns0:is>
-          <ns0:t>{3|0.1,3|0.2,6|0.3,7|0.4,8|0.5,13|0.6,14|0.7,8|0.8,15|0.9}</ns0:t>
+          <ns0:t>{30201|0.100000,30202|0.200000,30203|0.300000,30204|0.400000,30205|0.500000,30206|0.600000,30207|0.700000,30208|0.800000,30209|0.900000}</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="D23" s="1" t="n">
-        <ns0:v>10000000000</ns0:v>
+        <ns0:v>1107737222003781</ns0:v>
       </ns0:c>
       <ns0:c r="E23" s="1" t="n">
-        <ns0:v>10000000000</ns0:v>
+        <ns0:v>1107737222003781</ns0:v>
       </ns0:c>
       <ns0:c r="F23" s="1" t="n">
-        <ns0:v>500000</ns0:v>
+        <ns0:v>34673132095468.54</ns0:v>
       </ns0:c>
       <ns0:c r="G23" s="1" t="n">
         <ns0:v>4.8</ns0:v>
       </ns0:c>
       <ns0:c r="H23" s="1" t="n">
-        <ns0:v>1</ns0:v>
+        <ns0:v>0</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="24">
@@ -1855,15 +1828,15 @@
       </ns0:c>
       <ns0:c r="D24" s="1">
         <ns0:f>ROUND(D23*10,0)</ns0:f>
-        <ns0:v>100000000000</ns0:v>
+        <ns0:v>1.1077372220037806e+16</ns0:v>
       </ns0:c>
       <ns0:c r="E24" s="1">
         <ns0:f>D24</ns0:f>
-        <ns0:v>100000000000</ns0:v>
+        <ns0:v>1.1077372220037806e+16</ns0:v>
       </ns0:c>
       <ns0:c r="F24" s="1">
         <ns0:f>ROUND(F23*1.4,-5)</ns0:f>
-        <ns0:v>700000</ns0:v>
+        <ns0:v>48542384899999.99</ns0:v>
       </ns0:c>
       <ns0:c r="G24" s="1" t="n">
         <ns0:v>5</ns0:v>
@@ -1886,15 +1859,15 @@
       </ns0:c>
       <ns0:c r="D25" s="1">
         <ns0:f>ROUND(D24*10,0)</ns0:f>
-        <ns0:v>1000000000000</ns0:v>
+        <ns0:v>1.1077372220037806e+17</ns0:v>
       </ns0:c>
       <ns0:c r="E25" s="1">
         <ns0:f>D25</ns0:f>
-        <ns0:v>1000000000000</ns0:v>
+        <ns0:v>1.1077372220037806e+17</ns0:v>
       </ns0:c>
       <ns0:c r="F25" s="1">
         <ns0:f>ROUND(F24*1.4,-5)</ns0:f>
-        <ns0:v>1000000</ns0:v>
+        <ns0:v>67959338899999.99</ns0:v>
       </ns0:c>
       <ns0:c r="G25" s="1" t="n">
         <ns0:v>5.2</ns0:v>
@@ -1917,15 +1890,15 @@
       </ns0:c>
       <ns0:c r="D26" s="1">
         <ns0:f>ROUND(D25*10,0)</ns0:f>
-        <ns0:v>10000000000000</ns0:v>
+        <ns0:v>1.1077372220037806e+18</ns0:v>
       </ns0:c>
       <ns0:c r="E26" s="1">
         <ns0:f>D26</ns0:f>
-        <ns0:v>10000000000000</ns0:v>
+        <ns0:v>1.1077372220037806e+18</ns0:v>
       </ns0:c>
       <ns0:c r="F26" s="1">
         <ns0:f>ROUND(F25*1.4,-5)</ns0:f>
-        <ns0:v>1400000</ns0:v>
+        <ns0:v>95143074500000.0</ns0:v>
       </ns0:c>
       <ns0:c r="G26" s="1" t="n">
         <ns0:v>5.4</ns0:v>
@@ -1948,15 +1921,15 @@
       </ns0:c>
       <ns0:c r="D27" s="1">
         <ns0:f>ROUND(D26*10,0)</ns0:f>
-        <ns0:v>100000000000000</ns0:v>
+        <ns0:v>1.1077372220037806e+19</ns0:v>
       </ns0:c>
       <ns0:c r="E27" s="1">
         <ns0:f>D27</ns0:f>
-        <ns0:v>100000000000000</ns0:v>
+        <ns0:v>1.1077372220037806e+19</ns0:v>
       </ns0:c>
       <ns0:c r="F27" s="1">
         <ns0:f>ROUND(F26*1.4,-5)</ns0:f>
-        <ns0:v>2000000</ns0:v>
+        <ns0:v>133200304299999.98</ns0:v>
       </ns0:c>
       <ns0:c r="G27" s="1" t="n">
         <ns0:v>5.6</ns0:v>
@@ -1979,15 +1952,15 @@
       </ns0:c>
       <ns0:c r="D28" s="1">
         <ns0:f>ROUND(D27*10,0)</ns0:f>
-        <ns0:v>1000000000000000</ns0:v>
+        <ns0:v>1.1077372220037806e+20</ns0:v>
       </ns0:c>
       <ns0:c r="E28" s="1">
         <ns0:f>D28</ns0:f>
-        <ns0:v>1000000000000000</ns0:v>
+        <ns0:v>1.1077372220037806e+20</ns0:v>
       </ns0:c>
       <ns0:c r="F28" s="1">
         <ns0:f>ROUND(F27*1.4,-5)</ns0:f>
-        <ns0:v>2800000</ns0:v>
+        <ns0:v>186480426000000.0</ns0:v>
       </ns0:c>
       <ns0:c r="G28" s="1" t="n">
         <ns0:v>5.8</ns0:v>
@@ -2010,15 +1983,15 @@
       </ns0:c>
       <ns0:c r="D29" s="1">
         <ns0:f>ROUND(D28*10,0)</ns0:f>
-        <ns0:v>1e+16</ns0:v>
+        <ns0:v>1.1077372220037806e+21</ns0:v>
       </ns0:c>
       <ns0:c r="E29" s="1">
         <ns0:f>D29</ns0:f>
-        <ns0:v>1e+16</ns0:v>
+        <ns0:v>1.1077372220037806e+21</ns0:v>
       </ns0:c>
       <ns0:c r="F29" s="1">
         <ns0:f>ROUND(F28*1.4,-5)</ns0:f>
-        <ns0:v>3900000</ns0:v>
+        <ns0:v>261072596399999.97</ns0:v>
       </ns0:c>
       <ns0:c r="G29" s="1" t="n">
         <ns0:v>6</ns0:v>
@@ -2041,15 +2014,15 @@
       </ns0:c>
       <ns0:c r="D30" s="1">
         <ns0:f>ROUND(D29*10,0)</ns0:f>
-        <ns0:v>1e+17</ns0:v>
+        <ns0:v>1.1077372220037805e+22</ns0:v>
       </ns0:c>
       <ns0:c r="E30" s="1">
         <ns0:f>D30</ns0:f>
-        <ns0:v>1e+17</ns0:v>
+        <ns0:v>1.1077372220037805e+22</ns0:v>
       </ns0:c>
       <ns0:c r="F30" s="1">
         <ns0:f>ROUND(F29*1.4,-5)</ns0:f>
-        <ns0:v>5500000</ns0:v>
+        <ns0:v>365501635000000.0</ns0:v>
       </ns0:c>
       <ns0:c r="G30" s="1" t="n">
         <ns0:v>6.2</ns0:v>
@@ -2072,15 +2045,15 @@
       </ns0:c>
       <ns0:c r="D31" s="1">
         <ns0:f>ROUND(D30*10,0)</ns0:f>
-        <ns0:v>1e+18</ns0:v>
+        <ns0:v>1.1077372220037805e+23</ns0:v>
       </ns0:c>
       <ns0:c r="E31" s="1">
         <ns0:f>D31</ns0:f>
-        <ns0:v>1e+18</ns0:v>
+        <ns0:v>1.1077372220037805e+23</ns0:v>
       </ns0:c>
       <ns0:c r="F31" s="1">
         <ns0:f>ROUND(F30*1.4,-5)</ns0:f>
-        <ns0:v>7700000</ns0:v>
+        <ns0:v>511702288999999.94</ns0:v>
       </ns0:c>
       <ns0:c r="G31" s="1" t="n">
         <ns0:v>6.4</ns0:v>
@@ -2103,15 +2076,15 @@
       </ns0:c>
       <ns0:c r="D32" s="1">
         <ns0:f>ROUND(D31*10,0)</ns0:f>
-        <ns0:v>1e+19</ns0:v>
+        <ns0:v>1.1077372220037805e+24</ns0:v>
       </ns0:c>
       <ns0:c r="E32" s="1">
         <ns0:f>D32</ns0:f>
-        <ns0:v>1e+19</ns0:v>
+        <ns0:v>1.1077372220037805e+24</ns0:v>
       </ns0:c>
       <ns0:c r="F32" s="1">
         <ns0:f>ROUND(F31*1.4,-5)</ns0:f>
-        <ns0:v>10800000</ns0:v>
+        <ns0:v>716383204600000.0</ns0:v>
       </ns0:c>
       <ns0:c r="G32" s="1" t="n">
         <ns0:v>6.6</ns0:v>
@@ -2134,15 +2107,15 @@
       </ns0:c>
       <ns0:c r="D33" s="1">
         <ns0:f>ROUND(D32*10,0)</ns0:f>
-        <ns0:v>1e+20</ns0:v>
+        <ns0:v>1.1077372220037805e+25</ns0:v>
       </ns0:c>
       <ns0:c r="E33" s="1">
         <ns0:f>D33</ns0:f>
-        <ns0:v>1e+20</ns0:v>
+        <ns0:v>1.1077372220037805e+25</ns0:v>
       </ns0:c>
       <ns0:c r="F33" s="1">
         <ns0:f>ROUND(F32*1.4,-5)</ns0:f>
-        <ns0:v>15100000</ns0:v>
+        <ns0:v>1002936486399999.9</ns0:v>
       </ns0:c>
       <ns0:c r="G33" s="1" t="n">
         <ns0:v>6.8</ns0:v>
@@ -2165,15 +2138,15 @@
       </ns0:c>
       <ns0:c r="D34" s="1">
         <ns0:f>ROUND(D33*10,0)</ns0:f>
-        <ns0:v>1e+21</ns0:v>
+        <ns0:v>1.1077372220037805e+26</ns0:v>
       </ns0:c>
       <ns0:c r="E34" s="1">
         <ns0:f>D34</ns0:f>
-        <ns0:v>1e+21</ns0:v>
+        <ns0:v>1.1077372220037805e+26</ns0:v>
       </ns0:c>
       <ns0:c r="F34" s="1">
         <ns0:f>ROUND(F33*1.4,-5)</ns0:f>
-        <ns0:v>21100000</ns0:v>
+        <ns0:v>1404111081000000.0</ns0:v>
       </ns0:c>
       <ns0:c r="G34" s="1" t="n">
         <ns0:v>7</ns0:v>
@@ -2196,15 +2169,15 @@
       </ns0:c>
       <ns0:c r="D35" s="1">
         <ns0:f>ROUND(D34*10,0)</ns0:f>
-        <ns0:v>1e+22</ns0:v>
+        <ns0:v>1.1077372220037804e+27</ns0:v>
       </ns0:c>
       <ns0:c r="E35" s="1">
         <ns0:f>D35</ns0:f>
-        <ns0:v>1e+22</ns0:v>
+        <ns0:v>1.1077372220037804e+27</ns0:v>
       </ns0:c>
       <ns0:c r="F35" s="1">
         <ns0:f>ROUND(F34*1.4,-5)</ns0:f>
-        <ns0:v>29500000</ns0:v>
+        <ns0:v>1965755513399999.8</ns0:v>
       </ns0:c>
       <ns0:c r="G35" s="1" t="n">
         <ns0:v>7.2</ns0:v>
@@ -2227,15 +2200,15 @@
       </ns0:c>
       <ns0:c r="D36" s="1">
         <ns0:f>ROUND(D35*10,0)</ns0:f>
-        <ns0:v>1e+23</ns0:v>
+        <ns0:v>1.1077372220037803e+28</ns0:v>
       </ns0:c>
       <ns0:c r="E36" s="1">
         <ns0:f>D36</ns0:f>
-        <ns0:v>1e+23</ns0:v>
+        <ns0:v>1.1077372220037803e+28</ns0:v>
       </ns0:c>
       <ns0:c r="F36" s="1">
         <ns0:f>ROUND(F35*1.4,-5)</ns0:f>
-        <ns0:v>41300000</ns0:v>
+        <ns0:v>2752057718800000.0</ns0:v>
       </ns0:c>
       <ns0:c r="G36" s="1" t="n">
         <ns0:v>7.4</ns0:v>
@@ -2258,15 +2231,15 @@
       </ns0:c>
       <ns0:c r="D37" s="1">
         <ns0:f>ROUND(D36*10,0)</ns0:f>
-        <ns0:v>1e+24</ns0:v>
+        <ns0:v>1.1077372220037803e+29</ns0:v>
       </ns0:c>
       <ns0:c r="E37" s="1">
         <ns0:f>D37</ns0:f>
-        <ns0:v>1e+24</ns0:v>
+        <ns0:v>1.1077372220037803e+29</ns0:v>
       </ns0:c>
       <ns0:c r="F37" s="1">
         <ns0:f>ROUND(F36*1.4,-5)</ns0:f>
-        <ns0:v>57800000</ns0:v>
+        <ns0:v>3852880806299999.5</ns0:v>
       </ns0:c>
       <ns0:c r="G37" s="1" t="n">
         <ns0:v>7.6</ns0:v>
@@ -2289,15 +2262,15 @@
       </ns0:c>
       <ns0:c r="D38" s="1">
         <ns0:f>ROUND(D37*10,0)</ns0:f>
-        <ns0:v>1e+25</ns0:v>
+        <ns0:v>1.1077372220037803e+30</ns0:v>
       </ns0:c>
       <ns0:c r="E38" s="1">
         <ns0:f>D38</ns0:f>
-        <ns0:v>1e+25</ns0:v>
+        <ns0:v>1.1077372220037803e+30</ns0:v>
       </ns0:c>
       <ns0:c r="F38" s="1">
         <ns0:f>ROUND(F37*1.4,-5)</ns0:f>
-        <ns0:v>80900000</ns0:v>
+        <ns0:v>5394033128800000.0</ns0:v>
       </ns0:c>
       <ns0:c r="G38" s="1" t="n">
         <ns0:v>7.8</ns0:v>
@@ -2320,15 +2293,15 @@
       </ns0:c>
       <ns0:c r="D39" s="1">
         <ns0:f>ROUND(D38*10,0)</ns0:f>
-        <ns0:v>1e+26</ns0:v>
+        <ns0:v>1.1077372220037803e+31</ns0:v>
       </ns0:c>
       <ns0:c r="E39" s="1">
         <ns0:f>D39</ns0:f>
-        <ns0:v>1e+26</ns0:v>
+        <ns0:v>1.1077372220037803e+31</ns0:v>
       </ns0:c>
       <ns0:c r="F39" s="1">
         <ns0:f>ROUND(F38*1.4,-5)</ns0:f>
-        <ns0:v>113300000</ns0:v>
+        <ns0:v>7551646380299999.0</ns0:v>
       </ns0:c>
       <ns0:c r="G39" s="1" t="n">
         <ns0:v>8</ns0:v>
@@ -2351,15 +2324,15 @@
       </ns0:c>
       <ns0:c r="D40" s="1">
         <ns0:f>ROUND(D39*10,0)</ns0:f>
-        <ns0:v>1e+27</ns0:v>
+        <ns0:v>1.1077372220037804e+32</ns0:v>
       </ns0:c>
       <ns0:c r="E40" s="1">
         <ns0:f>D40</ns0:f>
-        <ns0:v>1e+27</ns0:v>
+        <ns0:v>1.1077372220037804e+32</ns0:v>
       </ns0:c>
       <ns0:c r="F40" s="1">
         <ns0:f>ROUND(F39*1.4,-5)</ns0:f>
-        <ns0:v>158600000</ns0:v>
+        <ns0:v>1.05723049324e+16</ns0:v>
       </ns0:c>
       <ns0:c r="G40" s="1" t="n">
         <ns0:v>8.199999999999999</ns0:v>
@@ -2382,15 +2355,15 @@
       </ns0:c>
       <ns0:c r="D41" s="1">
         <ns0:f>ROUND(D40*10,0)</ns0:f>
-        <ns0:v>1e+28</ns0:v>
+        <ns0:v>1.1077372220037804e+33</ns0:v>
       </ns0:c>
       <ns0:c r="E41" s="1">
         <ns0:f>D41</ns0:f>
-        <ns0:v>1e+28</ns0:v>
+        <ns0:v>1.1077372220037804e+33</ns0:v>
       </ns0:c>
       <ns0:c r="F41" s="1">
         <ns0:f>ROUND(F40*1.4,-5)</ns0:f>
-        <ns0:v>222000000</ns0:v>
+        <ns0:v>1.4801226905399998e+16</ns0:v>
       </ns0:c>
       <ns0:c r="G41" s="1" t="n">
         <ns0:v>8.4</ns0:v>
@@ -2413,15 +2386,15 @@
       </ns0:c>
       <ns0:c r="D42" s="1">
         <ns0:f>ROUND(D41*10,0)</ns0:f>
-        <ns0:v>1e+29</ns0:v>
+        <ns0:v>1.1077372220037804e+34</ns0:v>
       </ns0:c>
       <ns0:c r="E42" s="1">
         <ns0:f>D42</ns0:f>
-        <ns0:v>1e+29</ns0:v>
+        <ns0:v>1.1077372220037804e+34</ns0:v>
       </ns0:c>
       <ns0:c r="F42" s="1">
         <ns0:f>ROUND(F41*1.4,-5)</ns0:f>
-        <ns0:v>310800000</ns0:v>
+        <ns0:v>2.07217176676e+16</ns0:v>
       </ns0:c>
       <ns0:c r="G42" s="1" t="n">
         <ns0:v>8.6</ns0:v>
@@ -2444,15 +2417,15 @@
       </ns0:c>
       <ns0:c r="D43" s="1">
         <ns0:f>ROUND(D42*10,0)</ns0:f>
-        <ns0:v>1e+30</ns0:v>
+        <ns0:v>1.1077372220037804e+35</ns0:v>
       </ns0:c>
       <ns0:c r="E43" s="1">
         <ns0:f>D43</ns0:f>
-        <ns0:v>1e+30</ns0:v>
+        <ns0:v>1.1077372220037804e+35</ns0:v>
       </ns0:c>
       <ns0:c r="F43" s="1">
         <ns0:f>ROUND(F42*1.4,-5)</ns0:f>
-        <ns0:v>435100000</ns0:v>
+        <ns0:v>2.9010404734599996e+16</ns0:v>
       </ns0:c>
       <ns0:c r="G43" s="1" t="n">
         <ns0:v>8.800000000000001</ns0:v>
@@ -2475,15 +2448,15 @@
       </ns0:c>
       <ns0:c r="D44" s="1">
         <ns0:f>ROUND(D43*10,0)</ns0:f>
-        <ns0:v>1e+31</ns0:v>
+        <ns0:v>1.1077372220037803e+36</ns0:v>
       </ns0:c>
       <ns0:c r="E44" s="1">
         <ns0:f>D44</ns0:f>
-        <ns0:v>1e+31</ns0:v>
+        <ns0:v>1.1077372220037803e+36</ns0:v>
       </ns0:c>
       <ns0:c r="F44" s="1">
         <ns0:f>ROUND(F43*1.4,-5)</ns0:f>
-        <ns0:v>609100000</ns0:v>
+        <ns0:v>4.06145666284e+16</ns0:v>
       </ns0:c>
       <ns0:c r="G44" s="1" t="n">
         <ns0:v>9</ns0:v>
@@ -2506,15 +2479,15 @@
       </ns0:c>
       <ns0:c r="D45" s="1">
         <ns0:f>ROUND(D44*10,0)</ns0:f>
-        <ns0:v>1e+32</ns0:v>
+        <ns0:v>1.1077372220037803e+37</ns0:v>
       </ns0:c>
       <ns0:c r="E45" s="1">
         <ns0:f>D45</ns0:f>
-        <ns0:v>1e+32</ns0:v>
+        <ns0:v>1.1077372220037803e+37</ns0:v>
       </ns0:c>
       <ns0:c r="F45" s="1">
         <ns0:f>ROUND(F44*1.4,-5)</ns0:f>
-        <ns0:v>852700000</ns0:v>
+        <ns0:v>5.686039327979999e+16</ns0:v>
       </ns0:c>
       <ns0:c r="G45" s="1" t="n">
         <ns0:v>9.199999999999999</ns0:v>
@@ -2537,15 +2510,15 @@
       </ns0:c>
       <ns0:c r="D46" s="1">
         <ns0:f>ROUND(D45*10,0)</ns0:f>
-        <ns0:v>1e+33</ns0:v>
+        <ns0:v>1.1077372220037804e+38</ns0:v>
       </ns0:c>
       <ns0:c r="E46" s="1">
         <ns0:f>D46</ns0:f>
-        <ns0:v>1e+33</ns0:v>
+        <ns0:v>1.1077372220037804e+38</ns0:v>
       </ns0:c>
       <ns0:c r="F46" s="1">
         <ns0:f>ROUND(F45*1.4,-5)</ns0:f>
-        <ns0:v>1193800000</ns0:v>
+        <ns0:v>7.96045505917e+16</ns0:v>
       </ns0:c>
       <ns0:c r="G46" s="1" t="n">
         <ns0:v>9.4</ns0:v>
@@ -2568,15 +2541,15 @@
       </ns0:c>
       <ns0:c r="D47" s="1">
         <ns0:f>ROUND(D46*10,0)</ns0:f>
-        <ns0:v>1e+34</ns0:v>
+        <ns0:v>1.1077372220037804e+39</ns0:v>
       </ns0:c>
       <ns0:c r="E47" s="1">
         <ns0:f>D47</ns0:f>
-        <ns0:v>1e+34</ns0:v>
+        <ns0:v>1.1077372220037804e+39</ns0:v>
       </ns0:c>
       <ns0:c r="F47" s="1">
         <ns0:f>ROUND(F46*1.4,-5)</ns0:f>
-        <ns0:v>1671300000</ns0:v>
+        <ns0:v>1.1144637082839998e+17</ns0:v>
       </ns0:c>
       <ns0:c r="G47" s="1" t="n">
         <ns0:v>9.6</ns0:v>
@@ -2599,15 +2572,15 @@
       </ns0:c>
       <ns0:c r="D48" s="1">
         <ns0:f>ROUND(D47*10,0)</ns0:f>
-        <ns0:v>1e+35</ns0:v>
+        <ns0:v>1.1077372220037803e+40</ns0:v>
       </ns0:c>
       <ns0:c r="E48" s="1">
         <ns0:f>D48</ns0:f>
-        <ns0:v>1e+35</ns0:v>
+        <ns0:v>1.1077372220037803e+40</ns0:v>
       </ns0:c>
       <ns0:c r="F48" s="1">
         <ns0:f>ROUND(F47*1.4,-5)</ns0:f>
-        <ns0:v>2339800000</ns0:v>
+        <ns0:v>1.560249191598e+17</ns0:v>
       </ns0:c>
       <ns0:c r="G48" s="1" t="n">
         <ns0:v>9.800000000000001</ns0:v>
@@ -2630,15 +2603,15 @@
       </ns0:c>
       <ns0:c r="D49" s="1">
         <ns0:f>ROUND(D48*10,0)</ns0:f>
-        <ns0:v>1e+36</ns0:v>
+        <ns0:v>1.1077372220037803e+41</ns0:v>
       </ns0:c>
       <ns0:c r="E49" s="1">
         <ns0:f>D49</ns0:f>
-        <ns0:v>1e+36</ns0:v>
+        <ns0:v>1.1077372220037803e+41</ns0:v>
       </ns0:c>
       <ns0:c r="F49" s="1">
         <ns0:f>ROUND(F48*1.4,-5)</ns0:f>
-        <ns0:v>3275700000</ns0:v>
+        <ns0:v>2.1843488682369997e+17</ns0:v>
       </ns0:c>
       <ns0:c r="G49" s="1" t="n">
         <ns0:v>10</ns0:v>
@@ -2661,15 +2634,15 @@
       </ns0:c>
       <ns0:c r="D50" s="1">
         <ns0:f>ROUND(D49*10,0)</ns0:f>
-        <ns0:v>1e+37</ns0:v>
+        <ns0:v>1.1077372220037803e+42</ns0:v>
       </ns0:c>
       <ns0:c r="E50" s="1">
         <ns0:f>D50</ns0:f>
-        <ns0:v>1e+37</ns0:v>
+        <ns0:v>1.1077372220037803e+42</ns0:v>
       </ns0:c>
       <ns0:c r="F50" s="1">
         <ns0:f>ROUND(F49*1.4,-5)</ns0:f>
-        <ns0:v>4586000000</ns0:v>
+        <ns0:v>3.058088415532e+17</ns0:v>
       </ns0:c>
       <ns0:c r="G50" s="1" t="n">
         <ns0:v>10.2</ns0:v>
@@ -2692,15 +2665,15 @@
       </ns0:c>
       <ns0:c r="D51" s="1">
         <ns0:f>ROUND(D50*10,0)</ns0:f>
-        <ns0:v>1e+38</ns0:v>
+        <ns0:v>1.1077372220037803e+43</ns0:v>
       </ns0:c>
       <ns0:c r="E51" s="1">
         <ns0:f>D51</ns0:f>
-        <ns0:v>1e+38</ns0:v>
+        <ns0:v>1.1077372220037803e+43</ns0:v>
       </ns0:c>
       <ns0:c r="F51" s="1">
         <ns0:f>ROUND(F50*1.4,-5)</ns0:f>
-        <ns0:v>6420400000</ns0:v>
+        <ns0:v>4.281323781745e+17</ns0:v>
       </ns0:c>
       <ns0:c r="G51" s="1" t="n">
         <ns0:v>10.4</ns0:v>
@@ -2723,15 +2696,15 @@
       </ns0:c>
       <ns0:c r="D52" s="1">
         <ns0:f>ROUND(D51*10,0)</ns0:f>
-        <ns0:v>1e+39</ns0:v>
+        <ns0:v>1.1077372220037804e+44</ns0:v>
       </ns0:c>
       <ns0:c r="E52" s="1">
         <ns0:f>D52</ns0:f>
-        <ns0:v>1e+39</ns0:v>
+        <ns0:v>1.1077372220037804e+44</ns0:v>
       </ns0:c>
       <ns0:c r="F52" s="1">
         <ns0:f>ROUND(F51*1.4,-5)</ns0:f>
-        <ns0:v>8988600000</ns0:v>
+        <ns0:v>5.993853294442999e+17</ns0:v>
       </ns0:c>
       <ns0:c r="G52" s="1" t="n">
         <ns0:v>10.6</ns0:v>
@@ -2754,15 +2727,15 @@
       </ns0:c>
       <ns0:c r="D53" s="1">
         <ns0:f>ROUND(D52*10,0)</ns0:f>
-        <ns0:v>1e+40</ns0:v>
+        <ns0:v>1.1077372220037804e+45</ns0:v>
       </ns0:c>
       <ns0:c r="E53" s="1">
         <ns0:f>D53</ns0:f>
-        <ns0:v>1e+40</ns0:v>
+        <ns0:v>1.1077372220037804e+45</ns0:v>
       </ns0:c>
       <ns0:c r="F53" s="1">
         <ns0:f>ROUND(F52*1.4,-5)</ns0:f>
-        <ns0:v>12584000000</ns0:v>
+        <ns0:v>8.391394612219999e+17</ns0:v>
       </ns0:c>
       <ns0:c r="G53" s="1" t="n">
         <ns0:v>10.8</ns0:v>
@@ -2785,15 +2758,15 @@
       </ns0:c>
       <ns0:c r="D54" s="1">
         <ns0:f>ROUND(D53*10,0)</ns0:f>
-        <ns0:v>1e+41</ns0:v>
+        <ns0:v>1.1077372220037804e+46</ns0:v>
       </ns0:c>
       <ns0:c r="E54" s="1">
         <ns0:f>D54</ns0:f>
-        <ns0:v>1e+41</ns0:v>
+        <ns0:v>1.1077372220037804e+46</ns0:v>
       </ns0:c>
       <ns0:c r="F54" s="1">
         <ns0:f>ROUND(F53*1.4,-5)</ns0:f>
-        <ns0:v>17617600000</ns0:v>
+        <ns0:v>1.1747952457108e+18</ns0:v>
       </ns0:c>
       <ns0:c r="G54" s="1" t="n">
         <ns0:v>11</ns0:v>
@@ -2816,15 +2789,15 @@
       </ns0:c>
       <ns0:c r="D55" s="1">
         <ns0:f>ROUND(D54*10,0)</ns0:f>
-        <ns0:v>1e+42</ns0:v>
+        <ns0:v>1.1077372220037803e+47</ns0:v>
       </ns0:c>
       <ns0:c r="E55" s="1">
         <ns0:f>D55</ns0:f>
-        <ns0:v>1e+42</ns0:v>
+        <ns0:v>1.1077372220037803e+47</ns0:v>
       </ns0:c>
       <ns0:c r="F55" s="1">
         <ns0:f>ROUND(F54*1.4,-5)</ns0:f>
-        <ns0:v>24664600000</ns0:v>
+        <ns0:v>1.6447133439951e+18</ns0:v>
       </ns0:c>
       <ns0:c r="G55" s="1" t="n">
         <ns0:v>11.2</ns0:v>
@@ -2847,15 +2820,15 @@
       </ns0:c>
       <ns0:c r="D56" s="1">
         <ns0:f>ROUND(D55*10,0)</ns0:f>
-        <ns0:v>1e+43</ns0:v>
+        <ns0:v>1.1077372220037804e+48</ns0:v>
       </ns0:c>
       <ns0:c r="E56" s="1">
         <ns0:f>D56</ns0:f>
-        <ns0:v>1e+43</ns0:v>
+        <ns0:v>1.1077372220037804e+48</ns0:v>
       </ns0:c>
       <ns0:c r="F56" s="1">
         <ns0:f>ROUND(F55*1.4,-5)</ns0:f>
-        <ns0:v>34530400000</ns0:v>
+        <ns0:v>2.3025986815930998e+18</ns0:v>
       </ns0:c>
       <ns0:c r="G56" s="1" t="n">
         <ns0:v>11.4</ns0:v>
@@ -2878,15 +2851,15 @@
       </ns0:c>
       <ns0:c r="D57" s="1">
         <ns0:f>ROUND(D56*10,0)</ns0:f>
-        <ns0:v>1e+44</ns0:v>
+        <ns0:v>1.1077372220037804e+49</ns0:v>
       </ns0:c>
       <ns0:c r="E57" s="1">
         <ns0:f>D57</ns0:f>
-        <ns0:v>1e+44</ns0:v>
+        <ns0:v>1.1077372220037804e+49</ns0:v>
       </ns0:c>
       <ns0:c r="F57" s="1">
         <ns0:f>ROUND(F56*1.4,-5)</ns0:f>
-        <ns0:v>48342600000</ns0:v>
+        <ns0:v>3.2236381542302996e+18</ns0:v>
       </ns0:c>
       <ns0:c r="G57" s="1" t="n">
         <ns0:v>11.6</ns0:v>
@@ -2909,15 +2882,15 @@
       </ns0:c>
       <ns0:c r="D58" s="1">
         <ns0:f>ROUND(D57*10,0)</ns0:f>
-        <ns0:v>1e+45</ns0:v>
+        <ns0:v>1.1077372220037804e+50</ns0:v>
       </ns0:c>
       <ns0:c r="E58" s="1">
         <ns0:f>D58</ns0:f>
-        <ns0:v>1e+45</ns0:v>
+        <ns0:v>1.1077372220037804e+50</ns0:v>
       </ns0:c>
       <ns0:c r="F58" s="1">
         <ns0:f>ROUND(F57*1.4,-5)</ns0:f>
-        <ns0:v>67679600000</ns0:v>
+        <ns0:v>4.5130934159223997e+18</ns0:v>
       </ns0:c>
       <ns0:c r="G58" s="1" t="n">
         <ns0:v>11.8</ns0:v>
@@ -2940,15 +2913,15 @@
       </ns0:c>
       <ns0:c r="D59" s="1">
         <ns0:f>ROUND(D58*10,0)</ns0:f>
-        <ns0:v>1e+46</ns0:v>
+        <ns0:v>1.1077372220037804e+51</ns0:v>
       </ns0:c>
       <ns0:c r="E59" s="1">
         <ns0:f>D59</ns0:f>
-        <ns0:v>1e+46</ns0:v>
+        <ns0:v>1.1077372220037804e+51</ns0:v>
       </ns0:c>
       <ns0:c r="F59" s="1">
         <ns0:f>ROUND(F58*1.4,-5)</ns0:f>
-        <ns0:v>94751400000</ns0:v>
+        <ns0:v>6.3183307822914e+18</ns0:v>
       </ns0:c>
       <ns0:c r="G59" s="1" t="n">
         <ns0:v>12</ns0:v>
@@ -2971,15 +2944,15 @@
       </ns0:c>
       <ns0:c r="D60" s="1">
         <ns0:f>ROUND(D59*10,0)</ns0:f>
-        <ns0:v>1e+47</ns0:v>
+        <ns0:v>1.1077372220037804e+52</ns0:v>
       </ns0:c>
       <ns0:c r="E60" s="1">
         <ns0:f>D60</ns0:f>
-        <ns0:v>1e+47</ns0:v>
+        <ns0:v>1.1077372220037804e+52</ns0:v>
       </ns0:c>
       <ns0:c r="F60" s="1">
         <ns0:f>ROUND(F59*1.4,-5)</ns0:f>
-        <ns0:v>132652000000</ns0:v>
+        <ns0:v>8.845663095208e+18</ns0:v>
       </ns0:c>
       <ns0:c r="G60" s="1" t="n">
         <ns0:v>12.2</ns0:v>
@@ -3002,15 +2975,15 @@
       </ns0:c>
       <ns0:c r="D61" s="1">
         <ns0:f>ROUND(D60*10,0)</ns0:f>
-        <ns0:v>1e+48</ns0:v>
+        <ns0:v>1.1077372220037804e+53</ns0:v>
       </ns0:c>
       <ns0:c r="E61" s="1">
         <ns0:f>D61</ns0:f>
-        <ns0:v>1e+48</ns0:v>
+        <ns0:v>1.1077372220037804e+53</ns0:v>
       </ns0:c>
       <ns0:c r="F61" s="1">
         <ns0:f>ROUND(F60*1.4,-5)</ns0:f>
-        <ns0:v>185712800000</ns0:v>
+        <ns0:v>1.2383928333291198e+19</ns0:v>
       </ns0:c>
       <ns0:c r="G61" s="1" t="n">
         <ns0:v>12.4</ns0:v>
@@ -3033,15 +3006,15 @@
       </ns0:c>
       <ns0:c r="D62" s="1">
         <ns0:f>ROUND(D61*10,0)</ns0:f>
-        <ns0:v>1e+49</ns0:v>
+        <ns0:v>1.1077372220037804e+54</ns0:v>
       </ns0:c>
       <ns0:c r="E62" s="1">
         <ns0:f>D62</ns0:f>
-        <ns0:v>1e+49</ns0:v>
+        <ns0:v>1.1077372220037804e+54</ns0:v>
       </ns0:c>
       <ns0:c r="F62" s="1">
         <ns0:f>ROUND(F61*1.4,-5)</ns0:f>
-        <ns0:v>259997900000</ns0:v>
+        <ns0:v>1.7337499666607698e+19</ns0:v>
       </ns0:c>
       <ns0:c r="G62" s="1" t="n">
         <ns0:v>12.6</ns0:v>
@@ -3064,15 +3037,15 @@
       </ns0:c>
       <ns0:c r="D63" s="1">
         <ns0:f>ROUND(D62*10,0)</ns0:f>
-        <ns0:v>1e+50</ns0:v>
+        <ns0:v>1.1077372220037803e+55</ns0:v>
       </ns0:c>
       <ns0:c r="E63" s="1">
         <ns0:f>D63</ns0:f>
-        <ns0:v>1e+50</ns0:v>
+        <ns0:v>1.1077372220037803e+55</ns0:v>
       </ns0:c>
       <ns0:c r="F63" s="1">
         <ns0:f>ROUND(F62*1.4,-5)</ns0:f>
-        <ns0:v>363997100000</ns0:v>
+        <ns0:v>2.4272499533250798e+19</ns0:v>
       </ns0:c>
       <ns0:c r="G63" s="1" t="n">
         <ns0:v>12.8</ns0:v>
@@ -3095,15 +3068,15 @@
       </ns0:c>
       <ns0:c r="D64" s="1">
         <ns0:f>ROUND(D63*10,0)</ns0:f>
-        <ns0:v>1e+51</ns0:v>
+        <ns0:v>1.1077372220037803e+56</ns0:v>
       </ns0:c>
       <ns0:c r="E64" s="1">
         <ns0:f>D64</ns0:f>
-        <ns0:v>1e+51</ns0:v>
+        <ns0:v>1.1077372220037803e+56</ns0:v>
       </ns0:c>
       <ns0:c r="F64" s="1">
         <ns0:f>ROUND(F63*1.4,-5)</ns0:f>
-        <ns0:v>509595900000</ns0:v>
+        <ns0:v>3.3981499346551095e+19</ns0:v>
       </ns0:c>
       <ns0:c r="G64" s="1" t="n">
         <ns0:v>13</ns0:v>
@@ -3126,15 +3099,15 @@
       </ns0:c>
       <ns0:c r="D65" s="1">
         <ns0:f>ROUND(D64*10,0)</ns0:f>
-        <ns0:v>1e+52</ns0:v>
+        <ns0:v>1.1077372220037802e+57</ns0:v>
       </ns0:c>
       <ns0:c r="E65" s="1">
         <ns0:f>D65</ns0:f>
-        <ns0:v>1e+52</ns0:v>
+        <ns0:v>1.1077372220037802e+57</ns0:v>
       </ns0:c>
       <ns0:c r="F65" s="1">
         <ns0:f>ROUND(F64*1.4,-5)</ns0:f>
-        <ns0:v>713434300000</ns0:v>
+        <ns0:v>4.75740990851715e+19</ns0:v>
       </ns0:c>
       <ns0:c r="G65" s="1" t="n">
         <ns0:v>13.2</ns0:v>
@@ -3157,15 +3130,15 @@
       </ns0:c>
       <ns0:c r="D66" s="1">
         <ns0:f>ROUND(D65*10,0)</ns0:f>
-        <ns0:v>1e+53</ns0:v>
+        <ns0:v>1.1077372220037802e+58</ns0:v>
       </ns0:c>
       <ns0:c r="E66" s="1">
         <ns0:f>D66</ns0:f>
-        <ns0:v>1e+53</ns0:v>
+        <ns0:v>1.1077372220037802e+58</ns0:v>
       </ns0:c>
       <ns0:c r="F66" s="1">
         <ns0:f>ROUND(F65*1.4,-5)</ns0:f>
-        <ns0:v>998808000000</ns0:v>
+        <ns0:v>6.660373871924009e+19</ns0:v>
       </ns0:c>
       <ns0:c r="G66" s="1" t="n">
         <ns0:v>13.4</ns0:v>
@@ -3188,15 +3161,15 @@
       </ns0:c>
       <ns0:c r="D67" s="1">
         <ns0:f>ROUND(D66*10,0)</ns0:f>
-        <ns0:v>1e+54</ns0:v>
+        <ns0:v>1.1077372220037803e+59</ns0:v>
       </ns0:c>
       <ns0:c r="E67" s="1">
         <ns0:f>D67</ns0:f>
-        <ns0:v>1e+54</ns0:v>
+        <ns0:v>1.1077372220037803e+59</ns0:v>
       </ns0:c>
       <ns0:c r="F67" s="1">
         <ns0:f>ROUND(F66*1.4,-5)</ns0:f>
-        <ns0:v>1398331200000</ns0:v>
+        <ns0:v>9.324523420693609e+19</ns0:v>
       </ns0:c>
       <ns0:c r="G67" s="1" t="n">
         <ns0:v>13.6</ns0:v>
@@ -3219,15 +3192,15 @@
       </ns0:c>
       <ns0:c r="D68" s="1">
         <ns0:f>ROUND(D67*10,0)</ns0:f>
-        <ns0:v>1e+55</ns0:v>
+        <ns0:v>1.1077372220037803e+60</ns0:v>
       </ns0:c>
       <ns0:c r="E68" s="1">
         <ns0:f>D68</ns0:f>
-        <ns0:v>1e+55</ns0:v>
+        <ns0:v>1.1077372220037803e+60</ns0:v>
       </ns0:c>
       <ns0:c r="F68" s="1">
         <ns0:f>ROUND(F67*1.4,-5)</ns0:f>
-        <ns0:v>1957663700000</ns0:v>
+        <ns0:v>1.3054332788971048e+20</ns0:v>
       </ns0:c>
       <ns0:c r="G68" s="1" t="n">
         <ns0:v>13.8</ns0:v>
@@ -3250,15 +3223,15 @@
       </ns0:c>
       <ns0:c r="D69" s="1">
         <ns0:f>ROUND(D68*10,0)</ns0:f>
-        <ns0:v>1e+56</ns0:v>
+        <ns0:v>1.1077372220037802e+61</ns0:v>
       </ns0:c>
       <ns0:c r="E69" s="1">
         <ns0:f>D69</ns0:f>
-        <ns0:v>1e+56</ns0:v>
+        <ns0:v>1.1077372220037802e+61</ns0:v>
       </ns0:c>
       <ns0:c r="F69" s="1">
         <ns0:f>ROUND(F68*1.4,-5)</ns0:f>
-        <ns0:v>2740729200000</ns0:v>
+        <ns0:v>1.827606590455947e+20</ns0:v>
       </ns0:c>
       <ns0:c r="G69" s="1" t="n">
         <ns0:v>14</ns0:v>
@@ -3281,15 +3254,15 @@
       </ns0:c>
       <ns0:c r="D70" s="1">
         <ns0:f>ROUND(D69*10,0)</ns0:f>
-        <ns0:v>1e+57</ns0:v>
+        <ns0:v>1.1077372220037803e+62</ns0:v>
       </ns0:c>
       <ns0:c r="E70" s="1">
         <ns0:f>D70</ns0:f>
-        <ns0:v>1e+57</ns0:v>
+        <ns0:v>1.1077372220037803e+62</ns0:v>
       </ns0:c>
       <ns0:c r="F70" s="1">
         <ns0:f>ROUND(F69*1.4,-5)</ns0:f>
-        <ns0:v>3837020900000</ns0:v>
+        <ns0:v>2.558649226638326e+20</ns0:v>
       </ns0:c>
       <ns0:c r="G70" s="1" t="n">
         <ns0:v>14.2</ns0:v>
@@ -3312,15 +3285,15 @@
       </ns0:c>
       <ns0:c r="D71" s="1">
         <ns0:f>ROUND(D70*10,0)</ns0:f>
-        <ns0:v>1e+58</ns0:v>
+        <ns0:v>1.1077372220037803e+63</ns0:v>
       </ns0:c>
       <ns0:c r="E71" s="1">
         <ns0:f>D71</ns0:f>
-        <ns0:v>1e+58</ns0:v>
+        <ns0:v>1.1077372220037803e+63</ns0:v>
       </ns0:c>
       <ns0:c r="F71" s="1">
         <ns0:f>ROUND(F70*1.4,-5)</ns0:f>
-        <ns0:v>5371829300000</ns0:v>
+        <ns0:v>3.5821089172936557e+20</ns0:v>
       </ns0:c>
       <ns0:c r="G71" s="1" t="n">
         <ns0:v>14.4</ns0:v>
@@ -3343,15 +3316,15 @@
       </ns0:c>
       <ns0:c r="D72" s="1">
         <ns0:f>ROUND(D71*10,0)</ns0:f>
-        <ns0:v>1e+59</ns0:v>
+        <ns0:v>1.1077372220037803e+64</ns0:v>
       </ns0:c>
       <ns0:c r="E72" s="1">
         <ns0:f>D72</ns0:f>
-        <ns0:v>1e+59</ns0:v>
+        <ns0:v>1.1077372220037803e+64</ns0:v>
       </ns0:c>
       <ns0:c r="F72" s="1">
         <ns0:f>ROUND(F71*1.4,-5)</ns0:f>
-        <ns0:v>7520561000000</ns0:v>
+        <ns0:v>5.014952484211118e+20</ns0:v>
       </ns0:c>
       <ns0:c r="G72" s="1" t="n">
         <ns0:v>14.6</ns0:v>
@@ -3374,15 +3347,15 @@
       </ns0:c>
       <ns0:c r="D73" s="1">
         <ns0:f>ROUND(D72*10,0)</ns0:f>
-        <ns0:v>1e+60</ns0:v>
+        <ns0:v>1.1077372220037803e+65</ns0:v>
       </ns0:c>
       <ns0:c r="E73" s="1">
         <ns0:f>D73</ns0:f>
-        <ns0:v>1e+60</ns0:v>
+        <ns0:v>1.1077372220037803e+65</ns0:v>
       </ns0:c>
       <ns0:c r="F73" s="1">
         <ns0:f>ROUND(F72*1.4,-5)</ns0:f>
-        <ns0:v>10528785400000</ns0:v>
+        <ns0:v>7.020933477895565e+20</ns0:v>
       </ns0:c>
       <ns0:c r="G73" s="1" t="n">
         <ns0:v>14.8</ns0:v>
@@ -3405,15 +3378,15 @@
       </ns0:c>
       <ns0:c r="D74" s="1">
         <ns0:f>ROUND(D73*10,0)</ns0:f>
-        <ns0:v>1e+61</ns0:v>
+        <ns0:v>1.1077372220037803e+66</ns0:v>
       </ns0:c>
       <ns0:c r="E74" s="1">
         <ns0:f>D74</ns0:f>
-        <ns0:v>1e+61</ns0:v>
+        <ns0:v>1.1077372220037803e+66</ns0:v>
       </ns0:c>
       <ns0:c r="F74" s="1">
         <ns0:f>ROUND(F73*1.4,-5)</ns0:f>
-        <ns0:v>14740299600000</ns0:v>
+        <ns0:v>9.82930686905379e+20</ns0:v>
       </ns0:c>
       <ns0:c r="G74" s="1" t="n">
         <ns0:v>15</ns0:v>
@@ -3437,15 +3410,15 @@
       </ns0:c>
       <ns0:c r="D75" s="1">
         <ns0:f>ROUND(D74*10,0)</ns0:f>
-        <ns0:v>1e+62</ns0:v>
+        <ns0:v>1.1077372220037803e+67</ns0:v>
       </ns0:c>
       <ns0:c r="E75" s="1">
         <ns0:f>D75</ns0:f>
-        <ns0:v>1e+62</ns0:v>
+        <ns0:v>1.1077372220037803e+67</ns0:v>
       </ns0:c>
       <ns0:c r="F75" s="1">
         <ns0:f>ROUND(F74*1.4,-5)</ns0:f>
-        <ns0:v>20636419400000</ns0:v>
+        <ns0:v>1.3761029616675306e+21</ns0:v>
       </ns0:c>
       <ns0:c r="G75" s="1" t="n">
         <ns0:v>15.2</ns0:v>
@@ -3469,15 +3442,15 @@
       </ns0:c>
       <ns0:c r="D76" s="1">
         <ns0:f>ROUND(D75*10,0)</ns0:f>
-        <ns0:v>1e+63</ns0:v>
+        <ns0:v>1.1077372220037802e+68</ns0:v>
       </ns0:c>
       <ns0:c r="E76" s="1">
         <ns0:f>D76</ns0:f>
-        <ns0:v>1e+63</ns0:v>
+        <ns0:v>1.1077372220037802e+68</ns0:v>
       </ns0:c>
       <ns0:c r="F76" s="1">
         <ns0:f>ROUND(F75*1.4,-5)</ns0:f>
-        <ns0:v>28890987200000</ns0:v>
+        <ns0:v>1.9265441463345427e+21</ns0:v>
       </ns0:c>
       <ns0:c r="G76" s="1" t="n">
         <ns0:v>15.4</ns0:v>
@@ -3501,15 +3474,15 @@
       </ns0:c>
       <ns0:c r="D77" s="1">
         <ns0:f>ROUND(D76*10,0)</ns0:f>
-        <ns0:v>1e+64</ns0:v>
+        <ns0:v>1.1077372220037801e+69</ns0:v>
       </ns0:c>
       <ns0:c r="E77" s="1">
         <ns0:f>D77</ns0:f>
-        <ns0:v>1e+64</ns0:v>
+        <ns0:v>1.1077372220037801e+69</ns0:v>
       </ns0:c>
       <ns0:c r="F77" s="1">
         <ns0:f>ROUND(F76*1.4,-5)</ns0:f>
-        <ns0:v>40447382100000</ns0:v>
+        <ns0:v>2.69716180486836e+21</ns0:v>
       </ns0:c>
       <ns0:c r="G77" s="1" t="n">
         <ns0:v>15.6</ns0:v>
@@ -3533,15 +3506,15 @@
       </ns0:c>
       <ns0:c r="D78" s="1">
         <ns0:f>ROUND(D77*10,0)</ns0:f>
-        <ns0:v>1e+65</ns0:v>
+        <ns0:v>1.1077372220037801e+70</ns0:v>
       </ns0:c>
       <ns0:c r="E78" s="1">
         <ns0:f>D78</ns0:f>
-        <ns0:v>1e+65</ns0:v>
+        <ns0:v>1.1077372220037801e+70</ns0:v>
       </ns0:c>
       <ns0:c r="F78" s="1">
         <ns0:f>ROUND(F77*1.4,-5)</ns0:f>
-        <ns0:v>56626334900000</ns0:v>
+        <ns0:v>3.7760265268157035e+21</ns0:v>
       </ns0:c>
       <ns0:c r="G78" s="1" t="n">
         <ns0:v>15.8</ns0:v>
@@ -3565,15 +3538,15 @@
       </ns0:c>
       <ns0:c r="D79" s="1">
         <ns0:f>ROUND(D78*10,0)</ns0:f>
-        <ns0:v>1e+66</ns0:v>
+        <ns0:v>1.10773722200378e+71</ns0:v>
       </ns0:c>
       <ns0:c r="E79" s="1">
         <ns0:f>D79</ns0:f>
-        <ns0:v>1e+66</ns0:v>
+        <ns0:v>1.10773722200378e+71</ns0:v>
       </ns0:c>
       <ns0:c r="F79" s="1">
         <ns0:f>ROUND(F78*1.4,-5)</ns0:f>
-        <ns0:v>79276868900000</ns0:v>
+        <ns0:v>5.286437137541984e+21</ns0:v>
       </ns0:c>
       <ns0:c r="G79" s="1" t="n">
         <ns0:v>16</ns0:v>
@@ -3597,15 +3570,15 @@
       </ns0:c>
       <ns0:c r="D80" s="1">
         <ns0:f>ROUND(D79*10,0)</ns0:f>
-        <ns0:v>1e+67</ns0:v>
+        <ns0:v>1.1077372220037801e+72</ns0:v>
       </ns0:c>
       <ns0:c r="E80" s="1">
         <ns0:f>D80</ns0:f>
-        <ns0:v>1e+67</ns0:v>
+        <ns0:v>1.1077372220037801e+72</ns0:v>
       </ns0:c>
       <ns0:c r="F80" s="1">
         <ns0:f>ROUND(F79*1.4,-5)</ns0:f>
-        <ns0:v>110987616500000</ns0:v>
+        <ns0:v>7.401011992558778e+21</ns0:v>
       </ns0:c>
       <ns0:c r="G80" s="1" t="n">
         <ns0:v>16.2</ns0:v>
@@ -3629,15 +3602,15 @@
       </ns0:c>
       <ns0:c r="D81" s="1">
         <ns0:f>ROUND(D80*10,0)</ns0:f>
-        <ns0:v>1e+68</ns0:v>
+        <ns0:v>1.10773722200378e+73</ns0:v>
       </ns0:c>
       <ns0:c r="E81" s="1">
         <ns0:f>D81</ns0:f>
-        <ns0:v>1e+68</ns0:v>
+        <ns0:v>1.10773722200378e+73</ns0:v>
       </ns0:c>
       <ns0:c r="F81" s="1">
         <ns0:f>ROUND(F80*1.4,-5)</ns0:f>
-        <ns0:v>155382663100000</ns0:v>
+        <ns0:v>1.0361416789582288e+22</ns0:v>
       </ns0:c>
       <ns0:c r="G81" s="1" t="n">
         <ns0:v>16.4</ns0:v>
@@ -3661,15 +3634,15 @@
       </ns0:c>
       <ns0:c r="D82" s="1">
         <ns0:f>ROUND(D81*10,0)</ns0:f>
-        <ns0:v>1e+69</ns0:v>
+        <ns0:v>1.1077372220037801e+74</ns0:v>
       </ns0:c>
       <ns0:c r="E82" s="1">
         <ns0:f>D82</ns0:f>
-        <ns0:v>1e+69</ns0:v>
+        <ns0:v>1.1077372220037801e+74</ns0:v>
       </ns0:c>
       <ns0:c r="F82" s="1">
         <ns0:f>ROUND(F81*1.4,-5)</ns0:f>
-        <ns0:v>217535728300000</ns0:v>
+        <ns0:v>1.4505983505415201e+22</ns0:v>
       </ns0:c>
       <ns0:c r="G82" s="1" t="n">
         <ns0:v>16.6</ns0:v>
@@ -3693,15 +3666,15 @@
       </ns0:c>
       <ns0:c r="D83" s="1">
         <ns0:f>ROUND(D82*10,0)</ns0:f>
-        <ns0:v>1e+70</ns0:v>
+        <ns0:v>1.10773722200378e+75</ns0:v>
       </ns0:c>
       <ns0:c r="E83" s="1">
         <ns0:f>D83</ns0:f>
-        <ns0:v>1e+70</ns0:v>
+        <ns0:v>1.10773722200378e+75</ns0:v>
       </ns0:c>
       <ns0:c r="F83" s="1">
         <ns0:f>ROUND(F82*1.4,-5)</ns0:f>
-        <ns0:v>304550019600000</ns0:v>
+        <ns0:v>2.030837690758128e+22</ns0:v>
       </ns0:c>
       <ns0:c r="G83" s="1" t="n">
         <ns0:v>16.8</ns0:v>
@@ -3725,15 +3698,15 @@
       </ns0:c>
       <ns0:c r="D84" s="1">
         <ns0:f>ROUND(D83*20,2-INT(LOG10(ABS(D83*20))))</ns0:f>
-        <ns0:v>2e+71</ns0:v>
+        <ns0:v>2.2200000000000002e+76</ns0:v>
       </ns0:c>
       <ns0:c r="E84" s="1">
         <ns0:f>D84</ns0:f>
-        <ns0:v>2e+71</ns0:v>
+        <ns0:v>2.2200000000000002e+76</ns0:v>
       </ns0:c>
       <ns0:c r="F84" s="1">
         <ns0:f>ROUND(F83*1.4,-5)</ns0:f>
-        <ns0:v>426370027400000</ns0:v>
+        <ns0:v>2.8431727670613793e+22</ns0:v>
       </ns0:c>
       <ns0:c r="G84" s="1" t="n">
         <ns0:v>17</ns0:v>
@@ -3757,15 +3730,15 @@
       </ns0:c>
       <ns0:c r="D85" s="1">
         <ns0:f>ROUND(D84*20,2-INT(LOG10(ABS(D84*20))))</ns0:f>
-        <ns0:v>4e+72</ns0:v>
+        <ns0:v>4.44e+77</ns0:v>
       </ns0:c>
       <ns0:c r="E85" s="1">
         <ns0:f>D85</ns0:f>
-        <ns0:v>4e+72</ns0:v>
+        <ns0:v>4.44e+77</ns0:v>
       </ns0:c>
       <ns0:c r="F85" s="1">
         <ns0:f>ROUND(F84*1.4,-5)</ns0:f>
-        <ns0:v>596918038400000</ns0:v>
+        <ns0:v>3.9804418738859306e+22</ns0:v>
       </ns0:c>
       <ns0:c r="G85" s="1" t="n">
         <ns0:v>17.2</ns0:v>
@@ -3789,15 +3762,15 @@
       </ns0:c>
       <ns0:c r="D86" s="1">
         <ns0:f>ROUND(D85*20,2-INT(LOG10(ABS(D85*20))))</ns0:f>
-        <ns0:v>8e+73</ns0:v>
+        <ns0:v>8.88e+78</ns0:v>
       </ns0:c>
       <ns0:c r="E86" s="1">
         <ns0:f>D86</ns0:f>
-        <ns0:v>8e+73</ns0:v>
+        <ns0:v>8.88e+78</ns0:v>
       </ns0:c>
       <ns0:c r="F86" s="1">
         <ns0:f>ROUND(F85*1.4,-5)</ns0:f>
-        <ns0:v>835685253800000</ns0:v>
+        <ns0:v>5.572618623440302e+22</ns0:v>
       </ns0:c>
       <ns0:c r="G86" s="1" t="n">
         <ns0:v>17.4</ns0:v>
@@ -3821,15 +3794,15 @@
       </ns0:c>
       <ns0:c r="D87" s="1">
         <ns0:f>ROUND(D86*20,2-INT(LOG10(ABS(D86*20))))</ns0:f>
-        <ns0:v>1.6e+75</ns0:v>
+        <ns0:v>1.78e+80</ns0:v>
       </ns0:c>
       <ns0:c r="E87" s="1">
         <ns0:f>D87</ns0:f>
-        <ns0:v>1.6e+75</ns0:v>
+        <ns0:v>1.78e+80</ns0:v>
       </ns0:c>
       <ns0:c r="F87" s="1">
         <ns0:f>ROUND(F86*1.4,-5)</ns0:f>
-        <ns0:v>1169959355300000</ns0:v>
+        <ns0:v>7.801666072816423e+22</ns0:v>
       </ns0:c>
       <ns0:c r="G87" s="1" t="n">
         <ns0:v>17.6</ns0:v>
@@ -3853,15 +3826,15 @@
       </ns0:c>
       <ns0:c r="D88" s="1">
         <ns0:f>ROUND(D87*20,2-INT(LOG10(ABS(D87*20))))</ns0:f>
-        <ns0:v>3.2e+76</ns0:v>
+        <ns0:v>3.56e+81</ns0:v>
       </ns0:c>
       <ns0:c r="E88" s="1">
         <ns0:f>D88</ns0:f>
-        <ns0:v>3.2e+76</ns0:v>
+        <ns0:v>3.56e+81</ns0:v>
       </ns0:c>
       <ns0:c r="F88" s="1">
         <ns0:f>ROUND(F87*1.4,-5)</ns0:f>
-        <ns0:v>1637943097400000</ns0:v>
+        <ns0:v>1.092233250194299e+23</ns0:v>
       </ns0:c>
       <ns0:c r="G88" s="1" t="n">
         <ns0:v>17.8</ns0:v>
@@ -3885,15 +3858,15 @@
       </ns0:c>
       <ns0:c r="D89" s="1">
         <ns0:f>ROUND(D88*20,2-INT(LOG10(ABS(D88*20))))</ns0:f>
-        <ns0:v>6.4e+77</ns0:v>
+        <ns0:v>7.12e+82</ns0:v>
       </ns0:c>
       <ns0:c r="E89" s="1">
         <ns0:f>D89</ns0:f>
-        <ns0:v>6.4e+77</ns0:v>
+        <ns0:v>7.12e+82</ns0:v>
       </ns0:c>
       <ns0:c r="F89" s="1">
         <ns0:f>ROUND(F88*1.4,-5)</ns0:f>
-        <ns0:v>2293120336400000</ns0:v>
+        <ns0:v>1.5291265502720185e+23</ns0:v>
       </ns0:c>
       <ns0:c r="G89" s="1" t="n">
         <ns0:v>18</ns0:v>
@@ -3917,15 +3890,15 @@
       </ns0:c>
       <ns0:c r="D90" s="1">
         <ns0:f>ROUND(D89*20,2-INT(LOG10(ABS(D89*20))))</ns0:f>
-        <ns0:v>1.28e+79</ns0:v>
+        <ns0:v>1.42e+84</ns0:v>
       </ns0:c>
       <ns0:c r="E90" s="1">
         <ns0:f>D90</ns0:f>
-        <ns0:v>1.28e+79</ns0:v>
+        <ns0:v>1.42e+84</ns0:v>
       </ns0:c>
       <ns0:c r="F90" s="1">
         <ns0:f>ROUND(F89*1.4,-5)</ns0:f>
-        <ns0:v>3210368471000000</ns0:v>
+        <ns0:v>2.140777170380826e+23</ns0:v>
       </ns0:c>
       <ns0:c r="G90" s="1" t="n">
         <ns0:v>18.2</ns0:v>
@@ -3949,15 +3922,15 @@
       </ns0:c>
       <ns0:c r="D91" s="1">
         <ns0:f>ROUND(D90*20,2-INT(LOG10(ABS(D90*20))))</ns0:f>
-        <ns0:v>2.56e+80</ns0:v>
+        <ns0:v>2.84e+85</ns0:v>
       </ns0:c>
       <ns0:c r="E91" s="1">
         <ns0:f>D91</ns0:f>
-        <ns0:v>2.56e+80</ns0:v>
+        <ns0:v>2.84e+85</ns0:v>
       </ns0:c>
       <ns0:c r="F91" s="1">
         <ns0:f>ROUND(F90*1.4,-5)</ns0:f>
-        <ns0:v>4494515859400000</ns0:v>
+        <ns0:v>2.997088038533156e+23</ns0:v>
       </ns0:c>
       <ns0:c r="G91" s="1" t="n">
         <ns0:v>18.4</ns0:v>
@@ -3981,15 +3954,15 @@
       </ns0:c>
       <ns0:c r="D92" s="1">
         <ns0:f>ROUND(D91*20,2-INT(LOG10(ABS(D91*20))))</ns0:f>
-        <ns0:v>5.12e+81</ns0:v>
+        <ns0:v>5.679999999999999e+86</ns0:v>
       </ns0:c>
       <ns0:c r="E92" s="1">
         <ns0:f>D92</ns0:f>
-        <ns0:v>5.12e+81</ns0:v>
+        <ns0:v>5.679999999999999e+86</ns0:v>
       </ns0:c>
       <ns0:c r="F92" s="1">
         <ns0:f>ROUND(F91*1.4,-5)</ns0:f>
-        <ns0:v>6292322203200000</ns0:v>
+        <ns0:v>4.195923253946418e+23</ns0:v>
       </ns0:c>
       <ns0:c r="G92" s="1" t="n">
         <ns0:v>18.6</ns0:v>
@@ -4013,15 +3986,15 @@
       </ns0:c>
       <ns0:c r="D93" s="1">
         <ns0:f>ROUND(D92*20,2-INT(LOG10(ABS(D92*20))))</ns0:f>
-        <ns0:v>1.02e+83</ns0:v>
+        <ns0:v>1.1399999999999999e+88</ns0:v>
       </ns0:c>
       <ns0:c r="E93" s="1">
         <ns0:f>D93</ns0:f>
-        <ns0:v>1.02e+83</ns0:v>
+        <ns0:v>1.1399999999999999e+88</ns0:v>
       </ns0:c>
       <ns0:c r="F93" s="1">
         <ns0:f>ROUND(F92*1.4,-5)</ns0:f>
-        <ns0:v>8809251084500000</ns0:v>
+        <ns0:v>5.8742925555249847e+23</ns0:v>
       </ns0:c>
       <ns0:c r="G93" s="1" t="n">
         <ns0:v>18.8</ns0:v>
@@ -4045,15 +4018,15 @@
       </ns0:c>
       <ns0:c r="D94" s="1">
         <ns0:f>ROUND(D93*20,2-INT(LOG10(ABS(D93*20))))</ns0:f>
-        <ns0:v>2.04e+84</ns0:v>
+        <ns0:v>2.28e+89</ns0:v>
       </ns0:c>
       <ns0:c r="E94" s="1">
         <ns0:f>D94</ns0:f>
-        <ns0:v>2.04e+84</ns0:v>
+        <ns0:v>2.28e+89</ns0:v>
       </ns0:c>
       <ns0:c r="F94" s="1">
         <ns0:f>ROUND(F93*1.4,-5)</ns0:f>
-        <ns0:v>1.23329515183e+16</ns0:v>
+        <ns0:v>8.224009577734978e+23</ns0:v>
       </ns0:c>
       <ns0:c r="G94" s="1" t="n">
         <ns0:v>19</ns0:v>
@@ -4077,15 +4050,15 @@
       </ns0:c>
       <ns0:c r="D95" s="1">
         <ns0:f>ROUND(D94*20,2-INT(LOG10(ABS(D94*20))))</ns0:f>
-        <ns0:v>4.08e+85</ns0:v>
+        <ns0:v>4.5600000000000005e+90</ns0:v>
       </ns0:c>
       <ns0:c r="E95" s="1">
         <ns0:f>D95</ns0:f>
-        <ns0:v>4.08e+85</ns0:v>
+        <ns0:v>4.5600000000000005e+90</ns0:v>
       </ns0:c>
       <ns0:c r="F95" s="1">
         <ns0:f>ROUND(F94*1.4,-5)</ns0:f>
-        <ns0:v>1.72661321256e+16</ns0:v>
+        <ns0:v>1.1513613408828967e+24</ns0:v>
       </ns0:c>
       <ns0:c r="G95" s="1" t="n">
         <ns0:v>19.2</ns0:v>
@@ -4109,15 +4082,15 @@
       </ns0:c>
       <ns0:c r="D96" s="1">
         <ns0:f>ROUND(D95*20,2-INT(LOG10(ABS(D95*20))))</ns0:f>
-        <ns0:v>8.16e+86</ns0:v>
+        <ns0:v>9.12e+91</ns0:v>
       </ns0:c>
       <ns0:c r="E96" s="1">
         <ns0:f>D96</ns0:f>
-        <ns0:v>8.16e+86</ns0:v>
+        <ns0:v>9.12e+91</ns0:v>
       </ns0:c>
       <ns0:c r="F96" s="1">
         <ns0:f>ROUND(F95*1.4,-5)</ns0:f>
-        <ns0:v>2.41725849758e+16</ns0:v>
+        <ns0:v>1.6119058772360553e+24</ns0:v>
       </ns0:c>
       <ns0:c r="G96" s="1" t="n">
         <ns0:v>19.4</ns0:v>
@@ -4141,15 +4114,15 @@
       </ns0:c>
       <ns0:c r="D97" s="1">
         <ns0:f>ROUND(D96*20,2-INT(LOG10(ABS(D96*20))))</ns0:f>
-        <ns0:v>1.63e+88</ns0:v>
+        <ns0:v>1.8199999999999999e+93</ns0:v>
       </ns0:c>
       <ns0:c r="E97" s="1">
         <ns0:f>D97</ns0:f>
-        <ns0:v>1.63e+88</ns0:v>
+        <ns0:v>1.8199999999999999e+93</ns0:v>
       </ns0:c>
       <ns0:c r="F97" s="1">
         <ns0:f>ROUND(F96*1.4,-5)</ns0:f>
-        <ns0:v>3.38416189661e+16</ns0:v>
+        <ns0:v>2.2566682281304774e+24</ns0:v>
       </ns0:c>
       <ns0:c r="G97" s="1" t="n">
         <ns0:v>19.6</ns0:v>
@@ -4173,15 +4146,15 @@
       </ns0:c>
       <ns0:c r="D98" s="1">
         <ns0:f>ROUND(D97*20,2-INT(LOG10(ABS(D97*20))))</ns0:f>
-        <ns0:v>3.26e+89</ns0:v>
+        <ns0:v>3.64e+94</ns0:v>
       </ns0:c>
       <ns0:c r="E98" s="1">
         <ns0:f>D98</ns0:f>
-        <ns0:v>3.26e+89</ns0:v>
+        <ns0:v>3.64e+94</ns0:v>
       </ns0:c>
       <ns0:c r="F98" s="1">
         <ns0:f>ROUND(F97*1.4,-5)</ns0:f>
-        <ns0:v>4.73782665525e+16</ns0:v>
+        <ns0:v>3.159335519382668e+24</ns0:v>
       </ns0:c>
       <ns0:c r="G98" s="1" t="n">
         <ns0:v>19.8</ns0:v>
@@ -4205,15 +4178,15 @@
       </ns0:c>
       <ns0:c r="D99" s="1">
         <ns0:f>ROUND(D98*20,2-INT(LOG10(ABS(D98*20))))</ns0:f>
-        <ns0:v>6.52e+90</ns0:v>
+        <ns0:v>7.28e+95</ns0:v>
       </ns0:c>
       <ns0:c r="E99" s="1">
         <ns0:f>D99</ns0:f>
-        <ns0:v>6.52e+90</ns0:v>
+        <ns0:v>7.28e+95</ns0:v>
       </ns0:c>
       <ns0:c r="F99" s="1">
         <ns0:f>ROUND(F98*1.4,-5)</ns0:f>
-        <ns0:v>6.63295731735e+16</ns0:v>
+        <ns0:v>4.423069727135735e+24</ns0:v>
       </ns0:c>
       <ns0:c r="G99" s="1" t="n">
         <ns0:v>20</ns0:v>
@@ -4237,15 +4210,15 @@
       </ns0:c>
       <ns0:c r="D100" s="1">
         <ns0:f>ROUND(D99*20,2-INT(LOG10(ABS(D99*20))))</ns0:f>
-        <ns0:v>1.3e+92</ns0:v>
+        <ns0:v>1.46e+97</ns0:v>
       </ns0:c>
       <ns0:c r="E100" s="1">
         <ns0:f>D100</ns0:f>
-        <ns0:v>1.3e+92</ns0:v>
+        <ns0:v>1.46e+97</ns0:v>
       </ns0:c>
       <ns0:c r="F100" s="1">
         <ns0:f>ROUND(F99*1.4,-5)</ns0:f>
-        <ns0:v>9.28614024429e+16</ns0:v>
+        <ns0:v>6.192297617990029e+24</ns0:v>
       </ns0:c>
       <ns0:c r="G100" s="1" t="n">
         <ns0:v>20.2</ns0:v>
@@ -4269,15 +4242,15 @@
       </ns0:c>
       <ns0:c r="D101" s="1">
         <ns0:f>ROUND(D100*20,2-INT(LOG10(ABS(D100*20))))</ns0:f>
-        <ns0:v>2.6e+93</ns0:v>
+        <ns0:v>2.9200000000000005e+98</ns0:v>
       </ns0:c>
       <ns0:c r="E101" s="1">
         <ns0:f>D101</ns0:f>
-        <ns0:v>2.6e+93</ns0:v>
+        <ns0:v>2.9200000000000005e+98</ns0:v>
       </ns0:c>
       <ns0:c r="F101" s="1">
         <ns0:f>ROUND(F100*1.4,-5)</ns0:f>
-        <ns0:v>1.300059634201e+17</ns0:v>
+        <ns0:v>8.669216665186042e+24</ns0:v>
       </ns0:c>
       <ns0:c r="G101" s="1" t="n">
         <ns0:v>20.4</ns0:v>
@@ -4301,15 +4274,15 @@
       </ns0:c>
       <ns0:c r="D102" s="1">
         <ns0:f>ROUND(D101*20,2-INT(LOG10(ABS(D101*20))))</ns0:f>
-        <ns0:v>5.2e+94</ns0:v>
+        <ns0:v>5.84e+99</ns0:v>
       </ns0:c>
       <ns0:c r="E102" s="1">
         <ns0:f>D102</ns0:f>
-        <ns0:v>5.2e+94</ns0:v>
+        <ns0:v>5.84e+99</ns0:v>
       </ns0:c>
       <ns0:c r="F102" s="1">
         <ns0:f>ROUND(F101*1.4,-5)</ns0:f>
-        <ns0:v>1.820083487881e+17</ns0:v>
+        <ns0:v>1.2136903331260458e+25</ns0:v>
       </ns0:c>
       <ns0:c r="G102" s="1" t="n">
         <ns0:v>20.6</ns0:v>
@@ -4333,15 +4306,15 @@
       </ns0:c>
       <ns0:c r="D103" s="1">
         <ns0:f>ROUND(D102*20,2-INT(LOG10(ABS(D102*20))))</ns0:f>
-        <ns0:v>1.04e+96</ns0:v>
+        <ns0:v>1.17e+101</ns0:v>
       </ns0:c>
       <ns0:c r="E103" s="1">
         <ns0:f>D103</ns0:f>
-        <ns0:v>1.04e+96</ns0:v>
+        <ns0:v>1.17e+101</ns0:v>
       </ns0:c>
       <ns0:c r="F103" s="1">
         <ns0:f>ROUND(F102*1.4,-5)</ns0:f>
-        <ns0:v>2.548116883033e+17</ns0:v>
+        <ns0:v>1.699166466376464e+25</ns0:v>
       </ns0:c>
       <ns0:c r="G103" s="1" t="n">
         <ns0:v>20.8</ns0:v>
@@ -4365,15 +4338,15 @@
       </ns0:c>
       <ns0:c r="D104" s="1">
         <ns0:f>ROUND(D103*20,2-INT(LOG10(ABS(D103*20))))</ns0:f>
-        <ns0:v>2.08e+97</ns0:v>
+        <ns0:v>2.34e+102</ns0:v>
       </ns0:c>
       <ns0:c r="E104" s="1">
         <ns0:f>D104</ns0:f>
-        <ns0:v>2.08e+97</ns0:v>
+        <ns0:v>2.34e+102</ns0:v>
       </ns0:c>
       <ns0:c r="F104" s="1">
         <ns0:f>ROUND(F103*1.4,-5)</ns0:f>
-        <ns0:v>3.567363636246e+17</ns0:v>
+        <ns0:v>2.3788330529270497e+25</ns0:v>
       </ns0:c>
       <ns0:c r="G104" s="1" t="n">
         <ns0:v>21</ns0:v>
@@ -4397,15 +4370,15 @@
       </ns0:c>
       <ns0:c r="D105" s="1">
         <ns0:f>ROUND(D104*20,2-INT(LOG10(ABS(D104*20))))</ns0:f>
-        <ns0:v>4.16e+98</ns0:v>
+        <ns0:v>4.68e+103</ns0:v>
       </ns0:c>
       <ns0:c r="E105" s="1">
         <ns0:f>D105</ns0:f>
-        <ns0:v>4.16e+98</ns0:v>
+        <ns0:v>4.68e+103</ns0:v>
       </ns0:c>
       <ns0:c r="F105" s="1">
         <ns0:f>ROUND(F104*1.4,-5)</ns0:f>
-        <ns0:v>4.994309090744e+17</ns0:v>
+        <ns0:v>3.3303662740978692e+25</ns0:v>
       </ns0:c>
       <ns0:c r="G105" s="1" t="n">
         <ns0:v>21.2</ns0:v>
@@ -4429,15 +4402,15 @@
       </ns0:c>
       <ns0:c r="D106" s="1">
         <ns0:f>ROUND(D105*20,2-INT(LOG10(ABS(D105*20))))</ns0:f>
-        <ns0:v>8.32e+99</ns0:v>
+        <ns0:v>9.360000000000001e+104</ns0:v>
       </ns0:c>
       <ns0:c r="E106" s="1">
         <ns0:f>D106</ns0:f>
-        <ns0:v>8.32e+99</ns0:v>
+        <ns0:v>9.360000000000001e+104</ns0:v>
       </ns0:c>
       <ns0:c r="F106" s="1">
         <ns0:f>ROUND(F105*1.4,-5)</ns0:f>
-        <ns0:v>6.992032727042e+17</ns0:v>
+        <ns0:v>4.6625127837370165e+25</ns0:v>
       </ns0:c>
       <ns0:c r="G106" s="1" t="n">
         <ns0:v>21.4</ns0:v>
@@ -4461,15 +4434,15 @@
       </ns0:c>
       <ns0:c r="D107" s="1">
         <ns0:f>ROUND(D106*20,2-INT(LOG10(ABS(D106*20))))</ns0:f>
-        <ns0:v>1.66e+101</ns0:v>
+        <ns0:v>1.8700000000000003e+106</ns0:v>
       </ns0:c>
       <ns0:c r="E107" s="1">
         <ns0:f>D107</ns0:f>
-        <ns0:v>1.66e+101</ns0:v>
+        <ns0:v>1.8700000000000003e+106</ns0:v>
       </ns0:c>
       <ns0:c r="F107" s="1">
         <ns0:f>ROUND(F106*1.4,-5)</ns0:f>
-        <ns0:v>9.788845817859e+17</ns0:v>
+        <ns0:v>6.527517897231822e+25</ns0:v>
       </ns0:c>
       <ns0:c r="G107" s="1" t="n">
         <ns0:v>21.6</ns0:v>
@@ -4493,15 +4466,15 @@
       </ns0:c>
       <ns0:c r="D108" s="1">
         <ns0:f>ROUND(D107*20,2-INT(LOG10(ABS(D107*20))))</ns0:f>
-        <ns0:v>3.32e+102</ns0:v>
+        <ns0:v>3.74e+107</ns0:v>
       </ns0:c>
       <ns0:c r="E108" s="1">
         <ns0:f>D108</ns0:f>
-        <ns0:v>3.32e+102</ns0:v>
+        <ns0:v>3.74e+107</ns0:v>
       </ns0:c>
       <ns0:c r="F108" s="1">
         <ns0:f>ROUND(F107*1.4,-5)</ns0:f>
-        <ns0:v>1.3704384145003e+18</ns0:v>
+        <ns0:v>9.13852505612455e+25</ns0:v>
       </ns0:c>
       <ns0:c r="G108" s="1" t="n">
         <ns0:v>21.8</ns0:v>
@@ -4525,15 +4498,15 @@
       </ns0:c>
       <ns0:c r="D109" s="1">
         <ns0:f>ROUND(D108*20,2-INT(LOG10(ABS(D108*20))))</ns0:f>
-        <ns0:v>6.64e+103</ns0:v>
+        <ns0:v>7.480000000000001e+108</ns0:v>
       </ns0:c>
       <ns0:c r="E109" s="1">
         <ns0:f>D109</ns0:f>
-        <ns0:v>6.64e+103</ns0:v>
+        <ns0:v>7.480000000000001e+108</ns0:v>
       </ns0:c>
       <ns0:c r="F109" s="1">
         <ns0:f>ROUND(F108*1.4,-5)</ns0:f>
-        <ns0:v>1.9186137803004e+18</ns0:v>
+        <ns0:v>1.279393507857437e+26</ns0:v>
       </ns0:c>
       <ns0:c r="G109" s="1" t="n">
         <ns0:v>22</ns0:v>
@@ -4557,15 +4530,15 @@
       </ns0:c>
       <ns0:c r="D110" s="1">
         <ns0:f>ROUND(D109*20,2-INT(LOG10(ABS(D109*20))))</ns0:f>
-        <ns0:v>1.33e+105</ns0:v>
+        <ns0:v>1.4999999999999999e+110</ns0:v>
       </ns0:c>
       <ns0:c r="E110" s="1">
         <ns0:f>D110</ns0:f>
-        <ns0:v>1.33e+105</ns0:v>
+        <ns0:v>1.4999999999999999e+110</ns0:v>
       </ns0:c>
       <ns0:c r="F110" s="1">
         <ns0:f>ROUND(F109*1.4,-5)</ns0:f>
-        <ns0:v>2.6860592924206e+18</ns0:v>
+        <ns0:v>1.7911509110004117e+26</ns0:v>
       </ns0:c>
       <ns0:c r="G110" s="1" t="n">
         <ns0:v>22.2</ns0:v>
@@ -4589,15 +4562,15 @@
       </ns0:c>
       <ns0:c r="D111" s="1">
         <ns0:f>ROUND(D110*20,2-INT(LOG10(ABS(D110*20))))</ns0:f>
-        <ns0:v>2.66e+106</ns0:v>
+        <ns0:v>3e+111</ns0:v>
       </ns0:c>
       <ns0:c r="E111" s="1">
         <ns0:f>D111</ns0:f>
-        <ns0:v>2.66e+106</ns0:v>
+        <ns0:v>3e+111</ns0:v>
       </ns0:c>
       <ns0:c r="F111" s="1">
         <ns0:f>ROUND(F110*1.4,-5)</ns0:f>
-        <ns0:v>3.7604830093888e+18</ns0:v>
+        <ns0:v>2.5076112754005763e+26</ns0:v>
       </ns0:c>
       <ns0:c r="G111" s="1" t="n">
         <ns0:v>22.4</ns0:v>
@@ -4621,15 +4594,15 @@
       </ns0:c>
       <ns0:c r="D112" s="1">
         <ns0:f>ROUND(D111*20,2-INT(LOG10(ABS(D111*20))))</ns0:f>
-        <ns0:v>5.32e+107</ns0:v>
+        <ns0:v>6e+112</ns0:v>
       </ns0:c>
       <ns0:c r="E112" s="1">
         <ns0:f>D112</ns0:f>
-        <ns0:v>5.32e+107</ns0:v>
+        <ns0:v>6e+112</ns0:v>
       </ns0:c>
       <ns0:c r="F112" s="1">
         <ns0:f>ROUND(F111*1.4,-5)</ns0:f>
-        <ns0:v>5.2646762131443e+18</ns0:v>
+        <ns0:v>3.510655785560806e+26</ns0:v>
       </ns0:c>
       <ns0:c r="G112" s="1" t="n">
         <ns0:v>22.6</ns0:v>
@@ -4653,15 +4626,15 @@
       </ns0:c>
       <ns0:c r="D113" s="1">
         <ns0:f>ROUND(D112*20,2-INT(LOG10(ABS(D112*20))))</ns0:f>
-        <ns0:v>1.06e+109</ns0:v>
+        <ns0:v>1.2e+114</ns0:v>
       </ns0:c>
       <ns0:c r="E113" s="1">
         <ns0:f>D113</ns0:f>
-        <ns0:v>1.06e+109</ns0:v>
+        <ns0:v>1.2e+114</ns0:v>
       </ns0:c>
       <ns0:c r="F113" s="1">
         <ns0:f>ROUND(F112*1.4,-5)</ns0:f>
-        <ns0:v>7.370546698402e+18</ns0:v>
+        <ns0:v>4.9149180997851284e+26</ns0:v>
       </ns0:c>
       <ns0:c r="G113" s="1" t="n">
         <ns0:v>22.8</ns0:v>
@@ -4685,15 +4658,15 @@
       </ns0:c>
       <ns0:c r="D114" s="1">
         <ns0:f>ROUND(D113*20,2-INT(LOG10(ABS(D113*20))))</ns0:f>
-        <ns0:v>2.12e+110</ns0:v>
+        <ns0:v>2.4e+115</ns0:v>
       </ns0:c>
       <ns0:c r="E114" s="1">
         <ns0:f>D114</ns0:f>
-        <ns0:v>2.12e+110</ns0:v>
+        <ns0:v>2.4e+115</ns0:v>
       </ns0:c>
       <ns0:c r="F114" s="1">
         <ns0:f>ROUND(F113*1.4,-5)</ns0:f>
-        <ns0:v>1.03187653777628e+19</ns0:v>
+        <ns0:v>6.880885339699179e+26</ns0:v>
       </ns0:c>
       <ns0:c r="G114" s="1" t="n">
         <ns0:v>23</ns0:v>
@@ -4717,15 +4690,15 @@
       </ns0:c>
       <ns0:c r="D115" s="1">
         <ns0:f>ROUND(D114*20,2-INT(LOG10(ABS(D114*20))))</ns0:f>
-        <ns0:v>4.24e+111</ns0:v>
+        <ns0:v>4.8e+116</ns0:v>
       </ns0:c>
       <ns0:c r="E115" s="1">
         <ns0:f>D115</ns0:f>
-        <ns0:v>4.24e+111</ns0:v>
+        <ns0:v>4.8e+116</ns0:v>
       </ns0:c>
       <ns0:c r="F115" s="1">
         <ns0:f>ROUND(F114*1.4,-5)</ns0:f>
-        <ns0:v>1.44462715288679e+19</ns0:v>
+        <ns0:v>9.633239475578852e+26</ns0:v>
       </ns0:c>
       <ns0:c r="G115" s="1" t="n">
         <ns0:v>23.2</ns0:v>
@@ -4749,15 +4722,15 @@
       </ns0:c>
       <ns0:c r="D116" s="1">
         <ns0:f>ROUND(D115*20,2-INT(LOG10(ABS(D115*20))))</ns0:f>
-        <ns0:v>8.48e+112</ns0:v>
+        <ns0:v>9.6e+117</ns0:v>
       </ns0:c>
       <ns0:c r="E116" s="1">
         <ns0:f>D116</ns0:f>
-        <ns0:v>8.48e+112</ns0:v>
+        <ns0:v>9.6e+117</ns0:v>
       </ns0:c>
       <ns0:c r="F116" s="1">
         <ns0:f>ROUND(F115*1.4,-5)</ns0:f>
-        <ns0:v>2.02247801404151e+19</ns0:v>
+        <ns0:v>1.3486535265810393e+27</ns0:v>
       </ns0:c>
       <ns0:c r="G116" s="1" t="n">
         <ns0:v>23.4</ns0:v>
@@ -4781,15 +4754,15 @@
       </ns0:c>
       <ns0:c r="D117" s="1">
         <ns0:f>ROUND(D116*20,2-INT(LOG10(ABS(D116*20))))</ns0:f>
-        <ns0:v>1.7e+114</ns0:v>
+        <ns0:v>1.92e+119</ns0:v>
       </ns0:c>
       <ns0:c r="E117" s="1">
         <ns0:f>D117</ns0:f>
-        <ns0:v>1.7e+114</ns0:v>
+        <ns0:v>1.92e+119</ns0:v>
       </ns0:c>
       <ns0:c r="F117" s="1">
         <ns0:f>ROUND(F116*1.4,-5)</ns0:f>
-        <ns0:v>2.83146921965811e+19</ns0:v>
+        <ns0:v>1.8881149372134549e+27</ns0:v>
       </ns0:c>
       <ns0:c r="G117" s="1" t="n">
         <ns0:v>23.6</ns0:v>
@@ -4813,15 +4786,15 @@
       </ns0:c>
       <ns0:c r="D118" s="1">
         <ns0:f>ROUND(D117*20,2-INT(LOG10(ABS(D117*20))))</ns0:f>
-        <ns0:v>3.4e+115</ns0:v>
+        <ns0:v>3.84e+120</ns0:v>
       </ns0:c>
       <ns0:c r="E118" s="1">
         <ns0:f>D118</ns0:f>
-        <ns0:v>3.4e+115</ns0:v>
+        <ns0:v>3.84e+120</ns0:v>
       </ns0:c>
       <ns0:c r="F118" s="1">
         <ns0:f>ROUND(F117*1.4,-5)</ns0:f>
-        <ns0:v>3.96405690752135e+19</ns0:v>
+        <ns0:v>2.6433609120988366e+27</ns0:v>
       </ns0:c>
       <ns0:c r="G118" s="1" t="n">
         <ns0:v>23.8</ns0:v>
@@ -4845,15 +4818,15 @@
       </ns0:c>
       <ns0:c r="D119" s="1">
         <ns0:f>ROUND(D118*20,2-INT(LOG10(ABS(D118*20))))</ns0:f>
-        <ns0:v>6.8e+116</ns0:v>
+        <ns0:v>7.68e+121</ns0:v>
       </ns0:c>
       <ns0:c r="E119" s="1">
         <ns0:f>D119</ns0:f>
-        <ns0:v>6.8e+116</ns0:v>
+        <ns0:v>7.68e+121</ns0:v>
       </ns0:c>
       <ns0:c r="F119" s="1">
         <ns0:f>ROUND(F118*1.4,-5)</ns0:f>
-        <ns0:v>5.54967967052989e+19</ns0:v>
+        <ns0:v>3.700705276938371e+27</ns0:v>
       </ns0:c>
       <ns0:c r="G119" s="1" t="n">
         <ns0:v>24</ns0:v>
@@ -4877,15 +4850,15 @@
       </ns0:c>
       <ns0:c r="D120" s="1">
         <ns0:f>ROUND(D119*20,2-INT(LOG10(ABS(D119*20))))</ns0:f>
-        <ns0:v>1.36e+118</ns0:v>
+        <ns0:v>1.54e+123</ns0:v>
       </ns0:c>
       <ns0:c r="E120" s="1">
         <ns0:f>D120</ns0:f>
-        <ns0:v>1.36e+118</ns0:v>
+        <ns0:v>1.54e+123</ns0:v>
       </ns0:c>
       <ns0:c r="F120" s="1">
         <ns0:f>ROUND(F119*1.4,-5)</ns0:f>
-        <ns0:v>7.76955153874185e+19</ns0:v>
+        <ns0:v>5.180987387713719e+27</ns0:v>
       </ns0:c>
       <ns0:c r="G120" s="1" t="n">
         <ns0:v>24.2000000000001</ns0:v>
@@ -4909,15 +4882,15 @@
       </ns0:c>
       <ns0:c r="D121" s="1">
         <ns0:f>ROUND(D120*20,2-INT(LOG10(ABS(D120*20))))</ns0:f>
-        <ns0:v>2.72e+119</ns0:v>
+        <ns0:v>3.08e+124</ns0:v>
       </ns0:c>
       <ns0:c r="E121" s="1">
         <ns0:f>D121</ns0:f>
-        <ns0:v>2.72e+119</ns0:v>
+        <ns0:v>3.08e+124</ns0:v>
       </ns0:c>
       <ns0:c r="F121" s="1">
         <ns0:f>ROUND(F120*1.4,-5)</ns0:f>
-        <ns0:v>1.08773721542386e+20</ns0:v>
+        <ns0:v>7.253382342799206e+27</ns0:v>
       </ns0:c>
       <ns0:c r="G121" s="1" t="n">
         <ns0:v>24.4000000000001</ns0:v>
@@ -4941,15 +4914,15 @@
       </ns0:c>
       <ns0:c r="D122" s="1">
         <ns0:f>ROUND(D121*20,2-INT(LOG10(ABS(D121*20))))</ns0:f>
-        <ns0:v>5.44e+120</ns0:v>
+        <ns0:v>6.16e+125</ns0:v>
       </ns0:c>
       <ns0:c r="E122" s="1">
         <ns0:f>D122</ns0:f>
-        <ns0:v>5.44e+120</ns0:v>
+        <ns0:v>6.16e+125</ns0:v>
       </ns0:c>
       <ns0:c r="F122" s="1">
         <ns0:f>ROUND(F121*1.4,-5)</ns0:f>
-        <ns0:v>1.5228321015934e+20</ns0:v>
+        <ns0:v>1.0154735279918888e+28</ns0:v>
       </ns0:c>
       <ns0:c r="G122" s="1" t="n">
         <ns0:v>24.6000000000001</ns0:v>
@@ -4973,15 +4946,15 @@
       </ns0:c>
       <ns0:c r="D123" s="1">
         <ns0:f>ROUND(D122*20,2-INT(LOG10(ABS(D122*20))))</ns0:f>
-        <ns0:v>1.09e+122</ns0:v>
+        <ns0:v>1.23e+127</ns0:v>
       </ns0:c>
       <ns0:c r="E123" s="1">
         <ns0:f>D123</ns0:f>
-        <ns0:v>1.09e+122</ns0:v>
+        <ns0:v>1.23e+127</ns0:v>
       </ns0:c>
       <ns0:c r="F123" s="1">
         <ns0:f>ROUND(F122*1.4,-5)</ns0:f>
-        <ns0:v>2.13196494223076e+20</ns0:v>
+        <ns0:v>1.4216629391886442e+28</ns0:v>
       </ns0:c>
       <ns0:c r="G123" s="1" t="n">
         <ns0:v>24.8000000000001</ns0:v>
@@ -5005,15 +4978,15 @@
       </ns0:c>
       <ns0:c r="D124" s="1">
         <ns0:f>ROUND(D123*20,2-INT(LOG10(ABS(D123*20))))</ns0:f>
-        <ns0:v>2.18e+123</ns0:v>
+        <ns0:v>2.46e+128</ns0:v>
       </ns0:c>
       <ns0:c r="E124" s="1">
         <ns0:f>D124</ns0:f>
-        <ns0:v>2.18e+123</ns0:v>
+        <ns0:v>2.46e+128</ns0:v>
       </ns0:c>
       <ns0:c r="F124" s="1">
         <ns0:f>ROUND(F123*1.4,-5)</ns0:f>
-        <ns0:v>2.98475091912306e+20</ns0:v>
+        <ns0:v>1.990328114864102e+28</ns0:v>
       </ns0:c>
       <ns0:c r="G124" s="1" t="n">
         <ns0:v>25.0000000000001</ns0:v>
@@ -5037,15 +5010,15 @@
       </ns0:c>
       <ns0:c r="D125" s="1">
         <ns0:f>ROUND(D124*20,2-INT(LOG10(ABS(D124*20))))</ns0:f>
-        <ns0:v>4.36e+124</ns0:v>
+        <ns0:v>4.92e+129</ns0:v>
       </ns0:c>
       <ns0:c r="E125" s="1">
         <ns0:f>D125</ns0:f>
-        <ns0:v>4.36e+124</ns0:v>
+        <ns0:v>4.92e+129</ns0:v>
       </ns0:c>
       <ns0:c r="F125" s="1">
         <ns0:f>ROUND(F124*1.4,-5)</ns0:f>
-        <ns0:v>4.17865128677228e+20</ns0:v>
+        <ns0:v>2.7864593608097423e+28</ns0:v>
       </ns0:c>
       <ns0:c r="G125" s="1" t="n">
         <ns0:v>25.2000000000001</ns0:v>
@@ -5069,15 +5042,15 @@
       </ns0:c>
       <ns0:c r="D126" s="1">
         <ns0:f>ROUND(D125*20,2-INT(LOG10(ABS(D125*20))))</ns0:f>
-        <ns0:v>8.72e+125</ns0:v>
+        <ns0:v>9.839999999999999e+130</ns0:v>
       </ns0:c>
       <ns0:c r="E126" s="1">
         <ns0:f>D126</ns0:f>
-        <ns0:v>8.72e+125</ns0:v>
+        <ns0:v>9.839999999999999e+130</ns0:v>
       </ns0:c>
       <ns0:c r="F126" s="1">
         <ns0:f>ROUND(F125*1.4,-5)</ns0:f>
-        <ns0:v>5.85011180148119e+20</ns0:v>
+        <ns0:v>3.9010431051336393e+28</ns0:v>
       </ns0:c>
       <ns0:c r="G126" s="1" t="n">
         <ns0:v>25.4000000000001</ns0:v>
@@ -5101,15 +5074,15 @@
       </ns0:c>
       <ns0:c r="D127" s="1">
         <ns0:f>ROUND(D126*20,2-INT(LOG10(ABS(D126*20))))</ns0:f>
-        <ns0:v>1.74e+127</ns0:v>
+        <ns0:v>1.97e+132</ns0:v>
       </ns0:c>
       <ns0:c r="E127" s="1">
         <ns0:f>D127</ns0:f>
-        <ns0:v>1.74e+127</ns0:v>
+        <ns0:v>1.97e+132</ns0:v>
       </ns0:c>
       <ns0:c r="F127" s="1">
         <ns0:f>ROUND(F126*1.4,-5)</ns0:f>
-        <ns0:v>8.19015652207367e+20</ns0:v>
+        <ns0:v>5.461460347187095e+28</ns0:v>
       </ns0:c>
       <ns0:c r="G127" s="1" t="n">
         <ns0:v>25.6000000000001</ns0:v>
@@ -5133,15 +5106,15 @@
       </ns0:c>
       <ns0:c r="D128" s="1">
         <ns0:f>ROUND(D127*20,2-INT(LOG10(ABS(D127*20))))</ns0:f>
-        <ns0:v>3.48e+128</ns0:v>
+        <ns0:v>3.94e+133</ns0:v>
       </ns0:c>
       <ns0:c r="E128" s="1">
         <ns0:f>D128</ns0:f>
-        <ns0:v>3.48e+128</ns0:v>
+        <ns0:v>3.94e+133</ns0:v>
       </ns0:c>
       <ns0:c r="F128" s="1">
         <ns0:f>ROUND(F127*1.4,-5)</ns0:f>
-        <ns0:v>1.14662191309031e+21</ns0:v>
+        <ns0:v>7.646044486061932e+28</ns0:v>
       </ns0:c>
       <ns0:c r="G128" s="1" t="n">
         <ns0:v>25.8000000000001</ns0:v>
@@ -5165,15 +5138,15 @@
       </ns0:c>
       <ns0:c r="D129" s="1">
         <ns0:f>ROUND(D128*20,2-INT(LOG10(ABS(D128*20))))</ns0:f>
-        <ns0:v>6.96e+129</ns0:v>
+        <ns0:v>7.880000000000001e+134</ns0:v>
       </ns0:c>
       <ns0:c r="E129" s="1">
         <ns0:f>D129</ns0:f>
-        <ns0:v>6.96e+129</ns0:v>
+        <ns0:v>7.880000000000001e+134</ns0:v>
       </ns0:c>
       <ns0:c r="F129" s="1">
         <ns0:f>ROUND(F128*1.4,-5)</ns0:f>
-        <ns0:v>1.60527067832643e+21</ns0:v>
+        <ns0:v>1.0704462280486704e+29</ns0:v>
       </ns0:c>
       <ns0:c r="G129" s="1" t="n">
         <ns0:v>26.0000000000001</ns0:v>
@@ -5197,15 +5170,15 @@
       </ns0:c>
       <ns0:c r="D130" s="1">
         <ns0:f>ROUND(D129*20,2-INT(LOG10(ABS(D129*20))))</ns0:f>
-        <ns0:v>1.39e+131</ns0:v>
+        <ns0:v>1.58e+136</ns0:v>
       </ns0:c>
       <ns0:c r="E130" s="1">
         <ns0:f>D130</ns0:f>
-        <ns0:v>1.39e+131</ns0:v>
+        <ns0:v>1.58e+136</ns0:v>
       </ns0:c>
       <ns0:c r="F130" s="1">
         <ns0:f>ROUND(F129*1.4,-5)</ns0:f>
-        <ns0:v>2.247378949657e+21</ns0:v>
+        <ns0:v>1.4986247192681385e+29</ns0:v>
       </ns0:c>
       <ns0:c r="G130" s="1" t="n">
         <ns0:v>26.2000000000001</ns0:v>
@@ -5229,15 +5202,15 @@
       </ns0:c>
       <ns0:c r="D131" s="1">
         <ns0:f>ROUND(D130*20,2-INT(LOG10(ABS(D130*20))))</ns0:f>
-        <ns0:v>2.78e+132</ns0:v>
+        <ns0:v>3.1599999999999998e+137</ns0:v>
       </ns0:c>
       <ns0:c r="E131" s="1">
         <ns0:f>D131</ns0:f>
-        <ns0:v>2.78e+132</ns0:v>
+        <ns0:v>3.1599999999999998e+137</ns0:v>
       </ns0:c>
       <ns0:c r="F131" s="1">
         <ns0:f>ROUND(F130*1.4,-5)</ns0:f>
-        <ns0:v>3.1463305295198e+21</ns0:v>
+        <ns0:v>2.0980746069753937e+29</ns0:v>
       </ns0:c>
       <ns0:c r="G131" s="1" t="n">
         <ns0:v>26.4000000000001</ns0:v>
@@ -5261,15 +5234,15 @@
       </ns0:c>
       <ns0:c r="D132" s="1">
         <ns0:f>ROUND(D131*20,2-INT(LOG10(ABS(D131*20))))</ns0:f>
-        <ns0:v>5.56e+133</ns0:v>
+        <ns0:v>6.32e+138</ns0:v>
       </ns0:c>
       <ns0:c r="E132" s="1">
         <ns0:f>D132</ns0:f>
-        <ns0:v>5.56e+133</ns0:v>
+        <ns0:v>6.32e+138</ns0:v>
       </ns0:c>
       <ns0:c r="F132" s="1">
         <ns0:f>ROUND(F131*1.4,-5)</ns0:f>
-        <ns0:v>4.40486274132772e+21</ns0:v>
+        <ns0:v>2.9373044497655515e+29</ns0:v>
       </ns0:c>
       <ns0:c r="G132" s="1" t="n">
         <ns0:v>26.6000000000001</ns0:v>
@@ -5293,15 +5266,15 @@
       </ns0:c>
       <ns0:c r="D133" s="1">
         <ns0:f>ROUND(D132*20,2-INT(LOG10(ABS(D132*20))))</ns0:f>
-        <ns0:v>1.11e+135</ns0:v>
+        <ns0:v>1.2599999999999998e+140</ns0:v>
       </ns0:c>
       <ns0:c r="E133" s="1">
         <ns0:f>D133</ns0:f>
-        <ns0:v>1.11e+135</ns0:v>
+        <ns0:v>1.2599999999999998e+140</ns0:v>
       </ns0:c>
       <ns0:c r="F133" s="1">
         <ns0:f>ROUND(F132*1.4,-5)</ns0:f>
-        <ns0:v>6.16680783785881e+21</ns0:v>
+        <ns0:v>4.112226229671772e+29</ns0:v>
       </ns0:c>
       <ns0:c r="G133" s="1" t="n">
         <ns0:v>26.8000000000001</ns0:v>
@@ -5325,15 +5298,15 @@
       </ns0:c>
       <ns0:c r="D134" s="1">
         <ns0:f>ROUND(D133*20,2-INT(LOG10(ABS(D133*20))))</ns0:f>
-        <ns0:v>2.22e+136</ns0:v>
+        <ns0:v>2.52e+141</ns0:v>
       </ns0:c>
       <ns0:c r="E134" s="1">
         <ns0:f>D134</ns0:f>
-        <ns0:v>2.22e+136</ns0:v>
+        <ns0:v>2.52e+141</ns0:v>
       </ns0:c>
       <ns0:c r="F134" s="1">
         <ns0:f>ROUND(F133*1.4,-5)</ns0:f>
-        <ns0:v>8.63353097300233e+21</ns0:v>
+        <ns0:v>5.7571167215404806e+29</ns0:v>
       </ns0:c>
       <ns0:c r="G134" s="1" t="n">
         <ns0:v>27.0000000000001</ns0:v>
@@ -5357,15 +5330,15 @@
       </ns0:c>
       <ns0:c r="D135" s="1">
         <ns0:f>ROUND(D134*20,2-INT(LOG10(ABS(D134*20))))</ns0:f>
-        <ns0:v>4.44e+137</ns0:v>
+        <ns0:v>5.04e+142</ns0:v>
       </ns0:c>
       <ns0:c r="E135" s="1">
         <ns0:f>D135</ns0:f>
-        <ns0:v>4.44e+137</ns0:v>
+        <ns0:v>5.04e+142</ns0:v>
       </ns0:c>
       <ns0:c r="F135" s="1">
         <ns0:f>ROUND(F134*1.4,-5)</ns0:f>
-        <ns0:v>1.20869433622033e+22</ns0:v>
+        <ns0:v>8.059963410156672e+29</ns0:v>
       </ns0:c>
       <ns0:c r="G135" s="1" t="n">
         <ns0:v>27.2000000000001</ns0:v>
@@ -5389,15 +5362,15 @@
       </ns0:c>
       <ns0:c r="D136" s="1">
         <ns0:f>ROUND(D135*20,2-INT(LOG10(ABS(D135*20))))</ns0:f>
-        <ns0:v>8.88e+138</ns0:v>
+        <ns0:v>1.0099999999999999e+144</ns0:v>
       </ns0:c>
       <ns0:c r="E136" s="1">
         <ns0:f>D136</ns0:f>
-        <ns0:v>8.88e+138</ns0:v>
+        <ns0:v>1.0099999999999999e+144</ns0:v>
       </ns0:c>
       <ns0:c r="F136" s="1">
         <ns0:f>ROUND(F135*1.4,-5)</ns0:f>
-        <ns0:v>1.69217207070846e+22</ns0:v>
+        <ns0:v>1.128394877421934e+30</ns0:v>
       </ns0:c>
       <ns0:c r="G136" s="1" t="n">
         <ns0:v>27.4000000000001</ns0:v>
@@ -5421,15 +5394,15 @@
       </ns0:c>
       <ns0:c r="D137" s="1">
         <ns0:f>ROUND(D136*20,2-INT(LOG10(ABS(D136*20))))</ns0:f>
-        <ns0:v>1.78e+140</ns0:v>
+        <ns0:v>2.0200000000000002e+145</ns0:v>
       </ns0:c>
       <ns0:c r="E137" s="1">
         <ns0:f>D137</ns0:f>
-        <ns0:v>1.78e+140</ns0:v>
+        <ns0:v>2.0200000000000002e+145</ns0:v>
       </ns0:c>
       <ns0:c r="F137" s="1">
         <ns0:f>ROUND(F136*1.4,-5)</ns0:f>
-        <ns0:v>2.36904089899184e+22</ns0:v>
+        <ns0:v>1.5797528283907075e+30</ns0:v>
       </ns0:c>
       <ns0:c r="G137" s="1" t="n">
         <ns0:v>27.6000000000001</ns0:v>
@@ -5453,15 +5426,15 @@
       </ns0:c>
       <ns0:c r="D138" s="1">
         <ns0:f>ROUND(D137*20,2-INT(LOG10(ABS(D137*20))))</ns0:f>
-        <ns0:v>3.56e+141</ns0:v>
+        <ns0:v>4.04e+146</ns0:v>
       </ns0:c>
       <ns0:c r="E138" s="1">
         <ns0:f>D138</ns0:f>
-        <ns0:v>3.56e+141</ns0:v>
+        <ns0:v>4.04e+146</ns0:v>
       </ns0:c>
       <ns0:c r="F138" s="1">
         <ns0:f>ROUND(F137*1.4,-5)</ns0:f>
-        <ns0:v>3.31665725858858e+22</ns0:v>
+        <ns0:v>2.2116539597469903e+30</ns0:v>
       </ns0:c>
       <ns0:c r="G138" s="1" t="n">
         <ns0:v>27.8000000000001</ns0:v>
@@ -5485,15 +5458,15 @@
       </ns0:c>
       <ns0:c r="D139" s="1">
         <ns0:f>ROUND(D138*20,2-INT(LOG10(ABS(D138*20))))</ns0:f>
-        <ns0:v>7.12e+142</ns0:v>
+        <ns0:v>8.080000000000001e+147</ns0:v>
       </ns0:c>
       <ns0:c r="E139" s="1">
         <ns0:f>D139</ns0:f>
-        <ns0:v>7.12e+142</ns0:v>
+        <ns0:v>8.080000000000001e+147</ns0:v>
       </ns0:c>
       <ns0:c r="F139" s="1">
         <ns0:f>ROUND(F138*1.4,-5)</ns0:f>
-        <ns0:v>4.64332016202401e+22</ns0:v>
+        <ns0:v>3.096315543645786e+30</ns0:v>
       </ns0:c>
       <ns0:c r="G139" s="1" t="n">
         <ns0:v>28.0000000000001</ns0:v>
@@ -5517,15 +5490,15 @@
       </ns0:c>
       <ns0:c r="D140" s="1">
         <ns0:f>ROUND(D139*20,2-INT(LOG10(ABS(D139*20))))</ns0:f>
-        <ns0:v>1.42e+144</ns0:v>
+        <ns0:v>1.62e+149</ns0:v>
       </ns0:c>
       <ns0:c r="E140" s="1">
         <ns0:f>D140</ns0:f>
-        <ns0:v>1.42e+144</ns0:v>
+        <ns0:v>1.62e+149</ns0:v>
       </ns0:c>
       <ns0:c r="F140" s="1">
         <ns0:f>ROUND(F139*1.4,-5)</ns0:f>
-        <ns0:v>6.50064822683361e+22</ns0:v>
+        <ns0:v>4.3348417611040996e+30</ns0:v>
       </ns0:c>
       <ns0:c r="G140" s="1" t="n">
         <ns0:v>28.2000000000001</ns0:v>
@@ -5549,15 +5522,15 @@
       </ns0:c>
       <ns0:c r="D141" s="1">
         <ns0:f>ROUND(D140*20,2-INT(LOG10(ABS(D140*20))))</ns0:f>
-        <ns0:v>2.84e+145</ns0:v>
+        <ns0:v>3.24e+150</ns0:v>
       </ns0:c>
       <ns0:c r="E141" s="1">
         <ns0:f>D141</ns0:f>
-        <ns0:v>2.84e+145</ns0:v>
+        <ns0:v>3.24e+150</ns0:v>
       </ns0:c>
       <ns0:c r="F141" s="1">
         <ns0:f>ROUND(F140*1.4,-5)</ns0:f>
-        <ns0:v>9.10090751756705e+22</ns0:v>
+        <ns0:v>6.068778465545739e+30</ns0:v>
       </ns0:c>
       <ns0:c r="G141" s="1" t="n">
         <ns0:v>28.4000000000001</ns0:v>
@@ -5581,15 +5554,15 @@
       </ns0:c>
       <ns0:c r="D142" s="1">
         <ns0:f>ROUND(D141*20,2-INT(LOG10(ABS(D141*20))))</ns0:f>
-        <ns0:v>5.68e+146</ns0:v>
+        <ns0:v>6.48e+151</ns0:v>
       </ns0:c>
       <ns0:c r="E142" s="1">
         <ns0:f>D142</ns0:f>
-        <ns0:v>5.68e+146</ns0:v>
+        <ns0:v>6.48e+151</ns0:v>
       </ns0:c>
       <ns0:c r="F142" s="1">
         <ns0:f>ROUND(F141*1.4,-5)</ns0:f>
-        <ns0:v>1.27412705245939e+23</ns0:v>
+        <ns0:v>8.496289851764034e+30</ns0:v>
       </ns0:c>
       <ns0:c r="G142" s="1" t="n">
         <ns0:v>28.6000000000001</ns0:v>
@@ -5613,15 +5586,15 @@
       </ns0:c>
       <ns0:c r="D143" s="1">
         <ns0:f>ROUND(D142*20,2-INT(LOG10(ABS(D142*20))))</ns0:f>
-        <ns0:v>1.14e+148</ns0:v>
+        <ns0:v>1.3000000000000001e+153</ns0:v>
       </ns0:c>
       <ns0:c r="E143" s="1">
         <ns0:f>D143</ns0:f>
-        <ns0:v>1.14e+148</ns0:v>
+        <ns0:v>1.3000000000000001e+153</ns0:v>
       </ns0:c>
       <ns0:c r="F143" s="1">
         <ns0:f>ROUND(F142*1.4,-5)</ns0:f>
-        <ns0:v>1.78377787344315e+23</ns0:v>
+        <ns0:v>1.1894805792469646e+31</ns0:v>
       </ns0:c>
       <ns0:c r="G143" s="1" t="n">
         <ns0:v>28.8000000000001</ns0:v>
@@ -5645,15 +5618,15 @@
       </ns0:c>
       <ns0:c r="D144" s="1">
         <ns0:f>ROUND(D143*20,2-INT(LOG10(ABS(D143*20))))</ns0:f>
-        <ns0:v>2.28e+149</ns0:v>
+        <ns0:v>2.6e+154</ns0:v>
       </ns0:c>
       <ns0:c r="E144" s="1">
         <ns0:f>D144</ns0:f>
-        <ns0:v>2.28e+149</ns0:v>
+        <ns0:v>2.6e+154</ns0:v>
       </ns0:c>
       <ns0:c r="F144" s="1">
         <ns0:f>ROUND(F143*1.4,-5)</ns0:f>
-        <ns0:v>2.49728902282041e+23</ns0:v>
+        <ns0:v>1.6652728109457504e+31</ns0:v>
       </ns0:c>
       <ns0:c r="G144" s="1" t="n">
         <ns0:v>29.0000000000001</ns0:v>
@@ -5677,15 +5650,15 @@
       </ns0:c>
       <ns0:c r="D145" s="1">
         <ns0:f>ROUND(D144*20,2-INT(LOG10(ABS(D144*20))))</ns0:f>
-        <ns0:v>4.56e+150</ns0:v>
+        <ns0:v>5.199999999999999e+155</ns0:v>
       </ns0:c>
       <ns0:c r="E145" s="1">
         <ns0:f>D145</ns0:f>
-        <ns0:v>4.56e+150</ns0:v>
+        <ns0:v>5.199999999999999e+155</ns0:v>
       </ns0:c>
       <ns0:c r="F145" s="1">
         <ns0:f>ROUND(F144*1.4,-5)</ns0:f>
-        <ns0:v>3.49620463194857e+23</ns0:v>
+        <ns0:v>2.3313819353240506e+31</ns0:v>
       </ns0:c>
       <ns0:c r="G145" s="1" t="n">
         <ns0:v>29.2000000000001</ns0:v>
@@ -5709,15 +5682,15 @@
       </ns0:c>
       <ns0:c r="D146" s="1">
         <ns0:f>ROUND(D145*20,2-INT(LOG10(ABS(D145*20))))</ns0:f>
-        <ns0:v>9.12e+151</ns0:v>
+        <ns0:v>1.0399999999999999e+157</ns0:v>
       </ns0:c>
       <ns0:c r="E146" s="1">
         <ns0:f>D146</ns0:f>
-        <ns0:v>9.12e+151</ns0:v>
+        <ns0:v>1.0399999999999999e+157</ns0:v>
       </ns0:c>
       <ns0:c r="F146" s="1">
         <ns0:f>ROUND(F145*1.4,-5)</ns0:f>
-        <ns0:v>4.894686484728e+23</ns0:v>
+        <ns0:v>3.263934709453671e+31</ns0:v>
       </ns0:c>
       <ns0:c r="G146" s="1" t="n">
         <ns0:v>29.4000000000001</ns0:v>
@@ -5741,15 +5714,15 @@
       </ns0:c>
       <ns0:c r="D147" s="1">
         <ns0:f>ROUND(D146*20,2-INT(LOG10(ABS(D146*20))))</ns0:f>
-        <ns0:v>1.82e+153</ns0:v>
+        <ns0:v>2.0799999999999998e+158</ns0:v>
       </ns0:c>
       <ns0:c r="E147" s="1">
         <ns0:f>D147</ns0:f>
-        <ns0:v>1.82e+153</ns0:v>
+        <ns0:v>2.0799999999999998e+158</ns0:v>
       </ns0:c>
       <ns0:c r="F147" s="1">
         <ns0:f>ROUND(F146*1.4,-5)</ns0:f>
-        <ns0:v>6.8525610786192e+23</ns0:v>
+        <ns0:v>4.569508593235139e+31</ns0:v>
       </ns0:c>
       <ns0:c r="G147" s="1" t="n">
         <ns0:v>29.6000000000001</ns0:v>
@@ -5773,15 +5746,15 @@
       </ns0:c>
       <ns0:c r="D148" s="1">
         <ns0:f>ROUND(D147*20,2-INT(LOG10(ABS(D147*20))))</ns0:f>
-        <ns0:v>3.64e+154</ns0:v>
+        <ns0:v>4.16e+159</ns0:v>
       </ns0:c>
       <ns0:c r="E148" s="1">
         <ns0:f>D148</ns0:f>
-        <ns0:v>3.64e+154</ns0:v>
+        <ns0:v>4.16e+159</ns0:v>
       </ns0:c>
       <ns0:c r="F148" s="1">
         <ns0:f>ROUND(F147*1.4,-5)</ns0:f>
-        <ns0:v>9.59358551006688e+23</ns0:v>
+        <ns0:v>6.397312030529194e+31</ns0:v>
       </ns0:c>
       <ns0:c r="G148" s="1" t="n">
         <ns0:v>29.8000000000001</ns0:v>
@@ -5805,15 +5778,15 @@
       </ns0:c>
       <ns0:c r="D149" s="1">
         <ns0:f>ROUND(D148*20,2-INT(LOG10(ABS(D148*20))))</ns0:f>
-        <ns0:v>7.28e+155</ns0:v>
+        <ns0:v>8.319999999999999e+160</ns0:v>
       </ns0:c>
       <ns0:c r="E149" s="1">
         <ns0:f>D149</ns0:f>
-        <ns0:v>7.28e+155</ns0:v>
+        <ns0:v>8.319999999999999e+160</ns0:v>
       </ns0:c>
       <ns0:c r="F149" s="1">
         <ns0:f>ROUND(F148*1.4,-5)</ns0:f>
-        <ns0:v>1.34310197140936e+24</ns0:v>
+        <ns0:v>8.95623684274087e+31</ns0:v>
       </ns0:c>
       <ns0:c r="G149" s="1" t="n">
         <ns0:v>30.0000000000001</ns0:v>
@@ -5837,15 +5810,15 @@
       </ns0:c>
       <ns0:c r="D150" s="1">
         <ns0:f>ROUND(D149*20,2-INT(LOG10(ABS(D149*20))))</ns0:f>
-        <ns0:v>1.46e+157</ns0:v>
+        <ns0:v>1.66e+162</ns0:v>
       </ns0:c>
       <ns0:c r="E150" s="1">
         <ns0:f>D150</ns0:f>
-        <ns0:v>1.46e+157</ns0:v>
+        <ns0:v>1.66e+162</ns0:v>
       </ns0:c>
       <ns0:c r="F150" s="1">
         <ns0:f>ROUND(F149*1.4,-5)</ns0:f>
-        <ns0:v>1.8803427599731e+24</ns0:v>
+        <ns0:v>1.253873157983722e+32</ns0:v>
       </ns0:c>
       <ns0:c r="G150" s="1" t="n">
         <ns0:v>30.2000000000001</ns0:v>
@@ -5869,15 +5842,15 @@
       </ns0:c>
       <ns0:c r="D151" s="1">
         <ns0:f>ROUND(D150*20,2-INT(LOG10(ABS(D150*20))))</ns0:f>
-        <ns0:v>2.92e+158</ns0:v>
+        <ns0:v>3.32e+163</ns0:v>
       </ns0:c>
       <ns0:c r="E151" s="1">
         <ns0:f>D151</ns0:f>
-        <ns0:v>2.92e+158</ns0:v>
+        <ns0:v>3.32e+163</ns0:v>
       </ns0:c>
       <ns0:c r="F151" s="1">
         <ns0:f>ROUND(F150*1.4,-5)</ns0:f>
-        <ns0:v>2.63247986396234e+24</ns0:v>
+        <ns0:v>1.7554224211772108e+32</ns0:v>
       </ns0:c>
       <ns0:c r="G151" s="1" t="n">
         <ns0:v>30.4000000000001</ns0:v>
@@ -5901,15 +5874,15 @@
       </ns0:c>
       <ns0:c r="D152" s="1">
         <ns0:f>ROUND(D151*20,2-INT(LOG10(ABS(D151*20))))</ns0:f>
-        <ns0:v>5.84e+159</ns0:v>
+        <ns0:v>6.64e+164</ns0:v>
       </ns0:c>
       <ns0:c r="E152" s="1">
         <ns0:f>D152</ns0:f>
-        <ns0:v>5.84e+159</ns0:v>
+        <ns0:v>6.64e+164</ns0:v>
       </ns0:c>
       <ns0:c r="F152" s="1">
         <ns0:f>ROUND(F151*1.4,-5)</ns0:f>
-        <ns0:v>3.68547180954728e+24</ns0:v>
+        <ns0:v>2.457591389648095e+32</ns0:v>
       </ns0:c>
       <ns0:c r="G152" s="1" t="n">
         <ns0:v>30.6000000000001</ns0:v>
@@ -5933,15 +5906,15 @@
       </ns0:c>
       <ns0:c r="D153" s="1">
         <ns0:f>ROUND(D152*20,2-INT(LOG10(ABS(D152*20))))</ns0:f>
-        <ns0:v>1.17e+161</ns0:v>
+        <ns0:v>1.3300000000000001e+166</ns0:v>
       </ns0:c>
       <ns0:c r="E153" s="1">
         <ns0:f>D153</ns0:f>
-        <ns0:v>1.17e+161</ns0:v>
+        <ns0:v>1.3300000000000001e+166</ns0:v>
       </ns0:c>
       <ns0:c r="F153" s="1">
         <ns0:f>ROUND(F152*1.4,-5)</ns0:f>
-        <ns0:v>5.15966053336619e+24</ns0:v>
+        <ns0:v>3.440627945507332e+32</ns0:v>
       </ns0:c>
       <ns0:c r="G153" s="1" t="n">
         <ns0:v>30.8000000000001</ns0:v>
@@ -5965,15 +5938,15 @@
       </ns0:c>
       <ns0:c r="D154" s="1">
         <ns0:f>ROUND(D153*20,2-INT(LOG10(ABS(D153*20))))</ns0:f>
-        <ns0:v>2.34e+162</ns0:v>
+        <ns0:v>2.66e+167</ns0:v>
       </ns0:c>
       <ns0:c r="E154" s="1">
         <ns0:f>D154</ns0:f>
-        <ns0:v>2.34e+162</ns0:v>
+        <ns0:v>2.66e+167</ns0:v>
       </ns0:c>
       <ns0:c r="F154" s="1">
         <ns0:f>ROUND(F153*1.4,-5)</ns0:f>
-        <ns0:v>7.22352474671267e+24</ns0:v>
+        <ns0:v>4.816879123710265e+32</ns0:v>
       </ns0:c>
       <ns0:c r="G154" s="1" t="n">
         <ns0:v>31.0000000000001</ns0:v>
@@ -5997,15 +5970,15 @@
       </ns0:c>
       <ns0:c r="D155" s="1">
         <ns0:f>ROUND(D154*20,2-INT(LOG10(ABS(D154*20))))</ns0:f>
-        <ns0:v>4.68e+163</ns0:v>
+        <ns0:v>5.32e+168</ns0:v>
       </ns0:c>
       <ns0:c r="E155" s="1">
         <ns0:f>D155</ns0:f>
-        <ns0:v>4.68e+163</ns0:v>
+        <ns0:v>5.32e+168</ns0:v>
       </ns0:c>
       <ns0:c r="F155" s="1">
         <ns0:f>ROUND(F154*1.4,-5)</ns0:f>
-        <ns0:v>1.01129346453977e+25</ns0:v>
+        <ns0:v>6.743630773194371e+32</ns0:v>
       </ns0:c>
       <ns0:c r="G155" s="1" t="n">
         <ns0:v>31.2000000000001</ns0:v>
@@ -6029,15 +6002,15 @@
       </ns0:c>
       <ns0:c r="D156" s="1">
         <ns0:f>ROUND(D155*20,2-INT(LOG10(ABS(D155*20))))</ns0:f>
-        <ns0:v>9.36e+164</ns0:v>
+        <ns0:v>1.06e+170</ns0:v>
       </ns0:c>
       <ns0:c r="E156" s="1">
         <ns0:f>D156</ns0:f>
-        <ns0:v>9.36e+164</ns0:v>
+        <ns0:v>1.06e+170</ns0:v>
       </ns0:c>
       <ns0:c r="F156" s="1">
         <ns0:f>ROUND(F155*1.4,-5)</ns0:f>
-        <ns0:v>1.41581085035568e+25</ns0:v>
+        <ns0:v>9.441083082472119e+32</ns0:v>
       </ns0:c>
       <ns0:c r="G156" s="1" t="n">
         <ns0:v>31.4000000000001</ns0:v>
@@ -6061,15 +6034,15 @@
       </ns0:c>
       <ns0:c r="D157" s="1">
         <ns0:f>ROUND(D156*20,2-INT(LOG10(ABS(D156*20))))</ns0:f>
-        <ns0:v>1.87e+166</ns0:v>
+        <ns0:v>2.12e+171</ns0:v>
       </ns0:c>
       <ns0:c r="E157" s="1">
         <ns0:f>D157</ns0:f>
-        <ns0:v>1.87e+166</ns0:v>
+        <ns0:v>2.12e+171</ns0:v>
       </ns0:c>
       <ns0:c r="F157" s="1">
         <ns0:f>ROUND(F156*1.4,-5)</ns0:f>
-        <ns0:v>1.98213519049795e+25</ns0:v>
+        <ns0:v>1.3217516315460965e+33</ns0:v>
       </ns0:c>
       <ns0:c r="G157" s="1" t="n">
         <ns0:v>31.6000000000001</ns0:v>
@@ -6093,15 +6066,15 @@
       </ns0:c>
       <ns0:c r="D158" s="1">
         <ns0:f>ROUND(D157*20,2-INT(LOG10(ABS(D157*20))))</ns0:f>
-        <ns0:v>3.74e+167</ns0:v>
+        <ns0:v>4.24e+172</ns0:v>
       </ns0:c>
       <ns0:c r="E158" s="1">
         <ns0:f>D158</ns0:f>
-        <ns0:v>3.74e+167</ns0:v>
+        <ns0:v>4.24e+172</ns0:v>
       </ns0:c>
       <ns0:c r="F158" s="1">
         <ns0:f>ROUND(F157*1.4,-5)</ns0:f>
-        <ns0:v>2.77498926669713e+25</ns0:v>
+        <ns0:v>1.850452284164535e+33</ns0:v>
       </ns0:c>
       <ns0:c r="G158" s="1" t="n">
         <ns0:v>31.8000000000001</ns0:v>
@@ -6125,15 +6098,15 @@
       </ns0:c>
       <ns0:c r="D159" s="1">
         <ns0:f>ROUND(D158*20,2-INT(LOG10(ABS(D158*20))))</ns0:f>
-        <ns0:v>7.48e+168</ns0:v>
+        <ns0:v>8.48e+173</ns0:v>
       </ns0:c>
       <ns0:c r="E159" s="1">
         <ns0:f>D159</ns0:f>
-        <ns0:v>7.48e+168</ns0:v>
+        <ns0:v>8.48e+173</ns0:v>
       </ns0:c>
       <ns0:c r="F159" s="1">
         <ns0:f>ROUND(F158*1.4,-5)</ns0:f>
-        <ns0:v>3.88498497337598e+25</ns0:v>
+        <ns0:v>2.590633197830349e+33</ns0:v>
       </ns0:c>
       <ns0:c r="G159" s="1" t="n">
         <ns0:v>32.0000000000001</ns0:v>
@@ -6157,15 +6130,15 @@
       </ns0:c>
       <ns0:c r="D160" s="1">
         <ns0:f>ROUND(D159*20,2-INT(LOG10(ABS(D159*20))))</ns0:f>
-        <ns0:v>1.5e+170</ns0:v>
+        <ns0:v>1.6999999999999998e+175</ns0:v>
       </ns0:c>
       <ns0:c r="E160" s="1">
         <ns0:f>D160</ns0:f>
-        <ns0:v>1.5e+170</ns0:v>
+        <ns0:v>1.6999999999999998e+175</ns0:v>
       </ns0:c>
       <ns0:c r="F160" s="1">
         <ns0:f>ROUND(F159*1.4,-5)</ns0:f>
-        <ns0:v>5.43897896272637e+25</ns0:v>
+        <ns0:v>3.6268864769624885e+33</ns0:v>
       </ns0:c>
       <ns0:c r="G160" s="1" t="n">
         <ns0:v>32.2000000000001</ns0:v>
@@ -6189,15 +6162,15 @@
       </ns0:c>
       <ns0:c r="D161" s="1">
         <ns0:f>ROUND(D160*20,2-INT(LOG10(ABS(D160*20))))</ns0:f>
-        <ns0:v>3e+171</ns0:v>
+        <ns0:v>3.4e+176</ns0:v>
       </ns0:c>
       <ns0:c r="E161" s="1">
         <ns0:f>D161</ns0:f>
-        <ns0:v>3e+171</ns0:v>
+        <ns0:v>3.4e+176</ns0:v>
       </ns0:c>
       <ns0:c r="F161" s="1">
         <ns0:f>ROUND(F160*1.4,-5)</ns0:f>
-        <ns0:v>7.61457054781692e+25</ns0:v>
+        <ns0:v>5.077641067747484e+33</ns0:v>
       </ns0:c>
       <ns0:c r="G161" s="1" t="n">
         <ns0:v>32.4000000000001</ns0:v>
@@ -6221,15 +6194,15 @@
       </ns0:c>
       <ns0:c r="D162" s="1">
         <ns0:f>ROUND(D161*20,2-INT(LOG10(ABS(D161*20))))</ns0:f>
-        <ns0:v>6e+172</ns0:v>
+        <ns0:v>6.8e+177</ns0:v>
       </ns0:c>
       <ns0:c r="E162" s="1">
         <ns0:f>D162</ns0:f>
-        <ns0:v>6e+172</ns0:v>
+        <ns0:v>6.8e+177</ns0:v>
       </ns0:c>
       <ns0:c r="F162" s="1">
         <ns0:f>ROUND(F161*1.4,-5)</ns0:f>
-        <ns0:v>1.06603987669437e+26</ns0:v>
+        <ns0:v>7.108697494846477e+33</ns0:v>
       </ns0:c>
       <ns0:c r="G162" s="1" t="n">
         <ns0:v>32.6000000000001</ns0:v>
@@ -6253,15 +6226,15 @@
       </ns0:c>
       <ns0:c r="D163" s="1">
         <ns0:f>ROUND(D162*20,2-INT(LOG10(ABS(D162*20))))</ns0:f>
-        <ns0:v>1.2e+174</ns0:v>
+        <ns0:v>1.36e+179</ns0:v>
       </ns0:c>
       <ns0:c r="E163" s="1">
         <ns0:f>D163</ns0:f>
-        <ns0:v>1.2e+174</ns0:v>
+        <ns0:v>1.36e+179</ns0:v>
       </ns0:c>
       <ns0:c r="F163" s="1">
         <ns0:f>ROUND(F162*1.4,-5)</ns0:f>
-        <ns0:v>1.49245582737212e+26</ns0:v>
+        <ns0:v>9.952176492785067e+33</ns0:v>
       </ns0:c>
       <ns0:c r="G163" s="1" t="n">
         <ns0:v>32.8000000000001</ns0:v>
@@ -6285,15 +6258,15 @@
       </ns0:c>
       <ns0:c r="D164" s="1">
         <ns0:f>ROUND(D163*20,2-INT(LOG10(ABS(D163*20))))</ns0:f>
-        <ns0:v>2.4e+175</ns0:v>
+        <ns0:v>2.72e+180</ns0:v>
       </ns0:c>
       <ns0:c r="E164" s="1">
         <ns0:f>D164</ns0:f>
-        <ns0:v>2.4e+175</ns0:v>
+        <ns0:v>2.72e+180</ns0:v>
       </ns0:c>
       <ns0:c r="F164" s="1">
         <ns0:f>ROUND(F163*1.4,-5)</ns0:f>
-        <ns0:v>2.08943815832097e+26</ns0:v>
+        <ns0:v>1.3933047089899093e+34</ns0:v>
       </ns0:c>
       <ns0:c r="G164" s="1" t="n">
         <ns0:v>33.0000000000001</ns0:v>
@@ -6317,15 +6290,15 @@
       </ns0:c>
       <ns0:c r="D165" s="1">
         <ns0:f>ROUND(D164*20,2-INT(LOG10(ABS(D164*20))))</ns0:f>
-        <ns0:v>4.8e+176</ns0:v>
+        <ns0:v>5.44e+181</ns0:v>
       </ns0:c>
       <ns0:c r="E165" s="1">
         <ns0:f>D165</ns0:f>
-        <ns0:v>4.8e+176</ns0:v>
+        <ns0:v>5.44e+181</ns0:v>
       </ns0:c>
       <ns0:c r="F165" s="1">
         <ns0:f>ROUND(F164*1.4,-5)</ns0:f>
-        <ns0:v>2.92521342164936e+26</ns0:v>
+        <ns0:v>1.950626592585873e+34</ns0:v>
       </ns0:c>
       <ns0:c r="G165" s="1" t="n">
         <ns0:v>33.2000000000001</ns0:v>
@@ -6349,15 +6322,15 @@
       </ns0:c>
       <ns0:c r="D166" s="1">
         <ns0:f>ROUND(D165*20,2-INT(LOG10(ABS(D165*20))))</ns0:f>
-        <ns0:v>9.6e+177</ns0:v>
+        <ns0:v>1.09e+183</ns0:v>
       </ns0:c>
       <ns0:c r="E166" s="1">
         <ns0:f>D166</ns0:f>
-        <ns0:v>9.6e+177</ns0:v>
+        <ns0:v>1.09e+183</ns0:v>
       </ns0:c>
       <ns0:c r="F166" s="1">
         <ns0:f>ROUND(F165*1.4,-5)</ns0:f>
-        <ns0:v>4.0952987903091e+26</ns0:v>
+        <ns0:v>2.730877229620222e+34</ns0:v>
       </ns0:c>
       <ns0:c r="G166" s="1" t="n">
         <ns0:v>33.4000000000001</ns0:v>
@@ -6381,15 +6354,15 @@
       </ns0:c>
       <ns0:c r="D167" s="1">
         <ns0:f>ROUND(D166*20,2-INT(LOG10(ABS(D166*20))))</ns0:f>
-        <ns0:v>1.92e+179</ns0:v>
+        <ns0:v>2.18e+184</ns0:v>
       </ns0:c>
       <ns0:c r="E167" s="1">
         <ns0:f>D167</ns0:f>
-        <ns0:v>1.92e+179</ns0:v>
+        <ns0:v>2.18e+184</ns0:v>
       </ns0:c>
       <ns0:c r="F167" s="1">
         <ns0:f>ROUND(F166*1.4,-5)</ns0:f>
-        <ns0:v>5.73341830643274e+26</ns0:v>
+        <ns0:v>3.823228121468311e+34</ns0:v>
       </ns0:c>
       <ns0:c r="G167" s="1" t="n">
         <ns0:v>33.6000000000001</ns0:v>
@@ -6413,15 +6386,15 @@
       </ns0:c>
       <ns0:c r="D168" s="1">
         <ns0:f>ROUND(D167*20,2-INT(LOG10(ABS(D167*20))))</ns0:f>
-        <ns0:v>3.84e+180</ns0:v>
+        <ns0:v>4.36e+185</ns0:v>
       </ns0:c>
       <ns0:c r="E168" s="1">
         <ns0:f>D168</ns0:f>
-        <ns0:v>3.84e+180</ns0:v>
+        <ns0:v>4.36e+185</ns0:v>
       </ns0:c>
       <ns0:c r="F168" s="1">
         <ns0:f>ROUND(F167*1.4,-5)</ns0:f>
-        <ns0:v>8.02678562900584e+26</ns0:v>
+        <ns0:v>5.352519370055635e+34</ns0:v>
       </ns0:c>
       <ns0:c r="G168" s="1" t="n">
         <ns0:v>33.8000000000001</ns0:v>
@@ -6445,15 +6418,15 @@
       </ns0:c>
       <ns0:c r="D169" s="1">
         <ns0:f>ROUND(D168*20,2-INT(LOG10(ABS(D168*20))))</ns0:f>
-        <ns0:v>7.68e+181</ns0:v>
+        <ns0:v>8.72e+186</ns0:v>
       </ns0:c>
       <ns0:c r="E169" s="1">
         <ns0:f>D169</ns0:f>
-        <ns0:v>7.68e+181</ns0:v>
+        <ns0:v>8.72e+186</ns0:v>
       </ns0:c>
       <ns0:c r="F169" s="1">
         <ns0:f>ROUND(F168*1.4,-5)</ns0:f>
-        <ns0:v>1.12374998806082e+27</ns0:v>
+        <ns0:v>7.493527118077889e+34</ns0:v>
       </ns0:c>
       <ns0:c r="G169" s="1" t="n">
         <ns0:v>34.0000000000001</ns0:v>
@@ -6477,15 +6450,15 @@
       </ns0:c>
       <ns0:c r="D170" s="1">
         <ns0:f>ROUND(D169*20,2-INT(LOG10(ABS(D169*20))))</ns0:f>
-        <ns0:v>1.54e+183</ns0:v>
+        <ns0:v>1.7400000000000002e+188</ns0:v>
       </ns0:c>
       <ns0:c r="E170" s="1">
         <ns0:f>D170</ns0:f>
-        <ns0:v>1.54e+183</ns0:v>
+        <ns0:v>1.7400000000000002e+188</ns0:v>
       </ns0:c>
       <ns0:c r="F170" s="1">
         <ns0:f>ROUND(F169*1.4,-5)</ns0:f>
-        <ns0:v>1.57324998328515e+27</ns0:v>
+        <ns0:v>1.0490937965309043e+35</ns0:v>
       </ns0:c>
       <ns0:c r="G170" s="1" t="n">
         <ns0:v>34.2000000000001</ns0:v>
@@ -6509,15 +6482,15 @@
       </ns0:c>
       <ns0:c r="D171" s="1">
         <ns0:f>ROUND(D170*20,2-INT(LOG10(ABS(D170*20))))</ns0:f>
-        <ns0:v>3.08e+184</ns0:v>
+        <ns0:v>3.48e+189</ns0:v>
       </ns0:c>
       <ns0:c r="E171" s="1">
         <ns0:f>D171</ns0:f>
-        <ns0:v>3.08e+184</ns0:v>
+        <ns0:v>3.48e+189</ns0:v>
       </ns0:c>
       <ns0:c r="F171" s="1">
         <ns0:f>ROUND(F170*1.4,-5)</ns0:f>
-        <ns0:v>2.20254997659921e+27</ns0:v>
+        <ns0:v>1.468731315143266e+35</ns0:v>
       </ns0:c>
       <ns0:c r="G171" s="1" t="n">
         <ns0:v>34.4000000000001</ns0:v>
@@ -6541,15 +6514,15 @@
       </ns0:c>
       <ns0:c r="D172" s="1">
         <ns0:f>ROUND(D171*20,2-INT(LOG10(ABS(D171*20))))</ns0:f>
-        <ns0:v>6.16e+185</ns0:v>
+        <ns0:v>6.96e+190</ns0:v>
       </ns0:c>
       <ns0:c r="E172" s="1">
         <ns0:f>D172</ns0:f>
-        <ns0:v>6.16e+185</ns0:v>
+        <ns0:v>6.96e+190</ns0:v>
       </ns0:c>
       <ns0:c r="F172" s="1">
         <ns0:f>ROUND(F171*1.4,-5)</ns0:f>
-        <ns0:v>3.08356996723889e+27</ns0:v>
+        <ns0:v>2.056223841200572e+35</ns0:v>
       </ns0:c>
       <ns0:c r="G172" s="1" t="n">
         <ns0:v>34.6000000000001</ns0:v>
@@ -6573,15 +6546,15 @@
       </ns0:c>
       <ns0:c r="D173" s="1">
         <ns0:f>ROUND(D172*20,2-INT(LOG10(ABS(D172*20))))</ns0:f>
-        <ns0:v>1.23e+187</ns0:v>
+        <ns0:v>1.39e+192</ns0:v>
       </ns0:c>
       <ns0:c r="E173" s="1">
         <ns0:f>D173</ns0:f>
-        <ns0:v>1.23e+187</ns0:v>
+        <ns0:v>1.39e+192</ns0:v>
       </ns0:c>
       <ns0:c r="F173" s="1">
         <ns0:f>ROUND(F172*1.4,-5)</ns0:f>
-        <ns0:v>4.31699795413445e+27</ns0:v>
+        <ns0:v>2.8787133776808006e+35</ns0:v>
       </ns0:c>
       <ns0:c r="G173" s="1" t="n">
         <ns0:v>34.8000000000001</ns0:v>
@@ -6605,15 +6578,15 @@
       </ns0:c>
       <ns0:c r="D174" s="1">
         <ns0:f>ROUND(D173*20,2-INT(LOG10(ABS(D173*20))))</ns0:f>
-        <ns0:v>2.46e+188</ns0:v>
+        <ns0:v>2.78e+193</ns0:v>
       </ns0:c>
       <ns0:c r="E174" s="1">
         <ns0:f>D174</ns0:f>
-        <ns0:v>2.46e+188</ns0:v>
+        <ns0:v>2.78e+193</ns0:v>
       </ns0:c>
       <ns0:c r="F174" s="1">
         <ns0:f>ROUND(F173*1.4,-5)</ns0:f>
-        <ns0:v>6.04379713578823e+27</ns0:v>
+        <ns0:v>4.03019872875312e+35</ns0:v>
       </ns0:c>
       <ns0:c r="G174" s="1" t="n">
         <ns0:v>35.0000000000001</ns0:v>
@@ -6637,15 +6610,15 @@
       </ns0:c>
       <ns0:c r="D175" s="1">
         <ns0:f>ROUND(D174*20,2-INT(LOG10(ABS(D174*20))))</ns0:f>
-        <ns0:v>4.92e+189</ns0:v>
+        <ns0:v>5.5599999999999995e+194</ns0:v>
       </ns0:c>
       <ns0:c r="E175" s="1">
         <ns0:f>D175</ns0:f>
-        <ns0:v>4.92e+189</ns0:v>
+        <ns0:v>5.5599999999999995e+194</ns0:v>
       </ns0:c>
       <ns0:c r="F175" s="1">
         <ns0:f>ROUND(F174*1.4,-5)</ns0:f>
-        <ns0:v>8.46131599010352e+27</ns0:v>
+        <ns0:v>5.642278220254368e+35</ns0:v>
       </ns0:c>
       <ns0:c r="G175" s="1" t="n">
         <ns0:v>35.2000000000001</ns0:v>
@@ -6669,15 +6642,15 @@
       </ns0:c>
       <ns0:c r="D176" s="1">
         <ns0:f>ROUND(D175*20,2-INT(LOG10(ABS(D175*20))))</ns0:f>
-        <ns0:v>9.84e+190</ns0:v>
+        <ns0:v>1.11e+196</ns0:v>
       </ns0:c>
       <ns0:c r="E176" s="1">
         <ns0:f>D176</ns0:f>
-        <ns0:v>9.84e+190</ns0:v>
+        <ns0:v>1.11e+196</ns0:v>
       </ns0:c>
       <ns0:c r="F176" s="1">
         <ns0:f>ROUND(F175*1.4,-5)</ns0:f>
-        <ns0:v>1.18458423861449e+28</ns0:v>
+        <ns0:v>7.899189508356115e+35</ns0:v>
       </ns0:c>
       <ns0:c r="G176" s="1" t="n">
         <ns0:v>35.4000000000001</ns0:v>
@@ -6701,15 +6674,15 @@
       </ns0:c>
       <ns0:c r="D177" s="1">
         <ns0:f>ROUND(D176*20,2-INT(LOG10(ABS(D176*20))))</ns0:f>
-        <ns0:v>1.97e+192</ns0:v>
+        <ns0:v>2.22e+197</ns0:v>
       </ns0:c>
       <ns0:c r="E177" s="1">
         <ns0:f>D177</ns0:f>
-        <ns0:v>1.97e+192</ns0:v>
+        <ns0:v>2.22e+197</ns0:v>
       </ns0:c>
       <ns0:c r="F177" s="1">
         <ns0:f>ROUND(F176*1.4,-5)</ns0:f>
-        <ns0:v>1.65841793406029e+28</ns0:v>
+        <ns0:v>1.105886531169856e+36</ns0:v>
       </ns0:c>
       <ns0:c r="G177" s="1" t="n">
         <ns0:v>35.6000000000001</ns0:v>
@@ -6733,15 +6706,15 @@
       </ns0:c>
       <ns0:c r="D178" s="1">
         <ns0:f>ROUND(D177*20,2-INT(LOG10(ABS(D177*20))))</ns0:f>
-        <ns0:v>3.94e+193</ns0:v>
+        <ns0:v>4.44e+198</ns0:v>
       </ns0:c>
       <ns0:c r="E178" s="1">
         <ns0:f>D178</ns0:f>
-        <ns0:v>3.94e+193</ns0:v>
+        <ns0:v>4.44e+198</ns0:v>
       </ns0:c>
       <ns0:c r="F178" s="1">
         <ns0:f>ROUND(F177*1.4,-5)</ns0:f>
-        <ns0:v>2.32178510768441e+28</ns0:v>
+        <ns0:v>1.5482411436377982e+36</ns0:v>
       </ns0:c>
       <ns0:c r="G178" s="1" t="n">
         <ns0:v>35.8000000000001</ns0:v>
@@ -6765,15 +6738,15 @@
       </ns0:c>
       <ns0:c r="D179" s="1">
         <ns0:f>ROUND(D178*20,2-INT(LOG10(ABS(D178*20))))</ns0:f>
-        <ns0:v>7.88e+194</ns0:v>
+        <ns0:v>8.88e+199</ns0:v>
       </ns0:c>
       <ns0:c r="E179" s="1">
         <ns0:f>D179</ns0:f>
-        <ns0:v>7.88e+194</ns0:v>
+        <ns0:v>8.88e+199</ns0:v>
       </ns0:c>
       <ns0:c r="F179" s="1">
         <ns0:f>ROUND(F178*1.4,-5)</ns0:f>
-        <ns0:v>3.25049915075817e+28</ns0:v>
+        <ns0:v>2.1675376010929173e+36</ns0:v>
       </ns0:c>
       <ns0:c r="G179" s="1" t="n">
         <ns0:v>36.0000000000001</ns0:v>
@@ -6797,15 +6770,15 @@
       </ns0:c>
       <ns0:c r="D180" s="1">
         <ns0:f>ROUND(D179*20,2-INT(LOG10(ABS(D179*20))))</ns0:f>
-        <ns0:v>1.58e+196</ns0:v>
+        <ns0:v>1.78e+201</ns0:v>
       </ns0:c>
       <ns0:c r="E180" s="1">
         <ns0:f>D180</ns0:f>
-        <ns0:v>1.58e+196</ns0:v>
+        <ns0:v>1.78e+201</ns0:v>
       </ns0:c>
       <ns0:c r="F180" s="1">
         <ns0:f>ROUND(F179*1.4,-5)</ns0:f>
-        <ns0:v>4.55069881106144e+28</ns0:v>
+        <ns0:v>3.034552641530084e+36</ns0:v>
       </ns0:c>
       <ns0:c r="G180" s="1" t="n">
         <ns0:v>36.2000000000001</ns0:v>
@@ -6829,15 +6802,15 @@
       </ns0:c>
       <ns0:c r="D181" s="1">
         <ns0:f>ROUND(D180*20,2-INT(LOG10(ABS(D180*20))))</ns0:f>
-        <ns0:v>3.16e+197</ns0:v>
+        <ns0:v>3.5600000000000003e+202</ns0:v>
       </ns0:c>
       <ns0:c r="E181" s="1">
         <ns0:f>D181</ns0:f>
-        <ns0:v>3.16e+197</ns0:v>
+        <ns0:v>3.5600000000000003e+202</ns0:v>
       </ns0:c>
       <ns0:c r="F181" s="1">
         <ns0:f>ROUND(F180*1.4,-5)</ns0:f>
-        <ns0:v>6.37097833548602e+28</ns0:v>
+        <ns0:v>4.2483736981421174e+36</ns0:v>
       </ns0:c>
       <ns0:c r="G181" s="1" t="n">
         <ns0:v>36.4000000000001</ns0:v>
@@ -6861,15 +6834,15 @@
       </ns0:c>
       <ns0:c r="D182" s="1">
         <ns0:f>ROUND(D181*20,2-INT(LOG10(ABS(D181*20))))</ns0:f>
-        <ns0:v>6.32e+198</ns0:v>
+        <ns0:v>7.120000000000001e+203</ns0:v>
       </ns0:c>
       <ns0:c r="E182" s="1">
         <ns0:f>D182</ns0:f>
-        <ns0:v>6.32e+198</ns0:v>
+        <ns0:v>7.120000000000001e+203</ns0:v>
       </ns0:c>
       <ns0:c r="F182" s="1">
         <ns0:f>ROUND(F181*1.4,-5)</ns0:f>
-        <ns0:v>8.91936966968043e+28</ns0:v>
+        <ns0:v>5.947723177398964e+36</ns0:v>
       </ns0:c>
       <ns0:c r="G182" s="1" t="n">
         <ns0:v>36.6000000000001</ns0:v>
@@ -6893,15 +6866,15 @@
       </ns0:c>
       <ns0:c r="D183" s="1">
         <ns0:f>ROUND(D182*20,2-INT(LOG10(ABS(D182*20))))</ns0:f>
-        <ns0:v>1.26e+200</ns0:v>
+        <ns0:v>1.42e+205</ns0:v>
       </ns0:c>
       <ns0:c r="E183" s="1">
         <ns0:f>D183</ns0:f>
-        <ns0:v>1.26e+200</ns0:v>
+        <ns0:v>1.42e+205</ns0:v>
       </ns0:c>
       <ns0:c r="F183" s="1">
         <ns0:f>ROUND(F182*1.4,-5)</ns0:f>
-        <ns0:v>1.24871175375526e+29</ns0:v>
+        <ns0:v>8.326812448358549e+36</ns0:v>
       </ns0:c>
       <ns0:c r="G183" s="1" t="n">
         <ns0:v>36.8000000000001</ns0:v>
@@ -6925,15 +6898,15 @@
       </ns0:c>
       <ns0:c r="D184" s="1">
         <ns0:f>ROUND(D183*20,2-INT(LOG10(ABS(D183*20))))</ns0:f>
-        <ns0:v>2.52e+201</ns0:v>
+        <ns0:v>2.84e+206</ns0:v>
       </ns0:c>
       <ns0:c r="E184" s="1">
         <ns0:f>D184</ns0:f>
-        <ns0:v>2.52e+201</ns0:v>
+        <ns0:v>2.84e+206</ns0:v>
       </ns0:c>
       <ns0:c r="F184" s="1">
         <ns0:f>ROUND(F183*1.4,-5)</ns0:f>
-        <ns0:v>1.74819645525736e+29</ns0:v>
+        <ns0:v>1.1657537427701967e+37</ns0:v>
       </ns0:c>
       <ns0:c r="G184" s="1" t="n">
         <ns0:v>37.0000000000001</ns0:v>
@@ -6957,15 +6930,15 @@
       </ns0:c>
       <ns0:c r="D185" s="1">
         <ns0:f>ROUND(D184*20,2-INT(LOG10(ABS(D184*20))))</ns0:f>
-        <ns0:v>5.04e+202</ns0:v>
+        <ns0:v>5.68e+207</ns0:v>
       </ns0:c>
       <ns0:c r="E185" s="1">
         <ns0:f>D185</ns0:f>
-        <ns0:v>5.04e+202</ns0:v>
+        <ns0:v>5.68e+207</ns0:v>
       </ns0:c>
       <ns0:c r="F185" s="1">
         <ns0:f>ROUND(F184*1.4,-5)</ns0:f>
-        <ns0:v>2.4474750373603e+29</ns0:v>
+        <ns0:v>1.6320552398782752e+37</ns0:v>
       </ns0:c>
       <ns0:c r="G185" s="1" t="n">
         <ns0:v>37.2000000000001</ns0:v>
@@ -6989,15 +6962,15 @@
       </ns0:c>
       <ns0:c r="D186" s="1">
         <ns0:f>ROUND(D185*20,2-INT(LOG10(ABS(D185*20))))</ns0:f>
-        <ns0:v>1.01e+204</ns0:v>
+        <ns0:v>1.14e+209</ns0:v>
       </ns0:c>
       <ns0:c r="E186" s="1">
         <ns0:f>D186</ns0:f>
-        <ns0:v>1.01e+204</ns0:v>
+        <ns0:v>1.14e+209</ns0:v>
       </ns0:c>
       <ns0:c r="F186" s="1">
         <ns0:f>ROUND(F185*1.4,-5)</ns0:f>
-        <ns0:v>3.42646505230442e+29</ns0:v>
+        <ns0:v>2.284877335829585e+37</ns0:v>
       </ns0:c>
       <ns0:c r="G186" s="1" t="n">
         <ns0:v>37.4000000000001</ns0:v>
@@ -7021,15 +6994,15 @@
       </ns0:c>
       <ns0:c r="D187" s="1">
         <ns0:f>ROUND(D186*20,2-INT(LOG10(ABS(D186*20))))</ns0:f>
-        <ns0:v>2.02e+205</ns0:v>
+        <ns0:v>2.2799999999999998e+210</ns0:v>
       </ns0:c>
       <ns0:c r="E187" s="1">
         <ns0:f>D187</ns0:f>
-        <ns0:v>2.02e+205</ns0:v>
+        <ns0:v>2.2799999999999998e+210</ns0:v>
       </ns0:c>
       <ns0:c r="F187" s="1">
         <ns0:f>ROUND(F186*1.4,-5)</ns0:f>
-        <ns0:v>4.79705107322619e+29</ns0:v>
+        <ns0:v>3.198828270161419e+37</ns0:v>
       </ns0:c>
       <ns0:c r="G187" s="1" t="n">
         <ns0:v>37.6000000000001</ns0:v>
@@ -7053,15 +7026,15 @@
       </ns0:c>
       <ns0:c r="D188" s="1">
         <ns0:f>ROUND(D187*20,2-INT(LOG10(ABS(D187*20))))</ns0:f>
-        <ns0:v>4.04e+206</ns0:v>
+        <ns0:v>4.56e+211</ns0:v>
       </ns0:c>
       <ns0:c r="E188" s="1">
         <ns0:f>D188</ns0:f>
-        <ns0:v>4.04e+206</ns0:v>
+        <ns0:v>4.56e+211</ns0:v>
       </ns0:c>
       <ns0:c r="F188" s="1">
         <ns0:f>ROUND(F187*1.4,-5)</ns0:f>
-        <ns0:v>6.71587150251667e+29</ns0:v>
+        <ns0:v>4.478359578225986e+37</ns0:v>
       </ns0:c>
       <ns0:c r="G188" s="1" t="n">
         <ns0:v>37.8000000000001</ns0:v>
@@ -7085,15 +7058,15 @@
       </ns0:c>
       <ns0:c r="D189" s="1">
         <ns0:f>ROUND(D188*20,2-INT(LOG10(ABS(D188*20))))</ns0:f>
-        <ns0:v>8.08e+207</ns0:v>
+        <ns0:v>9.12e+212</ns0:v>
       </ns0:c>
       <ns0:c r="E189" s="1">
         <ns0:f>D189</ns0:f>
-        <ns0:v>8.08e+207</ns0:v>
+        <ns0:v>9.12e+212</ns0:v>
       </ns0:c>
       <ns0:c r="F189" s="1">
         <ns0:f>ROUND(F188*1.4,-5)</ns0:f>
-        <ns0:v>9.40222010352334e+29</ns0:v>
+        <ns0:v>6.26970340951638e+37</ns0:v>
       </ns0:c>
       <ns0:c r="G189" s="1" t="n">
         <ns0:v>38.0000000000001</ns0:v>
@@ -7117,15 +7090,15 @@
       </ns0:c>
       <ns0:c r="D190" s="1">
         <ns0:f>ROUND(D189*20,2-INT(LOG10(ABS(D189*20))))</ns0:f>
-        <ns0:v>1.62e+209</ns0:v>
+        <ns0:v>1.8200000000000001e+214</ns0:v>
       </ns0:c>
       <ns0:c r="E190" s="1">
         <ns0:f>D190</ns0:f>
-        <ns0:v>1.62e+209</ns0:v>
+        <ns0:v>1.8200000000000001e+214</ns0:v>
       </ns0:c>
       <ns0:c r="F190" s="1">
         <ns0:f>ROUND(F189*1.4,-5)</ns0:f>
-        <ns0:v>1.31631081449327e+30</ns0:v>
+        <ns0:v>8.777584773322933e+37</ns0:v>
       </ns0:c>
       <ns0:c r="G190" s="1" t="n">
         <ns0:v>38.2000000000001</ns0:v>
@@ -7149,15 +7122,15 @@
       </ns0:c>
       <ns0:c r="D191" s="1">
         <ns0:f>ROUND(D190*20,2-INT(LOG10(ABS(D190*20))))</ns0:f>
-        <ns0:v>3.24e+210</ns0:v>
+        <ns0:v>3.64e+215</ns0:v>
       </ns0:c>
       <ns0:c r="E191" s="1">
         <ns0:f>D191</ns0:f>
-        <ns0:v>3.24e+210</ns0:v>
+        <ns0:v>3.64e+215</ns0:v>
       </ns0:c>
       <ns0:c r="F191" s="1">
         <ns0:f>ROUND(F190*1.4,-5)</ns0:f>
-        <ns0:v>1.84283514029058e+30</ns0:v>
+        <ns0:v>1.2288618682652105e+38</ns0:v>
       </ns0:c>
       <ns0:c r="G191" s="1" t="n">
         <ns0:v>38.4000000000001</ns0:v>
@@ -7181,15 +7154,15 @@
       </ns0:c>
       <ns0:c r="D192" s="1">
         <ns0:f>ROUND(D191*20,2-INT(LOG10(ABS(D191*20))))</ns0:f>
-        <ns0:v>6.48e+211</ns0:v>
+        <ns0:v>7.28e+216</ns0:v>
       </ns0:c>
       <ns0:c r="E192" s="1">
         <ns0:f>D192</ns0:f>
-        <ns0:v>6.48e+211</ns0:v>
+        <ns0:v>7.28e+216</ns0:v>
       </ns0:c>
       <ns0:c r="F192" s="1">
         <ns0:f>ROUND(F191*1.4,-5)</ns0:f>
-        <ns0:v>2.57996919640681e+30</ns0:v>
+        <ns0:v>1.7204066155712946e+38</ns0:v>
       </ns0:c>
       <ns0:c r="G192" s="1" t="n">
         <ns0:v>38.6000000000001</ns0:v>
@@ -7213,15 +7186,15 @@
       </ns0:c>
       <ns0:c r="D193" s="1">
         <ns0:f>ROUND(D192*20,2-INT(LOG10(ABS(D192*20))))</ns0:f>
-        <ns0:v>1.3e+213</ns0:v>
+        <ns0:v>1.4599999999999999e+218</ns0:v>
       </ns0:c>
       <ns0:c r="E193" s="1">
         <ns0:f>D193</ns0:f>
-        <ns0:v>1.3e+213</ns0:v>
+        <ns0:v>1.4599999999999999e+218</ns0:v>
       </ns0:c>
       <ns0:c r="F193" s="1">
         <ns0:f>ROUND(F192*1.4,-5)</ns0:f>
-        <ns0:v>3.61195687496953e+30</ns0:v>
+        <ns0:v>2.4085692617998124e+38</ns0:v>
       </ns0:c>
       <ns0:c r="G193" s="1" t="n">
         <ns0:v>38.8000000000001</ns0:v>
@@ -7245,15 +7218,15 @@
       </ns0:c>
       <ns0:c r="D194" s="1">
         <ns0:f>ROUND(D193*20,2-INT(LOG10(ABS(D193*20))))</ns0:f>
-        <ns0:v>2.6e+214</ns0:v>
+        <ns0:v>2.9199999999999997e+219</ns0:v>
       </ns0:c>
       <ns0:c r="E194" s="1">
         <ns0:f>D194</ns0:f>
-        <ns0:v>2.6e+214</ns0:v>
+        <ns0:v>2.9199999999999997e+219</ns0:v>
       </ns0:c>
       <ns0:c r="F194" s="1">
         <ns0:f>ROUND(F193*1.4,-5)</ns0:f>
-        <ns0:v>5.05673962495734e+30</ns0:v>
+        <ns0:v>3.371996966519737e+38</ns0:v>
       </ns0:c>
       <ns0:c r="G194" s="1" t="n">
         <ns0:v>39.0000000000001</ns0:v>
@@ -7277,15 +7250,15 @@
       </ns0:c>
       <ns0:c r="D195" s="1">
         <ns0:f>ROUND(D194*20,2-INT(LOG10(ABS(D194*20))))</ns0:f>
-        <ns0:v>5.2e+215</ns0:v>
+        <ns0:v>5.84e+220</ns0:v>
       </ns0:c>
       <ns0:c r="E195" s="1">
         <ns0:f>D195</ns0:f>
-        <ns0:v>5.2e+215</ns0:v>
+        <ns0:v>5.84e+220</ns0:v>
       </ns0:c>
       <ns0:c r="F195" s="1">
         <ns0:f>ROUND(F194*1.4,-5)</ns0:f>
-        <ns0:v>7.07943547494028e+30</ns0:v>
+        <ns0:v>4.720795753127631e+38</ns0:v>
       </ns0:c>
       <ns0:c r="G195" s="1" t="n">
         <ns0:v>39.2000000000001</ns0:v>
@@ -7309,15 +7282,15 @@
       </ns0:c>
       <ns0:c r="D196" s="1">
         <ns0:f>ROUND(D195*20,2-INT(LOG10(ABS(D195*20))))</ns0:f>
-        <ns0:v>1.04e+217</ns0:v>
+        <ns0:v>1.17e+222</ns0:v>
       </ns0:c>
       <ns0:c r="E196" s="1">
         <ns0:f>D196</ns0:f>
-        <ns0:v>1.04e+217</ns0:v>
+        <ns0:v>1.17e+222</ns0:v>
       </ns0:c>
       <ns0:c r="F196" s="1">
         <ns0:f>ROUND(F195*1.4,-5)</ns0:f>
-        <ns0:v>9.91120966491639e+30</ns0:v>
+        <ns0:v>6.6091140543786836e+38</ns0:v>
       </ns0:c>
       <ns0:c r="G196" s="1" t="n">
         <ns0:v>39.4000000000001</ns0:v>
@@ -7341,15 +7314,15 @@
       </ns0:c>
       <ns0:c r="D197" s="1">
         <ns0:f>ROUND(D196*20,2-INT(LOG10(ABS(D196*20))))</ns0:f>
-        <ns0:v>2.08e+218</ns0:v>
+        <ns0:v>2.34e+223</ns0:v>
       </ns0:c>
       <ns0:c r="E197" s="1">
         <ns0:f>D197</ns0:f>
-        <ns0:v>2.08e+218</ns0:v>
+        <ns0:v>2.34e+223</ns0:v>
       </ns0:c>
       <ns0:c r="F197" s="1">
         <ns0:f>ROUND(F196*1.4,-5)</ns0:f>
-        <ns0:v>1.38756935308829e+31</ns0:v>
+        <ns0:v>9.252759676130156e+38</ns0:v>
       </ns0:c>
       <ns0:c r="G197" s="1" t="n">
         <ns0:v>39.6000000000001</ns0:v>
@@ -7373,15 +7346,15 @@
       </ns0:c>
       <ns0:c r="D198" s="1">
         <ns0:f>ROUND(D197*20,2-INT(LOG10(ABS(D197*20))))</ns0:f>
-        <ns0:v>4.16e+219</ns0:v>
+        <ns0:v>4.6799999999999994e+224</ns0:v>
       </ns0:c>
       <ns0:c r="E198" s="1">
         <ns0:f>D198</ns0:f>
-        <ns0:v>4.16e+219</ns0:v>
+        <ns0:v>4.6799999999999994e+224</ns0:v>
       </ns0:c>
       <ns0:c r="F198" s="1">
         <ns0:f>ROUND(F197*1.4,-5)</ns0:f>
-        <ns0:v>1.94259709432361e+31</ns0:v>
+        <ns0:v>1.2953863546582217e+39</ns0:v>
       </ns0:c>
       <ns0:c r="G198" s="1" t="n">
         <ns0:v>39.8000000000001</ns0:v>
@@ -7405,15 +7378,15 @@
       </ns0:c>
       <ns0:c r="D199" s="1">
         <ns0:f>ROUND(D198*20,2-INT(LOG10(ABS(D198*20))))</ns0:f>
-        <ns0:v>8.32e+220</ns0:v>
+        <ns0:v>9.360000000000001e+225</ns0:v>
       </ns0:c>
       <ns0:c r="E199" s="1">
         <ns0:f>D199</ns0:f>
-        <ns0:v>8.32e+220</ns0:v>
+        <ns0:v>9.360000000000001e+225</ns0:v>
       </ns0:c>
       <ns0:c r="F199" s="1">
         <ns0:f>ROUND(F198*1.4,-5)</ns0:f>
-        <ns0:v>2.71963593205305e+31</ns0:v>
+        <ns0:v>1.8135408965215102e+39</ns0:v>
       </ns0:c>
       <ns0:c r="G199" s="1" t="n">
         <ns0:v>40.0000000000001</ns0:v>
@@ -7437,15 +7410,15 @@
       </ns0:c>
       <ns0:c r="D200" s="1">
         <ns0:f>ROUND(D199*20,2-INT(LOG10(ABS(D199*20))))</ns0:f>
-        <ns0:v>1.66e+222</ns0:v>
+        <ns0:v>1.8700000000000002e+227</ns0:v>
       </ns0:c>
       <ns0:c r="E200" s="1">
         <ns0:f>D200</ns0:f>
-        <ns0:v>1.66e+222</ns0:v>
+        <ns0:v>1.8700000000000002e+227</ns0:v>
       </ns0:c>
       <ns0:c r="F200" s="1">
         <ns0:f>ROUND(F199*1.4,-5)</ns0:f>
-        <ns0:v>3.80749030487427e+31</ns0:v>
+        <ns0:v>2.538957255130114e+39</ns0:v>
       </ns0:c>
       <ns0:c r="G200" s="1" t="n">
         <ns0:v>40.2000000000001</ns0:v>
@@ -7469,15 +7442,15 @@
       </ns0:c>
       <ns0:c r="D201" s="1">
         <ns0:f>ROUND(D200*20,2-INT(LOG10(ABS(D200*20))))</ns0:f>
-        <ns0:v>3.32e+223</ns0:v>
+        <ns0:v>3.7400000000000006e+228</ns0:v>
       </ns0:c>
       <ns0:c r="E201" s="1">
         <ns0:f>D201</ns0:f>
-        <ns0:v>3.32e+223</ns0:v>
+        <ns0:v>3.7400000000000006e+228</ns0:v>
       </ns0:c>
       <ns0:c r="F201" s="1">
         <ns0:f>ROUND(F200*1.4,-5)</ns0:f>
-        <ns0:v>5.33048642682398e+31</ns0:v>
+        <ns0:v>3.5545401571821595e+39</ns0:v>
       </ns0:c>
       <ns0:c r="G201" s="1" t="n">
         <ns0:v>40.4000000000001</ns0:v>
@@ -7501,15 +7474,15 @@
       </ns0:c>
       <ns0:c r="D202" s="1">
         <ns0:f>ROUND(D201*20,2-INT(LOG10(ABS(D201*20))))</ns0:f>
-        <ns0:v>6.64e+224</ns0:v>
+        <ns0:v>7.48e+229</ns0:v>
       </ns0:c>
       <ns0:c r="E202" s="1">
         <ns0:f>D202</ns0:f>
-        <ns0:v>6.64e+224</ns0:v>
+        <ns0:v>7.48e+229</ns0:v>
       </ns0:c>
       <ns0:c r="F202" s="1">
         <ns0:f>ROUND(F201*1.4,-5)</ns0:f>
-        <ns0:v>7.46268099755357e+31</ns0:v>
+        <ns0:v>4.976356220055024e+39</ns0:v>
       </ns0:c>
       <ns0:c r="G202" s="1" t="n">
         <ns0:v>40.6000000000001</ns0:v>
@@ -7533,15 +7506,15 @@
       </ns0:c>
       <ns0:c r="D203" s="1">
         <ns0:f>ROUND(D202*20,2-INT(LOG10(ABS(D202*20))))</ns0:f>
-        <ns0:v>1.33e+226</ns0:v>
+        <ns0:v>1.4999999999999999e+231</ns0:v>
       </ns0:c>
       <ns0:c r="E203" s="1">
         <ns0:f>D203</ns0:f>
-        <ns0:v>1.33e+226</ns0:v>
+        <ns0:v>1.4999999999999999e+231</ns0:v>
       </ns0:c>
       <ns0:c r="F203" s="1">
         <ns0:f>ROUND(F202*1.4,-5)</ns0:f>
-        <ns0:v>1.0447753396575e+32</ns0:v>
+        <ns0:v>6.966898708077033e+39</ns0:v>
       </ns0:c>
       <ns0:c r="G203" s="1" t="n">
         <ns0:v>40.8000000000001</ns0:v>
@@ -7565,15 +7538,15 @@
       </ns0:c>
       <ns0:c r="D204" s="1">
         <ns0:f>ROUND(D203*20,2-INT(LOG10(ABS(D203*20))))</ns0:f>
-        <ns0:v>2.66e+227</ns0:v>
+        <ns0:v>3e+232</ns0:v>
       </ns0:c>
       <ns0:c r="E204" s="1">
         <ns0:f>D204</ns0:f>
-        <ns0:v>2.66e+227</ns0:v>
+        <ns0:v>3e+232</ns0:v>
       </ns0:c>
       <ns0:c r="F204" s="1">
         <ns0:f>ROUND(F203*1.4,-5)</ns0:f>
-        <ns0:v>1.4626854755205e+32</ns0:v>
+        <ns0:v>9.753658191307845e+39</ns0:v>
       </ns0:c>
       <ns0:c r="G204" s="1" t="n">
         <ns0:v>41.0000000000001</ns0:v>
@@ -7597,15 +7570,15 @@
       </ns0:c>
       <ns0:c r="D205" s="1">
         <ns0:f>ROUND(D204*20,2-INT(LOG10(ABS(D204*20))))</ns0:f>
-        <ns0:v>5.32e+228</ns0:v>
+        <ns0:v>6e+233</ns0:v>
       </ns0:c>
       <ns0:c r="E205" s="1">
         <ns0:f>D205</ns0:f>
-        <ns0:v>5.32e+228</ns0:v>
+        <ns0:v>6e+233</ns0:v>
       </ns0:c>
       <ns0:c r="F205" s="1">
         <ns0:f>ROUND(F204*1.4,-5)</ns0:f>
-        <ns0:v>2.0477596657287e+32</ns0:v>
+        <ns0:v>1.3655121467830982e+40</ns0:v>
       </ns0:c>
       <ns0:c r="G205" s="1" t="n">
         <ns0:v>41.2000000000001</ns0:v>
@@ -7629,15 +7602,15 @@
       </ns0:c>
       <ns0:c r="D206" s="1">
         <ns0:f>ROUND(D205*20,2-INT(LOG10(ABS(D205*20))))</ns0:f>
-        <ns0:v>1.06e+230</ns0:v>
+        <ns0:v>1.2000000000000001e+235</ns0:v>
       </ns0:c>
       <ns0:c r="E206" s="1">
         <ns0:f>D206</ns0:f>
-        <ns0:v>1.06e+230</ns0:v>
+        <ns0:v>1.2000000000000001e+235</ns0:v>
       </ns0:c>
       <ns0:c r="F206" s="1">
         <ns0:f>ROUND(F205*1.4,-5)</ns0:f>
-        <ns0:v>2.86686353202018e+32</ns0:v>
+        <ns0:v>1.9117170054963372e+40</ns0:v>
       </ns0:c>
       <ns0:c r="G206" s="1" t="n">
         <ns0:v>41.4000000000001</ns0:v>
@@ -7661,15 +7634,15 @@
       </ns0:c>
       <ns0:c r="D207" s="1">
         <ns0:f>ROUND(D206*20,2-INT(LOG10(ABS(D206*20))))</ns0:f>
-        <ns0:v>2.12e+231</ns0:v>
+        <ns0:v>2.4e+236</ns0:v>
       </ns0:c>
       <ns0:c r="E207" s="1">
         <ns0:f>D207</ns0:f>
-        <ns0:v>2.12e+231</ns0:v>
+        <ns0:v>2.4e+236</ns0:v>
       </ns0:c>
       <ns0:c r="F207" s="1">
         <ns0:f>ROUND(F206*1.4,-5)</ns0:f>
-        <ns0:v>4.01360894482825e+32</ns0:v>
+        <ns0:v>2.676403807694872e+40</ns0:v>
       </ns0:c>
       <ns0:c r="G207" s="1" t="n">
         <ns0:v>41.6000000000001</ns0:v>
@@ -7693,15 +7666,15 @@
       </ns0:c>
       <ns0:c r="D208" s="1">
         <ns0:f>ROUND(D207*20,2-INT(LOG10(ABS(D207*20))))</ns0:f>
-        <ns0:v>4.24e+232</ns0:v>
+        <ns0:v>4.8000000000000004e+237</ns0:v>
       </ns0:c>
       <ns0:c r="E208" s="1">
         <ns0:f>D208</ns0:f>
-        <ns0:v>4.24e+232</ns0:v>
+        <ns0:v>4.8000000000000004e+237</ns0:v>
       </ns0:c>
       <ns0:c r="F208" s="1">
         <ns0:f>ROUND(F207*1.4,-5)</ns0:f>
-        <ns0:v>5.61905252275955e+32</ns0:v>
+        <ns0:v>3.7469653307728205e+40</ns0:v>
       </ns0:c>
       <ns0:c r="G208" s="1" t="n">
         <ns0:v>41.8000000000001</ns0:v>
@@ -7725,15 +7698,15 @@
       </ns0:c>
       <ns0:c r="D209" s="1">
         <ns0:f>ROUND(D208*20,2-INT(LOG10(ABS(D208*20))))</ns0:f>
-        <ns0:v>8.48e+233</ns0:v>
+        <ns0:v>9.6e+238</ns0:v>
       </ns0:c>
       <ns0:c r="E209" s="1">
         <ns0:f>D209</ns0:f>
-        <ns0:v>8.48e+233</ns0:v>
+        <ns0:v>9.6e+238</ns0:v>
       </ns0:c>
       <ns0:c r="F209" s="1">
         <ns0:f>ROUND(F208*1.4,-5)</ns0:f>
-        <ns0:v>7.86667353186337e+32</ns0:v>
+        <ns0:v>5.245751463081948e+40</ns0:v>
       </ns0:c>
       <ns0:c r="G209" s="1" t="n">
         <ns0:v>42.0000000000001</ns0:v>
@@ -7757,15 +7730,15 @@
       </ns0:c>
       <ns0:c r="D210" s="1">
         <ns0:f>ROUND(D209*20,2-INT(LOG10(ABS(D209*20))))</ns0:f>
-        <ns0:v>1.7e+235</ns0:v>
+        <ns0:v>1.92e+240</ns0:v>
       </ns0:c>
       <ns0:c r="E210" s="1">
         <ns0:f>D210</ns0:f>
-        <ns0:v>1.7e+235</ns0:v>
+        <ns0:v>1.92e+240</ns0:v>
       </ns0:c>
       <ns0:c r="F210" s="1">
         <ns0:f>ROUND(F209*1.4,-5)</ns0:f>
-        <ns0:v>1.10133429446087e+33</ns0:v>
+        <ns0:v>7.344052048314727e+40</ns0:v>
       </ns0:c>
       <ns0:c r="G210" s="1" t="n">
         <ns0:v>42.2000000000001</ns0:v>
@@ -7789,15 +7762,15 @@
       </ns0:c>
       <ns0:c r="D211" s="1">
         <ns0:f>ROUND(D210*20,2-INT(LOG10(ABS(D210*20))))</ns0:f>
-        <ns0:v>3.4e+236</ns0:v>
+        <ns0:v>3.84e+241</ns0:v>
       </ns0:c>
       <ns0:c r="E211" s="1">
         <ns0:f>D211</ns0:f>
-        <ns0:v>3.4e+236</ns0:v>
+        <ns0:v>3.84e+241</ns0:v>
       </ns0:c>
       <ns0:c r="F211" s="1">
         <ns0:f>ROUND(F210*1.4,-5)</ns0:f>
-        <ns0:v>1.54186801224522e+33</ns0:v>
+        <ns0:v>1.0281672867640618e+41</ns0:v>
       </ns0:c>
       <ns0:c r="G211" s="1" t="n">
         <ns0:v>42.4000000000001</ns0:v>
@@ -7821,15 +7794,15 @@
       </ns0:c>
       <ns0:c r="D212" s="1">
         <ns0:f>ROUND(D211*20,2-INT(LOG10(ABS(D211*20))))</ns0:f>
-        <ns0:v>6.8e+237</ns0:v>
+        <ns0:v>7.680000000000001e+242</ns0:v>
       </ns0:c>
       <ns0:c r="E212" s="1">
         <ns0:f>D212</ns0:f>
-        <ns0:v>6.8e+237</ns0:v>
+        <ns0:v>7.680000000000001e+242</ns0:v>
       </ns0:c>
       <ns0:c r="F212" s="1">
         <ns0:f>ROUND(F211*1.4,-5)</ns0:f>
-        <ns0:v>2.15861521714331e+33</ns0:v>
+        <ns0:v>1.4394342014696866e+41</ns0:v>
       </ns0:c>
       <ns0:c r="G212" s="1" t="n">
         <ns0:v>42.6000000000002</ns0:v>
@@ -7853,15 +7826,15 @@
       </ns0:c>
       <ns0:c r="D213" s="1">
         <ns0:f>ROUND(D212*20,2-INT(LOG10(ABS(D212*20))))</ns0:f>
-        <ns0:v>1.36e+239</ns0:v>
+        <ns0:v>1.54e+244</ns0:v>
       </ns0:c>
       <ns0:c r="E213" s="1">
         <ns0:f>D213</ns0:f>
-        <ns0:v>1.36e+239</ns0:v>
+        <ns0:v>1.54e+244</ns0:v>
       </ns0:c>
       <ns0:c r="F213" s="1">
         <ns0:f>ROUND(F212*1.4,-5)</ns0:f>
-        <ns0:v>3.02206130400063e+33</ns0:v>
+        <ns0:v>2.0152078820575612e+41</ns0:v>
       </ns0:c>
       <ns0:c r="G213" s="1" t="n">
         <ns0:v>42.8000000000002</ns0:v>
@@ -7885,15 +7858,15 @@
       </ns0:c>
       <ns0:c r="D214" s="1">
         <ns0:f>ROUND(D213*20,2-INT(LOG10(ABS(D213*20))))</ns0:f>
-        <ns0:v>2.72e+240</ns0:v>
+        <ns0:v>3.08e+245</ns0:v>
       </ns0:c>
       <ns0:c r="E214" s="1">
         <ns0:f>D214</ns0:f>
-        <ns0:v>2.72e+240</ns0:v>
+        <ns0:v>3.08e+245</ns0:v>
       </ns0:c>
       <ns0:c r="F214" s="1">
         <ns0:f>ROUND(F213*1.4,-5)</ns0:f>
-        <ns0:v>4.23088582560088e+33</ns0:v>
+        <ns0:v>2.8212910348805854e+41</ns0:v>
       </ns0:c>
       <ns0:c r="G214" s="1" t="n">
         <ns0:v>43.0000000000001</ns0:v>
@@ -7917,15 +7890,15 @@
       </ns0:c>
       <ns0:c r="D215" s="1">
         <ns0:f>ROUND(D214*20,2-INT(LOG10(ABS(D214*20))))</ns0:f>
-        <ns0:v>5.44e+241</ns0:v>
+        <ns0:v>6.1600000000000006e+246</ns0:v>
       </ns0:c>
       <ns0:c r="E215" s="1">
         <ns0:f>D215</ns0:f>
-        <ns0:v>5.44e+241</ns0:v>
+        <ns0:v>6.1600000000000006e+246</ns0:v>
       </ns0:c>
       <ns0:c r="F215" s="1">
         <ns0:f>ROUND(F214*1.4,-5)</ns0:f>
-        <ns0:v>5.92324015584123e+33</ns0:v>
+        <ns0:v>3.949807448832819e+41</ns0:v>
       </ns0:c>
       <ns0:c r="G215" s="1" t="n">
         <ns0:v>43.2000000000002</ns0:v>
@@ -7949,15 +7922,15 @@
       </ns0:c>
       <ns0:c r="D216" s="1">
         <ns0:f>ROUND(D215*20,2-INT(LOG10(ABS(D215*20))))</ns0:f>
-        <ns0:v>1.09e+243</ns0:v>
+        <ns0:v>1.23e+248</ns0:v>
       </ns0:c>
       <ns0:c r="E216" s="1">
         <ns0:f>D216</ns0:f>
-        <ns0:v>1.09e+243</ns0:v>
+        <ns0:v>1.23e+248</ns0:v>
       </ns0:c>
       <ns0:c r="F216" s="1">
         <ns0:f>ROUND(F215*1.4,-5)</ns0:f>
-        <ns0:v>8.29253621817772e+33</ns0:v>
+        <ns0:v>5.529730428365947e+41</ns0:v>
       </ns0:c>
       <ns0:c r="G216" s="1" t="n">
         <ns0:v>43.4000000000002</ns0:v>
@@ -7981,15 +7954,15 @@
       </ns0:c>
       <ns0:c r="D217" s="1">
         <ns0:f>ROUND(D216*20,2-INT(LOG10(ABS(D216*20))))</ns0:f>
-        <ns0:v>2.18e+244</ns0:v>
+        <ns0:v>2.46e+249</ns0:v>
       </ns0:c>
       <ns0:c r="E217" s="1">
         <ns0:f>D217</ns0:f>
-        <ns0:v>2.18e+244</ns0:v>
+        <ns0:v>2.46e+249</ns0:v>
       </ns0:c>
       <ns0:c r="F217" s="1">
         <ns0:f>ROUND(F216*1.4,-5)</ns0:f>
-        <ns0:v>1.16095507054488e+34</ns0:v>
+        <ns0:v>7.741622599712325e+41</ns0:v>
       </ns0:c>
       <ns0:c r="G217" s="1" t="n">
         <ns0:v>43.6000000000002</ns0:v>
@@ -8013,15 +7986,15 @@
       </ns0:c>
       <ns0:c r="D218" s="1">
         <ns0:f>ROUND(D217*20,2-INT(LOG10(ABS(D217*20))))</ns0:f>
-        <ns0:v>4.36e+245</ns0:v>
+        <ns0:v>4.92e+250</ns0:v>
       </ns0:c>
       <ns0:c r="E218" s="1">
         <ns0:f>D218</ns0:f>
-        <ns0:v>4.36e+245</ns0:v>
+        <ns0:v>4.92e+250</ns0:v>
       </ns0:c>
       <ns0:c r="F218" s="1">
         <ns0:f>ROUND(F217*1.4,-5)</ns0:f>
-        <ns0:v>1.62533709876283e+34</ns0:v>
+        <ns0:v>1.0838271639597256e+42</ns0:v>
       </ns0:c>
       <ns0:c r="G218" s="1" t="n">
         <ns0:v>43.8000000000002</ns0:v>
@@ -8045,15 +8018,15 @@
       </ns0:c>
       <ns0:c r="D219" s="1">
         <ns0:f>ROUND(D218*20,2-INT(LOG10(ABS(D218*20))))</ns0:f>
-        <ns0:v>8.72e+246</ns0:v>
+        <ns0:v>9.84e+251</ns0:v>
       </ns0:c>
       <ns0:c r="E219" s="1">
         <ns0:f>D219</ns0:f>
-        <ns0:v>8.72e+246</ns0:v>
+        <ns0:v>9.84e+251</ns0:v>
       </ns0:c>
       <ns0:c r="F219" s="1">
         <ns0:f>ROUND(F218*1.4,-5)</ns0:f>
-        <ns0:v>2.27547193826796e+34</ns0:v>
+        <ns0:v>1.5173580295436157e+42</ns0:v>
       </ns0:c>
       <ns0:c r="G219" s="1" t="n">
         <ns0:v>44.0000000000002</ns0:v>
@@ -8077,15 +8050,15 @@
       </ns0:c>
       <ns0:c r="D220" s="1">
         <ns0:f>ROUND(D219*20,2-INT(LOG10(ABS(D219*20))))</ns0:f>
-        <ns0:v>1.74e+248</ns0:v>
+        <ns0:v>1.97e+253</ns0:v>
       </ns0:c>
       <ns0:c r="E220" s="1">
         <ns0:f>D220</ns0:f>
-        <ns0:v>1.74e+248</ns0:v>
+        <ns0:v>1.97e+253</ns0:v>
       </ns0:c>
       <ns0:c r="F220" s="1">
         <ns0:f>ROUND(F219*1.4,-5)</ns0:f>
-        <ns0:v>3.18566071357514e+34</ns0:v>
+        <ns0:v>2.1243012413610618e+42</ns0:v>
       </ns0:c>
       <ns0:c r="G220" s="1" t="n">
         <ns0:v>44.2000000000002</ns0:v>
@@ -8109,15 +8082,15 @@
       </ns0:c>
       <ns0:c r="D221" s="1">
         <ns0:f>ROUND(D220*20,2-INT(LOG10(ABS(D220*20))))</ns0:f>
-        <ns0:v>3.48e+249</ns0:v>
+        <ns0:v>3.94e+254</ns0:v>
       </ns0:c>
       <ns0:c r="E221" s="1">
         <ns0:f>D221</ns0:f>
-        <ns0:v>3.48e+249</ns0:v>
+        <ns0:v>3.94e+254</ns0:v>
       </ns0:c>
       <ns0:c r="F221" s="1">
         <ns0:f>ROUND(F220*1.4,-5)</ns0:f>
-        <ns0:v>4.4599249990052e+34</ns0:v>
+        <ns0:v>2.9740217379054866e+42</ns0:v>
       </ns0:c>
       <ns0:c r="G221" s="1" t="n">
         <ns0:v>44.4000000000002</ns0:v>
@@ -8141,15 +8114,15 @@
       </ns0:c>
       <ns0:c r="D222" s="1">
         <ns0:f>ROUND(D221*20,2-INT(LOG10(ABS(D221*20))))</ns0:f>
-        <ns0:v>6.96e+250</ns0:v>
+        <ns0:v>7.879999999999999e+255</ns0:v>
       </ns0:c>
       <ns0:c r="E222" s="1">
         <ns0:f>D222</ns0:f>
-        <ns0:v>6.96e+250</ns0:v>
+        <ns0:v>7.879999999999999e+255</ns0:v>
       </ns0:c>
       <ns0:c r="F222" s="1">
         <ns0:f>ROUND(F221*1.4,-5)</ns0:f>
-        <ns0:v>6.24389499860728e+34</ns0:v>
+        <ns0:v>4.163630433067681e+42</ns0:v>
       </ns0:c>
       <ns0:c r="G222" s="1" t="n">
         <ns0:v>44.6000000000002</ns0:v>
@@ -8173,15 +8146,15 @@
       </ns0:c>
       <ns0:c r="D223" s="1">
         <ns0:f>ROUND(D222*20,2-INT(LOG10(ABS(D222*20))))</ns0:f>
-        <ns0:v>1.39e+252</ns0:v>
+        <ns0:v>1.58e+257</ns0:v>
       </ns0:c>
       <ns0:c r="E223" s="1">
         <ns0:f>D223</ns0:f>
-        <ns0:v>1.39e+252</ns0:v>
+        <ns0:v>1.58e+257</ns0:v>
       </ns0:c>
       <ns0:c r="F223" s="1">
         <ns0:f>ROUND(F222*1.4,-5)</ns0:f>
-        <ns0:v>8.74145299805019e+34</ns0:v>
+        <ns0:v>5.829082606294754e+42</ns0:v>
       </ns0:c>
       <ns0:c r="G223" s="1" t="n">
         <ns0:v>44.8000000000002</ns0:v>

</xml_diff>

<commit_message>
Freeze v5 late-income candidate, all-level roster, diagnostic checkpoints and failed v4 evidence
</commit_message>
<xml_diff>
--- a/space-battleship/config_excel/level.xlsx
+++ b/space-battleship/config_excel/level.xlsx
@@ -1553,7 +1553,7 @@
         <ns0:v>602880.1175788565</ns0:v>
       </ns0:c>
       <ns0:c r="F14" s="1" t="n">
-        <ns0:v>18870.66854784442</ns0:v>
+        <ns0:v>188.7066854784442</ns0:v>
       </ns0:c>
       <ns0:c r="G14" s="1" t="n">
         <ns0:v>3</ns0:v>
@@ -1581,7 +1581,7 @@
         <ns0:v>6450407.623907364</ns0:v>
       </ns0:c>
       <ns0:c r="F15" s="1" t="n">
-        <ns0:v>201903.3315579912</ns0:v>
+        <ns0:v>2019.033315579911</ns0:v>
       </ns0:c>
       <ns0:c r="G15" s="1" t="n">
         <ns0:v>3.2</ns0:v>
@@ -1609,7 +1609,7 @@
         <ns0:v>69014978.76834521</ns0:v>
       </ns0:c>
       <ns0:c r="F16" s="1" t="n">
-        <ns0:v>2160228.462010301</ns0:v>
+        <ns0:v>21602.284620103</ns0:v>
       </ns0:c>
       <ns0:c r="G16" s="1" t="n">
         <ns0:v>3.4</ns0:v>
@@ -1637,7 +1637,7 @@
         <ns0:v>738413379.7593849</ns0:v>
       </ns0:c>
       <ns0:c r="F17" s="1" t="n">
-        <ns0:v>23112976.75015848</ns0:v>
+        <ns0:v>231129.7675015848</ns0:v>
       </ns0:c>
       <ns0:c r="G17" s="1" t="n">
         <ns0:v>3.6</ns0:v>
@@ -1665,7 +1665,7 @@
         <ns0:v>7900521439.525051</ns0:v>
       </ns0:c>
       <ns0:c r="F18" s="1" t="n">
-        <ns0:v>247293146.8351421</ns0:v>
+        <ns0:v>2472931.468351421</ns0:v>
       </ns0:c>
       <ns0:c r="G18" s="1" t="n">
         <ns0:v>3.8</ns0:v>
@@ -1693,7 +1693,7 @@
         <ns0:v>84530211298.0865</ns0:v>
       </ns0:c>
       <ns0:c r="F19" s="1" t="n">
-        <ns0:v>2645868644.816936</ns0:v>
+        <ns0:v>26458686.44816936</ns0:v>
       </ns0:c>
       <ns0:c r="G19" s="1" t="n">
         <ns0:v>4</ns0:v>
@@ -1721,7 +1721,7 @@
         <ns0:v>904415825815.2517</ns0:v>
       </ns0:c>
       <ns0:c r="F20" s="1" t="n">
-        <ns0:v>28308996732.09452</ns0:v>
+        <ns0:v>283089967.3209452</ns0:v>
       </ns0:c>
       <ns0:c r="G20" s="1" t="n">
         <ns0:v>4.2</ns0:v>
@@ -1749,7 +1749,7 @@
         <ns0:v>9676634819953.418</ns0:v>
       </ns0:c>
       <ns0:c r="F21" s="1" t="n">
-        <ns0:v>302887030143.2465</ns0:v>
+        <ns0:v>3028870301.432466</ns0:v>
       </ns0:c>
       <ns0:c r="G21" s="1" t="n">
         <ns0:v>4.4</ns0:v>
@@ -1777,7 +1777,7 @@
         <ns0:v>103533417666955.5</ns0:v>
       </ns0:c>
       <ns0:c r="F22" s="1" t="n">
-        <ns0:v>3240685422277.354</ns0:v>
+        <ns0:v>32406854222.77353</ns0:v>
       </ns0:c>
       <ns0:c r="G22" s="1" t="n">
         <ns0:v>4.6</ns0:v>
@@ -1805,7 +1805,7 @@
         <ns0:v>1107737222003781</ns0:v>
       </ns0:c>
       <ns0:c r="F23" s="1" t="n">
-        <ns0:v>34673132095468.54</ns0:v>
+        <ns0:v>346731320954.6854</ns0:v>
       </ns0:c>
       <ns0:c r="G23" s="1" t="n">
         <ns0:v>4.8</ns0:v>
@@ -1823,7 +1823,7 @@
       </ns0:c>
       <ns0:c r="C24" s="1" t="inlineStr">
         <ns0:is>
-          <ns0:t>{60|0.1,109|0.2,96|0.3,39|0.4,106|0.5,17|0.6,51|0.7,52|0.8,37|0.9}</ns0:t>
+          <ns0:t>{30211|0.100000,30212|0.200000,30213|0.300000,30214|0.400000,30215|0.500000,30216|0.600000,30217|0.700000,30218|0.800000,30219|0.900000}</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="D24" s="1">
@@ -1836,7 +1836,7 @@
       </ns0:c>
       <ns0:c r="F24" s="1">
         <ns0:f>ROUND(F23*1.4,-5)</ns0:f>
-        <ns0:v>48542384899999.99</ns0:v>
+        <ns0:v>485423799999.99994</ns0:v>
       </ns0:c>
       <ns0:c r="G24" s="1" t="n">
         <ns0:v>5</ns0:v>
@@ -1854,7 +1854,7 @@
       </ns0:c>
       <ns0:c r="C25" s="1" t="inlineStr">
         <ns0:is>
-          <ns0:t>{123|0.1,185|0.2,49|0.3,30|0.4,67|0.5,121|0.6,28|0.7,32|0.8,91|0.9}</ns0:t>
+          <ns0:t>{30221|0.100000,30222|0.200000,30223|0.300000,30224|0.400000,30225|0.500000,30226|0.600000,30227|0.700000,30228|0.800000,30229|0.900000}</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="D25" s="1">
@@ -1867,7 +1867,7 @@
       </ns0:c>
       <ns0:c r="F25" s="1">
         <ns0:f>ROUND(F24*1.4,-5)</ns0:f>
-        <ns0:v>67959338899999.99</ns0:v>
+        <ns0:v>679593300000.0</ns0:v>
       </ns0:c>
       <ns0:c r="G25" s="1" t="n">
         <ns0:v>5.2</ns0:v>
@@ -1885,7 +1885,7 @@
       </ns0:c>
       <ns0:c r="C26" s="1" t="inlineStr">
         <ns0:is>
-          <ns0:t>{202|0.1,193|0.2,203|0.3,224|0.4,201|0.5,229|0.6,195|0.7,199|0.8,209|0.9}</ns0:t>
+          <ns0:t>{30231|0.100000,30232|0.200000,30233|0.300000,30234|0.400000,30235|0.500000,30236|0.600000,30237|0.700000,30238|0.800000,30239|0.900000}</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="D26" s="1">
@@ -1898,7 +1898,7 @@
       </ns0:c>
       <ns0:c r="F26" s="1">
         <ns0:f>ROUND(F25*1.4,-5)</ns0:f>
-        <ns0:v>95143074500000.0</ns0:v>
+        <ns0:v>951430599999.9999</ns0:v>
       </ns0:c>
       <ns0:c r="G26" s="1" t="n">
         <ns0:v>5.4</ns0:v>
@@ -1916,7 +1916,7 @@
       </ns0:c>
       <ns0:c r="C27" s="1" t="inlineStr">
         <ns0:is>
-          <ns0:t>{226|0.1,190|0.2,262|0.3,225|0.4,222|0.5,228|0.6,196|0.7,198|0.8,211|0.9}</ns0:t>
+          <ns0:t>{30241|0.100000,30242|0.200000,30243|0.300000,30244|0.400000,30245|0.500000,30246|0.600000,30247|0.700000,30248|0.800000,30249|0.900000}</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="D27" s="1">
@@ -1929,7 +1929,7 @@
       </ns0:c>
       <ns0:c r="F27" s="1">
         <ns0:f>ROUND(F26*1.4,-5)</ns0:f>
-        <ns0:v>133200304299999.98</ns0:v>
+        <ns0:v>1332002800000.0</ns0:v>
       </ns0:c>
       <ns0:c r="G27" s="1" t="n">
         <ns0:v>5.6</ns0:v>
@@ -1947,7 +1947,7 @@
       </ns0:c>
       <ns0:c r="C28" s="1" t="inlineStr">
         <ns0:is>
-          <ns0:t>{234|0.1,241|0.2,236|0.3,219|0.4,223|0.5,240|0.6,245|0.7,256|0.8,258|0.9}</ns0:t>
+          <ns0:t>{30251|0.100000,30252|0.200000,30253|0.300000,30254|0.400000,30255|0.500000,30256|0.600000,30257|0.700000,30258|0.800000,30259|0.900000}</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="D28" s="1">
@@ -1960,7 +1960,7 @@
       </ns0:c>
       <ns0:c r="F28" s="1">
         <ns0:f>ROUND(F27*1.4,-5)</ns0:f>
-        <ns0:v>186480426000000.0</ns0:v>
+        <ns0:v>1864803899999.9998</ns0:v>
       </ns0:c>
       <ns0:c r="G28" s="1" t="n">
         <ns0:v>5.8</ns0:v>
@@ -1978,7 +1978,7 @@
       </ns0:c>
       <ns0:c r="C29" s="1" t="inlineStr">
         <ns0:is>
-          <ns0:t>{117|0.1,125|0.2,120|0.3,126|0.4,108|0.5,145|0.6,169|0.7,107|0.8,110|0.9}</ns0:t>
+          <ns0:t>{30261|0.100000,30262|0.200000,30263|0.300000,30264|0.400000,30265|0.500000,30266|0.600000,30267|0.700000,30268|0.800000,30269|0.900000}</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="D29" s="1">
@@ -1991,7 +1991,7 @@
       </ns0:c>
       <ns0:c r="F29" s="1">
         <ns0:f>ROUND(F28*1.4,-5)</ns0:f>
-        <ns0:v>261072596399999.97</ns0:v>
+        <ns0:v>2610725500000.0</ns0:v>
       </ns0:c>
       <ns0:c r="G29" s="1" t="n">
         <ns0:v>6</ns0:v>
@@ -2009,7 +2009,7 @@
       </ns0:c>
       <ns0:c r="C30" s="1" t="inlineStr">
         <ns0:is>
-          <ns0:t>{73|0.1,171|0.2,22|0.3,146|0.4,133|0.5,57|0.6,47|0.7,71|0.8,151|0.9}</ns0:t>
+          <ns0:t>{30271|0.100000,30272|0.200000,30273|0.300000,30274|0.400000,30275|0.500000,30276|0.600000,30277|0.700000,30278|0.800000,30279|0.900000}</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="D30" s="1">
@@ -2022,7 +2022,7 @@
       </ns0:c>
       <ns0:c r="F30" s="1">
         <ns0:f>ROUND(F29*1.4,-5)</ns0:f>
-        <ns0:v>365501635000000.0</ns0:v>
+        <ns0:v>3655015699999.9995</ns0:v>
       </ns0:c>
       <ns0:c r="G30" s="1" t="n">
         <ns0:v>6.2</ns0:v>
@@ -2040,7 +2040,7 @@
       </ns0:c>
       <ns0:c r="C31" s="1" t="inlineStr">
         <ns0:is>
-          <ns0:t>{192|0.1,194|0.2,215|0.3,197|0.4,200|0.5,191|0.6,204|0.7,206|0.8,216|0.9}</ns0:t>
+          <ns0:t>{30281|0.100000,30282|0.200000,30283|0.300000,30284|0.400000,30285|0.500000,30286|0.600000,30287|0.700000,30288|0.800000,30289|0.900000}</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="D31" s="1">
@@ -2053,7 +2053,7 @@
       </ns0:c>
       <ns0:c r="F31" s="1">
         <ns0:f>ROUND(F30*1.4,-5)</ns0:f>
-        <ns0:v>511702288999999.94</ns0:v>
+        <ns0:v>5117022000000.0</ns0:v>
       </ns0:c>
       <ns0:c r="G31" s="1" t="n">
         <ns0:v>6.4</ns0:v>
@@ -2071,7 +2071,7 @@
       </ns0:c>
       <ns0:c r="C32" s="1" t="inlineStr">
         <ns0:is>
-          <ns0:t>{227|0.1,218|0.2,210|0.3,207|0.4,212|0.5,213|0.6,205|0.7,190|0.8,228|0.9}</ns0:t>
+          <ns0:t>{30291|0.100000,30292|0.200000,30293|0.300000,30294|0.400000,30295|0.500000,30296|0.600000,30297|0.700000,30298|0.800000,30299|0.900000}</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="D32" s="1">
@@ -2084,7 +2084,7 @@
       </ns0:c>
       <ns0:c r="F32" s="1">
         <ns0:f>ROUND(F31*1.4,-5)</ns0:f>
-        <ns0:v>716383204600000.0</ns0:v>
+        <ns0:v>7163830799999.999</ns0:v>
       </ns0:c>
       <ns0:c r="G32" s="1" t="n">
         <ns0:v>6.6</ns0:v>
@@ -2102,7 +2102,7 @@
       </ns0:c>
       <ns0:c r="C33" s="1" t="inlineStr">
         <ns0:is>
-          <ns0:t>{264|0.1,261|0.2,252|0.3,260|0.4,247|0.5,265|0.6,253|0.7,255|0.8,251|0.9}</ns0:t>
+          <ns0:t>{30301|0.100000,30302|0.200000,30303|0.300000,30304|0.400000,30305|0.500000,30306|0.600000,30307|0.700000,30308|0.800000,30309|0.900000}</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="D33" s="1">
@@ -2115,7 +2115,7 @@
       </ns0:c>
       <ns0:c r="F33" s="1">
         <ns0:f>ROUND(F32*1.4,-5)</ns0:f>
-        <ns0:v>1002936486399999.9</ns0:v>
+        <ns0:v>10029363100000.0</ns0:v>
       </ns0:c>
       <ns0:c r="G33" s="1" t="n">
         <ns0:v>6.8</ns0:v>
@@ -2133,7 +2133,7 @@
       </ns0:c>
       <ns0:c r="C34" s="1" t="inlineStr">
         <ns0:is>
-          <ns0:t>{166|0.1,83|0.2,38|0.3,23|0.4,131|0.5,54|0.6,66|0.7,159|0.8,162|0.9}</ns0:t>
+          <ns0:t>{30311|0.100000,30312|0.200000,30313|0.300000,30314|0.400000,30315|0.500000,30316|0.600000,30317|0.700000,30318|0.800000,30319|0.900000}</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="D34" s="1">
@@ -2146,7 +2146,7 @@
       </ns0:c>
       <ns0:c r="F34" s="1">
         <ns0:f>ROUND(F33*1.4,-5)</ns0:f>
-        <ns0:v>1404111081000000.0</ns0:v>
+        <ns0:v>14041108299999.998</ns0:v>
       </ns0:c>
       <ns0:c r="G34" s="1" t="n">
         <ns0:v>7</ns0:v>
@@ -2164,7 +2164,7 @@
       </ns0:c>
       <ns0:c r="C35" s="1" t="inlineStr">
         <ns0:is>
-          <ns0:t>{59|0.1,103|0.2,87|0.3,135|0.4,88|0.5,177|0.6,98|0.7,175|0.8,189|0.9}</ns0:t>
+          <ns0:t>{30321|0.100000,30322|0.200000,30323|0.300000,30324|0.400000,30325|0.500000,30326|0.600000,30327|0.700000,30328|0.800000,30329|0.900000}</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="D35" s="1">
@@ -2177,7 +2177,7 @@
       </ns0:c>
       <ns0:c r="F35" s="1">
         <ns0:f>ROUND(F34*1.4,-5)</ns0:f>
-        <ns0:v>1965755513399999.8</ns0:v>
+        <ns0:v>19657551600000.0</ns0:v>
       </ns0:c>
       <ns0:c r="G35" s="1" t="n">
         <ns0:v>7.2</ns0:v>
@@ -2195,7 +2195,7 @@
       </ns0:c>
       <ns0:c r="C36" s="1" t="inlineStr">
         <ns0:is>
-          <ns0:t>{242|0.1,238|0.2,217|0.3,221|0.4,215|0.5,199|0.6,202|0.7,203|0.8,201|0.9}</ns0:t>
+          <ns0:t>{30331|0.100000,30332|0.200000,30333|0.300000,30334|0.400000,30335|0.500000,30336|0.600000,30337|0.700000,30338|0.800000,30339|0.900000}</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="D36" s="1">
@@ -2208,7 +2208,7 @@
       </ns0:c>
       <ns0:c r="F36" s="1">
         <ns0:f>ROUND(F35*1.4,-5)</ns0:f>
-        <ns0:v>2752057718800000.0</ns0:v>
+        <ns0:v>27520572199999.996</ns0:v>
       </ns0:c>
       <ns0:c r="G36" s="1" t="n">
         <ns0:v>7.4</ns0:v>
@@ -2226,7 +2226,7 @@
       </ns0:c>
       <ns0:c r="C37" s="1" t="inlineStr">
         <ns0:is>
-          <ns0:t>{192|0.1,196|0.2,256|0.3,209|0.4,222|0.5,231|0.6,225|0.7,198|0.8,194|0.9}</ns0:t>
+          <ns0:t>{30341|0.100000,30342|0.200000,30343|0.300000,30344|0.400000,30345|0.500000,30346|0.600000,30347|0.700000,30348|0.800000,30349|0.900000}</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="D37" s="1">
@@ -2239,7 +2239,7 @@
       </ns0:c>
       <ns0:c r="F37" s="1">
         <ns0:f>ROUND(F36*1.4,-5)</ns0:f>
-        <ns0:v>3852880806299999.5</ns0:v>
+        <ns0:v>38528801100000.0</ns0:v>
       </ns0:c>
       <ns0:c r="G37" s="1" t="n">
         <ns0:v>7.6</ns0:v>
@@ -2257,7 +2257,7 @@
       </ns0:c>
       <ns0:c r="C38" s="1" t="inlineStr">
         <ns0:is>
-          <ns0:t>{230|0.1,239|0.2,257|0.3,220|0.4,243|0.5,233|0.6,237|0.7,232|0.8,246|0.9}</ns0:t>
+          <ns0:t>{30351|0.100000,30352|0.200000,30353|0.300000,30354|0.400000,30355|0.500000,30356|0.600000,30357|0.700000,30358|0.800000,30359|0.900000}</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="D38" s="1">
@@ -2270,7 +2270,7 @@
       </ns0:c>
       <ns0:c r="F38" s="1">
         <ns0:f>ROUND(F37*1.4,-5)</ns0:f>
-        <ns0:v>5394033128800000.0</ns0:v>
+        <ns0:v>53940321499999.99</ns0:v>
       </ns0:c>
       <ns0:c r="G38" s="1" t="n">
         <ns0:v>7.8</ns0:v>
@@ -2288,7 +2288,7 @@
       </ns0:c>
       <ns0:c r="C39" s="1" t="inlineStr">
         <ns0:is>
-          <ns0:t>{173|0.1,148|0.2,112|0.3,77|0.4,34|0.5,84|0.6,20|0.7,130|0.8,134|0.9}</ns0:t>
+          <ns0:t>{30361|0.100000,30362|0.200000,30363|0.300000,30364|0.400000,30365|0.500000,30366|0.600000,30367|0.700000,30368|0.800000,30369|0.900000}</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="D39" s="1">
@@ -2301,7 +2301,7 @@
       </ns0:c>
       <ns0:c r="F39" s="1">
         <ns0:f>ROUND(F38*1.4,-5)</ns0:f>
-        <ns0:v>7551646380299999.0</ns0:v>
+        <ns0:v>75516450100000.0</ns0:v>
       </ns0:c>
       <ns0:c r="G39" s="1" t="n">
         <ns0:v>8</ns0:v>
@@ -2319,7 +2319,7 @@
       </ns0:c>
       <ns0:c r="C40" s="1" t="inlineStr">
         <ns0:is>
-          <ns0:t>{70|0.1,104|0.2,97|0.3,158|0.4,40|0.5,167|0.6,21|0.7,86|0.8,180|0.9}</ns0:t>
+          <ns0:t>{30371|0.100000,30372|0.200000,30373|0.300000,30374|0.400000,30375|0.500000,30376|0.600000,30377|0.700000,30378|0.800000,30379|0.900000}</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="D40" s="1">
@@ -2332,7 +2332,7 @@
       </ns0:c>
       <ns0:c r="F40" s="1">
         <ns0:f>ROUND(F39*1.4,-5)</ns0:f>
-        <ns0:v>1.05723049324e+16</ns0:v>
+        <ns0:v>105723030099999.98</ns0:v>
       </ns0:c>
       <ns0:c r="G40" s="1" t="n">
         <ns0:v>8.199999999999999</ns0:v>
@@ -2350,7 +2350,7 @@
       </ns0:c>
       <ns0:c r="C41" s="1" t="inlineStr">
         <ns0:is>
-          <ns0:t>{214|0.1,234|0.2,241|0.3,204|0.4,197|0.5,193|0.6,195|0.7,216|0.8,200|0.9}</ns0:t>
+          <ns0:t>{30381|0.100000,30382|0.200000,30383|0.300000,30384|0.400000,30385|0.500000,30386|0.600000,30387|0.700000,30388|0.800000,30389|0.900000}</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="D41" s="1">
@@ -2363,7 +2363,7 @@
       </ns0:c>
       <ns0:c r="F41" s="1">
         <ns0:f>ROUND(F40*1.4,-5)</ns0:f>
-        <ns0:v>1.4801226905399998e+16</ns0:v>
+        <ns0:v>148012242100000.0</ns0:v>
       </ns0:c>
       <ns0:c r="G41" s="1" t="n">
         <ns0:v>8.4</ns0:v>
@@ -2381,7 +2381,7 @@
       </ns0:c>
       <ns0:c r="C42" s="1" t="inlineStr">
         <ns0:is>
-          <ns0:t>{227|0.1,212|0.2,226|0.3,210|0.4,262|0.5,208|0.6,211|0.7,213|0.8,207|0.9}</ns0:t>
+          <ns0:t>{30391|0.100000,30392|0.200000,30393|0.300000,30394|0.400000,30395|0.500000,30396|0.600000,30397|0.700000,30398|0.800000,30399|0.900000}</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="D42" s="1">
@@ -2394,7 +2394,7 @@
       </ns0:c>
       <ns0:c r="F42" s="1">
         <ns0:f>ROUND(F41*1.4,-5)</ns0:f>
-        <ns0:v>2.07217176676e+16</ns0:v>
+        <ns0:v>207217138899999.97</ns0:v>
       </ns0:c>
       <ns0:c r="G42" s="1" t="n">
         <ns0:v>8.6</ns0:v>
@@ -2412,7 +2412,7 @@
       </ns0:c>
       <ns0:c r="C43" s="1" t="inlineStr">
         <ns0:is>
-          <ns0:t>{259|0.1,249|0.2,250|0.3,248|0.4,268|0.5,252|0.6,229|0.7,255|0.8,260|0.9}</ns0:t>
+          <ns0:t>{30401|0.100000,30402|0.200000,30403|0.300000,30404|0.400000,30405|0.500000,30406|0.600000,30407|0.700000,30408|0.800000,30409|0.900000}</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="D43" s="1">
@@ -2425,7 +2425,7 @@
       </ns0:c>
       <ns0:c r="F43" s="1">
         <ns0:f>ROUND(F42*1.4,-5)</ns0:f>
-        <ns0:v>2.9010404734599996e+16</ns0:v>
+        <ns0:v>290103994500000.0</ns0:v>
       </ns0:c>
       <ns0:c r="G43" s="1" t="n">
         <ns0:v>8.800000000000001</ns0:v>
@@ -2443,7 +2443,7 @@
       </ns0:c>
       <ns0:c r="C44" s="1" t="inlineStr">
         <ns0:is>
-          <ns0:t>{43|0.1,16|0.2,74|0.3,55|0.4,94|0.5,48|0.6,79|0.7,19|0.8,168|0.9}</ns0:t>
+          <ns0:t>{30411|0.100000,30412|0.200000,30413|0.300000,30414|0.400000,30415|0.500000,30416|0.600000,30417|0.700000,30418|0.800000,30419|0.900000}</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="D44" s="1">
@@ -2456,7 +2456,7 @@
       </ns0:c>
       <ns0:c r="F44" s="1">
         <ns0:f>ROUND(F43*1.4,-5)</ns0:f>
-        <ns0:v>4.06145666284e+16</ns0:v>
+        <ns0:v>406145592299999.94</ns0:v>
       </ns0:c>
       <ns0:c r="G44" s="1" t="n">
         <ns0:v>9</ns0:v>
@@ -2474,7 +2474,7 @@
       </ns0:c>
       <ns0:c r="C45" s="1" t="inlineStr">
         <ns0:is>
-          <ns0:t>{58|0.1,165|0.2,156|0.3,127|0.4,152|0.5,75|0.6,176|0.7,111|0.8,129|0.9}</ns0:t>
+          <ns0:t>{30421|0.100000,30422|0.200000,30423|0.300000,30424|0.400000,30425|0.500000,30426|0.600000,30427|0.700000,30428|0.800000,30429|0.900000}</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="D45" s="1">
@@ -2487,7 +2487,7 @@
       </ns0:c>
       <ns0:c r="F45" s="1">
         <ns0:f>ROUND(F44*1.4,-5)</ns0:f>
-        <ns0:v>5.686039327979999e+16</ns0:v>
+        <ns0:v>568603829200000.0</ns0:v>
       </ns0:c>
       <ns0:c r="G45" s="1" t="n">
         <ns0:v>9.199999999999999</ns0:v>
@@ -2505,7 +2505,7 @@
       </ns0:c>
       <ns0:c r="C46" s="1" t="inlineStr">
         <ns0:is>
-          <ns0:t>{244|0.1,217|0.2,238|0.3,206|0.4,224|0.5,215|0.6,202|0.7,199|0.8,203|0.9}</ns0:t>
+          <ns0:t>{30431|0.100000,30432|0.200000,30433|0.300000,30434|0.400000,30435|0.500000,30436|0.600000,30437|0.700000,30438|0.800000,30439|0.900000}</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="D46" s="1">
@@ -2518,7 +2518,7 @@
       </ns0:c>
       <ns0:c r="F46" s="1">
         <ns0:f>ROUND(F45*1.4,-5)</ns0:f>
-        <ns0:v>7.96045505917e+16</ns0:v>
+        <ns0:v>796045360899999.9</ns0:v>
       </ns0:c>
       <ns0:c r="G46" s="1" t="n">
         <ns0:v>9.4</ns0:v>
@@ -2536,7 +2536,7 @@
       </ns0:c>
       <ns0:c r="C47" s="1" t="inlineStr">
         <ns0:is>
-          <ns0:t>{191|0.1,205|0.2,256|0.3,190|0.4,201|0.5,228|0.6,218|0.7,245|0.8,198|0.9}</ns0:t>
+          <ns0:t>{30441|0.100000,30442|0.200000,30443|0.300000,30444|0.400000,30445|0.500000,30446|0.600000,30447|0.700000,30448|0.800000,30449|0.900000}</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="D47" s="1">
@@ -2549,7 +2549,7 @@
       </ns0:c>
       <ns0:c r="F47" s="1">
         <ns0:f>ROUND(F46*1.4,-5)</ns0:f>
-        <ns0:v>1.1144637082839998e+17</ns0:v>
+        <ns0:v>1114463505299999.9</ns0:v>
       </ns0:c>
       <ns0:c r="G47" s="1" t="n">
         <ns0:v>9.6</ns0:v>
@@ -2567,7 +2567,7 @@
       </ns0:c>
       <ns0:c r="C48" s="1" t="inlineStr">
         <ns0:is>
-          <ns0:t>{235|0.1,230|0.2,257|0.3,219|0.4,223|0.5,258|0.6,254|0.7,240|0.8,243|0.9}</ns0:t>
+          <ns0:t>{30451|0.100000,30452|0.200000,30453|0.300000,30454|0.400000,30455|0.500000,30456|0.600000,30457|0.700000,30458|0.800000,30459|0.900000}</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="D48" s="1">
@@ -2580,7 +2580,7 @@
       </ns0:c>
       <ns0:c r="F48" s="1">
         <ns0:f>ROUND(F47*1.4,-5)</ns0:f>
-        <ns0:v>1.560249191598e+17</ns0:v>
+        <ns0:v>1560248907399999.8</ns0:v>
       </ns0:c>
       <ns0:c r="G48" s="1" t="n">
         <ns0:v>9.800000000000001</ns0:v>
@@ -2598,7 +2598,7 @@
       </ns0:c>
       <ns0:c r="C49" s="1" t="inlineStr">
         <ns0:is>
-          <ns0:t>{144|0.1,69|0.2,82|0.3,18|0.4,65|0.5,50|0.6,183|0.7,161|0.8,78|0.9}</ns0:t>
+          <ns0:t>{30461|0.100000,30462|0.200000,30463|0.300000,30464|0.400000,30465|0.500000,30466|0.600000,30467|0.700000,30468|0.800000,30469|0.900000}</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="D49" s="1">
@@ -2611,7 +2611,7 @@
       </ns0:c>
       <ns0:c r="F49" s="1">
         <ns0:f>ROUND(F48*1.4,-5)</ns0:f>
-        <ns0:v>2.1843488682369997e+17</ns0:v>
+        <ns0:v>2184348470399999.8</ns0:v>
       </ns0:c>
       <ns0:c r="G49" s="1" t="n">
         <ns0:v>10</ns0:v>
@@ -2629,7 +2629,7 @@
       </ns0:c>
       <ns0:c r="C50" s="1" t="inlineStr">
         <ns0:is>
-          <ns0:t>{29|0.1,153|0.2,44|0.3,155|0.4,114|0.5,138|0.6,99|0.7,118|0.8,105|0.9}</ns0:t>
+          <ns0:t>{30471|0.100000,30472|0.200000,30473|0.300000,30474|0.400000,30475|0.500000,30476|0.600000,30477|0.700000,30478|0.800000,30479|0.900000}</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="D50" s="1">
@@ -2642,7 +2642,7 @@
       </ns0:c>
       <ns0:c r="F50" s="1">
         <ns0:f>ROUND(F49*1.4,-5)</ns0:f>
-        <ns0:v>3.058088415532e+17</ns0:v>
+        <ns0:v>3058087858599999.5</ns0:v>
       </ns0:c>
       <ns0:c r="G50" s="1" t="n">
         <ns0:v>10.2</ns0:v>
@@ -2660,7 +2660,7 @@
       </ns0:c>
       <ns0:c r="C51" s="1" t="inlineStr">
         <ns0:is>
-          <ns0:t>{221|0.1,242|0.2,193|0.3,224|0.4,195|0.5,194|0.6,197|0.7,234|0.8,200|0.9}</ns0:t>
+          <ns0:t>{30481|0.100000,30482|0.200000,30483|0.300000,30484|0.400000,30485|0.500000,30486|0.600000,30487|0.700000,30488|0.800000,30489|0.900000}</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="D51" s="1">
@@ -2673,7 +2673,7 @@
       </ns0:c>
       <ns0:c r="F51" s="1">
         <ns0:f>ROUND(F50*1.4,-5)</ns0:f>
-        <ns0:v>4.281323781745e+17</ns0:v>
+        <ns0:v>4281323001999999.5</ns0:v>
       </ns0:c>
       <ns0:c r="G51" s="1" t="n">
         <ns0:v>10.4</ns0:v>
@@ -2691,7 +2691,7 @@
       </ns0:c>
       <ns0:c r="C52" s="1" t="inlineStr">
         <ns0:is>
-          <ns0:t>{231|0.1,262|0.2,225|0.3,222|0.4,192|0.5,191|0.6,209|0.7,211|0.8,213|0.9}</ns0:t>
+          <ns0:t>{30491|0.100000,30492|0.200000,30493|0.300000,30494|0.400000,30495|0.500000,30496|0.600000,30497|0.700000,30498|0.800000,30499|0.900000}</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="D52" s="1">
@@ -2704,7 +2704,7 @@
       </ns0:c>
       <ns0:c r="F52" s="1">
         <ns0:f>ROUND(F51*1.4,-5)</ns0:f>
-        <ns0:v>5.993853294442999e+17</ns0:v>
+        <ns0:v>5993852202800000.0</ns0:v>
       </ns0:c>
       <ns0:c r="G52" s="1" t="n">
         <ns0:v>10.6</ns0:v>
@@ -2722,7 +2722,7 @@
       </ns0:c>
       <ns0:c r="C53" s="1" t="inlineStr">
         <ns0:is>
-          <ns0:t>{250|0.1,261|0.2,251|0.3,248|0.4,249|0.5,259|0.6,268|0.7,264|0.8,253|0.9}</ns0:t>
+          <ns0:t>{30501|0.100000,30502|0.200000,30503|0.300000,30504|0.400000,30505|0.500000,30506|0.600000,30507|0.700000,30508|0.800000,30509|0.900000}</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="D53" s="1">
@@ -2735,7 +2735,7 @@
       </ns0:c>
       <ns0:c r="F53" s="1">
         <ns0:f>ROUND(F52*1.4,-5)</ns0:f>
-        <ns0:v>8.391394612219999e+17</ns0:v>
+        <ns0:v>8391393083899999.0</ns0:v>
       </ns0:c>
       <ns0:c r="G53" s="1" t="n">
         <ns0:v>10.8</ns0:v>
@@ -2753,7 +2753,7 @@
       </ns0:c>
       <ns0:c r="C54" s="1" t="inlineStr">
         <ns0:is>
-          <ns0:t>{163|0.1,62|0.2,24|0.3,95|0.4,81|0.5,64|0.6,172|0.7,182|0.8,25|0.9}</ns0:t>
+          <ns0:t>{30511|0.100000,30512|0.200000,30513|0.300000,30514|0.400000,30515|0.500000,30516|0.600000,30517|0.700000,30518|0.800000,30519|0.900000}</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="D54" s="1">
@@ -2766,7 +2766,7 @@
       </ns0:c>
       <ns0:c r="F54" s="1">
         <ns0:f>ROUND(F53*1.4,-5)</ns0:f>
-        <ns0:v>1.1747952457108e+18</ns0:v>
+        <ns0:v>1.17479503175e+16</ns0:v>
       </ns0:c>
       <ns0:c r="G54" s="1" t="n">
         <ns0:v>11</ns0:v>
@@ -2784,7 +2784,7 @@
       </ns0:c>
       <ns0:c r="C55" s="1" t="inlineStr">
         <ns0:is>
-          <ns0:t>{56|0.1,113|0.2,141|0.3,102|0.4,119|0.5,36|0.6,116|0.7,154|0.8,170|0.9}</ns0:t>
+          <ns0:t>{30521|0.100000,30522|0.200000,30523|0.300000,30524|0.400000,30525|0.500000,30526|0.600000,30527|0.700000,30528|0.800000,30529|0.900000}</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="D55" s="1">
@@ -2797,7 +2797,7 @@
       </ns0:c>
       <ns0:c r="F55" s="1">
         <ns0:f>ROUND(F54*1.4,-5)</ns0:f>
-        <ns0:v>1.6447133439951e+18</ns0:v>
+        <ns0:v>1.6447130444499998e+16</ns0:v>
       </ns0:c>
       <ns0:c r="G55" s="1" t="n">
         <ns0:v>11.2</ns0:v>
@@ -2815,7 +2815,7 @@
       </ns0:c>
       <ns0:c r="C56" s="1" t="inlineStr">
         <ns0:is>
-          <ns0:t>{244|0.1,217|0.2,216|0.3,238|0.4,204|0.5,241|0.6,207|0.7,206|0.8,229|0.9}</ns0:t>
+          <ns0:t>{30531|0.100000,30532|0.200000,30533|0.300000,30534|0.400000,30535|0.500000,30536|0.600000,30537|0.700000,30538|0.800000,30539|0.900000}</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="D56" s="1">
@@ -2828,7 +2828,7 @@
       </ns0:c>
       <ns0:c r="F56" s="1">
         <ns0:f>ROUND(F55*1.4,-5)</ns0:f>
-        <ns0:v>2.3025986815930998e+18</ns0:v>
+        <ns0:v>2.30259826223e+16</ns0:v>
       </ns0:c>
       <ns0:c r="G56" s="1" t="n">
         <ns0:v>11.4</ns0:v>
@@ -2846,7 +2846,7 @@
       </ns0:c>
       <ns0:c r="C57" s="1" t="inlineStr">
         <ns0:is>
-          <ns0:t>{208|0.1,227|0.2,210|0.3,212|0.4,226|0.5,205|0.6,190|0.7,228|0.8,201|0.9}</ns0:t>
+          <ns0:t>{30541|0.100000,30542|0.200000,30543|0.300000,30544|0.400000,30545|0.500000,30546|0.600000,30547|0.700000,30548|0.800000,30549|0.900000}</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="D57" s="1">
@@ -2859,7 +2859,7 @@
       </ns0:c>
       <ns0:c r="F57" s="1">
         <ns0:f>ROUND(F56*1.4,-5)</ns0:f>
-        <ns0:v>3.2236381542302996e+18</ns0:v>
+        <ns0:v>3.2236375671199996e+16</ns0:v>
       </ns0:c>
       <ns0:c r="G57" s="1" t="n">
         <ns0:v>11.6</ns0:v>
@@ -2877,7 +2877,7 @@
       </ns0:c>
       <ns0:c r="C58" s="1" t="inlineStr">
         <ns0:is>
-          <ns0:t>{236|0.1,233|0.2,237|0.3,239|0.4,232|0.5,246|0.6,220|0.7,254|0.8,219|0.9}</ns0:t>
+          <ns0:t>{30551|0.100000,30552|0.200000,30553|0.300000,30554|0.400000,30555|0.500000,30556|0.600000,30557|0.700000,30558|0.800000,30559|0.900000}</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="D58" s="1">
@@ -2890,7 +2890,7 @@
       </ns0:c>
       <ns0:c r="F58" s="1">
         <ns0:f>ROUND(F57*1.4,-5)</ns0:f>
-        <ns0:v>4.5130934159223997e+18</ns0:v>
+        <ns0:v>4.51309259397e+16</ns0:v>
       </ns0:c>
       <ns0:c r="G58" s="1" t="n">
         <ns0:v>11.8</ns0:v>
@@ -2908,7 +2908,7 @@
       </ns0:c>
       <ns0:c r="C59" s="1" t="inlineStr">
         <ns0:is>
-          <ns0:t>{93|0.1,92|0.2,41|0.3,184|0.4,26|0.5,142|0.6,132|0.7,90|0.8,101|0.9}</ns0:t>
+          <ns0:t>{30561|0.100000,30562|0.200000,30563|0.300000,30564|0.400000,30565|0.500000,30566|0.600000,30567|0.700000,30568|0.800000,30569|0.900000}</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="D59" s="1">
@@ -2921,7 +2921,7 @@
       </ns0:c>
       <ns0:c r="F59" s="1">
         <ns0:f>ROUND(F58*1.4,-5)</ns0:f>
-        <ns0:v>6.3183307822914e+18</ns0:v>
+        <ns0:v>6.318329631559999e+16</ns0:v>
       </ns0:c>
       <ns0:c r="G59" s="1" t="n">
         <ns0:v>12</ns0:v>
@@ -2939,7 +2939,7 @@
       </ns0:c>
       <ns0:c r="C60" s="1" t="inlineStr">
         <ns0:is>
-          <ns0:t>{31|0.1,33|0.2,85|0.3,53|0.4,76|0.5,147|0.6,136|0.7,187|0.8,35|0.9}</ns0:t>
+          <ns0:t>{30571|0.100000,30572|0.200000,30573|0.300000,30574|0.400000,30575|0.500000,30576|0.600000,30577|0.700000,30578|0.800000,30579|0.900000}</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="D60" s="1">
@@ -2952,7 +2952,7 @@
       </ns0:c>
       <ns0:c r="F60" s="1">
         <ns0:f>ROUND(F59*1.4,-5)</ns0:f>
-        <ns0:v>8.845663095208e+18</ns0:v>
+        <ns0:v>8.84566148418e+16</ns0:v>
       </ns0:c>
       <ns0:c r="G60" s="1" t="n">
         <ns0:v>12.2</ns0:v>
@@ -2970,7 +2970,7 @@
       </ns0:c>
       <ns0:c r="C61" s="1" t="inlineStr">
         <ns0:is>
-          <ns0:t>{214|0.1,223|0.2,196|0.3,193|0.4,197|0.5,203|0.6,202|0.7,199|0.8,195|0.9}</ns0:t>
+          <ns0:t>{30581|0.100000,30582|0.200000,30583|0.300000,30584|0.400000,30585|0.500000,30586|0.600000,30587|0.700000,30588|0.800000,30589|0.900000}</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="D61" s="1">
@@ -2983,7 +2983,7 @@
       </ns0:c>
       <ns0:c r="F61" s="1">
         <ns0:f>ROUND(F60*1.4,-5)</ns0:f>
-        <ns0:v>1.2383928333291198e+19</ns0:v>
+        <ns0:v>1.2383926077849998e+17</ns0:v>
       </ns0:c>
       <ns0:c r="G61" s="1" t="n">
         <ns0:v>12.4</ns0:v>
@@ -3001,7 +3001,7 @@
       </ns0:c>
       <ns0:c r="C62" s="1" t="inlineStr">
         <ns0:is>
-          <ns0:t>{256|0.1,205|0.2,192|0.3,218|0.4,245|0.5,225|0.6,222|0.7,198|0.8,262|0.9}</ns0:t>
+          <ns0:t>{30591|0.100000,30592|0.200000,30593|0.300000,30594|0.400000,30595|0.500000,30596|0.600000,30597|0.700000,30598|0.800000,30599|0.900000}</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="D62" s="1">
@@ -3014,7 +3014,7 @@
       </ns0:c>
       <ns0:c r="F62" s="1">
         <ns0:f>ROUND(F61*1.4,-5)</ns0:f>
-        <ns0:v>1.7337499666607698e+19</ns0:v>
+        <ns0:v>1.733749650899e+17</ns0:v>
       </ns0:c>
       <ns0:c r="G62" s="1" t="n">
         <ns0:v>12.6</ns0:v>
@@ -3032,7 +3032,7 @@
       </ns0:c>
       <ns0:c r="C63" s="1" t="inlineStr">
         <ns0:is>
-          <ns0:t>{247|0.1,265|0.2,260|0.3,255|0.4,252|0.5,259|0.6,264|0.7,261|0.8,251|0.9}</ns0:t>
+          <ns0:t>{30601|0.100000,30602|0.200000,30603|0.300000,30604|0.400000,30605|0.500000,30606|0.600000,30607|0.700000,30608|0.800000,30609|0.900000}</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="D63" s="1">
@@ -3045,7 +3045,7 @@
       </ns0:c>
       <ns0:c r="F63" s="1">
         <ns0:f>ROUND(F62*1.4,-5)</ns0:f>
-        <ns0:v>2.4272499533250798e+19</ns0:v>
+        <ns0:v>2.4272495112589997e+17</ns0:v>
       </ns0:c>
       <ns0:c r="G63" s="1" t="n">
         <ns0:v>12.8</ns0:v>
@@ -3063,7 +3063,7 @@
       </ns0:c>
       <ns0:c r="C64" s="1" t="inlineStr">
         <ns0:is>
-          <ns0:t>{63|0.1,68|0.2,100|0.3,160|0.4,181|0.5,188|0.6,186|0.7,150|0.8,178|0.9}</ns0:t>
+          <ns0:t>{30611|0.100000,30612|0.200000,30613|0.300000,30614|0.400000,30615|0.500000,30616|0.600000,30617|0.700000,30618|0.800000,30619|0.900000}</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="D64" s="1">
@@ -3076,7 +3076,7 @@
       </ns0:c>
       <ns0:c r="F64" s="1">
         <ns0:f>ROUND(F63*1.4,-5)</ns0:f>
-        <ns0:v>3.3981499346551095e+19</ns0:v>
+        <ns0:v>3.3981493157629997e+17</ns0:v>
       </ns0:c>
       <ns0:c r="G64" s="1" t="n">
         <ns0:v>13</ns0:v>
@@ -3094,7 +3094,7 @@
       </ns0:c>
       <ns0:c r="C65" s="1" t="inlineStr">
         <ns0:is>
-          <ns0:t>{128|0.1,124|0.2,45|0.3,80|0.4,122|0.5,140|0.6,72|0.7,143|0.8,137|0.9}</ns0:t>
+          <ns0:t>{30621|0.100000,30622|0.200000,30623|0.300000,30624|0.400000,30625|0.500000,30626|0.600000,30627|0.700000,30628|0.800000,30629|0.900000}</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="D65" s="1">
@@ -3107,7 +3107,7 @@
       </ns0:c>
       <ns0:c r="F65" s="1">
         <ns0:f>ROUND(F64*1.4,-5)</ns0:f>
-        <ns0:v>4.75740990851715e+19</ns0:v>
+        <ns0:v>4.7574090420679994e+17</ns0:v>
       </ns0:c>
       <ns0:c r="G65" s="1" t="n">
         <ns0:v>13.2</ns0:v>
@@ -3125,7 +3125,7 @@
       </ns0:c>
       <ns0:c r="C66" s="1" t="inlineStr">
         <ns0:is>
-          <ns0:t>{221|0.1,242|0.2,217|0.3,194|0.4,215|0.5,234|0.6,200|0.7,241|0.8,204|0.9}</ns0:t>
+          <ns0:t>{30631|0.100000,30632|0.200000,30633|0.300000,30634|0.400000,30635|0.500000,30636|0.600000,30637|0.700000,30638|0.800000,30639|0.900000}</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="D66" s="1">
@@ -3138,7 +3138,7 @@
       </ns0:c>
       <ns0:c r="F66" s="1">
         <ns0:f>ROUND(F65*1.4,-5)</ns0:f>
-        <ns0:v>6.660373871924009e+19</ns0:v>
+        <ns0:v>6.660372658894999e+17</ns0:v>
       </ns0:c>
       <ns0:c r="G66" s="1" t="n">
         <ns0:v>13.4</ns0:v>
@@ -3156,7 +3156,7 @@
       </ns0:c>
       <ns0:c r="C67" s="1" t="inlineStr">
         <ns0:is>
-          <ns0:t>{231|0.1,227|0.2,191|0.3,209|0.4,211|0.5,213|0.6,210|0.7,207|0.8,212|0.9}</ns0:t>
+          <ns0:t>{30641|0.100000,30642|0.200000,30643|0.300000,30644|0.400000,30645|0.500000,30646|0.600000,30647|0.700000,30648|0.800000,30649|0.900000}</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="D67" s="1">
@@ -3169,7 +3169,7 @@
       </ns0:c>
       <ns0:c r="F67" s="1">
         <ns0:f>ROUND(F66*1.4,-5)</ns0:f>
-        <ns0:v>9.324523420693609e+19</ns0:v>
+        <ns0:v>9.324521722453e+17</ns0:v>
       </ns0:c>
       <ns0:c r="G67" s="1" t="n">
         <ns0:v>13.6</ns0:v>
@@ -3187,7 +3187,7 @@
       </ns0:c>
       <ns0:c r="C68" s="1" t="inlineStr">
         <ns0:is>
-          <ns0:t>{257|0.1,230|0.2,235|0.3,232|0.4,233|0.5,240|0.6,244|0.7,243|0.8,236|0.9}</ns0:t>
+          <ns0:t>{30651|0.100000,30652|0.200000,30653|0.300000,30654|0.400000,30655|0.500000,30656|0.600000,30657|0.700000,30658|0.800000,30659|0.900000}</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="D68" s="1">
@@ -3200,7 +3200,7 @@
       </ns0:c>
       <ns0:c r="F68" s="1">
         <ns0:f>ROUND(F67*1.4,-5)</ns0:f>
-        <ns0:v>1.3054332788971048e+20</ns0:v>
+        <ns0:v>1.3054330411434e+18</ns0:v>
       </ns0:c>
       <ns0:c r="G68" s="1" t="n">
         <ns0:v>13.8</ns0:v>
@@ -3218,7 +3218,7 @@
       </ns0:c>
       <ns0:c r="C69" s="1" t="inlineStr">
         <ns0:is>
-          <ns0:t>{42|0.1,164|0.2,149|0.3,179|0.4,157|0.5,46|0.6,27|0.7,174|0.8,89|0.9}</ns0:t>
+          <ns0:t>{30661|0.100000,30662|0.200000,30663|0.300000,30664|0.400000,30665|0.500000,30666|0.600000,30667|0.700000,30668|0.800000,30669|0.900000}</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="D69" s="1">
@@ -3231,7 +3231,7 @@
       </ns0:c>
       <ns0:c r="F69" s="1">
         <ns0:f>ROUND(F68*1.4,-5)</ns0:f>
-        <ns0:v>1.827606590455947e+20</ns0:v>
+        <ns0:v>1.8276062576007997e+18</ns0:v>
       </ns0:c>
       <ns0:c r="G69" s="1" t="n">
         <ns0:v>14</ns0:v>
@@ -3249,7 +3249,7 @@
       </ns0:c>
       <ns0:c r="C70" s="1" t="inlineStr">
         <ns0:is>
-          <ns0:t>{61|0.1,115|0.2,67|0.3,130|0.4,52|0.5,106|0.6,37|0.7,17|0.8,96|0.9}</ns0:t>
+          <ns0:t>{30671|0.100000,30672|0.200000,30673|0.300000,30674|0.400000,30675|0.500000,30676|0.600000,30677|0.700000,30678|0.800000,30679|0.900000}</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="D70" s="1">
@@ -3262,7 +3262,7 @@
       </ns0:c>
       <ns0:c r="F70" s="1">
         <ns0:f>ROUND(F69*1.4,-5)</ns0:f>
-        <ns0:v>2.558649226638326e+20</ns0:v>
+        <ns0:v>2.5586487606411e+18</ns0:v>
       </ns0:c>
       <ns0:c r="G70" s="1" t="n">
         <ns0:v>14.2</ns0:v>
@@ -3280,7 +3280,7 @@
       </ns0:c>
       <ns0:c r="C71" s="1" t="inlineStr">
         <ns0:is>
-          <ns0:t>{239|0.1,216|0.2,238|0.3,224|0.4,229|0.5,196|0.6,206|0.7,234|0.8,201|0.9}</ns0:t>
+          <ns0:t>{30681|0.100000,30682|0.200000,30683|0.300000,30684|0.400000,30685|0.500000,30686|0.600000,30687|0.700000,30688|0.800000,30689|0.900000}</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="D71" s="1">
@@ -3293,7 +3293,7 @@
       </ns0:c>
       <ns0:c r="F71" s="1">
         <ns0:f>ROUND(F70*1.4,-5)</ns0:f>
-        <ns0:v>3.5821089172936557e+20</ns0:v>
+        <ns0:v>3.5821082648974996e+18</ns0:v>
       </ns0:c>
       <ns0:c r="G71" s="1" t="n">
         <ns0:v>14.4</ns0:v>
@@ -3311,7 +3311,7 @@
       </ns0:c>
       <ns0:c r="C72" s="1" t="inlineStr">
         <ns0:is>
-          <ns0:t>{208|0.1,226|0.2,190|0.3,228|0.4,191|0.5,256|0.6,225|0.7,209|0.8,198|0.9}</ns0:t>
+          <ns0:t>{30691|0.100000,30692|0.200000,30693|0.300000,30694|0.400000,30695|0.500000,30696|0.600000,30697|0.700000,30698|0.800000,30699|0.900000}</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="D72" s="1">
@@ -3324,7 +3324,7 @@
       </ns0:c>
       <ns0:c r="F72" s="1">
         <ns0:f>ROUND(F71*1.4,-5)</ns0:f>
-        <ns0:v>5.014952484211118e+20</ns0:v>
+        <ns0:v>5.014951570856499e+18</ns0:v>
       </ns0:c>
       <ns0:c r="G72" s="1" t="n">
         <ns0:v>14.6</ns0:v>
@@ -3342,7 +3342,7 @@
       </ns0:c>
       <ns0:c r="C73" s="1" t="inlineStr">
         <ns0:is>
-          <ns0:t>{253|0.1,265|0.2,268|0.3,247|0.4,250|0.5,249|0.6,252|0.7,255|0.8,260|0.9}</ns0:t>
+          <ns0:t>{30701|0.100000,30702|0.200000,30703|0.300000,30704|0.400000,30705|0.500000,30706|0.600000,30707|0.700000,30708|0.800000,30709|0.900000}</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="D73" s="1">
@@ -3355,7 +3355,7 @@
       </ns0:c>
       <ns0:c r="F73" s="1">
         <ns0:f>ROUND(F72*1.4,-5)</ns0:f>
-        <ns0:v>7.020933477895565e+20</ns0:v>
+        <ns0:v>7.0209321991991e+18</ns0:v>
       </ns0:c>
       <ns0:c r="G73" s="1" t="n">
         <ns0:v>14.8</ns0:v>
@@ -3373,7 +3373,7 @@
       </ns0:c>
       <ns0:c r="C74" s="1" t="inlineStr">
         <ns0:is>
-          <ns0:t>{139|0.1,121|0.2,51|0.3,73|0.4,69|0.5,39|0.6,49|0.7,91|0.8,120|0.9}</ns0:t>
+          <ns0:t>{30711|0.100000,30712|0.200000,30713|0.300000,30714|0.400000,30715|0.500000,30716|0.600000,30717|0.700000,30718|0.800000,30719|0.900000}</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="D74" s="1">
@@ -3386,7 +3386,7 @@
       </ns0:c>
       <ns0:c r="F74" s="1">
         <ns0:f>ROUND(F73*1.4,-5)</ns0:f>
-        <ns0:v>9.82930686905379e+20</ns0:v>
+        <ns0:v>9.8293050788787e+18</ns0:v>
       </ns0:c>
       <ns0:c r="G74" s="1" t="n">
         <ns0:v>15</ns0:v>
@@ -3405,7 +3405,7 @@
       </ns0:c>
       <ns0:c r="C75" s="1" t="inlineStr">
         <ns0:is>
-          <ns0:t>{23|0.1,119|0.2,22|0.3,145|0.4,57|0.5,98|0.6,127|0.7,64|0.8,161|0.9}</ns0:t>
+          <ns0:t>{30721|0.100000,30722|0.200000,30723|0.300000,30724|0.400000,30725|0.500000,30726|0.600000,30727|0.700000,30728|0.800000,30729|0.900000}</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="D75" s="1">
@@ -3418,7 +3418,7 @@
       </ns0:c>
       <ns0:c r="F75" s="1">
         <ns0:f>ROUND(F74*1.4,-5)</ns0:f>
-        <ns0:v>1.3761029616675306e+21</ns0:v>
+        <ns0:v>1.37610271104302e+19</ns0:v>
       </ns0:c>
       <ns0:c r="G75" s="1" t="n">
         <ns0:v>15.2</ns0:v>
@@ -3437,7 +3437,7 @@
       </ns0:c>
       <ns0:c r="C76" s="1" t="inlineStr">
         <ns0:is>
-          <ns0:t>{214|0.1,223|0.2,197|0.3,193|0.4,203|0.5,202|0.6,195|0.7,199|0.8,215|0.9}</ns0:t>
+          <ns0:t>{30731|0.100000,30732|0.200000,30733|0.300000,30734|0.400000,30735|0.500000,30736|0.600000,30737|0.700000,30738|0.800000,30739|0.900000}</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="D76" s="1">
@@ -3450,7 +3450,7 @@
       </ns0:c>
       <ns0:c r="F76" s="1">
         <ns0:f>ROUND(F75*1.4,-5)</ns0:f>
-        <ns0:v>1.9265441463345427e+21</ns0:v>
+        <ns0:v>1.92654379546023e+19</ns0:v>
       </ns0:c>
       <ns0:c r="G76" s="1" t="n">
         <ns0:v>15.4</ns0:v>
@@ -3469,7 +3469,7 @@
       </ns0:c>
       <ns0:c r="C77" s="1" t="inlineStr">
         <ns0:is>
-          <ns0:t>{192|0.1,262|0.2,231|0.3,212|0.4,222|0.5,194|0.6,211|0.7,213|0.8,210|0.9}</ns0:t>
+          <ns0:t>{30741|0.100000,30742|0.200000,30743|0.300000,30744|0.400000,30745|0.500000,30746|0.600000,30747|0.700000,30748|0.800000,30749|0.900000}</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="D77" s="1">
@@ -3482,7 +3482,7 @@
       </ns0:c>
       <ns0:c r="F77" s="1">
         <ns0:f>ROUND(F76*1.4,-5)</ns0:f>
-        <ns0:v>2.69716180486836e+21</ns0:v>
+        <ns0:v>2.69716131364432e+19</ns0:v>
       </ns0:c>
       <ns0:c r="G77" s="1" t="n">
         <ns0:v>15.6</ns0:v>
@@ -3501,7 +3501,7 @@
       </ns0:c>
       <ns0:c r="C78" s="1" t="inlineStr">
         <ns0:is>
-          <ns0:t>{220|0.1,246|0.2,258|0.3,248|0.4,237|0.5,219|0.6,254|0.7,236|0.8,221|0.9}</ns0:t>
+          <ns0:t>{30751|0.100000,30752|0.200000,30753|0.300000,30754|0.400000,30755|0.500000,30756|0.600000,30757|0.700000,30758|0.800000,30759|0.900000}</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="D78" s="1">
@@ -3514,7 +3514,7 @@
       </ns0:c>
       <ns0:c r="F78" s="1">
         <ns0:f>ROUND(F77*1.4,-5)</ns0:f>
-        <ns0:v>3.7760265268157035e+21</ns0:v>
+        <ns0:v>3.7760258391020495e+19</ns0:v>
       </ns0:c>
       <ns0:c r="G78" s="1" t="n">
         <ns0:v>15.8</ns0:v>
@@ -3533,7 +3533,7 @@
       </ns0:c>
       <ns0:c r="C79" s="1" t="inlineStr">
         <ns0:is>
-          <ns0:t>{59|0.1,34|0.2,54|0.3,108|0.4,107|0.5,74|0.6,104|0.7,71|0.8,103|0.9}</ns0:t>
+          <ns0:t>{30761|0.100000,30762|0.200000,30763|0.300000,30764|0.400000,30765|0.500000,30766|0.600000,30767|0.700000,30768|0.800000,30769|0.900000}</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="D79" s="1">
@@ -3546,7 +3546,7 @@
       </ns0:c>
       <ns0:c r="F79" s="1">
         <ns0:f>ROUND(F78*1.4,-5)</ns0:f>
-        <ns0:v>5.286437137541984e+21</ns0:v>
+        <ns0:v>5.28643617474287e+19</ns0:v>
       </ns0:c>
       <ns0:c r="G79" s="1" t="n">
         <ns0:v>16</ns0:v>
@@ -3565,7 +3565,7 @@
       </ns0:c>
       <ns0:c r="C80" s="1" t="inlineStr">
         <ns0:is>
-          <ns0:t>{146|0.1,55|0.2,154|0.3,28|0.4,133|0.5,48|0.6,47|0.7,88|0.8,94|0.9}</ns0:t>
+          <ns0:t>{30771|0.100000,30772|0.200000,30773|0.300000,30774|0.400000,30775|0.500000,30776|0.600000,30777|0.700000,30778|0.800000,30779|0.900000}</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="D80" s="1">
@@ -3578,7 +3578,7 @@
       </ns0:c>
       <ns0:c r="F80" s="1">
         <ns0:f>ROUND(F79*1.4,-5)</ns0:f>
-        <ns0:v>7.401011992558778e+21</ns0:v>
+        <ns0:v>7.40101064464002e+19</ns0:v>
       </ns0:c>
       <ns0:c r="G80" s="1" t="n">
         <ns0:v>16.2</ns0:v>
@@ -3597,7 +3597,7 @@
       </ns0:c>
       <ns0:c r="C81" s="1" t="inlineStr">
         <ns0:is>
-          <ns0:t>{242|0.1,244|0.2,204|0.3,241|0.4,216|0.5,217|0.6,200|0.7,207|0.8,238|0.9}</ns0:t>
+          <ns0:t>{30781|0.100000,30782|0.200000,30783|0.300000,30784|0.400000,30785|0.500000,30786|0.600000,30787|0.700000,30788|0.800000,30789|0.900000}</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="D81" s="1">
@@ -3610,7 +3610,7 @@
       </ns0:c>
       <ns0:c r="F81" s="1">
         <ns0:f>ROUND(F80*1.4,-5)</ns0:f>
-        <ns0:v>1.0361416789582288e+22</ns0:v>
+        <ns0:v>1.036141490249603e+20</ns0:v>
       </ns0:c>
       <ns0:c r="G81" s="1" t="n">
         <ns0:v>16.4</ns0:v>
@@ -3629,7 +3629,7 @@
       </ns0:c>
       <ns0:c r="C82" s="1" t="inlineStr">
         <ns0:is>
-          <ns0:t>{218|0.1,227|0.2,245|0.3,205|0.4,196|0.5,190|0.6,228|0.7,201|0.8,222|0.9}</ns0:t>
+          <ns0:t>{30791|0.100000,30792|0.200000,30793|0.300000,30794|0.400000,30795|0.500000,30796|0.600000,30797|0.700000,30798|0.800000,30799|0.900000}</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="D82" s="1">
@@ -3642,7 +3642,7 @@
       </ns0:c>
       <ns0:c r="F82" s="1">
         <ns0:f>ROUND(F81*1.4,-5)</ns0:f>
-        <ns0:v>1.4505983505415201e+22</ns0:v>
+        <ns0:v>1.4505980863494439e+20</ns0:v>
       </ns0:c>
       <ns0:c r="G82" s="1" t="n">
         <ns0:v>16.6</ns0:v>
@@ -3661,7 +3661,7 @@
       </ns0:c>
       <ns0:c r="C83" s="1" t="inlineStr">
         <ns0:is>
-          <ns0:t>{249|0.1,264|0.2,261|0.3,251|0.4,248|0.5,259|0.6,268|0.7,250|0.8,257|0.9}</ns0:t>
+          <ns0:t>{30801|0.100000,30802|0.200000,30803|0.300000,30804|0.400000,30805|0.500000,30806|0.600000,30807|0.700000,30808|0.800000,30809|0.900000}</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="D83" s="1">
@@ -3674,7 +3674,7 @@
       </ns0:c>
       <ns0:c r="F83" s="1">
         <ns0:f>ROUND(F82*1.4,-5)</ns0:f>
-        <ns0:v>2.030837690758128e+22</ns0:v>
+        <ns0:v>2.0308373208892218e+20</ns0:v>
       </ns0:c>
       <ns0:c r="G83" s="1" t="n">
         <ns0:v>16.8</ns0:v>
@@ -3693,7 +3693,7 @@
       </ns0:c>
       <ns0:c r="C84" s="1" t="inlineStr">
         <ns0:is>
-          <ns0:t>{58|0.1,16|0.2,87|0.3,32|0.4,159|0.5,30|0.6,112|0.7,33|0.8,152|0.9}</ns0:t>
+          <ns0:t>{30811|0.100000,30812|0.200000,30813|0.300000,30814|0.400000,30815|0.500000,30816|0.600000,30817|0.700000,30818|0.800000,30819|0.900000}</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="D84" s="1">
@@ -3706,7 +3706,7 @@
       </ns0:c>
       <ns0:c r="F84" s="1">
         <ns0:f>ROUND(F83*1.4,-5)</ns0:f>
-        <ns0:v>2.8431727670613793e+22</ns0:v>
+        <ns0:v>2.843172249244911e+20</ns0:v>
       </ns0:c>
       <ns0:c r="G84" s="1" t="n">
         <ns0:v>17</ns0:v>
@@ -3725,7 +3725,7 @@
       </ns0:c>
       <ns0:c r="C85" s="1" t="inlineStr">
         <ns0:is>
-          <ns0:t>{125|0.1,84|0.2,155|0.3,66|0.4,113|0.5,131|0.6,18|0.7,77|0.8,134|0.9}</ns0:t>
+          <ns0:t>{30821|0.100000,30822|0.200000,30823|0.300000,30824|0.400000,30825|0.500000,30826|0.600000,30827|0.700000,30828|0.800000,30829|0.900000}</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="D85" s="1">
@@ -3738,7 +3738,7 @@
       </ns0:c>
       <ns0:c r="F85" s="1">
         <ns0:f>ROUND(F84*1.4,-5)</ns0:f>
-        <ns0:v>3.9804418738859306e+22</ns0:v>
+        <ns0:v>3.980441148942875e+20</ns0:v>
       </ns0:c>
       <ns0:c r="G85" s="1" t="n">
         <ns0:v>17.2</ns0:v>
@@ -3757,7 +3757,7 @@
       </ns0:c>
       <ns0:c r="C86" s="1" t="inlineStr">
         <ns0:is>
-          <ns0:t>{239|0.1,224|0.2,229|0.3,206|0.4,193|0.5,202|0.6,199|0.7,195|0.8,203|0.9}</ns0:t>
+          <ns0:t>{30831|0.100000,30832|0.200000,30833|0.300000,30834|0.400000,30835|0.500000,30836|0.600000,30837|0.700000,30838|0.800000,30839|0.900000}</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="D86" s="1">
@@ -3770,7 +3770,7 @@
       </ns0:c>
       <ns0:c r="F86" s="1">
         <ns0:f>ROUND(F85*1.4,-5)</ns0:f>
-        <ns0:v>5.572618623440302e+22</ns0:v>
+        <ns0:v>5.5726176085200254e+20</ns0:v>
       </ns0:c>
       <ns0:c r="G86" s="1" t="n">
         <ns0:v>17.4</ns0:v>
@@ -3789,7 +3789,7 @@
       </ns0:c>
       <ns0:c r="C87" s="1" t="inlineStr">
         <ns0:is>
-          <ns0:t>{210|0.1,205|0.2,192|0.3,225|0.4,211|0.5,256|0.6,208|0.7,226|0.8,191|0.9}</ns0:t>
+          <ns0:t>{30841|0.100000,30842|0.200000,30843|0.300000,30844|0.400000,30845|0.500000,30846|0.600000,30847|0.700000,30848|0.800000,30849|0.900000}</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="D87" s="1">
@@ -3802,7 +3802,7 @@
       </ns0:c>
       <ns0:c r="F87" s="1">
         <ns0:f>ROUND(F86*1.4,-5)</ns0:f>
-        <ns0:v>7.801666072816423e+22</ns0:v>
+        <ns0:v>7.801664651928036e+20</ns0:v>
       </ns0:c>
       <ns0:c r="G87" s="1" t="n">
         <ns0:v>17.6</ns0:v>
@@ -3821,7 +3821,7 @@
       </ns0:c>
       <ns0:c r="C88" s="1" t="inlineStr">
         <ns0:is>
-          <ns0:t>{258|0.1,230|0.2,235|0.3,240|0.4,254|0.5,246|0.6,243|0.7,220|0.8,232|0.9}</ns0:t>
+          <ns0:t>{30851|0.100000,30852|0.200000,30853|0.300000,30854|0.400000,30855|0.500000,30856|0.600000,30857|0.700000,30858|0.800000,30859|0.900000}</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="D88" s="1">
@@ -3834,7 +3834,7 @@
       </ns0:c>
       <ns0:c r="F88" s="1">
         <ns0:f>ROUND(F87*1.4,-5)</ns0:f>
-        <ns0:v>1.092233250194299e+23</ns0:v>
+        <ns0:v>1.0922330512699249e+21</ns0:v>
       </ns0:c>
       <ns0:c r="G88" s="1" t="n">
         <ns0:v>17.8</ns0:v>
@@ -3853,7 +3853,7 @@
       </ns0:c>
       <ns0:c r="C89" s="1" t="inlineStr">
         <ns0:is>
-          <ns0:t>{95|0.1,144|0.2,21|0.3,20|0.4,75|0.5,81|0.6,38|0.7,79|0.8,177|0.9}</ns0:t>
+          <ns0:t>{30861|0.100000,30862|0.200000,30863|0.300000,30864|0.400000,30865|0.500000,30866|0.600000,30867|0.700000,30868|0.800000,30869|0.900000}</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="D89" s="1">
@@ -3866,7 +3866,7 @@
       </ns0:c>
       <ns0:c r="F89" s="1">
         <ns0:f>ROUND(F88*1.4,-5)</ns0:f>
-        <ns0:v>1.5291265502720185e+23</ns0:v>
+        <ns0:v>1.5291262717778948e+21</ns0:v>
       </ns0:c>
       <ns0:c r="G89" s="1" t="n">
         <ns0:v>18</ns0:v>
@@ -3885,7 +3885,7 @@
       </ns0:c>
       <ns0:c r="C90" s="1" t="inlineStr">
         <ns0:is>
-          <ns0:t>{26|0.1,171|0.2,114|0.3,129|0.4,175|0.5,189|0.6,65|0.7,148|0.8,182|0.9}</ns0:t>
+          <ns0:t>{30871|0.100000,30872|0.200000,30873|0.300000,30874|0.400000,30875|0.500000,30876|0.600000,30877|0.700000,30878|0.800000,30879|0.900000}</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="D90" s="1">
@@ -3898,7 +3898,7 @@
       </ns0:c>
       <ns0:c r="F90" s="1">
         <ns0:f>ROUND(F89*1.4,-5)</ns0:f>
-        <ns0:v>2.140777170380826e+23</ns0:v>
+        <ns0:v>2.1407767804890527e+21</ns0:v>
       </ns0:c>
       <ns0:c r="G90" s="1" t="n">
         <ns0:v>18.2</ns0:v>
@@ -3917,7 +3917,7 @@
       </ns0:c>
       <ns0:c r="C91" s="1" t="inlineStr">
         <ns0:is>
-          <ns0:t>{214|0.1,223|0.2,197|0.3,234|0.4,215|0.5,204|0.6,217|0.7,238|0.8,216|0.9}</ns0:t>
+          <ns0:t>{30881|0.100000,30882|0.200000,30883|0.300000,30884|0.400000,30885|0.500000,30886|0.600000,30887|0.700000,30888|0.800000,30889|0.900000}</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="D91" s="1">
@@ -3930,7 +3930,7 @@
       </ns0:c>
       <ns0:c r="F91" s="1">
         <ns0:f>ROUND(F90*1.4,-5)</ns0:f>
-        <ns0:v>2.997088038533156e+23</ns0:v>
+        <ns0:v>2.9970874926846737e+21</ns0:v>
       </ns0:c>
       <ns0:c r="G91" s="1" t="n">
         <ns0:v>18.4</ns0:v>
@@ -3949,7 +3949,7 @@
       </ns0:c>
       <ns0:c r="C92" s="1" t="inlineStr">
         <ns0:is>
-          <ns0:t>{218|0.1,262|0.2,212|0.3,209|0.4,198|0.5,194|0.6,245|0.7,213|0.8,227|0.9}</ns0:t>
+          <ns0:t>{30891|0.100000,30892|0.200000,30893|0.300000,30894|0.400000,30895|0.500000,30896|0.600000,30897|0.700000,30898|0.800000,30899|0.900000}</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="D92" s="1">
@@ -3962,7 +3962,7 @@
       </ns0:c>
       <ns0:c r="F92" s="1">
         <ns0:f>ROUND(F91*1.4,-5)</ns0:f>
-        <ns0:v>4.195923253946418e+23</ns0:v>
+        <ns0:v>4.195922489758543e+21</ns0:v>
       </ns0:c>
       <ns0:c r="G92" s="1" t="n">
         <ns0:v>18.6</ns0:v>
@@ -3981,7 +3981,7 @@
       </ns0:c>
       <ns0:c r="C93" s="1" t="inlineStr">
         <ns0:is>
-          <ns0:t>{253|0.1,265|0.2,247|0.3,261|0.4,252|0.5,260|0.6,264|0.7,255|0.8,251|0.9}</ns0:t>
+          <ns0:t>{30901|0.100000,30902|0.200000,30903|0.300000,30904|0.400000,30905|0.500000,30906|0.600000,30907|0.700000,30908|0.800000,30909|0.900000}</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="D93" s="1">
@@ -3994,7 +3994,7 @@
       </ns0:c>
       <ns0:c r="F93" s="1">
         <ns0:f>ROUND(F92*1.4,-5)</ns0:f>
-        <ns0:v>5.8742925555249847e+23</ns0:v>
+        <ns0:v>5.87429148566196e+21</ns0:v>
       </ns0:c>
       <ns0:c r="G93" s="1" t="n">
         <ns0:v>18.8</ns0:v>
@@ -4013,7 +4013,7 @@
       </ns0:c>
       <ns0:c r="C94" s="1" t="inlineStr">
         <ns0:is>
-          <ns0:t>{139|0.1,167|0.2,40|0.3,156|0.4,29|0.5,169|0.6,44|0.7,86|0.8,180|0.9}</ns0:t>
+          <ns0:t>{30911|0.100000,30912|0.200000,30913|0.300000,30914|0.400000,30915|0.500000,30916|0.600000,30917|0.700000,30918|0.800000,30919|0.900000}</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="D94" s="1">
@@ -4026,7 +4026,7 @@
       </ns0:c>
       <ns0:c r="F94" s="1">
         <ns0:f>ROUND(F93*1.4,-5)</ns0:f>
-        <ns0:v>8.224009577734978e+23</ns0:v>
+        <ns0:v>8.224008079926744e+21</ns0:v>
       </ns0:c>
       <ns0:c r="G94" s="1" t="n">
         <ns0:v>19</ns0:v>
@@ -4045,7 +4045,7 @@
       </ns0:c>
       <ns0:c r="C95" s="1" t="inlineStr">
         <ns0:is>
-          <ns0:t>{149|0.1,153|0.2,101|0.3,102|0.4,183|0.5,31|0.6,50|0.7,19|0.8,164|0.9}</ns0:t>
+          <ns0:t>{30921|0.100000,30922|0.200000,30923|0.300000,30924|0.400000,30925|0.500000,30926|0.600000,30927|0.700000,30928|0.800000,30929|0.900000}</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="D95" s="1">
@@ -4058,7 +4058,7 @@
       </ns0:c>
       <ns0:c r="F95" s="1">
         <ns0:f>ROUND(F94*1.4,-5)</ns0:f>
-        <ns0:v>1.1513613408828967e+24</ns0:v>
+        <ns0:v>1.151361131189744e+22</ns0:v>
       </ns0:c>
       <ns0:c r="G95" s="1" t="n">
         <ns0:v>19.2</ns0:v>
@@ -4077,7 +4077,7 @@
       </ns0:c>
       <ns0:c r="C96" s="1" t="inlineStr">
         <ns0:is>
-          <ns0:t>{221|0.1,242|0.2,241|0.3,200|0.4,207|0.5,224|0.6,196|0.7,234|0.8,201|0.9}</ns0:t>
+          <ns0:t>{30931|0.100000,30932|0.200000,30933|0.300000,30934|0.400000,30935|0.500000,30936|0.600000,30937|0.700000,30938|0.800000,30939|0.900000}</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="D96" s="1">
@@ -4090,7 +4090,7 @@
       </ns0:c>
       <ns0:c r="F96" s="1">
         <ns0:f>ROUND(F95*1.4,-5)</ns0:f>
-        <ns0:v>1.6119058772360553e+24</ns0:v>
+        <ns0:v>1.6119055836656414e+22</ns0:v>
       </ns0:c>
       <ns0:c r="G96" s="1" t="n">
         <ns0:v>19.4</ns0:v>
@@ -4109,7 +4109,7 @@
       </ns0:c>
       <ns0:c r="C97" s="1" t="inlineStr">
         <ns0:is>
-          <ns0:t>{231|0.1,228|0.2,256|0.3,190|0.4,191|0.5,222|0.6,225|0.7,209|0.8,198|0.9}</ns0:t>
+          <ns0:t>{30941|0.100000,30942|0.200000,30943|0.300000,30944|0.400000,30945|0.500000,30946|0.600000,30947|0.700000,30948|0.800000,30949|0.900000}</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="D97" s="1">
@@ -4122,7 +4122,7 @@
       </ns0:c>
       <ns0:c r="F97" s="1">
         <ns0:f>ROUND(F96*1.4,-5)</ns0:f>
-        <ns0:v>2.2566682281304774e+24</ns0:v>
+        <ns0:v>2.256667817131898e+22</ns0:v>
       </ns0:c>
       <ns0:c r="G97" s="1" t="n">
         <ns0:v>19.6</ns0:v>
@@ -4141,7 +4141,7 @@
       </ns0:c>
       <ns0:c r="C98" s="1" t="inlineStr">
         <ns0:is>
-          <ns0:t>{237|0.1,233|0.2,230|0.3,219|0.4,257|0.5,244|0.6,240|0.7,232|0.8,243|0.9}</ns0:t>
+          <ns0:t>{30951|0.100000,30952|0.200000,30953|0.300000,30954|0.400000,30955|0.500000,30956|0.600000,30957|0.700000,30958|0.800000,30959|0.900000}</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="D98" s="1">
@@ -4154,7 +4154,7 @@
       </ns0:c>
       <ns0:c r="F98" s="1">
         <ns0:f>ROUND(F97*1.4,-5)</ns0:f>
-        <ns0:v>3.159335519382668e+24</ns0:v>
+        <ns0:v>3.159334943984657e+22</ns0:v>
       </ns0:c>
       <ns0:c r="G98" s="1" t="n">
         <ns0:v>19.8</ns0:v>
@@ -4173,7 +4173,7 @@
       </ns0:c>
       <ns0:c r="C99" s="1" t="inlineStr">
         <ns0:is>
-          <ns0:t>{76|0.1,100|0.2,97|0.3,110|0.4,118|0.5,62|0.6,126|0.7,172|0.8,128|0.9}</ns0:t>
+          <ns0:t>{30961|0.100000,30962|0.200000,30963|0.300000,30964|0.400000,30965|0.500000,30966|0.600000,30967|0.700000,30968|0.800000,30969|0.900000}</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="D99" s="1">
@@ -4186,7 +4186,7 @@
       </ns0:c>
       <ns0:c r="F99" s="1">
         <ns0:f>ROUND(F98*1.4,-5)</ns0:f>
-        <ns0:v>4.423069727135735e+24</ns0:v>
+        <ns0:v>4.4230689215785195e+22</ns0:v>
       </ns0:c>
       <ns0:c r="G99" s="1" t="n">
         <ns0:v>20</ns0:v>
@@ -4205,7 +4205,7 @@
       </ns0:c>
       <ns0:c r="C100" s="1" t="inlineStr">
         <ns0:is>
-          <ns0:t>{174|0.1,184|0.2,168|0.3,135|0.4,151|0.5,36|0.6,99|0.7,162|0.8,158|0.9}</ns0:t>
+          <ns0:t>{30971|0.100000,30972|0.200000,30973|0.300000,30974|0.400000,30975|0.500000,30976|0.600000,30977|0.700000,30978|0.800000,30979|0.900000}</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="D100" s="1">
@@ -4218,7 +4218,7 @@
       </ns0:c>
       <ns0:c r="F100" s="1">
         <ns0:f>ROUND(F99*1.4,-5)</ns0:f>
-        <ns0:v>6.192297617990029e+24</ns0:v>
+        <ns0:v>6.192296490209927e+22</ns0:v>
       </ns0:c>
       <ns0:c r="G100" s="1" t="n">
         <ns0:v>20.2</ns0:v>
@@ -4237,7 +4237,7 @@
       </ns0:c>
       <ns0:c r="C101" s="1" t="inlineStr">
         <ns0:is>
-          <ns0:t>{239|0.1,229|0.2,206|0.3,193|0.4,241|0.5,202|0.6,199|0.7,195|0.8,203|0.9}</ns0:t>
+          <ns0:t>{30981|0.100000,30982|0.200000,30983|0.300000,30984|0.400000,30985|0.500000,30986|0.600000,30987|0.700000,30988|0.800000,30989|0.900000}</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="D101" s="1">
@@ -4250,7 +4250,7 @@
       </ns0:c>
       <ns0:c r="F101" s="1">
         <ns0:f>ROUND(F100*1.4,-5)</ns0:f>
-        <ns0:v>8.669216665186042e+24</ns0:v>
+        <ns0:v>8.669215086293898e+22</ns0:v>
       </ns0:c>
       <ns0:c r="G101" s="1" t="n">
         <ns0:v>20.4</ns0:v>
@@ -4269,7 +4269,7 @@
       </ns0:c>
       <ns0:c r="C102" s="1" t="inlineStr">
         <ns0:is>
-          <ns0:t>{227|0.1,205|0.2,192|0.3,211|0.4,213|0.5,210|0.6,208|0.7,226|0.8,194|0.9}</ns0:t>
+          <ns0:t>{30991|0.100000,30992|0.200000,30993|0.300000,30994|0.400000,30995|0.500000,30996|0.600000,30997|0.700000,30998|0.800000,30999|0.900000}</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="D102" s="1">
@@ -4282,7 +4282,7 @@
       </ns0:c>
       <ns0:c r="F102" s="1">
         <ns0:f>ROUND(F101*1.4,-5)</ns0:f>
-        <ns0:v>1.2136903331260458e+25</ns0:v>
+        <ns0:v>1.2136901120811458e+23</ns0:v>
       </ns0:c>
       <ns0:c r="G102" s="1" t="n">
         <ns0:v>20.6</ns0:v>
@@ -4301,7 +4301,7 @@
       </ns0:c>
       <ns0:c r="C103" s="1" t="inlineStr">
         <ns0:is>
-          <ns0:t>{259|0.1,265|0.2,250|0.3,247|0.4,268|0.5,253|0.6,249|0.7,252|0.8,255|0.9}</ns0:t>
+          <ns0:t>{31001|0.100000,31002|0.200000,31003|0.300000,31004|0.400000,31005|0.500000,31006|0.600000,31007|0.700000,31008|0.800000,31009|0.900000}</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="D103" s="1">
@@ -4314,7 +4314,7 @@
       </ns0:c>
       <ns0:c r="F103" s="1">
         <ns0:f>ROUND(F102*1.4,-5)</ns0:f>
-        <ns0:v>1.699166466376464e+25</ns0:v>
+        <ns0:v>1.699166156913604e+23</ns0:v>
       </ns0:c>
       <ns0:c r="G103" s="1" t="n">
         <ns0:v>20.8</ns0:v>
@@ -4333,7 +4333,7 @@
       </ns0:c>
       <ns0:c r="C104" s="1" t="inlineStr">
         <ns0:is>
-          <ns0:t>{143|0.1,82|0.2,56|0.3,176|0.4,78|0.5,165|0.6,150|0.7,61|0.8,122|0.9}</ns0:t>
+          <ns0:t>{31011|0.100000,31012|0.200000,31013|0.300000,31014|0.400000,31015|0.500000,31016|0.600000,31017|0.700000,31018|0.800000,31019|0.900000}</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="D104" s="1">
@@ -4346,7 +4346,7 @@
       </ns0:c>
       <ns0:c r="F104" s="1">
         <ns0:f>ROUND(F103*1.4,-5)</ns0:f>
-        <ns0:v>2.3788330529270497e+25</ns0:v>
+        <ns0:v>2.3788326196790453e+23</ns0:v>
       </ns0:c>
       <ns0:c r="G104" s="1" t="n">
         <ns0:v>21</ns0:v>
@@ -4365,7 +4365,7 @@
       </ns0:c>
       <ns0:c r="C105" s="1" t="inlineStr">
         <ns0:is>
-          <ns0:t>{24|0.1,92|0.2,70|0.3,186|0.4,136|0.5,138|0.6,132|0.7,179|0.8,90|0.9}</ns0:t>
+          <ns0:t>{31021|0.100000,31022|0.200000,31023|0.300000,31024|0.400000,31025|0.500000,31026|0.600000,31027|0.700000,31028|0.800000,31029|0.900000}</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="D105" s="1">
@@ -4378,7 +4378,7 @@
       </ns0:c>
       <ns0:c r="F105" s="1">
         <ns0:f>ROUND(F104*1.4,-5)</ns0:f>
-        <ns0:v>3.3303662740978692e+25</ns0:v>
+        <ns0:v>3.3303656675506634e+23</ns0:v>
       </ns0:c>
       <ns0:c r="G105" s="1" t="n">
         <ns0:v>21.2</ns0:v>
@@ -4397,7 +4397,7 @@
       </ns0:c>
       <ns0:c r="C106" s="1" t="inlineStr">
         <ns0:is>
-          <ns0:t>{214|0.1,223|0.2,224|0.3,204|0.4,197|0.5,216|0.6,215|0.7,200|0.8,207|0.9}</ns0:t>
+          <ns0:t>{31031|0.100000,31032|0.200000,31033|0.300000,31034|0.400000,31035|0.500000,31036|0.600000,31037|0.700000,31038|0.800000,31039|0.900000}</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="D106" s="1">
@@ -4410,7 +4410,7 @@
       </ns0:c>
       <ns0:c r="F106" s="1">
         <ns0:f>ROUND(F105*1.4,-5)</ns0:f>
-        <ns0:v>4.6625127837370165e+25</ns0:v>
+        <ns0:v>4.662511934570929e+23</ns0:v>
       </ns0:c>
       <ns0:c r="G106" s="1" t="n">
         <ns0:v>21.4</ns0:v>
@@ -4429,7 +4429,7 @@
       </ns0:c>
       <ns0:c r="C107" s="1" t="inlineStr">
         <ns0:is>
-          <ns0:t>{218|0.1,262|0.2,212|0.3,245|0.4,190|0.5,228|0.6,201|0.7,222|0.8,198|0.9}</ns0:t>
+          <ns0:t>{31041|0.100000,31042|0.200000,31043|0.300000,31044|0.400000,31045|0.500000,31046|0.600000,31047|0.700000,31048|0.800000,31049|0.900000}</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="D107" s="1">
@@ -4442,7 +4442,7 @@
       </ns0:c>
       <ns0:c r="F107" s="1">
         <ns0:f>ROUND(F106*1.4,-5)</ns0:f>
-        <ns0:v>6.527517897231822e+25</ns0:v>
+        <ns0:v>6.5275167083993e+23</ns0:v>
       </ns0:c>
       <ns0:c r="G107" s="1" t="n">
         <ns0:v>21.6</ns0:v>
@@ -4461,7 +4461,7 @@
       </ns0:c>
       <ns0:c r="C108" s="1" t="inlineStr">
         <ns0:is>
-          <ns0:t>{235|0.1,236|0.2,258|0.3,246|0.4,220|0.5,233|0.6,254|0.7,248|0.8,219|0.9}</ns0:t>
+          <ns0:t>{31051|0.100000,31052|0.200000,31053|0.300000,31054|0.400000,31055|0.500000,31056|0.600000,31057|0.700000,31058|0.800000,31059|0.900000}</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="D108" s="1">
@@ -4474,7 +4474,7 @@
       </ns0:c>
       <ns0:c r="F108" s="1">
         <ns0:f>ROUND(F107*1.4,-5)</ns0:f>
-        <ns0:v>9.13852505612455e+25</ns0:v>
+        <ns0:v>9.138523391759019e+23</ns0:v>
       </ns0:c>
       <ns0:c r="G108" s="1" t="n">
         <ns0:v>21.8</ns0:v>
@@ -4493,7 +4493,7 @@
       </ns0:c>
       <ns0:c r="C109" s="1" t="inlineStr">
         <ns0:is>
-          <ns0:t>{46|0.1,68|0.2,53|0.3,141|0.4,85|0.5,123|0.6,188|0.7,187|0.8,173|0.9}</ns0:t>
+          <ns0:t>{31061|0.100000,31062|0.200000,31063|0.300000,31064|0.400000,31065|0.500000,31066|0.600000,31067|0.700000,31068|0.800000,31069|0.900000}</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="D109" s="1">
@@ -4506,7 +4506,7 @@
       </ns0:c>
       <ns0:c r="F109" s="1">
         <ns0:f>ROUND(F108*1.4,-5)</ns0:f>
-        <ns0:v>1.279393507857437e+26</ns0:v>
+        <ns0:v>1.2793932748462625e+24</ns0:v>
       </ns0:c>
       <ns0:c r="G109" s="1" t="n">
         <ns0:v>22</ns0:v>
@@ -4525,7 +4525,7 @@
       </ns0:c>
       <ns0:c r="C110" s="1" t="inlineStr">
         <ns0:is>
-          <ns0:t>{35|0.1,140|0.2,147|0.3,72|0.4,25|0.5,160|0.6,163|0.7,111|0.8,181|0.9}</ns0:t>
+          <ns0:t>{31071|0.100000,31072|0.200000,31073|0.300000,31074|0.400000,31075|0.500000,31076|0.600000,31077|0.700000,31078|0.800000,31079|0.900000}</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="D110" s="1">
@@ -4538,7 +4538,7 @@
       </ns0:c>
       <ns0:c r="F110" s="1">
         <ns0:f>ROUND(F109*1.4,-5)</ns0:f>
-        <ns0:v>1.7911509110004117e+26</ns0:v>
+        <ns0:v>1.7911505847847674e+24</ns0:v>
       </ns0:c>
       <ns0:c r="G110" s="1" t="n">
         <ns0:v>22.2</ns0:v>
@@ -4557,7 +4557,7 @@
       </ns0:c>
       <ns0:c r="C111" s="1" t="inlineStr">
         <ns0:is>
-          <ns0:t>{221|0.1,242|0.2,217|0.3,238|0.4,196|0.5,193|0.6,202|0.7,199|0.8,203|0.9}</ns0:t>
+          <ns0:t>{31081|0.100000,31082|0.200000,31083|0.300000,31084|0.400000,31085|0.500000,31086|0.600000,31087|0.700000,31088|0.800000,31089|0.900000}</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="D111" s="1">
@@ -4570,7 +4570,7 @@
       </ns0:c>
       <ns0:c r="F111" s="1">
         <ns0:f>ROUND(F110*1.4,-5)</ns0:f>
-        <ns0:v>2.5076112754005763e+26</ns0:v>
+        <ns0:v>2.507610818698674e+24</ns0:v>
       </ns0:c>
       <ns0:c r="G111" s="1" t="n">
         <ns0:v>22.4</ns0:v>
@@ -4589,7 +4589,7 @@
       </ns0:c>
       <ns0:c r="C112" s="1" t="inlineStr">
         <ns0:is>
-          <ns0:t>{210|0.1,192|0.2,196|0.3,225|0.4,209|0.5,211|0.6,231|0.7,256|0.8,194|0.9}</ns0:t>
+          <ns0:t>{31091|0.100000,31092|0.200000,31093|0.300000,31094|0.400000,31095|0.500000,31096|0.600000,31097|0.700000,31098|0.800000,31099|0.900000}</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="D112" s="1">
@@ -4602,7 +4602,7 @@
       </ns0:c>
       <ns0:c r="F112" s="1">
         <ns0:f>ROUND(F111*1.4,-5)</ns0:f>
-        <ns0:v>3.510655785560806e+26</ns0:v>
+        <ns0:v>3.5106551461781433e+24</ns0:v>
       </ns0:c>
       <ns0:c r="G112" s="1" t="n">
         <ns0:v>22.6</ns0:v>
@@ -4621,7 +4621,7 @@
       </ns0:c>
       <ns0:c r="C113" s="1" t="inlineStr">
         <ns0:is>
-          <ns0:t>{251|0.1,260|0.2,261|0.3,248|0.4,250|0.5,249|0.6,253|0.7,257|0.8,268|0.9}</ns0:t>
+          <ns0:t>{31101|0.100000,31102|0.200000,31103|0.300000,31104|0.400000,31105|0.500000,31106|0.600000,31107|0.700000,31108|0.800000,31109|0.900000}</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="D113" s="1">
@@ -4634,7 +4634,7 @@
       </ns0:c>
       <ns0:c r="F113" s="1">
         <ns0:f>ROUND(F112*1.4,-5)</ns0:f>
-        <ns0:v>4.9149180997851284e+26</ns0:v>
+        <ns0:v>4.9149172046494e+24</ns0:v>
       </ns0:c>
       <ns0:c r="G113" s="1" t="n">
         <ns0:v>22.8</ns0:v>
@@ -4653,7 +4653,7 @@
       </ns0:c>
       <ns0:c r="C114" s="1" t="inlineStr">
         <ns0:is>
-          <ns0:t>{157|0.1,83|0.2,116|0.3,178|0.4,124|0.5,166|0.6,185|0.7,45|0.8,105|0.9}</ns0:t>
+          <ns0:t>{31111|0.100000,31112|0.200000,31113|0.300000,31114|0.400000,31115|0.500000,31116|0.600000,31117|0.700000,31118|0.800000,31119|0.900000}</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="D114" s="1">
@@ -4666,7 +4666,7 @@
       </ns0:c>
       <ns0:c r="F114" s="1">
         <ns0:f>ROUND(F113*1.4,-5)</ns0:f>
-        <ns0:v>6.880885339699179e+26</ns0:v>
+        <ns0:v>6.88088408650916e+24</ns0:v>
       </ns0:c>
       <ns0:c r="G114" s="1" t="n">
         <ns0:v>23</ns0:v>
@@ -4685,7 +4685,7 @@
       </ns0:c>
       <ns0:c r="C115" s="1" t="inlineStr">
         <ns0:is>
-          <ns0:t>{80|0.1,115|0.2,137|0.3,41|0.4,109|0.5,63|0.6,170|0.7,27|0.8,89|0.9}</ns0:t>
+          <ns0:t>{31121|0.100000,31122|0.200000,31123|0.300000,31124|0.400000,31125|0.500000,31126|0.600000,31127|0.700000,31128|0.800000,31129|0.900000}</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="D115" s="1">
@@ -4698,7 +4698,7 @@
       </ns0:c>
       <ns0:c r="F115" s="1">
         <ns0:f>ROUND(F114*1.4,-5)</ns0:f>
-        <ns0:v>9.633239475578852e+26</ns0:v>
+        <ns0:v>9.633237721112824e+24</ns0:v>
       </ns0:c>
       <ns0:c r="G115" s="1" t="n">
         <ns0:v>23.2</ns0:v>
@@ -4717,7 +4717,7 @@
       </ns0:c>
       <ns0:c r="C116" s="1" t="inlineStr">
         <ns0:is>
-          <ns0:t>{244|0.1,206|0.2,229|0.3,224|0.4,195|0.5,215|0.6,234|0.7,204|0.8,197|0.9}</ns0:t>
+          <ns0:t>{31131|0.100000,31132|0.200000,31133|0.300000,31134|0.400000,31135|0.500000,31136|0.600000,31137|0.700000,31138|0.800000,31139|0.900000}</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="D116" s="1">
@@ -4730,7 +4730,7 @@
       </ns0:c>
       <ns0:c r="F116" s="1">
         <ns0:f>ROUND(F115*1.4,-5)</ns0:f>
-        <ns0:v>1.3486535265810393e+27</ns0:v>
+        <ns0:v>1.3486532809557953e+25</ns0:v>
       </ns0:c>
       <ns0:c r="G116" s="1" t="n">
         <ns0:v>23.4</ns0:v>
@@ -4749,7 +4749,7 @@
       </ns0:c>
       <ns0:c r="C117" s="1" t="inlineStr">
         <ns0:is>
-          <ns0:t>{208|0.1,226|0.2,262|0.3,191|0.4,205|0.5,213|0.6,227|0.7,207|0.8,212|0.9}</ns0:t>
+          <ns0:t>{31141|0.100000,31142|0.200000,31143|0.300000,31144|0.400000,31145|0.500000,31146|0.600000,31147|0.700000,31148|0.800000,31149|0.900000}</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="D117" s="1">
@@ -4762,7 +4762,7 @@
       </ns0:c>
       <ns0:c r="F117" s="1">
         <ns0:f>ROUND(F116*1.4,-5)</ns0:f>
-        <ns0:v>1.8881149372134549e+27</ns0:v>
+        <ns0:v>1.8881145933381136e+25</ns0:v>
       </ns0:c>
       <ns0:c r="G117" s="1" t="n">
         <ns0:v>23.6</ns0:v>
@@ -4781,7 +4781,7 @@
       </ns0:c>
       <ns0:c r="C118" s="1" t="inlineStr">
         <ns0:is>
-          <ns0:t>{237|0.1,246|0.2,236|0.3,220|0.4,240|0.5,233|0.6,243|0.7,239|0.8,230|0.9}</ns0:t>
+          <ns0:t>{31151|0.100000,31152|0.200000,31153|0.300000,31154|0.400000,31155|0.500000,31156|0.600000,31157|0.700000,31158|0.800000,31159|0.900000}</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="D118" s="1">
@@ -4794,7 +4794,7 @@
       </ns0:c>
       <ns0:c r="F118" s="1">
         <ns0:f>ROUND(F117*1.4,-5)</ns0:f>
-        <ns0:v>2.6433609120988366e+27</ns0:v>
+        <ns0:v>2.643360430673359e+25</ns0:v>
       </ns0:c>
       <ns0:c r="G118" s="1" t="n">
         <ns0:v>23.8</ns0:v>
@@ -4813,7 +4813,7 @@
       </ns0:c>
       <ns0:c r="C119" s="1" t="inlineStr">
         <ns0:is>
-          <ns0:t>{117|0.1,43|0.2,142|0.3,60|0.4,93|0.5,30|0.6,49|0.7,96|0.8,52|0.9}</ns0:t>
+          <ns0:t>{31161|0.100000,31162|0.200000,31163|0.300000,31164|0.400000,31165|0.500000,31166|0.600000,31167|0.700000,31168|0.800000,31169|0.900000}</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="D119" s="1">
@@ -4826,7 +4826,7 @@
       </ns0:c>
       <ns0:c r="F119" s="1">
         <ns0:f>ROUND(F118*1.4,-5)</ns0:f>
-        <ns0:v>3.700705276938371e+27</ns0:v>
+        <ns0:v>3.700704602942702e+25</ns0:v>
       </ns0:c>
       <ns0:c r="G119" s="1" t="n">
         <ns0:v>24</ns0:v>
@@ -4845,7 +4845,7 @@
       </ns0:c>
       <ns0:c r="C120" s="1" t="inlineStr">
         <ns0:is>
-          <ns0:t>{42|0.1,53|0.2,37|0.3,54|0.4,51|0.5,57|0.6,17|0.7,28|0.8,108|0.9}</ns0:t>
+          <ns0:t>{31171|0.100000,31172|0.200000,31173|0.300000,31174|0.400000,31175|0.500000,31176|0.600000,31177|0.700000,31178|0.800000,31179|0.900000}</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="D120" s="1">
@@ -4858,7 +4858,7 @@
       </ns0:c>
       <ns0:c r="F120" s="1">
         <ns0:f>ROUND(F119*1.4,-5)</ns0:f>
-        <ns0:v>5.180987387713719e+27</ns0:v>
+        <ns0:v>5.1809864441197824e+25</ns0:v>
       </ns0:c>
       <ns0:c r="G120" s="1" t="n">
         <ns0:v>24.2000000000001</ns0:v>
@@ -4877,7 +4877,7 @@
       </ns0:c>
       <ns0:c r="C121" s="1" t="inlineStr">
         <ns0:is>
-          <ns0:t>{214|0.1,223|0.2,217|0.3,238|0.4,241|0.5,200|0.6,216|0.7,215|0.8,202|0.9}</ns0:t>
+          <ns0:t>{31181|0.100000,31182|0.200000,31183|0.300000,31184|0.400000,31185|0.500000,31186|0.600000,31187|0.700000,31188|0.800000,31189|0.900000}</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="D121" s="1">
@@ -4890,7 +4890,7 @@
       </ns0:c>
       <ns0:c r="F121" s="1">
         <ns0:f>ROUND(F120*1.4,-5)</ns0:f>
-        <ns0:v>7.253382342799206e+27</ns0:v>
+        <ns0:v>7.253381021767694e+25</ns0:v>
       </ns0:c>
       <ns0:c r="G121" s="1" t="n">
         <ns0:v>24.4000000000001</ns0:v>
@@ -4909,7 +4909,7 @@
       </ns0:c>
       <ns0:c r="C122" s="1" t="inlineStr">
         <ns0:is>
-          <ns0:t>{218|0.1,225|0.2,190|0.3,191|0.4,245|0.5,228|0.6,256|0.7,209|0.8,198|0.9}</ns0:t>
+          <ns0:t>{31191|0.100000,31192|0.200000,31193|0.300000,31194|0.400000,31195|0.500000,31196|0.600000,31197|0.700000,31198|0.800000,31199|0.900000}</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="D122" s="1">
@@ -4922,7 +4922,7 @@
       </ns0:c>
       <ns0:c r="F122" s="1">
         <ns0:f>ROUND(F121*1.4,-5)</ns0:f>
-        <ns0:v>1.0154735279918888e+28</ns0:v>
+        <ns0:v>1.015473343047477e+26</ns0:v>
       </ns0:c>
       <ns0:c r="G122" s="1" t="n">
         <ns0:v>24.6000000000001</ns0:v>
@@ -4941,7 +4941,7 @@
       </ns0:c>
       <ns0:c r="C123" s="1" t="inlineStr">
         <ns0:is>
-          <ns0:t>{259|0.1,265|0.2,264|0.3,252|0.4,247|0.5,260|0.6,261|0.7,255|0.8,251|0.9}</ns0:t>
+          <ns0:t>{31201|0.100000,31202|0.200000,31203|0.300000,31204|0.400000,31205|0.500000,31206|0.600000,31207|0.700000,31208|0.800000,31209|0.900000}</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="D123" s="1">
@@ -4954,7 +4954,7 @@
       </ns0:c>
       <ns0:c r="F123" s="1">
         <ns0:f>ROUND(F122*1.4,-5)</ns0:f>
-        <ns0:v>1.4216629391886442e+28</ns0:v>
+        <ns0:v>1.4216626802664678e+26</ns0:v>
       </ns0:c>
       <ns0:c r="G123" s="1" t="n">
         <ns0:v>24.8000000000001</ns0:v>
@@ -4973,7 +4973,7 @@
       </ns0:c>
       <ns0:c r="C124" s="1" t="inlineStr">
         <ns0:is>
-          <ns0:t>{171|0.1,114|0.2,55|0.3,73|0.4,120|0.5,145|0.6,106|0.7,91|0.8,67|0.9}</ns0:t>
+          <ns0:t>{31211|0.100000,31212|0.200000,31213|0.300000,31214|0.400000,31215|0.500000,31216|0.600000,31217|0.700000,31218|0.800000,31219|0.900000}</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="D124" s="1">
@@ -4986,7 +4986,7 @@
       </ns0:c>
       <ns0:c r="F124" s="1">
         <ns0:f>ROUND(F123*1.4,-5)</ns0:f>
-        <ns0:v>1.990328114864102e+28</ns0:v>
+        <ns0:v>1.9903277523730548e+26</ns0:v>
       </ns0:c>
       <ns0:c r="G124" s="1" t="n">
         <ns0:v>25.0000000000001</ns0:v>
@@ -5005,7 +5005,7 @@
       </ns0:c>
       <ns0:c r="C125" s="1" t="inlineStr">
         <ns0:is>
-          <ns0:t>{86|0.1,154|0.2,87|0.3,39|0.4,107|0.5,48|0.6,127|0.7,125|0.8,79|0.9}</ns0:t>
+          <ns0:t>{31221|0.100000,31222|0.200000,31223|0.300000,31224|0.400000,31225|0.500000,31226|0.600000,31227|0.700000,31228|0.800000,31229|0.900000}</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="D125" s="1">
@@ -5018,7 +5018,7 @@
       </ns0:c>
       <ns0:c r="F125" s="1">
         <ns0:f>ROUND(F124*1.4,-5)</ns0:f>
-        <ns0:v>2.7864593608097423e+28</ns0:v>
+        <ns0:v>2.7864588533222764e+26</ns0:v>
       </ns0:c>
       <ns0:c r="G125" s="1" t="n">
         <ns0:v>25.2000000000001</ns0:v>
@@ -5037,7 +5037,7 @@
       </ns0:c>
       <ns0:c r="C126" s="1" t="inlineStr">
         <ns0:is>
-          <ns0:t>{221|0.1,242|0.2,201|0.3,193|0.4,224|0.5,195|0.6,203|0.7,199|0.8,197|0.9}</ns0:t>
+          <ns0:t>{31231|0.100000,31232|0.200000,31233|0.300000,31234|0.400000,31235|0.500000,31236|0.600000,31237|0.700000,31238|0.800000,31239|0.900000}</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="D126" s="1">
@@ -5050,7 +5050,7 @@
       </ns0:c>
       <ns0:c r="F126" s="1">
         <ns0:f>ROUND(F125*1.4,-5)</ns0:f>
-        <ns0:v>3.9010431051336393e+28</ns0:v>
+        <ns0:v>3.9010423946511864e+26</ns0:v>
       </ns0:c>
       <ns0:c r="G126" s="1" t="n">
         <ns0:v>25.4000000000001</ns0:v>
@@ -5069,7 +5069,7 @@
       </ns0:c>
       <ns0:c r="C127" s="1" t="inlineStr">
         <ns0:is>
-          <ns0:t>{262|0.1,205|0.2,192|0.3,222|0.4,231|0.5,194|0.6,211|0.7,196|0.8,210|0.9}</ns0:t>
+          <ns0:t>{31241|0.100000,31242|0.200000,31243|0.300000,31244|0.400000,31245|0.500000,31246|0.600000,31247|0.700000,31248|0.800000,31249|0.900000}</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="D127" s="1">
@@ -5082,7 +5082,7 @@
       </ns0:c>
       <ns0:c r="F127" s="1">
         <ns0:f>ROUND(F126*1.4,-5)</ns0:f>
-        <ns0:v>5.461460347187095e+28</ns0:v>
+        <ns0:v>5.4614593525116606e+26</ns0:v>
       </ns0:c>
       <ns0:c r="G127" s="1" t="n">
         <ns0:v>25.6000000000001</ns0:v>
@@ -5101,7 +5101,7 @@
       </ns0:c>
       <ns0:c r="C128" s="1" t="inlineStr">
         <ns0:is>
-          <ns0:t>{232|0.1,258|0.2,230|0.3,219|0.4,235|0.5,246|0.6,254|0.7,240|0.8,244|0.9}</ns0:t>
+          <ns0:t>{31251|0.100000,31252|0.200000,31253|0.300000,31254|0.400000,31255|0.500000,31256|0.600000,31257|0.700000,31258|0.800000,31259|0.900000}</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="D128" s="1">
@@ -5114,7 +5114,7 @@
       </ns0:c>
       <ns0:c r="F128" s="1">
         <ns0:f>ROUND(F127*1.4,-5)</ns0:f>
-        <ns0:v>7.646044486061932e+28</ns0:v>
+        <ns0:v>7.646043093516325e+26</ns0:v>
       </ns0:c>
       <ns0:c r="G128" s="1" t="n">
         <ns0:v>25.8000000000001</ns0:v>
@@ -5133,7 +5133,7 @@
       </ns0:c>
       <ns0:c r="C129" s="1" t="inlineStr">
         <ns0:is>
-          <ns0:t>{152|0.1,21|0.2,22|0.3,121|0.4,131|0.5,66|0.6,103|0.7,104|0.8,40|0.9}</ns0:t>
+          <ns0:t>{31261|0.100000,31262|0.200000,31263|0.300000,31264|0.400000,31265|0.500000,31266|0.600000,31267|0.700000,31268|0.800000,31269|0.900000}</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="D129" s="1">
@@ -5146,7 +5146,7 @@
       </ns0:c>
       <ns0:c r="F129" s="1">
         <ns0:f>ROUND(F128*1.4,-5)</ns0:f>
-        <ns0:v>1.0704462280486704e+29</ns0:v>
+        <ns0:v>1.0704460330922856e+27</ns0:v>
       </ns0:c>
       <ns0:c r="G129" s="1" t="n">
         <ns0:v>26.0000000000001</ns0:v>
@@ -5165,7 +5165,7 @@
       </ns0:c>
       <ns0:c r="C130" s="1" t="inlineStr">
         <ns0:is>
-          <ns0:t>{175|0.1,119|0.2,153|0.3,88|0.4,135|0.5,65|0.6,100|0.7,146|0.8,160|0.9}</ns0:t>
+          <ns0:t>{31271|0.100000,31272|0.200000,31273|0.300000,31274|0.400000,31275|0.500000,31276|0.600000,31277|0.700000,31278|0.800000,31279|0.900000}</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="D130" s="1">
@@ -5178,7 +5178,7 @@
       </ns0:c>
       <ns0:c r="F130" s="1">
         <ns0:f>ROUND(F129*1.4,-5)</ns0:f>
-        <ns0:v>1.4986247192681385e+29</ns0:v>
+        <ns0:v>1.4986244463291998e+27</ns0:v>
       </ns0:c>
       <ns0:c r="G130" s="1" t="n">
         <ns0:v>26.2000000000001</ns0:v>
@@ -5197,7 +5197,7 @@
       </ns0:c>
       <ns0:c r="C131" s="1" t="inlineStr">
         <ns0:is>
-          <ns0:t>{239|0.1,229|0.2,206|0.3,234|0.4,241|0.5,204|0.6,200|0.7,216|0.8,217|0.9}</ns0:t>
+          <ns0:t>{31281|0.100000,31282|0.200000,31283|0.300000,31284|0.400000,31285|0.500000,31286|0.600000,31287|0.700000,31288|0.800000,31289|0.900000}</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="D131" s="1">
@@ -5210,7 +5210,7 @@
       </ns0:c>
       <ns0:c r="F131" s="1">
         <ns0:f>ROUND(F130*1.4,-5)</ns0:f>
-        <ns0:v>2.0980746069753937e+29</ns0:v>
+        <ns0:v>2.0980742248608796e+27</ns0:v>
       </ns0:c>
       <ns0:c r="G131" s="1" t="n">
         <ns0:v>26.4000000000001</ns0:v>
@@ -5229,7 +5229,7 @@
       </ns0:c>
       <ns0:c r="C132" s="1" t="inlineStr">
         <ns0:is>
-          <ns0:t>{226|0.1,227|0.2,212|0.3,207|0.4,213|0.5,208|0.6,190|0.7,228|0.8,225|0.9}</ns0:t>
+          <ns0:t>{31291|0.100000,31292|0.200000,31293|0.300000,31294|0.400000,31295|0.500000,31296|0.600000,31297|0.700000,31298|0.800000,31299|0.900000}</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="D132" s="1">
@@ -5242,7 +5242,7 @@
       </ns0:c>
       <ns0:c r="F132" s="1">
         <ns0:f>ROUND(F131*1.4,-5)</ns0:f>
-        <ns0:v>2.9373044497655515e+29</ns0:v>
+        <ns0:v>2.9373039148052314e+27</ns0:v>
       </ns0:c>
       <ns0:c r="G132" s="1" t="n">
         <ns0:v>26.6000000000001</ns0:v>
@@ -5261,7 +5261,7 @@
       </ns0:c>
       <ns0:c r="C133" s="1" t="inlineStr">
         <ns0:is>
-          <ns0:t>{249|0.1,250|0.2,265|0.3,264|0.4,257|0.5,268|0.6,253|0.7,259|0.8,247|0.9}</ns0:t>
+          <ns0:t>{31301|0.100000,31302|0.200000,31303|0.300000,31304|0.400000,31305|0.500000,31306|0.600000,31307|0.700000,31308|0.800000,31309|0.900000}</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="D133" s="1">
@@ -5274,7 +5274,7 @@
       </ns0:c>
       <ns0:c r="F133" s="1">
         <ns0:f>ROUND(F132*1.4,-5)</ns0:f>
-        <ns0:v>4.112226229671772e+29</ns0:v>
+        <ns0:v>4.112225480727324e+27</ns0:v>
       </ns0:c>
       <ns0:c r="G133" s="1" t="n">
         <ns0:v>26.8000000000001</ns0:v>
@@ -5293,7 +5293,7 @@
       </ns0:c>
       <ns0:c r="C134" s="1" t="inlineStr">
         <ns0:is>
-          <ns0:t>{69|0.1,68|0.2,44|0.3,167|0.4,26|0.5,189|0.6,20|0.7,161|0.8,50|0.9}</ns0:t>
+          <ns0:t>{31311|0.100000,31312|0.200000,31313|0.300000,31314|0.400000,31315|0.500000,31316|0.600000,31317|0.700000,31318|0.800000,31319|0.900000}</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="D134" s="1">
@@ -5306,7 +5306,7 @@
       </ns0:c>
       <ns0:c r="F134" s="1">
         <ns0:f>ROUND(F133*1.4,-5)</ns0:f>
-        <ns0:v>5.7571167215404806e+29</ns0:v>
+        <ns0:v>5.757115673018253e+27</ns0:v>
       </ns0:c>
       <ns0:c r="G134" s="1" t="n">
         <ns0:v>27.0000000000001</ns0:v>
@@ -5325,7 +5325,7 @@
       </ns0:c>
       <ns0:c r="C135" s="1" t="inlineStr">
         <ns0:is>
-          <ns0:t>{82|0.1,29|0.2,118|0.3,98|0.4,18|0.5,148|0.6,23|0.7,110|0.8,138|0.9}</ns0:t>
+          <ns0:t>{31321|0.100000,31322|0.200000,31323|0.300000,31324|0.400000,31325|0.500000,31326|0.600000,31327|0.700000,31328|0.800000,31329|0.900000}</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="D135" s="1">
@@ -5338,7 +5338,7 @@
       </ns0:c>
       <ns0:c r="F135" s="1">
         <ns0:f>ROUND(F134*1.4,-5)</ns0:f>
-        <ns0:v>8.059963410156672e+29</ns0:v>
+        <ns0:v>8.059961942225552e+27</ns0:v>
       </ns0:c>
       <ns0:c r="G135" s="1" t="n">
         <ns0:v>27.2000000000001</ns0:v>
@@ -5357,7 +5357,7 @@
       </ns0:c>
       <ns0:c r="C136" s="1" t="inlineStr">
         <ns0:is>
-          <ns0:t>{214|0.1,223|0.2,238|0.3,193|0.4,241|0.5,201|0.6,202|0.7,203|0.8,199|0.9}</ns0:t>
+          <ns0:t>{31331|0.100000,31332|0.200000,31333|0.300000,31334|0.400000,31335|0.500000,31336|0.600000,31337|0.700000,31338|0.800000,31339|0.900000}</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="D136" s="1">
@@ -5370,7 +5370,7 @@
       </ns0:c>
       <ns0:c r="F136" s="1">
         <ns0:f>ROUND(F135*1.4,-5)</ns0:f>
-        <ns0:v>1.128394877421934e+30</ns0:v>
+        <ns0:v>1.1283946719115773e+28</ns0:v>
       </ns0:c>
       <ns0:c r="G136" s="1" t="n">
         <ns0:v>27.4000000000001</ns0:v>
@@ -5389,7 +5389,7 @@
       </ns0:c>
       <ns0:c r="C137" s="1" t="inlineStr">
         <ns0:is>
-          <ns0:t>{196|0.1,256|0.2,192|0.3,209|0.4,222|0.5,231|0.6,198|0.7,194|0.8,262|0.9}</ns0:t>
+          <ns0:t>{31341|0.100000,31342|0.200000,31343|0.300000,31344|0.400000,31345|0.500000,31346|0.600000,31347|0.700000,31348|0.800000,31349|0.900000}</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="D137" s="1">
@@ -5402,7 +5402,7 @@
       </ns0:c>
       <ns0:c r="F137" s="1">
         <ns0:f>ROUND(F136*1.4,-5)</ns0:f>
-        <ns0:v>1.5797528283907075e+30</ns0:v>
+        <ns0:v>1.5797525406762081e+28</ns0:v>
       </ns0:c>
       <ns0:c r="G137" s="1" t="n">
         <ns0:v>27.6000000000001</ns0:v>
@@ -5421,7 +5421,7 @@
       </ns0:c>
       <ns0:c r="C138" s="1" t="inlineStr">
         <ns0:is>
-          <ns0:t>{235|0.1,236|0.2,232|0.3,243|0.4,248|0.5,220|0.6,233|0.7,258|0.8,254|0.9}</ns0:t>
+          <ns0:t>{31351|0.100000,31352|0.200000,31353|0.300000,31354|0.400000,31355|0.500000,31356|0.600000,31357|0.700000,31358|0.800000,31359|0.900000}</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="D138" s="1">
@@ -5434,7 +5434,7 @@
       </ns0:c>
       <ns0:c r="F138" s="1">
         <ns0:f>ROUND(F137*1.4,-5)</ns0:f>
-        <ns0:v>2.2116539597469903e+30</ns0:v>
+        <ns0:v>2.211653556946691e+28</ns0:v>
       </ns0:c>
       <ns0:c r="G138" s="1" t="n">
         <ns0:v>27.8000000000001</ns0:v>
@@ -5453,7 +5453,7 @@
       </ns0:c>
       <ns0:c r="C139" s="1" t="inlineStr">
         <ns0:is>
-          <ns0:t>{143|0.1,19|0.2,58|0.3,184|0.4,133|0.5,112|0.6,38|0.7,172|0.8,113|0.9}</ns0:t>
+          <ns0:t>{31361|0.100000,31362|0.200000,31363|0.300000,31364|0.400000,31365|0.500000,31366|0.600000,31367|0.700000,31368|0.800000,31369|0.900000}</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="D139" s="1">
@@ -5466,7 +5466,7 @@
       </ns0:c>
       <ns0:c r="F139" s="1">
         <ns0:f>ROUND(F138*1.4,-5)</ns0:f>
-        <ns0:v>3.096315543645786e+30</ns0:v>
+        <ns0:v>3.096314979725367e+28</ns0:v>
       </ns0:c>
       <ns0:c r="G139" s="1" t="n">
         <ns0:v>28.0000000000001</ns0:v>
@@ -5485,7 +5485,7 @@
       </ns0:c>
       <ns0:c r="C140" s="1" t="inlineStr">
         <ns0:is>
-          <ns0:t>{85|0.1,129|0.2,169|0.3,94|0.4,64|0.5,155|0.6,74|0.7,182|0.8,59|0.9}</ns0:t>
+          <ns0:t>{31371|0.100000,31372|0.200000,31373|0.300000,31374|0.400000,31375|0.500000,31376|0.600000,31377|0.700000,31378|0.800000,31379|0.900000}</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="D140" s="1">
@@ -5498,7 +5498,7 @@
       </ns0:c>
       <ns0:c r="F140" s="1">
         <ns0:f>ROUND(F139*1.4,-5)</ns0:f>
-        <ns0:v>4.3348417611040996e+30</ns0:v>
+        <ns0:v>4.334840971615514e+28</ns0:v>
       </ns0:c>
       <ns0:c r="G140" s="1" t="n">
         <ns0:v>28.2000000000001</ns0:v>
@@ -5517,7 +5517,7 @@
       </ns0:c>
       <ns0:c r="C141" s="1" t="inlineStr">
         <ns0:is>
-          <ns0:t>{242|0.1,221|0.2,197|0.3,234|0.4,195|0.5,215|0.6,204|0.7,224|0.8,200|0.9}</ns0:t>
+          <ns0:t>{31381|0.100000,31382|0.200000,31383|0.300000,31384|0.400000,31385|0.500000,31386|0.600000,31387|0.700000,31388|0.800000,31389|0.900000}</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="D141" s="1">
@@ -5530,7 +5530,7 @@
       </ns0:c>
       <ns0:c r="F141" s="1">
         <ns0:f>ROUND(F140*1.4,-5)</ns0:f>
-        <ns0:v>6.068778465545739e+30</ns0:v>
+        <ns0:v>6.0687773602617194e+28</ns0:v>
       </ns0:c>
       <ns0:c r="G141" s="1" t="n">
         <ns0:v>28.4000000000001</ns0:v>
@@ -5549,7 +5549,7 @@
       </ns0:c>
       <ns0:c r="C142" s="1" t="inlineStr">
         <ns0:is>
-          <ns0:t>{245|0.1,218|0.2,227|0.3,191|0.4,205|0.5,210|0.6,207|0.7,211|0.8,213|0.9}</ns0:t>
+          <ns0:t>{31391|0.100000,31392|0.200000,31393|0.300000,31394|0.400000,31395|0.500000,31396|0.600000,31397|0.700000,31398|0.800000,31399|0.900000}</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="D142" s="1">
@@ -5562,7 +5562,7 @@
       </ns0:c>
       <ns0:c r="F142" s="1">
         <ns0:f>ROUND(F141*1.4,-5)</ns0:f>
-        <ns0:v>8.496289851764034e+30</ns0:v>
+        <ns0:v>8.496288304366406e+28</ns0:v>
       </ns0:c>
       <ns0:c r="G142" s="1" t="n">
         <ns0:v>28.6000000000001</ns0:v>
@@ -5581,7 +5581,7 @@
       </ns0:c>
       <ns0:c r="C143" s="1" t="inlineStr">
         <ns0:is>
-          <ns0:t>{251|0.1,260|0.2,255|0.3,247|0.4,252|0.5,248|0.6,268|0.7,261|0.8,253|0.9}</ns0:t>
+          <ns0:t>{31401|0.100000,31402|0.200000,31403|0.300000,31404|0.400000,31405|0.500000,31406|0.600000,31407|0.700000,31408|0.800000,31409|0.900000}</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="D143" s="1">
@@ -5594,7 +5594,7 @@
       </ns0:c>
       <ns0:c r="F143" s="1">
         <ns0:f>ROUND(F142*1.4,-5)</ns0:f>
-        <ns0:v>1.1894805792469646e+31</ns0:v>
+        <ns0:v>1.1894803626112967e+29</ns0:v>
       </ns0:c>
       <ns0:c r="G143" s="1" t="n">
         <ns0:v>28.8000000000001</ns0:v>
@@ -5613,7 +5613,7 @@
       </ns0:c>
       <ns0:c r="C144" s="1" t="inlineStr">
         <ns0:is>
-          <ns0:t>{25|0.1,47|0.2,95|0.3,99|0.4,81|0.5,183|0.6,159|0.7,176|0.8,34|0.9}</ns0:t>
+          <ns0:t>{31411|0.100000,31412|0.200000,31413|0.300000,31414|0.400000,31415|0.500000,31416|0.600000,31417|0.700000,31418|0.800000,31419|0.900000}</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="D144" s="1">
@@ -5626,7 +5626,7 @@
       </ns0:c>
       <ns0:c r="F144" s="1">
         <ns0:f>ROUND(F143*1.4,-5)</ns0:f>
-        <ns0:v>1.6652728109457504e+31</ns0:v>
+        <ns0:v>1.665272507655815e+29</ns0:v>
       </ns0:c>
       <ns0:c r="G144" s="1" t="n">
         <ns0:v>29.0000000000001</ns0:v>
@@ -5645,7 +5645,7 @@
       </ns0:c>
       <ns0:c r="C145" s="1" t="inlineStr">
         <ns0:is>
-          <ns0:t>{71|0.1,76|0.2,90|0.3,32|0.4,165|0.5,180|0.6,174|0.7,162|0.8,36|0.9}</ns0:t>
+          <ns0:t>{31421|0.100000,31422|0.200000,31423|0.300000,31424|0.400000,31425|0.500000,31426|0.600000,31427|0.700000,31428|0.800000,31429|0.900000}</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="D145" s="1">
@@ -5658,7 +5658,7 @@
       </ns0:c>
       <ns0:c r="F145" s="1">
         <ns0:f>ROUND(F144*1.4,-5)</ns0:f>
-        <ns0:v>2.3313819353240506e+31</ns0:v>
+        <ns0:v>2.331381510718141e+29</ns0:v>
       </ns0:c>
       <ns0:c r="G145" s="1" t="n">
         <ns0:v>29.2000000000001</ns0:v>
@@ -5677,7 +5677,7 @@
       </ns0:c>
       <ns0:c r="C146" s="1" t="inlineStr">
         <ns0:is>
-          <ns0:t>{239|0.1,229|0.2,206|0.3,217|0.4,216|0.5,238|0.6,193|0.7,202|0.8,199|0.9}</ns0:t>
+          <ns0:t>{31431|0.100000,31432|0.200000,31433|0.300000,31434|0.400000,31435|0.500000,31436|0.600000,31437|0.700000,31438|0.800000,31439|0.900000}</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="D146" s="1">
@@ -5690,7 +5690,7 @@
       </ns0:c>
       <ns0:c r="F146" s="1">
         <ns0:f>ROUND(F145*1.4,-5)</ns0:f>
-        <ns0:v>3.263934709453671e+31</ns0:v>
+        <ns0:v>3.263934115005397e+29</ns0:v>
       </ns0:c>
       <ns0:c r="G146" s="1" t="n">
         <ns0:v>29.4000000000001</ns0:v>
@@ -5709,7 +5709,7 @@
       </ns0:c>
       <ns0:c r="C147" s="1" t="inlineStr">
         <ns0:is>
-          <ns0:t>{226|0.1,212|0.2,208|0.3,192|0.4,256|0.5,201|0.6,228|0.7,222|0.8,198|0.9}</ns0:t>
+          <ns0:t>{31441|0.100000,31442|0.200000,31443|0.300000,31444|0.400000,31445|0.500000,31446|0.600000,31447|0.700000,31448|0.800000,31449|0.900000}</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="D147" s="1">
@@ -5722,7 +5722,7 @@
       </ns0:c>
       <ns0:c r="F147" s="1">
         <ns0:f>ROUND(F146*1.4,-5)</ns0:f>
-        <ns0:v>4.569508593235139e+31</ns0:v>
+        <ns0:v>4.569507761007556e+29</ns0:v>
       </ns0:c>
       <ns0:c r="G147" s="1" t="n">
         <ns0:v>29.6000000000001</ns0:v>
@@ -5741,7 +5741,7 @@
       </ns0:c>
       <ns0:c r="C148" s="1" t="inlineStr">
         <ns0:is>
-          <ns0:t>{237|0.1,230|0.2,257|0.3,244|0.4,240|0.5,219|0.6,233|0.7,220|0.8,243|0.9}</ns0:t>
+          <ns0:t>{31451|0.100000,31452|0.200000,31453|0.300000,31454|0.400000,31455|0.500000,31456|0.600000,31457|0.700000,31458|0.800000,31459|0.900000}</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="D148" s="1">
@@ -5754,7 +5754,7 @@
       </ns0:c>
       <ns0:c r="F148" s="1">
         <ns0:f>ROUND(F147*1.4,-5)</ns0:f>
-        <ns0:v>6.397312030529194e+31</ns0:v>
+        <ns0:v>6.397310865410578e+29</ns0:v>
       </ns0:c>
       <ns0:c r="G148" s="1" t="n">
         <ns0:v>29.8000000000001</ns0:v>
@@ -5773,7 +5773,7 @@
       </ns0:c>
       <ns0:c r="C149" s="1" t="inlineStr">
         <ns0:is>
-          <ns0:t>{128|0.1,16|0.2,142|0.3,33|0.4,149|0.5,102|0.6,130|0.7,177|0.8,62|0.9}</ns0:t>
+          <ns0:t>{31461|0.100000,31462|0.200000,31463|0.300000,31464|0.400000,31465|0.500000,31466|0.600000,31467|0.700000,31468|0.800000,31469|0.900000}</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="D149" s="1">
@@ -5786,7 +5786,7 @@
       </ns0:c>
       <ns0:c r="F149" s="1">
         <ns0:f>ROUND(F148*1.4,-5)</ns0:f>
-        <ns0:v>8.95623684274087e+31</ns0:v>
+        <ns0:v>8.956235211574808e+29</ns0:v>
       </ns0:c>
       <ns0:c r="G149" s="1" t="n">
         <ns0:v>30.0000000000001</ns0:v>
@@ -5805,7 +5805,7 @@
       </ns0:c>
       <ns0:c r="C150" s="1" t="inlineStr">
         <ns0:is>
-          <ns0:t>{97|0.1,136|0.2,173|0.3,70|0.4,126|0.5,77|0.6,134|0.7,78|0.8,84|0.9}</ns0:t>
+          <ns0:t>{31471|0.100000,31472|0.200000,31473|0.300000,31474|0.400000,31475|0.500000,31476|0.600000,31477|0.700000,31478|0.800000,31479|0.900000}</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="D150" s="1">
@@ -5818,7 +5818,7 @@
       </ns0:c>
       <ns0:c r="F150" s="1">
         <ns0:f>ROUND(F149*1.4,-5)</ns0:f>
-        <ns0:v>1.253873157983722e+32</ns0:v>
+        <ns0:v>1.2538729296204731e+30</ns0:v>
       </ns0:c>
       <ns0:c r="G150" s="1" t="n">
         <ns0:v>30.2000000000001</ns0:v>
@@ -5837,7 +5837,7 @@
       </ns0:c>
       <ns0:c r="C151" s="1" t="inlineStr">
         <ns0:is>
-          <ns0:t>{214|0.1,223|0.2,241|0.3,234|0.4,195|0.5,215|0.6,203|0.7,197|0.8,200|0.9}</ns0:t>
+          <ns0:t>{31481|0.100000,31482|0.200000,31483|0.300000,31484|0.400000,31485|0.500000,31486|0.600000,31487|0.700000,31488|0.800000,31489|0.900000}</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="D151" s="1">
@@ -5850,7 +5850,7 @@
       </ns0:c>
       <ns0:c r="F151" s="1">
         <ns0:f>ROUND(F150*1.4,-5)</ns0:f>
-        <ns0:v>1.7554224211772108e+32</ns0:v>
+        <ns0:v>1.7554221014686622e+30</ns0:v>
       </ns0:c>
       <ns0:c r="G151" s="1" t="n">
         <ns0:v>30.4000000000001</ns0:v>
@@ -5869,7 +5869,7 @@
       </ns0:c>
       <ns0:c r="C152" s="1" t="inlineStr">
         <ns0:is>
-          <ns0:t>{227|0.1,225|0.2,190|0.3,212|0.4,218|0.5,245|0.6,209|0.7,194|0.8,213|0.9}</ns0:t>
+          <ns0:t>{31491|0.100000,31492|0.200000,31493|0.300000,31494|0.400000,31495|0.500000,31496|0.600000,31497|0.700000,31498|0.800000,31499|0.900000}</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="D152" s="1">
@@ -5882,7 +5882,7 @@
       </ns0:c>
       <ns0:c r="F152" s="1">
         <ns0:f>ROUND(F151*1.4,-5)</ns0:f>
-        <ns0:v>2.457591389648095e+32</ns0:v>
+        <ns0:v>2.4575909420561268e+30</ns0:v>
       </ns0:c>
       <ns0:c r="G152" s="1" t="n">
         <ns0:v>30.6000000000001</ns0:v>
@@ -5901,7 +5901,7 @@
       </ns0:c>
       <ns0:c r="C153" s="1" t="inlineStr">
         <ns0:is>
-          <ns0:t>{249|0.1,259|0.2,250|0.3,265|0.4,264|0.5,252|0.6,255|0.7,260|0.8,261|0.9}</ns0:t>
+          <ns0:t>{31501|0.100000,31502|0.200000,31503|0.300000,31504|0.400000,31505|0.500000,31506|0.600000,31507|0.700000,31508|0.800000,31509|0.900000}</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="D153" s="1">
@@ -5914,7 +5914,7 @@
       </ns0:c>
       <ns0:c r="F153" s="1">
         <ns0:f>ROUND(F152*1.4,-5)</ns0:f>
-        <ns0:v>3.440627945507332e+32</ns0:v>
+        <ns0:v>3.440627318878577e+30</ns0:v>
       </ns0:c>
       <ns0:c r="G153" s="1" t="n">
         <ns0:v>30.8000000000001</ns0:v>
@@ -5933,7 +5933,7 @@
       </ns0:c>
       <ns0:c r="C154" s="1" t="inlineStr">
         <ns0:is>
-          <ns0:t>{27|0.1,75|0.2,132|0.3,158|0.4,151|0.5,179|0.6,156|0.7,31|0.8,101|0.9}</ns0:t>
+          <ns0:t>{31511|0.100000,31512|0.200000,31513|0.300000,31514|0.400000,31515|0.500000,31516|0.600000,31517|0.700000,31518|0.800000,31519|0.900000}</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="D154" s="1">
@@ -5946,7 +5946,7 @@
       </ns0:c>
       <ns0:c r="F154" s="1">
         <ns0:f>ROUND(F153*1.4,-5)</ns0:f>
-        <ns0:v>4.816879123710265e+32</ns0:v>
+        <ns0:v>4.8168782464300075e+30</ns0:v>
       </ns0:c>
       <ns0:c r="G154" s="1" t="n">
         <ns0:v>31.0000000000001</ns0:v>
@@ -5965,7 +5965,7 @@
       </ns0:c>
       <ns0:c r="C155" s="1" t="inlineStr">
         <ns0:is>
-          <ns0:t>{163|0.1,83|0.2,56|0.3,168|0.4,72|0.5,116|0.6,147|0.7,188|0.8,150|0.9}</ns0:t>
+          <ns0:t>{31521|0.100000,31522|0.200000,31523|0.300000,31524|0.400000,31525|0.500000,31526|0.600000,31527|0.700000,31528|0.800000,31529|0.900000}</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="D155" s="1">
@@ -5978,7 +5978,7 @@
       </ns0:c>
       <ns0:c r="F155" s="1">
         <ns0:f>ROUND(F154*1.4,-5)</ns0:f>
-        <ns0:v>6.743630773194371e+32</ns0:v>
+        <ns0:v>6.74362954500201e+30</ns0:v>
       </ns0:c>
       <ns0:c r="G155" s="1" t="n">
         <ns0:v>31.2000000000001</ns0:v>
@@ -5997,7 +5997,7 @@
       </ns0:c>
       <ns0:c r="C156" s="1" t="inlineStr">
         <ns0:is>
-          <ns0:t>{221|0.1,242|0.2,217|0.3,238|0.4,204|0.5,207|0.6,216|0.7,224|0.8,196|0.9}</ns0:t>
+          <ns0:t>{31531|0.100000,31532|0.200000,31533|0.300000,31534|0.400000,31535|0.500000,31536|0.600000,31537|0.700000,31538|0.800000,31539|0.900000}</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="D156" s="1">
@@ -6010,7 +6010,7 @@
       </ns0:c>
       <ns0:c r="F156" s="1">
         <ns0:f>ROUND(F155*1.4,-5)</ns0:f>
-        <ns0:v>9.441083082472119e+32</ns0:v>
+        <ns0:v>9.441081363002813e+30</ns0:v>
       </ns0:c>
       <ns0:c r="G156" s="1" t="n">
         <ns0:v>31.4000000000001</ns0:v>
@@ -6029,7 +6029,7 @@
       </ns0:c>
       <ns0:c r="C157" s="1" t="inlineStr">
         <ns0:is>
-          <ns0:t>{231|0.1,262|0.2,205|0.3,210|0.4,211|0.5,190|0.6,191|0.7,228|0.8,225|0.9}</ns0:t>
+          <ns0:t>{31541|0.100000,31542|0.200000,31543|0.300000,31544|0.400000,31545|0.500000,31546|0.600000,31547|0.700000,31548|0.800000,31549|0.900000}</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="D157" s="1">
@@ -6042,7 +6042,7 @@
       </ns0:c>
       <ns0:c r="F157" s="1">
         <ns0:f>ROUND(F156*1.4,-5)</ns0:f>
-        <ns0:v>1.3217516315460965e+33</ns0:v>
+        <ns0:v>1.3217513908203938e+31</ns0:v>
       </ns0:c>
       <ns0:c r="G157" s="1" t="n">
         <ns0:v>31.6000000000001</ns0:v>
@@ -6061,7 +6061,7 @@
       </ns0:c>
       <ns0:c r="C158" s="1" t="inlineStr">
         <ns0:is>
-          <ns0:t>{236|0.1,254|0.2,237|0.3,258|0.4,246|0.5,232|0.6,219|0.7,244|0.8,240|0.9}</ns0:t>
+          <ns0:t>{31551|0.100000,31552|0.200000,31553|0.300000,31554|0.400000,31555|0.500000,31556|0.600000,31557|0.700000,31558|0.800000,31559|0.900000}</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="D158" s="1">
@@ -6074,7 +6074,7 @@
       </ns0:c>
       <ns0:c r="F158" s="1">
         <ns0:f>ROUND(F157*1.4,-5)</ns0:f>
-        <ns0:v>1.850452284164535e+33</ns0:v>
+        <ns0:v>1.8504519471485511e+31</ns0:v>
       </ns0:c>
       <ns0:c r="G158" s="1" t="n">
         <ns0:v>31.8000000000001</ns0:v>
@@ -6093,7 +6093,7 @@
       </ns0:c>
       <ns0:c r="C159" s="1" t="inlineStr">
         <ns0:is>
-          <ns0:t>{117|0.1,122|0.2,185|0.3,181|0.4,105|0.5,92|0.6,111|0.7,186|0.8,157|0.9}</ns0:t>
+          <ns0:t>{31561|0.100000,31562|0.200000,31563|0.300000,31564|0.400000,31565|0.500000,31566|0.600000,31567|0.700000,31568|0.800000,31569|0.900000}</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="D159" s="1">
@@ -6106,7 +6106,7 @@
       </ns0:c>
       <ns0:c r="F159" s="1">
         <ns0:f>ROUND(F158*1.4,-5)</ns0:f>
-        <ns0:v>2.590633197830349e+33</ns0:v>
+        <ns0:v>2.5906327260079714e+31</ns0:v>
       </ns0:c>
       <ns0:c r="G159" s="1" t="n">
         <ns0:v>32.0000000000001</ns0:v>
@@ -6125,7 +6125,7 @@
       </ns0:c>
       <ns0:c r="C160" s="1" t="inlineStr">
         <ns0:is>
-          <ns0:t>{141|0.1,24|0.2,166|0.3,187|0.4,45|0.5,123|0.6,80|0.7,89|0.8,35|0.9}</ns0:t>
+          <ns0:t>{31571|0.100000,31572|0.200000,31573|0.300000,31574|0.400000,31575|0.500000,31576|0.600000,31577|0.700000,31578|0.800000,31579|0.900000}</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="D160" s="1">
@@ -6138,7 +6138,7 @@
       </ns0:c>
       <ns0:c r="F160" s="1">
         <ns0:f>ROUND(F159*1.4,-5)</ns0:f>
-        <ns0:v>3.6268864769624885e+33</ns0:v>
+        <ns0:v>3.6268858164111598e+31</ns0:v>
       </ns0:c>
       <ns0:c r="G160" s="1" t="n">
         <ns0:v>32.2000000000001</ns0:v>
@@ -6157,7 +6157,7 @@
       </ns0:c>
       <ns0:c r="C161" s="1" t="inlineStr">
         <ns0:is>
-          <ns0:t>{239|0.1,229|0.2,206|0.3,197|0.4,193|0.5,199|0.6,202|0.7,195|0.8,201|0.9}</ns0:t>
+          <ns0:t>{31581|0.100000,31582|0.200000,31583|0.300000,31584|0.400000,31585|0.500000,31586|0.600000,31587|0.700000,31588|0.800000,31589|0.900000}</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="D161" s="1">
@@ -6170,7 +6170,7 @@
       </ns0:c>
       <ns0:c r="F161" s="1">
         <ns0:f>ROUND(F160*1.4,-5)</ns0:f>
-        <ns0:v>5.077641067747484e+33</ns0:v>
+        <ns0:v>5.0776401429756235e+31</ns0:v>
       </ns0:c>
       <ns0:c r="G161" s="1" t="n">
         <ns0:v>32.4000000000001</ns0:v>
@@ -6189,7 +6189,7 @@
       </ns0:c>
       <ns0:c r="C162" s="1" t="inlineStr">
         <ns0:is>
-          <ns0:t>{208|0.1,226|0.2,192|0.3,205|0.4,256|0.5,222|0.6,198|0.7,262|0.8,194|0.9}</ns0:t>
+          <ns0:t>{31591|0.100000,31592|0.200000,31593|0.300000,31594|0.400000,31595|0.500000,31596|0.600000,31597|0.700000,31598|0.800000,31599|0.900000}</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="D162" s="1">
@@ -6202,7 +6202,7 @@
       </ns0:c>
       <ns0:c r="F162" s="1">
         <ns0:f>ROUND(F161*1.4,-5)</ns0:f>
-        <ns0:v>7.108697494846477e+33</ns0:v>
+        <ns0:v>7.108696200165872e+31</ns0:v>
       </ns0:c>
       <ns0:c r="G162" s="1" t="n">
         <ns0:v>32.6000000000001</ns0:v>
@@ -6221,7 +6221,7 @@
       </ns0:c>
       <ns0:c r="C163" s="1" t="inlineStr">
         <ns0:is>
-          <ns0:t>{251|0.1,257|0.2,247|0.3,248|0.4,250|0.5,264|0.6,268|0.7,259|0.8,253|0.9}</ns0:t>
+          <ns0:t>{31601|0.100000,31602|0.200000,31603|0.300000,31604|0.400000,31605|0.500000,31606|0.600000,31607|0.700000,31608|0.800000,31609|0.900000}</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="D163" s="1">
@@ -6234,7 +6234,7 @@
       </ns0:c>
       <ns0:c r="F163" s="1">
         <ns0:f>ROUND(F162*1.4,-5)</ns0:f>
-        <ns0:v>9.952176492785067e+33</ns0:v>
+        <ns0:v>9.95217468023222e+31</ns0:v>
       </ns0:c>
       <ns0:c r="G163" s="1" t="n">
         <ns0:v>32.8000000000001</ns0:v>
@@ -6253,7 +6253,7 @@
       </ns0:c>
       <ns0:c r="C164" s="1" t="inlineStr">
         <ns0:is>
-          <ns0:t>{93|0.1,124|0.2,41|0.3,140|0.4,115|0.5,164|0.6,60|0.7,63|0.8,170|0.9}</ns0:t>
+          <ns0:t>{31611|0.100000,31612|0.200000,31613|0.300000,31614|0.400000,31615|0.500000,31616|0.600000,31617|0.700000,31618|0.800000,31619|0.900000}</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="D164" s="1">
@@ -6266,7 +6266,7 @@
       </ns0:c>
       <ns0:c r="F164" s="1">
         <ns0:f>ROUND(F163*1.4,-5)</ns0:f>
-        <ns0:v>1.3933047089899093e+34</ns0:v>
+        <ns0:v>1.3933044552325108e+32</ns0:v>
       </ns0:c>
       <ns0:c r="G164" s="1" t="n">
         <ns0:v>33.0000000000001</ns0:v>
@@ -6285,7 +6285,7 @@
       </ns0:c>
       <ns0:c r="C165" s="1" t="inlineStr">
         <ns0:is>
-          <ns0:t>{61|0.1,109|0.2,178|0.3,137|0.4,144|0.5,46|0.6,88|0.7,52|0.8,37|0.9}</ns0:t>
+          <ns0:t>{31621|0.100000,31622|0.200000,31623|0.300000,31624|0.400000,31625|0.500000,31626|0.600000,31627|0.700000,31628|0.800000,31629|0.900000}</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="D165" s="1">
@@ -6298,7 +6298,7 @@
       </ns0:c>
       <ns0:c r="F165" s="1">
         <ns0:f>ROUND(F164*1.4,-5)</ns0:f>
-        <ns0:v>1.950626592585873e+34</ns0:v>
+        <ns0:v>1.950626237325515e+32</ns0:v>
       </ns0:c>
       <ns0:c r="G165" s="1" t="n">
         <ns0:v>33.2000000000001</ns0:v>
@@ -6317,7 +6317,7 @@
       </ns0:c>
       <ns0:c r="C166" s="1" t="inlineStr">
         <ns0:is>
-          <ns0:t>{214|0.1,223|0.2,215|0.3,203|0.4,217|0.5,234|0.6,238|0.7,241|0.8,204|0.9}</ns0:t>
+          <ns0:t>{31631|0.100000,31632|0.200000,31633|0.300000,31634|0.400000,31635|0.500000,31636|0.600000,31637|0.700000,31638|0.800000,31639|0.900000}</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="D166" s="1">
@@ -6330,7 +6330,7 @@
       </ns0:c>
       <ns0:c r="F166" s="1">
         <ns0:f>ROUND(F165*1.4,-5)</ns0:f>
-        <ns0:v>2.730877229620222e+34</ns0:v>
+        <ns0:v>2.7308767322557203e+32</ns0:v>
       </ns0:c>
       <ns0:c r="G166" s="1" t="n">
         <ns0:v>33.4000000000001</ns0:v>
@@ -6349,7 +6349,7 @@
       </ns0:c>
       <ns0:c r="C167" s="1" t="inlineStr">
         <ns0:is>
-          <ns0:t>{227|0.1,245|0.2,218|0.3,191|0.4,209|0.5,210|0.6,213|0.7,211|0.8,207|0.9}</ns0:t>
+          <ns0:t>{31641|0.100000,31642|0.200000,31643|0.300000,31644|0.400000,31645|0.500000,31646|0.600000,31647|0.700000,31648|0.800000,31649|0.900000}</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="D167" s="1">
@@ -6362,7 +6362,7 @@
       </ns0:c>
       <ns0:c r="F167" s="1">
         <ns0:f>ROUND(F166*1.4,-5)</ns0:f>
-        <ns0:v>3.823228121468311e+34</ns0:v>
+        <ns0:v>3.823227425158008e+32</ns0:v>
       </ns0:c>
       <ns0:c r="G167" s="1" t="n">
         <ns0:v>33.6000000000001</ns0:v>
@@ -6381,7 +6381,7 @@
       </ns0:c>
       <ns0:c r="C168" s="1" t="inlineStr">
         <ns0:is>
-          <ns0:t>{232|0.1,236|0.2,246|0.3,233|0.4,258|0.5,235|0.6,243|0.7,230|0.8,220|0.9}</ns0:t>
+          <ns0:t>{31651|0.100000,31652|0.200000,31653|0.300000,31654|0.400000,31655|0.500000,31656|0.600000,31657|0.700000,31658|0.800000,31659|0.900000}</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="D168" s="1">
@@ -6394,7 +6394,7 @@
       </ns0:c>
       <ns0:c r="F168" s="1">
         <ns0:f>ROUND(F167*1.4,-5)</ns0:f>
-        <ns0:v>5.352519370055635e+34</ns0:v>
+        <ns0:v>5.352518395221211e+32</ns0:v>
       </ns0:c>
       <ns0:c r="G168" s="1" t="n">
         <ns0:v>33.8000000000001</ns0:v>
@@ -6413,7 +6413,7 @@
       </ns0:c>
       <ns0:c r="C169" s="1" t="inlineStr">
         <ns0:is>
-          <ns0:t>{43|0.1,42|0.2,139|0.3,51|0.4,54|0.5,141|0.6,106|0.7,96|0.8,17|0.9}</ns0:t>
+          <ns0:t>{31661|0.100000,31662|0.200000,31663|0.300000,31664|0.400000,31665|0.500000,31666|0.600000,31667|0.700000,31668|0.800000,31669|0.900000}</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="D169" s="1">
@@ -6426,7 +6426,7 @@
       </ns0:c>
       <ns0:c r="F169" s="1">
         <ns0:f>ROUND(F168*1.4,-5)</ns0:f>
-        <ns0:v>7.493527118077889e+34</ns0:v>
+        <ns0:v>7.493525753309694e+32</ns0:v>
       </ns0:c>
       <ns0:c r="G169" s="1" t="n">
         <ns0:v>34.0000000000001</ns0:v>
@@ -6445,7 +6445,7 @@
       </ns0:c>
       <ns0:c r="C170" s="1" t="inlineStr">
         <ns0:is>
-          <ns0:t>{27|0.1,32|0.2,146|0.3,148|0.4,57|0.5,28|0.6,121|0.7,91|0.8,120|0.9}</ns0:t>
+          <ns0:t>{31671|0.100000,31672|0.200000,31673|0.300000,31674|0.400000,31675|0.500000,31676|0.600000,31677|0.700000,31678|0.800000,31679|0.900000}</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="D170" s="1">
@@ -6458,7 +6458,7 @@
       </ns0:c>
       <ns0:c r="F170" s="1">
         <ns0:f>ROUND(F169*1.4,-5)</ns0:f>
-        <ns0:v>1.0490937965309043e+35</ns0:v>
+        <ns0:v>1.0490936054633572e+33</ns0:v>
       </ns0:c>
       <ns0:c r="G170" s="1" t="n">
         <ns0:v>34.2000000000001</ns0:v>
@@ -6477,7 +6477,7 @@
       </ns0:c>
       <ns0:c r="C171" s="1" t="inlineStr">
         <ns0:is>
-          <ns0:t>{221|0.1,242|0.2,224|0.3,216|0.4,200|0.5,196|0.6,193|0.7,202|0.8,201|0.9}</ns0:t>
+          <ns0:t>{31681|0.100000,31682|0.200000,31683|0.300000,31684|0.400000,31685|0.500000,31686|0.600000,31687|0.700000,31688|0.800000,31689|0.900000}</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="D171" s="1">
@@ -6490,7 +6490,7 @@
       </ns0:c>
       <ns0:c r="F171" s="1">
         <ns0:f>ROUND(F170*1.4,-5)</ns0:f>
-        <ns0:v>1.468731315143266e+35</ns0:v>
+        <ns0:v>1.4687310476486998e+33</ns0:v>
       </ns0:c>
       <ns0:c r="G171" s="1" t="n">
         <ns0:v>34.4000000000001</ns0:v>
@@ -6509,7 +6509,7 @@
       </ns0:c>
       <ns0:c r="C172" s="1" t="inlineStr">
         <ns0:is>
-          <ns0:t>{231|0.1,190|0.2,228|0.3,212|0.4,256|0.5,222|0.6,225|0.7,198|0.8,209|0.9}</ns0:t>
+          <ns0:t>{31691|0.100000,31692|0.200000,31693|0.300000,31694|0.400000,31695|0.500000,31696|0.600000,31697|0.700000,31698|0.800000,31699|0.900000}</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="D172" s="1">
@@ -6522,7 +6522,7 @@
       </ns0:c>
       <ns0:c r="F172" s="1">
         <ns0:f>ROUND(F171*1.4,-5)</ns0:f>
-        <ns0:v>2.056223841200572e+35</ns0:v>
+        <ns0:v>2.0562234667081797e+33</ns0:v>
       </ns0:c>
       <ns0:c r="G172" s="1" t="n">
         <ns0:v>34.6000000000001</ns0:v>
@@ -6541,7 +6541,7 @@
       </ns0:c>
       <ns0:c r="C173" s="1" t="inlineStr">
         <ns0:is>
-          <ns0:t>{265|0.1,249|0.2,260|0.3,252|0.4,255|0.5,259|0.6,264|0.7,261|0.8,251|0.9}</ns0:t>
+          <ns0:t>{31701|0.100000,31702|0.200000,31703|0.300000,31704|0.400000,31705|0.500000,31706|0.600000,31707|0.700000,31708|0.800000,31709|0.900000}</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="D173" s="1">
@@ -6554,7 +6554,7 @@
       </ns0:c>
       <ns0:c r="F173" s="1">
         <ns0:f>ROUND(F172*1.4,-5)</ns0:f>
-        <ns0:v>2.8787133776808006e+35</ns0:v>
+        <ns0:v>2.878712853391451e+33</ns0:v>
       </ns0:c>
       <ns0:c r="G173" s="1" t="n">
         <ns0:v>34.8000000000001</ns0:v>
@@ -6573,7 +6573,7 @@
       </ns0:c>
       <ns0:c r="C174" s="1" t="inlineStr">
         <ns0:is>
-          <ns0:t>{154|0.1,103|0.2,108|0.3,67|0.4,38|0.5,39|0.6,107|0.7,127|0.8,125|0.9}</ns0:t>
+          <ns0:t>{31711|0.100000,31712|0.200000,31713|0.300000,31714|0.400000,31715|0.500000,31716|0.600000,31717|0.700000,31718|0.800000,31719|0.900000}</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="D174" s="1">
@@ -6586,7 +6586,7 @@
       </ns0:c>
       <ns0:c r="F174" s="1">
         <ns0:f>ROUND(F173*1.4,-5)</ns0:f>
-        <ns0:v>4.03019872875312e+35</ns0:v>
+        <ns0:v>4.0301979947480315e+33</ns0:v>
       </ns0:c>
       <ns0:c r="G174" s="1" t="n">
         <ns0:v>35.0000000000001</ns0:v>
@@ -6605,7 +6605,7 @@
       </ns0:c>
       <ns0:c r="C175" s="1" t="inlineStr">
         <ns0:is>
-          <ns0:t>{114|0.1,155|0.2,98|0.3,30|0.4,49|0.5,33|0.6,21|0.7,129|0.8,112|0.9}</ns0:t>
+          <ns0:t>{31721|0.100000,31722|0.200000,31723|0.300000,31724|0.400000,31725|0.500000,31726|0.600000,31727|0.700000,31728|0.800000,31729|0.900000}</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="D175" s="1">
@@ -6618,7 +6618,7 @@
       </ns0:c>
       <ns0:c r="F175" s="1">
         <ns0:f>ROUND(F174*1.4,-5)</ns0:f>
-        <ns0:v>5.642278220254368e+35</ns0:v>
+        <ns0:v>5.642277192647244e+33</ns0:v>
       </ns0:c>
       <ns0:c r="G175" s="1" t="n">
         <ns0:v>35.2000000000001</ns0:v>
@@ -6637,7 +6637,7 @@
       </ns0:c>
       <ns0:c r="C176" s="1" t="inlineStr">
         <ns0:is>
-          <ns0:t>{244|0.1,206|0.2,229|0.3,224|0.4,215|0.5,199|0.6,234|0.7,195|0.8,203|0.9}</ns0:t>
+          <ns0:t>{31731|0.100000,31732|0.200000,31733|0.300000,31734|0.400000,31735|0.500000,31736|0.600000,31737|0.700000,31738|0.800000,31739|0.900000}</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="D176" s="1">
@@ -6650,7 +6650,7 @@
       </ns0:c>
       <ns0:c r="F176" s="1">
         <ns0:f>ROUND(F175*1.4,-5)</ns0:f>
-        <ns0:v>7.899189508356115e+35</ns0:v>
+        <ns0:v>7.899188069706141e+33</ns0:v>
       </ns0:c>
       <ns0:c r="G176" s="1" t="n">
         <ns0:v>35.4000000000001</ns0:v>
@@ -6669,7 +6669,7 @@
       </ns0:c>
       <ns0:c r="C177" s="1" t="inlineStr">
         <ns0:is>
-          <ns0:t>{227|0.1,192|0.2,191|0.3,211|0.4,205|0.5,262|0.6,208|0.7,226|0.8,194|0.9}</ns0:t>
+          <ns0:t>{31741|0.100000,31742|0.200000,31743|0.300000,31744|0.400000,31745|0.500000,31746|0.600000,31747|0.700000,31748|0.800000,31749|0.900000}</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="D177" s="1">
@@ -6682,7 +6682,7 @@
       </ns0:c>
       <ns0:c r="F177" s="1">
         <ns0:f>ROUND(F176*1.4,-5)</ns0:f>
-        <ns0:v>1.105886531169856e+36</ns0:v>
+        <ns0:v>1.1058863297588596e+34</ns0:v>
       </ns0:c>
       <ns0:c r="G177" s="1" t="n">
         <ns0:v>35.6000000000001</ns0:v>
@@ -6701,7 +6701,7 @@
       </ns0:c>
       <ns0:c r="C178" s="1" t="inlineStr">
         <ns0:is>
-          <ns0:t>{254|0.1,235|0.2,230|0.3,257|0.4,219|0.5,240|0.6,220|0.7,243|0.8,239|0.9}</ns0:t>
+          <ns0:t>{31751|0.100000,31752|0.200000,31753|0.300000,31754|0.400000,31755|0.500000,31756|0.600000,31757|0.700000,31758|0.800000,31759|0.900000}</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="D178" s="1">
@@ -6714,7 +6714,7 @@
       </ns0:c>
       <ns0:c r="F178" s="1">
         <ns0:f>ROUND(F177*1.4,-5)</ns0:f>
-        <ns0:v>1.5482411436377982e+36</ns0:v>
+        <ns0:v>1.5482408616624033e+34</ns0:v>
       </ns0:c>
       <ns0:c r="G178" s="1" t="n">
         <ns0:v>35.8000000000001</ns0:v>
@@ -6733,7 +6733,7 @@
       </ns0:c>
       <ns0:c r="C179" s="1" t="inlineStr">
         <ns0:is>
-          <ns0:t>{149|0.1,73|0.2,165|0.3,145|0.4,71|0.5,50|0.6,169|0.7,79|0.8,183|0.9}</ns0:t>
+          <ns0:t>{31761|0.100000,31762|0.200000,31763|0.300000,31764|0.400000,31765|0.500000,31766|0.600000,31767|0.700000,31768|0.800000,31769|0.900000}</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="D179" s="1">
@@ -6746,7 +6746,7 @@
       </ns0:c>
       <ns0:c r="F179" s="1">
         <ns0:f>ROUND(F178*1.4,-5)</ns0:f>
-        <ns0:v>2.1675376010929173e+36</ns0:v>
+        <ns0:v>2.1675372063273644e+34</ns0:v>
       </ns0:c>
       <ns0:c r="G179" s="1" t="n">
         <ns0:v>36.0000000000001</ns0:v>
@@ -6765,7 +6765,7 @@
       </ns0:c>
       <ns0:c r="C180" s="1" t="inlineStr">
         <ns0:is>
-          <ns0:t>{119|0.1,66|0.2,34|0.3,87|0.4,77|0.5,172|0.6,167|0.7,64|0.8,134|0.9}</ns0:t>
+          <ns0:t>{31771|0.100000,31772|0.200000,31773|0.300000,31774|0.400000,31775|0.500000,31776|0.600000,31777|0.700000,31778|0.800000,31779|0.900000}</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="D180" s="1">
@@ -6778,7 +6778,7 @@
       </ns0:c>
       <ns0:c r="F180" s="1">
         <ns0:f>ROUND(F179*1.4,-5)</ns0:f>
-        <ns0:v>3.034552641530084e+36</ns0:v>
+        <ns0:v>3.03455208885831e+34</ns0:v>
       </ns0:c>
       <ns0:c r="G180" s="1" t="n">
         <ns0:v>36.2000000000001</ns0:v>
@@ -6797,7 +6797,7 @@
       </ns0:c>
       <ns0:c r="C181" s="1" t="inlineStr">
         <ns0:is>
-          <ns0:t>{214|0.1,223|0.2,241|0.3,204|0.4,197|0.5,216|0.6,200|0.7,217|0.8,207|0.9}</ns0:t>
+          <ns0:t>{31781|0.100000,31782|0.200000,31783|0.300000,31784|0.400000,31785|0.500000,31786|0.600000,31787|0.700000,31788|0.800000,31789|0.900000}</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="D181" s="1">
@@ -6810,7 +6810,7 @@
       </ns0:c>
       <ns0:c r="F181" s="1">
         <ns0:f>ROUND(F180*1.4,-5)</ns0:f>
-        <ns0:v>4.2483736981421174e+36</ns0:v>
+        <ns0:v>4.248372924401634e+34</ns0:v>
       </ns0:c>
       <ns0:c r="G181" s="1" t="n">
         <ns0:v>36.4000000000001</ns0:v>
@@ -6829,7 +6829,7 @@
       </ns0:c>
       <ns0:c r="C182" s="1" t="inlineStr">
         <ns0:is>
-          <ns0:t>{218|0.1,210|0.2,212|0.3,245|0.4,213|0.5,190|0.6,228|0.7,225|0.8,222|0.9}</ns0:t>
+          <ns0:t>{31791|0.100000,31792|0.200000,31793|0.300000,31794|0.400000,31795|0.500000,31796|0.600000,31797|0.700000,31798|0.800000,31799|0.900000}</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="D182" s="1">
@@ -6842,7 +6842,7 @@
       </ns0:c>
       <ns0:c r="F182" s="1">
         <ns0:f>ROUND(F181*1.4,-5)</ns0:f>
-        <ns0:v>5.947723177398964e+36</ns0:v>
+        <ns0:v>5.9477220941622865e+34</ns0:v>
       </ns0:c>
       <ns0:c r="G182" s="1" t="n">
         <ns0:v>36.6000000000001</ns0:v>
@@ -6861,7 +6861,7 @@
       </ns0:c>
       <ns0:c r="C183" s="1" t="inlineStr">
         <ns0:is>
-          <ns0:t>{249|0.1,250|0.2,265|0.3,253|0.4,268|0.5,247|0.6,252|0.7,260|0.8,261|0.9}</ns0:t>
+          <ns0:t>{31801|0.100000,31802|0.200000,31803|0.300000,31804|0.400000,31805|0.500000,31806|0.600000,31807|0.700000,31808|0.800000,31809|0.900000}</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="D183" s="1">
@@ -6874,7 +6874,7 @@
       </ns0:c>
       <ns0:c r="F183" s="1">
         <ns0:f>ROUND(F182*1.4,-5)</ns0:f>
-        <ns0:v>8.326812448358549e+36</ns0:v>
+        <ns0:v>8.3268109318272e+34</ns0:v>
       </ns0:c>
       <ns0:c r="G183" s="1" t="n">
         <ns0:v>36.8000000000001</ns0:v>
@@ -6893,7 +6893,7 @@
       </ns0:c>
       <ns0:c r="C184" s="1" t="inlineStr">
         <ns0:is>
-          <ns0:t>{59|0.1,23|0.2,16|0.3,65|0.4,40|0.5,29|0.6,20|0.7,152|0.8,113|0.9}</ns0:t>
+          <ns0:t>{31811|0.100000,31812|0.200000,31813|0.300000,31814|0.400000,31815|0.500000,31816|0.600000,31817|0.700000,31818|0.800000,31819|0.900000}</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="D184" s="1">
@@ -6906,7 +6906,7 @@
       </ns0:c>
       <ns0:c r="F184" s="1">
         <ns0:f>ROUND(F183*1.4,-5)</ns0:f>
-        <ns0:v>1.1657537427701967e+37</ns0:v>
+        <ns0:v>1.165753530455808e+35</ns0:v>
       </ns0:c>
       <ns0:c r="G184" s="1" t="n">
         <ns0:v>37.0000000000001</ns0:v>
@@ -6925,7 +6925,7 @@
       </ns0:c>
       <ns0:c r="C185" s="1" t="inlineStr">
         <ns0:is>
-          <ns0:t>{85|0.1,133|0.2,176|0.3,184|0.4,94|0.5,175|0.6,135|0.7,82|0.8,45|0.9}</ns0:t>
+          <ns0:t>{31821|0.100000,31822|0.200000,31823|0.300000,31824|0.400000,31825|0.500000,31826|0.600000,31827|0.700000,31828|0.800000,31829|0.900000}</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="D185" s="1">
@@ -6938,7 +6938,7 @@
       </ns0:c>
       <ns0:c r="F185" s="1">
         <ns0:f>ROUND(F184*1.4,-5)</ns0:f>
-        <ns0:v>1.6320552398782752e+37</ns0:v>
+        <ns0:v>1.6320549426381312e+35</ns0:v>
       </ns0:c>
       <ns0:c r="G185" s="1" t="n">
         <ns0:v>37.2000000000001</ns0:v>
@@ -6957,7 +6957,7 @@
       </ns0:c>
       <ns0:c r="C186" s="1" t="inlineStr">
         <ns0:is>
-          <ns0:t>{239|0.1,229|0.2,206|0.3,238|0.4,196|0.5,215|0.6,241|0.7,201|0.8,202|0.9}</ns0:t>
+          <ns0:t>{31831|0.100000,31832|0.200000,31833|0.300000,31834|0.400000,31835|0.500000,31836|0.600000,31837|0.700000,31838|0.800000,31839|0.900000}</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="D186" s="1">
@@ -6970,7 +6970,7 @@
       </ns0:c>
       <ns0:c r="F186" s="1">
         <ns0:f>ROUND(F185*1.4,-5)</ns0:f>
-        <ns0:v>2.284877335829585e+37</ns0:v>
+        <ns0:v>2.2848769196933836e+35</ns0:v>
       </ns0:c>
       <ns0:c r="G186" s="1" t="n">
         <ns0:v>37.4000000000001</ns0:v>
@@ -6989,7 +6989,7 @@
       </ns0:c>
       <ns0:c r="C187" s="1" t="inlineStr">
         <ns0:is>
-          <ns0:t>{231|0.1,256|0.2,191|0.3,209|0.4,192|0.5,198|0.6,194|0.7,262|0.8,211|0.9}</ns0:t>
+          <ns0:t>{31841|0.100000,31842|0.200000,31843|0.300000,31844|0.400000,31845|0.500000,31846|0.600000,31847|0.700000,31848|0.800000,31849|0.900000}</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="D187" s="1">
@@ -7002,7 +7002,7 @@
       </ns0:c>
       <ns0:c r="F187" s="1">
         <ns0:f>ROUND(F186*1.4,-5)</ns0:f>
-        <ns0:v>3.198828270161419e+37</ns0:v>
+        <ns0:v>3.1988276875707367e+35</ns0:v>
       </ns0:c>
       <ns0:c r="G187" s="1" t="n">
         <ns0:v>37.6000000000001</ns0:v>
@@ -7021,7 +7021,7 @@
       </ns0:c>
       <ns0:c r="C188" s="1" t="inlineStr">
         <ns0:is>
-          <ns0:t>{236|0.1,258|0.2,246|0.3,232|0.4,254|0.5,248|0.6,237|0.7,233|0.8,219|0.9}</ns0:t>
+          <ns0:t>{31851|0.100000,31852|0.200000,31853|0.300000,31854|0.400000,31855|0.500000,31856|0.600000,31857|0.700000,31858|0.800000,31859|0.900000}</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="D188" s="1">
@@ -7034,7 +7034,7 @@
       </ns0:c>
       <ns0:c r="F188" s="1">
         <ns0:f>ROUND(F187*1.4,-5)</ns0:f>
-        <ns0:v>4.478359578225986e+37</ns0:v>
+        <ns0:v>4.478358762599031e+35</ns0:v>
       </ns0:c>
       <ns0:c r="G188" s="1" t="n">
         <ns0:v>37.8000000000001</ns0:v>
@@ -7053,7 +7053,7 @@
       </ns0:c>
       <ns0:c r="C189" s="1" t="inlineStr">
         <ns0:is>
-          <ns0:t>{163|0.1,24|0.2,74|0.3,104|0.4,151|0.5,70|0.6,36|0.7,110|0.8,22|0.9}</ns0:t>
+          <ns0:t>{31861|0.100000,31862|0.200000,31863|0.300000,31864|0.400000,31865|0.500000,31866|0.600000,31867|0.700000,31868|0.800000,31869|0.900000}</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="D189" s="1">
@@ -7066,7 +7066,7 @@
       </ns0:c>
       <ns0:c r="F189" s="1">
         <ns0:f>ROUND(F188*1.4,-5)</ns0:f>
-        <ns0:v>6.26970340951638e+37</ns0:v>
+        <ns0:v>6.269702267638643e+35</ns0:v>
       </ns0:c>
       <ns0:c r="G189" s="1" t="n">
         <ns0:v>38.0000000000001</ns0:v>
@@ -7085,7 +7085,7 @@
       </ns0:c>
       <ns0:c r="C190" s="1" t="inlineStr">
         <ns0:is>
-          <ns0:t>{171|0.1,81|0.2,56|0.3,131|0.4,182|0.5,18|0.6,158|0.7,86|0.8,189|0.9}</ns0:t>
+          <ns0:t>{31871|0.100000,31872|0.200000,31873|0.300000,31874|0.400000,31875|0.500000,31876|0.600000,31877|0.700000,31878|0.800000,31879|0.900000}</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="D190" s="1">
@@ -7098,7 +7098,7 @@
       </ns0:c>
       <ns0:c r="F190" s="1">
         <ns0:f>ROUND(F189*1.4,-5)</ns0:f>
-        <ns0:v>8.777584773322933e+37</ns0:v>
+        <ns0:v>8.7775831746941e+35</ns0:v>
       </ns0:c>
       <ns0:c r="G190" s="1" t="n">
         <ns0:v>38.2000000000001</ns0:v>
@@ -7117,7 +7117,7 @@
       </ns0:c>
       <ns0:c r="C191" s="1" t="inlineStr">
         <ns0:is>
-          <ns0:t>{221|0.1,242|0.2,193|0.3,217|0.4,199|0.5,203|0.6,195|0.7,234|0.8,197|0.9}</ns0:t>
+          <ns0:t>{31881|0.100000,31882|0.200000,31883|0.300000,31884|0.400000,31885|0.500000,31886|0.600000,31887|0.700000,31888|0.800000,31889|0.900000}</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="D191" s="1">
@@ -7130,7 +7130,7 @@
       </ns0:c>
       <ns0:c r="F191" s="1">
         <ns0:f>ROUND(F190*1.4,-5)</ns0:f>
-        <ns0:v>1.2288618682652105e+38</ns0:v>
+        <ns0:v>1.228861644457174e+36</ns0:v>
       </ns0:c>
       <ns0:c r="G191" s="1" t="n">
         <ns0:v>38.4000000000001</ns0:v>
@@ -7149,7 +7149,7 @@
       </ns0:c>
       <ns0:c r="C192" s="1" t="inlineStr">
         <ns0:is>
-          <ns0:t>{205|0.1,227|0.2,207|0.3,208|0.4,226|0.5,210|0.6,213|0.7,196|0.8,190|0.9}</ns0:t>
+          <ns0:t>{31891|0.100000,31892|0.200000,31893|0.300000,31894|0.400000,31895|0.500000,31896|0.600000,31897|0.700000,31898|0.800000,31899|0.900000}</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="D192" s="1">
@@ -7162,7 +7162,7 @@
       </ns0:c>
       <ns0:c r="F192" s="1">
         <ns0:f>ROUND(F191*1.4,-5)</ns0:f>
-        <ns0:v>1.7204066155712946e+38</ns0:v>
+        <ns0:v>1.7204063022400436e+36</ns0:v>
       </ns0:c>
       <ns0:c r="G192" s="1" t="n">
         <ns0:v>38.6000000000001</ns0:v>
@@ -7181,7 +7181,7 @@
       </ns0:c>
       <ns0:c r="C193" s="1" t="inlineStr">
         <ns0:is>
-          <ns0:t>{255|0.1,265|0.2,268|0.3,249|0.4,251|0.5,264|0.6,257|0.7,253|0.8,259|0.9}</ns0:t>
+          <ns0:t>{31901|0.100000,31902|0.200000,31903|0.300000,31904|0.400000,31905|0.500000,31906|0.600000,31907|0.700000,31908|0.800000,31909|0.900000}</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="D193" s="1">
@@ -7194,7 +7194,7 @@
       </ns0:c>
       <ns0:c r="F193" s="1">
         <ns0:f>ROUND(F192*1.4,-5)</ns0:f>
-        <ns0:v>2.4085692617998124e+38</ns0:v>
+        <ns0:v>2.4085688231360608e+36</ns0:v>
       </ns0:c>
       <ns0:c r="G193" s="1" t="n">
         <ns0:v>38.8000000000001</ns0:v>
@@ -7213,7 +7213,7 @@
       </ns0:c>
       <ns0:c r="C194" s="1" t="inlineStr">
         <ns0:is>
-          <ns0:t>{42|0.1,62|0.2,58|0.3,55|0.4,159|0.5,48|0.6,126|0.7,118|0.8,179|0.9}</ns0:t>
+          <ns0:t>{31911|0.100000,31912|0.200000,31913|0.300000,31914|0.400000,31915|0.500000,31916|0.600000,31917|0.700000,31918|0.800000,31919|0.900000}</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="D194" s="1">
@@ -7226,7 +7226,7 @@
       </ns0:c>
       <ns0:c r="F194" s="1">
         <ns0:f>ROUND(F193*1.4,-5)</ns0:f>
-        <ns0:v>3.371996966519737e+38</ns0:v>
+        <ns0:v>3.371996352390485e+36</ns0:v>
       </ns0:c>
       <ns0:c r="G194" s="1" t="n">
         <ns0:v>39.0000000000001</ns0:v>
@@ -7245,7 +7245,7 @@
       </ns0:c>
       <ns0:c r="C195" s="1" t="inlineStr">
         <ns0:is>
-          <ns0:t>{153|0.1,185|0.2,162|0.3,44|0.4,75|0.5,102|0.6,76|0.7,128|0.8,177|0.9}</ns0:t>
+          <ns0:t>{31921|0.100000,31922|0.200000,31923|0.300000,31924|0.400000,31925|0.500000,31926|0.600000,31927|0.700000,31928|0.800000,31929|0.900000}</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="D195" s="1">
@@ -7258,7 +7258,7 @@
       </ns0:c>
       <ns0:c r="F195" s="1">
         <ns0:f>ROUND(F194*1.4,-5)</ns0:f>
-        <ns0:v>4.720795753127631e+38</ns0:v>
+        <ns0:v>4.720794893346679e+36</ns0:v>
       </ns0:c>
       <ns0:c r="G195" s="1" t="n">
         <ns0:v>39.2000000000001</ns0:v>
@@ -7277,7 +7277,7 @@
       </ns0:c>
       <ns0:c r="C196" s="1" t="inlineStr">
         <ns0:is>
-          <ns0:t>{214|0.1,223|0.2,224|0.3,204|0.4,238|0.5,216|0.6,200|0.7,193|0.8,202|0.9}</ns0:t>
+          <ns0:t>{31931|0.100000,31932|0.200000,31933|0.300000,31934|0.400000,31935|0.500000,31936|0.600000,31937|0.700000,31938|0.800000,31939|0.900000}</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="D196" s="1">
@@ -7290,7 +7290,7 @@
       </ns0:c>
       <ns0:c r="F196" s="1">
         <ns0:f>ROUND(F195*1.4,-5)</ns0:f>
-        <ns0:v>6.6091140543786836e+38</ns0:v>
+        <ns0:v>6.60911285068535e+36</ns0:v>
       </ns0:c>
       <ns0:c r="G196" s="1" t="n">
         <ns0:v>39.4000000000001</ns0:v>
@@ -7309,7 +7309,7 @@
       </ns0:c>
       <ns0:c r="C197" s="1" t="inlineStr">
         <ns0:is>
-          <ns0:t>{218|0.1,212|0.2,192|0.3,245|0.4,256|0.5,228|0.6,225|0.7,222|0.8,201|0.9}</ns0:t>
+          <ns0:t>{31941|0.100000,31942|0.200000,31943|0.300000,31944|0.400000,31945|0.500000,31946|0.600000,31947|0.700000,31948|0.800000,31949|0.900000}</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="D197" s="1">
@@ -7322,7 +7322,7 @@
       </ns0:c>
       <ns0:c r="F197" s="1">
         <ns0:f>ROUND(F196*1.4,-5)</ns0:f>
-        <ns0:v>9.252759676130156e+38</ns0:v>
+        <ns0:v>9.252757990959492e+36</ns0:v>
       </ns0:c>
       <ns0:c r="G197" s="1" t="n">
         <ns0:v>39.6000000000001</ns0:v>
@@ -7341,7 +7341,7 @@
       </ns0:c>
       <ns0:c r="C198" s="1" t="inlineStr">
         <ns0:is>
-          <ns0:t>{235|0.1,232|0.2,230|0.3,246|0.4,233|0.5,244|0.6,240|0.7,243|0.8,220|0.9}</ns0:t>
+          <ns0:t>{31951|0.100000,31952|0.200000,31953|0.300000,31954|0.400000,31955|0.500000,31956|0.600000,31957|0.700000,31958|0.800000,31959|0.900000}</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="D198" s="1">
@@ -7354,7 +7354,7 @@
       </ns0:c>
       <ns0:c r="F198" s="1">
         <ns0:f>ROUND(F197*1.4,-5)</ns0:f>
-        <ns0:v>1.2953863546582217e+39</ns0:v>
+        <ns0:v>1.2953861187343288e+37</ns0:v>
       </ns0:c>
       <ns0:c r="G198" s="1" t="n">
         <ns0:v>39.8000000000001</ns0:v>
@@ -7373,7 +7373,7 @@
       </ns0:c>
       <ns0:c r="C199" s="1" t="inlineStr">
         <ns0:is>
-          <ns0:t>{132|0.1,63|0.2,95|0.3,161|0.4,168|0.5,47|0.6,130|0.7,84|0.8,188|0.9}</ns0:t>
+          <ns0:t>{31961|0.100000,31962|0.200000,31963|0.300000,31964|0.400000,31965|0.500000,31966|0.600000,31967|0.700000,31968|0.800000,31969|0.900000}</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="D199" s="1">
@@ -7386,7 +7386,7 @@
       </ns0:c>
       <ns0:c r="F199" s="1">
         <ns0:f>ROUND(F198*1.4,-5)</ns0:f>
-        <ns0:v>1.8135408965215102e+39</ns0:v>
+        <ns0:v>1.8135405662280603e+37</ns0:v>
       </ns0:c>
       <ns0:c r="G199" s="1" t="n">
         <ns0:v>40.0000000000001</ns0:v>
@@ -7405,7 +7405,7 @@
       </ns0:c>
       <ns0:c r="C200" s="1" t="inlineStr">
         <ns0:is>
-          <ns0:t>{116|0.1,26|0.2,69|0.3,90|0.4,92|0.5,180|0.6,173|0.7,25|0.8,142|0.9}</ns0:t>
+          <ns0:t>{31971|0.100000,31972|0.200000,31973|0.300000,31974|0.400000,31975|0.500000,31976|0.600000,31977|0.700000,31978|0.800000,31979|0.900000}</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="D200" s="1">
@@ -7418,7 +7418,7 @@
       </ns0:c>
       <ns0:c r="F200" s="1">
         <ns0:f>ROUND(F199*1.4,-5)</ns0:f>
-        <ns0:v>2.538957255130114e+39</ns0:v>
+        <ns0:v>2.5389567927192844e+37</ns0:v>
       </ns0:c>
       <ns0:c r="G200" s="1" t="n">
         <ns0:v>40.2000000000001</ns0:v>
@@ -7437,7 +7437,7 @@
       </ns0:c>
       <ns0:c r="C201" s="1" t="inlineStr">
         <ns0:is>
-          <ns0:t>{221|0.1,242|0.2,198|0.3,215|0.4,241|0.5,234|0.6,195|0.7,199|0.8,203|0.9}</ns0:t>
+          <ns0:t>{31981|0.100000,31982|0.200000,31983|0.300000,31984|0.400000,31985|0.500000,31986|0.600000,31987|0.700000,31988|0.800000,31989|0.900000}</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="D201" s="1">
@@ -7450,7 +7450,7 @@
       </ns0:c>
       <ns0:c r="F201" s="1">
         <ns0:f>ROUND(F200*1.4,-5)</ns0:f>
-        <ns0:v>3.5545401571821595e+39</ns0:v>
+        <ns0:v>3.554539509806998e+37</ns0:v>
       </ns0:c>
       <ns0:c r="G201" s="1" t="n">
         <ns0:v>40.4000000000001</ns0:v>
@@ -7469,7 +7469,7 @@
       </ns0:c>
       <ns0:c r="C202" s="1" t="inlineStr">
         <ns0:is>
-          <ns0:t>{227|0.1,205|0.2,211|0.3,191|0.4,262|0.5,194|0.6,231|0.7,213|0.8,209|0.9}</ns0:t>
+          <ns0:t>{31991|0.100000,31992|0.200000,31993|0.300000,31994|0.400000,31995|0.500000,31996|0.600000,31997|0.700000,31998|0.800000,31999|0.900000}</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="D202" s="1">
@@ -7482,7 +7482,7 @@
       </ns0:c>
       <ns0:c r="F202" s="1">
         <ns0:f>ROUND(F201*1.4,-5)</ns0:f>
-        <ns0:v>4.976356220055024e+39</ns0:v>
+        <ns0:v>4.976355313729797e+37</ns0:v>
       </ns0:c>
       <ns0:c r="G202" s="1" t="n">
         <ns0:v>40.6000000000001</ns0:v>
@@ -7501,7 +7501,7 @@
       </ns0:c>
       <ns0:c r="C203" s="1" t="inlineStr">
         <ns0:is>
-          <ns0:t>{248|0.1,247|0.2,250|0.3,260|0.4,252|0.5,261|0.6,255|0.7,251|0.8,259|0.9}</ns0:t>
+          <ns0:t>{32001|0.100000,32002|0.200000,32003|0.300000,32004|0.400000,32005|0.500000,32006|0.600000,32007|0.700000,32008|0.800000,32009|0.900000}</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="D203" s="1">
@@ -7514,7 +7514,7 @@
       </ns0:c>
       <ns0:c r="F203" s="1">
         <ns0:f>ROUND(F202*1.4,-5)</ns0:f>
-        <ns0:v>6.966898708077033e+39</ns0:v>
+        <ns0:v>6.966897439221714e+37</ns0:v>
       </ns0:c>
       <ns0:c r="G203" s="1" t="n">
         <ns0:v>40.8000000000001</ns0:v>
@@ -7533,7 +7533,7 @@
       </ns0:c>
       <ns0:c r="C204" s="1" t="inlineStr">
         <ns0:is>
-          <ns0:t>{31|0.1,166|0.2,138|0.3,178|0.4,101|0.5,80|0.6,160|0.7,78|0.8,53|0.9}</ns0:t>
+          <ns0:t>{32011|0.100000,32012|0.200000,32013|0.300000,32014|0.400000,32015|0.500000,32016|0.600000,32017|0.700000,32018|0.800000,32019|0.900000}</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="D204" s="1">
@@ -7546,7 +7546,7 @@
       </ns0:c>
       <ns0:c r="F204" s="1">
         <ns0:f>ROUND(F203*1.4,-5)</ns0:f>
-        <ns0:v>9.753658191307845e+39</ns0:v>
+        <ns0:v>9.753656414910399e+37</ns0:v>
       </ns0:c>
       <ns0:c r="G204" s="1" t="n">
         <ns0:v>41.0000000000001</ns0:v>
@@ -7565,7 +7565,7 @@
       </ns0:c>
       <ns0:c r="C205" s="1" t="inlineStr">
         <ns0:is>
-          <ns0:t>{105|0.1,72|0.2,136|0.3,99|0.4,147|0.5,111|0.6,187|0.7,83|0.8,181|0.9}</ns0:t>
+          <ns0:t>{32021|0.100000,32022|0.200000,32023|0.300000,32024|0.400000,32025|0.500000,32026|0.600000,32027|0.700000,32028|0.800000,32029|0.900000}</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="D205" s="1">
@@ -7578,7 +7578,7 @@
       </ns0:c>
       <ns0:c r="F205" s="1">
         <ns0:f>ROUND(F204*1.4,-5)</ns0:f>
-        <ns0:v>1.3655121467830982e+40</ns0:v>
+        <ns0:v>1.3655118980874558e+38</ns0:v>
       </ns0:c>
       <ns0:c r="G205" s="1" t="n">
         <ns0:v>41.2000000000001</ns0:v>
@@ -7597,7 +7597,7 @@
       </ns0:c>
       <ns0:c r="C206" s="1" t="inlineStr">
         <ns0:is>
-          <ns0:t>{244|0.1,206|0.2,229|0.3,197|0.4,217|0.5,204|0.6,200|0.7,216|0.8,207|0.9}</ns0:t>
+          <ns0:t>{32031|0.100000,32032|0.200000,32033|0.300000,32034|0.400000,32035|0.500000,32036|0.600000,32037|0.700000,32038|0.800000,32039|0.900000}</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="D206" s="1">
@@ -7610,7 +7610,7 @@
       </ns0:c>
       <ns0:c r="F206" s="1">
         <ns0:f>ROUND(F205*1.4,-5)</ns0:f>
-        <ns0:v>1.9117170054963372e+40</ns0:v>
+        <ns0:v>1.9117166573224382e+38</ns0:v>
       </ns0:c>
       <ns0:c r="G206" s="1" t="n">
         <ns0:v>41.4000000000001</ns0:v>
@@ -7629,7 +7629,7 @@
       </ns0:c>
       <ns0:c r="C207" s="1" t="inlineStr">
         <ns0:is>
-          <ns0:t>{226|0.1,210|0.2,212|0.3,190|0.4,228|0.5,208|0.6,225|0.7,222|0.8,201|0.9}</ns0:t>
+          <ns0:t>{32041|0.100000,32042|0.200000,32043|0.300000,32044|0.400000,32045|0.500000,32046|0.600000,32047|0.700000,32048|0.800000,32049|0.900000}</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="D207" s="1">
@@ -7642,7 +7642,7 @@
       </ns0:c>
       <ns0:c r="F207" s="1">
         <ns0:f>ROUND(F206*1.4,-5)</ns0:f>
-        <ns0:v>2.676403807694872e+40</ns0:v>
+        <ns0:v>2.6764033202514134e+38</ns0:v>
       </ns0:c>
       <ns0:c r="G207" s="1" t="n">
         <ns0:v>41.6000000000001</ns0:v>
@@ -7661,7 +7661,7 @@
       </ns0:c>
       <ns0:c r="C208" s="1" t="inlineStr">
         <ns0:is>
-          <ns0:t>{237|0.1,236|0.2,258|0.3,254|0.4,257|0.5,219|0.6,240|0.7,239|0.8,243|0.9}</ns0:t>
+          <ns0:t>{32051|0.100000,32052|0.200000,32053|0.300000,32054|0.400000,32055|0.500000,32056|0.600000,32057|0.700000,32058|0.800000,32059|0.900000}</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="D208" s="1">
@@ -7674,7 +7674,7 @@
       </ns0:c>
       <ns0:c r="F208" s="1">
         <ns0:f>ROUND(F207*1.4,-5)</ns0:f>
-        <ns0:v>3.7469653307728205e+40</ns0:v>
+        <ns0:v>3.746964648351978e+38</ns0:v>
       </ns0:c>
       <ns0:c r="G208" s="1" t="n">
         <ns0:v>41.8000000000001</ns0:v>
@@ -7693,7 +7693,7 @@
       </ns0:c>
       <ns0:c r="C209" s="1" t="inlineStr">
         <ns0:is>
-          <ns0:t>{144|0.1,68|0.2,150|0.3,35|0.4,19|0.5,97|0.6,100|0.7,93|0.8,174|0.9}</ns0:t>
+          <ns0:t>{32061|0.100000,32062|0.200000,32063|0.300000,32064|0.400000,32065|0.500000,32066|0.600000,32067|0.700000,32068|0.800000,32069|0.900000}</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="D209" s="1">
@@ -7706,7 +7706,7 @@
       </ns0:c>
       <ns0:c r="F209" s="1">
         <ns0:f>ROUND(F208*1.4,-5)</ns0:f>
-        <ns0:v>5.245751463081948e+40</ns0:v>
+        <ns0:v>5.245750507692769e+38</ns0:v>
       </ns0:c>
       <ns0:c r="G209" s="1" t="n">
         <ns0:v>42.0000000000001</ns0:v>
@@ -7725,7 +7725,7 @@
       </ns0:c>
       <ns0:c r="C210" s="1" t="inlineStr">
         <ns0:is>
-          <ns0:t>{123|0.1,41|0.2,124|0.3,170|0.4,140|0.5,60|0.6,156|0.7,89|0.8,122|0.9}</ns0:t>
+          <ns0:t>{32071|0.100000,32072|0.200000,32073|0.300000,32074|0.400000,32075|0.500000,32076|0.600000,32077|0.700000,32078|0.800000,32079|0.900000}</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="D210" s="1">
@@ -7738,7 +7738,7 @@
       </ns0:c>
       <ns0:c r="F210" s="1">
         <ns0:f>ROUND(F209*1.4,-5)</ns0:f>
-        <ns0:v>7.344052048314727e+40</ns0:v>
+        <ns0:v>7.344050710769877e+38</ns0:v>
       </ns0:c>
       <ns0:c r="G210" s="1" t="n">
         <ns0:v>42.2000000000001</ns0:v>
@@ -7757,7 +7757,7 @@
       </ns0:c>
       <ns0:c r="C211" s="1" t="inlineStr">
         <ns0:is>
-          <ns0:t>{214|0.1,223|0.2,224|0.3,238|0.4,196|0.5,193|0.6,202|0.7,203|0.8,199|0.9}</ns0:t>
+          <ns0:t>{32081|0.100000,32082|0.200000,32083|0.300000,32084|0.400000,32085|0.500000,32086|0.600000,32087|0.700000,32088|0.800000,32089|0.900000}</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="D211" s="1">
@@ -7770,7 +7770,7 @@
       </ns0:c>
       <ns0:c r="F211" s="1">
         <ns0:f>ROUND(F210*1.4,-5)</ns0:f>
-        <ns0:v>1.0281672867640618e+41</ns0:v>
+        <ns0:v>1.0281670995077828e+39</ns0:v>
       </ns0:c>
       <ns0:c r="G211" s="1" t="n">
         <ns0:v>42.4000000000001</ns0:v>
@@ -7789,7 +7789,7 @@
       </ns0:c>
       <ns0:c r="C212" s="1" t="inlineStr">
         <ns0:is>
-          <ns0:t>{198|0.1,256|0.2,191|0.3,209|0.4,192|0.5,218|0.6,245|0.7,262|0.8,194|0.9}</ns0:t>
+          <ns0:t>{32091|0.100000,32092|0.200000,32093|0.300000,32094|0.400000,32095|0.500000,32096|0.600000,32097|0.700000,32098|0.800000,32099|0.900000}</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="D212" s="1">
@@ -7802,7 +7802,7 @@
       </ns0:c>
       <ns0:c r="F212" s="1">
         <ns0:f>ROUND(F211*1.4,-5)</ns0:f>
-        <ns0:v>1.4394342014696866e+41</ns0:v>
+        <ns0:v>1.439433939310896e+39</ns0:v>
       </ns0:c>
       <ns0:c r="G212" s="1" t="n">
         <ns0:v>42.6000000000002</ns0:v>
@@ -7821,7 +7821,7 @@
       </ns0:c>
       <ns0:c r="C213" s="1" t="inlineStr">
         <ns0:is>
-          <ns0:t>{247|0.1,253|0.2,265|0.3,268|0.4,250|0.5,264|0.6,249|0.7,252|0.8,260|0.9}</ns0:t>
+          <ns0:t>{32101|0.100000,32102|0.200000,32103|0.300000,32104|0.400000,32105|0.500000,32106|0.600000,32107|0.700000,32108|0.800000,32109|0.900000}</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="D213" s="1">
@@ -7834,7 +7834,7 @@
       </ns0:c>
       <ns0:c r="F213" s="1">
         <ns0:f>ROUND(F212*1.4,-5)</ns0:f>
-        <ns0:v>2.0152078820575612e+41</ns0:v>
+        <ns0:v>2.015207515035254e+39</ns0:v>
       </ns0:c>
       <ns0:c r="G213" s="1" t="n">
         <ns0:v>42.8000000000002</ns0:v>
@@ -7853,7 +7853,7 @@
       </ns0:c>
       <ns0:c r="C214" s="1" t="inlineStr">
         <ns0:is>
-          <ns0:t>{157|0.1,46|0.2,115|0.3,164|0.4,109|0.5,186|0.6,61|0.7,52|0.8,57|0.9}</ns0:t>
+          <ns0:t>{32111|0.100000,32112|0.200000,32113|0.300000,32114|0.400000,32115|0.500000,32116|0.600000,32117|0.700000,32118|0.800000,32119|0.900000}</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="D214" s="1">
@@ -7866,7 +7866,7 @@
       </ns0:c>
       <ns0:c r="F214" s="1">
         <ns0:f>ROUND(F213*1.4,-5)</ns0:f>
-        <ns0:v>2.8212910348805854e+41</ns0:v>
+        <ns0:v>2.8212905210493555e+39</ns0:v>
       </ns0:c>
       <ns0:c r="G214" s="1" t="n">
         <ns0:v>43.0000000000001</ns0:v>
@@ -7885,7 +7885,7 @@
       </ns0:c>
       <ns0:c r="C215" s="1" t="inlineStr">
         <ns0:is>
-          <ns0:t>{117|0.1,43|0.2,143|0.3,176|0.4,139|0.5,37|0.6,146|0.7,51|0.8,17|0.9}</ns0:t>
+          <ns0:t>{32121|0.100000,32122|0.200000,32123|0.300000,32124|0.400000,32125|0.500000,32126|0.600000,32127|0.700000,32128|0.800000,32129|0.900000}</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="D215" s="1">
@@ -7898,7 +7898,7 @@
       </ns0:c>
       <ns0:c r="F215" s="1">
         <ns0:f>ROUND(F214*1.4,-5)</ns0:f>
-        <ns0:v>3.949807448832819e+41</ns0:v>
+        <ns0:v>3.9498067294690976e+39</ns0:v>
       </ns0:c>
       <ns0:c r="G215" s="1" t="n">
         <ns0:v>43.2000000000002</ns0:v>
@@ -7917,7 +7917,7 @@
       </ns0:c>
       <ns0:c r="C216" s="1" t="inlineStr">
         <ns0:is>
-          <ns0:t>{221|0.1,242|0.2,241|0.3,234|0.4,195|0.5,215|0.6,204|0.7,197|0.8,200|0.9}</ns0:t>
+          <ns0:t>{32131|0.100000,32132|0.200000,32133|0.300000,32134|0.400000,32135|0.500000,32136|0.600000,32137|0.700000,32138|0.800000,32139|0.900000}</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="D216" s="1">
@@ -7930,7 +7930,7 @@
       </ns0:c>
       <ns0:c r="F216" s="1">
         <ns0:f>ROUND(F215*1.4,-5)</ns0:f>
-        <ns0:v>5.529730428365947e+41</ns0:v>
+        <ns0:v>5.529729421256736e+39</ns0:v>
       </ns0:c>
       <ns0:c r="G216" s="1" t="n">
         <ns0:v>43.4000000000002</ns0:v>
@@ -7949,7 +7949,7 @@
       </ns0:c>
       <ns0:c r="C217" s="1" t="inlineStr">
         <ns0:is>
-          <ns0:t>{231|0.1,227|0.2,212|0.3,211|0.4,210|0.5,213|0.6,207|0.7,205|0.8,190|0.9}</ns0:t>
+          <ns0:t>{32141|0.100000,32142|0.200000,32143|0.300000,32144|0.400000,32145|0.500000,32146|0.600000,32147|0.700000,32148|0.800000,32149|0.900000}</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="D217" s="1">
@@ -7962,7 +7962,7 @@
       </ns0:c>
       <ns0:c r="F217" s="1">
         <ns0:f>ROUND(F216*1.4,-5)</ns0:f>
-        <ns0:v>7.741622599712325e+41</ns0:v>
+        <ns0:v>7.74162118975943e+39</ns0:v>
       </ns0:c>
       <ns0:c r="G217" s="1" t="n">
         <ns0:v>43.6000000000002</ns0:v>
@@ -7981,7 +7981,7 @@
       </ns0:c>
       <ns0:c r="C218" s="1" t="inlineStr">
         <ns0:is>
-          <ns0:t>{230|0.1,237|0.2,233|0.3,220|0.4,232|0.5,236|0.6,246|0.7,258|0.8,254|0.9}</ns0:t>
+          <ns0:t>{32151|0.100000,32152|0.200000,32153|0.300000,32154|0.400000,32155|0.500000,32156|0.600000,32157|0.700000,32158|0.800000,32159|0.900000}</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="D218" s="1">
@@ -7994,7 +7994,7 @@
       </ns0:c>
       <ns0:c r="F218" s="1">
         <ns0:f>ROUND(F217*1.4,-5)</ns0:f>
-        <ns0:v>1.0838271639597256e+42</ns0:v>
+        <ns0:v>1.0838269665663202e+40</ns0:v>
       </ns0:c>
       <ns0:c r="G218" s="1" t="n">
         <ns0:v>43.8000000000002</ns0:v>
@@ -8013,7 +8013,7 @@
       </ns0:c>
       <ns0:c r="C219" s="1" t="inlineStr">
         <ns0:is>
-          <ns0:t>{137|0.1,100|0.2,96|0.3,114|0.4,73|0.5,54|0.6,49|0.7,152|0.8,91|0.9}</ns0:t>
+          <ns0:t>{32161|0.100000,32162|0.200000,32163|0.300000,32164|0.400000,32165|0.500000,32166|0.600000,32167|0.700000,32168|0.800000,32169|0.900000}</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="D219" s="1">
@@ -8026,7 +8026,7 @@
       </ns0:c>
       <ns0:c r="F219" s="1">
         <ns0:f>ROUND(F218*1.4,-5)</ns0:f>
-        <ns0:v>1.5173580295436157e+42</ns0:v>
+        <ns0:v>1.5173577531928483e+40</ns0:v>
       </ns0:c>
       <ns0:c r="G219" s="1" t="n">
         <ns0:v>44.0000000000002</ns0:v>
@@ -8045,7 +8045,7 @@
       </ns0:c>
       <ns0:c r="C220" s="1" t="inlineStr">
         <ns0:is>
-          <ns0:t>{36|0.1,32|0.2,171|0.3,39|0.4,106|0.5,98|0.6,120|0.7,121|0.8,65|0.9}</ns0:t>
+          <ns0:t>{32171|0.100000,32172|0.200000,32173|0.300000,32174|0.400000,32175|0.500000,32176|0.600000,32177|0.700000,32178|0.800000,32179|0.900000}</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="D220" s="1">
@@ -8058,7 +8058,7 @@
       </ns0:c>
       <ns0:c r="F220" s="1">
         <ns0:f>ROUND(F219*1.4,-5)</ns0:f>
-        <ns0:v>2.1243012413610618e+42</ns0:v>
+        <ns0:v>2.1243008544699876e+40</ns0:v>
       </ns0:c>
       <ns0:c r="G220" s="1" t="n">
         <ns0:v>44.2000000000002</ns0:v>
@@ -8077,7 +8077,7 @@
       </ns0:c>
       <ns0:c r="C221" s="1" t="inlineStr">
         <ns0:is>
-          <ns0:t>{239|0.1,229|0.2,206|0.3,224|0.4,216|0.5,238|0.6,217|0.7,196|0.8,193|0.9}</ns0:t>
+          <ns0:t>{32181|0.100000,32182|0.200000,32183|0.300000,32184|0.400000,32185|0.500000,32186|0.600000,32187|0.700000,32188|0.800000,32189|0.900000}</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="D221" s="1">
@@ -8090,7 +8090,7 @@
       </ns0:c>
       <ns0:c r="F221" s="1">
         <ns0:f>ROUND(F220*1.4,-5)</ns0:f>
-        <ns0:v>2.9740217379054866e+42</ns0:v>
+        <ns0:v>2.9740211962579824e+40</ns0:v>
       </ns0:c>
       <ns0:c r="G221" s="1" t="n">
         <ns0:v>44.4000000000002</ns0:v>
@@ -8109,7 +8109,7 @@
       </ns0:c>
       <ns0:c r="C222" s="1" t="inlineStr">
         <ns0:is>
-          <ns0:t>{226|0.1,228|0.2,208|0.3,256|0.4,192|0.5,191|0.6,225|0.7,209|0.8,222|0.9}</ns0:t>
+          <ns0:t>{32191|0.100000,32192|0.200000,32193|0.300000,32194|0.400000,32195|0.500000,32196|0.600000,32197|0.700000,32198|0.800000,32199|0.900000}</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="D222" s="1">
@@ -8122,7 +8122,7 @@
       </ns0:c>
       <ns0:c r="F222" s="1">
         <ns0:f>ROUND(F221*1.4,-5)</ns0:f>
-        <ns0:v>4.163630433067681e+42</ns0:v>
+        <ns0:v>4.1636296747611744e+40</ns0:v>
       </ns0:c>
       <ns0:c r="G222" s="1" t="n">
         <ns0:v>44.6000000000002</ns0:v>
@@ -8141,7 +8141,7 @@
       </ns0:c>
       <ns0:c r="C223" s="1" t="inlineStr">
         <ns0:is>
-          <ns0:t>{248|0.1,247|0.2,268|0.3,261|0.4,251|0.5,255|0.6,253|0.7,259|0.8,257|0.9}</ns0:t>
+          <ns0:t>{32201|0.100000,32202|0.200000,32203|0.300000,32204|0.400000,32205|0.500000,32206|0.600000,32207|0.700000,32208|0.800000,32209|0.900000}</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="D223" s="1">
@@ -8154,7 +8154,7 @@
       </ns0:c>
       <ns0:c r="F223" s="1">
         <ns0:f>ROUND(F222*1.4,-5)</ns0:f>
-        <ns0:v>5.829082606294754e+42</ns0:v>
+        <ns0:v>5.829081544665644e+40</ns0:v>
       </ns0:c>
       <ns0:c r="G223" s="1" t="n">
         <ns0:v>44.8000000000002</ns0:v>

</xml_diff>

<commit_message>
Prototype explicit stage30-60 reforge budgets and fix in-flight builder import; lock source transactions
</commit_message>
<xml_diff>
--- a/space-battleship/config_excel/level.xlsx
+++ b/space-battleship/config_excel/level.xlsx
@@ -1826,23 +1826,20 @@
           <ns0:t>{30211|0.100000,30212|0.200000,30213|0.300000,30214|0.400000,30215|0.500000,30216|0.600000,30217|0.700000,30218|0.800000,30219|0.900000}</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="D24" s="1">
-        <ns0:f>ROUND(D23*10,0)</ns0:f>
-        <ns0:v>1.1077372220037806e+16</ns0:v>
-      </ns0:c>
-      <ns0:c r="E24" s="1">
-        <ns0:f>D24</ns0:f>
-        <ns0:v>1.1077372220037806e+16</ns0:v>
-      </ns0:c>
-      <ns0:c r="F24" s="1">
-        <ns0:f>ROUND(F23*1.4,-5)</ns0:f>
-        <ns0:v>485423799999.99994</ns0:v>
+      <ns0:c r="D24" s="1" t="n">
+        <ns0:v>4763067294395140</ns0:v>
+      </ns0:c>
+      <ns0:c r="E24" s="1" t="n">
+        <ns0:v>4763067294395140</ns0:v>
+      </ns0:c>
+      <ns0:c r="F24" s="1" t="n">
+        <ns0:v>5963524857616.636</ns0:v>
       </ns0:c>
       <ns0:c r="G24" s="1" t="n">
         <ns0:v>5</ns0:v>
       </ns0:c>
       <ns0:c r="H24" s="1" t="n">
-        <ns0:v>1</ns0:v>
+        <ns0:v>0</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="25">
@@ -1857,23 +1854,20 @@
           <ns0:t>{30221|0.100000,30222|0.200000,30223|0.300000,30224|0.400000,30225|0.500000,30226|0.600000,30227|0.700000,30228|0.800000,30229|0.900000}</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="D25" s="1">
-        <ns0:f>ROUND(D24*10,0)</ns0:f>
-        <ns0:v>1.1077372220037806e+17</ns0:v>
-      </ns0:c>
-      <ns0:c r="E25" s="1">
-        <ns0:f>D25</ns0:f>
-        <ns0:v>1.1077372220037806e+17</ns0:v>
-      </ns0:c>
-      <ns0:c r="F25" s="1">
-        <ns0:f>ROUND(F24*1.4,-5)</ns0:f>
-        <ns0:v>679593300000.0</ns0:v>
+      <ns0:c r="D25" s="1" t="n">
+        <ns0:v>2.048031753406153e+16</ns0:v>
+      </ns0:c>
+      <ns0:c r="E25" s="1" t="n">
+        <ns0:v>2.048031753406153e+16</ns0:v>
+      </ns0:c>
+      <ns0:c r="F25" s="1" t="n">
+        <ns0:v>25642065324161.59</ns0:v>
       </ns0:c>
       <ns0:c r="G25" s="1" t="n">
         <ns0:v>5.2</ns0:v>
       </ns0:c>
       <ns0:c r="H25" s="1" t="n">
-        <ns0:v>1</ns0:v>
+        <ns0:v>0</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="26">
@@ -1888,23 +1882,20 @@
           <ns0:t>{30231|0.100000,30232|0.200000,30233|0.300000,30234|0.400000,30235|0.500000,30236|0.600000,30237|0.700000,30238|0.800000,30239|0.900000}</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="D26" s="1">
-        <ns0:f>ROUND(D25*10,0)</ns0:f>
-        <ns0:v>1.1077372220037806e+18</ns0:v>
-      </ns0:c>
-      <ns0:c r="E26" s="1">
-        <ns0:f>D26</ns0:f>
-        <ns0:v>1.1077372220037806e+18</ns0:v>
-      </ns0:c>
-      <ns0:c r="F26" s="1">
-        <ns0:f>ROUND(F25*1.4,-5)</ns0:f>
-        <ns0:v>951430599999.9999</ns0:v>
+      <ns0:c r="D26" s="1" t="n">
+        <ns0:v>8.80616166791431e+16</ns0:v>
+      </ns0:c>
+      <ns0:c r="E26" s="1" t="n">
+        <ns0:v>8.80616166791431e+16</ns0:v>
+      </ns0:c>
+      <ns0:c r="F26" s="1" t="n">
+        <ns0:v>110256187370257.9</ns0:v>
       </ns0:c>
       <ns0:c r="G26" s="1" t="n">
         <ns0:v>5.4</ns0:v>
       </ns0:c>
       <ns0:c r="H26" s="1" t="n">
-        <ns0:v>1</ns0:v>
+        <ns0:v>0</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="27">
@@ -1919,23 +1910,20 @@
           <ns0:t>{30241|0.100000,30242|0.200000,30243|0.300000,30244|0.400000,30245|0.500000,30246|0.600000,30247|0.700000,30248|0.800000,30249|0.900000}</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="D27" s="1">
-        <ns0:f>ROUND(D26*10,0)</ns0:f>
-        <ns0:v>1.1077372220037806e+19</ns0:v>
-      </ns0:c>
-      <ns0:c r="E27" s="1">
-        <ns0:f>D27</ns0:f>
-        <ns0:v>1.1077372220037806e+19</ns0:v>
-      </ns0:c>
-      <ns0:c r="F27" s="1">
-        <ns0:f>ROUND(F26*1.4,-5)</ns0:f>
-        <ns0:v>1332002800000.0</ns0:v>
+      <ns0:c r="D27" s="1" t="n">
+        <ns0:v>3.786488329219983e+17</ns0:v>
+      </ns0:c>
+      <ns0:c r="E27" s="1" t="n">
+        <ns0:v>3.786488329219983e+17</ns0:v>
+      </ns0:c>
+      <ns0:c r="F27" s="1" t="n">
+        <ns0:v>474081424399572.5</ns0:v>
       </ns0:c>
       <ns0:c r="G27" s="1" t="n">
         <ns0:v>5.6</ns0:v>
       </ns0:c>
       <ns0:c r="H27" s="1" t="n">
-        <ns0:v>1</ns0:v>
+        <ns0:v>0</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="28">
@@ -1950,23 +1938,20 @@
           <ns0:t>{30251|0.100000,30252|0.200000,30253|0.300000,30254|0.400000,30255|0.500000,30256|0.600000,30257|0.700000,30258|0.800000,30259|0.900000}</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="D28" s="1">
-        <ns0:f>ROUND(D27*10,0)</ns0:f>
-        <ns0:v>1.1077372220037806e+20</ns0:v>
-      </ns0:c>
-      <ns0:c r="E28" s="1">
-        <ns0:f>D28</ns0:f>
-        <ns0:v>1.1077372220037806e+20</ns0:v>
-      </ns0:c>
-      <ns0:c r="F28" s="1">
-        <ns0:f>ROUND(F27*1.4,-5)</ns0:f>
-        <ns0:v>1864803899999.9998</ns0:v>
+      <ns0:c r="D28" s="1" t="n">
+        <ns0:v>1.628120673682214e+18</ns0:v>
+      </ns0:c>
+      <ns0:c r="E28" s="1" t="n">
+        <ns0:v>1.628120673682214e+18</ns0:v>
+      </ns0:c>
+      <ns0:c r="F28" s="1" t="n">
+        <ns0:v>2038463349054239</ns0:v>
       </ns0:c>
       <ns0:c r="G28" s="1" t="n">
         <ns0:v>5.8</ns0:v>
       </ns0:c>
       <ns0:c r="H28" s="1" t="n">
-        <ns0:v>1</ns0:v>
+        <ns0:v>0</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="29">
@@ -1981,23 +1966,20 @@
           <ns0:t>{30261|0.100000,30262|0.200000,30263|0.300000,30264|0.400000,30265|0.500000,30266|0.600000,30267|0.700000,30268|0.800000,30269|0.900000}</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="D29" s="1">
-        <ns0:f>ROUND(D28*10,0)</ns0:f>
-        <ns0:v>1.1077372220037806e+21</ns0:v>
-      </ns0:c>
-      <ns0:c r="E29" s="1">
-        <ns0:f>D29</ns0:f>
-        <ns0:v>1.1077372220037806e+21</ns0:v>
-      </ns0:c>
-      <ns0:c r="F29" s="1">
-        <ns0:f>ROUND(F28*1.4,-5)</ns0:f>
-        <ns0:v>2610725500000.0</ns0:v>
+      <ns0:c r="D29" s="1" t="n">
+        <ns0:v>7.000620885625409e+18</ns0:v>
+      </ns0:c>
+      <ns0:c r="E29" s="1" t="n">
+        <ns0:v>7.000620885625409e+18</ns0:v>
+      </ns0:c>
+      <ns0:c r="F29" s="1" t="n">
+        <ns0:v>8765019280601813</ns0:v>
       </ns0:c>
       <ns0:c r="G29" s="1" t="n">
         <ns0:v>6</ns0:v>
       </ns0:c>
       <ns0:c r="H29" s="1" t="n">
-        <ns0:v>1</ns0:v>
+        <ns0:v>0</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="30">
@@ -2012,23 +1994,20 @@
           <ns0:t>{30271|0.100000,30272|0.200000,30273|0.300000,30274|0.400000,30275|0.500000,30276|0.600000,30277|0.700000,30278|0.800000,30279|0.900000}</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="D30" s="1">
-        <ns0:f>ROUND(D29*10,0)</ns0:f>
-        <ns0:v>1.1077372220037805e+22</ns0:v>
-      </ns0:c>
-      <ns0:c r="E30" s="1">
-        <ns0:f>D30</ns0:f>
-        <ns0:v>1.1077372220037805e+22</ns0:v>
-      </ns0:c>
-      <ns0:c r="F30" s="1">
-        <ns0:f>ROUND(F29*1.4,-5)</ns0:f>
-        <ns0:v>3655015699999.9995</ns0:v>
+      <ns0:c r="D30" s="1" t="n">
+        <ns0:v>3.010138841454234e+19</ns0:v>
+      </ns0:c>
+      <ns0:c r="E30" s="1" t="n">
+        <ns0:v>3.010138841454234e+19</ns0:v>
+      </ns0:c>
+      <ns0:c r="F30" s="1" t="n">
+        <ns0:v>3.768797855745866e+16</ns0:v>
       </ns0:c>
       <ns0:c r="G30" s="1" t="n">
         <ns0:v>6.2</ns0:v>
       </ns0:c>
       <ns0:c r="H30" s="1" t="n">
-        <ns0:v>1</ns0:v>
+        <ns0:v>0</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="31">
@@ -2043,23 +2022,20 @@
           <ns0:t>{30281|0.100000,30282|0.200000,30283|0.300000,30284|0.400000,30285|0.500000,30286|0.600000,30287|0.700000,30288|0.800000,30289|0.900000}</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="D31" s="1">
-        <ns0:f>ROUND(D30*10,0)</ns0:f>
-        <ns0:v>1.1077372220037805e+23</ns0:v>
-      </ns0:c>
-      <ns0:c r="E31" s="1">
-        <ns0:f>D31</ns0:f>
-        <ns0:v>1.1077372220037805e+23</ns0:v>
-      </ns0:c>
-      <ns0:c r="F31" s="1">
-        <ns0:f>ROUND(F30*1.4,-5)</ns0:f>
-        <ns0:v>5117022000000.0</ns0:v>
+      <ns0:c r="D31" s="1" t="n">
+        <ns0:v>1.294304604243966e+20</ns0:v>
+      </ns0:c>
+      <ns0:c r="E31" s="1" t="n">
+        <ns0:v>1.294304604243966e+20</ns0:v>
+      </ns0:c>
+      <ns0:c r="F31" s="1" t="n">
+        <ns0:v>1.620514093894771e+17</ns0:v>
       </ns0:c>
       <ns0:c r="G31" s="1" t="n">
         <ns0:v>6.4</ns0:v>
       </ns0:c>
       <ns0:c r="H31" s="1" t="n">
-        <ns0:v>1</ns0:v>
+        <ns0:v>0</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="32">
@@ -2074,23 +2050,20 @@
           <ns0:t>{30291|0.100000,30292|0.200000,30293|0.300000,30294|0.400000,30295|0.500000,30296|0.600000,30297|0.700000,30298|0.800000,30299|0.900000}</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="D32" s="1">
-        <ns0:f>ROUND(D31*10,0)</ns0:f>
-        <ns0:v>1.1077372220037805e+24</ns0:v>
-      </ns0:c>
-      <ns0:c r="E32" s="1">
-        <ns0:f>D32</ns0:f>
-        <ns0:v>1.1077372220037805e+24</ns0:v>
-      </ns0:c>
-      <ns0:c r="F32" s="1">
-        <ns0:f>ROUND(F31*1.4,-5)</ns0:f>
-        <ns0:v>7163830799999.999</ns0:v>
+      <ns0:c r="D32" s="1" t="n">
+        <ns0:v>5.565272888734292e+20</ns0:v>
+      </ns0:c>
+      <ns0:c r="E32" s="1" t="n">
+        <ns0:v>5.565272888734292e+20</ns0:v>
+      </ns0:c>
+      <ns0:c r="F32" s="1" t="n">
+        <ns0:v>6.967913984847764e+17</ns0:v>
       </ns0:c>
       <ns0:c r="G32" s="1" t="n">
         <ns0:v>6.6</ns0:v>
       </ns0:c>
       <ns0:c r="H32" s="1" t="n">
-        <ns0:v>1</ns0:v>
+        <ns0:v>0</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="33">
@@ -2105,17 +2078,14 @@
           <ns0:t>{30301|0.100000,30302|0.200000,30303|0.300000,30304|0.400000,30305|0.500000,30306|0.600000,30307|0.700000,30308|0.800000,30309|0.900000}</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="D33" s="1">
-        <ns0:f>ROUND(D32*10,0)</ns0:f>
-        <ns0:v>1.1077372220037805e+25</ns0:v>
-      </ns0:c>
-      <ns0:c r="E33" s="1">
-        <ns0:f>D33</ns0:f>
-        <ns0:v>1.1077372220037805e+25</ns0:v>
-      </ns0:c>
-      <ns0:c r="F33" s="1">
-        <ns0:f>ROUND(F32*1.4,-5)</ns0:f>
-        <ns0:v>10029363100000.0</ns0:v>
+      <ns0:c r="D33" s="1" t="n">
+        <ns0:v>2.39296547540079e+21</ns0:v>
+      </ns0:c>
+      <ns0:c r="E33" s="1" t="n">
+        <ns0:v>2.39296547540079e+21</ns0:v>
+      </ns0:c>
+      <ns0:c r="F33" s="1" t="n">
+        <ns0:v>2.99607547278696e+18</ns0:v>
       </ns0:c>
       <ns0:c r="G33" s="1" t="n">
         <ns0:v>6.8</ns0:v>
@@ -2136,23 +2106,20 @@
           <ns0:t>{30311|0.100000,30312|0.200000,30313|0.300000,30314|0.400000,30315|0.500000,30316|0.600000,30317|0.700000,30318|0.800000,30319|0.900000}</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="D34" s="1">
-        <ns0:f>ROUND(D33*10,0)</ns0:f>
-        <ns0:v>1.1077372220037805e+26</ns0:v>
-      </ns0:c>
-      <ns0:c r="E34" s="1">
-        <ns0:f>D34</ns0:f>
-        <ns0:v>1.1077372220037805e+26</ns0:v>
-      </ns0:c>
-      <ns0:c r="F34" s="1">
-        <ns0:f>ROUND(F33*1.4,-5)</ns0:f>
-        <ns0:v>14041108299999.998</ns0:v>
+      <ns0:c r="D34" s="1" t="n">
+        <ns0:v>1.028931353582277e+22</ns0:v>
+      </ns0:c>
+      <ns0:c r="E34" s="1" t="n">
+        <ns0:v>1.028931353582277e+22</ns0:v>
+      </ns0:c>
+      <ns0:c r="F34" s="1" t="n">
+        <ns0:v>2.99607547278696e+18</ns0:v>
       </ns0:c>
       <ns0:c r="G34" s="1" t="n">
         <ns0:v>7</ns0:v>
       </ns0:c>
       <ns0:c r="H34" s="1" t="n">
-        <ns0:v>1.2</ns0:v>
+        <ns0:v>1.037137289336648</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="35">
@@ -2167,23 +2134,20 @@
           <ns0:t>{30321|0.100000,30322|0.200000,30323|0.300000,30324|0.400000,30325|0.500000,30326|0.600000,30327|0.700000,30328|0.800000,30329|0.900000}</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="D35" s="1">
-        <ns0:f>ROUND(D34*10,0)</ns0:f>
-        <ns0:v>1.1077372220037804e+27</ns0:v>
-      </ns0:c>
-      <ns0:c r="E35" s="1">
-        <ns0:f>D35</ns0:f>
-        <ns0:v>1.1077372220037804e+27</ns0:v>
-      </ns0:c>
-      <ns0:c r="F35" s="1">
-        <ns0:f>ROUND(F34*1.4,-5)</ns0:f>
-        <ns0:v>19657551600000.0</ns0:v>
+      <ns0:c r="D35" s="1" t="n">
+        <ns0:v>4.424216484808832e+22</ns0:v>
+      </ns0:c>
+      <ns0:c r="E35" s="1" t="n">
+        <ns0:v>4.424216484808832e+22</ns0:v>
+      </ns0:c>
+      <ns0:c r="F35" s="1" t="n">
+        <ns0:v>2.99607547278696e+18</ns0:v>
       </ns0:c>
       <ns0:c r="G35" s="1" t="n">
         <ns0:v>7.2</ns0:v>
       </ns0:c>
       <ns0:c r="H35" s="1" t="n">
-        <ns0:v>1.44</ns0:v>
+        <ns0:v>1.07565375693257</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="36">
@@ -2198,23 +2162,20 @@
           <ns0:t>{30331|0.100000,30332|0.200000,30333|0.300000,30334|0.400000,30335|0.500000,30336|0.600000,30337|0.700000,30338|0.800000,30339|0.900000}</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="D36" s="1">
-        <ns0:f>ROUND(D35*10,0)</ns0:f>
-        <ns0:v>1.1077372220037803e+28</ns0:v>
-      </ns0:c>
-      <ns0:c r="E36" s="1">
-        <ns0:f>D36</ns0:f>
-        <ns0:v>1.1077372220037803e+28</ns0:v>
-      </ns0:c>
-      <ns0:c r="F36" s="1">
-        <ns0:f>ROUND(F35*1.4,-5)</ns0:f>
-        <ns0:v>27520572199999.996</ns0:v>
+      <ns0:c r="D36" s="1" t="n">
+        <ns0:v>8.179679859850836e+23</ns0:v>
+      </ns0:c>
+      <ns0:c r="E36" s="1" t="n">
+        <ns0:v>8.179679859850836e+23</ns0:v>
+      </ns0:c>
+      <ns0:c r="F36" s="1" t="n">
+        <ns0:v>6.212662100371039e+18</ns0:v>
       </ns0:c>
       <ns0:c r="G36" s="1" t="n">
         <ns0:v>7.4</ns0:v>
       </ns0:c>
       <ns0:c r="H36" s="1" t="n">
-        <ns0:v>1.73</ns0:v>
+        <ns0:v>1.115600621729828</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="37">
@@ -2229,23 +2190,20 @@
           <ns0:t>{30341|0.100000,30342|0.200000,30343|0.300000,30344|0.400000,30345|0.500000,30346|0.600000,30347|0.700000,30348|0.800000,30349|0.900000}</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="D37" s="1">
-        <ns0:f>ROUND(D36*10,0)</ns0:f>
-        <ns0:v>1.1077372220037803e+29</ns0:v>
-      </ns0:c>
-      <ns0:c r="E37" s="1">
-        <ns0:f>D37</ns0:f>
-        <ns0:v>1.1077372220037803e+29</ns0:v>
-      </ns0:c>
-      <ns0:c r="F37" s="1">
-        <ns0:f>ROUND(F36*1.4,-5)</ns0:f>
-        <ns0:v>38528801100000.0</ns0:v>
+      <ns0:c r="D37" s="1" t="n">
+        <ns0:v>1.512294048887176e+25</ns0:v>
+      </ns0:c>
+      <ns0:c r="E37" s="1" t="n">
+        <ns0:v>1.512294048887176e+25</ns0:v>
+      </ns0:c>
+      <ns0:c r="F37" s="1" t="n">
+        <ns0:v>6.212662100371039e+18</ns0:v>
       </ns0:c>
       <ns0:c r="G37" s="1" t="n">
         <ns0:v>7.6</ns0:v>
       </ns0:c>
       <ns0:c r="H37" s="1" t="n">
-        <ns0:v>2.08</ns0:v>
+        <ns0:v>1.157031004803153</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="38">
@@ -2260,23 +2218,20 @@
           <ns0:t>{30351|0.100000,30352|0.200000,30353|0.300000,30354|0.400000,30355|0.500000,30356|0.600000,30357|0.700000,30358|0.800000,30359|0.900000}</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="D38" s="1">
-        <ns0:f>ROUND(D37*10,0)</ns0:f>
-        <ns0:v>1.1077372220037803e+30</ns0:v>
-      </ns0:c>
-      <ns0:c r="E38" s="1">
-        <ns0:f>D38</ns0:f>
-        <ns0:v>1.1077372220037803e+30</ns0:v>
-      </ns0:c>
-      <ns0:c r="F38" s="1">
-        <ns0:f>ROUND(F37*1.4,-5)</ns0:f>
-        <ns0:v>53940321499999.99</ns0:v>
+      <ns0:c r="D38" s="1" t="n">
+        <ns0:v>5.797772421440058e+26</ns0:v>
+      </ns0:c>
+      <ns0:c r="E38" s="1" t="n">
+        <ns0:v>5.797772421440058e+26</ns0:v>
+      </ns0:c>
+      <ns0:c r="F38" s="1" t="n">
+        <ns0:v>1.855090962911431e+19</ns0:v>
       </ns0:c>
       <ns0:c r="G38" s="1" t="n">
         <ns0:v>7.8</ns0:v>
       </ns0:c>
       <ns0:c r="H38" s="1" t="n">
-        <ns0:v>2.5</ns0:v>
+        <ns0:v>1.2</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="39">
@@ -2291,23 +2246,20 @@
           <ns0:t>{30361|0.100000,30362|0.200000,30363|0.300000,30364|0.400000,30365|0.500000,30366|0.600000,30367|0.700000,30368|0.800000,30369|0.900000}</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="D39" s="1">
-        <ns0:f>ROUND(D38*10,0)</ns0:f>
-        <ns0:v>1.1077372220037803e+31</ns0:v>
-      </ns0:c>
-      <ns0:c r="E39" s="1">
-        <ns0:f>D39</ns0:f>
-        <ns0:v>1.1077372220037803e+31</ns0:v>
-      </ns0:c>
-      <ns0:c r="F39" s="1">
-        <ns0:f>ROUND(F38*1.4,-5)</ns0:f>
-        <ns0:v>75516450100000.0</ns0:v>
+      <ns0:c r="D39" s="1" t="n">
+        <ns0:v>1.731205568606127e+27</ns0:v>
+      </ns0:c>
+      <ns0:c r="E39" s="1" t="n">
+        <ns0:v>1.731205568606127e+27</ns0:v>
+      </ns0:c>
+      <ns0:c r="F39" s="1" t="n">
+        <ns0:v>3.846716620693144e+19</ns0:v>
       </ns0:c>
       <ns0:c r="G39" s="1" t="n">
         <ns0:v>8</ns0:v>
       </ns0:c>
       <ns0:c r="H39" s="1" t="n">
-        <ns0:v>3</ns0:v>
+        <ns0:v>1.244564747203978</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="40">
@@ -2322,23 +2274,20 @@
           <ns0:t>{30371|0.100000,30372|0.200000,30373|0.300000,30374|0.400000,30375|0.500000,30376|0.600000,30377|0.700000,30378|0.800000,30379|0.900000}</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="D40" s="1">
-        <ns0:f>ROUND(D39*10,0)</ns0:f>
-        <ns0:v>1.1077372220037804e+32</ns0:v>
-      </ns0:c>
-      <ns0:c r="E40" s="1">
-        <ns0:f>D40</ns0:f>
-        <ns0:v>1.1077372220037804e+32</ns0:v>
-      </ns0:c>
-      <ns0:c r="F40" s="1">
-        <ns0:f>ROUND(F39*1.4,-5)</ns0:f>
-        <ns0:v>105723030099999.98</ns0:v>
+      <ns0:c r="D40" s="1" t="n">
+        <ns0:v>5.169352128568795e+27</ns0:v>
+      </ns0:c>
+      <ns0:c r="E40" s="1" t="n">
+        <ns0:v>5.169352128568795e+27</ns0:v>
+      </ns0:c>
+      <ns0:c r="F40" s="1" t="n">
+        <ns0:v>7.9765515846693e+19</ns0:v>
       </ns0:c>
       <ns0:c r="G40" s="1" t="n">
         <ns0:v>8.199999999999999</ns0:v>
       </ns0:c>
       <ns0:c r="H40" s="1" t="n">
-        <ns0:v>3.6</ns0:v>
+        <ns0:v>1.290784508319084</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="41">
@@ -2353,23 +2302,20 @@
           <ns0:t>{30381|0.100000,30382|0.200000,30383|0.300000,30384|0.400000,30385|0.500000,30386|0.600000,30387|0.700000,30388|0.800000,30389|0.900000}</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="D41" s="1">
-        <ns0:f>ROUND(D40*10,0)</ns0:f>
-        <ns0:v>1.1077372220037804e+33</ns0:v>
-      </ns0:c>
-      <ns0:c r="E41" s="1">
-        <ns0:f>D41</ns0:f>
-        <ns0:v>1.1077372220037804e+33</ns0:v>
-      </ns0:c>
-      <ns0:c r="F41" s="1">
-        <ns0:f>ROUND(F40*1.4,-5)</ns0:f>
-        <ns0:v>148012242100000.0</ns0:v>
+      <ns0:c r="D41" s="1" t="n">
+        <ns0:v>1.543560274627236e+28</ns0:v>
+      </ns0:c>
+      <ns0:c r="E41" s="1" t="n">
+        <ns0:v>1.543560274627236e+28</ns0:v>
+      </ns0:c>
+      <ns0:c r="F41" s="1" t="n">
+        <ns0:v>1.654017736597026e+20</ns0:v>
       </ns0:c>
       <ns0:c r="G41" s="1" t="n">
         <ns0:v>8.4</ns0:v>
       </ns0:c>
       <ns0:c r="H41" s="1" t="n">
-        <ns0:v>4.32</ns0:v>
+        <ns0:v>1.338720746075793</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="42">
@@ -2384,23 +2330,20 @@
           <ns0:t>{30391|0.100000,30392|0.200000,30393|0.300000,30394|0.400000,30395|0.500000,30396|0.600000,30397|0.700000,30398|0.800000,30399|0.900000}</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="D42" s="1">
-        <ns0:f>ROUND(D41*10,0)</ns0:f>
-        <ns0:v>1.1077372220037804e+34</ns0:v>
-      </ns0:c>
-      <ns0:c r="E42" s="1">
-        <ns0:f>D42</ns0:f>
-        <ns0:v>1.1077372220037804e+34</ns0:v>
-      </ns0:c>
-      <ns0:c r="F42" s="1">
-        <ns0:f>ROUND(F41*1.4,-5)</ns0:f>
-        <ns0:v>207217138899999.97</ns0:v>
+      <ns0:c r="D42" s="1" t="n">
+        <ns0:v>1.376253845651405e+29</ns0:v>
+      </ns0:c>
+      <ns0:c r="E42" s="1" t="n">
+        <ns0:v>1.376253845651405e+29</ns0:v>
+      </ns0:c>
+      <ns0:c r="F42" s="1" t="n">
+        <ns0:v>7.111973515960703e+20</ns0:v>
       </ns0:c>
       <ns0:c r="G42" s="1" t="n">
         <ns0:v>8.6</ns0:v>
       </ns0:c>
       <ns0:c r="H42" s="1" t="n">
-        <ns0:v>5.18</ns0:v>
+        <ns0:v>1.388437205763783</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="43">
@@ -2415,23 +2358,20 @@
           <ns0:t>{30401|0.100000,30402|0.200000,30403|0.300000,30404|0.400000,30405|0.500000,30406|0.600000,30407|0.700000,30408|0.800000,30409|0.900000}</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="D43" s="1">
-        <ns0:f>ROUND(D42*10,0)</ns0:f>
-        <ns0:v>1.1077372220037804e+35</ns0:v>
-      </ns0:c>
-      <ns0:c r="E43" s="1">
-        <ns0:f>D43</ns0:f>
-        <ns0:v>1.1077372220037804e+35</ns0:v>
-      </ns0:c>
-      <ns0:c r="F43" s="1">
-        <ns0:f>ROUND(F42*1.4,-5)</ns0:f>
-        <ns0:v>290103994500000.0</ns0:v>
+      <ns0:c r="D43" s="1" t="n">
+        <ns0:v>5.276226932910335e+30</ns0:v>
+      </ns0:c>
+      <ns0:c r="E43" s="1" t="n">
+        <ns0:v>5.276226932910335e+30</ns0:v>
+      </ns0:c>
+      <ns0:c r="F43" s="1" t="n">
+        <ns0:v>6.341107025364199e+21</ns0:v>
       </ns0:c>
       <ns0:c r="G43" s="1" t="n">
         <ns0:v>8.800000000000001</ns0:v>
       </ns0:c>
       <ns0:c r="H43" s="1" t="n">
-        <ns0:v>6.22</ns0:v>
+        <ns0:v>1.44</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="44">
@@ -2446,23 +2386,20 @@
           <ns0:t>{30411|0.100000,30412|0.200000,30413|0.300000,30414|0.400000,30415|0.500000,30416|0.600000,30417|0.700000,30418|0.800000,30419|0.900000}</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="D44" s="1">
-        <ns0:f>ROUND(D43*10,0)</ns0:f>
-        <ns0:v>1.1077372220037803e+36</ns0:v>
-      </ns0:c>
-      <ns0:c r="E44" s="1">
-        <ns0:f>D44</ns0:f>
-        <ns0:v>1.1077372220037803e+36</ns0:v>
-      </ns0:c>
-      <ns0:c r="F44" s="1">
-        <ns0:f>ROUND(F43*1.4,-5)</ns0:f>
-        <ns0:v>406145592299999.94</ns0:v>
+      <ns0:c r="D44" s="1" t="n">
+        <ns0:v>1.575472920203933e+31</ns0:v>
+      </ns0:c>
+      <ns0:c r="E44" s="1" t="n">
+        <ns0:v>1.575472920203933e+31</ns0:v>
+      </ns0:c>
+      <ns0:c r="F44" s="1" t="n">
+        <ns0:v>1.31489195277952e+22</ns0:v>
       </ns0:c>
       <ns0:c r="G44" s="1" t="n">
         <ns0:v>9</ns0:v>
       </ns0:c>
       <ns0:c r="H44" s="1" t="n">
-        <ns0:v>7.46</ns0:v>
+        <ns0:v>1.493477696644773</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="45">
@@ -2477,23 +2414,20 @@
           <ns0:t>{30421|0.100000,30422|0.200000,30423|0.300000,30424|0.400000,30425|0.500000,30426|0.600000,30427|0.700000,30428|0.800000,30429|0.900000}</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="D45" s="1">
-        <ns0:f>ROUND(D44*10,0)</ns0:f>
-        <ns0:v>1.1077372220037803e+37</ns0:v>
-      </ns0:c>
-      <ns0:c r="E45" s="1">
-        <ns0:f>D45</ns0:f>
-        <ns0:v>1.1077372220037803e+37</ns0:v>
-      </ns0:c>
-      <ns0:c r="F45" s="1">
-        <ns0:f>ROUND(F44*1.4,-5)</ns0:f>
-        <ns0:v>568603829200000.0</ns0:v>
+      <ns0:c r="D45" s="1" t="n">
+        <ns0:v>4.704336932162219e+31</ns0:v>
+      </ns0:c>
+      <ns0:c r="E45" s="1" t="n">
+        <ns0:v>4.704336932162219e+31</ns0:v>
+      </ns0:c>
+      <ns0:c r="F45" s="1" t="n">
+        <ns0:v>2.726559953283612e+22</ns0:v>
       </ns0:c>
       <ns0:c r="G45" s="1" t="n">
         <ns0:v>9.199999999999999</ns0:v>
       </ns0:c>
       <ns0:c r="H45" s="1" t="n">
-        <ns0:v>8.949999999999999</ns0:v>
+        <ns0:v>1.548941409982901</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="46">
@@ -2508,23 +2442,20 @@
           <ns0:t>{30431|0.100000,30432|0.200000,30433|0.300000,30434|0.400000,30435|0.500000,30436|0.600000,30437|0.700000,30438|0.800000,30439|0.900000}</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="D46" s="1">
-        <ns0:f>ROUND(D45*10,0)</ns0:f>
-        <ns0:v>1.1077372220037804e+38</ns0:v>
-      </ns0:c>
-      <ns0:c r="E46" s="1">
-        <ns0:f>D46</ns0:f>
-        <ns0:v>1.1077372220037804e+38</ns0:v>
-      </ns0:c>
-      <ns0:c r="F46" s="1">
-        <ns0:f>ROUND(F45*1.4,-5)</ns0:f>
-        <ns0:v>796045360899999.9</ns0:v>
+      <ns0:c r="D46" s="1" t="n">
+        <ns0:v>1.404707481004547e+32</ns0:v>
+      </ns0:c>
+      <ns0:c r="E46" s="1" t="n">
+        <ns0:v>1.404707481004547e+32</ns0:v>
+      </ns0:c>
+      <ns0:c r="F46" s="1" t="n">
+        <ns0:v>5.653794719128898e+22</ns0:v>
       </ns0:c>
       <ns0:c r="G46" s="1" t="n">
         <ns0:v>9.4</ns0:v>
       </ns0:c>
       <ns0:c r="H46" s="1" t="n">
-        <ns0:v>10.74</ns0:v>
+        <ns0:v>1.606464895290951</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="47">
@@ -2539,23 +2470,20 @@
           <ns0:t>{30441|0.100000,30442|0.200000,30443|0.300000,30444|0.400000,30445|0.500000,30446|0.600000,30447|0.700000,30448|0.800000,30449|0.900000}</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="D47" s="1">
-        <ns0:f>ROUND(D46*10,0)</ns0:f>
-        <ns0:v>1.1077372220037804e+39</ns0:v>
-      </ns0:c>
-      <ns0:c r="E47" s="1">
-        <ns0:f>D47</ns0:f>
-        <ns0:v>1.1077372220037804e+39</ns0:v>
-      </ns0:c>
-      <ns0:c r="F47" s="1">
-        <ns0:f>ROUND(F46*1.4,-5)</ns0:f>
-        <ns0:v>1114463505299999.9</ns0:v>
+      <ns0:c r="D47" s="1" t="n">
+        <ns0:v>1.252451300105319e+33</ns0:v>
+      </ns0:c>
+      <ns0:c r="E47" s="1" t="n">
+        <ns0:v>1.252451300105319e+33</ns0:v>
+      </ns0:c>
+      <ns0:c r="F47" s="1" t="n">
+        <ns0:v>2.431028242166887e+23</ns0:v>
       </ns0:c>
       <ns0:c r="G47" s="1" t="n">
         <ns0:v>9.6</ns0:v>
       </ns0:c>
       <ns0:c r="H47" s="1" t="n">
-        <ns0:v>12.89</ns0:v>
+        <ns0:v>1.66612464691654</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="48">
@@ -2570,23 +2498,20 @@
           <ns0:t>{30451|0.100000,30452|0.200000,30453|0.300000,30454|0.400000,30455|0.500000,30456|0.600000,30457|0.700000,30458|0.800000,30459|0.900000}</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="D48" s="1">
-        <ns0:f>ROUND(D47*10,0)</ns0:f>
-        <ns0:v>1.1077372220037803e+40</ns0:v>
-      </ns0:c>
-      <ns0:c r="E48" s="1">
-        <ns0:f>D48</ns0:f>
-        <ns0:v>1.1077372220037803e+40</ns0:v>
-      </ns0:c>
-      <ns0:c r="F48" s="1">
-        <ns0:f>ROUND(F47*1.4,-5)</ns0:f>
-        <ns0:v>1560248907399999.8</ns0:v>
+      <ns0:c r="D48" s="1" t="n">
+        <ns0:v>4.801597686832596e+34</ns0:v>
+      </ns0:c>
+      <ns0:c r="E48" s="1" t="n">
+        <ns0:v>4.801597686832596e+34</ns0:v>
+      </ns0:c>
+      <ns0:c r="F48" s="1" t="n">
+        <ns0:v>2.167529199970716e+24</ns0:v>
       </ns0:c>
       <ns0:c r="G48" s="1" t="n">
         <ns0:v>9.800000000000001</ns0:v>
       </ns0:c>
       <ns0:c r="H48" s="1" t="n">
-        <ns0:v>15.47</ns0:v>
+        <ns0:v>1.728</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="49">
@@ -2601,23 +2526,20 @@
           <ns0:t>{30461|0.100000,30462|0.200000,30463|0.300000,30464|0.400000,30465|0.500000,30466|0.600000,30467|0.700000,30468|0.800000,30469|0.900000}</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="D49" s="1">
-        <ns0:f>ROUND(D48*10,0)</ns0:f>
-        <ns0:v>1.1077372220037803e+41</ns0:v>
-      </ns0:c>
-      <ns0:c r="E49" s="1">
-        <ns0:f>D49</ns0:f>
-        <ns0:v>1.1077372220037803e+41</ns0:v>
-      </ns0:c>
-      <ns0:c r="F49" s="1">
-        <ns0:f>ROUND(F48*1.4,-5)</ns0:f>
-        <ns0:v>2184348470399999.8</ns0:v>
+      <ns0:c r="D49" s="1" t="n">
+        <ns0:v>1.433749386731914e+35</ns0:v>
+      </ns0:c>
+      <ns0:c r="E49" s="1" t="n">
+        <ns0:v>1.433749386731914e+35</ns0:v>
+      </ns0:c>
+      <ns0:c r="F49" s="1" t="n">
+        <ns0:v>4.494588549059277e+24</ns0:v>
       </ns0:c>
       <ns0:c r="G49" s="1" t="n">
         <ns0:v>10</ns0:v>
       </ns0:c>
       <ns0:c r="H49" s="1" t="n">
-        <ns0:v>18.56</ns0:v>
+        <ns0:v>1.792173235973728</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="50">
@@ -2632,23 +2554,20 @@
           <ns0:t>{30471|0.100000,30472|0.200000,30473|0.300000,30474|0.400000,30475|0.500000,30476|0.600000,30477|0.700000,30478|0.800000,30479|0.900000}</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="D50" s="1">
-        <ns0:f>ROUND(D49*10,0)</ns0:f>
-        <ns0:v>1.1077372220037803e+42</ns0:v>
-      </ns0:c>
-      <ns0:c r="E50" s="1">
-        <ns0:f>D50</ns0:f>
-        <ns0:v>1.1077372220037803e+42</ns0:v>
-      </ns0:c>
-      <ns0:c r="F50" s="1">
-        <ns0:f>ROUND(F49*1.4,-5)</ns0:f>
-        <ns0:v>3058087858599999.5</ns0:v>
+      <ns0:c r="D50" s="1" t="n">
+        <ns0:v>4.281152728791306e+35</ns0:v>
+      </ns0:c>
+      <ns0:c r="E50" s="1" t="n">
+        <ns0:v>4.281152728791306e+35</ns0:v>
+      </ns0:c>
+      <ns0:c r="F50" s="1" t="n">
+        <ns0:v>9.319978815329315e+24</ns0:v>
       </ns0:c>
       <ns0:c r="G50" s="1" t="n">
         <ns0:v>10.2</ns0:v>
       </ns0:c>
       <ns0:c r="H50" s="1" t="n">
-        <ns0:v>22.27</ns0:v>
+        <ns0:v>1.858729691979481</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="51">
@@ -2663,23 +2582,20 @@
           <ns0:t>{30481|0.100000,30482|0.200000,30483|0.300000,30484|0.400000,30485|0.500000,30486|0.600000,30487|0.700000,30488|0.800000,30489|0.900000}</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="D51" s="1">
-        <ns0:f>ROUND(D50*10,0)</ns0:f>
-        <ns0:v>1.1077372220037803e+43</ns0:v>
-      </ns0:c>
-      <ns0:c r="E51" s="1">
-        <ns0:f>D51</ns0:f>
-        <ns0:v>1.1077372220037803e+43</ns0:v>
-      </ns0:c>
-      <ns0:c r="F51" s="1">
-        <ns0:f>ROUND(F50*1.4,-5)</ns0:f>
-        <ns0:v>4281323001999999.5</ns0:v>
+      <ns0:c r="D51" s="1" t="n">
+        <ns0:v>1.278345354972718e+36</ns0:v>
+      </ns0:c>
+      <ns0:c r="E51" s="1" t="n">
+        <ns0:v>1.278345354972718e+36</ns0:v>
+      </ns0:c>
+      <ns0:c r="F51" s="1" t="n">
+        <ns0:v>1.932590807146687e+25</ns0:v>
       </ns0:c>
       <ns0:c r="G51" s="1" t="n">
         <ns0:v>10.4</ns0:v>
       </ns0:c>
       <ns0:c r="H51" s="1" t="n">
-        <ns0:v>26.72</ns0:v>
+        <ns0:v>1.927757874349142</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="52">
@@ -2694,23 +2610,20 @@
           <ns0:t>{30491|0.100000,30492|0.200000,30493|0.300000,30494|0.400000,30495|0.500000,30496|0.600000,30497|0.700000,30498|0.800000,30499|0.900000}</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="D52" s="1">
-        <ns0:f>ROUND(D51*10,0)</ns0:f>
-        <ns0:v>1.1077372220037804e+44</ns0:v>
-      </ns0:c>
-      <ns0:c r="E52" s="1">
-        <ns0:f>D52</ns0:f>
-        <ns0:v>1.1077372220037804e+44</ns0:v>
-      </ns0:c>
-      <ns0:c r="F52" s="1">
-        <ns0:f>ROUND(F51*1.4,-5)</ns0:f>
-        <ns0:v>5993852202800000.0</ns0:v>
+      <ns0:c r="D52" s="1" t="n">
+        <ns0:v>1.139785559249822e+37</ns0:v>
+      </ns0:c>
+      <ns0:c r="E52" s="1" t="n">
+        <ns0:v>1.139785559249822e+37</ns0:v>
+      </ns0:c>
+      <ns0:c r="F52" s="1" t="n">
+        <ns0:v>8.30978672930941e+25</ns0:v>
       </ns0:c>
       <ns0:c r="G52" s="1" t="n">
         <ns0:v>10.6</ns0:v>
       </ns0:c>
       <ns0:c r="H52" s="1" t="n">
-        <ns0:v>32.06</ns0:v>
+        <ns0:v>1.999349576299847</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="53">
@@ -2725,23 +2638,20 @@
           <ns0:t>{30501|0.100000,30502|0.200000,30503|0.300000,30504|0.400000,30505|0.500000,30506|0.600000,30507|0.700000,30508|0.800000,30509|0.900000}</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="D53" s="1">
-        <ns0:f>ROUND(D52*10,0)</ns0:f>
-        <ns0:v>1.1077372220037804e+45</ns0:v>
-      </ns0:c>
-      <ns0:c r="E53" s="1">
-        <ns0:f>D53</ns0:f>
-        <ns0:v>1.1077372220037804e+45</ns0:v>
-      </ns0:c>
-      <ns0:c r="F53" s="1">
-        <ns0:f>ROUND(F52*1.4,-5)</ns0:f>
-        <ns0:v>8391393083899999.0</ns0:v>
+      <ns0:c r="D53" s="1" t="n">
+        <ns0:v>4.369664277021335e+38</ns0:v>
+      </ns0:c>
+      <ns0:c r="E53" s="1" t="n">
+        <ns0:v>4.369664277021335e+38</ns0:v>
+      </ns0:c>
+      <ns0:c r="F53" s="1" t="n">
+        <ns0:v>7.409089318210736e+26</ns0:v>
       </ns0:c>
       <ns0:c r="G53" s="1" t="n">
         <ns0:v>10.8</ns0:v>
       </ns0:c>
       <ns0:c r="H53" s="1" t="n">
-        <ns0:v>38.47</ns0:v>
+        <ns0:v>2.0736</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="54">
@@ -2756,23 +2666,20 @@
           <ns0:t>{30511|0.100000,30512|0.200000,30513|0.300000,30514|0.400000,30515|0.500000,30516|0.600000,30517|0.700000,30518|0.800000,30519|0.900000}</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="D54" s="1">
-        <ns0:f>ROUND(D53*10,0)</ns0:f>
-        <ns0:v>1.1077372220037804e+46</ns0:v>
-      </ns0:c>
-      <ns0:c r="E54" s="1">
-        <ns0:f>D54</ns0:f>
-        <ns0:v>1.1077372220037804e+46</ns0:v>
-      </ns0:c>
-      <ns0:c r="F54" s="1">
-        <ns0:f>ROUND(F53*1.4,-5)</ns0:f>
-        <ns0:v>1.17479503175e+16</ns0:v>
+      <ns0:c r="D54" s="1" t="n">
+        <ns0:v>1.304774761655727e+39</ns0:v>
+      </ns0:c>
+      <ns0:c r="E54" s="1" t="n">
+        <ns0:v>1.304774761655727e+39</ns0:v>
+      </ns0:c>
+      <ns0:c r="F54" s="1" t="n">
+        <ns0:v>1.536348761024178e+27</ns0:v>
       </ns0:c>
       <ns0:c r="G54" s="1" t="n">
         <ns0:v>11</ns0:v>
       </ns0:c>
       <ns0:c r="H54" s="1" t="n">
-        <ns0:v>46.16</ns0:v>
+        <ns0:v>2.150607883168473</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="55">
@@ -2787,23 +2694,20 @@
           <ns0:t>{30521|0.100000,30522|0.200000,30523|0.300000,30524|0.400000,30525|0.500000,30526|0.600000,30527|0.700000,30528|0.800000,30529|0.900000}</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="D55" s="1">
-        <ns0:f>ROUND(D54*10,0)</ns0:f>
-        <ns0:v>1.1077372220037803e+47</ns0:v>
-      </ns0:c>
-      <ns0:c r="E55" s="1">
-        <ns0:f>D55</ns0:f>
-        <ns0:v>1.1077372220037803e+47</ns0:v>
-      </ns0:c>
-      <ns0:c r="F55" s="1">
-        <ns0:f>ROUND(F54*1.4,-5)</ns0:f>
-        <ns0:v>1.6447130444499998e+16</ns0:v>
+      <ns0:c r="D55" s="1" t="n">
+        <ns0:v>3.896036561907814e+39</ns0:v>
+      </ns0:c>
+      <ns0:c r="E55" s="1" t="n">
+        <ns0:v>3.896036561907814e+39</ns0:v>
+      </ns0:c>
+      <ns0:c r="F55" s="1" t="n">
+        <ns0:v>3.185772790859734e+27</ns0:v>
       </ns0:c>
       <ns0:c r="G55" s="1" t="n">
         <ns0:v>11.2</ns0:v>
       </ns0:c>
       <ns0:c r="H55" s="1" t="n">
-        <ns0:v>55.39</ns0:v>
+        <ns0:v>2.230475630375377</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="56">
@@ -2818,23 +2722,20 @@
           <ns0:t>{30531|0.100000,30532|0.200000,30533|0.300000,30534|0.400000,30535|0.500000,30536|0.600000,30537|0.700000,30538|0.800000,30539|0.900000}</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="D56" s="1">
-        <ns0:f>ROUND(D55*10,0)</ns0:f>
-        <ns0:v>1.1077372220037804e+48</ns0:v>
-      </ns0:c>
-      <ns0:c r="E56" s="1">
-        <ns0:f>D56</ns0:f>
-        <ns0:v>1.1077372220037804e+48</ns0:v>
-      </ns0:c>
-      <ns0:c r="F56" s="1">
-        <ns0:f>ROUND(F55*1.4,-5)</ns0:f>
-        <ns0:v>2.30259826223e+16</ns0:v>
+      <ns0:c r="D56" s="1" t="n">
+        <ns0:v>1.163350283727174e+40</ns0:v>
+      </ns0:c>
+      <ns0:c r="E56" s="1" t="n">
+        <ns0:v>1.163350283727174e+40</ns0:v>
+      </ns0:c>
+      <ns0:c r="F56" s="1" t="n">
+        <ns0:v>6.606018459126745e+27</ns0:v>
       </ns0:c>
       <ns0:c r="G56" s="1" t="n">
         <ns0:v>11.4</ns0:v>
       </ns0:c>
       <ns0:c r="H56" s="1" t="n">
-        <ns0:v>66.47</ns0:v>
+        <ns0:v>2.31330944921897</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="57">
@@ -2849,23 +2750,20 @@
           <ns0:t>{30541|0.100000,30542|0.200000,30543|0.300000,30544|0.400000,30545|0.500000,30546|0.600000,30547|0.700000,30548|0.800000,30549|0.900000}</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="D57" s="1">
-        <ns0:f>ROUND(D56*10,0)</ns0:f>
-        <ns0:v>1.1077372220037804e+49</ns0:v>
-      </ns0:c>
-      <ns0:c r="E57" s="1">
-        <ns0:f>D57</ns0:f>
-        <ns0:v>1.1077372220037804e+49</ns0:v>
-      </ns0:c>
-      <ns0:c r="F57" s="1">
-        <ns0:f>ROUND(F56*1.4,-5)</ns0:f>
-        <ns0:v>3.2236375671199996e+16</ns0:v>
+      <ns0:c r="D57" s="1" t="n">
+        <ns0:v>1.03725479862186e+41</ns0:v>
+      </ns0:c>
+      <ns0:c r="E57" s="1" t="n">
+        <ns0:v>1.03725479862186e+41</ns0:v>
+      </ns0:c>
+      <ns0:c r="F57" s="1" t="n">
+        <ns0:v>2.840467020862624e+28</ns0:v>
       </ns0:c>
       <ns0:c r="G57" s="1" t="n">
         <ns0:v>11.6</ns0:v>
       </ns0:c>
       <ns0:c r="H57" s="1" t="n">
-        <ns0:v>79.76000000000001</ns0:v>
+        <ns0:v>2.399219491559817</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="58">
@@ -2880,23 +2778,20 @@
           <ns0:t>{30551|0.100000,30552|0.200000,30553|0.300000,30554|0.400000,30555|0.500000,30556|0.600000,30557|0.700000,30558|0.800000,30559|0.900000}</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="D58" s="1">
-        <ns0:f>ROUND(D57*10,0)</ns0:f>
-        <ns0:v>1.1077372220037804e+50</ns0:v>
-      </ns0:c>
-      <ns0:c r="E58" s="1">
-        <ns0:f>D58</ns0:f>
-        <ns0:v>1.1077372220037804e+50</ns0:v>
-      </ns0:c>
-      <ns0:c r="F58" s="1">
-        <ns0:f>ROUND(F57*1.4,-5)</ns0:f>
-        <ns0:v>4.51309259397e+16</ns0:v>
+      <ns0:c r="D58" s="1" t="n">
+        <ns0:v>3.976585948930645e+42</ns0:v>
+      </ns0:c>
+      <ns0:c r="E58" s="1" t="n">
+        <ns0:v>3.976585948930645e+42</ns0:v>
+      </ns0:c>
+      <ns0:c r="F58" s="1" t="n">
+        <ns0:v>2.532588927796961e+29</ns0:v>
       </ns0:c>
       <ns0:c r="G58" s="1" t="n">
         <ns0:v>11.8</ns0:v>
       </ns0:c>
       <ns0:c r="H58" s="1" t="n">
-        <ns0:v>95.70999999999999</ns0:v>
+        <ns0:v>2.488319999999999</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="59">
@@ -2911,23 +2806,20 @@
           <ns0:t>{30561|0.100000,30562|0.200000,30563|0.300000,30564|0.400000,30565|0.500000,30566|0.600000,30567|0.700000,30568|0.800000,30569|0.900000}</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="D59" s="1">
-        <ns0:f>ROUND(D58*10,0)</ns0:f>
-        <ns0:v>1.1077372220037804e+51</ns0:v>
-      </ns0:c>
-      <ns0:c r="E59" s="1">
-        <ns0:f>D59</ns0:f>
-        <ns0:v>1.1077372220037804e+51</ns0:v>
-      </ns0:c>
-      <ns0:c r="F59" s="1">
-        <ns0:f>ROUND(F58*1.4,-5)</ns0:f>
-        <ns0:v>6.318329631559999e+16</ns0:v>
+      <ns0:c r="D59" s="1" t="n">
+        <ns0:v>1.187402201813172e+43</ns0:v>
+      </ns0:c>
+      <ns0:c r="E59" s="1" t="n">
+        <ns0:v>1.187402201813172e+43</ns0:v>
+      </ns0:c>
+      <ns0:c r="F59" s="1" t="n">
+        <ns0:v>5.251576400679779e+29</ns0:v>
       </ns0:c>
       <ns0:c r="G59" s="1" t="n">
         <ns0:v>12</ns0:v>
       </ns0:c>
       <ns0:c r="H59" s="1" t="n">
-        <ns0:v>114.85</ns0:v>
+        <ns0:v>2.580729459802168</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="60">
@@ -2942,23 +2834,20 @@
           <ns0:t>{30571|0.100000,30572|0.200000,30573|0.300000,30574|0.400000,30575|0.500000,30576|0.600000,30577|0.700000,30578|0.800000,30579|0.900000}</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="D60" s="1">
-        <ns0:f>ROUND(D59*10,0)</ns0:f>
-        <ns0:v>1.1077372220037804e+52</ns0:v>
-      </ns0:c>
-      <ns0:c r="E60" s="1">
-        <ns0:f>D60</ns0:f>
-        <ns0:v>1.1077372220037804e+52</ns0:v>
-      </ns0:c>
-      <ns0:c r="F60" s="1">
-        <ns0:f>ROUND(F59*1.4,-5)</ns0:f>
-        <ns0:v>8.84566148418e+16</ns0:v>
+      <ns0:c r="D60" s="1" t="n">
+        <ns0:v>3.545563976178901e+43</ns0:v>
+      </ns0:c>
+      <ns0:c r="E60" s="1" t="n">
+        <ns0:v>3.545563976178901e+43</ns0:v>
+      </ns0:c>
+      <ns0:c r="F60" s="1" t="n">
+        <ns0:v>1.088966882444959e+30</ns0:v>
       </ns0:c>
       <ns0:c r="G60" s="1" t="n">
         <ns0:v>12.2</ns0:v>
       </ns0:c>
       <ns0:c r="H60" s="1" t="n">
-        <ns0:v>137.82</ns0:v>
+        <ns0:v>2.676570756450452</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="61">
@@ -2973,23 +2862,20 @@
           <ns0:t>{30581|0.100000,30582|0.200000,30583|0.300000,30584|0.400000,30585|0.500000,30586|0.600000,30587|0.700000,30588|0.800000,30589|0.900000}</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="D61" s="1">
-        <ns0:f>ROUND(D60*10,0)</ns0:f>
-        <ns0:v>1.1077372220037804e+53</ns0:v>
-      </ns0:c>
-      <ns0:c r="E61" s="1">
-        <ns0:f>D61</ns0:f>
-        <ns0:v>1.1077372220037804e+53</ns0:v>
-      </ns0:c>
-      <ns0:c r="F61" s="1">
-        <ns0:f>ROUND(F60*1.4,-5)</ns0:f>
-        <ns0:v>1.2383926077849998e+17</ns0:v>
+      <ns0:c r="D61" s="1" t="n">
+        <ns0:v>1.058699730384658e+44</ns0:v>
+      </ns0:c>
+      <ns0:c r="E61" s="1" t="n">
+        <ns0:v>1.058699730384658e+44</ns0:v>
+      </ns0:c>
+      <ns0:c r="F61" s="1" t="n">
+        <ns0:v>2.258081727437866e+30</ns0:v>
       </ns0:c>
       <ns0:c r="G61" s="1" t="n">
         <ns0:v>12.4</ns0:v>
       </ns0:c>
       <ns0:c r="H61" s="1" t="n">
-        <ns0:v>165.38</ns0:v>
+        <ns0:v>2.775971339062764</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="62">
@@ -3004,23 +2890,20 @@
           <ns0:t>{30591|0.100000,30592|0.200000,30593|0.300000,30594|0.400000,30595|0.500000,30596|0.600000,30597|0.700000,30598|0.800000,30599|0.900000}</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="D62" s="1">
-        <ns0:f>ROUND(D61*10,0)</ns0:f>
-        <ns0:v>1.1077372220037804e+54</ns0:v>
-      </ns0:c>
-      <ns0:c r="E62" s="1">
-        <ns0:f>D62</ns0:f>
-        <ns0:v>1.1077372220037804e+54</ns0:v>
-      </ns0:c>
-      <ns0:c r="F62" s="1">
-        <ns0:f>ROUND(F61*1.4,-5)</ns0:f>
-        <ns0:v>1.733749650899e+17</ns0:v>
+      <ns0:c r="D62" s="1" t="n">
+        <ns0:v>9.43947314065115e+44</ns0:v>
+      </ns0:c>
+      <ns0:c r="E62" s="1" t="n">
+        <ns0:v>9.43947314065115e+44</ns0:v>
+      </ns0:c>
+      <ns0:c r="F62" s="1" t="n">
+        <ns0:v>9.709338108703431e+30</ns0:v>
       </ns0:c>
       <ns0:c r="G62" s="1" t="n">
         <ns0:v>12.6</ns0:v>
       </ns0:c>
       <ns0:c r="H62" s="1" t="n">
-        <ns0:v>198.46</ns0:v>
+        <ns0:v>2.87906338987178</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="63">
@@ -3035,23 +2918,20 @@
           <ns0:t>{30601|0.100000,30602|0.200000,30603|0.300000,30604|0.400000,30605|0.500000,30606|0.600000,30607|0.700000,30608|0.800000,30609|0.900000}</ns0:t>
         </ns0:is>
       </ns0:c>
-      <ns0:c r="D63" s="1">
-        <ns0:f>ROUND(D62*10,0)</ns0:f>
-        <ns0:v>1.1077372220037803e+55</ns0:v>
-      </ns0:c>
-      <ns0:c r="E63" s="1">
-        <ns0:f>D63</ns0:f>
-        <ns0:v>1.1077372220037803e+55</ns0:v>
-      </ns0:c>
-      <ns0:c r="F63" s="1">
-        <ns0:f>ROUND(F62*1.4,-5)</ns0:f>
-        <ns0:v>2.4272495112589997e+17</ns0:v>
+      <ns0:c r="D63" s="1" t="n">
+        <ns0:v>3.618867447641087e+46</ns0:v>
+      </ns0:c>
+      <ns0:c r="E63" s="1" t="n">
+        <ns0:v>3.618867447641087e+46</ns0:v>
+      </ns0:c>
+      <ns0:c r="F63" s="1" t="n">
+        <ns0:v>8.656943386327968e+31</ns0:v>
       </ns0:c>
       <ns0:c r="G63" s="1" t="n">
         <ns0:v>12.8</ns0:v>
       </ns0:c>
       <ns0:c r="H63" s="1" t="n">
-        <ns0:v>238.15</ns0:v>
+        <ns0:v>2.985983999999999</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="64">
@@ -3068,15 +2948,15 @@
       </ns0:c>
       <ns0:c r="D64" s="1">
         <ns0:f>ROUND(D63*10,0)</ns0:f>
-        <ns0:v>1.1077372220037803e+56</ns0:v>
+        <ns0:v>3.6188674476410877e+47</ns0:v>
       </ns0:c>
       <ns0:c r="E64" s="1">
         <ns0:f>D64</ns0:f>
-        <ns0:v>1.1077372220037803e+56</ns0:v>
+        <ns0:v>3.6188674476410877e+47</ns0:v>
       </ns0:c>
       <ns0:c r="F64" s="1">
         <ns0:f>ROUND(F63*1.4,-5)</ns0:f>
-        <ns0:v>3.3981493157629997e+17</ns0:v>
+        <ns0:v>1.2119720740859155e+32</ns0:v>
       </ns0:c>
       <ns0:c r="G64" s="1" t="n">
         <ns0:v>13</ns0:v>
@@ -3099,15 +2979,15 @@
       </ns0:c>
       <ns0:c r="D65" s="1">
         <ns0:f>ROUND(D64*10,0)</ns0:f>
-        <ns0:v>1.1077372220037802e+57</ns0:v>
+        <ns0:v>3.6188674476410873e+48</ns0:v>
       </ns0:c>
       <ns0:c r="E65" s="1">
         <ns0:f>D65</ns0:f>
-        <ns0:v>1.1077372220037802e+57</ns0:v>
+        <ns0:v>3.6188674476410873e+48</ns0:v>
       </ns0:c>
       <ns0:c r="F65" s="1">
         <ns0:f>ROUND(F64*1.4,-5)</ns0:f>
-        <ns0:v>4.7574090420679994e+17</ns0:v>
+        <ns0:v>1.6967609037202817e+32</ns0:v>
       </ns0:c>
       <ns0:c r="G65" s="1" t="n">
         <ns0:v>13.2</ns0:v>
@@ -3130,15 +3010,15 @@
       </ns0:c>
       <ns0:c r="D66" s="1">
         <ns0:f>ROUND(D65*10,0)</ns0:f>
-        <ns0:v>1.1077372220037802e+58</ns0:v>
+        <ns0:v>3.6188674476410876e+49</ns0:v>
       </ns0:c>
       <ns0:c r="E66" s="1">
         <ns0:f>D66</ns0:f>
-        <ns0:v>1.1077372220037802e+58</ns0:v>
+        <ns0:v>3.6188674476410876e+49</ns0:v>
       </ns0:c>
       <ns0:c r="F66" s="1">
         <ns0:f>ROUND(F65*1.4,-5)</ns0:f>
-        <ns0:v>6.660372658894999e+17</ns0:v>
+        <ns0:v>2.3754652652083943e+32</ns0:v>
       </ns0:c>
       <ns0:c r="G66" s="1" t="n">
         <ns0:v>13.4</ns0:v>
@@ -3161,15 +3041,15 @@
       </ns0:c>
       <ns0:c r="D67" s="1">
         <ns0:f>ROUND(D66*10,0)</ns0:f>
-        <ns0:v>1.1077372220037803e+59</ns0:v>
+        <ns0:v>3.6188674476410874e+50</ns0:v>
       </ns0:c>
       <ns0:c r="E67" s="1">
         <ns0:f>D67</ns0:f>
-        <ns0:v>1.1077372220037803e+59</ns0:v>
+        <ns0:v>3.6188674476410874e+50</ns0:v>
       </ns0:c>
       <ns0:c r="F67" s="1">
         <ns0:f>ROUND(F66*1.4,-5)</ns0:f>
-        <ns0:v>9.324521722453e+17</ns0:v>
+        <ns0:v>3.325651371291752e+32</ns0:v>
       </ns0:c>
       <ns0:c r="G67" s="1" t="n">
         <ns0:v>13.6</ns0:v>
@@ -3192,15 +3072,15 @@
       </ns0:c>
       <ns0:c r="D68" s="1">
         <ns0:f>ROUND(D67*10,0)</ns0:f>
-        <ns0:v>1.1077372220037803e+60</ns0:v>
+        <ns0:v>3.6188674476410876e+51</ns0:v>
       </ns0:c>
       <ns0:c r="E68" s="1">
         <ns0:f>D68</ns0:f>
-        <ns0:v>1.1077372220037803e+60</ns0:v>
+        <ns0:v>3.6188674476410876e+51</ns0:v>
       </ns0:c>
       <ns0:c r="F68" s="1">
         <ns0:f>ROUND(F67*1.4,-5)</ns0:f>
-        <ns0:v>1.3054330411434e+18</ns0:v>
+        <ns0:v>4.655911919808452e+32</ns0:v>
       </ns0:c>
       <ns0:c r="G68" s="1" t="n">
         <ns0:v>13.8</ns0:v>
@@ -3223,15 +3103,15 @@
       </ns0:c>
       <ns0:c r="D69" s="1">
         <ns0:f>ROUND(D68*10,0)</ns0:f>
-        <ns0:v>1.1077372220037802e+61</ns0:v>
+        <ns0:v>3.6188674476410876e+52</ns0:v>
       </ns0:c>
       <ns0:c r="E69" s="1">
         <ns0:f>D69</ns0:f>
-        <ns0:v>1.1077372220037802e+61</ns0:v>
+        <ns0:v>3.6188674476410876e+52</ns0:v>
       </ns0:c>
       <ns0:c r="F69" s="1">
         <ns0:f>ROUND(F68*1.4,-5)</ns0:f>
-        <ns0:v>1.8276062576007997e+18</ns0:v>
+        <ns0:v>6.518276687731834e+32</ns0:v>
       </ns0:c>
       <ns0:c r="G69" s="1" t="n">
         <ns0:v>14</ns0:v>
@@ -3254,15 +3134,15 @@
       </ns0:c>
       <ns0:c r="D70" s="1">
         <ns0:f>ROUND(D69*10,0)</ns0:f>
-        <ns0:v>1.1077372220037803e+62</ns0:v>
+        <ns0:v>3.6188674476410878e+53</ns0:v>
       </ns0:c>
       <ns0:c r="E70" s="1">
         <ns0:f>D70</ns0:f>
-        <ns0:v>1.1077372220037803e+62</ns0:v>
+        <ns0:v>3.6188674476410878e+53</ns0:v>
       </ns0:c>
       <ns0:c r="F70" s="1">
         <ns0:f>ROUND(F69*1.4,-5)</ns0:f>
-        <ns0:v>2.5586487606411e+18</ns0:v>
+        <ns0:v>9.125587362824566e+32</ns0:v>
       </ns0:c>
       <ns0:c r="G70" s="1" t="n">
         <ns0:v>14.2</ns0:v>
@@ -3285,15 +3165,15 @@
       </ns0:c>
       <ns0:c r="D71" s="1">
         <ns0:f>ROUND(D70*10,0)</ns0:f>
-        <ns0:v>1.1077372220037803e+63</ns0:v>
+        <ns0:v>3.6188674476410876e+54</ns0:v>
       </ns0:c>
       <ns0:c r="E71" s="1">
         <ns0:f>D71</ns0:f>
-        <ns0:v>1.1077372220037803e+63</ns0:v>
+        <ns0:v>3.6188674476410876e+54</ns0:v>
       </ns0:c>
       <ns0:c r="F71" s="1">
         <ns0:f>ROUND(F70*1.4,-5)</ns0:f>
-        <ns0:v>3.5821082648974996e+18</ns0:v>
+        <ns0:v>1.2775822307954391e+33</ns0:v>
       </ns0:c>
       <ns0:c r="G71" s="1" t="n">
         <ns0:v>14.4</ns0:v>
@@ -3316,15 +3196,15 @@
       </ns0:c>
       <ns0:c r="D72" s="1">
         <ns0:f>ROUND(D71*10,0)</ns0:f>
-        <ns0:v>1.1077372220037803e+64</ns0:v>
+        <ns0:v>3.6188674476410875e+55</ns0:v>
       </ns0:c>
       <ns0:c r="E72" s="1">
         <ns0:f>D72</ns0:f>
-        <ns0:v>1.1077372220037803e+64</ns0:v>
+        <ns0:v>3.6188674476410875e+55</ns0:v>
       </ns0:c>
       <ns0:c r="F72" s="1">
         <ns0:f>ROUND(F71*1.4,-5)</ns0:f>
-        <ns0:v>5.014951570856499e+18</ns0:v>
+        <ns0:v>1.7886151231136147e+33</ns0:v>
       </ns0:c>
       <ns0:c r="G72" s="1" t="n">
         <ns0:v>14.6</ns0:v>
@@ -3347,15 +3227,15 @@
       </ns0:c>
       <ns0:c r="D73" s="1">
         <ns0:f>ROUND(D72*10,0)</ns0:f>
-        <ns0:v>1.1077372220037803e+65</ns0:v>
+        <ns0:v>3.6188674476410876e+56</ns0:v>
       </ns0:c>
       <ns0:c r="E73" s="1">
         <ns0:f>D73</ns0:f>
-        <ns0:v>1.1077372220037803e+65</ns0:v>
+        <ns0:v>3.6188674476410876e+56</ns0:v>
       </ns0:c>
       <ns0:c r="F73" s="1">
         <ns0:f>ROUND(F72*1.4,-5)</ns0:f>
-        <ns0:v>7.0209321991991e+18</ns0:v>
+        <ns0:v>2.5040611723590604e+33</ns0:v>
       </ns0:c>
       <ns0:c r="G73" s="1" t="n">
         <ns0:v>14.8</ns0:v>
@@ -3378,15 +3258,15 @@
       </ns0:c>
       <ns0:c r="D74" s="1">
         <ns0:f>ROUND(D73*10,0)</ns0:f>
-        <ns0:v>1.1077372220037803e+66</ns0:v>
+        <ns0:v>3.6188674476410876e+57</ns0:v>
       </ns0:c>
       <ns0:c r="E74" s="1">
         <ns0:f>D74</ns0:f>
-        <ns0:v>1.1077372220037803e+66</ns0:v>
+        <ns0:v>3.6188674476410876e+57</ns0:v>
       </ns0:c>
       <ns0:c r="F74" s="1">
         <ns0:f>ROUND(F73*1.4,-5)</ns0:f>
-        <ns0:v>9.8293050788787e+18</ns0:v>
+        <ns0:v>3.5056856413026845e+33</ns0:v>
       </ns0:c>
       <ns0:c r="G74" s="1" t="n">
         <ns0:v>15</ns0:v>
@@ -3410,15 +3290,15 @@
       </ns0:c>
       <ns0:c r="D75" s="1">
         <ns0:f>ROUND(D74*10,0)</ns0:f>
-        <ns0:v>1.1077372220037803e+67</ns0:v>
+        <ns0:v>3.6188674476410877e+58</ns0:v>
       </ns0:c>
       <ns0:c r="E75" s="1">
         <ns0:f>D75</ns0:f>
-        <ns0:v>1.1077372220037803e+67</ns0:v>
+        <ns0:v>3.6188674476410877e+58</ns0:v>
       </ns0:c>
       <ns0:c r="F75" s="1">
         <ns0:f>ROUND(F74*1.4,-5)</ns0:f>
-        <ns0:v>1.37610271104302e+19</ns0:v>
+        <ns0:v>4.907959897823758e+33</ns0:v>
       </ns0:c>
       <ns0:c r="G75" s="1" t="n">
         <ns0:v>15.2</ns0:v>
@@ -3442,15 +3322,15 @@
       </ns0:c>
       <ns0:c r="D76" s="1">
         <ns0:f>ROUND(D75*10,0)</ns0:f>
-        <ns0:v>1.1077372220037802e+68</ns0:v>
+        <ns0:v>3.6188674476410875e+59</ns0:v>
       </ns0:c>
       <ns0:c r="E76" s="1">
         <ns0:f>D76</ns0:f>
-        <ns0:v>1.1077372220037802e+68</ns0:v>
+        <ns0:v>3.6188674476410875e+59</ns0:v>
       </ns0:c>
       <ns0:c r="F76" s="1">
         <ns0:f>ROUND(F75*1.4,-5)</ns0:f>
-        <ns0:v>1.92654379546023e+19</ns0:v>
+        <ns0:v>6.87114385695326e+33</ns0:v>
       </ns0:c>
       <ns0:c r="G76" s="1" t="n">
         <ns0:v>15.4</ns0:v>
@@ -3474,15 +3354,15 @@
       </ns0:c>
       <ns0:c r="D77" s="1">
         <ns0:f>ROUND(D76*10,0)</ns0:f>
-        <ns0:v>1.1077372220037801e+69</ns0:v>
+        <ns0:v>3.618867447641087e+60</ns0:v>
       </ns0:c>
       <ns0:c r="E77" s="1">
         <ns0:f>D77</ns0:f>
-        <ns0:v>1.1077372220037801e+69</ns0:v>
+        <ns0:v>3.618867447641087e+60</ns0:v>
       </ns0:c>
       <ns0:c r="F77" s="1">
         <ns0:f>ROUND(F76*1.4,-5)</ns0:f>
-        <ns0:v>2.69716131364432e+19</ns0:v>
+        <ns0:v>9.619601399734563e+33</ns0:v>
       </ns0:c>
       <ns0:c r="G77" s="1" t="n">
         <ns0:v>15.6</ns0:v>
@@ -3506,15 +3386,15 @@
       </ns0:c>
       <ns0:c r="D78" s="1">
         <ns0:f>ROUND(D77*10,0)</ns0:f>
-        <ns0:v>1.1077372220037801e+70</ns0:v>
+        <ns0:v>3.6188674476410876e+61</ns0:v>
       </ns0:c>
       <ns0:c r="E78" s="1">
         <ns0:f>D78</ns0:f>
-        <ns0:v>1.1077372220037801e+70</ns0:v>
+        <ns0:v>3.6188674476410876e+61</ns0:v>
       </ns0:c>
       <ns0:c r="F78" s="1">
         <ns0:f>ROUND(F77*1.4,-5)</ns0:f>
-        <ns0:v>3.7760258391020495e+19</ns0:v>
+        <ns0:v>1.3467441959628388e+34</ns0:v>
       </ns0:c>
       <ns0:c r="G78" s="1" t="n">
         <ns0:v>15.8</ns0:v>
@@ -3538,15 +3418,15 @@
       </ns0:c>
       <ns0:c r="D79" s="1">
         <ns0:f>ROUND(D78*10,0)</ns0:f>
-        <ns0:v>1.10773722200378e+71</ns0:v>
+        <ns0:v>3.618867447641088e+62</ns0:v>
       </ns0:c>
       <ns0:c r="E79" s="1">
         <ns0:f>D79</ns0:f>
-        <ns0:v>1.10773722200378e+71</ns0:v>
+        <ns0:v>3.618867447641088e+62</ns0:v>
       </ns0:c>
       <ns0:c r="F79" s="1">
         <ns0:f>ROUND(F78*1.4,-5)</ns0:f>
-        <ns0:v>5.28643617474287e+19</ns0:v>
+        <ns0:v>1.885441874347974e+34</ns0:v>
       </ns0:c>
       <ns0:c r="G79" s="1" t="n">
         <ns0:v>16</ns0:v>
@@ -3570,15 +3450,15 @@
       </ns0:c>
       <ns0:c r="D80" s="1">
         <ns0:f>ROUND(D79*10,0)</ns0:f>
-        <ns0:v>1.1077372220037801e+72</ns0:v>
+        <ns0:v>3.618867447641088e+63</ns0:v>
       </ns0:c>
       <ns0:c r="E80" s="1">
         <ns0:f>D80</ns0:f>
-        <ns0:v>1.1077372220037801e+72</ns0:v>
+        <ns0:v>3.618867447641088e+63</ns0:v>
       </ns0:c>
       <ns0:c r="F80" s="1">
         <ns0:f>ROUND(F79*1.4,-5)</ns0:f>
-        <ns0:v>7.40101064464002e+19</ns0:v>
+        <ns0:v>2.6396186240871637e+34</ns0:v>
       </ns0:c>
       <ns0:c r="G80" s="1" t="n">
         <ns0:v>16.2</ns0:v>
@@ -3602,15 +3482,15 @@
       </ns0:c>
       <ns0:c r="D81" s="1">
         <ns0:f>ROUND(D80*10,0)</ns0:f>
-        <ns0:v>1.10773722200378e+73</ns0:v>
+        <ns0:v>3.6188674476410876e+64</ns0:v>
       </ns0:c>
       <ns0:c r="E81" s="1">
         <ns0:f>D81</ns0:f>
-        <ns0:v>1.10773722200378e+73</ns0:v>
+        <ns0:v>3.6188674476410876e+64</ns0:v>
       </ns0:c>
       <ns0:c r="F81" s="1">
         <ns0:f>ROUND(F80*1.4,-5)</ns0:f>
-        <ns0:v>1.036141490249603e+20</ns0:v>
+        <ns0:v>3.6954660737220284e+34</ns0:v>
       </ns0:c>
       <ns0:c r="G81" s="1" t="n">
         <ns0:v>16.4</ns0:v>
@@ -3634,15 +3514,15 @@
       </ns0:c>
       <ns0:c r="D82" s="1">
         <ns0:f>ROUND(D81*10,0)</ns0:f>
-        <ns0:v>1.1077372220037801e+74</ns0:v>
+        <ns0:v>3.6188674476410874e+65</ns0:v>
       </ns0:c>
       <ns0:c r="E82" s="1">
         <ns0:f>D82</ns0:f>
-        <ns0:v>1.1077372220037801e+74</ns0:v>
+        <ns0:v>3.6188674476410874e+65</ns0:v>
       </ns0:c>
       <ns0:c r="F82" s="1">
         <ns0:f>ROUND(F81*1.4,-5)</ns0:f>
-        <ns0:v>1.4505980863494439e+20</ns0:v>
+        <ns0:v>5.173652503210839e+34</ns0:v>
       </ns0:c>
       <ns0:c r="G82" s="1" t="n">
         <ns0:v>16.6</ns0:v>
@@ -3666,15 +3546,15 @@
       </ns0:c>
       <ns0:c r="D83" s="1">
         <ns0:f>ROUND(D82*10,0)</ns0:f>
-        <ns0:v>1.10773722200378e+75</ns0:v>
+        <ns0:v>3.618867447641088e+66</ns0:v>
       </ns0:c>
       <ns0:c r="E83" s="1">
         <ns0:f>D83</ns0:f>
-        <ns0:v>1.10773722200378e+75</ns0:v>
+        <ns0:v>3.618867447641088e+66</ns0:v>
       </ns0:c>
       <ns0:c r="F83" s="1">
         <ns0:f>ROUND(F82*1.4,-5)</ns0:f>
-        <ns0:v>2.0308373208892218e+20</ns0:v>
+        <ns0:v>7.243113504495176e+34</ns0:v>
       </ns0:c>
       <ns0:c r="G83" s="1" t="n">
         <ns0:v>16.8</ns0:v>
@@ -3698,15 +3578,15 @@
       </ns0:c>
       <ns0:c r="D84" s="1">
         <ns0:f>ROUND(D83*20,2-INT(LOG10(ABS(D83*20))))</ns0:f>
-        <ns0:v>2.2200000000000002e+76</ns0:v>
+        <ns0:v>7.24e+67</ns0:v>
       </ns0:c>
       <ns0:c r="E84" s="1">
         <ns0:f>D84</ns0:f>
-        <ns0:v>2.2200000000000002e+76</ns0:v>
+        <ns0:v>7.24e+67</ns0:v>
       </ns0:c>
       <ns0:c r="F84" s="1">
         <ns0:f>ROUND(F83*1.4,-5)</ns0:f>
-        <ns0:v>2.843172249244911e+20</ns0:v>
+        <ns0:v>1.0140358906293245e+35</ns0:v>
       </ns0:c>
       <ns0:c r="G84" s="1" t="n">
         <ns0:v>17</ns0:v>
@@ -3730,15 +3610,15 @@
       </ns0:c>
       <ns0:c r="D85" s="1">
         <ns0:f>ROUND(D84*20,2-INT(LOG10(ABS(D84*20))))</ns0:f>
-        <ns0:v>4.44e+77</ns0:v>
+        <ns0:v>1.4500000000000001e+69</ns0:v>
       </ns0:c>
       <ns0:c r="E85" s="1">
         <ns0:f>D85</ns0:f>
-        <ns0:v>4.44e+77</ns0:v>
+        <ns0:v>1.4500000000000001e+69</ns0:v>
       </ns0:c>
       <ns0:c r="F85" s="1">
         <ns0:f>ROUND(F84*1.4,-5)</ns0:f>
-        <ns0:v>3.980441148942875e+20</ns0:v>
+        <ns0:v>1.4196502468810543e+35</ns0:v>
       </ns0:c>
       <ns0:c r="G85" s="1" t="n">
         <ns0:v>17.2</ns0:v>
@@ -3762,15 +3642,15 @@
       </ns0:c>
       <ns0:c r="D86" s="1">
         <ns0:f>ROUND(D85*20,2-INT(LOG10(ABS(D85*20))))</ns0:f>
-        <ns0:v>8.88e+78</ns0:v>
+        <ns0:v>2.9e+70</ns0:v>
       </ns0:c>
       <ns0:c r="E86" s="1">
         <ns0:f>D86</ns0:f>
-        <ns0:v>8.88e+78</ns0:v>
+        <ns0:v>2.9e+70</ns0:v>
       </ns0:c>
       <ns0:c r="F86" s="1">
         <ns0:f>ROUND(F85*1.4,-5)</ns0:f>
-        <ns0:v>5.5726176085200254e+20</ns0:v>
+        <ns0:v>1.987510345633476e+35</ns0:v>
       </ns0:c>
       <ns0:c r="G86" s="1" t="n">
         <ns0:v>17.4</ns0:v>
@@ -3794,15 +3674,15 @@
       </ns0:c>
       <ns0:c r="D87" s="1">
         <ns0:f>ROUND(D86*20,2-INT(LOG10(ABS(D86*20))))</ns0:f>
-        <ns0:v>1.78e+80</ns0:v>
+        <ns0:v>5.8e+71</ns0:v>
       </ns0:c>
       <ns0:c r="E87" s="1">
         <ns0:f>D87</ns0:f>
-        <ns0:v>1.78e+80</ns0:v>
+        <ns0:v>5.8e+71</ns0:v>
       </ns0:c>
       <ns0:c r="F87" s="1">
         <ns0:f>ROUND(F86*1.4,-5)</ns0:f>
-        <ns0:v>7.801664651928036e+20</ns0:v>
+        <ns0:v>2.782514483886866e+35</ns0:v>
       </ns0:c>
       <ns0:c r="G87" s="1" t="n">
         <ns0:v>17.6</ns0:v>
@@ -3826,15 +3706,15 @@
       </ns0:c>
       <ns0:c r="D88" s="1">
         <ns0:f>ROUND(D87*20,2-INT(LOG10(ABS(D87*20))))</ns0:f>
-        <ns0:v>3.56e+81</ns0:v>
+        <ns0:v>1.16e+73</ns0:v>
       </ns0:c>
       <ns0:c r="E88" s="1">
         <ns0:f>D88</ns0:f>
-        <ns0:v>3.56e+81</ns0:v>
+        <ns0:v>1.16e+73</ns0:v>
       </ns0:c>
       <ns0:c r="F88" s="1">
         <ns0:f>ROUND(F87*1.4,-5)</ns0:f>
-        <ns0:v>1.0922330512699249e+21</ns0:v>
+        <ns0:v>3.8955202774416125e+35</ns0:v>
       </ns0:c>
       <ns0:c r="G88" s="1" t="n">
         <ns0:v>17.8</ns0:v>
@@ -3858,15 +3738,15 @@
       </ns0:c>
       <ns0:c r="D89" s="1">
         <ns0:f>ROUND(D88*20,2-INT(LOG10(ABS(D88*20))))</ns0:f>
-        <ns0:v>7.12e+82</ns0:v>
+        <ns0:v>2.32e+74</ns0:v>
       </ns0:c>
       <ns0:c r="E89" s="1">
         <ns0:f>D89</ns0:f>
-        <ns0:v>7.12e+82</ns0:v>
+        <ns0:v>2.32e+74</ns0:v>
       </ns0:c>
       <ns0:c r="F89" s="1">
         <ns0:f>ROUND(F88*1.4,-5)</ns0:f>
-        <ns0:v>1.5291262717778948e+21</ns0:v>
+        <ns0:v>5.453728388418258e+35</ns0:v>
       </ns0:c>
       <ns0:c r="G89" s="1" t="n">
         <ns0:v>18</ns0:v>
@@ -3890,15 +3770,15 @@
       </ns0:c>
       <ns0:c r="D90" s="1">
         <ns0:f>ROUND(D89*20,2-INT(LOG10(ABS(D89*20))))</ns0:f>
-        <ns0:v>1.42e+84</ns0:v>
+        <ns0:v>4.64e+75</ns0:v>
       </ns0:c>
       <ns0:c r="E90" s="1">
         <ns0:f>D90</ns0:f>
-        <ns0:v>1.42e+84</ns0:v>
+        <ns0:v>4.64e+75</ns0:v>
       </ns0:c>
       <ns0:c r="F90" s="1">
         <ns0:f>ROUND(F89*1.4,-5)</ns0:f>
-        <ns0:v>2.1407767804890527e+21</ns0:v>
+        <ns0:v>7.635219743785561e+35</ns0:v>
       </ns0:c>
       <ns0:c r="G90" s="1" t="n">
         <ns0:v>18.2</ns0:v>
@@ -3922,15 +3802,15 @@
       </ns0:c>
       <ns0:c r="D91" s="1">
         <ns0:f>ROUND(D90*20,2-INT(LOG10(ABS(D90*20))))</ns0:f>
-        <ns0:v>2.84e+85</ns0:v>
+        <ns0:v>9.280000000000001e+76</ns0:v>
       </ns0:c>
       <ns0:c r="E91" s="1">
         <ns0:f>D91</ns0:f>
-        <ns0:v>2.84e+85</ns0:v>
+        <ns0:v>9.280000000000001e+76</ns0:v>
       </ns0:c>
       <ns0:c r="F91" s="1">
         <ns0:f>ROUND(F90*1.4,-5)</ns0:f>
-        <ns0:v>2.9970874926846737e+21</ns0:v>
+        <ns0:v>1.0689307641299785e+36</ns0:v>
       </ns0:c>
       <ns0:c r="G91" s="1" t="n">
         <ns0:v>18.4</ns0:v>
@@ -3954,15 +3834,15 @@
       </ns0:c>
       <ns0:c r="D92" s="1">
         <ns0:f>ROUND(D91*20,2-INT(LOG10(ABS(D91*20))))</ns0:f>
-        <ns0:v>5.679999999999999e+86</ns0:v>
+        <ns0:v>1.86e+78</ns0:v>
       </ns0:c>
       <ns0:c r="E92" s="1">
         <ns0:f>D92</ns0:f>
-        <ns0:v>5.679999999999999e+86</ns0:v>
+        <ns0:v>1.86e+78</ns0:v>
       </ns0:c>
       <ns0:c r="F92" s="1">
         <ns0:f>ROUND(F91*1.4,-5)</ns0:f>
-        <ns0:v>4.195922489758543e+21</ns0:v>
+        <ns0:v>1.4965030697819698e+36</ns0:v>
       </ns0:c>
       <ns0:c r="G92" s="1" t="n">
         <ns0:v>18.6</ns0:v>
@@ -3986,15 +3866,15 @@
       </ns0:c>
       <ns0:c r="D93" s="1">
         <ns0:f>ROUND(D92*20,2-INT(LOG10(ABS(D92*20))))</ns0:f>
-        <ns0:v>1.1399999999999999e+88</ns0:v>
+        <ns0:v>3.7200000000000005e+79</ns0:v>
       </ns0:c>
       <ns0:c r="E93" s="1">
         <ns0:f>D93</ns0:f>
-        <ns0:v>1.1399999999999999e+88</ns0:v>
+        <ns0:v>3.7200000000000005e+79</ns0:v>
       </ns0:c>
       <ns0:c r="F93" s="1">
         <ns0:f>ROUND(F92*1.4,-5)</ns0:f>
-        <ns0:v>5.87429148566196e+21</ns0:v>
+        <ns0:v>2.0951042976947578e+36</ns0:v>
       </ns0:c>
       <ns0:c r="G93" s="1" t="n">
         <ns0:v>18.8</ns0:v>
@@ -4018,15 +3898,15 @@
       </ns0:c>
       <ns0:c r="D94" s="1">
         <ns0:f>ROUND(D93*20,2-INT(LOG10(ABS(D93*20))))</ns0:f>
-        <ns0:v>2.28e+89</ns0:v>
+        <ns0:v>7.44e+80</ns0:v>
       </ns0:c>
       <ns0:c r="E94" s="1">
         <ns0:f>D94</ns0:f>
-        <ns0:v>2.28e+89</ns0:v>
+        <ns0:v>7.44e+80</ns0:v>
       </ns0:c>
       <ns0:c r="F94" s="1">
         <ns0:f>ROUND(F93*1.4,-5)</ns0:f>
-        <ns0:v>8.224008079926744e+21</ns0:v>
+        <ns0:v>2.933146016772661e+36</ns0:v>
       </ns0:c>
       <ns0:c r="G94" s="1" t="n">
         <ns0:v>19</ns0:v>
@@ -4050,15 +3930,15 @@
       </ns0:c>
       <ns0:c r="D95" s="1">
         <ns0:f>ROUND(D94*20,2-INT(LOG10(ABS(D94*20))))</ns0:f>
-        <ns0:v>4.5600000000000005e+90</ns0:v>
+        <ns0:v>1.49e+82</ns0:v>
       </ns0:c>
       <ns0:c r="E95" s="1">
         <ns0:f>D95</ns0:f>
-        <ns0:v>4.5600000000000005e+90</ns0:v>
+        <ns0:v>1.49e+82</ns0:v>
       </ns0:c>
       <ns0:c r="F95" s="1">
         <ns0:f>ROUND(F94*1.4,-5)</ns0:f>
-        <ns0:v>1.151361131189744e+22</ns0:v>
+        <ns0:v>4.106404423481725e+36</ns0:v>
       </ns0:c>
       <ns0:c r="G95" s="1" t="n">
         <ns0:v>19.2</ns0:v>
@@ -4082,15 +3962,15 @@
       </ns0:c>
       <ns0:c r="D96" s="1">
         <ns0:f>ROUND(D95*20,2-INT(LOG10(ABS(D95*20))))</ns0:f>
-        <ns0:v>9.12e+91</ns0:v>
+        <ns0:v>2.98e+83</ns0:v>
       </ns0:c>
       <ns0:c r="E96" s="1">
         <ns0:f>D96</ns0:f>
-        <ns0:v>9.12e+91</ns0:v>
+        <ns0:v>2.98e+83</ns0:v>
       </ns0:c>
       <ns0:c r="F96" s="1">
         <ns0:f>ROUND(F95*1.4,-5)</ns0:f>
-        <ns0:v>1.6119055836656414e+22</ns0:v>
+        <ns0:v>5.748966192874415e+36</ns0:v>
       </ns0:c>
       <ns0:c r="G96" s="1" t="n">
         <ns0:v>19.4</ns0:v>
@@ -4114,15 +3994,15 @@
       </ns0:c>
       <ns0:c r="D97" s="1">
         <ns0:f>ROUND(D96*20,2-INT(LOG10(ABS(D96*20))))</ns0:f>
-        <ns0:v>1.8199999999999999e+93</ns0:v>
+        <ns0:v>5.960000000000001e+84</ns0:v>
       </ns0:c>
       <ns0:c r="E97" s="1">
         <ns0:f>D97</ns0:f>
-        <ns0:v>1.8199999999999999e+93</ns0:v>
+        <ns0:v>5.960000000000001e+84</ns0:v>
       </ns0:c>
       <ns0:c r="F97" s="1">
         <ns0:f>ROUND(F96*1.4,-5)</ns0:f>
-        <ns0:v>2.256667817131898e+22</ns0:v>
+        <ns0:v>8.048552670024181e+36</ns0:v>
       </ns0:c>
       <ns0:c r="G97" s="1" t="n">
         <ns0:v>19.6</ns0:v>
@@ -4146,15 +4026,15 @@
       </ns0:c>
       <ns0:c r="D98" s="1">
         <ns0:f>ROUND(D97*20,2-INT(LOG10(ABS(D97*20))))</ns0:f>
-        <ns0:v>3.64e+94</ns0:v>
+        <ns0:v>1.19e+86</ns0:v>
       </ns0:c>
       <ns0:c r="E98" s="1">
         <ns0:f>D98</ns0:f>
-        <ns0:v>3.64e+94</ns0:v>
+        <ns0:v>1.19e+86</ns0:v>
       </ns0:c>
       <ns0:c r="F98" s="1">
         <ns0:f>ROUND(F97*1.4,-5)</ns0:f>
-        <ns0:v>3.159334943984657e+22</ns0:v>
+        <ns0:v>1.1267973738033853e+37</ns0:v>
       </ns0:c>
       <ns0:c r="G98" s="1" t="n">
         <ns0:v>19.8</ns0:v>
@@ -4178,15 +4058,15 @@
       </ns0:c>
       <ns0:c r="D99" s="1">
         <ns0:f>ROUND(D98*20,2-INT(LOG10(ABS(D98*20))))</ns0:f>
-        <ns0:v>7.28e+95</ns0:v>
+        <ns0:v>2.38e+87</ns0:v>
       </ns0:c>
       <ns0:c r="E99" s="1">
         <ns0:f>D99</ns0:f>
-        <ns0:v>7.28e+95</ns0:v>
+        <ns0:v>2.38e+87</ns0:v>
       </ns0:c>
       <ns0:c r="F99" s="1">
         <ns0:f>ROUND(F98*1.4,-5)</ns0:f>
-        <ns0:v>4.4230689215785195e+22</ns0:v>
+        <ns0:v>1.5775163233247394e+37</ns0:v>
       </ns0:c>
       <ns0:c r="G99" s="1" t="n">
         <ns0:v>20</ns0:v>
@@ -4210,15 +4090,15 @@
       </ns0:c>
       <ns0:c r="D100" s="1">
         <ns0:f>ROUND(D99*20,2-INT(LOG10(ABS(D99*20))))</ns0:f>
-        <ns0:v>1.46e+97</ns0:v>
+        <ns0:v>4.76e+88</ns0:v>
       </ns0:c>
       <ns0:c r="E100" s="1">
         <ns0:f>D100</ns0:f>
-        <ns0:v>1.46e+97</ns0:v>
+        <ns0:v>4.76e+88</ns0:v>
       </ns0:c>
       <ns0:c r="F100" s="1">
         <ns0:f>ROUND(F99*1.4,-5)</ns0:f>
-        <ns0:v>6.192296490209927e+22</ns0:v>
+        <ns0:v>2.208522852654635e+37</ns0:v>
       </ns0:c>
       <ns0:c r="G100" s="1" t="n">
         <ns0:v>20.2</ns0:v>
@@ -4242,15 +4122,15 @@
       </ns0:c>
       <ns0:c r="D101" s="1">
         <ns0:f>ROUND(D100*20,2-INT(LOG10(ABS(D100*20))))</ns0:f>
-        <ns0:v>2.9200000000000005e+98</ns0:v>
+        <ns0:v>9.52e+89</ns0:v>
       </ns0:c>
       <ns0:c r="E101" s="1">
         <ns0:f>D101</ns0:f>
-        <ns0:v>2.9200000000000005e+98</ns0:v>
+        <ns0:v>9.52e+89</ns0:v>
       </ns0:c>
       <ns0:c r="F101" s="1">
         <ns0:f>ROUND(F100*1.4,-5)</ns0:f>
-        <ns0:v>8.669215086293898e+22</ns0:v>
+        <ns0:v>3.091931993716489e+37</ns0:v>
       </ns0:c>
       <ns0:c r="G101" s="1" t="n">
         <ns0:v>20.4</ns0:v>
@@ -4274,15 +4154,15 @@
       </ns0:c>
       <ns0:c r="D102" s="1">
         <ns0:f>ROUND(D101*20,2-INT(LOG10(ABS(D101*20))))</ns0:f>
-        <ns0:v>5.84e+99</ns0:v>
+        <ns0:v>1.9e+91</ns0:v>
       </ns0:c>
       <ns0:c r="E102" s="1">
         <ns0:f>D102</ns0:f>
-        <ns0:v>5.84e+99</ns0:v>
+        <ns0:v>1.9e+91</ns0:v>
       </ns0:c>
       <ns0:c r="F102" s="1">
         <ns0:f>ROUND(F101*1.4,-5)</ns0:f>
-        <ns0:v>1.2136901120811458e+23</ns0:v>
+        <ns0:v>4.328704791203084e+37</ns0:v>
       </ns0:c>
       <ns0:c r="G102" s="1" t="n">
         <ns0:v>20.6</ns0:v>
@@ -4306,15 +4186,15 @@
       </ns0:c>
       <ns0:c r="D103" s="1">
         <ns0:f>ROUND(D102*20,2-INT(LOG10(ABS(D102*20))))</ns0:f>
-        <ns0:v>1.17e+101</ns0:v>
+        <ns0:v>3.8e+92</ns0:v>
       </ns0:c>
       <ns0:c r="E103" s="1">
         <ns0:f>D103</ns0:f>
-        <ns0:v>1.17e+101</ns0:v>
+        <ns0:v>3.8e+92</ns0:v>
       </ns0:c>
       <ns0:c r="F103" s="1">
         <ns0:f>ROUND(F102*1.4,-5)</ns0:f>
-        <ns0:v>1.699166156913604e+23</ns0:v>
+        <ns0:v>6.060186707684317e+37</ns0:v>
       </ns0:c>
       <ns0:c r="G103" s="1" t="n">
         <ns0:v>20.8</ns0:v>
@@ -4338,15 +4218,15 @@
       </ns0:c>
       <ns0:c r="D104" s="1">
         <ns0:f>ROUND(D103*20,2-INT(LOG10(ABS(D103*20))))</ns0:f>
-        <ns0:v>2.34e+102</ns0:v>
+        <ns0:v>7.6e+93</ns0:v>
       </ns0:c>
       <ns0:c r="E104" s="1">
         <ns0:f>D104</ns0:f>
-        <ns0:v>2.34e+102</ns0:v>
+        <ns0:v>7.6e+93</ns0:v>
       </ns0:c>
       <ns0:c r="F104" s="1">
         <ns0:f>ROUND(F103*1.4,-5)</ns0:f>
-        <ns0:v>2.3788326196790453e+23</ns0:v>
+        <ns0:v>8.484261390758044e+37</ns0:v>
       </ns0:c>
       <ns0:c r="G104" s="1" t="n">
         <ns0:v>21</ns0:v>
@@ -4370,15 +4250,15 @@
       </ns0:c>
       <ns0:c r="D105" s="1">
         <ns0:f>ROUND(D104*20,2-INT(LOG10(ABS(D104*20))))</ns0:f>
-        <ns0:v>4.68e+103</ns0:v>
+        <ns0:v>1.5200000000000001e+95</ns0:v>
       </ns0:c>
       <ns0:c r="E105" s="1">
         <ns0:f>D105</ns0:f>
-        <ns0:v>4.68e+103</ns0:v>
+        <ns0:v>1.5200000000000001e+95</ns0:v>
       </ns0:c>
       <ns0:c r="F105" s="1">
         <ns0:f>ROUND(F104*1.4,-5)</ns0:f>
-        <ns0:v>3.3303656675506634e+23</ns0:v>
+        <ns0:v>1.1877965947061261e+38</ns0:v>
       </ns0:c>
       <ns0:c r="G105" s="1" t="n">
         <ns0:v>21.2</ns0:v>
@@ -4402,15 +4282,15 @@
       </ns0:c>
       <ns0:c r="D106" s="1">
         <ns0:f>ROUND(D105*20,2-INT(LOG10(ABS(D105*20))))</ns0:f>
-        <ns0:v>9.360000000000001e+104</ns0:v>
+        <ns0:v>3.04e+96</ns0:v>
       </ns0:c>
       <ns0:c r="E106" s="1">
         <ns0:f>D106</ns0:f>
-        <ns0:v>9.360000000000001e+104</ns0:v>
+        <ns0:v>3.04e+96</ns0:v>
       </ns0:c>
       <ns0:c r="F106" s="1">
         <ns0:f>ROUND(F105*1.4,-5)</ns0:f>
-        <ns0:v>4.662511934570929e+23</ns0:v>
+        <ns0:v>1.6629152325885765e+38</ns0:v>
       </ns0:c>
       <ns0:c r="G106" s="1" t="n">
         <ns0:v>21.4</ns0:v>
@@ -4434,15 +4314,15 @@
       </ns0:c>
       <ns0:c r="D107" s="1">
         <ns0:f>ROUND(D106*20,2-INT(LOG10(ABS(D106*20))))</ns0:f>
-        <ns0:v>1.8700000000000003e+106</ns0:v>
+        <ns0:v>6.08e+97</ns0:v>
       </ns0:c>
       <ns0:c r="E107" s="1">
         <ns0:f>D107</ns0:f>
-        <ns0:v>1.8700000000000003e+106</ns0:v>
+        <ns0:v>6.08e+97</ns0:v>
       </ns0:c>
       <ns0:c r="F107" s="1">
         <ns0:f>ROUND(F106*1.4,-5)</ns0:f>
-        <ns0:v>6.5275167083993e+23</ns0:v>
+        <ns0:v>2.328081325624007e+38</ns0:v>
       </ns0:c>
       <ns0:c r="G107" s="1" t="n">
         <ns0:v>21.6</ns0:v>
@@ -4466,15 +4346,15 @@
       </ns0:c>
       <ns0:c r="D108" s="1">
         <ns0:f>ROUND(D107*20,2-INT(LOG10(ABS(D107*20))))</ns0:f>
-        <ns0:v>3.74e+107</ns0:v>
+        <ns0:v>1.22e+99</ns0:v>
       </ns0:c>
       <ns0:c r="E108" s="1">
         <ns0:f>D108</ns0:f>
-        <ns0:v>3.74e+107</ns0:v>
+        <ns0:v>1.22e+99</ns0:v>
       </ns0:c>
       <ns0:c r="F108" s="1">
         <ns0:f>ROUND(F107*1.4,-5)</ns0:f>
-        <ns0:v>9.138523391759019e+23</ns0:v>
+        <ns0:v>3.25931385587361e+38</ns0:v>
       </ns0:c>
       <ns0:c r="G108" s="1" t="n">
         <ns0:v>21.8</ns0:v>
@@ -4498,15 +4378,15 @@
       </ns0:c>
       <ns0:c r="D109" s="1">
         <ns0:f>ROUND(D108*20,2-INT(LOG10(ABS(D108*20))))</ns0:f>
-        <ns0:v>7.480000000000001e+108</ns0:v>
+        <ns0:v>2.4400000000000003e+100</ns0:v>
       </ns0:c>
       <ns0:c r="E109" s="1">
         <ns0:f>D109</ns0:f>
-        <ns0:v>7.480000000000001e+108</ns0:v>
+        <ns0:v>2.4400000000000003e+100</ns0:v>
       </ns0:c>
       <ns0:c r="F109" s="1">
         <ns0:f>ROUND(F108*1.4,-5)</ns0:f>
-        <ns0:v>1.2793932748462625e+24</ns0:v>
+        <ns0:v>4.563039398223054e+38</ns0:v>
       </ns0:c>
       <ns0:c r="G109" s="1" t="n">
         <ns0:v>22</ns0:v>
@@ -4530,15 +4410,15 @@
       </ns0:c>
       <ns0:c r="D110" s="1">
         <ns0:f>ROUND(D109*20,2-INT(LOG10(ABS(D109*20))))</ns0:f>
-        <ns0:v>1.4999999999999999e+110</ns0:v>
+        <ns0:v>4.88e+101</ns0:v>
       </ns0:c>
       <ns0:c r="E110" s="1">
         <ns0:f>D110</ns0:f>
-        <ns0:v>1.4999999999999999e+110</ns0:v>
+        <ns0:v>4.88e+101</ns0:v>
       </ns0:c>
       <ns0:c r="F110" s="1">
         <ns0:f>ROUND(F109*1.4,-5)</ns0:f>
-        <ns0:v>1.7911505847847674e+24</ns0:v>
+        <ns0:v>6.388255157512275e+38</ns0:v>
       </ns0:c>
       <ns0:c r="G110" s="1" t="n">
         <ns0:v>22.2</ns0:v>
@@ -4562,15 +4442,15 @@
       </ns0:c>
       <ns0:c r="D111" s="1">
         <ns0:f>ROUND(D110*20,2-INT(LOG10(ABS(D110*20))))</ns0:f>
-        <ns0:v>3e+111</ns0:v>
+        <ns0:v>9.76e+102</ns0:v>
       </ns0:c>
       <ns0:c r="E111" s="1">
         <ns0:f>D111</ns0:f>
-        <ns0:v>3e+111</ns0:v>
+        <ns0:v>9.76e+102</ns0:v>
       </ns0:c>
       <ns0:c r="F111" s="1">
         <ns0:f>ROUND(F110*1.4,-5)</ns0:f>
-        <ns0:v>2.507610818698674e+24</ns0:v>
+        <ns0:v>8.943557220517185e+38</ns0:v>
       </ns0:c>
       <ns0:c r="G111" s="1" t="n">
         <ns0:v>22.4</ns0:v>
@@ -4594,15 +4474,15 @@
       </ns0:c>
       <ns0:c r="D112" s="1">
         <ns0:f>ROUND(D111*20,2-INT(LOG10(ABS(D111*20))))</ns0:f>
-        <ns0:v>6e+112</ns0:v>
+        <ns0:v>1.95e+104</ns0:v>
       </ns0:c>
       <ns0:c r="E112" s="1">
         <ns0:f>D112</ns0:f>
-        <ns0:v>6e+112</ns0:v>
+        <ns0:v>1.95e+104</ns0:v>
       </ns0:c>
       <ns0:c r="F112" s="1">
         <ns0:f>ROUND(F111*1.4,-5)</ns0:f>
-        <ns0:v>3.5106551461781433e+24</ns0:v>
+        <ns0:v>1.2520980108724058e+39</ns0:v>
       </ns0:c>
       <ns0:c r="G112" s="1" t="n">
         <ns0:v>22.6</ns0:v>
@@ -4626,15 +4506,15 @@
       </ns0:c>
       <ns0:c r="D113" s="1">
         <ns0:f>ROUND(D112*20,2-INT(LOG10(ABS(D112*20))))</ns0:f>
-        <ns0:v>1.2e+114</ns0:v>
+        <ns0:v>3.9000000000000003e+105</ns0:v>
       </ns0:c>
       <ns0:c r="E113" s="1">
         <ns0:f>D113</ns0:f>
-        <ns0:v>1.2e+114</ns0:v>
+        <ns0:v>3.9000000000000003e+105</ns0:v>
       </ns0:c>
       <ns0:c r="F113" s="1">
         <ns0:f>ROUND(F112*1.4,-5)</ns0:f>
-        <ns0:v>4.9149172046494e+24</ns0:v>
+        <ns0:v>1.752937215221368e+39</ns0:v>
       </ns0:c>
       <ns0:c r="G113" s="1" t="n">
         <ns0:v>22.8</ns0:v>
@@ -4658,15 +4538,15 @@
       </ns0:c>
       <ns0:c r="D114" s="1">
         <ns0:f>ROUND(D113*20,2-INT(LOG10(ABS(D113*20))))</ns0:f>
-        <ns0:v>2.4e+115</ns0:v>
+        <ns0:v>7.800000000000001e+106</ns0:v>
       </ns0:c>
       <ns0:c r="E114" s="1">
         <ns0:f>D114</ns0:f>
-        <ns0:v>2.4e+115</ns0:v>
+        <ns0:v>7.800000000000001e+106</ns0:v>
       </ns0:c>
       <ns0:c r="F114" s="1">
         <ns0:f>ROUND(F113*1.4,-5)</ns0:f>
-        <ns0:v>6.88088408650916e+24</ns0:v>
+        <ns0:v>2.454112101309915e+39</ns0:v>
       </ns0:c>
       <ns0:c r="G114" s="1" t="n">
         <ns0:v>23</ns0:v>
@@ -4690,15 +4570,15 @@
       </ns0:c>
       <ns0:c r="D115" s="1">
         <ns0:f>ROUND(D114*20,2-INT(LOG10(ABS(D114*20))))</ns0:f>
-        <ns0:v>4.8e+116</ns0:v>
+        <ns0:v>1.5600000000000002e+108</ns0:v>
       </ns0:c>
       <ns0:c r="E115" s="1">
         <ns0:f>D115</ns0:f>
-        <ns0:v>4.8e+116</ns0:v>
+        <ns0:v>1.5600000000000002e+108</ns0:v>
       </ns0:c>
       <ns0:c r="F115" s="1">
         <ns0:f>ROUND(F114*1.4,-5)</ns0:f>
-        <ns0:v>9.633237721112824e+24</ns0:v>
+        <ns0:v>3.4357569418338807e+39</ns0:v>
       </ns0:c>
       <ns0:c r="G115" s="1" t="n">
         <ns0:v>23.2</ns0:v>
@@ -4722,15 +4602,15 @@
       </ns0:c>
       <ns0:c r="D116" s="1">
         <ns0:f>ROUND(D115*20,2-INT(LOG10(ABS(D115*20))))</ns0:f>
-        <ns0:v>9.6e+117</ns0:v>
+        <ns0:v>3.12e+109</ns0:v>
       </ns0:c>
       <ns0:c r="E116" s="1">
         <ns0:f>D116</ns0:f>
-        <ns0:v>9.6e+117</ns0:v>
+        <ns0:v>3.12e+109</ns0:v>
       </ns0:c>
       <ns0:c r="F116" s="1">
         <ns0:f>ROUND(F115*1.4,-5)</ns0:f>
-        <ns0:v>1.3486532809557953e+25</ns0:v>
+        <ns0:v>4.810059718567433e+39</ns0:v>
       </ns0:c>
       <ns0:c r="G116" s="1" t="n">
         <ns0:v>23.4</ns0:v>
@@ -4754,15 +4634,15 @@
       </ns0:c>
       <ns0:c r="D117" s="1">
         <ns0:f>ROUND(D116*20,2-INT(LOG10(ABS(D116*20))))</ns0:f>
-        <ns0:v>1.92e+119</ns0:v>
+        <ns0:v>6.24e+110</ns0:v>
       </ns0:c>
       <ns0:c r="E117" s="1">
         <ns0:f>D117</ns0:f>
-        <ns0:v>1.92e+119</ns0:v>
+        <ns0:v>6.24e+110</ns0:v>
       </ns0:c>
       <ns0:c r="F117" s="1">
         <ns0:f>ROUND(F116*1.4,-5)</ns0:f>
-        <ns0:v>1.8881145933381136e+25</ns0:v>
+        <ns0:v>6.734083605994406e+39</ns0:v>
       </ns0:c>
       <ns0:c r="G117" s="1" t="n">
         <ns0:v>23.6</ns0:v>
@@ -4786,15 +4666,15 @@
       </ns0:c>
       <ns0:c r="D118" s="1">
         <ns0:f>ROUND(D117*20,2-INT(LOG10(ABS(D117*20))))</ns0:f>
-        <ns0:v>3.84e+120</ns0:v>
+        <ns0:v>1.25e+112</ns0:v>
       </ns0:c>
       <ns0:c r="E118" s="1">
         <ns0:f>D118</ns0:f>
-        <ns0:v>3.84e+120</ns0:v>
+        <ns0:v>1.25e+112</ns0:v>
       </ns0:c>
       <ns0:c r="F118" s="1">
         <ns0:f>ROUND(F117*1.4,-5)</ns0:f>
-        <ns0:v>2.643360430673359e+25</ns0:v>
+        <ns0:v>9.427717048392167e+39</ns0:v>
       </ns0:c>
       <ns0:c r="G118" s="1" t="n">
         <ns0:v>23.8</ns0:v>
@@ -4818,15 +4698,15 @@
       </ns0:c>
       <ns0:c r="D119" s="1">
         <ns0:f>ROUND(D118*20,2-INT(LOG10(ABS(D118*20))))</ns0:f>
-        <ns0:v>7.68e+121</ns0:v>
+        <ns0:v>2.4999999999999997e+113</ns0:v>
       </ns0:c>
       <ns0:c r="E119" s="1">
         <ns0:f>D119</ns0:f>
-        <ns0:v>7.68e+121</ns0:v>
+        <ns0:v>2.4999999999999997e+113</ns0:v>
       </ns0:c>
       <ns0:c r="F119" s="1">
         <ns0:f>ROUND(F118*1.4,-5)</ns0:f>
-        <ns0:v>3.700704602942702e+25</ns0:v>
+        <ns0:v>1.3198803867749033e+40</ns0:v>
       </ns0:c>
       <ns0:c r="G119" s="1" t="n">
         <ns0:v>24</ns0:v>
@@ -4850,15 +4730,15 @@
       </ns0:c>
       <ns0:c r="D120" s="1">
         <ns0:f>ROUND(D119*20,2-INT(LOG10(ABS(D119*20))))</ns0:f>
-        <ns0:v>1.54e+123</ns0:v>
+        <ns0:v>5e+114</ns0:v>
       </ns0:c>
       <ns0:c r="E120" s="1">
         <ns0:f>D120</ns0:f>
-        <ns0:v>1.54e+123</ns0:v>
+        <ns0:v>5e+114</ns0:v>
       </ns0:c>
       <ns0:c r="F120" s="1">
         <ns0:f>ROUND(F119*1.4,-5)</ns0:f>
-        <ns0:v>5.1809864441197824e+25</ns0:v>
+        <ns0:v>1.8478325414848646e+40</ns0:v>
       </ns0:c>
       <ns0:c r="G120" s="1" t="n">
         <ns0:v>24.2000000000001</ns0:v>
@@ -4882,15 +4762,15 @@
       </ns0:c>
       <ns0:c r="D121" s="1">
         <ns0:f>ROUND(D120*20,2-INT(LOG10(ABS(D120*20))))</ns0:f>
-        <ns0:v>3.08e+124</ns0:v>
+        <ns0:v>1e+116</ns0:v>
       </ns0:c>
       <ns0:c r="E121" s="1">
         <ns0:f>D121</ns0:f>
-        <ns0:v>3.08e+124</ns0:v>
+        <ns0:v>1e+116</ns0:v>
       </ns0:c>
       <ns0:c r="F121" s="1">
         <ns0:f>ROUND(F120*1.4,-5)</ns0:f>
-        <ns0:v>7.253381021767694e+25</ns0:v>
+        <ns0:v>2.58696555807881e+40</ns0:v>
       </ns0:c>
       <ns0:c r="G121" s="1" t="n">
         <ns0:v>24.4000000000001</ns0:v>
@@ -4914,15 +4794,15 @@
       </ns0:c>
       <ns0:c r="D122" s="1">
         <ns0:f>ROUND(D121*20,2-INT(LOG10(ABS(D121*20))))</ns0:f>
-        <ns0:v>6.16e+125</ns0:v>
+        <ns0:v>1.9999999999999998e+117</ns0:v>
       </ns0:c>
       <ns0:c r="E122" s="1">
         <ns0:f>D122</ns0:f>
-        <ns0:v>6.16e+125</ns0:v>
+        <ns0:v>1.9999999999999998e+117</ns0:v>
       </ns0:c>
       <ns0:c r="F122" s="1">
         <ns0:f>ROUND(F121*1.4,-5)</ns0:f>
-        <ns0:v>1.015473343047477e+26</ns0:v>
+        <ns0:v>3.6217517813103335e+40</ns0:v>
       </ns0:c>
       <ns0:c r="G122" s="1" t="n">
         <ns0:v>24.6000000000001</ns0:v>
@@ -4946,15 +4826,15 @@
       </ns0:c>
       <ns0:c r="D123" s="1">
         <ns0:f>ROUND(D122*20,2-INT(LOG10(ABS(D122*20))))</ns0:f>
-        <ns0:v>1.23e+127</ns0:v>
+        <ns0:v>4e+118</ns0:v>
       </ns0:c>
       <ns0:c r="E123" s="1">
         <ns0:f>D123</ns0:f>
-        <ns0:v>1.23e+127</ns0:v>
+        <ns0:v>4e+118</ns0:v>
       </ns0:c>
       <ns0:c r="F123" s="1">
         <ns0:f>ROUND(F122*1.4,-5)</ns0:f>
-        <ns0:v>1.4216626802664678e+26</ns0:v>
+        <ns0:v>5.070452493834467e+40</ns0:v>
       </ns0:c>
       <ns0:c r="G123" s="1" t="n">
         <ns0:v>24.8000000000001</ns0:v>
@@ -4978,15 +4858,15 @@
       </ns0:c>
       <ns0:c r="D124" s="1">
         <ns0:f>ROUND(D123*20,2-INT(LOG10(ABS(D123*20))))</ns0:f>
-        <ns0:v>2.46e+128</ns0:v>
+        <ns0:v>8e+119</ns0:v>
       </ns0:c>
       <ns0:c r="E124" s="1">
         <ns0:f>D124</ns0:f>
-        <ns0:v>2.46e+128</ns0:v>
+        <ns0:v>8e+119</ns0:v>
       </ns0:c>
       <ns0:c r="F124" s="1">
         <ns0:f>ROUND(F123*1.4,-5)</ns0:f>
-        <ns0:v>1.9903277523730548e+26</ns0:v>
+        <ns0:v>7.098633491368252e+40</ns0:v>
       </ns0:c>
       <ns0:c r="G124" s="1" t="n">
         <ns0:v>25.0000000000001</ns0:v>
@@ -5010,15 +4890,15 @@
       </ns0:c>
       <ns0:c r="D125" s="1">
         <ns0:f>ROUND(D124*20,2-INT(LOG10(ABS(D124*20))))</ns0:f>
-        <ns0:v>4.92e+129</ns0:v>
+        <ns0:v>1.6e+121</ns0:v>
       </ns0:c>
       <ns0:c r="E125" s="1">
         <ns0:f>D125</ns0:f>
-        <ns0:v>4.92e+129</ns0:v>
+        <ns0:v>1.6e+121</ns0:v>
       </ns0:c>
       <ns0:c r="F125" s="1">
         <ns0:f>ROUND(F124*1.4,-5)</ns0:f>
-        <ns0:v>2.7864588533222764e+26</ns0:v>
+        <ns0:v>9.938086887915552e+40</ns0:v>
       </ns0:c>
       <ns0:c r="G125" s="1" t="n">
         <ns0:v>25.2000000000001</ns0:v>
@@ -5042,15 +4922,15 @@
       </ns0:c>
       <ns0:c r="D126" s="1">
         <ns0:f>ROUND(D125*20,2-INT(LOG10(ABS(D125*20))))</ns0:f>
-        <ns0:v>9.839999999999999e+130</ns0:v>
+        <ns0:v>3.2e+122</ns0:v>
       </ns0:c>
       <ns0:c r="E126" s="1">
         <ns0:f>D126</ns0:f>
-        <ns0:v>9.839999999999999e+130</ns0:v>
+        <ns0:v>3.2e+122</ns0:v>
       </ns0:c>
       <ns0:c r="F126" s="1">
         <ns0:f>ROUND(F125*1.4,-5)</ns0:f>
-        <ns0:v>3.9010423946511864e+26</ns0:v>
+        <ns0:v>1.3913321643081771e+41</ns0:v>
       </ns0:c>
       <ns0:c r="G126" s="1" t="n">
         <ns0:v>25.4000000000001</ns0:v>
@@ -5074,15 +4954,15 @@
       </ns0:c>
       <ns0:c r="D127" s="1">
         <ns0:f>ROUND(D126*20,2-INT(LOG10(ABS(D126*20))))</ns0:f>
-        <ns0:v>1.97e+132</ns0:v>
+        <ns0:v>6.4e+123</ns0:v>
       </ns0:c>
       <ns0:c r="E127" s="1">
         <ns0:f>D127</ns0:f>
-        <ns0:v>1.97e+132</ns0:v>
+        <ns0:v>6.4e+123</ns0:v>
       </ns0:c>
       <ns0:c r="F127" s="1">
         <ns0:f>ROUND(F126*1.4,-5)</ns0:f>
-        <ns0:v>5.4614593525116606e+26</ns0:v>
+        <ns0:v>1.9478650300314477e+41</ns0:v>
       </ns0:c>
       <ns0:c r="G127" s="1" t="n">
         <ns0:v>25.6000000000001</ns0:v>
@@ -5106,15 +4986,15 @@
       </ns0:c>
       <ns0:c r="D128" s="1">
         <ns0:f>ROUND(D127*20,2-INT(LOG10(ABS(D127*20))))</ns0:f>
-        <ns0:v>3.94e+133</ns0:v>
+        <ns0:v>1.28e+125</ns0:v>
       </ns0:c>
       <ns0:c r="E128" s="1">
         <ns0:f>D128</ns0:f>
-        <ns0:v>3.94e+133</ns0:v>
+        <ns0:v>1.28e+125</ns0:v>
       </ns0:c>
       <ns0:c r="F128" s="1">
         <ns0:f>ROUND(F127*1.4,-5)</ns0:f>
-        <ns0:v>7.646043093516325e+26</ns0:v>
+        <ns0:v>2.7270110420440267e+41</ns0:v>
       </ns0:c>
       <ns0:c r="G128" s="1" t="n">
         <ns0:v>25.8000000000001</ns0:v>
@@ -5138,15 +5018,15 @@
       </ns0:c>
       <ns0:c r="D129" s="1">
         <ns0:f>ROUND(D128*20,2-INT(LOG10(ABS(D128*20))))</ns0:f>
-        <ns0:v>7.880000000000001e+134</ns0:v>
+        <ns0:v>2.5600000000000002e+126</ns0:v>
       </ns0:c>
       <ns0:c r="E129" s="1">
         <ns0:f>D129</ns0:f>
-        <ns0:v>7.880000000000001e+134</ns0:v>
+        <ns0:v>2.5600000000000002e+126</ns0:v>
       </ns0:c>
       <ns0:c r="F129" s="1">
         <ns0:f>ROUND(F128*1.4,-5)</ns0:f>
-        <ns0:v>1.0704460330922856e+27</ns0:v>
+        <ns0:v>3.817815458861637e+41</ns0:v>
       </ns0:c>
       <ns0:c r="G129" s="1" t="n">
         <ns0:v>26.0000000000001</ns0:v>
@@ -5170,15 +5050,15 @@
       </ns0:c>
       <ns0:c r="D130" s="1">
         <ns0:f>ROUND(D129*20,2-INT(LOG10(ABS(D129*20))))</ns0:f>
-        <ns0:v>1.58e+136</ns0:v>
+        <ns0:v>5.12e+127</ns0:v>
       </ns0:c>
       <ns0:c r="E130" s="1">
         <ns0:f>D130</ns0:f>
-        <ns0:v>1.58e+136</ns0:v>
+        <ns0:v>5.12e+127</ns0:v>
       </ns0:c>
       <ns0:c r="F130" s="1">
         <ns0:f>ROUND(F129*1.4,-5)</ns0:f>
-        <ns0:v>1.4986244463291998e+27</ns0:v>
+        <ns0:v>5.3449416424062916e+41</ns0:v>
       </ns0:c>
       <ns0:c r="G130" s="1" t="n">
         <ns0:v>26.2000000000001</ns0:v>
@@ -5202,15 +5082,15 @@
       </ns0:c>
       <ns0:c r="D131" s="1">
         <ns0:f>ROUND(D130*20,2-INT(LOG10(ABS(D130*20))))</ns0:f>
-        <ns0:v>3.1599999999999998e+137</ns0:v>
+        <ns0:v>1.02e+129</ns0:v>
       </ns0:c>
       <ns0:c r="E131" s="1">
         <ns0:f>D131</ns0:f>
-        <ns0:v>3.1599999999999998e+137</ns0:v>
+        <ns0:v>1.02e+129</ns0:v>
       </ns0:c>
       <ns0:c r="F131" s="1">
         <ns0:f>ROUND(F130*1.4,-5)</ns0:f>
-        <ns0:v>2.0980742248608796e+27</ns0:v>
+        <ns0:v>7.482918299368808e+41</ns0:v>
       </ns0:c>
       <ns0:c r="G131" s="1" t="n">
         <ns0:v>26.4000000000001</ns0:v>
@@ -5234,15 +5114,15 @@
       </ns0:c>
       <ns0:c r="D132" s="1">
         <ns0:f>ROUND(D131*20,2-INT(LOG10(ABS(D131*20))))</ns0:f>
-        <ns0:v>6.32e+138</ns0:v>
+        <ns0:v>2.04e+130</ns0:v>
       </ns0:c>
       <ns0:c r="E132" s="1">
         <ns0:f>D132</ns0:f>
-        <ns0:v>6.32e+138</ns0:v>
+        <ns0:v>2.04e+130</ns0:v>
       </ns0:c>
       <ns0:c r="F132" s="1">
         <ns0:f>ROUND(F131*1.4,-5)</ns0:f>
-        <ns0:v>2.9373039148052314e+27</ns0:v>
+        <ns0:v>1.0476085619116331e+42</ns0:v>
       </ns0:c>
       <ns0:c r="G132" s="1" t="n">
         <ns0:v>26.6000000000001</ns0:v>
@@ -5266,15 +5146,15 @@
       </ns0:c>
       <ns0:c r="D133" s="1">
         <ns0:f>ROUND(D132*20,2-INT(LOG10(ABS(D132*20))))</ns0:f>
-        <ns0:v>1.2599999999999998e+140</ns0:v>
+        <ns0:v>4.0800000000000005e+131</ns0:v>
       </ns0:c>
       <ns0:c r="E133" s="1">
         <ns0:f>D133</ns0:f>
-        <ns0:v>1.2599999999999998e+140</ns0:v>
+        <ns0:v>4.0800000000000005e+131</ns0:v>
       </ns0:c>
       <ns0:c r="F133" s="1">
         <ns0:f>ROUND(F132*1.4,-5)</ns0:f>
-        <ns0:v>4.112225480727324e+27</ns0:v>
+        <ns0:v>1.4666519866762864e+42</ns0:v>
       </ns0:c>
       <ns0:c r="G133" s="1" t="n">
         <ns0:v>26.8000000000001</ns0:v>
@@ -5298,15 +5178,15 @@
       </ns0:c>
       <ns0:c r="D134" s="1">
         <ns0:f>ROUND(D133*20,2-INT(LOG10(ABS(D133*20))))</ns0:f>
-        <ns0:v>2.52e+141</ns0:v>
+        <ns0:v>8.159999999999999e+132</ns0:v>
       </ns0:c>
       <ns0:c r="E134" s="1">
         <ns0:f>D134</ns0:f>
-        <ns0:v>2.52e+141</ns0:v>
+        <ns0:v>8.159999999999999e+132</ns0:v>
       </ns0:c>
       <ns0:c r="F134" s="1">
         <ns0:f>ROUND(F133*1.4,-5)</ns0:f>
-        <ns0:v>5.757115673018253e+27</ns0:v>
+        <ns0:v>2.053312781346801e+42</ns0:v>
       </ns0:c>
       <ns0:c r="G134" s="1" t="n">
         <ns0:v>27.0000000000001</ns0:v>
@@ -5330,15 +5210,15 @@
       </ns0:c>
       <ns0:c r="D135" s="1">
         <ns0:f>ROUND(D134*20,2-INT(LOG10(ABS(D134*20))))</ns0:f>
-        <ns0:v>5.04e+142</ns0:v>
+        <ns0:v>1.63e+134</ns0:v>
       </ns0:c>
       <ns0:c r="E135" s="1">
         <ns0:f>D135</ns0:f>
-        <ns0:v>5.04e+142</ns0:v>
+        <ns0:v>1.63e+134</ns0:v>
       </ns0:c>
       <ns0:c r="F135" s="1">
         <ns0:f>ROUND(F134*1.4,-5)</ns0:f>
-        <ns0:v>8.059961942225552e+27</ns0:v>
+        <ns0:v>2.8746378938855214e+42</ns0:v>
       </ns0:c>
       <ns0:c r="G135" s="1" t="n">
         <ns0:v>27.2000000000001</ns0:v>
@@ -5362,15 +5242,15 @@
       </ns0:c>
       <ns0:c r="D136" s="1">
         <ns0:f>ROUND(D135*20,2-INT(LOG10(ABS(D135*20))))</ns0:f>
-        <ns0:v>1.0099999999999999e+144</ns0:v>
+        <ns0:v>3.26e+135</ns0:v>
       </ns0:c>
       <ns0:c r="E136" s="1">
         <ns0:f>D136</ns0:f>
-        <ns0:v>1.0099999999999999e+144</ns0:v>
+        <ns0:v>3.26e+135</ns0:v>
       </ns0:c>
       <ns0:c r="F136" s="1">
         <ns0:f>ROUND(F135*1.4,-5)</ns0:f>
-        <ns0:v>1.1283946719115773e+28</ns0:v>
+        <ns0:v>4.0244930514397294e+42</ns0:v>
       </ns0:c>
       <ns0:c r="G136" s="1" t="n">
         <ns0:v>27.4000000000001</ns0:v>
@@ -5394,15 +5274,15 @@
       </ns0:c>
       <ns0:c r="D137" s="1">
         <ns0:f>ROUND(D136*20,2-INT(LOG10(ABS(D136*20))))</ns0:f>
-        <ns0:v>2.0200000000000002e+145</ns0:v>
+        <ns0:v>6.52e+136</ns0:v>
       </ns0:c>
       <ns0:c r="E137" s="1">
         <ns0:f>D137</ns0:f>
-        <ns0:v>2.0200000000000002e+145</ns0:v>
+        <ns0:v>6.52e+136</ns0:v>
       </ns0:c>
       <ns0:c r="F137" s="1">
         <ns0:f>ROUND(F136*1.4,-5)</ns0:f>
-        <ns0:v>1.5797525406762081e+28</ns0:v>
+        <ns0:v>5.634290272015621e+42</ns0:v>
       </ns0:c>
       <ns0:c r="G137" s="1" t="n">
         <ns0:v>27.6000000000001</ns0:v>
@@ -5426,15 +5306,15 @@
       </ns0:c>
       <ns0:c r="D138" s="1">
         <ns0:f>ROUND(D137*20,2-INT(LOG10(ABS(D137*20))))</ns0:f>
-        <ns0:v>4.04e+146</ns0:v>
+        <ns0:v>1.3e+138</ns0:v>
       </ns0:c>
       <ns0:c r="E138" s="1">
         <ns0:f>D138</ns0:f>
-        <ns0:v>4.04e+146</ns0:v>
+        <ns0:v>1.3e+138</ns0:v>
       </ns0:c>
       <ns0:c r="F138" s="1">
         <ns0:f>ROUND(F137*1.4,-5)</ns0:f>
-        <ns0:v>2.211653556946691e+28</ns0:v>
+        <ns0:v>7.888006380821869e+42</ns0:v>
       </ns0:c>
       <ns0:c r="G138" s="1" t="n">
         <ns0:v>27.8000000000001</ns0:v>
@@ -5458,15 +5338,15 @@
       </ns0:c>
       <ns0:c r="D139" s="1">
         <ns0:f>ROUND(D138*20,2-INT(LOG10(ABS(D138*20))))</ns0:f>
-        <ns0:v>8.080000000000001e+147</ns0:v>
+        <ns0:v>2.6e+139</ns0:v>
       </ns0:c>
       <ns0:c r="E139" s="1">
         <ns0:f>D139</ns0:f>
-        <ns0:v>8.080000000000001e+147</ns0:v>
+        <ns0:v>2.6e+139</ns0:v>
       </ns0:c>
       <ns0:c r="F139" s="1">
         <ns0:f>ROUND(F138*1.4,-5)</ns0:f>
-        <ns0:v>3.096314979725367e+28</ns0:v>
+        <ns0:v>1.1043208933150617e+43</ns0:v>
       </ns0:c>
       <ns0:c r="G139" s="1" t="n">
         <ns0:v>28.0000000000001</ns0:v>
@@ -5490,15 +5370,15 @@
       </ns0:c>
       <ns0:c r="D140" s="1">
         <ns0:f>ROUND(D139*20,2-INT(LOG10(ABS(D139*20))))</ns0:f>
-        <ns0:v>1.62e+149</ns0:v>
+        <ns0:v>5.199999999999999e+140</ns0:v>
       </ns0:c>
       <ns0:c r="E140" s="1">
         <ns0:f>D140</ns0:f>
-        <ns0:v>1.62e+149</ns0:v>
+        <ns0:v>5.199999999999999e+140</ns0:v>
       </ns0:c>
       <ns0:c r="F140" s="1">
         <ns0:f>ROUND(F139*1.4,-5)</ns0:f>
-        <ns0:v>4.334840971615514e+28</ns0:v>
+        <ns0:v>1.5460492506410863e+43</ns0:v>
       </ns0:c>
       <ns0:c r="G140" s="1" t="n">
         <ns0:v>28.2000000000001</ns0:v>
@@ -5522,15 +5402,15 @@
       </ns0:c>
       <ns0:c r="D141" s="1">
         <ns0:f>ROUND(D140*20,2-INT(LOG10(ABS(D140*20))))</ns0:f>
-        <ns0:v>3.24e+150</ns0:v>
+        <ns0:v>1.04e+142</ns0:v>
       </ns0:c>
       <ns0:c r="E141" s="1">
         <ns0:f>D141</ns0:f>
-        <ns0:v>3.24e+150</ns0:v>
+        <ns0:v>1.04e+142</ns0:v>
       </ns0:c>
       <ns0:c r="F141" s="1">
         <ns0:f>ROUND(F140*1.4,-5)</ns0:f>
-        <ns0:v>6.0687773602617194e+28</ns0:v>
+        <ns0:v>2.1644689508975208e+43</ns0:v>
       </ns0:c>
       <ns0:c r="G141" s="1" t="n">
         <ns0:v>28.4000000000001</ns0:v>
@@ -5554,15 +5434,15 @@
       </ns0:c>
       <ns0:c r="D142" s="1">
         <ns0:f>ROUND(D141*20,2-INT(LOG10(ABS(D141*20))))</ns0:f>
-        <ns0:v>6.48e+151</ns0:v>
+        <ns0:v>2.0799999999999997e+143</ns0:v>
       </ns0:c>
       <ns0:c r="E142" s="1">
         <ns0:f>D142</ns0:f>
-        <ns0:v>6.48e+151</ns0:v>
+        <ns0:v>2.0799999999999997e+143</ns0:v>
       </ns0:c>
       <ns0:c r="F142" s="1">
         <ns0:f>ROUND(F141*1.4,-5)</ns0:f>
-        <ns0:v>8.496288304366406e+28</ns0:v>
+        <ns0:v>3.030256531256529e+43</ns0:v>
       </ns0:c>
       <ns0:c r="G142" s="1" t="n">
         <ns0:v>28.6000000000001</ns0:v>
@@ -5586,15 +5466,15 @@
       </ns0:c>
       <ns0:c r="D143" s="1">
         <ns0:f>ROUND(D142*20,2-INT(LOG10(ABS(D142*20))))</ns0:f>
-        <ns0:v>1.3000000000000001e+153</ns0:v>
+        <ns0:v>4.16e+144</ns0:v>
       </ns0:c>
       <ns0:c r="E143" s="1">
         <ns0:f>D143</ns0:f>
-        <ns0:v>1.3000000000000001e+153</ns0:v>
+        <ns0:v>4.16e+144</ns0:v>
       </ns0:c>
       <ns0:c r="F143" s="1">
         <ns0:f>ROUND(F142*1.4,-5)</ns0:f>
-        <ns0:v>1.1894803626112967e+29</ns0:v>
+        <ns0:v>4.24235914375914e+43</ns0:v>
       </ns0:c>
       <ns0:c r="G143" s="1" t="n">
         <ns0:v>28.8000000000001</ns0:v>
@@ -5618,15 +5498,15 @@
       </ns0:c>
       <ns0:c r="D144" s="1">
         <ns0:f>ROUND(D143*20,2-INT(LOG10(ABS(D143*20))))</ns0:f>
-        <ns0:v>2.6e+154</ns0:v>
+        <ns0:v>8.320000000000001e+145</ns0:v>
       </ns0:c>
       <ns0:c r="E144" s="1">
         <ns0:f>D144</ns0:f>
-        <ns0:v>2.6e+154</ns0:v>
+        <ns0:v>8.320000000000001e+145</ns0:v>
       </ns0:c>
       <ns0:c r="F144" s="1">
         <ns0:f>ROUND(F143*1.4,-5)</ns0:f>
-        <ns0:v>1.665272507655815e+29</ns0:v>
+        <ns0:v>5.939302801262796e+43</ns0:v>
       </ns0:c>
       <ns0:c r="G144" s="1" t="n">
         <ns0:v>29.0000000000001</ns0:v>
@@ -5650,15 +5530,15 @@
       </ns0:c>
       <ns0:c r="D145" s="1">
         <ns0:f>ROUND(D144*20,2-INT(LOG10(ABS(D144*20))))</ns0:f>
-        <ns0:v>5.199999999999999e+155</ns0:v>
+        <ns0:v>1.66e+147</ns0:v>
       </ns0:c>
       <ns0:c r="E145" s="1">
         <ns0:f>D145</ns0:f>
-        <ns0:v>5.199999999999999e+155</ns0:v>
+        <ns0:v>1.66e+147</ns0:v>
       </ns0:c>
       <ns0:c r="F145" s="1">
         <ns0:f>ROUND(F144*1.4,-5)</ns0:f>
-        <ns0:v>2.331381510718141e+29</ns0:v>
+        <ns0:v>8.315023921767913e+43</ns0:v>
       </ns0:c>
       <ns0:c r="G145" s="1" t="n">
         <ns0:v>29.2000000000001</ns0:v>
@@ -5682,15 +5562,15 @@
       </ns0:c>
       <ns0:c r="D146" s="1">
         <ns0:f>ROUND(D145*20,2-INT(LOG10(ABS(D145*20))))</ns0:f>
-        <ns0:v>1.0399999999999999e+157</ns0:v>
+        <ns0:v>3.32e+148</ns0:v>
       </ns0:c>
       <ns0:c r="E146" s="1">
         <ns0:f>D146</ns0:f>
-        <ns0:v>1.0399999999999999e+157</ns0:v>
+        <ns0:v>3.32e+148</ns0:v>
       </ns0:c>
       <ns0:c r="F146" s="1">
         <ns0:f>ROUND(F145*1.4,-5)</ns0:f>
-        <ns0:v>3.263934115005397e+29</ns0:v>
+        <ns0:v>1.1641033490475078e+44</ns0:v>
       </ns0:c>
       <ns0:c r="G146" s="1" t="n">
         <ns0:v>29.4000000000001</ns0:v>
@@ -5714,15 +5594,15 @@
       </ns0:c>
       <ns0:c r="D147" s="1">
         <ns0:f>ROUND(D146*20,2-INT(LOG10(ABS(D146*20))))</ns0:f>
-        <ns0:v>2.0799999999999998e+158</ns0:v>
+        <ns0:v>6.64e+149</ns0:v>
       </ns0:c>
       <ns0:c r="E147" s="1">
         <ns0:f>D147</ns0:f>
-        <ns0:v>2.0799999999999998e+158</ns0:v>
+        <ns0:v>6.64e+149</ns0:v>
       </ns0:c>
       <ns0:c r="F147" s="1">
         <ns0:f>ROUND(F146*1.4,-5)</ns0:f>
-        <ns0:v>4.569507761007556e+29</ns0:v>
+        <ns0:v>1.6297446886665107e+44</ns0:v>
       </ns0:c>
       <ns0:c r="G147" s="1" t="n">
         <ns0:v>29.6000000000001</ns0:v>
@@ -5746,15 +5626,15 @@
       </ns0:c>
       <ns0:c r="D148" s="1">
         <ns0:f>ROUND(D147*20,2-INT(LOG10(ABS(D147*20))))</ns0:f>
-        <ns0:v>4.16e+159</ns0:v>
+        <ns0:v>1.33e+151</ns0:v>
       </ns0:c>
       <ns0:c r="E148" s="1">
         <ns0:f>D148</ns0:f>
-        <ns0:v>4.16e+159</ns0:v>
+        <ns0:v>1.33e+151</ns0:v>
       </ns0:c>
       <ns0:c r="F148" s="1">
         <ns0:f>ROUND(F147*1.4,-5)</ns0:f>
-        <ns0:v>6.397310865410578e+29</ns0:v>
+        <ns0:v>2.2816425641331147e+44</ns0:v>
       </ns0:c>
       <ns0:c r="G148" s="1" t="n">
         <ns0:v>29.8000000000001</ns0:v>
@@ -5778,15 +5658,15 @@
       </ns0:c>
       <ns0:c r="D149" s="1">
         <ns0:f>ROUND(D148*20,2-INT(LOG10(ABS(D148*20))))</ns0:f>
-        <ns0:v>8.319999999999999e+160</ns0:v>
+        <ns0:v>2.66e+152</ns0:v>
       </ns0:c>
       <ns0:c r="E149" s="1">
         <ns0:f>D149</ns0:f>
-        <ns0:v>8.319999999999999e+160</ns0:v>
+        <ns0:v>2.66e+152</ns0:v>
       </ns0:c>
       <ns0:c r="F149" s="1">
         <ns0:f>ROUND(F148*1.4,-5)</ns0:f>
-        <ns0:v>8.956235211574808e+29</ns0:v>
+        <ns0:v>3.1942995897863605e+44</ns0:v>
       </ns0:c>
       <ns0:c r="G149" s="1" t="n">
         <ns0:v>30.0000000000001</ns0:v>
@@ -5810,15 +5690,15 @@
       </ns0:c>
       <ns0:c r="D150" s="1">
         <ns0:f>ROUND(D149*20,2-INT(LOG10(ABS(D149*20))))</ns0:f>
-        <ns0:v>1.66e+162</ns0:v>
+        <ns0:v>5.3200000000000004e+153</ns0:v>
       </ns0:c>
       <ns0:c r="E150" s="1">
         <ns0:f>D150</ns0:f>
-        <ns0:v>1.66e+162</ns0:v>
+        <ns0:v>5.3200000000000004e+153</ns0:v>
       </ns0:c>
       <ns0:c r="F150" s="1">
         <ns0:f>ROUND(F149*1.4,-5)</ns0:f>
-        <ns0:v>1.2538729296204731e+30</ns0:v>
+        <ns0:v>4.472019425700905e+44</ns0:v>
       </ns0:c>
       <ns0:c r="G150" s="1" t="n">
         <ns0:v>30.2000000000001</ns0:v>
@@ -5842,15 +5722,15 @@
       </ns0:c>
       <ns0:c r="D151" s="1">
         <ns0:f>ROUND(D150*20,2-INT(LOG10(ABS(D150*20))))</ns0:f>
-        <ns0:v>3.32e+163</ns0:v>
+        <ns0:v>1.0599999999999999e+155</ns0:v>
       </ns0:c>
       <ns0:c r="E151" s="1">
         <ns0:f>D151</ns0:f>
-        <ns0:v>3.32e+163</ns0:v>
+        <ns0:v>1.0599999999999999e+155</ns0:v>
       </ns0:c>
       <ns0:c r="F151" s="1">
         <ns0:f>ROUND(F150*1.4,-5)</ns0:f>
-        <ns0:v>1.7554221014686622e+30</ns0:v>
+        <ns0:v>6.260827195981266e+44</ns0:v>
       </ns0:c>
       <ns0:c r="G151" s="1" t="n">
         <ns0:v>30.4000000000001</ns0:v>
@@ -5874,15 +5754,15 @@
       </ns0:c>
       <ns0:c r="D152" s="1">
         <ns0:f>ROUND(D151*20,2-INT(LOG10(ABS(D151*20))))</ns0:f>
-        <ns0:v>6.64e+164</ns0:v>
+        <ns0:v>2.1200000000000002e+156</ns0:v>
       </ns0:c>
       <ns0:c r="E152" s="1">
         <ns0:f>D152</ns0:f>
-        <ns0:v>6.64e+164</ns0:v>
+        <ns0:v>2.1200000000000002e+156</ns0:v>
       </ns0:c>
       <ns0:c r="F152" s="1">
         <ns0:f>ROUND(F151*1.4,-5)</ns0:f>
-        <ns0:v>2.4575909420561268e+30</ns0:v>
+        <ns0:v>8.765158074373773e+44</ns0:v>
       </ns0:c>
       <ns0:c r="G152" s="1" t="n">
         <ns0:v>30.6000000000001</ns0:v>
@@ -5906,15 +5786,15 @@
       </ns0:c>
       <ns0:c r="D153" s="1">
         <ns0:f>ROUND(D152*20,2-INT(LOG10(ABS(D152*20))))</ns0:f>
-        <ns0:v>1.3300000000000001e+166</ns0:v>
+        <ns0:v>4.24e+157</ns0:v>
       </ns0:c>
       <ns0:c r="E153" s="1">
         <ns0:f>D153</ns0:f>
-        <ns0:v>1.3300000000000001e+166</ns0:v>
+        <ns0:v>4.24e+157</ns0:v>
       </ns0:c>
       <ns0:c r="F153" s="1">
         <ns0:f>ROUND(F152*1.4,-5)</ns0:f>
-        <ns0:v>3.440627318878577e+30</ns0:v>
+        <ns0:v>1.2271221304123282e+45</ns0:v>
       </ns0:c>
       <ns0:c r="G153" s="1" t="n">
         <ns0:v>30.8000000000001</ns0:v>
@@ -5938,15 +5818,15 @@
       </ns0:c>
       <ns0:c r="D154" s="1">
         <ns0:f>ROUND(D153*20,2-INT(LOG10(ABS(D153*20))))</ns0:f>
-        <ns0:v>2.66e+167</ns0:v>
+        <ns0:v>8.48e+158</ns0:v>
       </ns0:c>
       <ns0:c r="E154" s="1">
         <ns0:f>D154</ns0:f>
-        <ns0:v>2.66e+167</ns0:v>
+        <ns0:v>8.48e+158</ns0:v>
       </ns0:c>
       <ns0:c r="F154" s="1">
         <ns0:f>ROUND(F153*1.4,-5)</ns0:f>
-        <ns0:v>4.8168782464300075e+30</ns0:v>
+        <ns0:v>1.7179709825772595e+45</ns0:v>
       </ns0:c>
       <ns0:c r="G154" s="1" t="n">
         <ns0:v>31.0000000000001</ns0:v>
@@ -5970,15 +5850,15 @@
       </ns0:c>
       <ns0:c r="D155" s="1">
         <ns0:f>ROUND(D154*20,2-INT(LOG10(ABS(D154*20))))</ns0:f>
-        <ns0:v>5.32e+168</ns0:v>
+        <ns0:v>1.6999999999999998e+160</ns0:v>
       </ns0:c>
       <ns0:c r="E155" s="1">
         <ns0:f>D155</ns0:f>
-        <ns0:v>5.32e+168</ns0:v>
+        <ns0:v>1.6999999999999998e+160</ns0:v>
       </ns0:c>
       <ns0:c r="F155" s="1">
         <ns0:f>ROUND(F154*1.4,-5)</ns0:f>
-        <ns0:v>6.74362954500201e+30</ns0:v>
+        <ns0:v>2.405159375608163e+45</ns0:v>
       </ns0:c>
       <ns0:c r="G155" s="1" t="n">
         <ns0:v>31.2000000000001</ns0:v>
@@ -6002,15 +5882,15 @@
       </ns0:c>
       <ns0:c r="D156" s="1">
         <ns0:f>ROUND(D155*20,2-INT(LOG10(ABS(D155*20))))</ns0:f>
-        <ns0:v>1.06e+170</ns0:v>
+        <ns0:v>3.4e+161</ns0:v>
       </ns0:c>
       <ns0:c r="E156" s="1">
         <ns0:f>D156</ns0:f>
-        <ns0:v>1.06e+170</ns0:v>
+        <ns0:v>3.4e+161</ns0:v>
       </ns0:c>
       <ns0:c r="F156" s="1">
         <ns0:f>ROUND(F155*1.4,-5)</ns0:f>
-        <ns0:v>9.441081363002813e+30</ns0:v>
+        <ns0:v>3.367223125851428e+45</ns0:v>
       </ns0:c>
       <ns0:c r="G156" s="1" t="n">
         <ns0:v>31.4000000000001</ns0:v>
@@ -6034,15 +5914,15 @@
       </ns0:c>
       <ns0:c r="D157" s="1">
         <ns0:f>ROUND(D156*20,2-INT(LOG10(ABS(D156*20))))</ns0:f>
-        <ns0:v>2.12e+171</ns0:v>
+        <ns0:v>6.8e+162</ns0:v>
       </ns0:c>
       <ns0:c r="E157" s="1">
         <ns0:f>D157</ns0:f>
-        <ns0:v>2.12e+171</ns0:v>
+        <ns0:v>6.8e+162</ns0:v>
       </ns0:c>
       <ns0:c r="F157" s="1">
         <ns0:f>ROUND(F156*1.4,-5)</ns0:f>
-        <ns0:v>1.3217513908203938e+31</ns0:v>
+        <ns0:v>4.714112376191999e+45</ns0:v>
       </ns0:c>
       <ns0:c r="G157" s="1" t="n">
         <ns0:v>31.6000000000001</ns0:v>
@@ -6066,15 +5946,15 @@
       </ns0:c>
       <ns0:c r="D158" s="1">
         <ns0:f>ROUND(D157*20,2-INT(LOG10(ABS(D157*20))))</ns0:f>
-        <ns0:v>4.24e+172</ns0:v>
+        <ns0:v>1.36e+164</ns0:v>
       </ns0:c>
       <ns0:c r="E158" s="1">
         <ns0:f>D158</ns0:f>
-        <ns0:v>4.24e+172</ns0:v>
+        <ns0:v>1.36e+164</ns0:v>
       </ns0:c>
       <ns0:c r="F158" s="1">
         <ns0:f>ROUND(F157*1.4,-5)</ns0:f>
-        <ns0:v>1.8504519471485511e+31</ns0:v>
+        <ns0:v>6.599757326668798e+45</ns0:v>
       </ns0:c>
       <ns0:c r="G158" s="1" t="n">
         <ns0:v>31.8000000000001</ns0:v>
@@ -6098,15 +5978,15 @@
       </ns0:c>
       <ns0:c r="D159" s="1">
         <ns0:f>ROUND(D158*20,2-INT(LOG10(ABS(D158*20))))</ns0:f>
-        <ns0:v>8.48e+173</ns0:v>
+        <ns0:v>2.72e+165</ns0:v>
       </ns0:c>
       <ns0:c r="E159" s="1">
         <ns0:f>D159</ns0:f>
-        <ns0:v>8.48e+173</ns0:v>
+        <ns0:v>2.72e+165</ns0:v>
       </ns0:c>
       <ns0:c r="F159" s="1">
         <ns0:f>ROUND(F158*1.4,-5)</ns0:f>
-        <ns0:v>2.5906327260079714e+31</ns0:v>
+        <ns0:v>9.239660257336316e+45</ns0:v>
       </ns0:c>
       <ns0:c r="G159" s="1" t="n">
         <ns0:v>32.0000000000001</ns0:v>
@@ -6130,15 +6010,15 @@
       </ns0:c>
       <ns0:c r="D160" s="1">
         <ns0:f>ROUND(D159*20,2-INT(LOG10(ABS(D159*20))))</ns0:f>
-        <ns0:v>1.6999999999999998e+175</ns0:v>
+        <ns0:v>5.44e+166</ns0:v>
       </ns0:c>
       <ns0:c r="E160" s="1">
         <ns0:f>D160</ns0:f>
-        <ns0:v>1.6999999999999998e+175</ns0:v>
+        <ns0:v>5.44e+166</ns0:v>
       </ns0:c>
       <ns0:c r="F160" s="1">
         <ns0:f>ROUND(F159*1.4,-5)</ns0:f>
-        <ns0:v>3.6268858164111598e+31</ns0:v>
+        <ns0:v>1.2935524360270842e+46</ns0:v>
       </ns0:c>
       <ns0:c r="G160" s="1" t="n">
         <ns0:v>32.2000000000001</ns0:v>
@@ -6162,15 +6042,15 @@
       </ns0:c>
       <ns0:c r="D161" s="1">
         <ns0:f>ROUND(D160*20,2-INT(LOG10(ABS(D160*20))))</ns0:f>
-        <ns0:v>3.4e+176</ns0:v>
+        <ns0:v>1.09e+168</ns0:v>
       </ns0:c>
       <ns0:c r="E161" s="1">
         <ns0:f>D161</ns0:f>
-        <ns0:v>3.4e+176</ns0:v>
+        <ns0:v>1.09e+168</ns0:v>
       </ns0:c>
       <ns0:c r="F161" s="1">
         <ns0:f>ROUND(F160*1.4,-5)</ns0:f>
-        <ns0:v>5.0776401429756235e+31</ns0:v>
+        <ns0:v>1.8109734104379178e+46</ns0:v>
       </ns0:c>
       <ns0:c r="G161" s="1" t="n">
         <ns0:v>32.4000000000001</ns0:v>
@@ -6194,15 +6074,15 @@
       </ns0:c>
       <ns0:c r="D162" s="1">
         <ns0:f>ROUND(D161*20,2-INT(LOG10(ABS(D161*20))))</ns0:f>
-        <ns0:v>6.8e+177</ns0:v>
+        <ns0:v>2.18e+169</ns0:v>
       </ns0:c>
       <ns0:c r="E162" s="1">
         <ns0:f>D162</ns0:f>
-        <ns0:v>6.8e+177</ns0:v>
+        <ns0:v>2.18e+169</ns0:v>
       </ns0:c>
       <ns0:c r="F162" s="1">
         <ns0:f>ROUND(F161*1.4,-5)</ns0:f>
-        <ns0:v>7.108696200165872e+31</ns0:v>
+        <ns0:v>2.5353627746130845e+46</ns0:v>
       </ns0:c>
       <ns0:c r="G162" s="1" t="n">
         <ns0:v>32.6000000000001</ns0:v>
@@ -6226,15 +6106,15 @@
       </ns0:c>
       <ns0:c r="D163" s="1">
         <ns0:f>ROUND(D162*20,2-INT(LOG10(ABS(D162*20))))</ns0:f>
-        <ns0:v>1.36e+179</ns0:v>
+        <ns0:v>4.36e+170</ns0:v>
       </ns0:c>
       <ns0:c r="E163" s="1">
         <ns0:f>D163</ns0:f>
-        <ns0:v>1.36e+179</ns0:v>
+        <ns0:v>4.36e+170</ns0:v>
       </ns0:c>
       <ns0:c r="F163" s="1">
         <ns0:f>ROUND(F162*1.4,-5)</ns0:f>
-        <ns0:v>9.95217468023222e+31</ns0:v>
+        <ns0:v>3.5495078844583184e+46</ns0:v>
       </ns0:c>
       <ns0:c r="G163" s="1" t="n">
         <ns0:v>32.8000000000001</ns0:v>
@@ -6258,15 +6138,15 @@
       </ns0:c>
       <ns0:c r="D164" s="1">
         <ns0:f>ROUND(D163*20,2-INT(LOG10(ABS(D163*20))))</ns0:f>
-        <ns0:v>2.72e+180</ns0:v>
+        <ns0:v>8.72e+171</ns0:v>
       </ns0:c>
       <ns0:c r="E164" s="1">
         <ns0:f>D164</ns0:f>
-        <ns0:v>2.72e+180</ns0:v>
+        <ns0:v>8.72e+171</ns0:v>
       </ns0:c>
       <ns0:c r="F164" s="1">
         <ns0:f>ROUND(F163*1.4,-5)</ns0:f>
-        <ns0:v>1.3933044552325108e+32</ns0:v>
+        <ns0:v>4.969311038241645e+46</ns0:v>
       </ns0:c>
       <ns0:c r="G164" s="1" t="n">
         <ns0:v>33.0000000000001</ns0:v>
@@ -6290,15 +6170,15 @@
       </ns0:c>
       <ns0:c r="D165" s="1">
         <ns0:f>ROUND(D164*20,2-INT(LOG10(ABS(D164*20))))</ns0:f>
-        <ns0:v>5.44e+181</ns0:v>
+        <ns0:v>1.74e+173</ns0:v>
       </ns0:c>
       <ns0:c r="E165" s="1">
         <ns0:f>D165</ns0:f>
-        <ns0:v>5.44e+181</ns0:v>
+        <ns0:v>1.74e+173</ns0:v>
       </ns0:c>
       <ns0:c r="F165" s="1">
         <ns0:f>ROUND(F164*1.4,-5)</ns0:f>
-        <ns0:v>1.950626237325515e+32</ns0:v>
+        <ns0:v>6.957035453538303e+46</ns0:v>
       </ns0:c>
       <ns0:c r="G165" s="1" t="n">
         <ns0:v>33.2000000000001</ns0:v>
@@ -6322,15 +6202,15 @@
       </ns0:c>
       <ns0:c r="D166" s="1">
         <ns0:f>ROUND(D165*20,2-INT(LOG10(ABS(D165*20))))</ns0:f>
-        <ns0:v>1.09e+183</ns0:v>
+        <ns0:v>3.48e+174</ns0:v>
       </ns0:c>
       <ns0:c r="E166" s="1">
         <ns0:f>D166</ns0:f>
-        <ns0:v>1.09e+183</ns0:v>
+        <ns0:v>3.48e+174</ns0:v>
       </ns0:c>
       <ns0:c r="F166" s="1">
         <ns0:f>ROUND(F165*1.4,-5)</ns0:f>
-        <ns0:v>2.7308767322557203e+32</ns0:v>
+        <ns0:v>9.739849634953624e+46</ns0:v>
       </ns0:c>
       <ns0:c r="G166" s="1" t="n">
         <ns0:v>33.4000000000001</ns0:v>
@@ -6354,15 +6234,15 @@
       </ns0:c>
       <ns0:c r="D167" s="1">
         <ns0:f>ROUND(D166*20,2-INT(LOG10(ABS(D166*20))))</ns0:f>
-        <ns0:v>2.18e+184</ns0:v>
+        <ns0:v>6.959999999999999e+175</ns0:v>
       </ns0:c>
       <ns0:c r="E167" s="1">
         <ns0:f>D167</ns0:f>
-        <ns0:v>2.18e+184</ns0:v>
+        <ns0:v>6.959999999999999e+175</ns0:v>
       </ns0:c>
       <ns0:c r="F167" s="1">
         <ns0:f>ROUND(F166*1.4,-5)</ns0:f>
-        <ns0:v>3.823227425158008e+32</ns0:v>
+        <ns0:v>1.3635789488935073e+47</ns0:v>
       </ns0:c>
       <ns0:c r="G167" s="1" t="n">
         <ns0:v>33.6000000000001</ns0:v>
@@ -6386,15 +6266,15 @@
       </ns0:c>
       <ns0:c r="D168" s="1">
         <ns0:f>ROUND(D167*20,2-INT(LOG10(ABS(D167*20))))</ns0:f>
-        <ns0:v>4.36e+185</ns0:v>
+        <ns0:v>1.39e+177</ns0:v>
       </ns0:c>
       <ns0:c r="E168" s="1">
         <ns0:f>D168</ns0:f>
-        <ns0:v>4.36e+185</ns0:v>
+        <ns0:v>1.39e+177</ns0:v>
       </ns0:c>
       <ns0:c r="F168" s="1">
         <ns0:f>ROUND(F167*1.4,-5)</ns0:f>
-        <ns0:v>5.352518395221211e+32</ns0:v>
+        <ns0:v>1.9090105284509103e+47</ns0:v>
       </ns0:c>
       <ns0:c r="G168" s="1" t="n">
         <ns0:v>33.8000000000001</ns0:v>
@@ -6418,15 +6298,15 @@
       </ns0:c>
       <ns0:c r="D169" s="1">
         <ns0:f>ROUND(D168*20,2-INT(LOG10(ABS(D168*20))))</ns0:f>
-        <ns0:v>8.72e+186</ns0:v>
+        <ns0:v>2.78e+178</ns0:v>
       </ns0:c>
       <ns0:c r="E169" s="1">
         <ns0:f>D169</ns0:f>
-        <ns0:v>8.72e+186</ns0:v>
+        <ns0:v>2.78e+178</ns0:v>
       </ns0:c>
       <ns0:c r="F169" s="1">
         <ns0:f>ROUND(F168*1.4,-5)</ns0:f>
-        <ns0:v>7.493525753309694e+32</ns0:v>
+        <ns0:v>2.6726147398312744e+47</ns0:v>
       </ns0:c>
       <ns0:c r="G169" s="1" t="n">
         <ns0:v>34.0000000000001</ns0:v>
@@ -6450,15 +6330,15 @@
       </ns0:c>
       <ns0:c r="D170" s="1">
         <ns0:f>ROUND(D169*20,2-INT(LOG10(ABS(D169*20))))</ns0:f>
-        <ns0:v>1.7400000000000002e+188</ns0:v>
+        <ns0:v>5.56e+179</ns0:v>
       </ns0:c>
       <ns0:c r="E170" s="1">
         <ns0:f>D170</ns0:f>
-        <ns0:v>1.7400000000000002e+188</ns0:v>
+        <ns0:v>5.56e+179</ns0:v>
       </ns0:c>
       <ns0:c r="F170" s="1">
         <ns0:f>ROUND(F169*1.4,-5)</ns0:f>
-        <ns0:v>1.0490936054633572e+33</ns0:v>
+        <ns0:v>3.741660635763784e+47</ns0:v>
       </ns0:c>
       <ns0:c r="G170" s="1" t="n">
         <ns0:v>34.2000000000001</ns0:v>
@@ -6482,15 +6362,15 @@
       </ns0:c>
       <ns0:c r="D171" s="1">
         <ns0:f>ROUND(D170*20,2-INT(LOG10(ABS(D170*20))))</ns0:f>
-        <ns0:v>3.48e+189</ns0:v>
+        <ns0:v>1.11e+181</ns0:v>
       </ns0:c>
       <ns0:c r="E171" s="1">
         <ns0:f>D171</ns0:f>
-        <ns0:v>3.48e+189</ns0:v>
+        <ns0:v>1.11e+181</ns0:v>
       </ns0:c>
       <ns0:c r="F171" s="1">
         <ns0:f>ROUND(F170*1.4,-5)</ns0:f>
-        <ns0:v>1.4687310476486998e+33</ns0:v>
+        <ns0:v>5.238324890069298e+47</ns0:v>
       </ns0:c>
       <ns0:c r="G171" s="1" t="n">
         <ns0:v>34.4000000000001</ns0:v>
@@ -6514,15 +6394,15 @@
       </ns0:c>
       <ns0:c r="D172" s="1">
         <ns0:f>ROUND(D171*20,2-INT(LOG10(ABS(D171*20))))</ns0:f>
-        <ns0:v>6.96e+190</ns0:v>
+        <ns0:v>2.22e+182</ns0:v>
       </ns0:c>
       <ns0:c r="E172" s="1">
         <ns0:f>D172</ns0:f>
-        <ns0:v>6.96e+190</ns0:v>
+        <ns0:v>2.22e+182</ns0:v>
       </ns0:c>
       <ns0:c r="F172" s="1">
         <ns0:f>ROUND(F171*1.4,-5)</ns0:f>
-        <ns0:v>2.0562234667081797e+33</ns0:v>
+        <ns0:v>7.333654846097016e+47</ns0:v>
       </ns0:c>
       <ns0:c r="G172" s="1" t="n">
         <ns0:v>34.6000000000001</ns0:v>
@@ -6546,15 +6426,15 @@
       </ns0:c>
       <ns0:c r="D173" s="1">
         <ns0:f>ROUND(D172*20,2-INT(LOG10(ABS(D172*20))))</ns0:f>
-        <ns0:v>1.39e+192</ns0:v>
+        <ns0:v>4.44e+183</ns0:v>
       </ns0:c>
       <ns0:c r="E173" s="1">
         <ns0:f>D173</ns0:f>
-        <ns0:v>1.39e+192</ns0:v>
+        <ns0:v>4.44e+183</ns0:v>
       </ns0:c>
       <ns0:c r="F173" s="1">
         <ns0:f>ROUND(F172*1.4,-5)</ns0:f>
-        <ns0:v>2.878712853391451e+33</ns0:v>
+        <ns0:v>1.0267116784535822e+48</ns0:v>
       </ns0:c>
       <ns0:c r="G173" s="1" t="n">
         <ns0:v>34.8000000000001</ns0:v>
@@ -6578,15 +6458,15 @@
       </ns0:c>
       <ns0:c r="D174" s="1">
         <ns0:f>ROUND(D173*20,2-INT(LOG10(ABS(D173*20))))</ns0:f>
-        <ns0:v>2.78e+193</ns0:v>
+        <ns0:v>8.88e+184</ns0:v>
       </ns0:c>
       <ns0:c r="E174" s="1">
         <ns0:f>D174</ns0:f>
-        <ns0:v>2.78e+193</ns0:v>
+        <ns0:v>8.88e+184</ns0:v>
       </ns0:c>
       <ns0:c r="F174" s="1">
         <ns0:f>ROUND(F173*1.4,-5)</ns0:f>
-        <ns0:v>4.0301979947480315e+33</ns0:v>
+        <ns0:v>1.437396349835015e+48</ns0:v>
       </ns0:c>
       <ns0:c r="G174" s="1" t="n">
         <ns0:v>35.0000000000001</ns0:v>
@@ -6610,15 +6490,15 @@
       </ns0:c>
       <ns0:c r="D175" s="1">
         <ns0:f>ROUND(D174*20,2-INT(LOG10(ABS(D174*20))))</ns0:f>
-        <ns0:v>5.5599999999999995e+194</ns0:v>
+        <ns0:v>1.7799999999999998e+186</ns0:v>
       </ns0:c>
       <ns0:c r="E175" s="1">
         <ns0:f>D175</ns0:f>
-        <ns0:v>5.5599999999999995e+194</ns0:v>
+        <ns0:v>1.7799999999999998e+186</ns0:v>
       </ns0:c>
       <ns0:c r="F175" s="1">
         <ns0:f>ROUND(F174*1.4,-5)</ns0:f>
-        <ns0:v>5.642277192647244e+33</ns0:v>
+        <ns0:v>2.012354889769021e+48</ns0:v>
       </ns0:c>
       <ns0:c r="G175" s="1" t="n">
         <ns0:v>35.2000000000001</ns0:v>
@@ -6642,15 +6522,15 @@
       </ns0:c>
       <ns0:c r="D176" s="1">
         <ns0:f>ROUND(D175*20,2-INT(LOG10(ABS(D175*20))))</ns0:f>
-        <ns0:v>1.11e+196</ns0:v>
+        <ns0:v>3.56e+187</ns0:v>
       </ns0:c>
       <ns0:c r="E176" s="1">
         <ns0:f>D176</ns0:f>
-        <ns0:v>1.11e+196</ns0:v>
+        <ns0:v>3.56e+187</ns0:v>
       </ns0:c>
       <ns0:c r="F176" s="1">
         <ns0:f>ROUND(F175*1.4,-5)</ns0:f>
-        <ns0:v>7.899188069706141e+33</ns0:v>
+        <ns0:v>2.817296845676629e+48</ns0:v>
       </ns0:c>
       <ns0:c r="G176" s="1" t="n">
         <ns0:v>35.4000000000001</ns0:v>
@@ -6674,15 +6554,15 @@
       </ns0:c>
       <ns0:c r="D177" s="1">
         <ns0:f>ROUND(D176*20,2-INT(LOG10(ABS(D176*20))))</ns0:f>
-        <ns0:v>2.22e+197</ns0:v>
+        <ns0:v>7.12e+188</ns0:v>
       </ns0:c>
       <ns0:c r="E177" s="1">
         <ns0:f>D177</ns0:f>
-        <ns0:v>2.22e+197</ns0:v>
+        <ns0:v>7.12e+188</ns0:v>
       </ns0:c>
       <ns0:c r="F177" s="1">
         <ns0:f>ROUND(F176*1.4,-5)</ns0:f>
-        <ns0:v>1.1058863297588596e+34</ns0:v>
+        <ns0:v>3.9442155839472805e+48</ns0:v>
       </ns0:c>
       <ns0:c r="G177" s="1" t="n">
         <ns0:v>35.6000000000001</ns0:v>
@@ -6706,15 +6586,15 @@
       </ns0:c>
       <ns0:c r="D178" s="1">
         <ns0:f>ROUND(D177*20,2-INT(LOG10(ABS(D177*20))))</ns0:f>
-        <ns0:v>4.44e+198</ns0:v>
+        <ns0:v>1.42e+190</ns0:v>
       </ns0:c>
       <ns0:c r="E178" s="1">
         <ns0:f>D178</ns0:f>
-        <ns0:v>4.44e+198</ns0:v>
+        <ns0:v>1.42e+190</ns0:v>
       </ns0:c>
       <ns0:c r="F178" s="1">
         <ns0:f>ROUND(F177*1.4,-5)</ns0:f>
-        <ns0:v>1.5482408616624033e+34</ns0:v>
+        <ns0:v>5.521901817526192e+48</ns0:v>
       </ns0:c>
       <ns0:c r="G178" s="1" t="n">
         <ns0:v>35.8000000000001</ns0:v>
@@ -6738,15 +6618,15 @@
       </ns0:c>
       <ns0:c r="D179" s="1">
         <ns0:f>ROUND(D178*20,2-INT(LOG10(ABS(D178*20))))</ns0:f>
-        <ns0:v>8.88e+199</ns0:v>
+        <ns0:v>2.84e+191</ns0:v>
       </ns0:c>
       <ns0:c r="E179" s="1">
         <ns0:f>D179</ns0:f>
-        <ns0:v>8.88e+199</ns0:v>
+        <ns0:v>2.84e+191</ns0:v>
       </ns0:c>
       <ns0:c r="F179" s="1">
         <ns0:f>ROUND(F178*1.4,-5)</ns0:f>
-        <ns0:v>2.1675372063273644e+34</ns0:v>
+        <ns0:v>7.730662544536668e+48</ns0:v>
       </ns0:c>
       <ns0:c r="G179" s="1" t="n">
         <ns0:v>36.0000000000001</ns0:v>
@@ -6770,15 +6650,15 @@
       </ns0:c>
       <ns0:c r="D180" s="1">
         <ns0:f>ROUND(D179*20,2-INT(LOG10(ABS(D179*20))))</ns0:f>
-        <ns0:v>1.78e+201</ns0:v>
+        <ns0:v>5.68e+192</ns0:v>
       </ns0:c>
       <ns0:c r="E180" s="1">
         <ns0:f>D180</ns0:f>
-        <ns0:v>1.78e+201</ns0:v>
+        <ns0:v>5.68e+192</ns0:v>
       </ns0:c>
       <ns0:c r="F180" s="1">
         <ns0:f>ROUND(F179*1.4,-5)</ns0:f>
-        <ns0:v>3.03455208885831e+34</ns0:v>
+        <ns0:v>1.0822927562351333e+49</ns0:v>
       </ns0:c>
       <ns0:c r="G180" s="1" t="n">
         <ns0:v>36.2000000000001</ns0:v>
@@ -6802,15 +6682,15 @@
       </ns0:c>
       <ns0:c r="D181" s="1">
         <ns0:f>ROUND(D180*20,2-INT(LOG10(ABS(D180*20))))</ns0:f>
-        <ns0:v>3.5600000000000003e+202</ns0:v>
+        <ns0:v>1.1399999999999998e+194</ns0:v>
       </ns0:c>
       <ns0:c r="E181" s="1">
         <ns0:f>D181</ns0:f>
-        <ns0:v>3.5600000000000003e+202</ns0:v>
+        <ns0:v>1.1399999999999998e+194</ns0:v>
       </ns0:c>
       <ns0:c r="F181" s="1">
         <ns0:f>ROUND(F180*1.4,-5)</ns0:f>
-        <ns0:v>4.248372924401634e+34</ns0:v>
+        <ns0:v>1.5152098587291864e+49</ns0:v>
       </ns0:c>
       <ns0:c r="G181" s="1" t="n">
         <ns0:v>36.4000000000001</ns0:v>
@@ -6834,15 +6714,15 @@
       </ns0:c>
       <ns0:c r="D182" s="1">
         <ns0:f>ROUND(D181*20,2-INT(LOG10(ABS(D181*20))))</ns0:f>
-        <ns0:v>7.120000000000001e+203</ns0:v>
+        <ns0:v>2.28e+195</ns0:v>
       </ns0:c>
       <ns0:c r="E182" s="1">
         <ns0:f>D182</ns0:f>
-        <ns0:v>7.120000000000001e+203</ns0:v>
+        <ns0:v>2.28e+195</ns0:v>
       </ns0:c>
       <ns0:c r="F182" s="1">
         <ns0:f>ROUND(F181*1.4,-5)</ns0:f>
-        <ns0:v>5.9477220941622865e+34</ns0:v>
+        <ns0:v>2.1212938022208608e+49</ns0:v>
       </ns0:c>
       <ns0:c r="G182" s="1" t="n">
         <ns0:v>36.6000000000001</ns0:v>
@@ -6866,15 +6746,15 @@
       </ns0:c>
       <ns0:c r="D183" s="1">
         <ns0:f>ROUND(D182*20,2-INT(LOG10(ABS(D182*20))))</ns0:f>
-        <ns0:v>1.42e+205</ns0:v>
+        <ns0:v>4.56e+196</ns0:v>
       </ns0:c>
       <ns0:c r="E183" s="1">
         <ns0:f>D183</ns0:f>
-        <ns0:v>1.42e+205</ns0:v>
+        <ns0:v>4.56e+196</ns0:v>
       </ns0:c>
       <ns0:c r="F183" s="1">
         <ns0:f>ROUND(F182*1.4,-5)</ns0:f>
-        <ns0:v>8.3268109318272e+34</ns0:v>
+        <ns0:v>2.9698113231092047e+49</ns0:v>
       </ns0:c>
       <ns0:c r="G183" s="1" t="n">
         <ns0:v>36.8000000000001</ns0:v>
@@ -6898,15 +6778,15 @@
       </ns0:c>
       <ns0:c r="D184" s="1">
         <ns0:f>ROUND(D183*20,2-INT(LOG10(ABS(D183*20))))</ns0:f>
-        <ns0:v>2.84e+206</ns0:v>
+        <ns0:v>9.119999999999999e+197</ns0:v>
       </ns0:c>
       <ns0:c r="E184" s="1">
         <ns0:f>D184</ns0:f>
-        <ns0:v>2.84e+206</ns0:v>
+        <ns0:v>9.119999999999999e+197</ns0:v>
       </ns0:c>
       <ns0:c r="F184" s="1">
         <ns0:f>ROUND(F183*1.4,-5)</ns0:f>
-        <ns0:v>1.165753530455808e+35</ns0:v>
+        <ns0:v>4.1577358523528863e+49</ns0:v>
       </ns0:c>
       <ns0:c r="G184" s="1" t="n">
         <ns0:v>37.0000000000001</ns0:v>
@@ -6930,15 +6810,15 @@
       </ns0:c>
       <ns0:c r="D185" s="1">
         <ns0:f>ROUND(D184*20,2-INT(LOG10(ABS(D184*20))))</ns0:f>
-        <ns0:v>5.68e+207</ns0:v>
+        <ns0:v>1.8200000000000001e+199</ns0:v>
       </ns0:c>
       <ns0:c r="E185" s="1">
         <ns0:f>D185</ns0:f>
-        <ns0:v>5.68e+207</ns0:v>
+        <ns0:v>1.8200000000000001e+199</ns0:v>
       </ns0:c>
       <ns0:c r="F185" s="1">
         <ns0:f>ROUND(F184*1.4,-5)</ns0:f>
-        <ns0:v>1.6320549426381312e+35</ns0:v>
+        <ns0:v>5.82083019329404e+49</ns0:v>
       </ns0:c>
       <ns0:c r="G185" s="1" t="n">
         <ns0:v>37.2000000000001</ns0:v>
@@ -6962,15 +6842,15 @@
       </ns0:c>
       <ns0:c r="D186" s="1">
         <ns0:f>ROUND(D185*20,2-INT(LOG10(ABS(D185*20))))</ns0:f>
-        <ns0:v>1.14e+209</ns0:v>
+        <ns0:v>3.64e+200</ns0:v>
       </ns0:c>
       <ns0:c r="E186" s="1">
         <ns0:f>D186</ns0:f>
-        <ns0:v>1.14e+209</ns0:v>
+        <ns0:v>3.64e+200</ns0:v>
       </ns0:c>
       <ns0:c r="F186" s="1">
         <ns0:f>ROUND(F185*1.4,-5)</ns0:f>
-        <ns0:v>2.2848769196933836e+35</ns0:v>
+        <ns0:v>8.149162270611656e+49</ns0:v>
       </ns0:c>
       <ns0:c r="G186" s="1" t="n">
         <ns0:v>37.4000000000001</ns0:v>
@@ -6994,15 +6874,15 @@
       </ns0:c>
       <ns0:c r="D187" s="1">
         <ns0:f>ROUND(D186*20,2-INT(LOG10(ABS(D186*20))))</ns0:f>
-        <ns0:v>2.2799999999999998e+210</ns0:v>
+        <ns0:v>7.28e+201</ns0:v>
       </ns0:c>
       <ns0:c r="E187" s="1">
         <ns0:f>D187</ns0:f>
-        <ns0:v>2.2799999999999998e+210</ns0:v>
+        <ns0:v>7.28e+201</ns0:v>
       </ns0:c>
       <ns0:c r="F187" s="1">
         <ns0:f>ROUND(F186*1.4,-5)</ns0:f>
-        <ns0:v>3.1988276875707367e+35</ns0:v>
+        <ns0:v>1.1408827178856317e+50</ns0:v>
       </ns0:c>
       <ns0:c r="G187" s="1" t="n">
         <ns0:v>37.6000000000001</ns0:v>
@@ -7026,15 +6906,15 @@
       </ns0:c>
       <ns0:c r="D188" s="1">
         <ns0:f>ROUND(D187*20,2-INT(LOG10(ABS(D187*20))))</ns0:f>
-        <ns0:v>4.56e+211</ns0:v>
+        <ns0:v>1.46e+203</ns0:v>
       </ns0:c>
       <ns0:c r="E188" s="1">
         <ns0:f>D188</ns0:f>
-        <ns0:v>4.56e+211</ns0:v>
+        <ns0:v>1.46e+203</ns0:v>
       </ns0:c>
       <ns0:c r="F188" s="1">
         <ns0:f>ROUND(F187*1.4,-5)</ns0:f>
-        <ns0:v>4.478358762599031e+35</ns0:v>
+        <ns0:v>1.5972358050398844e+50</ns0:v>
       </ns0:c>
       <ns0:c r="G188" s="1" t="n">
         <ns0:v>37.8000000000001</ns0:v>
@@ -7058,15 +6938,15 @@
       </ns0:c>
       <ns0:c r="D189" s="1">
         <ns0:f>ROUND(D188*20,2-INT(LOG10(ABS(D188*20))))</ns0:f>
-        <ns0:v>9.12e+212</ns0:v>
+        <ns0:v>2.9199999999999997e+204</ns0:v>
       </ns0:c>
       <ns0:c r="E189" s="1">
         <ns0:f>D189</ns0:f>
-        <ns0:v>9.12e+212</ns0:v>
+        <ns0:v>2.9199999999999997e+204</ns0:v>
       </ns0:c>
       <ns0:c r="F189" s="1">
         <ns0:f>ROUND(F188*1.4,-5)</ns0:f>
-        <ns0:v>6.269702267638643e+35</ns0:v>
+        <ns0:v>2.236130127055838e+50</ns0:v>
       </ns0:c>
       <ns0:c r="G189" s="1" t="n">
         <ns0:v>38.0000000000001</ns0:v>
@@ -7090,15 +6970,15 @@
       </ns0:c>
       <ns0:c r="D190" s="1">
         <ns0:f>ROUND(D189*20,2-INT(LOG10(ABS(D189*20))))</ns0:f>
-        <ns0:v>1.8200000000000001e+214</ns0:v>
+        <ns0:v>5.84e+205</ns0:v>
       </ns0:c>
       <ns0:c r="E190" s="1">
         <ns0:f>D190</ns0:f>
-        <ns0:v>1.8200000000000001e+214</ns0:v>
+        <ns0:v>5.84e+205</ns0:v>
       </ns0:c>
       <ns0:c r="F190" s="1">
         <ns0:f>ROUND(F189*1.4,-5)</ns0:f>
-        <ns0:v>8.7775831746941e+35</ns0:v>
+        <ns0:v>3.130582177878173e+50</ns0:v>
       </ns0:c>
       <ns0:c r="G190" s="1" t="n">
         <ns0:v>38.2000000000001</ns0:v>
@@ -7122,15 +7002,15 @@
       </ns0:c>
       <ns0:c r="D191" s="1">
         <ns0:f>ROUND(D190*20,2-INT(LOG10(ABS(D190*20))))</ns0:f>
-        <ns0:v>3.64e+215</ns0:v>
+        <ns0:v>1.17e+207</ns0:v>
       </ns0:c>
       <ns0:c r="E191" s="1">
         <ns0:f>D191</ns0:f>
-        <ns0:v>3.64e+215</ns0:v>
+        <ns0:v>1.17e+207</ns0:v>
       </ns0:c>
       <ns0:c r="F191" s="1">
         <ns0:f>ROUND(F190*1.4,-5)</ns0:f>
-        <ns0:v>1.228861644457174e+36</ns0:v>
+        <ns0:v>4.382815049029442e+50</ns0:v>
       </ns0:c>
       <ns0:c r="G191" s="1" t="n">
         <ns0:v>38.4000000000001</ns0:v>
@@ -7154,15 +7034,15 @@
       </ns0:c>
       <ns0:c r="D192" s="1">
         <ns0:f>ROUND(D191*20,2-INT(LOG10(ABS(D191*20))))</ns0:f>
-        <ns0:v>7.28e+216</ns0:v>
+        <ns0:v>2.34e+208</ns0:v>
       </ns0:c>
       <ns0:c r="E192" s="1">
         <ns0:f>D192</ns0:f>
-        <ns0:v>7.28e+216</ns0:v>
+        <ns0:v>2.34e+208</ns0:v>
       </ns0:c>
       <ns0:c r="F192" s="1">
         <ns0:f>ROUND(F191*1.4,-5)</ns0:f>
-        <ns0:v>1.7204063022400436e+36</ns0:v>
+        <ns0:v>6.135941068641219e+50</ns0:v>
       </ns0:c>
       <ns0:c r="G192" s="1" t="n">
         <ns0:v>38.6000000000001</ns0:v>
@@ -7186,15 +7066,15 @@
       </ns0:c>
       <ns0:c r="D193" s="1">
         <ns0:f>ROUND(D192*20,2-INT(LOG10(ABS(D192*20))))</ns0:f>
-        <ns0:v>1.4599999999999999e+218</ns0:v>
+        <ns0:v>4.68e+209</ns0:v>
       </ns0:c>
       <ns0:c r="E193" s="1">
         <ns0:f>D193</ns0:f>
-        <ns0:v>1.4599999999999999e+218</ns0:v>
+        <ns0:v>4.68e+209</ns0:v>
       </ns0:c>
       <ns0:c r="F193" s="1">
         <ns0:f>ROUND(F192*1.4,-5)</ns0:f>
-        <ns0:v>2.4085688231360608e+36</ns0:v>
+        <ns0:v>8.590317496097706e+50</ns0:v>
       </ns0:c>
       <ns0:c r="G193" s="1" t="n">
         <ns0:v>38.8000000000001</ns0:v>
@@ -7218,15 +7098,15 @@
       </ns0:c>
       <ns0:c r="D194" s="1">
         <ns0:f>ROUND(D193*20,2-INT(LOG10(ABS(D193*20))))</ns0:f>
-        <ns0:v>2.9199999999999997e+219</ns0:v>
+        <ns0:v>9.359999999999999e+210</ns0:v>
       </ns0:c>
       <ns0:c r="E194" s="1">
         <ns0:f>D194</ns0:f>
-        <ns0:v>2.9199999999999997e+219</ns0:v>
+        <ns0:v>9.359999999999999e+210</ns0:v>
       </ns0:c>
       <ns0:c r="F194" s="1">
         <ns0:f>ROUND(F193*1.4,-5)</ns0:f>
-        <ns0:v>3.371996352390485e+36</ns0:v>
+        <ns0:v>1.2026444494536786e+51</ns0:v>
       </ns0:c>
       <ns0:c r="G194" s="1" t="n">
         <ns0:v>39.0000000000001</ns0:v>
@@ -7250,15 +7130,15 @@
       </ns0:c>
       <ns0:c r="D195" s="1">
         <ns0:f>ROUND(D194*20,2-INT(LOG10(ABS(D194*20))))</ns0:f>
-        <ns0:v>5.84e+220</ns0:v>
+        <ns0:v>1.87e+212</ns0:v>
       </ns0:c>
       <ns0:c r="E195" s="1">
         <ns0:f>D195</ns0:f>
-        <ns0:v>5.84e+220</ns0:v>
+        <ns0:v>1.87e+212</ns0:v>
       </ns0:c>
       <ns0:c r="F195" s="1">
         <ns0:f>ROUND(F194*1.4,-5)</ns0:f>
-        <ns0:v>4.720794893346679e+36</ns0:v>
+        <ns0:v>1.68370222923515e+51</ns0:v>
       </ns0:c>
       <ns0:c r="G195" s="1" t="n">
         <ns0:v>39.2000000000001</ns0:v>
@@ -7282,15 +7162,15 @@
       </ns0:c>
       <ns0:c r="D196" s="1">
         <ns0:f>ROUND(D195*20,2-INT(LOG10(ABS(D195*20))))</ns0:f>
-        <ns0:v>1.17e+222</ns0:v>
+        <ns0:v>3.74e+213</ns0:v>
       </ns0:c>
       <ns0:c r="E196" s="1">
         <ns0:f>D196</ns0:f>
-        <ns0:v>1.17e+222</ns0:v>
+        <ns0:v>3.74e+213</ns0:v>
       </ns0:c>
       <ns0:c r="F196" s="1">
         <ns0:f>ROUND(F195*1.4,-5)</ns0:f>
-        <ns0:v>6.60911285068535e+36</ns0:v>
+        <ns0:v>2.35718312092921e+51</ns0:v>
       </ns0:c>
       <ns0:c r="G196" s="1" t="n">
         <ns0:v>39.4000000000001</ns0:v>
@@ -7314,15 +7194,15 @@
       </ns0:c>
       <ns0:c r="D197" s="1">
         <ns0:f>ROUND(D196*20,2-INT(LOG10(ABS(D196*20))))</ns0:f>
-        <ns0:v>2.34e+223</ns0:v>
+        <ns0:v>7.48e+214</ns0:v>
       </ns0:c>
       <ns0:c r="E197" s="1">
         <ns0:f>D197</ns0:f>
-        <ns0:v>2.34e+223</ns0:v>
+        <ns0:v>7.48e+214</ns0:v>
       </ns0:c>
       <ns0:c r="F197" s="1">
         <ns0:f>ROUND(F196*1.4,-5)</ns0:f>
-        <ns0:v>9.252757990959492e+36</ns0:v>
+        <ns0:v>3.300056369300893e+51</ns0:v>
       </ns0:c>
       <ns0:c r="G197" s="1" t="n">
         <ns0:v>39.6000000000001</ns0:v>
@@ -7346,15 +7226,15 @@
       </ns0:c>
       <ns0:c r="D198" s="1">
         <ns0:f>ROUND(D197*20,2-INT(LOG10(ABS(D197*20))))</ns0:f>
-        <ns0:v>4.6799999999999994e+224</ns0:v>
+        <ns0:v>1.5000000000000002e+216</ns0:v>
       </ns0:c>
       <ns0:c r="E198" s="1">
         <ns0:f>D198</ns0:f>
-        <ns0:v>4.6799999999999994e+224</ns0:v>
+        <ns0:v>1.5000000000000002e+216</ns0:v>
       </ns0:c>
       <ns0:c r="F198" s="1">
         <ns0:f>ROUND(F197*1.4,-5)</ns0:f>
-        <ns0:v>1.2953861187343288e+37</ns0:v>
+        <ns0:v>4.6200789170212506e+51</ns0:v>
       </ns0:c>
       <ns0:c r="G198" s="1" t="n">
         <ns0:v>39.8000000000001</ns0:v>
@@ -7378,15 +7258,15 @@
       </ns0:c>
       <ns0:c r="D199" s="1">
         <ns0:f>ROUND(D198*20,2-INT(LOG10(ABS(D198*20))))</ns0:f>
-        <ns0:v>9.360000000000001e+225</ns0:v>
+        <ns0:v>3e+217</ns0:v>
       </ns0:c>
       <ns0:c r="E199" s="1">
         <ns0:f>D199</ns0:f>
-        <ns0:v>9.360000000000001e+225</ns0:v>
+        <ns0:v>3e+217</ns0:v>
       </ns0:c>
       <ns0:c r="F199" s="1">
         <ns0:f>ROUND(F198*1.4,-5)</ns0:f>
-        <ns0:v>1.8135405662280603e+37</ns0:v>
+        <ns0:v>6.46811048382975e+51</ns0:v>
       </ns0:c>
       <ns0:c r="G199" s="1" t="n">
         <ns0:v>40.0000000000001</ns0:v>
@@ -7410,15 +7290,15 @@
       </ns0:c>
       <ns0:c r="D200" s="1">
         <ns0:f>ROUND(D199*20,2-INT(LOG10(ABS(D199*20))))</ns0:f>
-        <ns0:v>1.8700000000000002e+227</ns0:v>
+        <ns0:v>6e+218</ns0:v>
       </ns0:c>
       <ns0:c r="E200" s="1">
         <ns0:f>D200</ns0:f>
-        <ns0:v>1.8700000000000002e+227</ns0:v>
+        <ns0:v>6e+218</ns0:v>
       </ns0:c>
       <ns0:c r="F200" s="1">
         <ns0:f>ROUND(F199*1.4,-5)</ns0:f>
-        <ns0:v>2.5389567927192844e+37</ns0:v>
+        <ns0:v>9.05535467736165e+51</ns0:v>
       </ns0:c>
       <ns0:c r="G200" s="1" t="n">
         <ns0:v>40.2000000000001</ns0:v>
@@ -7442,15 +7322,15 @@
       </ns0:c>
       <ns0:c r="D201" s="1">
         <ns0:f>ROUND(D200*20,2-INT(LOG10(ABS(D200*20))))</ns0:f>
-        <ns0:v>3.7400000000000006e+228</ns0:v>
+        <ns0:v>1.2e+220</ns0:v>
       </ns0:c>
       <ns0:c r="E201" s="1">
         <ns0:f>D201</ns0:f>
-        <ns0:v>3.7400000000000006e+228</ns0:v>
+        <ns0:v>1.2e+220</ns0:v>
       </ns0:c>
       <ns0:c r="F201" s="1">
         <ns0:f>ROUND(F200*1.4,-5)</ns0:f>
-        <ns0:v>3.554539509806998e+37</ns0:v>
+        <ns0:v>1.267749654830631e+52</ns0:v>
       </ns0:c>
       <ns0:c r="G201" s="1" t="n">
         <ns0:v>40.4000000000001</ns0:v>
@@ -7474,15 +7354,15 @@
       </ns0:c>
       <ns0:c r="D202" s="1">
         <ns0:f>ROUND(D201*20,2-INT(LOG10(ABS(D201*20))))</ns0:f>
-        <ns0:v>7.48e+229</ns0:v>
+        <ns0:v>2.3999999999999998e+221</ns0:v>
       </ns0:c>
       <ns0:c r="E202" s="1">
         <ns0:f>D202</ns0:f>
-        <ns0:v>7.48e+229</ns0:v>
+        <ns0:v>2.3999999999999998e+221</ns0:v>
       </ns0:c>
       <ns0:c r="F202" s="1">
         <ns0:f>ROUND(F201*1.4,-5)</ns0:f>
-        <ns0:v>4.976355313729797e+37</ns0:v>
+        <ns0:v>1.774849516762883e+52</ns0:v>
       </ns0:c>
       <ns0:c r="G202" s="1" t="n">
         <ns0:v>40.6000000000001</ns0:v>
@@ -7506,15 +7386,15 @@
       </ns0:c>
       <ns0:c r="D203" s="1">
         <ns0:f>ROUND(D202*20,2-INT(LOG10(ABS(D202*20))))</ns0:f>
-        <ns0:v>1.4999999999999999e+231</ns0:v>
+        <ns0:v>4.8e+222</ns0:v>
       </ns0:c>
       <ns0:c r="E203" s="1">
         <ns0:f>D203</ns0:f>
-        <ns0:v>1.4999999999999999e+231</ns0:v>
+        <ns0:v>4.8e+222</ns0:v>
       </ns0:c>
       <ns0:c r="F203" s="1">
         <ns0:f>ROUND(F202*1.4,-5)</ns0:f>
-        <ns0:v>6.966897439221714e+37</ns0:v>
+        <ns0:v>2.484789323468036e+52</ns0:v>
       </ns0:c>
       <ns0:c r="G203" s="1" t="n">
         <ns0:v>40.8000000000001</ns0:v>
@@ -7538,15 +7418,15 @@
       </ns0:c>
       <ns0:c r="D204" s="1">
         <ns0:f>ROUND(D203*20,2-INT(LOG10(ABS(D203*20))))</ns0:f>
-        <ns0:v>3e+232</ns0:v>
+        <ns0:v>9.6e+223</ns0:v>
       </ns0:c>
       <ns0:c r="E204" s="1">
         <ns0:f>D204</ns0:f>
-        <ns0:v>3e+232</ns0:v>
+        <ns0:v>9.6e+223</ns0:v>
       </ns0:c>
       <ns0:c r="F204" s="1">
         <ns0:f>ROUND(F203*1.4,-5)</ns0:f>
-        <ns0:v>9.753656414910399e+37</ns0:v>
+        <ns0:v>3.47870505285525e+52</ns0:v>
       </ns0:c>
       <ns0:c r="G204" s="1" t="n">
         <ns0:v>41.0000000000001</ns0:v>
@@ -7570,15 +7450,15 @@
       </ns0:c>
       <ns0:c r="D205" s="1">
         <ns0:f>ROUND(D204*20,2-INT(LOG10(ABS(D204*20))))</ns0:f>
-        <ns0:v>6e+233</ns0:v>
+        <ns0:v>1.92e+225</ns0:v>
       </ns0:c>
       <ns0:c r="E205" s="1">
         <ns0:f>D205</ns0:f>
-        <ns0:v>6e+233</ns0:v>
+        <ns0:v>1.92e+225</ns0:v>
       </ns0:c>
       <ns0:c r="F205" s="1">
         <ns0:f>ROUND(F204*1.4,-5)</ns0:f>
-        <ns0:v>1.3655118980874558e+38</ns0:v>
+        <ns0:v>4.87018707399735e+52</ns0:v>
       </ns0:c>
       <ns0:c r="G205" s="1" t="n">
         <ns0:v>41.2000000000001</ns0:v>
@@ -7602,15 +7482,15 @@
       </ns0:c>
       <ns0:c r="D206" s="1">
         <ns0:f>ROUND(D205*20,2-INT(LOG10(ABS(D205*20))))</ns0:f>
-        <ns0:v>1.2000000000000001e+235</ns0:v>
+        <ns0:v>3.84e+226</ns0:v>
       </ns0:c>
       <ns0:c r="E206" s="1">
         <ns0:f>D206</ns0:f>
-        <ns0:v>1.2000000000000001e+235</ns0:v>
+        <ns0:v>3.84e+226</ns0:v>
       </ns0:c>
       <ns0:c r="F206" s="1">
         <ns0:f>ROUND(F205*1.4,-5)</ns0:f>
-        <ns0:v>1.9117166573224382e+38</ns0:v>
+        <ns0:v>6.81826190359629e+52</ns0:v>
       </ns0:c>
       <ns0:c r="G206" s="1" t="n">
         <ns0:v>41.4000000000001</ns0:v>
@@ -7634,15 +7514,15 @@
       </ns0:c>
       <ns0:c r="D207" s="1">
         <ns0:f>ROUND(D206*20,2-INT(LOG10(ABS(D206*20))))</ns0:f>
-        <ns0:v>2.4e+236</ns0:v>
+        <ns0:v>7.68e+227</ns0:v>
       </ns0:c>
       <ns0:c r="E207" s="1">
         <ns0:f>D207</ns0:f>
-        <ns0:v>2.4e+236</ns0:v>
+        <ns0:v>7.68e+227</ns0:v>
       </ns0:c>
       <ns0:c r="F207" s="1">
         <ns0:f>ROUND(F206*1.4,-5)</ns0:f>
-        <ns0:v>2.6764033202514134e+38</ns0:v>
+        <ns0:v>9.545566665034806e+52</ns0:v>
       </ns0:c>
       <ns0:c r="G207" s="1" t="n">
         <ns0:v>41.6000000000001</ns0:v>
@@ -7666,15 +7546,15 @@
       </ns0:c>
       <ns0:c r="D208" s="1">
         <ns0:f>ROUND(D207*20,2-INT(LOG10(ABS(D207*20))))</ns0:f>
-        <ns0:v>4.8000000000000004e+237</ns0:v>
+        <ns0:v>1.5400000000000002e+229</ns0:v>
       </ns0:c>
       <ns0:c r="E208" s="1">
         <ns0:f>D208</ns0:f>
-        <ns0:v>4.8000000000000004e+237</ns0:v>
+        <ns0:v>1.5400000000000002e+229</ns0:v>
       </ns0:c>
       <ns0:c r="F208" s="1">
         <ns0:f>ROUND(F207*1.4,-5)</ns0:f>
-        <ns0:v>3.746964648351978e+38</ns0:v>
+        <ns0:v>1.3363793331048728e+53</ns0:v>
       </ns0:c>
       <ns0:c r="G208" s="1" t="n">
         <ns0:v>41.8000000000001</ns0:v>
@@ -7698,15 +7578,15 @@
       </ns0:c>
       <ns0:c r="D209" s="1">
         <ns0:f>ROUND(D208*20,2-INT(LOG10(ABS(D208*20))))</ns0:f>
-        <ns0:v>9.6e+238</ns0:v>
+        <ns0:v>3.0799999999999998e+230</ns0:v>
       </ns0:c>
       <ns0:c r="E209" s="1">
         <ns0:f>D209</ns0:f>
-        <ns0:v>9.6e+238</ns0:v>
+        <ns0:v>3.0799999999999998e+230</ns0:v>
       </ns0:c>
       <ns0:c r="F209" s="1">
         <ns0:f>ROUND(F208*1.4,-5)</ns0:f>
-        <ns0:v>5.245750507692769e+38</ns0:v>
+        <ns0:v>1.8709310663468219e+53</ns0:v>
       </ns0:c>
       <ns0:c r="G209" s="1" t="n">
         <ns0:v>42.0000000000001</ns0:v>
@@ -7730,15 +7610,15 @@
       </ns0:c>
       <ns0:c r="D210" s="1">
         <ns0:f>ROUND(D209*20,2-INT(LOG10(ABS(D209*20))))</ns0:f>
-        <ns0:v>1.92e+240</ns0:v>
+        <ns0:v>6.16e+231</ns0:v>
       </ns0:c>
       <ns0:c r="E210" s="1">
         <ns0:f>D210</ns0:f>
-        <ns0:v>1.92e+240</ns0:v>
+        <ns0:v>6.16e+231</ns0:v>
       </ns0:c>
       <ns0:c r="F210" s="1">
         <ns0:f>ROUND(F209*1.4,-5)</ns0:f>
-        <ns0:v>7.344050710769877e+38</ns0:v>
+        <ns0:v>2.6193034928855506e+53</ns0:v>
       </ns0:c>
       <ns0:c r="G210" s="1" t="n">
         <ns0:v>42.2000000000001</ns0:v>
@@ -7762,15 +7642,15 @@
       </ns0:c>
       <ns0:c r="D211" s="1">
         <ns0:f>ROUND(D210*20,2-INT(LOG10(ABS(D210*20))))</ns0:f>
-        <ns0:v>3.84e+241</ns0:v>
+        <ns0:v>1.23e+233</ns0:v>
       </ns0:c>
       <ns0:c r="E211" s="1">
         <ns0:f>D211</ns0:f>
-        <ns0:v>3.84e+241</ns0:v>
+        <ns0:v>1.23e+233</ns0:v>
       </ns0:c>
       <ns0:c r="F211" s="1">
         <ns0:f>ROUND(F210*1.4,-5)</ns0:f>
-        <ns0:v>1.0281670995077828e+39</ns0:v>
+        <ns0:v>3.6670248900397707e+53</ns0:v>
       </ns0:c>
       <ns0:c r="G211" s="1" t="n">
         <ns0:v>42.4000000000001</ns0:v>
@@ -7794,15 +7674,15 @@
       </ns0:c>
       <ns0:c r="D212" s="1">
         <ns0:f>ROUND(D211*20,2-INT(LOG10(ABS(D211*20))))</ns0:f>
-        <ns0:v>7.680000000000001e+242</ns0:v>
+        <ns0:v>2.4599999999999998e+234</ns0:v>
       </ns0:c>
       <ns0:c r="E212" s="1">
         <ns0:f>D212</ns0:f>
-        <ns0:v>7.680000000000001e+242</ns0:v>
+        <ns0:v>2.4599999999999998e+234</ns0:v>
       </ns0:c>
       <ns0:c r="F212" s="1">
         <ns0:f>ROUND(F211*1.4,-5)</ns0:f>
-        <ns0:v>1.439433939310896e+39</ns0:v>
+        <ns0:v>5.133834846055678e+53</ns0:v>
       </ns0:c>
       <ns0:c r="G212" s="1" t="n">
         <ns0:v>42.6000000000002</ns0:v>
@@ -7826,15 +7706,15 @@
       </ns0:c>
       <ns0:c r="D213" s="1">
         <ns0:f>ROUND(D212*20,2-INT(LOG10(ABS(D212*20))))</ns0:f>
-        <ns0:v>1.54e+244</ns0:v>
+        <ns0:v>4.92e+235</ns0:v>
       </ns0:c>
       <ns0:c r="E213" s="1">
         <ns0:f>D213</ns0:f>
-        <ns0:v>1.54e+244</ns0:v>
+        <ns0:v>4.92e+235</ns0:v>
       </ns0:c>
       <ns0:c r="F213" s="1">
         <ns0:f>ROUND(F212*1.4,-5)</ns0:f>
-        <ns0:v>2.015207515035254e+39</ns0:v>
+        <ns0:v>7.187368784477949e+53</ns0:v>
       </ns0:c>
       <ns0:c r="G213" s="1" t="n">
         <ns0:v>42.8000000000002</ns0:v>
@@ -7858,15 +7738,15 @@
       </ns0:c>
       <ns0:c r="D214" s="1">
         <ns0:f>ROUND(D213*20,2-INT(LOG10(ABS(D213*20))))</ns0:f>
-        <ns0:v>3.08e+245</ns0:v>
+        <ns0:v>9.840000000000001e+236</ns0:v>
       </ns0:c>
       <ns0:c r="E214" s="1">
         <ns0:f>D214</ns0:f>
-        <ns0:v>3.08e+245</ns0:v>
+        <ns0:v>9.840000000000001e+236</ns0:v>
       </ns0:c>
       <ns0:c r="F214" s="1">
         <ns0:f>ROUND(F213*1.4,-5)</ns0:f>
-        <ns0:v>2.8212905210493555e+39</ns0:v>
+        <ns0:v>1.0062316298269128e+54</ns0:v>
       </ns0:c>
       <ns0:c r="G214" s="1" t="n">
         <ns0:v>43.0000000000001</ns0:v>
@@ -7890,15 +7770,15 @@
       </ns0:c>
       <ns0:c r="D215" s="1">
         <ns0:f>ROUND(D214*20,2-INT(LOG10(ABS(D214*20))))</ns0:f>
-        <ns0:v>6.1600000000000006e+246</ns0:v>
+        <ns0:v>1.97e+238</ns0:v>
       </ns0:c>
       <ns0:c r="E215" s="1">
         <ns0:f>D215</ns0:f>
-        <ns0:v>6.1600000000000006e+246</ns0:v>
+        <ns0:v>1.97e+238</ns0:v>
       </ns0:c>
       <ns0:c r="F215" s="1">
         <ns0:f>ROUND(F214*1.4,-5)</ns0:f>
-        <ns0:v>3.9498067294690976e+39</ns0:v>
+        <ns0:v>1.4087242817576779e+54</ns0:v>
       </ns0:c>
       <ns0:c r="G215" s="1" t="n">
         <ns0:v>43.2000000000002</ns0:v>
@@ -7922,15 +7802,15 @@
       </ns0:c>
       <ns0:c r="D216" s="1">
         <ns0:f>ROUND(D215*20,2-INT(LOG10(ABS(D215*20))))</ns0:f>
-        <ns0:v>1.23e+248</ns0:v>
+        <ns0:v>3.94e+239</ns0:v>
       </ns0:c>
       <ns0:c r="E216" s="1">
         <ns0:f>D216</ns0:f>
-        <ns0:v>1.23e+248</ns0:v>
+        <ns0:v>3.94e+239</ns0:v>
       </ns0:c>
       <ns0:c r="F216" s="1">
         <ns0:f>ROUND(F215*1.4,-5)</ns0:f>
-        <ns0:v>5.529729421256736e+39</ns0:v>
+        <ns0:v>1.9722139944607488e+54</ns0:v>
       </ns0:c>
       <ns0:c r="G216" s="1" t="n">
         <ns0:v>43.4000000000002</ns0:v>
@@ -7954,15 +7834,15 @@
       </ns0:c>
       <ns0:c r="D217" s="1">
         <ns0:f>ROUND(D216*20,2-INT(LOG10(ABS(D216*20))))</ns0:f>
-        <ns0:v>2.46e+249</ns0:v>
+        <ns0:v>7.88e+240</ns0:v>
       </ns0:c>
       <ns0:c r="E217" s="1">
         <ns0:f>D217</ns0:f>
-        <ns0:v>2.46e+249</ns0:v>
+        <ns0:v>7.88e+240</ns0:v>
       </ns0:c>
       <ns0:c r="F217" s="1">
         <ns0:f>ROUND(F216*1.4,-5)</ns0:f>
-        <ns0:v>7.74162118975943e+39</ns0:v>
+        <ns0:v>2.7610995922450485e+54</ns0:v>
       </ns0:c>
       <ns0:c r="G217" s="1" t="n">
         <ns0:v>43.6000000000002</ns0:v>
@@ -7986,15 +7866,15 @@
       </ns0:c>
       <ns0:c r="D218" s="1">
         <ns0:f>ROUND(D217*20,2-INT(LOG10(ABS(D217*20))))</ns0:f>
-        <ns0:v>4.92e+250</ns0:v>
+        <ns0:v>1.58e+242</ns0:v>
       </ns0:c>
       <ns0:c r="E218" s="1">
         <ns0:f>D218</ns0:f>
-        <ns0:v>4.92e+250</ns0:v>
+        <ns0:v>1.58e+242</ns0:v>
       </ns0:c>
       <ns0:c r="F218" s="1">
         <ns0:f>ROUND(F217*1.4,-5)</ns0:f>
-        <ns0:v>1.0838269665663202e+40</ns0:v>
+        <ns0:v>3.865539429143068e+54</ns0:v>
       </ns0:c>
       <ns0:c r="G218" s="1" t="n">
         <ns0:v>43.8000000000002</ns0:v>
@@ -8018,15 +7898,15 @@
       </ns0:c>
       <ns0:c r="D219" s="1">
         <ns0:f>ROUND(D218*20,2-INT(LOG10(ABS(D218*20))))</ns0:f>
-        <ns0:v>9.84e+251</ns0:v>
+        <ns0:v>3.16e+243</ns0:v>
       </ns0:c>
       <ns0:c r="E219" s="1">
         <ns0:f>D219</ns0:f>
-        <ns0:v>9.84e+251</ns0:v>
+        <ns0:v>3.16e+243</ns0:v>
       </ns0:c>
       <ns0:c r="F219" s="1">
         <ns0:f>ROUND(F218*1.4,-5)</ns0:f>
-        <ns0:v>1.5173577531928483e+40</ns0:v>
+        <ns0:v>5.4117552008002956e+54</ns0:v>
       </ns0:c>
       <ns0:c r="G219" s="1" t="n">
         <ns0:v>44.0000000000002</ns0:v>
@@ -8050,15 +7930,15 @@
       </ns0:c>
       <ns0:c r="D220" s="1">
         <ns0:f>ROUND(D219*20,2-INT(LOG10(ABS(D219*20))))</ns0:f>
-        <ns0:v>1.97e+253</ns0:v>
+        <ns0:v>6.32e+244</ns0:v>
       </ns0:c>
       <ns0:c r="E220" s="1">
         <ns0:f>D220</ns0:f>
-        <ns0:v>1.97e+253</ns0:v>
+        <ns0:v>6.32e+244</ns0:v>
       </ns0:c>
       <ns0:c r="F220" s="1">
         <ns0:f>ROUND(F219*1.4,-5)</ns0:f>
-        <ns0:v>2.1243008544699876e+40</ns0:v>
+        <ns0:v>7.576457281120413e+54</ns0:v>
       </ns0:c>
       <ns0:c r="G220" s="1" t="n">
         <ns0:v>44.2000000000002</ns0:v>
@@ -8082,15 +7962,15 @@
       </ns0:c>
       <ns0:c r="D221" s="1">
         <ns0:f>ROUND(D220*20,2-INT(LOG10(ABS(D220*20))))</ns0:f>
-        <ns0:v>3.94e+254</ns0:v>
+        <ns0:v>1.2600000000000001e+246</ns0:v>
       </ns0:c>
       <ns0:c r="E221" s="1">
         <ns0:f>D221</ns0:f>
-        <ns0:v>3.94e+254</ns0:v>
+        <ns0:v>1.2600000000000001e+246</ns0:v>
       </ns0:c>
       <ns0:c r="F221" s="1">
         <ns0:f>ROUND(F220*1.4,-5)</ns0:f>
-        <ns0:v>2.9740211962579824e+40</ns0:v>
+        <ns0:v>1.0607040193568578e+55</ns0:v>
       </ns0:c>
       <ns0:c r="G221" s="1" t="n">
         <ns0:v>44.4000000000002</ns0:v>
@@ -8114,15 +7994,15 @@
       </ns0:c>
       <ns0:c r="D222" s="1">
         <ns0:f>ROUND(D221*20,2-INT(LOG10(ABS(D221*20))))</ns0:f>
-        <ns0:v>7.879999999999999e+255</ns0:v>
+        <ns0:v>2.5200000000000003e+247</ns0:v>
       </ns0:c>
       <ns0:c r="E222" s="1">
         <ns0:f>D222</ns0:f>
-        <ns0:v>7.879999999999999e+255</ns0:v>
+        <ns0:v>2.5200000000000003e+247</ns0:v>
       </ns0:c>
       <ns0:c r="F222" s="1">
         <ns0:f>ROUND(F221*1.4,-5)</ns0:f>
-        <ns0:v>4.1636296747611744e+40</ns0:v>
+        <ns0:v>1.4849856270996007e+55</ns0:v>
       </ns0:c>
       <ns0:c r="G222" s="1" t="n">
         <ns0:v>44.6000000000002</ns0:v>
@@ -8146,15 +8026,15 @@
       </ns0:c>
       <ns0:c r="D223" s="1">
         <ns0:f>ROUND(D222*20,2-INT(LOG10(ABS(D222*20))))</ns0:f>
-        <ns0:v>1.58e+257</ns0:v>
+        <ns0:v>5.040000000000001e+248</ns0:v>
       </ns0:c>
       <ns0:c r="E223" s="1">
         <ns0:f>D223</ns0:f>
-        <ns0:v>1.58e+257</ns0:v>
+        <ns0:v>5.040000000000001e+248</ns0:v>
       </ns0:c>
       <ns0:c r="F223" s="1">
         <ns0:f>ROUND(F222*1.4,-5)</ns0:f>
-        <ns0:v>5.829081544665644e+40</ns0:v>
+        <ns0:v>2.0789798779394408e+55</ns0:v>
       </ns0:c>
       <ns0:c r="G223" s="1" t="n">
         <ns0:v>44.8000000000002</ns0:v>

</xml_diff>

<commit_message>
Correct QA combat engine to formal Presented path, add real scene comparison and cross-frame fixed clock
</commit_message>
<xml_diff>
--- a/space-battleship/config_excel/level.xlsx
+++ b/space-battleship/config_excel/level.xlsx
@@ -1553,7 +1553,7 @@
         <ns0:v>602880.1175788565</ns0:v>
       </ns0:c>
       <ns0:c r="F14" s="1" t="n">
-        <ns0:v>188.7066854784442</ns0:v>
+        <ns0:v>24692.16234188062</ns0:v>
       </ns0:c>
       <ns0:c r="G14" s="1" t="n">
         <ns0:v>3</ns0:v>
@@ -1581,7 +1581,7 @@
         <ns0:v>6450407.623907364</ns0:v>
       </ns0:c>
       <ns0:c r="F15" s="1" t="n">
-        <ns0:v>2019.033315579911</ns0:v>
+        <ns0:v>34569.02727863286</ns0:v>
       </ns0:c>
       <ns0:c r="G15" s="1" t="n">
         <ns0:v>3.2</ns0:v>
@@ -1609,7 +1609,7 @@
         <ns0:v>69014978.76834521</ns0:v>
       </ns0:c>
       <ns0:c r="F16" s="1" t="n">
-        <ns0:v>21602.284620103</ns0:v>
+        <ns0:v>48396.638190086</ns0:v>
       </ns0:c>
       <ns0:c r="G16" s="1" t="n">
         <ns0:v>3.4</ns0:v>

</xml_diff>

<commit_message>
Freeze v9 formal-scene candidate and retain teaching, clock and failed-run evidence
</commit_message>
<xml_diff>
--- a/space-battleship/config_excel/level.xlsx
+++ b/space-battleship/config_excel/level.xlsx
@@ -1553,7 +1553,7 @@
         <ns0:v>602880.1175788565</ns0:v>
       </ns0:c>
       <ns0:c r="F14" s="1" t="n">
-        <ns0:v>24692.16234188062</ns0:v>
+        <ns0:v>18870.66854784442</ns0:v>
       </ns0:c>
       <ns0:c r="G14" s="1" t="n">
         <ns0:v>3</ns0:v>
@@ -1581,7 +1581,7 @@
         <ns0:v>6450407.623907364</ns0:v>
       </ns0:c>
       <ns0:c r="F15" s="1" t="n">
-        <ns0:v>34569.02727863286</ns0:v>
+        <ns0:v>97368.504802272</ns0:v>
       </ns0:c>
       <ns0:c r="G15" s="1" t="n">
         <ns0:v>3.2</ns0:v>
@@ -1609,7 +1609,7 @@
         <ns0:v>69014978.76834521</ns0:v>
       </ns0:c>
       <ns0:c r="F16" s="1" t="n">
-        <ns0:v>48396.638190086</ns0:v>
+        <ns0:v>502400.0979823805</ns0:v>
       </ns0:c>
       <ns0:c r="G16" s="1" t="n">
         <ns0:v>3.4</ns0:v>
@@ -1637,7 +1637,7 @@
         <ns0:v>738413379.7593849</ns0:v>
       </ns0:c>
       <ns0:c r="F17" s="1" t="n">
-        <ns0:v>231129.7675015848</ns0:v>
+        <ns0:v>2592274.154412361</ns0:v>
       </ns0:c>
       <ns0:c r="G17" s="1" t="n">
         <ns0:v>3.6</ns0:v>
@@ -1665,7 +1665,7 @@
         <ns0:v>7900521439.525051</ns0:v>
       </ns0:c>
       <ns0:c r="F18" s="1" t="n">
-        <ns0:v>2472931.468351421</ns0:v>
+        <ns0:v>13375565.24893431</ns0:v>
       </ns0:c>
       <ns0:c r="G18" s="1" t="n">
         <ns0:v>3.8</ns0:v>
@@ -1693,7 +1693,7 @@
         <ns0:v>84530211298.0865</ns0:v>
       </ns0:c>
       <ns0:c r="F19" s="1" t="n">
-        <ns0:v>26458686.44816936</ns0:v>
+        <ns0:v>69014978.76834521</ns0:v>
       </ns0:c>
       <ns0:c r="G19" s="1" t="n">
         <ns0:v>4</ns0:v>
@@ -1721,7 +1721,7 @@
         <ns0:v>904415825815.2517</ns0:v>
       </ns0:c>
       <ns0:c r="F20" s="1" t="n">
-        <ns0:v>283089967.3209452</ns0:v>
+        <ns0:v>356102131.4426047</ns0:v>
       </ns0:c>
       <ns0:c r="G20" s="1" t="n">
         <ns0:v>4.2</ns0:v>
@@ -1749,7 +1749,7 @@
         <ns0:v>9676634819953.418</ns0:v>
       </ns0:c>
       <ns0:c r="F21" s="1" t="n">
-        <ns0:v>3028870301.432466</ns0:v>
+        <ns0:v>1837408781.122872</ns0:v>
       </ns0:c>
       <ns0:c r="G21" s="1" t="n">
         <ns0:v>4.4</ns0:v>
@@ -1777,7 +1777,7 @@
         <ns0:v>103533417666955.5</ns0:v>
       </ns0:c>
       <ns0:c r="F22" s="1" t="n">
-        <ns0:v>32406854222.77353</ns0:v>
+        <ns0:v>9480625727.430063</ns0:v>
       </ns0:c>
       <ns0:c r="G22" s="1" t="n">
         <ns0:v>4.6</ns0:v>
@@ -1805,7 +1805,7 @@
         <ns0:v>1107737222003781</ns0:v>
       </ns0:c>
       <ns0:c r="F23" s="1" t="n">
-        <ns0:v>346731320954.6854</ns0:v>
+        <ns0:v>48917946353.05933</ns0:v>
       </ns0:c>
       <ns0:c r="G23" s="1" t="n">
         <ns0:v>4.8</ns0:v>
@@ -2948,11 +2948,11 @@
       </ns0:c>
       <ns0:c r="D64" s="1">
         <ns0:f>ROUND(D63*10,0)</ns0:f>
-        <ns0:v>3.6188674476410877e+47</ns0:v>
+        <ns0:v>3.618867447641087e+47</ns0:v>
       </ns0:c>
       <ns0:c r="E64" s="1">
         <ns0:f>D64</ns0:f>
-        <ns0:v>3.6188674476410877e+47</ns0:v>
+        <ns0:v>3.618867447641087e+47</ns0:v>
       </ns0:c>
       <ns0:c r="F64" s="1">
         <ns0:f>ROUND(F63*1.4,-5)</ns0:f>
@@ -2979,11 +2979,11 @@
       </ns0:c>
       <ns0:c r="D65" s="1">
         <ns0:f>ROUND(D64*10,0)</ns0:f>
-        <ns0:v>3.6188674476410873e+48</ns0:v>
+        <ns0:v>3.618867447641087e+48</ns0:v>
       </ns0:c>
       <ns0:c r="E65" s="1">
         <ns0:f>D65</ns0:f>
-        <ns0:v>3.6188674476410873e+48</ns0:v>
+        <ns0:v>3.618867447641087e+48</ns0:v>
       </ns0:c>
       <ns0:c r="F65" s="1">
         <ns0:f>ROUND(F64*1.4,-5)</ns0:f>
@@ -3010,11 +3010,11 @@
       </ns0:c>
       <ns0:c r="D66" s="1">
         <ns0:f>ROUND(D65*10,0)</ns0:f>
-        <ns0:v>3.6188674476410876e+49</ns0:v>
+        <ns0:v>3.6188674476410866e+49</ns0:v>
       </ns0:c>
       <ns0:c r="E66" s="1">
         <ns0:f>D66</ns0:f>
-        <ns0:v>3.6188674476410876e+49</ns0:v>
+        <ns0:v>3.6188674476410866e+49</ns0:v>
       </ns0:c>
       <ns0:c r="F66" s="1">
         <ns0:f>ROUND(F65*1.4,-5)</ns0:f>
@@ -3041,11 +3041,11 @@
       </ns0:c>
       <ns0:c r="D67" s="1">
         <ns0:f>ROUND(D66*10,0)</ns0:f>
-        <ns0:v>3.6188674476410874e+50</ns0:v>
+        <ns0:v>3.6188674476410866e+50</ns0:v>
       </ns0:c>
       <ns0:c r="E67" s="1">
         <ns0:f>D67</ns0:f>
-        <ns0:v>3.6188674476410874e+50</ns0:v>
+        <ns0:v>3.6188674476410866e+50</ns0:v>
       </ns0:c>
       <ns0:c r="F67" s="1">
         <ns0:f>ROUND(F66*1.4,-5)</ns0:f>
@@ -3072,11 +3072,11 @@
       </ns0:c>
       <ns0:c r="D68" s="1">
         <ns0:f>ROUND(D67*10,0)</ns0:f>
-        <ns0:v>3.6188674476410876e+51</ns0:v>
+        <ns0:v>3.618867447641086e+51</ns0:v>
       </ns0:c>
       <ns0:c r="E68" s="1">
         <ns0:f>D68</ns0:f>
-        <ns0:v>3.6188674476410876e+51</ns0:v>
+        <ns0:v>3.618867447641086e+51</ns0:v>
       </ns0:c>
       <ns0:c r="F68" s="1">
         <ns0:f>ROUND(F67*1.4,-5)</ns0:f>
@@ -3103,11 +3103,11 @@
       </ns0:c>
       <ns0:c r="D69" s="1">
         <ns0:f>ROUND(D68*10,0)</ns0:f>
-        <ns0:v>3.6188674476410876e+52</ns0:v>
+        <ns0:v>3.6188674476410865e+52</ns0:v>
       </ns0:c>
       <ns0:c r="E69" s="1">
         <ns0:f>D69</ns0:f>
-        <ns0:v>3.6188674476410876e+52</ns0:v>
+        <ns0:v>3.6188674476410865e+52</ns0:v>
       </ns0:c>
       <ns0:c r="F69" s="1">
         <ns0:f>ROUND(F68*1.4,-5)</ns0:f>
@@ -3134,11 +3134,11 @@
       </ns0:c>
       <ns0:c r="D70" s="1">
         <ns0:f>ROUND(D69*10,0)</ns0:f>
-        <ns0:v>3.6188674476410878e+53</ns0:v>
+        <ns0:v>3.6188674476410865e+53</ns0:v>
       </ns0:c>
       <ns0:c r="E70" s="1">
         <ns0:f>D70</ns0:f>
-        <ns0:v>3.6188674476410878e+53</ns0:v>
+        <ns0:v>3.6188674476410865e+53</ns0:v>
       </ns0:c>
       <ns0:c r="F70" s="1">
         <ns0:f>ROUND(F69*1.4,-5)</ns0:f>
@@ -3165,11 +3165,11 @@
       </ns0:c>
       <ns0:c r="D71" s="1">
         <ns0:f>ROUND(D70*10,0)</ns0:f>
-        <ns0:v>3.6188674476410876e+54</ns0:v>
+        <ns0:v>3.618867447641086e+54</ns0:v>
       </ns0:c>
       <ns0:c r="E71" s="1">
         <ns0:f>D71</ns0:f>
-        <ns0:v>3.6188674476410876e+54</ns0:v>
+        <ns0:v>3.618867447641086e+54</ns0:v>
       </ns0:c>
       <ns0:c r="F71" s="1">
         <ns0:f>ROUND(F70*1.4,-5)</ns0:f>
@@ -3196,11 +3196,11 @@
       </ns0:c>
       <ns0:c r="D72" s="1">
         <ns0:f>ROUND(D71*10,0)</ns0:f>
-        <ns0:v>3.6188674476410875e+55</ns0:v>
+        <ns0:v>3.6188674476410864e+55</ns0:v>
       </ns0:c>
       <ns0:c r="E72" s="1">
         <ns0:f>D72</ns0:f>
-        <ns0:v>3.6188674476410875e+55</ns0:v>
+        <ns0:v>3.6188674476410864e+55</ns0:v>
       </ns0:c>
       <ns0:c r="F72" s="1">
         <ns0:f>ROUND(F71*1.4,-5)</ns0:f>
@@ -3227,11 +3227,11 @@
       </ns0:c>
       <ns0:c r="D73" s="1">
         <ns0:f>ROUND(D72*10,0)</ns0:f>
-        <ns0:v>3.6188674476410876e+56</ns0:v>
+        <ns0:v>3.6188674476410863e+56</ns0:v>
       </ns0:c>
       <ns0:c r="E73" s="1">
         <ns0:f>D73</ns0:f>
-        <ns0:v>3.6188674476410876e+56</ns0:v>
+        <ns0:v>3.6188674476410863e+56</ns0:v>
       </ns0:c>
       <ns0:c r="F73" s="1">
         <ns0:f>ROUND(F72*1.4,-5)</ns0:f>
@@ -3258,11 +3258,11 @@
       </ns0:c>
       <ns0:c r="D74" s="1">
         <ns0:f>ROUND(D73*10,0)</ns0:f>
-        <ns0:v>3.6188674476410876e+57</ns0:v>
+        <ns0:v>3.618867447641086e+57</ns0:v>
       </ns0:c>
       <ns0:c r="E74" s="1">
         <ns0:f>D74</ns0:f>
-        <ns0:v>3.6188674476410876e+57</ns0:v>
+        <ns0:v>3.618867447641086e+57</ns0:v>
       </ns0:c>
       <ns0:c r="F74" s="1">
         <ns0:f>ROUND(F73*1.4,-5)</ns0:f>
@@ -3290,11 +3290,11 @@
       </ns0:c>
       <ns0:c r="D75" s="1">
         <ns0:f>ROUND(D74*10,0)</ns0:f>
-        <ns0:v>3.6188674476410877e+58</ns0:v>
+        <ns0:v>3.618867447641086e+58</ns0:v>
       </ns0:c>
       <ns0:c r="E75" s="1">
         <ns0:f>D75</ns0:f>
-        <ns0:v>3.6188674476410877e+58</ns0:v>
+        <ns0:v>3.618867447641086e+58</ns0:v>
       </ns0:c>
       <ns0:c r="F75" s="1">
         <ns0:f>ROUND(F74*1.4,-5)</ns0:f>
@@ -3322,11 +3322,11 @@
       </ns0:c>
       <ns0:c r="D76" s="1">
         <ns0:f>ROUND(D75*10,0)</ns0:f>
-        <ns0:v>3.6188674476410875e+59</ns0:v>
+        <ns0:v>3.618867447641086e+59</ns0:v>
       </ns0:c>
       <ns0:c r="E76" s="1">
         <ns0:f>D76</ns0:f>
-        <ns0:v>3.6188674476410875e+59</ns0:v>
+        <ns0:v>3.618867447641086e+59</ns0:v>
       </ns0:c>
       <ns0:c r="F76" s="1">
         <ns0:f>ROUND(F75*1.4,-5)</ns0:f>
@@ -3354,11 +3354,11 @@
       </ns0:c>
       <ns0:c r="D77" s="1">
         <ns0:f>ROUND(D76*10,0)</ns0:f>
-        <ns0:v>3.618867447641087e+60</ns0:v>
+        <ns0:v>3.618867447641086e+60</ns0:v>
       </ns0:c>
       <ns0:c r="E77" s="1">
         <ns0:f>D77</ns0:f>
-        <ns0:v>3.618867447641087e+60</ns0:v>
+        <ns0:v>3.618867447641086e+60</ns0:v>
       </ns0:c>
       <ns0:c r="F77" s="1">
         <ns0:f>ROUND(F76*1.4,-5)</ns0:f>
@@ -3386,11 +3386,11 @@
       </ns0:c>
       <ns0:c r="D78" s="1">
         <ns0:f>ROUND(D77*10,0)</ns0:f>
-        <ns0:v>3.6188674476410876e+61</ns0:v>
+        <ns0:v>3.618867447641086e+61</ns0:v>
       </ns0:c>
       <ns0:c r="E78" s="1">
         <ns0:f>D78</ns0:f>
-        <ns0:v>3.6188674476410876e+61</ns0:v>
+        <ns0:v>3.618867447641086e+61</ns0:v>
       </ns0:c>
       <ns0:c r="F78" s="1">
         <ns0:f>ROUND(F77*1.4,-5)</ns0:f>
@@ -3418,11 +3418,11 @@
       </ns0:c>
       <ns0:c r="D79" s="1">
         <ns0:f>ROUND(D78*10,0)</ns0:f>
-        <ns0:v>3.618867447641088e+62</ns0:v>
+        <ns0:v>3.618867447641086e+62</ns0:v>
       </ns0:c>
       <ns0:c r="E79" s="1">
         <ns0:f>D79</ns0:f>
-        <ns0:v>3.618867447641088e+62</ns0:v>
+        <ns0:v>3.618867447641086e+62</ns0:v>
       </ns0:c>
       <ns0:c r="F79" s="1">
         <ns0:f>ROUND(F78*1.4,-5)</ns0:f>
@@ -3450,11 +3450,11 @@
       </ns0:c>
       <ns0:c r="D80" s="1">
         <ns0:f>ROUND(D79*10,0)</ns0:f>
-        <ns0:v>3.618867447641088e+63</ns0:v>
+        <ns0:v>3.618867447641086e+63</ns0:v>
       </ns0:c>
       <ns0:c r="E80" s="1">
         <ns0:f>D80</ns0:f>
-        <ns0:v>3.618867447641088e+63</ns0:v>
+        <ns0:v>3.618867447641086e+63</ns0:v>
       </ns0:c>
       <ns0:c r="F80" s="1">
         <ns0:f>ROUND(F79*1.4,-5)</ns0:f>
@@ -3482,11 +3482,11 @@
       </ns0:c>
       <ns0:c r="D81" s="1">
         <ns0:f>ROUND(D80*10,0)</ns0:f>
-        <ns0:v>3.6188674476410876e+64</ns0:v>
+        <ns0:v>3.6188674476410865e+64</ns0:v>
       </ns0:c>
       <ns0:c r="E81" s="1">
         <ns0:f>D81</ns0:f>
-        <ns0:v>3.6188674476410876e+64</ns0:v>
+        <ns0:v>3.6188674476410865e+64</ns0:v>
       </ns0:c>
       <ns0:c r="F81" s="1">
         <ns0:f>ROUND(F80*1.4,-5)</ns0:f>
@@ -3514,11 +3514,11 @@
       </ns0:c>
       <ns0:c r="D82" s="1">
         <ns0:f>ROUND(D81*10,0)</ns0:f>
-        <ns0:v>3.6188674476410874e+65</ns0:v>
+        <ns0:v>3.6188674476410865e+65</ns0:v>
       </ns0:c>
       <ns0:c r="E82" s="1">
         <ns0:f>D82</ns0:f>
-        <ns0:v>3.6188674476410874e+65</ns0:v>
+        <ns0:v>3.6188674476410865e+65</ns0:v>
       </ns0:c>
       <ns0:c r="F82" s="1">
         <ns0:f>ROUND(F81*1.4,-5)</ns0:f>
@@ -3546,11 +3546,11 @@
       </ns0:c>
       <ns0:c r="D83" s="1">
         <ns0:f>ROUND(D82*10,0)</ns0:f>
-        <ns0:v>3.618867447641088e+66</ns0:v>
+        <ns0:v>3.618867447641086e+66</ns0:v>
       </ns0:c>
       <ns0:c r="E83" s="1">
         <ns0:f>D83</ns0:f>
-        <ns0:v>3.618867447641088e+66</ns0:v>
+        <ns0:v>3.618867447641086e+66</ns0:v>
       </ns0:c>
       <ns0:c r="F83" s="1">
         <ns0:f>ROUND(F82*1.4,-5)</ns0:f>

</xml_diff>

<commit_message>
Freeze smooth7 candidate, preserve sparse timing and teaching failure, verify offline save contract
</commit_message>
<xml_diff>
--- a/space-battleship/config_excel/level.xlsx
+++ b/space-battleship/config_excel/level.xlsx
@@ -1385,7 +1385,7 @@
         <ns0:v>4.5</ns0:v>
       </ns0:c>
       <ns0:c r="F8" s="1" t="n">
-        <ns0:v>3.841599999999999</ns0:v>
+        <ns0:v>5.762399999999999</ns0:v>
       </ns0:c>
       <ns0:c r="G8" s="1" t="n">
         <ns0:v>1.8</ns0:v>
@@ -1581,7 +1581,7 @@
         <ns0:v>6450407.623907364</ns0:v>
       </ns0:c>
       <ns0:c r="F15" s="1" t="n">
-        <ns0:v>97368.504802272</ns0:v>
+        <ns0:v>67617.01722380001</ns0:v>
       </ns0:c>
       <ns0:c r="G15" s="1" t="n">
         <ns0:v>3.2</ns0:v>
@@ -1609,7 +1609,7 @@
         <ns0:v>69014978.76834521</ns0:v>
       </ns0:c>
       <ns0:c r="F16" s="1" t="n">
-        <ns0:v>502400.0979823805</ns0:v>
+        <ns0:v>242283.9978695894</ns0:v>
       </ns0:c>
       <ns0:c r="G16" s="1" t="n">
         <ns0:v>3.4</ns0:v>
@@ -1637,7 +1637,7 @@
         <ns0:v>738413379.7593849</ns0:v>
       </ns0:c>
       <ns0:c r="F17" s="1" t="n">
-        <ns0:v>2592274.154412361</ns0:v>
+        <ns0:v>868147.3693135534</ns0:v>
       </ns0:c>
       <ns0:c r="G17" s="1" t="n">
         <ns0:v>3.6</ns0:v>
@@ -1665,7 +1665,7 @@
         <ns0:v>7900521439.525051</ns0:v>
       </ns0:c>
       <ns0:c r="F18" s="1" t="n">
-        <ns0:v>13375565.24893431</ns0:v>
+        <ns0:v>3110728.985294833</ns0:v>
       </ns0:c>
       <ns0:c r="G18" s="1" t="n">
         <ns0:v>3.8</ns0:v>
@@ -1693,7 +1693,7 @@
         <ns0:v>84530211298.0865</ns0:v>
       </ns0:c>
       <ns0:c r="F19" s="1" t="n">
-        <ns0:v>69014978.76834521</ns0:v>
+        <ns0:v>11146304.37411193</ns0:v>
       </ns0:c>
       <ns0:c r="G19" s="1" t="n">
         <ns0:v>4</ns0:v>
@@ -1721,7 +1721,7 @@
         <ns0:v>904415825815.2517</ns0:v>
       </ns0:c>
       <ns0:c r="F20" s="1" t="n">
-        <ns0:v>356102131.4426047</ns0:v>
+        <ns0:v>39939223.82427385</ns0:v>
       </ns0:c>
       <ns0:c r="G20" s="1" t="n">
         <ns0:v>4.2</ns0:v>
@@ -1749,7 +1749,7 @@
         <ns0:v>9676634819953.418</ns0:v>
       </ns0:c>
       <ns0:c r="F21" s="1" t="n">
-        <ns0:v>1837408781.122872</ns0:v>
+        <ns0:v>143109459.9740406</ns0:v>
       </ns0:c>
       <ns0:c r="G21" s="1" t="n">
         <ns0:v>4.4</ns0:v>
@@ -1777,7 +1777,7 @@
         <ns0:v>103533417666955.5</ns0:v>
       </ns0:c>
       <ns0:c r="F22" s="1" t="n">
-        <ns0:v>9480625727.430063</ns0:v>
+        <ns0:v>512787069.2773507</ns0:v>
       </ns0:c>
       <ns0:c r="G22" s="1" t="n">
         <ns0:v>4.6</ns0:v>
@@ -1805,7 +1805,7 @@
         <ns0:v>1107737222003781</ns0:v>
       </ns0:c>
       <ns0:c r="F23" s="1" t="n">
-        <ns0:v>48917946353.05933</ns0:v>
+        <ns0:v>1837408781.122872</ns0:v>
       </ns0:c>
       <ns0:c r="G23" s="1" t="n">
         <ns0:v>4.8</ns0:v>

</xml_diff>

<commit_message>
Reanchor provisional stages 21-60 to current income; retain failures and prove full-event native prefix
</commit_message>
<xml_diff>
--- a/space-battleship/config_excel/level.xlsx
+++ b/space-battleship/config_excel/level.xlsx
@@ -1833,7 +1833,7 @@
         <ns0:v>4763067294395140</ns0:v>
       </ns0:c>
       <ns0:c r="F24" s="1" t="n">
-        <ns0:v>5963524857616.636</ns0:v>
+        <ns0:v>31602085758.1002</ns0:v>
       </ns0:c>
       <ns0:c r="G24" s="1" t="n">
         <ns0:v>5</ns0:v>
@@ -1861,7 +1861,7 @@
         <ns0:v>2.048031753406153e+16</ns0:v>
       </ns0:c>
       <ns0:c r="F25" s="1" t="n">
-        <ns0:v>25642065324161.59</ns0:v>
+        <ns0:v>135883184314.0537</ns0:v>
       </ns0:c>
       <ns0:c r="G25" s="1" t="n">
         <ns0:v>5.2</ns0:v>
@@ -1889,7 +1889,7 @@
         <ns0:v>8.80616166791431e+16</ns0:v>
       </ns0:c>
       <ns0:c r="F26" s="1" t="n">
-        <ns0:v>110256187370257.9</ns0:v>
+        <ns0:v>584272820492.3739</ns0:v>
       </ns0:c>
       <ns0:c r="G26" s="1" t="n">
         <ns0:v>5.4</ns0:v>
@@ -1917,7 +1917,7 @@
         <ns0:v>3.786488329219983e+17</ns0:v>
       </ns0:c>
       <ns0:c r="F27" s="1" t="n">
-        <ns0:v>474081424399572.5</ns0:v>
+        <ns0:v>2512266182820.144</ns0:v>
       </ns0:c>
       <ns0:c r="G27" s="1" t="n">
         <ns0:v>5.6</ns0:v>
@@ -1945,7 +1945,7 @@
         <ns0:v>1.628120673682214e+18</ns0:v>
       </ns0:c>
       <ns0:c r="F28" s="1" t="n">
-        <ns0:v>2038463349054239</ns0:v>
+        <ns0:v>10802284740924.51</ns0:v>
       </ns0:c>
       <ns0:c r="G28" s="1" t="n">
         <ns0:v>5.8</ns0:v>
@@ -1973,7 +1973,7 @@
         <ns0:v>7.000620885625409e+18</ns0:v>
       </ns0:c>
       <ns0:c r="F29" s="1" t="n">
-        <ns0:v>8765019280601813</ns0:v>
+        <ns0:v>46447847135776.41</ns0:v>
       </ns0:c>
       <ns0:c r="G29" s="1" t="n">
         <ns0:v>6</ns0:v>
@@ -2001,7 +2001,7 @@
         <ns0:v>3.010138841454234e+19</ns0:v>
       </ns0:c>
       <ns0:c r="F30" s="1" t="n">
-        <ns0:v>3.768797855745866e+16</ns0:v>
+        <ns0:v>199717240869898.8</ns0:v>
       </ns0:c>
       <ns0:c r="G30" s="1" t="n">
         <ns0:v>6.2</ns0:v>
@@ -2029,7 +2029,7 @@
         <ns0:v>1.294304604243966e+20</ns0:v>
       </ns0:c>
       <ns0:c r="F31" s="1" t="n">
-        <ns0:v>1.620514093894771e+17</ns0:v>
+        <ns0:v>858747579496795.6</ns0:v>
       </ns0:c>
       <ns0:c r="G31" s="1" t="n">
         <ns0:v>6.4</ns0:v>
@@ -2057,7 +2057,7 @@
         <ns0:v>5.565272888734292e+20</ns0:v>
       </ns0:c>
       <ns0:c r="F32" s="1" t="n">
-        <ns0:v>6.967913984847764e+17</ns0:v>
+        <ns0:v>3692457406679269</ns0:v>
       </ns0:c>
       <ns0:c r="G32" s="1" t="n">
         <ns0:v>6.6</ns0:v>
@@ -2085,7 +2085,7 @@
         <ns0:v>2.39296547540079e+21</ns0:v>
       </ns0:c>
       <ns0:c r="F33" s="1" t="n">
-        <ns0:v>2.99607547278696e+18</ns0:v>
+        <ns0:v>1.587689098131714e+16</ns0:v>
       </ns0:c>
       <ns0:c r="G33" s="1" t="n">
         <ns0:v>6.8</ns0:v>
@@ -2113,7 +2113,7 @@
         <ns0:v>1.028931353582277e+22</ns0:v>
       </ns0:c>
       <ns0:c r="F34" s="1" t="n">
-        <ns0:v>2.99607547278696e+18</ns0:v>
+        <ns0:v>1.587689098131714e+16</ns0:v>
       </ns0:c>
       <ns0:c r="G34" s="1" t="n">
         <ns0:v>7</ns0:v>
@@ -2141,7 +2141,7 @@
         <ns0:v>4.424216484808832e+22</ns0:v>
       </ns0:c>
       <ns0:c r="F35" s="1" t="n">
-        <ns0:v>2.99607547278696e+18</ns0:v>
+        <ns0:v>1.587689098131714e+16</ns0:v>
       </ns0:c>
       <ns0:c r="G35" s="1" t="n">
         <ns0:v>7.2</ns0:v>
@@ -2169,7 +2169,7 @@
         <ns0:v>8.179679859850836e+23</ns0:v>
       </ns0:c>
       <ns0:c r="F36" s="1" t="n">
-        <ns0:v>6.212662100371039e+18</ns0:v>
+        <ns0:v>3.292232113885921e+16</ns0:v>
       </ns0:c>
       <ns0:c r="G36" s="1" t="n">
         <ns0:v>7.4</ns0:v>
@@ -2197,7 +2197,7 @@
         <ns0:v>1.512294048887176e+25</ns0:v>
       </ns0:c>
       <ns0:c r="F37" s="1" t="n">
-        <ns0:v>6.212662100371039e+18</ns0:v>
+        <ns0:v>3.292232113885921e+16</ns0:v>
       </ns0:c>
       <ns0:c r="G37" s="1" t="n">
         <ns0:v>7.6</ns0:v>
@@ -2225,7 +2225,7 @@
         <ns0:v>5.797772421440058e+26</ns0:v>
       </ns0:c>
       <ns0:c r="F38" s="1" t="n">
-        <ns0:v>1.855090962911431e+19</ns0:v>
+        <ns0:v>9.830552416349534e+16</ns0:v>
       </ns0:c>
       <ns0:c r="G38" s="1" t="n">
         <ns0:v>7.8</ns0:v>
@@ -2253,7 +2253,7 @@
         <ns0:v>1.731205568606127e+27</ns0:v>
       </ns0:c>
       <ns0:c r="F39" s="1" t="n">
-        <ns0:v>3.846716620693144e+19</ns0:v>
+        <ns0:v>2.038463349054239e+17</ns0:v>
       </ns0:c>
       <ns0:c r="G39" s="1" t="n">
         <ns0:v>8</ns0:v>
@@ -2281,7 +2281,7 @@
         <ns0:v>5.169352128568795e+27</ns0:v>
       </ns0:c>
       <ns0:c r="F40" s="1" t="n">
-        <ns0:v>7.9765515846693e+19</ns0:v>
+        <ns0:v>4.226957600598869e+17</ns0:v>
       </ns0:c>
       <ns0:c r="G40" s="1" t="n">
         <ns0:v>8.199999999999999</ns0:v>
@@ -2309,7 +2309,7 @@
         <ns0:v>1.543560274627236e+28</ns0:v>
       </ns0:c>
       <ns0:c r="F41" s="1" t="n">
-        <ns0:v>1.654017736597026e+20</ns0:v>
+        <ns0:v>8.765019280601815e+17</ns0:v>
       </ns0:c>
       <ns0:c r="G41" s="1" t="n">
         <ns0:v>8.4</ns0:v>
@@ -2337,7 +2337,7 @@
         <ns0:v>1.376253845651405e+29</ns0:v>
       </ns0:c>
       <ns0:c r="F42" s="1" t="n">
-        <ns0:v>7.111973515960703e+20</ns0:v>
+        <ns0:v>3.768797855745867e+18</ns0:v>
       </ns0:c>
       <ns0:c r="G42" s="1" t="n">
         <ns0:v>8.6</ns0:v>
@@ -2365,7 +2365,7 @@
         <ns0:v>5.276226932910335e+30</ns0:v>
       </ns0:c>
       <ns0:c r="F43" s="1" t="n">
-        <ns0:v>6.341107025364199e+21</ns0:v>
+        <ns0:v>3.360298025100196e+19</ns0:v>
       </ns0:c>
       <ns0:c r="G43" s="1" t="n">
         <ns0:v>8.800000000000001</ns0:v>
@@ -2393,7 +2393,7 @@
         <ns0:v>1.575472920203933e+31</ns0:v>
       </ns0:c>
       <ns0:c r="F44" s="1" t="n">
-        <ns0:v>1.31489195277952e+22</ns0:v>
+        <ns0:v>6.967913984847766e+19</ns0:v>
       </ns0:c>
       <ns0:c r="G44" s="1" t="n">
         <ns0:v>9</ns0:v>
@@ -2421,7 +2421,7 @@
         <ns0:v>4.704336932162219e+31</ns0:v>
       </ns0:c>
       <ns0:c r="F45" s="1" t="n">
-        <ns0:v>2.726559953283612e+22</ns0:v>
+        <ns0:v>1.444866643898032e+20</ns0:v>
       </ns0:c>
       <ns0:c r="G45" s="1" t="n">
         <ns0:v>9.199999999999999</ns0:v>
@@ -2449,7 +2449,7 @@
         <ns0:v>1.404707481004547e+32</ns0:v>
       </ns0:c>
       <ns0:c r="F46" s="1" t="n">
-        <ns0:v>5.653794719128898e+22</ns0:v>
+        <ns0:v>2.99607547278696e+20</ns0:v>
       </ns0:c>
       <ns0:c r="G46" s="1" t="n">
         <ns0:v>9.4</ns0:v>
@@ -2477,7 +2477,7 @@
         <ns0:v>1.252451300105319e+33</ns0:v>
       </ns0:c>
       <ns0:c r="F47" s="1" t="n">
-        <ns0:v>2.431028242166887e+23</ns0:v>
+        <ns0:v>1.288257613132938e+21</ns0:v>
       </ns0:c>
       <ns0:c r="G47" s="1" t="n">
         <ns0:v>9.6</ns0:v>
@@ -2505,7 +2505,7 @@
         <ns0:v>4.801597686832596e+34</ns0:v>
       </ns0:c>
       <ns0:c r="F48" s="1" t="n">
-        <ns0:v>2.167529199970716e+24</ns0:v>
+        <ns0:v>1.148623428192379e+22</ns0:v>
       </ns0:c>
       <ns0:c r="G48" s="1" t="n">
         <ns0:v>9.800000000000001</ns0:v>
@@ -2533,7 +2533,7 @@
         <ns0:v>1.433749386731914e+35</ns0:v>
       </ns0:c>
       <ns0:c r="F49" s="1" t="n">
-        <ns0:v>4.494588549059277e+24</ns0:v>
+        <ns0:v>2.381785540699717e+22</ns0:v>
       </ns0:c>
       <ns0:c r="G49" s="1" t="n">
         <ns0:v>10</ns0:v>
@@ -2561,7 +2561,7 @@
         <ns0:v>4.281152728791306e+35</ns0:v>
       </ns0:c>
       <ns0:c r="F50" s="1" t="n">
-        <ns0:v>9.319978815329315e+24</ns0:v>
+        <ns0:v>4.938870497194933e+22</ns0:v>
       </ns0:c>
       <ns0:c r="G50" s="1" t="n">
         <ns0:v>10.2</ns0:v>
@@ -2589,7 +2589,7 @@
         <ns0:v>1.278345354972718e+36</ns0:v>
       </ns0:c>
       <ns0:c r="F51" s="1" t="n">
-        <ns0:v>1.932590807146687e+25</ns0:v>
+        <ns0:v>1.024124186298341e+23</ns0:v>
       </ns0:c>
       <ns0:c r="G51" s="1" t="n">
         <ns0:v>10.4</ns0:v>
@@ -2617,7 +2617,7 @@
         <ns0:v>1.139785559249822e+37</ns0:v>
       </ns0:c>
       <ns0:c r="F52" s="1" t="n">
-        <ns0:v>8.30978672930941e+25</ns0:v>
+        <ns0:v>4.403546545391806e+23</ns0:v>
       </ns0:c>
       <ns0:c r="G52" s="1" t="n">
         <ns0:v>10.6</ns0:v>
@@ -2645,7 +2645,7 @@
         <ns0:v>4.369664277021335e+38</ns0:v>
       </ns0:c>
       <ns0:c r="F53" s="1" t="n">
-        <ns0:v>7.409089318210736e+26</ns0:v>
+        <ns0:v>3.926246332728402e+24</ns0:v>
       </ns0:c>
       <ns0:c r="G53" s="1" t="n">
         <ns0:v>10.8</ns0:v>
@@ -2673,7 +2673,7 @@
         <ns0:v>1.304774761655727e+39</ns0:v>
       </ns0:c>
       <ns0:c r="F54" s="1" t="n">
-        <ns0:v>1.536348761024178e+27</ns0:v>
+        <ns0:v>8.141464395545614e+24</ns0:v>
       </ns0:c>
       <ns0:c r="G54" s="1" t="n">
         <ns0:v>11</ns0:v>
@@ -2701,7 +2701,7 @@
         <ns0:v>3.896036561907814e+39</ns0:v>
       </ns0:c>
       <ns0:c r="F55" s="1" t="n">
-        <ns0:v>3.185772790859734e+27</ns0:v>
+        <ns0:v>1.688214057060338e+25</ns0:v>
       </ns0:c>
       <ns0:c r="G55" s="1" t="n">
         <ns0:v>11.2</ns0:v>
@@ -2729,7 +2729,7 @@
         <ns0:v>1.163350283727174e+40</ns0:v>
       </ns0:c>
       <ns0:c r="F56" s="1" t="n">
-        <ns0:v>6.606018459126745e+27</ns0:v>
+        <ns0:v>3.500680668720316e+25</ns0:v>
       </ns0:c>
       <ns0:c r="G56" s="1" t="n">
         <ns0:v>11.4</ns0:v>
@@ -2757,7 +2757,7 @@
         <ns0:v>1.03725479862186e+41</ns0:v>
       </ns0:c>
       <ns0:c r="F57" s="1" t="n">
-        <ns0:v>2.840467020862624e+28</ns0:v>
+        <ns0:v>1.505228611090775e+26</ns0:v>
       </ns0:c>
       <ns0:c r="G57" s="1" t="n">
         <ns0:v>11.6</ns0:v>
@@ -2785,7 +2785,7 @@
         <ns0:v>3.976585948930645e+42</ns0:v>
       </ns0:c>
       <ns0:c r="F58" s="1" t="n">
-        <ns0:v>2.532588927796961e+29</ns0:v>
+        <ns0:v>1.342076949407421e+27</ns0:v>
       </ns0:c>
       <ns0:c r="G58" s="1" t="n">
         <ns0:v>11.8</ns0:v>
@@ -2813,7 +2813,7 @@
         <ns0:v>1.187402201813172e+43</ns0:v>
       </ns0:c>
       <ns0:c r="F59" s="1" t="n">
-        <ns0:v>5.251576400679779e+29</ns0:v>
+        <ns0:v>2.782930762291229e+27</ns0:v>
       </ns0:c>
       <ns0:c r="G59" s="1" t="n">
         <ns0:v>12</ns0:v>
@@ -2841,7 +2841,7 @@
         <ns0:v>3.545563976178901e+43</ns0:v>
       </ns0:c>
       <ns0:c r="F60" s="1" t="n">
-        <ns0:v>1.088966882444959e+30</ns0:v>
+        <ns0:v>5.77068522868709e+27</ns0:v>
       </ns0:c>
       <ns0:c r="G60" s="1" t="n">
         <ns0:v>12.2</ns0:v>
@@ -2869,7 +2869,7 @@
         <ns0:v>1.058699730384658e+44</ns0:v>
       </ns0:c>
       <ns0:c r="F61" s="1" t="n">
-        <ns0:v>2.258081727437866e+30</ns0:v>
+        <ns0:v>1.196609289020555e+28</ns0:v>
       </ns0:c>
       <ns0:c r="G61" s="1" t="n">
         <ns0:v>12.4</ns0:v>
@@ -2897,7 +2897,7 @@
         <ns0:v>9.43947314065115e+44</ns0:v>
       </ns0:c>
       <ns0:c r="F62" s="1" t="n">
-        <ns0:v>9.709338108703431e+30</ns0:v>
+        <ns0:v>5.145200915424123e+28</ns0:v>
       </ns0:c>
       <ns0:c r="G62" s="1" t="n">
         <ns0:v>12.6</ns0:v>
@@ -2925,7 +2925,7 @@
         <ns0:v>3.618867447641087e+46</ns0:v>
       </ns0:c>
       <ns0:c r="F63" s="1" t="n">
-        <ns0:v>8.656943386327968e+31</ns0:v>
+        <ns0:v>4.587512818838018e+29</ns0:v>
       </ns0:c>
       <ns0:c r="G63" s="1" t="n">
         <ns0:v>12.8</ns0:v>
@@ -2948,15 +2948,15 @@
       </ns0:c>
       <ns0:c r="D64" s="1">
         <ns0:f>ROUND(D63*10,0)</ns0:f>
-        <ns0:v>3.618867447641087e+47</ns0:v>
+        <ns0:v>3.6188674476410877e+47</ns0:v>
       </ns0:c>
       <ns0:c r="E64" s="1">
         <ns0:f>D64</ns0:f>
-        <ns0:v>3.618867447641087e+47</ns0:v>
+        <ns0:v>3.6188674476410877e+47</ns0:v>
       </ns0:c>
       <ns0:c r="F64" s="1">
         <ns0:f>ROUND(F63*1.4,-5)</ns0:f>
-        <ns0:v>1.2119720740859155e+32</ns0:v>
+        <ns0:v>6.422517946373224e+29</ns0:v>
       </ns0:c>
       <ns0:c r="G64" s="1" t="n">
         <ns0:v>13</ns0:v>
@@ -2979,15 +2979,15 @@
       </ns0:c>
       <ns0:c r="D65" s="1">
         <ns0:f>ROUND(D64*10,0)</ns0:f>
-        <ns0:v>3.618867447641087e+48</ns0:v>
+        <ns0:v>3.6188674476410873e+48</ns0:v>
       </ns0:c>
       <ns0:c r="E65" s="1">
         <ns0:f>D65</ns0:f>
-        <ns0:v>3.618867447641087e+48</ns0:v>
+        <ns0:v>3.6188674476410873e+48</ns0:v>
       </ns0:c>
       <ns0:c r="F65" s="1">
         <ns0:f>ROUND(F64*1.4,-5)</ns0:f>
-        <ns0:v>1.6967609037202817e+32</ns0:v>
+        <ns0:v>8.991525124922513e+29</ns0:v>
       </ns0:c>
       <ns0:c r="G65" s="1" t="n">
         <ns0:v>13.2</ns0:v>
@@ -3010,15 +3010,15 @@
       </ns0:c>
       <ns0:c r="D66" s="1">
         <ns0:f>ROUND(D65*10,0)</ns0:f>
-        <ns0:v>3.6188674476410866e+49</ns0:v>
+        <ns0:v>3.6188674476410876e+49</ns0:v>
       </ns0:c>
       <ns0:c r="E66" s="1">
         <ns0:f>D66</ns0:f>
-        <ns0:v>3.6188674476410866e+49</ns0:v>
+        <ns0:v>3.6188674476410876e+49</ns0:v>
       </ns0:c>
       <ns0:c r="F66" s="1">
         <ns0:f>ROUND(F65*1.4,-5)</ns0:f>
-        <ns0:v>2.3754652652083943e+32</ns0:v>
+        <ns0:v>1.2588135174891517e+30</ns0:v>
       </ns0:c>
       <ns0:c r="G66" s="1" t="n">
         <ns0:v>13.4</ns0:v>
@@ -3041,15 +3041,15 @@
       </ns0:c>
       <ns0:c r="D67" s="1">
         <ns0:f>ROUND(D66*10,0)</ns0:f>
-        <ns0:v>3.6188674476410866e+50</ns0:v>
+        <ns0:v>3.6188674476410874e+50</ns0:v>
       </ns0:c>
       <ns0:c r="E67" s="1">
         <ns0:f>D67</ns0:f>
-        <ns0:v>3.6188674476410866e+50</ns0:v>
+        <ns0:v>3.6188674476410874e+50</ns0:v>
       </ns0:c>
       <ns0:c r="F67" s="1">
         <ns0:f>ROUND(F66*1.4,-5)</ns0:f>
-        <ns0:v>3.325651371291752e+32</ns0:v>
+        <ns0:v>1.7623389244848124e+30</ns0:v>
       </ns0:c>
       <ns0:c r="G67" s="1" t="n">
         <ns0:v>13.6</ns0:v>
@@ -3072,15 +3072,15 @@
       </ns0:c>
       <ns0:c r="D68" s="1">
         <ns0:f>ROUND(D67*10,0)</ns0:f>
-        <ns0:v>3.618867447641086e+51</ns0:v>
+        <ns0:v>3.6188674476410876e+51</ns0:v>
       </ns0:c>
       <ns0:c r="E68" s="1">
         <ns0:f>D68</ns0:f>
-        <ns0:v>3.618867447641086e+51</ns0:v>
+        <ns0:v>3.6188674476410876e+51</ns0:v>
       </ns0:c>
       <ns0:c r="F68" s="1">
         <ns0:f>ROUND(F67*1.4,-5)</ns0:f>
-        <ns0:v>4.655911919808452e+32</ns0:v>
+        <ns0:v>2.4672744942787372e+30</ns0:v>
       </ns0:c>
       <ns0:c r="G68" s="1" t="n">
         <ns0:v>13.8</ns0:v>
@@ -3103,15 +3103,15 @@
       </ns0:c>
       <ns0:c r="D69" s="1">
         <ns0:f>ROUND(D68*10,0)</ns0:f>
-        <ns0:v>3.6188674476410865e+52</ns0:v>
+        <ns0:v>3.6188674476410876e+52</ns0:v>
       </ns0:c>
       <ns0:c r="E69" s="1">
         <ns0:f>D69</ns0:f>
-        <ns0:v>3.6188674476410865e+52</ns0:v>
+        <ns0:v>3.6188674476410876e+52</ns0:v>
       </ns0:c>
       <ns0:c r="F69" s="1">
         <ns0:f>ROUND(F68*1.4,-5)</ns0:f>
-        <ns0:v>6.518276687731834e+32</ns0:v>
+        <ns0:v>3.454184291990232e+30</ns0:v>
       </ns0:c>
       <ns0:c r="G69" s="1" t="n">
         <ns0:v>14</ns0:v>
@@ -3134,15 +3134,15 @@
       </ns0:c>
       <ns0:c r="D70" s="1">
         <ns0:f>ROUND(D69*10,0)</ns0:f>
-        <ns0:v>3.6188674476410865e+53</ns0:v>
+        <ns0:v>3.6188674476410878e+53</ns0:v>
       </ns0:c>
       <ns0:c r="E70" s="1">
         <ns0:f>D70</ns0:f>
-        <ns0:v>3.6188674476410865e+53</ns0:v>
+        <ns0:v>3.6188674476410878e+53</ns0:v>
       </ns0:c>
       <ns0:c r="F70" s="1">
         <ns0:f>ROUND(F69*1.4,-5)</ns0:f>
-        <ns0:v>9.125587362824566e+32</ns0:v>
+        <ns0:v>4.835858008786324e+30</ns0:v>
       </ns0:c>
       <ns0:c r="G70" s="1" t="n">
         <ns0:v>14.2</ns0:v>
@@ -3165,15 +3165,15 @@
       </ns0:c>
       <ns0:c r="D71" s="1">
         <ns0:f>ROUND(D70*10,0)</ns0:f>
-        <ns0:v>3.618867447641086e+54</ns0:v>
+        <ns0:v>3.6188674476410876e+54</ns0:v>
       </ns0:c>
       <ns0:c r="E71" s="1">
         <ns0:f>D71</ns0:f>
-        <ns0:v>3.618867447641086e+54</ns0:v>
+        <ns0:v>3.6188674476410876e+54</ns0:v>
       </ns0:c>
       <ns0:c r="F71" s="1">
         <ns0:f>ROUND(F70*1.4,-5)</ns0:f>
-        <ns0:v>1.2775822307954391e+33</ns0:v>
+        <ns0:v>6.770201212300853e+30</ns0:v>
       </ns0:c>
       <ns0:c r="G71" s="1" t="n">
         <ns0:v>14.4</ns0:v>
@@ -3196,15 +3196,15 @@
       </ns0:c>
       <ns0:c r="D72" s="1">
         <ns0:f>ROUND(D71*10,0)</ns0:f>
-        <ns0:v>3.6188674476410864e+55</ns0:v>
+        <ns0:v>3.6188674476410875e+55</ns0:v>
       </ns0:c>
       <ns0:c r="E72" s="1">
         <ns0:f>D72</ns0:f>
-        <ns0:v>3.6188674476410864e+55</ns0:v>
+        <ns0:v>3.6188674476410875e+55</ns0:v>
       </ns0:c>
       <ns0:c r="F72" s="1">
         <ns0:f>ROUND(F71*1.4,-5)</ns0:f>
-        <ns0:v>1.7886151231136147e+33</ns0:v>
+        <ns0:v>9.478281697221195e+30</ns0:v>
       </ns0:c>
       <ns0:c r="G72" s="1" t="n">
         <ns0:v>14.6</ns0:v>
@@ -3227,15 +3227,15 @@
       </ns0:c>
       <ns0:c r="D73" s="1">
         <ns0:f>ROUND(D72*10,0)</ns0:f>
-        <ns0:v>3.6188674476410863e+56</ns0:v>
+        <ns0:v>3.6188674476410876e+56</ns0:v>
       </ns0:c>
       <ns0:c r="E73" s="1">
         <ns0:f>D73</ns0:f>
-        <ns0:v>3.6188674476410863e+56</ns0:v>
+        <ns0:v>3.6188674476410876e+56</ns0:v>
       </ns0:c>
       <ns0:c r="F73" s="1">
         <ns0:f>ROUND(F72*1.4,-5)</ns0:f>
-        <ns0:v>2.5040611723590604e+33</ns0:v>
+        <ns0:v>1.3269594376109672e+31</ns0:v>
       </ns0:c>
       <ns0:c r="G73" s="1" t="n">
         <ns0:v>14.8</ns0:v>
@@ -3258,15 +3258,15 @@
       </ns0:c>
       <ns0:c r="D74" s="1">
         <ns0:f>ROUND(D73*10,0)</ns0:f>
-        <ns0:v>3.618867447641086e+57</ns0:v>
+        <ns0:v>3.6188674476410876e+57</ns0:v>
       </ns0:c>
       <ns0:c r="E74" s="1">
         <ns0:f>D74</ns0:f>
-        <ns0:v>3.618867447641086e+57</ns0:v>
+        <ns0:v>3.6188674476410876e+57</ns0:v>
       </ns0:c>
       <ns0:c r="F74" s="1">
         <ns0:f>ROUND(F73*1.4,-5)</ns0:f>
-        <ns0:v>3.5056856413026845e+33</ns0:v>
+        <ns0:v>1.8577432126553538e+31</ns0:v>
       </ns0:c>
       <ns0:c r="G74" s="1" t="n">
         <ns0:v>15</ns0:v>
@@ -3290,15 +3290,15 @@
       </ns0:c>
       <ns0:c r="D75" s="1">
         <ns0:f>ROUND(D74*10,0)</ns0:f>
-        <ns0:v>3.618867447641086e+58</ns0:v>
+        <ns0:v>3.6188674476410877e+58</ns0:v>
       </ns0:c>
       <ns0:c r="E75" s="1">
         <ns0:f>D75</ns0:f>
-        <ns0:v>3.618867447641086e+58</ns0:v>
+        <ns0:v>3.6188674476410877e+58</ns0:v>
       </ns0:c>
       <ns0:c r="F75" s="1">
         <ns0:f>ROUND(F74*1.4,-5)</ns0:f>
-        <ns0:v>4.907959897823758e+33</ns0:v>
+        <ns0:v>2.600840497717495e+31</ns0:v>
       </ns0:c>
       <ns0:c r="G75" s="1" t="n">
         <ns0:v>15.2</ns0:v>
@@ -3322,15 +3322,15 @@
       </ns0:c>
       <ns0:c r="D76" s="1">
         <ns0:f>ROUND(D75*10,0)</ns0:f>
-        <ns0:v>3.618867447641086e+59</ns0:v>
+        <ns0:v>3.6188674476410875e+59</ns0:v>
       </ns0:c>
       <ns0:c r="E76" s="1">
         <ns0:f>D76</ns0:f>
-        <ns0:v>3.618867447641086e+59</ns0:v>
+        <ns0:v>3.6188674476410875e+59</ns0:v>
       </ns0:c>
       <ns0:c r="F76" s="1">
         <ns0:f>ROUND(F75*1.4,-5)</ns0:f>
-        <ns0:v>6.87114385695326e+33</ns0:v>
+        <ns0:v>3.6411766968044923e+31</ns0:v>
       </ns0:c>
       <ns0:c r="G76" s="1" t="n">
         <ns0:v>15.4</ns0:v>
@@ -3354,15 +3354,15 @@
       </ns0:c>
       <ns0:c r="D77" s="1">
         <ns0:f>ROUND(D76*10,0)</ns0:f>
-        <ns0:v>3.618867447641086e+60</ns0:v>
+        <ns0:v>3.618867447641087e+60</ns0:v>
       </ns0:c>
       <ns0:c r="E77" s="1">
         <ns0:f>D77</ns0:f>
-        <ns0:v>3.618867447641086e+60</ns0:v>
+        <ns0:v>3.618867447641087e+60</ns0:v>
       </ns0:c>
       <ns0:c r="F77" s="1">
         <ns0:f>ROUND(F76*1.4,-5)</ns0:f>
-        <ns0:v>9.619601399734563e+33</ns0:v>
+        <ns0:v>5.097647375526289e+31</ns0:v>
       </ns0:c>
       <ns0:c r="G77" s="1" t="n">
         <ns0:v>15.6</ns0:v>
@@ -3386,15 +3386,15 @@
       </ns0:c>
       <ns0:c r="D78" s="1">
         <ns0:f>ROUND(D77*10,0)</ns0:f>
-        <ns0:v>3.618867447641086e+61</ns0:v>
+        <ns0:v>3.6188674476410876e+61</ns0:v>
       </ns0:c>
       <ns0:c r="E78" s="1">
         <ns0:f>D78</ns0:f>
-        <ns0:v>3.618867447641086e+61</ns0:v>
+        <ns0:v>3.6188674476410876e+61</ns0:v>
       </ns0:c>
       <ns0:c r="F78" s="1">
         <ns0:f>ROUND(F77*1.4,-5)</ns0:f>
-        <ns0:v>1.3467441959628388e+34</ns0:v>
+        <ns0:v>7.136706325736805e+31</ns0:v>
       </ns0:c>
       <ns0:c r="G78" s="1" t="n">
         <ns0:v>15.8</ns0:v>
@@ -3418,15 +3418,15 @@
       </ns0:c>
       <ns0:c r="D79" s="1">
         <ns0:f>ROUND(D78*10,0)</ns0:f>
-        <ns0:v>3.618867447641086e+62</ns0:v>
+        <ns0:v>3.618867447641088e+62</ns0:v>
       </ns0:c>
       <ns0:c r="E79" s="1">
         <ns0:f>D79</ns0:f>
-        <ns0:v>3.618867447641086e+62</ns0:v>
+        <ns0:v>3.618867447641088e+62</ns0:v>
       </ns0:c>
       <ns0:c r="F79" s="1">
         <ns0:f>ROUND(F78*1.4,-5)</ns0:f>
-        <ns0:v>1.885441874347974e+34</ns0:v>
+        <ns0:v>9.991388856031526e+31</ns0:v>
       </ns0:c>
       <ns0:c r="G79" s="1" t="n">
         <ns0:v>16</ns0:v>
@@ -3450,15 +3450,15 @@
       </ns0:c>
       <ns0:c r="D80" s="1">
         <ns0:f>ROUND(D79*10,0)</ns0:f>
-        <ns0:v>3.618867447641086e+63</ns0:v>
+        <ns0:v>3.618867447641088e+63</ns0:v>
       </ns0:c>
       <ns0:c r="E80" s="1">
         <ns0:f>D80</ns0:f>
-        <ns0:v>3.618867447641086e+63</ns0:v>
+        <ns0:v>3.618867447641088e+63</ns0:v>
       </ns0:c>
       <ns0:c r="F80" s="1">
         <ns0:f>ROUND(F79*1.4,-5)</ns0:f>
-        <ns0:v>2.6396186240871637e+34</ns0:v>
+        <ns0:v>1.3987944398444136e+32</ns0:v>
       </ns0:c>
       <ns0:c r="G80" s="1" t="n">
         <ns0:v>16.2</ns0:v>
@@ -3482,15 +3482,15 @@
       </ns0:c>
       <ns0:c r="D81" s="1">
         <ns0:f>ROUND(D80*10,0)</ns0:f>
-        <ns0:v>3.6188674476410865e+64</ns0:v>
+        <ns0:v>3.6188674476410876e+64</ns0:v>
       </ns0:c>
       <ns0:c r="E81" s="1">
         <ns0:f>D81</ns0:f>
-        <ns0:v>3.6188674476410865e+64</ns0:v>
+        <ns0:v>3.6188674476410876e+64</ns0:v>
       </ns0:c>
       <ns0:c r="F81" s="1">
         <ns0:f>ROUND(F80*1.4,-5)</ns0:f>
-        <ns0:v>3.6954660737220284e+34</ns0:v>
+        <ns0:v>1.958312215782179e+32</ns0:v>
       </ns0:c>
       <ns0:c r="G81" s="1" t="n">
         <ns0:v>16.4</ns0:v>
@@ -3514,15 +3514,15 @@
       </ns0:c>
       <ns0:c r="D82" s="1">
         <ns0:f>ROUND(D81*10,0)</ns0:f>
-        <ns0:v>3.6188674476410865e+65</ns0:v>
+        <ns0:v>3.6188674476410874e+65</ns0:v>
       </ns0:c>
       <ns0:c r="E82" s="1">
         <ns0:f>D82</ns0:f>
-        <ns0:v>3.6188674476410865e+65</ns0:v>
+        <ns0:v>3.6188674476410874e+65</ns0:v>
       </ns0:c>
       <ns0:c r="F82" s="1">
         <ns0:f>ROUND(F81*1.4,-5)</ns0:f>
-        <ns0:v>5.173652503210839e+34</ns0:v>
+        <ns0:v>2.74163710209505e+32</ns0:v>
       </ns0:c>
       <ns0:c r="G82" s="1" t="n">
         <ns0:v>16.6</ns0:v>
@@ -3546,15 +3546,15 @@
       </ns0:c>
       <ns0:c r="D83" s="1">
         <ns0:f>ROUND(D82*10,0)</ns0:f>
-        <ns0:v>3.618867447641086e+66</ns0:v>
+        <ns0:v>3.618867447641088e+66</ns0:v>
       </ns0:c>
       <ns0:c r="E83" s="1">
         <ns0:f>D83</ns0:f>
-        <ns0:v>3.618867447641086e+66</ns0:v>
+        <ns0:v>3.618867447641088e+66</ns0:v>
       </ns0:c>
       <ns0:c r="F83" s="1">
         <ns0:f>ROUND(F82*1.4,-5)</ns0:f>
-        <ns0:v>7.243113504495176e+34</ns0:v>
+        <ns0:v>3.83829194293307e+32</ns0:v>
       </ns0:c>
       <ns0:c r="G83" s="1" t="n">
         <ns0:v>16.8</ns0:v>
@@ -3586,7 +3586,7 @@
       </ns0:c>
       <ns0:c r="F84" s="1">
         <ns0:f>ROUND(F83*1.4,-5)</ns0:f>
-        <ns0:v>1.0140358906293245e+35</ns0:v>
+        <ns0:v>5.373608720106297e+32</ns0:v>
       </ns0:c>
       <ns0:c r="G84" s="1" t="n">
         <ns0:v>17</ns0:v>
@@ -3618,7 +3618,7 @@
       </ns0:c>
       <ns0:c r="F85" s="1">
         <ns0:f>ROUND(F84*1.4,-5)</ns0:f>
-        <ns0:v>1.4196502468810543e+35</ns0:v>
+        <ns0:v>7.523052208148816e+32</ns0:v>
       </ns0:c>
       <ns0:c r="G85" s="1" t="n">
         <ns0:v>17.2</ns0:v>
@@ -3650,7 +3650,7 @@
       </ns0:c>
       <ns0:c r="F86" s="1">
         <ns0:f>ROUND(F85*1.4,-5)</ns0:f>
-        <ns0:v>1.987510345633476e+35</ns0:v>
+        <ns0:v>1.0532273091408342e+33</ns0:v>
       </ns0:c>
       <ns0:c r="G86" s="1" t="n">
         <ns0:v>17.4</ns0:v>
@@ -3682,7 +3682,7 @@
       </ns0:c>
       <ns0:c r="F87" s="1">
         <ns0:f>ROUND(F86*1.4,-5)</ns0:f>
-        <ns0:v>2.782514483886866e+35</ns0:v>
+        <ns0:v>1.4745182327971676e+33</ns0:v>
       </ns0:c>
       <ns0:c r="G87" s="1" t="n">
         <ns0:v>17.6</ns0:v>
@@ -3714,7 +3714,7 @@
       </ns0:c>
       <ns0:c r="F88" s="1">
         <ns0:f>ROUND(F87*1.4,-5)</ns0:f>
-        <ns0:v>3.8955202774416125e+35</ns0:v>
+        <ns0:v>2.0643255259160346e+33</ns0:v>
       </ns0:c>
       <ns0:c r="G88" s="1" t="n">
         <ns0:v>17.8</ns0:v>
@@ -3746,7 +3746,7 @@
       </ns0:c>
       <ns0:c r="F89" s="1">
         <ns0:f>ROUND(F88*1.4,-5)</ns0:f>
-        <ns0:v>5.453728388418258e+35</ns0:v>
+        <ns0:v>2.890055736282448e+33</ns0:v>
       </ns0:c>
       <ns0:c r="G89" s="1" t="n">
         <ns0:v>18</ns0:v>
@@ -3778,7 +3778,7 @@
       </ns0:c>
       <ns0:c r="F90" s="1">
         <ns0:f>ROUND(F89*1.4,-5)</ns0:f>
-        <ns0:v>7.635219743785561e+35</ns0:v>
+        <ns0:v>4.046078030795427e+33</ns0:v>
       </ns0:c>
       <ns0:c r="G90" s="1" t="n">
         <ns0:v>18.2</ns0:v>
@@ -3810,7 +3810,7 @@
       </ns0:c>
       <ns0:c r="F91" s="1">
         <ns0:f>ROUND(F90*1.4,-5)</ns0:f>
-        <ns0:v>1.0689307641299785e+36</ns0:v>
+        <ns0:v>5.664509243113597e+33</ns0:v>
       </ns0:c>
       <ns0:c r="G91" s="1" t="n">
         <ns0:v>18.4</ns0:v>
@@ -3842,7 +3842,7 @@
       </ns0:c>
       <ns0:c r="F92" s="1">
         <ns0:f>ROUND(F91*1.4,-5)</ns0:f>
-        <ns0:v>1.4965030697819698e+36</ns0:v>
+        <ns0:v>7.930312940359036e+33</ns0:v>
       </ns0:c>
       <ns0:c r="G92" s="1" t="n">
         <ns0:v>18.6</ns0:v>
@@ -3874,7 +3874,7 @@
       </ns0:c>
       <ns0:c r="F93" s="1">
         <ns0:f>ROUND(F92*1.4,-5)</ns0:f>
-        <ns0:v>2.0951042976947578e+36</ns0:v>
+        <ns0:v>1.110243811650265e+34</ns0:v>
       </ns0:c>
       <ns0:c r="G93" s="1" t="n">
         <ns0:v>18.8</ns0:v>
@@ -3906,7 +3906,7 @@
       </ns0:c>
       <ns0:c r="F94" s="1">
         <ns0:f>ROUND(F93*1.4,-5)</ns0:f>
-        <ns0:v>2.933146016772661e+36</ns0:v>
+        <ns0:v>1.554341336310371e+34</ns0:v>
       </ns0:c>
       <ns0:c r="G94" s="1" t="n">
         <ns0:v>19</ns0:v>
@@ -3938,7 +3938,7 @@
       </ns0:c>
       <ns0:c r="F95" s="1">
         <ns0:f>ROUND(F94*1.4,-5)</ns0:f>
-        <ns0:v>4.106404423481725e+36</ns0:v>
+        <ns0:v>2.176077870834519e+34</ns0:v>
       </ns0:c>
       <ns0:c r="G95" s="1" t="n">
         <ns0:v>19.2</ns0:v>
@@ -3970,7 +3970,7 @@
       </ns0:c>
       <ns0:c r="F96" s="1">
         <ns0:f>ROUND(F95*1.4,-5)</ns0:f>
-        <ns0:v>5.748966192874415e+36</ns0:v>
+        <ns0:v>3.0465090191683266e+34</ns0:v>
       </ns0:c>
       <ns0:c r="G96" s="1" t="n">
         <ns0:v>19.4</ns0:v>
@@ -4002,7 +4002,7 @@
       </ns0:c>
       <ns0:c r="F97" s="1">
         <ns0:f>ROUND(F96*1.4,-5)</ns0:f>
-        <ns0:v>8.048552670024181e+36</ns0:v>
+        <ns0:v>4.265112626835657e+34</ns0:v>
       </ns0:c>
       <ns0:c r="G97" s="1" t="n">
         <ns0:v>19.6</ns0:v>
@@ -4034,7 +4034,7 @@
       </ns0:c>
       <ns0:c r="F98" s="1">
         <ns0:f>ROUND(F97*1.4,-5)</ns0:f>
-        <ns0:v>1.1267973738033853e+37</ns0:v>
+        <ns0:v>5.97115767756992e+34</ns0:v>
       </ns0:c>
       <ns0:c r="G98" s="1" t="n">
         <ns0:v>19.8</ns0:v>
@@ -4066,7 +4066,7 @@
       </ns0:c>
       <ns0:c r="F99" s="1">
         <ns0:f>ROUND(F98*1.4,-5)</ns0:f>
-        <ns0:v>1.5775163233247394e+37</ns0:v>
+        <ns0:v>8.359620748597887e+34</ns0:v>
       </ns0:c>
       <ns0:c r="G99" s="1" t="n">
         <ns0:v>20</ns0:v>
@@ -4098,7 +4098,7 @@
       </ns0:c>
       <ns0:c r="F100" s="1">
         <ns0:f>ROUND(F99*1.4,-5)</ns0:f>
-        <ns0:v>2.208522852654635e+37</ns0:v>
+        <ns0:v>1.170346904803704e+35</ns0:v>
       </ns0:c>
       <ns0:c r="G100" s="1" t="n">
         <ns0:v>20.2</ns0:v>
@@ -4130,7 +4130,7 @@
       </ns0:c>
       <ns0:c r="F101" s="1">
         <ns0:f>ROUND(F100*1.4,-5)</ns0:f>
-        <ns0:v>3.091931993716489e+37</ns0:v>
+        <ns0:v>1.6384856667251856e+35</ns0:v>
       </ns0:c>
       <ns0:c r="G101" s="1" t="n">
         <ns0:v>20.4</ns0:v>
@@ -4162,7 +4162,7 @@
       </ns0:c>
       <ns0:c r="F102" s="1">
         <ns0:f>ROUND(F101*1.4,-5)</ns0:f>
-        <ns0:v>4.328704791203084e+37</ns0:v>
+        <ns0:v>2.2938799334152597e+35</ns0:v>
       </ns0:c>
       <ns0:c r="G102" s="1" t="n">
         <ns0:v>20.6</ns0:v>
@@ -4194,7 +4194,7 @@
       </ns0:c>
       <ns0:c r="F103" s="1">
         <ns0:f>ROUND(F102*1.4,-5)</ns0:f>
-        <ns0:v>6.060186707684317e+37</ns0:v>
+        <ns0:v>3.2114319067813633e+35</ns0:v>
       </ns0:c>
       <ns0:c r="G103" s="1" t="n">
         <ns0:v>20.8</ns0:v>
@@ -4226,7 +4226,7 @@
       </ns0:c>
       <ns0:c r="F104" s="1">
         <ns0:f>ROUND(F103*1.4,-5)</ns0:f>
-        <ns0:v>8.484261390758044e+37</ns0:v>
+        <ns0:v>4.4960046694939086e+35</ns0:v>
       </ns0:c>
       <ns0:c r="G104" s="1" t="n">
         <ns0:v>21</ns0:v>
@@ -4258,7 +4258,7 @@
       </ns0:c>
       <ns0:c r="F105" s="1">
         <ns0:f>ROUND(F104*1.4,-5)</ns0:f>
-        <ns0:v>1.1877965947061261e+38</ns0:v>
+        <ns0:v>6.294406537291471e+35</ns0:v>
       </ns0:c>
       <ns0:c r="G105" s="1" t="n">
         <ns0:v>21.2</ns0:v>
@@ -4290,7 +4290,7 @@
       </ns0:c>
       <ns0:c r="F106" s="1">
         <ns0:f>ROUND(F105*1.4,-5)</ns0:f>
-        <ns0:v>1.6629152325885765e+38</ns0:v>
+        <ns0:v>8.812169152208059e+35</ns0:v>
       </ns0:c>
       <ns0:c r="G106" s="1" t="n">
         <ns0:v>21.4</ns0:v>
@@ -4322,7 +4322,7 @@
       </ns0:c>
       <ns0:c r="F107" s="1">
         <ns0:f>ROUND(F106*1.4,-5)</ns0:f>
-        <ns0:v>2.328081325624007e+38</ns0:v>
+        <ns0:v>1.2337036813091281e+36</ns0:v>
       </ns0:c>
       <ns0:c r="G107" s="1" t="n">
         <ns0:v>21.6</ns0:v>
@@ -4354,7 +4354,7 @@
       </ns0:c>
       <ns0:c r="F108" s="1">
         <ns0:f>ROUND(F107*1.4,-5)</ns0:f>
-        <ns0:v>3.25931385587361e+38</ns0:v>
+        <ns0:v>1.7271851538327794e+36</ns0:v>
       </ns0:c>
       <ns0:c r="G108" s="1" t="n">
         <ns0:v>21.8</ns0:v>
@@ -4386,7 +4386,7 @@
       </ns0:c>
       <ns0:c r="F109" s="1">
         <ns0:f>ROUND(F108*1.4,-5)</ns0:f>
-        <ns0:v>4.563039398223054e+38</ns0:v>
+        <ns0:v>2.418059215365891e+36</ns0:v>
       </ns0:c>
       <ns0:c r="G109" s="1" t="n">
         <ns0:v>22</ns0:v>
@@ -4418,7 +4418,7 @@
       </ns0:c>
       <ns0:c r="F110" s="1">
         <ns0:f>ROUND(F109*1.4,-5)</ns0:f>
-        <ns0:v>6.388255157512275e+38</ns0:v>
+        <ns0:v>3.385282901512247e+36</ns0:v>
       </ns0:c>
       <ns0:c r="G110" s="1" t="n">
         <ns0:v>22.2</ns0:v>
@@ -4450,7 +4450,7 @@
       </ns0:c>
       <ns0:c r="F111" s="1">
         <ns0:f>ROUND(F110*1.4,-5)</ns0:f>
-        <ns0:v>8.943557220517185e+38</ns0:v>
+        <ns0:v>4.7393960621171457e+36</ns0:v>
       </ns0:c>
       <ns0:c r="G111" s="1" t="n">
         <ns0:v>22.4</ns0:v>
@@ -4482,7 +4482,7 @@
       </ns0:c>
       <ns0:c r="F112" s="1">
         <ns0:f>ROUND(F111*1.4,-5)</ns0:f>
-        <ns0:v>1.2520980108724058e+39</ns0:v>
+        <ns0:v>6.635154486964003e+36</ns0:v>
       </ns0:c>
       <ns0:c r="G112" s="1" t="n">
         <ns0:v>22.6</ns0:v>
@@ -4514,7 +4514,7 @@
       </ns0:c>
       <ns0:c r="F113" s="1">
         <ns0:f>ROUND(F112*1.4,-5)</ns0:f>
-        <ns0:v>1.752937215221368e+39</ns0:v>
+        <ns0:v>9.289216281749605e+36</ns0:v>
       </ns0:c>
       <ns0:c r="G113" s="1" t="n">
         <ns0:v>22.8</ns0:v>
@@ -4546,7 +4546,7 @@
       </ns0:c>
       <ns0:c r="F114" s="1">
         <ns0:f>ROUND(F113*1.4,-5)</ns0:f>
-        <ns0:v>2.454112101309915e+39</ns0:v>
+        <ns0:v>1.3004902794449445e+37</ns0:v>
       </ns0:c>
       <ns0:c r="G114" s="1" t="n">
         <ns0:v>23</ns0:v>
@@ -4578,7 +4578,7 @@
       </ns0:c>
       <ns0:c r="F115" s="1">
         <ns0:f>ROUND(F114*1.4,-5)</ns0:f>
-        <ns0:v>3.4357569418338807e+39</ns0:v>
+        <ns0:v>1.8206863912229223e+37</ns0:v>
       </ns0:c>
       <ns0:c r="G115" s="1" t="n">
         <ns0:v>23.2</ns0:v>
@@ -4610,7 +4610,7 @@
       </ns0:c>
       <ns0:c r="F116" s="1">
         <ns0:f>ROUND(F115*1.4,-5)</ns0:f>
-        <ns0:v>4.810059718567433e+39</ns0:v>
+        <ns0:v>2.5489609477120913e+37</ns0:v>
       </ns0:c>
       <ns0:c r="G116" s="1" t="n">
         <ns0:v>23.4</ns0:v>
@@ -4642,7 +4642,7 @@
       </ns0:c>
       <ns0:c r="F117" s="1">
         <ns0:f>ROUND(F116*1.4,-5)</ns0:f>
-        <ns0:v>6.734083605994406e+39</ns0:v>
+        <ns0:v>3.5685453267969277e+37</ns0:v>
       </ns0:c>
       <ns0:c r="G117" s="1" t="n">
         <ns0:v>23.6</ns0:v>
@@ -4674,7 +4674,7 @@
       </ns0:c>
       <ns0:c r="F118" s="1">
         <ns0:f>ROUND(F117*1.4,-5)</ns0:f>
-        <ns0:v>9.427717048392167e+39</ns0:v>
+        <ns0:v>4.995963457515698e+37</ns0:v>
       </ns0:c>
       <ns0:c r="G118" s="1" t="n">
         <ns0:v>23.8</ns0:v>
@@ -4706,7 +4706,7 @@
       </ns0:c>
       <ns0:c r="F119" s="1">
         <ns0:f>ROUND(F118*1.4,-5)</ns0:f>
-        <ns0:v>1.3198803867749033e+40</ns0:v>
+        <ns0:v>6.994348840521976e+37</ns0:v>
       </ns0:c>
       <ns0:c r="G119" s="1" t="n">
         <ns0:v>24</ns0:v>
@@ -4738,7 +4738,7 @@
       </ns0:c>
       <ns0:c r="F120" s="1">
         <ns0:f>ROUND(F119*1.4,-5)</ns0:f>
-        <ns0:v>1.8478325414848646e+40</ns0:v>
+        <ns0:v>9.792088376730766e+37</ns0:v>
       </ns0:c>
       <ns0:c r="G120" s="1" t="n">
         <ns0:v>24.2000000000001</ns0:v>
@@ -4770,7 +4770,7 @@
       </ns0:c>
       <ns0:c r="F121" s="1">
         <ns0:f>ROUND(F120*1.4,-5)</ns0:f>
-        <ns0:v>2.58696555807881e+40</ns0:v>
+        <ns0:v>1.3708923727423071e+38</ns0:v>
       </ns0:c>
       <ns0:c r="G121" s="1" t="n">
         <ns0:v>24.4000000000001</ns0:v>
@@ -4802,7 +4802,7 @@
       </ns0:c>
       <ns0:c r="F122" s="1">
         <ns0:f>ROUND(F121*1.4,-5)</ns0:f>
-        <ns0:v>3.6217517813103335e+40</ns0:v>
+        <ns0:v>1.91924932183923e+38</ns0:v>
       </ns0:c>
       <ns0:c r="G122" s="1" t="n">
         <ns0:v>24.6000000000001</ns0:v>
@@ -4834,7 +4834,7 @@
       </ns0:c>
       <ns0:c r="F123" s="1">
         <ns0:f>ROUND(F122*1.4,-5)</ns0:f>
-        <ns0:v>5.070452493834467e+40</ns0:v>
+        <ns0:v>2.6869490505749215e+38</ns0:v>
       </ns0:c>
       <ns0:c r="G123" s="1" t="n">
         <ns0:v>24.8000000000001</ns0:v>
@@ -4866,7 +4866,7 @@
       </ns0:c>
       <ns0:c r="F124" s="1">
         <ns0:f>ROUND(F123*1.4,-5)</ns0:f>
-        <ns0:v>7.098633491368252e+40</ns0:v>
+        <ns0:v>3.76172867080489e+38</ns0:v>
       </ns0:c>
       <ns0:c r="G124" s="1" t="n">
         <ns0:v>25.0000000000001</ns0:v>
@@ -4898,7 +4898,7 @@
       </ns0:c>
       <ns0:c r="F125" s="1">
         <ns0:f>ROUND(F124*1.4,-5)</ns0:f>
-        <ns0:v>9.938086887915552e+40</ns0:v>
+        <ns0:v>5.266420139126845e+38</ns0:v>
       </ns0:c>
       <ns0:c r="G125" s="1" t="n">
         <ns0:v>25.2000000000001</ns0:v>
@@ -4930,7 +4930,7 @@
       </ns0:c>
       <ns0:c r="F126" s="1">
         <ns0:f>ROUND(F125*1.4,-5)</ns0:f>
-        <ns0:v>1.3913321643081771e+41</ns0:v>
+        <ns0:v>7.372988194777583e+38</ns0:v>
       </ns0:c>
       <ns0:c r="G126" s="1" t="n">
         <ns0:v>25.4000000000001</ns0:v>
@@ -4962,7 +4962,7 @@
       </ns0:c>
       <ns0:c r="F127" s="1">
         <ns0:f>ROUND(F126*1.4,-5)</ns0:f>
-        <ns0:v>1.9478650300314477e+41</ns0:v>
+        <ns0:v>1.0322183472688616e+39</ns0:v>
       </ns0:c>
       <ns0:c r="G127" s="1" t="n">
         <ns0:v>25.6000000000001</ns0:v>
@@ -4994,7 +4994,7 @@
       </ns0:c>
       <ns0:c r="F128" s="1">
         <ns0:f>ROUND(F127*1.4,-5)</ns0:f>
-        <ns0:v>2.7270110420440267e+41</ns0:v>
+        <ns0:v>1.445105686176406e+39</ns0:v>
       </ns0:c>
       <ns0:c r="G128" s="1" t="n">
         <ns0:v>25.8000000000001</ns0:v>
@@ -5026,7 +5026,7 @@
       </ns0:c>
       <ns0:c r="F129" s="1">
         <ns0:f>ROUND(F128*1.4,-5)</ns0:f>
-        <ns0:v>3.817815458861637e+41</ns0:v>
+        <ns0:v>2.0231479606469683e+39</ns0:v>
       </ns0:c>
       <ns0:c r="G129" s="1" t="n">
         <ns0:v>26.0000000000001</ns0:v>
@@ -5058,7 +5058,7 @@
       </ns0:c>
       <ns0:c r="F130" s="1">
         <ns0:f>ROUND(F129*1.4,-5)</ns0:f>
-        <ns0:v>5.3449416424062916e+41</ns0:v>
+        <ns0:v>2.8324071449057554e+39</ns0:v>
       </ns0:c>
       <ns0:c r="G130" s="1" t="n">
         <ns0:v>26.2000000000001</ns0:v>
@@ -5090,7 +5090,7 @@
       </ns0:c>
       <ns0:c r="F131" s="1">
         <ns0:f>ROUND(F130*1.4,-5)</ns0:f>
-        <ns0:v>7.482918299368808e+41</ns0:v>
+        <ns0:v>3.9653700028680576e+39</ns0:v>
       </ns0:c>
       <ns0:c r="G131" s="1" t="n">
         <ns0:v>26.4000000000001</ns0:v>
@@ -5122,7 +5122,7 @@
       </ns0:c>
       <ns0:c r="F132" s="1">
         <ns0:f>ROUND(F131*1.4,-5)</ns0:f>
-        <ns0:v>1.0476085619116331e+42</ns0:v>
+        <ns0:v>5.55151800401528e+39</ns0:v>
       </ns0:c>
       <ns0:c r="G132" s="1" t="n">
         <ns0:v>26.6000000000001</ns0:v>
@@ -5154,7 +5154,7 @@
       </ns0:c>
       <ns0:c r="F133" s="1">
         <ns0:f>ROUND(F132*1.4,-5)</ns0:f>
-        <ns0:v>1.4666519866762864e+42</ns0:v>
+        <ns0:v>7.772125205621392e+39</ns0:v>
       </ns0:c>
       <ns0:c r="G133" s="1" t="n">
         <ns0:v>26.8000000000001</ns0:v>
@@ -5186,7 +5186,7 @@
       </ns0:c>
       <ns0:c r="F134" s="1">
         <ns0:f>ROUND(F133*1.4,-5)</ns0:f>
-        <ns0:v>2.053312781346801e+42</ns0:v>
+        <ns0:v>1.0880975287869949e+40</ns0:v>
       </ns0:c>
       <ns0:c r="G134" s="1" t="n">
         <ns0:v>27.0000000000001</ns0:v>
@@ -5218,7 +5218,7 @@
       </ns0:c>
       <ns0:c r="F135" s="1">
         <ns0:f>ROUND(F134*1.4,-5)</ns0:f>
-        <ns0:v>2.8746378938855214e+42</ns0:v>
+        <ns0:v>1.5233365403017927e+40</ns0:v>
       </ns0:c>
       <ns0:c r="G135" s="1" t="n">
         <ns0:v>27.2000000000001</ns0:v>
@@ -5250,7 +5250,7 @@
       </ns0:c>
       <ns0:c r="F136" s="1">
         <ns0:f>ROUND(F135*1.4,-5)</ns0:f>
-        <ns0:v>4.0244930514397294e+42</ns0:v>
+        <ns0:v>2.1326711564225094e+40</ns0:v>
       </ns0:c>
       <ns0:c r="G136" s="1" t="n">
         <ns0:v>27.4000000000001</ns0:v>
@@ -5282,7 +5282,7 @@
       </ns0:c>
       <ns0:c r="F137" s="1">
         <ns0:f>ROUND(F136*1.4,-5)</ns0:f>
-        <ns0:v>5.634290272015621e+42</ns0:v>
+        <ns0:v>2.985739618991513e+40</ns0:v>
       </ns0:c>
       <ns0:c r="G137" s="1" t="n">
         <ns0:v>27.6000000000001</ns0:v>
@@ -5314,7 +5314,7 @@
       </ns0:c>
       <ns0:c r="F138" s="1">
         <ns0:f>ROUND(F137*1.4,-5)</ns0:f>
-        <ns0:v>7.888006380821869e+42</ns0:v>
+        <ns0:v>4.1800354665881186e+40</ns0:v>
       </ns0:c>
       <ns0:c r="G138" s="1" t="n">
         <ns0:v>27.8000000000001</ns0:v>
@@ -5346,7 +5346,7 @@
       </ns0:c>
       <ns0:c r="F139" s="1">
         <ns0:f>ROUND(F138*1.4,-5)</ns0:f>
-        <ns0:v>1.1043208933150617e+43</ns0:v>
+        <ns0:v>5.852049653223366e+40</ns0:v>
       </ns0:c>
       <ns0:c r="G139" s="1" t="n">
         <ns0:v>28.0000000000001</ns0:v>
@@ -5378,7 +5378,7 @@
       </ns0:c>
       <ns0:c r="F140" s="1">
         <ns0:f>ROUND(F139*1.4,-5)</ns0:f>
-        <ns0:v>1.5460492506410863e+43</ns0:v>
+        <ns0:v>8.192869514512712e+40</ns0:v>
       </ns0:c>
       <ns0:c r="G140" s="1" t="n">
         <ns0:v>28.2000000000001</ns0:v>
@@ -5410,7 +5410,7 @@
       </ns0:c>
       <ns0:c r="F141" s="1">
         <ns0:f>ROUND(F140*1.4,-5)</ns0:f>
-        <ns0:v>2.1644689508975208e+43</ns0:v>
+        <ns0:v>1.1470017320317795e+41</ns0:v>
       </ns0:c>
       <ns0:c r="G141" s="1" t="n">
         <ns0:v>28.4000000000001</ns0:v>
@@ -5442,7 +5442,7 @@
       </ns0:c>
       <ns0:c r="F142" s="1">
         <ns0:f>ROUND(F141*1.4,-5)</ns0:f>
-        <ns0:v>3.030256531256529e+43</ns0:v>
+        <ns0:v>1.6058024248444911e+41</ns0:v>
       </ns0:c>
       <ns0:c r="G142" s="1" t="n">
         <ns0:v>28.6000000000001</ns0:v>
@@ -5474,7 +5474,7 @@
       </ns0:c>
       <ns0:c r="F143" s="1">
         <ns0:f>ROUND(F142*1.4,-5)</ns0:f>
-        <ns0:v>4.24235914375914e+43</ns0:v>
+        <ns0:v>2.2481233947822873e+41</ns0:v>
       </ns0:c>
       <ns0:c r="G143" s="1" t="n">
         <ns0:v>28.8000000000001</ns0:v>
@@ -5506,7 +5506,7 @@
       </ns0:c>
       <ns0:c r="F144" s="1">
         <ns0:f>ROUND(F143*1.4,-5)</ns0:f>
-        <ns0:v>5.939302801262796e+43</ns0:v>
+        <ns0:v>3.1473727526952024e+41</ns0:v>
       </ns0:c>
       <ns0:c r="G144" s="1" t="n">
         <ns0:v>29.0000000000001</ns0:v>
@@ -5538,7 +5538,7 @@
       </ns0:c>
       <ns0:c r="F145" s="1">
         <ns0:f>ROUND(F144*1.4,-5)</ns0:f>
-        <ns0:v>8.315023921767913e+43</ns0:v>
+        <ns0:v>4.406321853773283e+41</ns0:v>
       </ns0:c>
       <ns0:c r="G145" s="1" t="n">
         <ns0:v>29.2000000000001</ns0:v>
@@ -5570,7 +5570,7 @@
       </ns0:c>
       <ns0:c r="F146" s="1">
         <ns0:f>ROUND(F145*1.4,-5)</ns0:f>
-        <ns0:v>1.1641033490475078e+44</ns0:v>
+        <ns0:v>6.168850595282596e+41</ns0:v>
       </ns0:c>
       <ns0:c r="G146" s="1" t="n">
         <ns0:v>29.4000000000001</ns0:v>
@@ -5602,7 +5602,7 @@
       </ns0:c>
       <ns0:c r="F147" s="1">
         <ns0:f>ROUND(F146*1.4,-5)</ns0:f>
-        <ns0:v>1.6297446886665107e+44</ns0:v>
+        <ns0:v>8.636390833395633e+41</ns0:v>
       </ns0:c>
       <ns0:c r="G147" s="1" t="n">
         <ns0:v>29.6000000000001</ns0:v>
@@ -5634,7 +5634,7 @@
       </ns0:c>
       <ns0:c r="F148" s="1">
         <ns0:f>ROUND(F147*1.4,-5)</ns0:f>
-        <ns0:v>2.2816425641331147e+44</ns0:v>
+        <ns0:v>1.2090947166753886e+42</ns0:v>
       </ns0:c>
       <ns0:c r="G148" s="1" t="n">
         <ns0:v>29.8000000000001</ns0:v>
@@ -5666,7 +5666,7 @@
       </ns0:c>
       <ns0:c r="F149" s="1">
         <ns0:f>ROUND(F148*1.4,-5)</ns0:f>
-        <ns0:v>3.1942995897863605e+44</ns0:v>
+        <ns0:v>1.692732603345544e+42</ns0:v>
       </ns0:c>
       <ns0:c r="G149" s="1" t="n">
         <ns0:v>30.0000000000001</ns0:v>
@@ -5698,7 +5698,7 @@
       </ns0:c>
       <ns0:c r="F150" s="1">
         <ns0:f>ROUND(F149*1.4,-5)</ns0:f>
-        <ns0:v>4.472019425700905e+44</ns0:v>
+        <ns0:v>2.369825644683761e+42</ns0:v>
       </ns0:c>
       <ns0:c r="G150" s="1" t="n">
         <ns0:v>30.2000000000001</ns0:v>
@@ -5730,7 +5730,7 @@
       </ns0:c>
       <ns0:c r="F151" s="1">
         <ns0:f>ROUND(F150*1.4,-5)</ns0:f>
-        <ns0:v>6.260827195981266e+44</ns0:v>
+        <ns0:v>3.317755902557265e+42</ns0:v>
       </ns0:c>
       <ns0:c r="G151" s="1" t="n">
         <ns0:v>30.4000000000001</ns0:v>
@@ -5762,7 +5762,7 @@
       </ns0:c>
       <ns0:c r="F152" s="1">
         <ns0:f>ROUND(F151*1.4,-5)</ns0:f>
-        <ns0:v>8.765158074373773e+44</ns0:v>
+        <ns0:v>4.644858263580172e+42</ns0:v>
       </ns0:c>
       <ns0:c r="G152" s="1" t="n">
         <ns0:v>30.6000000000001</ns0:v>
@@ -5794,7 +5794,7 @@
       </ns0:c>
       <ns0:c r="F153" s="1">
         <ns0:f>ROUND(F152*1.4,-5)</ns0:f>
-        <ns0:v>1.2271221304123282e+45</ns0:v>
+        <ns0:v>6.50280156901224e+42</ns0:v>
       </ns0:c>
       <ns0:c r="G153" s="1" t="n">
         <ns0:v>30.8000000000001</ns0:v>
@@ -5826,7 +5826,7 @@
       </ns0:c>
       <ns0:c r="F154" s="1">
         <ns0:f>ROUND(F153*1.4,-5)</ns0:f>
-        <ns0:v>1.7179709825772595e+45</ns0:v>
+        <ns0:v>9.103922196617134e+42</ns0:v>
       </ns0:c>
       <ns0:c r="G154" s="1" t="n">
         <ns0:v>31.0000000000001</ns0:v>
@@ -5858,7 +5858,7 @@
       </ns0:c>
       <ns0:c r="F155" s="1">
         <ns0:f>ROUND(F154*1.4,-5)</ns0:f>
-        <ns0:v>2.405159375608163e+45</ns0:v>
+        <ns0:v>1.2745491075263987e+43</ns0:v>
       </ns0:c>
       <ns0:c r="G155" s="1" t="n">
         <ns0:v>31.2000000000001</ns0:v>
@@ -5890,7 +5890,7 @@
       </ns0:c>
       <ns0:c r="F156" s="1">
         <ns0:f>ROUND(F155*1.4,-5)</ns0:f>
-        <ns0:v>3.367223125851428e+45</ns0:v>
+        <ns0:v>1.7843687505369578e+43</ns0:v>
       </ns0:c>
       <ns0:c r="G156" s="1" t="n">
         <ns0:v>31.4000000000001</ns0:v>
@@ -5922,7 +5922,7 @@
       </ns0:c>
       <ns0:c r="F157" s="1">
         <ns0:f>ROUND(F156*1.4,-5)</ns0:f>
-        <ns0:v>4.714112376191999e+45</ns0:v>
+        <ns0:v>2.4981162507517407e+43</ns0:v>
       </ns0:c>
       <ns0:c r="G157" s="1" t="n">
         <ns0:v>31.6000000000001</ns0:v>
@@ -5954,7 +5954,7 @@
       </ns0:c>
       <ns0:c r="F158" s="1">
         <ns0:f>ROUND(F157*1.4,-5)</ns0:f>
-        <ns0:v>6.599757326668798e+45</ns0:v>
+        <ns0:v>3.497362751052437e+43</ns0:v>
       </ns0:c>
       <ns0:c r="G158" s="1" t="n">
         <ns0:v>31.8000000000001</ns0:v>
@@ -5986,7 +5986,7 @@
       </ns0:c>
       <ns0:c r="F159" s="1">
         <ns0:f>ROUND(F158*1.4,-5)</ns0:f>
-        <ns0:v>9.239660257336316e+45</ns0:v>
+        <ns0:v>4.896307851473411e+43</ns0:v>
       </ns0:c>
       <ns0:c r="G159" s="1" t="n">
         <ns0:v>32.0000000000001</ns0:v>
@@ -6018,7 +6018,7 @@
       </ns0:c>
       <ns0:c r="F160" s="1">
         <ns0:f>ROUND(F159*1.4,-5)</ns0:f>
-        <ns0:v>1.2935524360270842e+46</ns0:v>
+        <ns0:v>6.854830992062775e+43</ns0:v>
       </ns0:c>
       <ns0:c r="G160" s="1" t="n">
         <ns0:v>32.2000000000001</ns0:v>
@@ -6050,7 +6050,7 @@
       </ns0:c>
       <ns0:c r="F161" s="1">
         <ns0:f>ROUND(F160*1.4,-5)</ns0:f>
-        <ns0:v>1.8109734104379178e+46</ns0:v>
+        <ns0:v>9.596763388887884e+43</ns0:v>
       </ns0:c>
       <ns0:c r="G161" s="1" t="n">
         <ns0:v>32.4000000000001</ns0:v>
@@ -6082,7 +6082,7 @@
       </ns0:c>
       <ns0:c r="F162" s="1">
         <ns0:f>ROUND(F161*1.4,-5)</ns0:f>
-        <ns0:v>2.5353627746130845e+46</ns0:v>
+        <ns0:v>1.3435468744443037e+44</ns0:v>
       </ns0:c>
       <ns0:c r="G162" s="1" t="n">
         <ns0:v>32.6000000000001</ns0:v>
@@ -6114,7 +6114,7 @@
       </ns0:c>
       <ns0:c r="F163" s="1">
         <ns0:f>ROUND(F162*1.4,-5)</ns0:f>
-        <ns0:v>3.5495078844583184e+46</ns0:v>
+        <ns0:v>1.880965624222025e+44</ns0:v>
       </ns0:c>
       <ns0:c r="G163" s="1" t="n">
         <ns0:v>32.8000000000001</ns0:v>
@@ -6146,7 +6146,7 @@
       </ns0:c>
       <ns0:c r="F164" s="1">
         <ns0:f>ROUND(F163*1.4,-5)</ns0:f>
-        <ns0:v>4.969311038241645e+46</ns0:v>
+        <ns0:v>2.633351873910835e+44</ns0:v>
       </ns0:c>
       <ns0:c r="G164" s="1" t="n">
         <ns0:v>33.0000000000001</ns0:v>
@@ -6178,7 +6178,7 @@
       </ns0:c>
       <ns0:c r="F165" s="1">
         <ns0:f>ROUND(F164*1.4,-5)</ns0:f>
-        <ns0:v>6.957035453538303e+46</ns0:v>
+        <ns0:v>3.686692623475169e+44</ns0:v>
       </ns0:c>
       <ns0:c r="G165" s="1" t="n">
         <ns0:v>33.2000000000001</ns0:v>
@@ -6210,7 +6210,7 @@
       </ns0:c>
       <ns0:c r="F166" s="1">
         <ns0:f>ROUND(F165*1.4,-5)</ns0:f>
-        <ns0:v>9.739849634953624e+46</ns0:v>
+        <ns0:v>5.161369672865237e+44</ns0:v>
       </ns0:c>
       <ns0:c r="G166" s="1" t="n">
         <ns0:v>33.4000000000001</ns0:v>
@@ -6242,7 +6242,7 @@
       </ns0:c>
       <ns0:c r="F167" s="1">
         <ns0:f>ROUND(F166*1.4,-5)</ns0:f>
-        <ns0:v>1.3635789488935073e+47</ns0:v>
+        <ns0:v>7.225917542011331e+44</ns0:v>
       </ns0:c>
       <ns0:c r="G167" s="1" t="n">
         <ns0:v>33.6000000000001</ns0:v>
@@ -6274,7 +6274,7 @@
       </ns0:c>
       <ns0:c r="F168" s="1">
         <ns0:f>ROUND(F167*1.4,-5)</ns0:f>
-        <ns0:v>1.9090105284509103e+47</ns0:v>
+        <ns0:v>1.0116284558815864e+45</ns0:v>
       </ns0:c>
       <ns0:c r="G168" s="1" t="n">
         <ns0:v>33.8000000000001</ns0:v>
@@ -6306,7 +6306,7 @@
       </ns0:c>
       <ns0:c r="F169" s="1">
         <ns0:f>ROUND(F168*1.4,-5)</ns0:f>
-        <ns0:v>2.6726147398312744e+47</ns0:v>
+        <ns0:v>1.4162798382342208e+45</ns0:v>
       </ns0:c>
       <ns0:c r="G169" s="1" t="n">
         <ns0:v>34.0000000000001</ns0:v>
@@ -6338,7 +6338,7 @@
       </ns0:c>
       <ns0:c r="F170" s="1">
         <ns0:f>ROUND(F169*1.4,-5)</ns0:f>
-        <ns0:v>3.741660635763784e+47</ns0:v>
+        <ns0:v>1.982791773527909e+45</ns0:v>
       </ns0:c>
       <ns0:c r="G170" s="1" t="n">
         <ns0:v>34.2000000000001</ns0:v>
@@ -6370,7 +6370,7 @@
       </ns0:c>
       <ns0:c r="F171" s="1">
         <ns0:f>ROUND(F170*1.4,-5)</ns0:f>
-        <ns0:v>5.238324890069298e+47</ns0:v>
+        <ns0:v>2.7759084829390727e+45</ns0:v>
       </ns0:c>
       <ns0:c r="G171" s="1" t="n">
         <ns0:v>34.4000000000001</ns0:v>
@@ -6402,7 +6402,7 @@
       </ns0:c>
       <ns0:c r="F172" s="1">
         <ns0:f>ROUND(F171*1.4,-5)</ns0:f>
-        <ns0:v>7.333654846097016e+47</ns0:v>
+        <ns0:v>3.886271876114702e+45</ns0:v>
       </ns0:c>
       <ns0:c r="G172" s="1" t="n">
         <ns0:v>34.6000000000001</ns0:v>
@@ -6434,7 +6434,7 @@
       </ns0:c>
       <ns0:c r="F173" s="1">
         <ns0:f>ROUND(F172*1.4,-5)</ns0:f>
-        <ns0:v>1.0267116784535822e+48</ns0:v>
+        <ns0:v>5.4407806265605814e+45</ns0:v>
       </ns0:c>
       <ns0:c r="G173" s="1" t="n">
         <ns0:v>34.8000000000001</ns0:v>
@@ -6466,7 +6466,7 @@
       </ns0:c>
       <ns0:c r="F174" s="1">
         <ns0:f>ROUND(F173*1.4,-5)</ns0:f>
-        <ns0:v>1.437396349835015e+48</ns0:v>
+        <ns0:v>7.617092877184813e+45</ns0:v>
       </ns0:c>
       <ns0:c r="G174" s="1" t="n">
         <ns0:v>35.0000000000001</ns0:v>
@@ -6498,7 +6498,7 @@
       </ns0:c>
       <ns0:c r="F175" s="1">
         <ns0:f>ROUND(F174*1.4,-5)</ns0:f>
-        <ns0:v>2.012354889769021e+48</ns0:v>
+        <ns0:v>1.0663930028058737e+46</ns0:v>
       </ns0:c>
       <ns0:c r="G175" s="1" t="n">
         <ns0:v>35.2000000000001</ns0:v>
@@ -6530,7 +6530,7 @@
       </ns0:c>
       <ns0:c r="F176" s="1">
         <ns0:f>ROUND(F175*1.4,-5)</ns0:f>
-        <ns0:v>2.817296845676629e+48</ns0:v>
+        <ns0:v>1.492950203928223e+46</ns0:v>
       </ns0:c>
       <ns0:c r="G176" s="1" t="n">
         <ns0:v>35.4000000000001</ns0:v>
@@ -6562,7 +6562,7 @@
       </ns0:c>
       <ns0:c r="F177" s="1">
         <ns0:f>ROUND(F176*1.4,-5)</ns0:f>
-        <ns0:v>3.9442155839472805e+48</ns0:v>
+        <ns0:v>2.0901302854995122e+46</ns0:v>
       </ns0:c>
       <ns0:c r="G177" s="1" t="n">
         <ns0:v>35.6000000000001</ns0:v>
@@ -6594,7 +6594,7 @@
       </ns0:c>
       <ns0:c r="F178" s="1">
         <ns0:f>ROUND(F177*1.4,-5)</ns0:f>
-        <ns0:v>5.521901817526192e+48</ns0:v>
+        <ns0:v>2.926182399699317e+46</ns0:v>
       </ns0:c>
       <ns0:c r="G178" s="1" t="n">
         <ns0:v>35.8000000000001</ns0:v>
@@ -6626,7 +6626,7 @@
       </ns0:c>
       <ns0:c r="F179" s="1">
         <ns0:f>ROUND(F178*1.4,-5)</ns0:f>
-        <ns0:v>7.730662544536668e+48</ns0:v>
+        <ns0:v>4.096655359579043e+46</ns0:v>
       </ns0:c>
       <ns0:c r="G179" s="1" t="n">
         <ns0:v>36.0000000000001</ns0:v>
@@ -6658,7 +6658,7 @@
       </ns0:c>
       <ns0:c r="F180" s="1">
         <ns0:f>ROUND(F179*1.4,-5)</ns0:f>
-        <ns0:v>1.0822927562351333e+49</ns0:v>
+        <ns0:v>5.73531750341066e+46</ns0:v>
       </ns0:c>
       <ns0:c r="G180" s="1" t="n">
         <ns0:v>36.2000000000001</ns0:v>
@@ -6690,7 +6690,7 @@
       </ns0:c>
       <ns0:c r="F181" s="1">
         <ns0:f>ROUND(F180*1.4,-5)</ns0:f>
-        <ns0:v>1.5152098587291864e+49</ns0:v>
+        <ns0:v>8.029444504774923e+46</ns0:v>
       </ns0:c>
       <ns0:c r="G181" s="1" t="n">
         <ns0:v>36.4000000000001</ns0:v>
@@ -6722,7 +6722,7 @@
       </ns0:c>
       <ns0:c r="F182" s="1">
         <ns0:f>ROUND(F181*1.4,-5)</ns0:f>
-        <ns0:v>2.1212938022208608e+49</ns0:v>
+        <ns0:v>1.1241222306684891e+47</ns0:v>
       </ns0:c>
       <ns0:c r="G182" s="1" t="n">
         <ns0:v>36.6000000000001</ns0:v>
@@ -6754,7 +6754,7 @@
       </ns0:c>
       <ns0:c r="F183" s="1">
         <ns0:f>ROUND(F182*1.4,-5)</ns0:f>
-        <ns0:v>2.9698113231092047e+49</ns0:v>
+        <ns0:v>1.5737711229358847e+47</ns0:v>
       </ns0:c>
       <ns0:c r="G183" s="1" t="n">
         <ns0:v>36.8000000000001</ns0:v>
@@ -6786,7 +6786,7 @@
       </ns0:c>
       <ns0:c r="F184" s="1">
         <ns0:f>ROUND(F183*1.4,-5)</ns0:f>
-        <ns0:v>4.1577358523528863e+49</ns0:v>
+        <ns0:v>2.2032795721102382e+47</ns0:v>
       </ns0:c>
       <ns0:c r="G184" s="1" t="n">
         <ns0:v>37.0000000000001</ns0:v>
@@ -6818,7 +6818,7 @@
       </ns0:c>
       <ns0:c r="F185" s="1">
         <ns0:f>ROUND(F184*1.4,-5)</ns0:f>
-        <ns0:v>5.82083019329404e+49</ns0:v>
+        <ns0:v>3.0845914009543333e+47</ns0:v>
       </ns0:c>
       <ns0:c r="G185" s="1" t="n">
         <ns0:v>37.2000000000001</ns0:v>
@@ -6850,7 +6850,7 @@
       </ns0:c>
       <ns0:c r="F186" s="1">
         <ns0:f>ROUND(F185*1.4,-5)</ns0:f>
-        <ns0:v>8.149162270611656e+49</ns0:v>
+        <ns0:v>4.3184279613360664e+47</ns0:v>
       </ns0:c>
       <ns0:c r="G186" s="1" t="n">
         <ns0:v>37.4000000000001</ns0:v>
@@ -6882,7 +6882,7 @@
       </ns0:c>
       <ns0:c r="F187" s="1">
         <ns0:f>ROUND(F186*1.4,-5)</ns0:f>
-        <ns0:v>1.1408827178856317e+50</ns0:v>
+        <ns0:v>6.045799145870493e+47</ns0:v>
       </ns0:c>
       <ns0:c r="G187" s="1" t="n">
         <ns0:v>37.6000000000001</ns0:v>
@@ -6914,7 +6914,7 @@
       </ns0:c>
       <ns0:c r="F188" s="1">
         <ns0:f>ROUND(F187*1.4,-5)</ns0:f>
-        <ns0:v>1.5972358050398844e+50</ns0:v>
+        <ns0:v>8.464118804218689e+47</ns0:v>
       </ns0:c>
       <ns0:c r="G188" s="1" t="n">
         <ns0:v>37.8000000000001</ns0:v>
@@ -6946,7 +6946,7 @@
       </ns0:c>
       <ns0:c r="F189" s="1">
         <ns0:f>ROUND(F188*1.4,-5)</ns0:f>
-        <ns0:v>2.236130127055838e+50</ns0:v>
+        <ns0:v>1.1849766325906162e+48</ns0:v>
       </ns0:c>
       <ns0:c r="G189" s="1" t="n">
         <ns0:v>38.0000000000001</ns0:v>
@@ -6978,7 +6978,7 @@
       </ns0:c>
       <ns0:c r="F190" s="1">
         <ns0:f>ROUND(F189*1.4,-5)</ns0:f>
-        <ns0:v>3.130582177878173e+50</ns0:v>
+        <ns0:v>1.6589672856268625e+48</ns0:v>
       </ns0:c>
       <ns0:c r="G190" s="1" t="n">
         <ns0:v>38.2000000000001</ns0:v>
@@ -7010,7 +7010,7 @@
       </ns0:c>
       <ns0:c r="F191" s="1">
         <ns0:f>ROUND(F190*1.4,-5)</ns0:f>
-        <ns0:v>4.382815049029442e+50</ns0:v>
+        <ns0:v>2.3225541998776073e+48</ns0:v>
       </ns0:c>
       <ns0:c r="G191" s="1" t="n">
         <ns0:v>38.4000000000001</ns0:v>
@@ -7042,7 +7042,7 @@
       </ns0:c>
       <ns0:c r="F192" s="1">
         <ns0:f>ROUND(F191*1.4,-5)</ns0:f>
-        <ns0:v>6.135941068641219e+50</ns0:v>
+        <ns0:v>3.2515758798286497e+48</ns0:v>
       </ns0:c>
       <ns0:c r="G192" s="1" t="n">
         <ns0:v>38.6000000000001</ns0:v>
@@ -7074,7 +7074,7 @@
       </ns0:c>
       <ns0:c r="F193" s="1">
         <ns0:f>ROUND(F192*1.4,-5)</ns0:f>
-        <ns0:v>8.590317496097706e+50</ns0:v>
+        <ns0:v>4.55220623176011e+48</ns0:v>
       </ns0:c>
       <ns0:c r="G193" s="1" t="n">
         <ns0:v>38.8000000000001</ns0:v>
@@ -7106,7 +7106,7 @@
       </ns0:c>
       <ns0:c r="F194" s="1">
         <ns0:f>ROUND(F193*1.4,-5)</ns0:f>
-        <ns0:v>1.2026444494536786e+51</ns0:v>
+        <ns0:v>6.373088724464154e+48</ns0:v>
       </ns0:c>
       <ns0:c r="G194" s="1" t="n">
         <ns0:v>39.0000000000001</ns0:v>
@@ -7138,7 +7138,7 @@
       </ns0:c>
       <ns0:c r="F195" s="1">
         <ns0:f>ROUND(F194*1.4,-5)</ns0:f>
-        <ns0:v>1.68370222923515e+51</ns0:v>
+        <ns0:v>8.922324214249816e+48</ns0:v>
       </ns0:c>
       <ns0:c r="G195" s="1" t="n">
         <ns0:v>39.2000000000001</ns0:v>
@@ -7170,7 +7170,7 @@
       </ns0:c>
       <ns0:c r="F196" s="1">
         <ns0:f>ROUND(F195*1.4,-5)</ns0:f>
-        <ns0:v>2.35718312092921e+51</ns0:v>
+        <ns0:v>1.249125389994974e+49</ns0:v>
       </ns0:c>
       <ns0:c r="G196" s="1" t="n">
         <ns0:v>39.4000000000001</ns0:v>
@@ -7202,7 +7202,7 @@
       </ns0:c>
       <ns0:c r="F197" s="1">
         <ns0:f>ROUND(F196*1.4,-5)</ns0:f>
-        <ns0:v>3.300056369300893e+51</ns0:v>
+        <ns0:v>1.7487755459929634e+49</ns0:v>
       </ns0:c>
       <ns0:c r="G197" s="1" t="n">
         <ns0:v>39.6000000000001</ns0:v>
@@ -7234,7 +7234,7 @@
       </ns0:c>
       <ns0:c r="F198" s="1">
         <ns0:f>ROUND(F197*1.4,-5)</ns0:f>
-        <ns0:v>4.6200789170212506e+51</ns0:v>
+        <ns0:v>2.4482857643901485e+49</ns0:v>
       </ns0:c>
       <ns0:c r="G198" s="1" t="n">
         <ns0:v>39.8000000000001</ns0:v>
@@ -7266,7 +7266,7 @@
       </ns0:c>
       <ns0:c r="F199" s="1">
         <ns0:f>ROUND(F198*1.4,-5)</ns0:f>
-        <ns0:v>6.46811048382975e+51</ns0:v>
+        <ns0:v>3.427600070146208e+49</ns0:v>
       </ns0:c>
       <ns0:c r="G199" s="1" t="n">
         <ns0:v>40.0000000000001</ns0:v>
@@ -7298,7 +7298,7 @@
       </ns0:c>
       <ns0:c r="F200" s="1">
         <ns0:f>ROUND(F199*1.4,-5)</ns0:f>
-        <ns0:v>9.05535467736165e+51</ns0:v>
+        <ns0:v>4.798640098204691e+49</ns0:v>
       </ns0:c>
       <ns0:c r="G200" s="1" t="n">
         <ns0:v>40.2000000000001</ns0:v>
@@ -7330,7 +7330,7 @@
       </ns0:c>
       <ns0:c r="F201" s="1">
         <ns0:f>ROUND(F200*1.4,-5)</ns0:f>
-        <ns0:v>1.267749654830631e+52</ns0:v>
+        <ns0:v>6.718096137486567e+49</ns0:v>
       </ns0:c>
       <ns0:c r="G201" s="1" t="n">
         <ns0:v>40.4000000000001</ns0:v>
@@ -7362,7 +7362,7 @@
       </ns0:c>
       <ns0:c r="F202" s="1">
         <ns0:f>ROUND(F201*1.4,-5)</ns0:f>
-        <ns0:v>1.774849516762883e+52</ns0:v>
+        <ns0:v>9.405334592481194e+49</ns0:v>
       </ns0:c>
       <ns0:c r="G202" s="1" t="n">
         <ns0:v>40.6000000000001</ns0:v>
@@ -7394,7 +7394,7 @@
       </ns0:c>
       <ns0:c r="F203" s="1">
         <ns0:f>ROUND(F202*1.4,-5)</ns0:f>
-        <ns0:v>2.484789323468036e+52</ns0:v>
+        <ns0:v>1.3167468429473672e+50</ns0:v>
       </ns0:c>
       <ns0:c r="G203" s="1" t="n">
         <ns0:v>40.8000000000001</ns0:v>
@@ -7426,7 +7426,7 @@
       </ns0:c>
       <ns0:c r="F204" s="1">
         <ns0:f>ROUND(F203*1.4,-5)</ns0:f>
-        <ns0:v>3.47870505285525e+52</ns0:v>
+        <ns0:v>1.8434455801263142e+50</ns0:v>
       </ns0:c>
       <ns0:c r="G204" s="1" t="n">
         <ns0:v>41.0000000000001</ns0:v>
@@ -7458,7 +7458,7 @@
       </ns0:c>
       <ns0:c r="F205" s="1">
         <ns0:f>ROUND(F204*1.4,-5)</ns0:f>
-        <ns0:v>4.87018707399735e+52</ns0:v>
+        <ns0:v>2.58082381217684e+50</ns0:v>
       </ns0:c>
       <ns0:c r="G205" s="1" t="n">
         <ns0:v>41.2000000000001</ns0:v>
@@ -7490,7 +7490,7 @@
       </ns0:c>
       <ns0:c r="F206" s="1">
         <ns0:f>ROUND(F205*1.4,-5)</ns0:f>
-        <ns0:v>6.81826190359629e+52</ns0:v>
+        <ns0:v>3.613153337047575e+50</ns0:v>
       </ns0:c>
       <ns0:c r="G206" s="1" t="n">
         <ns0:v>41.4000000000001</ns0:v>
@@ -7522,7 +7522,7 @@
       </ns0:c>
       <ns0:c r="F207" s="1">
         <ns0:f>ROUND(F206*1.4,-5)</ns0:f>
-        <ns0:v>9.545566665034806e+52</ns0:v>
+        <ns0:v>5.058414671866605e+50</ns0:v>
       </ns0:c>
       <ns0:c r="G207" s="1" t="n">
         <ns0:v>41.6000000000001</ns0:v>
@@ -7554,7 +7554,7 @@
       </ns0:c>
       <ns0:c r="F208" s="1">
         <ns0:f>ROUND(F207*1.4,-5)</ns0:f>
-        <ns0:v>1.3363793331048728e+53</ns0:v>
+        <ns0:v>7.081780540613247e+50</ns0:v>
       </ns0:c>
       <ns0:c r="G208" s="1" t="n">
         <ns0:v>41.8000000000001</ns0:v>
@@ -7586,7 +7586,7 @@
       </ns0:c>
       <ns0:c r="F209" s="1">
         <ns0:f>ROUND(F208*1.4,-5)</ns0:f>
-        <ns0:v>1.8709310663468219e+53</ns0:v>
+        <ns0:v>9.914492756858545e+50</ns0:v>
       </ns0:c>
       <ns0:c r="G209" s="1" t="n">
         <ns0:v>42.0000000000001</ns0:v>
@@ -7618,7 +7618,7 @@
       </ns0:c>
       <ns0:c r="F210" s="1">
         <ns0:f>ROUND(F209*1.4,-5)</ns0:f>
-        <ns0:v>2.6193034928855506e+53</ns0:v>
+        <ns0:v>1.3880289859601963e+51</ns0:v>
       </ns0:c>
       <ns0:c r="G210" s="1" t="n">
         <ns0:v>42.2000000000001</ns0:v>
@@ -7650,7 +7650,7 @@
       </ns0:c>
       <ns0:c r="F211" s="1">
         <ns0:f>ROUND(F210*1.4,-5)</ns0:f>
-        <ns0:v>3.6670248900397707e+53</ns0:v>
+        <ns0:v>1.9432405803442746e+51</ns0:v>
       </ns0:c>
       <ns0:c r="G211" s="1" t="n">
         <ns0:v>42.4000000000001</ns0:v>
@@ -7682,7 +7682,7 @@
       </ns0:c>
       <ns0:c r="F212" s="1">
         <ns0:f>ROUND(F211*1.4,-5)</ns0:f>
-        <ns0:v>5.133834846055678e+53</ns0:v>
+        <ns0:v>2.7205368124819845e+51</ns0:v>
       </ns0:c>
       <ns0:c r="G212" s="1" t="n">
         <ns0:v>42.6000000000002</ns0:v>
@@ -7714,7 +7714,7 @@
       </ns0:c>
       <ns0:c r="F213" s="1">
         <ns0:f>ROUND(F212*1.4,-5)</ns0:f>
-        <ns0:v>7.187368784477949e+53</ns0:v>
+        <ns0:v>3.808751537474778e+51</ns0:v>
       </ns0:c>
       <ns0:c r="G213" s="1" t="n">
         <ns0:v>42.8000000000002</ns0:v>
@@ -7746,7 +7746,7 @@
       </ns0:c>
       <ns0:c r="F214" s="1">
         <ns0:f>ROUND(F213*1.4,-5)</ns0:f>
-        <ns0:v>1.0062316298269128e+54</ns0:v>
+        <ns0:v>5.33225215246469e+51</ns0:v>
       </ns0:c>
       <ns0:c r="G214" s="1" t="n">
         <ns0:v>43.0000000000001</ns0:v>
@@ -7778,7 +7778,7 @@
       </ns0:c>
       <ns0:c r="F215" s="1">
         <ns0:f>ROUND(F214*1.4,-5)</ns0:f>
-        <ns0:v>1.4087242817576779e+54</ns0:v>
+        <ns0:v>7.465153013450565e+51</ns0:v>
       </ns0:c>
       <ns0:c r="G215" s="1" t="n">
         <ns0:v>43.2000000000002</ns0:v>
@@ -7810,7 +7810,7 @@
       </ns0:c>
       <ns0:c r="F216" s="1">
         <ns0:f>ROUND(F215*1.4,-5)</ns0:f>
-        <ns0:v>1.9722139944607488e+54</ns0:v>
+        <ns0:v>1.0451214218830791e+52</ns0:v>
       </ns0:c>
       <ns0:c r="G216" s="1" t="n">
         <ns0:v>43.4000000000002</ns0:v>
@@ -7842,7 +7842,7 @@
       </ns0:c>
       <ns0:c r="F217" s="1">
         <ns0:f>ROUND(F216*1.4,-5)</ns0:f>
-        <ns0:v>2.7610995922450485e+54</ns0:v>
+        <ns0:v>1.4631699906363107e+52</ns0:v>
       </ns0:c>
       <ns0:c r="G217" s="1" t="n">
         <ns0:v>43.6000000000002</ns0:v>
@@ -7874,7 +7874,7 @@
       </ns0:c>
       <ns0:c r="F218" s="1">
         <ns0:f>ROUND(F217*1.4,-5)</ns0:f>
-        <ns0:v>3.865539429143068e+54</ns0:v>
+        <ns0:v>2.0484379868908348e+52</ns0:v>
       </ns0:c>
       <ns0:c r="G218" s="1" t="n">
         <ns0:v>43.8000000000002</ns0:v>
@@ -7906,7 +7906,7 @@
       </ns0:c>
       <ns0:c r="F219" s="1">
         <ns0:f>ROUND(F218*1.4,-5)</ns0:f>
-        <ns0:v>5.4117552008002956e+54</ns0:v>
+        <ns0:v>2.867813181647169e+52</ns0:v>
       </ns0:c>
       <ns0:c r="G219" s="1" t="n">
         <ns0:v>44.0000000000002</ns0:v>
@@ -7938,7 +7938,7 @@
       </ns0:c>
       <ns0:c r="F220" s="1">
         <ns0:f>ROUND(F219*1.4,-5)</ns0:f>
-        <ns0:v>7.576457281120413e+54</ns0:v>
+        <ns0:v>4.014938454306036e+52</ns0:v>
       </ns0:c>
       <ns0:c r="G220" s="1" t="n">
         <ns0:v>44.2000000000002</ns0:v>
@@ -7970,7 +7970,7 @@
       </ns0:c>
       <ns0:c r="F221" s="1">
         <ns0:f>ROUND(F220*1.4,-5)</ns0:f>
-        <ns0:v>1.0607040193568578e+55</ns0:v>
+        <ns0:v>5.620913836028451e+52</ns0:v>
       </ns0:c>
       <ns0:c r="G221" s="1" t="n">
         <ns0:v>44.4000000000002</ns0:v>
@@ -8002,7 +8002,7 @@
       </ns0:c>
       <ns0:c r="F222" s="1">
         <ns0:f>ROUND(F221*1.4,-5)</ns0:f>
-        <ns0:v>1.4849856270996007e+55</ns0:v>
+        <ns0:v>7.86927937043983e+52</ns0:v>
       </ns0:c>
       <ns0:c r="G222" s="1" t="n">
         <ns0:v>44.6000000000002</ns0:v>
@@ -8034,7 +8034,7 @@
       </ns0:c>
       <ns0:c r="F223" s="1">
         <ns0:f>ROUND(F222*1.4,-5)</ns0:f>
-        <ns0:v>2.0789798779394408e+55</ns0:v>
+        <ns0:v>1.1016991118615762e+53</ns0:v>
       </ns0:c>
       <ns0:c r="G223" s="1" t="n">
         <ns0:v>44.8000000000002</ns0:v>

</xml_diff>

<commit_message>
Preserve fractional saved resources and freeze income-step 6.7 diagnostic candidate
</commit_message>
<xml_diff>
--- a/space-battleship/config_excel/level.xlsx
+++ b/space-battleship/config_excel/level.xlsx
@@ -1581,7 +1581,7 @@
         <ns0:v>6450407.623907364</ns0:v>
       </ns0:c>
       <ns0:c r="F15" s="1" t="n">
-        <ns0:v>67617.01722380001</ns0:v>
+        <ns0:v>64017.93115473424</ns0:v>
       </ns0:c>
       <ns0:c r="G15" s="1" t="n">
         <ns0:v>3.2</ns0:v>
@@ -1609,7 +1609,7 @@
         <ns0:v>69014978.76834521</ns0:v>
       </ns0:c>
       <ns0:c r="F16" s="1" t="n">
-        <ns0:v>242283.9978695894</ns0:v>
+        <ns0:v>217178.0771275556</ns0:v>
       </ns0:c>
       <ns0:c r="G16" s="1" t="n">
         <ns0:v>3.4</ns0:v>
@@ -1637,7 +1637,7 @@
         <ns0:v>738413379.7593849</ns0:v>
       </ns0:c>
       <ns0:c r="F17" s="1" t="n">
-        <ns0:v>868147.3693135534</ns0:v>
+        <ns0:v>736767.2827605028</ns0:v>
       </ns0:c>
       <ns0:c r="G17" s="1" t="n">
         <ns0:v>3.6</ns0:v>
@@ -1665,7 +1665,7 @@
         <ns0:v>7900521439.525051</ns0:v>
       </ns0:c>
       <ns0:c r="F18" s="1" t="n">
-        <ns0:v>3110728.985294833</ns0:v>
+        <ns0:v>2499451.308004148</ns0:v>
       </ns0:c>
       <ns0:c r="G18" s="1" t="n">
         <ns0:v>3.8</ns0:v>
@@ -1693,7 +1693,7 @@
         <ns0:v>84530211298.0865</ns0:v>
       </ns0:c>
       <ns0:c r="F19" s="1" t="n">
-        <ns0:v>11146304.37411193</ns0:v>
+        <ns0:v>8479281.025721673</ns0:v>
       </ns0:c>
       <ns0:c r="G19" s="1" t="n">
         <ns0:v>4</ns0:v>
@@ -1721,7 +1721,7 @@
         <ns0:v>904415825815.2517</ns0:v>
       </ns0:c>
       <ns0:c r="F20" s="1" t="n">
-        <ns0:v>39939223.82427385</ns0:v>
+        <ns0:v>28765596.06619243</ns0:v>
       </ns0:c>
       <ns0:c r="G20" s="1" t="n">
         <ns0:v>4.2</ns0:v>
@@ -1749,7 +1749,7 @@
         <ns0:v>9676634819953.418</ns0:v>
       </ns0:c>
       <ns0:c r="F21" s="1" t="n">
-        <ns0:v>143109459.9740406</ns0:v>
+        <ns0:v>97586047.04022282</ns0:v>
       </ns0:c>
       <ns0:c r="G21" s="1" t="n">
         <ns0:v>4.4</ns0:v>
@@ -1777,7 +1777,7 @@
         <ns0:v>103533417666955.5</ns0:v>
       </ns0:c>
       <ns0:c r="F22" s="1" t="n">
-        <ns0:v>512787069.2773507</ns0:v>
+        <ns0:v>331056466.0305722</ns0:v>
       </ns0:c>
       <ns0:c r="G22" s="1" t="n">
         <ns0:v>4.6</ns0:v>
@@ -1805,7 +1805,7 @@
         <ns0:v>1107737222003781</ns0:v>
       </ns0:c>
       <ns0:c r="F23" s="1" t="n">
-        <ns0:v>1837408781.122872</ns0:v>
+        <ns0:v>1123094817.597001</ns0:v>
       </ns0:c>
       <ns0:c r="G23" s="1" t="n">
         <ns0:v>4.8</ns0:v>
@@ -1833,7 +1833,7 @@
         <ns0:v>4763067294395140</ns0:v>
       </ns0:c>
       <ns0:c r="F24" s="1" t="n">
-        <ns0:v>31602085758.1002</ns0:v>
+        <ns0:v>19316408577.56676</ns0:v>
       </ns0:c>
       <ns0:c r="G24" s="1" t="n">
         <ns0:v>5</ns0:v>
@@ -1861,7 +1861,7 @@
         <ns0:v>2.048031753406153e+16</ns0:v>
       </ns0:c>
       <ns0:c r="F25" s="1" t="n">
-        <ns0:v>135883184314.0537</ns0:v>
+        <ns0:v>83057021208.11101</ns0:v>
       </ns0:c>
       <ns0:c r="G25" s="1" t="n">
         <ns0:v>5.2</ns0:v>
@@ -1889,7 +1889,7 @@
         <ns0:v>8.80616166791431e+16</ns0:v>
       </ns0:c>
       <ns0:c r="F26" s="1" t="n">
-        <ns0:v>584272820492.3739</ns0:v>
+        <ns0:v>357129988437.7153</ns0:v>
       </ns0:c>
       <ns0:c r="G26" s="1" t="n">
         <ns0:v>5.4</ns0:v>
@@ -1917,7 +1917,7 @@
         <ns0:v>3.786488329219983e+17</ns0:v>
       </ns0:c>
       <ns0:c r="F27" s="1" t="n">
-        <ns0:v>2512266182820.144</ns0:v>
+        <ns0:v>1535593581209.092</ns0:v>
       </ns0:c>
       <ns0:c r="G27" s="1" t="n">
         <ns0:v>5.6</ns0:v>
@@ -1945,7 +1945,7 @@
         <ns0:v>1.628120673682214e+18</ns0:v>
       </ns0:c>
       <ns0:c r="F28" s="1" t="n">
-        <ns0:v>10802284740924.51</ns0:v>
+        <ns0:v>6602771324149.988</ns0:v>
       </ns0:c>
       <ns0:c r="G28" s="1" t="n">
         <ns0:v>5.8</ns0:v>
@@ -1973,7 +1973,7 @@
         <ns0:v>7.000620885625409e+18</ns0:v>
       </ns0:c>
       <ns0:c r="F29" s="1" t="n">
-        <ns0:v>46447847135776.41</ns0:v>
+        <ns0:v>28390708122581.77</ns0:v>
       </ns0:c>
       <ns0:c r="G29" s="1" t="n">
         <ns0:v>6</ns0:v>
@@ -2001,7 +2001,7 @@
         <ns0:v>3.010138841454234e+19</ns0:v>
       </ns0:c>
       <ns0:c r="F30" s="1" t="n">
-        <ns0:v>199717240869898.8</ns0:v>
+        <ns0:v>122074848291886.8</ns0:v>
       </ns0:c>
       <ns0:c r="G30" s="1" t="n">
         <ns0:v>6.2</ns0:v>
@@ -2029,7 +2029,7 @@
         <ns0:v>1.294304604243966e+20</ns0:v>
       </ns0:c>
       <ns0:c r="F31" s="1" t="n">
-        <ns0:v>858747579496795.6</ns0:v>
+        <ns0:v>524899503074881.8</ns0:v>
       </ns0:c>
       <ns0:c r="G31" s="1" t="n">
         <ns0:v>6.4</ns0:v>
@@ -2057,7 +2057,7 @@
         <ns0:v>5.565272888734292e+20</ns0:v>
       </ns0:c>
       <ns0:c r="F32" s="1" t="n">
-        <ns0:v>3692457406679269</ns0:v>
+        <ns0:v>2256971785616948</ns0:v>
       </ns0:c>
       <ns0:c r="G32" s="1" t="n">
         <ns0:v>6.6</ns0:v>
@@ -2085,7 +2085,7 @@
         <ns0:v>2.39296547540079e+21</ns0:v>
       </ns0:c>
       <ns0:c r="F33" s="1" t="n">
-        <ns0:v>1.587689098131714e+16</ns0:v>
+        <ns0:v>9704565562037236</ns0:v>
       </ns0:c>
       <ns0:c r="G33" s="1" t="n">
         <ns0:v>6.8</ns0:v>
@@ -2113,7 +2113,7 @@
         <ns0:v>1.028931353582277e+22</ns0:v>
       </ns0:c>
       <ns0:c r="F34" s="1" t="n">
-        <ns0:v>1.587689098131714e+16</ns0:v>
+        <ns0:v>9704565562037236</ns0:v>
       </ns0:c>
       <ns0:c r="G34" s="1" t="n">
         <ns0:v>7</ns0:v>
@@ -2141,7 +2141,7 @@
         <ns0:v>4.424216484808832e+22</ns0:v>
       </ns0:c>
       <ns0:c r="F35" s="1" t="n">
-        <ns0:v>1.587689098131714e+16</ns0:v>
+        <ns0:v>9704565562037236</ns0:v>
       </ns0:c>
       <ns0:c r="G35" s="1" t="n">
         <ns0:v>7.2</ns0:v>
@@ -2169,7 +2169,7 @@
         <ns0:v>8.179679859850836e+23</ns0:v>
       </ns0:c>
       <ns0:c r="F36" s="1" t="n">
-        <ns0:v>3.292232113885921e+16</ns0:v>
+        <ns0:v>2.012338714944041e+16</ns0:v>
       </ns0:c>
       <ns0:c r="G36" s="1" t="n">
         <ns0:v>7.4</ns0:v>
@@ -2197,7 +2197,7 @@
         <ns0:v>1.512294048887176e+25</ns0:v>
       </ns0:c>
       <ns0:c r="F37" s="1" t="n">
-        <ns0:v>3.292232113885921e+16</ns0:v>
+        <ns0:v>2.012338714944041e+16</ns0:v>
       </ns0:c>
       <ns0:c r="G37" s="1" t="n">
         <ns0:v>7.6</ns0:v>
@@ -2225,7 +2225,7 @@
         <ns0:v>5.797772421440058e+26</ns0:v>
       </ns0:c>
       <ns0:c r="F38" s="1" t="n">
-        <ns0:v>9.830552416349534e+16</ns0:v>
+        <ns0:v>6.008811205403466e+16</ns0:v>
       </ns0:c>
       <ns0:c r="G38" s="1" t="n">
         <ns0:v>7.8</ns0:v>
@@ -2253,7 +2253,7 @@
         <ns0:v>1.731205568606127e+27</ns0:v>
       </ns0:c>
       <ns0:c r="F39" s="1" t="n">
-        <ns0:v>2.038463349054239e+17</ns0:v>
+        <ns0:v>1.245987091552463e+17</ns0:v>
       </ns0:c>
       <ns0:c r="G39" s="1" t="n">
         <ns0:v>8</ns0:v>
@@ -2281,7 +2281,7 @@
         <ns0:v>5.169352128568795e+27</ns0:v>
       </ns0:c>
       <ns0:c r="F40" s="1" t="n">
-        <ns0:v>4.226957600598869e+17</ns0:v>
+        <ns0:v>2.583678833043186e+17</ns0:v>
       </ns0:c>
       <ns0:c r="G40" s="1" t="n">
         <ns0:v>8.199999999999999</ns0:v>
@@ -2309,7 +2309,7 @@
         <ns0:v>1.543560274627236e+28</ns0:v>
       </ns0:c>
       <ns0:c r="F41" s="1" t="n">
-        <ns0:v>8.765019280601815e+17</ns0:v>
+        <ns0:v>5.357516428198349e+17</ns0:v>
       </ns0:c>
       <ns0:c r="G41" s="1" t="n">
         <ns0:v>8.4</ns0:v>
@@ -2337,7 +2337,7 @@
         <ns0:v>1.376253845651405e+29</ns0:v>
       </ns0:c>
       <ns0:c r="F42" s="1" t="n">
-        <ns0:v>3.768797855745867e+18</ns0:v>
+        <ns0:v>2.303634000144588e+18</ns0:v>
       </ns0:c>
       <ns0:c r="G42" s="1" t="n">
         <ns0:v>8.6</ns0:v>
@@ -2365,7 +2365,7 @@
         <ns0:v>5.276226932910335e+30</ns0:v>
       </ns0:c>
       <ns0:c r="F43" s="1" t="n">
-        <ns0:v>3.360298025100196e+19</ns0:v>
+        <ns0:v>2.053943214130691e+19</ns0:v>
       </ns0:c>
       <ns0:c r="G43" s="1" t="n">
         <ns0:v>8.800000000000001</ns0:v>
@@ -2393,7 +2393,7 @@
         <ns0:v>1.575472920203933e+31</ns0:v>
       </ns0:c>
       <ns0:c r="F44" s="1" t="n">
-        <ns0:v>6.967913984847766e+19</ns0:v>
+        <ns0:v>4.259056648821401e+19</ns0:v>
       </ns0:c>
       <ns0:c r="G44" s="1" t="n">
         <ns0:v>9</ns0:v>
@@ -2421,7 +2421,7 @@
         <ns0:v>4.704336932162219e+31</ns0:v>
       </ns0:c>
       <ns0:c r="F45" s="1" t="n">
-        <ns0:v>1.444866643898032e+20</ns0:v>
+        <ns0:v>8.831579866996054e+19</ns0:v>
       </ns0:c>
       <ns0:c r="G45" s="1" t="n">
         <ns0:v>9.199999999999999</ns0:v>
@@ -2449,7 +2449,7 @@
         <ns0:v>1.404707481004547e+32</ns0:v>
       </ns0:c>
       <ns0:c r="F46" s="1" t="n">
-        <ns0:v>2.99607547278696e+20</ns0:v>
+        <ns0:v>1.831316401220302e+20</ns0:v>
       </ns0:c>
       <ns0:c r="G46" s="1" t="n">
         <ns0:v>9.4</ns0:v>
@@ -2477,7 +2477,7 @@
         <ns0:v>1.252451300105319e+33</ns0:v>
       </ns0:c>
       <ns0:c r="F47" s="1" t="n">
-        <ns0:v>1.288257613132938e+21</ns0:v>
+        <ns0:v>7.874325321093216e+20</ns0:v>
       </ns0:c>
       <ns0:c r="G47" s="1" t="n">
         <ns0:v>9.6</ns0:v>
@@ -2505,7 +2505,7 @@
         <ns0:v>4.801597686832596e+34</ns0:v>
       </ns0:c>
       <ns0:c r="F48" s="1" t="n">
-        <ns0:v>1.148623428192379e+22</ns0:v>
+        <ns0:v>7.020827552511277e+21</ns0:v>
       </ns0:c>
       <ns0:c r="G48" s="1" t="n">
         <ns0:v>9.800000000000001</ns0:v>
@@ -2533,7 +2533,7 @@
         <ns0:v>1.433749386731914e+35</ns0:v>
       </ns0:c>
       <ns0:c r="F49" s="1" t="n">
-        <ns0:v>2.381785540699717e+22</ns0:v>
+        <ns0:v>1.455838801288738e+22</ns0:v>
       </ns0:c>
       <ns0:c r="G49" s="1" t="n">
         <ns0:v>10</ns0:v>
@@ -2561,7 +2561,7 @@
         <ns0:v>4.281152728791306e+35</ns0:v>
       </ns0:c>
       <ns0:c r="F50" s="1" t="n">
-        <ns0:v>4.938870497194933e+22</ns0:v>
+        <ns0:v>3.018827338352327e+22</ns0:v>
       </ns0:c>
       <ns0:c r="G50" s="1" t="n">
         <ns0:v>10.2</ns0:v>
@@ -2589,7 +2589,7 @@
         <ns0:v>1.278345354972718e+36</ns0:v>
       </ns0:c>
       <ns0:c r="F51" s="1" t="n">
-        <ns0:v>1.024124186298341e+23</ns0:v>
+        <ns0:v>6.259840368807384e+22</ns0:v>
       </ns0:c>
       <ns0:c r="G51" s="1" t="n">
         <ns0:v>10.4</ns0:v>
@@ -2617,7 +2617,7 @@
         <ns0:v>1.139785559249822e+37</ns0:v>
       </ns0:c>
       <ns0:c r="F52" s="1" t="n">
-        <ns0:v>4.403546545391806e+23</ns0:v>
+        <ns0:v>2.691616778469064e+23</ns0:v>
       </ns0:c>
       <ns0:c r="G52" s="1" t="n">
         <ns0:v>10.6</ns0:v>
@@ -2645,7 +2645,7 @@
         <ns0:v>4.369664277021335e+38</ns0:v>
       </ns0:c>
       <ns0:c r="F53" s="1" t="n">
-        <ns0:v>3.926246332728402e+24</ns0:v>
+        <ns0:v>2.399872556504138e+24</ns0:v>
       </ns0:c>
       <ns0:c r="G53" s="1" t="n">
         <ns0:v>10.8</ns0:v>
@@ -2673,7 +2673,7 @@
         <ns0:v>1.304774761655727e+39</ns0:v>
       </ns0:c>
       <ns0:c r="F54" s="1" t="n">
-        <ns0:v>8.141464395545614e+24</ns0:v>
+        <ns0:v>4.976375733166981e+24</ns0:v>
       </ns0:c>
       <ns0:c r="G54" s="1" t="n">
         <ns0:v>11</ns0:v>
@@ -2701,7 +2701,7 @@
         <ns0:v>3.896036561907814e+39</ns0:v>
       </ns0:c>
       <ns0:c r="F55" s="1" t="n">
-        <ns0:v>1.688214057060338e+25</ns0:v>
+        <ns0:v>1.031901272029505e+25</ns0:v>
       </ns0:c>
       <ns0:c r="G55" s="1" t="n">
         <ns0:v>11.2</ns0:v>
@@ -2729,7 +2729,7 @@
         <ns0:v>1.163350283727174e+40</ns0:v>
       </ns0:c>
       <ns0:c r="F56" s="1" t="n">
-        <ns0:v>3.500680668720316e+25</ns0:v>
+        <ns0:v>2.139750477680381e+25</ns0:v>
       </ns0:c>
       <ns0:c r="G56" s="1" t="n">
         <ns0:v>11.4</ns0:v>
@@ -2757,7 +2757,7 @@
         <ns0:v>1.03725479862186e+41</ns0:v>
       </ns0:c>
       <ns0:c r="F57" s="1" t="n">
-        <ns0:v>1.505228611090775e+26</ns0:v>
+        <ns0:v>9.200535394098201e+25</ns0:v>
       </ns0:c>
       <ns0:c r="G57" s="1" t="n">
         <ns0:v>11.6</ns0:v>
@@ -2785,7 +2785,7 @@
         <ns0:v>3.976585948930645e+42</ns0:v>
       </ns0:c>
       <ns0:c r="F58" s="1" t="n">
-        <ns0:v>1.342076949407421e+27</ns0:v>
+        <ns0:v>8.203289775151412e+26</ns0:v>
       </ns0:c>
       <ns0:c r="G58" s="1" t="n">
         <ns0:v>11.8</ns0:v>
@@ -2813,7 +2813,7 @@
         <ns0:v>1.187402201813172e+43</ns0:v>
       </ns0:c>
       <ns0:c r="F59" s="1" t="n">
-        <ns0:v>2.782930762291229e+27</ns0:v>
+        <ns0:v>1.701034167775397e+27</ns0:v>
       </ns0:c>
       <ns0:c r="G59" s="1" t="n">
         <ns0:v>12</ns0:v>
@@ -2841,7 +2841,7 @@
         <ns0:v>3.545563976178901e+43</ns0:v>
       </ns0:c>
       <ns0:c r="F60" s="1" t="n">
-        <ns0:v>5.77068522868709e+27</ns0:v>
+        <ns0:v>3.527264450299061e+27</ns0:v>
       </ns0:c>
       <ns0:c r="G60" s="1" t="n">
         <ns0:v>12.2</ns0:v>
@@ -2869,7 +2869,7 @@
         <ns0:v>1.058699730384658e+44</ns0:v>
       </ns0:c>
       <ns0:c r="F61" s="1" t="n">
-        <ns0:v>1.196609289020555e+28</ns0:v>
+        <ns0:v>7.314135564140134e+27</ns0:v>
       </ns0:c>
       <ns0:c r="G61" s="1" t="n">
         <ns0:v>12.4</ns0:v>
@@ -2897,7 +2897,7 @@
         <ns0:v>9.43947314065115e+44</ns0:v>
       </ns0:c>
       <ns0:c r="F62" s="1" t="n">
-        <ns0:v>5.145200915424123e+28</ns0:v>
+        <ns0:v>3.14494441464289e+28</ns0:v>
       </ns0:c>
       <ns0:c r="G62" s="1" t="n">
         <ns0:v>12.6</ns0:v>
@@ -2925,7 +2925,7 @@
         <ns0:v>3.618867447641087e+46</ns0:v>
       </ns0:c>
       <ns0:c r="F63" s="1" t="n">
-        <ns0:v>4.587512818838018e+29</ns0:v>
+        <ns0:v>2.804064030513767e+29</ns0:v>
       </ns0:c>
       <ns0:c r="G63" s="1" t="n">
         <ns0:v>12.8</ns0:v>
@@ -2956,7 +2956,7 @@
       </ns0:c>
       <ns0:c r="F64" s="1">
         <ns0:f>ROUND(F63*1.4,-5)</ns0:f>
-        <ns0:v>6.422517946373224e+29</ns0:v>
+        <ns0:v>3.925689642719273e+29</ns0:v>
       </ns0:c>
       <ns0:c r="G64" s="1" t="n">
         <ns0:v>13</ns0:v>
@@ -2987,7 +2987,7 @@
       </ns0:c>
       <ns0:c r="F65" s="1">
         <ns0:f>ROUND(F64*1.4,-5)</ns0:f>
-        <ns0:v>8.991525124922513e+29</ns0:v>
+        <ns0:v>5.495965499806982e+29</ns0:v>
       </ns0:c>
       <ns0:c r="G65" s="1" t="n">
         <ns0:v>13.2</ns0:v>
@@ -3018,7 +3018,7 @@
       </ns0:c>
       <ns0:c r="F66" s="1">
         <ns0:f>ROUND(F65*1.4,-5)</ns0:f>
-        <ns0:v>1.2588135174891517e+30</ns0:v>
+        <ns0:v>7.694351699729775e+29</ns0:v>
       </ns0:c>
       <ns0:c r="G66" s="1" t="n">
         <ns0:v>13.4</ns0:v>
@@ -3049,7 +3049,7 @@
       </ns0:c>
       <ns0:c r="F67" s="1">
         <ns0:f>ROUND(F66*1.4,-5)</ns0:f>
-        <ns0:v>1.7623389244848124e+30</ns0:v>
+        <ns0:v>1.0772092379621684e+30</ns0:v>
       </ns0:c>
       <ns0:c r="G67" s="1" t="n">
         <ns0:v>13.6</ns0:v>
@@ -3080,7 +3080,7 @@
       </ns0:c>
       <ns0:c r="F68" s="1">
         <ns0:f>ROUND(F67*1.4,-5)</ns0:f>
-        <ns0:v>2.4672744942787372e+30</ns0:v>
+        <ns0:v>1.5080929331470357e+30</ns0:v>
       </ns0:c>
       <ns0:c r="G68" s="1" t="n">
         <ns0:v>13.8</ns0:v>
@@ -3111,7 +3111,7 @@
       </ns0:c>
       <ns0:c r="F69" s="1">
         <ns0:f>ROUND(F68*1.4,-5)</ns0:f>
-        <ns0:v>3.454184291990232e+30</ns0:v>
+        <ns0:v>2.11133010640585e+30</ns0:v>
       </ns0:c>
       <ns0:c r="G69" s="1" t="n">
         <ns0:v>14</ns0:v>
@@ -3142,7 +3142,7 @@
       </ns0:c>
       <ns0:c r="F70" s="1">
         <ns0:f>ROUND(F69*1.4,-5)</ns0:f>
-        <ns0:v>4.835858008786324e+30</ns0:v>
+        <ns0:v>2.95586214896819e+30</ns0:v>
       </ns0:c>
       <ns0:c r="G70" s="1" t="n">
         <ns0:v>14.2</ns0:v>
@@ -3173,7 +3173,7 @@
       </ns0:c>
       <ns0:c r="F71" s="1">
         <ns0:f>ROUND(F70*1.4,-5)</ns0:f>
-        <ns0:v>6.770201212300853e+30</ns0:v>
+        <ns0:v>4.138207008555466e+30</ns0:v>
       </ns0:c>
       <ns0:c r="G71" s="1" t="n">
         <ns0:v>14.4</ns0:v>
@@ -3204,7 +3204,7 @@
       </ns0:c>
       <ns0:c r="F72" s="1">
         <ns0:f>ROUND(F71*1.4,-5)</ns0:f>
-        <ns0:v>9.478281697221195e+30</ns0:v>
+        <ns0:v>5.793489811977652e+30</ns0:v>
       </ns0:c>
       <ns0:c r="G72" s="1" t="n">
         <ns0:v>14.6</ns0:v>
@@ -3235,7 +3235,7 @@
       </ns0:c>
       <ns0:c r="F73" s="1">
         <ns0:f>ROUND(F72*1.4,-5)</ns0:f>
-        <ns0:v>1.3269594376109672e+31</ns0:v>
+        <ns0:v>8.110885736768713e+30</ns0:v>
       </ns0:c>
       <ns0:c r="G73" s="1" t="n">
         <ns0:v>14.8</ns0:v>
@@ -3266,7 +3266,7 @@
       </ns0:c>
       <ns0:c r="F74" s="1">
         <ns0:f>ROUND(F73*1.4,-5)</ns0:f>
-        <ns0:v>1.8577432126553538e+31</ns0:v>
+        <ns0:v>1.1355240031476196e+31</ns0:v>
       </ns0:c>
       <ns0:c r="G74" s="1" t="n">
         <ns0:v>15</ns0:v>
@@ -3298,7 +3298,7 @@
       </ns0:c>
       <ns0:c r="F75" s="1">
         <ns0:f>ROUND(F74*1.4,-5)</ns0:f>
-        <ns0:v>2.600840497717495e+31</ns0:v>
+        <ns0:v>1.5897336044066675e+31</ns0:v>
       </ns0:c>
       <ns0:c r="G75" s="1" t="n">
         <ns0:v>15.2</ns0:v>
@@ -3330,7 +3330,7 @@
       </ns0:c>
       <ns0:c r="F76" s="1">
         <ns0:f>ROUND(F75*1.4,-5)</ns0:f>
-        <ns0:v>3.6411766968044923e+31</ns0:v>
+        <ns0:v>2.2256270461693345e+31</ns0:v>
       </ns0:c>
       <ns0:c r="G76" s="1" t="n">
         <ns0:v>15.4</ns0:v>
@@ -3362,7 +3362,7 @@
       </ns0:c>
       <ns0:c r="F77" s="1">
         <ns0:f>ROUND(F76*1.4,-5)</ns0:f>
-        <ns0:v>5.097647375526289e+31</ns0:v>
+        <ns0:v>3.1158778646370687e+31</ns0:v>
       </ns0:c>
       <ns0:c r="G77" s="1" t="n">
         <ns0:v>15.6</ns0:v>
@@ -3394,7 +3394,7 @@
       </ns0:c>
       <ns0:c r="F78" s="1">
         <ns0:f>ROUND(F77*1.4,-5)</ns0:f>
-        <ns0:v>7.136706325736805e+31</ns0:v>
+        <ns0:v>4.3622290104918955e+31</ns0:v>
       </ns0:c>
       <ns0:c r="G78" s="1" t="n">
         <ns0:v>15.8</ns0:v>
@@ -3426,7 +3426,7 @@
       </ns0:c>
       <ns0:c r="F79" s="1">
         <ns0:f>ROUND(F78*1.4,-5)</ns0:f>
-        <ns0:v>9.991388856031526e+31</ns0:v>
+        <ns0:v>6.107120614688653e+31</ns0:v>
       </ns0:c>
       <ns0:c r="G79" s="1" t="n">
         <ns0:v>16</ns0:v>
@@ -3458,7 +3458,7 @@
       </ns0:c>
       <ns0:c r="F80" s="1">
         <ns0:f>ROUND(F79*1.4,-5)</ns0:f>
-        <ns0:v>1.3987944398444136e+32</ns0:v>
+        <ns0:v>8.549968860564114e+31</ns0:v>
       </ns0:c>
       <ns0:c r="G80" s="1" t="n">
         <ns0:v>16.2</ns0:v>
@@ -3490,7 +3490,7 @@
       </ns0:c>
       <ns0:c r="F81" s="1">
         <ns0:f>ROUND(F80*1.4,-5)</ns0:f>
-        <ns0:v>1.958312215782179e+32</ns0:v>
+        <ns0:v>1.1969956404789758e+32</ns0:v>
       </ns0:c>
       <ns0:c r="G81" s="1" t="n">
         <ns0:v>16.4</ns0:v>
@@ -3522,7 +3522,7 @@
       </ns0:c>
       <ns0:c r="F82" s="1">
         <ns0:f>ROUND(F81*1.4,-5)</ns0:f>
-        <ns0:v>2.74163710209505e+32</ns0:v>
+        <ns0:v>1.675793896670566e+32</ns0:v>
       </ns0:c>
       <ns0:c r="G82" s="1" t="n">
         <ns0:v>16.6</ns0:v>
@@ -3554,7 +3554,7 @@
       </ns0:c>
       <ns0:c r="F83" s="1">
         <ns0:f>ROUND(F82*1.4,-5)</ns0:f>
-        <ns0:v>3.83829194293307e+32</ns0:v>
+        <ns0:v>2.346111455338792e+32</ns0:v>
       </ns0:c>
       <ns0:c r="G83" s="1" t="n">
         <ns0:v>16.8</ns0:v>
@@ -3586,7 +3586,7 @@
       </ns0:c>
       <ns0:c r="F84" s="1">
         <ns0:f>ROUND(F83*1.4,-5)</ns0:f>
-        <ns0:v>5.373608720106297e+32</ns0:v>
+        <ns0:v>3.284556037474309e+32</ns0:v>
       </ns0:c>
       <ns0:c r="G84" s="1" t="n">
         <ns0:v>17</ns0:v>
@@ -3618,7 +3618,7 @@
       </ns0:c>
       <ns0:c r="F85" s="1">
         <ns0:f>ROUND(F84*1.4,-5)</ns0:f>
-        <ns0:v>7.523052208148816e+32</ns0:v>
+        <ns0:v>4.5983784524640325e+32</ns0:v>
       </ns0:c>
       <ns0:c r="G85" s="1" t="n">
         <ns0:v>17.2</ns0:v>
@@ -3650,7 +3650,7 @@
       </ns0:c>
       <ns0:c r="F86" s="1">
         <ns0:f>ROUND(F85*1.4,-5)</ns0:f>
-        <ns0:v>1.0532273091408342e+33</ns0:v>
+        <ns0:v>6.437729833449646e+32</ns0:v>
       </ns0:c>
       <ns0:c r="G86" s="1" t="n">
         <ns0:v>17.4</ns0:v>
@@ -3682,7 +3682,7 @@
       </ns0:c>
       <ns0:c r="F87" s="1">
         <ns0:f>ROUND(F86*1.4,-5)</ns0:f>
-        <ns0:v>1.4745182327971676e+33</ns0:v>
+        <ns0:v>9.012821766829504e+32</ns0:v>
       </ns0:c>
       <ns0:c r="G87" s="1" t="n">
         <ns0:v>17.6</ns0:v>
@@ -3714,7 +3714,7 @@
       </ns0:c>
       <ns0:c r="F88" s="1">
         <ns0:f>ROUND(F87*1.4,-5)</ns0:f>
-        <ns0:v>2.0643255259160346e+33</ns0:v>
+        <ns0:v>1.2617950473561304e+33</ns0:v>
       </ns0:c>
       <ns0:c r="G88" s="1" t="n">
         <ns0:v>17.8</ns0:v>
@@ -3746,7 +3746,7 @@
       </ns0:c>
       <ns0:c r="F89" s="1">
         <ns0:f>ROUND(F88*1.4,-5)</ns0:f>
-        <ns0:v>2.890055736282448e+33</ns0:v>
+        <ns0:v>1.7665130662985825e+33</ns0:v>
       </ns0:c>
       <ns0:c r="G89" s="1" t="n">
         <ns0:v>18</ns0:v>
@@ -3778,7 +3778,7 @@
       </ns0:c>
       <ns0:c r="F90" s="1">
         <ns0:f>ROUND(F89*1.4,-5)</ns0:f>
-        <ns0:v>4.046078030795427e+33</ns0:v>
+        <ns0:v>2.4731182928180153e+33</ns0:v>
       </ns0:c>
       <ns0:c r="G90" s="1" t="n">
         <ns0:v>18.2</ns0:v>
@@ -3810,7 +3810,7 @@
       </ns0:c>
       <ns0:c r="F91" s="1">
         <ns0:f>ROUND(F90*1.4,-5)</ns0:f>
-        <ns0:v>5.664509243113597e+33</ns0:v>
+        <ns0:v>3.462365609945221e+33</ns0:v>
       </ns0:c>
       <ns0:c r="G91" s="1" t="n">
         <ns0:v>18.4</ns0:v>
@@ -3842,7 +3842,7 @@
       </ns0:c>
       <ns0:c r="F92" s="1">
         <ns0:f>ROUND(F91*1.4,-5)</ns0:f>
-        <ns0:v>7.930312940359036e+33</ns0:v>
+        <ns0:v>4.8473118539233087e+33</ns0:v>
       </ns0:c>
       <ns0:c r="G92" s="1" t="n">
         <ns0:v>18.6</ns0:v>
@@ -3874,7 +3874,7 @@
       </ns0:c>
       <ns0:c r="F93" s="1">
         <ns0:f>ROUND(F92*1.4,-5)</ns0:f>
-        <ns0:v>1.110243811650265e+34</ns0:v>
+        <ns0:v>6.786236595492632e+33</ns0:v>
       </ns0:c>
       <ns0:c r="G93" s="1" t="n">
         <ns0:v>18.8</ns0:v>
@@ -3906,7 +3906,7 @@
       </ns0:c>
       <ns0:c r="F94" s="1">
         <ns0:f>ROUND(F93*1.4,-5)</ns0:f>
-        <ns0:v>1.554341336310371e+34</ns0:v>
+        <ns0:v>9.500731233689683e+33</ns0:v>
       </ns0:c>
       <ns0:c r="G94" s="1" t="n">
         <ns0:v>19</ns0:v>
@@ -3938,7 +3938,7 @@
       </ns0:c>
       <ns0:c r="F95" s="1">
         <ns0:f>ROUND(F94*1.4,-5)</ns0:f>
-        <ns0:v>2.176077870834519e+34</ns0:v>
+        <ns0:v>1.3301023727165556e+34</ns0:v>
       </ns0:c>
       <ns0:c r="G95" s="1" t="n">
         <ns0:v>19.2</ns0:v>
@@ -3970,7 +3970,7 @@
       </ns0:c>
       <ns0:c r="F96" s="1">
         <ns0:f>ROUND(F95*1.4,-5)</ns0:f>
-        <ns0:v>3.0465090191683266e+34</ns0:v>
+        <ns0:v>1.8621433218031776e+34</ns0:v>
       </ns0:c>
       <ns0:c r="G96" s="1" t="n">
         <ns0:v>19.4</ns0:v>
@@ -4002,7 +4002,7 @@
       </ns0:c>
       <ns0:c r="F97" s="1">
         <ns0:f>ROUND(F96*1.4,-5)</ns0:f>
-        <ns0:v>4.265112626835657e+34</ns0:v>
+        <ns0:v>2.6070006505244486e+34</ns0:v>
       </ns0:c>
       <ns0:c r="G97" s="1" t="n">
         <ns0:v>19.6</ns0:v>
@@ -4034,7 +4034,7 @@
       </ns0:c>
       <ns0:c r="F98" s="1">
         <ns0:f>ROUND(F97*1.4,-5)</ns0:f>
-        <ns0:v>5.97115767756992e+34</ns0:v>
+        <ns0:v>3.6498009107342274e+34</ns0:v>
       </ns0:c>
       <ns0:c r="G98" s="1" t="n">
         <ns0:v>19.8</ns0:v>
@@ -4066,7 +4066,7 @@
       </ns0:c>
       <ns0:c r="F99" s="1">
         <ns0:f>ROUND(F98*1.4,-5)</ns0:f>
-        <ns0:v>8.359620748597887e+34</ns0:v>
+        <ns0:v>5.109721275027918e+34</ns0:v>
       </ns0:c>
       <ns0:c r="G99" s="1" t="n">
         <ns0:v>20</ns0:v>
@@ -4098,7 +4098,7 @@
       </ns0:c>
       <ns0:c r="F100" s="1">
         <ns0:f>ROUND(F99*1.4,-5)</ns0:f>
-        <ns0:v>1.170346904803704e+35</ns0:v>
+        <ns0:v>7.153609785039085e+34</ns0:v>
       </ns0:c>
       <ns0:c r="G100" s="1" t="n">
         <ns0:v>20.2</ns0:v>
@@ -4130,7 +4130,7 @@
       </ns0:c>
       <ns0:c r="F101" s="1">
         <ns0:f>ROUND(F100*1.4,-5)</ns0:f>
-        <ns0:v>1.6384856667251856e+35</ns0:v>
+        <ns0:v>1.0015053699054717e+35</ns0:v>
       </ns0:c>
       <ns0:c r="G101" s="1" t="n">
         <ns0:v>20.4</ns0:v>
@@ -4162,7 +4162,7 @@
       </ns0:c>
       <ns0:c r="F102" s="1">
         <ns0:f>ROUND(F101*1.4,-5)</ns0:f>
-        <ns0:v>2.2938799334152597e+35</ns0:v>
+        <ns0:v>1.4021075178676604e+35</ns0:v>
       </ns0:c>
       <ns0:c r="G102" s="1" t="n">
         <ns0:v>20.6</ns0:v>
@@ -4194,7 +4194,7 @@
       </ns0:c>
       <ns0:c r="F103" s="1">
         <ns0:f>ROUND(F102*1.4,-5)</ns0:f>
-        <ns0:v>3.2114319067813633e+35</ns0:v>
+        <ns0:v>1.9629505250147243e+35</ns0:v>
       </ns0:c>
       <ns0:c r="G103" s="1" t="n">
         <ns0:v>20.8</ns0:v>
@@ -4226,7 +4226,7 @@
       </ns0:c>
       <ns0:c r="F104" s="1">
         <ns0:f>ROUND(F103*1.4,-5)</ns0:f>
-        <ns0:v>4.4960046694939086e+35</ns0:v>
+        <ns0:v>2.7481307350206138e+35</ns0:v>
       </ns0:c>
       <ns0:c r="G104" s="1" t="n">
         <ns0:v>21</ns0:v>
@@ -4258,7 +4258,7 @@
       </ns0:c>
       <ns0:c r="F105" s="1">
         <ns0:f>ROUND(F104*1.4,-5)</ns0:f>
-        <ns0:v>6.294406537291471e+35</ns0:v>
+        <ns0:v>3.847383029028859e+35</ns0:v>
       </ns0:c>
       <ns0:c r="G105" s="1" t="n">
         <ns0:v>21.2</ns0:v>
@@ -4290,7 +4290,7 @@
       </ns0:c>
       <ns0:c r="F106" s="1">
         <ns0:f>ROUND(F105*1.4,-5)</ns0:f>
-        <ns0:v>8.812169152208059e+35</ns0:v>
+        <ns0:v>5.386336240640402e+35</ns0:v>
       </ns0:c>
       <ns0:c r="G106" s="1" t="n">
         <ns0:v>21.4</ns0:v>
@@ -4322,7 +4322,7 @@
       </ns0:c>
       <ns0:c r="F107" s="1">
         <ns0:f>ROUND(F106*1.4,-5)</ns0:f>
-        <ns0:v>1.2337036813091281e+36</ns0:v>
+        <ns0:v>7.540870736896562e+35</ns0:v>
       </ns0:c>
       <ns0:c r="G107" s="1" t="n">
         <ns0:v>21.6</ns0:v>
@@ -4354,7 +4354,7 @@
       </ns0:c>
       <ns0:c r="F108" s="1">
         <ns0:f>ROUND(F107*1.4,-5)</ns0:f>
-        <ns0:v>1.7271851538327794e+36</ns0:v>
+        <ns0:v>1.0557219031655186e+36</ns0:v>
       </ns0:c>
       <ns0:c r="G108" s="1" t="n">
         <ns0:v>21.8</ns0:v>
@@ -4386,7 +4386,7 @@
       </ns0:c>
       <ns0:c r="F109" s="1">
         <ns0:f>ROUND(F108*1.4,-5)</ns0:f>
-        <ns0:v>2.418059215365891e+36</ns0:v>
+        <ns0:v>1.478010664431726e+36</ns0:v>
       </ns0:c>
       <ns0:c r="G109" s="1" t="n">
         <ns0:v>22</ns0:v>
@@ -4418,7 +4418,7 @@
       </ns0:c>
       <ns0:c r="F110" s="1">
         <ns0:f>ROUND(F109*1.4,-5)</ns0:f>
-        <ns0:v>3.385282901512247e+36</ns0:v>
+        <ns0:v>2.0692149302044165e+36</ns0:v>
       </ns0:c>
       <ns0:c r="G110" s="1" t="n">
         <ns0:v>22.2</ns0:v>
@@ -4450,7 +4450,7 @@
       </ns0:c>
       <ns0:c r="F111" s="1">
         <ns0:f>ROUND(F110*1.4,-5)</ns0:f>
-        <ns0:v>4.7393960621171457e+36</ns0:v>
+        <ns0:v>2.896900902286183e+36</ns0:v>
       </ns0:c>
       <ns0:c r="G111" s="1" t="n">
         <ns0:v>22.4</ns0:v>
@@ -4482,7 +4482,7 @@
       </ns0:c>
       <ns0:c r="F112" s="1">
         <ns0:f>ROUND(F111*1.4,-5)</ns0:f>
-        <ns0:v>6.635154486964003e+36</ns0:v>
+        <ns0:v>4.055661263200656e+36</ns0:v>
       </ns0:c>
       <ns0:c r="G112" s="1" t="n">
         <ns0:v>22.6</ns0:v>
@@ -4514,7 +4514,7 @@
       </ns0:c>
       <ns0:c r="F113" s="1">
         <ns0:f>ROUND(F112*1.4,-5)</ns0:f>
-        <ns0:v>9.289216281749605e+36</ns0:v>
+        <ns0:v>5.677925768480918e+36</ns0:v>
       </ns0:c>
       <ns0:c r="G113" s="1" t="n">
         <ns0:v>22.8</ns0:v>
@@ -4546,7 +4546,7 @@
       </ns0:c>
       <ns0:c r="F114" s="1">
         <ns0:f>ROUND(F113*1.4,-5)</ns0:f>
-        <ns0:v>1.3004902794449445e+37</ns0:v>
+        <ns0:v>7.949096075873285e+36</ns0:v>
       </ns0:c>
       <ns0:c r="G114" s="1" t="n">
         <ns0:v>23</ns0:v>
@@ -4578,7 +4578,7 @@
       </ns0:c>
       <ns0:c r="F115" s="1">
         <ns0:f>ROUND(F114*1.4,-5)</ns0:f>
-        <ns0:v>1.8206863912229223e+37</ns0:v>
+        <ns0:v>1.1128734506222598e+37</ns0:v>
       </ns0:c>
       <ns0:c r="G115" s="1" t="n">
         <ns0:v>23.2</ns0:v>
@@ -4610,7 +4610,7 @@
       </ns0:c>
       <ns0:c r="F116" s="1">
         <ns0:f>ROUND(F115*1.4,-5)</ns0:f>
-        <ns0:v>2.5489609477120913e+37</ns0:v>
+        <ns0:v>1.5580228308711636e+37</ns0:v>
       </ns0:c>
       <ns0:c r="G116" s="1" t="n">
         <ns0:v>23.4</ns0:v>
@@ -4642,7 +4642,7 @@
       </ns0:c>
       <ns0:c r="F117" s="1">
         <ns0:f>ROUND(F116*1.4,-5)</ns0:f>
-        <ns0:v>3.5685453267969277e+37</ns0:v>
+        <ns0:v>2.181231963219629e+37</ns0:v>
       </ns0:c>
       <ns0:c r="G117" s="1" t="n">
         <ns0:v>23.6</ns0:v>
@@ -4674,7 +4674,7 @@
       </ns0:c>
       <ns0:c r="F118" s="1">
         <ns0:f>ROUND(F117*1.4,-5)</ns0:f>
-        <ns0:v>4.995963457515698e+37</ns0:v>
+        <ns0:v>3.0537247485074806e+37</ns0:v>
       </ns0:c>
       <ns0:c r="G118" s="1" t="n">
         <ns0:v>23.8</ns0:v>
@@ -4706,7 +4706,7 @@
       </ns0:c>
       <ns0:c r="F119" s="1">
         <ns0:f>ROUND(F118*1.4,-5)</ns0:f>
-        <ns0:v>6.994348840521976e+37</ns0:v>
+        <ns0:v>4.275214647910472e+37</ns0:v>
       </ns0:c>
       <ns0:c r="G119" s="1" t="n">
         <ns0:v>24</ns0:v>
@@ -4738,7 +4738,7 @@
       </ns0:c>
       <ns0:c r="F120" s="1">
         <ns0:f>ROUND(F119*1.4,-5)</ns0:f>
-        <ns0:v>9.792088376730766e+37</ns0:v>
+        <ns0:v>5.9853005070746605e+37</ns0:v>
       </ns0:c>
       <ns0:c r="G120" s="1" t="n">
         <ns0:v>24.2000000000001</ns0:v>
@@ -4770,7 +4770,7 @@
       </ns0:c>
       <ns0:c r="F121" s="1">
         <ns0:f>ROUND(F120*1.4,-5)</ns0:f>
-        <ns0:v>1.3708923727423071e+38</ns0:v>
+        <ns0:v>8.379420709904523e+37</ns0:v>
       </ns0:c>
       <ns0:c r="G121" s="1" t="n">
         <ns0:v>24.4000000000001</ns0:v>
@@ -4802,7 +4802,7 @@
       </ns0:c>
       <ns0:c r="F122" s="1">
         <ns0:f>ROUND(F121*1.4,-5)</ns0:f>
-        <ns0:v>1.91924932183923e+38</ns0:v>
+        <ns0:v>1.1731188993866332e+38</ns0:v>
       </ns0:c>
       <ns0:c r="G122" s="1" t="n">
         <ns0:v>24.6000000000001</ns0:v>
@@ -4834,7 +4834,7 @@
       </ns0:c>
       <ns0:c r="F123" s="1">
         <ns0:f>ROUND(F122*1.4,-5)</ns0:f>
-        <ns0:v>2.6869490505749215e+38</ns0:v>
+        <ns0:v>1.6423664591412864e+38</ns0:v>
       </ns0:c>
       <ns0:c r="G123" s="1" t="n">
         <ns0:v>24.8000000000001</ns0:v>
@@ -4866,7 +4866,7 @@
       </ns0:c>
       <ns0:c r="F124" s="1">
         <ns0:f>ROUND(F123*1.4,-5)</ns0:f>
-        <ns0:v>3.76172867080489e+38</ns0:v>
+        <ns0:v>2.299313042797801e+38</ns0:v>
       </ns0:c>
       <ns0:c r="G124" s="1" t="n">
         <ns0:v>25.0000000000001</ns0:v>
@@ -4898,7 +4898,7 @@
       </ns0:c>
       <ns0:c r="F125" s="1">
         <ns0:f>ROUND(F124*1.4,-5)</ns0:f>
-        <ns0:v>5.266420139126845e+38</ns0:v>
+        <ns0:v>3.2190382599169213e+38</ns0:v>
       </ns0:c>
       <ns0:c r="G125" s="1" t="n">
         <ns0:v>25.2000000000001</ns0:v>
@@ -4930,7 +4930,7 @@
       </ns0:c>
       <ns0:c r="F126" s="1">
         <ns0:f>ROUND(F125*1.4,-5)</ns0:f>
-        <ns0:v>7.372988194777583e+38</ns0:v>
+        <ns0:v>4.50665356388369e+38</ns0:v>
       </ns0:c>
       <ns0:c r="G126" s="1" t="n">
         <ns0:v>25.4000000000001</ns0:v>
@@ -4962,7 +4962,7 @@
       </ns0:c>
       <ns0:c r="F127" s="1">
         <ns0:f>ROUND(F126*1.4,-5)</ns0:f>
-        <ns0:v>1.0322183472688616e+39</ns0:v>
+        <ns0:v>6.309314989437165e+38</ns0:v>
       </ns0:c>
       <ns0:c r="G127" s="1" t="n">
         <ns0:v>25.6000000000001</ns0:v>
@@ -4994,7 +4994,7 @@
       </ns0:c>
       <ns0:c r="F128" s="1">
         <ns0:f>ROUND(F127*1.4,-5)</ns0:f>
-        <ns0:v>1.445105686176406e+39</ns0:v>
+        <ns0:v>8.83304098521203e+38</ns0:v>
       </ns0:c>
       <ns0:c r="G128" s="1" t="n">
         <ns0:v>25.8000000000001</ns0:v>
@@ -5026,7 +5026,7 @@
       </ns0:c>
       <ns0:c r="F129" s="1">
         <ns0:f>ROUND(F128*1.4,-5)</ns0:f>
-        <ns0:v>2.0231479606469683e+39</ns0:v>
+        <ns0:v>1.2366257379296841e+39</ns0:v>
       </ns0:c>
       <ns0:c r="G129" s="1" t="n">
         <ns0:v>26.0000000000001</ns0:v>
@@ -5058,7 +5058,7 @@
       </ns0:c>
       <ns0:c r="F130" s="1">
         <ns0:f>ROUND(F129*1.4,-5)</ns0:f>
-        <ns0:v>2.8324071449057554e+39</ns0:v>
+        <ns0:v>1.7312760331015576e+39</ns0:v>
       </ns0:c>
       <ns0:c r="G130" s="1" t="n">
         <ns0:v>26.2000000000001</ns0:v>
@@ -5090,7 +5090,7 @@
       </ns0:c>
       <ns0:c r="F131" s="1">
         <ns0:f>ROUND(F130*1.4,-5)</ns0:f>
-        <ns0:v>3.9653700028680576e+39</ns0:v>
+        <ns0:v>2.4237864463421808e+39</ns0:v>
       </ns0:c>
       <ns0:c r="G131" s="1" t="n">
         <ns0:v>26.4000000000001</ns0:v>
@@ -5122,7 +5122,7 @@
       </ns0:c>
       <ns0:c r="F132" s="1">
         <ns0:f>ROUND(F131*1.4,-5)</ns0:f>
-        <ns0:v>5.55151800401528e+39</ns0:v>
+        <ns0:v>3.393301024879053e+39</ns0:v>
       </ns0:c>
       <ns0:c r="G132" s="1" t="n">
         <ns0:v>26.6000000000001</ns0:v>
@@ -5154,7 +5154,7 @@
       </ns0:c>
       <ns0:c r="F133" s="1">
         <ns0:f>ROUND(F132*1.4,-5)</ns0:f>
-        <ns0:v>7.772125205621392e+39</ns0:v>
+        <ns0:v>4.750621434830674e+39</ns0:v>
       </ns0:c>
       <ns0:c r="G133" s="1" t="n">
         <ns0:v>26.8000000000001</ns0:v>
@@ -5186,7 +5186,7 @@
       </ns0:c>
       <ns0:c r="F134" s="1">
         <ns0:f>ROUND(F133*1.4,-5)</ns0:f>
-        <ns0:v>1.0880975287869949e+40</ns0:v>
+        <ns0:v>6.650870008762943e+39</ns0:v>
       </ns0:c>
       <ns0:c r="G134" s="1" t="n">
         <ns0:v>27.0000000000001</ns0:v>
@@ -5218,7 +5218,7 @@
       </ns0:c>
       <ns0:c r="F135" s="1">
         <ns0:f>ROUND(F134*1.4,-5)</ns0:f>
-        <ns0:v>1.5233365403017927e+40</ns0:v>
+        <ns0:v>9.31121801226812e+39</ns0:v>
       </ns0:c>
       <ns0:c r="G135" s="1" t="n">
         <ns0:v>27.2000000000001</ns0:v>
@@ -5250,7 +5250,7 @@
       </ns0:c>
       <ns0:c r="F136" s="1">
         <ns0:f>ROUND(F135*1.4,-5)</ns0:f>
-        <ns0:v>2.1326711564225094e+40</ns0:v>
+        <ns0:v>1.3035705217175366e+40</ns0:v>
       </ns0:c>
       <ns0:c r="G136" s="1" t="n">
         <ns0:v>27.4000000000001</ns0:v>
@@ -5282,7 +5282,7 @@
       </ns0:c>
       <ns0:c r="F137" s="1">
         <ns0:f>ROUND(F136*1.4,-5)</ns0:f>
-        <ns0:v>2.985739618991513e+40</ns0:v>
+        <ns0:v>1.824998730404551e+40</ns0:v>
       </ns0:c>
       <ns0:c r="G137" s="1" t="n">
         <ns0:v>27.6000000000001</ns0:v>
@@ -5314,7 +5314,7 @@
       </ns0:c>
       <ns0:c r="F138" s="1">
         <ns0:f>ROUND(F137*1.4,-5)</ns0:f>
-        <ns0:v>4.1800354665881186e+40</ns0:v>
+        <ns0:v>2.5549982225663714e+40</ns0:v>
       </ns0:c>
       <ns0:c r="G138" s="1" t="n">
         <ns0:v>27.8000000000001</ns0:v>
@@ -5346,7 +5346,7 @@
       </ns0:c>
       <ns0:c r="F139" s="1">
         <ns0:f>ROUND(F138*1.4,-5)</ns0:f>
-        <ns0:v>5.852049653223366e+40</ns0:v>
+        <ns0:v>3.57699751159292e+40</ns0:v>
       </ns0:c>
       <ns0:c r="G139" s="1" t="n">
         <ns0:v>28.0000000000001</ns0:v>
@@ -5378,7 +5378,7 @@
       </ns0:c>
       <ns0:c r="F140" s="1">
         <ns0:f>ROUND(F139*1.4,-5)</ns0:f>
-        <ns0:v>8.192869514512712e+40</ns0:v>
+        <ns0:v>5.007796516230087e+40</ns0:v>
       </ns0:c>
       <ns0:c r="G140" s="1" t="n">
         <ns0:v>28.2000000000001</ns0:v>
@@ -5410,7 +5410,7 @@
       </ns0:c>
       <ns0:c r="F141" s="1">
         <ns0:f>ROUND(F140*1.4,-5)</ns0:f>
-        <ns0:v>1.1470017320317795e+41</ns0:v>
+        <ns0:v>7.010915122722121e+40</ns0:v>
       </ns0:c>
       <ns0:c r="G141" s="1" t="n">
         <ns0:v>28.4000000000001</ns0:v>
@@ -5442,7 +5442,7 @@
       </ns0:c>
       <ns0:c r="F142" s="1">
         <ns0:f>ROUND(F141*1.4,-5)</ns0:f>
-        <ns0:v>1.6058024248444911e+41</ns0:v>
+        <ns0:v>9.81528117181097e+40</ns0:v>
       </ns0:c>
       <ns0:c r="G142" s="1" t="n">
         <ns0:v>28.6000000000001</ns0:v>
@@ -5474,7 +5474,7 @@
       </ns0:c>
       <ns0:c r="F143" s="1">
         <ns0:f>ROUND(F142*1.4,-5)</ns0:f>
-        <ns0:v>2.2481233947822873e+41</ns0:v>
+        <ns0:v>1.3741393640535355e+41</ns0:v>
       </ns0:c>
       <ns0:c r="G143" s="1" t="n">
         <ns0:v>28.8000000000001</ns0:v>
@@ -5506,7 +5506,7 @@
       </ns0:c>
       <ns0:c r="F144" s="1">
         <ns0:f>ROUND(F143*1.4,-5)</ns0:f>
-        <ns0:v>3.1473727526952024e+41</ns0:v>
+        <ns0:v>1.9237951096749496e+41</ns0:v>
       </ns0:c>
       <ns0:c r="G144" s="1" t="n">
         <ns0:v>29.0000000000001</ns0:v>
@@ -5538,7 +5538,7 @@
       </ns0:c>
       <ns0:c r="F145" s="1">
         <ns0:f>ROUND(F144*1.4,-5)</ns0:f>
-        <ns0:v>4.406321853773283e+41</ns0:v>
+        <ns0:v>2.693313153544929e+41</ns0:v>
       </ns0:c>
       <ns0:c r="G145" s="1" t="n">
         <ns0:v>29.2000000000001</ns0:v>
@@ -5570,7 +5570,7 @@
       </ns0:c>
       <ns0:c r="F146" s="1">
         <ns0:f>ROUND(F145*1.4,-5)</ns0:f>
-        <ns0:v>6.168850595282596e+41</ns0:v>
+        <ns0:v>3.7706384149629006e+41</ns0:v>
       </ns0:c>
       <ns0:c r="G146" s="1" t="n">
         <ns0:v>29.4000000000001</ns0:v>
@@ -5602,7 +5602,7 @@
       </ns0:c>
       <ns0:c r="F147" s="1">
         <ns0:f>ROUND(F146*1.4,-5)</ns0:f>
-        <ns0:v>8.636390833395633e+41</ns0:v>
+        <ns0:v>5.2788937809480605e+41</ns0:v>
       </ns0:c>
       <ns0:c r="G147" s="1" t="n">
         <ns0:v>29.6000000000001</ns0:v>
@@ -5634,7 +5634,7 @@
       </ns0:c>
       <ns0:c r="F148" s="1">
         <ns0:f>ROUND(F147*1.4,-5)</ns0:f>
-        <ns0:v>1.2090947166753886e+42</ns0:v>
+        <ns0:v>7.390451293327283e+41</ns0:v>
       </ns0:c>
       <ns0:c r="G148" s="1" t="n">
         <ns0:v>29.8000000000001</ns0:v>
@@ -5666,7 +5666,7 @@
       </ns0:c>
       <ns0:c r="F149" s="1">
         <ns0:f>ROUND(F148*1.4,-5)</ns0:f>
-        <ns0:v>1.692732603345544e+42</ns0:v>
+        <ns0:v>1.0346631810658196e+42</ns0:v>
       </ns0:c>
       <ns0:c r="G149" s="1" t="n">
         <ns0:v>30.0000000000001</ns0:v>
@@ -5698,7 +5698,7 @@
       </ns0:c>
       <ns0:c r="F150" s="1">
         <ns0:f>ROUND(F149*1.4,-5)</ns0:f>
-        <ns0:v>2.369825644683761e+42</ns0:v>
+        <ns0:v>1.4485284534921475e+42</ns0:v>
       </ns0:c>
       <ns0:c r="G150" s="1" t="n">
         <ns0:v>30.2000000000001</ns0:v>
@@ -5730,7 +5730,7 @@
       </ns0:c>
       <ns0:c r="F151" s="1">
         <ns0:f>ROUND(F150*1.4,-5)</ns0:f>
-        <ns0:v>3.317755902557265e+42</ns0:v>
+        <ns0:v>2.0279398348890064e+42</ns0:v>
       </ns0:c>
       <ns0:c r="G151" s="1" t="n">
         <ns0:v>30.4000000000001</ns0:v>
@@ -5762,7 +5762,7 @@
       </ns0:c>
       <ns0:c r="F152" s="1">
         <ns0:f>ROUND(F151*1.4,-5)</ns0:f>
-        <ns0:v>4.644858263580172e+42</ns0:v>
+        <ns0:v>2.8391157688446086e+42</ns0:v>
       </ns0:c>
       <ns0:c r="G152" s="1" t="n">
         <ns0:v>30.6000000000001</ns0:v>
@@ -5794,7 +5794,7 @@
       </ns0:c>
       <ns0:c r="F153" s="1">
         <ns0:f>ROUND(F152*1.4,-5)</ns0:f>
-        <ns0:v>6.50280156901224e+42</ns0:v>
+        <ns0:v>3.974762076382452e+42</ns0:v>
       </ns0:c>
       <ns0:c r="G153" s="1" t="n">
         <ns0:v>30.8000000000001</ns0:v>
@@ -5826,7 +5826,7 @@
       </ns0:c>
       <ns0:c r="F154" s="1">
         <ns0:f>ROUND(F153*1.4,-5)</ns0:f>
-        <ns0:v>9.103922196617134e+42</ns0:v>
+        <ns0:v>5.5646669069354325e+42</ns0:v>
       </ns0:c>
       <ns0:c r="G154" s="1" t="n">
         <ns0:v>31.0000000000001</ns0:v>
@@ -5858,7 +5858,7 @@
       </ns0:c>
       <ns0:c r="F155" s="1">
         <ns0:f>ROUND(F154*1.4,-5)</ns0:f>
-        <ns0:v>1.2745491075263987e+43</ns0:v>
+        <ns0:v>7.790533669709605e+42</ns0:v>
       </ns0:c>
       <ns0:c r="G155" s="1" t="n">
         <ns0:v>31.2000000000001</ns0:v>
@@ -5890,7 +5890,7 @@
       </ns0:c>
       <ns0:c r="F156" s="1">
         <ns0:f>ROUND(F155*1.4,-5)</ns0:f>
-        <ns0:v>1.7843687505369578e+43</ns0:v>
+        <ns0:v>1.0906747137593445e+43</ns0:v>
       </ns0:c>
       <ns0:c r="G156" s="1" t="n">
         <ns0:v>31.4000000000001</ns0:v>
@@ -5922,7 +5922,7 @@
       </ns0:c>
       <ns0:c r="F157" s="1">
         <ns0:f>ROUND(F156*1.4,-5)</ns0:f>
-        <ns0:v>2.4981162507517407e+43</ns0:v>
+        <ns0:v>1.5269445992630822e+43</ns0:v>
       </ns0:c>
       <ns0:c r="G157" s="1" t="n">
         <ns0:v>31.6000000000001</ns0:v>
@@ -5954,7 +5954,7 @@
       </ns0:c>
       <ns0:c r="F158" s="1">
         <ns0:f>ROUND(F157*1.4,-5)</ns0:f>
-        <ns0:v>3.497362751052437e+43</ns0:v>
+        <ns0:v>2.137722438968315e+43</ns0:v>
       </ns0:c>
       <ns0:c r="G158" s="1" t="n">
         <ns0:v>31.8000000000001</ns0:v>
@@ -5986,7 +5986,7 @@
       </ns0:c>
       <ns0:c r="F159" s="1">
         <ns0:f>ROUND(F158*1.4,-5)</ns0:f>
-        <ns0:v>4.896307851473411e+43</ns0:v>
+        <ns0:v>2.9928114145556406e+43</ns0:v>
       </ns0:c>
       <ns0:c r="G159" s="1" t="n">
         <ns0:v>32.0000000000001</ns0:v>
@@ -6018,7 +6018,7 @@
       </ns0:c>
       <ns0:c r="F160" s="1">
         <ns0:f>ROUND(F159*1.4,-5)</ns0:f>
-        <ns0:v>6.854830992062775e+43</ns0:v>
+        <ns0:v>4.1899359803778964e+43</ns0:v>
       </ns0:c>
       <ns0:c r="G160" s="1" t="n">
         <ns0:v>32.2000000000001</ns0:v>
@@ -6050,7 +6050,7 @@
       </ns0:c>
       <ns0:c r="F161" s="1">
         <ns0:f>ROUND(F160*1.4,-5)</ns0:f>
-        <ns0:v>9.596763388887884e+43</ns0:v>
+        <ns0:v>5.865910372529055e+43</ns0:v>
       </ns0:c>
       <ns0:c r="G161" s="1" t="n">
         <ns0:v>32.4000000000001</ns0:v>
@@ -6082,7 +6082,7 @@
       </ns0:c>
       <ns0:c r="F162" s="1">
         <ns0:f>ROUND(F161*1.4,-5)</ns0:f>
-        <ns0:v>1.3435468744443037e+44</ns0:v>
+        <ns0:v>8.212274521540677e+43</ns0:v>
       </ns0:c>
       <ns0:c r="G162" s="1" t="n">
         <ns0:v>32.6000000000001</ns0:v>
@@ -6114,7 +6114,7 @@
       </ns0:c>
       <ns0:c r="F163" s="1">
         <ns0:f>ROUND(F162*1.4,-5)</ns0:f>
-        <ns0:v>1.880965624222025e+44</ns0:v>
+        <ns0:v>1.1497184330156946e+44</ns0:v>
       </ns0:c>
       <ns0:c r="G163" s="1" t="n">
         <ns0:v>32.8000000000001</ns0:v>
@@ -6146,7 +6146,7 @@
       </ns0:c>
       <ns0:c r="F164" s="1">
         <ns0:f>ROUND(F163*1.4,-5)</ns0:f>
-        <ns0:v>2.633351873910835e+44</ns0:v>
+        <ns0:v>1.609605806221972e+44</ns0:v>
       </ns0:c>
       <ns0:c r="G164" s="1" t="n">
         <ns0:v>33.0000000000001</ns0:v>
@@ -6178,7 +6178,7 @@
       </ns0:c>
       <ns0:c r="F165" s="1">
         <ns0:f>ROUND(F164*1.4,-5)</ns0:f>
-        <ns0:v>3.686692623475169e+44</ns0:v>
+        <ns0:v>2.253448128710761e+44</ns0:v>
       </ns0:c>
       <ns0:c r="G165" s="1" t="n">
         <ns0:v>33.2000000000001</ns0:v>
@@ -6210,7 +6210,7 @@
       </ns0:c>
       <ns0:c r="F166" s="1">
         <ns0:f>ROUND(F165*1.4,-5)</ns0:f>
-        <ns0:v>5.161369672865237e+44</ns0:v>
+        <ns0:v>3.154827380195065e+44</ns0:v>
       </ns0:c>
       <ns0:c r="G166" s="1" t="n">
         <ns0:v>33.4000000000001</ns0:v>
@@ -6242,7 +6242,7 @@
       </ns0:c>
       <ns0:c r="F167" s="1">
         <ns0:f>ROUND(F166*1.4,-5)</ns0:f>
-        <ns0:v>7.225917542011331e+44</ns0:v>
+        <ns0:v>4.416758332273091e+44</ns0:v>
       </ns0:c>
       <ns0:c r="G167" s="1" t="n">
         <ns0:v>33.6000000000001</ns0:v>
@@ -6274,7 +6274,7 @@
       </ns0:c>
       <ns0:c r="F168" s="1">
         <ns0:f>ROUND(F167*1.4,-5)</ns0:f>
-        <ns0:v>1.0116284558815864e+45</ns0:v>
+        <ns0:v>6.183461665182327e+44</ns0:v>
       </ns0:c>
       <ns0:c r="G168" s="1" t="n">
         <ns0:v>33.8000000000001</ns0:v>
@@ -6306,7 +6306,7 @@
       </ns0:c>
       <ns0:c r="F169" s="1">
         <ns0:f>ROUND(F168*1.4,-5)</ns0:f>
-        <ns0:v>1.4162798382342208e+45</ns0:v>
+        <ns0:v>8.656846331255258e+44</ns0:v>
       </ns0:c>
       <ns0:c r="G169" s="1" t="n">
         <ns0:v>34.0000000000001</ns0:v>
@@ -6338,7 +6338,7 @@
       </ns0:c>
       <ns0:c r="F170" s="1">
         <ns0:f>ROUND(F169*1.4,-5)</ns0:f>
-        <ns0:v>1.982791773527909e+45</ns0:v>
+        <ns0:v>1.211958486375736e+45</ns0:v>
       </ns0:c>
       <ns0:c r="G170" s="1" t="n">
         <ns0:v>34.2000000000001</ns0:v>
@@ -6370,7 +6370,7 @@
       </ns0:c>
       <ns0:c r="F171" s="1">
         <ns0:f>ROUND(F170*1.4,-5)</ns0:f>
-        <ns0:v>2.7759084829390727e+45</ns0:v>
+        <ns0:v>1.6967418809260303e+45</ns0:v>
       </ns0:c>
       <ns0:c r="G171" s="1" t="n">
         <ns0:v>34.4000000000001</ns0:v>
@@ -6402,7 +6402,7 @@
       </ns0:c>
       <ns0:c r="F172" s="1">
         <ns0:f>ROUND(F171*1.4,-5)</ns0:f>
-        <ns0:v>3.886271876114702e+45</ns0:v>
+        <ns0:v>2.3754386332964422e+45</ns0:v>
       </ns0:c>
       <ns0:c r="G172" s="1" t="n">
         <ns0:v>34.6000000000001</ns0:v>
@@ -6434,7 +6434,7 @@
       </ns0:c>
       <ns0:c r="F173" s="1">
         <ns0:f>ROUND(F172*1.4,-5)</ns0:f>
-        <ns0:v>5.4407806265605814e+45</ns0:v>
+        <ns0:v>3.325614086615019e+45</ns0:v>
       </ns0:c>
       <ns0:c r="G173" s="1" t="n">
         <ns0:v>34.8000000000001</ns0:v>
@@ -6466,7 +6466,7 @@
       </ns0:c>
       <ns0:c r="F174" s="1">
         <ns0:f>ROUND(F173*1.4,-5)</ns0:f>
-        <ns0:v>7.617092877184813e+45</ns0:v>
+        <ns0:v>4.655859721261025e+45</ns0:v>
       </ns0:c>
       <ns0:c r="G174" s="1" t="n">
         <ns0:v>35.0000000000001</ns0:v>
@@ -6498,7 +6498,7 @@
       </ns0:c>
       <ns0:c r="F175" s="1">
         <ns0:f>ROUND(F174*1.4,-5)</ns0:f>
-        <ns0:v>1.0663930028058737e+46</ns0:v>
+        <ns0:v>6.518203609765435e+45</ns0:v>
       </ns0:c>
       <ns0:c r="G175" s="1" t="n">
         <ns0:v>35.2000000000001</ns0:v>
@@ -6530,7 +6530,7 @@
       </ns0:c>
       <ns0:c r="F176" s="1">
         <ns0:f>ROUND(F175*1.4,-5)</ns0:f>
-        <ns0:v>1.492950203928223e+46</ns0:v>
+        <ns0:v>9.125485053671609e+45</ns0:v>
       </ns0:c>
       <ns0:c r="G176" s="1" t="n">
         <ns0:v>35.4000000000001</ns0:v>
@@ -6562,7 +6562,7 @@
       </ns0:c>
       <ns0:c r="F177" s="1">
         <ns0:f>ROUND(F176*1.4,-5)</ns0:f>
-        <ns0:v>2.0901302854995122e+46</ns0:v>
+        <ns0:v>1.2775679075140252e+46</ns0:v>
       </ns0:c>
       <ns0:c r="G177" s="1" t="n">
         <ns0:v>35.6000000000001</ns0:v>
@@ -6594,7 +6594,7 @@
       </ns0:c>
       <ns0:c r="F178" s="1">
         <ns0:f>ROUND(F177*1.4,-5)</ns0:f>
-        <ns0:v>2.926182399699317e+46</ns0:v>
+        <ns0:v>1.7885950705196354e+46</ns0:v>
       </ns0:c>
       <ns0:c r="G178" s="1" t="n">
         <ns0:v>35.8000000000001</ns0:v>
@@ -6626,7 +6626,7 @@
       </ns0:c>
       <ns0:c r="F179" s="1">
         <ns0:f>ROUND(F178*1.4,-5)</ns0:f>
-        <ns0:v>4.096655359579043e+46</ns0:v>
+        <ns0:v>2.5040330987274893e+46</ns0:v>
       </ns0:c>
       <ns0:c r="G179" s="1" t="n">
         <ns0:v>36.0000000000001</ns0:v>
@@ -6658,7 +6658,7 @@
       </ns0:c>
       <ns0:c r="F180" s="1">
         <ns0:f>ROUND(F179*1.4,-5)</ns0:f>
-        <ns0:v>5.73531750341066e+46</ns0:v>
+        <ns0:v>3.5056463382184853e+46</ns0:v>
       </ns0:c>
       <ns0:c r="G180" s="1" t="n">
         <ns0:v>36.2000000000001</ns0:v>
@@ -6690,7 +6690,7 @@
       </ns0:c>
       <ns0:c r="F181" s="1">
         <ns0:f>ROUND(F180*1.4,-5)</ns0:f>
-        <ns0:v>8.029444504774923e+46</ns0:v>
+        <ns0:v>4.907904873505879e+46</ns0:v>
       </ns0:c>
       <ns0:c r="G181" s="1" t="n">
         <ns0:v>36.4000000000001</ns0:v>
@@ -6722,7 +6722,7 @@
       </ns0:c>
       <ns0:c r="F182" s="1">
         <ns0:f>ROUND(F181*1.4,-5)</ns0:f>
-        <ns0:v>1.1241222306684891e+47</ns0:v>
+        <ns0:v>6.87106682290823e+46</ns0:v>
       </ns0:c>
       <ns0:c r="G182" s="1" t="n">
         <ns0:v>36.6000000000001</ns0:v>
@@ -6754,7 +6754,7 @@
       </ns0:c>
       <ns0:c r="F183" s="1">
         <ns0:f>ROUND(F182*1.4,-5)</ns0:f>
-        <ns0:v>1.5737711229358847e+47</ns0:v>
+        <ns0:v>9.619493552071522e+46</ns0:v>
       </ns0:c>
       <ns0:c r="G183" s="1" t="n">
         <ns0:v>36.8000000000001</ns0:v>
@@ -6786,7 +6786,7 @@
       </ns0:c>
       <ns0:c r="F184" s="1">
         <ns0:f>ROUND(F183*1.4,-5)</ns0:f>
-        <ns0:v>2.2032795721102382e+47</ns0:v>
+        <ns0:v>1.346729097290013e+47</ns0:v>
       </ns0:c>
       <ns0:c r="G184" s="1" t="n">
         <ns0:v>37.0000000000001</ns0:v>
@@ -6818,7 +6818,7 @@
       </ns0:c>
       <ns0:c r="F185" s="1">
         <ns0:f>ROUND(F184*1.4,-5)</ns0:f>
-        <ns0:v>3.0845914009543333e+47</ns0:v>
+        <ns0:v>1.885420736206018e+47</ns0:v>
       </ns0:c>
       <ns0:c r="G185" s="1" t="n">
         <ns0:v>37.2000000000001</ns0:v>
@@ -6850,7 +6850,7 @@
       </ns0:c>
       <ns0:c r="F186" s="1">
         <ns0:f>ROUND(F185*1.4,-5)</ns0:f>
-        <ns0:v>4.3184279613360664e+47</ns0:v>
+        <ns0:v>2.639589030688425e+47</ns0:v>
       </ns0:c>
       <ns0:c r="G186" s="1" t="n">
         <ns0:v>37.4000000000001</ns0:v>
@@ -6882,7 +6882,7 @@
       </ns0:c>
       <ns0:c r="F187" s="1">
         <ns0:f>ROUND(F186*1.4,-5)</ns0:f>
-        <ns0:v>6.045799145870493e+47</ns0:v>
+        <ns0:v>3.695424642963795e+47</ns0:v>
       </ns0:c>
       <ns0:c r="G187" s="1" t="n">
         <ns0:v>37.6000000000001</ns0:v>
@@ -6914,7 +6914,7 @@
       </ns0:c>
       <ns0:c r="F188" s="1">
         <ns0:f>ROUND(F187*1.4,-5)</ns0:f>
-        <ns0:v>8.464118804218689e+47</ns0:v>
+        <ns0:v>5.173594500149313e+47</ns0:v>
       </ns0:c>
       <ns0:c r="G188" s="1" t="n">
         <ns0:v>37.8000000000001</ns0:v>
@@ -6946,7 +6946,7 @@
       </ns0:c>
       <ns0:c r="F189" s="1">
         <ns0:f>ROUND(F188*1.4,-5)</ns0:f>
-        <ns0:v>1.1849766325906162e+48</ns0:v>
+        <ns0:v>7.243032300209037e+47</ns0:v>
       </ns0:c>
       <ns0:c r="G189" s="1" t="n">
         <ns0:v>38.0000000000001</ns0:v>
@@ -6978,7 +6978,7 @@
       </ns0:c>
       <ns0:c r="F190" s="1">
         <ns0:f>ROUND(F189*1.4,-5)</ns0:f>
-        <ns0:v>1.6589672856268625e+48</ns0:v>
+        <ns0:v>1.0140245220292651e+48</ns0:v>
       </ns0:c>
       <ns0:c r="G190" s="1" t="n">
         <ns0:v>38.2000000000001</ns0:v>
@@ -7010,7 +7010,7 @@
       </ns0:c>
       <ns0:c r="F191" s="1">
         <ns0:f>ROUND(F190*1.4,-5)</ns0:f>
-        <ns0:v>2.3225541998776073e+48</ns0:v>
+        <ns0:v>1.4196343308409709e+48</ns0:v>
       </ns0:c>
       <ns0:c r="G191" s="1" t="n">
         <ns0:v>38.4000000000001</ns0:v>
@@ -7042,7 +7042,7 @@
       </ns0:c>
       <ns0:c r="F192" s="1">
         <ns0:f>ROUND(F191*1.4,-5)</ns0:f>
-        <ns0:v>3.2515758798286497e+48</ns0:v>
+        <ns0:v>1.987488063177359e+48</ns0:v>
       </ns0:c>
       <ns0:c r="G192" s="1" t="n">
         <ns0:v>38.6000000000001</ns0:v>
@@ -7074,7 +7074,7 @@
       </ns0:c>
       <ns0:c r="F193" s="1">
         <ns0:f>ROUND(F192*1.4,-5)</ns0:f>
-        <ns0:v>4.55220623176011e+48</ns0:v>
+        <ns0:v>2.782483288448303e+48</ns0:v>
       </ns0:c>
       <ns0:c r="G193" s="1" t="n">
         <ns0:v>38.8000000000001</ns0:v>
@@ -7106,7 +7106,7 @@
       </ns0:c>
       <ns0:c r="F194" s="1">
         <ns0:f>ROUND(F193*1.4,-5)</ns0:f>
-        <ns0:v>6.373088724464154e+48</ns0:v>
+        <ns0:v>3.895476603827624e+48</ns0:v>
       </ns0:c>
       <ns0:c r="G194" s="1" t="n">
         <ns0:v>39.0000000000001</ns0:v>
@@ -7138,7 +7138,7 @@
       </ns0:c>
       <ns0:c r="F195" s="1">
         <ns0:f>ROUND(F194*1.4,-5)</ns0:f>
-        <ns0:v>8.922324214249816e+48</ns0:v>
+        <ns0:v>5.453667245358673e+48</ns0:v>
       </ns0:c>
       <ns0:c r="G195" s="1" t="n">
         <ns0:v>39.2000000000001</ns0:v>
@@ -7170,7 +7170,7 @@
       </ns0:c>
       <ns0:c r="F196" s="1">
         <ns0:f>ROUND(F195*1.4,-5)</ns0:f>
-        <ns0:v>1.249125389994974e+49</ns0:v>
+        <ns0:v>7.635134143502141e+48</ns0:v>
       </ns0:c>
       <ns0:c r="G196" s="1" t="n">
         <ns0:v>39.4000000000001</ns0:v>
@@ -7202,7 +7202,7 @@
       </ns0:c>
       <ns0:c r="F197" s="1">
         <ns0:f>ROUND(F196*1.4,-5)</ns0:f>
-        <ns0:v>1.7487755459929634e+49</ns0:v>
+        <ns0:v>1.0689187800902998e+49</ns0:v>
       </ns0:c>
       <ns0:c r="G197" s="1" t="n">
         <ns0:v>39.6000000000001</ns0:v>
@@ -7234,7 +7234,7 @@
       </ns0:c>
       <ns0:c r="F198" s="1">
         <ns0:f>ROUND(F197*1.4,-5)</ns0:f>
-        <ns0:v>2.4482857643901485e+49</ns0:v>
+        <ns0:v>1.4964862921264196e+49</ns0:v>
       </ns0:c>
       <ns0:c r="G198" s="1" t="n">
         <ns0:v>39.8000000000001</ns0:v>
@@ -7266,7 +7266,7 @@
       </ns0:c>
       <ns0:c r="F199" s="1">
         <ns0:f>ROUND(F198*1.4,-5)</ns0:f>
-        <ns0:v>3.427600070146208e+49</ns0:v>
+        <ns0:v>2.0950808089769872e+49</ns0:v>
       </ns0:c>
       <ns0:c r="G199" s="1" t="n">
         <ns0:v>40.0000000000001</ns0:v>
@@ -7298,7 +7298,7 @@
       </ns0:c>
       <ns0:c r="F200" s="1">
         <ns0:f>ROUND(F199*1.4,-5)</ns0:f>
-        <ns0:v>4.798640098204691e+49</ns0:v>
+        <ns0:v>2.9331131325677817e+49</ns0:v>
       </ns0:c>
       <ns0:c r="G200" s="1" t="n">
         <ns0:v>40.2000000000001</ns0:v>
@@ -7330,7 +7330,7 @@
       </ns0:c>
       <ns0:c r="F201" s="1">
         <ns0:f>ROUND(F200*1.4,-5)</ns0:f>
-        <ns0:v>6.718096137486567e+49</ns0:v>
+        <ns0:v>4.106358385594894e+49</ns0:v>
       </ns0:c>
       <ns0:c r="G201" s="1" t="n">
         <ns0:v>40.4000000000001</ns0:v>
@@ -7362,7 +7362,7 @@
       </ns0:c>
       <ns0:c r="F202" s="1">
         <ns0:f>ROUND(F201*1.4,-5)</ns0:f>
-        <ns0:v>9.405334592481194e+49</ns0:v>
+        <ns0:v>5.748901739832851e+49</ns0:v>
       </ns0:c>
       <ns0:c r="G202" s="1" t="n">
         <ns0:v>40.6000000000001</ns0:v>
@@ -7394,7 +7394,7 @@
       </ns0:c>
       <ns0:c r="F203" s="1">
         <ns0:f>ROUND(F202*1.4,-5)</ns0:f>
-        <ns0:v>1.3167468429473672e+50</ns0:v>
+        <ns0:v>8.048462435765991e+49</ns0:v>
       </ns0:c>
       <ns0:c r="G203" s="1" t="n">
         <ns0:v>40.8000000000001</ns0:v>
@@ -7426,7 +7426,7 @@
       </ns0:c>
       <ns0:c r="F204" s="1">
         <ns0:f>ROUND(F203*1.4,-5)</ns0:f>
-        <ns0:v>1.8434455801263142e+50</ns0:v>
+        <ns0:v>1.1267847410072387e+50</ns0:v>
       </ns0:c>
       <ns0:c r="G204" s="1" t="n">
         <ns0:v>41.0000000000001</ns0:v>
@@ -7458,7 +7458,7 @@
       </ns0:c>
       <ns0:c r="F205" s="1">
         <ns0:f>ROUND(F204*1.4,-5)</ns0:f>
-        <ns0:v>2.58082381217684e+50</ns0:v>
+        <ns0:v>1.5774986374101342e+50</ns0:v>
       </ns0:c>
       <ns0:c r="G205" s="1" t="n">
         <ns0:v>41.2000000000001</ns0:v>
@@ -7490,7 +7490,7 @@
       </ns0:c>
       <ns0:c r="F206" s="1">
         <ns0:f>ROUND(F205*1.4,-5)</ns0:f>
-        <ns0:v>3.613153337047575e+50</ns0:v>
+        <ns0:v>2.208498092374188e+50</ns0:v>
       </ns0:c>
       <ns0:c r="G206" s="1" t="n">
         <ns0:v>41.4000000000001</ns0:v>
@@ -7522,7 +7522,7 @@
       </ns0:c>
       <ns0:c r="F207" s="1">
         <ns0:f>ROUND(F206*1.4,-5)</ns0:f>
-        <ns0:v>5.058414671866605e+50</ns0:v>
+        <ns0:v>3.091897329323863e+50</ns0:v>
       </ns0:c>
       <ns0:c r="G207" s="1" t="n">
         <ns0:v>41.6000000000001</ns0:v>
@@ -7554,7 +7554,7 @@
       </ns0:c>
       <ns0:c r="F208" s="1">
         <ns0:f>ROUND(F207*1.4,-5)</ns0:f>
-        <ns0:v>7.081780540613247e+50</ns0:v>
+        <ns0:v>4.328656261053408e+50</ns0:v>
       </ns0:c>
       <ns0:c r="G208" s="1" t="n">
         <ns0:v>41.8000000000001</ns0:v>
@@ -7586,7 +7586,7 @@
       </ns0:c>
       <ns0:c r="F209" s="1">
         <ns0:f>ROUND(F208*1.4,-5)</ns0:f>
-        <ns0:v>9.914492756858545e+50</ns0:v>
+        <ns0:v>6.06011876547477e+50</ns0:v>
       </ns0:c>
       <ns0:c r="G209" s="1" t="n">
         <ns0:v>42.0000000000001</ns0:v>
@@ -7618,7 +7618,7 @@
       </ns0:c>
       <ns0:c r="F210" s="1">
         <ns0:f>ROUND(F209*1.4,-5)</ns0:f>
-        <ns0:v>1.3880289859601963e+51</ns0:v>
+        <ns0:v>8.484166271664678e+50</ns0:v>
       </ns0:c>
       <ns0:c r="G210" s="1" t="n">
         <ns0:v>42.2000000000001</ns0:v>
@@ -7650,7 +7650,7 @@
       </ns0:c>
       <ns0:c r="F211" s="1">
         <ns0:f>ROUND(F210*1.4,-5)</ns0:f>
-        <ns0:v>1.9432405803442746e+51</ns0:v>
+        <ns0:v>1.187783278033055e+51</ns0:v>
       </ns0:c>
       <ns0:c r="G211" s="1" t="n">
         <ns0:v>42.4000000000001</ns0:v>
@@ -7682,7 +7682,7 @@
       </ns0:c>
       <ns0:c r="F212" s="1">
         <ns0:f>ROUND(F211*1.4,-5)</ns0:f>
-        <ns0:v>2.7205368124819845e+51</ns0:v>
+        <ns0:v>1.662896589246277e+51</ns0:v>
       </ns0:c>
       <ns0:c r="G212" s="1" t="n">
         <ns0:v>42.6000000000002</ns0:v>
@@ -7714,7 +7714,7 @@
       </ns0:c>
       <ns0:c r="F213" s="1">
         <ns0:f>ROUND(F212*1.4,-5)</ns0:f>
-        <ns0:v>3.808751537474778e+51</ns0:v>
+        <ns0:v>2.3280552249447878e+51</ns0:v>
       </ns0:c>
       <ns0:c r="G213" s="1" t="n">
         <ns0:v>42.8000000000002</ns0:v>
@@ -7746,7 +7746,7 @@
       </ns0:c>
       <ns0:c r="F214" s="1">
         <ns0:f>ROUND(F213*1.4,-5)</ns0:f>
-        <ns0:v>5.33225215246469e+51</ns0:v>
+        <ns0:v>3.2592773149227023e+51</ns0:v>
       </ns0:c>
       <ns0:c r="G214" s="1" t="n">
         <ns0:v>43.0000000000001</ns0:v>
@@ -7778,7 +7778,7 @@
       </ns0:c>
       <ns0:c r="F215" s="1">
         <ns0:f>ROUND(F214*1.4,-5)</ns0:f>
-        <ns0:v>7.465153013450565e+51</ns0:v>
+        <ns0:v>4.562988240891783e+51</ns0:v>
       </ns0:c>
       <ns0:c r="G215" s="1" t="n">
         <ns0:v>43.2000000000002</ns0:v>
@@ -7810,7 +7810,7 @@
       </ns0:c>
       <ns0:c r="F216" s="1">
         <ns0:f>ROUND(F215*1.4,-5)</ns0:f>
-        <ns0:v>1.0451214218830791e+52</ns0:v>
+        <ns0:v>6.388183537248496e+51</ns0:v>
       </ns0:c>
       <ns0:c r="G216" s="1" t="n">
         <ns0:v>43.4000000000002</ns0:v>
@@ -7842,7 +7842,7 @@
       </ns0:c>
       <ns0:c r="F217" s="1">
         <ns0:f>ROUND(F216*1.4,-5)</ns0:f>
-        <ns0:v>1.4631699906363107e+52</ns0:v>
+        <ns0:v>8.943456952147894e+51</ns0:v>
       </ns0:c>
       <ns0:c r="G217" s="1" t="n">
         <ns0:v>43.6000000000002</ns0:v>
@@ -7874,7 +7874,7 @@
       </ns0:c>
       <ns0:c r="F218" s="1">
         <ns0:f>ROUND(F217*1.4,-5)</ns0:f>
-        <ns0:v>2.0484379868908348e+52</ns0:v>
+        <ns0:v>1.2520839733007052e+52</ns0:v>
       </ns0:c>
       <ns0:c r="G218" s="1" t="n">
         <ns0:v>43.8000000000002</ns0:v>
@@ -7906,7 +7906,7 @@
       </ns0:c>
       <ns0:c r="F219" s="1">
         <ns0:f>ROUND(F218*1.4,-5)</ns0:f>
-        <ns0:v>2.867813181647169e+52</ns0:v>
+        <ns0:v>1.752917562620987e+52</ns0:v>
       </ns0:c>
       <ns0:c r="G219" s="1" t="n">
         <ns0:v>44.0000000000002</ns0:v>
@@ -7938,7 +7938,7 @@
       </ns0:c>
       <ns0:c r="F220" s="1">
         <ns0:f>ROUND(F219*1.4,-5)</ns0:f>
-        <ns0:v>4.014938454306036e+52</ns0:v>
+        <ns0:v>2.454084587669382e+52</ns0:v>
       </ns0:c>
       <ns0:c r="G220" s="1" t="n">
         <ns0:v>44.2000000000002</ns0:v>
@@ -7970,7 +7970,7 @@
       </ns0:c>
       <ns0:c r="F221" s="1">
         <ns0:f>ROUND(F220*1.4,-5)</ns0:f>
-        <ns0:v>5.620913836028451e+52</ns0:v>
+        <ns0:v>3.4357184227371343e+52</ns0:v>
       </ns0:c>
       <ns0:c r="G221" s="1" t="n">
         <ns0:v>44.4000000000002</ns0:v>
@@ -8002,7 +8002,7 @@
       </ns0:c>
       <ns0:c r="F222" s="1">
         <ns0:f>ROUND(F221*1.4,-5)</ns0:f>
-        <ns0:v>7.86927937043983e+52</ns0:v>
+        <ns0:v>4.810005791831987e+52</ns0:v>
       </ns0:c>
       <ns0:c r="G222" s="1" t="n">
         <ns0:v>44.6000000000002</ns0:v>
@@ -8034,7 +8034,7 @@
       </ns0:c>
       <ns0:c r="F223" s="1">
         <ns0:f>ROUND(F222*1.4,-5)</ns0:f>
-        <ns0:v>1.1016991118615762e+53</ns0:v>
+        <ns0:v>6.734008108564782e+52</ns0:v>
       </ns0:c>
       <ns0:c r="G223" s="1" t="n">
         <ns0:v>44.8000000000002</ns0:v>

</xml_diff>

<commit_message>
Separate combat tiers from final-wave completion; strengthen provisional reforge wall
</commit_message>
<xml_diff>
--- a/space-battleship/config_excel/level.xlsx
+++ b/space-battleship/config_excel/level.xlsx
@@ -2191,10 +2191,10 @@
         </ns0:is>
       </ns0:c>
       <ns0:c r="D37" s="1" t="n">
-        <ns0:v>1.512294048887176e+25</ns0:v>
+        <ns0:v>4.026230848222263e+26</ns0:v>
       </ns0:c>
       <ns0:c r="E37" s="1" t="n">
-        <ns0:v>1.512294048887176e+25</ns0:v>
+        <ns0:v>4.026230848222263e+26</ns0:v>
       </ns0:c>
       <ns0:c r="F37" s="1" t="n">
         <ns0:v>2.012338714944041e+16</ns0:v>
@@ -2219,10 +2219,10 @@
         </ns0:is>
       </ns0:c>
       <ns0:c r="D38" s="1" t="n">
-        <ns0:v>5.797772421440058e+26</ns0:v>
+        <ns0:v>1.543560274627236e+28</ns0:v>
       </ns0:c>
       <ns0:c r="E38" s="1" t="n">
-        <ns0:v>5.797772421440058e+26</ns0:v>
+        <ns0:v>1.543560274627236e+28</ns0:v>
       </ns0:c>
       <ns0:c r="F38" s="1" t="n">
         <ns0:v>6.008811205403466e+16</ns0:v>
@@ -2247,10 +2247,10 @@
         </ns0:is>
       </ns0:c>
       <ns0:c r="D39" s="1" t="n">
-        <ns0:v>1.731205568606127e+27</ns0:v>
+        <ns0:v>4.609046283072532e+28</ns0:v>
       </ns0:c>
       <ns0:c r="E39" s="1" t="n">
-        <ns0:v>1.731205568606127e+27</ns0:v>
+        <ns0:v>4.609046283072532e+28</ns0:v>
       </ns0:c>
       <ns0:c r="F39" s="1" t="n">
         <ns0:v>1.245987091552463e+17</ns0:v>
@@ -2275,10 +2275,10 @@
         </ns0:is>
       </ns0:c>
       <ns0:c r="D40" s="1" t="n">
-        <ns0:v>5.169352128568795e+27</ns0:v>
+        <ns0:v>1.376253845651405e+29</ns0:v>
       </ns0:c>
       <ns0:c r="E40" s="1" t="n">
-        <ns0:v>5.169352128568795e+27</ns0:v>
+        <ns0:v>1.376253845651405e+29</ns0:v>
       </ns0:c>
       <ns0:c r="F40" s="1" t="n">
         <ns0:v>2.583678833043186e+17</ns0:v>
@@ -2303,10 +2303,10 @@
         </ns0:is>
       </ns0:c>
       <ns0:c r="D41" s="1" t="n">
-        <ns0:v>1.543560274627236e+28</ns0:v>
+        <ns0:v>4.109471963053564e+29</ns0:v>
       </ns0:c>
       <ns0:c r="E41" s="1" t="n">
-        <ns0:v>1.543560274627236e+28</ns0:v>
+        <ns0:v>4.109471963053564e+29</ns0:v>
       </ns0:c>
       <ns0:c r="F41" s="1" t="n">
         <ns0:v>5.357516428198349e+17</ns0:v>
@@ -2331,10 +2331,10 @@
         </ns0:is>
       </ns0:c>
       <ns0:c r="D42" s="1" t="n">
-        <ns0:v>1.376253845651405e+29</ns0:v>
+        <ns0:v>3.664046481187733e+30</ns0:v>
       </ns0:c>
       <ns0:c r="E42" s="1" t="n">
-        <ns0:v>1.376253845651405e+29</ns0:v>
+        <ns0:v>3.664046481187733e+30</ns0:v>
       </ns0:c>
       <ns0:c r="F42" s="1" t="n">
         <ns0:v>2.303634000144588e+18</ns0:v>
@@ -2359,10 +2359,10 @@
         </ns0:is>
       </ns0:c>
       <ns0:c r="D43" s="1" t="n">
-        <ns0:v>5.276226932910335e+30</ns0:v>
+        <ns0:v>1.404707481004547e+32</ns0:v>
       </ns0:c>
       <ns0:c r="E43" s="1" t="n">
-        <ns0:v>5.276226932910335e+30</ns0:v>
+        <ns0:v>1.404707481004547e+32</ns0:v>
       </ns0:c>
       <ns0:c r="F43" s="1" t="n">
         <ns0:v>2.053943214130691e+19</ns0:v>
@@ -2387,10 +2387,10 @@
         </ns0:is>
       </ns0:c>
       <ns0:c r="D44" s="1" t="n">
-        <ns0:v>1.575472920203933e+31</ns0:v>
+        <ns0:v>4.19443406295988e+32</ns0:v>
       </ns0:c>
       <ns0:c r="E44" s="1" t="n">
-        <ns0:v>1.575472920203933e+31</ns0:v>
+        <ns0:v>4.19443406295988e+32</ns0:v>
       </ns0:c>
       <ns0:c r="F44" s="1" t="n">
         <ns0:v>4.259056648821401e+19</ns0:v>
@@ -2415,10 +2415,10 @@
         </ns0:is>
       </ns0:c>
       <ns0:c r="D45" s="1" t="n">
-        <ns0:v>4.704336932162219e+31</ns0:v>
+        <ns0:v>1.252451300105319e+33</ns0:v>
       </ns0:c>
       <ns0:c r="E45" s="1" t="n">
-        <ns0:v>4.704336932162219e+31</ns0:v>
+        <ns0:v>1.252451300105319e+33</ns0:v>
       </ns0:c>
       <ns0:c r="F45" s="1" t="n">
         <ns0:v>8.831579866996054e+19</ns0:v>
@@ -2443,10 +2443,10 @@
         </ns0:is>
       </ns0:c>
       <ns0:c r="D46" s="1" t="n">
-        <ns0:v>1.404707481004547e+32</ns0:v>
+        <ns0:v>3.739799542893681e+33</ns0:v>
       </ns0:c>
       <ns0:c r="E46" s="1" t="n">
-        <ns0:v>1.404707481004547e+32</ns0:v>
+        <ns0:v>3.739799542893681e+33</ns0:v>
       </ns0:c>
       <ns0:c r="F46" s="1" t="n">
         <ns0:v>1.831316401220302e+20</ns0:v>
@@ -2471,10 +2471,10 @@
         </ns0:is>
       </ns0:c>
       <ns0:c r="D47" s="1" t="n">
-        <ns0:v>1.252451300105319e+33</ns0:v>
+        <ns0:v>3.334442838078192e+34</ns0:v>
       </ns0:c>
       <ns0:c r="E47" s="1" t="n">
-        <ns0:v>1.252451300105319e+33</ns0:v>
+        <ns0:v>3.334442838078192e+34</ns0:v>
       </ns0:c>
       <ns0:c r="F47" s="1" t="n">
         <ns0:v>7.874325321093216e+20</ns0:v>
@@ -2499,10 +2499,10 @@
         </ns0:is>
       </ns0:c>
       <ns0:c r="D48" s="1" t="n">
-        <ns0:v>4.801597686832596e+34</ns0:v>
+        <ns0:v>1.278345354972718e+36</ns0:v>
       </ns0:c>
       <ns0:c r="E48" s="1" t="n">
-        <ns0:v>4.801597686832596e+34</ns0:v>
+        <ns0:v>1.278345354972718e+36</ns0:v>
       </ns0:c>
       <ns0:c r="F48" s="1" t="n">
         <ns0:v>7.020827552511277e+21</ns0:v>
@@ -2527,10 +2527,10 @@
         </ns0:is>
       </ns0:c>
       <ns0:c r="D49" s="1" t="n">
-        <ns0:v>1.433749386731914e+35</ns0:v>
+        <ns0:v>3.817118776422855e+36</ns0:v>
       </ns0:c>
       <ns0:c r="E49" s="1" t="n">
-        <ns0:v>1.433749386731914e+35</ns0:v>
+        <ns0:v>3.817118776422855e+36</ns0:v>
       </ns0:c>
       <ns0:c r="F49" s="1" t="n">
         <ns0:v>1.455838801288738e+22</ns0:v>
@@ -2555,10 +2555,10 @@
         </ns0:is>
       </ns0:c>
       <ns0:c r="D50" s="1" t="n">
-        <ns0:v>4.281152728791306e+35</ns0:v>
+        <ns0:v>1.139785559249822e+37</ns0:v>
       </ns0:c>
       <ns0:c r="E50" s="1" t="n">
-        <ns0:v>4.281152728791306e+35</ns0:v>
+        <ns0:v>1.139785559249822e+37</ns0:v>
       </ns0:c>
       <ns0:c r="F50" s="1" t="n">
         <ns0:v>3.018827338352327e+22</ns0:v>
@@ -2583,10 +2583,10 @@
         </ns0:is>
       </ns0:c>
       <ns0:c r="D51" s="1" t="n">
-        <ns0:v>1.278345354972718e+36</ns0:v>
+        <ns0:v>3.40338144335102e+37</ns0:v>
       </ns0:c>
       <ns0:c r="E51" s="1" t="n">
-        <ns0:v>1.278345354972718e+36</ns0:v>
+        <ns0:v>3.40338144335102e+37</ns0:v>
       </ns0:c>
       <ns0:c r="F51" s="1" t="n">
         <ns0:v>6.259840368807384e+22</ns0:v>
@@ -2611,10 +2611,10 @@
         </ns0:is>
       </ns0:c>
       <ns0:c r="D52" s="1" t="n">
-        <ns0:v>1.139785559249822e+37</ns0:v>
+        <ns0:v>3.034489081264816e+38</ns0:v>
       </ns0:c>
       <ns0:c r="E52" s="1" t="n">
-        <ns0:v>1.139785559249822e+37</ns0:v>
+        <ns0:v>3.034489081264816e+38</ns0:v>
       </ns0:c>
       <ns0:c r="F52" s="1" t="n">
         <ns0:v>2.691616778469064e+23</ns0:v>
@@ -2639,10 +2639,10 @@
         </ns0:is>
       </ns0:c>
       <ns0:c r="D53" s="1" t="n">
-        <ns0:v>4.369664277021335e+38</ns0:v>
+        <ns0:v>1.163350283727174e+40</ns0:v>
       </ns0:c>
       <ns0:c r="E53" s="1" t="n">
-        <ns0:v>4.369664277021335e+38</ns0:v>
+        <ns0:v>1.163350283727174e+40</ns0:v>
       </ns0:c>
       <ns0:c r="F53" s="1" t="n">
         <ns0:v>2.399872556504138e+24</ns0:v>
@@ -2667,10 +2667,10 @@
         </ns0:is>
       </ns0:c>
       <ns0:c r="D54" s="1" t="n">
-        <ns0:v>1.304774761655727e+39</ns0:v>
+        <ns0:v>3.473745333604802e+40</ns0:v>
       </ns0:c>
       <ns0:c r="E54" s="1" t="n">
-        <ns0:v>1.304774761655727e+39</ns0:v>
+        <ns0:v>3.473745333604802e+40</ns0:v>
       </ns0:c>
       <ns0:c r="F54" s="1" t="n">
         <ns0:v>4.976375733166981e+24</ns0:v>
@@ -2695,10 +2695,10 @@
         </ns0:is>
       </ns0:c>
       <ns0:c r="D55" s="1" t="n">
-        <ns0:v>3.896036561907814e+39</ns0:v>
+        <ns0:v>1.03725479862186e+41</ns0:v>
       </ns0:c>
       <ns0:c r="E55" s="1" t="n">
-        <ns0:v>3.896036561907814e+39</ns0:v>
+        <ns0:v>1.03725479862186e+41</ns0:v>
       </ns0:c>
       <ns0:c r="F55" s="1" t="n">
         <ns0:v>1.031901272029505e+25</ns0:v>
@@ -2723,10 +2723,10 @@
         </ns0:is>
       </ns0:c>
       <ns0:c r="D56" s="1" t="n">
-        <ns0:v>1.163350283727174e+40</ns0:v>
+        <ns0:v>3.097226232608094e+41</ns0:v>
       </ns0:c>
       <ns0:c r="E56" s="1" t="n">
-        <ns0:v>1.163350283727174e+40</ns0:v>
+        <ns0:v>3.097226232608094e+41</ns0:v>
       </ns0:c>
       <ns0:c r="F56" s="1" t="n">
         <ns0:v>2.139750477680381e+25</ns0:v>
@@ -2751,10 +2751,10 @@
         </ns0:is>
       </ns0:c>
       <ns0:c r="D57" s="1" t="n">
-        <ns0:v>1.03725479862186e+41</ns0:v>
+        <ns0:v>2.761518020090726e+42</ns0:v>
       </ns0:c>
       <ns0:c r="E57" s="1" t="n">
-        <ns0:v>1.03725479862186e+41</ns0:v>
+        <ns0:v>2.761518020090726e+42</ns0:v>
       </ns0:c>
       <ns0:c r="F57" s="1" t="n">
         <ns0:v>9.200535394098201e+25</ns0:v>
@@ -2779,10 +2779,10 @@
         </ns0:is>
       </ns0:c>
       <ns0:c r="D58" s="1" t="n">
-        <ns0:v>3.976585948930645e+42</ns0:v>
+        <ns0:v>1.058699730384658e+44</ns0:v>
       </ns0:c>
       <ns0:c r="E58" s="1" t="n">
-        <ns0:v>3.976585948930645e+42</ns0:v>
+        <ns0:v>1.058699730384658e+44</ns0:v>
       </ns0:c>
       <ns0:c r="F58" s="1" t="n">
         <ns0:v>8.203289775151412e+26</ns0:v>
@@ -2807,10 +2807,10 @@
         </ns0:is>
       </ns0:c>
       <ns0:c r="D59" s="1" t="n">
-        <ns0:v>1.187402201813172e+43</ns0:v>
+        <ns0:v>3.161260455732902e+44</ns0:v>
       </ns0:c>
       <ns0:c r="E59" s="1" t="n">
-        <ns0:v>1.187402201813172e+43</ns0:v>
+        <ns0:v>3.161260455732902e+44</ns0:v>
       </ns0:c>
       <ns0:c r="F59" s="1" t="n">
         <ns0:v>1.701034167775397e+27</ns0:v>
@@ -2835,10 +2835,10 @@
         </ns0:is>
       </ns0:c>
       <ns0:c r="D60" s="1" t="n">
-        <ns0:v>3.545563976178901e+43</ns0:v>
+        <ns0:v>9.439473140651152e+44</ns0:v>
       </ns0:c>
       <ns0:c r="E60" s="1" t="n">
-        <ns0:v>3.545563976178901e+43</ns0:v>
+        <ns0:v>9.439473140651152e+44</ns0:v>
       </ns0:c>
       <ns0:c r="F60" s="1" t="n">
         <ns0:v>3.527264450299061e+27</ns0:v>
@@ -2863,10 +2863,10 @@
         </ns0:is>
       </ns0:c>
       <ns0:c r="D61" s="1" t="n">
-        <ns0:v>1.058699730384658e+44</ns0:v>
+        <ns0:v>2.818611576641408e+45</ns0:v>
       </ns0:c>
       <ns0:c r="E61" s="1" t="n">
-        <ns0:v>1.058699730384658e+44</ns0:v>
+        <ns0:v>2.818611576641408e+45</ns0:v>
       </ns0:c>
       <ns0:c r="F61" s="1" t="n">
         <ns0:v>7.314135564140134e+27</ns0:v>
@@ -2891,10 +2891,10 @@
         </ns0:is>
       </ns0:c>
       <ns0:c r="D62" s="1" t="n">
-        <ns0:v>9.43947314065115e+44</ns0:v>
+        <ns0:v>2.5131023941952e+46</ns0:v>
       </ns0:c>
       <ns0:c r="E62" s="1" t="n">
-        <ns0:v>9.43947314065115e+44</ns0:v>
+        <ns0:v>2.5131023941952e+46</ns0:v>
       </ns0:c>
       <ns0:c r="F62" s="1" t="n">
         <ns0:v>3.14494441464289e+28</ns0:v>
@@ -2919,10 +2919,10 @@
         </ns0:is>
       </ns0:c>
       <ns0:c r="D63" s="1" t="n">
-        <ns0:v>3.618867447641087e+46</ns0:v>
+        <ns0:v>9.634631415789515e+47</ns0:v>
       </ns0:c>
       <ns0:c r="E63" s="1" t="n">
-        <ns0:v>3.618867447641087e+46</ns0:v>
+        <ns0:v>9.634631415789515e+47</ns0:v>
       </ns0:c>
       <ns0:c r="F63" s="1" t="n">
         <ns0:v>2.804064030513767e+29</ns0:v>
@@ -2948,11 +2948,11 @@
       </ns0:c>
       <ns0:c r="D64" s="1">
         <ns0:f>ROUND(D63*10,0)</ns0:f>
-        <ns0:v>3.6188674476410877e+47</ns0:v>
+        <ns0:v>9.634631415789514e+48</ns0:v>
       </ns0:c>
       <ns0:c r="E64" s="1">
         <ns0:f>D64</ns0:f>
-        <ns0:v>3.6188674476410877e+47</ns0:v>
+        <ns0:v>9.634631415789514e+48</ns0:v>
       </ns0:c>
       <ns0:c r="F64" s="1">
         <ns0:f>ROUND(F63*1.4,-5)</ns0:f>
@@ -2979,11 +2979,11 @@
       </ns0:c>
       <ns0:c r="D65" s="1">
         <ns0:f>ROUND(D64*10,0)</ns0:f>
-        <ns0:v>3.6188674476410873e+48</ns0:v>
+        <ns0:v>9.634631415789515e+49</ns0:v>
       </ns0:c>
       <ns0:c r="E65" s="1">
         <ns0:f>D65</ns0:f>
-        <ns0:v>3.6188674476410873e+48</ns0:v>
+        <ns0:v>9.634631415789515e+49</ns0:v>
       </ns0:c>
       <ns0:c r="F65" s="1">
         <ns0:f>ROUND(F64*1.4,-5)</ns0:f>
@@ -3010,11 +3010,11 @@
       </ns0:c>
       <ns0:c r="D66" s="1">
         <ns0:f>ROUND(D65*10,0)</ns0:f>
-        <ns0:v>3.6188674476410876e+49</ns0:v>
+        <ns0:v>9.634631415789514e+50</ns0:v>
       </ns0:c>
       <ns0:c r="E66" s="1">
         <ns0:f>D66</ns0:f>
-        <ns0:v>3.6188674476410876e+49</ns0:v>
+        <ns0:v>9.634631415789514e+50</ns0:v>
       </ns0:c>
       <ns0:c r="F66" s="1">
         <ns0:f>ROUND(F65*1.4,-5)</ns0:f>
@@ -3041,11 +3041,11 @@
       </ns0:c>
       <ns0:c r="D67" s="1">
         <ns0:f>ROUND(D66*10,0)</ns0:f>
-        <ns0:v>3.6188674476410874e+50</ns0:v>
+        <ns0:v>9.634631415789515e+51</ns0:v>
       </ns0:c>
       <ns0:c r="E67" s="1">
         <ns0:f>D67</ns0:f>
-        <ns0:v>3.6188674476410874e+50</ns0:v>
+        <ns0:v>9.634631415789515e+51</ns0:v>
       </ns0:c>
       <ns0:c r="F67" s="1">
         <ns0:f>ROUND(F66*1.4,-5)</ns0:f>
@@ -3072,11 +3072,11 @@
       </ns0:c>
       <ns0:c r="D68" s="1">
         <ns0:f>ROUND(D67*10,0)</ns0:f>
-        <ns0:v>3.6188674476410876e+51</ns0:v>
+        <ns0:v>9.634631415789515e+52</ns0:v>
       </ns0:c>
       <ns0:c r="E68" s="1">
         <ns0:f>D68</ns0:f>
-        <ns0:v>3.6188674476410876e+51</ns0:v>
+        <ns0:v>9.634631415789515e+52</ns0:v>
       </ns0:c>
       <ns0:c r="F68" s="1">
         <ns0:f>ROUND(F67*1.4,-5)</ns0:f>
@@ -3103,11 +3103,11 @@
       </ns0:c>
       <ns0:c r="D69" s="1">
         <ns0:f>ROUND(D68*10,0)</ns0:f>
-        <ns0:v>3.6188674476410876e+52</ns0:v>
+        <ns0:v>9.634631415789514e+53</ns0:v>
       </ns0:c>
       <ns0:c r="E69" s="1">
         <ns0:f>D69</ns0:f>
-        <ns0:v>3.6188674476410876e+52</ns0:v>
+        <ns0:v>9.634631415789514e+53</ns0:v>
       </ns0:c>
       <ns0:c r="F69" s="1">
         <ns0:f>ROUND(F68*1.4,-5)</ns0:f>
@@ -3134,11 +3134,11 @@
       </ns0:c>
       <ns0:c r="D70" s="1">
         <ns0:f>ROUND(D69*10,0)</ns0:f>
-        <ns0:v>3.6188674476410878e+53</ns0:v>
+        <ns0:v>9.634631415789514e+54</ns0:v>
       </ns0:c>
       <ns0:c r="E70" s="1">
         <ns0:f>D70</ns0:f>
-        <ns0:v>3.6188674476410878e+53</ns0:v>
+        <ns0:v>9.634631415789514e+54</ns0:v>
       </ns0:c>
       <ns0:c r="F70" s="1">
         <ns0:f>ROUND(F69*1.4,-5)</ns0:f>
@@ -3165,11 +3165,11 @@
       </ns0:c>
       <ns0:c r="D71" s="1">
         <ns0:f>ROUND(D70*10,0)</ns0:f>
-        <ns0:v>3.6188674476410876e+54</ns0:v>
+        <ns0:v>9.634631415789515e+55</ns0:v>
       </ns0:c>
       <ns0:c r="E71" s="1">
         <ns0:f>D71</ns0:f>
-        <ns0:v>3.6188674476410876e+54</ns0:v>
+        <ns0:v>9.634631415789515e+55</ns0:v>
       </ns0:c>
       <ns0:c r="F71" s="1">
         <ns0:f>ROUND(F70*1.4,-5)</ns0:f>
@@ -3196,11 +3196,11 @@
       </ns0:c>
       <ns0:c r="D72" s="1">
         <ns0:f>ROUND(D71*10,0)</ns0:f>
-        <ns0:v>3.6188674476410875e+55</ns0:v>
+        <ns0:v>9.634631415789514e+56</ns0:v>
       </ns0:c>
       <ns0:c r="E72" s="1">
         <ns0:f>D72</ns0:f>
-        <ns0:v>3.6188674476410875e+55</ns0:v>
+        <ns0:v>9.634631415789514e+56</ns0:v>
       </ns0:c>
       <ns0:c r="F72" s="1">
         <ns0:f>ROUND(F71*1.4,-5)</ns0:f>
@@ -3227,11 +3227,11 @@
       </ns0:c>
       <ns0:c r="D73" s="1">
         <ns0:f>ROUND(D72*10,0)</ns0:f>
-        <ns0:v>3.6188674476410876e+56</ns0:v>
+        <ns0:v>9.634631415789514e+57</ns0:v>
       </ns0:c>
       <ns0:c r="E73" s="1">
         <ns0:f>D73</ns0:f>
-        <ns0:v>3.6188674476410876e+56</ns0:v>
+        <ns0:v>9.634631415789514e+57</ns0:v>
       </ns0:c>
       <ns0:c r="F73" s="1">
         <ns0:f>ROUND(F72*1.4,-5)</ns0:f>
@@ -3258,11 +3258,11 @@
       </ns0:c>
       <ns0:c r="D74" s="1">
         <ns0:f>ROUND(D73*10,0)</ns0:f>
-        <ns0:v>3.6188674476410876e+57</ns0:v>
+        <ns0:v>9.634631415789514e+58</ns0:v>
       </ns0:c>
       <ns0:c r="E74" s="1">
         <ns0:f>D74</ns0:f>
-        <ns0:v>3.6188674476410876e+57</ns0:v>
+        <ns0:v>9.634631415789514e+58</ns0:v>
       </ns0:c>
       <ns0:c r="F74" s="1">
         <ns0:f>ROUND(F73*1.4,-5)</ns0:f>
@@ -3290,11 +3290,11 @@
       </ns0:c>
       <ns0:c r="D75" s="1">
         <ns0:f>ROUND(D74*10,0)</ns0:f>
-        <ns0:v>3.6188674476410877e+58</ns0:v>
+        <ns0:v>9.634631415789515e+59</ns0:v>
       </ns0:c>
       <ns0:c r="E75" s="1">
         <ns0:f>D75</ns0:f>
-        <ns0:v>3.6188674476410877e+58</ns0:v>
+        <ns0:v>9.634631415789515e+59</ns0:v>
       </ns0:c>
       <ns0:c r="F75" s="1">
         <ns0:f>ROUND(F74*1.4,-5)</ns0:f>
@@ -3322,11 +3322,11 @@
       </ns0:c>
       <ns0:c r="D76" s="1">
         <ns0:f>ROUND(D75*10,0)</ns0:f>
-        <ns0:v>3.6188674476410875e+59</ns0:v>
+        <ns0:v>9.634631415789514e+60</ns0:v>
       </ns0:c>
       <ns0:c r="E76" s="1">
         <ns0:f>D76</ns0:f>
-        <ns0:v>3.6188674476410875e+59</ns0:v>
+        <ns0:v>9.634631415789514e+60</ns0:v>
       </ns0:c>
       <ns0:c r="F76" s="1">
         <ns0:f>ROUND(F75*1.4,-5)</ns0:f>
@@ -3354,11 +3354,11 @@
       </ns0:c>
       <ns0:c r="D77" s="1">
         <ns0:f>ROUND(D76*10,0)</ns0:f>
-        <ns0:v>3.618867447641087e+60</ns0:v>
+        <ns0:v>9.634631415789515e+61</ns0:v>
       </ns0:c>
       <ns0:c r="E77" s="1">
         <ns0:f>D77</ns0:f>
-        <ns0:v>3.618867447641087e+60</ns0:v>
+        <ns0:v>9.634631415789515e+61</ns0:v>
       </ns0:c>
       <ns0:c r="F77" s="1">
         <ns0:f>ROUND(F76*1.4,-5)</ns0:f>
@@ -3386,11 +3386,11 @@
       </ns0:c>
       <ns0:c r="D78" s="1">
         <ns0:f>ROUND(D77*10,0)</ns0:f>
-        <ns0:v>3.6188674476410876e+61</ns0:v>
+        <ns0:v>9.634631415789515e+62</ns0:v>
       </ns0:c>
       <ns0:c r="E78" s="1">
         <ns0:f>D78</ns0:f>
-        <ns0:v>3.6188674476410876e+61</ns0:v>
+        <ns0:v>9.634631415789515e+62</ns0:v>
       </ns0:c>
       <ns0:c r="F78" s="1">
         <ns0:f>ROUND(F77*1.4,-5)</ns0:f>
@@ -3418,11 +3418,11 @@
       </ns0:c>
       <ns0:c r="D79" s="1">
         <ns0:f>ROUND(D78*10,0)</ns0:f>
-        <ns0:v>3.618867447641088e+62</ns0:v>
+        <ns0:v>9.634631415789514e+63</ns0:v>
       </ns0:c>
       <ns0:c r="E79" s="1">
         <ns0:f>D79</ns0:f>
-        <ns0:v>3.618867447641088e+62</ns0:v>
+        <ns0:v>9.634631415789514e+63</ns0:v>
       </ns0:c>
       <ns0:c r="F79" s="1">
         <ns0:f>ROUND(F78*1.4,-5)</ns0:f>
@@ -3450,11 +3450,11 @@
       </ns0:c>
       <ns0:c r="D80" s="1">
         <ns0:f>ROUND(D79*10,0)</ns0:f>
-        <ns0:v>3.618867447641088e+63</ns0:v>
+        <ns0:v>9.634631415789513e+64</ns0:v>
       </ns0:c>
       <ns0:c r="E80" s="1">
         <ns0:f>D80</ns0:f>
-        <ns0:v>3.618867447641088e+63</ns0:v>
+        <ns0:v>9.634631415789513e+64</ns0:v>
       </ns0:c>
       <ns0:c r="F80" s="1">
         <ns0:f>ROUND(F79*1.4,-5)</ns0:f>
@@ -3482,11 +3482,11 @@
       </ns0:c>
       <ns0:c r="D81" s="1">
         <ns0:f>ROUND(D80*10,0)</ns0:f>
-        <ns0:v>3.6188674476410876e+64</ns0:v>
+        <ns0:v>9.634631415789514e+65</ns0:v>
       </ns0:c>
       <ns0:c r="E81" s="1">
         <ns0:f>D81</ns0:f>
-        <ns0:v>3.6188674476410876e+64</ns0:v>
+        <ns0:v>9.634631415789514e+65</ns0:v>
       </ns0:c>
       <ns0:c r="F81" s="1">
         <ns0:f>ROUND(F80*1.4,-5)</ns0:f>
@@ -3514,11 +3514,11 @@
       </ns0:c>
       <ns0:c r="D82" s="1">
         <ns0:f>ROUND(D81*10,0)</ns0:f>
-        <ns0:v>3.6188674476410874e+65</ns0:v>
+        <ns0:v>9.634631415789514e+66</ns0:v>
       </ns0:c>
       <ns0:c r="E82" s="1">
         <ns0:f>D82</ns0:f>
-        <ns0:v>3.6188674476410874e+65</ns0:v>
+        <ns0:v>9.634631415789514e+66</ns0:v>
       </ns0:c>
       <ns0:c r="F82" s="1">
         <ns0:f>ROUND(F81*1.4,-5)</ns0:f>
@@ -3546,11 +3546,11 @@
       </ns0:c>
       <ns0:c r="D83" s="1">
         <ns0:f>ROUND(D82*10,0)</ns0:f>
-        <ns0:v>3.618867447641088e+66</ns0:v>
+        <ns0:v>9.634631415789514e+67</ns0:v>
       </ns0:c>
       <ns0:c r="E83" s="1">
         <ns0:f>D83</ns0:f>
-        <ns0:v>3.618867447641088e+66</ns0:v>
+        <ns0:v>9.634631415789514e+67</ns0:v>
       </ns0:c>
       <ns0:c r="F83" s="1">
         <ns0:f>ROUND(F82*1.4,-5)</ns0:f>
@@ -3578,11 +3578,11 @@
       </ns0:c>
       <ns0:c r="D84" s="1">
         <ns0:f>ROUND(D83*20,2-INT(LOG10(ABS(D83*20))))</ns0:f>
-        <ns0:v>7.24e+67</ns0:v>
+        <ns0:v>1.93e+69</ns0:v>
       </ns0:c>
       <ns0:c r="E84" s="1">
         <ns0:f>D84</ns0:f>
-        <ns0:v>7.24e+67</ns0:v>
+        <ns0:v>1.93e+69</ns0:v>
       </ns0:c>
       <ns0:c r="F84" s="1">
         <ns0:f>ROUND(F83*1.4,-5)</ns0:f>
@@ -3610,11 +3610,11 @@
       </ns0:c>
       <ns0:c r="D85" s="1">
         <ns0:f>ROUND(D84*20,2-INT(LOG10(ABS(D84*20))))</ns0:f>
-        <ns0:v>1.4500000000000001e+69</ns0:v>
+        <ns0:v>3.86e+70</ns0:v>
       </ns0:c>
       <ns0:c r="E85" s="1">
         <ns0:f>D85</ns0:f>
-        <ns0:v>1.4500000000000001e+69</ns0:v>
+        <ns0:v>3.86e+70</ns0:v>
       </ns0:c>
       <ns0:c r="F85" s="1">
         <ns0:f>ROUND(F84*1.4,-5)</ns0:f>
@@ -3642,11 +3642,11 @@
       </ns0:c>
       <ns0:c r="D86" s="1">
         <ns0:f>ROUND(D85*20,2-INT(LOG10(ABS(D85*20))))</ns0:f>
-        <ns0:v>2.9e+70</ns0:v>
+        <ns0:v>7.72e+71</ns0:v>
       </ns0:c>
       <ns0:c r="E86" s="1">
         <ns0:f>D86</ns0:f>
-        <ns0:v>2.9e+70</ns0:v>
+        <ns0:v>7.72e+71</ns0:v>
       </ns0:c>
       <ns0:c r="F86" s="1">
         <ns0:f>ROUND(F85*1.4,-5)</ns0:f>
@@ -3674,11 +3674,11 @@
       </ns0:c>
       <ns0:c r="D87" s="1">
         <ns0:f>ROUND(D86*20,2-INT(LOG10(ABS(D86*20))))</ns0:f>
-        <ns0:v>5.8e+71</ns0:v>
+        <ns0:v>1.54e+73</ns0:v>
       </ns0:c>
       <ns0:c r="E87" s="1">
         <ns0:f>D87</ns0:f>
-        <ns0:v>5.8e+71</ns0:v>
+        <ns0:v>1.54e+73</ns0:v>
       </ns0:c>
       <ns0:c r="F87" s="1">
         <ns0:f>ROUND(F86*1.4,-5)</ns0:f>
@@ -3706,11 +3706,11 @@
       </ns0:c>
       <ns0:c r="D88" s="1">
         <ns0:f>ROUND(D87*20,2-INT(LOG10(ABS(D87*20))))</ns0:f>
-        <ns0:v>1.16e+73</ns0:v>
+        <ns0:v>3.08e+74</ns0:v>
       </ns0:c>
       <ns0:c r="E88" s="1">
         <ns0:f>D88</ns0:f>
-        <ns0:v>1.16e+73</ns0:v>
+        <ns0:v>3.08e+74</ns0:v>
       </ns0:c>
       <ns0:c r="F88" s="1">
         <ns0:f>ROUND(F87*1.4,-5)</ns0:f>
@@ -3738,11 +3738,11 @@
       </ns0:c>
       <ns0:c r="D89" s="1">
         <ns0:f>ROUND(D88*20,2-INT(LOG10(ABS(D88*20))))</ns0:f>
-        <ns0:v>2.32e+74</ns0:v>
+        <ns0:v>6.16e+75</ns0:v>
       </ns0:c>
       <ns0:c r="E89" s="1">
         <ns0:f>D89</ns0:f>
-        <ns0:v>2.32e+74</ns0:v>
+        <ns0:v>6.16e+75</ns0:v>
       </ns0:c>
       <ns0:c r="F89" s="1">
         <ns0:f>ROUND(F88*1.4,-5)</ns0:f>
@@ -3770,11 +3770,11 @@
       </ns0:c>
       <ns0:c r="D90" s="1">
         <ns0:f>ROUND(D89*20,2-INT(LOG10(ABS(D89*20))))</ns0:f>
-        <ns0:v>4.64e+75</ns0:v>
+        <ns0:v>1.23e+77</ns0:v>
       </ns0:c>
       <ns0:c r="E90" s="1">
         <ns0:f>D90</ns0:f>
-        <ns0:v>4.64e+75</ns0:v>
+        <ns0:v>1.23e+77</ns0:v>
       </ns0:c>
       <ns0:c r="F90" s="1">
         <ns0:f>ROUND(F89*1.4,-5)</ns0:f>
@@ -3802,11 +3802,11 @@
       </ns0:c>
       <ns0:c r="D91" s="1">
         <ns0:f>ROUND(D90*20,2-INT(LOG10(ABS(D90*20))))</ns0:f>
-        <ns0:v>9.280000000000001e+76</ns0:v>
+        <ns0:v>2.46e+78</ns0:v>
       </ns0:c>
       <ns0:c r="E91" s="1">
         <ns0:f>D91</ns0:f>
-        <ns0:v>9.280000000000001e+76</ns0:v>
+        <ns0:v>2.46e+78</ns0:v>
       </ns0:c>
       <ns0:c r="F91" s="1">
         <ns0:f>ROUND(F90*1.4,-5)</ns0:f>
@@ -3834,11 +3834,11 @@
       </ns0:c>
       <ns0:c r="D92" s="1">
         <ns0:f>ROUND(D91*20,2-INT(LOG10(ABS(D91*20))))</ns0:f>
-        <ns0:v>1.86e+78</ns0:v>
+        <ns0:v>4.92e+79</ns0:v>
       </ns0:c>
       <ns0:c r="E92" s="1">
         <ns0:f>D92</ns0:f>
-        <ns0:v>1.86e+78</ns0:v>
+        <ns0:v>4.92e+79</ns0:v>
       </ns0:c>
       <ns0:c r="F92" s="1">
         <ns0:f>ROUND(F91*1.4,-5)</ns0:f>
@@ -3866,11 +3866,11 @@
       </ns0:c>
       <ns0:c r="D93" s="1">
         <ns0:f>ROUND(D92*20,2-INT(LOG10(ABS(D92*20))))</ns0:f>
-        <ns0:v>3.7200000000000005e+79</ns0:v>
+        <ns0:v>9.84e+80</ns0:v>
       </ns0:c>
       <ns0:c r="E93" s="1">
         <ns0:f>D93</ns0:f>
-        <ns0:v>3.7200000000000005e+79</ns0:v>
+        <ns0:v>9.84e+80</ns0:v>
       </ns0:c>
       <ns0:c r="F93" s="1">
         <ns0:f>ROUND(F92*1.4,-5)</ns0:f>
@@ -3898,11 +3898,11 @@
       </ns0:c>
       <ns0:c r="D94" s="1">
         <ns0:f>ROUND(D93*20,2-INT(LOG10(ABS(D93*20))))</ns0:f>
-        <ns0:v>7.44e+80</ns0:v>
+        <ns0:v>1.97e+82</ns0:v>
       </ns0:c>
       <ns0:c r="E94" s="1">
         <ns0:f>D94</ns0:f>
-        <ns0:v>7.44e+80</ns0:v>
+        <ns0:v>1.97e+82</ns0:v>
       </ns0:c>
       <ns0:c r="F94" s="1">
         <ns0:f>ROUND(F93*1.4,-5)</ns0:f>
@@ -3930,11 +3930,11 @@
       </ns0:c>
       <ns0:c r="D95" s="1">
         <ns0:f>ROUND(D94*20,2-INT(LOG10(ABS(D94*20))))</ns0:f>
-        <ns0:v>1.49e+82</ns0:v>
+        <ns0:v>3.94e+83</ns0:v>
       </ns0:c>
       <ns0:c r="E95" s="1">
         <ns0:f>D95</ns0:f>
-        <ns0:v>1.49e+82</ns0:v>
+        <ns0:v>3.94e+83</ns0:v>
       </ns0:c>
       <ns0:c r="F95" s="1">
         <ns0:f>ROUND(F94*1.4,-5)</ns0:f>
@@ -3962,11 +3962,11 @@
       </ns0:c>
       <ns0:c r="D96" s="1">
         <ns0:f>ROUND(D95*20,2-INT(LOG10(ABS(D95*20))))</ns0:f>
-        <ns0:v>2.98e+83</ns0:v>
+        <ns0:v>7.88e+84</ns0:v>
       </ns0:c>
       <ns0:c r="E96" s="1">
         <ns0:f>D96</ns0:f>
-        <ns0:v>2.98e+83</ns0:v>
+        <ns0:v>7.88e+84</ns0:v>
       </ns0:c>
       <ns0:c r="F96" s="1">
         <ns0:f>ROUND(F95*1.4,-5)</ns0:f>
@@ -3994,11 +3994,11 @@
       </ns0:c>
       <ns0:c r="D97" s="1">
         <ns0:f>ROUND(D96*20,2-INT(LOG10(ABS(D96*20))))</ns0:f>
-        <ns0:v>5.960000000000001e+84</ns0:v>
+        <ns0:v>1.58e+86</ns0:v>
       </ns0:c>
       <ns0:c r="E97" s="1">
         <ns0:f>D97</ns0:f>
-        <ns0:v>5.960000000000001e+84</ns0:v>
+        <ns0:v>1.58e+86</ns0:v>
       </ns0:c>
       <ns0:c r="F97" s="1">
         <ns0:f>ROUND(F96*1.4,-5)</ns0:f>
@@ -4026,11 +4026,11 @@
       </ns0:c>
       <ns0:c r="D98" s="1">
         <ns0:f>ROUND(D97*20,2-INT(LOG10(ABS(D97*20))))</ns0:f>
-        <ns0:v>1.19e+86</ns0:v>
+        <ns0:v>3.16e+87</ns0:v>
       </ns0:c>
       <ns0:c r="E98" s="1">
         <ns0:f>D98</ns0:f>
-        <ns0:v>1.19e+86</ns0:v>
+        <ns0:v>3.16e+87</ns0:v>
       </ns0:c>
       <ns0:c r="F98" s="1">
         <ns0:f>ROUND(F97*1.4,-5)</ns0:f>
@@ -4058,11 +4058,11 @@
       </ns0:c>
       <ns0:c r="D99" s="1">
         <ns0:f>ROUND(D98*20,2-INT(LOG10(ABS(D98*20))))</ns0:f>
-        <ns0:v>2.38e+87</ns0:v>
+        <ns0:v>6.32e+88</ns0:v>
       </ns0:c>
       <ns0:c r="E99" s="1">
         <ns0:f>D99</ns0:f>
-        <ns0:v>2.38e+87</ns0:v>
+        <ns0:v>6.32e+88</ns0:v>
       </ns0:c>
       <ns0:c r="F99" s="1">
         <ns0:f>ROUND(F98*1.4,-5)</ns0:f>
@@ -4090,11 +4090,11 @@
       </ns0:c>
       <ns0:c r="D100" s="1">
         <ns0:f>ROUND(D99*20,2-INT(LOG10(ABS(D99*20))))</ns0:f>
-        <ns0:v>4.76e+88</ns0:v>
+        <ns0:v>1.26e+90</ns0:v>
       </ns0:c>
       <ns0:c r="E100" s="1">
         <ns0:f>D100</ns0:f>
-        <ns0:v>4.76e+88</ns0:v>
+        <ns0:v>1.26e+90</ns0:v>
       </ns0:c>
       <ns0:c r="F100" s="1">
         <ns0:f>ROUND(F99*1.4,-5)</ns0:f>
@@ -4122,11 +4122,11 @@
       </ns0:c>
       <ns0:c r="D101" s="1">
         <ns0:f>ROUND(D100*20,2-INT(LOG10(ABS(D100*20))))</ns0:f>
-        <ns0:v>9.52e+89</ns0:v>
+        <ns0:v>2.52e+91</ns0:v>
       </ns0:c>
       <ns0:c r="E101" s="1">
         <ns0:f>D101</ns0:f>
-        <ns0:v>9.52e+89</ns0:v>
+        <ns0:v>2.52e+91</ns0:v>
       </ns0:c>
       <ns0:c r="F101" s="1">
         <ns0:f>ROUND(F100*1.4,-5)</ns0:f>
@@ -4154,11 +4154,11 @@
       </ns0:c>
       <ns0:c r="D102" s="1">
         <ns0:f>ROUND(D101*20,2-INT(LOG10(ABS(D101*20))))</ns0:f>
-        <ns0:v>1.9e+91</ns0:v>
+        <ns0:v>5.04e+92</ns0:v>
       </ns0:c>
       <ns0:c r="E102" s="1">
         <ns0:f>D102</ns0:f>
-        <ns0:v>1.9e+91</ns0:v>
+        <ns0:v>5.04e+92</ns0:v>
       </ns0:c>
       <ns0:c r="F102" s="1">
         <ns0:f>ROUND(F101*1.4,-5)</ns0:f>
@@ -4186,11 +4186,11 @@
       </ns0:c>
       <ns0:c r="D103" s="1">
         <ns0:f>ROUND(D102*20,2-INT(LOG10(ABS(D102*20))))</ns0:f>
-        <ns0:v>3.8e+92</ns0:v>
+        <ns0:v>1.01e+94</ns0:v>
       </ns0:c>
       <ns0:c r="E103" s="1">
         <ns0:f>D103</ns0:f>
-        <ns0:v>3.8e+92</ns0:v>
+        <ns0:v>1.01e+94</ns0:v>
       </ns0:c>
       <ns0:c r="F103" s="1">
         <ns0:f>ROUND(F102*1.4,-5)</ns0:f>
@@ -4218,11 +4218,11 @@
       </ns0:c>
       <ns0:c r="D104" s="1">
         <ns0:f>ROUND(D103*20,2-INT(LOG10(ABS(D103*20))))</ns0:f>
-        <ns0:v>7.6e+93</ns0:v>
+        <ns0:v>2.0200000000000002e+95</ns0:v>
       </ns0:c>
       <ns0:c r="E104" s="1">
         <ns0:f>D104</ns0:f>
-        <ns0:v>7.6e+93</ns0:v>
+        <ns0:v>2.0200000000000002e+95</ns0:v>
       </ns0:c>
       <ns0:c r="F104" s="1">
         <ns0:f>ROUND(F103*1.4,-5)</ns0:f>
@@ -4250,11 +4250,11 @@
       </ns0:c>
       <ns0:c r="D105" s="1">
         <ns0:f>ROUND(D104*20,2-INT(LOG10(ABS(D104*20))))</ns0:f>
-        <ns0:v>1.5200000000000001e+95</ns0:v>
+        <ns0:v>4.04e+96</ns0:v>
       </ns0:c>
       <ns0:c r="E105" s="1">
         <ns0:f>D105</ns0:f>
-        <ns0:v>1.5200000000000001e+95</ns0:v>
+        <ns0:v>4.04e+96</ns0:v>
       </ns0:c>
       <ns0:c r="F105" s="1">
         <ns0:f>ROUND(F104*1.4,-5)</ns0:f>
@@ -4282,11 +4282,11 @@
       </ns0:c>
       <ns0:c r="D106" s="1">
         <ns0:f>ROUND(D105*20,2-INT(LOG10(ABS(D105*20))))</ns0:f>
-        <ns0:v>3.04e+96</ns0:v>
+        <ns0:v>8.08e+97</ns0:v>
       </ns0:c>
       <ns0:c r="E106" s="1">
         <ns0:f>D106</ns0:f>
-        <ns0:v>3.04e+96</ns0:v>
+        <ns0:v>8.08e+97</ns0:v>
       </ns0:c>
       <ns0:c r="F106" s="1">
         <ns0:f>ROUND(F105*1.4,-5)</ns0:f>
@@ -4314,11 +4314,11 @@
       </ns0:c>
       <ns0:c r="D107" s="1">
         <ns0:f>ROUND(D106*20,2-INT(LOG10(ABS(D106*20))))</ns0:f>
-        <ns0:v>6.08e+97</ns0:v>
+        <ns0:v>1.62e+99</ns0:v>
       </ns0:c>
       <ns0:c r="E107" s="1">
         <ns0:f>D107</ns0:f>
-        <ns0:v>6.08e+97</ns0:v>
+        <ns0:v>1.62e+99</ns0:v>
       </ns0:c>
       <ns0:c r="F107" s="1">
         <ns0:f>ROUND(F106*1.4,-5)</ns0:f>
@@ -4346,11 +4346,11 @@
       </ns0:c>
       <ns0:c r="D108" s="1">
         <ns0:f>ROUND(D107*20,2-INT(LOG10(ABS(D107*20))))</ns0:f>
-        <ns0:v>1.22e+99</ns0:v>
+        <ns0:v>3.24e+100</ns0:v>
       </ns0:c>
       <ns0:c r="E108" s="1">
         <ns0:f>D108</ns0:f>
-        <ns0:v>1.22e+99</ns0:v>
+        <ns0:v>3.24e+100</ns0:v>
       </ns0:c>
       <ns0:c r="F108" s="1">
         <ns0:f>ROUND(F107*1.4,-5)</ns0:f>
@@ -4378,11 +4378,11 @@
       </ns0:c>
       <ns0:c r="D109" s="1">
         <ns0:f>ROUND(D108*20,2-INT(LOG10(ABS(D108*20))))</ns0:f>
-        <ns0:v>2.4400000000000003e+100</ns0:v>
+        <ns0:v>6.48e+101</ns0:v>
       </ns0:c>
       <ns0:c r="E109" s="1">
         <ns0:f>D109</ns0:f>
-        <ns0:v>2.4400000000000003e+100</ns0:v>
+        <ns0:v>6.48e+101</ns0:v>
       </ns0:c>
       <ns0:c r="F109" s="1">
         <ns0:f>ROUND(F108*1.4,-5)</ns0:f>
@@ -4410,11 +4410,11 @@
       </ns0:c>
       <ns0:c r="D110" s="1">
         <ns0:f>ROUND(D109*20,2-INT(LOG10(ABS(D109*20))))</ns0:f>
-        <ns0:v>4.88e+101</ns0:v>
+        <ns0:v>1.2999999999999999e+103</ns0:v>
       </ns0:c>
       <ns0:c r="E110" s="1">
         <ns0:f>D110</ns0:f>
-        <ns0:v>4.88e+101</ns0:v>
+        <ns0:v>1.2999999999999999e+103</ns0:v>
       </ns0:c>
       <ns0:c r="F110" s="1">
         <ns0:f>ROUND(F109*1.4,-5)</ns0:f>
@@ -4442,11 +4442,11 @@
       </ns0:c>
       <ns0:c r="D111" s="1">
         <ns0:f>ROUND(D110*20,2-INT(LOG10(ABS(D110*20))))</ns0:f>
-        <ns0:v>9.76e+102</ns0:v>
+        <ns0:v>2.6000000000000003e+104</ns0:v>
       </ns0:c>
       <ns0:c r="E111" s="1">
         <ns0:f>D111</ns0:f>
-        <ns0:v>9.76e+102</ns0:v>
+        <ns0:v>2.6000000000000003e+104</ns0:v>
       </ns0:c>
       <ns0:c r="F111" s="1">
         <ns0:f>ROUND(F110*1.4,-5)</ns0:f>
@@ -4474,11 +4474,11 @@
       </ns0:c>
       <ns0:c r="D112" s="1">
         <ns0:f>ROUND(D111*20,2-INT(LOG10(ABS(D111*20))))</ns0:f>
-        <ns0:v>1.95e+104</ns0:v>
+        <ns0:v>5.2e+105</ns0:v>
       </ns0:c>
       <ns0:c r="E112" s="1">
         <ns0:f>D112</ns0:f>
-        <ns0:v>1.95e+104</ns0:v>
+        <ns0:v>5.2e+105</ns0:v>
       </ns0:c>
       <ns0:c r="F112" s="1">
         <ns0:f>ROUND(F111*1.4,-5)</ns0:f>
@@ -4506,11 +4506,11 @@
       </ns0:c>
       <ns0:c r="D113" s="1">
         <ns0:f>ROUND(D112*20,2-INT(LOG10(ABS(D112*20))))</ns0:f>
-        <ns0:v>3.9000000000000003e+105</ns0:v>
+        <ns0:v>1.04e+107</ns0:v>
       </ns0:c>
       <ns0:c r="E113" s="1">
         <ns0:f>D113</ns0:f>
-        <ns0:v>3.9000000000000003e+105</ns0:v>
+        <ns0:v>1.04e+107</ns0:v>
       </ns0:c>
       <ns0:c r="F113" s="1">
         <ns0:f>ROUND(F112*1.4,-5)</ns0:f>
@@ -4538,11 +4538,11 @@
       </ns0:c>
       <ns0:c r="D114" s="1">
         <ns0:f>ROUND(D113*20,2-INT(LOG10(ABS(D113*20))))</ns0:f>
-        <ns0:v>7.800000000000001e+106</ns0:v>
+        <ns0:v>2.08e+108</ns0:v>
       </ns0:c>
       <ns0:c r="E114" s="1">
         <ns0:f>D114</ns0:f>
-        <ns0:v>7.800000000000001e+106</ns0:v>
+        <ns0:v>2.08e+108</ns0:v>
       </ns0:c>
       <ns0:c r="F114" s="1">
         <ns0:f>ROUND(F113*1.4,-5)</ns0:f>
@@ -4570,11 +4570,11 @@
       </ns0:c>
       <ns0:c r="D115" s="1">
         <ns0:f>ROUND(D114*20,2-INT(LOG10(ABS(D114*20))))</ns0:f>
-        <ns0:v>1.5600000000000002e+108</ns0:v>
+        <ns0:v>4.16e+109</ns0:v>
       </ns0:c>
       <ns0:c r="E115" s="1">
         <ns0:f>D115</ns0:f>
-        <ns0:v>1.5600000000000002e+108</ns0:v>
+        <ns0:v>4.16e+109</ns0:v>
       </ns0:c>
       <ns0:c r="F115" s="1">
         <ns0:f>ROUND(F114*1.4,-5)</ns0:f>
@@ -4602,11 +4602,11 @@
       </ns0:c>
       <ns0:c r="D116" s="1">
         <ns0:f>ROUND(D115*20,2-INT(LOG10(ABS(D115*20))))</ns0:f>
-        <ns0:v>3.12e+109</ns0:v>
+        <ns0:v>8.32e+110</ns0:v>
       </ns0:c>
       <ns0:c r="E116" s="1">
         <ns0:f>D116</ns0:f>
-        <ns0:v>3.12e+109</ns0:v>
+        <ns0:v>8.32e+110</ns0:v>
       </ns0:c>
       <ns0:c r="F116" s="1">
         <ns0:f>ROUND(F115*1.4,-5)</ns0:f>
@@ -4634,11 +4634,11 @@
       </ns0:c>
       <ns0:c r="D117" s="1">
         <ns0:f>ROUND(D116*20,2-INT(LOG10(ABS(D116*20))))</ns0:f>
-        <ns0:v>6.24e+110</ns0:v>
+        <ns0:v>1.66e+112</ns0:v>
       </ns0:c>
       <ns0:c r="E117" s="1">
         <ns0:f>D117</ns0:f>
-        <ns0:v>6.24e+110</ns0:v>
+        <ns0:v>1.66e+112</ns0:v>
       </ns0:c>
       <ns0:c r="F117" s="1">
         <ns0:f>ROUND(F116*1.4,-5)</ns0:f>
@@ -4666,11 +4666,11 @@
       </ns0:c>
       <ns0:c r="D118" s="1">
         <ns0:f>ROUND(D117*20,2-INT(LOG10(ABS(D117*20))))</ns0:f>
-        <ns0:v>1.25e+112</ns0:v>
+        <ns0:v>3.3199999999999995e+113</ns0:v>
       </ns0:c>
       <ns0:c r="E118" s="1">
         <ns0:f>D118</ns0:f>
-        <ns0:v>1.25e+112</ns0:v>
+        <ns0:v>3.3199999999999995e+113</ns0:v>
       </ns0:c>
       <ns0:c r="F118" s="1">
         <ns0:f>ROUND(F117*1.4,-5)</ns0:f>
@@ -4698,11 +4698,11 @@
       </ns0:c>
       <ns0:c r="D119" s="1">
         <ns0:f>ROUND(D118*20,2-INT(LOG10(ABS(D118*20))))</ns0:f>
-        <ns0:v>2.4999999999999997e+113</ns0:v>
+        <ns0:v>6.64e+114</ns0:v>
       </ns0:c>
       <ns0:c r="E119" s="1">
         <ns0:f>D119</ns0:f>
-        <ns0:v>2.4999999999999997e+113</ns0:v>
+        <ns0:v>6.64e+114</ns0:v>
       </ns0:c>
       <ns0:c r="F119" s="1">
         <ns0:f>ROUND(F118*1.4,-5)</ns0:f>
@@ -4730,11 +4730,11 @@
       </ns0:c>
       <ns0:c r="D120" s="1">
         <ns0:f>ROUND(D119*20,2-INT(LOG10(ABS(D119*20))))</ns0:f>
-        <ns0:v>5e+114</ns0:v>
+        <ns0:v>1.3299999999999999e+116</ns0:v>
       </ns0:c>
       <ns0:c r="E120" s="1">
         <ns0:f>D120</ns0:f>
-        <ns0:v>5e+114</ns0:v>
+        <ns0:v>1.3299999999999999e+116</ns0:v>
       </ns0:c>
       <ns0:c r="F120" s="1">
         <ns0:f>ROUND(F119*1.4,-5)</ns0:f>
@@ -4762,11 +4762,11 @@
       </ns0:c>
       <ns0:c r="D121" s="1">
         <ns0:f>ROUND(D120*20,2-INT(LOG10(ABS(D120*20))))</ns0:f>
-        <ns0:v>1e+116</ns0:v>
+        <ns0:v>2.66e+117</ns0:v>
       </ns0:c>
       <ns0:c r="E121" s="1">
         <ns0:f>D121</ns0:f>
-        <ns0:v>1e+116</ns0:v>
+        <ns0:v>2.66e+117</ns0:v>
       </ns0:c>
       <ns0:c r="F121" s="1">
         <ns0:f>ROUND(F120*1.4,-5)</ns0:f>
@@ -4794,11 +4794,11 @@
       </ns0:c>
       <ns0:c r="D122" s="1">
         <ns0:f>ROUND(D121*20,2-INT(LOG10(ABS(D121*20))))</ns0:f>
-        <ns0:v>1.9999999999999998e+117</ns0:v>
+        <ns0:v>5.32e+118</ns0:v>
       </ns0:c>
       <ns0:c r="E122" s="1">
         <ns0:f>D122</ns0:f>
-        <ns0:v>1.9999999999999998e+117</ns0:v>
+        <ns0:v>5.32e+118</ns0:v>
       </ns0:c>
       <ns0:c r="F122" s="1">
         <ns0:f>ROUND(F121*1.4,-5)</ns0:f>
@@ -4826,11 +4826,11 @@
       </ns0:c>
       <ns0:c r="D123" s="1">
         <ns0:f>ROUND(D122*20,2-INT(LOG10(ABS(D122*20))))</ns0:f>
-        <ns0:v>4e+118</ns0:v>
+        <ns0:v>1.06e+120</ns0:v>
       </ns0:c>
       <ns0:c r="E123" s="1">
         <ns0:f>D123</ns0:f>
-        <ns0:v>4e+118</ns0:v>
+        <ns0:v>1.06e+120</ns0:v>
       </ns0:c>
       <ns0:c r="F123" s="1">
         <ns0:f>ROUND(F122*1.4,-5)</ns0:f>
@@ -4858,11 +4858,11 @@
       </ns0:c>
       <ns0:c r="D124" s="1">
         <ns0:f>ROUND(D123*20,2-INT(LOG10(ABS(D123*20))))</ns0:f>
-        <ns0:v>8e+119</ns0:v>
+        <ns0:v>2.12e+121</ns0:v>
       </ns0:c>
       <ns0:c r="E124" s="1">
         <ns0:f>D124</ns0:f>
-        <ns0:v>8e+119</ns0:v>
+        <ns0:v>2.12e+121</ns0:v>
       </ns0:c>
       <ns0:c r="F124" s="1">
         <ns0:f>ROUND(F123*1.4,-5)</ns0:f>
@@ -4890,11 +4890,11 @@
       </ns0:c>
       <ns0:c r="D125" s="1">
         <ns0:f>ROUND(D124*20,2-INT(LOG10(ABS(D124*20))))</ns0:f>
-        <ns0:v>1.6e+121</ns0:v>
+        <ns0:v>4.24e+122</ns0:v>
       </ns0:c>
       <ns0:c r="E125" s="1">
         <ns0:f>D125</ns0:f>
-        <ns0:v>1.6e+121</ns0:v>
+        <ns0:v>4.24e+122</ns0:v>
       </ns0:c>
       <ns0:c r="F125" s="1">
         <ns0:f>ROUND(F124*1.4,-5)</ns0:f>
@@ -4922,11 +4922,11 @@
       </ns0:c>
       <ns0:c r="D126" s="1">
         <ns0:f>ROUND(D125*20,2-INT(LOG10(ABS(D125*20))))</ns0:f>
-        <ns0:v>3.2e+122</ns0:v>
+        <ns0:v>8.48e+123</ns0:v>
       </ns0:c>
       <ns0:c r="E126" s="1">
         <ns0:f>D126</ns0:f>
-        <ns0:v>3.2e+122</ns0:v>
+        <ns0:v>8.48e+123</ns0:v>
       </ns0:c>
       <ns0:c r="F126" s="1">
         <ns0:f>ROUND(F125*1.4,-5)</ns0:f>
@@ -4954,11 +4954,11 @@
       </ns0:c>
       <ns0:c r="D127" s="1">
         <ns0:f>ROUND(D126*20,2-INT(LOG10(ABS(D126*20))))</ns0:f>
-        <ns0:v>6.4e+123</ns0:v>
+        <ns0:v>1.7e+125</ns0:v>
       </ns0:c>
       <ns0:c r="E127" s="1">
         <ns0:f>D127</ns0:f>
-        <ns0:v>6.4e+123</ns0:v>
+        <ns0:v>1.7e+125</ns0:v>
       </ns0:c>
       <ns0:c r="F127" s="1">
         <ns0:f>ROUND(F126*1.4,-5)</ns0:f>
@@ -4986,11 +4986,11 @@
       </ns0:c>
       <ns0:c r="D128" s="1">
         <ns0:f>ROUND(D127*20,2-INT(LOG10(ABS(D127*20))))</ns0:f>
-        <ns0:v>1.28e+125</ns0:v>
+        <ns0:v>3.4000000000000005e+126</ns0:v>
       </ns0:c>
       <ns0:c r="E128" s="1">
         <ns0:f>D128</ns0:f>
-        <ns0:v>1.28e+125</ns0:v>
+        <ns0:v>3.4000000000000005e+126</ns0:v>
       </ns0:c>
       <ns0:c r="F128" s="1">
         <ns0:f>ROUND(F127*1.4,-5)</ns0:f>
@@ -5018,11 +5018,11 @@
       </ns0:c>
       <ns0:c r="D129" s="1">
         <ns0:f>ROUND(D128*20,2-INT(LOG10(ABS(D128*20))))</ns0:f>
-        <ns0:v>2.5600000000000002e+126</ns0:v>
+        <ns0:v>6.8e+127</ns0:v>
       </ns0:c>
       <ns0:c r="E129" s="1">
         <ns0:f>D129</ns0:f>
-        <ns0:v>2.5600000000000002e+126</ns0:v>
+        <ns0:v>6.8e+127</ns0:v>
       </ns0:c>
       <ns0:c r="F129" s="1">
         <ns0:f>ROUND(F128*1.4,-5)</ns0:f>
@@ -5050,11 +5050,11 @@
       </ns0:c>
       <ns0:c r="D130" s="1">
         <ns0:f>ROUND(D129*20,2-INT(LOG10(ABS(D129*20))))</ns0:f>
-        <ns0:v>5.12e+127</ns0:v>
+        <ns0:v>1.36e+129</ns0:v>
       </ns0:c>
       <ns0:c r="E130" s="1">
         <ns0:f>D130</ns0:f>
-        <ns0:v>5.12e+127</ns0:v>
+        <ns0:v>1.36e+129</ns0:v>
       </ns0:c>
       <ns0:c r="F130" s="1">
         <ns0:f>ROUND(F129*1.4,-5)</ns0:f>
@@ -5082,11 +5082,11 @@
       </ns0:c>
       <ns0:c r="D131" s="1">
         <ns0:f>ROUND(D130*20,2-INT(LOG10(ABS(D130*20))))</ns0:f>
-        <ns0:v>1.02e+129</ns0:v>
+        <ns0:v>2.7199999999999997e+130</ns0:v>
       </ns0:c>
       <ns0:c r="E131" s="1">
         <ns0:f>D131</ns0:f>
-        <ns0:v>1.02e+129</ns0:v>
+        <ns0:v>2.7199999999999997e+130</ns0:v>
       </ns0:c>
       <ns0:c r="F131" s="1">
         <ns0:f>ROUND(F130*1.4,-5)</ns0:f>
@@ -5114,11 +5114,11 @@
       </ns0:c>
       <ns0:c r="D132" s="1">
         <ns0:f>ROUND(D131*20,2-INT(LOG10(ABS(D131*20))))</ns0:f>
-        <ns0:v>2.04e+130</ns0:v>
+        <ns0:v>5.44e+131</ns0:v>
       </ns0:c>
       <ns0:c r="E132" s="1">
         <ns0:f>D132</ns0:f>
-        <ns0:v>2.04e+130</ns0:v>
+        <ns0:v>5.44e+131</ns0:v>
       </ns0:c>
       <ns0:c r="F132" s="1">
         <ns0:f>ROUND(F131*1.4,-5)</ns0:f>
@@ -5146,11 +5146,11 @@
       </ns0:c>
       <ns0:c r="D133" s="1">
         <ns0:f>ROUND(D132*20,2-INT(LOG10(ABS(D132*20))))</ns0:f>
-        <ns0:v>4.0800000000000005e+131</ns0:v>
+        <ns0:v>1.09e+133</ns0:v>
       </ns0:c>
       <ns0:c r="E133" s="1">
         <ns0:f>D133</ns0:f>
-        <ns0:v>4.0800000000000005e+131</ns0:v>
+        <ns0:v>1.09e+133</ns0:v>
       </ns0:c>
       <ns0:c r="F133" s="1">
         <ns0:f>ROUND(F132*1.4,-5)</ns0:f>
@@ -5178,11 +5178,11 @@
       </ns0:c>
       <ns0:c r="D134" s="1">
         <ns0:f>ROUND(D133*20,2-INT(LOG10(ABS(D133*20))))</ns0:f>
-        <ns0:v>8.159999999999999e+132</ns0:v>
+        <ns0:v>2.18e+134</ns0:v>
       </ns0:c>
       <ns0:c r="E134" s="1">
         <ns0:f>D134</ns0:f>
-        <ns0:v>8.159999999999999e+132</ns0:v>
+        <ns0:v>2.18e+134</ns0:v>
       </ns0:c>
       <ns0:c r="F134" s="1">
         <ns0:f>ROUND(F133*1.4,-5)</ns0:f>
@@ -5210,11 +5210,11 @@
       </ns0:c>
       <ns0:c r="D135" s="1">
         <ns0:f>ROUND(D134*20,2-INT(LOG10(ABS(D134*20))))</ns0:f>
-        <ns0:v>1.63e+134</ns0:v>
+        <ns0:v>4.36e+135</ns0:v>
       </ns0:c>
       <ns0:c r="E135" s="1">
         <ns0:f>D135</ns0:f>
-        <ns0:v>1.63e+134</ns0:v>
+        <ns0:v>4.36e+135</ns0:v>
       </ns0:c>
       <ns0:c r="F135" s="1">
         <ns0:f>ROUND(F134*1.4,-5)</ns0:f>
@@ -5242,11 +5242,11 @@
       </ns0:c>
       <ns0:c r="D136" s="1">
         <ns0:f>ROUND(D135*20,2-INT(LOG10(ABS(D135*20))))</ns0:f>
-        <ns0:v>3.26e+135</ns0:v>
+        <ns0:v>8.719999999999999e+136</ns0:v>
       </ns0:c>
       <ns0:c r="E136" s="1">
         <ns0:f>D136</ns0:f>
-        <ns0:v>3.26e+135</ns0:v>
+        <ns0:v>8.719999999999999e+136</ns0:v>
       </ns0:c>
       <ns0:c r="F136" s="1">
         <ns0:f>ROUND(F135*1.4,-5)</ns0:f>
@@ -5274,11 +5274,11 @@
       </ns0:c>
       <ns0:c r="D137" s="1">
         <ns0:f>ROUND(D136*20,2-INT(LOG10(ABS(D136*20))))</ns0:f>
-        <ns0:v>6.52e+136</ns0:v>
+        <ns0:v>1.74e+138</ns0:v>
       </ns0:c>
       <ns0:c r="E137" s="1">
         <ns0:f>D137</ns0:f>
-        <ns0:v>6.52e+136</ns0:v>
+        <ns0:v>1.74e+138</ns0:v>
       </ns0:c>
       <ns0:c r="F137" s="1">
         <ns0:f>ROUND(F136*1.4,-5)</ns0:f>
@@ -5306,11 +5306,11 @@
       </ns0:c>
       <ns0:c r="D138" s="1">
         <ns0:f>ROUND(D137*20,2-INT(LOG10(ABS(D137*20))))</ns0:f>
-        <ns0:v>1.3e+138</ns0:v>
+        <ns0:v>3.48e+139</ns0:v>
       </ns0:c>
       <ns0:c r="E138" s="1">
         <ns0:f>D138</ns0:f>
-        <ns0:v>1.3e+138</ns0:v>
+        <ns0:v>3.48e+139</ns0:v>
       </ns0:c>
       <ns0:c r="F138" s="1">
         <ns0:f>ROUND(F137*1.4,-5)</ns0:f>
@@ -5338,11 +5338,11 @@
       </ns0:c>
       <ns0:c r="D139" s="1">
         <ns0:f>ROUND(D138*20,2-INT(LOG10(ABS(D138*20))))</ns0:f>
-        <ns0:v>2.6e+139</ns0:v>
+        <ns0:v>6.96e+140</ns0:v>
       </ns0:c>
       <ns0:c r="E139" s="1">
         <ns0:f>D139</ns0:f>
-        <ns0:v>2.6e+139</ns0:v>
+        <ns0:v>6.96e+140</ns0:v>
       </ns0:c>
       <ns0:c r="F139" s="1">
         <ns0:f>ROUND(F138*1.4,-5)</ns0:f>
@@ -5370,11 +5370,11 @@
       </ns0:c>
       <ns0:c r="D140" s="1">
         <ns0:f>ROUND(D139*20,2-INT(LOG10(ABS(D139*20))))</ns0:f>
-        <ns0:v>5.199999999999999e+140</ns0:v>
+        <ns0:v>1.39e+142</ns0:v>
       </ns0:c>
       <ns0:c r="E140" s="1">
         <ns0:f>D140</ns0:f>
-        <ns0:v>5.199999999999999e+140</ns0:v>
+        <ns0:v>1.39e+142</ns0:v>
       </ns0:c>
       <ns0:c r="F140" s="1">
         <ns0:f>ROUND(F139*1.4,-5)</ns0:f>
@@ -5402,11 +5402,11 @@
       </ns0:c>
       <ns0:c r="D141" s="1">
         <ns0:f>ROUND(D140*20,2-INT(LOG10(ABS(D140*20))))</ns0:f>
-        <ns0:v>1.04e+142</ns0:v>
+        <ns0:v>2.78e+143</ns0:v>
       </ns0:c>
       <ns0:c r="E141" s="1">
         <ns0:f>D141</ns0:f>
-        <ns0:v>1.04e+142</ns0:v>
+        <ns0:v>2.78e+143</ns0:v>
       </ns0:c>
       <ns0:c r="F141" s="1">
         <ns0:f>ROUND(F140*1.4,-5)</ns0:f>
@@ -5434,11 +5434,11 @@
       </ns0:c>
       <ns0:c r="D142" s="1">
         <ns0:f>ROUND(D141*20,2-INT(LOG10(ABS(D141*20))))</ns0:f>
-        <ns0:v>2.0799999999999997e+143</ns0:v>
+        <ns0:v>5.56e+144</ns0:v>
       </ns0:c>
       <ns0:c r="E142" s="1">
         <ns0:f>D142</ns0:f>
-        <ns0:v>2.0799999999999997e+143</ns0:v>
+        <ns0:v>5.56e+144</ns0:v>
       </ns0:c>
       <ns0:c r="F142" s="1">
         <ns0:f>ROUND(F141*1.4,-5)</ns0:f>
@@ -5466,11 +5466,11 @@
       </ns0:c>
       <ns0:c r="D143" s="1">
         <ns0:f>ROUND(D142*20,2-INT(LOG10(ABS(D142*20))))</ns0:f>
-        <ns0:v>4.16e+144</ns0:v>
+        <ns0:v>1.1100000000000001e+146</ns0:v>
       </ns0:c>
       <ns0:c r="E143" s="1">
         <ns0:f>D143</ns0:f>
-        <ns0:v>4.16e+144</ns0:v>
+        <ns0:v>1.1100000000000001e+146</ns0:v>
       </ns0:c>
       <ns0:c r="F143" s="1">
         <ns0:f>ROUND(F142*1.4,-5)</ns0:f>
@@ -5498,11 +5498,11 @@
       </ns0:c>
       <ns0:c r="D144" s="1">
         <ns0:f>ROUND(D143*20,2-INT(LOG10(ABS(D143*20))))</ns0:f>
-        <ns0:v>8.320000000000001e+145</ns0:v>
+        <ns0:v>2.22e+147</ns0:v>
       </ns0:c>
       <ns0:c r="E144" s="1">
         <ns0:f>D144</ns0:f>
-        <ns0:v>8.320000000000001e+145</ns0:v>
+        <ns0:v>2.22e+147</ns0:v>
       </ns0:c>
       <ns0:c r="F144" s="1">
         <ns0:f>ROUND(F143*1.4,-5)</ns0:f>
@@ -5530,11 +5530,11 @@
       </ns0:c>
       <ns0:c r="D145" s="1">
         <ns0:f>ROUND(D144*20,2-INT(LOG10(ABS(D144*20))))</ns0:f>
-        <ns0:v>1.66e+147</ns0:v>
+        <ns0:v>4.44e+148</ns0:v>
       </ns0:c>
       <ns0:c r="E145" s="1">
         <ns0:f>D145</ns0:f>
-        <ns0:v>1.66e+147</ns0:v>
+        <ns0:v>4.44e+148</ns0:v>
       </ns0:c>
       <ns0:c r="F145" s="1">
         <ns0:f>ROUND(F144*1.4,-5)</ns0:f>
@@ -5562,11 +5562,11 @@
       </ns0:c>
       <ns0:c r="D146" s="1">
         <ns0:f>ROUND(D145*20,2-INT(LOG10(ABS(D145*20))))</ns0:f>
-        <ns0:v>3.32e+148</ns0:v>
+        <ns0:v>8.88e+149</ns0:v>
       </ns0:c>
       <ns0:c r="E146" s="1">
         <ns0:f>D146</ns0:f>
-        <ns0:v>3.32e+148</ns0:v>
+        <ns0:v>8.88e+149</ns0:v>
       </ns0:c>
       <ns0:c r="F146" s="1">
         <ns0:f>ROUND(F145*1.4,-5)</ns0:f>
@@ -5594,11 +5594,11 @@
       </ns0:c>
       <ns0:c r="D147" s="1">
         <ns0:f>ROUND(D146*20,2-INT(LOG10(ABS(D146*20))))</ns0:f>
-        <ns0:v>6.64e+149</ns0:v>
+        <ns0:v>1.78e+151</ns0:v>
       </ns0:c>
       <ns0:c r="E147" s="1">
         <ns0:f>D147</ns0:f>
-        <ns0:v>6.64e+149</ns0:v>
+        <ns0:v>1.78e+151</ns0:v>
       </ns0:c>
       <ns0:c r="F147" s="1">
         <ns0:f>ROUND(F146*1.4,-5)</ns0:f>
@@ -5626,11 +5626,11 @@
       </ns0:c>
       <ns0:c r="D148" s="1">
         <ns0:f>ROUND(D147*20,2-INT(LOG10(ABS(D147*20))))</ns0:f>
-        <ns0:v>1.33e+151</ns0:v>
+        <ns0:v>3.5599999999999998e+152</ns0:v>
       </ns0:c>
       <ns0:c r="E148" s="1">
         <ns0:f>D148</ns0:f>
-        <ns0:v>1.33e+151</ns0:v>
+        <ns0:v>3.5599999999999998e+152</ns0:v>
       </ns0:c>
       <ns0:c r="F148" s="1">
         <ns0:f>ROUND(F147*1.4,-5)</ns0:f>
@@ -5658,11 +5658,11 @@
       </ns0:c>
       <ns0:c r="D149" s="1">
         <ns0:f>ROUND(D148*20,2-INT(LOG10(ABS(D148*20))))</ns0:f>
-        <ns0:v>2.66e+152</ns0:v>
+        <ns0:v>7.12e+153</ns0:v>
       </ns0:c>
       <ns0:c r="E149" s="1">
         <ns0:f>D149</ns0:f>
-        <ns0:v>2.66e+152</ns0:v>
+        <ns0:v>7.12e+153</ns0:v>
       </ns0:c>
       <ns0:c r="F149" s="1">
         <ns0:f>ROUND(F148*1.4,-5)</ns0:f>
@@ -5690,11 +5690,11 @@
       </ns0:c>
       <ns0:c r="D150" s="1">
         <ns0:f>ROUND(D149*20,2-INT(LOG10(ABS(D149*20))))</ns0:f>
-        <ns0:v>5.3200000000000004e+153</ns0:v>
+        <ns0:v>1.42e+155</ns0:v>
       </ns0:c>
       <ns0:c r="E150" s="1">
         <ns0:f>D150</ns0:f>
-        <ns0:v>5.3200000000000004e+153</ns0:v>
+        <ns0:v>1.42e+155</ns0:v>
       </ns0:c>
       <ns0:c r="F150" s="1">
         <ns0:f>ROUND(F149*1.4,-5)</ns0:f>
@@ -5722,11 +5722,11 @@
       </ns0:c>
       <ns0:c r="D151" s="1">
         <ns0:f>ROUND(D150*20,2-INT(LOG10(ABS(D150*20))))</ns0:f>
-        <ns0:v>1.0599999999999999e+155</ns0:v>
+        <ns0:v>2.84e+156</ns0:v>
       </ns0:c>
       <ns0:c r="E151" s="1">
         <ns0:f>D151</ns0:f>
-        <ns0:v>1.0599999999999999e+155</ns0:v>
+        <ns0:v>2.84e+156</ns0:v>
       </ns0:c>
       <ns0:c r="F151" s="1">
         <ns0:f>ROUND(F150*1.4,-5)</ns0:f>
@@ -5754,11 +5754,11 @@
       </ns0:c>
       <ns0:c r="D152" s="1">
         <ns0:f>ROUND(D151*20,2-INT(LOG10(ABS(D151*20))))</ns0:f>
-        <ns0:v>2.1200000000000002e+156</ns0:v>
+        <ns0:v>5.68e+157</ns0:v>
       </ns0:c>
       <ns0:c r="E152" s="1">
         <ns0:f>D152</ns0:f>
-        <ns0:v>2.1200000000000002e+156</ns0:v>
+        <ns0:v>5.68e+157</ns0:v>
       </ns0:c>
       <ns0:c r="F152" s="1">
         <ns0:f>ROUND(F151*1.4,-5)</ns0:f>
@@ -5786,11 +5786,11 @@
       </ns0:c>
       <ns0:c r="D153" s="1">
         <ns0:f>ROUND(D152*20,2-INT(LOG10(ABS(D152*20))))</ns0:f>
-        <ns0:v>4.24e+157</ns0:v>
+        <ns0:v>1.14e+159</ns0:v>
       </ns0:c>
       <ns0:c r="E153" s="1">
         <ns0:f>D153</ns0:f>
-        <ns0:v>4.24e+157</ns0:v>
+        <ns0:v>1.14e+159</ns0:v>
       </ns0:c>
       <ns0:c r="F153" s="1">
         <ns0:f>ROUND(F152*1.4,-5)</ns0:f>
@@ -5818,11 +5818,11 @@
       </ns0:c>
       <ns0:c r="D154" s="1">
         <ns0:f>ROUND(D153*20,2-INT(LOG10(ABS(D153*20))))</ns0:f>
-        <ns0:v>8.48e+158</ns0:v>
+        <ns0:v>2.28e+160</ns0:v>
       </ns0:c>
       <ns0:c r="E154" s="1">
         <ns0:f>D154</ns0:f>
-        <ns0:v>8.48e+158</ns0:v>
+        <ns0:v>2.28e+160</ns0:v>
       </ns0:c>
       <ns0:c r="F154" s="1">
         <ns0:f>ROUND(F153*1.4,-5)</ns0:f>
@@ -5850,11 +5850,11 @@
       </ns0:c>
       <ns0:c r="D155" s="1">
         <ns0:f>ROUND(D154*20,2-INT(LOG10(ABS(D154*20))))</ns0:f>
-        <ns0:v>1.6999999999999998e+160</ns0:v>
+        <ns0:v>4.56e+161</ns0:v>
       </ns0:c>
       <ns0:c r="E155" s="1">
         <ns0:f>D155</ns0:f>
-        <ns0:v>1.6999999999999998e+160</ns0:v>
+        <ns0:v>4.56e+161</ns0:v>
       </ns0:c>
       <ns0:c r="F155" s="1">
         <ns0:f>ROUND(F154*1.4,-5)</ns0:f>
@@ -5882,11 +5882,11 @@
       </ns0:c>
       <ns0:c r="D156" s="1">
         <ns0:f>ROUND(D155*20,2-INT(LOG10(ABS(D155*20))))</ns0:f>
-        <ns0:v>3.4e+161</ns0:v>
+        <ns0:v>9.12e+162</ns0:v>
       </ns0:c>
       <ns0:c r="E156" s="1">
         <ns0:f>D156</ns0:f>
-        <ns0:v>3.4e+161</ns0:v>
+        <ns0:v>9.12e+162</ns0:v>
       </ns0:c>
       <ns0:c r="F156" s="1">
         <ns0:f>ROUND(F155*1.4,-5)</ns0:f>
@@ -5914,11 +5914,11 @@
       </ns0:c>
       <ns0:c r="D157" s="1">
         <ns0:f>ROUND(D156*20,2-INT(LOG10(ABS(D156*20))))</ns0:f>
-        <ns0:v>6.8e+162</ns0:v>
+        <ns0:v>1.82e+164</ns0:v>
       </ns0:c>
       <ns0:c r="E157" s="1">
         <ns0:f>D157</ns0:f>
-        <ns0:v>6.8e+162</ns0:v>
+        <ns0:v>1.82e+164</ns0:v>
       </ns0:c>
       <ns0:c r="F157" s="1">
         <ns0:f>ROUND(F156*1.4,-5)</ns0:f>
@@ -5946,11 +5946,11 @@
       </ns0:c>
       <ns0:c r="D158" s="1">
         <ns0:f>ROUND(D157*20,2-INT(LOG10(ABS(D157*20))))</ns0:f>
-        <ns0:v>1.36e+164</ns0:v>
+        <ns0:v>3.6400000000000005e+165</ns0:v>
       </ns0:c>
       <ns0:c r="E158" s="1">
         <ns0:f>D158</ns0:f>
-        <ns0:v>1.36e+164</ns0:v>
+        <ns0:v>3.6400000000000005e+165</ns0:v>
       </ns0:c>
       <ns0:c r="F158" s="1">
         <ns0:f>ROUND(F157*1.4,-5)</ns0:f>
@@ -5978,11 +5978,11 @@
       </ns0:c>
       <ns0:c r="D159" s="1">
         <ns0:f>ROUND(D158*20,2-INT(LOG10(ABS(D158*20))))</ns0:f>
-        <ns0:v>2.72e+165</ns0:v>
+        <ns0:v>7.28e+166</ns0:v>
       </ns0:c>
       <ns0:c r="E159" s="1">
         <ns0:f>D159</ns0:f>
-        <ns0:v>2.72e+165</ns0:v>
+        <ns0:v>7.28e+166</ns0:v>
       </ns0:c>
       <ns0:c r="F159" s="1">
         <ns0:f>ROUND(F158*1.4,-5)</ns0:f>
@@ -6010,11 +6010,11 @@
       </ns0:c>
       <ns0:c r="D160" s="1">
         <ns0:f>ROUND(D159*20,2-INT(LOG10(ABS(D159*20))))</ns0:f>
-        <ns0:v>5.44e+166</ns0:v>
+        <ns0:v>1.46e+168</ns0:v>
       </ns0:c>
       <ns0:c r="E160" s="1">
         <ns0:f>D160</ns0:f>
-        <ns0:v>5.44e+166</ns0:v>
+        <ns0:v>1.46e+168</ns0:v>
       </ns0:c>
       <ns0:c r="F160" s="1">
         <ns0:f>ROUND(F159*1.4,-5)</ns0:f>
@@ -6042,11 +6042,11 @@
       </ns0:c>
       <ns0:c r="D161" s="1">
         <ns0:f>ROUND(D160*20,2-INT(LOG10(ABS(D160*20))))</ns0:f>
-        <ns0:v>1.09e+168</ns0:v>
+        <ns0:v>2.92e+169</ns0:v>
       </ns0:c>
       <ns0:c r="E161" s="1">
         <ns0:f>D161</ns0:f>
-        <ns0:v>1.09e+168</ns0:v>
+        <ns0:v>2.92e+169</ns0:v>
       </ns0:c>
       <ns0:c r="F161" s="1">
         <ns0:f>ROUND(F160*1.4,-5)</ns0:f>
@@ -6074,11 +6074,11 @@
       </ns0:c>
       <ns0:c r="D162" s="1">
         <ns0:f>ROUND(D161*20,2-INT(LOG10(ABS(D161*20))))</ns0:f>
-        <ns0:v>2.18e+169</ns0:v>
+        <ns0:v>5.84e+170</ns0:v>
       </ns0:c>
       <ns0:c r="E162" s="1">
         <ns0:f>D162</ns0:f>
-        <ns0:v>2.18e+169</ns0:v>
+        <ns0:v>5.84e+170</ns0:v>
       </ns0:c>
       <ns0:c r="F162" s="1">
         <ns0:f>ROUND(F161*1.4,-5)</ns0:f>
@@ -6106,11 +6106,11 @@
       </ns0:c>
       <ns0:c r="D163" s="1">
         <ns0:f>ROUND(D162*20,2-INT(LOG10(ABS(D162*20))))</ns0:f>
-        <ns0:v>4.36e+170</ns0:v>
+        <ns0:v>1.17e+172</ns0:v>
       </ns0:c>
       <ns0:c r="E163" s="1">
         <ns0:f>D163</ns0:f>
-        <ns0:v>4.36e+170</ns0:v>
+        <ns0:v>1.17e+172</ns0:v>
       </ns0:c>
       <ns0:c r="F163" s="1">
         <ns0:f>ROUND(F162*1.4,-5)</ns0:f>
@@ -6138,11 +6138,11 @@
       </ns0:c>
       <ns0:c r="D164" s="1">
         <ns0:f>ROUND(D163*20,2-INT(LOG10(ABS(D163*20))))</ns0:f>
-        <ns0:v>8.72e+171</ns0:v>
+        <ns0:v>2.34e+173</ns0:v>
       </ns0:c>
       <ns0:c r="E164" s="1">
         <ns0:f>D164</ns0:f>
-        <ns0:v>8.72e+171</ns0:v>
+        <ns0:v>2.34e+173</ns0:v>
       </ns0:c>
       <ns0:c r="F164" s="1">
         <ns0:f>ROUND(F163*1.4,-5)</ns0:f>
@@ -6170,11 +6170,11 @@
       </ns0:c>
       <ns0:c r="D165" s="1">
         <ns0:f>ROUND(D164*20,2-INT(LOG10(ABS(D164*20))))</ns0:f>
-        <ns0:v>1.74e+173</ns0:v>
+        <ns0:v>4.68e+174</ns0:v>
       </ns0:c>
       <ns0:c r="E165" s="1">
         <ns0:f>D165</ns0:f>
-        <ns0:v>1.74e+173</ns0:v>
+        <ns0:v>4.68e+174</ns0:v>
       </ns0:c>
       <ns0:c r="F165" s="1">
         <ns0:f>ROUND(F164*1.4,-5)</ns0:f>
@@ -6202,11 +6202,11 @@
       </ns0:c>
       <ns0:c r="D166" s="1">
         <ns0:f>ROUND(D165*20,2-INT(LOG10(ABS(D165*20))))</ns0:f>
-        <ns0:v>3.48e+174</ns0:v>
+        <ns0:v>9.36e+175</ns0:v>
       </ns0:c>
       <ns0:c r="E166" s="1">
         <ns0:f>D166</ns0:f>
-        <ns0:v>3.48e+174</ns0:v>
+        <ns0:v>9.36e+175</ns0:v>
       </ns0:c>
       <ns0:c r="F166" s="1">
         <ns0:f>ROUND(F165*1.4,-5)</ns0:f>
@@ -6234,11 +6234,11 @@
       </ns0:c>
       <ns0:c r="D167" s="1">
         <ns0:f>ROUND(D166*20,2-INT(LOG10(ABS(D166*20))))</ns0:f>
-        <ns0:v>6.959999999999999e+175</ns0:v>
+        <ns0:v>1.87e+177</ns0:v>
       </ns0:c>
       <ns0:c r="E167" s="1">
         <ns0:f>D167</ns0:f>
-        <ns0:v>6.959999999999999e+175</ns0:v>
+        <ns0:v>1.87e+177</ns0:v>
       </ns0:c>
       <ns0:c r="F167" s="1">
         <ns0:f>ROUND(F166*1.4,-5)</ns0:f>
@@ -6266,11 +6266,11 @@
       </ns0:c>
       <ns0:c r="D168" s="1">
         <ns0:f>ROUND(D167*20,2-INT(LOG10(ABS(D167*20))))</ns0:f>
-        <ns0:v>1.39e+177</ns0:v>
+        <ns0:v>3.74e+178</ns0:v>
       </ns0:c>
       <ns0:c r="E168" s="1">
         <ns0:f>D168</ns0:f>
-        <ns0:v>1.39e+177</ns0:v>
+        <ns0:v>3.74e+178</ns0:v>
       </ns0:c>
       <ns0:c r="F168" s="1">
         <ns0:f>ROUND(F167*1.4,-5)</ns0:f>
@@ -6298,11 +6298,11 @@
       </ns0:c>
       <ns0:c r="D169" s="1">
         <ns0:f>ROUND(D168*20,2-INT(LOG10(ABS(D168*20))))</ns0:f>
-        <ns0:v>2.78e+178</ns0:v>
+        <ns0:v>7.48e+179</ns0:v>
       </ns0:c>
       <ns0:c r="E169" s="1">
         <ns0:f>D169</ns0:f>
-        <ns0:v>2.78e+178</ns0:v>
+        <ns0:v>7.48e+179</ns0:v>
       </ns0:c>
       <ns0:c r="F169" s="1">
         <ns0:f>ROUND(F168*1.4,-5)</ns0:f>
@@ -6330,11 +6330,11 @@
       </ns0:c>
       <ns0:c r="D170" s="1">
         <ns0:f>ROUND(D169*20,2-INT(LOG10(ABS(D169*20))))</ns0:f>
-        <ns0:v>5.56e+179</ns0:v>
+        <ns0:v>1.5e+181</ns0:v>
       </ns0:c>
       <ns0:c r="E170" s="1">
         <ns0:f>D170</ns0:f>
-        <ns0:v>5.56e+179</ns0:v>
+        <ns0:v>1.5e+181</ns0:v>
       </ns0:c>
       <ns0:c r="F170" s="1">
         <ns0:f>ROUND(F169*1.4,-5)</ns0:f>
@@ -6362,11 +6362,11 @@
       </ns0:c>
       <ns0:c r="D171" s="1">
         <ns0:f>ROUND(D170*20,2-INT(LOG10(ABS(D170*20))))</ns0:f>
-        <ns0:v>1.11e+181</ns0:v>
+        <ns0:v>3e+182</ns0:v>
       </ns0:c>
       <ns0:c r="E171" s="1">
         <ns0:f>D171</ns0:f>
-        <ns0:v>1.11e+181</ns0:v>
+        <ns0:v>3e+182</ns0:v>
       </ns0:c>
       <ns0:c r="F171" s="1">
         <ns0:f>ROUND(F170*1.4,-5)</ns0:f>
@@ -6394,11 +6394,11 @@
       </ns0:c>
       <ns0:c r="D172" s="1">
         <ns0:f>ROUND(D171*20,2-INT(LOG10(ABS(D171*20))))</ns0:f>
-        <ns0:v>2.22e+182</ns0:v>
+        <ns0:v>6e+183</ns0:v>
       </ns0:c>
       <ns0:c r="E172" s="1">
         <ns0:f>D172</ns0:f>
-        <ns0:v>2.22e+182</ns0:v>
+        <ns0:v>6e+183</ns0:v>
       </ns0:c>
       <ns0:c r="F172" s="1">
         <ns0:f>ROUND(F171*1.4,-5)</ns0:f>
@@ -6426,11 +6426,11 @@
       </ns0:c>
       <ns0:c r="D173" s="1">
         <ns0:f>ROUND(D172*20,2-INT(LOG10(ABS(D172*20))))</ns0:f>
-        <ns0:v>4.44e+183</ns0:v>
+        <ns0:v>1.2e+185</ns0:v>
       </ns0:c>
       <ns0:c r="E173" s="1">
         <ns0:f>D173</ns0:f>
-        <ns0:v>4.44e+183</ns0:v>
+        <ns0:v>1.2e+185</ns0:v>
       </ns0:c>
       <ns0:c r="F173" s="1">
         <ns0:f>ROUND(F172*1.4,-5)</ns0:f>
@@ -6458,11 +6458,11 @@
       </ns0:c>
       <ns0:c r="D174" s="1">
         <ns0:f>ROUND(D173*20,2-INT(LOG10(ABS(D173*20))))</ns0:f>
-        <ns0:v>8.88e+184</ns0:v>
+        <ns0:v>2.4e+186</ns0:v>
       </ns0:c>
       <ns0:c r="E174" s="1">
         <ns0:f>D174</ns0:f>
-        <ns0:v>8.88e+184</ns0:v>
+        <ns0:v>2.4e+186</ns0:v>
       </ns0:c>
       <ns0:c r="F174" s="1">
         <ns0:f>ROUND(F173*1.4,-5)</ns0:f>
@@ -6490,11 +6490,11 @@
       </ns0:c>
       <ns0:c r="D175" s="1">
         <ns0:f>ROUND(D174*20,2-INT(LOG10(ABS(D174*20))))</ns0:f>
-        <ns0:v>1.7799999999999998e+186</ns0:v>
+        <ns0:v>4.8e+187</ns0:v>
       </ns0:c>
       <ns0:c r="E175" s="1">
         <ns0:f>D175</ns0:f>
-        <ns0:v>1.7799999999999998e+186</ns0:v>
+        <ns0:v>4.8e+187</ns0:v>
       </ns0:c>
       <ns0:c r="F175" s="1">
         <ns0:f>ROUND(F174*1.4,-5)</ns0:f>
@@ -6522,11 +6522,11 @@
       </ns0:c>
       <ns0:c r="D176" s="1">
         <ns0:f>ROUND(D175*20,2-INT(LOG10(ABS(D175*20))))</ns0:f>
-        <ns0:v>3.56e+187</ns0:v>
+        <ns0:v>9.600000000000001e+188</ns0:v>
       </ns0:c>
       <ns0:c r="E176" s="1">
         <ns0:f>D176</ns0:f>
-        <ns0:v>3.56e+187</ns0:v>
+        <ns0:v>9.600000000000001e+188</ns0:v>
       </ns0:c>
       <ns0:c r="F176" s="1">
         <ns0:f>ROUND(F175*1.4,-5)</ns0:f>
@@ -6554,11 +6554,11 @@
       </ns0:c>
       <ns0:c r="D177" s="1">
         <ns0:f>ROUND(D176*20,2-INT(LOG10(ABS(D176*20))))</ns0:f>
-        <ns0:v>7.12e+188</ns0:v>
+        <ns0:v>1.92e+190</ns0:v>
       </ns0:c>
       <ns0:c r="E177" s="1">
         <ns0:f>D177</ns0:f>
-        <ns0:v>7.12e+188</ns0:v>
+        <ns0:v>1.92e+190</ns0:v>
       </ns0:c>
       <ns0:c r="F177" s="1">
         <ns0:f>ROUND(F176*1.4,-5)</ns0:f>
@@ -6586,11 +6586,11 @@
       </ns0:c>
       <ns0:c r="D178" s="1">
         <ns0:f>ROUND(D177*20,2-INT(LOG10(ABS(D177*20))))</ns0:f>
-        <ns0:v>1.42e+190</ns0:v>
+        <ns0:v>3.84e+191</ns0:v>
       </ns0:c>
       <ns0:c r="E178" s="1">
         <ns0:f>D178</ns0:f>
-        <ns0:v>1.42e+190</ns0:v>
+        <ns0:v>3.84e+191</ns0:v>
       </ns0:c>
       <ns0:c r="F178" s="1">
         <ns0:f>ROUND(F177*1.4,-5)</ns0:f>
@@ -6618,11 +6618,11 @@
       </ns0:c>
       <ns0:c r="D179" s="1">
         <ns0:f>ROUND(D178*20,2-INT(LOG10(ABS(D178*20))))</ns0:f>
-        <ns0:v>2.84e+191</ns0:v>
+        <ns0:v>7.68e+192</ns0:v>
       </ns0:c>
       <ns0:c r="E179" s="1">
         <ns0:f>D179</ns0:f>
-        <ns0:v>2.84e+191</ns0:v>
+        <ns0:v>7.68e+192</ns0:v>
       </ns0:c>
       <ns0:c r="F179" s="1">
         <ns0:f>ROUND(F178*1.4,-5)</ns0:f>
@@ -6650,11 +6650,11 @@
       </ns0:c>
       <ns0:c r="D180" s="1">
         <ns0:f>ROUND(D179*20,2-INT(LOG10(ABS(D179*20))))</ns0:f>
-        <ns0:v>5.68e+192</ns0:v>
+        <ns0:v>1.54e+194</ns0:v>
       </ns0:c>
       <ns0:c r="E180" s="1">
         <ns0:f>D180</ns0:f>
-        <ns0:v>5.68e+192</ns0:v>
+        <ns0:v>1.54e+194</ns0:v>
       </ns0:c>
       <ns0:c r="F180" s="1">
         <ns0:f>ROUND(F179*1.4,-5)</ns0:f>
@@ -6682,11 +6682,11 @@
       </ns0:c>
       <ns0:c r="D181" s="1">
         <ns0:f>ROUND(D180*20,2-INT(LOG10(ABS(D180*20))))</ns0:f>
-        <ns0:v>1.1399999999999998e+194</ns0:v>
+        <ns0:v>3.08e+195</ns0:v>
       </ns0:c>
       <ns0:c r="E181" s="1">
         <ns0:f>D181</ns0:f>
-        <ns0:v>1.1399999999999998e+194</ns0:v>
+        <ns0:v>3.08e+195</ns0:v>
       </ns0:c>
       <ns0:c r="F181" s="1">
         <ns0:f>ROUND(F180*1.4,-5)</ns0:f>
@@ -6714,11 +6714,11 @@
       </ns0:c>
       <ns0:c r="D182" s="1">
         <ns0:f>ROUND(D181*20,2-INT(LOG10(ABS(D181*20))))</ns0:f>
-        <ns0:v>2.28e+195</ns0:v>
+        <ns0:v>6.16e+196</ns0:v>
       </ns0:c>
       <ns0:c r="E182" s="1">
         <ns0:f>D182</ns0:f>
-        <ns0:v>2.28e+195</ns0:v>
+        <ns0:v>6.16e+196</ns0:v>
       </ns0:c>
       <ns0:c r="F182" s="1">
         <ns0:f>ROUND(F181*1.4,-5)</ns0:f>
@@ -6746,11 +6746,11 @@
       </ns0:c>
       <ns0:c r="D183" s="1">
         <ns0:f>ROUND(D182*20,2-INT(LOG10(ABS(D182*20))))</ns0:f>
-        <ns0:v>4.56e+196</ns0:v>
+        <ns0:v>1.23e+198</ns0:v>
       </ns0:c>
       <ns0:c r="E183" s="1">
         <ns0:f>D183</ns0:f>
-        <ns0:v>4.56e+196</ns0:v>
+        <ns0:v>1.23e+198</ns0:v>
       </ns0:c>
       <ns0:c r="F183" s="1">
         <ns0:f>ROUND(F182*1.4,-5)</ns0:f>
@@ -6778,11 +6778,11 @@
       </ns0:c>
       <ns0:c r="D184" s="1">
         <ns0:f>ROUND(D183*20,2-INT(LOG10(ABS(D183*20))))</ns0:f>
-        <ns0:v>9.119999999999999e+197</ns0:v>
+        <ns0:v>2.46e+199</ns0:v>
       </ns0:c>
       <ns0:c r="E184" s="1">
         <ns0:f>D184</ns0:f>
-        <ns0:v>9.119999999999999e+197</ns0:v>
+        <ns0:v>2.46e+199</ns0:v>
       </ns0:c>
       <ns0:c r="F184" s="1">
         <ns0:f>ROUND(F183*1.4,-5)</ns0:f>
@@ -6810,11 +6810,11 @@
       </ns0:c>
       <ns0:c r="D185" s="1">
         <ns0:f>ROUND(D184*20,2-INT(LOG10(ABS(D184*20))))</ns0:f>
-        <ns0:v>1.8200000000000001e+199</ns0:v>
+        <ns0:v>4.920000000000001e+200</ns0:v>
       </ns0:c>
       <ns0:c r="E185" s="1">
         <ns0:f>D185</ns0:f>
-        <ns0:v>1.8200000000000001e+199</ns0:v>
+        <ns0:v>4.920000000000001e+200</ns0:v>
       </ns0:c>
       <ns0:c r="F185" s="1">
         <ns0:f>ROUND(F184*1.4,-5)</ns0:f>
@@ -6842,11 +6842,11 @@
       </ns0:c>
       <ns0:c r="D186" s="1">
         <ns0:f>ROUND(D185*20,2-INT(LOG10(ABS(D185*20))))</ns0:f>
-        <ns0:v>3.64e+200</ns0:v>
+        <ns0:v>9.84e+201</ns0:v>
       </ns0:c>
       <ns0:c r="E186" s="1">
         <ns0:f>D186</ns0:f>
-        <ns0:v>3.64e+200</ns0:v>
+        <ns0:v>9.84e+201</ns0:v>
       </ns0:c>
       <ns0:c r="F186" s="1">
         <ns0:f>ROUND(F185*1.4,-5)</ns0:f>
@@ -6874,11 +6874,11 @@
       </ns0:c>
       <ns0:c r="D187" s="1">
         <ns0:f>ROUND(D186*20,2-INT(LOG10(ABS(D186*20))))</ns0:f>
-        <ns0:v>7.28e+201</ns0:v>
+        <ns0:v>1.9700000000000003e+203</ns0:v>
       </ns0:c>
       <ns0:c r="E187" s="1">
         <ns0:f>D187</ns0:f>
-        <ns0:v>7.28e+201</ns0:v>
+        <ns0:v>1.9700000000000003e+203</ns0:v>
       </ns0:c>
       <ns0:c r="F187" s="1">
         <ns0:f>ROUND(F186*1.4,-5)</ns0:f>
@@ -6906,11 +6906,11 @@
       </ns0:c>
       <ns0:c r="D188" s="1">
         <ns0:f>ROUND(D187*20,2-INT(LOG10(ABS(D187*20))))</ns0:f>
-        <ns0:v>1.46e+203</ns0:v>
+        <ns0:v>3.94e+204</ns0:v>
       </ns0:c>
       <ns0:c r="E188" s="1">
         <ns0:f>D188</ns0:f>
-        <ns0:v>1.46e+203</ns0:v>
+        <ns0:v>3.94e+204</ns0:v>
       </ns0:c>
       <ns0:c r="F188" s="1">
         <ns0:f>ROUND(F187*1.4,-5)</ns0:f>
@@ -6938,11 +6938,11 @@
       </ns0:c>
       <ns0:c r="D189" s="1">
         <ns0:f>ROUND(D188*20,2-INT(LOG10(ABS(D188*20))))</ns0:f>
-        <ns0:v>2.9199999999999997e+204</ns0:v>
+        <ns0:v>7.8799999999999995e+205</ns0:v>
       </ns0:c>
       <ns0:c r="E189" s="1">
         <ns0:f>D189</ns0:f>
-        <ns0:v>2.9199999999999997e+204</ns0:v>
+        <ns0:v>7.8799999999999995e+205</ns0:v>
       </ns0:c>
       <ns0:c r="F189" s="1">
         <ns0:f>ROUND(F188*1.4,-5)</ns0:f>
@@ -6970,11 +6970,11 @@
       </ns0:c>
       <ns0:c r="D190" s="1">
         <ns0:f>ROUND(D189*20,2-INT(LOG10(ABS(D189*20))))</ns0:f>
-        <ns0:v>5.84e+205</ns0:v>
+        <ns0:v>1.58e+207</ns0:v>
       </ns0:c>
       <ns0:c r="E190" s="1">
         <ns0:f>D190</ns0:f>
-        <ns0:v>5.84e+205</ns0:v>
+        <ns0:v>1.58e+207</ns0:v>
       </ns0:c>
       <ns0:c r="F190" s="1">
         <ns0:f>ROUND(F189*1.4,-5)</ns0:f>
@@ -7002,11 +7002,11 @@
       </ns0:c>
       <ns0:c r="D191" s="1">
         <ns0:f>ROUND(D190*20,2-INT(LOG10(ABS(D190*20))))</ns0:f>
-        <ns0:v>1.17e+207</ns0:v>
+        <ns0:v>3.1599999999999997e+208</ns0:v>
       </ns0:c>
       <ns0:c r="E191" s="1">
         <ns0:f>D191</ns0:f>
-        <ns0:v>1.17e+207</ns0:v>
+        <ns0:v>3.1599999999999997e+208</ns0:v>
       </ns0:c>
       <ns0:c r="F191" s="1">
         <ns0:f>ROUND(F190*1.4,-5)</ns0:f>
@@ -7034,11 +7034,11 @@
       </ns0:c>
       <ns0:c r="D192" s="1">
         <ns0:f>ROUND(D191*20,2-INT(LOG10(ABS(D191*20))))</ns0:f>
-        <ns0:v>2.34e+208</ns0:v>
+        <ns0:v>6.320000000000001e+209</ns0:v>
       </ns0:c>
       <ns0:c r="E192" s="1">
         <ns0:f>D192</ns0:f>
-        <ns0:v>2.34e+208</ns0:v>
+        <ns0:v>6.320000000000001e+209</ns0:v>
       </ns0:c>
       <ns0:c r="F192" s="1">
         <ns0:f>ROUND(F191*1.4,-5)</ns0:f>
@@ -7066,11 +7066,11 @@
       </ns0:c>
       <ns0:c r="D193" s="1">
         <ns0:f>ROUND(D192*20,2-INT(LOG10(ABS(D192*20))))</ns0:f>
-        <ns0:v>4.68e+209</ns0:v>
+        <ns0:v>1.26e+211</ns0:v>
       </ns0:c>
       <ns0:c r="E193" s="1">
         <ns0:f>D193</ns0:f>
-        <ns0:v>4.68e+209</ns0:v>
+        <ns0:v>1.26e+211</ns0:v>
       </ns0:c>
       <ns0:c r="F193" s="1">
         <ns0:f>ROUND(F192*1.4,-5)</ns0:f>
@@ -7098,11 +7098,11 @@
       </ns0:c>
       <ns0:c r="D194" s="1">
         <ns0:f>ROUND(D193*20,2-INT(LOG10(ABS(D193*20))))</ns0:f>
-        <ns0:v>9.359999999999999e+210</ns0:v>
+        <ns0:v>2.5199999999999998e+212</ns0:v>
       </ns0:c>
       <ns0:c r="E194" s="1">
         <ns0:f>D194</ns0:f>
-        <ns0:v>9.359999999999999e+210</ns0:v>
+        <ns0:v>2.5199999999999998e+212</ns0:v>
       </ns0:c>
       <ns0:c r="F194" s="1">
         <ns0:f>ROUND(F193*1.4,-5)</ns0:f>
@@ -7130,11 +7130,11 @@
       </ns0:c>
       <ns0:c r="D195" s="1">
         <ns0:f>ROUND(D194*20,2-INT(LOG10(ABS(D194*20))))</ns0:f>
-        <ns0:v>1.87e+212</ns0:v>
+        <ns0:v>5.0399999999999996e+213</ns0:v>
       </ns0:c>
       <ns0:c r="E195" s="1">
         <ns0:f>D195</ns0:f>
-        <ns0:v>1.87e+212</ns0:v>
+        <ns0:v>5.0399999999999996e+213</ns0:v>
       </ns0:c>
       <ns0:c r="F195" s="1">
         <ns0:f>ROUND(F194*1.4,-5)</ns0:f>
@@ -7162,11 +7162,11 @@
       </ns0:c>
       <ns0:c r="D196" s="1">
         <ns0:f>ROUND(D195*20,2-INT(LOG10(ABS(D195*20))))</ns0:f>
-        <ns0:v>3.74e+213</ns0:v>
+        <ns0:v>1.01e+215</ns0:v>
       </ns0:c>
       <ns0:c r="E196" s="1">
         <ns0:f>D196</ns0:f>
-        <ns0:v>3.74e+213</ns0:v>
+        <ns0:v>1.01e+215</ns0:v>
       </ns0:c>
       <ns0:c r="F196" s="1">
         <ns0:f>ROUND(F195*1.4,-5)</ns0:f>
@@ -7194,11 +7194,11 @@
       </ns0:c>
       <ns0:c r="D197" s="1">
         <ns0:f>ROUND(D196*20,2-INT(LOG10(ABS(D196*20))))</ns0:f>
-        <ns0:v>7.48e+214</ns0:v>
+        <ns0:v>2.02e+216</ns0:v>
       </ns0:c>
       <ns0:c r="E197" s="1">
         <ns0:f>D197</ns0:f>
-        <ns0:v>7.48e+214</ns0:v>
+        <ns0:v>2.02e+216</ns0:v>
       </ns0:c>
       <ns0:c r="F197" s="1">
         <ns0:f>ROUND(F196*1.4,-5)</ns0:f>
@@ -7226,11 +7226,11 @@
       </ns0:c>
       <ns0:c r="D198" s="1">
         <ns0:f>ROUND(D197*20,2-INT(LOG10(ABS(D197*20))))</ns0:f>
-        <ns0:v>1.5000000000000002e+216</ns0:v>
+        <ns0:v>4.0399999999999997e+217</ns0:v>
       </ns0:c>
       <ns0:c r="E198" s="1">
         <ns0:f>D198</ns0:f>
-        <ns0:v>1.5000000000000002e+216</ns0:v>
+        <ns0:v>4.0399999999999997e+217</ns0:v>
       </ns0:c>
       <ns0:c r="F198" s="1">
         <ns0:f>ROUND(F197*1.4,-5)</ns0:f>
@@ -7258,11 +7258,11 @@
       </ns0:c>
       <ns0:c r="D199" s="1">
         <ns0:f>ROUND(D198*20,2-INT(LOG10(ABS(D198*20))))</ns0:f>
-        <ns0:v>3e+217</ns0:v>
+        <ns0:v>8.08e+218</ns0:v>
       </ns0:c>
       <ns0:c r="E199" s="1">
         <ns0:f>D199</ns0:f>
-        <ns0:v>3e+217</ns0:v>
+        <ns0:v>8.08e+218</ns0:v>
       </ns0:c>
       <ns0:c r="F199" s="1">
         <ns0:f>ROUND(F198*1.4,-5)</ns0:f>
@@ -7290,11 +7290,11 @@
       </ns0:c>
       <ns0:c r="D200" s="1">
         <ns0:f>ROUND(D199*20,2-INT(LOG10(ABS(D199*20))))</ns0:f>
-        <ns0:v>6e+218</ns0:v>
+        <ns0:v>1.62e+220</ns0:v>
       </ns0:c>
       <ns0:c r="E200" s="1">
         <ns0:f>D200</ns0:f>
-        <ns0:v>6e+218</ns0:v>
+        <ns0:v>1.62e+220</ns0:v>
       </ns0:c>
       <ns0:c r="F200" s="1">
         <ns0:f>ROUND(F199*1.4,-5)</ns0:f>
@@ -7322,11 +7322,11 @@
       </ns0:c>
       <ns0:c r="D201" s="1">
         <ns0:f>ROUND(D200*20,2-INT(LOG10(ABS(D200*20))))</ns0:f>
-        <ns0:v>1.2e+220</ns0:v>
+        <ns0:v>3.2399999999999997e+221</ns0:v>
       </ns0:c>
       <ns0:c r="E201" s="1">
         <ns0:f>D201</ns0:f>
-        <ns0:v>1.2e+220</ns0:v>
+        <ns0:v>3.2399999999999997e+221</ns0:v>
       </ns0:c>
       <ns0:c r="F201" s="1">
         <ns0:f>ROUND(F200*1.4,-5)</ns0:f>
@@ -7354,11 +7354,11 @@
       </ns0:c>
       <ns0:c r="D202" s="1">
         <ns0:f>ROUND(D201*20,2-INT(LOG10(ABS(D201*20))))</ns0:f>
-        <ns0:v>2.3999999999999998e+221</ns0:v>
+        <ns0:v>6.48e+222</ns0:v>
       </ns0:c>
       <ns0:c r="E202" s="1">
         <ns0:f>D202</ns0:f>
-        <ns0:v>2.3999999999999998e+221</ns0:v>
+        <ns0:v>6.48e+222</ns0:v>
       </ns0:c>
       <ns0:c r="F202" s="1">
         <ns0:f>ROUND(F201*1.4,-5)</ns0:f>
@@ -7386,11 +7386,11 @@
       </ns0:c>
       <ns0:c r="D203" s="1">
         <ns0:f>ROUND(D202*20,2-INT(LOG10(ABS(D202*20))))</ns0:f>
-        <ns0:v>4.8e+222</ns0:v>
+        <ns0:v>1.3e+224</ns0:v>
       </ns0:c>
       <ns0:c r="E203" s="1">
         <ns0:f>D203</ns0:f>
-        <ns0:v>4.8e+222</ns0:v>
+        <ns0:v>1.3e+224</ns0:v>
       </ns0:c>
       <ns0:c r="F203" s="1">
         <ns0:f>ROUND(F202*1.4,-5)</ns0:f>
@@ -7418,11 +7418,11 @@
       </ns0:c>
       <ns0:c r="D204" s="1">
         <ns0:f>ROUND(D203*20,2-INT(LOG10(ABS(D203*20))))</ns0:f>
-        <ns0:v>9.6e+223</ns0:v>
+        <ns0:v>2.6e+225</ns0:v>
       </ns0:c>
       <ns0:c r="E204" s="1">
         <ns0:f>D204</ns0:f>
-        <ns0:v>9.6e+223</ns0:v>
+        <ns0:v>2.6e+225</ns0:v>
       </ns0:c>
       <ns0:c r="F204" s="1">
         <ns0:f>ROUND(F203*1.4,-5)</ns0:f>
@@ -7450,11 +7450,11 @@
       </ns0:c>
       <ns0:c r="D205" s="1">
         <ns0:f>ROUND(D204*20,2-INT(LOG10(ABS(D204*20))))</ns0:f>
-        <ns0:v>1.92e+225</ns0:v>
+        <ns0:v>5.199999999999999e+226</ns0:v>
       </ns0:c>
       <ns0:c r="E205" s="1">
         <ns0:f>D205</ns0:f>
-        <ns0:v>1.92e+225</ns0:v>
+        <ns0:v>5.199999999999999e+226</ns0:v>
       </ns0:c>
       <ns0:c r="F205" s="1">
         <ns0:f>ROUND(F204*1.4,-5)</ns0:f>
@@ -7482,11 +7482,11 @@
       </ns0:c>
       <ns0:c r="D206" s="1">
         <ns0:f>ROUND(D205*20,2-INT(LOG10(ABS(D205*20))))</ns0:f>
-        <ns0:v>3.84e+226</ns0:v>
+        <ns0:v>1.0400000000000001e+228</ns0:v>
       </ns0:c>
       <ns0:c r="E206" s="1">
         <ns0:f>D206</ns0:f>
-        <ns0:v>3.84e+226</ns0:v>
+        <ns0:v>1.0400000000000001e+228</ns0:v>
       </ns0:c>
       <ns0:c r="F206" s="1">
         <ns0:f>ROUND(F205*1.4,-5)</ns0:f>
@@ -7514,11 +7514,11 @@
       </ns0:c>
       <ns0:c r="D207" s="1">
         <ns0:f>ROUND(D206*20,2-INT(LOG10(ABS(D206*20))))</ns0:f>
-        <ns0:v>7.68e+227</ns0:v>
+        <ns0:v>2.08e+229</ns0:v>
       </ns0:c>
       <ns0:c r="E207" s="1">
         <ns0:f>D207</ns0:f>
-        <ns0:v>7.68e+227</ns0:v>
+        <ns0:v>2.08e+229</ns0:v>
       </ns0:c>
       <ns0:c r="F207" s="1">
         <ns0:f>ROUND(F206*1.4,-5)</ns0:f>
@@ -7546,11 +7546,11 @@
       </ns0:c>
       <ns0:c r="D208" s="1">
         <ns0:f>ROUND(D207*20,2-INT(LOG10(ABS(D207*20))))</ns0:f>
-        <ns0:v>1.5400000000000002e+229</ns0:v>
+        <ns0:v>4.16e+230</ns0:v>
       </ns0:c>
       <ns0:c r="E208" s="1">
         <ns0:f>D208</ns0:f>
-        <ns0:v>1.5400000000000002e+229</ns0:v>
+        <ns0:v>4.16e+230</ns0:v>
       </ns0:c>
       <ns0:c r="F208" s="1">
         <ns0:f>ROUND(F207*1.4,-5)</ns0:f>
@@ -7578,11 +7578,11 @@
       </ns0:c>
       <ns0:c r="D209" s="1">
         <ns0:f>ROUND(D208*20,2-INT(LOG10(ABS(D208*20))))</ns0:f>
-        <ns0:v>3.0799999999999998e+230</ns0:v>
+        <ns0:v>8.32e+231</ns0:v>
       </ns0:c>
       <ns0:c r="E209" s="1">
         <ns0:f>D209</ns0:f>
-        <ns0:v>3.0799999999999998e+230</ns0:v>
+        <ns0:v>8.32e+231</ns0:v>
       </ns0:c>
       <ns0:c r="F209" s="1">
         <ns0:f>ROUND(F208*1.4,-5)</ns0:f>
@@ -7610,11 +7610,11 @@
       </ns0:c>
       <ns0:c r="D210" s="1">
         <ns0:f>ROUND(D209*20,2-INT(LOG10(ABS(D209*20))))</ns0:f>
-        <ns0:v>6.16e+231</ns0:v>
+        <ns0:v>1.66e+233</ns0:v>
       </ns0:c>
       <ns0:c r="E210" s="1">
         <ns0:f>D210</ns0:f>
-        <ns0:v>6.16e+231</ns0:v>
+        <ns0:v>1.66e+233</ns0:v>
       </ns0:c>
       <ns0:c r="F210" s="1">
         <ns0:f>ROUND(F209*1.4,-5)</ns0:f>
@@ -7642,11 +7642,11 @@
       </ns0:c>
       <ns0:c r="D211" s="1">
         <ns0:f>ROUND(D210*20,2-INT(LOG10(ABS(D210*20))))</ns0:f>
-        <ns0:v>1.23e+233</ns0:v>
+        <ns0:v>3.32e+234</ns0:v>
       </ns0:c>
       <ns0:c r="E211" s="1">
         <ns0:f>D211</ns0:f>
-        <ns0:v>1.23e+233</ns0:v>
+        <ns0:v>3.32e+234</ns0:v>
       </ns0:c>
       <ns0:c r="F211" s="1">
         <ns0:f>ROUND(F210*1.4,-5)</ns0:f>
@@ -7674,11 +7674,11 @@
       </ns0:c>
       <ns0:c r="D212" s="1">
         <ns0:f>ROUND(D211*20,2-INT(LOG10(ABS(D211*20))))</ns0:f>
-        <ns0:v>2.4599999999999998e+234</ns0:v>
+        <ns0:v>6.64e+235</ns0:v>
       </ns0:c>
       <ns0:c r="E212" s="1">
         <ns0:f>D212</ns0:f>
-        <ns0:v>2.4599999999999998e+234</ns0:v>
+        <ns0:v>6.64e+235</ns0:v>
       </ns0:c>
       <ns0:c r="F212" s="1">
         <ns0:f>ROUND(F211*1.4,-5)</ns0:f>
@@ -7706,11 +7706,11 @@
       </ns0:c>
       <ns0:c r="D213" s="1">
         <ns0:f>ROUND(D212*20,2-INT(LOG10(ABS(D212*20))))</ns0:f>
-        <ns0:v>4.92e+235</ns0:v>
+        <ns0:v>1.33e+237</ns0:v>
       </ns0:c>
       <ns0:c r="E213" s="1">
         <ns0:f>D213</ns0:f>
-        <ns0:v>4.92e+235</ns0:v>
+        <ns0:v>1.33e+237</ns0:v>
       </ns0:c>
       <ns0:c r="F213" s="1">
         <ns0:f>ROUND(F212*1.4,-5)</ns0:f>
@@ -7738,11 +7738,11 @@
       </ns0:c>
       <ns0:c r="D214" s="1">
         <ns0:f>ROUND(D213*20,2-INT(LOG10(ABS(D213*20))))</ns0:f>
-        <ns0:v>9.840000000000001e+236</ns0:v>
+        <ns0:v>2.66e+238</ns0:v>
       </ns0:c>
       <ns0:c r="E214" s="1">
         <ns0:f>D214</ns0:f>
-        <ns0:v>9.840000000000001e+236</ns0:v>
+        <ns0:v>2.66e+238</ns0:v>
       </ns0:c>
       <ns0:c r="F214" s="1">
         <ns0:f>ROUND(F213*1.4,-5)</ns0:f>
@@ -7770,11 +7770,11 @@
       </ns0:c>
       <ns0:c r="D215" s="1">
         <ns0:f>ROUND(D214*20,2-INT(LOG10(ABS(D214*20))))</ns0:f>
-        <ns0:v>1.97e+238</ns0:v>
+        <ns0:v>5.32e+239</ns0:v>
       </ns0:c>
       <ns0:c r="E215" s="1">
         <ns0:f>D215</ns0:f>
-        <ns0:v>1.97e+238</ns0:v>
+        <ns0:v>5.32e+239</ns0:v>
       </ns0:c>
       <ns0:c r="F215" s="1">
         <ns0:f>ROUND(F214*1.4,-5)</ns0:f>
@@ -7802,11 +7802,11 @@
       </ns0:c>
       <ns0:c r="D216" s="1">
         <ns0:f>ROUND(D215*20,2-INT(LOG10(ABS(D215*20))))</ns0:f>
-        <ns0:v>3.94e+239</ns0:v>
+        <ns0:v>1.0599999999999999e+241</ns0:v>
       </ns0:c>
       <ns0:c r="E216" s="1">
         <ns0:f>D216</ns0:f>
-        <ns0:v>3.94e+239</ns0:v>
+        <ns0:v>1.0599999999999999e+241</ns0:v>
       </ns0:c>
       <ns0:c r="F216" s="1">
         <ns0:f>ROUND(F215*1.4,-5)</ns0:f>
@@ -7834,11 +7834,11 @@
       </ns0:c>
       <ns0:c r="D217" s="1">
         <ns0:f>ROUND(D216*20,2-INT(LOG10(ABS(D216*20))))</ns0:f>
-        <ns0:v>7.88e+240</ns0:v>
+        <ns0:v>2.12e+242</ns0:v>
       </ns0:c>
       <ns0:c r="E217" s="1">
         <ns0:f>D217</ns0:f>
-        <ns0:v>7.88e+240</ns0:v>
+        <ns0:v>2.12e+242</ns0:v>
       </ns0:c>
       <ns0:c r="F217" s="1">
         <ns0:f>ROUND(F216*1.4,-5)</ns0:f>
@@ -7866,11 +7866,11 @@
       </ns0:c>
       <ns0:c r="D218" s="1">
         <ns0:f>ROUND(D217*20,2-INT(LOG10(ABS(D217*20))))</ns0:f>
-        <ns0:v>1.58e+242</ns0:v>
+        <ns0:v>4.24e+243</ns0:v>
       </ns0:c>
       <ns0:c r="E218" s="1">
         <ns0:f>D218</ns0:f>
-        <ns0:v>1.58e+242</ns0:v>
+        <ns0:v>4.24e+243</ns0:v>
       </ns0:c>
       <ns0:c r="F218" s="1">
         <ns0:f>ROUND(F217*1.4,-5)</ns0:f>
@@ -7898,11 +7898,11 @@
       </ns0:c>
       <ns0:c r="D219" s="1">
         <ns0:f>ROUND(D218*20,2-INT(LOG10(ABS(D218*20))))</ns0:f>
-        <ns0:v>3.16e+243</ns0:v>
+        <ns0:v>8.480000000000001e+244</ns0:v>
       </ns0:c>
       <ns0:c r="E219" s="1">
         <ns0:f>D219</ns0:f>
-        <ns0:v>3.16e+243</ns0:v>
+        <ns0:v>8.480000000000001e+244</ns0:v>
       </ns0:c>
       <ns0:c r="F219" s="1">
         <ns0:f>ROUND(F218*1.4,-5)</ns0:f>
@@ -7930,11 +7930,11 @@
       </ns0:c>
       <ns0:c r="D220" s="1">
         <ns0:f>ROUND(D219*20,2-INT(LOG10(ABS(D219*20))))</ns0:f>
-        <ns0:v>6.32e+244</ns0:v>
+        <ns0:v>1.7000000000000001e+246</ns0:v>
       </ns0:c>
       <ns0:c r="E220" s="1">
         <ns0:f>D220</ns0:f>
-        <ns0:v>6.32e+244</ns0:v>
+        <ns0:v>1.7000000000000001e+246</ns0:v>
       </ns0:c>
       <ns0:c r="F220" s="1">
         <ns0:f>ROUND(F219*1.4,-5)</ns0:f>
@@ -7962,11 +7962,11 @@
       </ns0:c>
       <ns0:c r="D221" s="1">
         <ns0:f>ROUND(D220*20,2-INT(LOG10(ABS(D220*20))))</ns0:f>
-        <ns0:v>1.2600000000000001e+246</ns0:v>
+        <ns0:v>3.4000000000000004e+247</ns0:v>
       </ns0:c>
       <ns0:c r="E221" s="1">
         <ns0:f>D221</ns0:f>
-        <ns0:v>1.2600000000000001e+246</ns0:v>
+        <ns0:v>3.4000000000000004e+247</ns0:v>
       </ns0:c>
       <ns0:c r="F221" s="1">
         <ns0:f>ROUND(F220*1.4,-5)</ns0:f>
@@ -7994,11 +7994,11 @@
       </ns0:c>
       <ns0:c r="D222" s="1">
         <ns0:f>ROUND(D221*20,2-INT(LOG10(ABS(D221*20))))</ns0:f>
-        <ns0:v>2.5200000000000003e+247</ns0:v>
+        <ns0:v>6.8e+248</ns0:v>
       </ns0:c>
       <ns0:c r="E222" s="1">
         <ns0:f>D222</ns0:f>
-        <ns0:v>2.5200000000000003e+247</ns0:v>
+        <ns0:v>6.8e+248</ns0:v>
       </ns0:c>
       <ns0:c r="F222" s="1">
         <ns0:f>ROUND(F221*1.4,-5)</ns0:f>
@@ -8026,11 +8026,11 @@
       </ns0:c>
       <ns0:c r="D223" s="1">
         <ns0:f>ROUND(D222*20,2-INT(LOG10(ABS(D222*20))))</ns0:f>
-        <ns0:v>5.040000000000001e+248</ns0:v>
+        <ns0:v>1.36e+250</ns0:v>
       </ns0:c>
       <ns0:c r="E223" s="1">
         <ns0:f>D223</ns0:f>
-        <ns0:v>5.040000000000001e+248</ns0:v>
+        <ns0:v>1.36e+250</ns0:v>
       </ns0:c>
       <ns0:c r="F223" s="1">
         <ns0:f>ROUND(F222*1.4,-5)</ns0:f>

</xml_diff>

<commit_message>
Fix obsolete reforge UI cards, scene refresh and sparse visit enhancement behavior
</commit_message>
<xml_diff>
--- a/space-battleship/config_excel/level.xlsx
+++ b/space-battleship/config_excel/level.xlsx
@@ -2107,10 +2107,10 @@
         </ns0:is>
       </ns0:c>
       <ns0:c r="D34" s="1" t="n">
-        <ns0:v>1.028931353582277e+22</ns0:v>
+        <ns0:v>3.944675858338559e+23</ns0:v>
       </ns0:c>
       <ns0:c r="E34" s="1" t="n">
-        <ns0:v>1.028931353582277e+22</ns0:v>
+        <ns0:v>3.944675858338559e+23</ns0:v>
       </ns0:c>
       <ns0:c r="F34" s="1" t="n">
         <ns0:v>9704565562037236</ns0:v>
@@ -2135,10 +2135,10 @@
         </ns0:is>
       </ns0:c>
       <ns0:c r="D35" s="1" t="n">
-        <ns0:v>4.424216484808832e+22</ns0:v>
+        <ns0:v>5.064642171181013e+24</ns0:v>
       </ns0:c>
       <ns0:c r="E35" s="1" t="n">
-        <ns0:v>4.424216484808832e+22</ns0:v>
+        <ns0:v>5.064642171181013e+24</ns0:v>
       </ns0:c>
       <ns0:c r="F35" s="1" t="n">
         <ns0:v>9704565562037236</ns0:v>
@@ -2163,10 +2163,10 @@
         </ns0:is>
       </ns0:c>
       <ns0:c r="D36" s="1" t="n">
-        <ns0:v>8.179679859850836e+23</ns0:v>
+        <ns0:v>4.515685833272325e+25</ns0:v>
       </ns0:c>
       <ns0:c r="E36" s="1" t="n">
-        <ns0:v>8.179679859850836e+23</ns0:v>
+        <ns0:v>4.515685833272325e+25</ns0:v>
       </ns0:c>
       <ns0:c r="F36" s="1" t="n">
         <ns0:v>2.012338714944041e+16</ns0:v>
@@ -2191,10 +2191,10 @@
         </ns0:is>
       </ns0:c>
       <ns0:c r="D37" s="1" t="n">
-        <ns0:v>4.026230848222263e+26</ns0:v>
+        <ns0:v>2.492936018792822e+27</ns0:v>
       </ns0:c>
       <ns0:c r="E37" s="1" t="n">
-        <ns0:v>4.026230848222263e+26</ns0:v>
+        <ns0:v>2.492936018792822e+27</ns0:v>
       </ns0:c>
       <ns0:c r="F37" s="1" t="n">
         <ns0:v>2.012338714944041e+16</ns0:v>
@@ -2219,10 +2219,10 @@
         </ns0:is>
       </ns0:c>
       <ns0:c r="D38" s="1" t="n">
-        <ns0:v>1.543560274627236e+28</ns0:v>
+        <ns0:v>1.981805537738023e+29</ns0:v>
       </ns0:c>
       <ns0:c r="E38" s="1" t="n">
-        <ns0:v>1.543560274627236e+28</ns0:v>
+        <ns0:v>1.981805537738023e+29</ns0:v>
       </ns0:c>
       <ns0:c r="F38" s="1" t="n">
         <ns0:v>6.008811205403466e+16</ns0:v>
@@ -2247,10 +2247,10 @@
         </ns0:is>
       </ns0:c>
       <ns0:c r="D39" s="1" t="n">
-        <ns0:v>4.609046283072532e+28</ns0:v>
+        <ns0:v>5.917639626797131e+29</ns0:v>
       </ns0:c>
       <ns0:c r="E39" s="1" t="n">
-        <ns0:v>4.609046283072532e+28</ns0:v>
+        <ns0:v>5.917639626797131e+29</ns0:v>
       </ns0:c>
       <ns0:c r="F39" s="1" t="n">
         <ns0:v>1.245987091552463e+17</ns0:v>
@@ -2275,10 +2275,10 @@
         </ns0:is>
       </ns0:c>
       <ns0:c r="D40" s="1" t="n">
-        <ns0:v>1.376253845651405e+29</ns0:v>
+        <ns0:v>1.76699772433822e+30</ns0:v>
       </ns0:c>
       <ns0:c r="E40" s="1" t="n">
-        <ns0:v>1.376253845651405e+29</ns0:v>
+        <ns0:v>1.76699772433822e+30</ns0:v>
       </ns0:c>
       <ns0:c r="F40" s="1" t="n">
         <ns0:v>2.583678833043186e+17</ns0:v>
@@ -2303,10 +2303,10 @@
         </ns0:is>
       </ns0:c>
       <ns0:c r="D41" s="1" t="n">
-        <ns0:v>4.109471963053564e+29</ns0:v>
+        <ns0:v>5.276226932910335e+30</ns0:v>
       </ns0:c>
       <ns0:c r="E41" s="1" t="n">
-        <ns0:v>4.109471963053564e+29</ns0:v>
+        <ns0:v>5.276226932910335e+30</ns0:v>
       </ns0:c>
       <ns0:c r="F41" s="1" t="n">
         <ns0:v>5.357516428198349e+17</ns0:v>
@@ -2331,10 +2331,10 @@
         </ns0:is>
       </ns0:c>
       <ns0:c r="D42" s="1" t="n">
-        <ns0:v>3.664046481187733e+30</ns0:v>
+        <ns0:v>4.704336932162219e+31</ns0:v>
       </ns0:c>
       <ns0:c r="E42" s="1" t="n">
-        <ns0:v>3.664046481187733e+30</ns0:v>
+        <ns0:v>4.704336932162219e+31</ns0:v>
       </ns0:c>
       <ns0:c r="F42" s="1" t="n">
         <ns0:v>2.303634000144588e+18</ns0:v>
@@ -2359,10 +2359,10 @@
         </ns0:is>
       </ns0:c>
       <ns0:c r="D43" s="1" t="n">
-        <ns0:v>1.404707481004547e+32</ns0:v>
+        <ns0:v>1.80352987215166e+33</ns0:v>
       </ns0:c>
       <ns0:c r="E43" s="1" t="n">
-        <ns0:v>1.404707481004547e+32</ns0:v>
+        <ns0:v>1.80352987215166e+33</ns0:v>
       </ns0:c>
       <ns0:c r="F43" s="1" t="n">
         <ns0:v>2.053943214130691e+19</ns0:v>
@@ -2387,10 +2387,10 @@
         </ns0:is>
       </ns0:c>
       <ns0:c r="D44" s="1" t="n">
-        <ns0:v>4.19443406295988e+32</ns0:v>
+        <ns0:v>5.3853113417669e+33</ns0:v>
       </ns0:c>
       <ns0:c r="E44" s="1" t="n">
-        <ns0:v>4.19443406295988e+32</ns0:v>
+        <ns0:v>5.3853113417669e+33</ns0:v>
       </ns0:c>
       <ns0:c r="F44" s="1" t="n">
         <ns0:v>4.259056648821401e+19</ns0:v>
@@ -2415,10 +2415,10 @@
         </ns0:is>
       </ns0:c>
       <ns0:c r="D45" s="1" t="n">
-        <ns0:v>1.252451300105319e+33</ns0:v>
+        <ns0:v>1.608045350153449e+34</ns0:v>
       </ns0:c>
       <ns0:c r="E45" s="1" t="n">
-        <ns0:v>1.252451300105319e+33</ns0:v>
+        <ns0:v>1.608045350153449e+34</ns0:v>
       </ns0:c>
       <ns0:c r="F45" s="1" t="n">
         <ns0:v>8.831579866996054e+19</ns0:v>
@@ -2443,10 +2443,10 @@
         </ns0:is>
       </ns0:c>
       <ns0:c r="D46" s="1" t="n">
-        <ns0:v>3.739799542893681e+33</ns0:v>
+        <ns0:v>4.801597686832596e+34</ns0:v>
       </ns0:c>
       <ns0:c r="E46" s="1" t="n">
-        <ns0:v>3.739799542893681e+33</ns0:v>
+        <ns0:v>4.801597686832596e+34</ns0:v>
       </ns0:c>
       <ns0:c r="F46" s="1" t="n">
         <ns0:v>1.831316401220302e+20</ns0:v>
@@ -2471,10 +2471,10 @@
         </ns0:is>
       </ns0:c>
       <ns0:c r="D47" s="1" t="n">
-        <ns0:v>3.334442838078192e+34</ns0:v>
+        <ns0:v>4.281152728791306e+35</ns0:v>
       </ns0:c>
       <ns0:c r="E47" s="1" t="n">
-        <ns0:v>3.334442838078192e+34</ns0:v>
+        <ns0:v>4.281152728791306e+35</ns0:v>
       </ns0:c>
       <ns0:c r="F47" s="1" t="n">
         <ns0:v>7.874325321093216e+20</ns0:v>
@@ -2499,10 +2499,10 @@
         </ns0:is>
       </ns0:c>
       <ns0:c r="D48" s="1" t="n">
-        <ns0:v>1.278345354972718e+36</ns0:v>
+        <ns0:v>1.641291205319743e+37</ns0:v>
       </ns0:c>
       <ns0:c r="E48" s="1" t="n">
-        <ns0:v>1.278345354972718e+36</ns0:v>
+        <ns0:v>1.641291205319743e+37</ns0:v>
       </ns0:c>
       <ns0:c r="F48" s="1" t="n">
         <ns0:v>7.020827552511277e+21</ns0:v>
@@ -2527,10 +2527,10 @@
         </ns0:is>
       </ns0:c>
       <ns0:c r="D49" s="1" t="n">
-        <ns0:v>3.817118776422855e+36</ns0:v>
+        <ns0:v>4.900869278425468e+37</ns0:v>
       </ns0:c>
       <ns0:c r="E49" s="1" t="n">
-        <ns0:v>3.817118776422855e+36</ns0:v>
+        <ns0:v>4.900869278425468e+37</ns0:v>
       </ns0:c>
       <ns0:c r="F49" s="1" t="n">
         <ns0:v>1.455838801288738e+22</ns0:v>
@@ -2555,10 +2555,10 @@
         </ns0:is>
       </ns0:c>
       <ns0:c r="D50" s="1" t="n">
-        <ns0:v>1.139785559249822e+37</ns0:v>
+        <ns0:v>1.463391725146999e+38</ns0:v>
       </ns0:c>
       <ns0:c r="E50" s="1" t="n">
-        <ns0:v>1.139785559249822e+37</ns0:v>
+        <ns0:v>1.463391725146999e+38</ns0:v>
       </ns0:c>
       <ns0:c r="F50" s="1" t="n">
         <ns0:v>3.018827338352327e+22</ns0:v>
@@ -2583,10 +2583,10 @@
         </ns0:is>
       </ns0:c>
       <ns0:c r="D51" s="1" t="n">
-        <ns0:v>3.40338144335102e+37</ns0:v>
+        <ns0:v>4.369664277021335e+38</ns0:v>
       </ns0:c>
       <ns0:c r="E51" s="1" t="n">
-        <ns0:v>3.40338144335102e+37</ns0:v>
+        <ns0:v>4.369664277021335e+38</ns0:v>
       </ns0:c>
       <ns0:c r="F51" s="1" t="n">
         <ns0:v>6.259840368807384e+22</ns0:v>
@@ -2611,10 +2611,10 @@
         </ns0:is>
       </ns0:c>
       <ns0:c r="D52" s="1" t="n">
-        <ns0:v>3.034489081264816e+38</ns0:v>
+        <ns0:v>3.896036561907814e+39</ns0:v>
       </ns0:c>
       <ns0:c r="E52" s="1" t="n">
-        <ns0:v>3.034489081264816e+38</ns0:v>
+        <ns0:v>3.896036561907814e+39</ns0:v>
       </ns0:c>
       <ns0:c r="F52" s="1" t="n">
         <ns0:v>2.691616778469064e+23</ns0:v>
@@ -2639,10 +2639,10 @@
         </ns0:is>
       </ns0:c>
       <ns0:c r="D53" s="1" t="n">
-        <ns0:v>1.163350283727174e+40</ns0:v>
+        <ns0:v>1.493646910015478e+41</ns0:v>
       </ns0:c>
       <ns0:c r="E53" s="1" t="n">
-        <ns0:v>1.163350283727174e+40</ns0:v>
+        <ns0:v>1.493646910015478e+41</ns0:v>
       </ns0:c>
       <ns0:c r="F53" s="1" t="n">
         <ns0:v>2.399872556504138e+24</ns0:v>
@@ -2667,10 +2667,10 @@
         </ns0:is>
       </ns0:c>
       <ns0:c r="D54" s="1" t="n">
-        <ns0:v>3.473745333604802e+40</ns0:v>
+        <ns0:v>4.460005774955655e+41</ns0:v>
       </ns0:c>
       <ns0:c r="E54" s="1" t="n">
-        <ns0:v>3.473745333604802e+40</ns0:v>
+        <ns0:v>4.460005774955655e+41</ns0:v>
       </ns0:c>
       <ns0:c r="F54" s="1" t="n">
         <ns0:v>4.976375733166981e+24</ns0:v>
@@ -2695,10 +2695,10 @@
         </ns0:is>
       </ns0:c>
       <ns0:c r="D55" s="1" t="n">
-        <ns0:v>1.03725479862186e+41</ns0:v>
+        <ns0:v>1.331750588392518e+42</ns0:v>
       </ns0:c>
       <ns0:c r="E55" s="1" t="n">
-        <ns0:v>1.03725479862186e+41</ns0:v>
+        <ns0:v>1.331750588392518e+42</ns0:v>
       </ns0:c>
       <ns0:c r="F55" s="1" t="n">
         <ns0:v>1.031901272029505e+25</ns0:v>
@@ -2723,10 +2723,10 @@
         </ns0:is>
       </ns0:c>
       <ns0:c r="D56" s="1" t="n">
-        <ns0:v>3.097226232608094e+41</ns0:v>
+        <ns0:v>3.976585948930645e+42</ns0:v>
       </ns0:c>
       <ns0:c r="E56" s="1" t="n">
-        <ns0:v>3.097226232608094e+41</ns0:v>
+        <ns0:v>3.976585948930645e+42</ns0:v>
       </ns0:c>
       <ns0:c r="F56" s="1" t="n">
         <ns0:v>2.139750477680381e+25</ns0:v>
@@ -2751,10 +2751,10 @@
         </ns0:is>
       </ns0:c>
       <ns0:c r="D57" s="1" t="n">
-        <ns0:v>2.761518020090726e+42</ns0:v>
+        <ns0:v>3.545563976178902e+43</ns0:v>
       </ns0:c>
       <ns0:c r="E57" s="1" t="n">
-        <ns0:v>2.761518020090726e+42</ns0:v>
+        <ns0:v>3.545563976178902e+43</ns0:v>
       </ns0:c>
       <ns0:c r="F57" s="1" t="n">
         <ns0:v>9.200535394098201e+25</ns0:v>
@@ -2779,10 +2779,10 @@
         </ns0:is>
       </ns0:c>
       <ns0:c r="D58" s="1" t="n">
-        <ns0:v>1.058699730384658e+44</ns0:v>
+        <ns0:v>1.359284132253766e+45</ns0:v>
       </ns0:c>
       <ns0:c r="E58" s="1" t="n">
-        <ns0:v>1.058699730384658e+44</ns0:v>
+        <ns0:v>1.359284132253766e+45</ns0:v>
       </ns0:c>
       <ns0:c r="F58" s="1" t="n">
         <ns0:v>8.203289775151412e+26</ns0:v>
@@ -2807,10 +2807,10 @@
         </ns0:is>
       </ns0:c>
       <ns0:c r="D59" s="1" t="n">
-        <ns0:v>3.161260455732902e+44</ns0:v>
+        <ns0:v>4.058800670363627e+45</ns0:v>
       </ns0:c>
       <ns0:c r="E59" s="1" t="n">
-        <ns0:v>3.161260455732902e+44</ns0:v>
+        <ns0:v>4.058800670363627e+45</ns0:v>
       </ns0:c>
       <ns0:c r="F59" s="1" t="n">
         <ns0:v>1.701034167775397e+27</ns0:v>
@@ -2835,10 +2835,10 @@
         </ns0:is>
       </ns0:c>
       <ns0:c r="D60" s="1" t="n">
-        <ns0:v>9.439473140651152e+44</ns0:v>
+        <ns0:v>1.211951386089506e+46</ns0:v>
       </ns0:c>
       <ns0:c r="E60" s="1" t="n">
-        <ns0:v>9.439473140651152e+44</ns0:v>
+        <ns0:v>1.211951386089506e+46</ns0:v>
       </ns0:c>
       <ns0:c r="F60" s="1" t="n">
         <ns0:v>3.527264450299061e+27</ns0:v>
@@ -2863,10 +2863,10 @@
         </ns0:is>
       </ns0:c>
       <ns0:c r="D61" s="1" t="n">
-        <ns0:v>2.818611576641408e+45</ns0:v>
+        <ns0:v>3.618867447641087e+46</ns0:v>
       </ns0:c>
       <ns0:c r="E61" s="1" t="n">
-        <ns0:v>2.818611576641408e+45</ns0:v>
+        <ns0:v>3.618867447641087e+46</ns0:v>
       </ns0:c>
       <ns0:c r="F61" s="1" t="n">
         <ns0:v>7.314135564140134e+27</ns0:v>
@@ -2891,10 +2891,10 @@
         </ns0:is>
       </ns0:c>
       <ns0:c r="D62" s="1" t="n">
-        <ns0:v>2.5131023941952e+46</ns0:v>
+        <ns0:v>3.226618567209173e+47</ns0:v>
       </ns0:c>
       <ns0:c r="E62" s="1" t="n">
-        <ns0:v>2.5131023941952e+46</ns0:v>
+        <ns0:v>3.226618567209173e+47</ns0:v>
       </ns0:c>
       <ns0:c r="F62" s="1" t="n">
         <ns0:v>3.14494441464289e+28</ns0:v>
@@ -2919,10 +2919,10 @@
         </ns0:is>
       </ns0:c>
       <ns0:c r="D63" s="1" t="n">
-        <ns0:v>9.634631415789515e+47</ns0:v>
+        <ns0:v>1.237008117385472e+49</ns0:v>
       </ns0:c>
       <ns0:c r="E63" s="1" t="n">
-        <ns0:v>9.634631415789515e+47</ns0:v>
+        <ns0:v>1.237008117385472e+49</ns0:v>
       </ns0:c>
       <ns0:c r="F63" s="1" t="n">
         <ns0:v>2.804064030513767e+29</ns0:v>
@@ -2948,11 +2948,11 @@
       </ns0:c>
       <ns0:c r="D64" s="1">
         <ns0:f>ROUND(D63*10,0)</ns0:f>
-        <ns0:v>9.634631415789514e+48</ns0:v>
+        <ns0:v>1.2370081173854715e+50</ns0:v>
       </ns0:c>
       <ns0:c r="E64" s="1">
         <ns0:f>D64</ns0:f>
-        <ns0:v>9.634631415789514e+48</ns0:v>
+        <ns0:v>1.2370081173854715e+50</ns0:v>
       </ns0:c>
       <ns0:c r="F64" s="1">
         <ns0:f>ROUND(F63*1.4,-5)</ns0:f>
@@ -2979,11 +2979,11 @@
       </ns0:c>
       <ns0:c r="D65" s="1">
         <ns0:f>ROUND(D64*10,0)</ns0:f>
-        <ns0:v>9.634631415789515e+49</ns0:v>
+        <ns0:v>1.2370081173854714e+51</ns0:v>
       </ns0:c>
       <ns0:c r="E65" s="1">
         <ns0:f>D65</ns0:f>
-        <ns0:v>9.634631415789515e+49</ns0:v>
+        <ns0:v>1.2370081173854714e+51</ns0:v>
       </ns0:c>
       <ns0:c r="F65" s="1">
         <ns0:f>ROUND(F64*1.4,-5)</ns0:f>
@@ -3010,11 +3010,11 @@
       </ns0:c>
       <ns0:c r="D66" s="1">
         <ns0:f>ROUND(D65*10,0)</ns0:f>
-        <ns0:v>9.634631415789514e+50</ns0:v>
+        <ns0:v>1.2370081173854714e+52</ns0:v>
       </ns0:c>
       <ns0:c r="E66" s="1">
         <ns0:f>D66</ns0:f>
-        <ns0:v>9.634631415789514e+50</ns0:v>
+        <ns0:v>1.2370081173854714e+52</ns0:v>
       </ns0:c>
       <ns0:c r="F66" s="1">
         <ns0:f>ROUND(F65*1.4,-5)</ns0:f>
@@ -3041,11 +3041,11 @@
       </ns0:c>
       <ns0:c r="D67" s="1">
         <ns0:f>ROUND(D66*10,0)</ns0:f>
-        <ns0:v>9.634631415789515e+51</ns0:v>
+        <ns0:v>1.2370081173854714e+53</ns0:v>
       </ns0:c>
       <ns0:c r="E67" s="1">
         <ns0:f>D67</ns0:f>
-        <ns0:v>9.634631415789515e+51</ns0:v>
+        <ns0:v>1.2370081173854714e+53</ns0:v>
       </ns0:c>
       <ns0:c r="F67" s="1">
         <ns0:f>ROUND(F66*1.4,-5)</ns0:f>
@@ -3072,11 +3072,11 @@
       </ns0:c>
       <ns0:c r="D68" s="1">
         <ns0:f>ROUND(D67*10,0)</ns0:f>
-        <ns0:v>9.634631415789515e+52</ns0:v>
+        <ns0:v>1.2370081173854715e+54</ns0:v>
       </ns0:c>
       <ns0:c r="E68" s="1">
         <ns0:f>D68</ns0:f>
-        <ns0:v>9.634631415789515e+52</ns0:v>
+        <ns0:v>1.2370081173854715e+54</ns0:v>
       </ns0:c>
       <ns0:c r="F68" s="1">
         <ns0:f>ROUND(F67*1.4,-5)</ns0:f>
@@ -3103,11 +3103,11 @@
       </ns0:c>
       <ns0:c r="D69" s="1">
         <ns0:f>ROUND(D68*10,0)</ns0:f>
-        <ns0:v>9.634631415789514e+53</ns0:v>
+        <ns0:v>1.2370081173854714e+55</ns0:v>
       </ns0:c>
       <ns0:c r="E69" s="1">
         <ns0:f>D69</ns0:f>
-        <ns0:v>9.634631415789514e+53</ns0:v>
+        <ns0:v>1.2370081173854714e+55</ns0:v>
       </ns0:c>
       <ns0:c r="F69" s="1">
         <ns0:f>ROUND(F68*1.4,-5)</ns0:f>
@@ -3134,11 +3134,11 @@
       </ns0:c>
       <ns0:c r="D70" s="1">
         <ns0:f>ROUND(D69*10,0)</ns0:f>
-        <ns0:v>9.634631415789514e+54</ns0:v>
+        <ns0:v>1.2370081173854714e+56</ns0:v>
       </ns0:c>
       <ns0:c r="E70" s="1">
         <ns0:f>D70</ns0:f>
-        <ns0:v>9.634631415789514e+54</ns0:v>
+        <ns0:v>1.2370081173854714e+56</ns0:v>
       </ns0:c>
       <ns0:c r="F70" s="1">
         <ns0:f>ROUND(F69*1.4,-5)</ns0:f>
@@ -3165,11 +3165,11 @@
       </ns0:c>
       <ns0:c r="D71" s="1">
         <ns0:f>ROUND(D70*10,0)</ns0:f>
-        <ns0:v>9.634631415789515e+55</ns0:v>
+        <ns0:v>1.2370081173854715e+57</ns0:v>
       </ns0:c>
       <ns0:c r="E71" s="1">
         <ns0:f>D71</ns0:f>
-        <ns0:v>9.634631415789515e+55</ns0:v>
+        <ns0:v>1.2370081173854715e+57</ns0:v>
       </ns0:c>
       <ns0:c r="F71" s="1">
         <ns0:f>ROUND(F70*1.4,-5)</ns0:f>
@@ -3196,11 +3196,11 @@
       </ns0:c>
       <ns0:c r="D72" s="1">
         <ns0:f>ROUND(D71*10,0)</ns0:f>
-        <ns0:v>9.634631415789514e+56</ns0:v>
+        <ns0:v>1.2370081173854714e+58</ns0:v>
       </ns0:c>
       <ns0:c r="E72" s="1">
         <ns0:f>D72</ns0:f>
-        <ns0:v>9.634631415789514e+56</ns0:v>
+        <ns0:v>1.2370081173854714e+58</ns0:v>
       </ns0:c>
       <ns0:c r="F72" s="1">
         <ns0:f>ROUND(F71*1.4,-5)</ns0:f>
@@ -3227,11 +3227,11 @@
       </ns0:c>
       <ns0:c r="D73" s="1">
         <ns0:f>ROUND(D72*10,0)</ns0:f>
-        <ns0:v>9.634631415789514e+57</ns0:v>
+        <ns0:v>1.2370081173854714e+59</ns0:v>
       </ns0:c>
       <ns0:c r="E73" s="1">
         <ns0:f>D73</ns0:f>
-        <ns0:v>9.634631415789514e+57</ns0:v>
+        <ns0:v>1.2370081173854714e+59</ns0:v>
       </ns0:c>
       <ns0:c r="F73" s="1">
         <ns0:f>ROUND(F72*1.4,-5)</ns0:f>
@@ -3258,11 +3258,11 @@
       </ns0:c>
       <ns0:c r="D74" s="1">
         <ns0:f>ROUND(D73*10,0)</ns0:f>
-        <ns0:v>9.634631415789514e+58</ns0:v>
+        <ns0:v>1.2370081173854713e+60</ns0:v>
       </ns0:c>
       <ns0:c r="E74" s="1">
         <ns0:f>D74</ns0:f>
-        <ns0:v>9.634631415789514e+58</ns0:v>
+        <ns0:v>1.2370081173854713e+60</ns0:v>
       </ns0:c>
       <ns0:c r="F74" s="1">
         <ns0:f>ROUND(F73*1.4,-5)</ns0:f>
@@ -3290,11 +3290,11 @@
       </ns0:c>
       <ns0:c r="D75" s="1">
         <ns0:f>ROUND(D74*10,0)</ns0:f>
-        <ns0:v>9.634631415789515e+59</ns0:v>
+        <ns0:v>1.2370081173854713e+61</ns0:v>
       </ns0:c>
       <ns0:c r="E75" s="1">
         <ns0:f>D75</ns0:f>
-        <ns0:v>9.634631415789515e+59</ns0:v>
+        <ns0:v>1.2370081173854713e+61</ns0:v>
       </ns0:c>
       <ns0:c r="F75" s="1">
         <ns0:f>ROUND(F74*1.4,-5)</ns0:f>
@@ -3322,11 +3322,11 @@
       </ns0:c>
       <ns0:c r="D76" s="1">
         <ns0:f>ROUND(D75*10,0)</ns0:f>
-        <ns0:v>9.634631415789514e+60</ns0:v>
+        <ns0:v>1.2370081173854713e+62</ns0:v>
       </ns0:c>
       <ns0:c r="E76" s="1">
         <ns0:f>D76</ns0:f>
-        <ns0:v>9.634631415789514e+60</ns0:v>
+        <ns0:v>1.2370081173854713e+62</ns0:v>
       </ns0:c>
       <ns0:c r="F76" s="1">
         <ns0:f>ROUND(F75*1.4,-5)</ns0:f>
@@ -3354,11 +3354,11 @@
       </ns0:c>
       <ns0:c r="D77" s="1">
         <ns0:f>ROUND(D76*10,0)</ns0:f>
-        <ns0:v>9.634631415789515e+61</ns0:v>
+        <ns0:v>1.2370081173854712e+63</ns0:v>
       </ns0:c>
       <ns0:c r="E77" s="1">
         <ns0:f>D77</ns0:f>
-        <ns0:v>9.634631415789515e+61</ns0:v>
+        <ns0:v>1.2370081173854712e+63</ns0:v>
       </ns0:c>
       <ns0:c r="F77" s="1">
         <ns0:f>ROUND(F76*1.4,-5)</ns0:f>
@@ -3386,11 +3386,11 @@
       </ns0:c>
       <ns0:c r="D78" s="1">
         <ns0:f>ROUND(D77*10,0)</ns0:f>
-        <ns0:v>9.634631415789515e+62</ns0:v>
+        <ns0:v>1.2370081173854713e+64</ns0:v>
       </ns0:c>
       <ns0:c r="E78" s="1">
         <ns0:f>D78</ns0:f>
-        <ns0:v>9.634631415789515e+62</ns0:v>
+        <ns0:v>1.2370081173854713e+64</ns0:v>
       </ns0:c>
       <ns0:c r="F78" s="1">
         <ns0:f>ROUND(F77*1.4,-5)</ns0:f>
@@ -3418,11 +3418,11 @@
       </ns0:c>
       <ns0:c r="D79" s="1">
         <ns0:f>ROUND(D78*10,0)</ns0:f>
-        <ns0:v>9.634631415789514e+63</ns0:v>
+        <ns0:v>1.2370081173854713e+65</ns0:v>
       </ns0:c>
       <ns0:c r="E79" s="1">
         <ns0:f>D79</ns0:f>
-        <ns0:v>9.634631415789514e+63</ns0:v>
+        <ns0:v>1.2370081173854713e+65</ns0:v>
       </ns0:c>
       <ns0:c r="F79" s="1">
         <ns0:f>ROUND(F78*1.4,-5)</ns0:f>
@@ -3450,11 +3450,11 @@
       </ns0:c>
       <ns0:c r="D80" s="1">
         <ns0:f>ROUND(D79*10,0)</ns0:f>
-        <ns0:v>9.634631415789513e+64</ns0:v>
+        <ns0:v>1.2370081173854713e+66</ns0:v>
       </ns0:c>
       <ns0:c r="E80" s="1">
         <ns0:f>D80</ns0:f>
-        <ns0:v>9.634631415789513e+64</ns0:v>
+        <ns0:v>1.2370081173854713e+66</ns0:v>
       </ns0:c>
       <ns0:c r="F80" s="1">
         <ns0:f>ROUND(F79*1.4,-5)</ns0:f>
@@ -3482,11 +3482,11 @@
       </ns0:c>
       <ns0:c r="D81" s="1">
         <ns0:f>ROUND(D80*10,0)</ns0:f>
-        <ns0:v>9.634631415789514e+65</ns0:v>
+        <ns0:v>1.2370081173854713e+67</ns0:v>
       </ns0:c>
       <ns0:c r="E81" s="1">
         <ns0:f>D81</ns0:f>
-        <ns0:v>9.634631415789514e+65</ns0:v>
+        <ns0:v>1.2370081173854713e+67</ns0:v>
       </ns0:c>
       <ns0:c r="F81" s="1">
         <ns0:f>ROUND(F80*1.4,-5)</ns0:f>
@@ -3514,11 +3514,11 @@
       </ns0:c>
       <ns0:c r="D82" s="1">
         <ns0:f>ROUND(D81*10,0)</ns0:f>
-        <ns0:v>9.634631415789514e+66</ns0:v>
+        <ns0:v>1.2370081173854713e+68</ns0:v>
       </ns0:c>
       <ns0:c r="E82" s="1">
         <ns0:f>D82</ns0:f>
-        <ns0:v>9.634631415789514e+66</ns0:v>
+        <ns0:v>1.2370081173854713e+68</ns0:v>
       </ns0:c>
       <ns0:c r="F82" s="1">
         <ns0:f>ROUND(F81*1.4,-5)</ns0:f>
@@ -3546,11 +3546,11 @@
       </ns0:c>
       <ns0:c r="D83" s="1">
         <ns0:f>ROUND(D82*10,0)</ns0:f>
-        <ns0:v>9.634631415789514e+67</ns0:v>
+        <ns0:v>1.2370081173854714e+69</ns0:v>
       </ns0:c>
       <ns0:c r="E83" s="1">
         <ns0:f>D83</ns0:f>
-        <ns0:v>9.634631415789514e+67</ns0:v>
+        <ns0:v>1.2370081173854714e+69</ns0:v>
       </ns0:c>
       <ns0:c r="F83" s="1">
         <ns0:f>ROUND(F82*1.4,-5)</ns0:f>
@@ -3578,11 +3578,11 @@
       </ns0:c>
       <ns0:c r="D84" s="1">
         <ns0:f>ROUND(D83*20,2-INT(LOG10(ABS(D83*20))))</ns0:f>
-        <ns0:v>1.93e+69</ns0:v>
+        <ns0:v>2.4699999999999998e+70</ns0:v>
       </ns0:c>
       <ns0:c r="E84" s="1">
         <ns0:f>D84</ns0:f>
-        <ns0:v>1.93e+69</ns0:v>
+        <ns0:v>2.4699999999999998e+70</ns0:v>
       </ns0:c>
       <ns0:c r="F84" s="1">
         <ns0:f>ROUND(F83*1.4,-5)</ns0:f>
@@ -3610,11 +3610,11 @@
       </ns0:c>
       <ns0:c r="D85" s="1">
         <ns0:f>ROUND(D84*20,2-INT(LOG10(ABS(D84*20))))</ns0:f>
-        <ns0:v>3.86e+70</ns0:v>
+        <ns0:v>4.94e+71</ns0:v>
       </ns0:c>
       <ns0:c r="E85" s="1">
         <ns0:f>D85</ns0:f>
-        <ns0:v>3.86e+70</ns0:v>
+        <ns0:v>4.94e+71</ns0:v>
       </ns0:c>
       <ns0:c r="F85" s="1">
         <ns0:f>ROUND(F84*1.4,-5)</ns0:f>
@@ -3642,11 +3642,11 @@
       </ns0:c>
       <ns0:c r="D86" s="1">
         <ns0:f>ROUND(D85*20,2-INT(LOG10(ABS(D85*20))))</ns0:f>
-        <ns0:v>7.72e+71</ns0:v>
+        <ns0:v>9.88e+72</ns0:v>
       </ns0:c>
       <ns0:c r="E86" s="1">
         <ns0:f>D86</ns0:f>
-        <ns0:v>7.72e+71</ns0:v>
+        <ns0:v>9.88e+72</ns0:v>
       </ns0:c>
       <ns0:c r="F86" s="1">
         <ns0:f>ROUND(F85*1.4,-5)</ns0:f>
@@ -3674,11 +3674,11 @@
       </ns0:c>
       <ns0:c r="D87" s="1">
         <ns0:f>ROUND(D86*20,2-INT(LOG10(ABS(D86*20))))</ns0:f>
-        <ns0:v>1.54e+73</ns0:v>
+        <ns0:v>1.98e+74</ns0:v>
       </ns0:c>
       <ns0:c r="E87" s="1">
         <ns0:f>D87</ns0:f>
-        <ns0:v>1.54e+73</ns0:v>
+        <ns0:v>1.98e+74</ns0:v>
       </ns0:c>
       <ns0:c r="F87" s="1">
         <ns0:f>ROUND(F86*1.4,-5)</ns0:f>
@@ -3706,11 +3706,11 @@
       </ns0:c>
       <ns0:c r="D88" s="1">
         <ns0:f>ROUND(D87*20,2-INT(LOG10(ABS(D87*20))))</ns0:f>
-        <ns0:v>3.08e+74</ns0:v>
+        <ns0:v>3.96e+75</ns0:v>
       </ns0:c>
       <ns0:c r="E88" s="1">
         <ns0:f>D88</ns0:f>
-        <ns0:v>3.08e+74</ns0:v>
+        <ns0:v>3.96e+75</ns0:v>
       </ns0:c>
       <ns0:c r="F88" s="1">
         <ns0:f>ROUND(F87*1.4,-5)</ns0:f>
@@ -3738,11 +3738,11 @@
       </ns0:c>
       <ns0:c r="D89" s="1">
         <ns0:f>ROUND(D88*20,2-INT(LOG10(ABS(D88*20))))</ns0:f>
-        <ns0:v>6.16e+75</ns0:v>
+        <ns0:v>7.920000000000001e+76</ns0:v>
       </ns0:c>
       <ns0:c r="E89" s="1">
         <ns0:f>D89</ns0:f>
-        <ns0:v>6.16e+75</ns0:v>
+        <ns0:v>7.920000000000001e+76</ns0:v>
       </ns0:c>
       <ns0:c r="F89" s="1">
         <ns0:f>ROUND(F88*1.4,-5)</ns0:f>
@@ -3770,11 +3770,11 @@
       </ns0:c>
       <ns0:c r="D90" s="1">
         <ns0:f>ROUND(D89*20,2-INT(LOG10(ABS(D89*20))))</ns0:f>
-        <ns0:v>1.23e+77</ns0:v>
+        <ns0:v>1.58e+78</ns0:v>
       </ns0:c>
       <ns0:c r="E90" s="1">
         <ns0:f>D90</ns0:f>
-        <ns0:v>1.23e+77</ns0:v>
+        <ns0:v>1.58e+78</ns0:v>
       </ns0:c>
       <ns0:c r="F90" s="1">
         <ns0:f>ROUND(F89*1.4,-5)</ns0:f>
@@ -3802,11 +3802,11 @@
       </ns0:c>
       <ns0:c r="D91" s="1">
         <ns0:f>ROUND(D90*20,2-INT(LOG10(ABS(D90*20))))</ns0:f>
-        <ns0:v>2.46e+78</ns0:v>
+        <ns0:v>3.1600000000000005e+79</ns0:v>
       </ns0:c>
       <ns0:c r="E91" s="1">
         <ns0:f>D91</ns0:f>
-        <ns0:v>2.46e+78</ns0:v>
+        <ns0:v>3.1600000000000005e+79</ns0:v>
       </ns0:c>
       <ns0:c r="F91" s="1">
         <ns0:f>ROUND(F90*1.4,-5)</ns0:f>
@@ -3834,11 +3834,11 @@
       </ns0:c>
       <ns0:c r="D92" s="1">
         <ns0:f>ROUND(D91*20,2-INT(LOG10(ABS(D91*20))))</ns0:f>
-        <ns0:v>4.92e+79</ns0:v>
+        <ns0:v>6.32e+80</ns0:v>
       </ns0:c>
       <ns0:c r="E92" s="1">
         <ns0:f>D92</ns0:f>
-        <ns0:v>4.92e+79</ns0:v>
+        <ns0:v>6.32e+80</ns0:v>
       </ns0:c>
       <ns0:c r="F92" s="1">
         <ns0:f>ROUND(F91*1.4,-5)</ns0:f>
@@ -3866,11 +3866,11 @@
       </ns0:c>
       <ns0:c r="D93" s="1">
         <ns0:f>ROUND(D92*20,2-INT(LOG10(ABS(D92*20))))</ns0:f>
-        <ns0:v>9.84e+80</ns0:v>
+        <ns0:v>1.26e+82</ns0:v>
       </ns0:c>
       <ns0:c r="E93" s="1">
         <ns0:f>D93</ns0:f>
-        <ns0:v>9.84e+80</ns0:v>
+        <ns0:v>1.26e+82</ns0:v>
       </ns0:c>
       <ns0:c r="F93" s="1">
         <ns0:f>ROUND(F92*1.4,-5)</ns0:f>
@@ -3898,11 +3898,11 @@
       </ns0:c>
       <ns0:c r="D94" s="1">
         <ns0:f>ROUND(D93*20,2-INT(LOG10(ABS(D93*20))))</ns0:f>
-        <ns0:v>1.97e+82</ns0:v>
+        <ns0:v>2.52e+83</ns0:v>
       </ns0:c>
       <ns0:c r="E94" s="1">
         <ns0:f>D94</ns0:f>
-        <ns0:v>1.97e+82</ns0:v>
+        <ns0:v>2.52e+83</ns0:v>
       </ns0:c>
       <ns0:c r="F94" s="1">
         <ns0:f>ROUND(F93*1.4,-5)</ns0:f>
@@ -3930,11 +3930,11 @@
       </ns0:c>
       <ns0:c r="D95" s="1">
         <ns0:f>ROUND(D94*20,2-INT(LOG10(ABS(D94*20))))</ns0:f>
-        <ns0:v>3.94e+83</ns0:v>
+        <ns0:v>5.04e+84</ns0:v>
       </ns0:c>
       <ns0:c r="E95" s="1">
         <ns0:f>D95</ns0:f>
-        <ns0:v>3.94e+83</ns0:v>
+        <ns0:v>5.04e+84</ns0:v>
       </ns0:c>
       <ns0:c r="F95" s="1">
         <ns0:f>ROUND(F94*1.4,-5)</ns0:f>
@@ -3962,11 +3962,11 @@
       </ns0:c>
       <ns0:c r="D96" s="1">
         <ns0:f>ROUND(D95*20,2-INT(LOG10(ABS(D95*20))))</ns0:f>
-        <ns0:v>7.88e+84</ns0:v>
+        <ns0:v>1.0099999999999999e+86</ns0:v>
       </ns0:c>
       <ns0:c r="E96" s="1">
         <ns0:f>D96</ns0:f>
-        <ns0:v>7.88e+84</ns0:v>
+        <ns0:v>1.0099999999999999e+86</ns0:v>
       </ns0:c>
       <ns0:c r="F96" s="1">
         <ns0:f>ROUND(F95*1.4,-5)</ns0:f>
@@ -3994,11 +3994,11 @@
       </ns0:c>
       <ns0:c r="D97" s="1">
         <ns0:f>ROUND(D96*20,2-INT(LOG10(ABS(D96*20))))</ns0:f>
-        <ns0:v>1.58e+86</ns0:v>
+        <ns0:v>2.02e+87</ns0:v>
       </ns0:c>
       <ns0:c r="E97" s="1">
         <ns0:f>D97</ns0:f>
-        <ns0:v>1.58e+86</ns0:v>
+        <ns0:v>2.02e+87</ns0:v>
       </ns0:c>
       <ns0:c r="F97" s="1">
         <ns0:f>ROUND(F96*1.4,-5)</ns0:f>
@@ -4026,11 +4026,11 @@
       </ns0:c>
       <ns0:c r="D98" s="1">
         <ns0:f>ROUND(D97*20,2-INT(LOG10(ABS(D97*20))))</ns0:f>
-        <ns0:v>3.16e+87</ns0:v>
+        <ns0:v>4.04e+88</ns0:v>
       </ns0:c>
       <ns0:c r="E98" s="1">
         <ns0:f>D98</ns0:f>
-        <ns0:v>3.16e+87</ns0:v>
+        <ns0:v>4.04e+88</ns0:v>
       </ns0:c>
       <ns0:c r="F98" s="1">
         <ns0:f>ROUND(F97*1.4,-5)</ns0:f>
@@ -4058,11 +4058,11 @@
       </ns0:c>
       <ns0:c r="D99" s="1">
         <ns0:f>ROUND(D98*20,2-INT(LOG10(ABS(D98*20))))</ns0:f>
-        <ns0:v>6.32e+88</ns0:v>
+        <ns0:v>8.08e+89</ns0:v>
       </ns0:c>
       <ns0:c r="E99" s="1">
         <ns0:f>D99</ns0:f>
-        <ns0:v>6.32e+88</ns0:v>
+        <ns0:v>8.08e+89</ns0:v>
       </ns0:c>
       <ns0:c r="F99" s="1">
         <ns0:f>ROUND(F98*1.4,-5)</ns0:f>
@@ -4090,11 +4090,11 @@
       </ns0:c>
       <ns0:c r="D100" s="1">
         <ns0:f>ROUND(D99*20,2-INT(LOG10(ABS(D99*20))))</ns0:f>
-        <ns0:v>1.26e+90</ns0:v>
+        <ns0:v>1.62e+91</ns0:v>
       </ns0:c>
       <ns0:c r="E100" s="1">
         <ns0:f>D100</ns0:f>
-        <ns0:v>1.26e+90</ns0:v>
+        <ns0:v>1.62e+91</ns0:v>
       </ns0:c>
       <ns0:c r="F100" s="1">
         <ns0:f>ROUND(F99*1.4,-5)</ns0:f>
@@ -4122,11 +4122,11 @@
       </ns0:c>
       <ns0:c r="D101" s="1">
         <ns0:f>ROUND(D100*20,2-INT(LOG10(ABS(D100*20))))</ns0:f>
-        <ns0:v>2.52e+91</ns0:v>
+        <ns0:v>3.24e+92</ns0:v>
       </ns0:c>
       <ns0:c r="E101" s="1">
         <ns0:f>D101</ns0:f>
-        <ns0:v>2.52e+91</ns0:v>
+        <ns0:v>3.24e+92</ns0:v>
       </ns0:c>
       <ns0:c r="F101" s="1">
         <ns0:f>ROUND(F100*1.4,-5)</ns0:f>
@@ -4154,11 +4154,11 @@
       </ns0:c>
       <ns0:c r="D102" s="1">
         <ns0:f>ROUND(D101*20,2-INT(LOG10(ABS(D101*20))))</ns0:f>
-        <ns0:v>5.04e+92</ns0:v>
+        <ns0:v>6.48e+93</ns0:v>
       </ns0:c>
       <ns0:c r="E102" s="1">
         <ns0:f>D102</ns0:f>
-        <ns0:v>5.04e+92</ns0:v>
+        <ns0:v>6.48e+93</ns0:v>
       </ns0:c>
       <ns0:c r="F102" s="1">
         <ns0:f>ROUND(F101*1.4,-5)</ns0:f>
@@ -4186,11 +4186,11 @@
       </ns0:c>
       <ns0:c r="D103" s="1">
         <ns0:f>ROUND(D102*20,2-INT(LOG10(ABS(D102*20))))</ns0:f>
-        <ns0:v>1.01e+94</ns0:v>
+        <ns0:v>1.3000000000000001e+95</ns0:v>
       </ns0:c>
       <ns0:c r="E103" s="1">
         <ns0:f>D103</ns0:f>
-        <ns0:v>1.01e+94</ns0:v>
+        <ns0:v>1.3000000000000001e+95</ns0:v>
       </ns0:c>
       <ns0:c r="F103" s="1">
         <ns0:f>ROUND(F102*1.4,-5)</ns0:f>
@@ -4218,11 +4218,11 @@
       </ns0:c>
       <ns0:c r="D104" s="1">
         <ns0:f>ROUND(D103*20,2-INT(LOG10(ABS(D103*20))))</ns0:f>
-        <ns0:v>2.0200000000000002e+95</ns0:v>
+        <ns0:v>2.6e+96</ns0:v>
       </ns0:c>
       <ns0:c r="E104" s="1">
         <ns0:f>D104</ns0:f>
-        <ns0:v>2.0200000000000002e+95</ns0:v>
+        <ns0:v>2.6e+96</ns0:v>
       </ns0:c>
       <ns0:c r="F104" s="1">
         <ns0:f>ROUND(F103*1.4,-5)</ns0:f>
@@ -4250,11 +4250,11 @@
       </ns0:c>
       <ns0:c r="D105" s="1">
         <ns0:f>ROUND(D104*20,2-INT(LOG10(ABS(D104*20))))</ns0:f>
-        <ns0:v>4.04e+96</ns0:v>
+        <ns0:v>5.2e+97</ns0:v>
       </ns0:c>
       <ns0:c r="E105" s="1">
         <ns0:f>D105</ns0:f>
-        <ns0:v>4.04e+96</ns0:v>
+        <ns0:v>5.2e+97</ns0:v>
       </ns0:c>
       <ns0:c r="F105" s="1">
         <ns0:f>ROUND(F104*1.4,-5)</ns0:f>
@@ -4282,11 +4282,11 @@
       </ns0:c>
       <ns0:c r="D106" s="1">
         <ns0:f>ROUND(D105*20,2-INT(LOG10(ABS(D105*20))))</ns0:f>
-        <ns0:v>8.08e+97</ns0:v>
+        <ns0:v>1.04e+99</ns0:v>
       </ns0:c>
       <ns0:c r="E106" s="1">
         <ns0:f>D106</ns0:f>
-        <ns0:v>8.08e+97</ns0:v>
+        <ns0:v>1.04e+99</ns0:v>
       </ns0:c>
       <ns0:c r="F106" s="1">
         <ns0:f>ROUND(F105*1.4,-5)</ns0:f>
@@ -4314,11 +4314,11 @@
       </ns0:c>
       <ns0:c r="D107" s="1">
         <ns0:f>ROUND(D106*20,2-INT(LOG10(ABS(D106*20))))</ns0:f>
-        <ns0:v>1.62e+99</ns0:v>
+        <ns0:v>2.08e+100</ns0:v>
       </ns0:c>
       <ns0:c r="E107" s="1">
         <ns0:f>D107</ns0:f>
-        <ns0:v>1.62e+99</ns0:v>
+        <ns0:v>2.08e+100</ns0:v>
       </ns0:c>
       <ns0:c r="F107" s="1">
         <ns0:f>ROUND(F106*1.4,-5)</ns0:f>
@@ -4346,11 +4346,11 @@
       </ns0:c>
       <ns0:c r="D108" s="1">
         <ns0:f>ROUND(D107*20,2-INT(LOG10(ABS(D107*20))))</ns0:f>
-        <ns0:v>3.24e+100</ns0:v>
+        <ns0:v>4.1599999999999996e+101</ns0:v>
       </ns0:c>
       <ns0:c r="E108" s="1">
         <ns0:f>D108</ns0:f>
-        <ns0:v>3.24e+100</ns0:v>
+        <ns0:v>4.1599999999999996e+101</ns0:v>
       </ns0:c>
       <ns0:c r="F108" s="1">
         <ns0:f>ROUND(F107*1.4,-5)</ns0:f>
@@ -4378,11 +4378,11 @@
       </ns0:c>
       <ns0:c r="D109" s="1">
         <ns0:f>ROUND(D108*20,2-INT(LOG10(ABS(D108*20))))</ns0:f>
-        <ns0:v>6.48e+101</ns0:v>
+        <ns0:v>8.32e+102</ns0:v>
       </ns0:c>
       <ns0:c r="E109" s="1">
         <ns0:f>D109</ns0:f>
-        <ns0:v>6.48e+101</ns0:v>
+        <ns0:v>8.32e+102</ns0:v>
       </ns0:c>
       <ns0:c r="F109" s="1">
         <ns0:f>ROUND(F108*1.4,-5)</ns0:f>
@@ -4410,11 +4410,11 @@
       </ns0:c>
       <ns0:c r="D110" s="1">
         <ns0:f>ROUND(D109*20,2-INT(LOG10(ABS(D109*20))))</ns0:f>
-        <ns0:v>1.2999999999999999e+103</ns0:v>
+        <ns0:v>1.66e+104</ns0:v>
       </ns0:c>
       <ns0:c r="E110" s="1">
         <ns0:f>D110</ns0:f>
-        <ns0:v>1.2999999999999999e+103</ns0:v>
+        <ns0:v>1.66e+104</ns0:v>
       </ns0:c>
       <ns0:c r="F110" s="1">
         <ns0:f>ROUND(F109*1.4,-5)</ns0:f>
@@ -4442,11 +4442,11 @@
       </ns0:c>
       <ns0:c r="D111" s="1">
         <ns0:f>ROUND(D110*20,2-INT(LOG10(ABS(D110*20))))</ns0:f>
-        <ns0:v>2.6000000000000003e+104</ns0:v>
+        <ns0:v>3.32e+105</ns0:v>
       </ns0:c>
       <ns0:c r="E111" s="1">
         <ns0:f>D111</ns0:f>
-        <ns0:v>2.6000000000000003e+104</ns0:v>
+        <ns0:v>3.32e+105</ns0:v>
       </ns0:c>
       <ns0:c r="F111" s="1">
         <ns0:f>ROUND(F110*1.4,-5)</ns0:f>
@@ -4474,11 +4474,11 @@
       </ns0:c>
       <ns0:c r="D112" s="1">
         <ns0:f>ROUND(D111*20,2-INT(LOG10(ABS(D111*20))))</ns0:f>
-        <ns0:v>5.2e+105</ns0:v>
+        <ns0:v>6.640000000000001e+106</ns0:v>
       </ns0:c>
       <ns0:c r="E112" s="1">
         <ns0:f>D112</ns0:f>
-        <ns0:v>5.2e+105</ns0:v>
+        <ns0:v>6.640000000000001e+106</ns0:v>
       </ns0:c>
       <ns0:c r="F112" s="1">
         <ns0:f>ROUND(F111*1.4,-5)</ns0:f>
@@ -4506,11 +4506,11 @@
       </ns0:c>
       <ns0:c r="D113" s="1">
         <ns0:f>ROUND(D112*20,2-INT(LOG10(ABS(D112*20))))</ns0:f>
-        <ns0:v>1.04e+107</ns0:v>
+        <ns0:v>1.33e+108</ns0:v>
       </ns0:c>
       <ns0:c r="E113" s="1">
         <ns0:f>D113</ns0:f>
-        <ns0:v>1.04e+107</ns0:v>
+        <ns0:v>1.33e+108</ns0:v>
       </ns0:c>
       <ns0:c r="F113" s="1">
         <ns0:f>ROUND(F112*1.4,-5)</ns0:f>
@@ -4538,11 +4538,11 @@
       </ns0:c>
       <ns0:c r="D114" s="1">
         <ns0:f>ROUND(D113*20,2-INT(LOG10(ABS(D113*20))))</ns0:f>
-        <ns0:v>2.08e+108</ns0:v>
+        <ns0:v>2.66e+109</ns0:v>
       </ns0:c>
       <ns0:c r="E114" s="1">
         <ns0:f>D114</ns0:f>
-        <ns0:v>2.08e+108</ns0:v>
+        <ns0:v>2.66e+109</ns0:v>
       </ns0:c>
       <ns0:c r="F114" s="1">
         <ns0:f>ROUND(F113*1.4,-5)</ns0:f>
@@ -4570,11 +4570,11 @@
       </ns0:c>
       <ns0:c r="D115" s="1">
         <ns0:f>ROUND(D114*20,2-INT(LOG10(ABS(D114*20))))</ns0:f>
-        <ns0:v>4.16e+109</ns0:v>
+        <ns0:v>5.32e+110</ns0:v>
       </ns0:c>
       <ns0:c r="E115" s="1">
         <ns0:f>D115</ns0:f>
-        <ns0:v>4.16e+109</ns0:v>
+        <ns0:v>5.32e+110</ns0:v>
       </ns0:c>
       <ns0:c r="F115" s="1">
         <ns0:f>ROUND(F114*1.4,-5)</ns0:f>
@@ -4602,11 +4602,11 @@
       </ns0:c>
       <ns0:c r="D116" s="1">
         <ns0:f>ROUND(D115*20,2-INT(LOG10(ABS(D115*20))))</ns0:f>
-        <ns0:v>8.32e+110</ns0:v>
+        <ns0:v>1.06e+112</ns0:v>
       </ns0:c>
       <ns0:c r="E116" s="1">
         <ns0:f>D116</ns0:f>
-        <ns0:v>8.32e+110</ns0:v>
+        <ns0:v>1.06e+112</ns0:v>
       </ns0:c>
       <ns0:c r="F116" s="1">
         <ns0:f>ROUND(F115*1.4,-5)</ns0:f>
@@ -4634,11 +4634,11 @@
       </ns0:c>
       <ns0:c r="D117" s="1">
         <ns0:f>ROUND(D116*20,2-INT(LOG10(ABS(D116*20))))</ns0:f>
-        <ns0:v>1.66e+112</ns0:v>
+        <ns0:v>2.1199999999999997e+113</ns0:v>
       </ns0:c>
       <ns0:c r="E117" s="1">
         <ns0:f>D117</ns0:f>
-        <ns0:v>1.66e+112</ns0:v>
+        <ns0:v>2.1199999999999997e+113</ns0:v>
       </ns0:c>
       <ns0:c r="F117" s="1">
         <ns0:f>ROUND(F116*1.4,-5)</ns0:f>
@@ -4666,11 +4666,11 @@
       </ns0:c>
       <ns0:c r="D118" s="1">
         <ns0:f>ROUND(D117*20,2-INT(LOG10(ABS(D117*20))))</ns0:f>
-        <ns0:v>3.3199999999999995e+113</ns0:v>
+        <ns0:v>4.2400000000000003e+114</ns0:v>
       </ns0:c>
       <ns0:c r="E118" s="1">
         <ns0:f>D118</ns0:f>
-        <ns0:v>3.3199999999999995e+113</ns0:v>
+        <ns0:v>4.2400000000000003e+114</ns0:v>
       </ns0:c>
       <ns0:c r="F118" s="1">
         <ns0:f>ROUND(F117*1.4,-5)</ns0:f>
@@ -4698,11 +4698,11 @@
       </ns0:c>
       <ns0:c r="D119" s="1">
         <ns0:f>ROUND(D118*20,2-INT(LOG10(ABS(D118*20))))</ns0:f>
-        <ns0:v>6.64e+114</ns0:v>
+        <ns0:v>8.48e+115</ns0:v>
       </ns0:c>
       <ns0:c r="E119" s="1">
         <ns0:f>D119</ns0:f>
-        <ns0:v>6.64e+114</ns0:v>
+        <ns0:v>8.48e+115</ns0:v>
       </ns0:c>
       <ns0:c r="F119" s="1">
         <ns0:f>ROUND(F118*1.4,-5)</ns0:f>
@@ -4730,11 +4730,11 @@
       </ns0:c>
       <ns0:c r="D120" s="1">
         <ns0:f>ROUND(D119*20,2-INT(LOG10(ABS(D119*20))))</ns0:f>
-        <ns0:v>1.3299999999999999e+116</ns0:v>
+        <ns0:v>1.7e+117</ns0:v>
       </ns0:c>
       <ns0:c r="E120" s="1">
         <ns0:f>D120</ns0:f>
-        <ns0:v>1.3299999999999999e+116</ns0:v>
+        <ns0:v>1.7e+117</ns0:v>
       </ns0:c>
       <ns0:c r="F120" s="1">
         <ns0:f>ROUND(F119*1.4,-5)</ns0:f>
@@ -4762,11 +4762,11 @@
       </ns0:c>
       <ns0:c r="D121" s="1">
         <ns0:f>ROUND(D120*20,2-INT(LOG10(ABS(D120*20))))</ns0:f>
-        <ns0:v>2.66e+117</ns0:v>
+        <ns0:v>3.4e+118</ns0:v>
       </ns0:c>
       <ns0:c r="E121" s="1">
         <ns0:f>D121</ns0:f>
-        <ns0:v>2.66e+117</ns0:v>
+        <ns0:v>3.4e+118</ns0:v>
       </ns0:c>
       <ns0:c r="F121" s="1">
         <ns0:f>ROUND(F120*1.4,-5)</ns0:f>
@@ -4794,11 +4794,11 @@
       </ns0:c>
       <ns0:c r="D122" s="1">
         <ns0:f>ROUND(D121*20,2-INT(LOG10(ABS(D121*20))))</ns0:f>
-        <ns0:v>5.32e+118</ns0:v>
+        <ns0:v>6.8e+119</ns0:v>
       </ns0:c>
       <ns0:c r="E122" s="1">
         <ns0:f>D122</ns0:f>
-        <ns0:v>5.32e+118</ns0:v>
+        <ns0:v>6.8e+119</ns0:v>
       </ns0:c>
       <ns0:c r="F122" s="1">
         <ns0:f>ROUND(F121*1.4,-5)</ns0:f>
@@ -4826,11 +4826,11 @@
       </ns0:c>
       <ns0:c r="D123" s="1">
         <ns0:f>ROUND(D122*20,2-INT(LOG10(ABS(D122*20))))</ns0:f>
-        <ns0:v>1.06e+120</ns0:v>
+        <ns0:v>1.36e+121</ns0:v>
       </ns0:c>
       <ns0:c r="E123" s="1">
         <ns0:f>D123</ns0:f>
-        <ns0:v>1.06e+120</ns0:v>
+        <ns0:v>1.36e+121</ns0:v>
       </ns0:c>
       <ns0:c r="F123" s="1">
         <ns0:f>ROUND(F122*1.4,-5)</ns0:f>
@@ -4858,11 +4858,11 @@
       </ns0:c>
       <ns0:c r="D124" s="1">
         <ns0:f>ROUND(D123*20,2-INT(LOG10(ABS(D123*20))))</ns0:f>
-        <ns0:v>2.12e+121</ns0:v>
+        <ns0:v>2.72e+122</ns0:v>
       </ns0:c>
       <ns0:c r="E124" s="1">
         <ns0:f>D124</ns0:f>
-        <ns0:v>2.12e+121</ns0:v>
+        <ns0:v>2.72e+122</ns0:v>
       </ns0:c>
       <ns0:c r="F124" s="1">
         <ns0:f>ROUND(F123*1.4,-5)</ns0:f>
@@ -4890,11 +4890,11 @@
       </ns0:c>
       <ns0:c r="D125" s="1">
         <ns0:f>ROUND(D124*20,2-INT(LOG10(ABS(D124*20))))</ns0:f>
-        <ns0:v>4.24e+122</ns0:v>
+        <ns0:v>5.44e+123</ns0:v>
       </ns0:c>
       <ns0:c r="E125" s="1">
         <ns0:f>D125</ns0:f>
-        <ns0:v>4.24e+122</ns0:v>
+        <ns0:v>5.44e+123</ns0:v>
       </ns0:c>
       <ns0:c r="F125" s="1">
         <ns0:f>ROUND(F124*1.4,-5)</ns0:f>
@@ -4922,11 +4922,11 @@
       </ns0:c>
       <ns0:c r="D126" s="1">
         <ns0:f>ROUND(D125*20,2-INT(LOG10(ABS(D125*20))))</ns0:f>
-        <ns0:v>8.48e+123</ns0:v>
+        <ns0:v>1.09e+125</ns0:v>
       </ns0:c>
       <ns0:c r="E126" s="1">
         <ns0:f>D126</ns0:f>
-        <ns0:v>8.48e+123</ns0:v>
+        <ns0:v>1.09e+125</ns0:v>
       </ns0:c>
       <ns0:c r="F126" s="1">
         <ns0:f>ROUND(F125*1.4,-5)</ns0:f>
@@ -4954,11 +4954,11 @@
       </ns0:c>
       <ns0:c r="D127" s="1">
         <ns0:f>ROUND(D126*20,2-INT(LOG10(ABS(D126*20))))</ns0:f>
-        <ns0:v>1.7e+125</ns0:v>
+        <ns0:v>2.18e+126</ns0:v>
       </ns0:c>
       <ns0:c r="E127" s="1">
         <ns0:f>D127</ns0:f>
-        <ns0:v>1.7e+125</ns0:v>
+        <ns0:v>2.18e+126</ns0:v>
       </ns0:c>
       <ns0:c r="F127" s="1">
         <ns0:f>ROUND(F126*1.4,-5)</ns0:f>
@@ -4986,11 +4986,11 @@
       </ns0:c>
       <ns0:c r="D128" s="1">
         <ns0:f>ROUND(D127*20,2-INT(LOG10(ABS(D127*20))))</ns0:f>
-        <ns0:v>3.4000000000000005e+126</ns0:v>
+        <ns0:v>4.36e+127</ns0:v>
       </ns0:c>
       <ns0:c r="E128" s="1">
         <ns0:f>D128</ns0:f>
-        <ns0:v>3.4000000000000005e+126</ns0:v>
+        <ns0:v>4.36e+127</ns0:v>
       </ns0:c>
       <ns0:c r="F128" s="1">
         <ns0:f>ROUND(F127*1.4,-5)</ns0:f>
@@ -5018,11 +5018,11 @@
       </ns0:c>
       <ns0:c r="D129" s="1">
         <ns0:f>ROUND(D128*20,2-INT(LOG10(ABS(D128*20))))</ns0:f>
-        <ns0:v>6.8e+127</ns0:v>
+        <ns0:v>8.72e+128</ns0:v>
       </ns0:c>
       <ns0:c r="E129" s="1">
         <ns0:f>D129</ns0:f>
-        <ns0:v>6.8e+127</ns0:v>
+        <ns0:v>8.72e+128</ns0:v>
       </ns0:c>
       <ns0:c r="F129" s="1">
         <ns0:f>ROUND(F128*1.4,-5)</ns0:f>
@@ -5050,11 +5050,11 @@
       </ns0:c>
       <ns0:c r="D130" s="1">
         <ns0:f>ROUND(D129*20,2-INT(LOG10(ABS(D129*20))))</ns0:f>
-        <ns0:v>1.36e+129</ns0:v>
+        <ns0:v>1.74e+130</ns0:v>
       </ns0:c>
       <ns0:c r="E130" s="1">
         <ns0:f>D130</ns0:f>
-        <ns0:v>1.36e+129</ns0:v>
+        <ns0:v>1.74e+130</ns0:v>
       </ns0:c>
       <ns0:c r="F130" s="1">
         <ns0:f>ROUND(F129*1.4,-5)</ns0:f>
@@ -5082,11 +5082,11 @@
       </ns0:c>
       <ns0:c r="D131" s="1">
         <ns0:f>ROUND(D130*20,2-INT(LOG10(ABS(D130*20))))</ns0:f>
-        <ns0:v>2.7199999999999997e+130</ns0:v>
+        <ns0:v>3.4800000000000003e+131</ns0:v>
       </ns0:c>
       <ns0:c r="E131" s="1">
         <ns0:f>D131</ns0:f>
-        <ns0:v>2.7199999999999997e+130</ns0:v>
+        <ns0:v>3.4800000000000003e+131</ns0:v>
       </ns0:c>
       <ns0:c r="F131" s="1">
         <ns0:f>ROUND(F130*1.4,-5)</ns0:f>
@@ -5114,11 +5114,11 @@
       </ns0:c>
       <ns0:c r="D132" s="1">
         <ns0:f>ROUND(D131*20,2-INT(LOG10(ABS(D131*20))))</ns0:f>
-        <ns0:v>5.44e+131</ns0:v>
+        <ns0:v>6.96e+132</ns0:v>
       </ns0:c>
       <ns0:c r="E132" s="1">
         <ns0:f>D132</ns0:f>
-        <ns0:v>5.44e+131</ns0:v>
+        <ns0:v>6.96e+132</ns0:v>
       </ns0:c>
       <ns0:c r="F132" s="1">
         <ns0:f>ROUND(F131*1.4,-5)</ns0:f>
@@ -5146,11 +5146,11 @@
       </ns0:c>
       <ns0:c r="D133" s="1">
         <ns0:f>ROUND(D132*20,2-INT(LOG10(ABS(D132*20))))</ns0:f>
-        <ns0:v>1.09e+133</ns0:v>
+        <ns0:v>1.39e+134</ns0:v>
       </ns0:c>
       <ns0:c r="E133" s="1">
         <ns0:f>D133</ns0:f>
-        <ns0:v>1.09e+133</ns0:v>
+        <ns0:v>1.39e+134</ns0:v>
       </ns0:c>
       <ns0:c r="F133" s="1">
         <ns0:f>ROUND(F132*1.4,-5)</ns0:f>
@@ -5178,11 +5178,11 @@
       </ns0:c>
       <ns0:c r="D134" s="1">
         <ns0:f>ROUND(D133*20,2-INT(LOG10(ABS(D133*20))))</ns0:f>
-        <ns0:v>2.18e+134</ns0:v>
+        <ns0:v>2.7799999999999997e+135</ns0:v>
       </ns0:c>
       <ns0:c r="E134" s="1">
         <ns0:f>D134</ns0:f>
-        <ns0:v>2.18e+134</ns0:v>
+        <ns0:v>2.7799999999999997e+135</ns0:v>
       </ns0:c>
       <ns0:c r="F134" s="1">
         <ns0:f>ROUND(F133*1.4,-5)</ns0:f>
@@ -5210,11 +5210,11 @@
       </ns0:c>
       <ns0:c r="D135" s="1">
         <ns0:f>ROUND(D134*20,2-INT(LOG10(ABS(D134*20))))</ns0:f>
-        <ns0:v>4.36e+135</ns0:v>
+        <ns0:v>5.56e+136</ns0:v>
       </ns0:c>
       <ns0:c r="E135" s="1">
         <ns0:f>D135</ns0:f>
-        <ns0:v>4.36e+135</ns0:v>
+        <ns0:v>5.56e+136</ns0:v>
       </ns0:c>
       <ns0:c r="F135" s="1">
         <ns0:f>ROUND(F134*1.4,-5)</ns0:f>
@@ -5242,11 +5242,11 @@
       </ns0:c>
       <ns0:c r="D136" s="1">
         <ns0:f>ROUND(D135*20,2-INT(LOG10(ABS(D135*20))))</ns0:f>
-        <ns0:v>8.719999999999999e+136</ns0:v>
+        <ns0:v>1.11e+138</ns0:v>
       </ns0:c>
       <ns0:c r="E136" s="1">
         <ns0:f>D136</ns0:f>
-        <ns0:v>8.719999999999999e+136</ns0:v>
+        <ns0:v>1.11e+138</ns0:v>
       </ns0:c>
       <ns0:c r="F136" s="1">
         <ns0:f>ROUND(F135*1.4,-5)</ns0:f>
@@ -5274,11 +5274,11 @@
       </ns0:c>
       <ns0:c r="D137" s="1">
         <ns0:f>ROUND(D136*20,2-INT(LOG10(ABS(D136*20))))</ns0:f>
-        <ns0:v>1.74e+138</ns0:v>
+        <ns0:v>2.22e+139</ns0:v>
       </ns0:c>
       <ns0:c r="E137" s="1">
         <ns0:f>D137</ns0:f>
-        <ns0:v>1.74e+138</ns0:v>
+        <ns0:v>2.22e+139</ns0:v>
       </ns0:c>
       <ns0:c r="F137" s="1">
         <ns0:f>ROUND(F136*1.4,-5)</ns0:f>
@@ -5306,11 +5306,11 @@
       </ns0:c>
       <ns0:c r="D138" s="1">
         <ns0:f>ROUND(D137*20,2-INT(LOG10(ABS(D137*20))))</ns0:f>
-        <ns0:v>3.48e+139</ns0:v>
+        <ns0:v>4.44e+140</ns0:v>
       </ns0:c>
       <ns0:c r="E138" s="1">
         <ns0:f>D138</ns0:f>
-        <ns0:v>3.48e+139</ns0:v>
+        <ns0:v>4.44e+140</ns0:v>
       </ns0:c>
       <ns0:c r="F138" s="1">
         <ns0:f>ROUND(F137*1.4,-5)</ns0:f>
@@ -5338,11 +5338,11 @@
       </ns0:c>
       <ns0:c r="D139" s="1">
         <ns0:f>ROUND(D138*20,2-INT(LOG10(ABS(D138*20))))</ns0:f>
-        <ns0:v>6.96e+140</ns0:v>
+        <ns0:v>8.88e+141</ns0:v>
       </ns0:c>
       <ns0:c r="E139" s="1">
         <ns0:f>D139</ns0:f>
-        <ns0:v>6.96e+140</ns0:v>
+        <ns0:v>8.88e+141</ns0:v>
       </ns0:c>
       <ns0:c r="F139" s="1">
         <ns0:f>ROUND(F138*1.4,-5)</ns0:f>
@@ -5370,11 +5370,11 @@
       </ns0:c>
       <ns0:c r="D140" s="1">
         <ns0:f>ROUND(D139*20,2-INT(LOG10(ABS(D139*20))))</ns0:f>
-        <ns0:v>1.39e+142</ns0:v>
+        <ns0:v>1.78e+143</ns0:v>
       </ns0:c>
       <ns0:c r="E140" s="1">
         <ns0:f>D140</ns0:f>
-        <ns0:v>1.39e+142</ns0:v>
+        <ns0:v>1.78e+143</ns0:v>
       </ns0:c>
       <ns0:c r="F140" s="1">
         <ns0:f>ROUND(F139*1.4,-5)</ns0:f>
@@ -5402,11 +5402,11 @@
       </ns0:c>
       <ns0:c r="D141" s="1">
         <ns0:f>ROUND(D140*20,2-INT(LOG10(ABS(D140*20))))</ns0:f>
-        <ns0:v>2.78e+143</ns0:v>
+        <ns0:v>3.5599999999999996e+144</ns0:v>
       </ns0:c>
       <ns0:c r="E141" s="1">
         <ns0:f>D141</ns0:f>
-        <ns0:v>2.78e+143</ns0:v>
+        <ns0:v>3.5599999999999996e+144</ns0:v>
       </ns0:c>
       <ns0:c r="F141" s="1">
         <ns0:f>ROUND(F140*1.4,-5)</ns0:f>
@@ -5434,11 +5434,11 @@
       </ns0:c>
       <ns0:c r="D142" s="1">
         <ns0:f>ROUND(D141*20,2-INT(LOG10(ABS(D141*20))))</ns0:f>
-        <ns0:v>5.56e+144</ns0:v>
+        <ns0:v>7.120000000000001e+145</ns0:v>
       </ns0:c>
       <ns0:c r="E142" s="1">
         <ns0:f>D142</ns0:f>
-        <ns0:v>5.56e+144</ns0:v>
+        <ns0:v>7.120000000000001e+145</ns0:v>
       </ns0:c>
       <ns0:c r="F142" s="1">
         <ns0:f>ROUND(F141*1.4,-5)</ns0:f>
@@ -5466,11 +5466,11 @@
       </ns0:c>
       <ns0:c r="D143" s="1">
         <ns0:f>ROUND(D142*20,2-INT(LOG10(ABS(D142*20))))</ns0:f>
-        <ns0:v>1.1100000000000001e+146</ns0:v>
+        <ns0:v>1.4200000000000002e+147</ns0:v>
       </ns0:c>
       <ns0:c r="E143" s="1">
         <ns0:f>D143</ns0:f>
-        <ns0:v>1.1100000000000001e+146</ns0:v>
+        <ns0:v>1.4200000000000002e+147</ns0:v>
       </ns0:c>
       <ns0:c r="F143" s="1">
         <ns0:f>ROUND(F142*1.4,-5)</ns0:f>
@@ -5498,11 +5498,11 @@
       </ns0:c>
       <ns0:c r="D144" s="1">
         <ns0:f>ROUND(D143*20,2-INT(LOG10(ABS(D143*20))))</ns0:f>
-        <ns0:v>2.22e+147</ns0:v>
+        <ns0:v>2.84e+148</ns0:v>
       </ns0:c>
       <ns0:c r="E144" s="1">
         <ns0:f>D144</ns0:f>
-        <ns0:v>2.22e+147</ns0:v>
+        <ns0:v>2.84e+148</ns0:v>
       </ns0:c>
       <ns0:c r="F144" s="1">
         <ns0:f>ROUND(F143*1.4,-5)</ns0:f>
@@ -5530,11 +5530,11 @@
       </ns0:c>
       <ns0:c r="D145" s="1">
         <ns0:f>ROUND(D144*20,2-INT(LOG10(ABS(D144*20))))</ns0:f>
-        <ns0:v>4.44e+148</ns0:v>
+        <ns0:v>5.68e+149</ns0:v>
       </ns0:c>
       <ns0:c r="E145" s="1">
         <ns0:f>D145</ns0:f>
-        <ns0:v>4.44e+148</ns0:v>
+        <ns0:v>5.68e+149</ns0:v>
       </ns0:c>
       <ns0:c r="F145" s="1">
         <ns0:f>ROUND(F144*1.4,-5)</ns0:f>
@@ -5562,11 +5562,11 @@
       </ns0:c>
       <ns0:c r="D146" s="1">
         <ns0:f>ROUND(D145*20,2-INT(LOG10(ABS(D145*20))))</ns0:f>
-        <ns0:v>8.88e+149</ns0:v>
+        <ns0:v>1.14e+151</ns0:v>
       </ns0:c>
       <ns0:c r="E146" s="1">
         <ns0:f>D146</ns0:f>
-        <ns0:v>8.88e+149</ns0:v>
+        <ns0:v>1.14e+151</ns0:v>
       </ns0:c>
       <ns0:c r="F146" s="1">
         <ns0:f>ROUND(F145*1.4,-5)</ns0:f>
@@ -5594,11 +5594,11 @@
       </ns0:c>
       <ns0:c r="D147" s="1">
         <ns0:f>ROUND(D146*20,2-INT(LOG10(ABS(D146*20))))</ns0:f>
-        <ns0:v>1.78e+151</ns0:v>
+        <ns0:v>2.28e+152</ns0:v>
       </ns0:c>
       <ns0:c r="E147" s="1">
         <ns0:f>D147</ns0:f>
-        <ns0:v>1.78e+151</ns0:v>
+        <ns0:v>2.28e+152</ns0:v>
       </ns0:c>
       <ns0:c r="F147" s="1">
         <ns0:f>ROUND(F146*1.4,-5)</ns0:f>
@@ -5626,11 +5626,11 @@
       </ns0:c>
       <ns0:c r="D148" s="1">
         <ns0:f>ROUND(D147*20,2-INT(LOG10(ABS(D147*20))))</ns0:f>
-        <ns0:v>3.5599999999999998e+152</ns0:v>
+        <ns0:v>4.56e+153</ns0:v>
       </ns0:c>
       <ns0:c r="E148" s="1">
         <ns0:f>D148</ns0:f>
-        <ns0:v>3.5599999999999998e+152</ns0:v>
+        <ns0:v>4.56e+153</ns0:v>
       </ns0:c>
       <ns0:c r="F148" s="1">
         <ns0:f>ROUND(F147*1.4,-5)</ns0:f>
@@ -5658,11 +5658,11 @@
       </ns0:c>
       <ns0:c r="D149" s="1">
         <ns0:f>ROUND(D148*20,2-INT(LOG10(ABS(D148*20))))</ns0:f>
-        <ns0:v>7.12e+153</ns0:v>
+        <ns0:v>9.12e+154</ns0:v>
       </ns0:c>
       <ns0:c r="E149" s="1">
         <ns0:f>D149</ns0:f>
-        <ns0:v>7.12e+153</ns0:v>
+        <ns0:v>9.12e+154</ns0:v>
       </ns0:c>
       <ns0:c r="F149" s="1">
         <ns0:f>ROUND(F148*1.4,-5)</ns0:f>
@@ -5690,11 +5690,11 @@
       </ns0:c>
       <ns0:c r="D150" s="1">
         <ns0:f>ROUND(D149*20,2-INT(LOG10(ABS(D149*20))))</ns0:f>
-        <ns0:v>1.42e+155</ns0:v>
+        <ns0:v>1.82e+156</ns0:v>
       </ns0:c>
       <ns0:c r="E150" s="1">
         <ns0:f>D150</ns0:f>
-        <ns0:v>1.42e+155</ns0:v>
+        <ns0:v>1.82e+156</ns0:v>
       </ns0:c>
       <ns0:c r="F150" s="1">
         <ns0:f>ROUND(F149*1.4,-5)</ns0:f>
@@ -5722,11 +5722,11 @@
       </ns0:c>
       <ns0:c r="D151" s="1">
         <ns0:f>ROUND(D150*20,2-INT(LOG10(ABS(D150*20))))</ns0:f>
-        <ns0:v>2.84e+156</ns0:v>
+        <ns0:v>3.64e+157</ns0:v>
       </ns0:c>
       <ns0:c r="E151" s="1">
         <ns0:f>D151</ns0:f>
-        <ns0:v>2.84e+156</ns0:v>
+        <ns0:v>3.64e+157</ns0:v>
       </ns0:c>
       <ns0:c r="F151" s="1">
         <ns0:f>ROUND(F150*1.4,-5)</ns0:f>
@@ -5754,11 +5754,11 @@
       </ns0:c>
       <ns0:c r="D152" s="1">
         <ns0:f>ROUND(D151*20,2-INT(LOG10(ABS(D151*20))))</ns0:f>
-        <ns0:v>5.68e+157</ns0:v>
+        <ns0:v>7.28e+158</ns0:v>
       </ns0:c>
       <ns0:c r="E152" s="1">
         <ns0:f>D152</ns0:f>
-        <ns0:v>5.68e+157</ns0:v>
+        <ns0:v>7.28e+158</ns0:v>
       </ns0:c>
       <ns0:c r="F152" s="1">
         <ns0:f>ROUND(F151*1.4,-5)</ns0:f>
@@ -5786,11 +5786,11 @@
       </ns0:c>
       <ns0:c r="D153" s="1">
         <ns0:f>ROUND(D152*20,2-INT(LOG10(ABS(D152*20))))</ns0:f>
-        <ns0:v>1.14e+159</ns0:v>
+        <ns0:v>1.4599999999999998e+160</ns0:v>
       </ns0:c>
       <ns0:c r="E153" s="1">
         <ns0:f>D153</ns0:f>
-        <ns0:v>1.14e+159</ns0:v>
+        <ns0:v>1.4599999999999998e+160</ns0:v>
       </ns0:c>
       <ns0:c r="F153" s="1">
         <ns0:f>ROUND(F152*1.4,-5)</ns0:f>
@@ -5818,11 +5818,11 @@
       </ns0:c>
       <ns0:c r="D154" s="1">
         <ns0:f>ROUND(D153*20,2-INT(LOG10(ABS(D153*20))))</ns0:f>
-        <ns0:v>2.28e+160</ns0:v>
+        <ns0:v>2.92e+161</ns0:v>
       </ns0:c>
       <ns0:c r="E154" s="1">
         <ns0:f>D154</ns0:f>
-        <ns0:v>2.28e+160</ns0:v>
+        <ns0:v>2.92e+161</ns0:v>
       </ns0:c>
       <ns0:c r="F154" s="1">
         <ns0:f>ROUND(F153*1.4,-5)</ns0:f>
@@ -5850,11 +5850,11 @@
       </ns0:c>
       <ns0:c r="D155" s="1">
         <ns0:f>ROUND(D154*20,2-INT(LOG10(ABS(D154*20))))</ns0:f>
-        <ns0:v>4.56e+161</ns0:v>
+        <ns0:v>5.84e+162</ns0:v>
       </ns0:c>
       <ns0:c r="E155" s="1">
         <ns0:f>D155</ns0:f>
-        <ns0:v>4.56e+161</ns0:v>
+        <ns0:v>5.84e+162</ns0:v>
       </ns0:c>
       <ns0:c r="F155" s="1">
         <ns0:f>ROUND(F154*1.4,-5)</ns0:f>
@@ -5882,11 +5882,11 @@
       </ns0:c>
       <ns0:c r="D156" s="1">
         <ns0:f>ROUND(D155*20,2-INT(LOG10(ABS(D155*20))))</ns0:f>
-        <ns0:v>9.12e+162</ns0:v>
+        <ns0:v>1.17e+164</ns0:v>
       </ns0:c>
       <ns0:c r="E156" s="1">
         <ns0:f>D156</ns0:f>
-        <ns0:v>9.12e+162</ns0:v>
+        <ns0:v>1.17e+164</ns0:v>
       </ns0:c>
       <ns0:c r="F156" s="1">
         <ns0:f>ROUND(F155*1.4,-5)</ns0:f>
@@ -5914,11 +5914,11 @@
       </ns0:c>
       <ns0:c r="D157" s="1">
         <ns0:f>ROUND(D156*20,2-INT(LOG10(ABS(D156*20))))</ns0:f>
-        <ns0:v>1.82e+164</ns0:v>
+        <ns0:v>2.34e+165</ns0:v>
       </ns0:c>
       <ns0:c r="E157" s="1">
         <ns0:f>D157</ns0:f>
-        <ns0:v>1.82e+164</ns0:v>
+        <ns0:v>2.34e+165</ns0:v>
       </ns0:c>
       <ns0:c r="F157" s="1">
         <ns0:f>ROUND(F156*1.4,-5)</ns0:f>
@@ -5946,11 +5946,11 @@
       </ns0:c>
       <ns0:c r="D158" s="1">
         <ns0:f>ROUND(D157*20,2-INT(LOG10(ABS(D157*20))))</ns0:f>
-        <ns0:v>3.6400000000000005e+165</ns0:v>
+        <ns0:v>4.68e+166</ns0:v>
       </ns0:c>
       <ns0:c r="E158" s="1">
         <ns0:f>D158</ns0:f>
-        <ns0:v>3.6400000000000005e+165</ns0:v>
+        <ns0:v>4.68e+166</ns0:v>
       </ns0:c>
       <ns0:c r="F158" s="1">
         <ns0:f>ROUND(F157*1.4,-5)</ns0:f>
@@ -5978,11 +5978,11 @@
       </ns0:c>
       <ns0:c r="D159" s="1">
         <ns0:f>ROUND(D158*20,2-INT(LOG10(ABS(D158*20))))</ns0:f>
-        <ns0:v>7.28e+166</ns0:v>
+        <ns0:v>9.36e+167</ns0:v>
       </ns0:c>
       <ns0:c r="E159" s="1">
         <ns0:f>D159</ns0:f>
-        <ns0:v>7.28e+166</ns0:v>
+        <ns0:v>9.36e+167</ns0:v>
       </ns0:c>
       <ns0:c r="F159" s="1">
         <ns0:f>ROUND(F158*1.4,-5)</ns0:f>
@@ -6010,11 +6010,11 @@
       </ns0:c>
       <ns0:c r="D160" s="1">
         <ns0:f>ROUND(D159*20,2-INT(LOG10(ABS(D159*20))))</ns0:f>
-        <ns0:v>1.46e+168</ns0:v>
+        <ns0:v>1.87e+169</ns0:v>
       </ns0:c>
       <ns0:c r="E160" s="1">
         <ns0:f>D160</ns0:f>
-        <ns0:v>1.46e+168</ns0:v>
+        <ns0:v>1.87e+169</ns0:v>
       </ns0:c>
       <ns0:c r="F160" s="1">
         <ns0:f>ROUND(F159*1.4,-5)</ns0:f>
@@ -6042,11 +6042,11 @@
       </ns0:c>
       <ns0:c r="D161" s="1">
         <ns0:f>ROUND(D160*20,2-INT(LOG10(ABS(D160*20))))</ns0:f>
-        <ns0:v>2.92e+169</ns0:v>
+        <ns0:v>3.74e+170</ns0:v>
       </ns0:c>
       <ns0:c r="E161" s="1">
         <ns0:f>D161</ns0:f>
-        <ns0:v>2.92e+169</ns0:v>
+        <ns0:v>3.74e+170</ns0:v>
       </ns0:c>
       <ns0:c r="F161" s="1">
         <ns0:f>ROUND(F160*1.4,-5)</ns0:f>
@@ -6074,11 +6074,11 @@
       </ns0:c>
       <ns0:c r="D162" s="1">
         <ns0:f>ROUND(D161*20,2-INT(LOG10(ABS(D161*20))))</ns0:f>
-        <ns0:v>5.84e+170</ns0:v>
+        <ns0:v>7.4799999999999995e+171</ns0:v>
       </ns0:c>
       <ns0:c r="E162" s="1">
         <ns0:f>D162</ns0:f>
-        <ns0:v>5.84e+170</ns0:v>
+        <ns0:v>7.4799999999999995e+171</ns0:v>
       </ns0:c>
       <ns0:c r="F162" s="1">
         <ns0:f>ROUND(F161*1.4,-5)</ns0:f>
@@ -6106,11 +6106,11 @@
       </ns0:c>
       <ns0:c r="D163" s="1">
         <ns0:f>ROUND(D162*20,2-INT(LOG10(ABS(D162*20))))</ns0:f>
-        <ns0:v>1.17e+172</ns0:v>
+        <ns0:v>1.5000000000000002e+173</ns0:v>
       </ns0:c>
       <ns0:c r="E163" s="1">
         <ns0:f>D163</ns0:f>
-        <ns0:v>1.17e+172</ns0:v>
+        <ns0:v>1.5000000000000002e+173</ns0:v>
       </ns0:c>
       <ns0:c r="F163" s="1">
         <ns0:f>ROUND(F162*1.4,-5)</ns0:f>
@@ -6138,11 +6138,11 @@
       </ns0:c>
       <ns0:c r="D164" s="1">
         <ns0:f>ROUND(D163*20,2-INT(LOG10(ABS(D163*20))))</ns0:f>
-        <ns0:v>2.34e+173</ns0:v>
+        <ns0:v>3e+174</ns0:v>
       </ns0:c>
       <ns0:c r="E164" s="1">
         <ns0:f>D164</ns0:f>
-        <ns0:v>2.34e+173</ns0:v>
+        <ns0:v>3e+174</ns0:v>
       </ns0:c>
       <ns0:c r="F164" s="1">
         <ns0:f>ROUND(F163*1.4,-5)</ns0:f>
@@ -6170,11 +6170,11 @@
       </ns0:c>
       <ns0:c r="D165" s="1">
         <ns0:f>ROUND(D164*20,2-INT(LOG10(ABS(D164*20))))</ns0:f>
-        <ns0:v>4.68e+174</ns0:v>
+        <ns0:v>5.9999999999999996e+175</ns0:v>
       </ns0:c>
       <ns0:c r="E165" s="1">
         <ns0:f>D165</ns0:f>
-        <ns0:v>4.68e+174</ns0:v>
+        <ns0:v>5.9999999999999996e+175</ns0:v>
       </ns0:c>
       <ns0:c r="F165" s="1">
         <ns0:f>ROUND(F164*1.4,-5)</ns0:f>
@@ -6202,11 +6202,11 @@
       </ns0:c>
       <ns0:c r="D166" s="1">
         <ns0:f>ROUND(D165*20,2-INT(LOG10(ABS(D165*20))))</ns0:f>
-        <ns0:v>9.36e+175</ns0:v>
+        <ns0:v>1.2e+177</ns0:v>
       </ns0:c>
       <ns0:c r="E166" s="1">
         <ns0:f>D166</ns0:f>
-        <ns0:v>9.36e+175</ns0:v>
+        <ns0:v>1.2e+177</ns0:v>
       </ns0:c>
       <ns0:c r="F166" s="1">
         <ns0:f>ROUND(F165*1.4,-5)</ns0:f>
@@ -6234,11 +6234,11 @@
       </ns0:c>
       <ns0:c r="D167" s="1">
         <ns0:f>ROUND(D166*20,2-INT(LOG10(ABS(D166*20))))</ns0:f>
-        <ns0:v>1.87e+177</ns0:v>
+        <ns0:v>2.4e+178</ns0:v>
       </ns0:c>
       <ns0:c r="E167" s="1">
         <ns0:f>D167</ns0:f>
-        <ns0:v>1.87e+177</ns0:v>
+        <ns0:v>2.4e+178</ns0:v>
       </ns0:c>
       <ns0:c r="F167" s="1">
         <ns0:f>ROUND(F166*1.4,-5)</ns0:f>
@@ -6266,11 +6266,11 @@
       </ns0:c>
       <ns0:c r="D168" s="1">
         <ns0:f>ROUND(D167*20,2-INT(LOG10(ABS(D167*20))))</ns0:f>
-        <ns0:v>3.74e+178</ns0:v>
+        <ns0:v>4.8e+179</ns0:v>
       </ns0:c>
       <ns0:c r="E168" s="1">
         <ns0:f>D168</ns0:f>
-        <ns0:v>3.74e+178</ns0:v>
+        <ns0:v>4.8e+179</ns0:v>
       </ns0:c>
       <ns0:c r="F168" s="1">
         <ns0:f>ROUND(F167*1.4,-5)</ns0:f>
@@ -6298,11 +6298,11 @@
       </ns0:c>
       <ns0:c r="D169" s="1">
         <ns0:f>ROUND(D168*20,2-INT(LOG10(ABS(D168*20))))</ns0:f>
-        <ns0:v>7.48e+179</ns0:v>
+        <ns0:v>9.600000000000001e+180</ns0:v>
       </ns0:c>
       <ns0:c r="E169" s="1">
         <ns0:f>D169</ns0:f>
-        <ns0:v>7.48e+179</ns0:v>
+        <ns0:v>9.600000000000001e+180</ns0:v>
       </ns0:c>
       <ns0:c r="F169" s="1">
         <ns0:f>ROUND(F168*1.4,-5)</ns0:f>
@@ -6330,11 +6330,11 @@
       </ns0:c>
       <ns0:c r="D170" s="1">
         <ns0:f>ROUND(D169*20,2-INT(LOG10(ABS(D169*20))))</ns0:f>
-        <ns0:v>1.5e+181</ns0:v>
+        <ns0:v>1.92e+182</ns0:v>
       </ns0:c>
       <ns0:c r="E170" s="1">
         <ns0:f>D170</ns0:f>
-        <ns0:v>1.5e+181</ns0:v>
+        <ns0:v>1.92e+182</ns0:v>
       </ns0:c>
       <ns0:c r="F170" s="1">
         <ns0:f>ROUND(F169*1.4,-5)</ns0:f>
@@ -6362,11 +6362,11 @@
       </ns0:c>
       <ns0:c r="D171" s="1">
         <ns0:f>ROUND(D170*20,2-INT(LOG10(ABS(D170*20))))</ns0:f>
-        <ns0:v>3e+182</ns0:v>
+        <ns0:v>3.8399999999999997e+183</ns0:v>
       </ns0:c>
       <ns0:c r="E171" s="1">
         <ns0:f>D171</ns0:f>
-        <ns0:v>3e+182</ns0:v>
+        <ns0:v>3.8399999999999997e+183</ns0:v>
       </ns0:c>
       <ns0:c r="F171" s="1">
         <ns0:f>ROUND(F170*1.4,-5)</ns0:f>
@@ -6394,11 +6394,11 @@
       </ns0:c>
       <ns0:c r="D172" s="1">
         <ns0:f>ROUND(D171*20,2-INT(LOG10(ABS(D171*20))))</ns0:f>
-        <ns0:v>6e+183</ns0:v>
+        <ns0:v>7.679999999999999e+184</ns0:v>
       </ns0:c>
       <ns0:c r="E172" s="1">
         <ns0:f>D172</ns0:f>
-        <ns0:v>6e+183</ns0:v>
+        <ns0:v>7.679999999999999e+184</ns0:v>
       </ns0:c>
       <ns0:c r="F172" s="1">
         <ns0:f>ROUND(F171*1.4,-5)</ns0:f>
@@ -6426,11 +6426,11 @@
       </ns0:c>
       <ns0:c r="D173" s="1">
         <ns0:f>ROUND(D172*20,2-INT(LOG10(ABS(D172*20))))</ns0:f>
-        <ns0:v>1.2e+185</ns0:v>
+        <ns0:v>1.54e+186</ns0:v>
       </ns0:c>
       <ns0:c r="E173" s="1">
         <ns0:f>D173</ns0:f>
-        <ns0:v>1.2e+185</ns0:v>
+        <ns0:v>1.54e+186</ns0:v>
       </ns0:c>
       <ns0:c r="F173" s="1">
         <ns0:f>ROUND(F172*1.4,-5)</ns0:f>
@@ -6458,11 +6458,11 @@
       </ns0:c>
       <ns0:c r="D174" s="1">
         <ns0:f>ROUND(D173*20,2-INT(LOG10(ABS(D173*20))))</ns0:f>
-        <ns0:v>2.4e+186</ns0:v>
+        <ns0:v>3.08e+187</ns0:v>
       </ns0:c>
       <ns0:c r="E174" s="1">
         <ns0:f>D174</ns0:f>
-        <ns0:v>2.4e+186</ns0:v>
+        <ns0:v>3.08e+187</ns0:v>
       </ns0:c>
       <ns0:c r="F174" s="1">
         <ns0:f>ROUND(F173*1.4,-5)</ns0:f>
@@ -6490,11 +6490,11 @@
       </ns0:c>
       <ns0:c r="D175" s="1">
         <ns0:f>ROUND(D174*20,2-INT(LOG10(ABS(D174*20))))</ns0:f>
-        <ns0:v>4.8e+187</ns0:v>
+        <ns0:v>6.160000000000001e+188</ns0:v>
       </ns0:c>
       <ns0:c r="E175" s="1">
         <ns0:f>D175</ns0:f>
-        <ns0:v>4.8e+187</ns0:v>
+        <ns0:v>6.160000000000001e+188</ns0:v>
       </ns0:c>
       <ns0:c r="F175" s="1">
         <ns0:f>ROUND(F174*1.4,-5)</ns0:f>
@@ -6522,11 +6522,11 @@
       </ns0:c>
       <ns0:c r="D176" s="1">
         <ns0:f>ROUND(D175*20,2-INT(LOG10(ABS(D175*20))))</ns0:f>
-        <ns0:v>9.600000000000001e+188</ns0:v>
+        <ns0:v>1.23e+190</ns0:v>
       </ns0:c>
       <ns0:c r="E176" s="1">
         <ns0:f>D176</ns0:f>
-        <ns0:v>9.600000000000001e+188</ns0:v>
+        <ns0:v>1.23e+190</ns0:v>
       </ns0:c>
       <ns0:c r="F176" s="1">
         <ns0:f>ROUND(F175*1.4,-5)</ns0:f>
@@ -6554,11 +6554,11 @@
       </ns0:c>
       <ns0:c r="D177" s="1">
         <ns0:f>ROUND(D176*20,2-INT(LOG10(ABS(D176*20))))</ns0:f>
-        <ns0:v>1.92e+190</ns0:v>
+        <ns0:v>2.4599999999999998e+191</ns0:v>
       </ns0:c>
       <ns0:c r="E177" s="1">
         <ns0:f>D177</ns0:f>
-        <ns0:v>1.92e+190</ns0:v>
+        <ns0:v>2.4599999999999998e+191</ns0:v>
       </ns0:c>
       <ns0:c r="F177" s="1">
         <ns0:f>ROUND(F176*1.4,-5)</ns0:f>
@@ -6586,11 +6586,11 @@
       </ns0:c>
       <ns0:c r="D178" s="1">
         <ns0:f>ROUND(D177*20,2-INT(LOG10(ABS(D177*20))))</ns0:f>
-        <ns0:v>3.84e+191</ns0:v>
+        <ns0:v>4.92e+192</ns0:v>
       </ns0:c>
       <ns0:c r="E178" s="1">
         <ns0:f>D178</ns0:f>
-        <ns0:v>3.84e+191</ns0:v>
+        <ns0:v>4.92e+192</ns0:v>
       </ns0:c>
       <ns0:c r="F178" s="1">
         <ns0:f>ROUND(F177*1.4,-5)</ns0:f>
@@ -6618,11 +6618,11 @@
       </ns0:c>
       <ns0:c r="D179" s="1">
         <ns0:f>ROUND(D178*20,2-INT(LOG10(ABS(D178*20))))</ns0:f>
-        <ns0:v>7.68e+192</ns0:v>
+        <ns0:v>9.84e+193</ns0:v>
       </ns0:c>
       <ns0:c r="E179" s="1">
         <ns0:f>D179</ns0:f>
-        <ns0:v>7.68e+192</ns0:v>
+        <ns0:v>9.84e+193</ns0:v>
       </ns0:c>
       <ns0:c r="F179" s="1">
         <ns0:f>ROUND(F178*1.4,-5)</ns0:f>
@@ -6650,11 +6650,11 @@
       </ns0:c>
       <ns0:c r="D180" s="1">
         <ns0:f>ROUND(D179*20,2-INT(LOG10(ABS(D179*20))))</ns0:f>
-        <ns0:v>1.54e+194</ns0:v>
+        <ns0:v>1.9699999999999998e+195</ns0:v>
       </ns0:c>
       <ns0:c r="E180" s="1">
         <ns0:f>D180</ns0:f>
-        <ns0:v>1.54e+194</ns0:v>
+        <ns0:v>1.9699999999999998e+195</ns0:v>
       </ns0:c>
       <ns0:c r="F180" s="1">
         <ns0:f>ROUND(F179*1.4,-5)</ns0:f>
@@ -6682,11 +6682,11 @@
       </ns0:c>
       <ns0:c r="D181" s="1">
         <ns0:f>ROUND(D180*20,2-INT(LOG10(ABS(D180*20))))</ns0:f>
-        <ns0:v>3.08e+195</ns0:v>
+        <ns0:v>3.94e+196</ns0:v>
       </ns0:c>
       <ns0:c r="E181" s="1">
         <ns0:f>D181</ns0:f>
-        <ns0:v>3.08e+195</ns0:v>
+        <ns0:v>3.94e+196</ns0:v>
       </ns0:c>
       <ns0:c r="F181" s="1">
         <ns0:f>ROUND(F180*1.4,-5)</ns0:f>
@@ -6714,11 +6714,11 @@
       </ns0:c>
       <ns0:c r="D182" s="1">
         <ns0:f>ROUND(D181*20,2-INT(LOG10(ABS(D181*20))))</ns0:f>
-        <ns0:v>6.16e+196</ns0:v>
+        <ns0:v>7.88e+197</ns0:v>
       </ns0:c>
       <ns0:c r="E182" s="1">
         <ns0:f>D182</ns0:f>
-        <ns0:v>6.16e+196</ns0:v>
+        <ns0:v>7.88e+197</ns0:v>
       </ns0:c>
       <ns0:c r="F182" s="1">
         <ns0:f>ROUND(F181*1.4,-5)</ns0:f>
@@ -6746,11 +6746,11 @@
       </ns0:c>
       <ns0:c r="D183" s="1">
         <ns0:f>ROUND(D182*20,2-INT(LOG10(ABS(D182*20))))</ns0:f>
-        <ns0:v>1.23e+198</ns0:v>
+        <ns0:v>1.5800000000000001e+199</ns0:v>
       </ns0:c>
       <ns0:c r="E183" s="1">
         <ns0:f>D183</ns0:f>
-        <ns0:v>1.23e+198</ns0:v>
+        <ns0:v>1.5800000000000001e+199</ns0:v>
       </ns0:c>
       <ns0:c r="F183" s="1">
         <ns0:f>ROUND(F182*1.4,-5)</ns0:f>
@@ -6778,11 +6778,11 @@
       </ns0:c>
       <ns0:c r="D184" s="1">
         <ns0:f>ROUND(D183*20,2-INT(LOG10(ABS(D183*20))))</ns0:f>
-        <ns0:v>2.46e+199</ns0:v>
+        <ns0:v>3.1600000000000006e+200</ns0:v>
       </ns0:c>
       <ns0:c r="E184" s="1">
         <ns0:f>D184</ns0:f>
-        <ns0:v>2.46e+199</ns0:v>
+        <ns0:v>3.1600000000000006e+200</ns0:v>
       </ns0:c>
       <ns0:c r="F184" s="1">
         <ns0:f>ROUND(F183*1.4,-5)</ns0:f>
@@ -6810,11 +6810,11 @@
       </ns0:c>
       <ns0:c r="D185" s="1">
         <ns0:f>ROUND(D184*20,2-INT(LOG10(ABS(D184*20))))</ns0:f>
-        <ns0:v>4.920000000000001e+200</ns0:v>
+        <ns0:v>6.320000000000001e+201</ns0:v>
       </ns0:c>
       <ns0:c r="E185" s="1">
         <ns0:f>D185</ns0:f>
-        <ns0:v>4.920000000000001e+200</ns0:v>
+        <ns0:v>6.320000000000001e+201</ns0:v>
       </ns0:c>
       <ns0:c r="F185" s="1">
         <ns0:f>ROUND(F184*1.4,-5)</ns0:f>
@@ -6842,11 +6842,11 @@
       </ns0:c>
       <ns0:c r="D186" s="1">
         <ns0:f>ROUND(D185*20,2-INT(LOG10(ABS(D185*20))))</ns0:f>
-        <ns0:v>9.84e+201</ns0:v>
+        <ns0:v>1.26e+203</ns0:v>
       </ns0:c>
       <ns0:c r="E186" s="1">
         <ns0:f>D186</ns0:f>
-        <ns0:v>9.84e+201</ns0:v>
+        <ns0:v>1.26e+203</ns0:v>
       </ns0:c>
       <ns0:c r="F186" s="1">
         <ns0:f>ROUND(F185*1.4,-5)</ns0:f>
@@ -6874,11 +6874,11 @@
       </ns0:c>
       <ns0:c r="D187" s="1">
         <ns0:f>ROUND(D186*20,2-INT(LOG10(ABS(D186*20))))</ns0:f>
-        <ns0:v>1.9700000000000003e+203</ns0:v>
+        <ns0:v>2.52e+204</ns0:v>
       </ns0:c>
       <ns0:c r="E187" s="1">
         <ns0:f>D187</ns0:f>
-        <ns0:v>1.9700000000000003e+203</ns0:v>
+        <ns0:v>2.52e+204</ns0:v>
       </ns0:c>
       <ns0:c r="F187" s="1">
         <ns0:f>ROUND(F186*1.4,-5)</ns0:f>
@@ -6906,11 +6906,11 @@
       </ns0:c>
       <ns0:c r="D188" s="1">
         <ns0:f>ROUND(D187*20,2-INT(LOG10(ABS(D187*20))))</ns0:f>
-        <ns0:v>3.94e+204</ns0:v>
+        <ns0:v>5.04e+205</ns0:v>
       </ns0:c>
       <ns0:c r="E188" s="1">
         <ns0:f>D188</ns0:f>
-        <ns0:v>3.94e+204</ns0:v>
+        <ns0:v>5.04e+205</ns0:v>
       </ns0:c>
       <ns0:c r="F188" s="1">
         <ns0:f>ROUND(F187*1.4,-5)</ns0:f>
@@ -6938,11 +6938,11 @@
       </ns0:c>
       <ns0:c r="D189" s="1">
         <ns0:f>ROUND(D188*20,2-INT(LOG10(ABS(D188*20))))</ns0:f>
-        <ns0:v>7.8799999999999995e+205</ns0:v>
+        <ns0:v>1.01e+207</ns0:v>
       </ns0:c>
       <ns0:c r="E189" s="1">
         <ns0:f>D189</ns0:f>
-        <ns0:v>7.8799999999999995e+205</ns0:v>
+        <ns0:v>1.01e+207</ns0:v>
       </ns0:c>
       <ns0:c r="F189" s="1">
         <ns0:f>ROUND(F188*1.4,-5)</ns0:f>
@@ -6970,11 +6970,11 @@
       </ns0:c>
       <ns0:c r="D190" s="1">
         <ns0:f>ROUND(D189*20,2-INT(LOG10(ABS(D189*20))))</ns0:f>
-        <ns0:v>1.58e+207</ns0:v>
+        <ns0:v>2.02e+208</ns0:v>
       </ns0:c>
       <ns0:c r="E190" s="1">
         <ns0:f>D190</ns0:f>
-        <ns0:v>1.58e+207</ns0:v>
+        <ns0:v>2.02e+208</ns0:v>
       </ns0:c>
       <ns0:c r="F190" s="1">
         <ns0:f>ROUND(F189*1.4,-5)</ns0:f>
@@ -7002,11 +7002,11 @@
       </ns0:c>
       <ns0:c r="D191" s="1">
         <ns0:f>ROUND(D190*20,2-INT(LOG10(ABS(D190*20))))</ns0:f>
-        <ns0:v>3.1599999999999997e+208</ns0:v>
+        <ns0:v>4.04e+209</ns0:v>
       </ns0:c>
       <ns0:c r="E191" s="1">
         <ns0:f>D191</ns0:f>
-        <ns0:v>3.1599999999999997e+208</ns0:v>
+        <ns0:v>4.04e+209</ns0:v>
       </ns0:c>
       <ns0:c r="F191" s="1">
         <ns0:f>ROUND(F190*1.4,-5)</ns0:f>
@@ -7034,11 +7034,11 @@
       </ns0:c>
       <ns0:c r="D192" s="1">
         <ns0:f>ROUND(D191*20,2-INT(LOG10(ABS(D191*20))))</ns0:f>
-        <ns0:v>6.320000000000001e+209</ns0:v>
+        <ns0:v>8.079999999999999e+210</ns0:v>
       </ns0:c>
       <ns0:c r="E192" s="1">
         <ns0:f>D192</ns0:f>
-        <ns0:v>6.320000000000001e+209</ns0:v>
+        <ns0:v>8.079999999999999e+210</ns0:v>
       </ns0:c>
       <ns0:c r="F192" s="1">
         <ns0:f>ROUND(F191*1.4,-5)</ns0:f>
@@ -7066,11 +7066,11 @@
       </ns0:c>
       <ns0:c r="D193" s="1">
         <ns0:f>ROUND(D192*20,2-INT(LOG10(ABS(D192*20))))</ns0:f>
-        <ns0:v>1.26e+211</ns0:v>
+        <ns0:v>1.62e+212</ns0:v>
       </ns0:c>
       <ns0:c r="E193" s="1">
         <ns0:f>D193</ns0:f>
-        <ns0:v>1.26e+211</ns0:v>
+        <ns0:v>1.62e+212</ns0:v>
       </ns0:c>
       <ns0:c r="F193" s="1">
         <ns0:f>ROUND(F192*1.4,-5)</ns0:f>
@@ -7098,11 +7098,11 @@
       </ns0:c>
       <ns0:c r="D194" s="1">
         <ns0:f>ROUND(D193*20,2-INT(LOG10(ABS(D193*20))))</ns0:f>
-        <ns0:v>2.5199999999999998e+212</ns0:v>
+        <ns0:v>3.2399999999999995e+213</ns0:v>
       </ns0:c>
       <ns0:c r="E194" s="1">
         <ns0:f>D194</ns0:f>
-        <ns0:v>2.5199999999999998e+212</ns0:v>
+        <ns0:v>3.2399999999999995e+213</ns0:v>
       </ns0:c>
       <ns0:c r="F194" s="1">
         <ns0:f>ROUND(F193*1.4,-5)</ns0:f>
@@ -7130,11 +7130,11 @@
       </ns0:c>
       <ns0:c r="D195" s="1">
         <ns0:f>ROUND(D194*20,2-INT(LOG10(ABS(D194*20))))</ns0:f>
-        <ns0:v>5.0399999999999996e+213</ns0:v>
+        <ns0:v>6.48e+214</ns0:v>
       </ns0:c>
       <ns0:c r="E195" s="1">
         <ns0:f>D195</ns0:f>
-        <ns0:v>5.0399999999999996e+213</ns0:v>
+        <ns0:v>6.48e+214</ns0:v>
       </ns0:c>
       <ns0:c r="F195" s="1">
         <ns0:f>ROUND(F194*1.4,-5)</ns0:f>
@@ -7162,11 +7162,11 @@
       </ns0:c>
       <ns0:c r="D196" s="1">
         <ns0:f>ROUND(D195*20,2-INT(LOG10(ABS(D195*20))))</ns0:f>
-        <ns0:v>1.01e+215</ns0:v>
+        <ns0:v>1.3000000000000001e+216</ns0:v>
       </ns0:c>
       <ns0:c r="E196" s="1">
         <ns0:f>D196</ns0:f>
-        <ns0:v>1.01e+215</ns0:v>
+        <ns0:v>1.3000000000000001e+216</ns0:v>
       </ns0:c>
       <ns0:c r="F196" s="1">
         <ns0:f>ROUND(F195*1.4,-5)</ns0:f>
@@ -7194,11 +7194,11 @@
       </ns0:c>
       <ns0:c r="D197" s="1">
         <ns0:f>ROUND(D196*20,2-INT(LOG10(ABS(D196*20))))</ns0:f>
-        <ns0:v>2.02e+216</ns0:v>
+        <ns0:v>2.6e+217</ns0:v>
       </ns0:c>
       <ns0:c r="E197" s="1">
         <ns0:f>D197</ns0:f>
-        <ns0:v>2.02e+216</ns0:v>
+        <ns0:v>2.6e+217</ns0:v>
       </ns0:c>
       <ns0:c r="F197" s="1">
         <ns0:f>ROUND(F196*1.4,-5)</ns0:f>
@@ -7226,11 +7226,11 @@
       </ns0:c>
       <ns0:c r="D198" s="1">
         <ns0:f>ROUND(D197*20,2-INT(LOG10(ABS(D197*20))))</ns0:f>
-        <ns0:v>4.0399999999999997e+217</ns0:v>
+        <ns0:v>5.2e+218</ns0:v>
       </ns0:c>
       <ns0:c r="E198" s="1">
         <ns0:f>D198</ns0:f>
-        <ns0:v>4.0399999999999997e+217</ns0:v>
+        <ns0:v>5.2e+218</ns0:v>
       </ns0:c>
       <ns0:c r="F198" s="1">
         <ns0:f>ROUND(F197*1.4,-5)</ns0:f>
@@ -7258,11 +7258,11 @@
       </ns0:c>
       <ns0:c r="D199" s="1">
         <ns0:f>ROUND(D198*20,2-INT(LOG10(ABS(D198*20))))</ns0:f>
-        <ns0:v>8.08e+218</ns0:v>
+        <ns0:v>1.04e+220</ns0:v>
       </ns0:c>
       <ns0:c r="E199" s="1">
         <ns0:f>D199</ns0:f>
-        <ns0:v>8.08e+218</ns0:v>
+        <ns0:v>1.04e+220</ns0:v>
       </ns0:c>
       <ns0:c r="F199" s="1">
         <ns0:f>ROUND(F198*1.4,-5)</ns0:f>
@@ -7290,11 +7290,11 @@
       </ns0:c>
       <ns0:c r="D200" s="1">
         <ns0:f>ROUND(D199*20,2-INT(LOG10(ABS(D199*20))))</ns0:f>
-        <ns0:v>1.62e+220</ns0:v>
+        <ns0:v>2.08e+221</ns0:v>
       </ns0:c>
       <ns0:c r="E200" s="1">
         <ns0:f>D200</ns0:f>
-        <ns0:v>1.62e+220</ns0:v>
+        <ns0:v>2.08e+221</ns0:v>
       </ns0:c>
       <ns0:c r="F200" s="1">
         <ns0:f>ROUND(F199*1.4,-5)</ns0:f>
@@ -7322,11 +7322,11 @@
       </ns0:c>
       <ns0:c r="D201" s="1">
         <ns0:f>ROUND(D200*20,2-INT(LOG10(ABS(D200*20))))</ns0:f>
-        <ns0:v>3.2399999999999997e+221</ns0:v>
+        <ns0:v>4.16e+222</ns0:v>
       </ns0:c>
       <ns0:c r="E201" s="1">
         <ns0:f>D201</ns0:f>
-        <ns0:v>3.2399999999999997e+221</ns0:v>
+        <ns0:v>4.16e+222</ns0:v>
       </ns0:c>
       <ns0:c r="F201" s="1">
         <ns0:f>ROUND(F200*1.4,-5)</ns0:f>
@@ -7354,11 +7354,11 @@
       </ns0:c>
       <ns0:c r="D202" s="1">
         <ns0:f>ROUND(D201*20,2-INT(LOG10(ABS(D201*20))))</ns0:f>
-        <ns0:v>6.48e+222</ns0:v>
+        <ns0:v>8.319999999999999e+223</ns0:v>
       </ns0:c>
       <ns0:c r="E202" s="1">
         <ns0:f>D202</ns0:f>
-        <ns0:v>6.48e+222</ns0:v>
+        <ns0:v>8.319999999999999e+223</ns0:v>
       </ns0:c>
       <ns0:c r="F202" s="1">
         <ns0:f>ROUND(F201*1.4,-5)</ns0:f>
@@ -7386,11 +7386,11 @@
       </ns0:c>
       <ns0:c r="D203" s="1">
         <ns0:f>ROUND(D202*20,2-INT(LOG10(ABS(D202*20))))</ns0:f>
-        <ns0:v>1.3e+224</ns0:v>
+        <ns0:v>1.6600000000000002e+225</ns0:v>
       </ns0:c>
       <ns0:c r="E203" s="1">
         <ns0:f>D203</ns0:f>
-        <ns0:v>1.3e+224</ns0:v>
+        <ns0:v>1.6600000000000002e+225</ns0:v>
       </ns0:c>
       <ns0:c r="F203" s="1">
         <ns0:f>ROUND(F202*1.4,-5)</ns0:f>
@@ -7418,11 +7418,11 @@
       </ns0:c>
       <ns0:c r="D204" s="1">
         <ns0:f>ROUND(D203*20,2-INT(LOG10(ABS(D203*20))))</ns0:f>
-        <ns0:v>2.6e+225</ns0:v>
+        <ns0:v>3.3199999999999997e+226</ns0:v>
       </ns0:c>
       <ns0:c r="E204" s="1">
         <ns0:f>D204</ns0:f>
-        <ns0:v>2.6e+225</ns0:v>
+        <ns0:v>3.3199999999999997e+226</ns0:v>
       </ns0:c>
       <ns0:c r="F204" s="1">
         <ns0:f>ROUND(F203*1.4,-5)</ns0:f>
@@ -7450,11 +7450,11 @@
       </ns0:c>
       <ns0:c r="D205" s="1">
         <ns0:f>ROUND(D204*20,2-INT(LOG10(ABS(D204*20))))</ns0:f>
-        <ns0:v>5.199999999999999e+226</ns0:v>
+        <ns0:v>6.640000000000001e+227</ns0:v>
       </ns0:c>
       <ns0:c r="E205" s="1">
         <ns0:f>D205</ns0:f>
-        <ns0:v>5.199999999999999e+226</ns0:v>
+        <ns0:v>6.640000000000001e+227</ns0:v>
       </ns0:c>
       <ns0:c r="F205" s="1">
         <ns0:f>ROUND(F204*1.4,-5)</ns0:f>
@@ -7482,11 +7482,11 @@
       </ns0:c>
       <ns0:c r="D206" s="1">
         <ns0:f>ROUND(D205*20,2-INT(LOG10(ABS(D205*20))))</ns0:f>
-        <ns0:v>1.0400000000000001e+228</ns0:v>
+        <ns0:v>1.3300000000000002e+229</ns0:v>
       </ns0:c>
       <ns0:c r="E206" s="1">
         <ns0:f>D206</ns0:f>
-        <ns0:v>1.0400000000000001e+228</ns0:v>
+        <ns0:v>1.3300000000000002e+229</ns0:v>
       </ns0:c>
       <ns0:c r="F206" s="1">
         <ns0:f>ROUND(F205*1.4,-5)</ns0:f>
@@ -7514,11 +7514,11 @@
       </ns0:c>
       <ns0:c r="D207" s="1">
         <ns0:f>ROUND(D206*20,2-INT(LOG10(ABS(D206*20))))</ns0:f>
-        <ns0:v>2.08e+229</ns0:v>
+        <ns0:v>2.66e+230</ns0:v>
       </ns0:c>
       <ns0:c r="E207" s="1">
         <ns0:f>D207</ns0:f>
-        <ns0:v>2.08e+229</ns0:v>
+        <ns0:v>2.66e+230</ns0:v>
       </ns0:c>
       <ns0:c r="F207" s="1">
         <ns0:f>ROUND(F206*1.4,-5)</ns0:f>
@@ -7546,11 +7546,11 @@
       </ns0:c>
       <ns0:c r="D208" s="1">
         <ns0:f>ROUND(D207*20,2-INT(LOG10(ABS(D207*20))))</ns0:f>
-        <ns0:v>4.16e+230</ns0:v>
+        <ns0:v>5.3199999999999994e+231</ns0:v>
       </ns0:c>
       <ns0:c r="E208" s="1">
         <ns0:f>D208</ns0:f>
-        <ns0:v>4.16e+230</ns0:v>
+        <ns0:v>5.3199999999999994e+231</ns0:v>
       </ns0:c>
       <ns0:c r="F208" s="1">
         <ns0:f>ROUND(F207*1.4,-5)</ns0:f>
@@ -7578,11 +7578,11 @@
       </ns0:c>
       <ns0:c r="D209" s="1">
         <ns0:f>ROUND(D208*20,2-INT(LOG10(ABS(D208*20))))</ns0:f>
-        <ns0:v>8.32e+231</ns0:v>
+        <ns0:v>1.06e+233</ns0:v>
       </ns0:c>
       <ns0:c r="E209" s="1">
         <ns0:f>D209</ns0:f>
-        <ns0:v>8.32e+231</ns0:v>
+        <ns0:v>1.06e+233</ns0:v>
       </ns0:c>
       <ns0:c r="F209" s="1">
         <ns0:f>ROUND(F208*1.4,-5)</ns0:f>
@@ -7610,11 +7610,11 @@
       </ns0:c>
       <ns0:c r="D210" s="1">
         <ns0:f>ROUND(D209*20,2-INT(LOG10(ABS(D209*20))))</ns0:f>
-        <ns0:v>1.66e+233</ns0:v>
+        <ns0:v>2.12e+234</ns0:v>
       </ns0:c>
       <ns0:c r="E210" s="1">
         <ns0:f>D210</ns0:f>
-        <ns0:v>1.66e+233</ns0:v>
+        <ns0:v>2.12e+234</ns0:v>
       </ns0:c>
       <ns0:c r="F210" s="1">
         <ns0:f>ROUND(F209*1.4,-5)</ns0:f>
@@ -7642,11 +7642,11 @@
       </ns0:c>
       <ns0:c r="D211" s="1">
         <ns0:f>ROUND(D210*20,2-INT(LOG10(ABS(D210*20))))</ns0:f>
-        <ns0:v>3.32e+234</ns0:v>
+        <ns0:v>4.24e+235</ns0:v>
       </ns0:c>
       <ns0:c r="E211" s="1">
         <ns0:f>D211</ns0:f>
-        <ns0:v>3.32e+234</ns0:v>
+        <ns0:v>4.24e+235</ns0:v>
       </ns0:c>
       <ns0:c r="F211" s="1">
         <ns0:f>ROUND(F210*1.4,-5)</ns0:f>
@@ -7674,11 +7674,11 @@
       </ns0:c>
       <ns0:c r="D212" s="1">
         <ns0:f>ROUND(D211*20,2-INT(LOG10(ABS(D211*20))))</ns0:f>
-        <ns0:v>6.64e+235</ns0:v>
+        <ns0:v>8.480000000000001e+236</ns0:v>
       </ns0:c>
       <ns0:c r="E212" s="1">
         <ns0:f>D212</ns0:f>
-        <ns0:v>6.64e+235</ns0:v>
+        <ns0:v>8.480000000000001e+236</ns0:v>
       </ns0:c>
       <ns0:c r="F212" s="1">
         <ns0:f>ROUND(F211*1.4,-5)</ns0:f>
@@ -7706,11 +7706,11 @@
       </ns0:c>
       <ns0:c r="D213" s="1">
         <ns0:f>ROUND(D212*20,2-INT(LOG10(ABS(D212*20))))</ns0:f>
-        <ns0:v>1.33e+237</ns0:v>
+        <ns0:v>1.7e+238</ns0:v>
       </ns0:c>
       <ns0:c r="E213" s="1">
         <ns0:f>D213</ns0:f>
-        <ns0:v>1.33e+237</ns0:v>
+        <ns0:v>1.7e+238</ns0:v>
       </ns0:c>
       <ns0:c r="F213" s="1">
         <ns0:f>ROUND(F212*1.4,-5)</ns0:f>
@@ -7738,11 +7738,11 @@
       </ns0:c>
       <ns0:c r="D214" s="1">
         <ns0:f>ROUND(D213*20,2-INT(LOG10(ABS(D213*20))))</ns0:f>
-        <ns0:v>2.66e+238</ns0:v>
+        <ns0:v>3.4e+239</ns0:v>
       </ns0:c>
       <ns0:c r="E214" s="1">
         <ns0:f>D214</ns0:f>
-        <ns0:v>2.66e+238</ns0:v>
+        <ns0:v>3.4e+239</ns0:v>
       </ns0:c>
       <ns0:c r="F214" s="1">
         <ns0:f>ROUND(F213*1.4,-5)</ns0:f>
@@ -7770,11 +7770,11 @@
       </ns0:c>
       <ns0:c r="D215" s="1">
         <ns0:f>ROUND(D214*20,2-INT(LOG10(ABS(D214*20))))</ns0:f>
-        <ns0:v>5.32e+239</ns0:v>
+        <ns0:v>6.8e+240</ns0:v>
       </ns0:c>
       <ns0:c r="E215" s="1">
         <ns0:f>D215</ns0:f>
-        <ns0:v>5.32e+239</ns0:v>
+        <ns0:v>6.8e+240</ns0:v>
       </ns0:c>
       <ns0:c r="F215" s="1">
         <ns0:f>ROUND(F214*1.4,-5)</ns0:f>
@@ -7802,11 +7802,11 @@
       </ns0:c>
       <ns0:c r="D216" s="1">
         <ns0:f>ROUND(D215*20,2-INT(LOG10(ABS(D215*20))))</ns0:f>
-        <ns0:v>1.0599999999999999e+241</ns0:v>
+        <ns0:v>1.36e+242</ns0:v>
       </ns0:c>
       <ns0:c r="E216" s="1">
         <ns0:f>D216</ns0:f>
-        <ns0:v>1.0599999999999999e+241</ns0:v>
+        <ns0:v>1.36e+242</ns0:v>
       </ns0:c>
       <ns0:c r="F216" s="1">
         <ns0:f>ROUND(F215*1.4,-5)</ns0:f>
@@ -7834,11 +7834,11 @@
       </ns0:c>
       <ns0:c r="D217" s="1">
         <ns0:f>ROUND(D216*20,2-INT(LOG10(ABS(D216*20))))</ns0:f>
-        <ns0:v>2.12e+242</ns0:v>
+        <ns0:v>2.7200000000000002e+243</ns0:v>
       </ns0:c>
       <ns0:c r="E217" s="1">
         <ns0:f>D217</ns0:f>
-        <ns0:v>2.12e+242</ns0:v>
+        <ns0:v>2.7200000000000002e+243</ns0:v>
       </ns0:c>
       <ns0:c r="F217" s="1">
         <ns0:f>ROUND(F216*1.4,-5)</ns0:f>
@@ -7866,11 +7866,11 @@
       </ns0:c>
       <ns0:c r="D218" s="1">
         <ns0:f>ROUND(D217*20,2-INT(LOG10(ABS(D217*20))))</ns0:f>
-        <ns0:v>4.24e+243</ns0:v>
+        <ns0:v>5.44e+244</ns0:v>
       </ns0:c>
       <ns0:c r="E218" s="1">
         <ns0:f>D218</ns0:f>
-        <ns0:v>4.24e+243</ns0:v>
+        <ns0:v>5.44e+244</ns0:v>
       </ns0:c>
       <ns0:c r="F218" s="1">
         <ns0:f>ROUND(F217*1.4,-5)</ns0:f>
@@ -7898,11 +7898,11 @@
       </ns0:c>
       <ns0:c r="D219" s="1">
         <ns0:f>ROUND(D218*20,2-INT(LOG10(ABS(D218*20))))</ns0:f>
-        <ns0:v>8.480000000000001e+244</ns0:v>
+        <ns0:v>1.0900000000000001e+246</ns0:v>
       </ns0:c>
       <ns0:c r="E219" s="1">
         <ns0:f>D219</ns0:f>
-        <ns0:v>8.480000000000001e+244</ns0:v>
+        <ns0:v>1.0900000000000001e+246</ns0:v>
       </ns0:c>
       <ns0:c r="F219" s="1">
         <ns0:f>ROUND(F218*1.4,-5)</ns0:f>
@@ -7930,11 +7930,11 @@
       </ns0:c>
       <ns0:c r="D220" s="1">
         <ns0:f>ROUND(D219*20,2-INT(LOG10(ABS(D219*20))))</ns0:f>
-        <ns0:v>1.7000000000000001e+246</ns0:v>
+        <ns0:v>2.1800000000000002e+247</ns0:v>
       </ns0:c>
       <ns0:c r="E220" s="1">
         <ns0:f>D220</ns0:f>
-        <ns0:v>1.7000000000000001e+246</ns0:v>
+        <ns0:v>2.1800000000000002e+247</ns0:v>
       </ns0:c>
       <ns0:c r="F220" s="1">
         <ns0:f>ROUND(F219*1.4,-5)</ns0:f>
@@ -7962,11 +7962,11 @@
       </ns0:c>
       <ns0:c r="D221" s="1">
         <ns0:f>ROUND(D220*20,2-INT(LOG10(ABS(D220*20))))</ns0:f>
-        <ns0:v>3.4000000000000004e+247</ns0:v>
+        <ns0:v>4.3600000000000004e+248</ns0:v>
       </ns0:c>
       <ns0:c r="E221" s="1">
         <ns0:f>D221</ns0:f>
-        <ns0:v>3.4000000000000004e+247</ns0:v>
+        <ns0:v>4.3600000000000004e+248</ns0:v>
       </ns0:c>
       <ns0:c r="F221" s="1">
         <ns0:f>ROUND(F220*1.4,-5)</ns0:f>
@@ -7994,11 +7994,11 @@
       </ns0:c>
       <ns0:c r="D222" s="1">
         <ns0:f>ROUND(D221*20,2-INT(LOG10(ABS(D221*20))))</ns0:f>
-        <ns0:v>6.8e+248</ns0:v>
+        <ns0:v>8.72e+249</ns0:v>
       </ns0:c>
       <ns0:c r="E222" s="1">
         <ns0:f>D222</ns0:f>
-        <ns0:v>6.8e+248</ns0:v>
+        <ns0:v>8.72e+249</ns0:v>
       </ns0:c>
       <ns0:c r="F222" s="1">
         <ns0:f>ROUND(F221*1.4,-5)</ns0:f>
@@ -8026,11 +8026,11 @@
       </ns0:c>
       <ns0:c r="D223" s="1">
         <ns0:f>ROUND(D222*20,2-INT(LOG10(ABS(D222*20))))</ns0:f>
-        <ns0:v>1.36e+250</ns0:v>
+        <ns0:v>1.74e+251</ns0:v>
       </ns0:c>
       <ns0:c r="E223" s="1">
         <ns0:f>D223</ns0:f>
-        <ns0:v>1.36e+250</ns0:v>
+        <ns0:v>1.74e+251</ns0:v>
       </ns0:c>
       <ns0:c r="F223" s="1">
         <ns0:f>ROUND(F222*1.4,-5)</ns0:f>

</xml_diff>

<commit_message>
Test distributed first-planet growth and enforce QA code fingerprint reloads
</commit_message>
<xml_diff>
--- a/space-battleship/config_excel/level.xlsx
+++ b/space-battleship/config_excel/level.xlsx
@@ -2107,10 +2107,10 @@
         </ns0:is>
       </ns0:c>
       <ns0:c r="D34" s="1" t="n">
-        <ns0:v>3.944675858338559e+23</ns0:v>
+        <ns0:v>2.442439318663683e+24</ns0:v>
       </ns0:c>
       <ns0:c r="E34" s="1" t="n">
-        <ns0:v>3.944675858338559e+23</ns0:v>
+        <ns0:v>2.442439318663683e+24</ns0:v>
       </ns0:c>
       <ns0:c r="F34" s="1" t="n">
         <ns0:v>9704565562037236</ns0:v>
@@ -2135,10 +2135,10 @@
         </ns0:is>
       </ns0:c>
       <ns0:c r="D35" s="1" t="n">
-        <ns0:v>5.064642171181013e+24</ns0:v>
+        <ns0:v>3.135892939772448e+25</ns0:v>
       </ns0:c>
       <ns0:c r="E35" s="1" t="n">
-        <ns0:v>5.064642171181013e+24</ns0:v>
+        <ns0:v>3.135892939772448e+25</ns0:v>
       </ns0:c>
       <ns0:c r="F35" s="1" t="n">
         <ns0:v>9704565562037236</ns0:v>
@@ -2163,10 +2163,10 @@
         </ns0:is>
       </ns0:c>
       <ns0:c r="D36" s="1" t="n">
-        <ns0:v>4.515685833272325e+25</ns0:v>
+        <ns0:v>4.026230848222263e+26</ns0:v>
       </ns0:c>
       <ns0:c r="E36" s="1" t="n">
-        <ns0:v>4.515685833272325e+25</ns0:v>
+        <ns0:v>4.026230848222263e+26</ns0:v>
       </ns0:c>
       <ns0:c r="F36" s="1" t="n">
         <ns0:v>2.012338714944041e+16</ns0:v>
@@ -2191,10 +2191,10 @@
         </ns0:is>
       </ns0:c>
       <ns0:c r="D37" s="1" t="n">
-        <ns0:v>2.492936018792822e+27</ns0:v>
+        <ns0:v>1.543560274627236e+28</ns0:v>
       </ns0:c>
       <ns0:c r="E37" s="1" t="n">
-        <ns0:v>2.492936018792822e+27</ns0:v>
+        <ns0:v>1.543560274627236e+28</ns0:v>
       </ns0:c>
       <ns0:c r="F37" s="1" t="n">
         <ns0:v>2.012338714944041e+16</ns0:v>

</xml_diff>

<commit_message>
Calibrate late boss wave duration and preserve completed sparse and forge failures
</commit_message>
<xml_diff>
--- a/space-battleship/config_excel/level.xlsx
+++ b/space-battleship/config_excel/level.xlsx
@@ -2107,10 +2107,10 @@
         </ns0:is>
       </ns0:c>
       <ns0:c r="D34" s="1" t="n">
-        <ns0:v>2.442439318663683e+24</ns0:v>
+        <ns0:v>1.512294048887176e+25</ns0:v>
       </ns0:c>
       <ns0:c r="E34" s="1" t="n">
-        <ns0:v>2.442439318663683e+24</ns0:v>
+        <ns0:v>1.512294048887176e+25</ns0:v>
       </ns0:c>
       <ns0:c r="F34" s="1" t="n">
         <ns0:v>9704565562037236</ns0:v>
@@ -2135,10 +2135,10 @@
         </ns0:is>
       </ns0:c>
       <ns0:c r="D35" s="1" t="n">
-        <ns0:v>3.135892939772448e+25</ns0:v>
+        <ns0:v>1.941662253193607e+26</ns0:v>
       </ns0:c>
       <ns0:c r="E35" s="1" t="n">
-        <ns0:v>3.135892939772448e+25</ns0:v>
+        <ns0:v>1.941662253193607e+26</ns0:v>
       </ns0:c>
       <ns0:c r="F35" s="1" t="n">
         <ns0:v>9704565562037236</ns0:v>

</xml_diff>

<commit_message>
Raise first stage35 growth and record propagated Excel formula scope
</commit_message>
<xml_diff>
--- a/space-battleship/config_excel/level.xlsx
+++ b/space-battleship/config_excel/level.xlsx
@@ -2219,10 +2219,10 @@
         </ns0:is>
       </ns0:c>
       <ns0:c r="D38" s="1" t="n">
-        <ns0:v>1.981805537738023e+29</ns0:v>
+        <ns0:v>1.76699772433822e+30</ns0:v>
       </ns0:c>
       <ns0:c r="E38" s="1" t="n">
-        <ns0:v>1.981805537738023e+29</ns0:v>
+        <ns0:v>1.76699772433822e+30</ns0:v>
       </ns0:c>
       <ns0:c r="F38" s="1" t="n">
         <ns0:v>6.008811205403466e+16</ns0:v>
@@ -2247,10 +2247,10 @@
         </ns0:is>
       </ns0:c>
       <ns0:c r="D39" s="1" t="n">
-        <ns0:v>5.917639626797131e+29</ns0:v>
+        <ns0:v>5.276226932910335e+30</ns0:v>
       </ns0:c>
       <ns0:c r="E39" s="1" t="n">
-        <ns0:v>5.917639626797131e+29</ns0:v>
+        <ns0:v>5.276226932910335e+30</ns0:v>
       </ns0:c>
       <ns0:c r="F39" s="1" t="n">
         <ns0:v>1.245987091552463e+17</ns0:v>
@@ -2275,10 +2275,10 @@
         </ns0:is>
       </ns0:c>
       <ns0:c r="D40" s="1" t="n">
-        <ns0:v>1.76699772433822e+30</ns0:v>
+        <ns0:v>1.575472920203933e+31</ns0:v>
       </ns0:c>
       <ns0:c r="E40" s="1" t="n">
-        <ns0:v>1.76699772433822e+30</ns0:v>
+        <ns0:v>1.575472920203933e+31</ns0:v>
       </ns0:c>
       <ns0:c r="F40" s="1" t="n">
         <ns0:v>2.583678833043186e+17</ns0:v>
@@ -2303,10 +2303,10 @@
         </ns0:is>
       </ns0:c>
       <ns0:c r="D41" s="1" t="n">
-        <ns0:v>5.276226932910335e+30</ns0:v>
+        <ns0:v>4.70433693216222e+31</ns0:v>
       </ns0:c>
       <ns0:c r="E41" s="1" t="n">
-        <ns0:v>5.276226932910335e+30</ns0:v>
+        <ns0:v>4.70433693216222e+31</ns0:v>
       </ns0:c>
       <ns0:c r="F41" s="1" t="n">
         <ns0:v>5.357516428198349e+17</ns0:v>
@@ -2331,10 +2331,10 @@
         </ns0:is>
       </ns0:c>
       <ns0:c r="D42" s="1" t="n">
-        <ns0:v>4.704336932162219e+31</ns0:v>
+        <ns0:v>4.194434062959881e+32</ns0:v>
       </ns0:c>
       <ns0:c r="E42" s="1" t="n">
-        <ns0:v>4.704336932162219e+31</ns0:v>
+        <ns0:v>4.194434062959881e+32</ns0:v>
       </ns0:c>
       <ns0:c r="F42" s="1" t="n">
         <ns0:v>2.303634000144588e+18</ns0:v>
@@ -2359,10 +2359,10 @@
         </ns0:is>
       </ns0:c>
       <ns0:c r="D43" s="1" t="n">
-        <ns0:v>1.80352987215166e+33</ns0:v>
+        <ns0:v>1.608045350153449e+34</ns0:v>
       </ns0:c>
       <ns0:c r="E43" s="1" t="n">
-        <ns0:v>1.80352987215166e+33</ns0:v>
+        <ns0:v>1.608045350153449e+34</ns0:v>
       </ns0:c>
       <ns0:c r="F43" s="1" t="n">
         <ns0:v>2.053943214130691e+19</ns0:v>
@@ -2387,10 +2387,10 @@
         </ns0:is>
       </ns0:c>
       <ns0:c r="D44" s="1" t="n">
-        <ns0:v>5.3853113417669e+33</ns0:v>
+        <ns0:v>4.801597686832597e+34</ns0:v>
       </ns0:c>
       <ns0:c r="E44" s="1" t="n">
-        <ns0:v>5.3853113417669e+33</ns0:v>
+        <ns0:v>4.801597686832597e+34</ns0:v>
       </ns0:c>
       <ns0:c r="F44" s="1" t="n">
         <ns0:v>4.259056648821401e+19</ns0:v>
@@ -2415,10 +2415,10 @@
         </ns0:is>
       </ns0:c>
       <ns0:c r="D45" s="1" t="n">
-        <ns0:v>1.608045350153449e+34</ns0:v>
+        <ns0:v>1.433749386731914e+35</ns0:v>
       </ns0:c>
       <ns0:c r="E45" s="1" t="n">
-        <ns0:v>1.608045350153449e+34</ns0:v>
+        <ns0:v>1.433749386731914e+35</ns0:v>
       </ns0:c>
       <ns0:c r="F45" s="1" t="n">
         <ns0:v>8.831579866996054e+19</ns0:v>
@@ -2443,10 +2443,10 @@
         </ns0:is>
       </ns0:c>
       <ns0:c r="D46" s="1" t="n">
-        <ns0:v>4.801597686832596e+34</ns0:v>
+        <ns0:v>4.281152728791306e+35</ns0:v>
       </ns0:c>
       <ns0:c r="E46" s="1" t="n">
-        <ns0:v>4.801597686832596e+34</ns0:v>
+        <ns0:v>4.281152728791306e+35</ns0:v>
       </ns0:c>
       <ns0:c r="F46" s="1" t="n">
         <ns0:v>1.831316401220302e+20</ns0:v>
@@ -2471,10 +2471,10 @@
         </ns0:is>
       </ns0:c>
       <ns0:c r="D47" s="1" t="n">
-        <ns0:v>4.281152728791306e+35</ns0:v>
+        <ns0:v>3.817118776422855e+36</ns0:v>
       </ns0:c>
       <ns0:c r="E47" s="1" t="n">
-        <ns0:v>4.281152728791306e+35</ns0:v>
+        <ns0:v>3.817118776422855e+36</ns0:v>
       </ns0:c>
       <ns0:c r="F47" s="1" t="n">
         <ns0:v>7.874325321093216e+20</ns0:v>
@@ -2499,10 +2499,10 @@
         </ns0:is>
       </ns0:c>
       <ns0:c r="D48" s="1" t="n">
-        <ns0:v>1.641291205319743e+37</ns0:v>
+        <ns0:v>1.463391725146999e+38</ns0:v>
       </ns0:c>
       <ns0:c r="E48" s="1" t="n">
-        <ns0:v>1.641291205319743e+37</ns0:v>
+        <ns0:v>1.463391725146999e+38</ns0:v>
       </ns0:c>
       <ns0:c r="F48" s="1" t="n">
         <ns0:v>7.020827552511277e+21</ns0:v>
@@ -2527,10 +2527,10 @@
         </ns0:is>
       </ns0:c>
       <ns0:c r="D49" s="1" t="n">
-        <ns0:v>4.900869278425468e+37</ns0:v>
+        <ns0:v>4.369664277021336e+38</ns0:v>
       </ns0:c>
       <ns0:c r="E49" s="1" t="n">
-        <ns0:v>4.900869278425468e+37</ns0:v>
+        <ns0:v>4.369664277021336e+38</ns0:v>
       </ns0:c>
       <ns0:c r="F49" s="1" t="n">
         <ns0:v>1.455838801288738e+22</ns0:v>
@@ -2555,10 +2555,10 @@
         </ns0:is>
       </ns0:c>
       <ns0:c r="D50" s="1" t="n">
-        <ns0:v>1.463391725146999e+38</ns0:v>
+        <ns0:v>1.304774761655727e+39</ns0:v>
       </ns0:c>
       <ns0:c r="E50" s="1" t="n">
-        <ns0:v>1.463391725146999e+38</ns0:v>
+        <ns0:v>1.304774761655727e+39</ns0:v>
       </ns0:c>
       <ns0:c r="F50" s="1" t="n">
         <ns0:v>3.018827338352327e+22</ns0:v>
@@ -2583,10 +2583,10 @@
         </ns0:is>
       </ns0:c>
       <ns0:c r="D51" s="1" t="n">
-        <ns0:v>4.369664277021335e+38</ns0:v>
+        <ns0:v>3.896036561907815e+39</ns0:v>
       </ns0:c>
       <ns0:c r="E51" s="1" t="n">
-        <ns0:v>4.369664277021335e+38</ns0:v>
+        <ns0:v>3.896036561907815e+39</ns0:v>
       </ns0:c>
       <ns0:c r="F51" s="1" t="n">
         <ns0:v>6.259840368807384e+22</ns0:v>
@@ -2611,10 +2611,10 @@
         </ns0:is>
       </ns0:c>
       <ns0:c r="D52" s="1" t="n">
-        <ns0:v>3.896036561907814e+39</ns0:v>
+        <ns0:v>3.473745333604802e+40</ns0:v>
       </ns0:c>
       <ns0:c r="E52" s="1" t="n">
-        <ns0:v>3.896036561907814e+39</ns0:v>
+        <ns0:v>3.473745333604802e+40</ns0:v>
       </ns0:c>
       <ns0:c r="F52" s="1" t="n">
         <ns0:v>2.691616778469064e+23</ns0:v>
@@ -2639,10 +2639,10 @@
         </ns0:is>
       </ns0:c>
       <ns0:c r="D53" s="1" t="n">
-        <ns0:v>1.493646910015478e+41</ns0:v>
+        <ns0:v>1.331750588392519e+42</ns0:v>
       </ns0:c>
       <ns0:c r="E53" s="1" t="n">
-        <ns0:v>1.493646910015478e+41</ns0:v>
+        <ns0:v>1.331750588392519e+42</ns0:v>
       </ns0:c>
       <ns0:c r="F53" s="1" t="n">
         <ns0:v>2.399872556504138e+24</ns0:v>
@@ -2667,10 +2667,10 @@
         </ns0:is>
       </ns0:c>
       <ns0:c r="D54" s="1" t="n">
-        <ns0:v>4.460005774955655e+41</ns0:v>
+        <ns0:v>3.976585948930646e+42</ns0:v>
       </ns0:c>
       <ns0:c r="E54" s="1" t="n">
-        <ns0:v>4.460005774955655e+41</ns0:v>
+        <ns0:v>3.976585948930646e+42</ns0:v>
       </ns0:c>
       <ns0:c r="F54" s="1" t="n">
         <ns0:v>4.976375733166981e+24</ns0:v>
@@ -2695,10 +2695,10 @@
         </ns0:is>
       </ns0:c>
       <ns0:c r="D55" s="1" t="n">
-        <ns0:v>1.331750588392518e+42</ns0:v>
+        <ns0:v>1.187402201813172e+43</ns0:v>
       </ns0:c>
       <ns0:c r="E55" s="1" t="n">
-        <ns0:v>1.331750588392518e+42</ns0:v>
+        <ns0:v>1.187402201813172e+43</ns0:v>
       </ns0:c>
       <ns0:c r="F55" s="1" t="n">
         <ns0:v>1.031901272029505e+25</ns0:v>
@@ -2723,10 +2723,10 @@
         </ns0:is>
       </ns0:c>
       <ns0:c r="D56" s="1" t="n">
-        <ns0:v>3.976585948930645e+42</ns0:v>
+        <ns0:v>3.545563976178902e+43</ns0:v>
       </ns0:c>
       <ns0:c r="E56" s="1" t="n">
-        <ns0:v>3.976585948930645e+42</ns0:v>
+        <ns0:v>3.545563976178902e+43</ns0:v>
       </ns0:c>
       <ns0:c r="F56" s="1" t="n">
         <ns0:v>2.139750477680381e+25</ns0:v>
@@ -2751,10 +2751,10 @@
         </ns0:is>
       </ns0:c>
       <ns0:c r="D57" s="1" t="n">
-        <ns0:v>3.545563976178902e+43</ns0:v>
+        <ns0:v>3.161260455732902e+44</ns0:v>
       </ns0:c>
       <ns0:c r="E57" s="1" t="n">
-        <ns0:v>3.545563976178902e+43</ns0:v>
+        <ns0:v>3.161260455732902e+44</ns0:v>
       </ns0:c>
       <ns0:c r="F57" s="1" t="n">
         <ns0:v>9.200535394098201e+25</ns0:v>
@@ -2779,10 +2779,10 @@
         </ns0:is>
       </ns0:c>
       <ns0:c r="D58" s="1" t="n">
-        <ns0:v>1.359284132253766e+45</ns0:v>
+        <ns0:v>1.211951386089507e+46</ns0:v>
       </ns0:c>
       <ns0:c r="E58" s="1" t="n">
-        <ns0:v>1.359284132253766e+45</ns0:v>
+        <ns0:v>1.211951386089507e+46</ns0:v>
       </ns0:c>
       <ns0:c r="F58" s="1" t="n">
         <ns0:v>8.203289775151412e+26</ns0:v>
@@ -2807,10 +2807,10 @@
         </ns0:is>
       </ns0:c>
       <ns0:c r="D59" s="1" t="n">
-        <ns0:v>4.058800670363627e+45</ns0:v>
+        <ns0:v>3.618867447641088e+46</ns0:v>
       </ns0:c>
       <ns0:c r="E59" s="1" t="n">
-        <ns0:v>4.058800670363627e+45</ns0:v>
+        <ns0:v>3.618867447641088e+46</ns0:v>
       </ns0:c>
       <ns0:c r="F59" s="1" t="n">
         <ns0:v>1.701034167775397e+27</ns0:v>
@@ -2835,10 +2835,10 @@
         </ns0:is>
       </ns0:c>
       <ns0:c r="D60" s="1" t="n">
-        <ns0:v>1.211951386089506e+46</ns0:v>
+        <ns0:v>1.080588029677713e+47</ns0:v>
       </ns0:c>
       <ns0:c r="E60" s="1" t="n">
-        <ns0:v>1.211951386089506e+46</ns0:v>
+        <ns0:v>1.080588029677713e+47</ns0:v>
       </ns0:c>
       <ns0:c r="F60" s="1" t="n">
         <ns0:v>3.527264450299061e+27</ns0:v>
@@ -2863,10 +2863,10 @@
         </ns0:is>
       </ns0:c>
       <ns0:c r="D61" s="1" t="n">
-        <ns0:v>3.618867447641087e+46</ns0:v>
+        <ns0:v>3.226618567209174e+47</ns0:v>
       </ns0:c>
       <ns0:c r="E61" s="1" t="n">
-        <ns0:v>3.618867447641087e+46</ns0:v>
+        <ns0:v>3.226618567209174e+47</ns0:v>
       </ns0:c>
       <ns0:c r="F61" s="1" t="n">
         <ns0:v>7.314135564140134e+27</ns0:v>
@@ -2891,10 +2891,10 @@
         </ns0:is>
       </ns0:c>
       <ns0:c r="D62" s="1" t="n">
-        <ns0:v>3.226618567209173e+47</ns0:v>
+        <ns0:v>2.876885525344484e+48</ns0:v>
       </ns0:c>
       <ns0:c r="E62" s="1" t="n">
-        <ns0:v>3.226618567209173e+47</ns0:v>
+        <ns0:v>2.876885525344484e+48</ns0:v>
       </ns0:c>
       <ns0:c r="F62" s="1" t="n">
         <ns0:v>3.14494441464289e+28</ns0:v>
@@ -2919,10 +2919,10 @@
         </ns0:is>
       </ns0:c>
       <ns0:c r="D63" s="1" t="n">
-        <ns0:v>1.237008117385472e+49</ns0:v>
+        <ns0:v>1.102928862991691e+50</ns0:v>
       </ns0:c>
       <ns0:c r="E63" s="1" t="n">
-        <ns0:v>1.237008117385472e+49</ns0:v>
+        <ns0:v>1.102928862991691e+50</ns0:v>
       </ns0:c>
       <ns0:c r="F63" s="1" t="n">
         <ns0:v>2.804064030513767e+29</ns0:v>
@@ -2948,11 +2948,11 @@
       </ns0:c>
       <ns0:c r="D64" s="1">
         <ns0:f>ROUND(D63*10,0)</ns0:f>
-        <ns0:v>1.2370081173854715e+50</ns0:v>
+        <ns0:v>1.1029288629916913e+51</ns0:v>
       </ns0:c>
       <ns0:c r="E64" s="1">
         <ns0:f>D64</ns0:f>
-        <ns0:v>1.2370081173854715e+50</ns0:v>
+        <ns0:v>1.1029288629916913e+51</ns0:v>
       </ns0:c>
       <ns0:c r="F64" s="1">
         <ns0:f>ROUND(F63*1.4,-5)</ns0:f>
@@ -2979,11 +2979,11 @@
       </ns0:c>
       <ns0:c r="D65" s="1">
         <ns0:f>ROUND(D64*10,0)</ns0:f>
-        <ns0:v>1.2370081173854714e+51</ns0:v>
+        <ns0:v>1.1029288629916913e+52</ns0:v>
       </ns0:c>
       <ns0:c r="E65" s="1">
         <ns0:f>D65</ns0:f>
-        <ns0:v>1.2370081173854714e+51</ns0:v>
+        <ns0:v>1.1029288629916913e+52</ns0:v>
       </ns0:c>
       <ns0:c r="F65" s="1">
         <ns0:f>ROUND(F64*1.4,-5)</ns0:f>
@@ -3010,11 +3010,11 @@
       </ns0:c>
       <ns0:c r="D66" s="1">
         <ns0:f>ROUND(D65*10,0)</ns0:f>
-        <ns0:v>1.2370081173854714e+52</ns0:v>
+        <ns0:v>1.1029288629916914e+53</ns0:v>
       </ns0:c>
       <ns0:c r="E66" s="1">
         <ns0:f>D66</ns0:f>
-        <ns0:v>1.2370081173854714e+52</ns0:v>
+        <ns0:v>1.1029288629916914e+53</ns0:v>
       </ns0:c>
       <ns0:c r="F66" s="1">
         <ns0:f>ROUND(F65*1.4,-5)</ns0:f>
@@ -3041,11 +3041,11 @@
       </ns0:c>
       <ns0:c r="D67" s="1">
         <ns0:f>ROUND(D66*10,0)</ns0:f>
-        <ns0:v>1.2370081173854714e+53</ns0:v>
+        <ns0:v>1.1029288629916914e+54</ns0:v>
       </ns0:c>
       <ns0:c r="E67" s="1">
         <ns0:f>D67</ns0:f>
-        <ns0:v>1.2370081173854714e+53</ns0:v>
+        <ns0:v>1.1029288629916914e+54</ns0:v>
       </ns0:c>
       <ns0:c r="F67" s="1">
         <ns0:f>ROUND(F66*1.4,-5)</ns0:f>
@@ -3072,11 +3072,11 @@
       </ns0:c>
       <ns0:c r="D68" s="1">
         <ns0:f>ROUND(D67*10,0)</ns0:f>
-        <ns0:v>1.2370081173854715e+54</ns0:v>
+        <ns0:v>1.1029288629916915e+55</ns0:v>
       </ns0:c>
       <ns0:c r="E68" s="1">
         <ns0:f>D68</ns0:f>
-        <ns0:v>1.2370081173854715e+54</ns0:v>
+        <ns0:v>1.1029288629916915e+55</ns0:v>
       </ns0:c>
       <ns0:c r="F68" s="1">
         <ns0:f>ROUND(F67*1.4,-5)</ns0:f>
@@ -3103,11 +3103,11 @@
       </ns0:c>
       <ns0:c r="D69" s="1">
         <ns0:f>ROUND(D68*10,0)</ns0:f>
-        <ns0:v>1.2370081173854714e+55</ns0:v>
+        <ns0:v>1.1029288629916915e+56</ns0:v>
       </ns0:c>
       <ns0:c r="E69" s="1">
         <ns0:f>D69</ns0:f>
-        <ns0:v>1.2370081173854714e+55</ns0:v>
+        <ns0:v>1.1029288629916915e+56</ns0:v>
       </ns0:c>
       <ns0:c r="F69" s="1">
         <ns0:f>ROUND(F68*1.4,-5)</ns0:f>
@@ -3134,11 +3134,11 @@
       </ns0:c>
       <ns0:c r="D70" s="1">
         <ns0:f>ROUND(D69*10,0)</ns0:f>
-        <ns0:v>1.2370081173854714e+56</ns0:v>
+        <ns0:v>1.1029288629916915e+57</ns0:v>
       </ns0:c>
       <ns0:c r="E70" s="1">
         <ns0:f>D70</ns0:f>
-        <ns0:v>1.2370081173854714e+56</ns0:v>
+        <ns0:v>1.1029288629916915e+57</ns0:v>
       </ns0:c>
       <ns0:c r="F70" s="1">
         <ns0:f>ROUND(F69*1.4,-5)</ns0:f>
@@ -3165,11 +3165,11 @@
       </ns0:c>
       <ns0:c r="D71" s="1">
         <ns0:f>ROUND(D70*10,0)</ns0:f>
-        <ns0:v>1.2370081173854715e+57</ns0:v>
+        <ns0:v>1.1029288629916915e+58</ns0:v>
       </ns0:c>
       <ns0:c r="E71" s="1">
         <ns0:f>D71</ns0:f>
-        <ns0:v>1.2370081173854715e+57</ns0:v>
+        <ns0:v>1.1029288629916915e+58</ns0:v>
       </ns0:c>
       <ns0:c r="F71" s="1">
         <ns0:f>ROUND(F70*1.4,-5)</ns0:f>
@@ -3196,11 +3196,11 @@
       </ns0:c>
       <ns0:c r="D72" s="1">
         <ns0:f>ROUND(D71*10,0)</ns0:f>
-        <ns0:v>1.2370081173854714e+58</ns0:v>
+        <ns0:v>1.1029288629916914e+59</ns0:v>
       </ns0:c>
       <ns0:c r="E72" s="1">
         <ns0:f>D72</ns0:f>
-        <ns0:v>1.2370081173854714e+58</ns0:v>
+        <ns0:v>1.1029288629916914e+59</ns0:v>
       </ns0:c>
       <ns0:c r="F72" s="1">
         <ns0:f>ROUND(F71*1.4,-5)</ns0:f>
@@ -3227,11 +3227,11 @@
       </ns0:c>
       <ns0:c r="D73" s="1">
         <ns0:f>ROUND(D72*10,0)</ns0:f>
-        <ns0:v>1.2370081173854714e+59</ns0:v>
+        <ns0:v>1.1029288629916914e+60</ns0:v>
       </ns0:c>
       <ns0:c r="E73" s="1">
         <ns0:f>D73</ns0:f>
-        <ns0:v>1.2370081173854714e+59</ns0:v>
+        <ns0:v>1.1029288629916914e+60</ns0:v>
       </ns0:c>
       <ns0:c r="F73" s="1">
         <ns0:f>ROUND(F72*1.4,-5)</ns0:f>
@@ -3258,11 +3258,11 @@
       </ns0:c>
       <ns0:c r="D74" s="1">
         <ns0:f>ROUND(D73*10,0)</ns0:f>
-        <ns0:v>1.2370081173854713e+60</ns0:v>
+        <ns0:v>1.1029288629916915e+61</ns0:v>
       </ns0:c>
       <ns0:c r="E74" s="1">
         <ns0:f>D74</ns0:f>
-        <ns0:v>1.2370081173854713e+60</ns0:v>
+        <ns0:v>1.1029288629916915e+61</ns0:v>
       </ns0:c>
       <ns0:c r="F74" s="1">
         <ns0:f>ROUND(F73*1.4,-5)</ns0:f>
@@ -3290,11 +3290,11 @@
       </ns0:c>
       <ns0:c r="D75" s="1">
         <ns0:f>ROUND(D74*10,0)</ns0:f>
-        <ns0:v>1.2370081173854713e+61</ns0:v>
+        <ns0:v>1.1029288629916914e+62</ns0:v>
       </ns0:c>
       <ns0:c r="E75" s="1">
         <ns0:f>D75</ns0:f>
-        <ns0:v>1.2370081173854713e+61</ns0:v>
+        <ns0:v>1.1029288629916914e+62</ns0:v>
       </ns0:c>
       <ns0:c r="F75" s="1">
         <ns0:f>ROUND(F74*1.4,-5)</ns0:f>
@@ -3322,11 +3322,11 @@
       </ns0:c>
       <ns0:c r="D76" s="1">
         <ns0:f>ROUND(D75*10,0)</ns0:f>
-        <ns0:v>1.2370081173854713e+62</ns0:v>
+        <ns0:v>1.1029288629916915e+63</ns0:v>
       </ns0:c>
       <ns0:c r="E76" s="1">
         <ns0:f>D76</ns0:f>
-        <ns0:v>1.2370081173854713e+62</ns0:v>
+        <ns0:v>1.1029288629916915e+63</ns0:v>
       </ns0:c>
       <ns0:c r="F76" s="1">
         <ns0:f>ROUND(F75*1.4,-5)</ns0:f>
@@ -3354,11 +3354,11 @@
       </ns0:c>
       <ns0:c r="D77" s="1">
         <ns0:f>ROUND(D76*10,0)</ns0:f>
-        <ns0:v>1.2370081173854712e+63</ns0:v>
+        <ns0:v>1.1029288629916914e+64</ns0:v>
       </ns0:c>
       <ns0:c r="E77" s="1">
         <ns0:f>D77</ns0:f>
-        <ns0:v>1.2370081173854712e+63</ns0:v>
+        <ns0:v>1.1029288629916914e+64</ns0:v>
       </ns0:c>
       <ns0:c r="F77" s="1">
         <ns0:f>ROUND(F76*1.4,-5)</ns0:f>
@@ -3386,11 +3386,11 @@
       </ns0:c>
       <ns0:c r="D78" s="1">
         <ns0:f>ROUND(D77*10,0)</ns0:f>
-        <ns0:v>1.2370081173854713e+64</ns0:v>
+        <ns0:v>1.1029288629916914e+65</ns0:v>
       </ns0:c>
       <ns0:c r="E78" s="1">
         <ns0:f>D78</ns0:f>
-        <ns0:v>1.2370081173854713e+64</ns0:v>
+        <ns0:v>1.1029288629916914e+65</ns0:v>
       </ns0:c>
       <ns0:c r="F78" s="1">
         <ns0:f>ROUND(F77*1.4,-5)</ns0:f>
@@ -3418,11 +3418,11 @@
       </ns0:c>
       <ns0:c r="D79" s="1">
         <ns0:f>ROUND(D78*10,0)</ns0:f>
-        <ns0:v>1.2370081173854713e+65</ns0:v>
+        <ns0:v>1.1029288629916914e+66</ns0:v>
       </ns0:c>
       <ns0:c r="E79" s="1">
         <ns0:f>D79</ns0:f>
-        <ns0:v>1.2370081173854713e+65</ns0:v>
+        <ns0:v>1.1029288629916914e+66</ns0:v>
       </ns0:c>
       <ns0:c r="F79" s="1">
         <ns0:f>ROUND(F78*1.4,-5)</ns0:f>
@@ -3450,11 +3450,11 @@
       </ns0:c>
       <ns0:c r="D80" s="1">
         <ns0:f>ROUND(D79*10,0)</ns0:f>
-        <ns0:v>1.2370081173854713e+66</ns0:v>
+        <ns0:v>1.1029288629916915e+67</ns0:v>
       </ns0:c>
       <ns0:c r="E80" s="1">
         <ns0:f>D80</ns0:f>
-        <ns0:v>1.2370081173854713e+66</ns0:v>
+        <ns0:v>1.1029288629916915e+67</ns0:v>
       </ns0:c>
       <ns0:c r="F80" s="1">
         <ns0:f>ROUND(F79*1.4,-5)</ns0:f>
@@ -3482,11 +3482,11 @@
       </ns0:c>
       <ns0:c r="D81" s="1">
         <ns0:f>ROUND(D80*10,0)</ns0:f>
-        <ns0:v>1.2370081173854713e+67</ns0:v>
+        <ns0:v>1.1029288629916915e+68</ns0:v>
       </ns0:c>
       <ns0:c r="E81" s="1">
         <ns0:f>D81</ns0:f>
-        <ns0:v>1.2370081173854713e+67</ns0:v>
+        <ns0:v>1.1029288629916915e+68</ns0:v>
       </ns0:c>
       <ns0:c r="F81" s="1">
         <ns0:f>ROUND(F80*1.4,-5)</ns0:f>
@@ -3514,11 +3514,11 @@
       </ns0:c>
       <ns0:c r="D82" s="1">
         <ns0:f>ROUND(D81*10,0)</ns0:f>
-        <ns0:v>1.2370081173854713e+68</ns0:v>
+        <ns0:v>1.1029288629916916e+69</ns0:v>
       </ns0:c>
       <ns0:c r="E82" s="1">
         <ns0:f>D82</ns0:f>
-        <ns0:v>1.2370081173854713e+68</ns0:v>
+        <ns0:v>1.1029288629916916e+69</ns0:v>
       </ns0:c>
       <ns0:c r="F82" s="1">
         <ns0:f>ROUND(F81*1.4,-5)</ns0:f>
@@ -3546,11 +3546,11 @@
       </ns0:c>
       <ns0:c r="D83" s="1">
         <ns0:f>ROUND(D82*10,0)</ns0:f>
-        <ns0:v>1.2370081173854714e+69</ns0:v>
+        <ns0:v>1.1029288629916916e+70</ns0:v>
       </ns0:c>
       <ns0:c r="E83" s="1">
         <ns0:f>D83</ns0:f>
-        <ns0:v>1.2370081173854714e+69</ns0:v>
+        <ns0:v>1.1029288629916916e+70</ns0:v>
       </ns0:c>
       <ns0:c r="F83" s="1">
         <ns0:f>ROUND(F82*1.4,-5)</ns0:f>
@@ -3578,11 +3578,11 @@
       </ns0:c>
       <ns0:c r="D84" s="1">
         <ns0:f>ROUND(D83*20,2-INT(LOG10(ABS(D83*20))))</ns0:f>
-        <ns0:v>2.4699999999999998e+70</ns0:v>
+        <ns0:v>2.21e+71</ns0:v>
       </ns0:c>
       <ns0:c r="E84" s="1">
         <ns0:f>D84</ns0:f>
-        <ns0:v>2.4699999999999998e+70</ns0:v>
+        <ns0:v>2.21e+71</ns0:v>
       </ns0:c>
       <ns0:c r="F84" s="1">
         <ns0:f>ROUND(F83*1.4,-5)</ns0:f>
@@ -3610,11 +3610,11 @@
       </ns0:c>
       <ns0:c r="D85" s="1">
         <ns0:f>ROUND(D84*20,2-INT(LOG10(ABS(D84*20))))</ns0:f>
-        <ns0:v>4.94e+71</ns0:v>
+        <ns0:v>4.42e+72</ns0:v>
       </ns0:c>
       <ns0:c r="E85" s="1">
         <ns0:f>D85</ns0:f>
-        <ns0:v>4.94e+71</ns0:v>
+        <ns0:v>4.42e+72</ns0:v>
       </ns0:c>
       <ns0:c r="F85" s="1">
         <ns0:f>ROUND(F84*1.4,-5)</ns0:f>
@@ -3642,11 +3642,11 @@
       </ns0:c>
       <ns0:c r="D86" s="1">
         <ns0:f>ROUND(D85*20,2-INT(LOG10(ABS(D85*20))))</ns0:f>
-        <ns0:v>9.88e+72</ns0:v>
+        <ns0:v>8.840000000000001e+73</ns0:v>
       </ns0:c>
       <ns0:c r="E86" s="1">
         <ns0:f>D86</ns0:f>
-        <ns0:v>9.88e+72</ns0:v>
+        <ns0:v>8.840000000000001e+73</ns0:v>
       </ns0:c>
       <ns0:c r="F86" s="1">
         <ns0:f>ROUND(F85*1.4,-5)</ns0:f>
@@ -3674,11 +3674,11 @@
       </ns0:c>
       <ns0:c r="D87" s="1">
         <ns0:f>ROUND(D86*20,2-INT(LOG10(ABS(D86*20))))</ns0:f>
-        <ns0:v>1.98e+74</ns0:v>
+        <ns0:v>1.77e+75</ns0:v>
       </ns0:c>
       <ns0:c r="E87" s="1">
         <ns0:f>D87</ns0:f>
-        <ns0:v>1.98e+74</ns0:v>
+        <ns0:v>1.77e+75</ns0:v>
       </ns0:c>
       <ns0:c r="F87" s="1">
         <ns0:f>ROUND(F86*1.4,-5)</ns0:f>
@@ -3706,11 +3706,11 @@
       </ns0:c>
       <ns0:c r="D88" s="1">
         <ns0:f>ROUND(D87*20,2-INT(LOG10(ABS(D87*20))))</ns0:f>
-        <ns0:v>3.96e+75</ns0:v>
+        <ns0:v>3.5400000000000004e+76</ns0:v>
       </ns0:c>
       <ns0:c r="E88" s="1">
         <ns0:f>D88</ns0:f>
-        <ns0:v>3.96e+75</ns0:v>
+        <ns0:v>3.5400000000000004e+76</ns0:v>
       </ns0:c>
       <ns0:c r="F88" s="1">
         <ns0:f>ROUND(F87*1.4,-5)</ns0:f>
@@ -3738,11 +3738,11 @@
       </ns0:c>
       <ns0:c r="D89" s="1">
         <ns0:f>ROUND(D88*20,2-INT(LOG10(ABS(D88*20))))</ns0:f>
-        <ns0:v>7.920000000000001e+76</ns0:v>
+        <ns0:v>7.08e+77</ns0:v>
       </ns0:c>
       <ns0:c r="E89" s="1">
         <ns0:f>D89</ns0:f>
-        <ns0:v>7.920000000000001e+76</ns0:v>
+        <ns0:v>7.08e+77</ns0:v>
       </ns0:c>
       <ns0:c r="F89" s="1">
         <ns0:f>ROUND(F88*1.4,-5)</ns0:f>
@@ -3770,11 +3770,11 @@
       </ns0:c>
       <ns0:c r="D90" s="1">
         <ns0:f>ROUND(D89*20,2-INT(LOG10(ABS(D89*20))))</ns0:f>
-        <ns0:v>1.58e+78</ns0:v>
+        <ns0:v>1.4200000000000001e+79</ns0:v>
       </ns0:c>
       <ns0:c r="E90" s="1">
         <ns0:f>D90</ns0:f>
-        <ns0:v>1.58e+78</ns0:v>
+        <ns0:v>1.4200000000000001e+79</ns0:v>
       </ns0:c>
       <ns0:c r="F90" s="1">
         <ns0:f>ROUND(F89*1.4,-5)</ns0:f>
@@ -3802,11 +3802,11 @@
       </ns0:c>
       <ns0:c r="D91" s="1">
         <ns0:f>ROUND(D90*20,2-INT(LOG10(ABS(D90*20))))</ns0:f>
-        <ns0:v>3.1600000000000005e+79</ns0:v>
+        <ns0:v>2.84e+80</ns0:v>
       </ns0:c>
       <ns0:c r="E91" s="1">
         <ns0:f>D91</ns0:f>
-        <ns0:v>3.1600000000000005e+79</ns0:v>
+        <ns0:v>2.84e+80</ns0:v>
       </ns0:c>
       <ns0:c r="F91" s="1">
         <ns0:f>ROUND(F90*1.4,-5)</ns0:f>
@@ -3834,11 +3834,11 @@
       </ns0:c>
       <ns0:c r="D92" s="1">
         <ns0:f>ROUND(D91*20,2-INT(LOG10(ABS(D91*20))))</ns0:f>
-        <ns0:v>6.32e+80</ns0:v>
+        <ns0:v>5.68e+81</ns0:v>
       </ns0:c>
       <ns0:c r="E92" s="1">
         <ns0:f>D92</ns0:f>
-        <ns0:v>6.32e+80</ns0:v>
+        <ns0:v>5.68e+81</ns0:v>
       </ns0:c>
       <ns0:c r="F92" s="1">
         <ns0:f>ROUND(F91*1.4,-5)</ns0:f>
@@ -3866,11 +3866,11 @@
       </ns0:c>
       <ns0:c r="D93" s="1">
         <ns0:f>ROUND(D92*20,2-INT(LOG10(ABS(D92*20))))</ns0:f>
-        <ns0:v>1.26e+82</ns0:v>
+        <ns0:v>1.14e+83</ns0:v>
       </ns0:c>
       <ns0:c r="E93" s="1">
         <ns0:f>D93</ns0:f>
-        <ns0:v>1.26e+82</ns0:v>
+        <ns0:v>1.14e+83</ns0:v>
       </ns0:c>
       <ns0:c r="F93" s="1">
         <ns0:f>ROUND(F92*1.4,-5)</ns0:f>
@@ -3898,11 +3898,11 @@
       </ns0:c>
       <ns0:c r="D94" s="1">
         <ns0:f>ROUND(D93*20,2-INT(LOG10(ABS(D93*20))))</ns0:f>
-        <ns0:v>2.52e+83</ns0:v>
+        <ns0:v>2.2800000000000002e+84</ns0:v>
       </ns0:c>
       <ns0:c r="E94" s="1">
         <ns0:f>D94</ns0:f>
-        <ns0:v>2.52e+83</ns0:v>
+        <ns0:v>2.2800000000000002e+84</ns0:v>
       </ns0:c>
       <ns0:c r="F94" s="1">
         <ns0:f>ROUND(F93*1.4,-5)</ns0:f>
@@ -3930,11 +3930,11 @@
       </ns0:c>
       <ns0:c r="D95" s="1">
         <ns0:f>ROUND(D94*20,2-INT(LOG10(ABS(D94*20))))</ns0:f>
-        <ns0:v>5.04e+84</ns0:v>
+        <ns0:v>4.56e+85</ns0:v>
       </ns0:c>
       <ns0:c r="E95" s="1">
         <ns0:f>D95</ns0:f>
-        <ns0:v>5.04e+84</ns0:v>
+        <ns0:v>4.56e+85</ns0:v>
       </ns0:c>
       <ns0:c r="F95" s="1">
         <ns0:f>ROUND(F94*1.4,-5)</ns0:f>
@@ -3962,11 +3962,11 @@
       </ns0:c>
       <ns0:c r="D96" s="1">
         <ns0:f>ROUND(D95*20,2-INT(LOG10(ABS(D95*20))))</ns0:f>
-        <ns0:v>1.0099999999999999e+86</ns0:v>
+        <ns0:v>9.119999999999999e+86</ns0:v>
       </ns0:c>
       <ns0:c r="E96" s="1">
         <ns0:f>D96</ns0:f>
-        <ns0:v>1.0099999999999999e+86</ns0:v>
+        <ns0:v>9.119999999999999e+86</ns0:v>
       </ns0:c>
       <ns0:c r="F96" s="1">
         <ns0:f>ROUND(F95*1.4,-5)</ns0:f>
@@ -3994,11 +3994,11 @@
       </ns0:c>
       <ns0:c r="D97" s="1">
         <ns0:f>ROUND(D96*20,2-INT(LOG10(ABS(D96*20))))</ns0:f>
-        <ns0:v>2.02e+87</ns0:v>
+        <ns0:v>1.8199999999999998e+88</ns0:v>
       </ns0:c>
       <ns0:c r="E97" s="1">
         <ns0:f>D97</ns0:f>
-        <ns0:v>2.02e+87</ns0:v>
+        <ns0:v>1.8199999999999998e+88</ns0:v>
       </ns0:c>
       <ns0:c r="F97" s="1">
         <ns0:f>ROUND(F96*1.4,-5)</ns0:f>
@@ -4026,11 +4026,11 @@
       </ns0:c>
       <ns0:c r="D98" s="1">
         <ns0:f>ROUND(D97*20,2-INT(LOG10(ABS(D97*20))))</ns0:f>
-        <ns0:v>4.04e+88</ns0:v>
+        <ns0:v>3.64e+89</ns0:v>
       </ns0:c>
       <ns0:c r="E98" s="1">
         <ns0:f>D98</ns0:f>
-        <ns0:v>4.04e+88</ns0:v>
+        <ns0:v>3.64e+89</ns0:v>
       </ns0:c>
       <ns0:c r="F98" s="1">
         <ns0:f>ROUND(F97*1.4,-5)</ns0:f>
@@ -4058,11 +4058,11 @@
       </ns0:c>
       <ns0:c r="D99" s="1">
         <ns0:f>ROUND(D98*20,2-INT(LOG10(ABS(D98*20))))</ns0:f>
-        <ns0:v>8.08e+89</ns0:v>
+        <ns0:v>7.280000000000001e+90</ns0:v>
       </ns0:c>
       <ns0:c r="E99" s="1">
         <ns0:f>D99</ns0:f>
-        <ns0:v>8.08e+89</ns0:v>
+        <ns0:v>7.280000000000001e+90</ns0:v>
       </ns0:c>
       <ns0:c r="F99" s="1">
         <ns0:f>ROUND(F98*1.4,-5)</ns0:f>
@@ -4090,11 +4090,11 @@
       </ns0:c>
       <ns0:c r="D100" s="1">
         <ns0:f>ROUND(D99*20,2-INT(LOG10(ABS(D99*20))))</ns0:f>
-        <ns0:v>1.62e+91</ns0:v>
+        <ns0:v>1.46e+92</ns0:v>
       </ns0:c>
       <ns0:c r="E100" s="1">
         <ns0:f>D100</ns0:f>
-        <ns0:v>1.62e+91</ns0:v>
+        <ns0:v>1.46e+92</ns0:v>
       </ns0:c>
       <ns0:c r="F100" s="1">
         <ns0:f>ROUND(F99*1.4,-5)</ns0:f>
@@ -4122,11 +4122,11 @@
       </ns0:c>
       <ns0:c r="D101" s="1">
         <ns0:f>ROUND(D100*20,2-INT(LOG10(ABS(D100*20))))</ns0:f>
-        <ns0:v>3.24e+92</ns0:v>
+        <ns0:v>2.9199999999999997e+93</ns0:v>
       </ns0:c>
       <ns0:c r="E101" s="1">
         <ns0:f>D101</ns0:f>
-        <ns0:v>3.24e+92</ns0:v>
+        <ns0:v>2.9199999999999997e+93</ns0:v>
       </ns0:c>
       <ns0:c r="F101" s="1">
         <ns0:f>ROUND(F100*1.4,-5)</ns0:f>
@@ -4154,11 +4154,11 @@
       </ns0:c>
       <ns0:c r="D102" s="1">
         <ns0:f>ROUND(D101*20,2-INT(LOG10(ABS(D101*20))))</ns0:f>
-        <ns0:v>6.48e+93</ns0:v>
+        <ns0:v>5.84e+94</ns0:v>
       </ns0:c>
       <ns0:c r="E102" s="1">
         <ns0:f>D102</ns0:f>
-        <ns0:v>6.48e+93</ns0:v>
+        <ns0:v>5.84e+94</ns0:v>
       </ns0:c>
       <ns0:c r="F102" s="1">
         <ns0:f>ROUND(F101*1.4,-5)</ns0:f>
@@ -4186,11 +4186,11 @@
       </ns0:c>
       <ns0:c r="D103" s="1">
         <ns0:f>ROUND(D102*20,2-INT(LOG10(ABS(D102*20))))</ns0:f>
-        <ns0:v>1.3000000000000001e+95</ns0:v>
+        <ns0:v>1.17e+96</ns0:v>
       </ns0:c>
       <ns0:c r="E103" s="1">
         <ns0:f>D103</ns0:f>
-        <ns0:v>1.3000000000000001e+95</ns0:v>
+        <ns0:v>1.17e+96</ns0:v>
       </ns0:c>
       <ns0:c r="F103" s="1">
         <ns0:f>ROUND(F102*1.4,-5)</ns0:f>
@@ -4218,11 +4218,11 @@
       </ns0:c>
       <ns0:c r="D104" s="1">
         <ns0:f>ROUND(D103*20,2-INT(LOG10(ABS(D103*20))))</ns0:f>
-        <ns0:v>2.6e+96</ns0:v>
+        <ns0:v>2.34e+97</ns0:v>
       </ns0:c>
       <ns0:c r="E104" s="1">
         <ns0:f>D104</ns0:f>
-        <ns0:v>2.6e+96</ns0:v>
+        <ns0:v>2.34e+97</ns0:v>
       </ns0:c>
       <ns0:c r="F104" s="1">
         <ns0:f>ROUND(F103*1.4,-5)</ns0:f>
@@ -4250,11 +4250,11 @@
       </ns0:c>
       <ns0:c r="D105" s="1">
         <ns0:f>ROUND(D104*20,2-INT(LOG10(ABS(D104*20))))</ns0:f>
-        <ns0:v>5.2e+97</ns0:v>
+        <ns0:v>4.6800000000000005e+98</ns0:v>
       </ns0:c>
       <ns0:c r="E105" s="1">
         <ns0:f>D105</ns0:f>
-        <ns0:v>5.2e+97</ns0:v>
+        <ns0:v>4.6800000000000005e+98</ns0:v>
       </ns0:c>
       <ns0:c r="F105" s="1">
         <ns0:f>ROUND(F104*1.4,-5)</ns0:f>
@@ -4282,11 +4282,11 @@
       </ns0:c>
       <ns0:c r="D106" s="1">
         <ns0:f>ROUND(D105*20,2-INT(LOG10(ABS(D105*20))))</ns0:f>
-        <ns0:v>1.04e+99</ns0:v>
+        <ns0:v>9.36e+99</ns0:v>
       </ns0:c>
       <ns0:c r="E106" s="1">
         <ns0:f>D106</ns0:f>
-        <ns0:v>1.04e+99</ns0:v>
+        <ns0:v>9.36e+99</ns0:v>
       </ns0:c>
       <ns0:c r="F106" s="1">
         <ns0:f>ROUND(F105*1.4,-5)</ns0:f>
@@ -4314,11 +4314,11 @@
       </ns0:c>
       <ns0:c r="D107" s="1">
         <ns0:f>ROUND(D106*20,2-INT(LOG10(ABS(D106*20))))</ns0:f>
-        <ns0:v>2.08e+100</ns0:v>
+        <ns0:v>1.87e+101</ns0:v>
       </ns0:c>
       <ns0:c r="E107" s="1">
         <ns0:f>D107</ns0:f>
-        <ns0:v>2.08e+100</ns0:v>
+        <ns0:v>1.87e+101</ns0:v>
       </ns0:c>
       <ns0:c r="F107" s="1">
         <ns0:f>ROUND(F106*1.4,-5)</ns0:f>
@@ -4346,11 +4346,11 @@
       </ns0:c>
       <ns0:c r="D108" s="1">
         <ns0:f>ROUND(D107*20,2-INT(LOG10(ABS(D107*20))))</ns0:f>
-        <ns0:v>4.1599999999999996e+101</ns0:v>
+        <ns0:v>3.74e+102</ns0:v>
       </ns0:c>
       <ns0:c r="E108" s="1">
         <ns0:f>D108</ns0:f>
-        <ns0:v>4.1599999999999996e+101</ns0:v>
+        <ns0:v>3.74e+102</ns0:v>
       </ns0:c>
       <ns0:c r="F108" s="1">
         <ns0:f>ROUND(F107*1.4,-5)</ns0:f>
@@ -4378,11 +4378,11 @@
       </ns0:c>
       <ns0:c r="D109" s="1">
         <ns0:f>ROUND(D108*20,2-INT(LOG10(ABS(D108*20))))</ns0:f>
-        <ns0:v>8.32e+102</ns0:v>
+        <ns0:v>7.48e+103</ns0:v>
       </ns0:c>
       <ns0:c r="E109" s="1">
         <ns0:f>D109</ns0:f>
-        <ns0:v>8.32e+102</ns0:v>
+        <ns0:v>7.48e+103</ns0:v>
       </ns0:c>
       <ns0:c r="F109" s="1">
         <ns0:f>ROUND(F108*1.4,-5)</ns0:f>
@@ -4410,11 +4410,11 @@
       </ns0:c>
       <ns0:c r="D110" s="1">
         <ns0:f>ROUND(D109*20,2-INT(LOG10(ABS(D109*20))))</ns0:f>
-        <ns0:v>1.66e+104</ns0:v>
+        <ns0:v>1.5e+105</ns0:v>
       </ns0:c>
       <ns0:c r="E110" s="1">
         <ns0:f>D110</ns0:f>
-        <ns0:v>1.66e+104</ns0:v>
+        <ns0:v>1.5e+105</ns0:v>
       </ns0:c>
       <ns0:c r="F110" s="1">
         <ns0:f>ROUND(F109*1.4,-5)</ns0:f>
@@ -4442,11 +4442,11 @@
       </ns0:c>
       <ns0:c r="D111" s="1">
         <ns0:f>ROUND(D110*20,2-INT(LOG10(ABS(D110*20))))</ns0:f>
-        <ns0:v>3.32e+105</ns0:v>
+        <ns0:v>3e+106</ns0:v>
       </ns0:c>
       <ns0:c r="E111" s="1">
         <ns0:f>D111</ns0:f>
-        <ns0:v>3.32e+105</ns0:v>
+        <ns0:v>3e+106</ns0:v>
       </ns0:c>
       <ns0:c r="F111" s="1">
         <ns0:f>ROUND(F110*1.4,-5)</ns0:f>
@@ -4474,11 +4474,11 @@
       </ns0:c>
       <ns0:c r="D112" s="1">
         <ns0:f>ROUND(D111*20,2-INT(LOG10(ABS(D111*20))))</ns0:f>
-        <ns0:v>6.640000000000001e+106</ns0:v>
+        <ns0:v>6e+107</ns0:v>
       </ns0:c>
       <ns0:c r="E112" s="1">
         <ns0:f>D112</ns0:f>
-        <ns0:v>6.640000000000001e+106</ns0:v>
+        <ns0:v>6e+107</ns0:v>
       </ns0:c>
       <ns0:c r="F112" s="1">
         <ns0:f>ROUND(F111*1.4,-5)</ns0:f>
@@ -4506,11 +4506,11 @@
       </ns0:c>
       <ns0:c r="D113" s="1">
         <ns0:f>ROUND(D112*20,2-INT(LOG10(ABS(D112*20))))</ns0:f>
-        <ns0:v>1.33e+108</ns0:v>
+        <ns0:v>1.2e+109</ns0:v>
       </ns0:c>
       <ns0:c r="E113" s="1">
         <ns0:f>D113</ns0:f>
-        <ns0:v>1.33e+108</ns0:v>
+        <ns0:v>1.2e+109</ns0:v>
       </ns0:c>
       <ns0:c r="F113" s="1">
         <ns0:f>ROUND(F112*1.4,-5)</ns0:f>
@@ -4538,11 +4538,11 @@
       </ns0:c>
       <ns0:c r="D114" s="1">
         <ns0:f>ROUND(D113*20,2-INT(LOG10(ABS(D113*20))))</ns0:f>
-        <ns0:v>2.66e+109</ns0:v>
+        <ns0:v>2.3999999999999998e+110</ns0:v>
       </ns0:c>
       <ns0:c r="E114" s="1">
         <ns0:f>D114</ns0:f>
-        <ns0:v>2.66e+109</ns0:v>
+        <ns0:v>2.3999999999999998e+110</ns0:v>
       </ns0:c>
       <ns0:c r="F114" s="1">
         <ns0:f>ROUND(F113*1.4,-5)</ns0:f>
@@ -4570,11 +4570,11 @@
       </ns0:c>
       <ns0:c r="D115" s="1">
         <ns0:f>ROUND(D114*20,2-INT(LOG10(ABS(D114*20))))</ns0:f>
-        <ns0:v>5.32e+110</ns0:v>
+        <ns0:v>4.8e+111</ns0:v>
       </ns0:c>
       <ns0:c r="E115" s="1">
         <ns0:f>D115</ns0:f>
-        <ns0:v>5.32e+110</ns0:v>
+        <ns0:v>4.8e+111</ns0:v>
       </ns0:c>
       <ns0:c r="F115" s="1">
         <ns0:f>ROUND(F114*1.4,-5)</ns0:f>
@@ -4602,11 +4602,11 @@
       </ns0:c>
       <ns0:c r="D116" s="1">
         <ns0:f>ROUND(D115*20,2-INT(LOG10(ABS(D115*20))))</ns0:f>
-        <ns0:v>1.06e+112</ns0:v>
+        <ns0:v>9.6e+112</ns0:v>
       </ns0:c>
       <ns0:c r="E116" s="1">
         <ns0:f>D116</ns0:f>
-        <ns0:v>1.06e+112</ns0:v>
+        <ns0:v>9.6e+112</ns0:v>
       </ns0:c>
       <ns0:c r="F116" s="1">
         <ns0:f>ROUND(F115*1.4,-5)</ns0:f>
@@ -4634,11 +4634,11 @@
       </ns0:c>
       <ns0:c r="D117" s="1">
         <ns0:f>ROUND(D116*20,2-INT(LOG10(ABS(D116*20))))</ns0:f>
-        <ns0:v>2.1199999999999997e+113</ns0:v>
+        <ns0:v>1.9200000000000001e+114</ns0:v>
       </ns0:c>
       <ns0:c r="E117" s="1">
         <ns0:f>D117</ns0:f>
-        <ns0:v>2.1199999999999997e+113</ns0:v>
+        <ns0:v>1.9200000000000001e+114</ns0:v>
       </ns0:c>
       <ns0:c r="F117" s="1">
         <ns0:f>ROUND(F116*1.4,-5)</ns0:f>
@@ -4666,11 +4666,11 @@
       </ns0:c>
       <ns0:c r="D118" s="1">
         <ns0:f>ROUND(D117*20,2-INT(LOG10(ABS(D117*20))))</ns0:f>
-        <ns0:v>4.2400000000000003e+114</ns0:v>
+        <ns0:v>3.84e+115</ns0:v>
       </ns0:c>
       <ns0:c r="E118" s="1">
         <ns0:f>D118</ns0:f>
-        <ns0:v>4.2400000000000003e+114</ns0:v>
+        <ns0:v>3.84e+115</ns0:v>
       </ns0:c>
       <ns0:c r="F118" s="1">
         <ns0:f>ROUND(F117*1.4,-5)</ns0:f>
@@ -4698,11 +4698,11 @@
       </ns0:c>
       <ns0:c r="D119" s="1">
         <ns0:f>ROUND(D118*20,2-INT(LOG10(ABS(D118*20))))</ns0:f>
-        <ns0:v>8.48e+115</ns0:v>
+        <ns0:v>7.68e+116</ns0:v>
       </ns0:c>
       <ns0:c r="E119" s="1">
         <ns0:f>D119</ns0:f>
-        <ns0:v>8.48e+115</ns0:v>
+        <ns0:v>7.68e+116</ns0:v>
       </ns0:c>
       <ns0:c r="F119" s="1">
         <ns0:f>ROUND(F118*1.4,-5)</ns0:f>
@@ -4730,11 +4730,11 @@
       </ns0:c>
       <ns0:c r="D120" s="1">
         <ns0:f>ROUND(D119*20,2-INT(LOG10(ABS(D119*20))))</ns0:f>
-        <ns0:v>1.7e+117</ns0:v>
+        <ns0:v>1.54e+118</ns0:v>
       </ns0:c>
       <ns0:c r="E120" s="1">
         <ns0:f>D120</ns0:f>
-        <ns0:v>1.7e+117</ns0:v>
+        <ns0:v>1.54e+118</ns0:v>
       </ns0:c>
       <ns0:c r="F120" s="1">
         <ns0:f>ROUND(F119*1.4,-5)</ns0:f>
@@ -4762,11 +4762,11 @@
       </ns0:c>
       <ns0:c r="D121" s="1">
         <ns0:f>ROUND(D120*20,2-INT(LOG10(ABS(D120*20))))</ns0:f>
-        <ns0:v>3.4e+118</ns0:v>
+        <ns0:v>3.08e+119</ns0:v>
       </ns0:c>
       <ns0:c r="E121" s="1">
         <ns0:f>D121</ns0:f>
-        <ns0:v>3.4e+118</ns0:v>
+        <ns0:v>3.08e+119</ns0:v>
       </ns0:c>
       <ns0:c r="F121" s="1">
         <ns0:f>ROUND(F120*1.4,-5)</ns0:f>
@@ -4794,11 +4794,11 @@
       </ns0:c>
       <ns0:c r="D122" s="1">
         <ns0:f>ROUND(D121*20,2-INT(LOG10(ABS(D121*20))))</ns0:f>
-        <ns0:v>6.8e+119</ns0:v>
+        <ns0:v>6.16e+120</ns0:v>
       </ns0:c>
       <ns0:c r="E122" s="1">
         <ns0:f>D122</ns0:f>
-        <ns0:v>6.8e+119</ns0:v>
+        <ns0:v>6.16e+120</ns0:v>
       </ns0:c>
       <ns0:c r="F122" s="1">
         <ns0:f>ROUND(F121*1.4,-5)</ns0:f>
@@ -4826,11 +4826,11 @@
       </ns0:c>
       <ns0:c r="D123" s="1">
         <ns0:f>ROUND(D122*20,2-INT(LOG10(ABS(D122*20))))</ns0:f>
-        <ns0:v>1.36e+121</ns0:v>
+        <ns0:v>1.2300000000000001e+122</ns0:v>
       </ns0:c>
       <ns0:c r="E123" s="1">
         <ns0:f>D123</ns0:f>
-        <ns0:v>1.36e+121</ns0:v>
+        <ns0:v>1.2300000000000001e+122</ns0:v>
       </ns0:c>
       <ns0:c r="F123" s="1">
         <ns0:f>ROUND(F122*1.4,-5)</ns0:f>
@@ -4858,11 +4858,11 @@
       </ns0:c>
       <ns0:c r="D124" s="1">
         <ns0:f>ROUND(D123*20,2-INT(LOG10(ABS(D123*20))))</ns0:f>
-        <ns0:v>2.72e+122</ns0:v>
+        <ns0:v>2.46e+123</ns0:v>
       </ns0:c>
       <ns0:c r="E124" s="1">
         <ns0:f>D124</ns0:f>
-        <ns0:v>2.72e+122</ns0:v>
+        <ns0:v>2.46e+123</ns0:v>
       </ns0:c>
       <ns0:c r="F124" s="1">
         <ns0:f>ROUND(F123*1.4,-5)</ns0:f>
@@ -4890,11 +4890,11 @@
       </ns0:c>
       <ns0:c r="D125" s="1">
         <ns0:f>ROUND(D124*20,2-INT(LOG10(ABS(D124*20))))</ns0:f>
-        <ns0:v>5.44e+123</ns0:v>
+        <ns0:v>4.92e+124</ns0:v>
       </ns0:c>
       <ns0:c r="E125" s="1">
         <ns0:f>D125</ns0:f>
-        <ns0:v>5.44e+123</ns0:v>
+        <ns0:v>4.92e+124</ns0:v>
       </ns0:c>
       <ns0:c r="F125" s="1">
         <ns0:f>ROUND(F124*1.4,-5)</ns0:f>
@@ -4922,11 +4922,11 @@
       </ns0:c>
       <ns0:c r="D126" s="1">
         <ns0:f>ROUND(D125*20,2-INT(LOG10(ABS(D125*20))))</ns0:f>
-        <ns0:v>1.09e+125</ns0:v>
+        <ns0:v>9.839999999999999e+125</ns0:v>
       </ns0:c>
       <ns0:c r="E126" s="1">
         <ns0:f>D126</ns0:f>
-        <ns0:v>1.09e+125</ns0:v>
+        <ns0:v>9.839999999999999e+125</ns0:v>
       </ns0:c>
       <ns0:c r="F126" s="1">
         <ns0:f>ROUND(F125*1.4,-5)</ns0:f>
@@ -4954,11 +4954,11 @@
       </ns0:c>
       <ns0:c r="D127" s="1">
         <ns0:f>ROUND(D126*20,2-INT(LOG10(ABS(D126*20))))</ns0:f>
-        <ns0:v>2.18e+126</ns0:v>
+        <ns0:v>1.9699999999999999e+127</ns0:v>
       </ns0:c>
       <ns0:c r="E127" s="1">
         <ns0:f>D127</ns0:f>
-        <ns0:v>2.18e+126</ns0:v>
+        <ns0:v>1.9699999999999999e+127</ns0:v>
       </ns0:c>
       <ns0:c r="F127" s="1">
         <ns0:f>ROUND(F126*1.4,-5)</ns0:f>
@@ -4986,11 +4986,11 @@
       </ns0:c>
       <ns0:c r="D128" s="1">
         <ns0:f>ROUND(D127*20,2-INT(LOG10(ABS(D127*20))))</ns0:f>
-        <ns0:v>4.36e+127</ns0:v>
+        <ns0:v>3.94e+128</ns0:v>
       </ns0:c>
       <ns0:c r="E128" s="1">
         <ns0:f>D128</ns0:f>
-        <ns0:v>4.36e+127</ns0:v>
+        <ns0:v>3.94e+128</ns0:v>
       </ns0:c>
       <ns0:c r="F128" s="1">
         <ns0:f>ROUND(F127*1.4,-5)</ns0:f>
@@ -5018,11 +5018,11 @@
       </ns0:c>
       <ns0:c r="D129" s="1">
         <ns0:f>ROUND(D128*20,2-INT(LOG10(ABS(D128*20))))</ns0:f>
-        <ns0:v>8.72e+128</ns0:v>
+        <ns0:v>7.88e+129</ns0:v>
       </ns0:c>
       <ns0:c r="E129" s="1">
         <ns0:f>D129</ns0:f>
-        <ns0:v>8.72e+128</ns0:v>
+        <ns0:v>7.88e+129</ns0:v>
       </ns0:c>
       <ns0:c r="F129" s="1">
         <ns0:f>ROUND(F128*1.4,-5)</ns0:f>
@@ -5050,11 +5050,11 @@
       </ns0:c>
       <ns0:c r="D130" s="1">
         <ns0:f>ROUND(D129*20,2-INT(LOG10(ABS(D129*20))))</ns0:f>
-        <ns0:v>1.74e+130</ns0:v>
+        <ns0:v>1.58e+131</ns0:v>
       </ns0:c>
       <ns0:c r="E130" s="1">
         <ns0:f>D130</ns0:f>
-        <ns0:v>1.74e+130</ns0:v>
+        <ns0:v>1.58e+131</ns0:v>
       </ns0:c>
       <ns0:c r="F130" s="1">
         <ns0:f>ROUND(F129*1.4,-5)</ns0:f>
@@ -5082,11 +5082,11 @@
       </ns0:c>
       <ns0:c r="D131" s="1">
         <ns0:f>ROUND(D130*20,2-INT(LOG10(ABS(D130*20))))</ns0:f>
-        <ns0:v>3.4800000000000003e+131</ns0:v>
+        <ns0:v>3.16e+132</ns0:v>
       </ns0:c>
       <ns0:c r="E131" s="1">
         <ns0:f>D131</ns0:f>
-        <ns0:v>3.4800000000000003e+131</ns0:v>
+        <ns0:v>3.16e+132</ns0:v>
       </ns0:c>
       <ns0:c r="F131" s="1">
         <ns0:f>ROUND(F130*1.4,-5)</ns0:f>
@@ -5114,11 +5114,11 @@
       </ns0:c>
       <ns0:c r="D132" s="1">
         <ns0:f>ROUND(D131*20,2-INT(LOG10(ABS(D131*20))))</ns0:f>
-        <ns0:v>6.96e+132</ns0:v>
+        <ns0:v>6.32e+133</ns0:v>
       </ns0:c>
       <ns0:c r="E132" s="1">
         <ns0:f>D132</ns0:f>
-        <ns0:v>6.96e+132</ns0:v>
+        <ns0:v>6.32e+133</ns0:v>
       </ns0:c>
       <ns0:c r="F132" s="1">
         <ns0:f>ROUND(F131*1.4,-5)</ns0:f>
@@ -5146,11 +5146,11 @@
       </ns0:c>
       <ns0:c r="D133" s="1">
         <ns0:f>ROUND(D132*20,2-INT(LOG10(ABS(D132*20))))</ns0:f>
-        <ns0:v>1.39e+134</ns0:v>
+        <ns0:v>1.2599999999999999e+135</ns0:v>
       </ns0:c>
       <ns0:c r="E133" s="1">
         <ns0:f>D133</ns0:f>
-        <ns0:v>1.39e+134</ns0:v>
+        <ns0:v>1.2599999999999999e+135</ns0:v>
       </ns0:c>
       <ns0:c r="F133" s="1">
         <ns0:f>ROUND(F132*1.4,-5)</ns0:f>
@@ -5178,11 +5178,11 @@
       </ns0:c>
       <ns0:c r="D134" s="1">
         <ns0:f>ROUND(D133*20,2-INT(LOG10(ABS(D133*20))))</ns0:f>
-        <ns0:v>2.7799999999999997e+135</ns0:v>
+        <ns0:v>2.52e+136</ns0:v>
       </ns0:c>
       <ns0:c r="E134" s="1">
         <ns0:f>D134</ns0:f>
-        <ns0:v>2.7799999999999997e+135</ns0:v>
+        <ns0:v>2.52e+136</ns0:v>
       </ns0:c>
       <ns0:c r="F134" s="1">
         <ns0:f>ROUND(F133*1.4,-5)</ns0:f>
@@ -5210,11 +5210,11 @@
       </ns0:c>
       <ns0:c r="D135" s="1">
         <ns0:f>ROUND(D134*20,2-INT(LOG10(ABS(D134*20))))</ns0:f>
-        <ns0:v>5.56e+136</ns0:v>
+        <ns0:v>5.04e+137</ns0:v>
       </ns0:c>
       <ns0:c r="E135" s="1">
         <ns0:f>D135</ns0:f>
-        <ns0:v>5.56e+136</ns0:v>
+        <ns0:v>5.04e+137</ns0:v>
       </ns0:c>
       <ns0:c r="F135" s="1">
         <ns0:f>ROUND(F134*1.4,-5)</ns0:f>
@@ -5242,11 +5242,11 @@
       </ns0:c>
       <ns0:c r="D136" s="1">
         <ns0:f>ROUND(D135*20,2-INT(LOG10(ABS(D135*20))))</ns0:f>
-        <ns0:v>1.11e+138</ns0:v>
+        <ns0:v>1.0100000000000001e+139</ns0:v>
       </ns0:c>
       <ns0:c r="E136" s="1">
         <ns0:f>D136</ns0:f>
-        <ns0:v>1.11e+138</ns0:v>
+        <ns0:v>1.0100000000000001e+139</ns0:v>
       </ns0:c>
       <ns0:c r="F136" s="1">
         <ns0:f>ROUND(F135*1.4,-5)</ns0:f>
@@ -5274,11 +5274,11 @@
       </ns0:c>
       <ns0:c r="D137" s="1">
         <ns0:f>ROUND(D136*20,2-INT(LOG10(ABS(D136*20))))</ns0:f>
-        <ns0:v>2.22e+139</ns0:v>
+        <ns0:v>2.0199999999999997e+140</ns0:v>
       </ns0:c>
       <ns0:c r="E137" s="1">
         <ns0:f>D137</ns0:f>
-        <ns0:v>2.22e+139</ns0:v>
+        <ns0:v>2.0199999999999997e+140</ns0:v>
       </ns0:c>
       <ns0:c r="F137" s="1">
         <ns0:f>ROUND(F136*1.4,-5)</ns0:f>
@@ -5306,11 +5306,11 @@
       </ns0:c>
       <ns0:c r="D138" s="1">
         <ns0:f>ROUND(D137*20,2-INT(LOG10(ABS(D137*20))))</ns0:f>
-        <ns0:v>4.44e+140</ns0:v>
+        <ns0:v>4.0399999999999996e+141</ns0:v>
       </ns0:c>
       <ns0:c r="E138" s="1">
         <ns0:f>D138</ns0:f>
-        <ns0:v>4.44e+140</ns0:v>
+        <ns0:v>4.0399999999999996e+141</ns0:v>
       </ns0:c>
       <ns0:c r="F138" s="1">
         <ns0:f>ROUND(F137*1.4,-5)</ns0:f>
@@ -5338,11 +5338,11 @@
       </ns0:c>
       <ns0:c r="D139" s="1">
         <ns0:f>ROUND(D138*20,2-INT(LOG10(ABS(D138*20))))</ns0:f>
-        <ns0:v>8.88e+141</ns0:v>
+        <ns0:v>8.08e+142</ns0:v>
       </ns0:c>
       <ns0:c r="E139" s="1">
         <ns0:f>D139</ns0:f>
-        <ns0:v>8.88e+141</ns0:v>
+        <ns0:v>8.08e+142</ns0:v>
       </ns0:c>
       <ns0:c r="F139" s="1">
         <ns0:f>ROUND(F138*1.4,-5)</ns0:f>
@@ -5370,11 +5370,11 @@
       </ns0:c>
       <ns0:c r="D140" s="1">
         <ns0:f>ROUND(D139*20,2-INT(LOG10(ABS(D139*20))))</ns0:f>
-        <ns0:v>1.78e+143</ns0:v>
+        <ns0:v>1.62e+144</ns0:v>
       </ns0:c>
       <ns0:c r="E140" s="1">
         <ns0:f>D140</ns0:f>
-        <ns0:v>1.78e+143</ns0:v>
+        <ns0:v>1.62e+144</ns0:v>
       </ns0:c>
       <ns0:c r="F140" s="1">
         <ns0:f>ROUND(F139*1.4,-5)</ns0:f>
@@ -5402,11 +5402,11 @@
       </ns0:c>
       <ns0:c r="D141" s="1">
         <ns0:f>ROUND(D140*20,2-INT(LOG10(ABS(D140*20))))</ns0:f>
-        <ns0:v>3.5599999999999996e+144</ns0:v>
+        <ns0:v>3.24e+145</ns0:v>
       </ns0:c>
       <ns0:c r="E141" s="1">
         <ns0:f>D141</ns0:f>
-        <ns0:v>3.5599999999999996e+144</ns0:v>
+        <ns0:v>3.24e+145</ns0:v>
       </ns0:c>
       <ns0:c r="F141" s="1">
         <ns0:f>ROUND(F140*1.4,-5)</ns0:f>
@@ -5434,11 +5434,11 @@
       </ns0:c>
       <ns0:c r="D142" s="1">
         <ns0:f>ROUND(D141*20,2-INT(LOG10(ABS(D141*20))))</ns0:f>
-        <ns0:v>7.120000000000001e+145</ns0:v>
+        <ns0:v>6.48e+146</ns0:v>
       </ns0:c>
       <ns0:c r="E142" s="1">
         <ns0:f>D142</ns0:f>
-        <ns0:v>7.120000000000001e+145</ns0:v>
+        <ns0:v>6.48e+146</ns0:v>
       </ns0:c>
       <ns0:c r="F142" s="1">
         <ns0:f>ROUND(F141*1.4,-5)</ns0:f>
@@ -5466,11 +5466,11 @@
       </ns0:c>
       <ns0:c r="D143" s="1">
         <ns0:f>ROUND(D142*20,2-INT(LOG10(ABS(D142*20))))</ns0:f>
-        <ns0:v>1.4200000000000002e+147</ns0:v>
+        <ns0:v>1.3e+148</ns0:v>
       </ns0:c>
       <ns0:c r="E143" s="1">
         <ns0:f>D143</ns0:f>
-        <ns0:v>1.4200000000000002e+147</ns0:v>
+        <ns0:v>1.3e+148</ns0:v>
       </ns0:c>
       <ns0:c r="F143" s="1">
         <ns0:f>ROUND(F142*1.4,-5)</ns0:f>
@@ -5498,11 +5498,11 @@
       </ns0:c>
       <ns0:c r="D144" s="1">
         <ns0:f>ROUND(D143*20,2-INT(LOG10(ABS(D143*20))))</ns0:f>
-        <ns0:v>2.84e+148</ns0:v>
+        <ns0:v>2.6000000000000002e+149</ns0:v>
       </ns0:c>
       <ns0:c r="E144" s="1">
         <ns0:f>D144</ns0:f>
-        <ns0:v>2.84e+148</ns0:v>
+        <ns0:v>2.6000000000000002e+149</ns0:v>
       </ns0:c>
       <ns0:c r="F144" s="1">
         <ns0:f>ROUND(F143*1.4,-5)</ns0:f>
@@ -5530,11 +5530,11 @@
       </ns0:c>
       <ns0:c r="D145" s="1">
         <ns0:f>ROUND(D144*20,2-INT(LOG10(ABS(D144*20))))</ns0:f>
-        <ns0:v>5.68e+149</ns0:v>
+        <ns0:v>5.2e+150</ns0:v>
       </ns0:c>
       <ns0:c r="E145" s="1">
         <ns0:f>D145</ns0:f>
-        <ns0:v>5.68e+149</ns0:v>
+        <ns0:v>5.2e+150</ns0:v>
       </ns0:c>
       <ns0:c r="F145" s="1">
         <ns0:f>ROUND(F144*1.4,-5)</ns0:f>
@@ -5562,11 +5562,11 @@
       </ns0:c>
       <ns0:c r="D146" s="1">
         <ns0:f>ROUND(D145*20,2-INT(LOG10(ABS(D145*20))))</ns0:f>
-        <ns0:v>1.14e+151</ns0:v>
+        <ns0:v>1.0399999999999999e+152</ns0:v>
       </ns0:c>
       <ns0:c r="E146" s="1">
         <ns0:f>D146</ns0:f>
-        <ns0:v>1.14e+151</ns0:v>
+        <ns0:v>1.0399999999999999e+152</ns0:v>
       </ns0:c>
       <ns0:c r="F146" s="1">
         <ns0:f>ROUND(F145*1.4,-5)</ns0:f>
@@ -5594,11 +5594,11 @@
       </ns0:c>
       <ns0:c r="D147" s="1">
         <ns0:f>ROUND(D146*20,2-INT(LOG10(ABS(D146*20))))</ns0:f>
-        <ns0:v>2.28e+152</ns0:v>
+        <ns0:v>2.08e+153</ns0:v>
       </ns0:c>
       <ns0:c r="E147" s="1">
         <ns0:f>D147</ns0:f>
-        <ns0:v>2.28e+152</ns0:v>
+        <ns0:v>2.08e+153</ns0:v>
       </ns0:c>
       <ns0:c r="F147" s="1">
         <ns0:f>ROUND(F146*1.4,-5)</ns0:f>
@@ -5626,11 +5626,11 @@
       </ns0:c>
       <ns0:c r="D148" s="1">
         <ns0:f>ROUND(D147*20,2-INT(LOG10(ABS(D147*20))))</ns0:f>
-        <ns0:v>4.56e+153</ns0:v>
+        <ns0:v>4.16e+154</ns0:v>
       </ns0:c>
       <ns0:c r="E148" s="1">
         <ns0:f>D148</ns0:f>
-        <ns0:v>4.56e+153</ns0:v>
+        <ns0:v>4.16e+154</ns0:v>
       </ns0:c>
       <ns0:c r="F148" s="1">
         <ns0:f>ROUND(F147*1.4,-5)</ns0:f>
@@ -5658,11 +5658,11 @@
       </ns0:c>
       <ns0:c r="D149" s="1">
         <ns0:f>ROUND(D148*20,2-INT(LOG10(ABS(D148*20))))</ns0:f>
-        <ns0:v>9.12e+154</ns0:v>
+        <ns0:v>8.32e+155</ns0:v>
       </ns0:c>
       <ns0:c r="E149" s="1">
         <ns0:f>D149</ns0:f>
-        <ns0:v>9.12e+154</ns0:v>
+        <ns0:v>8.32e+155</ns0:v>
       </ns0:c>
       <ns0:c r="F149" s="1">
         <ns0:f>ROUND(F148*1.4,-5)</ns0:f>
@@ -5690,11 +5690,11 @@
       </ns0:c>
       <ns0:c r="D150" s="1">
         <ns0:f>ROUND(D149*20,2-INT(LOG10(ABS(D149*20))))</ns0:f>
-        <ns0:v>1.82e+156</ns0:v>
+        <ns0:v>1.66e+157</ns0:v>
       </ns0:c>
       <ns0:c r="E150" s="1">
         <ns0:f>D150</ns0:f>
-        <ns0:v>1.82e+156</ns0:v>
+        <ns0:v>1.66e+157</ns0:v>
       </ns0:c>
       <ns0:c r="F150" s="1">
         <ns0:f>ROUND(F149*1.4,-5)</ns0:f>
@@ -5722,11 +5722,11 @@
       </ns0:c>
       <ns0:c r="D151" s="1">
         <ns0:f>ROUND(D150*20,2-INT(LOG10(ABS(D150*20))))</ns0:f>
-        <ns0:v>3.64e+157</ns0:v>
+        <ns0:v>3.3199999999999997e+158</ns0:v>
       </ns0:c>
       <ns0:c r="E151" s="1">
         <ns0:f>D151</ns0:f>
-        <ns0:v>3.64e+157</ns0:v>
+        <ns0:v>3.3199999999999997e+158</ns0:v>
       </ns0:c>
       <ns0:c r="F151" s="1">
         <ns0:f>ROUND(F150*1.4,-5)</ns0:f>
@@ -5754,11 +5754,11 @@
       </ns0:c>
       <ns0:c r="D152" s="1">
         <ns0:f>ROUND(D151*20,2-INT(LOG10(ABS(D151*20))))</ns0:f>
-        <ns0:v>7.28e+158</ns0:v>
+        <ns0:v>6.64e+159</ns0:v>
       </ns0:c>
       <ns0:c r="E152" s="1">
         <ns0:f>D152</ns0:f>
-        <ns0:v>7.28e+158</ns0:v>
+        <ns0:v>6.64e+159</ns0:v>
       </ns0:c>
       <ns0:c r="F152" s="1">
         <ns0:f>ROUND(F151*1.4,-5)</ns0:f>
@@ -5786,11 +5786,11 @@
       </ns0:c>
       <ns0:c r="D153" s="1">
         <ns0:f>ROUND(D152*20,2-INT(LOG10(ABS(D152*20))))</ns0:f>
-        <ns0:v>1.4599999999999998e+160</ns0:v>
+        <ns0:v>1.3300000000000001e+161</ns0:v>
       </ns0:c>
       <ns0:c r="E153" s="1">
         <ns0:f>D153</ns0:f>
-        <ns0:v>1.4599999999999998e+160</ns0:v>
+        <ns0:v>1.3300000000000001e+161</ns0:v>
       </ns0:c>
       <ns0:c r="F153" s="1">
         <ns0:f>ROUND(F152*1.4,-5)</ns0:f>
@@ -5818,11 +5818,11 @@
       </ns0:c>
       <ns0:c r="D154" s="1">
         <ns0:f>ROUND(D153*20,2-INT(LOG10(ABS(D153*20))))</ns0:f>
-        <ns0:v>2.92e+161</ns0:v>
+        <ns0:v>2.66e+162</ns0:v>
       </ns0:c>
       <ns0:c r="E154" s="1">
         <ns0:f>D154</ns0:f>
-        <ns0:v>2.92e+161</ns0:v>
+        <ns0:v>2.66e+162</ns0:v>
       </ns0:c>
       <ns0:c r="F154" s="1">
         <ns0:f>ROUND(F153*1.4,-5)</ns0:f>
@@ -5850,11 +5850,11 @@
       </ns0:c>
       <ns0:c r="D155" s="1">
         <ns0:f>ROUND(D154*20,2-INT(LOG10(ABS(D154*20))))</ns0:f>
-        <ns0:v>5.84e+162</ns0:v>
+        <ns0:v>5.32e+163</ns0:v>
       </ns0:c>
       <ns0:c r="E155" s="1">
         <ns0:f>D155</ns0:f>
-        <ns0:v>5.84e+162</ns0:v>
+        <ns0:v>5.32e+163</ns0:v>
       </ns0:c>
       <ns0:c r="F155" s="1">
         <ns0:f>ROUND(F154*1.4,-5)</ns0:f>
@@ -5882,11 +5882,11 @@
       </ns0:c>
       <ns0:c r="D156" s="1">
         <ns0:f>ROUND(D155*20,2-INT(LOG10(ABS(D155*20))))</ns0:f>
-        <ns0:v>1.17e+164</ns0:v>
+        <ns0:v>1.06e+165</ns0:v>
       </ns0:c>
       <ns0:c r="E156" s="1">
         <ns0:f>D156</ns0:f>
-        <ns0:v>1.17e+164</ns0:v>
+        <ns0:v>1.06e+165</ns0:v>
       </ns0:c>
       <ns0:c r="F156" s="1">
         <ns0:f>ROUND(F155*1.4,-5)</ns0:f>
@@ -5914,11 +5914,11 @@
       </ns0:c>
       <ns0:c r="D157" s="1">
         <ns0:f>ROUND(D156*20,2-INT(LOG10(ABS(D156*20))))</ns0:f>
-        <ns0:v>2.34e+165</ns0:v>
+        <ns0:v>2.12e+166</ns0:v>
       </ns0:c>
       <ns0:c r="E157" s="1">
         <ns0:f>D157</ns0:f>
-        <ns0:v>2.34e+165</ns0:v>
+        <ns0:v>2.12e+166</ns0:v>
       </ns0:c>
       <ns0:c r="F157" s="1">
         <ns0:f>ROUND(F156*1.4,-5)</ns0:f>
@@ -5946,11 +5946,11 @@
       </ns0:c>
       <ns0:c r="D158" s="1">
         <ns0:f>ROUND(D157*20,2-INT(LOG10(ABS(D157*20))))</ns0:f>
-        <ns0:v>4.68e+166</ns0:v>
+        <ns0:v>4.24e+167</ns0:v>
       </ns0:c>
       <ns0:c r="E158" s="1">
         <ns0:f>D158</ns0:f>
-        <ns0:v>4.68e+166</ns0:v>
+        <ns0:v>4.24e+167</ns0:v>
       </ns0:c>
       <ns0:c r="F158" s="1">
         <ns0:f>ROUND(F157*1.4,-5)</ns0:f>
@@ -5978,11 +5978,11 @@
       </ns0:c>
       <ns0:c r="D159" s="1">
         <ns0:f>ROUND(D158*20,2-INT(LOG10(ABS(D158*20))))</ns0:f>
-        <ns0:v>9.36e+167</ns0:v>
+        <ns0:v>8.48e+168</ns0:v>
       </ns0:c>
       <ns0:c r="E159" s="1">
         <ns0:f>D159</ns0:f>
-        <ns0:v>9.36e+167</ns0:v>
+        <ns0:v>8.48e+168</ns0:v>
       </ns0:c>
       <ns0:c r="F159" s="1">
         <ns0:f>ROUND(F158*1.4,-5)</ns0:f>
@@ -6010,11 +6010,11 @@
       </ns0:c>
       <ns0:c r="D160" s="1">
         <ns0:f>ROUND(D159*20,2-INT(LOG10(ABS(D159*20))))</ns0:f>
-        <ns0:v>1.87e+169</ns0:v>
+        <ns0:v>1.6999999999999998e+170</ns0:v>
       </ns0:c>
       <ns0:c r="E160" s="1">
         <ns0:f>D160</ns0:f>
-        <ns0:v>1.87e+169</ns0:v>
+        <ns0:v>1.6999999999999998e+170</ns0:v>
       </ns0:c>
       <ns0:c r="F160" s="1">
         <ns0:f>ROUND(F159*1.4,-5)</ns0:f>
@@ -6042,11 +6042,11 @@
       </ns0:c>
       <ns0:c r="D161" s="1">
         <ns0:f>ROUND(D160*20,2-INT(LOG10(ABS(D160*20))))</ns0:f>
-        <ns0:v>3.74e+170</ns0:v>
+        <ns0:v>3.4e+171</ns0:v>
       </ns0:c>
       <ns0:c r="E161" s="1">
         <ns0:f>D161</ns0:f>
-        <ns0:v>3.74e+170</ns0:v>
+        <ns0:v>3.4e+171</ns0:v>
       </ns0:c>
       <ns0:c r="F161" s="1">
         <ns0:f>ROUND(F160*1.4,-5)</ns0:f>
@@ -6074,11 +6074,11 @@
       </ns0:c>
       <ns0:c r="D162" s="1">
         <ns0:f>ROUND(D161*20,2-INT(LOG10(ABS(D161*20))))</ns0:f>
-        <ns0:v>7.4799999999999995e+171</ns0:v>
+        <ns0:v>6.8e+172</ns0:v>
       </ns0:c>
       <ns0:c r="E162" s="1">
         <ns0:f>D162</ns0:f>
-        <ns0:v>7.4799999999999995e+171</ns0:v>
+        <ns0:v>6.8e+172</ns0:v>
       </ns0:c>
       <ns0:c r="F162" s="1">
         <ns0:f>ROUND(F161*1.4,-5)</ns0:f>
@@ -6106,11 +6106,11 @@
       </ns0:c>
       <ns0:c r="D163" s="1">
         <ns0:f>ROUND(D162*20,2-INT(LOG10(ABS(D162*20))))</ns0:f>
-        <ns0:v>1.5000000000000002e+173</ns0:v>
+        <ns0:v>1.3599999999999999e+174</ns0:v>
       </ns0:c>
       <ns0:c r="E163" s="1">
         <ns0:f>D163</ns0:f>
-        <ns0:v>1.5000000000000002e+173</ns0:v>
+        <ns0:v>1.3599999999999999e+174</ns0:v>
       </ns0:c>
       <ns0:c r="F163" s="1">
         <ns0:f>ROUND(F162*1.4,-5)</ns0:f>
@@ -6138,11 +6138,11 @@
       </ns0:c>
       <ns0:c r="D164" s="1">
         <ns0:f>ROUND(D163*20,2-INT(LOG10(ABS(D163*20))))</ns0:f>
-        <ns0:v>3e+174</ns0:v>
+        <ns0:v>2.7199999999999997e+175</ns0:v>
       </ns0:c>
       <ns0:c r="E164" s="1">
         <ns0:f>D164</ns0:f>
-        <ns0:v>3e+174</ns0:v>
+        <ns0:v>2.7199999999999997e+175</ns0:v>
       </ns0:c>
       <ns0:c r="F164" s="1">
         <ns0:f>ROUND(F163*1.4,-5)</ns0:f>
@@ -6170,11 +6170,11 @@
       </ns0:c>
       <ns0:c r="D165" s="1">
         <ns0:f>ROUND(D164*20,2-INT(LOG10(ABS(D164*20))))</ns0:f>
-        <ns0:v>5.9999999999999996e+175</ns0:v>
+        <ns0:v>5.44e+176</ns0:v>
       </ns0:c>
       <ns0:c r="E165" s="1">
         <ns0:f>D165</ns0:f>
-        <ns0:v>5.9999999999999996e+175</ns0:v>
+        <ns0:v>5.44e+176</ns0:v>
       </ns0:c>
       <ns0:c r="F165" s="1">
         <ns0:f>ROUND(F164*1.4,-5)</ns0:f>
@@ -6202,11 +6202,11 @@
       </ns0:c>
       <ns0:c r="D166" s="1">
         <ns0:f>ROUND(D165*20,2-INT(LOG10(ABS(D165*20))))</ns0:f>
-        <ns0:v>1.2e+177</ns0:v>
+        <ns0:v>1.09e+178</ns0:v>
       </ns0:c>
       <ns0:c r="E166" s="1">
         <ns0:f>D166</ns0:f>
-        <ns0:v>1.2e+177</ns0:v>
+        <ns0:v>1.09e+178</ns0:v>
       </ns0:c>
       <ns0:c r="F166" s="1">
         <ns0:f>ROUND(F165*1.4,-5)</ns0:f>
@@ -6234,11 +6234,11 @@
       </ns0:c>
       <ns0:c r="D167" s="1">
         <ns0:f>ROUND(D166*20,2-INT(LOG10(ABS(D166*20))))</ns0:f>
-        <ns0:v>2.4e+178</ns0:v>
+        <ns0:v>2.1800000000000002e+179</ns0:v>
       </ns0:c>
       <ns0:c r="E167" s="1">
         <ns0:f>D167</ns0:f>
-        <ns0:v>2.4e+178</ns0:v>
+        <ns0:v>2.1800000000000002e+179</ns0:v>
       </ns0:c>
       <ns0:c r="F167" s="1">
         <ns0:f>ROUND(F166*1.4,-5)</ns0:f>
@@ -6266,11 +6266,11 @@
       </ns0:c>
       <ns0:c r="D168" s="1">
         <ns0:f>ROUND(D167*20,2-INT(LOG10(ABS(D167*20))))</ns0:f>
-        <ns0:v>4.8e+179</ns0:v>
+        <ns0:v>4.36e+180</ns0:v>
       </ns0:c>
       <ns0:c r="E168" s="1">
         <ns0:f>D168</ns0:f>
-        <ns0:v>4.8e+179</ns0:v>
+        <ns0:v>4.36e+180</ns0:v>
       </ns0:c>
       <ns0:c r="F168" s="1">
         <ns0:f>ROUND(F167*1.4,-5)</ns0:f>
@@ -6298,11 +6298,11 @@
       </ns0:c>
       <ns0:c r="D169" s="1">
         <ns0:f>ROUND(D168*20,2-INT(LOG10(ABS(D168*20))))</ns0:f>
-        <ns0:v>9.600000000000001e+180</ns0:v>
+        <ns0:v>8.72e+181</ns0:v>
       </ns0:c>
       <ns0:c r="E169" s="1">
         <ns0:f>D169</ns0:f>
-        <ns0:v>9.600000000000001e+180</ns0:v>
+        <ns0:v>8.72e+181</ns0:v>
       </ns0:c>
       <ns0:c r="F169" s="1">
         <ns0:f>ROUND(F168*1.4,-5)</ns0:f>
@@ -6330,11 +6330,11 @@
       </ns0:c>
       <ns0:c r="D170" s="1">
         <ns0:f>ROUND(D169*20,2-INT(LOG10(ABS(D169*20))))</ns0:f>
-        <ns0:v>1.92e+182</ns0:v>
+        <ns0:v>1.74e+183</ns0:v>
       </ns0:c>
       <ns0:c r="E170" s="1">
         <ns0:f>D170</ns0:f>
-        <ns0:v>1.92e+182</ns0:v>
+        <ns0:v>1.74e+183</ns0:v>
       </ns0:c>
       <ns0:c r="F170" s="1">
         <ns0:f>ROUND(F169*1.4,-5)</ns0:f>
@@ -6362,11 +6362,11 @@
       </ns0:c>
       <ns0:c r="D171" s="1">
         <ns0:f>ROUND(D170*20,2-INT(LOG10(ABS(D170*20))))</ns0:f>
-        <ns0:v>3.8399999999999997e+183</ns0:v>
+        <ns0:v>3.48e+184</ns0:v>
       </ns0:c>
       <ns0:c r="E171" s="1">
         <ns0:f>D171</ns0:f>
-        <ns0:v>3.8399999999999997e+183</ns0:v>
+        <ns0:v>3.48e+184</ns0:v>
       </ns0:c>
       <ns0:c r="F171" s="1">
         <ns0:f>ROUND(F170*1.4,-5)</ns0:f>
@@ -6394,11 +6394,11 @@
       </ns0:c>
       <ns0:c r="D172" s="1">
         <ns0:f>ROUND(D171*20,2-INT(LOG10(ABS(D171*20))))</ns0:f>
-        <ns0:v>7.679999999999999e+184</ns0:v>
+        <ns0:v>6.96e+185</ns0:v>
       </ns0:c>
       <ns0:c r="E172" s="1">
         <ns0:f>D172</ns0:f>
-        <ns0:v>7.679999999999999e+184</ns0:v>
+        <ns0:v>6.96e+185</ns0:v>
       </ns0:c>
       <ns0:c r="F172" s="1">
         <ns0:f>ROUND(F171*1.4,-5)</ns0:f>
@@ -6426,11 +6426,11 @@
       </ns0:c>
       <ns0:c r="D173" s="1">
         <ns0:f>ROUND(D172*20,2-INT(LOG10(ABS(D172*20))))</ns0:f>
-        <ns0:v>1.54e+186</ns0:v>
+        <ns0:v>1.39e+187</ns0:v>
       </ns0:c>
       <ns0:c r="E173" s="1">
         <ns0:f>D173</ns0:f>
-        <ns0:v>1.54e+186</ns0:v>
+        <ns0:v>1.39e+187</ns0:v>
       </ns0:c>
       <ns0:c r="F173" s="1">
         <ns0:f>ROUND(F172*1.4,-5)</ns0:f>
@@ -6458,11 +6458,11 @@
       </ns0:c>
       <ns0:c r="D174" s="1">
         <ns0:f>ROUND(D173*20,2-INT(LOG10(ABS(D173*20))))</ns0:f>
-        <ns0:v>3.08e+187</ns0:v>
+        <ns0:v>2.7800000000000002e+188</ns0:v>
       </ns0:c>
       <ns0:c r="E174" s="1">
         <ns0:f>D174</ns0:f>
-        <ns0:v>3.08e+187</ns0:v>
+        <ns0:v>2.7800000000000002e+188</ns0:v>
       </ns0:c>
       <ns0:c r="F174" s="1">
         <ns0:f>ROUND(F173*1.4,-5)</ns0:f>
@@ -6490,11 +6490,11 @@
       </ns0:c>
       <ns0:c r="D175" s="1">
         <ns0:f>ROUND(D174*20,2-INT(LOG10(ABS(D174*20))))</ns0:f>
-        <ns0:v>6.160000000000001e+188</ns0:v>
+        <ns0:v>5.56e+189</ns0:v>
       </ns0:c>
       <ns0:c r="E175" s="1">
         <ns0:f>D175</ns0:f>
-        <ns0:v>6.160000000000001e+188</ns0:v>
+        <ns0:v>5.56e+189</ns0:v>
       </ns0:c>
       <ns0:c r="F175" s="1">
         <ns0:f>ROUND(F174*1.4,-5)</ns0:f>
@@ -6522,11 +6522,11 @@
       </ns0:c>
       <ns0:c r="D176" s="1">
         <ns0:f>ROUND(D175*20,2-INT(LOG10(ABS(D175*20))))</ns0:f>
-        <ns0:v>1.23e+190</ns0:v>
+        <ns0:v>1.11e+191</ns0:v>
       </ns0:c>
       <ns0:c r="E176" s="1">
         <ns0:f>D176</ns0:f>
-        <ns0:v>1.23e+190</ns0:v>
+        <ns0:v>1.11e+191</ns0:v>
       </ns0:c>
       <ns0:c r="F176" s="1">
         <ns0:f>ROUND(F175*1.4,-5)</ns0:f>
@@ -6554,11 +6554,11 @@
       </ns0:c>
       <ns0:c r="D177" s="1">
         <ns0:f>ROUND(D176*20,2-INT(LOG10(ABS(D176*20))))</ns0:f>
-        <ns0:v>2.4599999999999998e+191</ns0:v>
+        <ns0:v>2.22e+192</ns0:v>
       </ns0:c>
       <ns0:c r="E177" s="1">
         <ns0:f>D177</ns0:f>
-        <ns0:v>2.4599999999999998e+191</ns0:v>
+        <ns0:v>2.22e+192</ns0:v>
       </ns0:c>
       <ns0:c r="F177" s="1">
         <ns0:f>ROUND(F176*1.4,-5)</ns0:f>
@@ -6586,11 +6586,11 @@
       </ns0:c>
       <ns0:c r="D178" s="1">
         <ns0:f>ROUND(D177*20,2-INT(LOG10(ABS(D177*20))))</ns0:f>
-        <ns0:v>4.92e+192</ns0:v>
+        <ns0:v>4.44e+193</ns0:v>
       </ns0:c>
       <ns0:c r="E178" s="1">
         <ns0:f>D178</ns0:f>
-        <ns0:v>4.92e+192</ns0:v>
+        <ns0:v>4.44e+193</ns0:v>
       </ns0:c>
       <ns0:c r="F178" s="1">
         <ns0:f>ROUND(F177*1.4,-5)</ns0:f>
@@ -6618,11 +6618,11 @@
       </ns0:c>
       <ns0:c r="D179" s="1">
         <ns0:f>ROUND(D178*20,2-INT(LOG10(ABS(D178*20))))</ns0:f>
-        <ns0:v>9.84e+193</ns0:v>
+        <ns0:v>8.879999999999999e+194</ns0:v>
       </ns0:c>
       <ns0:c r="E179" s="1">
         <ns0:f>D179</ns0:f>
-        <ns0:v>9.84e+193</ns0:v>
+        <ns0:v>8.879999999999999e+194</ns0:v>
       </ns0:c>
       <ns0:c r="F179" s="1">
         <ns0:f>ROUND(F178*1.4,-5)</ns0:f>
@@ -6650,11 +6650,11 @@
       </ns0:c>
       <ns0:c r="D180" s="1">
         <ns0:f>ROUND(D179*20,2-INT(LOG10(ABS(D179*20))))</ns0:f>
-        <ns0:v>1.9699999999999998e+195</ns0:v>
+        <ns0:v>1.78e+196</ns0:v>
       </ns0:c>
       <ns0:c r="E180" s="1">
         <ns0:f>D180</ns0:f>
-        <ns0:v>1.9699999999999998e+195</ns0:v>
+        <ns0:v>1.78e+196</ns0:v>
       </ns0:c>
       <ns0:c r="F180" s="1">
         <ns0:f>ROUND(F179*1.4,-5)</ns0:f>
@@ -6682,11 +6682,11 @@
       </ns0:c>
       <ns0:c r="D181" s="1">
         <ns0:f>ROUND(D180*20,2-INT(LOG10(ABS(D180*20))))</ns0:f>
-        <ns0:v>3.94e+196</ns0:v>
+        <ns0:v>3.56e+197</ns0:v>
       </ns0:c>
       <ns0:c r="E181" s="1">
         <ns0:f>D181</ns0:f>
-        <ns0:v>3.94e+196</ns0:v>
+        <ns0:v>3.56e+197</ns0:v>
       </ns0:c>
       <ns0:c r="F181" s="1">
         <ns0:f>ROUND(F180*1.4,-5)</ns0:f>
@@ -6714,11 +6714,11 @@
       </ns0:c>
       <ns0:c r="D182" s="1">
         <ns0:f>ROUND(D181*20,2-INT(LOG10(ABS(D181*20))))</ns0:f>
-        <ns0:v>7.88e+197</ns0:v>
+        <ns0:v>7.12e+198</ns0:v>
       </ns0:c>
       <ns0:c r="E182" s="1">
         <ns0:f>D182</ns0:f>
-        <ns0:v>7.88e+197</ns0:v>
+        <ns0:v>7.12e+198</ns0:v>
       </ns0:c>
       <ns0:c r="F182" s="1">
         <ns0:f>ROUND(F181*1.4,-5)</ns0:f>
@@ -6746,11 +6746,11 @@
       </ns0:c>
       <ns0:c r="D183" s="1">
         <ns0:f>ROUND(D182*20,2-INT(LOG10(ABS(D182*20))))</ns0:f>
-        <ns0:v>1.5800000000000001e+199</ns0:v>
+        <ns0:v>1.4200000000000001e+200</ns0:v>
       </ns0:c>
       <ns0:c r="E183" s="1">
         <ns0:f>D183</ns0:f>
-        <ns0:v>1.5800000000000001e+199</ns0:v>
+        <ns0:v>1.4200000000000001e+200</ns0:v>
       </ns0:c>
       <ns0:c r="F183" s="1">
         <ns0:f>ROUND(F182*1.4,-5)</ns0:f>
@@ -6778,11 +6778,11 @@
       </ns0:c>
       <ns0:c r="D184" s="1">
         <ns0:f>ROUND(D183*20,2-INT(LOG10(ABS(D183*20))))</ns0:f>
-        <ns0:v>3.1600000000000006e+200</ns0:v>
+        <ns0:v>2.84e+201</ns0:v>
       </ns0:c>
       <ns0:c r="E184" s="1">
         <ns0:f>D184</ns0:f>
-        <ns0:v>3.1600000000000006e+200</ns0:v>
+        <ns0:v>2.84e+201</ns0:v>
       </ns0:c>
       <ns0:c r="F184" s="1">
         <ns0:f>ROUND(F183*1.4,-5)</ns0:f>
@@ -6810,11 +6810,11 @@
       </ns0:c>
       <ns0:c r="D185" s="1">
         <ns0:f>ROUND(D184*20,2-INT(LOG10(ABS(D184*20))))</ns0:f>
-        <ns0:v>6.320000000000001e+201</ns0:v>
+        <ns0:v>5.68e+202</ns0:v>
       </ns0:c>
       <ns0:c r="E185" s="1">
         <ns0:f>D185</ns0:f>
-        <ns0:v>6.320000000000001e+201</ns0:v>
+        <ns0:v>5.68e+202</ns0:v>
       </ns0:c>
       <ns0:c r="F185" s="1">
         <ns0:f>ROUND(F184*1.4,-5)</ns0:f>
@@ -6842,11 +6842,11 @@
       </ns0:c>
       <ns0:c r="D186" s="1">
         <ns0:f>ROUND(D185*20,2-INT(LOG10(ABS(D185*20))))</ns0:f>
-        <ns0:v>1.26e+203</ns0:v>
+        <ns0:v>1.14e+204</ns0:v>
       </ns0:c>
       <ns0:c r="E186" s="1">
         <ns0:f>D186</ns0:f>
-        <ns0:v>1.26e+203</ns0:v>
+        <ns0:v>1.14e+204</ns0:v>
       </ns0:c>
       <ns0:c r="F186" s="1">
         <ns0:f>ROUND(F185*1.4,-5)</ns0:f>
@@ -6874,11 +6874,11 @@
       </ns0:c>
       <ns0:c r="D187" s="1">
         <ns0:f>ROUND(D186*20,2-INT(LOG10(ABS(D186*20))))</ns0:f>
-        <ns0:v>2.52e+204</ns0:v>
+        <ns0:v>2.28e+205</ns0:v>
       </ns0:c>
       <ns0:c r="E187" s="1">
         <ns0:f>D187</ns0:f>
-        <ns0:v>2.52e+204</ns0:v>
+        <ns0:v>2.28e+205</ns0:v>
       </ns0:c>
       <ns0:c r="F187" s="1">
         <ns0:f>ROUND(F186*1.4,-5)</ns0:f>
@@ -6906,11 +6906,11 @@
       </ns0:c>
       <ns0:c r="D188" s="1">
         <ns0:f>ROUND(D187*20,2-INT(LOG10(ABS(D187*20))))</ns0:f>
-        <ns0:v>5.04e+205</ns0:v>
+        <ns0:v>4.56e+206</ns0:v>
       </ns0:c>
       <ns0:c r="E188" s="1">
         <ns0:f>D188</ns0:f>
-        <ns0:v>5.04e+205</ns0:v>
+        <ns0:v>4.56e+206</ns0:v>
       </ns0:c>
       <ns0:c r="F188" s="1">
         <ns0:f>ROUND(F187*1.4,-5)</ns0:f>
@@ -6938,11 +6938,11 @@
       </ns0:c>
       <ns0:c r="D189" s="1">
         <ns0:f>ROUND(D188*20,2-INT(LOG10(ABS(D188*20))))</ns0:f>
-        <ns0:v>1.01e+207</ns0:v>
+        <ns0:v>9.12e+207</ns0:v>
       </ns0:c>
       <ns0:c r="E189" s="1">
         <ns0:f>D189</ns0:f>
-        <ns0:v>1.01e+207</ns0:v>
+        <ns0:v>9.12e+207</ns0:v>
       </ns0:c>
       <ns0:c r="F189" s="1">
         <ns0:f>ROUND(F188*1.4,-5)</ns0:f>
@@ -6970,11 +6970,11 @@
       </ns0:c>
       <ns0:c r="D190" s="1">
         <ns0:f>ROUND(D189*20,2-INT(LOG10(ABS(D189*20))))</ns0:f>
-        <ns0:v>2.02e+208</ns0:v>
+        <ns0:v>1.82e+209</ns0:v>
       </ns0:c>
       <ns0:c r="E190" s="1">
         <ns0:f>D190</ns0:f>
-        <ns0:v>2.02e+208</ns0:v>
+        <ns0:v>1.82e+209</ns0:v>
       </ns0:c>
       <ns0:c r="F190" s="1">
         <ns0:f>ROUND(F189*1.4,-5)</ns0:f>
@@ -7002,11 +7002,11 @@
       </ns0:c>
       <ns0:c r="D191" s="1">
         <ns0:f>ROUND(D190*20,2-INT(LOG10(ABS(D190*20))))</ns0:f>
-        <ns0:v>4.04e+209</ns0:v>
+        <ns0:v>3.64e+210</ns0:v>
       </ns0:c>
       <ns0:c r="E191" s="1">
         <ns0:f>D191</ns0:f>
-        <ns0:v>4.04e+209</ns0:v>
+        <ns0:v>3.64e+210</ns0:v>
       </ns0:c>
       <ns0:c r="F191" s="1">
         <ns0:f>ROUND(F190*1.4,-5)</ns0:f>
@@ -7034,11 +7034,11 @@
       </ns0:c>
       <ns0:c r="D192" s="1">
         <ns0:f>ROUND(D191*20,2-INT(LOG10(ABS(D191*20))))</ns0:f>
-        <ns0:v>8.079999999999999e+210</ns0:v>
+        <ns0:v>7.279999999999999e+211</ns0:v>
       </ns0:c>
       <ns0:c r="E192" s="1">
         <ns0:f>D192</ns0:f>
-        <ns0:v>8.079999999999999e+210</ns0:v>
+        <ns0:v>7.279999999999999e+211</ns0:v>
       </ns0:c>
       <ns0:c r="F192" s="1">
         <ns0:f>ROUND(F191*1.4,-5)</ns0:f>
@@ -7066,11 +7066,11 @@
       </ns0:c>
       <ns0:c r="D193" s="1">
         <ns0:f>ROUND(D192*20,2-INT(LOG10(ABS(D192*20))))</ns0:f>
-        <ns0:v>1.62e+212</ns0:v>
+        <ns0:v>1.46e+213</ns0:v>
       </ns0:c>
       <ns0:c r="E193" s="1">
         <ns0:f>D193</ns0:f>
-        <ns0:v>1.62e+212</ns0:v>
+        <ns0:v>1.46e+213</ns0:v>
       </ns0:c>
       <ns0:c r="F193" s="1">
         <ns0:f>ROUND(F192*1.4,-5)</ns0:f>
@@ -7098,11 +7098,11 @@
       </ns0:c>
       <ns0:c r="D194" s="1">
         <ns0:f>ROUND(D193*20,2-INT(LOG10(ABS(D193*20))))</ns0:f>
-        <ns0:v>3.2399999999999995e+213</ns0:v>
+        <ns0:v>2.9200000000000003e+214</ns0:v>
       </ns0:c>
       <ns0:c r="E194" s="1">
         <ns0:f>D194</ns0:f>
-        <ns0:v>3.2399999999999995e+213</ns0:v>
+        <ns0:v>2.9200000000000003e+214</ns0:v>
       </ns0:c>
       <ns0:c r="F194" s="1">
         <ns0:f>ROUND(F193*1.4,-5)</ns0:f>
@@ -7130,11 +7130,11 @@
       </ns0:c>
       <ns0:c r="D195" s="1">
         <ns0:f>ROUND(D194*20,2-INT(LOG10(ABS(D194*20))))</ns0:f>
-        <ns0:v>6.48e+214</ns0:v>
+        <ns0:v>5.84e+215</ns0:v>
       </ns0:c>
       <ns0:c r="E195" s="1">
         <ns0:f>D195</ns0:f>
-        <ns0:v>6.48e+214</ns0:v>
+        <ns0:v>5.84e+215</ns0:v>
       </ns0:c>
       <ns0:c r="F195" s="1">
         <ns0:f>ROUND(F194*1.4,-5)</ns0:f>
@@ -7162,11 +7162,11 @@
       </ns0:c>
       <ns0:c r="D196" s="1">
         <ns0:f>ROUND(D195*20,2-INT(LOG10(ABS(D195*20))))</ns0:f>
-        <ns0:v>1.3000000000000001e+216</ns0:v>
+        <ns0:v>1.17e+217</ns0:v>
       </ns0:c>
       <ns0:c r="E196" s="1">
         <ns0:f>D196</ns0:f>
-        <ns0:v>1.3000000000000001e+216</ns0:v>
+        <ns0:v>1.17e+217</ns0:v>
       </ns0:c>
       <ns0:c r="F196" s="1">
         <ns0:f>ROUND(F195*1.4,-5)</ns0:f>
@@ -7194,11 +7194,11 @@
       </ns0:c>
       <ns0:c r="D197" s="1">
         <ns0:f>ROUND(D196*20,2-INT(LOG10(ABS(D196*20))))</ns0:f>
-        <ns0:v>2.6e+217</ns0:v>
+        <ns0:v>2.34e+218</ns0:v>
       </ns0:c>
       <ns0:c r="E197" s="1">
         <ns0:f>D197</ns0:f>
-        <ns0:v>2.6e+217</ns0:v>
+        <ns0:v>2.34e+218</ns0:v>
       </ns0:c>
       <ns0:c r="F197" s="1">
         <ns0:f>ROUND(F196*1.4,-5)</ns0:f>
@@ -7226,11 +7226,11 @@
       </ns0:c>
       <ns0:c r="D198" s="1">
         <ns0:f>ROUND(D197*20,2-INT(LOG10(ABS(D197*20))))</ns0:f>
-        <ns0:v>5.2e+218</ns0:v>
+        <ns0:v>4.6799999999999996e+219</ns0:v>
       </ns0:c>
       <ns0:c r="E198" s="1">
         <ns0:f>D198</ns0:f>
-        <ns0:v>5.2e+218</ns0:v>
+        <ns0:v>4.6799999999999996e+219</ns0:v>
       </ns0:c>
       <ns0:c r="F198" s="1">
         <ns0:f>ROUND(F197*1.4,-5)</ns0:f>
@@ -7258,11 +7258,11 @@
       </ns0:c>
       <ns0:c r="D199" s="1">
         <ns0:f>ROUND(D198*20,2-INT(LOG10(ABS(D198*20))))</ns0:f>
-        <ns0:v>1.04e+220</ns0:v>
+        <ns0:v>9.359999999999999e+220</ns0:v>
       </ns0:c>
       <ns0:c r="E199" s="1">
         <ns0:f>D199</ns0:f>
-        <ns0:v>1.04e+220</ns0:v>
+        <ns0:v>9.359999999999999e+220</ns0:v>
       </ns0:c>
       <ns0:c r="F199" s="1">
         <ns0:f>ROUND(F198*1.4,-5)</ns0:f>
@@ -7290,11 +7290,11 @@
       </ns0:c>
       <ns0:c r="D200" s="1">
         <ns0:f>ROUND(D199*20,2-INT(LOG10(ABS(D199*20))))</ns0:f>
-        <ns0:v>2.08e+221</ns0:v>
+        <ns0:v>1.87e+222</ns0:v>
       </ns0:c>
       <ns0:c r="E200" s="1">
         <ns0:f>D200</ns0:f>
-        <ns0:v>2.08e+221</ns0:v>
+        <ns0:v>1.87e+222</ns0:v>
       </ns0:c>
       <ns0:c r="F200" s="1">
         <ns0:f>ROUND(F199*1.4,-5)</ns0:f>
@@ -7322,11 +7322,11 @@
       </ns0:c>
       <ns0:c r="D201" s="1">
         <ns0:f>ROUND(D200*20,2-INT(LOG10(ABS(D200*20))))</ns0:f>
-        <ns0:v>4.16e+222</ns0:v>
+        <ns0:v>3.74e+223</ns0:v>
       </ns0:c>
       <ns0:c r="E201" s="1">
         <ns0:f>D201</ns0:f>
-        <ns0:v>4.16e+222</ns0:v>
+        <ns0:v>3.74e+223</ns0:v>
       </ns0:c>
       <ns0:c r="F201" s="1">
         <ns0:f>ROUND(F200*1.4,-5)</ns0:f>
@@ -7354,11 +7354,11 @@
       </ns0:c>
       <ns0:c r="D202" s="1">
         <ns0:f>ROUND(D201*20,2-INT(LOG10(ABS(D201*20))))</ns0:f>
-        <ns0:v>8.319999999999999e+223</ns0:v>
+        <ns0:v>7.479999999999999e+224</ns0:v>
       </ns0:c>
       <ns0:c r="E202" s="1">
         <ns0:f>D202</ns0:f>
-        <ns0:v>8.319999999999999e+223</ns0:v>
+        <ns0:v>7.479999999999999e+224</ns0:v>
       </ns0:c>
       <ns0:c r="F202" s="1">
         <ns0:f>ROUND(F201*1.4,-5)</ns0:f>
@@ -7386,11 +7386,11 @@
       </ns0:c>
       <ns0:c r="D203" s="1">
         <ns0:f>ROUND(D202*20,2-INT(LOG10(ABS(D202*20))))</ns0:f>
-        <ns0:v>1.6600000000000002e+225</ns0:v>
+        <ns0:v>1.5e+226</ns0:v>
       </ns0:c>
       <ns0:c r="E203" s="1">
         <ns0:f>D203</ns0:f>
-        <ns0:v>1.6600000000000002e+225</ns0:v>
+        <ns0:v>1.5e+226</ns0:v>
       </ns0:c>
       <ns0:c r="F203" s="1">
         <ns0:f>ROUND(F202*1.4,-5)</ns0:f>
@@ -7418,11 +7418,11 @@
       </ns0:c>
       <ns0:c r="D204" s="1">
         <ns0:f>ROUND(D203*20,2-INT(LOG10(ABS(D203*20))))</ns0:f>
-        <ns0:v>3.3199999999999997e+226</ns0:v>
+        <ns0:v>3.0000000000000003e+227</ns0:v>
       </ns0:c>
       <ns0:c r="E204" s="1">
         <ns0:f>D204</ns0:f>
-        <ns0:v>3.3199999999999997e+226</ns0:v>
+        <ns0:v>3.0000000000000003e+227</ns0:v>
       </ns0:c>
       <ns0:c r="F204" s="1">
         <ns0:f>ROUND(F203*1.4,-5)</ns0:f>
@@ -7450,11 +7450,11 @@
       </ns0:c>
       <ns0:c r="D205" s="1">
         <ns0:f>ROUND(D204*20,2-INT(LOG10(ABS(D204*20))))</ns0:f>
-        <ns0:v>6.640000000000001e+227</ns0:v>
+        <ns0:v>6e+228</ns0:v>
       </ns0:c>
       <ns0:c r="E205" s="1">
         <ns0:f>D205</ns0:f>
-        <ns0:v>6.640000000000001e+227</ns0:v>
+        <ns0:v>6e+228</ns0:v>
       </ns0:c>
       <ns0:c r="F205" s="1">
         <ns0:f>ROUND(F204*1.4,-5)</ns0:f>
@@ -7482,11 +7482,11 @@
       </ns0:c>
       <ns0:c r="D206" s="1">
         <ns0:f>ROUND(D205*20,2-INT(LOG10(ABS(D205*20))))</ns0:f>
-        <ns0:v>1.3300000000000002e+229</ns0:v>
+        <ns0:v>1.2e+230</ns0:v>
       </ns0:c>
       <ns0:c r="E206" s="1">
         <ns0:f>D206</ns0:f>
-        <ns0:v>1.3300000000000002e+229</ns0:v>
+        <ns0:v>1.2e+230</ns0:v>
       </ns0:c>
       <ns0:c r="F206" s="1">
         <ns0:f>ROUND(F205*1.4,-5)</ns0:f>
@@ -7514,11 +7514,11 @@
       </ns0:c>
       <ns0:c r="D207" s="1">
         <ns0:f>ROUND(D206*20,2-INT(LOG10(ABS(D206*20))))</ns0:f>
-        <ns0:v>2.66e+230</ns0:v>
+        <ns0:v>2.3999999999999997e+231</ns0:v>
       </ns0:c>
       <ns0:c r="E207" s="1">
         <ns0:f>D207</ns0:f>
-        <ns0:v>2.66e+230</ns0:v>
+        <ns0:v>2.3999999999999997e+231</ns0:v>
       </ns0:c>
       <ns0:c r="F207" s="1">
         <ns0:f>ROUND(F206*1.4,-5)</ns0:f>
@@ -7546,11 +7546,11 @@
       </ns0:c>
       <ns0:c r="D208" s="1">
         <ns0:f>ROUND(D207*20,2-INT(LOG10(ABS(D207*20))))</ns0:f>
-        <ns0:v>5.3199999999999994e+231</ns0:v>
+        <ns0:v>4.7999999999999997e+232</ns0:v>
       </ns0:c>
       <ns0:c r="E208" s="1">
         <ns0:f>D208</ns0:f>
-        <ns0:v>5.3199999999999994e+231</ns0:v>
+        <ns0:v>4.7999999999999997e+232</ns0:v>
       </ns0:c>
       <ns0:c r="F208" s="1">
         <ns0:f>ROUND(F207*1.4,-5)</ns0:f>
@@ -7578,11 +7578,11 @@
       </ns0:c>
       <ns0:c r="D209" s="1">
         <ns0:f>ROUND(D208*20,2-INT(LOG10(ABS(D208*20))))</ns0:f>
-        <ns0:v>1.06e+233</ns0:v>
+        <ns0:v>9.6e+233</ns0:v>
       </ns0:c>
       <ns0:c r="E209" s="1">
         <ns0:f>D209</ns0:f>
-        <ns0:v>1.06e+233</ns0:v>
+        <ns0:v>9.6e+233</ns0:v>
       </ns0:c>
       <ns0:c r="F209" s="1">
         <ns0:f>ROUND(F208*1.4,-5)</ns0:f>
@@ -7610,11 +7610,11 @@
       </ns0:c>
       <ns0:c r="D210" s="1">
         <ns0:f>ROUND(D209*20,2-INT(LOG10(ABS(D209*20))))</ns0:f>
-        <ns0:v>2.12e+234</ns0:v>
+        <ns0:v>1.92e+235</ns0:v>
       </ns0:c>
       <ns0:c r="E210" s="1">
         <ns0:f>D210</ns0:f>
-        <ns0:v>2.12e+234</ns0:v>
+        <ns0:v>1.92e+235</ns0:v>
       </ns0:c>
       <ns0:c r="F210" s="1">
         <ns0:f>ROUND(F209*1.4,-5)</ns0:f>
@@ -7642,11 +7642,11 @@
       </ns0:c>
       <ns0:c r="D211" s="1">
         <ns0:f>ROUND(D210*20,2-INT(LOG10(ABS(D210*20))))</ns0:f>
-        <ns0:v>4.24e+235</ns0:v>
+        <ns0:v>3.8400000000000003e+236</ns0:v>
       </ns0:c>
       <ns0:c r="E211" s="1">
         <ns0:f>D211</ns0:f>
-        <ns0:v>4.24e+235</ns0:v>
+        <ns0:v>3.8400000000000003e+236</ns0:v>
       </ns0:c>
       <ns0:c r="F211" s="1">
         <ns0:f>ROUND(F210*1.4,-5)</ns0:f>
@@ -7674,11 +7674,11 @@
       </ns0:c>
       <ns0:c r="D212" s="1">
         <ns0:f>ROUND(D211*20,2-INT(LOG10(ABS(D211*20))))</ns0:f>
-        <ns0:v>8.480000000000001e+236</ns0:v>
+        <ns0:v>7.68e+237</ns0:v>
       </ns0:c>
       <ns0:c r="E212" s="1">
         <ns0:f>D212</ns0:f>
-        <ns0:v>8.480000000000001e+236</ns0:v>
+        <ns0:v>7.68e+237</ns0:v>
       </ns0:c>
       <ns0:c r="F212" s="1">
         <ns0:f>ROUND(F211*1.4,-5)</ns0:f>
@@ -7706,11 +7706,11 @@
       </ns0:c>
       <ns0:c r="D213" s="1">
         <ns0:f>ROUND(D212*20,2-INT(LOG10(ABS(D212*20))))</ns0:f>
-        <ns0:v>1.7e+238</ns0:v>
+        <ns0:v>1.54e+239</ns0:v>
       </ns0:c>
       <ns0:c r="E213" s="1">
         <ns0:f>D213</ns0:f>
-        <ns0:v>1.7e+238</ns0:v>
+        <ns0:v>1.54e+239</ns0:v>
       </ns0:c>
       <ns0:c r="F213" s="1">
         <ns0:f>ROUND(F212*1.4,-5)</ns0:f>
@@ -7738,11 +7738,11 @@
       </ns0:c>
       <ns0:c r="D214" s="1">
         <ns0:f>ROUND(D213*20,2-INT(LOG10(ABS(D213*20))))</ns0:f>
-        <ns0:v>3.4e+239</ns0:v>
+        <ns0:v>3.08e+240</ns0:v>
       </ns0:c>
       <ns0:c r="E214" s="1">
         <ns0:f>D214</ns0:f>
-        <ns0:v>3.4e+239</ns0:v>
+        <ns0:v>3.08e+240</ns0:v>
       </ns0:c>
       <ns0:c r="F214" s="1">
         <ns0:f>ROUND(F213*1.4,-5)</ns0:f>
@@ -7770,11 +7770,11 @@
       </ns0:c>
       <ns0:c r="D215" s="1">
         <ns0:f>ROUND(D214*20,2-INT(LOG10(ABS(D214*20))))</ns0:f>
-        <ns0:v>6.8e+240</ns0:v>
+        <ns0:v>6.16e+241</ns0:v>
       </ns0:c>
       <ns0:c r="E215" s="1">
         <ns0:f>D215</ns0:f>
-        <ns0:v>6.8e+240</ns0:v>
+        <ns0:v>6.16e+241</ns0:v>
       </ns0:c>
       <ns0:c r="F215" s="1">
         <ns0:f>ROUND(F214*1.4,-5)</ns0:f>
@@ -7802,11 +7802,11 @@
       </ns0:c>
       <ns0:c r="D216" s="1">
         <ns0:f>ROUND(D215*20,2-INT(LOG10(ABS(D215*20))))</ns0:f>
-        <ns0:v>1.36e+242</ns0:v>
+        <ns0:v>1.23e+243</ns0:v>
       </ns0:c>
       <ns0:c r="E216" s="1">
         <ns0:f>D216</ns0:f>
-        <ns0:v>1.36e+242</ns0:v>
+        <ns0:v>1.23e+243</ns0:v>
       </ns0:c>
       <ns0:c r="F216" s="1">
         <ns0:f>ROUND(F215*1.4,-5)</ns0:f>
@@ -7834,11 +7834,11 @@
       </ns0:c>
       <ns0:c r="D217" s="1">
         <ns0:f>ROUND(D216*20,2-INT(LOG10(ABS(D216*20))))</ns0:f>
-        <ns0:v>2.7200000000000002e+243</ns0:v>
+        <ns0:v>2.4600000000000002e+244</ns0:v>
       </ns0:c>
       <ns0:c r="E217" s="1">
         <ns0:f>D217</ns0:f>
-        <ns0:v>2.7200000000000002e+243</ns0:v>
+        <ns0:v>2.4600000000000002e+244</ns0:v>
       </ns0:c>
       <ns0:c r="F217" s="1">
         <ns0:f>ROUND(F216*1.4,-5)</ns0:f>
@@ -7866,11 +7866,11 @@
       </ns0:c>
       <ns0:c r="D218" s="1">
         <ns0:f>ROUND(D217*20,2-INT(LOG10(ABS(D217*20))))</ns0:f>
-        <ns0:v>5.44e+244</ns0:v>
+        <ns0:v>4.92e+245</ns0:v>
       </ns0:c>
       <ns0:c r="E218" s="1">
         <ns0:f>D218</ns0:f>
-        <ns0:v>5.44e+244</ns0:v>
+        <ns0:v>4.92e+245</ns0:v>
       </ns0:c>
       <ns0:c r="F218" s="1">
         <ns0:f>ROUND(F217*1.4,-5)</ns0:f>
@@ -7898,11 +7898,11 @@
       </ns0:c>
       <ns0:c r="D219" s="1">
         <ns0:f>ROUND(D218*20,2-INT(LOG10(ABS(D218*20))))</ns0:f>
-        <ns0:v>1.0900000000000001e+246</ns0:v>
+        <ns0:v>9.840000000000001e+246</ns0:v>
       </ns0:c>
       <ns0:c r="E219" s="1">
         <ns0:f>D219</ns0:f>
-        <ns0:v>1.0900000000000001e+246</ns0:v>
+        <ns0:v>9.840000000000001e+246</ns0:v>
       </ns0:c>
       <ns0:c r="F219" s="1">
         <ns0:f>ROUND(F218*1.4,-5)</ns0:f>
@@ -7930,11 +7930,11 @@
       </ns0:c>
       <ns0:c r="D220" s="1">
         <ns0:f>ROUND(D219*20,2-INT(LOG10(ABS(D219*20))))</ns0:f>
-        <ns0:v>2.1800000000000002e+247</ns0:v>
+        <ns0:v>1.9700000000000002e+248</ns0:v>
       </ns0:c>
       <ns0:c r="E220" s="1">
         <ns0:f>D220</ns0:f>
-        <ns0:v>2.1800000000000002e+247</ns0:v>
+        <ns0:v>1.9700000000000002e+248</ns0:v>
       </ns0:c>
       <ns0:c r="F220" s="1">
         <ns0:f>ROUND(F219*1.4,-5)</ns0:f>
@@ -7962,11 +7962,11 @@
       </ns0:c>
       <ns0:c r="D221" s="1">
         <ns0:f>ROUND(D220*20,2-INT(LOG10(ABS(D220*20))))</ns0:f>
-        <ns0:v>4.3600000000000004e+248</ns0:v>
+        <ns0:v>3.94e+249</ns0:v>
       </ns0:c>
       <ns0:c r="E221" s="1">
         <ns0:f>D221</ns0:f>
-        <ns0:v>4.3600000000000004e+248</ns0:v>
+        <ns0:v>3.94e+249</ns0:v>
       </ns0:c>
       <ns0:c r="F221" s="1">
         <ns0:f>ROUND(F220*1.4,-5)</ns0:f>
@@ -7994,11 +7994,11 @@
       </ns0:c>
       <ns0:c r="D222" s="1">
         <ns0:f>ROUND(D221*20,2-INT(LOG10(ABS(D221*20))))</ns0:f>
-        <ns0:v>8.72e+249</ns0:v>
+        <ns0:v>7.88e+250</ns0:v>
       </ns0:c>
       <ns0:c r="E222" s="1">
         <ns0:f>D222</ns0:f>
-        <ns0:v>8.72e+249</ns0:v>
+        <ns0:v>7.88e+250</ns0:v>
       </ns0:c>
       <ns0:c r="F222" s="1">
         <ns0:f>ROUND(F221*1.4,-5)</ns0:f>
@@ -8026,11 +8026,11 @@
       </ns0:c>
       <ns0:c r="D223" s="1">
         <ns0:f>ROUND(D222*20,2-INT(LOG10(ABS(D222*20))))</ns0:f>
-        <ns0:v>1.74e+251</ns0:v>
+        <ns0:v>1.5799999999999999e+252</ns0:v>
       </ns0:c>
       <ns0:c r="E223" s="1">
         <ns0:f>D223</ns0:f>
-        <ns0:v>1.74e+251</ns0:v>
+        <ns0:v>1.5799999999999999e+252</ns0:v>
       </ns0:c>
       <ns0:c r="F223" s="1">
         <ns0:f>ROUND(F222*1.4,-5)</ns0:f>

</xml_diff>

<commit_message>
balance: provisionally raise later cycle budgets for bounded diagnosis
</commit_message>
<xml_diff>
--- a/space-battleship/config_excel/level.xlsx
+++ b/space-battleship/config_excel/level.xlsx
@@ -2135,10 +2135,10 @@
         </ns0:is>
       </ns0:c>
       <ns0:c r="D35" s="1" t="n">
-        <ns0:v>1.941662253193607e+26</ns0:v>
+        <ns0:v>9.363726143873491e+25</ns0:v>
       </ns0:c>
       <ns0:c r="E35" s="1" t="n">
-        <ns0:v>1.941662253193607e+26</ns0:v>
+        <ns0:v>9.363726143873491e+25</ns0:v>
       </ns0:c>
       <ns0:c r="F35" s="1" t="n">
         <ns0:v>9704565562037236</ns0:v>
@@ -2163,10 +2163,10 @@
         </ns0:is>
       </ns0:c>
       <ns0:c r="D36" s="1" t="n">
-        <ns0:v>4.026230848222263e+26</ns0:v>
+        <ns0:v>3.589827867061663e+27</ns0:v>
       </ns0:c>
       <ns0:c r="E36" s="1" t="n">
-        <ns0:v>4.026230848222263e+26</ns0:v>
+        <ns0:v>3.589827867061663e+27</ns0:v>
       </ns0:c>
       <ns0:c r="F36" s="1" t="n">
         <ns0:v>2.012338714944041e+16</ns0:v>
@@ -2191,10 +2191,10 @@
         </ns0:is>
       </ns0:c>
       <ns0:c r="D37" s="1" t="n">
-        <ns0:v>1.543560274627236e+28</ns0:v>
+        <ns0:v>1.376253845651405e+29</ns0:v>
       </ns0:c>
       <ns0:c r="E37" s="1" t="n">
-        <ns0:v>1.543560274627236e+28</ns0:v>
+        <ns0:v>1.376253845651405e+29</ns0:v>
       </ns0:c>
       <ns0:c r="F37" s="1" t="n">
         <ns0:v>2.012338714944041e+16</ns0:v>
@@ -2219,10 +2219,10 @@
         </ns0:is>
       </ns0:c>
       <ns0:c r="D38" s="1" t="n">
-        <ns0:v>1.76699772433822e+30</ns0:v>
+        <ns0:v>1.890567504244719e+31</ns0:v>
       </ns0:c>
       <ns0:c r="E38" s="1" t="n">
-        <ns0:v>1.76699772433822e+30</ns0:v>
+        <ns0:v>1.890567504244719e+31</ns0:v>
       </ns0:c>
       <ns0:c r="F38" s="1" t="n">
         <ns0:v>6.008811205403466e+16</ns0:v>
@@ -2247,10 +2247,10 @@
         </ns0:is>
       </ns0:c>
       <ns0:c r="D39" s="1" t="n">
-        <ns0:v>5.276226932910335e+30</ns0:v>
+        <ns0:v>8.129094218776313e+31</ns0:v>
       </ns0:c>
       <ns0:c r="E39" s="1" t="n">
-        <ns0:v>5.276226932910335e+30</ns0:v>
+        <ns0:v>8.129094218776313e+31</ns0:v>
       </ns0:c>
       <ns0:c r="F39" s="1" t="n">
         <ns0:v>1.245987091552463e+17</ns0:v>
@@ -2275,10 +2275,10 @@
         </ns0:is>
       </ns0:c>
       <ns0:c r="D40" s="1" t="n">
-        <ns0:v>1.575472920203933e+31</ns0:v>
+        <ns0:v>3.495361719133234e+32</ns0:v>
       </ns0:c>
       <ns0:c r="E40" s="1" t="n">
-        <ns0:v>1.575472920203933e+31</ns0:v>
+        <ns0:v>3.495361719133234e+32</ns0:v>
       </ns0:c>
       <ns0:c r="F40" s="1" t="n">
         <ns0:v>2.583678833043186e+17</ns0:v>
@@ -2303,10 +2303,10 @@
         </ns0:is>
       </ns0:c>
       <ns0:c r="D41" s="1" t="n">
-        <ns0:v>4.70433693216222e+31</ns0:v>
+        <ns0:v>1.502941560126383e+33</ns0:v>
       </ns0:c>
       <ns0:c r="E41" s="1" t="n">
-        <ns0:v>4.70433693216222e+31</ns0:v>
+        <ns0:v>1.502941560126383e+33</ns0:v>
       </ns0:c>
       <ns0:c r="F41" s="1" t="n">
         <ns0:v>5.357516428198349e+17</ns0:v>
@@ -2331,10 +2331,10 @@
         </ns0:is>
       </ns0:c>
       <ns0:c r="D42" s="1" t="n">
-        <ns0:v>4.194434062959881e+32</ns0:v>
+        <ns0:v>4.001331405693829e+34</ns0:v>
       </ns0:c>
       <ns0:c r="E42" s="1" t="n">
-        <ns0:v>4.194434062959881e+32</ns0:v>
+        <ns0:v>4.001331405693829e+34</ns0:v>
       </ns0:c>
       <ns0:c r="F42" s="1" t="n">
         <ns0:v>2.303634000144588e+18</ns0:v>
@@ -2359,10 +2359,10 @@
         </ns0:is>
       </ns0:c>
       <ns0:c r="D43" s="1" t="n">
-        <ns0:v>1.608045350153449e+34</ns0:v>
+        <ns0:v>6.595981245658691e+36</ns0:v>
       </ns0:c>
       <ns0:c r="E43" s="1" t="n">
-        <ns0:v>1.608045350153449e+34</ns0:v>
+        <ns0:v>6.595981245658691e+36</ns0:v>
       </ns0:c>
       <ns0:c r="F43" s="1" t="n">
         <ns0:v>2.053943214130691e+19</ns0:v>
@@ -2387,10 +2387,10 @@
         </ns0:is>
       </ns0:c>
       <ns0:c r="D44" s="1" t="n">
-        <ns0:v>4.801597686832597e+34</ns0:v>
+        <ns0:v>2.836151202792515e+37</ns0:v>
       </ns0:c>
       <ns0:c r="E44" s="1" t="n">
-        <ns0:v>4.801597686832597e+34</ns0:v>
+        <ns0:v>2.836151202792515e+37</ns0:v>
       </ns0:c>
       <ns0:c r="F44" s="1" t="n">
         <ns0:v>4.259056648821401e+19</ns0:v>
@@ -2415,10 +2415,10 @@
         </ns0:is>
       </ns0:c>
       <ns0:c r="D45" s="1" t="n">
-        <ns0:v>1.433749386731914e+35</ns0:v>
+        <ns0:v>1.219493104289165e+38</ns0:v>
       </ns0:c>
       <ns0:c r="E45" s="1" t="n">
-        <ns0:v>1.433749386731914e+35</ns0:v>
+        <ns0:v>1.219493104289165e+38</ns0:v>
       </ns0:c>
       <ns0:c r="F45" s="1" t="n">
         <ns0:v>8.831579866996054e+19</ns0:v>
@@ -2443,10 +2443,10 @@
         </ns0:is>
       </ns0:c>
       <ns0:c r="D46" s="1" t="n">
-        <ns0:v>4.281152728791306e+35</ns0:v>
+        <ns0:v>5.2435971324256e+38</ns0:v>
       </ns0:c>
       <ns0:c r="E46" s="1" t="n">
-        <ns0:v>4.281152728791306e+35</ns0:v>
+        <ns0:v>5.2435971324256e+38</ns0:v>
       </ns0:c>
       <ns0:c r="F46" s="1" t="n">
         <ns0:v>1.831316401220302e+20</ns0:v>
@@ -2471,10 +2471,10 @@
         </ns0:is>
       </ns0:c>
       <ns0:c r="D47" s="1" t="n">
-        <ns0:v>3.817118776422855e+36</ns0:v>
+        <ns0:v>1.396020340472608e+40</ns0:v>
       </ns0:c>
       <ns0:c r="E47" s="1" t="n">
-        <ns0:v>3.817118776422855e+36</ns0:v>
+        <ns0:v>1.396020340472608e+40</ns0:v>
       </ns0:c>
       <ns0:c r="F47" s="1" t="n">
         <ns0:v>7.874325321093216e+20</ns0:v>
@@ -2499,10 +2499,10 @@
         </ns0:is>
       </ns0:c>
       <ns0:c r="D48" s="1" t="n">
-        <ns0:v>1.463391725146999e+38</ns0:v>
+        <ns0:v>2.301265016742271e+42</ns0:v>
       </ns0:c>
       <ns0:c r="E48" s="1" t="n">
-        <ns0:v>1.463391725146999e+38</ns0:v>
+        <ns0:v>2.301265016742271e+42</ns0:v>
       </ns0:c>
       <ns0:c r="F48" s="1" t="n">
         <ns0:v>7.020827552511277e+21</ns0:v>
@@ -2527,10 +2527,10 @@
         </ns0:is>
       </ns0:c>
       <ns0:c r="D49" s="1" t="n">
-        <ns0:v>4.369664277021336e+38</ns0:v>
+        <ns0:v>9.895018348443098e+42</ns0:v>
       </ns0:c>
       <ns0:c r="E49" s="1" t="n">
-        <ns0:v>4.369664277021336e+38</ns0:v>
+        <ns0:v>9.895018348443098e+42</ns0:v>
       </ns0:c>
       <ns0:c r="F49" s="1" t="n">
         <ns0:v>1.455838801288738e+22</ns0:v>
@@ -2555,10 +2555,10 @@
         </ns0:is>
       </ns0:c>
       <ns0:c r="D50" s="1" t="n">
-        <ns0:v>1.304774761655727e+39</ns0:v>
+        <ns0:v>4.254676771414681e+43</ns0:v>
       </ns0:c>
       <ns0:c r="E50" s="1" t="n">
-        <ns0:v>1.304774761655727e+39</ns0:v>
+        <ns0:v>4.254676771414681e+43</ns0:v>
       </ns0:c>
       <ns0:c r="F50" s="1" t="n">
         <ns0:v>3.018827338352327e+22</ns0:v>
@@ -2583,10 +2583,10 @@
         </ns0:is>
       </ns0:c>
       <ns0:c r="D51" s="1" t="n">
-        <ns0:v>3.896036561907815e+39</ns0:v>
+        <ns0:v>1.829433134104688e+44</ns0:v>
       </ns0:c>
       <ns0:c r="E51" s="1" t="n">
-        <ns0:v>3.896036561907815e+39</ns0:v>
+        <ns0:v>1.829433134104688e+44</ns0:v>
       </ns0:c>
       <ns0:c r="F51" s="1" t="n">
         <ns0:v>6.259840368807384e+22</ns0:v>
@@ -2611,10 +2611,10 @@
         </ns0:is>
       </ns0:c>
       <ns0:c r="D52" s="1" t="n">
-        <ns0:v>3.473745333604802e+40</ns0:v>
+        <ns0:v>4.870560804436351e+45</ns0:v>
       </ns0:c>
       <ns0:c r="E52" s="1" t="n">
-        <ns0:v>3.473745333604802e+40</ns0:v>
+        <ns0:v>4.870560804436351e+45</ns0:v>
       </ns0:c>
       <ns0:c r="F52" s="1" t="n">
         <ns0:v>2.691616778469064e+23</ns0:v>
@@ -2639,10 +2639,10 @@
         </ns0:is>
       </ns0:c>
       <ns0:c r="D53" s="1" t="n">
-        <ns0:v>1.331750588392519e+42</ns0:v>
+        <ns0:v>8.028859513157927e+47</ns0:v>
       </ns0:c>
       <ns0:c r="E53" s="1" t="n">
-        <ns0:v>1.331750588392519e+42</ns0:v>
+        <ns0:v>8.028859513157927e+47</ns0:v>
       </ns0:c>
       <ns0:c r="F53" s="1" t="n">
         <ns0:v>2.399872556504138e+24</ns0:v>
@@ -2667,10 +2667,10 @@
         </ns0:is>
       </ns0:c>
       <ns0:c r="D54" s="1" t="n">
-        <ns0:v>3.976585948930646e+42</ns0:v>
+        <ns0:v>3.452262630413378e+48</ns0:v>
       </ns0:c>
       <ns0:c r="E54" s="1" t="n">
-        <ns0:v>3.976585948930646e+42</ns0:v>
+        <ns0:v>3.452262630413378e+48</ns0:v>
       </ns0:c>
       <ns0:c r="F54" s="1" t="n">
         <ns0:v>4.976375733166981e+24</ns0:v>
@@ -2695,10 +2695,10 @@
         </ns0:is>
       </ns0:c>
       <ns0:c r="D55" s="1" t="n">
-        <ns0:v>1.187402201813172e+43</ns0:v>
+        <ns0:v>1.484409740862565e+49</ns0:v>
       </ns0:c>
       <ns0:c r="E55" s="1" t="n">
-        <ns0:v>1.187402201813172e+43</ns0:v>
+        <ns0:v>1.484409740862565e+49</ns0:v>
       </ns0:c>
       <ns0:c r="F55" s="1" t="n">
         <ns0:v>1.031901272029505e+25</ns0:v>
@@ -2723,10 +2723,10 @@
         </ns0:is>
       </ns0:c>
       <ns0:c r="D56" s="1" t="n">
-        <ns0:v>3.545563976178902e+43</ns0:v>
+        <ns0:v>6.382690179350061e+49</ns0:v>
       </ns0:c>
       <ns0:c r="E56" s="1" t="n">
-        <ns0:v>3.545563976178902e+43</ns0:v>
+        <ns0:v>6.382690179350061e+49</ns0:v>
       </ns0:c>
       <ns0:c r="F56" s="1" t="n">
         <ns0:v>2.139750477680381e+25</ns0:v>
@@ -2751,10 +2751,10 @@
         </ns0:is>
       </ns0:c>
       <ns0:c r="D57" s="1" t="n">
-        <ns0:v>3.161260455732902e+44</ns0:v>
+        <ns0:v>1.699284878734698e+51</ns0:v>
       </ns0:c>
       <ns0:c r="E57" s="1" t="n">
-        <ns0:v>3.161260455732902e+44</ns0:v>
+        <ns0:v>1.699284878734698e+51</ns0:v>
       </ns0:c>
       <ns0:c r="F57" s="1" t="n">
         <ns0:v>9.200535394098201e+25</ns0:v>
@@ -2779,10 +2779,10 @@
         </ns0:is>
       </ns0:c>
       <ns0:c r="D58" s="1" t="n">
-        <ns0:v>1.211951386089507e+46</ns0:v>
+        <ns0:v>2.80118042090091e+53</ns0:v>
       </ns0:c>
       <ns0:c r="E58" s="1" t="n">
-        <ns0:v>1.211951386089507e+46</ns0:v>
+        <ns0:v>2.80118042090091e+53</ns0:v>
       </ns0:c>
       <ns0:c r="F58" s="1" t="n">
         <ns0:v>8.203289775151412e+26</ns0:v>
@@ -2807,10 +2807,10 @@
         </ns0:is>
       </ns0:c>
       <ns0:c r="D59" s="1" t="n">
-        <ns0:v>3.618867447641088e+46</ns0:v>
+        <ns0:v>1.204456308180967e+54</ns0:v>
       </ns0:c>
       <ns0:c r="E59" s="1" t="n">
-        <ns0:v>3.618867447641088e+46</ns0:v>
+        <ns0:v>1.204456308180967e+54</ns0:v>
       </ns0:c>
       <ns0:c r="F59" s="1" t="n">
         <ns0:v>1.701034167775397e+27</ns0:v>
@@ -2835,10 +2835,10 @@
         </ns0:is>
       </ns0:c>
       <ns0:c r="D60" s="1" t="n">
-        <ns0:v>1.080588029677713e+47</ns0:v>
+        <ns0:v>5.178941661495506e+54</ns0:v>
       </ns0:c>
       <ns0:c r="E60" s="1" t="n">
-        <ns0:v>1.080588029677713e+47</ns0:v>
+        <ns0:v>5.178941661495506e+54</ns0:v>
       </ns0:c>
       <ns0:c r="F60" s="1" t="n">
         <ns0:v>3.527264450299061e+27</ns0:v>
@@ -2863,10 +2863,10 @@
         </ns0:is>
       </ns0:c>
       <ns0:c r="D61" s="1" t="n">
-        <ns0:v>3.226618567209174e+47</ns0:v>
+        <ns0:v>2.226850119094895e+55</ns0:v>
       </ns0:c>
       <ns0:c r="E61" s="1" t="n">
-        <ns0:v>3.226618567209174e+47</ns0:v>
+        <ns0:v>2.226850119094895e+55</ns0:v>
       </ns0:c>
       <ns0:c r="F61" s="1" t="n">
         <ns0:v>7.314135564140134e+27</ns0:v>
@@ -2891,10 +2891,10 @@
         </ns0:is>
       </ns0:c>
       <ns0:c r="D62" s="1" t="n">
-        <ns0:v>2.876885525344484e+48</ns0:v>
+        <ns0:v>5.928617288724234e+56</ns0:v>
       </ns0:c>
       <ns0:c r="E62" s="1" t="n">
-        <ns0:v>2.876885525344484e+48</ns0:v>
+        <ns0:v>5.928617288724234e+56</ns0:v>
       </ns0:c>
       <ns0:c r="F62" s="1" t="n">
         <ns0:v>3.14494441464289e+28</ns0:v>
@@ -2919,10 +2919,10 @@
         </ns0:is>
       </ns0:c>
       <ns0:c r="D63" s="1" t="n">
-        <ns0:v>1.102928862991691e+50</ns0:v>
+        <ns0:v>9.773009152270437e+58</ns0:v>
       </ns0:c>
       <ns0:c r="E63" s="1" t="n">
-        <ns0:v>1.102928862991691e+50</ns0:v>
+        <ns0:v>9.773009152270437e+58</ns0:v>
       </ns0:c>
       <ns0:c r="F63" s="1" t="n">
         <ns0:v>2.804064030513767e+29</ns0:v>
@@ -2948,11 +2948,11 @@
       </ns0:c>
       <ns0:c r="D64" s="1">
         <ns0:f>ROUND(D63*10,0)</ns0:f>
-        <ns0:v>1.1029288629916913e+51</ns0:v>
+        <ns0:v>9.773009152270437e+59</ns0:v>
       </ns0:c>
       <ns0:c r="E64" s="1">
         <ns0:f>D64</ns0:f>
-        <ns0:v>1.1029288629916913e+51</ns0:v>
+        <ns0:v>9.773009152270437e+59</ns0:v>
       </ns0:c>
       <ns0:c r="F64" s="1">
         <ns0:f>ROUND(F63*1.4,-5)</ns0:f>
@@ -2979,11 +2979,11 @@
       </ns0:c>
       <ns0:c r="D65" s="1">
         <ns0:f>ROUND(D64*10,0)</ns0:f>
-        <ns0:v>1.1029288629916913e+52</ns0:v>
+        <ns0:v>9.773009152270436e+60</ns0:v>
       </ns0:c>
       <ns0:c r="E65" s="1">
         <ns0:f>D65</ns0:f>
-        <ns0:v>1.1029288629916913e+52</ns0:v>
+        <ns0:v>9.773009152270436e+60</ns0:v>
       </ns0:c>
       <ns0:c r="F65" s="1">
         <ns0:f>ROUND(F64*1.4,-5)</ns0:f>
@@ -3010,11 +3010,11 @@
       </ns0:c>
       <ns0:c r="D66" s="1">
         <ns0:f>ROUND(D65*10,0)</ns0:f>
-        <ns0:v>1.1029288629916914e+53</ns0:v>
+        <ns0:v>9.773009152270436e+61</ns0:v>
       </ns0:c>
       <ns0:c r="E66" s="1">
         <ns0:f>D66</ns0:f>
-        <ns0:v>1.1029288629916914e+53</ns0:v>
+        <ns0:v>9.773009152270436e+61</ns0:v>
       </ns0:c>
       <ns0:c r="F66" s="1">
         <ns0:f>ROUND(F65*1.4,-5)</ns0:f>
@@ -3041,11 +3041,11 @@
       </ns0:c>
       <ns0:c r="D67" s="1">
         <ns0:f>ROUND(D66*10,0)</ns0:f>
-        <ns0:v>1.1029288629916914e+54</ns0:v>
+        <ns0:v>9.773009152270435e+62</ns0:v>
       </ns0:c>
       <ns0:c r="E67" s="1">
         <ns0:f>D67</ns0:f>
-        <ns0:v>1.1029288629916914e+54</ns0:v>
+        <ns0:v>9.773009152270435e+62</ns0:v>
       </ns0:c>
       <ns0:c r="F67" s="1">
         <ns0:f>ROUND(F66*1.4,-5)</ns0:f>
@@ -3072,11 +3072,11 @@
       </ns0:c>
       <ns0:c r="D68" s="1">
         <ns0:f>ROUND(D67*10,0)</ns0:f>
-        <ns0:v>1.1029288629916915e+55</ns0:v>
+        <ns0:v>9.773009152270435e+63</ns0:v>
       </ns0:c>
       <ns0:c r="E68" s="1">
         <ns0:f>D68</ns0:f>
-        <ns0:v>1.1029288629916915e+55</ns0:v>
+        <ns0:v>9.773009152270435e+63</ns0:v>
       </ns0:c>
       <ns0:c r="F68" s="1">
         <ns0:f>ROUND(F67*1.4,-5)</ns0:f>
@@ -3103,11 +3103,11 @@
       </ns0:c>
       <ns0:c r="D69" s="1">
         <ns0:f>ROUND(D68*10,0)</ns0:f>
-        <ns0:v>1.1029288629916915e+56</ns0:v>
+        <ns0:v>9.773009152270436e+64</ns0:v>
       </ns0:c>
       <ns0:c r="E69" s="1">
         <ns0:f>D69</ns0:f>
-        <ns0:v>1.1029288629916915e+56</ns0:v>
+        <ns0:v>9.773009152270436e+64</ns0:v>
       </ns0:c>
       <ns0:c r="F69" s="1">
         <ns0:f>ROUND(F68*1.4,-5)</ns0:f>
@@ -3134,11 +3134,11 @@
       </ns0:c>
       <ns0:c r="D70" s="1">
         <ns0:f>ROUND(D69*10,0)</ns0:f>
-        <ns0:v>1.1029288629916915e+57</ns0:v>
+        <ns0:v>9.773009152270435e+65</ns0:v>
       </ns0:c>
       <ns0:c r="E70" s="1">
         <ns0:f>D70</ns0:f>
-        <ns0:v>1.1029288629916915e+57</ns0:v>
+        <ns0:v>9.773009152270435e+65</ns0:v>
       </ns0:c>
       <ns0:c r="F70" s="1">
         <ns0:f>ROUND(F69*1.4,-5)</ns0:f>
@@ -3165,11 +3165,11 @@
       </ns0:c>
       <ns0:c r="D71" s="1">
         <ns0:f>ROUND(D70*10,0)</ns0:f>
-        <ns0:v>1.1029288629916915e+58</ns0:v>
+        <ns0:v>9.773009152270435e+66</ns0:v>
       </ns0:c>
       <ns0:c r="E71" s="1">
         <ns0:f>D71</ns0:f>
-        <ns0:v>1.1029288629916915e+58</ns0:v>
+        <ns0:v>9.773009152270435e+66</ns0:v>
       </ns0:c>
       <ns0:c r="F71" s="1">
         <ns0:f>ROUND(F70*1.4,-5)</ns0:f>
@@ -3196,11 +3196,11 @@
       </ns0:c>
       <ns0:c r="D72" s="1">
         <ns0:f>ROUND(D71*10,0)</ns0:f>
-        <ns0:v>1.1029288629916914e+59</ns0:v>
+        <ns0:v>9.773009152270435e+67</ns0:v>
       </ns0:c>
       <ns0:c r="E72" s="1">
         <ns0:f>D72</ns0:f>
-        <ns0:v>1.1029288629916914e+59</ns0:v>
+        <ns0:v>9.773009152270435e+67</ns0:v>
       </ns0:c>
       <ns0:c r="F72" s="1">
         <ns0:f>ROUND(F71*1.4,-5)</ns0:f>
@@ -3227,11 +3227,11 @@
       </ns0:c>
       <ns0:c r="D73" s="1">
         <ns0:f>ROUND(D72*10,0)</ns0:f>
-        <ns0:v>1.1029288629916914e+60</ns0:v>
+        <ns0:v>9.773009152270434e+68</ns0:v>
       </ns0:c>
       <ns0:c r="E73" s="1">
         <ns0:f>D73</ns0:f>
-        <ns0:v>1.1029288629916914e+60</ns0:v>
+        <ns0:v>9.773009152270434e+68</ns0:v>
       </ns0:c>
       <ns0:c r="F73" s="1">
         <ns0:f>ROUND(F72*1.4,-5)</ns0:f>
@@ -3258,11 +3258,11 @@
       </ns0:c>
       <ns0:c r="D74" s="1">
         <ns0:f>ROUND(D73*10,0)</ns0:f>
-        <ns0:v>1.1029288629916915e+61</ns0:v>
+        <ns0:v>9.773009152270435e+69</ns0:v>
       </ns0:c>
       <ns0:c r="E74" s="1">
         <ns0:f>D74</ns0:f>
-        <ns0:v>1.1029288629916915e+61</ns0:v>
+        <ns0:v>9.773009152270435e+69</ns0:v>
       </ns0:c>
       <ns0:c r="F74" s="1">
         <ns0:f>ROUND(F73*1.4,-5)</ns0:f>
@@ -3290,11 +3290,11 @@
       </ns0:c>
       <ns0:c r="D75" s="1">
         <ns0:f>ROUND(D74*10,0)</ns0:f>
-        <ns0:v>1.1029288629916914e+62</ns0:v>
+        <ns0:v>9.773009152270434e+70</ns0:v>
       </ns0:c>
       <ns0:c r="E75" s="1">
         <ns0:f>D75</ns0:f>
-        <ns0:v>1.1029288629916914e+62</ns0:v>
+        <ns0:v>9.773009152270434e+70</ns0:v>
       </ns0:c>
       <ns0:c r="F75" s="1">
         <ns0:f>ROUND(F74*1.4,-5)</ns0:f>
@@ -3322,11 +3322,11 @@
       </ns0:c>
       <ns0:c r="D76" s="1">
         <ns0:f>ROUND(D75*10,0)</ns0:f>
-        <ns0:v>1.1029288629916915e+63</ns0:v>
+        <ns0:v>9.773009152270434e+71</ns0:v>
       </ns0:c>
       <ns0:c r="E76" s="1">
         <ns0:f>D76</ns0:f>
-        <ns0:v>1.1029288629916915e+63</ns0:v>
+        <ns0:v>9.773009152270434e+71</ns0:v>
       </ns0:c>
       <ns0:c r="F76" s="1">
         <ns0:f>ROUND(F75*1.4,-5)</ns0:f>
@@ -3354,11 +3354,11 @@
       </ns0:c>
       <ns0:c r="D77" s="1">
         <ns0:f>ROUND(D76*10,0)</ns0:f>
-        <ns0:v>1.1029288629916914e+64</ns0:v>
+        <ns0:v>9.773009152270434e+72</ns0:v>
       </ns0:c>
       <ns0:c r="E77" s="1">
         <ns0:f>D77</ns0:f>
-        <ns0:v>1.1029288629916914e+64</ns0:v>
+        <ns0:v>9.773009152270434e+72</ns0:v>
       </ns0:c>
       <ns0:c r="F77" s="1">
         <ns0:f>ROUND(F76*1.4,-5)</ns0:f>
@@ -3386,11 +3386,11 @@
       </ns0:c>
       <ns0:c r="D78" s="1">
         <ns0:f>ROUND(D77*10,0)</ns0:f>
-        <ns0:v>1.1029288629916914e+65</ns0:v>
+        <ns0:v>9.773009152270433e+73</ns0:v>
       </ns0:c>
       <ns0:c r="E78" s="1">
         <ns0:f>D78</ns0:f>
-        <ns0:v>1.1029288629916914e+65</ns0:v>
+        <ns0:v>9.773009152270433e+73</ns0:v>
       </ns0:c>
       <ns0:c r="F78" s="1">
         <ns0:f>ROUND(F77*1.4,-5)</ns0:f>
@@ -3418,11 +3418,11 @@
       </ns0:c>
       <ns0:c r="D79" s="1">
         <ns0:f>ROUND(D78*10,0)</ns0:f>
-        <ns0:v>1.1029288629916914e+66</ns0:v>
+        <ns0:v>9.773009152270434e+74</ns0:v>
       </ns0:c>
       <ns0:c r="E79" s="1">
         <ns0:f>D79</ns0:f>
-        <ns0:v>1.1029288629916914e+66</ns0:v>
+        <ns0:v>9.773009152270434e+74</ns0:v>
       </ns0:c>
       <ns0:c r="F79" s="1">
         <ns0:f>ROUND(F78*1.4,-5)</ns0:f>
@@ -3450,11 +3450,11 @@
       </ns0:c>
       <ns0:c r="D80" s="1">
         <ns0:f>ROUND(D79*10,0)</ns0:f>
-        <ns0:v>1.1029288629916915e+67</ns0:v>
+        <ns0:v>9.773009152270435e+75</ns0:v>
       </ns0:c>
       <ns0:c r="E80" s="1">
         <ns0:f>D80</ns0:f>
-        <ns0:v>1.1029288629916915e+67</ns0:v>
+        <ns0:v>9.773009152270435e+75</ns0:v>
       </ns0:c>
       <ns0:c r="F80" s="1">
         <ns0:f>ROUND(F79*1.4,-5)</ns0:f>
@@ -3482,11 +3482,11 @@
       </ns0:c>
       <ns0:c r="D81" s="1">
         <ns0:f>ROUND(D80*10,0)</ns0:f>
-        <ns0:v>1.1029288629916915e+68</ns0:v>
+        <ns0:v>9.773009152270435e+76</ns0:v>
       </ns0:c>
       <ns0:c r="E81" s="1">
         <ns0:f>D81</ns0:f>
-        <ns0:v>1.1029288629916915e+68</ns0:v>
+        <ns0:v>9.773009152270435e+76</ns0:v>
       </ns0:c>
       <ns0:c r="F81" s="1">
         <ns0:f>ROUND(F80*1.4,-5)</ns0:f>
@@ -3514,11 +3514,11 @@
       </ns0:c>
       <ns0:c r="D82" s="1">
         <ns0:f>ROUND(D81*10,0)</ns0:f>
-        <ns0:v>1.1029288629916916e+69</ns0:v>
+        <ns0:v>9.773009152270435e+77</ns0:v>
       </ns0:c>
       <ns0:c r="E82" s="1">
         <ns0:f>D82</ns0:f>
-        <ns0:v>1.1029288629916916e+69</ns0:v>
+        <ns0:v>9.773009152270435e+77</ns0:v>
       </ns0:c>
       <ns0:c r="F82" s="1">
         <ns0:f>ROUND(F81*1.4,-5)</ns0:f>
@@ -3546,11 +3546,11 @@
       </ns0:c>
       <ns0:c r="D83" s="1">
         <ns0:f>ROUND(D82*10,0)</ns0:f>
-        <ns0:v>1.1029288629916916e+70</ns0:v>
+        <ns0:v>9.773009152270435e+78</ns0:v>
       </ns0:c>
       <ns0:c r="E83" s="1">
         <ns0:f>D83</ns0:f>
-        <ns0:v>1.1029288629916916e+70</ns0:v>
+        <ns0:v>9.773009152270435e+78</ns0:v>
       </ns0:c>
       <ns0:c r="F83" s="1">
         <ns0:f>ROUND(F82*1.4,-5)</ns0:f>
@@ -3578,11 +3578,11 @@
       </ns0:c>
       <ns0:c r="D84" s="1">
         <ns0:f>ROUND(D83*20,2-INT(LOG10(ABS(D83*20))))</ns0:f>
-        <ns0:v>2.21e+71</ns0:v>
+        <ns0:v>1.95e+80</ns0:v>
       </ns0:c>
       <ns0:c r="E84" s="1">
         <ns0:f>D84</ns0:f>
-        <ns0:v>2.21e+71</ns0:v>
+        <ns0:v>1.95e+80</ns0:v>
       </ns0:c>
       <ns0:c r="F84" s="1">
         <ns0:f>ROUND(F83*1.4,-5)</ns0:f>
@@ -3610,11 +3610,11 @@
       </ns0:c>
       <ns0:c r="D85" s="1">
         <ns0:f>ROUND(D84*20,2-INT(LOG10(ABS(D84*20))))</ns0:f>
-        <ns0:v>4.42e+72</ns0:v>
+        <ns0:v>3.9e+81</ns0:v>
       </ns0:c>
       <ns0:c r="E85" s="1">
         <ns0:f>D85</ns0:f>
-        <ns0:v>4.42e+72</ns0:v>
+        <ns0:v>3.9e+81</ns0:v>
       </ns0:c>
       <ns0:c r="F85" s="1">
         <ns0:f>ROUND(F84*1.4,-5)</ns0:f>
@@ -3642,11 +3642,11 @@
       </ns0:c>
       <ns0:c r="D86" s="1">
         <ns0:f>ROUND(D85*20,2-INT(LOG10(ABS(D85*20))))</ns0:f>
-        <ns0:v>8.840000000000001e+73</ns0:v>
+        <ns0:v>7.800000000000001e+82</ns0:v>
       </ns0:c>
       <ns0:c r="E86" s="1">
         <ns0:f>D86</ns0:f>
-        <ns0:v>8.840000000000001e+73</ns0:v>
+        <ns0:v>7.800000000000001e+82</ns0:v>
       </ns0:c>
       <ns0:c r="F86" s="1">
         <ns0:f>ROUND(F85*1.4,-5)</ns0:f>
@@ -3674,11 +3674,11 @@
       </ns0:c>
       <ns0:c r="D87" s="1">
         <ns0:f>ROUND(D86*20,2-INT(LOG10(ABS(D86*20))))</ns0:f>
-        <ns0:v>1.77e+75</ns0:v>
+        <ns0:v>1.56e+84</ns0:v>
       </ns0:c>
       <ns0:c r="E87" s="1">
         <ns0:f>D87</ns0:f>
-        <ns0:v>1.77e+75</ns0:v>
+        <ns0:v>1.56e+84</ns0:v>
       </ns0:c>
       <ns0:c r="F87" s="1">
         <ns0:f>ROUND(F86*1.4,-5)</ns0:f>
@@ -3706,11 +3706,11 @@
       </ns0:c>
       <ns0:c r="D88" s="1">
         <ns0:f>ROUND(D87*20,2-INT(LOG10(ABS(D87*20))))</ns0:f>
-        <ns0:v>3.5400000000000004e+76</ns0:v>
+        <ns0:v>3.12e+85</ns0:v>
       </ns0:c>
       <ns0:c r="E88" s="1">
         <ns0:f>D88</ns0:f>
-        <ns0:v>3.5400000000000004e+76</ns0:v>
+        <ns0:v>3.12e+85</ns0:v>
       </ns0:c>
       <ns0:c r="F88" s="1">
         <ns0:f>ROUND(F87*1.4,-5)</ns0:f>
@@ -3738,11 +3738,11 @@
       </ns0:c>
       <ns0:c r="D89" s="1">
         <ns0:f>ROUND(D88*20,2-INT(LOG10(ABS(D88*20))))</ns0:f>
-        <ns0:v>7.08e+77</ns0:v>
+        <ns0:v>6.239999999999999e+86</ns0:v>
       </ns0:c>
       <ns0:c r="E89" s="1">
         <ns0:f>D89</ns0:f>
-        <ns0:v>7.08e+77</ns0:v>
+        <ns0:v>6.239999999999999e+86</ns0:v>
       </ns0:c>
       <ns0:c r="F89" s="1">
         <ns0:f>ROUND(F88*1.4,-5)</ns0:f>
@@ -3770,11 +3770,11 @@
       </ns0:c>
       <ns0:c r="D90" s="1">
         <ns0:f>ROUND(D89*20,2-INT(LOG10(ABS(D89*20))))</ns0:f>
-        <ns0:v>1.4200000000000001e+79</ns0:v>
+        <ns0:v>1.2499999999999998e+88</ns0:v>
       </ns0:c>
       <ns0:c r="E90" s="1">
         <ns0:f>D90</ns0:f>
-        <ns0:v>1.4200000000000001e+79</ns0:v>
+        <ns0:v>1.2499999999999998e+88</ns0:v>
       </ns0:c>
       <ns0:c r="F90" s="1">
         <ns0:f>ROUND(F89*1.4,-5)</ns0:f>
@@ -3802,11 +3802,11 @@
       </ns0:c>
       <ns0:c r="D91" s="1">
         <ns0:f>ROUND(D90*20,2-INT(LOG10(ABS(D90*20))))</ns0:f>
-        <ns0:v>2.84e+80</ns0:v>
+        <ns0:v>2.5e+89</ns0:v>
       </ns0:c>
       <ns0:c r="E91" s="1">
         <ns0:f>D91</ns0:f>
-        <ns0:v>2.84e+80</ns0:v>
+        <ns0:v>2.5e+89</ns0:v>
       </ns0:c>
       <ns0:c r="F91" s="1">
         <ns0:f>ROUND(F90*1.4,-5)</ns0:f>
@@ -3834,11 +3834,11 @@
       </ns0:c>
       <ns0:c r="D92" s="1">
         <ns0:f>ROUND(D91*20,2-INT(LOG10(ABS(D91*20))))</ns0:f>
-        <ns0:v>5.68e+81</ns0:v>
+        <ns0:v>5e+90</ns0:v>
       </ns0:c>
       <ns0:c r="E92" s="1">
         <ns0:f>D92</ns0:f>
-        <ns0:v>5.68e+81</ns0:v>
+        <ns0:v>5e+90</ns0:v>
       </ns0:c>
       <ns0:c r="F92" s="1">
         <ns0:f>ROUND(F91*1.4,-5)</ns0:f>
@@ -3866,11 +3866,11 @@
       </ns0:c>
       <ns0:c r="D93" s="1">
         <ns0:f>ROUND(D92*20,2-INT(LOG10(ABS(D92*20))))</ns0:f>
-        <ns0:v>1.14e+83</ns0:v>
+        <ns0:v>1e+92</ns0:v>
       </ns0:c>
       <ns0:c r="E93" s="1">
         <ns0:f>D93</ns0:f>
-        <ns0:v>1.14e+83</ns0:v>
+        <ns0:v>1e+92</ns0:v>
       </ns0:c>
       <ns0:c r="F93" s="1">
         <ns0:f>ROUND(F92*1.4,-5)</ns0:f>
@@ -3898,11 +3898,11 @@
       </ns0:c>
       <ns0:c r="D94" s="1">
         <ns0:f>ROUND(D93*20,2-INT(LOG10(ABS(D93*20))))</ns0:f>
-        <ns0:v>2.2800000000000002e+84</ns0:v>
+        <ns0:v>1.9999999999999999e+93</ns0:v>
       </ns0:c>
       <ns0:c r="E94" s="1">
         <ns0:f>D94</ns0:f>
-        <ns0:v>2.2800000000000002e+84</ns0:v>
+        <ns0:v>1.9999999999999999e+93</ns0:v>
       </ns0:c>
       <ns0:c r="F94" s="1">
         <ns0:f>ROUND(F93*1.4,-5)</ns0:f>
@@ -3930,11 +3930,11 @@
       </ns0:c>
       <ns0:c r="D95" s="1">
         <ns0:f>ROUND(D94*20,2-INT(LOG10(ABS(D94*20))))</ns0:f>
-        <ns0:v>4.56e+85</ns0:v>
+        <ns0:v>4e+94</ns0:v>
       </ns0:c>
       <ns0:c r="E95" s="1">
         <ns0:f>D95</ns0:f>
-        <ns0:v>4.56e+85</ns0:v>
+        <ns0:v>4e+94</ns0:v>
       </ns0:c>
       <ns0:c r="F95" s="1">
         <ns0:f>ROUND(F94*1.4,-5)</ns0:f>
@@ -3962,11 +3962,11 @@
       </ns0:c>
       <ns0:c r="D96" s="1">
         <ns0:f>ROUND(D95*20,2-INT(LOG10(ABS(D95*20))))</ns0:f>
-        <ns0:v>9.119999999999999e+86</ns0:v>
+        <ns0:v>8.000000000000001e+95</ns0:v>
       </ns0:c>
       <ns0:c r="E96" s="1">
         <ns0:f>D96</ns0:f>
-        <ns0:v>9.119999999999999e+86</ns0:v>
+        <ns0:v>8.000000000000001e+95</ns0:v>
       </ns0:c>
       <ns0:c r="F96" s="1">
         <ns0:f>ROUND(F95*1.4,-5)</ns0:f>
@@ -3994,11 +3994,11 @@
       </ns0:c>
       <ns0:c r="D97" s="1">
         <ns0:f>ROUND(D96*20,2-INT(LOG10(ABS(D96*20))))</ns0:f>
-        <ns0:v>1.8199999999999998e+88</ns0:v>
+        <ns0:v>1.6e+97</ns0:v>
       </ns0:c>
       <ns0:c r="E97" s="1">
         <ns0:f>D97</ns0:f>
-        <ns0:v>1.8199999999999998e+88</ns0:v>
+        <ns0:v>1.6e+97</ns0:v>
       </ns0:c>
       <ns0:c r="F97" s="1">
         <ns0:f>ROUND(F96*1.4,-5)</ns0:f>
@@ -4026,11 +4026,11 @@
       </ns0:c>
       <ns0:c r="D98" s="1">
         <ns0:f>ROUND(D97*20,2-INT(LOG10(ABS(D97*20))))</ns0:f>
-        <ns0:v>3.64e+89</ns0:v>
+        <ns0:v>3.2e+98</ns0:v>
       </ns0:c>
       <ns0:c r="E98" s="1">
         <ns0:f>D98</ns0:f>
-        <ns0:v>3.64e+89</ns0:v>
+        <ns0:v>3.2e+98</ns0:v>
       </ns0:c>
       <ns0:c r="F98" s="1">
         <ns0:f>ROUND(F97*1.4,-5)</ns0:f>
@@ -4058,11 +4058,11 @@
       </ns0:c>
       <ns0:c r="D99" s="1">
         <ns0:f>ROUND(D98*20,2-INT(LOG10(ABS(D98*20))))</ns0:f>
-        <ns0:v>7.280000000000001e+90</ns0:v>
+        <ns0:v>6.4e+99</ns0:v>
       </ns0:c>
       <ns0:c r="E99" s="1">
         <ns0:f>D99</ns0:f>
-        <ns0:v>7.280000000000001e+90</ns0:v>
+        <ns0:v>6.4e+99</ns0:v>
       </ns0:c>
       <ns0:c r="F99" s="1">
         <ns0:f>ROUND(F98*1.4,-5)</ns0:f>
@@ -4090,11 +4090,11 @@
       </ns0:c>
       <ns0:c r="D100" s="1">
         <ns0:f>ROUND(D99*20,2-INT(LOG10(ABS(D99*20))))</ns0:f>
-        <ns0:v>1.46e+92</ns0:v>
+        <ns0:v>1.28e+101</ns0:v>
       </ns0:c>
       <ns0:c r="E100" s="1">
         <ns0:f>D100</ns0:f>
-        <ns0:v>1.46e+92</ns0:v>
+        <ns0:v>1.28e+101</ns0:v>
       </ns0:c>
       <ns0:c r="F100" s="1">
         <ns0:f>ROUND(F99*1.4,-5)</ns0:f>
@@ -4122,11 +4122,11 @@
       </ns0:c>
       <ns0:c r="D101" s="1">
         <ns0:f>ROUND(D100*20,2-INT(LOG10(ABS(D100*20))))</ns0:f>
-        <ns0:v>2.9199999999999997e+93</ns0:v>
+        <ns0:v>2.56e+102</ns0:v>
       </ns0:c>
       <ns0:c r="E101" s="1">
         <ns0:f>D101</ns0:f>
-        <ns0:v>2.9199999999999997e+93</ns0:v>
+        <ns0:v>2.56e+102</ns0:v>
       </ns0:c>
       <ns0:c r="F101" s="1">
         <ns0:f>ROUND(F100*1.4,-5)</ns0:f>
@@ -4154,11 +4154,11 @@
       </ns0:c>
       <ns0:c r="D102" s="1">
         <ns0:f>ROUND(D101*20,2-INT(LOG10(ABS(D101*20))))</ns0:f>
-        <ns0:v>5.84e+94</ns0:v>
+        <ns0:v>5.12e+103</ns0:v>
       </ns0:c>
       <ns0:c r="E102" s="1">
         <ns0:f>D102</ns0:f>
-        <ns0:v>5.84e+94</ns0:v>
+        <ns0:v>5.12e+103</ns0:v>
       </ns0:c>
       <ns0:c r="F102" s="1">
         <ns0:f>ROUND(F101*1.4,-5)</ns0:f>
@@ -4186,11 +4186,11 @@
       </ns0:c>
       <ns0:c r="D103" s="1">
         <ns0:f>ROUND(D102*20,2-INT(LOG10(ABS(D102*20))))</ns0:f>
-        <ns0:v>1.17e+96</ns0:v>
+        <ns0:v>1.02e+105</ns0:v>
       </ns0:c>
       <ns0:c r="E103" s="1">
         <ns0:f>D103</ns0:f>
-        <ns0:v>1.17e+96</ns0:v>
+        <ns0:v>1.02e+105</ns0:v>
       </ns0:c>
       <ns0:c r="F103" s="1">
         <ns0:f>ROUND(F102*1.4,-5)</ns0:f>
@@ -4218,11 +4218,11 @@
       </ns0:c>
       <ns0:c r="D104" s="1">
         <ns0:f>ROUND(D103*20,2-INT(LOG10(ABS(D103*20))))</ns0:f>
-        <ns0:v>2.34e+97</ns0:v>
+        <ns0:v>2.04e+106</ns0:v>
       </ns0:c>
       <ns0:c r="E104" s="1">
         <ns0:f>D104</ns0:f>
-        <ns0:v>2.34e+97</ns0:v>
+        <ns0:v>2.04e+106</ns0:v>
       </ns0:c>
       <ns0:c r="F104" s="1">
         <ns0:f>ROUND(F103*1.4,-5)</ns0:f>
@@ -4250,11 +4250,11 @@
       </ns0:c>
       <ns0:c r="D105" s="1">
         <ns0:f>ROUND(D104*20,2-INT(LOG10(ABS(D104*20))))</ns0:f>
-        <ns0:v>4.6800000000000005e+98</ns0:v>
+        <ns0:v>4.0800000000000004e+107</ns0:v>
       </ns0:c>
       <ns0:c r="E105" s="1">
         <ns0:f>D105</ns0:f>
-        <ns0:v>4.6800000000000005e+98</ns0:v>
+        <ns0:v>4.0800000000000004e+107</ns0:v>
       </ns0:c>
       <ns0:c r="F105" s="1">
         <ns0:f>ROUND(F104*1.4,-5)</ns0:f>
@@ -4282,11 +4282,11 @@
       </ns0:c>
       <ns0:c r="D106" s="1">
         <ns0:f>ROUND(D105*20,2-INT(LOG10(ABS(D105*20))))</ns0:f>
-        <ns0:v>9.36e+99</ns0:v>
+        <ns0:v>8.16e+108</ns0:v>
       </ns0:c>
       <ns0:c r="E106" s="1">
         <ns0:f>D106</ns0:f>
-        <ns0:v>9.36e+99</ns0:v>
+        <ns0:v>8.16e+108</ns0:v>
       </ns0:c>
       <ns0:c r="F106" s="1">
         <ns0:f>ROUND(F105*1.4,-5)</ns0:f>
@@ -4314,11 +4314,11 @@
       </ns0:c>
       <ns0:c r="D107" s="1">
         <ns0:f>ROUND(D106*20,2-INT(LOG10(ABS(D106*20))))</ns0:f>
-        <ns0:v>1.87e+101</ns0:v>
+        <ns0:v>1.63e+110</ns0:v>
       </ns0:c>
       <ns0:c r="E107" s="1">
         <ns0:f>D107</ns0:f>
-        <ns0:v>1.87e+101</ns0:v>
+        <ns0:v>1.63e+110</ns0:v>
       </ns0:c>
       <ns0:c r="F107" s="1">
         <ns0:f>ROUND(F106*1.4,-5)</ns0:f>
@@ -4346,11 +4346,11 @@
       </ns0:c>
       <ns0:c r="D108" s="1">
         <ns0:f>ROUND(D107*20,2-INT(LOG10(ABS(D107*20))))</ns0:f>
-        <ns0:v>3.74e+102</ns0:v>
+        <ns0:v>3.26e+111</ns0:v>
       </ns0:c>
       <ns0:c r="E108" s="1">
         <ns0:f>D108</ns0:f>
-        <ns0:v>3.74e+102</ns0:v>
+        <ns0:v>3.26e+111</ns0:v>
       </ns0:c>
       <ns0:c r="F108" s="1">
         <ns0:f>ROUND(F107*1.4,-5)</ns0:f>
@@ -4378,11 +4378,11 @@
       </ns0:c>
       <ns0:c r="D109" s="1">
         <ns0:f>ROUND(D108*20,2-INT(LOG10(ABS(D108*20))))</ns0:f>
-        <ns0:v>7.48e+103</ns0:v>
+        <ns0:v>6.52e+112</ns0:v>
       </ns0:c>
       <ns0:c r="E109" s="1">
         <ns0:f>D109</ns0:f>
-        <ns0:v>7.48e+103</ns0:v>
+        <ns0:v>6.52e+112</ns0:v>
       </ns0:c>
       <ns0:c r="F109" s="1">
         <ns0:f>ROUND(F108*1.4,-5)</ns0:f>
@@ -4410,11 +4410,11 @@
       </ns0:c>
       <ns0:c r="D110" s="1">
         <ns0:f>ROUND(D109*20,2-INT(LOG10(ABS(D109*20))))</ns0:f>
-        <ns0:v>1.5e+105</ns0:v>
+        <ns0:v>1.3e+114</ns0:v>
       </ns0:c>
       <ns0:c r="E110" s="1">
         <ns0:f>D110</ns0:f>
-        <ns0:v>1.5e+105</ns0:v>
+        <ns0:v>1.3e+114</ns0:v>
       </ns0:c>
       <ns0:c r="F110" s="1">
         <ns0:f>ROUND(F109*1.4,-5)</ns0:f>
@@ -4442,11 +4442,11 @@
       </ns0:c>
       <ns0:c r="D111" s="1">
         <ns0:f>ROUND(D110*20,2-INT(LOG10(ABS(D110*20))))</ns0:f>
-        <ns0:v>3e+106</ns0:v>
+        <ns0:v>2.6e+115</ns0:v>
       </ns0:c>
       <ns0:c r="E111" s="1">
         <ns0:f>D111</ns0:f>
-        <ns0:v>3e+106</ns0:v>
+        <ns0:v>2.6e+115</ns0:v>
       </ns0:c>
       <ns0:c r="F111" s="1">
         <ns0:f>ROUND(F110*1.4,-5)</ns0:f>
@@ -4474,11 +4474,11 @@
       </ns0:c>
       <ns0:c r="D112" s="1">
         <ns0:f>ROUND(D111*20,2-INT(LOG10(ABS(D111*20))))</ns0:f>
-        <ns0:v>6e+107</ns0:v>
+        <ns0:v>5.2e+116</ns0:v>
       </ns0:c>
       <ns0:c r="E112" s="1">
         <ns0:f>D112</ns0:f>
-        <ns0:v>6e+107</ns0:v>
+        <ns0:v>5.2e+116</ns0:v>
       </ns0:c>
       <ns0:c r="F112" s="1">
         <ns0:f>ROUND(F111*1.4,-5)</ns0:f>
@@ -4506,11 +4506,11 @@
       </ns0:c>
       <ns0:c r="D113" s="1">
         <ns0:f>ROUND(D112*20,2-INT(LOG10(ABS(D112*20))))</ns0:f>
-        <ns0:v>1.2e+109</ns0:v>
+        <ns0:v>1.04e+118</ns0:v>
       </ns0:c>
       <ns0:c r="E113" s="1">
         <ns0:f>D113</ns0:f>
-        <ns0:v>1.2e+109</ns0:v>
+        <ns0:v>1.04e+118</ns0:v>
       </ns0:c>
       <ns0:c r="F113" s="1">
         <ns0:f>ROUND(F112*1.4,-5)</ns0:f>
@@ -4538,11 +4538,11 @@
       </ns0:c>
       <ns0:c r="D114" s="1">
         <ns0:f>ROUND(D113*20,2-INT(LOG10(ABS(D113*20))))</ns0:f>
-        <ns0:v>2.3999999999999998e+110</ns0:v>
+        <ns0:v>2.0799999999999998e+119</ns0:v>
       </ns0:c>
       <ns0:c r="E114" s="1">
         <ns0:f>D114</ns0:f>
-        <ns0:v>2.3999999999999998e+110</ns0:v>
+        <ns0:v>2.0799999999999998e+119</ns0:v>
       </ns0:c>
       <ns0:c r="F114" s="1">
         <ns0:f>ROUND(F113*1.4,-5)</ns0:f>
@@ -4570,11 +4570,11 @@
       </ns0:c>
       <ns0:c r="D115" s="1">
         <ns0:f>ROUND(D114*20,2-INT(LOG10(ABS(D114*20))))</ns0:f>
-        <ns0:v>4.8e+111</ns0:v>
+        <ns0:v>4.16e+120</ns0:v>
       </ns0:c>
       <ns0:c r="E115" s="1">
         <ns0:f>D115</ns0:f>
-        <ns0:v>4.8e+111</ns0:v>
+        <ns0:v>4.16e+120</ns0:v>
       </ns0:c>
       <ns0:c r="F115" s="1">
         <ns0:f>ROUND(F114*1.4,-5)</ns0:f>
@@ -4602,11 +4602,11 @@
       </ns0:c>
       <ns0:c r="D116" s="1">
         <ns0:f>ROUND(D115*20,2-INT(LOG10(ABS(D115*20))))</ns0:f>
-        <ns0:v>9.6e+112</ns0:v>
+        <ns0:v>8.32e+121</ns0:v>
       </ns0:c>
       <ns0:c r="E116" s="1">
         <ns0:f>D116</ns0:f>
-        <ns0:v>9.6e+112</ns0:v>
+        <ns0:v>8.32e+121</ns0:v>
       </ns0:c>
       <ns0:c r="F116" s="1">
         <ns0:f>ROUND(F115*1.4,-5)</ns0:f>
@@ -4634,11 +4634,11 @@
       </ns0:c>
       <ns0:c r="D117" s="1">
         <ns0:f>ROUND(D116*20,2-INT(LOG10(ABS(D116*20))))</ns0:f>
-        <ns0:v>1.9200000000000001e+114</ns0:v>
+        <ns0:v>1.66e+123</ns0:v>
       </ns0:c>
       <ns0:c r="E117" s="1">
         <ns0:f>D117</ns0:f>
-        <ns0:v>1.9200000000000001e+114</ns0:v>
+        <ns0:v>1.66e+123</ns0:v>
       </ns0:c>
       <ns0:c r="F117" s="1">
         <ns0:f>ROUND(F116*1.4,-5)</ns0:f>
@@ -4666,11 +4666,11 @@
       </ns0:c>
       <ns0:c r="D118" s="1">
         <ns0:f>ROUND(D117*20,2-INT(LOG10(ABS(D117*20))))</ns0:f>
-        <ns0:v>3.84e+115</ns0:v>
+        <ns0:v>3.32e+124</ns0:v>
       </ns0:c>
       <ns0:c r="E118" s="1">
         <ns0:f>D118</ns0:f>
-        <ns0:v>3.84e+115</ns0:v>
+        <ns0:v>3.32e+124</ns0:v>
       </ns0:c>
       <ns0:c r="F118" s="1">
         <ns0:f>ROUND(F117*1.4,-5)</ns0:f>
@@ -4698,11 +4698,11 @@
       </ns0:c>
       <ns0:c r="D119" s="1">
         <ns0:f>ROUND(D118*20,2-INT(LOG10(ABS(D118*20))))</ns0:f>
-        <ns0:v>7.68e+116</ns0:v>
+        <ns0:v>6.6399999999999994e+125</ns0:v>
       </ns0:c>
       <ns0:c r="E119" s="1">
         <ns0:f>D119</ns0:f>
-        <ns0:v>7.68e+116</ns0:v>
+        <ns0:v>6.6399999999999994e+125</ns0:v>
       </ns0:c>
       <ns0:c r="F119" s="1">
         <ns0:f>ROUND(F118*1.4,-5)</ns0:f>
@@ -4730,11 +4730,11 @@
       </ns0:c>
       <ns0:c r="D120" s="1">
         <ns0:f>ROUND(D119*20,2-INT(LOG10(ABS(D119*20))))</ns0:f>
-        <ns0:v>1.54e+118</ns0:v>
+        <ns0:v>1.33e+127</ns0:v>
       </ns0:c>
       <ns0:c r="E120" s="1">
         <ns0:f>D120</ns0:f>
-        <ns0:v>1.54e+118</ns0:v>
+        <ns0:v>1.33e+127</ns0:v>
       </ns0:c>
       <ns0:c r="F120" s="1">
         <ns0:f>ROUND(F119*1.4,-5)</ns0:f>
@@ -4762,11 +4762,11 @@
       </ns0:c>
       <ns0:c r="D121" s="1">
         <ns0:f>ROUND(D120*20,2-INT(LOG10(ABS(D120*20))))</ns0:f>
-        <ns0:v>3.08e+119</ns0:v>
+        <ns0:v>2.66e+128</ns0:v>
       </ns0:c>
       <ns0:c r="E121" s="1">
         <ns0:f>D121</ns0:f>
-        <ns0:v>3.08e+119</ns0:v>
+        <ns0:v>2.66e+128</ns0:v>
       </ns0:c>
       <ns0:c r="F121" s="1">
         <ns0:f>ROUND(F120*1.4,-5)</ns0:f>
@@ -4794,11 +4794,11 @@
       </ns0:c>
       <ns0:c r="D122" s="1">
         <ns0:f>ROUND(D121*20,2-INT(LOG10(ABS(D121*20))))</ns0:f>
-        <ns0:v>6.16e+120</ns0:v>
+        <ns0:v>5.32e+129</ns0:v>
       </ns0:c>
       <ns0:c r="E122" s="1">
         <ns0:f>D122</ns0:f>
-        <ns0:v>6.16e+120</ns0:v>
+        <ns0:v>5.32e+129</ns0:v>
       </ns0:c>
       <ns0:c r="F122" s="1">
         <ns0:f>ROUND(F121*1.4,-5)</ns0:f>
@@ -4826,11 +4826,11 @@
       </ns0:c>
       <ns0:c r="D123" s="1">
         <ns0:f>ROUND(D122*20,2-INT(LOG10(ABS(D122*20))))</ns0:f>
-        <ns0:v>1.2300000000000001e+122</ns0:v>
+        <ns0:v>1.0600000000000001e+131</ns0:v>
       </ns0:c>
       <ns0:c r="E123" s="1">
         <ns0:f>D123</ns0:f>
-        <ns0:v>1.2300000000000001e+122</ns0:v>
+        <ns0:v>1.0600000000000001e+131</ns0:v>
       </ns0:c>
       <ns0:c r="F123" s="1">
         <ns0:f>ROUND(F122*1.4,-5)</ns0:f>
@@ -4858,11 +4858,11 @@
       </ns0:c>
       <ns0:c r="D124" s="1">
         <ns0:f>ROUND(D123*20,2-INT(LOG10(ABS(D123*20))))</ns0:f>
-        <ns0:v>2.46e+123</ns0:v>
+        <ns0:v>2.12e+132</ns0:v>
       </ns0:c>
       <ns0:c r="E124" s="1">
         <ns0:f>D124</ns0:f>
-        <ns0:v>2.46e+123</ns0:v>
+        <ns0:v>2.12e+132</ns0:v>
       </ns0:c>
       <ns0:c r="F124" s="1">
         <ns0:f>ROUND(F123*1.4,-5)</ns0:f>
@@ -4890,11 +4890,11 @@
       </ns0:c>
       <ns0:c r="D125" s="1">
         <ns0:f>ROUND(D124*20,2-INT(LOG10(ABS(D124*20))))</ns0:f>
-        <ns0:v>4.92e+124</ns0:v>
+        <ns0:v>4.24e+133</ns0:v>
       </ns0:c>
       <ns0:c r="E125" s="1">
         <ns0:f>D125</ns0:f>
-        <ns0:v>4.92e+124</ns0:v>
+        <ns0:v>4.24e+133</ns0:v>
       </ns0:c>
       <ns0:c r="F125" s="1">
         <ns0:f>ROUND(F124*1.4,-5)</ns0:f>
@@ -4922,11 +4922,11 @@
       </ns0:c>
       <ns0:c r="D126" s="1">
         <ns0:f>ROUND(D125*20,2-INT(LOG10(ABS(D125*20))))</ns0:f>
-        <ns0:v>9.839999999999999e+125</ns0:v>
+        <ns0:v>8.48e+134</ns0:v>
       </ns0:c>
       <ns0:c r="E126" s="1">
         <ns0:f>D126</ns0:f>
-        <ns0:v>9.839999999999999e+125</ns0:v>
+        <ns0:v>8.48e+134</ns0:v>
       </ns0:c>
       <ns0:c r="F126" s="1">
         <ns0:f>ROUND(F125*1.4,-5)</ns0:f>
@@ -4954,11 +4954,11 @@
       </ns0:c>
       <ns0:c r="D127" s="1">
         <ns0:f>ROUND(D126*20,2-INT(LOG10(ABS(D126*20))))</ns0:f>
-        <ns0:v>1.9699999999999999e+127</ns0:v>
+        <ns0:v>1.7e+136</ns0:v>
       </ns0:c>
       <ns0:c r="E127" s="1">
         <ns0:f>D127</ns0:f>
-        <ns0:v>1.9699999999999999e+127</ns0:v>
+        <ns0:v>1.7e+136</ns0:v>
       </ns0:c>
       <ns0:c r="F127" s="1">
         <ns0:f>ROUND(F126*1.4,-5)</ns0:f>
@@ -4986,11 +4986,11 @@
       </ns0:c>
       <ns0:c r="D128" s="1">
         <ns0:f>ROUND(D127*20,2-INT(LOG10(ABS(D127*20))))</ns0:f>
-        <ns0:v>3.94e+128</ns0:v>
+        <ns0:v>3.4e+137</ns0:v>
       </ns0:c>
       <ns0:c r="E128" s="1">
         <ns0:f>D128</ns0:f>
-        <ns0:v>3.94e+128</ns0:v>
+        <ns0:v>3.4e+137</ns0:v>
       </ns0:c>
       <ns0:c r="F128" s="1">
         <ns0:f>ROUND(F127*1.4,-5)</ns0:f>
@@ -5018,11 +5018,11 @@
       </ns0:c>
       <ns0:c r="D129" s="1">
         <ns0:f>ROUND(D128*20,2-INT(LOG10(ABS(D128*20))))</ns0:f>
-        <ns0:v>7.88e+129</ns0:v>
+        <ns0:v>6.8e+138</ns0:v>
       </ns0:c>
       <ns0:c r="E129" s="1">
         <ns0:f>D129</ns0:f>
-        <ns0:v>7.88e+129</ns0:v>
+        <ns0:v>6.8e+138</ns0:v>
       </ns0:c>
       <ns0:c r="F129" s="1">
         <ns0:f>ROUND(F128*1.4,-5)</ns0:f>
@@ -5050,11 +5050,11 @@
       </ns0:c>
       <ns0:c r="D130" s="1">
         <ns0:f>ROUND(D129*20,2-INT(LOG10(ABS(D129*20))))</ns0:f>
-        <ns0:v>1.58e+131</ns0:v>
+        <ns0:v>1.3599999999999999e+140</ns0:v>
       </ns0:c>
       <ns0:c r="E130" s="1">
         <ns0:f>D130</ns0:f>
-        <ns0:v>1.58e+131</ns0:v>
+        <ns0:v>1.3599999999999999e+140</ns0:v>
       </ns0:c>
       <ns0:c r="F130" s="1">
         <ns0:f>ROUND(F129*1.4,-5)</ns0:f>
@@ -5082,11 +5082,11 @@
       </ns0:c>
       <ns0:c r="D131" s="1">
         <ns0:f>ROUND(D130*20,2-INT(LOG10(ABS(D130*20))))</ns0:f>
-        <ns0:v>3.16e+132</ns0:v>
+        <ns0:v>2.72e+141</ns0:v>
       </ns0:c>
       <ns0:c r="E131" s="1">
         <ns0:f>D131</ns0:f>
-        <ns0:v>3.16e+132</ns0:v>
+        <ns0:v>2.72e+141</ns0:v>
       </ns0:c>
       <ns0:c r="F131" s="1">
         <ns0:f>ROUND(F130*1.4,-5)</ns0:f>
@@ -5114,11 +5114,11 @@
       </ns0:c>
       <ns0:c r="D132" s="1">
         <ns0:f>ROUND(D131*20,2-INT(LOG10(ABS(D131*20))))</ns0:f>
-        <ns0:v>6.32e+133</ns0:v>
+        <ns0:v>5.44e+142</ns0:v>
       </ns0:c>
       <ns0:c r="E132" s="1">
         <ns0:f>D132</ns0:f>
-        <ns0:v>6.32e+133</ns0:v>
+        <ns0:v>5.44e+142</ns0:v>
       </ns0:c>
       <ns0:c r="F132" s="1">
         <ns0:f>ROUND(F131*1.4,-5)</ns0:f>
@@ -5146,11 +5146,11 @@
       </ns0:c>
       <ns0:c r="D133" s="1">
         <ns0:f>ROUND(D132*20,2-INT(LOG10(ABS(D132*20))))</ns0:f>
-        <ns0:v>1.2599999999999999e+135</ns0:v>
+        <ns0:v>1.0899999999999999e+144</ns0:v>
       </ns0:c>
       <ns0:c r="E133" s="1">
         <ns0:f>D133</ns0:f>
-        <ns0:v>1.2599999999999999e+135</ns0:v>
+        <ns0:v>1.0899999999999999e+144</ns0:v>
       </ns0:c>
       <ns0:c r="F133" s="1">
         <ns0:f>ROUND(F132*1.4,-5)</ns0:f>
@@ -5178,11 +5178,11 @@
       </ns0:c>
       <ns0:c r="D134" s="1">
         <ns0:f>ROUND(D133*20,2-INT(LOG10(ABS(D133*20))))</ns0:f>
-        <ns0:v>2.52e+136</ns0:v>
+        <ns0:v>2.18e+145</ns0:v>
       </ns0:c>
       <ns0:c r="E134" s="1">
         <ns0:f>D134</ns0:f>
-        <ns0:v>2.52e+136</ns0:v>
+        <ns0:v>2.18e+145</ns0:v>
       </ns0:c>
       <ns0:c r="F134" s="1">
         <ns0:f>ROUND(F133*1.4,-5)</ns0:f>
@@ -5210,11 +5210,11 @@
       </ns0:c>
       <ns0:c r="D135" s="1">
         <ns0:f>ROUND(D134*20,2-INT(LOG10(ABS(D134*20))))</ns0:f>
-        <ns0:v>5.04e+137</ns0:v>
+        <ns0:v>4.36e+146</ns0:v>
       </ns0:c>
       <ns0:c r="E135" s="1">
         <ns0:f>D135</ns0:f>
-        <ns0:v>5.04e+137</ns0:v>
+        <ns0:v>4.36e+146</ns0:v>
       </ns0:c>
       <ns0:c r="F135" s="1">
         <ns0:f>ROUND(F134*1.4,-5)</ns0:f>
@@ -5242,11 +5242,11 @@
       </ns0:c>
       <ns0:c r="D136" s="1">
         <ns0:f>ROUND(D135*20,2-INT(LOG10(ABS(D135*20))))</ns0:f>
-        <ns0:v>1.0100000000000001e+139</ns0:v>
+        <ns0:v>8.720000000000001e+147</ns0:v>
       </ns0:c>
       <ns0:c r="E136" s="1">
         <ns0:f>D136</ns0:f>
-        <ns0:v>1.0100000000000001e+139</ns0:v>
+        <ns0:v>8.720000000000001e+147</ns0:v>
       </ns0:c>
       <ns0:c r="F136" s="1">
         <ns0:f>ROUND(F135*1.4,-5)</ns0:f>
@@ -5274,11 +5274,11 @@
       </ns0:c>
       <ns0:c r="D137" s="1">
         <ns0:f>ROUND(D136*20,2-INT(LOG10(ABS(D136*20))))</ns0:f>
-        <ns0:v>2.0199999999999997e+140</ns0:v>
+        <ns0:v>1.74e+149</ns0:v>
       </ns0:c>
       <ns0:c r="E137" s="1">
         <ns0:f>D137</ns0:f>
-        <ns0:v>2.0199999999999997e+140</ns0:v>
+        <ns0:v>1.74e+149</ns0:v>
       </ns0:c>
       <ns0:c r="F137" s="1">
         <ns0:f>ROUND(F136*1.4,-5)</ns0:f>
@@ -5306,11 +5306,11 @@
       </ns0:c>
       <ns0:c r="D138" s="1">
         <ns0:f>ROUND(D137*20,2-INT(LOG10(ABS(D137*20))))</ns0:f>
-        <ns0:v>4.0399999999999996e+141</ns0:v>
+        <ns0:v>3.4800000000000004e+150</ns0:v>
       </ns0:c>
       <ns0:c r="E138" s="1">
         <ns0:f>D138</ns0:f>
-        <ns0:v>4.0399999999999996e+141</ns0:v>
+        <ns0:v>3.4800000000000004e+150</ns0:v>
       </ns0:c>
       <ns0:c r="F138" s="1">
         <ns0:f>ROUND(F137*1.4,-5)</ns0:f>
@@ -5338,11 +5338,11 @@
       </ns0:c>
       <ns0:c r="D139" s="1">
         <ns0:f>ROUND(D138*20,2-INT(LOG10(ABS(D138*20))))</ns0:f>
-        <ns0:v>8.08e+142</ns0:v>
+        <ns0:v>6.96e+151</ns0:v>
       </ns0:c>
       <ns0:c r="E139" s="1">
         <ns0:f>D139</ns0:f>
-        <ns0:v>8.08e+142</ns0:v>
+        <ns0:v>6.96e+151</ns0:v>
       </ns0:c>
       <ns0:c r="F139" s="1">
         <ns0:f>ROUND(F138*1.4,-5)</ns0:f>
@@ -5370,11 +5370,11 @@
       </ns0:c>
       <ns0:c r="D140" s="1">
         <ns0:f>ROUND(D139*20,2-INT(LOG10(ABS(D139*20))))</ns0:f>
-        <ns0:v>1.62e+144</ns0:v>
+        <ns0:v>1.39e+153</ns0:v>
       </ns0:c>
       <ns0:c r="E140" s="1">
         <ns0:f>D140</ns0:f>
-        <ns0:v>1.62e+144</ns0:v>
+        <ns0:v>1.39e+153</ns0:v>
       </ns0:c>
       <ns0:c r="F140" s="1">
         <ns0:f>ROUND(F139*1.4,-5)</ns0:f>
@@ -5402,11 +5402,11 @@
       </ns0:c>
       <ns0:c r="D141" s="1">
         <ns0:f>ROUND(D140*20,2-INT(LOG10(ABS(D140*20))))</ns0:f>
-        <ns0:v>3.24e+145</ns0:v>
+        <ns0:v>2.7799999999999996e+154</ns0:v>
       </ns0:c>
       <ns0:c r="E141" s="1">
         <ns0:f>D141</ns0:f>
-        <ns0:v>3.24e+145</ns0:v>
+        <ns0:v>2.7799999999999996e+154</ns0:v>
       </ns0:c>
       <ns0:c r="F141" s="1">
         <ns0:f>ROUND(F140*1.4,-5)</ns0:f>
@@ -5434,11 +5434,11 @@
       </ns0:c>
       <ns0:c r="D142" s="1">
         <ns0:f>ROUND(D141*20,2-INT(LOG10(ABS(D141*20))))</ns0:f>
-        <ns0:v>6.48e+146</ns0:v>
+        <ns0:v>5.56e+155</ns0:v>
       </ns0:c>
       <ns0:c r="E142" s="1">
         <ns0:f>D142</ns0:f>
-        <ns0:v>6.48e+146</ns0:v>
+        <ns0:v>5.56e+155</ns0:v>
       </ns0:c>
       <ns0:c r="F142" s="1">
         <ns0:f>ROUND(F141*1.4,-5)</ns0:f>
@@ -5466,11 +5466,11 @@
       </ns0:c>
       <ns0:c r="D143" s="1">
         <ns0:f>ROUND(D142*20,2-INT(LOG10(ABS(D142*20))))</ns0:f>
-        <ns0:v>1.3e+148</ns0:v>
+        <ns0:v>1.11e+157</ns0:v>
       </ns0:c>
       <ns0:c r="E143" s="1">
         <ns0:f>D143</ns0:f>
-        <ns0:v>1.3e+148</ns0:v>
+        <ns0:v>1.11e+157</ns0:v>
       </ns0:c>
       <ns0:c r="F143" s="1">
         <ns0:f>ROUND(F142*1.4,-5)</ns0:f>
@@ -5498,11 +5498,11 @@
       </ns0:c>
       <ns0:c r="D144" s="1">
         <ns0:f>ROUND(D143*20,2-INT(LOG10(ABS(D143*20))))</ns0:f>
-        <ns0:v>2.6000000000000002e+149</ns0:v>
+        <ns0:v>2.2199999999999997e+158</ns0:v>
       </ns0:c>
       <ns0:c r="E144" s="1">
         <ns0:f>D144</ns0:f>
-        <ns0:v>2.6000000000000002e+149</ns0:v>
+        <ns0:v>2.2199999999999997e+158</ns0:v>
       </ns0:c>
       <ns0:c r="F144" s="1">
         <ns0:f>ROUND(F143*1.4,-5)</ns0:f>
@@ -5530,11 +5530,11 @@
       </ns0:c>
       <ns0:c r="D145" s="1">
         <ns0:f>ROUND(D144*20,2-INT(LOG10(ABS(D144*20))))</ns0:f>
-        <ns0:v>5.2e+150</ns0:v>
+        <ns0:v>4.44e+159</ns0:v>
       </ns0:c>
       <ns0:c r="E145" s="1">
         <ns0:f>D145</ns0:f>
-        <ns0:v>5.2e+150</ns0:v>
+        <ns0:v>4.44e+159</ns0:v>
       </ns0:c>
       <ns0:c r="F145" s="1">
         <ns0:f>ROUND(F144*1.4,-5)</ns0:f>
@@ -5562,11 +5562,11 @@
       </ns0:c>
       <ns0:c r="D146" s="1">
         <ns0:f>ROUND(D145*20,2-INT(LOG10(ABS(D145*20))))</ns0:f>
-        <ns0:v>1.0399999999999999e+152</ns0:v>
+        <ns0:v>8.88e+160</ns0:v>
       </ns0:c>
       <ns0:c r="E146" s="1">
         <ns0:f>D146</ns0:f>
-        <ns0:v>1.0399999999999999e+152</ns0:v>
+        <ns0:v>8.88e+160</ns0:v>
       </ns0:c>
       <ns0:c r="F146" s="1">
         <ns0:f>ROUND(F145*1.4,-5)</ns0:f>
@@ -5594,11 +5594,11 @@
       </ns0:c>
       <ns0:c r="D147" s="1">
         <ns0:f>ROUND(D146*20,2-INT(LOG10(ABS(D146*20))))</ns0:f>
-        <ns0:v>2.08e+153</ns0:v>
+        <ns0:v>1.78e+162</ns0:v>
       </ns0:c>
       <ns0:c r="E147" s="1">
         <ns0:f>D147</ns0:f>
-        <ns0:v>2.08e+153</ns0:v>
+        <ns0:v>1.78e+162</ns0:v>
       </ns0:c>
       <ns0:c r="F147" s="1">
         <ns0:f>ROUND(F146*1.4,-5)</ns0:f>
@@ -5626,11 +5626,11 @@
       </ns0:c>
       <ns0:c r="D148" s="1">
         <ns0:f>ROUND(D147*20,2-INT(LOG10(ABS(D147*20))))</ns0:f>
-        <ns0:v>4.16e+154</ns0:v>
+        <ns0:v>3.56e+163</ns0:v>
       </ns0:c>
       <ns0:c r="E148" s="1">
         <ns0:f>D148</ns0:f>
-        <ns0:v>4.16e+154</ns0:v>
+        <ns0:v>3.56e+163</ns0:v>
       </ns0:c>
       <ns0:c r="F148" s="1">
         <ns0:f>ROUND(F147*1.4,-5)</ns0:f>
@@ -5658,11 +5658,11 @@
       </ns0:c>
       <ns0:c r="D149" s="1">
         <ns0:f>ROUND(D148*20,2-INT(LOG10(ABS(D148*20))))</ns0:f>
-        <ns0:v>8.32e+155</ns0:v>
+        <ns0:v>7.120000000000001e+164</ns0:v>
       </ns0:c>
       <ns0:c r="E149" s="1">
         <ns0:f>D149</ns0:f>
-        <ns0:v>8.32e+155</ns0:v>
+        <ns0:v>7.120000000000001e+164</ns0:v>
       </ns0:c>
       <ns0:c r="F149" s="1">
         <ns0:f>ROUND(F148*1.4,-5)</ns0:f>
@@ -5690,11 +5690,11 @@
       </ns0:c>
       <ns0:c r="D150" s="1">
         <ns0:f>ROUND(D149*20,2-INT(LOG10(ABS(D149*20))))</ns0:f>
-        <ns0:v>1.66e+157</ns0:v>
+        <ns0:v>1.4200000000000001e+166</ns0:v>
       </ns0:c>
       <ns0:c r="E150" s="1">
         <ns0:f>D150</ns0:f>
-        <ns0:v>1.66e+157</ns0:v>
+        <ns0:v>1.4200000000000001e+166</ns0:v>
       </ns0:c>
       <ns0:c r="F150" s="1">
         <ns0:f>ROUND(F149*1.4,-5)</ns0:f>
@@ -5722,11 +5722,11 @@
       </ns0:c>
       <ns0:c r="D151" s="1">
         <ns0:f>ROUND(D150*20,2-INT(LOG10(ABS(D150*20))))</ns0:f>
-        <ns0:v>3.3199999999999997e+158</ns0:v>
+        <ns0:v>2.84e+167</ns0:v>
       </ns0:c>
       <ns0:c r="E151" s="1">
         <ns0:f>D151</ns0:f>
-        <ns0:v>3.3199999999999997e+158</ns0:v>
+        <ns0:v>2.84e+167</ns0:v>
       </ns0:c>
       <ns0:c r="F151" s="1">
         <ns0:f>ROUND(F150*1.4,-5)</ns0:f>
@@ -5754,11 +5754,11 @@
       </ns0:c>
       <ns0:c r="D152" s="1">
         <ns0:f>ROUND(D151*20,2-INT(LOG10(ABS(D151*20))))</ns0:f>
-        <ns0:v>6.64e+159</ns0:v>
+        <ns0:v>5.68e+168</ns0:v>
       </ns0:c>
       <ns0:c r="E152" s="1">
         <ns0:f>D152</ns0:f>
-        <ns0:v>6.64e+159</ns0:v>
+        <ns0:v>5.68e+168</ns0:v>
       </ns0:c>
       <ns0:c r="F152" s="1">
         <ns0:f>ROUND(F151*1.4,-5)</ns0:f>
@@ -5786,11 +5786,11 @@
       </ns0:c>
       <ns0:c r="D153" s="1">
         <ns0:f>ROUND(D152*20,2-INT(LOG10(ABS(D152*20))))</ns0:f>
-        <ns0:v>1.3300000000000001e+161</ns0:v>
+        <ns0:v>1.1399999999999999e+170</ns0:v>
       </ns0:c>
       <ns0:c r="E153" s="1">
         <ns0:f>D153</ns0:f>
-        <ns0:v>1.3300000000000001e+161</ns0:v>
+        <ns0:v>1.1399999999999999e+170</ns0:v>
       </ns0:c>
       <ns0:c r="F153" s="1">
         <ns0:f>ROUND(F152*1.4,-5)</ns0:f>
@@ -5818,11 +5818,11 @@
       </ns0:c>
       <ns0:c r="D154" s="1">
         <ns0:f>ROUND(D153*20,2-INT(LOG10(ABS(D153*20))))</ns0:f>
-        <ns0:v>2.66e+162</ns0:v>
+        <ns0:v>2.28e+171</ns0:v>
       </ns0:c>
       <ns0:c r="E154" s="1">
         <ns0:f>D154</ns0:f>
-        <ns0:v>2.66e+162</ns0:v>
+        <ns0:v>2.28e+171</ns0:v>
       </ns0:c>
       <ns0:c r="F154" s="1">
         <ns0:f>ROUND(F153*1.4,-5)</ns0:f>
@@ -5850,11 +5850,11 @@
       </ns0:c>
       <ns0:c r="D155" s="1">
         <ns0:f>ROUND(D154*20,2-INT(LOG10(ABS(D154*20))))</ns0:f>
-        <ns0:v>5.32e+163</ns0:v>
+        <ns0:v>4.56e+172</ns0:v>
       </ns0:c>
       <ns0:c r="E155" s="1">
         <ns0:f>D155</ns0:f>
-        <ns0:v>5.32e+163</ns0:v>
+        <ns0:v>4.56e+172</ns0:v>
       </ns0:c>
       <ns0:c r="F155" s="1">
         <ns0:f>ROUND(F154*1.4,-5)</ns0:f>
@@ -5882,11 +5882,11 @@
       </ns0:c>
       <ns0:c r="D156" s="1">
         <ns0:f>ROUND(D155*20,2-INT(LOG10(ABS(D155*20))))</ns0:f>
-        <ns0:v>1.06e+165</ns0:v>
+        <ns0:v>9.12e+173</ns0:v>
       </ns0:c>
       <ns0:c r="E156" s="1">
         <ns0:f>D156</ns0:f>
-        <ns0:v>1.06e+165</ns0:v>
+        <ns0:v>9.12e+173</ns0:v>
       </ns0:c>
       <ns0:c r="F156" s="1">
         <ns0:f>ROUND(F155*1.4,-5)</ns0:f>
@@ -5914,11 +5914,11 @@
       </ns0:c>
       <ns0:c r="D157" s="1">
         <ns0:f>ROUND(D156*20,2-INT(LOG10(ABS(D156*20))))</ns0:f>
-        <ns0:v>2.12e+166</ns0:v>
+        <ns0:v>1.8199999999999998e+175</ns0:v>
       </ns0:c>
       <ns0:c r="E157" s="1">
         <ns0:f>D157</ns0:f>
-        <ns0:v>2.12e+166</ns0:v>
+        <ns0:v>1.8199999999999998e+175</ns0:v>
       </ns0:c>
       <ns0:c r="F157" s="1">
         <ns0:f>ROUND(F156*1.4,-5)</ns0:f>
@@ -5946,11 +5946,11 @@
       </ns0:c>
       <ns0:c r="D158" s="1">
         <ns0:f>ROUND(D157*20,2-INT(LOG10(ABS(D157*20))))</ns0:f>
-        <ns0:v>4.24e+167</ns0:v>
+        <ns0:v>3.64e+176</ns0:v>
       </ns0:c>
       <ns0:c r="E158" s="1">
         <ns0:f>D158</ns0:f>
-        <ns0:v>4.24e+167</ns0:v>
+        <ns0:v>3.64e+176</ns0:v>
       </ns0:c>
       <ns0:c r="F158" s="1">
         <ns0:f>ROUND(F157*1.4,-5)</ns0:f>
@@ -5978,11 +5978,11 @@
       </ns0:c>
       <ns0:c r="D159" s="1">
         <ns0:f>ROUND(D158*20,2-INT(LOG10(ABS(D158*20))))</ns0:f>
-        <ns0:v>8.48e+168</ns0:v>
+        <ns0:v>7.28e+177</ns0:v>
       </ns0:c>
       <ns0:c r="E159" s="1">
         <ns0:f>D159</ns0:f>
-        <ns0:v>8.48e+168</ns0:v>
+        <ns0:v>7.28e+177</ns0:v>
       </ns0:c>
       <ns0:c r="F159" s="1">
         <ns0:f>ROUND(F158*1.4,-5)</ns0:f>
@@ -6010,11 +6010,11 @@
       </ns0:c>
       <ns0:c r="D160" s="1">
         <ns0:f>ROUND(D159*20,2-INT(LOG10(ABS(D159*20))))</ns0:f>
-        <ns0:v>1.6999999999999998e+170</ns0:v>
+        <ns0:v>1.46e+179</ns0:v>
       </ns0:c>
       <ns0:c r="E160" s="1">
         <ns0:f>D160</ns0:f>
-        <ns0:v>1.6999999999999998e+170</ns0:v>
+        <ns0:v>1.46e+179</ns0:v>
       </ns0:c>
       <ns0:c r="F160" s="1">
         <ns0:f>ROUND(F159*1.4,-5)</ns0:f>
@@ -6042,11 +6042,11 @@
       </ns0:c>
       <ns0:c r="D161" s="1">
         <ns0:f>ROUND(D160*20,2-INT(LOG10(ABS(D160*20))))</ns0:f>
-        <ns0:v>3.4e+171</ns0:v>
+        <ns0:v>2.9200000000000003e+180</ns0:v>
       </ns0:c>
       <ns0:c r="E161" s="1">
         <ns0:f>D161</ns0:f>
-        <ns0:v>3.4e+171</ns0:v>
+        <ns0:v>2.9200000000000003e+180</ns0:v>
       </ns0:c>
       <ns0:c r="F161" s="1">
         <ns0:f>ROUND(F160*1.4,-5)</ns0:f>
@@ -6074,11 +6074,11 @@
       </ns0:c>
       <ns0:c r="D162" s="1">
         <ns0:f>ROUND(D161*20,2-INT(LOG10(ABS(D161*20))))</ns0:f>
-        <ns0:v>6.8e+172</ns0:v>
+        <ns0:v>5.8399999999999996e+181</ns0:v>
       </ns0:c>
       <ns0:c r="E162" s="1">
         <ns0:f>D162</ns0:f>
-        <ns0:v>6.8e+172</ns0:v>
+        <ns0:v>5.8399999999999996e+181</ns0:v>
       </ns0:c>
       <ns0:c r="F162" s="1">
         <ns0:f>ROUND(F161*1.4,-5)</ns0:f>
@@ -6106,11 +6106,11 @@
       </ns0:c>
       <ns0:c r="D163" s="1">
         <ns0:f>ROUND(D162*20,2-INT(LOG10(ABS(D162*20))))</ns0:f>
-        <ns0:v>1.3599999999999999e+174</ns0:v>
+        <ns0:v>1.17e+183</ns0:v>
       </ns0:c>
       <ns0:c r="E163" s="1">
         <ns0:f>D163</ns0:f>
-        <ns0:v>1.3599999999999999e+174</ns0:v>
+        <ns0:v>1.17e+183</ns0:v>
       </ns0:c>
       <ns0:c r="F163" s="1">
         <ns0:f>ROUND(F162*1.4,-5)</ns0:f>
@@ -6138,11 +6138,11 @@
       </ns0:c>
       <ns0:c r="D164" s="1">
         <ns0:f>ROUND(D163*20,2-INT(LOG10(ABS(D163*20))))</ns0:f>
-        <ns0:v>2.7199999999999997e+175</ns0:v>
+        <ns0:v>2.3399999999999998e+184</ns0:v>
       </ns0:c>
       <ns0:c r="E164" s="1">
         <ns0:f>D164</ns0:f>
-        <ns0:v>2.7199999999999997e+175</ns0:v>
+        <ns0:v>2.3399999999999998e+184</ns0:v>
       </ns0:c>
       <ns0:c r="F164" s="1">
         <ns0:f>ROUND(F163*1.4,-5)</ns0:f>
@@ -6170,11 +6170,11 @@
       </ns0:c>
       <ns0:c r="D165" s="1">
         <ns0:f>ROUND(D164*20,2-INT(LOG10(ABS(D164*20))))</ns0:f>
-        <ns0:v>5.44e+176</ns0:v>
+        <ns0:v>4.68e+185</ns0:v>
       </ns0:c>
       <ns0:c r="E165" s="1">
         <ns0:f>D165</ns0:f>
-        <ns0:v>5.44e+176</ns0:v>
+        <ns0:v>4.68e+185</ns0:v>
       </ns0:c>
       <ns0:c r="F165" s="1">
         <ns0:f>ROUND(F164*1.4,-5)</ns0:f>
@@ -6202,11 +6202,11 @@
       </ns0:c>
       <ns0:c r="D166" s="1">
         <ns0:f>ROUND(D165*20,2-INT(LOG10(ABS(D165*20))))</ns0:f>
-        <ns0:v>1.09e+178</ns0:v>
+        <ns0:v>9.359999999999999e+186</ns0:v>
       </ns0:c>
       <ns0:c r="E166" s="1">
         <ns0:f>D166</ns0:f>
-        <ns0:v>1.09e+178</ns0:v>
+        <ns0:v>9.359999999999999e+186</ns0:v>
       </ns0:c>
       <ns0:c r="F166" s="1">
         <ns0:f>ROUND(F165*1.4,-5)</ns0:f>
@@ -6234,11 +6234,11 @@
       </ns0:c>
       <ns0:c r="D167" s="1">
         <ns0:f>ROUND(D166*20,2-INT(LOG10(ABS(D166*20))))</ns0:f>
-        <ns0:v>2.1800000000000002e+179</ns0:v>
+        <ns0:v>1.87e+188</ns0:v>
       </ns0:c>
       <ns0:c r="E167" s="1">
         <ns0:f>D167</ns0:f>
-        <ns0:v>2.1800000000000002e+179</ns0:v>
+        <ns0:v>1.87e+188</ns0:v>
       </ns0:c>
       <ns0:c r="F167" s="1">
         <ns0:f>ROUND(F166*1.4,-5)</ns0:f>
@@ -6266,11 +6266,11 @@
       </ns0:c>
       <ns0:c r="D168" s="1">
         <ns0:f>ROUND(D167*20,2-INT(LOG10(ABS(D167*20))))</ns0:f>
-        <ns0:v>4.36e+180</ns0:v>
+        <ns0:v>3.74e+189</ns0:v>
       </ns0:c>
       <ns0:c r="E168" s="1">
         <ns0:f>D168</ns0:f>
-        <ns0:v>4.36e+180</ns0:v>
+        <ns0:v>3.74e+189</ns0:v>
       </ns0:c>
       <ns0:c r="F168" s="1">
         <ns0:f>ROUND(F167*1.4,-5)</ns0:f>
@@ -6298,11 +6298,11 @@
       </ns0:c>
       <ns0:c r="D169" s="1">
         <ns0:f>ROUND(D168*20,2-INT(LOG10(ABS(D168*20))))</ns0:f>
-        <ns0:v>8.72e+181</ns0:v>
+        <ns0:v>7.48e+190</ns0:v>
       </ns0:c>
       <ns0:c r="E169" s="1">
         <ns0:f>D169</ns0:f>
-        <ns0:v>8.72e+181</ns0:v>
+        <ns0:v>7.48e+190</ns0:v>
       </ns0:c>
       <ns0:c r="F169" s="1">
         <ns0:f>ROUND(F168*1.4,-5)</ns0:f>
@@ -6330,11 +6330,11 @@
       </ns0:c>
       <ns0:c r="D170" s="1">
         <ns0:f>ROUND(D169*20,2-INT(LOG10(ABS(D169*20))))</ns0:f>
-        <ns0:v>1.74e+183</ns0:v>
+        <ns0:v>1.5e+192</ns0:v>
       </ns0:c>
       <ns0:c r="E170" s="1">
         <ns0:f>D170</ns0:f>
-        <ns0:v>1.74e+183</ns0:v>
+        <ns0:v>1.5e+192</ns0:v>
       </ns0:c>
       <ns0:c r="F170" s="1">
         <ns0:f>ROUND(F169*1.4,-5)</ns0:f>
@@ -6362,11 +6362,11 @@
       </ns0:c>
       <ns0:c r="D171" s="1">
         <ns0:f>ROUND(D170*20,2-INT(LOG10(ABS(D170*20))))</ns0:f>
-        <ns0:v>3.48e+184</ns0:v>
+        <ns0:v>3e+193</ns0:v>
       </ns0:c>
       <ns0:c r="E171" s="1">
         <ns0:f>D171</ns0:f>
-        <ns0:v>3.48e+184</ns0:v>
+        <ns0:v>3e+193</ns0:v>
       </ns0:c>
       <ns0:c r="F171" s="1">
         <ns0:f>ROUND(F170*1.4,-5)</ns0:f>
@@ -6394,11 +6394,11 @@
       </ns0:c>
       <ns0:c r="D172" s="1">
         <ns0:f>ROUND(D171*20,2-INT(LOG10(ABS(D171*20))))</ns0:f>
-        <ns0:v>6.96e+185</ns0:v>
+        <ns0:v>5.999999999999999e+194</ns0:v>
       </ns0:c>
       <ns0:c r="E172" s="1">
         <ns0:f>D172</ns0:f>
-        <ns0:v>6.96e+185</ns0:v>
+        <ns0:v>5.999999999999999e+194</ns0:v>
       </ns0:c>
       <ns0:c r="F172" s="1">
         <ns0:f>ROUND(F171*1.4,-5)</ns0:f>
@@ -6426,11 +6426,11 @@
       </ns0:c>
       <ns0:c r="D173" s="1">
         <ns0:f>ROUND(D172*20,2-INT(LOG10(ABS(D172*20))))</ns0:f>
-        <ns0:v>1.39e+187</ns0:v>
+        <ns0:v>1.2e+196</ns0:v>
       </ns0:c>
       <ns0:c r="E173" s="1">
         <ns0:f>D173</ns0:f>
-        <ns0:v>1.39e+187</ns0:v>
+        <ns0:v>1.2e+196</ns0:v>
       </ns0:c>
       <ns0:c r="F173" s="1">
         <ns0:f>ROUND(F172*1.4,-5)</ns0:f>
@@ -6458,11 +6458,11 @@
       </ns0:c>
       <ns0:c r="D174" s="1">
         <ns0:f>ROUND(D173*20,2-INT(LOG10(ABS(D173*20))))</ns0:f>
-        <ns0:v>2.7800000000000002e+188</ns0:v>
+        <ns0:v>2.4e+197</ns0:v>
       </ns0:c>
       <ns0:c r="E174" s="1">
         <ns0:f>D174</ns0:f>
-        <ns0:v>2.7800000000000002e+188</ns0:v>
+        <ns0:v>2.4e+197</ns0:v>
       </ns0:c>
       <ns0:c r="F174" s="1">
         <ns0:f>ROUND(F173*1.4,-5)</ns0:f>
@@ -6490,11 +6490,11 @@
       </ns0:c>
       <ns0:c r="D175" s="1">
         <ns0:f>ROUND(D174*20,2-INT(LOG10(ABS(D174*20))))</ns0:f>
-        <ns0:v>5.56e+189</ns0:v>
+        <ns0:v>4.8e+198</ns0:v>
       </ns0:c>
       <ns0:c r="E175" s="1">
         <ns0:f>D175</ns0:f>
-        <ns0:v>5.56e+189</ns0:v>
+        <ns0:v>4.8e+198</ns0:v>
       </ns0:c>
       <ns0:c r="F175" s="1">
         <ns0:f>ROUND(F174*1.4,-5)</ns0:f>
@@ -6522,11 +6522,11 @@
       </ns0:c>
       <ns0:c r="D176" s="1">
         <ns0:f>ROUND(D175*20,2-INT(LOG10(ABS(D175*20))))</ns0:f>
-        <ns0:v>1.11e+191</ns0:v>
+        <ns0:v>9.6e+199</ns0:v>
       </ns0:c>
       <ns0:c r="E176" s="1">
         <ns0:f>D176</ns0:f>
-        <ns0:v>1.11e+191</ns0:v>
+        <ns0:v>9.6e+199</ns0:v>
       </ns0:c>
       <ns0:c r="F176" s="1">
         <ns0:f>ROUND(F175*1.4,-5)</ns0:f>
@@ -6554,11 +6554,11 @@
       </ns0:c>
       <ns0:c r="D177" s="1">
         <ns0:f>ROUND(D176*20,2-INT(LOG10(ABS(D176*20))))</ns0:f>
-        <ns0:v>2.22e+192</ns0:v>
+        <ns0:v>1.92e+201</ns0:v>
       </ns0:c>
       <ns0:c r="E177" s="1">
         <ns0:f>D177</ns0:f>
-        <ns0:v>2.22e+192</ns0:v>
+        <ns0:v>1.92e+201</ns0:v>
       </ns0:c>
       <ns0:c r="F177" s="1">
         <ns0:f>ROUND(F176*1.4,-5)</ns0:f>
@@ -6586,11 +6586,11 @@
       </ns0:c>
       <ns0:c r="D178" s="1">
         <ns0:f>ROUND(D177*20,2-INT(LOG10(ABS(D177*20))))</ns0:f>
-        <ns0:v>4.44e+193</ns0:v>
+        <ns0:v>3.84e+202</ns0:v>
       </ns0:c>
       <ns0:c r="E178" s="1">
         <ns0:f>D178</ns0:f>
-        <ns0:v>4.44e+193</ns0:v>
+        <ns0:v>3.84e+202</ns0:v>
       </ns0:c>
       <ns0:c r="F178" s="1">
         <ns0:f>ROUND(F177*1.4,-5)</ns0:f>
@@ -6618,11 +6618,11 @@
       </ns0:c>
       <ns0:c r="D179" s="1">
         <ns0:f>ROUND(D178*20,2-INT(LOG10(ABS(D178*20))))</ns0:f>
-        <ns0:v>8.879999999999999e+194</ns0:v>
+        <ns0:v>7.68e+203</ns0:v>
       </ns0:c>
       <ns0:c r="E179" s="1">
         <ns0:f>D179</ns0:f>
-        <ns0:v>8.879999999999999e+194</ns0:v>
+        <ns0:v>7.68e+203</ns0:v>
       </ns0:c>
       <ns0:c r="F179" s="1">
         <ns0:f>ROUND(F178*1.4,-5)</ns0:f>
@@ -6650,11 +6650,11 @@
       </ns0:c>
       <ns0:c r="D180" s="1">
         <ns0:f>ROUND(D179*20,2-INT(LOG10(ABS(D179*20))))</ns0:f>
-        <ns0:v>1.78e+196</ns0:v>
+        <ns0:v>1.5399999999999999e+205</ns0:v>
       </ns0:c>
       <ns0:c r="E180" s="1">
         <ns0:f>D180</ns0:f>
-        <ns0:v>1.78e+196</ns0:v>
+        <ns0:v>1.5399999999999999e+205</ns0:v>
       </ns0:c>
       <ns0:c r="F180" s="1">
         <ns0:f>ROUND(F179*1.4,-5)</ns0:f>
@@ -6682,11 +6682,11 @@
       </ns0:c>
       <ns0:c r="D181" s="1">
         <ns0:f>ROUND(D180*20,2-INT(LOG10(ABS(D180*20))))</ns0:f>
-        <ns0:v>3.56e+197</ns0:v>
+        <ns0:v>3.08e+206</ns0:v>
       </ns0:c>
       <ns0:c r="E181" s="1">
         <ns0:f>D181</ns0:f>
-        <ns0:v>3.56e+197</ns0:v>
+        <ns0:v>3.08e+206</ns0:v>
       </ns0:c>
       <ns0:c r="F181" s="1">
         <ns0:f>ROUND(F180*1.4,-5)</ns0:f>
@@ -6714,11 +6714,11 @@
       </ns0:c>
       <ns0:c r="D182" s="1">
         <ns0:f>ROUND(D181*20,2-INT(LOG10(ABS(D181*20))))</ns0:f>
-        <ns0:v>7.12e+198</ns0:v>
+        <ns0:v>6.16e+207</ns0:v>
       </ns0:c>
       <ns0:c r="E182" s="1">
         <ns0:f>D182</ns0:f>
-        <ns0:v>7.12e+198</ns0:v>
+        <ns0:v>6.16e+207</ns0:v>
       </ns0:c>
       <ns0:c r="F182" s="1">
         <ns0:f>ROUND(F181*1.4,-5)</ns0:f>
@@ -6746,11 +6746,11 @@
       </ns0:c>
       <ns0:c r="D183" s="1">
         <ns0:f>ROUND(D182*20,2-INT(LOG10(ABS(D182*20))))</ns0:f>
-        <ns0:v>1.4200000000000001e+200</ns0:v>
+        <ns0:v>1.2300000000000001e+209</ns0:v>
       </ns0:c>
       <ns0:c r="E183" s="1">
         <ns0:f>D183</ns0:f>
-        <ns0:v>1.4200000000000001e+200</ns0:v>
+        <ns0:v>1.2300000000000001e+209</ns0:v>
       </ns0:c>
       <ns0:c r="F183" s="1">
         <ns0:f>ROUND(F182*1.4,-5)</ns0:f>
@@ -6778,11 +6778,11 @@
       </ns0:c>
       <ns0:c r="D184" s="1">
         <ns0:f>ROUND(D183*20,2-INT(LOG10(ABS(D183*20))))</ns0:f>
-        <ns0:v>2.84e+201</ns0:v>
+        <ns0:v>2.4599999999999997e+210</ns0:v>
       </ns0:c>
       <ns0:c r="E184" s="1">
         <ns0:f>D184</ns0:f>
-        <ns0:v>2.84e+201</ns0:v>
+        <ns0:v>2.4599999999999997e+210</ns0:v>
       </ns0:c>
       <ns0:c r="F184" s="1">
         <ns0:f>ROUND(F183*1.4,-5)</ns0:f>
@@ -6810,11 +6810,11 @@
       </ns0:c>
       <ns0:c r="D185" s="1">
         <ns0:f>ROUND(D184*20,2-INT(LOG10(ABS(D184*20))))</ns0:f>
-        <ns0:v>5.68e+202</ns0:v>
+        <ns0:v>4.92e+211</ns0:v>
       </ns0:c>
       <ns0:c r="E185" s="1">
         <ns0:f>D185</ns0:f>
-        <ns0:v>5.68e+202</ns0:v>
+        <ns0:v>4.92e+211</ns0:v>
       </ns0:c>
       <ns0:c r="F185" s="1">
         <ns0:f>ROUND(F184*1.4,-5)</ns0:f>
@@ -6842,11 +6842,11 @@
       </ns0:c>
       <ns0:c r="D186" s="1">
         <ns0:f>ROUND(D185*20,2-INT(LOG10(ABS(D185*20))))</ns0:f>
-        <ns0:v>1.14e+204</ns0:v>
+        <ns0:v>9.84e+212</ns0:v>
       </ns0:c>
       <ns0:c r="E186" s="1">
         <ns0:f>D186</ns0:f>
-        <ns0:v>1.14e+204</ns0:v>
+        <ns0:v>9.84e+212</ns0:v>
       </ns0:c>
       <ns0:c r="F186" s="1">
         <ns0:f>ROUND(F185*1.4,-5)</ns0:f>
@@ -6874,11 +6874,11 @@
       </ns0:c>
       <ns0:c r="D187" s="1">
         <ns0:f>ROUND(D186*20,2-INT(LOG10(ABS(D186*20))))</ns0:f>
-        <ns0:v>2.28e+205</ns0:v>
+        <ns0:v>1.9700000000000001e+214</ns0:v>
       </ns0:c>
       <ns0:c r="E187" s="1">
         <ns0:f>D187</ns0:f>
-        <ns0:v>2.28e+205</ns0:v>
+        <ns0:v>1.9700000000000001e+214</ns0:v>
       </ns0:c>
       <ns0:c r="F187" s="1">
         <ns0:f>ROUND(F186*1.4,-5)</ns0:f>
@@ -6906,11 +6906,11 @@
       </ns0:c>
       <ns0:c r="D188" s="1">
         <ns0:f>ROUND(D187*20,2-INT(LOG10(ABS(D187*20))))</ns0:f>
-        <ns0:v>4.56e+206</ns0:v>
+        <ns0:v>3.94e+215</ns0:v>
       </ns0:c>
       <ns0:c r="E188" s="1">
         <ns0:f>D188</ns0:f>
-        <ns0:v>4.56e+206</ns0:v>
+        <ns0:v>3.94e+215</ns0:v>
       </ns0:c>
       <ns0:c r="F188" s="1">
         <ns0:f>ROUND(F187*1.4,-5)</ns0:f>
@@ -6938,11 +6938,11 @@
       </ns0:c>
       <ns0:c r="D189" s="1">
         <ns0:f>ROUND(D188*20,2-INT(LOG10(ABS(D188*20))))</ns0:f>
-        <ns0:v>9.12e+207</ns0:v>
+        <ns0:v>7.880000000000001e+216</ns0:v>
       </ns0:c>
       <ns0:c r="E189" s="1">
         <ns0:f>D189</ns0:f>
-        <ns0:v>9.12e+207</ns0:v>
+        <ns0:v>7.880000000000001e+216</ns0:v>
       </ns0:c>
       <ns0:c r="F189" s="1">
         <ns0:f>ROUND(F188*1.4,-5)</ns0:f>
@@ -6970,11 +6970,11 @@
       </ns0:c>
       <ns0:c r="D190" s="1">
         <ns0:f>ROUND(D189*20,2-INT(LOG10(ABS(D189*20))))</ns0:f>
-        <ns0:v>1.82e+209</ns0:v>
+        <ns0:v>1.58e+218</ns0:v>
       </ns0:c>
       <ns0:c r="E190" s="1">
         <ns0:f>D190</ns0:f>
-        <ns0:v>1.82e+209</ns0:v>
+        <ns0:v>1.58e+218</ns0:v>
       </ns0:c>
       <ns0:c r="F190" s="1">
         <ns0:f>ROUND(F189*1.4,-5)</ns0:f>
@@ -7002,11 +7002,11 @@
       </ns0:c>
       <ns0:c r="D191" s="1">
         <ns0:f>ROUND(D190*20,2-INT(LOG10(ABS(D190*20))))</ns0:f>
-        <ns0:v>3.64e+210</ns0:v>
+        <ns0:v>3.16e+219</ns0:v>
       </ns0:c>
       <ns0:c r="E191" s="1">
         <ns0:f>D191</ns0:f>
-        <ns0:v>3.64e+210</ns0:v>
+        <ns0:v>3.16e+219</ns0:v>
       </ns0:c>
       <ns0:c r="F191" s="1">
         <ns0:f>ROUND(F190*1.4,-5)</ns0:f>
@@ -7034,11 +7034,11 @@
       </ns0:c>
       <ns0:c r="D192" s="1">
         <ns0:f>ROUND(D191*20,2-INT(LOG10(ABS(D191*20))))</ns0:f>
-        <ns0:v>7.279999999999999e+211</ns0:v>
+        <ns0:v>6.319999999999999e+220</ns0:v>
       </ns0:c>
       <ns0:c r="E192" s="1">
         <ns0:f>D192</ns0:f>
-        <ns0:v>7.279999999999999e+211</ns0:v>
+        <ns0:v>6.319999999999999e+220</ns0:v>
       </ns0:c>
       <ns0:c r="F192" s="1">
         <ns0:f>ROUND(F191*1.4,-5)</ns0:f>
@@ -7066,11 +7066,11 @@
       </ns0:c>
       <ns0:c r="D193" s="1">
         <ns0:f>ROUND(D192*20,2-INT(LOG10(ABS(D192*20))))</ns0:f>
-        <ns0:v>1.46e+213</ns0:v>
+        <ns0:v>1.26e+222</ns0:v>
       </ns0:c>
       <ns0:c r="E193" s="1">
         <ns0:f>D193</ns0:f>
-        <ns0:v>1.46e+213</ns0:v>
+        <ns0:v>1.26e+222</ns0:v>
       </ns0:c>
       <ns0:c r="F193" s="1">
         <ns0:f>ROUND(F192*1.4,-5)</ns0:f>
@@ -7098,11 +7098,11 @@
       </ns0:c>
       <ns0:c r="D194" s="1">
         <ns0:f>ROUND(D193*20,2-INT(LOG10(ABS(D193*20))))</ns0:f>
-        <ns0:v>2.9200000000000003e+214</ns0:v>
+        <ns0:v>2.52e+223</ns0:v>
       </ns0:c>
       <ns0:c r="E194" s="1">
         <ns0:f>D194</ns0:f>
-        <ns0:v>2.9200000000000003e+214</ns0:v>
+        <ns0:v>2.52e+223</ns0:v>
       </ns0:c>
       <ns0:c r="F194" s="1">
         <ns0:f>ROUND(F193*1.4,-5)</ns0:f>
@@ -7130,11 +7130,11 @@
       </ns0:c>
       <ns0:c r="D195" s="1">
         <ns0:f>ROUND(D194*20,2-INT(LOG10(ABS(D194*20))))</ns0:f>
-        <ns0:v>5.84e+215</ns0:v>
+        <ns0:v>5.0399999999999996e+224</ns0:v>
       </ns0:c>
       <ns0:c r="E195" s="1">
         <ns0:f>D195</ns0:f>
-        <ns0:v>5.84e+215</ns0:v>
+        <ns0:v>5.0399999999999996e+224</ns0:v>
       </ns0:c>
       <ns0:c r="F195" s="1">
         <ns0:f>ROUND(F194*1.4,-5)</ns0:f>
@@ -7162,11 +7162,11 @@
       </ns0:c>
       <ns0:c r="D196" s="1">
         <ns0:f>ROUND(D195*20,2-INT(LOG10(ABS(D195*20))))</ns0:f>
-        <ns0:v>1.17e+217</ns0:v>
+        <ns0:v>1.01e+226</ns0:v>
       </ns0:c>
       <ns0:c r="E196" s="1">
         <ns0:f>D196</ns0:f>
-        <ns0:v>1.17e+217</ns0:v>
+        <ns0:v>1.01e+226</ns0:v>
       </ns0:c>
       <ns0:c r="F196" s="1">
         <ns0:f>ROUND(F195*1.4,-5)</ns0:f>
@@ -7194,11 +7194,11 @@
       </ns0:c>
       <ns0:c r="D197" s="1">
         <ns0:f>ROUND(D196*20,2-INT(LOG10(ABS(D196*20))))</ns0:f>
-        <ns0:v>2.34e+218</ns0:v>
+        <ns0:v>2.02e+227</ns0:v>
       </ns0:c>
       <ns0:c r="E197" s="1">
         <ns0:f>D197</ns0:f>
-        <ns0:v>2.34e+218</ns0:v>
+        <ns0:v>2.02e+227</ns0:v>
       </ns0:c>
       <ns0:c r="F197" s="1">
         <ns0:f>ROUND(F196*1.4,-5)</ns0:f>
@@ -7226,11 +7226,11 @@
       </ns0:c>
       <ns0:c r="D198" s="1">
         <ns0:f>ROUND(D197*20,2-INT(LOG10(ABS(D197*20))))</ns0:f>
-        <ns0:v>4.6799999999999996e+219</ns0:v>
+        <ns0:v>4.0400000000000005e+228</ns0:v>
       </ns0:c>
       <ns0:c r="E198" s="1">
         <ns0:f>D198</ns0:f>
-        <ns0:v>4.6799999999999996e+219</ns0:v>
+        <ns0:v>4.0400000000000005e+228</ns0:v>
       </ns0:c>
       <ns0:c r="F198" s="1">
         <ns0:f>ROUND(F197*1.4,-5)</ns0:f>
@@ -7258,11 +7258,11 @@
       </ns0:c>
       <ns0:c r="D199" s="1">
         <ns0:f>ROUND(D198*20,2-INT(LOG10(ABS(D198*20))))</ns0:f>
-        <ns0:v>9.359999999999999e+220</ns0:v>
+        <ns0:v>8.08e+229</ns0:v>
       </ns0:c>
       <ns0:c r="E199" s="1">
         <ns0:f>D199</ns0:f>
-        <ns0:v>9.359999999999999e+220</ns0:v>
+        <ns0:v>8.08e+229</ns0:v>
       </ns0:c>
       <ns0:c r="F199" s="1">
         <ns0:f>ROUND(F198*1.4,-5)</ns0:f>
@@ -7290,11 +7290,11 @@
       </ns0:c>
       <ns0:c r="D200" s="1">
         <ns0:f>ROUND(D199*20,2-INT(LOG10(ABS(D199*20))))</ns0:f>
-        <ns0:v>1.87e+222</ns0:v>
+        <ns0:v>1.6199999999999998e+231</ns0:v>
       </ns0:c>
       <ns0:c r="E200" s="1">
         <ns0:f>D200</ns0:f>
-        <ns0:v>1.87e+222</ns0:v>
+        <ns0:v>1.6199999999999998e+231</ns0:v>
       </ns0:c>
       <ns0:c r="F200" s="1">
         <ns0:f>ROUND(F199*1.4,-5)</ns0:f>
@@ -7322,11 +7322,11 @@
       </ns0:c>
       <ns0:c r="D201" s="1">
         <ns0:f>ROUND(D200*20,2-INT(LOG10(ABS(D200*20))))</ns0:f>
-        <ns0:v>3.74e+223</ns0:v>
+        <ns0:v>3.2399999999999997e+232</ns0:v>
       </ns0:c>
       <ns0:c r="E201" s="1">
         <ns0:f>D201</ns0:f>
-        <ns0:v>3.74e+223</ns0:v>
+        <ns0:v>3.2399999999999997e+232</ns0:v>
       </ns0:c>
       <ns0:c r="F201" s="1">
         <ns0:f>ROUND(F200*1.4,-5)</ns0:f>
@@ -7354,11 +7354,11 @@
       </ns0:c>
       <ns0:c r="D202" s="1">
         <ns0:f>ROUND(D201*20,2-INT(LOG10(ABS(D201*20))))</ns0:f>
-        <ns0:v>7.479999999999999e+224</ns0:v>
+        <ns0:v>6.48e+233</ns0:v>
       </ns0:c>
       <ns0:c r="E202" s="1">
         <ns0:f>D202</ns0:f>
-        <ns0:v>7.479999999999999e+224</ns0:v>
+        <ns0:v>6.48e+233</ns0:v>
       </ns0:c>
       <ns0:c r="F202" s="1">
         <ns0:f>ROUND(F201*1.4,-5)</ns0:f>
@@ -7386,11 +7386,11 @@
       </ns0:c>
       <ns0:c r="D203" s="1">
         <ns0:f>ROUND(D202*20,2-INT(LOG10(ABS(D202*20))))</ns0:f>
-        <ns0:v>1.5e+226</ns0:v>
+        <ns0:v>1.3000000000000002e+235</ns0:v>
       </ns0:c>
       <ns0:c r="E203" s="1">
         <ns0:f>D203</ns0:f>
-        <ns0:v>1.5e+226</ns0:v>
+        <ns0:v>1.3000000000000002e+235</ns0:v>
       </ns0:c>
       <ns0:c r="F203" s="1">
         <ns0:f>ROUND(F202*1.4,-5)</ns0:f>
@@ -7418,11 +7418,11 @@
       </ns0:c>
       <ns0:c r="D204" s="1">
         <ns0:f>ROUND(D203*20,2-INT(LOG10(ABS(D203*20))))</ns0:f>
-        <ns0:v>3.0000000000000003e+227</ns0:v>
+        <ns0:v>2.6e+236</ns0:v>
       </ns0:c>
       <ns0:c r="E204" s="1">
         <ns0:f>D204</ns0:f>
-        <ns0:v>3.0000000000000003e+227</ns0:v>
+        <ns0:v>2.6e+236</ns0:v>
       </ns0:c>
       <ns0:c r="F204" s="1">
         <ns0:f>ROUND(F203*1.4,-5)</ns0:f>
@@ -7450,11 +7450,11 @@
       </ns0:c>
       <ns0:c r="D205" s="1">
         <ns0:f>ROUND(D204*20,2-INT(LOG10(ABS(D204*20))))</ns0:f>
-        <ns0:v>6e+228</ns0:v>
+        <ns0:v>5.2e+237</ns0:v>
       </ns0:c>
       <ns0:c r="E205" s="1">
         <ns0:f>D205</ns0:f>
-        <ns0:v>6e+228</ns0:v>
+        <ns0:v>5.2e+237</ns0:v>
       </ns0:c>
       <ns0:c r="F205" s="1">
         <ns0:f>ROUND(F204*1.4,-5)</ns0:f>
@@ -7482,11 +7482,11 @@
       </ns0:c>
       <ns0:c r="D206" s="1">
         <ns0:f>ROUND(D205*20,2-INT(LOG10(ABS(D205*20))))</ns0:f>
-        <ns0:v>1.2e+230</ns0:v>
+        <ns0:v>1.04e+239</ns0:v>
       </ns0:c>
       <ns0:c r="E206" s="1">
         <ns0:f>D206</ns0:f>
-        <ns0:v>1.2e+230</ns0:v>
+        <ns0:v>1.04e+239</ns0:v>
       </ns0:c>
       <ns0:c r="F206" s="1">
         <ns0:f>ROUND(F205*1.4,-5)</ns0:f>
@@ -7514,11 +7514,11 @@
       </ns0:c>
       <ns0:c r="D207" s="1">
         <ns0:f>ROUND(D206*20,2-INT(LOG10(ABS(D206*20))))</ns0:f>
-        <ns0:v>2.3999999999999997e+231</ns0:v>
+        <ns0:v>2.08e+240</ns0:v>
       </ns0:c>
       <ns0:c r="E207" s="1">
         <ns0:f>D207</ns0:f>
-        <ns0:v>2.3999999999999997e+231</ns0:v>
+        <ns0:v>2.08e+240</ns0:v>
       </ns0:c>
       <ns0:c r="F207" s="1">
         <ns0:f>ROUND(F206*1.4,-5)</ns0:f>
@@ -7546,11 +7546,11 @@
       </ns0:c>
       <ns0:c r="D208" s="1">
         <ns0:f>ROUND(D207*20,2-INT(LOG10(ABS(D207*20))))</ns0:f>
-        <ns0:v>4.7999999999999997e+232</ns0:v>
+        <ns0:v>4.1599999999999994e+241</ns0:v>
       </ns0:c>
       <ns0:c r="E208" s="1">
         <ns0:f>D208</ns0:f>
-        <ns0:v>4.7999999999999997e+232</ns0:v>
+        <ns0:v>4.1599999999999994e+241</ns0:v>
       </ns0:c>
       <ns0:c r="F208" s="1">
         <ns0:f>ROUND(F207*1.4,-5)</ns0:f>
@@ -7578,11 +7578,11 @@
       </ns0:c>
       <ns0:c r="D209" s="1">
         <ns0:f>ROUND(D208*20,2-INT(LOG10(ABS(D208*20))))</ns0:f>
-        <ns0:v>9.6e+233</ns0:v>
+        <ns0:v>8.32e+242</ns0:v>
       </ns0:c>
       <ns0:c r="E209" s="1">
         <ns0:f>D209</ns0:f>
-        <ns0:v>9.6e+233</ns0:v>
+        <ns0:v>8.32e+242</ns0:v>
       </ns0:c>
       <ns0:c r="F209" s="1">
         <ns0:f>ROUND(F208*1.4,-5)</ns0:f>
@@ -7610,11 +7610,11 @@
       </ns0:c>
       <ns0:c r="D210" s="1">
         <ns0:f>ROUND(D209*20,2-INT(LOG10(ABS(D209*20))))</ns0:f>
-        <ns0:v>1.92e+235</ns0:v>
+        <ns0:v>1.66e+244</ns0:v>
       </ns0:c>
       <ns0:c r="E210" s="1">
         <ns0:f>D210</ns0:f>
-        <ns0:v>1.92e+235</ns0:v>
+        <ns0:v>1.66e+244</ns0:v>
       </ns0:c>
       <ns0:c r="F210" s="1">
         <ns0:f>ROUND(F209*1.4,-5)</ns0:f>
@@ -7642,11 +7642,11 @@
       </ns0:c>
       <ns0:c r="D211" s="1">
         <ns0:f>ROUND(D210*20,2-INT(LOG10(ABS(D210*20))))</ns0:f>
-        <ns0:v>3.8400000000000003e+236</ns0:v>
+        <ns0:v>3.32e+245</ns0:v>
       </ns0:c>
       <ns0:c r="E211" s="1">
         <ns0:f>D211</ns0:f>
-        <ns0:v>3.8400000000000003e+236</ns0:v>
+        <ns0:v>3.32e+245</ns0:v>
       </ns0:c>
       <ns0:c r="F211" s="1">
         <ns0:f>ROUND(F210*1.4,-5)</ns0:f>
@@ -7674,11 +7674,11 @@
       </ns0:c>
       <ns0:c r="D212" s="1">
         <ns0:f>ROUND(D211*20,2-INT(LOG10(ABS(D211*20))))</ns0:f>
-        <ns0:v>7.68e+237</ns0:v>
+        <ns0:v>6.640000000000001e+246</ns0:v>
       </ns0:c>
       <ns0:c r="E212" s="1">
         <ns0:f>D212</ns0:f>
-        <ns0:v>7.68e+237</ns0:v>
+        <ns0:v>6.640000000000001e+246</ns0:v>
       </ns0:c>
       <ns0:c r="F212" s="1">
         <ns0:f>ROUND(F211*1.4,-5)</ns0:f>
@@ -7706,11 +7706,11 @@
       </ns0:c>
       <ns0:c r="D213" s="1">
         <ns0:f>ROUND(D212*20,2-INT(LOG10(ABS(D212*20))))</ns0:f>
-        <ns0:v>1.54e+239</ns0:v>
+        <ns0:v>1.33e+248</ns0:v>
       </ns0:c>
       <ns0:c r="E213" s="1">
         <ns0:f>D213</ns0:f>
-        <ns0:v>1.54e+239</ns0:v>
+        <ns0:v>1.33e+248</ns0:v>
       </ns0:c>
       <ns0:c r="F213" s="1">
         <ns0:f>ROUND(F212*1.4,-5)</ns0:f>
@@ -7738,11 +7738,11 @@
       </ns0:c>
       <ns0:c r="D214" s="1">
         <ns0:f>ROUND(D213*20,2-INT(LOG10(ABS(D213*20))))</ns0:f>
-        <ns0:v>3.08e+240</ns0:v>
+        <ns0:v>2.66e+249</ns0:v>
       </ns0:c>
       <ns0:c r="E214" s="1">
         <ns0:f>D214</ns0:f>
-        <ns0:v>3.08e+240</ns0:v>
+        <ns0:v>2.66e+249</ns0:v>
       </ns0:c>
       <ns0:c r="F214" s="1">
         <ns0:f>ROUND(F213*1.4,-5)</ns0:f>
@@ -7770,11 +7770,11 @@
       </ns0:c>
       <ns0:c r="D215" s="1">
         <ns0:f>ROUND(D214*20,2-INT(LOG10(ABS(D214*20))))</ns0:f>
-        <ns0:v>6.16e+241</ns0:v>
+        <ns0:v>5.32e+250</ns0:v>
       </ns0:c>
       <ns0:c r="E215" s="1">
         <ns0:f>D215</ns0:f>
-        <ns0:v>6.16e+241</ns0:v>
+        <ns0:v>5.32e+250</ns0:v>
       </ns0:c>
       <ns0:c r="F215" s="1">
         <ns0:f>ROUND(F214*1.4,-5)</ns0:f>
@@ -7802,11 +7802,11 @@
       </ns0:c>
       <ns0:c r="D216" s="1">
         <ns0:f>ROUND(D215*20,2-INT(LOG10(ABS(D215*20))))</ns0:f>
-        <ns0:v>1.23e+243</ns0:v>
+        <ns0:v>1.0599999999999999e+252</ns0:v>
       </ns0:c>
       <ns0:c r="E216" s="1">
         <ns0:f>D216</ns0:f>
-        <ns0:v>1.23e+243</ns0:v>
+        <ns0:v>1.0599999999999999e+252</ns0:v>
       </ns0:c>
       <ns0:c r="F216" s="1">
         <ns0:f>ROUND(F215*1.4,-5)</ns0:f>
@@ -7834,11 +7834,11 @@
       </ns0:c>
       <ns0:c r="D217" s="1">
         <ns0:f>ROUND(D216*20,2-INT(LOG10(ABS(D216*20))))</ns0:f>
-        <ns0:v>2.4600000000000002e+244</ns0:v>
+        <ns0:v>2.12e+253</ns0:v>
       </ns0:c>
       <ns0:c r="E217" s="1">
         <ns0:f>D217</ns0:f>
-        <ns0:v>2.4600000000000002e+244</ns0:v>
+        <ns0:v>2.12e+253</ns0:v>
       </ns0:c>
       <ns0:c r="F217" s="1">
         <ns0:f>ROUND(F216*1.4,-5)</ns0:f>
@@ -7866,11 +7866,11 @@
       </ns0:c>
       <ns0:c r="D218" s="1">
         <ns0:f>ROUND(D217*20,2-INT(LOG10(ABS(D217*20))))</ns0:f>
-        <ns0:v>4.92e+245</ns0:v>
+        <ns0:v>4.2400000000000004e+254</ns0:v>
       </ns0:c>
       <ns0:c r="E218" s="1">
         <ns0:f>D218</ns0:f>
-        <ns0:v>4.92e+245</ns0:v>
+        <ns0:v>4.2400000000000004e+254</ns0:v>
       </ns0:c>
       <ns0:c r="F218" s="1">
         <ns0:f>ROUND(F217*1.4,-5)</ns0:f>
@@ -7898,11 +7898,11 @@
       </ns0:c>
       <ns0:c r="D219" s="1">
         <ns0:f>ROUND(D218*20,2-INT(LOG10(ABS(D218*20))))</ns0:f>
-        <ns0:v>9.840000000000001e+246</ns0:v>
+        <ns0:v>8.48e+255</ns0:v>
       </ns0:c>
       <ns0:c r="E219" s="1">
         <ns0:f>D219</ns0:f>
-        <ns0:v>9.840000000000001e+246</ns0:v>
+        <ns0:v>8.48e+255</ns0:v>
       </ns0:c>
       <ns0:c r="F219" s="1">
         <ns0:f>ROUND(F218*1.4,-5)</ns0:f>
@@ -7930,11 +7930,11 @@
       </ns0:c>
       <ns0:c r="D220" s="1">
         <ns0:f>ROUND(D219*20,2-INT(LOG10(ABS(D219*20))))</ns0:f>
-        <ns0:v>1.9700000000000002e+248</ns0:v>
+        <ns0:v>1.7e+257</ns0:v>
       </ns0:c>
       <ns0:c r="E220" s="1">
         <ns0:f>D220</ns0:f>
-        <ns0:v>1.9700000000000002e+248</ns0:v>
+        <ns0:v>1.7e+257</ns0:v>
       </ns0:c>
       <ns0:c r="F220" s="1">
         <ns0:f>ROUND(F219*1.4,-5)</ns0:f>
@@ -7962,11 +7962,11 @@
       </ns0:c>
       <ns0:c r="D221" s="1">
         <ns0:f>ROUND(D220*20,2-INT(LOG10(ABS(D220*20))))</ns0:f>
-        <ns0:v>3.94e+249</ns0:v>
+        <ns0:v>3.4000000000000002e+258</ns0:v>
       </ns0:c>
       <ns0:c r="E221" s="1">
         <ns0:f>D221</ns0:f>
-        <ns0:v>3.94e+249</ns0:v>
+        <ns0:v>3.4000000000000002e+258</ns0:v>
       </ns0:c>
       <ns0:c r="F221" s="1">
         <ns0:f>ROUND(F220*1.4,-5)</ns0:f>
@@ -7994,11 +7994,11 @@
       </ns0:c>
       <ns0:c r="D222" s="1">
         <ns0:f>ROUND(D221*20,2-INT(LOG10(ABS(D221*20))))</ns0:f>
-        <ns0:v>7.88e+250</ns0:v>
+        <ns0:v>6.8e+259</ns0:v>
       </ns0:c>
       <ns0:c r="E222" s="1">
         <ns0:f>D222</ns0:f>
-        <ns0:v>7.88e+250</ns0:v>
+        <ns0:v>6.8e+259</ns0:v>
       </ns0:c>
       <ns0:c r="F222" s="1">
         <ns0:f>ROUND(F221*1.4,-5)</ns0:f>
@@ -8026,11 +8026,11 @@
       </ns0:c>
       <ns0:c r="D223" s="1">
         <ns0:f>ROUND(D222*20,2-INT(LOG10(ABS(D222*20))))</ns0:f>
-        <ns0:v>1.5799999999999999e+252</ns0:v>
+        <ns0:v>1.36e+261</ns0:v>
       </ns0:c>
       <ns0:c r="E223" s="1">
         <ns0:f>D223</ns0:f>
-        <ns0:v>1.5799999999999999e+252</ns0:v>
+        <ns0:v>1.36e+261</ns0:v>
       </ns0:c>
       <ns0:c r="F223" s="1">
         <ns0:f>ROUND(F222*1.4,-5)</ns0:f>

</xml_diff>

<commit_message>
source: v21 calibration and real crew preparation, full evidence remains in candidate history
</commit_message>
<xml_diff>
--- a/space-battleship/config_excel/level.xlsx
+++ b/space-battleship/config_excel/level.xlsx
@@ -1581,7 +1581,7 @@
         <ns0:v>6450407.623907364</ns0:v>
       </ns0:c>
       <ns0:c r="F15" s="1" t="n">
-        <ns0:v>64017.93115473424</ns0:v>
+        <ns0:v>61725.60934115101</ns0:v>
       </ns0:c>
       <ns0:c r="G15" s="1" t="n">
         <ns0:v>3.2</ns0:v>
@@ -1609,7 +1609,7 @@
         <ns0:v>69014978.76834521</ns0:v>
       </ns0:c>
       <ns0:c r="F16" s="1" t="n">
-        <ns0:v>217178.0771275556</ns0:v>
+        <ns0:v>201903.3315579912</ns0:v>
       </ns0:c>
       <ns0:c r="G16" s="1" t="n">
         <ns0:v>3.4</ns0:v>
@@ -1637,7 +1637,7 @@
         <ns0:v>738413379.7593849</ns0:v>
       </ns0:c>
       <ns0:c r="F17" s="1" t="n">
-        <ns0:v>736767.2827605028</ns0:v>
+        <ns0:v>660422.0797386132</ns0:v>
       </ns0:c>
       <ns0:c r="G17" s="1" t="n">
         <ns0:v>3.6</ns0:v>
@@ -1665,7 +1665,7 @@
         <ns0:v>7900521439.525051</ns0:v>
       </ns0:c>
       <ns0:c r="F18" s="1" t="n">
-        <ns0:v>2499451.308004148</ns0:v>
+        <ns0:v>2160228.462010301</ns0:v>
       </ns0:c>
       <ns0:c r="G18" s="1" t="n">
         <ns0:v>3.8</ns0:v>
@@ -1693,7 +1693,7 @@
         <ns0:v>84530211298.0865</ns0:v>
       </ns0:c>
       <ns0:c r="F19" s="1" t="n">
-        <ns0:v>8479281.025721673</ns0:v>
+        <ns0:v>7066067.521434727</ns0:v>
       </ns0:c>
       <ns0:c r="G19" s="1" t="n">
         <ns0:v>4</ns0:v>
@@ -1721,7 +1721,7 @@
         <ns0:v>904415825815.2517</ns0:v>
       </ns0:c>
       <ns0:c r="F20" s="1" t="n">
-        <ns0:v>28765596.06619243</ns0:v>
+        <ns0:v>23112976.75015849</ns0:v>
       </ns0:c>
       <ns0:c r="G20" s="1" t="n">
         <ns0:v>4.2</ns0:v>
@@ -1749,7 +1749,7 @@
         <ns0:v>9676634819953.418</ns0:v>
       </ns0:c>
       <ns0:c r="F21" s="1" t="n">
-        <ns0:v>97586047.04022282</ns0:v>
+        <ns0:v>75602121.35432556</ns0:v>
       </ns0:c>
       <ns0:c r="G21" s="1" t="n">
         <ns0:v>4.4</ns0:v>
@@ -1777,7 +1777,7 @@
         <ns0:v>103533417666955.5</ns0:v>
       </ns0:c>
       <ns0:c r="F22" s="1" t="n">
-        <ns0:v>331056466.0305722</ns0:v>
+        <ns0:v>247293146.8351422</ns0:v>
       </ns0:c>
       <ns0:c r="G22" s="1" t="n">
         <ns0:v>4.6</ns0:v>
@@ -1805,7 +1805,7 @@
         <ns0:v>1107737222003781</ns0:v>
       </ns0:c>
       <ns0:c r="F23" s="1" t="n">
-        <ns0:v>1123094817.597001</ns0:v>
+        <ns0:v>808891329.7156876</ns0:v>
       </ns0:c>
       <ns0:c r="G23" s="1" t="n">
         <ns0:v>4.8</ns0:v>
@@ -1833,7 +1833,7 @@
         <ns0:v>4763067294395140</ns0:v>
       </ns0:c>
       <ns0:c r="F24" s="1" t="n">
-        <ns0:v>19316408577.56676</ns0:v>
+        <ns0:v>13912338633.23386</ns0:v>
       </ns0:c>
       <ns0:c r="G24" s="1" t="n">
         <ns0:v>5</ns0:v>
@@ -1861,7 +1861,7 @@
         <ns0:v>2.048031753406153e+16</ns0:v>
       </ns0:c>
       <ns0:c r="F25" s="1" t="n">
-        <ns0:v>83057021208.11101</ns0:v>
+        <ns0:v>59820509608.44215</ns0:v>
       </ns0:c>
       <ns0:c r="G25" s="1" t="n">
         <ns0:v>5.2</ns0:v>
@@ -1889,7 +1889,7 @@
         <ns0:v>8.80616166791431e+16</ns0:v>
       </ns0:c>
       <ns0:c r="F26" s="1" t="n">
-        <ns0:v>357129988437.7153</ns0:v>
+        <ns0:v>257217241770.2224</ns0:v>
       </ns0:c>
       <ns0:c r="G26" s="1" t="n">
         <ns0:v>5.4</ns0:v>
@@ -1917,7 +1917,7 @@
         <ns0:v>3.786488329219983e+17</ns0:v>
       </ns0:c>
       <ns0:c r="F27" s="1" t="n">
-        <ns0:v>1535593581209.092</ns0:v>
+        <ns0:v>1105987058568.022</ns0:v>
       </ns0:c>
       <ns0:c r="G27" s="1" t="n">
         <ns0:v>5.6</ns0:v>
@@ -1945,7 +1945,7 @@
         <ns0:v>1.628120673682214e+18</ns0:v>
       </ns0:c>
       <ns0:c r="F28" s="1" t="n">
-        <ns0:v>6602771324149.988</ns0:v>
+        <ns0:v>4755541911971.295</ns0:v>
       </ns0:c>
       <ns0:c r="G28" s="1" t="n">
         <ns0:v>5.8</ns0:v>
@@ -1973,7 +1973,7 @@
         <ns0:v>7.000620885625409e+18</ns0:v>
       </ns0:c>
       <ns0:c r="F29" s="1" t="n">
-        <ns0:v>28390708122581.77</ns0:v>
+        <ns0:v>20447959767085</ns0:v>
       </ns0:c>
       <ns0:c r="G29" s="1" t="n">
         <ns0:v>6</ns0:v>
@@ -2001,7 +2001,7 @@
         <ns0:v>3.010138841454234e+19</ns0:v>
       </ns0:c>
       <ns0:c r="F30" s="1" t="n">
-        <ns0:v>122074848291886.8</ns0:v>
+        <ns0:v>87922484203909.69</ns0:v>
       </ns0:c>
       <ns0:c r="G30" s="1" t="n">
         <ns0:v>6.2</ns0:v>
@@ -2029,7 +2029,7 @@
         <ns0:v>1.294304604243966e+20</ns0:v>
       </ns0:c>
       <ns0:c r="F31" s="1" t="n">
-        <ns0:v>524899503074881.8</ns0:v>
+        <ns0:v>378050588745302.9</ns0:v>
       </ns0:c>
       <ns0:c r="G31" s="1" t="n">
         <ns0:v>6.4</ns0:v>
@@ -2057,7 +2057,7 @@
         <ns0:v>5.565272888734292e+20</ns0:v>
       </ns0:c>
       <ns0:c r="F32" s="1" t="n">
-        <ns0:v>2256971785616948</ns0:v>
+        <ns0:v>1625548333225038</ns0:v>
       </ns0:c>
       <ns0:c r="G32" s="1" t="n">
         <ns0:v>6.6</ns0:v>
@@ -2085,7 +2085,7 @@
         <ns0:v>2.39296547540079e+21</ns0:v>
       </ns0:c>
       <ns0:c r="F33" s="1" t="n">
-        <ns0:v>9704565562037236</ns0:v>
+        <ns0:v>6989560292500748</ns0:v>
       </ns0:c>
       <ns0:c r="G33" s="1" t="n">
         <ns0:v>6.8</ns0:v>
@@ -2113,7 +2113,7 @@
         <ns0:v>1.512294048887176e+25</ns0:v>
       </ns0:c>
       <ns0:c r="F34" s="1" t="n">
-        <ns0:v>9704565562037236</ns0:v>
+        <ns0:v>6989560292500748</ns0:v>
       </ns0:c>
       <ns0:c r="G34" s="1" t="n">
         <ns0:v>7</ns0:v>
@@ -2141,7 +2141,7 @@
         <ns0:v>9.363726143873491e+25</ns0:v>
       </ns0:c>
       <ns0:c r="F35" s="1" t="n">
-        <ns0:v>9704565562037236</ns0:v>
+        <ns0:v>6989560292500748</ns0:v>
       </ns0:c>
       <ns0:c r="G35" s="1" t="n">
         <ns0:v>7.2</ns0:v>
@@ -2163,13 +2163,13 @@
         </ns0:is>
       </ns0:c>
       <ns0:c r="D36" s="1" t="n">
-        <ns0:v>3.589827867061663e+27</ns0:v>
+        <ns0:v>8.348792286873683e+26</ns0:v>
       </ns0:c>
       <ns0:c r="E36" s="1" t="n">
-        <ns0:v>3.589827867061663e+27</ns0:v>
+        <ns0:v>8.348792286873683e+26</ns0:v>
       </ns0:c>
       <ns0:c r="F36" s="1" t="n">
-        <ns0:v>2.012338714944041e+16</ns0:v>
+        <ns0:v>1.449355222252955e+16</ns0:v>
       </ns0:c>
       <ns0:c r="G36" s="1" t="n">
         <ns0:v>7.4</ns0:v>
@@ -2197,7 +2197,7 @@
         <ns0:v>1.376253845651405e+29</ns0:v>
       </ns0:c>
       <ns0:c r="F37" s="1" t="n">
-        <ns0:v>2.012338714944041e+16</ns0:v>
+        <ns0:v>1.449355222252955e+16</ns0:v>
       </ns0:c>
       <ns0:c r="G37" s="1" t="n">
         <ns0:v>7.6</ns0:v>
@@ -2219,13 +2219,13 @@
         </ns0:is>
       </ns0:c>
       <ns0:c r="D38" s="1" t="n">
-        <ns0:v>1.890567504244719e+31</ns0:v>
+        <ns0:v>2.268681005093663e+31</ns0:v>
       </ns0:c>
       <ns0:c r="E38" s="1" t="n">
-        <ns0:v>1.890567504244719e+31</ns0:v>
+        <ns0:v>2.268681005093663e+31</ns0:v>
       </ns0:c>
       <ns0:c r="F38" s="1" t="n">
-        <ns0:v>6.008811205403466e+16</ns0:v>
+        <ns0:v>4.327751503963766e+16</ns0:v>
       </ns0:c>
       <ns0:c r="G38" s="1" t="n">
         <ns0:v>7.8</ns0:v>
@@ -2247,13 +2247,13 @@
         </ns0:is>
       </ns0:c>
       <ns0:c r="D39" s="1" t="n">
-        <ns0:v>8.129094218776313e+31</ns0:v>
+        <ns0:v>9.754913062531577e+31</ns0:v>
       </ns0:c>
       <ns0:c r="E39" s="1" t="n">
-        <ns0:v>8.129094218776313e+31</ns0:v>
+        <ns0:v>9.754913062531577e+31</ns0:v>
       </ns0:c>
       <ns0:c r="F39" s="1" t="n">
-        <ns0:v>1.245987091552463e+17</ns0:v>
+        <ns0:v>8.974025518619266e+16</ns0:v>
       </ns0:c>
       <ns0:c r="G39" s="1" t="n">
         <ns0:v>8</ns0:v>
@@ -2275,13 +2275,13 @@
         </ns0:is>
       </ns0:c>
       <ns0:c r="D40" s="1" t="n">
-        <ns0:v>3.495361719133234e+32</ns0:v>
+        <ns0:v>4.19443406295988e+32</ns0:v>
       </ns0:c>
       <ns0:c r="E40" s="1" t="n">
-        <ns0:v>3.495361719133234e+32</ns0:v>
+        <ns0:v>4.19443406295988e+32</ns0:v>
       </ns0:c>
       <ns0:c r="F40" s="1" t="n">
-        <ns0:v>2.583678833043186e+17</ns0:v>
+        <ns0:v>1.86085393154089e+17</ns0:v>
       </ns0:c>
       <ns0:c r="G40" s="1" t="n">
         <ns0:v>8.199999999999999</ns0:v>
@@ -2303,13 +2303,13 @@
         </ns0:is>
       </ns0:c>
       <ns0:c r="D41" s="1" t="n">
-        <ns0:v>1.502941560126383e+33</ns0:v>
+        <ns0:v>1.80352987215166e+33</ns0:v>
       </ns0:c>
       <ns0:c r="E41" s="1" t="n">
-        <ns0:v>1.502941560126383e+33</ns0:v>
+        <ns0:v>1.80352987215166e+33</ns0:v>
       </ns0:c>
       <ns0:c r="F41" s="1" t="n">
-        <ns0:v>5.357516428198349e+17</ns0:v>
+        <ns0:v>3.85866671244319e+17</ns0:v>
       </ns0:c>
       <ns0:c r="G41" s="1" t="n">
         <ns0:v>8.4</ns0:v>
@@ -2331,13 +2331,13 @@
         </ns0:is>
       </ns0:c>
       <ns0:c r="D42" s="1" t="n">
-        <ns0:v>4.001331405693829e+34</ns0:v>
+        <ns0:v>4.801597686832596e+34</ns0:v>
       </ns0:c>
       <ns0:c r="E42" s="1" t="n">
-        <ns0:v>4.001331405693829e+34</ns0:v>
+        <ns0:v>4.801597686832596e+34</ns0:v>
       </ns0:c>
       <ns0:c r="F42" s="1" t="n">
-        <ns0:v>2.303634000144588e+18</ns0:v>
+        <ns0:v>1.659156057315067e+18</ns0:v>
       </ns0:c>
       <ns0:c r="G42" s="1" t="n">
         <ns0:v>8.6</ns0:v>
@@ -2359,13 +2359,13 @@
         </ns0:is>
       </ns0:c>
       <ns0:c r="D43" s="1" t="n">
-        <ns0:v>6.595981245658691e+36</ns0:v>
+        <ns0:v>7.91517749479043e+36</ns0:v>
       </ns0:c>
       <ns0:c r="E43" s="1" t="n">
-        <ns0:v>6.595981245658691e+36</ns0:v>
+        <ns0:v>7.91517749479043e+36</ns0:v>
       </ns0:c>
       <ns0:c r="F43" s="1" t="n">
-        <ns0:v>2.053943214130691e+19</ns0:v>
+        <ns0:v>1.479320206635352e+19</ns0:v>
       </ns0:c>
       <ns0:c r="G43" s="1" t="n">
         <ns0:v>8.800000000000001</ns0:v>
@@ -2387,13 +2387,13 @@
         </ns0:is>
       </ns0:c>
       <ns0:c r="D44" s="1" t="n">
-        <ns0:v>2.836151202792515e+37</ns0:v>
+        <ns0:v>3.403381443351019e+37</ns0:v>
       </ns0:c>
       <ns0:c r="E44" s="1" t="n">
-        <ns0:v>2.836151202792515e+37</ns0:v>
+        <ns0:v>3.403381443351019e+37</ns0:v>
       </ns0:c>
       <ns0:c r="F44" s="1" t="n">
-        <ns0:v>4.259056648821401e+19</ns0:v>
+        <ns0:v>3.067518380479065e+19</ns0:v>
       </ns0:c>
       <ns0:c r="G44" s="1" t="n">
         <ns0:v>9</ns0:v>
@@ -2415,13 +2415,13 @@
         </ns0:is>
       </ns0:c>
       <ns0:c r="D45" s="1" t="n">
-        <ns0:v>1.219493104289165e+38</ns0:v>
+        <ns0:v>1.463391725146999e+38</ns0:v>
       </ns0:c>
       <ns0:c r="E45" s="1" t="n">
-        <ns0:v>1.219493104289165e+38</ns0:v>
+        <ns0:v>1.463391725146999e+38</ns0:v>
       </ns0:c>
       <ns0:c r="F45" s="1" t="n">
-        <ns0:v>8.831579866996054e+19</ns0:v>
+        <ns0:v>6.360806113761387e+19</ns0:v>
       </ns0:c>
       <ns0:c r="G45" s="1" t="n">
         <ns0:v>9.199999999999999</ns0:v>
@@ -2443,13 +2443,13 @@
         </ns0:is>
       </ns0:c>
       <ns0:c r="D46" s="1" t="n">
-        <ns0:v>5.2435971324256e+38</ns0:v>
+        <ns0:v>6.292316558910722e+38</ns0:v>
       </ns0:c>
       <ns0:c r="E46" s="1" t="n">
-        <ns0:v>5.2435971324256e+38</ns0:v>
+        <ns0:v>6.292316558910722e+38</ns0:v>
       </ns0:c>
       <ns0:c r="F46" s="1" t="n">
-        <ns0:v>1.831316401220302e+20</ns0:v>
+        <ns0:v>1.318976755749561e+20</ns0:v>
       </ns0:c>
       <ns0:c r="G46" s="1" t="n">
         <ns0:v>9.4</ns0:v>
@@ -2471,13 +2471,13 @@
         </ns0:is>
       </ns0:c>
       <ns0:c r="D47" s="1" t="n">
-        <ns0:v>1.396020340472608e+40</ns0:v>
+        <ns0:v>1.67522440856713e+40</ns0:v>
       </ns0:c>
       <ns0:c r="E47" s="1" t="n">
-        <ns0:v>1.396020340472608e+40</ns0:v>
+        <ns0:v>1.67522440856713e+40</ns0:v>
       </ns0:c>
       <ns0:c r="F47" s="1" t="n">
-        <ns0:v>7.874325321093216e+20</ns0:v>
+        <ns0:v>5.671358624217739e+20</ns0:v>
       </ns0:c>
       <ns0:c r="G47" s="1" t="n">
         <ns0:v>9.6</ns0:v>
@@ -2499,13 +2499,13 @@
         </ns0:is>
       </ns0:c>
       <ns0:c r="D48" s="1" t="n">
-        <ns0:v>2.301265016742271e+42</ns0:v>
+        <ns0:v>2.761518020090726e+42</ns0:v>
       </ns0:c>
       <ns0:c r="E48" s="1" t="n">
-        <ns0:v>2.301265016742271e+42</ns0:v>
+        <ns0:v>2.761518020090726e+42</ns0:v>
       </ns0:c>
       <ns0:c r="F48" s="1" t="n">
-        <ns0:v>7.020827552511277e+21</ns0:v>
+        <ns0:v>5.056640317160829e+21</ns0:v>
       </ns0:c>
       <ns0:c r="G48" s="1" t="n">
         <ns0:v>9.800000000000001</ns0:v>
@@ -2527,13 +2527,13 @@
         </ns0:is>
       </ns0:c>
       <ns0:c r="D49" s="1" t="n">
-        <ns0:v>9.895018348443098e+42</ns0:v>
+        <ns0:v>1.187402201813172e+43</ns0:v>
       </ns0:c>
       <ns0:c r="E49" s="1" t="n">
-        <ns0:v>9.895018348443098e+42</ns0:v>
+        <ns0:v>1.187402201813172e+43</ns0:v>
       </ns0:c>
       <ns0:c r="F49" s="1" t="n">
-        <ns0:v>1.455838801288738e+22</ns0:v>
+        <ns0:v>1.048544936166469e+22</ns0:v>
       </ns0:c>
       <ns0:c r="G49" s="1" t="n">
         <ns0:v>10</ns0:v>
@@ -2555,13 +2555,13 @@
         </ns0:is>
       </ns0:c>
       <ns0:c r="D50" s="1" t="n">
-        <ns0:v>4.254676771414681e+43</ns0:v>
+        <ns0:v>5.105612125697618e+43</ns0:v>
       </ns0:c>
       <ns0:c r="E50" s="1" t="n">
-        <ns0:v>4.254676771414681e+43</ns0:v>
+        <ns0:v>5.105612125697618e+43</ns0:v>
       </ns0:c>
       <ns0:c r="F50" s="1" t="n">
-        <ns0:v>3.018827338352327e+22</ns0:v>
+        <ns0:v>2.17426277963479e+22</ns0:v>
       </ns0:c>
       <ns0:c r="G50" s="1" t="n">
         <ns0:v>10.2</ns0:v>
@@ -2583,13 +2583,13 @@
         </ns0:is>
       </ns0:c>
       <ns0:c r="D51" s="1" t="n">
-        <ns0:v>1.829433134104688e+44</ns0:v>
+        <ns0:v>2.195319760925626e+44</ns0:v>
       </ns0:c>
       <ns0:c r="E51" s="1" t="n">
-        <ns0:v>1.829433134104688e+44</ns0:v>
+        <ns0:v>2.195319760925626e+44</ns0:v>
       </ns0:c>
       <ns0:c r="F51" s="1" t="n">
-        <ns0:v>6.259840368807384e+22</ns0:v>
+        <ns0:v>4.508551299850701e+22</ns0:v>
       </ns0:c>
       <ns0:c r="G51" s="1" t="n">
         <ns0:v>10.4</ns0:v>
@@ -2611,13 +2611,13 @@
         </ns0:is>
       </ns0:c>
       <ns0:c r="D52" s="1" t="n">
-        <ns0:v>4.870560804436351e+45</ns0:v>
+        <ns0:v>5.844672965323622e+45</ns0:v>
       </ns0:c>
       <ns0:c r="E52" s="1" t="n">
-        <ns0:v>4.870560804436351e+45</ns0:v>
+        <ns0:v>5.844672965323622e+45</ns0:v>
       </ns0:c>
       <ns0:c r="F52" s="1" t="n">
-        <ns0:v>2.691616778469064e+23</ns0:v>
+        <ns0:v>1.938594534412808e+23</ns0:v>
       </ns0:c>
       <ns0:c r="G52" s="1" t="n">
         <ns0:v>10.6</ns0:v>
@@ -2639,13 +2639,13 @@
         </ns0:is>
       </ns0:c>
       <ns0:c r="D53" s="1" t="n">
-        <ns0:v>8.028859513157927e+47</ns0:v>
+        <ns0:v>9.634631415789513e+47</ns0:v>
       </ns0:c>
       <ns0:c r="E53" s="1" t="n">
-        <ns0:v>8.028859513157927e+47</ns0:v>
+        <ns0:v>9.634631415789513e+47</ns0:v>
       </ns0:c>
       <ns0:c r="F53" s="1" t="n">
-        <ns0:v>2.399872556504138e+24</ns0:v>
+        <ns0:v>1.728470359726467e+24</ns0:v>
       </ns0:c>
       <ns0:c r="G53" s="1" t="n">
         <ns0:v>10.8</ns0:v>
@@ -2667,13 +2667,13 @@
         </ns0:is>
       </ns0:c>
       <ns0:c r="D54" s="1" t="n">
-        <ns0:v>3.452262630413378e+48</ns0:v>
+        <ns0:v>4.142715156496054e+48</ns0:v>
       </ns0:c>
       <ns0:c r="E54" s="1" t="n">
-        <ns0:v>3.452262630413378e+48</ns0:v>
+        <ns0:v>4.142715156496054e+48</ns0:v>
       </ns0:c>
       <ns0:c r="F54" s="1" t="n">
-        <ns0:v>4.976375733166981e+24</ns0:v>
+        <ns0:v>3.584156137928801e+24</ns0:v>
       </ns0:c>
       <ns0:c r="G54" s="1" t="n">
         <ns0:v>11</ns0:v>
@@ -2695,13 +2695,13 @@
         </ns0:is>
       </ns0:c>
       <ns0:c r="D55" s="1" t="n">
-        <ns0:v>1.484409740862565e+49</ns0:v>
+        <ns0:v>1.781291689035079e+49</ns0:v>
       </ns0:c>
       <ns0:c r="E55" s="1" t="n">
-        <ns0:v>1.484409740862565e+49</ns0:v>
+        <ns0:v>1.781291689035079e+49</ns0:v>
       </ns0:c>
       <ns0:c r="F55" s="1" t="n">
-        <ns0:v>1.031901272029505e+25</ns0:v>
+        <ns0:v>7.43210616760916e+24</ns0:v>
       </ns0:c>
       <ns0:c r="G55" s="1" t="n">
         <ns0:v>11.2</ns0:v>
@@ -2723,13 +2723,13 @@
         </ns0:is>
       </ns0:c>
       <ns0:c r="D56" s="1" t="n">
-        <ns0:v>6.382690179350061e+49</ns0:v>
+        <ns0:v>7.659228215220075e+49</ns0:v>
       </ns0:c>
       <ns0:c r="E56" s="1" t="n">
-        <ns0:v>6.382690179350061e+49</ns0:v>
+        <ns0:v>7.659228215220075e+49</ns0:v>
       </ns0:c>
       <ns0:c r="F56" s="1" t="n">
-        <ns0:v>2.139750477680381e+25</ns0:v>
+        <ns0:v>1.541121534915435e+25</ns0:v>
       </ns0:c>
       <ns0:c r="G56" s="1" t="n">
         <ns0:v>11.4</ns0:v>
@@ -2751,13 +2751,13 @@
         </ns0:is>
       </ns0:c>
       <ns0:c r="D57" s="1" t="n">
-        <ns0:v>1.699284878734698e+51</ns0:v>
+        <ns0:v>2.039141854481638e+51</ns0:v>
       </ns0:c>
       <ns0:c r="E57" s="1" t="n">
-        <ns0:v>1.699284878734698e+51</ns0:v>
+        <ns0:v>2.039141854481638e+51</ns0:v>
       </ns0:c>
       <ns0:c r="F57" s="1" t="n">
-        <ns0:v>9.200535394098201e+25</ns0:v>
+        <ns0:v>6.626540513250619e+25</ns0:v>
       </ns0:c>
       <ns0:c r="G57" s="1" t="n">
         <ns0:v>11.6</ns0:v>
@@ -2779,13 +2779,13 @@
         </ns0:is>
       </ns0:c>
       <ns0:c r="D58" s="1" t="n">
-        <ns0:v>2.80118042090091e+53</ns0:v>
+        <ns0:v>3.361416505081092e+53</ns0:v>
       </ns0:c>
       <ns0:c r="E58" s="1" t="n">
-        <ns0:v>2.80118042090091e+53</ns0:v>
+        <ns0:v>3.361416505081092e+53</ns0:v>
       </ns0:c>
       <ns0:c r="F58" s="1" t="n">
-        <ns0:v>8.203289775151412e+26</ns0:v>
+        <ns0:v>5.908290084058036e+26</ns0:v>
       </ns0:c>
       <ns0:c r="G58" s="1" t="n">
         <ns0:v>11.8</ns0:v>
@@ -2807,13 +2807,13 @@
         </ns0:is>
       </ns0:c>
       <ns0:c r="D59" s="1" t="n">
-        <ns0:v>1.204456308180967e+54</ns0:v>
+        <ns0:v>1.44534756981716e+54</ns0:v>
       </ns0:c>
       <ns0:c r="E59" s="1" t="n">
-        <ns0:v>1.204456308180967e+54</ns0:v>
+        <ns0:v>1.44534756981716e+54</ns0:v>
       </ns0:c>
       <ns0:c r="F59" s="1" t="n">
-        <ns0:v>1.701034167775397e+27</ns0:v>
+        <ns0:v>1.225143031830274e+27</ns0:v>
       </ns0:c>
       <ns0:c r="G59" s="1" t="n">
         <ns0:v>12</ns0:v>
@@ -2835,13 +2835,13 @@
         </ns0:is>
       </ns0:c>
       <ns0:c r="D60" s="1" t="n">
-        <ns0:v>5.178941661495506e+54</ns0:v>
+        <ns0:v>6.214729993794608e+54</ns0:v>
       </ns0:c>
       <ns0:c r="E60" s="1" t="n">
-        <ns0:v>5.178941661495506e+54</ns0:v>
+        <ns0:v>6.214729993794608e+54</ns0:v>
       </ns0:c>
       <ns0:c r="F60" s="1" t="n">
-        <ns0:v>3.527264450299061e+27</ns0:v>
+        <ns0:v>2.540456590803256e+27</ns0:v>
       </ns0:c>
       <ns0:c r="G60" s="1" t="n">
         <ns0:v>12.2</ns0:v>
@@ -2863,13 +2863,13 @@
         </ns0:is>
       </ns0:c>
       <ns0:c r="D61" s="1" t="n">
-        <ns0:v>2.226850119094895e+55</ns0:v>
+        <ns0:v>2.672220142913874e+55</ns0:v>
       </ns0:c>
       <ns0:c r="E61" s="1" t="n">
-        <ns0:v>2.226850119094895e+55</ns0:v>
+        <ns0:v>2.672220142913874e+55</ns0:v>
       </ns0:c>
       <ns0:c r="F61" s="1" t="n">
-        <ns0:v>7.314135564140134e+27</ns0:v>
+        <ns0:v>5.267890786689631e+27</ns0:v>
       </ns0:c>
       <ns0:c r="G61" s="1" t="n">
         <ns0:v>12.4</ns0:v>
@@ -2891,13 +2891,13 @@
         </ns0:is>
       </ns0:c>
       <ns0:c r="D62" s="1" t="n">
-        <ns0:v>5.928617288724234e+56</ns0:v>
+        <ns0:v>7.114340746469082e+56</ns0:v>
       </ns0:c>
       <ns0:c r="E62" s="1" t="n">
-        <ns0:v>5.928617288724234e+56</ns0:v>
+        <ns0:v>7.114340746469082e+56</ns0:v>
       </ns0:c>
       <ns0:c r="F62" s="1" t="n">
-        <ns0:v>3.14494441464289e+28</ns0:v>
+        <ns0:v>2.265096614803581e+28</ns0:v>
       </ns0:c>
       <ns0:c r="G62" s="1" t="n">
         <ns0:v>12.6</ns0:v>
@@ -2919,13 +2919,13 @@
         </ns0:is>
       </ns0:c>
       <ns0:c r="D63" s="1" t="n">
-        <ns0:v>9.773009152270437e+58</ns0:v>
+        <ns0:v>1.172761098272453e+59</ns0:v>
       </ns0:c>
       <ns0:c r="E63" s="1" t="n">
-        <ns0:v>9.773009152270437e+58</ns0:v>
+        <ns0:v>1.172761098272453e+59</ns0:v>
       </ns0:c>
       <ns0:c r="F63" s="1" t="n">
-        <ns0:v>2.804064030513767e+29</ns0:v>
+        <ns0:v>2.019582894259335e+29</ns0:v>
       </ns0:c>
       <ns0:c r="G63" s="1" t="n">
         <ns0:v>12.8</ns0:v>
@@ -2948,15 +2948,15 @@
       </ns0:c>
       <ns0:c r="D64" s="1">
         <ns0:f>ROUND(D63*10,0)</ns0:f>
-        <ns0:v>9.773009152270437e+59</ns0:v>
+        <ns0:v>1.1727610982724526e+60</ns0:v>
       </ns0:c>
       <ns0:c r="E64" s="1">
         <ns0:f>D64</ns0:f>
-        <ns0:v>9.773009152270437e+59</ns0:v>
+        <ns0:v>1.1727610982724526e+60</ns0:v>
       </ns0:c>
       <ns0:c r="F64" s="1">
         <ns0:f>ROUND(F63*1.4,-5)</ns0:f>
-        <ns0:v>3.925689642719273e+29</ns0:v>
+        <ns0:v>2.8274160519630688e+29</ns0:v>
       </ns0:c>
       <ns0:c r="G64" s="1" t="n">
         <ns0:v>13</ns0:v>
@@ -2979,15 +2979,15 @@
       </ns0:c>
       <ns0:c r="D65" s="1">
         <ns0:f>ROUND(D64*10,0)</ns0:f>
-        <ns0:v>9.773009152270436e+60</ns0:v>
+        <ns0:v>1.1727610982724527e+61</ns0:v>
       </ns0:c>
       <ns0:c r="E65" s="1">
         <ns0:f>D65</ns0:f>
-        <ns0:v>9.773009152270436e+60</ns0:v>
+        <ns0:v>1.1727610982724527e+61</ns0:v>
       </ns0:c>
       <ns0:c r="F65" s="1">
         <ns0:f>ROUND(F64*1.4,-5)</ns0:f>
-        <ns0:v>5.495965499806982e+29</ns0:v>
+        <ns0:v>3.958382472748296e+29</ns0:v>
       </ns0:c>
       <ns0:c r="G65" s="1" t="n">
         <ns0:v>13.2</ns0:v>
@@ -3010,15 +3010,15 @@
       </ns0:c>
       <ns0:c r="D66" s="1">
         <ns0:f>ROUND(D65*10,0)</ns0:f>
-        <ns0:v>9.773009152270436e+61</ns0:v>
+        <ns0:v>1.1727610982724528e+62</ns0:v>
       </ns0:c>
       <ns0:c r="E66" s="1">
         <ns0:f>D66</ns0:f>
-        <ns0:v>9.773009152270436e+61</ns0:v>
+        <ns0:v>1.1727610982724528e+62</ns0:v>
       </ns0:c>
       <ns0:c r="F66" s="1">
         <ns0:f>ROUND(F65*1.4,-5)</ns0:f>
-        <ns0:v>7.694351699729775e+29</ns0:v>
+        <ns0:v>5.541735461847614e+29</ns0:v>
       </ns0:c>
       <ns0:c r="G66" s="1" t="n">
         <ns0:v>13.4</ns0:v>
@@ -3041,15 +3041,15 @@
       </ns0:c>
       <ns0:c r="D67" s="1">
         <ns0:f>ROUND(D66*10,0)</ns0:f>
-        <ns0:v>9.773009152270435e+62</ns0:v>
+        <ns0:v>1.1727610982724528e+63</ns0:v>
       </ns0:c>
       <ns0:c r="E67" s="1">
         <ns0:f>D67</ns0:f>
-        <ns0:v>9.773009152270435e+62</ns0:v>
+        <ns0:v>1.1727610982724528e+63</ns0:v>
       </ns0:c>
       <ns0:c r="F67" s="1">
         <ns0:f>ROUND(F66*1.4,-5)</ns0:f>
-        <ns0:v>1.0772092379621684e+30</ns0:v>
+        <ns0:v>7.758429646586659e+29</ns0:v>
       </ns0:c>
       <ns0:c r="G67" s="1" t="n">
         <ns0:v>13.6</ns0:v>
@@ -3072,15 +3072,15 @@
       </ns0:c>
       <ns0:c r="D68" s="1">
         <ns0:f>ROUND(D67*10,0)</ns0:f>
-        <ns0:v>9.773009152270435e+63</ns0:v>
+        <ns0:v>1.1727610982724528e+64</ns0:v>
       </ns0:c>
       <ns0:c r="E68" s="1">
         <ns0:f>D68</ns0:f>
-        <ns0:v>9.773009152270435e+63</ns0:v>
+        <ns0:v>1.1727610982724528e+64</ns0:v>
       </ns0:c>
       <ns0:c r="F68" s="1">
         <ns0:f>ROUND(F67*1.4,-5)</ns0:f>
-        <ns0:v>1.5080929331470357e+30</ns0:v>
+        <ns0:v>1.0861801505221322e+30</ns0:v>
       </ns0:c>
       <ns0:c r="G68" s="1" t="n">
         <ns0:v>13.8</ns0:v>
@@ -3103,15 +3103,15 @@
       </ns0:c>
       <ns0:c r="D69" s="1">
         <ns0:f>ROUND(D68*10,0)</ns0:f>
-        <ns0:v>9.773009152270436e+64</ns0:v>
+        <ns0:v>1.172761098272453e+65</ns0:v>
       </ns0:c>
       <ns0:c r="E69" s="1">
         <ns0:f>D69</ns0:f>
-        <ns0:v>9.773009152270436e+64</ns0:v>
+        <ns0:v>1.172761098272453e+65</ns0:v>
       </ns0:c>
       <ns0:c r="F69" s="1">
         <ns0:f>ROUND(F68*1.4,-5)</ns0:f>
-        <ns0:v>2.11133010640585e+30</ns0:v>
+        <ns0:v>1.520652210730985e+30</ns0:v>
       </ns0:c>
       <ns0:c r="G69" s="1" t="n">
         <ns0:v>14</ns0:v>
@@ -3134,15 +3134,15 @@
       </ns0:c>
       <ns0:c r="D70" s="1">
         <ns0:f>ROUND(D69*10,0)</ns0:f>
-        <ns0:v>9.773009152270435e+65</ns0:v>
+        <ns0:v>1.1727610982724529e+66</ns0:v>
       </ns0:c>
       <ns0:c r="E70" s="1">
         <ns0:f>D70</ns0:f>
-        <ns0:v>9.773009152270435e+65</ns0:v>
+        <ns0:v>1.1727610982724529e+66</ns0:v>
       </ns0:c>
       <ns0:c r="F70" s="1">
         <ns0:f>ROUND(F69*1.4,-5)</ns0:f>
-        <ns0:v>2.95586214896819e+30</ns0:v>
+        <ns0:v>2.1289130950233787e+30</ns0:v>
       </ns0:c>
       <ns0:c r="G70" s="1" t="n">
         <ns0:v>14.2</ns0:v>
@@ -3165,15 +3165,15 @@
       </ns0:c>
       <ns0:c r="D71" s="1">
         <ns0:f>ROUND(D70*10,0)</ns0:f>
-        <ns0:v>9.773009152270435e+66</ns0:v>
+        <ns0:v>1.1727610982724529e+67</ns0:v>
       </ns0:c>
       <ns0:c r="E71" s="1">
         <ns0:f>D71</ns0:f>
-        <ns0:v>9.773009152270435e+66</ns0:v>
+        <ns0:v>1.1727610982724529e+67</ns0:v>
       </ns0:c>
       <ns0:c r="F71" s="1">
         <ns0:f>ROUND(F70*1.4,-5)</ns0:f>
-        <ns0:v>4.138207008555466e+30</ns0:v>
+        <ns0:v>2.98047833303273e+30</ns0:v>
       </ns0:c>
       <ns0:c r="G71" s="1" t="n">
         <ns0:v>14.4</ns0:v>
@@ -3196,15 +3196,15 @@
       </ns0:c>
       <ns0:c r="D72" s="1">
         <ns0:f>ROUND(D71*10,0)</ns0:f>
-        <ns0:v>9.773009152270435e+67</ns0:v>
+        <ns0:v>1.172761098272453e+68</ns0:v>
       </ns0:c>
       <ns0:c r="E72" s="1">
         <ns0:f>D72</ns0:f>
-        <ns0:v>9.773009152270435e+67</ns0:v>
+        <ns0:v>1.172761098272453e+68</ns0:v>
       </ns0:c>
       <ns0:c r="F72" s="1">
         <ns0:f>ROUND(F71*1.4,-5)</ns0:f>
-        <ns0:v>5.793489811977652e+30</ns0:v>
+        <ns0:v>4.172669666245821e+30</ns0:v>
       </ns0:c>
       <ns0:c r="G72" s="1" t="n">
         <ns0:v>14.6</ns0:v>
@@ -3227,15 +3227,15 @@
       </ns0:c>
       <ns0:c r="D73" s="1">
         <ns0:f>ROUND(D72*10,0)</ns0:f>
-        <ns0:v>9.773009152270434e+68</ns0:v>
+        <ns0:v>1.172761098272453e+69</ns0:v>
       </ns0:c>
       <ns0:c r="E73" s="1">
         <ns0:f>D73</ns0:f>
-        <ns0:v>9.773009152270434e+68</ns0:v>
+        <ns0:v>1.172761098272453e+69</ns0:v>
       </ns0:c>
       <ns0:c r="F73" s="1">
         <ns0:f>ROUND(F72*1.4,-5)</ns0:f>
-        <ns0:v>8.110885736768713e+30</ns0:v>
+        <ns0:v>5.841737532744149e+30</ns0:v>
       </ns0:c>
       <ns0:c r="G73" s="1" t="n">
         <ns0:v>14.8</ns0:v>
@@ -3258,15 +3258,15 @@
       </ns0:c>
       <ns0:c r="D74" s="1">
         <ns0:f>ROUND(D73*10,0)</ns0:f>
-        <ns0:v>9.773009152270435e+69</ns0:v>
+        <ns0:v>1.172761098272453e+70</ns0:v>
       </ns0:c>
       <ns0:c r="E74" s="1">
         <ns0:f>D74</ns0:f>
-        <ns0:v>9.773009152270435e+69</ns0:v>
+        <ns0:v>1.172761098272453e+70</ns0:v>
       </ns0:c>
       <ns0:c r="F74" s="1">
         <ns0:f>ROUND(F73*1.4,-5)</ns0:f>
-        <ns0:v>1.1355240031476196e+31</ns0:v>
+        <ns0:v>8.178432545841808e+30</ns0:v>
       </ns0:c>
       <ns0:c r="G74" s="1" t="n">
         <ns0:v>15</ns0:v>
@@ -3290,15 +3290,15 @@
       </ns0:c>
       <ns0:c r="D75" s="1">
         <ns0:f>ROUND(D74*10,0)</ns0:f>
-        <ns0:v>9.773009152270434e+70</ns0:v>
+        <ns0:v>1.172761098272453e+71</ns0:v>
       </ns0:c>
       <ns0:c r="E75" s="1">
         <ns0:f>D75</ns0:f>
-        <ns0:v>9.773009152270434e+70</ns0:v>
+        <ns0:v>1.172761098272453e+71</ns0:v>
       </ns0:c>
       <ns0:c r="F75" s="1">
         <ns0:f>ROUND(F74*1.4,-5)</ns0:f>
-        <ns0:v>1.5897336044066675e+31</ns0:v>
+        <ns0:v>1.144980556417853e+31</ns0:v>
       </ns0:c>
       <ns0:c r="G75" s="1" t="n">
         <ns0:v>15.2</ns0:v>
@@ -3322,15 +3322,15 @@
       </ns0:c>
       <ns0:c r="D76" s="1">
         <ns0:f>ROUND(D75*10,0)</ns0:f>
-        <ns0:v>9.773009152270434e+71</ns0:v>
+        <ns0:v>1.172761098272453e+72</ns0:v>
       </ns0:c>
       <ns0:c r="E76" s="1">
         <ns0:f>D76</ns0:f>
-        <ns0:v>9.773009152270434e+71</ns0:v>
+        <ns0:v>1.172761098272453e+72</ns0:v>
       </ns0:c>
       <ns0:c r="F76" s="1">
         <ns0:f>ROUND(F75*1.4,-5)</ns0:f>
-        <ns0:v>2.2256270461693345e+31</ns0:v>
+        <ns0:v>1.6029727789849941e+31</ns0:v>
       </ns0:c>
       <ns0:c r="G76" s="1" t="n">
         <ns0:v>15.4</ns0:v>
@@ -3354,15 +3354,15 @@
       </ns0:c>
       <ns0:c r="D77" s="1">
         <ns0:f>ROUND(D76*10,0)</ns0:f>
-        <ns0:v>9.773009152270434e+72</ns0:v>
+        <ns0:v>1.1727610982724531e+73</ns0:v>
       </ns0:c>
       <ns0:c r="E77" s="1">
         <ns0:f>D77</ns0:f>
-        <ns0:v>9.773009152270434e+72</ns0:v>
+        <ns0:v>1.1727610982724531e+73</ns0:v>
       </ns0:c>
       <ns0:c r="F77" s="1">
         <ns0:f>ROUND(F76*1.4,-5)</ns0:f>
-        <ns0:v>3.1158778646370687e+31</ns0:v>
+        <ns0:v>2.2441618905789915e+31</ns0:v>
       </ns0:c>
       <ns0:c r="G77" s="1" t="n">
         <ns0:v>15.6</ns0:v>
@@ -3386,15 +3386,15 @@
       </ns0:c>
       <ns0:c r="D78" s="1">
         <ns0:f>ROUND(D77*10,0)</ns0:f>
-        <ns0:v>9.773009152270433e+73</ns0:v>
+        <ns0:v>1.172761098272453e+74</ns0:v>
       </ns0:c>
       <ns0:c r="E78" s="1">
         <ns0:f>D78</ns0:f>
-        <ns0:v>9.773009152270433e+73</ns0:v>
+        <ns0:v>1.172761098272453e+74</ns0:v>
       </ns0:c>
       <ns0:c r="F78" s="1">
         <ns0:f>ROUND(F77*1.4,-5)</ns0:f>
-        <ns0:v>4.3622290104918955e+31</ns0:v>
+        <ns0:v>3.141826646810588e+31</ns0:v>
       </ns0:c>
       <ns0:c r="G78" s="1" t="n">
         <ns0:v>15.8</ns0:v>
@@ -3418,15 +3418,15 @@
       </ns0:c>
       <ns0:c r="D79" s="1">
         <ns0:f>ROUND(D78*10,0)</ns0:f>
-        <ns0:v>9.773009152270434e+74</ns0:v>
+        <ns0:v>1.1727610982724531e+75</ns0:v>
       </ns0:c>
       <ns0:c r="E79" s="1">
         <ns0:f>D79</ns0:f>
-        <ns0:v>9.773009152270434e+74</ns0:v>
+        <ns0:v>1.1727610982724531e+75</ns0:v>
       </ns0:c>
       <ns0:c r="F79" s="1">
         <ns0:f>ROUND(F78*1.4,-5)</ns0:f>
-        <ns0:v>6.107120614688653e+31</ns0:v>
+        <ns0:v>4.398557305534823e+31</ns0:v>
       </ns0:c>
       <ns0:c r="G79" s="1" t="n">
         <ns0:v>16</ns0:v>
@@ -3450,15 +3450,15 @@
       </ns0:c>
       <ns0:c r="D80" s="1">
         <ns0:f>ROUND(D79*10,0)</ns0:f>
-        <ns0:v>9.773009152270435e+75</ns0:v>
+        <ns0:v>1.1727610982724532e+76</ns0:v>
       </ns0:c>
       <ns0:c r="E80" s="1">
         <ns0:f>D80</ns0:f>
-        <ns0:v>9.773009152270435e+75</ns0:v>
+        <ns0:v>1.1727610982724532e+76</ns0:v>
       </ns0:c>
       <ns0:c r="F80" s="1">
         <ns0:f>ROUND(F79*1.4,-5)</ns0:f>
-        <ns0:v>8.549968860564114e+31</ns0:v>
+        <ns0:v>6.157980227748752e+31</ns0:v>
       </ns0:c>
       <ns0:c r="G80" s="1" t="n">
         <ns0:v>16.2</ns0:v>
@@ -3482,15 +3482,15 @@
       </ns0:c>
       <ns0:c r="D81" s="1">
         <ns0:f>ROUND(D80*10,0)</ns0:f>
-        <ns0:v>9.773009152270435e+76</ns0:v>
+        <ns0:v>1.1727610982724532e+77</ns0:v>
       </ns0:c>
       <ns0:c r="E81" s="1">
         <ns0:f>D81</ns0:f>
-        <ns0:v>9.773009152270435e+76</ns0:v>
+        <ns0:v>1.1727610982724532e+77</ns0:v>
       </ns0:c>
       <ns0:c r="F81" s="1">
         <ns0:f>ROUND(F80*1.4,-5)</ns0:f>
-        <ns0:v>1.1969956404789758e+32</ns0:v>
+        <ns0:v>8.621172318848253e+31</ns0:v>
       </ns0:c>
       <ns0:c r="G81" s="1" t="n">
         <ns0:v>16.4</ns0:v>
@@ -3514,15 +3514,15 @@
       </ns0:c>
       <ns0:c r="D82" s="1">
         <ns0:f>ROUND(D81*10,0)</ns0:f>
-        <ns0:v>9.773009152270435e+77</ns0:v>
+        <ns0:v>1.1727610982724532e+78</ns0:v>
       </ns0:c>
       <ns0:c r="E82" s="1">
         <ns0:f>D82</ns0:f>
-        <ns0:v>9.773009152270435e+77</ns0:v>
+        <ns0:v>1.1727610982724532e+78</ns0:v>
       </ns0:c>
       <ns0:c r="F82" s="1">
         <ns0:f>ROUND(F81*1.4,-5)</ns0:f>
-        <ns0:v>1.675793896670566e+32</ns0:v>
+        <ns0:v>1.2069641246387554e+32</ns0:v>
       </ns0:c>
       <ns0:c r="G82" s="1" t="n">
         <ns0:v>16.6</ns0:v>
@@ -3546,15 +3546,15 @@
       </ns0:c>
       <ns0:c r="D83" s="1">
         <ns0:f>ROUND(D82*10,0)</ns0:f>
-        <ns0:v>9.773009152270435e+78</ns0:v>
+        <ns0:v>1.1727610982724531e+79</ns0:v>
       </ns0:c>
       <ns0:c r="E83" s="1">
         <ns0:f>D83</ns0:f>
-        <ns0:v>9.773009152270435e+78</ns0:v>
+        <ns0:v>1.1727610982724531e+79</ns0:v>
       </ns0:c>
       <ns0:c r="F83" s="1">
         <ns0:f>ROUND(F82*1.4,-5)</ns0:f>
-        <ns0:v>2.346111455338792e+32</ns0:v>
+        <ns0:v>1.6897497744942575e+32</ns0:v>
       </ns0:c>
       <ns0:c r="G83" s="1" t="n">
         <ns0:v>16.8</ns0:v>
@@ -3578,15 +3578,15 @@
       </ns0:c>
       <ns0:c r="D84" s="1">
         <ns0:f>ROUND(D83*20,2-INT(LOG10(ABS(D83*20))))</ns0:f>
-        <ns0:v>1.95e+80</ns0:v>
+        <ns0:v>2.35e+80</ns0:v>
       </ns0:c>
       <ns0:c r="E84" s="1">
         <ns0:f>D84</ns0:f>
-        <ns0:v>1.95e+80</ns0:v>
+        <ns0:v>2.35e+80</ns0:v>
       </ns0:c>
       <ns0:c r="F84" s="1">
         <ns0:f>ROUND(F83*1.4,-5)</ns0:f>
-        <ns0:v>3.284556037474309e+32</ns0:v>
+        <ns0:v>2.3656496842919603e+32</ns0:v>
       </ns0:c>
       <ns0:c r="G84" s="1" t="n">
         <ns0:v>17</ns0:v>
@@ -3610,15 +3610,15 @@
       </ns0:c>
       <ns0:c r="D85" s="1">
         <ns0:f>ROUND(D84*20,2-INT(LOG10(ABS(D84*20))))</ns0:f>
-        <ns0:v>3.9e+81</ns0:v>
+        <ns0:v>4.7e+81</ns0:v>
       </ns0:c>
       <ns0:c r="E85" s="1">
         <ns0:f>D85</ns0:f>
-        <ns0:v>3.9e+81</ns0:v>
+        <ns0:v>4.7e+81</ns0:v>
       </ns0:c>
       <ns0:c r="F85" s="1">
         <ns0:f>ROUND(F84*1.4,-5)</ns0:f>
-        <ns0:v>4.5983784524640325e+32</ns0:v>
+        <ns0:v>3.3119095580087444e+32</ns0:v>
       </ns0:c>
       <ns0:c r="G85" s="1" t="n">
         <ns0:v>17.2</ns0:v>
@@ -3642,15 +3642,15 @@
       </ns0:c>
       <ns0:c r="D86" s="1">
         <ns0:f>ROUND(D85*20,2-INT(LOG10(ABS(D85*20))))</ns0:f>
-        <ns0:v>7.800000000000001e+82</ns0:v>
+        <ns0:v>9.4e+82</ns0:v>
       </ns0:c>
       <ns0:c r="E86" s="1">
         <ns0:f>D86</ns0:f>
-        <ns0:v>7.800000000000001e+82</ns0:v>
+        <ns0:v>9.4e+82</ns0:v>
       </ns0:c>
       <ns0:c r="F86" s="1">
         <ns0:f>ROUND(F85*1.4,-5)</ns0:f>
-        <ns0:v>6.437729833449646e+32</ns0:v>
+        <ns0:v>4.636673381212242e+32</ns0:v>
       </ns0:c>
       <ns0:c r="G86" s="1" t="n">
         <ns0:v>17.4</ns0:v>
@@ -3674,15 +3674,15 @@
       </ns0:c>
       <ns0:c r="D87" s="1">
         <ns0:f>ROUND(D86*20,2-INT(LOG10(ABS(D86*20))))</ns0:f>
-        <ns0:v>1.56e+84</ns0:v>
+        <ns0:v>1.8800000000000002e+84</ns0:v>
       </ns0:c>
       <ns0:c r="E87" s="1">
         <ns0:f>D87</ns0:f>
-        <ns0:v>1.56e+84</ns0:v>
+        <ns0:v>1.8800000000000002e+84</ns0:v>
       </ns0:c>
       <ns0:c r="F87" s="1">
         <ns0:f>ROUND(F86*1.4,-5)</ns0:f>
-        <ns0:v>9.012821766829504e+32</ns0:v>
+        <ns0:v>6.491342733697137e+32</ns0:v>
       </ns0:c>
       <ns0:c r="G87" s="1" t="n">
         <ns0:v>17.6</ns0:v>
@@ -3706,15 +3706,15 @@
       </ns0:c>
       <ns0:c r="D88" s="1">
         <ns0:f>ROUND(D87*20,2-INT(LOG10(ABS(D87*20))))</ns0:f>
-        <ns0:v>3.12e+85</ns0:v>
+        <ns0:v>3.76e+85</ns0:v>
       </ns0:c>
       <ns0:c r="E88" s="1">
         <ns0:f>D88</ns0:f>
-        <ns0:v>3.12e+85</ns0:v>
+        <ns0:v>3.76e+85</ns0:v>
       </ns0:c>
       <ns0:c r="F88" s="1">
         <ns0:f>ROUND(F87*1.4,-5)</ns0:f>
-        <ns0:v>1.2617950473561304e+33</ns0:v>
+        <ns0:v>9.087879827175992e+32</ns0:v>
       </ns0:c>
       <ns0:c r="G88" s="1" t="n">
         <ns0:v>17.8</ns0:v>
@@ -3738,15 +3738,15 @@
       </ns0:c>
       <ns0:c r="D89" s="1">
         <ns0:f>ROUND(D88*20,2-INT(LOG10(ABS(D88*20))))</ns0:f>
-        <ns0:v>6.239999999999999e+86</ns0:v>
+        <ns0:v>7.519999999999999e+86</ns0:v>
       </ns0:c>
       <ns0:c r="E89" s="1">
         <ns0:f>D89</ns0:f>
-        <ns0:v>6.239999999999999e+86</ns0:v>
+        <ns0:v>7.519999999999999e+86</ns0:v>
       </ns0:c>
       <ns0:c r="F89" s="1">
         <ns0:f>ROUND(F88*1.4,-5)</ns0:f>
-        <ns0:v>1.7665130662985825e+33</ns0:v>
+        <ns0:v>1.2723031758046388e+33</ns0:v>
       </ns0:c>
       <ns0:c r="G89" s="1" t="n">
         <ns0:v>18</ns0:v>
@@ -3770,15 +3770,15 @@
       </ns0:c>
       <ns0:c r="D90" s="1">
         <ns0:f>ROUND(D89*20,2-INT(LOG10(ABS(D89*20))))</ns0:f>
-        <ns0:v>1.2499999999999998e+88</ns0:v>
+        <ns0:v>1.4999999999999999e+88</ns0:v>
       </ns0:c>
       <ns0:c r="E90" s="1">
         <ns0:f>D90</ns0:f>
-        <ns0:v>1.2499999999999998e+88</ns0:v>
+        <ns0:v>1.4999999999999999e+88</ns0:v>
       </ns0:c>
       <ns0:c r="F90" s="1">
         <ns0:f>ROUND(F89*1.4,-5)</ns0:f>
-        <ns0:v>2.4731182928180153e+33</ns0:v>
+        <ns0:v>1.7812244461264942e+33</ns0:v>
       </ns0:c>
       <ns0:c r="G90" s="1" t="n">
         <ns0:v>18.2</ns0:v>
@@ -3802,15 +3802,15 @@
       </ns0:c>
       <ns0:c r="D91" s="1">
         <ns0:f>ROUND(D90*20,2-INT(LOG10(ABS(D90*20))))</ns0:f>
-        <ns0:v>2.5e+89</ns0:v>
+        <ns0:v>3e+89</ns0:v>
       </ns0:c>
       <ns0:c r="E91" s="1">
         <ns0:f>D91</ns0:f>
-        <ns0:v>2.5e+89</ns0:v>
+        <ns0:v>3e+89</ns0:v>
       </ns0:c>
       <ns0:c r="F91" s="1">
         <ns0:f>ROUND(F90*1.4,-5)</ns0:f>
-        <ns0:v>3.462365609945221e+33</ns0:v>
+        <ns0:v>2.4937142245770916e+33</ns0:v>
       </ns0:c>
       <ns0:c r="G91" s="1" t="n">
         <ns0:v>18.4</ns0:v>
@@ -3834,15 +3834,15 @@
       </ns0:c>
       <ns0:c r="D92" s="1">
         <ns0:f>ROUND(D91*20,2-INT(LOG10(ABS(D91*20))))</ns0:f>
-        <ns0:v>5e+90</ns0:v>
+        <ns0:v>6.0000000000000005e+90</ns0:v>
       </ns0:c>
       <ns0:c r="E92" s="1">
         <ns0:f>D92</ns0:f>
-        <ns0:v>5e+90</ns0:v>
+        <ns0:v>6.0000000000000005e+90</ns0:v>
       </ns0:c>
       <ns0:c r="F92" s="1">
         <ns0:f>ROUND(F91*1.4,-5)</ns0:f>
-        <ns0:v>4.8473118539233087e+33</ns0:v>
+        <ns0:v>3.491199914407928e+33</ns0:v>
       </ns0:c>
       <ns0:c r="G92" s="1" t="n">
         <ns0:v>18.6</ns0:v>
@@ -3866,15 +3866,15 @@
       </ns0:c>
       <ns0:c r="D93" s="1">
         <ns0:f>ROUND(D92*20,2-INT(LOG10(ABS(D92*20))))</ns0:f>
-        <ns0:v>1e+92</ns0:v>
+        <ns0:v>1.2e+92</ns0:v>
       </ns0:c>
       <ns0:c r="E93" s="1">
         <ns0:f>D93</ns0:f>
-        <ns0:v>1e+92</ns0:v>
+        <ns0:v>1.2e+92</ns0:v>
       </ns0:c>
       <ns0:c r="F93" s="1">
         <ns0:f>ROUND(F92*1.4,-5)</ns0:f>
-        <ns0:v>6.786236595492632e+33</ns0:v>
+        <ns0:v>4.8876798801710985e+33</ns0:v>
       </ns0:c>
       <ns0:c r="G93" s="1" t="n">
         <ns0:v>18.8</ns0:v>
@@ -3898,15 +3898,15 @@
       </ns0:c>
       <ns0:c r="D94" s="1">
         <ns0:f>ROUND(D93*20,2-INT(LOG10(ABS(D93*20))))</ns0:f>
-        <ns0:v>1.9999999999999999e+93</ns0:v>
+        <ns0:v>2.4e+93</ns0:v>
       </ns0:c>
       <ns0:c r="E94" s="1">
         <ns0:f>D94</ns0:f>
-        <ns0:v>1.9999999999999999e+93</ns0:v>
+        <ns0:v>2.4e+93</ns0:v>
       </ns0:c>
       <ns0:c r="F94" s="1">
         <ns0:f>ROUND(F93*1.4,-5)</ns0:f>
-        <ns0:v>9.500731233689683e+33</ns0:v>
+        <ns0:v>6.842751832239537e+33</ns0:v>
       </ns0:c>
       <ns0:c r="G94" s="1" t="n">
         <ns0:v>19</ns0:v>
@@ -3930,15 +3930,15 @@
       </ns0:c>
       <ns0:c r="D95" s="1">
         <ns0:f>ROUND(D94*20,2-INT(LOG10(ABS(D94*20))))</ns0:f>
-        <ns0:v>4e+94</ns0:v>
+        <ns0:v>4.8000000000000004e+94</ns0:v>
       </ns0:c>
       <ns0:c r="E95" s="1">
         <ns0:f>D95</ns0:f>
-        <ns0:v>4e+94</ns0:v>
+        <ns0:v>4.8000000000000004e+94</ns0:v>
       </ns0:c>
       <ns0:c r="F95" s="1">
         <ns0:f>ROUND(F94*1.4,-5)</ns0:f>
-        <ns0:v>1.3301023727165556e+34</ns0:v>
+        <ns0:v>9.579852565135353e+33</ns0:v>
       </ns0:c>
       <ns0:c r="G95" s="1" t="n">
         <ns0:v>19.2</ns0:v>
@@ -3962,15 +3962,15 @@
       </ns0:c>
       <ns0:c r="D96" s="1">
         <ns0:f>ROUND(D95*20,2-INT(LOG10(ABS(D95*20))))</ns0:f>
-        <ns0:v>8.000000000000001e+95</ns0:v>
+        <ns0:v>9.600000000000001e+95</ns0:v>
       </ns0:c>
       <ns0:c r="E96" s="1">
         <ns0:f>D96</ns0:f>
-        <ns0:v>8.000000000000001e+95</ns0:v>
+        <ns0:v>9.600000000000001e+95</ns0:v>
       </ns0:c>
       <ns0:c r="F96" s="1">
         <ns0:f>ROUND(F95*1.4,-5)</ns0:f>
-        <ns0:v>1.8621433218031776e+34</ns0:v>
+        <ns0:v>1.3411793591189494e+34</ns0:v>
       </ns0:c>
       <ns0:c r="G96" s="1" t="n">
         <ns0:v>19.4</ns0:v>
@@ -3994,15 +3994,15 @@
       </ns0:c>
       <ns0:c r="D97" s="1">
         <ns0:f>ROUND(D96*20,2-INT(LOG10(ABS(D96*20))))</ns0:f>
-        <ns0:v>1.6e+97</ns0:v>
+        <ns0:v>1.92e+97</ns0:v>
       </ns0:c>
       <ns0:c r="E97" s="1">
         <ns0:f>D97</ns0:f>
-        <ns0:v>1.6e+97</ns0:v>
+        <ns0:v>1.92e+97</ns0:v>
       </ns0:c>
       <ns0:c r="F97" s="1">
         <ns0:f>ROUND(F96*1.4,-5)</ns0:f>
-        <ns0:v>2.6070006505244486e+34</ns0:v>
+        <ns0:v>1.877651102766529e+34</ns0:v>
       </ns0:c>
       <ns0:c r="G97" s="1" t="n">
         <ns0:v>19.6</ns0:v>
@@ -4026,15 +4026,15 @@
       </ns0:c>
       <ns0:c r="D98" s="1">
         <ns0:f>ROUND(D97*20,2-INT(LOG10(ABS(D97*20))))</ns0:f>
-        <ns0:v>3.2e+98</ns0:v>
+        <ns0:v>3.8400000000000006e+98</ns0:v>
       </ns0:c>
       <ns0:c r="E98" s="1">
         <ns0:f>D98</ns0:f>
-        <ns0:v>3.2e+98</ns0:v>
+        <ns0:v>3.8400000000000006e+98</ns0:v>
       </ns0:c>
       <ns0:c r="F98" s="1">
         <ns0:f>ROUND(F97*1.4,-5)</ns0:f>
-        <ns0:v>3.6498009107342274e+34</ns0:v>
+        <ns0:v>2.6287115438731407e+34</ns0:v>
       </ns0:c>
       <ns0:c r="G98" s="1" t="n">
         <ns0:v>19.8</ns0:v>
@@ -4058,15 +4058,15 @@
       </ns0:c>
       <ns0:c r="D99" s="1">
         <ns0:f>ROUND(D98*20,2-INT(LOG10(ABS(D98*20))))</ns0:f>
-        <ns0:v>6.4e+99</ns0:v>
+        <ns0:v>7.68e+99</ns0:v>
       </ns0:c>
       <ns0:c r="E99" s="1">
         <ns0:f>D99</ns0:f>
-        <ns0:v>6.4e+99</ns0:v>
+        <ns0:v>7.68e+99</ns0:v>
       </ns0:c>
       <ns0:c r="F99" s="1">
         <ns0:f>ROUND(F98*1.4,-5)</ns0:f>
-        <ns0:v>5.109721275027918e+34</ns0:v>
+        <ns0:v>3.6801961614223965e+34</ns0:v>
       </ns0:c>
       <ns0:c r="G99" s="1" t="n">
         <ns0:v>20</ns0:v>
@@ -4090,15 +4090,15 @@
       </ns0:c>
       <ns0:c r="D100" s="1">
         <ns0:f>ROUND(D99*20,2-INT(LOG10(ABS(D99*20))))</ns0:f>
-        <ns0:v>1.28e+101</ns0:v>
+        <ns0:v>1.54e+101</ns0:v>
       </ns0:c>
       <ns0:c r="E100" s="1">
         <ns0:f>D100</ns0:f>
-        <ns0:v>1.28e+101</ns0:v>
+        <ns0:v>1.54e+101</ns0:v>
       </ns0:c>
       <ns0:c r="F100" s="1">
         <ns0:f>ROUND(F99*1.4,-5)</ns0:f>
-        <ns0:v>7.153609785039085e+34</ns0:v>
+        <ns0:v>5.152274625991355e+34</ns0:v>
       </ns0:c>
       <ns0:c r="G100" s="1" t="n">
         <ns0:v>20.2</ns0:v>
@@ -4122,15 +4122,15 @@
       </ns0:c>
       <ns0:c r="D101" s="1">
         <ns0:f>ROUND(D100*20,2-INT(LOG10(ABS(D100*20))))</ns0:f>
-        <ns0:v>2.56e+102</ns0:v>
+        <ns0:v>3.08e+102</ns0:v>
       </ns0:c>
       <ns0:c r="E101" s="1">
         <ns0:f>D101</ns0:f>
-        <ns0:v>2.56e+102</ns0:v>
+        <ns0:v>3.08e+102</ns0:v>
       </ns0:c>
       <ns0:c r="F101" s="1">
         <ns0:f>ROUND(F100*1.4,-5)</ns0:f>
-        <ns0:v>1.0015053699054717e+35</ns0:v>
+        <ns0:v>7.213184476387896e+34</ns0:v>
       </ns0:c>
       <ns0:c r="G101" s="1" t="n">
         <ns0:v>20.4</ns0:v>
@@ -4154,15 +4154,15 @@
       </ns0:c>
       <ns0:c r="D102" s="1">
         <ns0:f>ROUND(D101*20,2-INT(LOG10(ABS(D101*20))))</ns0:f>
-        <ns0:v>5.12e+103</ns0:v>
+        <ns0:v>6.159999999999999e+103</ns0:v>
       </ns0:c>
       <ns0:c r="E102" s="1">
         <ns0:f>D102</ns0:f>
-        <ns0:v>5.12e+103</ns0:v>
+        <ns0:v>6.159999999999999e+103</ns0:v>
       </ns0:c>
       <ns0:c r="F102" s="1">
         <ns0:f>ROUND(F101*1.4,-5)</ns0:f>
-        <ns0:v>1.4021075178676604e+35</ns0:v>
+        <ns0:v>1.0098458266943055e+35</ns0:v>
       </ns0:c>
       <ns0:c r="G102" s="1" t="n">
         <ns0:v>20.6</ns0:v>
@@ -4186,15 +4186,15 @@
       </ns0:c>
       <ns0:c r="D103" s="1">
         <ns0:f>ROUND(D102*20,2-INT(LOG10(ABS(D102*20))))</ns0:f>
-        <ns0:v>1.02e+105</ns0:v>
+        <ns0:v>1.23e+105</ns0:v>
       </ns0:c>
       <ns0:c r="E103" s="1">
         <ns0:f>D103</ns0:f>
-        <ns0:v>1.02e+105</ns0:v>
+        <ns0:v>1.23e+105</ns0:v>
       </ns0:c>
       <ns0:c r="F103" s="1">
         <ns0:f>ROUND(F102*1.4,-5)</ns0:f>
-        <ns0:v>1.9629505250147243e+35</ns0:v>
+        <ns0:v>1.4137841573720276e+35</ns0:v>
       </ns0:c>
       <ns0:c r="G103" s="1" t="n">
         <ns0:v>20.8</ns0:v>
@@ -4218,15 +4218,15 @@
       </ns0:c>
       <ns0:c r="D104" s="1">
         <ns0:f>ROUND(D103*20,2-INT(LOG10(ABS(D103*20))))</ns0:f>
-        <ns0:v>2.04e+106</ns0:v>
+        <ns0:v>2.46e+106</ns0:v>
       </ns0:c>
       <ns0:c r="E104" s="1">
         <ns0:f>D104</ns0:f>
-        <ns0:v>2.04e+106</ns0:v>
+        <ns0:v>2.46e+106</ns0:v>
       </ns0:c>
       <ns0:c r="F104" s="1">
         <ns0:f>ROUND(F103*1.4,-5)</ns0:f>
-        <ns0:v>2.7481307350206138e+35</ns0:v>
+        <ns0:v>1.9792978203208386e+35</ns0:v>
       </ns0:c>
       <ns0:c r="G104" s="1" t="n">
         <ns0:v>21</ns0:v>
@@ -4250,15 +4250,15 @@
       </ns0:c>
       <ns0:c r="D105" s="1">
         <ns0:f>ROUND(D104*20,2-INT(LOG10(ABS(D104*20))))</ns0:f>
-        <ns0:v>4.0800000000000004e+107</ns0:v>
+        <ns0:v>4.92e+107</ns0:v>
       </ns0:c>
       <ns0:c r="E105" s="1">
         <ns0:f>D105</ns0:f>
-        <ns0:v>4.0800000000000004e+107</ns0:v>
+        <ns0:v>4.92e+107</ns0:v>
       </ns0:c>
       <ns0:c r="F105" s="1">
         <ns0:f>ROUND(F104*1.4,-5)</ns0:f>
-        <ns0:v>3.847383029028859e+35</ns0:v>
+        <ns0:v>2.7710169484491734e+35</ns0:v>
       </ns0:c>
       <ns0:c r="G105" s="1" t="n">
         <ns0:v>21.2</ns0:v>
@@ -4282,15 +4282,15 @@
       </ns0:c>
       <ns0:c r="D106" s="1">
         <ns0:f>ROUND(D105*20,2-INT(LOG10(ABS(D105*20))))</ns0:f>
-        <ns0:v>8.16e+108</ns0:v>
+        <ns0:v>9.84e+108</ns0:v>
       </ns0:c>
       <ns0:c r="E106" s="1">
         <ns0:f>D106</ns0:f>
-        <ns0:v>8.16e+108</ns0:v>
+        <ns0:v>9.84e+108</ns0:v>
       </ns0:c>
       <ns0:c r="F106" s="1">
         <ns0:f>ROUND(F105*1.4,-5)</ns0:f>
-        <ns0:v>5.386336240640402e+35</ns0:v>
+        <ns0:v>3.879423727828843e+35</ns0:v>
       </ns0:c>
       <ns0:c r="G106" s="1" t="n">
         <ns0:v>21.4</ns0:v>
@@ -4314,15 +4314,15 @@
       </ns0:c>
       <ns0:c r="D107" s="1">
         <ns0:f>ROUND(D106*20,2-INT(LOG10(ABS(D106*20))))</ns0:f>
-        <ns0:v>1.63e+110</ns0:v>
+        <ns0:v>1.9699999999999998e+110</ns0:v>
       </ns0:c>
       <ns0:c r="E107" s="1">
         <ns0:f>D107</ns0:f>
-        <ns0:v>1.63e+110</ns0:v>
+        <ns0:v>1.9699999999999998e+110</ns0:v>
       </ns0:c>
       <ns0:c r="F107" s="1">
         <ns0:f>ROUND(F106*1.4,-5)</ns0:f>
-        <ns0:v>7.540870736896562e+35</ns0:v>
+        <ns0:v>5.431193218960379e+35</ns0:v>
       </ns0:c>
       <ns0:c r="G107" s="1" t="n">
         <ns0:v>21.6</ns0:v>
@@ -4346,15 +4346,15 @@
       </ns0:c>
       <ns0:c r="D108" s="1">
         <ns0:f>ROUND(D107*20,2-INT(LOG10(ABS(D107*20))))</ns0:f>
-        <ns0:v>3.26e+111</ns0:v>
+        <ns0:v>3.94e+111</ns0:v>
       </ns0:c>
       <ns0:c r="E108" s="1">
         <ns0:f>D108</ns0:f>
-        <ns0:v>3.26e+111</ns0:v>
+        <ns0:v>3.94e+111</ns0:v>
       </ns0:c>
       <ns0:c r="F108" s="1">
         <ns0:f>ROUND(F107*1.4,-5)</ns0:f>
-        <ns0:v>1.0557219031655186e+36</ns0:v>
+        <ns0:v>7.60367050654453e+35</ns0:v>
       </ns0:c>
       <ns0:c r="G108" s="1" t="n">
         <ns0:v>21.8</ns0:v>
@@ -4378,15 +4378,15 @@
       </ns0:c>
       <ns0:c r="D109" s="1">
         <ns0:f>ROUND(D108*20,2-INT(LOG10(ABS(D108*20))))</ns0:f>
-        <ns0:v>6.52e+112</ns0:v>
+        <ns0:v>7.88e+112</ns0:v>
       </ns0:c>
       <ns0:c r="E109" s="1">
         <ns0:f>D109</ns0:f>
-        <ns0:v>6.52e+112</ns0:v>
+        <ns0:v>7.88e+112</ns0:v>
       </ns0:c>
       <ns0:c r="F109" s="1">
         <ns0:f>ROUND(F108*1.4,-5)</ns0:f>
-        <ns0:v>1.478010664431726e+36</ns0:v>
+        <ns0:v>1.0645138709162343e+36</ns0:v>
       </ns0:c>
       <ns0:c r="G109" s="1" t="n">
         <ns0:v>22</ns0:v>
@@ -4410,15 +4410,15 @@
       </ns0:c>
       <ns0:c r="D110" s="1">
         <ns0:f>ROUND(D109*20,2-INT(LOG10(ABS(D109*20))))</ns0:f>
-        <ns0:v>1.3e+114</ns0:v>
+        <ns0:v>1.5800000000000002e+114</ns0:v>
       </ns0:c>
       <ns0:c r="E110" s="1">
         <ns0:f>D110</ns0:f>
-        <ns0:v>1.3e+114</ns0:v>
+        <ns0:v>1.5800000000000002e+114</ns0:v>
       </ns0:c>
       <ns0:c r="F110" s="1">
         <ns0:f>ROUND(F109*1.4,-5)</ns0:f>
-        <ns0:v>2.0692149302044165e+36</ns0:v>
+        <ns0:v>1.4903194192827278e+36</ns0:v>
       </ns0:c>
       <ns0:c r="G110" s="1" t="n">
         <ns0:v>22.2</ns0:v>
@@ -4442,15 +4442,15 @@
       </ns0:c>
       <ns0:c r="D111" s="1">
         <ns0:f>ROUND(D110*20,2-INT(LOG10(ABS(D110*20))))</ns0:f>
-        <ns0:v>2.6e+115</ns0:v>
+        <ns0:v>3.16e+115</ns0:v>
       </ns0:c>
       <ns0:c r="E111" s="1">
         <ns0:f>D111</ns0:f>
-        <ns0:v>2.6e+115</ns0:v>
+        <ns0:v>3.16e+115</ns0:v>
       </ns0:c>
       <ns0:c r="F111" s="1">
         <ns0:f>ROUND(F110*1.4,-5)</ns0:f>
-        <ns0:v>2.896900902286183e+36</ns0:v>
+        <ns0:v>2.0864471869958192e+36</ns0:v>
       </ns0:c>
       <ns0:c r="G111" s="1" t="n">
         <ns0:v>22.4</ns0:v>
@@ -4474,15 +4474,15 @@
       </ns0:c>
       <ns0:c r="D112" s="1">
         <ns0:f>ROUND(D111*20,2-INT(LOG10(ABS(D111*20))))</ns0:f>
-        <ns0:v>5.2e+116</ns0:v>
+        <ns0:v>6.32e+116</ns0:v>
       </ns0:c>
       <ns0:c r="E112" s="1">
         <ns0:f>D112</ns0:f>
-        <ns0:v>5.2e+116</ns0:v>
+        <ns0:v>6.32e+116</ns0:v>
       </ns0:c>
       <ns0:c r="F112" s="1">
         <ns0:f>ROUND(F111*1.4,-5)</ns0:f>
-        <ns0:v>4.055661263200656e+36</ns0:v>
+        <ns0:v>2.9210260617941466e+36</ns0:v>
       </ns0:c>
       <ns0:c r="G112" s="1" t="n">
         <ns0:v>22.6</ns0:v>
@@ -4506,15 +4506,15 @@
       </ns0:c>
       <ns0:c r="D113" s="1">
         <ns0:f>ROUND(D112*20,2-INT(LOG10(ABS(D112*20))))</ns0:f>
-        <ns0:v>1.04e+118</ns0:v>
+        <ns0:v>1.26e+118</ns0:v>
       </ns0:c>
       <ns0:c r="E113" s="1">
         <ns0:f>D113</ns0:f>
-        <ns0:v>1.04e+118</ns0:v>
+        <ns0:v>1.26e+118</ns0:v>
       </ns0:c>
       <ns0:c r="F113" s="1">
         <ns0:f>ROUND(F112*1.4,-5)</ns0:f>
-        <ns0:v>5.677925768480918e+36</ns0:v>
+        <ns0:v>4.0894364865118056e+36</ns0:v>
       </ns0:c>
       <ns0:c r="G113" s="1" t="n">
         <ns0:v>22.8</ns0:v>
@@ -4538,15 +4538,15 @@
       </ns0:c>
       <ns0:c r="D114" s="1">
         <ns0:f>ROUND(D113*20,2-INT(LOG10(ABS(D113*20))))</ns0:f>
-        <ns0:v>2.0799999999999998e+119</ns0:v>
+        <ns0:v>2.52e+119</ns0:v>
       </ns0:c>
       <ns0:c r="E114" s="1">
         <ns0:f>D114</ns0:f>
-        <ns0:v>2.0799999999999998e+119</ns0:v>
+        <ns0:v>2.52e+119</ns0:v>
       </ns0:c>
       <ns0:c r="F114" s="1">
         <ns0:f>ROUND(F113*1.4,-5)</ns0:f>
-        <ns0:v>7.949096075873285e+36</ns0:v>
+        <ns0:v>5.725211081116527e+36</ns0:v>
       </ns0:c>
       <ns0:c r="G114" s="1" t="n">
         <ns0:v>23</ns0:v>
@@ -4570,15 +4570,15 @@
       </ns0:c>
       <ns0:c r="D115" s="1">
         <ns0:f>ROUND(D114*20,2-INT(LOG10(ABS(D114*20))))</ns0:f>
-        <ns0:v>4.16e+120</ns0:v>
+        <ns0:v>5.04e+120</ns0:v>
       </ns0:c>
       <ns0:c r="E115" s="1">
         <ns0:f>D115</ns0:f>
-        <ns0:v>4.16e+120</ns0:v>
+        <ns0:v>5.04e+120</ns0:v>
       </ns0:c>
       <ns0:c r="F115" s="1">
         <ns0:f>ROUND(F114*1.4,-5)</ns0:f>
-        <ns0:v>1.1128734506222598e+37</ns0:v>
+        <ns0:v>8.015295513563137e+36</ns0:v>
       </ns0:c>
       <ns0:c r="G115" s="1" t="n">
         <ns0:v>23.2</ns0:v>
@@ -4602,15 +4602,15 @@
       </ns0:c>
       <ns0:c r="D116" s="1">
         <ns0:f>ROUND(D115*20,2-INT(LOG10(ABS(D115*20))))</ns0:f>
-        <ns0:v>8.32e+121</ns0:v>
+        <ns0:v>1.01e+122</ns0:v>
       </ns0:c>
       <ns0:c r="E116" s="1">
         <ns0:f>D116</ns0:f>
-        <ns0:v>8.32e+121</ns0:v>
+        <ns0:v>1.01e+122</ns0:v>
       </ns0:c>
       <ns0:c r="F116" s="1">
         <ns0:f>ROUND(F115*1.4,-5)</ns0:f>
-        <ns0:v>1.5580228308711636e+37</ns0:v>
+        <ns0:v>1.122141371898839e+37</ns0:v>
       </ns0:c>
       <ns0:c r="G116" s="1" t="n">
         <ns0:v>23.4</ns0:v>
@@ -4634,15 +4634,15 @@
       </ns0:c>
       <ns0:c r="D117" s="1">
         <ns0:f>ROUND(D116*20,2-INT(LOG10(ABS(D116*20))))</ns0:f>
-        <ns0:v>1.66e+123</ns0:v>
+        <ns0:v>2.02e+123</ns0:v>
       </ns0:c>
       <ns0:c r="E117" s="1">
         <ns0:f>D117</ns0:f>
-        <ns0:v>1.66e+123</ns0:v>
+        <ns0:v>2.02e+123</ns0:v>
       </ns0:c>
       <ns0:c r="F117" s="1">
         <ns0:f>ROUND(F116*1.4,-5)</ns0:f>
-        <ns0:v>2.181231963219629e+37</ns0:v>
+        <ns0:v>1.5709979206583747e+37</ns0:v>
       </ns0:c>
       <ns0:c r="G117" s="1" t="n">
         <ns0:v>23.6</ns0:v>
@@ -4666,15 +4666,15 @@
       </ns0:c>
       <ns0:c r="D118" s="1">
         <ns0:f>ROUND(D117*20,2-INT(LOG10(ABS(D117*20))))</ns0:f>
-        <ns0:v>3.32e+124</ns0:v>
+        <ns0:v>4.04e+124</ns0:v>
       </ns0:c>
       <ns0:c r="E118" s="1">
         <ns0:f>D118</ns0:f>
-        <ns0:v>3.32e+124</ns0:v>
+        <ns0:v>4.04e+124</ns0:v>
       </ns0:c>
       <ns0:c r="F118" s="1">
         <ns0:f>ROUND(F117*1.4,-5)</ns0:f>
-        <ns0:v>3.0537247485074806e+37</ns0:v>
+        <ns0:v>2.1993970889217245e+37</ns0:v>
       </ns0:c>
       <ns0:c r="G118" s="1" t="n">
         <ns0:v>23.8</ns0:v>
@@ -4698,15 +4698,15 @@
       </ns0:c>
       <ns0:c r="D119" s="1">
         <ns0:f>ROUND(D118*20,2-INT(LOG10(ABS(D118*20))))</ns0:f>
-        <ns0:v>6.6399999999999994e+125</ns0:v>
+        <ns0:v>8.08e+125</ns0:v>
       </ns0:c>
       <ns0:c r="E119" s="1">
         <ns0:f>D119</ns0:f>
-        <ns0:v>6.6399999999999994e+125</ns0:v>
+        <ns0:v>8.08e+125</ns0:v>
       </ns0:c>
       <ns0:c r="F119" s="1">
         <ns0:f>ROUND(F118*1.4,-5)</ns0:f>
-        <ns0:v>4.275214647910472e+37</ns0:v>
+        <ns0:v>3.079155924490414e+37</ns0:v>
       </ns0:c>
       <ns0:c r="G119" s="1" t="n">
         <ns0:v>24</ns0:v>
@@ -4730,15 +4730,15 @@
       </ns0:c>
       <ns0:c r="D120" s="1">
         <ns0:f>ROUND(D119*20,2-INT(LOG10(ABS(D119*20))))</ns0:f>
-        <ns0:v>1.33e+127</ns0:v>
+        <ns0:v>1.62e+127</ns0:v>
       </ns0:c>
       <ns0:c r="E120" s="1">
         <ns0:f>D120</ns0:f>
-        <ns0:v>1.33e+127</ns0:v>
+        <ns0:v>1.62e+127</ns0:v>
       </ns0:c>
       <ns0:c r="F120" s="1">
         <ns0:f>ROUND(F119*1.4,-5)</ns0:f>
-        <ns0:v>5.9853005070746605e+37</ns0:v>
+        <ns0:v>4.310818294286579e+37</ns0:v>
       </ns0:c>
       <ns0:c r="G120" s="1" t="n">
         <ns0:v>24.2000000000001</ns0:v>
@@ -4762,15 +4762,15 @@
       </ns0:c>
       <ns0:c r="D121" s="1">
         <ns0:f>ROUND(D120*20,2-INT(LOG10(ABS(D120*20))))</ns0:f>
-        <ns0:v>2.66e+128</ns0:v>
+        <ns0:v>3.2400000000000002e+128</ns0:v>
       </ns0:c>
       <ns0:c r="E121" s="1">
         <ns0:f>D121</ns0:f>
-        <ns0:v>2.66e+128</ns0:v>
+        <ns0:v>3.2400000000000002e+128</ns0:v>
       </ns0:c>
       <ns0:c r="F121" s="1">
         <ns0:f>ROUND(F120*1.4,-5)</ns0:f>
-        <ns0:v>8.379420709904523e+37</ns0:v>
+        <ns0:v>6.03514561200121e+37</ns0:v>
       </ns0:c>
       <ns0:c r="G121" s="1" t="n">
         <ns0:v>24.4000000000001</ns0:v>
@@ -4794,15 +4794,15 @@
       </ns0:c>
       <ns0:c r="D122" s="1">
         <ns0:f>ROUND(D121*20,2-INT(LOG10(ABS(D121*20))))</ns0:f>
-        <ns0:v>5.32e+129</ns0:v>
+        <ns0:v>6.48e+129</ns0:v>
       </ns0:c>
       <ns0:c r="E122" s="1">
         <ns0:f>D122</ns0:f>
-        <ns0:v>5.32e+129</ns0:v>
+        <ns0:v>6.48e+129</ns0:v>
       </ns0:c>
       <ns0:c r="F122" s="1">
         <ns0:f>ROUND(F121*1.4,-5)</ns0:f>
-        <ns0:v>1.1731188993866332e+38</ns0:v>
+        <ns0:v>8.449203856801694e+37</ns0:v>
       </ns0:c>
       <ns0:c r="G122" s="1" t="n">
         <ns0:v>24.6000000000001</ns0:v>
@@ -4826,15 +4826,15 @@
       </ns0:c>
       <ns0:c r="D123" s="1">
         <ns0:f>ROUND(D122*20,2-INT(LOG10(ABS(D122*20))))</ns0:f>
-        <ns0:v>1.0600000000000001e+131</ns0:v>
+        <ns0:v>1.3e+131</ns0:v>
       </ns0:c>
       <ns0:c r="E123" s="1">
         <ns0:f>D123</ns0:f>
-        <ns0:v>1.0600000000000001e+131</ns0:v>
+        <ns0:v>1.3e+131</ns0:v>
       </ns0:c>
       <ns0:c r="F123" s="1">
         <ns0:f>ROUND(F122*1.4,-5)</ns0:f>
-        <ns0:v>1.6423664591412864e+38</ns0:v>
+        <ns0:v>1.182888539952237e+38</ns0:v>
       </ns0:c>
       <ns0:c r="G123" s="1" t="n">
         <ns0:v>24.8000000000001</ns0:v>
@@ -4858,15 +4858,15 @@
       </ns0:c>
       <ns0:c r="D124" s="1">
         <ns0:f>ROUND(D123*20,2-INT(LOG10(ABS(D123*20))))</ns0:f>
-        <ns0:v>2.12e+132</ns0:v>
+        <ns0:v>2.5999999999999997e+132</ns0:v>
       </ns0:c>
       <ns0:c r="E124" s="1">
         <ns0:f>D124</ns0:f>
-        <ns0:v>2.12e+132</ns0:v>
+        <ns0:v>2.5999999999999997e+132</ns0:v>
       </ns0:c>
       <ns0:c r="F124" s="1">
         <ns0:f>ROUND(F123*1.4,-5)</ns0:f>
-        <ns0:v>2.299313042797801e+38</ns0:v>
+        <ns0:v>1.6560439559331319e+38</ns0:v>
       </ns0:c>
       <ns0:c r="G124" s="1" t="n">
         <ns0:v>25.0000000000001</ns0:v>
@@ -4890,15 +4890,15 @@
       </ns0:c>
       <ns0:c r="D125" s="1">
         <ns0:f>ROUND(D124*20,2-INT(LOG10(ABS(D124*20))))</ns0:f>
-        <ns0:v>4.24e+133</ns0:v>
+        <ns0:v>5.200000000000001e+133</ns0:v>
       </ns0:c>
       <ns0:c r="E125" s="1">
         <ns0:f>D125</ns0:f>
-        <ns0:v>4.24e+133</ns0:v>
+        <ns0:v>5.200000000000001e+133</ns0:v>
       </ns0:c>
       <ns0:c r="F125" s="1">
         <ns0:f>ROUND(F124*1.4,-5)</ns0:f>
-        <ns0:v>3.2190382599169213e+38</ns0:v>
+        <ns0:v>2.3184615383063845e+38</ns0:v>
       </ns0:c>
       <ns0:c r="G125" s="1" t="n">
         <ns0:v>25.2000000000001</ns0:v>
@@ -4922,15 +4922,15 @@
       </ns0:c>
       <ns0:c r="D126" s="1">
         <ns0:f>ROUND(D125*20,2-INT(LOG10(ABS(D125*20))))</ns0:f>
-        <ns0:v>8.48e+134</ns0:v>
+        <ns0:v>1.0399999999999999e+135</ns0:v>
       </ns0:c>
       <ns0:c r="E126" s="1">
         <ns0:f>D126</ns0:f>
-        <ns0:v>8.48e+134</ns0:v>
+        <ns0:v>1.0399999999999999e+135</ns0:v>
       </ns0:c>
       <ns0:c r="F126" s="1">
         <ns0:f>ROUND(F125*1.4,-5)</ns0:f>
-        <ns0:v>4.50665356388369e+38</ns0:v>
+        <ns0:v>3.245846153628938e+38</ns0:v>
       </ns0:c>
       <ns0:c r="G126" s="1" t="n">
         <ns0:v>25.4000000000001</ns0:v>
@@ -4954,15 +4954,15 @@
       </ns0:c>
       <ns0:c r="D127" s="1">
         <ns0:f>ROUND(D126*20,2-INT(LOG10(ABS(D126*20))))</ns0:f>
-        <ns0:v>1.7e+136</ns0:v>
+        <ns0:v>2.08e+136</ns0:v>
       </ns0:c>
       <ns0:c r="E127" s="1">
         <ns0:f>D127</ns0:f>
-        <ns0:v>1.7e+136</ns0:v>
+        <ns0:v>2.08e+136</ns0:v>
       </ns0:c>
       <ns0:c r="F127" s="1">
         <ns0:f>ROUND(F126*1.4,-5)</ns0:f>
-        <ns0:v>6.309314989437165e+38</ns0:v>
+        <ns0:v>4.544184615080513e+38</ns0:v>
       </ns0:c>
       <ns0:c r="G127" s="1" t="n">
         <ns0:v>25.6000000000001</ns0:v>
@@ -4986,15 +4986,15 @@
       </ns0:c>
       <ns0:c r="D128" s="1">
         <ns0:f>ROUND(D127*20,2-INT(LOG10(ABS(D127*20))))</ns0:f>
-        <ns0:v>3.4e+137</ns0:v>
+        <ns0:v>4.16e+137</ns0:v>
       </ns0:c>
       <ns0:c r="E128" s="1">
         <ns0:f>D128</ns0:f>
-        <ns0:v>3.4e+137</ns0:v>
+        <ns0:v>4.16e+137</ns0:v>
       </ns0:c>
       <ns0:c r="F128" s="1">
         <ns0:f>ROUND(F127*1.4,-5)</ns0:f>
-        <ns0:v>8.83304098521203e+38</ns0:v>
+        <ns0:v>6.361858461112718e+38</ns0:v>
       </ns0:c>
       <ns0:c r="G128" s="1" t="n">
         <ns0:v>25.8000000000001</ns0:v>
@@ -5018,15 +5018,15 @@
       </ns0:c>
       <ns0:c r="D129" s="1">
         <ns0:f>ROUND(D128*20,2-INT(LOG10(ABS(D128*20))))</ns0:f>
-        <ns0:v>6.8e+138</ns0:v>
+        <ns0:v>8.32e+138</ns0:v>
       </ns0:c>
       <ns0:c r="E129" s="1">
         <ns0:f>D129</ns0:f>
-        <ns0:v>6.8e+138</ns0:v>
+        <ns0:v>8.32e+138</ns0:v>
       </ns0:c>
       <ns0:c r="F129" s="1">
         <ns0:f>ROUND(F128*1.4,-5)</ns0:f>
-        <ns0:v>1.2366257379296841e+39</ns0:v>
+        <ns0:v>8.906601845557804e+38</ns0:v>
       </ns0:c>
       <ns0:c r="G129" s="1" t="n">
         <ns0:v>26.0000000000001</ns0:v>
@@ -5050,15 +5050,15 @@
       </ns0:c>
       <ns0:c r="D130" s="1">
         <ns0:f>ROUND(D129*20,2-INT(LOG10(ABS(D129*20))))</ns0:f>
-        <ns0:v>1.3599999999999999e+140</ns0:v>
+        <ns0:v>1.6599999999999999e+140</ns0:v>
       </ns0:c>
       <ns0:c r="E130" s="1">
         <ns0:f>D130</ns0:f>
-        <ns0:v>1.3599999999999999e+140</ns0:v>
+        <ns0:v>1.6599999999999999e+140</ns0:v>
       </ns0:c>
       <ns0:c r="F130" s="1">
         <ns0:f>ROUND(F129*1.4,-5)</ns0:f>
-        <ns0:v>1.7312760331015576e+39</ns0:v>
+        <ns0:v>1.2469242583780926e+39</ns0:v>
       </ns0:c>
       <ns0:c r="G130" s="1" t="n">
         <ns0:v>26.2000000000001</ns0:v>
@@ -5082,15 +5082,15 @@
       </ns0:c>
       <ns0:c r="D131" s="1">
         <ns0:f>ROUND(D130*20,2-INT(LOG10(ABS(D130*20))))</ns0:f>
-        <ns0:v>2.72e+141</ns0:v>
+        <ns0:v>3.32e+141</ns0:v>
       </ns0:c>
       <ns0:c r="E131" s="1">
         <ns0:f>D131</ns0:f>
-        <ns0:v>2.72e+141</ns0:v>
+        <ns0:v>3.32e+141</ns0:v>
       </ns0:c>
       <ns0:c r="F131" s="1">
         <ns0:f>ROUND(F130*1.4,-5)</ns0:f>
-        <ns0:v>2.4237864463421808e+39</ns0:v>
+        <ns0:v>1.7456939617293296e+39</ns0:v>
       </ns0:c>
       <ns0:c r="G131" s="1" t="n">
         <ns0:v>26.4000000000001</ns0:v>
@@ -5114,15 +5114,15 @@
       </ns0:c>
       <ns0:c r="D132" s="1">
         <ns0:f>ROUND(D131*20,2-INT(LOG10(ABS(D131*20))))</ns0:f>
-        <ns0:v>5.44e+142</ns0:v>
+        <ns0:v>6.64e+142</ns0:v>
       </ns0:c>
       <ns0:c r="E132" s="1">
         <ns0:f>D132</ns0:f>
-        <ns0:v>5.44e+142</ns0:v>
+        <ns0:v>6.64e+142</ns0:v>
       </ns0:c>
       <ns0:c r="F132" s="1">
         <ns0:f>ROUND(F131*1.4,-5)</ns0:f>
-        <ns0:v>3.393301024879053e+39</ns0:v>
+        <ns0:v>2.443971546421061e+39</ns0:v>
       </ns0:c>
       <ns0:c r="G132" s="1" t="n">
         <ns0:v>26.6000000000001</ns0:v>
@@ -5146,15 +5146,15 @@
       </ns0:c>
       <ns0:c r="D133" s="1">
         <ns0:f>ROUND(D132*20,2-INT(LOG10(ABS(D132*20))))</ns0:f>
-        <ns0:v>1.0899999999999999e+144</ns0:v>
+        <ns0:v>1.33e+144</ns0:v>
       </ns0:c>
       <ns0:c r="E133" s="1">
         <ns0:f>D133</ns0:f>
-        <ns0:v>1.0899999999999999e+144</ns0:v>
+        <ns0:v>1.33e+144</ns0:v>
       </ns0:c>
       <ns0:c r="F133" s="1">
         <ns0:f>ROUND(F132*1.4,-5)</ns0:f>
-        <ns0:v>4.750621434830674e+39</ns0:v>
+        <ns0:v>3.421560164989485e+39</ns0:v>
       </ns0:c>
       <ns0:c r="G133" s="1" t="n">
         <ns0:v>26.8000000000001</ns0:v>
@@ -5178,15 +5178,15 @@
       </ns0:c>
       <ns0:c r="D134" s="1">
         <ns0:f>ROUND(D133*20,2-INT(LOG10(ABS(D133*20))))</ns0:f>
-        <ns0:v>2.18e+145</ns0:v>
+        <ns0:v>2.66e+145</ns0:v>
       </ns0:c>
       <ns0:c r="E134" s="1">
         <ns0:f>D134</ns0:f>
-        <ns0:v>2.18e+145</ns0:v>
+        <ns0:v>2.66e+145</ns0:v>
       </ns0:c>
       <ns0:c r="F134" s="1">
         <ns0:f>ROUND(F133*1.4,-5)</ns0:f>
-        <ns0:v>6.650870008762943e+39</ns0:v>
+        <ns0:v>4.7901842309852785e+39</ns0:v>
       </ns0:c>
       <ns0:c r="G134" s="1" t="n">
         <ns0:v>27.0000000000001</ns0:v>
@@ -5210,15 +5210,15 @@
       </ns0:c>
       <ns0:c r="D135" s="1">
         <ns0:f>ROUND(D134*20,2-INT(LOG10(ABS(D134*20))))</ns0:f>
-        <ns0:v>4.36e+146</ns0:v>
+        <ns0:v>5.3200000000000005e+146</ns0:v>
       </ns0:c>
       <ns0:c r="E135" s="1">
         <ns0:f>D135</ns0:f>
-        <ns0:v>4.36e+146</ns0:v>
+        <ns0:v>5.3200000000000005e+146</ns0:v>
       </ns0:c>
       <ns0:c r="F135" s="1">
         <ns0:f>ROUND(F134*1.4,-5)</ns0:f>
-        <ns0:v>9.31121801226812e+39</ns0:v>
+        <ns0:v>6.70625792337939e+39</ns0:v>
       </ns0:c>
       <ns0:c r="G135" s="1" t="n">
         <ns0:v>27.2000000000001</ns0:v>
@@ -5242,15 +5242,15 @@
       </ns0:c>
       <ns0:c r="D136" s="1">
         <ns0:f>ROUND(D135*20,2-INT(LOG10(ABS(D135*20))))</ns0:f>
-        <ns0:v>8.720000000000001e+147</ns0:v>
+        <ns0:v>1.06e+148</ns0:v>
       </ns0:c>
       <ns0:c r="E136" s="1">
         <ns0:f>D136</ns0:f>
-        <ns0:v>8.720000000000001e+147</ns0:v>
+        <ns0:v>1.06e+148</ns0:v>
       </ns0:c>
       <ns0:c r="F136" s="1">
         <ns0:f>ROUND(F135*1.4,-5)</ns0:f>
-        <ns0:v>1.3035705217175366e+40</ns0:v>
+        <ns0:v>9.388761092731144e+39</ns0:v>
       </ns0:c>
       <ns0:c r="G136" s="1" t="n">
         <ns0:v>27.4000000000001</ns0:v>
@@ -5274,15 +5274,15 @@
       </ns0:c>
       <ns0:c r="D137" s="1">
         <ns0:f>ROUND(D136*20,2-INT(LOG10(ABS(D136*20))))</ns0:f>
-        <ns0:v>1.74e+149</ns0:v>
+        <ns0:v>2.12e+149</ns0:v>
       </ns0:c>
       <ns0:c r="E137" s="1">
         <ns0:f>D137</ns0:f>
-        <ns0:v>1.74e+149</ns0:v>
+        <ns0:v>2.12e+149</ns0:v>
       </ns0:c>
       <ns0:c r="F137" s="1">
         <ns0:f>ROUND(F136*1.4,-5)</ns0:f>
-        <ns0:v>1.824998730404551e+40</ns0:v>
+        <ns0:v>1.31442655298236e+40</ns0:v>
       </ns0:c>
       <ns0:c r="G137" s="1" t="n">
         <ns0:v>27.6000000000001</ns0:v>
@@ -5306,15 +5306,15 @@
       </ns0:c>
       <ns0:c r="D138" s="1">
         <ns0:f>ROUND(D137*20,2-INT(LOG10(ABS(D137*20))))</ns0:f>
-        <ns0:v>3.4800000000000004e+150</ns0:v>
+        <ns0:v>4.24e+150</ns0:v>
       </ns0:c>
       <ns0:c r="E138" s="1">
         <ns0:f>D138</ns0:f>
-        <ns0:v>3.4800000000000004e+150</ns0:v>
+        <ns0:v>4.24e+150</ns0:v>
       </ns0:c>
       <ns0:c r="F138" s="1">
         <ns0:f>ROUND(F137*1.4,-5)</ns0:f>
-        <ns0:v>2.5549982225663714e+40</ns0:v>
+        <ns0:v>1.8401971741753039e+40</ns0:v>
       </ns0:c>
       <ns0:c r="G138" s="1" t="n">
         <ns0:v>27.8000000000001</ns0:v>
@@ -5338,15 +5338,15 @@
       </ns0:c>
       <ns0:c r="D139" s="1">
         <ns0:f>ROUND(D138*20,2-INT(LOG10(ABS(D138*20))))</ns0:f>
-        <ns0:v>6.96e+151</ns0:v>
+        <ns0:v>8.48e+151</ns0:v>
       </ns0:c>
       <ns0:c r="E139" s="1">
         <ns0:f>D139</ns0:f>
-        <ns0:v>6.96e+151</ns0:v>
+        <ns0:v>8.48e+151</ns0:v>
       </ns0:c>
       <ns0:c r="F139" s="1">
         <ns0:f>ROUND(F138*1.4,-5)</ns0:f>
-        <ns0:v>3.57699751159292e+40</ns0:v>
+        <ns0:v>2.576276043845425e+40</ns0:v>
       </ns0:c>
       <ns0:c r="G139" s="1" t="n">
         <ns0:v>28.0000000000001</ns0:v>
@@ -5370,15 +5370,15 @@
       </ns0:c>
       <ns0:c r="D140" s="1">
         <ns0:f>ROUND(D139*20,2-INT(LOG10(ABS(D139*20))))</ns0:f>
-        <ns0:v>1.39e+153</ns0:v>
+        <ns0:v>1.7000000000000002e+153</ns0:v>
       </ns0:c>
       <ns0:c r="E140" s="1">
         <ns0:f>D140</ns0:f>
-        <ns0:v>1.39e+153</ns0:v>
+        <ns0:v>1.7000000000000002e+153</ns0:v>
       </ns0:c>
       <ns0:c r="F140" s="1">
         <ns0:f>ROUND(F139*1.4,-5)</ns0:f>
-        <ns0:v>5.007796516230087e+40</ns0:v>
+        <ns0:v>3.606786461383595e+40</ns0:v>
       </ns0:c>
       <ns0:c r="G140" s="1" t="n">
         <ns0:v>28.2000000000001</ns0:v>
@@ -5402,15 +5402,15 @@
       </ns0:c>
       <ns0:c r="D141" s="1">
         <ns0:f>ROUND(D140*20,2-INT(LOG10(ABS(D140*20))))</ns0:f>
-        <ns0:v>2.7799999999999996e+154</ns0:v>
+        <ns0:v>3.4e+154</ns0:v>
       </ns0:c>
       <ns0:c r="E141" s="1">
         <ns0:f>D141</ns0:f>
-        <ns0:v>2.7799999999999996e+154</ns0:v>
+        <ns0:v>3.4e+154</ns0:v>
       </ns0:c>
       <ns0:c r="F141" s="1">
         <ns0:f>ROUND(F140*1.4,-5)</ns0:f>
-        <ns0:v>7.010915122722121e+40</ns0:v>
+        <ns0:v>5.049501045937033e+40</ns0:v>
       </ns0:c>
       <ns0:c r="G141" s="1" t="n">
         <ns0:v>28.4000000000001</ns0:v>
@@ -5434,15 +5434,15 @@
       </ns0:c>
       <ns0:c r="D142" s="1">
         <ns0:f>ROUND(D141*20,2-INT(LOG10(ABS(D141*20))))</ns0:f>
-        <ns0:v>5.56e+155</ns0:v>
+        <ns0:v>6.8e+155</ns0:v>
       </ns0:c>
       <ns0:c r="E142" s="1">
         <ns0:f>D142</ns0:f>
-        <ns0:v>5.56e+155</ns0:v>
+        <ns0:v>6.8e+155</ns0:v>
       </ns0:c>
       <ns0:c r="F142" s="1">
         <ns0:f>ROUND(F141*1.4,-5)</ns0:f>
-        <ns0:v>9.81528117181097e+40</ns0:v>
+        <ns0:v>7.069301464311845e+40</ns0:v>
       </ns0:c>
       <ns0:c r="G142" s="1" t="n">
         <ns0:v>28.6000000000001</ns0:v>
@@ -5466,15 +5466,15 @@
       </ns0:c>
       <ns0:c r="D143" s="1">
         <ns0:f>ROUND(D142*20,2-INT(LOG10(ABS(D142*20))))</ns0:f>
-        <ns0:v>1.11e+157</ns0:v>
+        <ns0:v>1.36e+157</ns0:v>
       </ns0:c>
       <ns0:c r="E143" s="1">
         <ns0:f>D143</ns0:f>
-        <ns0:v>1.11e+157</ns0:v>
+        <ns0:v>1.36e+157</ns0:v>
       </ns0:c>
       <ns0:c r="F143" s="1">
         <ns0:f>ROUND(F142*1.4,-5)</ns0:f>
-        <ns0:v>1.3741393640535355e+41</ns0:v>
+        <ns0:v>9.897022050036582e+40</ns0:v>
       </ns0:c>
       <ns0:c r="G143" s="1" t="n">
         <ns0:v>28.8000000000001</ns0:v>
@@ -5498,15 +5498,15 @@
       </ns0:c>
       <ns0:c r="D144" s="1">
         <ns0:f>ROUND(D143*20,2-INT(LOG10(ABS(D143*20))))</ns0:f>
-        <ns0:v>2.2199999999999997e+158</ns0:v>
+        <ns0:v>2.72e+158</ns0:v>
       </ns0:c>
       <ns0:c r="E144" s="1">
         <ns0:f>D144</ns0:f>
-        <ns0:v>2.2199999999999997e+158</ns0:v>
+        <ns0:v>2.72e+158</ns0:v>
       </ns0:c>
       <ns0:c r="F144" s="1">
         <ns0:f>ROUND(F143*1.4,-5)</ns0:f>
-        <ns0:v>1.9237951096749496e+41</ns0:v>
+        <ns0:v>1.3855830870051214e+41</ns0:v>
       </ns0:c>
       <ns0:c r="G144" s="1" t="n">
         <ns0:v>29.0000000000001</ns0:v>
@@ -5530,15 +5530,15 @@
       </ns0:c>
       <ns0:c r="D145" s="1">
         <ns0:f>ROUND(D144*20,2-INT(LOG10(ABS(D144*20))))</ns0:f>
-        <ns0:v>4.44e+159</ns0:v>
+        <ns0:v>5.440000000000001e+159</ns0:v>
       </ns0:c>
       <ns0:c r="E145" s="1">
         <ns0:f>D145</ns0:f>
-        <ns0:v>4.44e+159</ns0:v>
+        <ns0:v>5.440000000000001e+159</ns0:v>
       </ns0:c>
       <ns0:c r="F145" s="1">
         <ns0:f>ROUND(F144*1.4,-5)</ns0:f>
-        <ns0:v>2.693313153544929e+41</ns0:v>
+        <ns0:v>1.9398163218071697e+41</ns0:v>
       </ns0:c>
       <ns0:c r="G145" s="1" t="n">
         <ns0:v>29.2000000000001</ns0:v>
@@ -5562,15 +5562,15 @@
       </ns0:c>
       <ns0:c r="D146" s="1">
         <ns0:f>ROUND(D145*20,2-INT(LOG10(ABS(D145*20))))</ns0:f>
-        <ns0:v>8.88e+160</ns0:v>
+        <ns0:v>1.09e+161</ns0:v>
       </ns0:c>
       <ns0:c r="E146" s="1">
         <ns0:f>D146</ns0:f>
-        <ns0:v>8.88e+160</ns0:v>
+        <ns0:v>1.09e+161</ns0:v>
       </ns0:c>
       <ns0:c r="F146" s="1">
         <ns0:f>ROUND(F145*1.4,-5)</ns0:f>
-        <ns0:v>3.7706384149629006e+41</ns0:v>
+        <ns0:v>2.7157428505300373e+41</ns0:v>
       </ns0:c>
       <ns0:c r="G146" s="1" t="n">
         <ns0:v>29.4000000000001</ns0:v>
@@ -5594,15 +5594,15 @@
       </ns0:c>
       <ns0:c r="D147" s="1">
         <ns0:f>ROUND(D146*20,2-INT(LOG10(ABS(D146*20))))</ns0:f>
-        <ns0:v>1.78e+162</ns0:v>
+        <ns0:v>2.18e+162</ns0:v>
       </ns0:c>
       <ns0:c r="E147" s="1">
         <ns0:f>D147</ns0:f>
-        <ns0:v>1.78e+162</ns0:v>
+        <ns0:v>2.18e+162</ns0:v>
       </ns0:c>
       <ns0:c r="F147" s="1">
         <ns0:f>ROUND(F146*1.4,-5)</ns0:f>
-        <ns0:v>5.2788937809480605e+41</ns0:v>
+        <ns0:v>3.802039990742052e+41</ns0:v>
       </ns0:c>
       <ns0:c r="G147" s="1" t="n">
         <ns0:v>29.6000000000001</ns0:v>
@@ -5626,15 +5626,15 @@
       </ns0:c>
       <ns0:c r="D148" s="1">
         <ns0:f>ROUND(D147*20,2-INT(LOG10(ABS(D147*20))))</ns0:f>
-        <ns0:v>3.56e+163</ns0:v>
+        <ns0:v>4.3599999999999997e+163</ns0:v>
       </ns0:c>
       <ns0:c r="E148" s="1">
         <ns0:f>D148</ns0:f>
-        <ns0:v>3.56e+163</ns0:v>
+        <ns0:v>4.3599999999999997e+163</ns0:v>
       </ns0:c>
       <ns0:c r="F148" s="1">
         <ns0:f>ROUND(F147*1.4,-5)</ns0:f>
-        <ns0:v>7.390451293327283e+41</ns0:v>
+        <ns0:v>5.322855987038872e+41</ns0:v>
       </ns0:c>
       <ns0:c r="G148" s="1" t="n">
         <ns0:v>29.8000000000001</ns0:v>
@@ -5658,15 +5658,15 @@
       </ns0:c>
       <ns0:c r="D149" s="1">
         <ns0:f>ROUND(D148*20,2-INT(LOG10(ABS(D148*20))))</ns0:f>
-        <ns0:v>7.120000000000001e+164</ns0:v>
+        <ns0:v>8.72e+164</ns0:v>
       </ns0:c>
       <ns0:c r="E149" s="1">
         <ns0:f>D149</ns0:f>
-        <ns0:v>7.120000000000001e+164</ns0:v>
+        <ns0:v>8.72e+164</ns0:v>
       </ns0:c>
       <ns0:c r="F149" s="1">
         <ns0:f>ROUND(F148*1.4,-5)</ns0:f>
-        <ns0:v>1.0346631810658196e+42</ns0:v>
+        <ns0:v>7.45199838185442e+41</ns0:v>
       </ns0:c>
       <ns0:c r="G149" s="1" t="n">
         <ns0:v>30.0000000000001</ns0:v>
@@ -5690,15 +5690,15 @@
       </ns0:c>
       <ns0:c r="D150" s="1">
         <ns0:f>ROUND(D149*20,2-INT(LOG10(ABS(D149*20))))</ns0:f>
-        <ns0:v>1.4200000000000001e+166</ns0:v>
+        <ns0:v>1.74e+166</ns0:v>
       </ns0:c>
       <ns0:c r="E150" s="1">
         <ns0:f>D150</ns0:f>
-        <ns0:v>1.4200000000000001e+166</ns0:v>
+        <ns0:v>1.74e+166</ns0:v>
       </ns0:c>
       <ns0:c r="F150" s="1">
         <ns0:f>ROUND(F149*1.4,-5)</ns0:f>
-        <ns0:v>1.4485284534921475e+42</ns0:v>
+        <ns0:v>1.0432797734596187e+42</ns0:v>
       </ns0:c>
       <ns0:c r="G150" s="1" t="n">
         <ns0:v>30.2000000000001</ns0:v>
@@ -5722,15 +5722,15 @@
       </ns0:c>
       <ns0:c r="D151" s="1">
         <ns0:f>ROUND(D150*20,2-INT(LOG10(ABS(D150*20))))</ns0:f>
-        <ns0:v>2.84e+167</ns0:v>
+        <ns0:v>3.48e+167</ns0:v>
       </ns0:c>
       <ns0:c r="E151" s="1">
         <ns0:f>D151</ns0:f>
-        <ns0:v>2.84e+167</ns0:v>
+        <ns0:v>3.48e+167</ns0:v>
       </ns0:c>
       <ns0:c r="F151" s="1">
         <ns0:f>ROUND(F150*1.4,-5)</ns0:f>
-        <ns0:v>2.0279398348890064e+42</ns0:v>
+        <ns0:v>1.4605916828434662e+42</ns0:v>
       </ns0:c>
       <ns0:c r="G151" s="1" t="n">
         <ns0:v>30.4000000000001</ns0:v>
@@ -5754,15 +5754,15 @@
       </ns0:c>
       <ns0:c r="D152" s="1">
         <ns0:f>ROUND(D151*20,2-INT(LOG10(ABS(D151*20))))</ns0:f>
-        <ns0:v>5.68e+168</ns0:v>
+        <ns0:v>6.96e+168</ns0:v>
       </ns0:c>
       <ns0:c r="E152" s="1">
         <ns0:f>D152</ns0:f>
-        <ns0:v>5.68e+168</ns0:v>
+        <ns0:v>6.96e+168</ns0:v>
       </ns0:c>
       <ns0:c r="F152" s="1">
         <ns0:f>ROUND(F151*1.4,-5)</ns0:f>
-        <ns0:v>2.8391157688446086e+42</ns0:v>
+        <ns0:v>2.0448283559808525e+42</ns0:v>
       </ns0:c>
       <ns0:c r="G152" s="1" t="n">
         <ns0:v>30.6000000000001</ns0:v>
@@ -5786,15 +5786,15 @@
       </ns0:c>
       <ns0:c r="D153" s="1">
         <ns0:f>ROUND(D152*20,2-INT(LOG10(ABS(D152*20))))</ns0:f>
-        <ns0:v>1.1399999999999999e+170</ns0:v>
+        <ns0:v>1.3899999999999998e+170</ns0:v>
       </ns0:c>
       <ns0:c r="E153" s="1">
         <ns0:f>D153</ns0:f>
-        <ns0:v>1.1399999999999999e+170</ns0:v>
+        <ns0:v>1.3899999999999998e+170</ns0:v>
       </ns0:c>
       <ns0:c r="F153" s="1">
         <ns0:f>ROUND(F152*1.4,-5)</ns0:f>
-        <ns0:v>3.974762076382452e+42</ns0:v>
+        <ns0:v>2.8627596983731936e+42</ns0:v>
       </ns0:c>
       <ns0:c r="G153" s="1" t="n">
         <ns0:v>30.8000000000001</ns0:v>
@@ -5818,15 +5818,15 @@
       </ns0:c>
       <ns0:c r="D154" s="1">
         <ns0:f>ROUND(D153*20,2-INT(LOG10(ABS(D153*20))))</ns0:f>
-        <ns0:v>2.28e+171</ns0:v>
+        <ns0:v>2.7799999999999997e+171</ns0:v>
       </ns0:c>
       <ns0:c r="E154" s="1">
         <ns0:f>D154</ns0:f>
-        <ns0:v>2.28e+171</ns0:v>
+        <ns0:v>2.7799999999999997e+171</ns0:v>
       </ns0:c>
       <ns0:c r="F154" s="1">
         <ns0:f>ROUND(F153*1.4,-5)</ns0:f>
-        <ns0:v>5.5646669069354325e+42</ns0:v>
+        <ns0:v>4.0078635777224706e+42</ns0:v>
       </ns0:c>
       <ns0:c r="G154" s="1" t="n">
         <ns0:v>31.0000000000001</ns0:v>
@@ -5850,15 +5850,15 @@
       </ns0:c>
       <ns0:c r="D155" s="1">
         <ns0:f>ROUND(D154*20,2-INT(LOG10(ABS(D154*20))))</ns0:f>
-        <ns0:v>4.56e+172</ns0:v>
+        <ns0:v>5.56e+172</ns0:v>
       </ns0:c>
       <ns0:c r="E155" s="1">
         <ns0:f>D155</ns0:f>
-        <ns0:v>4.56e+172</ns0:v>
+        <ns0:v>5.56e+172</ns0:v>
       </ns0:c>
       <ns0:c r="F155" s="1">
         <ns0:f>ROUND(F154*1.4,-5)</ns0:f>
-        <ns0:v>7.790533669709605e+42</ns0:v>
+        <ns0:v>5.611009008811459e+42</ns0:v>
       </ns0:c>
       <ns0:c r="G155" s="1" t="n">
         <ns0:v>31.2000000000001</ns0:v>
@@ -5882,15 +5882,15 @@
       </ns0:c>
       <ns0:c r="D156" s="1">
         <ns0:f>ROUND(D155*20,2-INT(LOG10(ABS(D155*20))))</ns0:f>
-        <ns0:v>9.12e+173</ns0:v>
+        <ns0:v>1.11e+174</ns0:v>
       </ns0:c>
       <ns0:c r="E156" s="1">
         <ns0:f>D156</ns0:f>
-        <ns0:v>9.12e+173</ns0:v>
+        <ns0:v>1.11e+174</ns0:v>
       </ns0:c>
       <ns0:c r="F156" s="1">
         <ns0:f>ROUND(F155*1.4,-5)</ns0:f>
-        <ns0:v>1.0906747137593445e+43</ns0:v>
+        <ns0:v>7.855412612336042e+42</ns0:v>
       </ns0:c>
       <ns0:c r="G156" s="1" t="n">
         <ns0:v>31.4000000000001</ns0:v>
@@ -5914,15 +5914,15 @@
       </ns0:c>
       <ns0:c r="D157" s="1">
         <ns0:f>ROUND(D156*20,2-INT(LOG10(ABS(D156*20))))</ns0:f>
-        <ns0:v>1.8199999999999998e+175</ns0:v>
+        <ns0:v>2.22e+175</ns0:v>
       </ns0:c>
       <ns0:c r="E157" s="1">
         <ns0:f>D157</ns0:f>
-        <ns0:v>1.8199999999999998e+175</ns0:v>
+        <ns0:v>2.22e+175</ns0:v>
       </ns0:c>
       <ns0:c r="F157" s="1">
         <ns0:f>ROUND(F156*1.4,-5)</ns0:f>
-        <ns0:v>1.5269445992630822e+43</ns0:v>
+        <ns0:v>1.0997577657270457e+43</ns0:v>
       </ns0:c>
       <ns0:c r="G157" s="1" t="n">
         <ns0:v>31.6000000000001</ns0:v>
@@ -5946,15 +5946,15 @@
       </ns0:c>
       <ns0:c r="D158" s="1">
         <ns0:f>ROUND(D157*20,2-INT(LOG10(ABS(D157*20))))</ns0:f>
-        <ns0:v>3.64e+176</ns0:v>
+        <ns0:v>4.44e+176</ns0:v>
       </ns0:c>
       <ns0:c r="E158" s="1">
         <ns0:f>D158</ns0:f>
-        <ns0:v>3.64e+176</ns0:v>
+        <ns0:v>4.44e+176</ns0:v>
       </ns0:c>
       <ns0:c r="F158" s="1">
         <ns0:f>ROUND(F157*1.4,-5)</ns0:f>
-        <ns0:v>2.137722438968315e+43</ns0:v>
+        <ns0:v>1.539660872017864e+43</ns0:v>
       </ns0:c>
       <ns0:c r="G158" s="1" t="n">
         <ns0:v>31.8000000000001</ns0:v>
@@ -5978,15 +5978,15 @@
       </ns0:c>
       <ns0:c r="D159" s="1">
         <ns0:f>ROUND(D158*20,2-INT(LOG10(ABS(D158*20))))</ns0:f>
-        <ns0:v>7.28e+177</ns0:v>
+        <ns0:v>8.88e+177</ns0:v>
       </ns0:c>
       <ns0:c r="E159" s="1">
         <ns0:f>D159</ns0:f>
-        <ns0:v>7.28e+177</ns0:v>
+        <ns0:v>8.88e+177</ns0:v>
       </ns0:c>
       <ns0:c r="F159" s="1">
         <ns0:f>ROUND(F158*1.4,-5)</ns0:f>
-        <ns0:v>2.9928114145556406e+43</ns0:v>
+        <ns0:v>2.1555252208250092e+43</ns0:v>
       </ns0:c>
       <ns0:c r="G159" s="1" t="n">
         <ns0:v>32.0000000000001</ns0:v>
@@ -6010,15 +6010,15 @@
       </ns0:c>
       <ns0:c r="D160" s="1">
         <ns0:f>ROUND(D159*20,2-INT(LOG10(ABS(D159*20))))</ns0:f>
-        <ns0:v>1.46e+179</ns0:v>
+        <ns0:v>1.78e+179</ns0:v>
       </ns0:c>
       <ns0:c r="E160" s="1">
         <ns0:f>D160</ns0:f>
-        <ns0:v>1.46e+179</ns0:v>
+        <ns0:v>1.78e+179</ns0:v>
       </ns0:c>
       <ns0:c r="F160" s="1">
         <ns0:f>ROUND(F159*1.4,-5)</ns0:f>
-        <ns0:v>4.1899359803778964e+43</ns0:v>
+        <ns0:v>3.0177353091550127e+43</ns0:v>
       </ns0:c>
       <ns0:c r="G160" s="1" t="n">
         <ns0:v>32.2000000000001</ns0:v>
@@ -6042,15 +6042,15 @@
       </ns0:c>
       <ns0:c r="D161" s="1">
         <ns0:f>ROUND(D160*20,2-INT(LOG10(ABS(D160*20))))</ns0:f>
-        <ns0:v>2.9200000000000003e+180</ns0:v>
+        <ns0:v>3.56e+180</ns0:v>
       </ns0:c>
       <ns0:c r="E161" s="1">
         <ns0:f>D161</ns0:f>
-        <ns0:v>2.9200000000000003e+180</ns0:v>
+        <ns0:v>3.56e+180</ns0:v>
       </ns0:c>
       <ns0:c r="F161" s="1">
         <ns0:f>ROUND(F160*1.4,-5)</ns0:f>
-        <ns0:v>5.865910372529055e+43</ns0:v>
+        <ns0:v>4.2248294328170174e+43</ns0:v>
       </ns0:c>
       <ns0:c r="G161" s="1" t="n">
         <ns0:v>32.4000000000001</ns0:v>
@@ -6074,15 +6074,15 @@
       </ns0:c>
       <ns0:c r="D162" s="1">
         <ns0:f>ROUND(D161*20,2-INT(LOG10(ABS(D161*20))))</ns0:f>
-        <ns0:v>5.8399999999999996e+181</ns0:v>
+        <ns0:v>7.12e+181</ns0:v>
       </ns0:c>
       <ns0:c r="E162" s="1">
         <ns0:f>D162</ns0:f>
-        <ns0:v>5.8399999999999996e+181</ns0:v>
+        <ns0:v>7.12e+181</ns0:v>
       </ns0:c>
       <ns0:c r="F162" s="1">
         <ns0:f>ROUND(F161*1.4,-5)</ns0:f>
-        <ns0:v>8.212274521540677e+43</ns0:v>
+        <ns0:v>5.914761205943824e+43</ns0:v>
       </ns0:c>
       <ns0:c r="G162" s="1" t="n">
         <ns0:v>32.6000000000001</ns0:v>
@@ -6106,15 +6106,15 @@
       </ns0:c>
       <ns0:c r="D163" s="1">
         <ns0:f>ROUND(D162*20,2-INT(LOG10(ABS(D162*20))))</ns0:f>
-        <ns0:v>1.17e+183</ns0:v>
+        <ns0:v>1.42e+183</ns0:v>
       </ns0:c>
       <ns0:c r="E163" s="1">
         <ns0:f>D163</ns0:f>
-        <ns0:v>1.17e+183</ns0:v>
+        <ns0:v>1.42e+183</ns0:v>
       </ns0:c>
       <ns0:c r="F163" s="1">
         <ns0:f>ROUND(F162*1.4,-5)</ns0:f>
-        <ns0:v>1.1497184330156946e+44</ns0:v>
+        <ns0:v>8.280665688321353e+43</ns0:v>
       </ns0:c>
       <ns0:c r="G163" s="1" t="n">
         <ns0:v>32.8000000000001</ns0:v>
@@ -6138,15 +6138,15 @@
       </ns0:c>
       <ns0:c r="D164" s="1">
         <ns0:f>ROUND(D163*20,2-INT(LOG10(ABS(D163*20))))</ns0:f>
-        <ns0:v>2.3399999999999998e+184</ns0:v>
+        <ns0:v>2.84e+184</ns0:v>
       </ns0:c>
       <ns0:c r="E164" s="1">
         <ns0:f>D164</ns0:f>
-        <ns0:v>2.3399999999999998e+184</ns0:v>
+        <ns0:v>2.84e+184</ns0:v>
       </ns0:c>
       <ns0:c r="F164" s="1">
         <ns0:f>ROUND(F163*1.4,-5)</ns0:f>
-        <ns0:v>1.609605806221972e+44</ns0:v>
+        <ns0:v>1.1592931963649895e+44</ns0:v>
       </ns0:c>
       <ns0:c r="G164" s="1" t="n">
         <ns0:v>33.0000000000001</ns0:v>
@@ -6170,15 +6170,15 @@
       </ns0:c>
       <ns0:c r="D165" s="1">
         <ns0:f>ROUND(D164*20,2-INT(LOG10(ABS(D164*20))))</ns0:f>
-        <ns0:v>4.68e+185</ns0:v>
+        <ns0:v>5.68e+185</ns0:v>
       </ns0:c>
       <ns0:c r="E165" s="1">
         <ns0:f>D165</ns0:f>
-        <ns0:v>4.68e+185</ns0:v>
+        <ns0:v>5.68e+185</ns0:v>
       </ns0:c>
       <ns0:c r="F165" s="1">
         <ns0:f>ROUND(F164*1.4,-5)</ns0:f>
-        <ns0:v>2.253448128710761e+44</ns0:v>
+        <ns0:v>1.6230104749109852e+44</ns0:v>
       </ns0:c>
       <ns0:c r="G165" s="1" t="n">
         <ns0:v>33.2000000000001</ns0:v>
@@ -6202,15 +6202,15 @@
       </ns0:c>
       <ns0:c r="D166" s="1">
         <ns0:f>ROUND(D165*20,2-INT(LOG10(ABS(D165*20))))</ns0:f>
-        <ns0:v>9.359999999999999e+186</ns0:v>
+        <ns0:v>1.14e+187</ns0:v>
       </ns0:c>
       <ns0:c r="E166" s="1">
         <ns0:f>D166</ns0:f>
-        <ns0:v>9.359999999999999e+186</ns0:v>
+        <ns0:v>1.14e+187</ns0:v>
       </ns0:c>
       <ns0:c r="F166" s="1">
         <ns0:f>ROUND(F165*1.4,-5)</ns0:f>
-        <ns0:v>3.154827380195065e+44</ns0:v>
+        <ns0:v>2.2722146648753793e+44</ns0:v>
       </ns0:c>
       <ns0:c r="G166" s="1" t="n">
         <ns0:v>33.4000000000001</ns0:v>
@@ -6234,15 +6234,15 @@
       </ns0:c>
       <ns0:c r="D167" s="1">
         <ns0:f>ROUND(D166*20,2-INT(LOG10(ABS(D166*20))))</ns0:f>
-        <ns0:v>1.87e+188</ns0:v>
+        <ns0:v>2.28e+188</ns0:v>
       </ns0:c>
       <ns0:c r="E167" s="1">
         <ns0:f>D167</ns0:f>
-        <ns0:v>1.87e+188</ns0:v>
+        <ns0:v>2.28e+188</ns0:v>
       </ns0:c>
       <ns0:c r="F167" s="1">
         <ns0:f>ROUND(F166*1.4,-5)</ns0:f>
-        <ns0:v>4.416758332273091e+44</ns0:v>
+        <ns0:v>3.181100530825531e+44</ns0:v>
       </ns0:c>
       <ns0:c r="G167" s="1" t="n">
         <ns0:v>33.6000000000001</ns0:v>
@@ -6266,15 +6266,15 @@
       </ns0:c>
       <ns0:c r="D168" s="1">
         <ns0:f>ROUND(D167*20,2-INT(LOG10(ABS(D167*20))))</ns0:f>
-        <ns0:v>3.74e+189</ns0:v>
+        <ns0:v>4.56e+189</ns0:v>
       </ns0:c>
       <ns0:c r="E168" s="1">
         <ns0:f>D168</ns0:f>
-        <ns0:v>3.74e+189</ns0:v>
+        <ns0:v>4.56e+189</ns0:v>
       </ns0:c>
       <ns0:c r="F168" s="1">
         <ns0:f>ROUND(F167*1.4,-5)</ns0:f>
-        <ns0:v>6.183461665182327e+44</ns0:v>
+        <ns0:v>4.4535407431557436e+44</ns0:v>
       </ns0:c>
       <ns0:c r="G168" s="1" t="n">
         <ns0:v>33.8000000000001</ns0:v>
@@ -6298,15 +6298,15 @@
       </ns0:c>
       <ns0:c r="D169" s="1">
         <ns0:f>ROUND(D168*20,2-INT(LOG10(ABS(D168*20))))</ns0:f>
-        <ns0:v>7.48e+190</ns0:v>
+        <ns0:v>9.12e+190</ns0:v>
       </ns0:c>
       <ns0:c r="E169" s="1">
         <ns0:f>D169</ns0:f>
-        <ns0:v>7.48e+190</ns0:v>
+        <ns0:v>9.12e+190</ns0:v>
       </ns0:c>
       <ns0:c r="F169" s="1">
         <ns0:f>ROUND(F168*1.4,-5)</ns0:f>
-        <ns0:v>8.656846331255258e+44</ns0:v>
+        <ns0:v>6.234957040418041e+44</ns0:v>
       </ns0:c>
       <ns0:c r="G169" s="1" t="n">
         <ns0:v>34.0000000000001</ns0:v>
@@ -6330,15 +6330,15 @@
       </ns0:c>
       <ns0:c r="D170" s="1">
         <ns0:f>ROUND(D169*20,2-INT(LOG10(ABS(D169*20))))</ns0:f>
-        <ns0:v>1.5e+192</ns0:v>
+        <ns0:v>1.82e+192</ns0:v>
       </ns0:c>
       <ns0:c r="E170" s="1">
         <ns0:f>D170</ns0:f>
-        <ns0:v>1.5e+192</ns0:v>
+        <ns0:v>1.82e+192</ns0:v>
       </ns0:c>
       <ns0:c r="F170" s="1">
         <ns0:f>ROUND(F169*1.4,-5)</ns0:f>
-        <ns0:v>1.211958486375736e+45</ns0:v>
+        <ns0:v>8.728939856585256e+44</ns0:v>
       </ns0:c>
       <ns0:c r="G170" s="1" t="n">
         <ns0:v>34.2000000000001</ns0:v>
@@ -6362,15 +6362,15 @@
       </ns0:c>
       <ns0:c r="D171" s="1">
         <ns0:f>ROUND(D170*20,2-INT(LOG10(ABS(D170*20))))</ns0:f>
-        <ns0:v>3e+193</ns0:v>
+        <ns0:v>3.64e+193</ns0:v>
       </ns0:c>
       <ns0:c r="E171" s="1">
         <ns0:f>D171</ns0:f>
-        <ns0:v>3e+193</ns0:v>
+        <ns0:v>3.64e+193</ns0:v>
       </ns0:c>
       <ns0:c r="F171" s="1">
         <ns0:f>ROUND(F170*1.4,-5)</ns0:f>
-        <ns0:v>1.6967418809260303e+45</ns0:v>
+        <ns0:v>1.2220515799219357e+45</ns0:v>
       </ns0:c>
       <ns0:c r="G171" s="1" t="n">
         <ns0:v>34.4000000000001</ns0:v>
@@ -6394,15 +6394,15 @@
       </ns0:c>
       <ns0:c r="D172" s="1">
         <ns0:f>ROUND(D171*20,2-INT(LOG10(ABS(D171*20))))</ns0:f>
-        <ns0:v>5.999999999999999e+194</ns0:v>
+        <ns0:v>7.279999999999999e+194</ns0:v>
       </ns0:c>
       <ns0:c r="E172" s="1">
         <ns0:f>D172</ns0:f>
-        <ns0:v>5.999999999999999e+194</ns0:v>
+        <ns0:v>7.279999999999999e+194</ns0:v>
       </ns0:c>
       <ns0:c r="F172" s="1">
         <ns0:f>ROUND(F171*1.4,-5)</ns0:f>
-        <ns0:v>2.3754386332964422e+45</ns0:v>
+        <ns0:v>1.71087221189071e+45</ns0:v>
       </ns0:c>
       <ns0:c r="G172" s="1" t="n">
         <ns0:v>34.6000000000001</ns0:v>
@@ -6426,15 +6426,15 @@
       </ns0:c>
       <ns0:c r="D173" s="1">
         <ns0:f>ROUND(D172*20,2-INT(LOG10(ABS(D172*20))))</ns0:f>
-        <ns0:v>1.2e+196</ns0:v>
+        <ns0:v>1.4599999999999999e+196</ns0:v>
       </ns0:c>
       <ns0:c r="E173" s="1">
         <ns0:f>D173</ns0:f>
-        <ns0:v>1.2e+196</ns0:v>
+        <ns0:v>1.4599999999999999e+196</ns0:v>
       </ns0:c>
       <ns0:c r="F173" s="1">
         <ns0:f>ROUND(F172*1.4,-5)</ns0:f>
-        <ns0:v>3.325614086615019e+45</ns0:v>
+        <ns0:v>2.395221096646994e+45</ns0:v>
       </ns0:c>
       <ns0:c r="G173" s="1" t="n">
         <ns0:v>34.8000000000001</ns0:v>
@@ -6458,15 +6458,15 @@
       </ns0:c>
       <ns0:c r="D174" s="1">
         <ns0:f>ROUND(D173*20,2-INT(LOG10(ABS(D173*20))))</ns0:f>
-        <ns0:v>2.4e+197</ns0:v>
+        <ns0:v>2.9199999999999997e+197</ns0:v>
       </ns0:c>
       <ns0:c r="E174" s="1">
         <ns0:f>D174</ns0:f>
-        <ns0:v>2.4e+197</ns0:v>
+        <ns0:v>2.9199999999999997e+197</ns0:v>
       </ns0:c>
       <ns0:c r="F174" s="1">
         <ns0:f>ROUND(F173*1.4,-5)</ns0:f>
-        <ns0:v>4.655859721261025e+45</ns0:v>
+        <ns0:v>3.3533095353057913e+45</ns0:v>
       </ns0:c>
       <ns0:c r="G174" s="1" t="n">
         <ns0:v>35.0000000000001</ns0:v>
@@ -6490,15 +6490,15 @@
       </ns0:c>
       <ns0:c r="D175" s="1">
         <ns0:f>ROUND(D174*20,2-INT(LOG10(ABS(D174*20))))</ns0:f>
-        <ns0:v>4.8e+198</ns0:v>
+        <ns0:v>5.84e+198</ns0:v>
       </ns0:c>
       <ns0:c r="E175" s="1">
         <ns0:f>D175</ns0:f>
-        <ns0:v>4.8e+198</ns0:v>
+        <ns0:v>5.84e+198</ns0:v>
       </ns0:c>
       <ns0:c r="F175" s="1">
         <ns0:f>ROUND(F174*1.4,-5)</ns0:f>
-        <ns0:v>6.518203609765435e+45</ns0:v>
+        <ns0:v>4.6946333494281075e+45</ns0:v>
       </ns0:c>
       <ns0:c r="G175" s="1" t="n">
         <ns0:v>35.2000000000001</ns0:v>
@@ -6522,15 +6522,15 @@
       </ns0:c>
       <ns0:c r="D176" s="1">
         <ns0:f>ROUND(D175*20,2-INT(LOG10(ABS(D175*20))))</ns0:f>
-        <ns0:v>9.6e+199</ns0:v>
+        <ns0:v>1.17e+200</ns0:v>
       </ns0:c>
       <ns0:c r="E176" s="1">
         <ns0:f>D176</ns0:f>
-        <ns0:v>9.6e+199</ns0:v>
+        <ns0:v>1.17e+200</ns0:v>
       </ns0:c>
       <ns0:c r="F176" s="1">
         <ns0:f>ROUND(F175*1.4,-5)</ns0:f>
-        <ns0:v>9.125485053671609e+45</ns0:v>
+        <ns0:v>6.57248668919935e+45</ns0:v>
       </ns0:c>
       <ns0:c r="G176" s="1" t="n">
         <ns0:v>35.4000000000001</ns0:v>
@@ -6554,15 +6554,15 @@
       </ns0:c>
       <ns0:c r="D177" s="1">
         <ns0:f>ROUND(D176*20,2-INT(LOG10(ABS(D176*20))))</ns0:f>
-        <ns0:v>1.92e+201</ns0:v>
+        <ns0:v>2.34e+201</ns0:v>
       </ns0:c>
       <ns0:c r="E177" s="1">
         <ns0:f>D177</ns0:f>
-        <ns0:v>1.92e+201</ns0:v>
+        <ns0:v>2.34e+201</ns0:v>
       </ns0:c>
       <ns0:c r="F177" s="1">
         <ns0:f>ROUND(F176*1.4,-5)</ns0:f>
-        <ns0:v>1.2775679075140252e+46</ns0:v>
+        <ns0:v>9.20148136487909e+45</ns0:v>
       </ns0:c>
       <ns0:c r="G177" s="1" t="n">
         <ns0:v>35.6000000000001</ns0:v>
@@ -6586,15 +6586,15 @@
       </ns0:c>
       <ns0:c r="D178" s="1">
         <ns0:f>ROUND(D177*20,2-INT(LOG10(ABS(D177*20))))</ns0:f>
-        <ns0:v>3.84e+202</ns0:v>
+        <ns0:v>4.6800000000000005e+202</ns0:v>
       </ns0:c>
       <ns0:c r="E178" s="1">
         <ns0:f>D178</ns0:f>
-        <ns0:v>3.84e+202</ns0:v>
+        <ns0:v>4.6800000000000005e+202</ns0:v>
       </ns0:c>
       <ns0:c r="F178" s="1">
         <ns0:f>ROUND(F177*1.4,-5)</ns0:f>
-        <ns0:v>1.7885950705196354e+46</ns0:v>
+        <ns0:v>1.2882073910830726e+46</ns0:v>
       </ns0:c>
       <ns0:c r="G178" s="1" t="n">
         <ns0:v>35.8000000000001</ns0:v>
@@ -6618,15 +6618,15 @@
       </ns0:c>
       <ns0:c r="D179" s="1">
         <ns0:f>ROUND(D178*20,2-INT(LOG10(ABS(D178*20))))</ns0:f>
-        <ns0:v>7.68e+203</ns0:v>
+        <ns0:v>9.36e+203</ns0:v>
       </ns0:c>
       <ns0:c r="E179" s="1">
         <ns0:f>D179</ns0:f>
-        <ns0:v>7.68e+203</ns0:v>
+        <ns0:v>9.36e+203</ns0:v>
       </ns0:c>
       <ns0:c r="F179" s="1">
         <ns0:f>ROUND(F178*1.4,-5)</ns0:f>
-        <ns0:v>2.5040330987274893e+46</ns0:v>
+        <ns0:v>1.8034903475163013e+46</ns0:v>
       </ns0:c>
       <ns0:c r="G179" s="1" t="n">
         <ns0:v>36.0000000000001</ns0:v>
@@ -6650,15 +6650,15 @@
       </ns0:c>
       <ns0:c r="D180" s="1">
         <ns0:f>ROUND(D179*20,2-INT(LOG10(ABS(D179*20))))</ns0:f>
-        <ns0:v>1.5399999999999999e+205</ns0:v>
+        <ns0:v>1.8699999999999999e+205</ns0:v>
       </ns0:c>
       <ns0:c r="E180" s="1">
         <ns0:f>D180</ns0:f>
-        <ns0:v>1.5399999999999999e+205</ns0:v>
+        <ns0:v>1.8699999999999999e+205</ns0:v>
       </ns0:c>
       <ns0:c r="F180" s="1">
         <ns0:f>ROUND(F179*1.4,-5)</ns0:f>
-        <ns0:v>3.5056463382184853e+46</ns0:v>
+        <ns0:v>2.524886486522822e+46</ns0:v>
       </ns0:c>
       <ns0:c r="G180" s="1" t="n">
         <ns0:v>36.2000000000001</ns0:v>
@@ -6682,15 +6682,15 @@
       </ns0:c>
       <ns0:c r="D181" s="1">
         <ns0:f>ROUND(D180*20,2-INT(LOG10(ABS(D180*20))))</ns0:f>
-        <ns0:v>3.08e+206</ns0:v>
+        <ns0:v>3.74e+206</ns0:v>
       </ns0:c>
       <ns0:c r="E181" s="1">
         <ns0:f>D181</ns0:f>
-        <ns0:v>3.08e+206</ns0:v>
+        <ns0:v>3.74e+206</ns0:v>
       </ns0:c>
       <ns0:c r="F181" s="1">
         <ns0:f>ROUND(F180*1.4,-5)</ns0:f>
-        <ns0:v>4.907904873505879e+46</ns0:v>
+        <ns0:v>3.5348410811319504e+46</ns0:v>
       </ns0:c>
       <ns0:c r="G181" s="1" t="n">
         <ns0:v>36.4000000000001</ns0:v>
@@ -6714,15 +6714,15 @@
       </ns0:c>
       <ns0:c r="D182" s="1">
         <ns0:f>ROUND(D181*20,2-INT(LOG10(ABS(D181*20))))</ns0:f>
-        <ns0:v>6.16e+207</ns0:v>
+        <ns0:v>7.48e+207</ns0:v>
       </ns0:c>
       <ns0:c r="E182" s="1">
         <ns0:f>D182</ns0:f>
-        <ns0:v>6.16e+207</ns0:v>
+        <ns0:v>7.48e+207</ns0:v>
       </ns0:c>
       <ns0:c r="F182" s="1">
         <ns0:f>ROUND(F181*1.4,-5)</ns0:f>
-        <ns0:v>6.87106682290823e+46</ns0:v>
+        <ns0:v>4.94877751358473e+46</ns0:v>
       </ns0:c>
       <ns0:c r="G182" s="1" t="n">
         <ns0:v>36.6000000000001</ns0:v>
@@ -6746,15 +6746,15 @@
       </ns0:c>
       <ns0:c r="D183" s="1">
         <ns0:f>ROUND(D182*20,2-INT(LOG10(ABS(D182*20))))</ns0:f>
-        <ns0:v>1.2300000000000001e+209</ns0:v>
+        <ns0:v>1.5000000000000001e+209</ns0:v>
       </ns0:c>
       <ns0:c r="E183" s="1">
         <ns0:f>D183</ns0:f>
-        <ns0:v>1.2300000000000001e+209</ns0:v>
+        <ns0:v>1.5000000000000001e+209</ns0:v>
       </ns0:c>
       <ns0:c r="F183" s="1">
         <ns0:f>ROUND(F182*1.4,-5)</ns0:f>
-        <ns0:v>9.619493552071522e+46</ns0:v>
+        <ns0:v>6.928288519018622e+46</ns0:v>
       </ns0:c>
       <ns0:c r="G183" s="1" t="n">
         <ns0:v>36.8000000000001</ns0:v>
@@ -6778,15 +6778,15 @@
       </ns0:c>
       <ns0:c r="D184" s="1">
         <ns0:f>ROUND(D183*20,2-INT(LOG10(ABS(D183*20))))</ns0:f>
-        <ns0:v>2.4599999999999997e+210</ns0:v>
+        <ns0:v>2.9999999999999996e+210</ns0:v>
       </ns0:c>
       <ns0:c r="E184" s="1">
         <ns0:f>D184</ns0:f>
-        <ns0:v>2.4599999999999997e+210</ns0:v>
+        <ns0:v>2.9999999999999996e+210</ns0:v>
       </ns0:c>
       <ns0:c r="F184" s="1">
         <ns0:f>ROUND(F183*1.4,-5)</ns0:f>
-        <ns0:v>1.346729097290013e+47</ns0:v>
+        <ns0:v>9.699603926626071e+46</ns0:v>
       </ns0:c>
       <ns0:c r="G184" s="1" t="n">
         <ns0:v>37.0000000000001</ns0:v>
@@ -6810,15 +6810,15 @@
       </ns0:c>
       <ns0:c r="D185" s="1">
         <ns0:f>ROUND(D184*20,2-INT(LOG10(ABS(D184*20))))</ns0:f>
-        <ns0:v>4.92e+211</ns0:v>
+        <ns0:v>5.999999999999999e+211</ns0:v>
       </ns0:c>
       <ns0:c r="E185" s="1">
         <ns0:f>D185</ns0:f>
-        <ns0:v>4.92e+211</ns0:v>
+        <ns0:v>5.999999999999999e+211</ns0:v>
       </ns0:c>
       <ns0:c r="F185" s="1">
         <ns0:f>ROUND(F184*1.4,-5)</ns0:f>
-        <ns0:v>1.885420736206018e+47</ns0:v>
+        <ns0:v>1.3579445497276498e+47</ns0:v>
       </ns0:c>
       <ns0:c r="G185" s="1" t="n">
         <ns0:v>37.2000000000001</ns0:v>
@@ -6842,15 +6842,15 @@
       </ns0:c>
       <ns0:c r="D186" s="1">
         <ns0:f>ROUND(D185*20,2-INT(LOG10(ABS(D185*20))))</ns0:f>
-        <ns0:v>9.84e+212</ns0:v>
+        <ns0:v>1.1999999999999999e+213</ns0:v>
       </ns0:c>
       <ns0:c r="E186" s="1">
         <ns0:f>D186</ns0:f>
-        <ns0:v>9.84e+212</ns0:v>
+        <ns0:v>1.1999999999999999e+213</ns0:v>
       </ns0:c>
       <ns0:c r="F186" s="1">
         <ns0:f>ROUND(F185*1.4,-5)</ns0:f>
-        <ns0:v>2.639589030688425e+47</ns0:v>
+        <ns0:v>1.9011223696187096e+47</ns0:v>
       </ns0:c>
       <ns0:c r="G186" s="1" t="n">
         <ns0:v>37.4000000000001</ns0:v>
@@ -6874,15 +6874,15 @@
       </ns0:c>
       <ns0:c r="D187" s="1">
         <ns0:f>ROUND(D186*20,2-INT(LOG10(ABS(D186*20))))</ns0:f>
-        <ns0:v>1.9700000000000001e+214</ns0:v>
+        <ns0:v>2.4e+214</ns0:v>
       </ns0:c>
       <ns0:c r="E187" s="1">
         <ns0:f>D187</ns0:f>
-        <ns0:v>1.9700000000000001e+214</ns0:v>
+        <ns0:v>2.4e+214</ns0:v>
       </ns0:c>
       <ns0:c r="F187" s="1">
         <ns0:f>ROUND(F186*1.4,-5)</ns0:f>
-        <ns0:v>3.695424642963795e+47</ns0:v>
+        <ns0:v>2.661571317466193e+47</ns0:v>
       </ns0:c>
       <ns0:c r="G187" s="1" t="n">
         <ns0:v>37.6000000000001</ns0:v>
@@ -6906,15 +6906,15 @@
       </ns0:c>
       <ns0:c r="D188" s="1">
         <ns0:f>ROUND(D187*20,2-INT(LOG10(ABS(D187*20))))</ns0:f>
-        <ns0:v>3.94e+215</ns0:v>
+        <ns0:v>4.8e+215</ns0:v>
       </ns0:c>
       <ns0:c r="E188" s="1">
         <ns0:f>D188</ns0:f>
-        <ns0:v>3.94e+215</ns0:v>
+        <ns0:v>4.8e+215</ns0:v>
       </ns0:c>
       <ns0:c r="F188" s="1">
         <ns0:f>ROUND(F187*1.4,-5)</ns0:f>
-        <ns0:v>5.173594500149313e+47</ns0:v>
+        <ns0:v>3.72619984445267e+47</ns0:v>
       </ns0:c>
       <ns0:c r="G188" s="1" t="n">
         <ns0:v>37.8000000000001</ns0:v>
@@ -6938,15 +6938,15 @@
       </ns0:c>
       <ns0:c r="D189" s="1">
         <ns0:f>ROUND(D188*20,2-INT(LOG10(ABS(D188*20))))</ns0:f>
-        <ns0:v>7.880000000000001e+216</ns0:v>
+        <ns0:v>9.600000000000001e+216</ns0:v>
       </ns0:c>
       <ns0:c r="E189" s="1">
         <ns0:f>D189</ns0:f>
-        <ns0:v>7.880000000000001e+216</ns0:v>
+        <ns0:v>9.600000000000001e+216</ns0:v>
       </ns0:c>
       <ns0:c r="F189" s="1">
         <ns0:f>ROUND(F188*1.4,-5)</ns0:f>
-        <ns0:v>7.243032300209037e+47</ns0:v>
+        <ns0:v>5.216679782233738e+47</ns0:v>
       </ns0:c>
       <ns0:c r="G189" s="1" t="n">
         <ns0:v>38.0000000000001</ns0:v>
@@ -6970,15 +6970,15 @@
       </ns0:c>
       <ns0:c r="D190" s="1">
         <ns0:f>ROUND(D189*20,2-INT(LOG10(ABS(D189*20))))</ns0:f>
-        <ns0:v>1.58e+218</ns0:v>
+        <ns0:v>1.92e+218</ns0:v>
       </ns0:c>
       <ns0:c r="E190" s="1">
         <ns0:f>D190</ns0:f>
-        <ns0:v>1.58e+218</ns0:v>
+        <ns0:v>1.92e+218</ns0:v>
       </ns0:c>
       <ns0:c r="F190" s="1">
         <ns0:f>ROUND(F189*1.4,-5)</ns0:f>
-        <ns0:v>1.0140245220292651e+48</ns0:v>
+        <ns0:v>7.3033516951272325e+47</ns0:v>
       </ns0:c>
       <ns0:c r="G190" s="1" t="n">
         <ns0:v>38.2000000000001</ns0:v>
@@ -7002,15 +7002,15 @@
       </ns0:c>
       <ns0:c r="D191" s="1">
         <ns0:f>ROUND(D190*20,2-INT(LOG10(ABS(D190*20))))</ns0:f>
-        <ns0:v>3.16e+219</ns0:v>
+        <ns0:v>3.84e+219</ns0:v>
       </ns0:c>
       <ns0:c r="E191" s="1">
         <ns0:f>D191</ns0:f>
-        <ns0:v>3.16e+219</ns0:v>
+        <ns0:v>3.84e+219</ns0:v>
       </ns0:c>
       <ns0:c r="F191" s="1">
         <ns0:f>ROUND(F190*1.4,-5)</ns0:f>
-        <ns0:v>1.4196343308409709e+48</ns0:v>
+        <ns0:v>1.0224692373178125e+48</ns0:v>
       </ns0:c>
       <ns0:c r="G191" s="1" t="n">
         <ns0:v>38.4000000000001</ns0:v>
@@ -7034,15 +7034,15 @@
       </ns0:c>
       <ns0:c r="D192" s="1">
         <ns0:f>ROUND(D191*20,2-INT(LOG10(ABS(D191*20))))</ns0:f>
-        <ns0:v>6.319999999999999e+220</ns0:v>
+        <ns0:v>7.68e+220</ns0:v>
       </ns0:c>
       <ns0:c r="E192" s="1">
         <ns0:f>D192</ns0:f>
-        <ns0:v>6.319999999999999e+220</ns0:v>
+        <ns0:v>7.68e+220</ns0:v>
       </ns0:c>
       <ns0:c r="F192" s="1">
         <ns0:f>ROUND(F191*1.4,-5)</ns0:f>
-        <ns0:v>1.987488063177359e+48</ns0:v>
+        <ns0:v>1.4314569322449375e+48</ns0:v>
       </ns0:c>
       <ns0:c r="G192" s="1" t="n">
         <ns0:v>38.6000000000001</ns0:v>
@@ -7066,15 +7066,15 @@
       </ns0:c>
       <ns0:c r="D193" s="1">
         <ns0:f>ROUND(D192*20,2-INT(LOG10(ABS(D192*20))))</ns0:f>
-        <ns0:v>1.26e+222</ns0:v>
+        <ns0:v>1.54e+222</ns0:v>
       </ns0:c>
       <ns0:c r="E193" s="1">
         <ns0:f>D193</ns0:f>
-        <ns0:v>1.26e+222</ns0:v>
+        <ns0:v>1.54e+222</ns0:v>
       </ns0:c>
       <ns0:c r="F193" s="1">
         <ns0:f>ROUND(F192*1.4,-5)</ns0:f>
-        <ns0:v>2.782483288448303e+48</ns0:v>
+        <ns0:v>2.0040397051429124e+48</ns0:v>
       </ns0:c>
       <ns0:c r="G193" s="1" t="n">
         <ns0:v>38.8000000000001</ns0:v>
@@ -7098,15 +7098,15 @@
       </ns0:c>
       <ns0:c r="D194" s="1">
         <ns0:f>ROUND(D193*20,2-INT(LOG10(ABS(D193*20))))</ns0:f>
-        <ns0:v>2.52e+223</ns0:v>
+        <ns0:v>3.08e+223</ns0:v>
       </ns0:c>
       <ns0:c r="E194" s="1">
         <ns0:f>D194</ns0:f>
-        <ns0:v>2.52e+223</ns0:v>
+        <ns0:v>3.08e+223</ns0:v>
       </ns0:c>
       <ns0:c r="F194" s="1">
         <ns0:f>ROUND(F193*1.4,-5)</ns0:f>
-        <ns0:v>3.895476603827624e+48</ns0:v>
+        <ns0:v>2.8056555872000773e+48</ns0:v>
       </ns0:c>
       <ns0:c r="G194" s="1" t="n">
         <ns0:v>39.0000000000001</ns0:v>
@@ -7130,15 +7130,15 @@
       </ns0:c>
       <ns0:c r="D195" s="1">
         <ns0:f>ROUND(D194*20,2-INT(LOG10(ABS(D194*20))))</ns0:f>
-        <ns0:v>5.0399999999999996e+224</ns0:v>
+        <ns0:v>6.16e+224</ns0:v>
       </ns0:c>
       <ns0:c r="E195" s="1">
         <ns0:f>D195</ns0:f>
-        <ns0:v>5.0399999999999996e+224</ns0:v>
+        <ns0:v>6.16e+224</ns0:v>
       </ns0:c>
       <ns0:c r="F195" s="1">
         <ns0:f>ROUND(F194*1.4,-5)</ns0:f>
-        <ns0:v>5.453667245358673e+48</ns0:v>
+        <ns0:v>3.927917822080108e+48</ns0:v>
       </ns0:c>
       <ns0:c r="G195" s="1" t="n">
         <ns0:v>39.2000000000001</ns0:v>
@@ -7162,15 +7162,15 @@
       </ns0:c>
       <ns0:c r="D196" s="1">
         <ns0:f>ROUND(D195*20,2-INT(LOG10(ABS(D195*20))))</ns0:f>
-        <ns0:v>1.01e+226</ns0:v>
+        <ns0:v>1.23e+226</ns0:v>
       </ns0:c>
       <ns0:c r="E196" s="1">
         <ns0:f>D196</ns0:f>
-        <ns0:v>1.01e+226</ns0:v>
+        <ns0:v>1.23e+226</ns0:v>
       </ns0:c>
       <ns0:c r="F196" s="1">
         <ns0:f>ROUND(F195*1.4,-5)</ns0:f>
-        <ns0:v>7.635134143502141e+48</ns0:v>
+        <ns0:v>5.49908495091215e+48</ns0:v>
       </ns0:c>
       <ns0:c r="G196" s="1" t="n">
         <ns0:v>39.4000000000001</ns0:v>
@@ -7194,15 +7194,15 @@
       </ns0:c>
       <ns0:c r="D197" s="1">
         <ns0:f>ROUND(D196*20,2-INT(LOG10(ABS(D196*20))))</ns0:f>
-        <ns0:v>2.02e+227</ns0:v>
+        <ns0:v>2.4600000000000002e+227</ns0:v>
       </ns0:c>
       <ns0:c r="E197" s="1">
         <ns0:f>D197</ns0:f>
-        <ns0:v>2.02e+227</ns0:v>
+        <ns0:v>2.4600000000000002e+227</ns0:v>
       </ns0:c>
       <ns0:c r="F197" s="1">
         <ns0:f>ROUND(F196*1.4,-5)</ns0:f>
-        <ns0:v>1.0689187800902998e+49</ns0:v>
+        <ns0:v>7.698718931277009e+48</ns0:v>
       </ns0:c>
       <ns0:c r="G197" s="1" t="n">
         <ns0:v>39.6000000000001</ns0:v>
@@ -7226,15 +7226,15 @@
       </ns0:c>
       <ns0:c r="D198" s="1">
         <ns0:f>ROUND(D197*20,2-INT(LOG10(ABS(D197*20))))</ns0:f>
-        <ns0:v>4.0400000000000005e+228</ns0:v>
+        <ns0:v>4.92e+228</ns0:v>
       </ns0:c>
       <ns0:c r="E198" s="1">
         <ns0:f>D198</ns0:f>
-        <ns0:v>4.0400000000000005e+228</ns0:v>
+        <ns0:v>4.92e+228</ns0:v>
       </ns0:c>
       <ns0:c r="F198" s="1">
         <ns0:f>ROUND(F197*1.4,-5)</ns0:f>
-        <ns0:v>1.4964862921264196e+49</ns0:v>
+        <ns0:v>1.0778206503787812e+49</ns0:v>
       </ns0:c>
       <ns0:c r="G198" s="1" t="n">
         <ns0:v>39.8000000000001</ns0:v>
@@ -7258,15 +7258,15 @@
       </ns0:c>
       <ns0:c r="D199" s="1">
         <ns0:f>ROUND(D198*20,2-INT(LOG10(ABS(D198*20))))</ns0:f>
-        <ns0:v>8.08e+229</ns0:v>
+        <ns0:v>9.84e+229</ns0:v>
       </ns0:c>
       <ns0:c r="E199" s="1">
         <ns0:f>D199</ns0:f>
-        <ns0:v>8.08e+229</ns0:v>
+        <ns0:v>9.84e+229</ns0:v>
       </ns0:c>
       <ns0:c r="F199" s="1">
         <ns0:f>ROUND(F198*1.4,-5)</ns0:f>
-        <ns0:v>2.0950808089769872e+49</ns0:v>
+        <ns0:v>1.5089489105302936e+49</ns0:v>
       </ns0:c>
       <ns0:c r="G199" s="1" t="n">
         <ns0:v>40.0000000000001</ns0:v>
@@ -7290,15 +7290,15 @@
       </ns0:c>
       <ns0:c r="D200" s="1">
         <ns0:f>ROUND(D199*20,2-INT(LOG10(ABS(D199*20))))</ns0:f>
-        <ns0:v>1.6199999999999998e+231</ns0:v>
+        <ns0:v>1.97e+231</ns0:v>
       </ns0:c>
       <ns0:c r="E200" s="1">
         <ns0:f>D200</ns0:f>
-        <ns0:v>1.6199999999999998e+231</ns0:v>
+        <ns0:v>1.97e+231</ns0:v>
       </ns0:c>
       <ns0:c r="F200" s="1">
         <ns0:f>ROUND(F199*1.4,-5)</ns0:f>
-        <ns0:v>2.9331131325677817e+49</ns0:v>
+        <ns0:v>2.112528474742411e+49</ns0:v>
       </ns0:c>
       <ns0:c r="G200" s="1" t="n">
         <ns0:v>40.2000000000001</ns0:v>
@@ -7322,15 +7322,15 @@
       </ns0:c>
       <ns0:c r="D201" s="1">
         <ns0:f>ROUND(D200*20,2-INT(LOG10(ABS(D200*20))))</ns0:f>
-        <ns0:v>3.2399999999999997e+232</ns0:v>
+        <ns0:v>3.94e+232</ns0:v>
       </ns0:c>
       <ns0:c r="E201" s="1">
         <ns0:f>D201</ns0:f>
-        <ns0:v>3.2399999999999997e+232</ns0:v>
+        <ns0:v>3.94e+232</ns0:v>
       </ns0:c>
       <ns0:c r="F201" s="1">
         <ns0:f>ROUND(F200*1.4,-5)</ns0:f>
-        <ns0:v>4.106358385594894e+49</ns0:v>
+        <ns0:v>2.957539864639375e+49</ns0:v>
       </ns0:c>
       <ns0:c r="G201" s="1" t="n">
         <ns0:v>40.4000000000001</ns0:v>
@@ -7354,15 +7354,15 @@
       </ns0:c>
       <ns0:c r="D202" s="1">
         <ns0:f>ROUND(D201*20,2-INT(LOG10(ABS(D201*20))))</ns0:f>
-        <ns0:v>6.48e+233</ns0:v>
+        <ns0:v>7.8800000000000005e+233</ns0:v>
       </ns0:c>
       <ns0:c r="E202" s="1">
         <ns0:f>D202</ns0:f>
-        <ns0:v>6.48e+233</ns0:v>
+        <ns0:v>7.8800000000000005e+233</ns0:v>
       </ns0:c>
       <ns0:c r="F202" s="1">
         <ns0:f>ROUND(F201*1.4,-5)</ns0:f>
-        <ns0:v>5.748901739832851e+49</ns0:v>
+        <ns0:v>4.1405558104951243e+49</ns0:v>
       </ns0:c>
       <ns0:c r="G202" s="1" t="n">
         <ns0:v>40.6000000000001</ns0:v>
@@ -7386,15 +7386,15 @@
       </ns0:c>
       <ns0:c r="D203" s="1">
         <ns0:f>ROUND(D202*20,2-INT(LOG10(ABS(D202*20))))</ns0:f>
-        <ns0:v>1.3000000000000002e+235</ns0:v>
+        <ns0:v>1.58e+235</ns0:v>
       </ns0:c>
       <ns0:c r="E203" s="1">
         <ns0:f>D203</ns0:f>
-        <ns0:v>1.3000000000000002e+235</ns0:v>
+        <ns0:v>1.58e+235</ns0:v>
       </ns0:c>
       <ns0:c r="F203" s="1">
         <ns0:f>ROUND(F202*1.4,-5)</ns0:f>
-        <ns0:v>8.048462435765991e+49</ns0:v>
+        <ns0:v>5.796778134693173e+49</ns0:v>
       </ns0:c>
       <ns0:c r="G203" s="1" t="n">
         <ns0:v>40.8000000000001</ns0:v>
@@ -7418,15 +7418,15 @@
       </ns0:c>
       <ns0:c r="D204" s="1">
         <ns0:f>ROUND(D203*20,2-INT(LOG10(ABS(D203*20))))</ns0:f>
-        <ns0:v>2.6e+236</ns0:v>
+        <ns0:v>3.16e+236</ns0:v>
       </ns0:c>
       <ns0:c r="E204" s="1">
         <ns0:f>D204</ns0:f>
-        <ns0:v>2.6e+236</ns0:v>
+        <ns0:v>3.16e+236</ns0:v>
       </ns0:c>
       <ns0:c r="F204" s="1">
         <ns0:f>ROUND(F203*1.4,-5)</ns0:f>
-        <ns0:v>1.1267847410072387e+50</ns0:v>
+        <ns0:v>8.115489388570442e+49</ns0:v>
       </ns0:c>
       <ns0:c r="G204" s="1" t="n">
         <ns0:v>41.0000000000001</ns0:v>
@@ -7450,15 +7450,15 @@
       </ns0:c>
       <ns0:c r="D205" s="1">
         <ns0:f>ROUND(D204*20,2-INT(LOG10(ABS(D204*20))))</ns0:f>
-        <ns0:v>5.2e+237</ns0:v>
+        <ns0:v>6.3200000000000006e+237</ns0:v>
       </ns0:c>
       <ns0:c r="E205" s="1">
         <ns0:f>D205</ns0:f>
-        <ns0:v>5.2e+237</ns0:v>
+        <ns0:v>6.3200000000000006e+237</ns0:v>
       </ns0:c>
       <ns0:c r="F205" s="1">
         <ns0:f>ROUND(F204*1.4,-5)</ns0:f>
-        <ns0:v>1.5774986374101342e+50</ns0:v>
+        <ns0:v>1.136168514399862e+50</ns0:v>
       </ns0:c>
       <ns0:c r="G205" s="1" t="n">
         <ns0:v>41.2000000000001</ns0:v>
@@ -7482,15 +7482,15 @@
       </ns0:c>
       <ns0:c r="D206" s="1">
         <ns0:f>ROUND(D205*20,2-INT(LOG10(ABS(D205*20))))</ns0:f>
-        <ns0:v>1.04e+239</ns0:v>
+        <ns0:v>1.26e+239</ns0:v>
       </ns0:c>
       <ns0:c r="E206" s="1">
         <ns0:f>D206</ns0:f>
-        <ns0:v>1.04e+239</ns0:v>
+        <ns0:v>1.26e+239</ns0:v>
       </ns0:c>
       <ns0:c r="F206" s="1">
         <ns0:f>ROUND(F205*1.4,-5)</ns0:f>
-        <ns0:v>2.208498092374188e+50</ns0:v>
+        <ns0:v>1.5906359201598066e+50</ns0:v>
       </ns0:c>
       <ns0:c r="G206" s="1" t="n">
         <ns0:v>41.4000000000001</ns0:v>
@@ -7514,15 +7514,15 @@
       </ns0:c>
       <ns0:c r="D207" s="1">
         <ns0:f>ROUND(D206*20,2-INT(LOG10(ABS(D206*20))))</ns0:f>
-        <ns0:v>2.08e+240</ns0:v>
+        <ns0:v>2.52e+240</ns0:v>
       </ns0:c>
       <ns0:c r="E207" s="1">
         <ns0:f>D207</ns0:f>
-        <ns0:v>2.08e+240</ns0:v>
+        <ns0:v>2.52e+240</ns0:v>
       </ns0:c>
       <ns0:c r="F207" s="1">
         <ns0:f>ROUND(F206*1.4,-5)</ns0:f>
-        <ns0:v>3.091897329323863e+50</ns0:v>
+        <ns0:v>2.226890288223729e+50</ns0:v>
       </ns0:c>
       <ns0:c r="G207" s="1" t="n">
         <ns0:v>41.6000000000001</ns0:v>
@@ -7546,15 +7546,15 @@
       </ns0:c>
       <ns0:c r="D208" s="1">
         <ns0:f>ROUND(D207*20,2-INT(LOG10(ABS(D207*20))))</ns0:f>
-        <ns0:v>4.1599999999999994e+241</ns0:v>
+        <ns0:v>5.04e+241</ns0:v>
       </ns0:c>
       <ns0:c r="E208" s="1">
         <ns0:f>D208</ns0:f>
-        <ns0:v>4.1599999999999994e+241</ns0:v>
+        <ns0:v>5.04e+241</ns0:v>
       </ns0:c>
       <ns0:c r="F208" s="1">
         <ns0:f>ROUND(F207*1.4,-5)</ns0:f>
-        <ns0:v>4.328656261053408e+50</ns0:v>
+        <ns0:v>3.117646403513221e+50</ns0:v>
       </ns0:c>
       <ns0:c r="G208" s="1" t="n">
         <ns0:v>41.8000000000001</ns0:v>
@@ -7578,15 +7578,15 @@
       </ns0:c>
       <ns0:c r="D209" s="1">
         <ns0:f>ROUND(D208*20,2-INT(LOG10(ABS(D208*20))))</ns0:f>
-        <ns0:v>8.32e+242</ns0:v>
+        <ns0:v>1.01e+243</ns0:v>
       </ns0:c>
       <ns0:c r="E209" s="1">
         <ns0:f>D209</ns0:f>
-        <ns0:v>8.32e+242</ns0:v>
+        <ns0:v>1.01e+243</ns0:v>
       </ns0:c>
       <ns0:c r="F209" s="1">
         <ns0:f>ROUND(F208*1.4,-5)</ns0:f>
-        <ns0:v>6.06011876547477e+50</ns0:v>
+        <ns0:v>4.3647049649185085e+50</ns0:v>
       </ns0:c>
       <ns0:c r="G209" s="1" t="n">
         <ns0:v>42.0000000000001</ns0:v>
@@ -7610,15 +7610,15 @@
       </ns0:c>
       <ns0:c r="D210" s="1">
         <ns0:f>ROUND(D209*20,2-INT(LOG10(ABS(D209*20))))</ns0:f>
-        <ns0:v>1.66e+244</ns0:v>
+        <ns0:v>2.02e+244</ns0:v>
       </ns0:c>
       <ns0:c r="E210" s="1">
         <ns0:f>D210</ns0:f>
-        <ns0:v>1.66e+244</ns0:v>
+        <ns0:v>2.02e+244</ns0:v>
       </ns0:c>
       <ns0:c r="F210" s="1">
         <ns0:f>ROUND(F209*1.4,-5)</ns0:f>
-        <ns0:v>8.484166271664678e+50</ns0:v>
+        <ns0:v>6.110586950885911e+50</ns0:v>
       </ns0:c>
       <ns0:c r="G210" s="1" t="n">
         <ns0:v>42.2000000000001</ns0:v>
@@ -7642,15 +7642,15 @@
       </ns0:c>
       <ns0:c r="D211" s="1">
         <ns0:f>ROUND(D210*20,2-INT(LOG10(ABS(D210*20))))</ns0:f>
-        <ns0:v>3.32e+245</ns0:v>
+        <ns0:v>4.04e+245</ns0:v>
       </ns0:c>
       <ns0:c r="E211" s="1">
         <ns0:f>D211</ns0:f>
-        <ns0:v>3.32e+245</ns0:v>
+        <ns0:v>4.04e+245</ns0:v>
       </ns0:c>
       <ns0:c r="F211" s="1">
         <ns0:f>ROUND(F210*1.4,-5)</ns0:f>
-        <ns0:v>1.187783278033055e+51</ns0:v>
+        <ns0:v>8.554821731240276e+50</ns0:v>
       </ns0:c>
       <ns0:c r="G211" s="1" t="n">
         <ns0:v>42.4000000000001</ns0:v>
@@ -7674,15 +7674,15 @@
       </ns0:c>
       <ns0:c r="D212" s="1">
         <ns0:f>ROUND(D211*20,2-INT(LOG10(ABS(D211*20))))</ns0:f>
-        <ns0:v>6.640000000000001e+246</ns0:v>
+        <ns0:v>8.08e+246</ns0:v>
       </ns0:c>
       <ns0:c r="E212" s="1">
         <ns0:f>D212</ns0:f>
-        <ns0:v>6.640000000000001e+246</ns0:v>
+        <ns0:v>8.08e+246</ns0:v>
       </ns0:c>
       <ns0:c r="F212" s="1">
         <ns0:f>ROUND(F211*1.4,-5)</ns0:f>
-        <ns0:v>1.662896589246277e+51</ns0:v>
+        <ns0:v>1.1976750423736385e+51</ns0:v>
       </ns0:c>
       <ns0:c r="G212" s="1" t="n">
         <ns0:v>42.6000000000002</ns0:v>
@@ -7706,15 +7706,15 @@
       </ns0:c>
       <ns0:c r="D213" s="1">
         <ns0:f>ROUND(D212*20,2-INT(LOG10(ABS(D212*20))))</ns0:f>
-        <ns0:v>1.33e+248</ns0:v>
+        <ns0:v>1.6200000000000001e+248</ns0:v>
       </ns0:c>
       <ns0:c r="E213" s="1">
         <ns0:f>D213</ns0:f>
-        <ns0:v>1.33e+248</ns0:v>
+        <ns0:v>1.6200000000000001e+248</ns0:v>
       </ns0:c>
       <ns0:c r="F213" s="1">
         <ns0:f>ROUND(F212*1.4,-5)</ns0:f>
-        <ns0:v>2.3280552249447878e+51</ns0:v>
+        <ns0:v>1.6767450593230938e+51</ns0:v>
       </ns0:c>
       <ns0:c r="G213" s="1" t="n">
         <ns0:v>42.8000000000002</ns0:v>
@@ -7738,15 +7738,15 @@
       </ns0:c>
       <ns0:c r="D214" s="1">
         <ns0:f>ROUND(D213*20,2-INT(LOG10(ABS(D213*20))))</ns0:f>
-        <ns0:v>2.66e+249</ns0:v>
+        <ns0:v>3.24e+249</ns0:v>
       </ns0:c>
       <ns0:c r="E214" s="1">
         <ns0:f>D214</ns0:f>
-        <ns0:v>2.66e+249</ns0:v>
+        <ns0:v>3.24e+249</ns0:v>
       </ns0:c>
       <ns0:c r="F214" s="1">
         <ns0:f>ROUND(F213*1.4,-5)</ns0:f>
-        <ns0:v>3.2592773149227023e+51</ns0:v>
+        <ns0:v>2.347443083052331e+51</ns0:v>
       </ns0:c>
       <ns0:c r="G214" s="1" t="n">
         <ns0:v>43.0000000000001</ns0:v>
@@ -7770,15 +7770,15 @@
       </ns0:c>
       <ns0:c r="D215" s="1">
         <ns0:f>ROUND(D214*20,2-INT(LOG10(ABS(D214*20))))</ns0:f>
-        <ns0:v>5.32e+250</ns0:v>
+        <ns0:v>6.480000000000001e+250</ns0:v>
       </ns0:c>
       <ns0:c r="E215" s="1">
         <ns0:f>D215</ns0:f>
-        <ns0:v>5.32e+250</ns0:v>
+        <ns0:v>6.480000000000001e+250</ns0:v>
       </ns0:c>
       <ns0:c r="F215" s="1">
         <ns0:f>ROUND(F214*1.4,-5)</ns0:f>
-        <ns0:v>4.562988240891783e+51</ns0:v>
+        <ns0:v>3.286420316273263e+51</ns0:v>
       </ns0:c>
       <ns0:c r="G215" s="1" t="n">
         <ns0:v>43.2000000000002</ns0:v>
@@ -7802,15 +7802,15 @@
       </ns0:c>
       <ns0:c r="D216" s="1">
         <ns0:f>ROUND(D215*20,2-INT(LOG10(ABS(D215*20))))</ns0:f>
-        <ns0:v>1.0599999999999999e+252</ns0:v>
+        <ns0:v>1.2999999999999999e+252</ns0:v>
       </ns0:c>
       <ns0:c r="E216" s="1">
         <ns0:f>D216</ns0:f>
-        <ns0:v>1.0599999999999999e+252</ns0:v>
+        <ns0:v>1.2999999999999999e+252</ns0:v>
       </ns0:c>
       <ns0:c r="F216" s="1">
         <ns0:f>ROUND(F215*1.4,-5)</ns0:f>
-        <ns0:v>6.388183537248496e+51</ns0:v>
+        <ns0:v>4.600988442782569e+51</ns0:v>
       </ns0:c>
       <ns0:c r="G216" s="1" t="n">
         <ns0:v>43.4000000000002</ns0:v>
@@ -7834,15 +7834,15 @@
       </ns0:c>
       <ns0:c r="D217" s="1">
         <ns0:f>ROUND(D216*20,2-INT(LOG10(ABS(D216*20))))</ns0:f>
-        <ns0:v>2.12e+253</ns0:v>
+        <ns0:v>2.6e+253</ns0:v>
       </ns0:c>
       <ns0:c r="E217" s="1">
         <ns0:f>D217</ns0:f>
-        <ns0:v>2.12e+253</ns0:v>
+        <ns0:v>2.6e+253</ns0:v>
       </ns0:c>
       <ns0:c r="F217" s="1">
         <ns0:f>ROUND(F216*1.4,-5)</ns0:f>
-        <ns0:v>8.943456952147894e+51</ns0:v>
+        <ns0:v>6.441383819895597e+51</ns0:v>
       </ns0:c>
       <ns0:c r="G217" s="1" t="n">
         <ns0:v>43.6000000000002</ns0:v>
@@ -7866,15 +7866,15 @@
       </ns0:c>
       <ns0:c r="D218" s="1">
         <ns0:f>ROUND(D217*20,2-INT(LOG10(ABS(D217*20))))</ns0:f>
-        <ns0:v>4.2400000000000004e+254</ns0:v>
+        <ns0:v>5.2e+254</ns0:v>
       </ns0:c>
       <ns0:c r="E218" s="1">
         <ns0:f>D218</ns0:f>
-        <ns0:v>4.2400000000000004e+254</ns0:v>
+        <ns0:v>5.2e+254</ns0:v>
       </ns0:c>
       <ns0:c r="F218" s="1">
         <ns0:f>ROUND(F217*1.4,-5)</ns0:f>
-        <ns0:v>1.2520839733007052e+52</ns0:v>
+        <ns0:v>9.017937347853835e+51</ns0:v>
       </ns0:c>
       <ns0:c r="G218" s="1" t="n">
         <ns0:v>43.8000000000002</ns0:v>
@@ -7898,15 +7898,15 @@
       </ns0:c>
       <ns0:c r="D219" s="1">
         <ns0:f>ROUND(D218*20,2-INT(LOG10(ABS(D218*20))))</ns0:f>
-        <ns0:v>8.48e+255</ns0:v>
+        <ns0:v>1.04e+256</ns0:v>
       </ns0:c>
       <ns0:c r="E219" s="1">
         <ns0:f>D219</ns0:f>
-        <ns0:v>8.48e+255</ns0:v>
+        <ns0:v>1.04e+256</ns0:v>
       </ns0:c>
       <ns0:c r="F219" s="1">
         <ns0:f>ROUND(F218*1.4,-5)</ns0:f>
-        <ns0:v>1.752917562620987e+52</ns0:v>
+        <ns0:v>1.2625112286995368e+52</ns0:v>
       </ns0:c>
       <ns0:c r="G219" s="1" t="n">
         <ns0:v>44.0000000000002</ns0:v>
@@ -7930,15 +7930,15 @@
       </ns0:c>
       <ns0:c r="D220" s="1">
         <ns0:f>ROUND(D219*20,2-INT(LOG10(ABS(D219*20))))</ns0:f>
-        <ns0:v>1.7e+257</ns0:v>
+        <ns0:v>2.08e+257</ns0:v>
       </ns0:c>
       <ns0:c r="E220" s="1">
         <ns0:f>D220</ns0:f>
-        <ns0:v>1.7e+257</ns0:v>
+        <ns0:v>2.08e+257</ns0:v>
       </ns0:c>
       <ns0:c r="F220" s="1">
         <ns0:f>ROUND(F219*1.4,-5)</ns0:f>
-        <ns0:v>2.454084587669382e+52</ns0:v>
+        <ns0:v>1.7675157201793514e+52</ns0:v>
       </ns0:c>
       <ns0:c r="G220" s="1" t="n">
         <ns0:v>44.2000000000002</ns0:v>
@@ -7962,15 +7962,15 @@
       </ns0:c>
       <ns0:c r="D221" s="1">
         <ns0:f>ROUND(D220*20,2-INT(LOG10(ABS(D220*20))))</ns0:f>
-        <ns0:v>3.4000000000000002e+258</ns0:v>
+        <ns0:v>4.16e+258</ns0:v>
       </ns0:c>
       <ns0:c r="E221" s="1">
         <ns0:f>D221</ns0:f>
-        <ns0:v>3.4000000000000002e+258</ns0:v>
+        <ns0:v>4.16e+258</ns0:v>
       </ns0:c>
       <ns0:c r="F221" s="1">
         <ns0:f>ROUND(F220*1.4,-5)</ns0:f>
-        <ns0:v>3.4357184227371343e+52</ns0:v>
+        <ns0:v>2.474522008251092e+52</ns0:v>
       </ns0:c>
       <ns0:c r="G221" s="1" t="n">
         <ns0:v>44.4000000000002</ns0:v>
@@ -7994,15 +7994,15 @@
       </ns0:c>
       <ns0:c r="D222" s="1">
         <ns0:f>ROUND(D221*20,2-INT(LOG10(ABS(D221*20))))</ns0:f>
-        <ns0:v>6.8e+259</ns0:v>
+        <ns0:v>8.32e+259</ns0:v>
       </ns0:c>
       <ns0:c r="E222" s="1">
         <ns0:f>D222</ns0:f>
-        <ns0:v>6.8e+259</ns0:v>
+        <ns0:v>8.32e+259</ns0:v>
       </ns0:c>
       <ns0:c r="F222" s="1">
         <ns0:f>ROUND(F221*1.4,-5)</ns0:f>
-        <ns0:v>4.810005791831987e+52</ns0:v>
+        <ns0:v>3.4643308115515286e+52</ns0:v>
       </ns0:c>
       <ns0:c r="G222" s="1" t="n">
         <ns0:v>44.6000000000002</ns0:v>
@@ -8026,15 +8026,15 @@
       </ns0:c>
       <ns0:c r="D223" s="1">
         <ns0:f>ROUND(D222*20,2-INT(LOG10(ABS(D222*20))))</ns0:f>
-        <ns0:v>1.36e+261</ns0:v>
+        <ns0:v>1.6599999999999999e+261</ns0:v>
       </ns0:c>
       <ns0:c r="E223" s="1">
         <ns0:f>D223</ns0:f>
-        <ns0:v>1.36e+261</ns0:v>
+        <ns0:v>1.6599999999999999e+261</ns0:v>
       </ns0:c>
       <ns0:c r="F223" s="1">
         <ns0:f>ROUND(F222*1.4,-5)</ns0:f>
-        <ns0:v>6.734008108564782e+52</ns0:v>
+        <ns0:v>4.85006313617214e+52</ns0:v>
       </ns0:c>
       <ns0:c r="G223" s="1" t="n">
         <ns0:v>44.8000000000002</ns0:v>

</xml_diff>

<commit_message>
balance: v22 source-only preparation candidate and explicit scoped verification
</commit_message>
<xml_diff>
--- a/space-battleship/config_excel/level.xlsx
+++ b/space-battleship/config_excel/level.xlsx
@@ -2247,10 +2247,10 @@
         </ns0:is>
       </ns0:c>
       <ns0:c r="D39" s="1" t="n">
-        <ns0:v>9.754913062531577e+31</ns0:v>
+        <ns0:v>4.70433693216222e+31</ns0:v>
       </ns0:c>
       <ns0:c r="E39" s="1" t="n">
-        <ns0:v>9.754913062531577e+31</ns0:v>
+        <ns0:v>4.70433693216222e+31</ns0:v>
       </ns0:c>
       <ns0:c r="F39" s="1" t="n">
         <ns0:v>8.974025518619266e+16</ns0:v>
@@ -2275,10 +2275,10 @@
         </ns0:is>
       </ns0:c>
       <ns0:c r="D40" s="1" t="n">
-        <ns0:v>4.19443406295988e+32</ns0:v>
+        <ns0:v>9.754913062531577e+31</ns0:v>
       </ns0:c>
       <ns0:c r="E40" s="1" t="n">
-        <ns0:v>4.19443406295988e+32</ns0:v>
+        <ns0:v>9.754913062531577e+31</ns0:v>
       </ns0:c>
       <ns0:c r="F40" s="1" t="n">
         <ns0:v>1.86085393154089e+17</ns0:v>
@@ -2303,10 +2303,10 @@
         </ns0:is>
       </ns0:c>
       <ns0:c r="D41" s="1" t="n">
-        <ns0:v>1.80352987215166e+33</ns0:v>
+        <ns0:v>2.022778772646547e+32</ns0:v>
       </ns0:c>
       <ns0:c r="E41" s="1" t="n">
-        <ns0:v>1.80352987215166e+33</ns0:v>
+        <ns0:v>2.022778772646547e+32</ns0:v>
       </ns0:c>
       <ns0:c r="F41" s="1" t="n">
         <ns0:v>3.85866671244319e+17</ns0:v>
@@ -2387,10 +2387,10 @@
         </ns0:is>
       </ns0:c>
       <ns0:c r="D44" s="1" t="n">
-        <ns0:v>3.403381443351019e+37</ns0:v>
+        <ns0:v>1.641291205319743e+37</ns0:v>
       </ns0:c>
       <ns0:c r="E44" s="1" t="n">
-        <ns0:v>3.403381443351019e+37</ns0:v>
+        <ns0:v>1.641291205319743e+37</ns0:v>
       </ns0:c>
       <ns0:c r="F44" s="1" t="n">
         <ns0:v>3.067518380479065e+19</ns0:v>
@@ -2415,10 +2415,10 @@
         </ns0:is>
       </ns0:c>
       <ns0:c r="D45" s="1" t="n">
-        <ns0:v>1.463391725146999e+38</ns0:v>
+        <ns0:v>3.403381443351019e+37</ns0:v>
       </ns0:c>
       <ns0:c r="E45" s="1" t="n">
-        <ns0:v>1.463391725146999e+38</ns0:v>
+        <ns0:v>3.403381443351019e+37</ns0:v>
       </ns0:c>
       <ns0:c r="F45" s="1" t="n">
         <ns0:v>6.360806113761387e+19</ns0:v>
@@ -2443,10 +2443,10 @@
         </ns0:is>
       </ns0:c>
       <ns0:c r="D46" s="1" t="n">
-        <ns0:v>6.292316558910722e+38</ns0:v>
+        <ns0:v>7.057251760932672e+37</ns0:v>
       </ns0:c>
       <ns0:c r="E46" s="1" t="n">
-        <ns0:v>6.292316558910722e+38</ns0:v>
+        <ns0:v>7.057251760932672e+37</ns0:v>
       </ns0:c>
       <ns0:c r="F46" s="1" t="n">
         <ns0:v>1.318976755749561e+20</ns0:v>
@@ -2527,10 +2527,10 @@
         </ns0:is>
       </ns0:c>
       <ns0:c r="D49" s="1" t="n">
-        <ns0:v>1.187402201813172e+43</ns0:v>
+        <ns0:v>5.726283766460129e+42</ns0:v>
       </ns0:c>
       <ns0:c r="E49" s="1" t="n">
-        <ns0:v>1.187402201813172e+43</ns0:v>
+        <ns0:v>5.726283766460129e+42</ns0:v>
       </ns0:c>
       <ns0:c r="F49" s="1" t="n">
         <ns0:v>1.048544936166469e+22</ns0:v>
@@ -2555,10 +2555,10 @@
         </ns0:is>
       </ns0:c>
       <ns0:c r="D50" s="1" t="n">
-        <ns0:v>5.105612125697618e+43</ns0:v>
+        <ns0:v>1.187402201813172e+43</ns0:v>
       </ns0:c>
       <ns0:c r="E50" s="1" t="n">
-        <ns0:v>5.105612125697618e+43</ns0:v>
+        <ns0:v>1.187402201813172e+43</ns0:v>
       </ns0:c>
       <ns0:c r="F50" s="1" t="n">
         <ns0:v>2.17426277963479e+22</ns0:v>
@@ -2583,10 +2583,10 @@
         </ns0:is>
       </ns0:c>
       <ns0:c r="D51" s="1" t="n">
-        <ns0:v>2.195319760925626e+44</ns0:v>
+        <ns0:v>2.462197205679793e+43</ns0:v>
       </ns0:c>
       <ns0:c r="E51" s="1" t="n">
-        <ns0:v>2.195319760925626e+44</ns0:v>
+        <ns0:v>2.462197205679793e+43</ns0:v>
       </ns0:c>
       <ns0:c r="F51" s="1" t="n">
         <ns0:v>4.508551299850701e+22</ns0:v>
@@ -2667,10 +2667,10 @@
         </ns0:is>
       </ns0:c>
       <ns0:c r="D54" s="1" t="n">
-        <ns0:v>4.142715156496054e+48</ns0:v>
+        <ns0:v>1.997837170378113e+48</ns0:v>
       </ns0:c>
       <ns0:c r="E54" s="1" t="n">
-        <ns0:v>4.142715156496054e+48</ns0:v>
+        <ns0:v>1.997837170378113e+48</ns0:v>
       </ns0:c>
       <ns0:c r="F54" s="1" t="n">
         <ns0:v>3.584156137928801e+24</ns0:v>
@@ -2695,10 +2695,10 @@
         </ns0:is>
       </ns0:c>
       <ns0:c r="D55" s="1" t="n">
-        <ns0:v>1.781291689035079e+49</ns0:v>
+        <ns0:v>4.142715156496054e+48</ns0:v>
       </ns0:c>
       <ns0:c r="E55" s="1" t="n">
-        <ns0:v>1.781291689035079e+49</ns0:v>
+        <ns0:v>4.142715156496054e+48</ns0:v>
       </ns0:c>
       <ns0:c r="F55" s="1" t="n">
         <ns0:v>7.43210616760916e+24</ns0:v>
@@ -2723,10 +2723,10 @@
         </ns0:is>
       </ns0:c>
       <ns0:c r="D56" s="1" t="n">
-        <ns0:v>7.659228215220075e+49</ns0:v>
+        <ns0:v>8.590334148510218e+48</ns0:v>
       </ns0:c>
       <ns0:c r="E56" s="1" t="n">
-        <ns0:v>7.659228215220075e+49</ns0:v>
+        <ns0:v>8.590334148510218e+48</ns0:v>
       </ns0:c>
       <ns0:c r="F56" s="1" t="n">
         <ns0:v>1.541121534915435e+25</ns0:v>
@@ -2807,10 +2807,10 @@
         </ns0:is>
       </ns0:c>
       <ns0:c r="D59" s="1" t="n">
-        <ns0:v>1.44534756981716e+54</ns0:v>
+        <ns0:v>6.970233264936152e+53</ns0:v>
       </ns0:c>
       <ns0:c r="E59" s="1" t="n">
-        <ns0:v>1.44534756981716e+54</ns0:v>
+        <ns0:v>6.970233264936152e+53</ns0:v>
       </ns0:c>
       <ns0:c r="F59" s="1" t="n">
         <ns0:v>1.225143031830274e+27</ns0:v>
@@ -2835,10 +2835,10 @@
         </ns0:is>
       </ns0:c>
       <ns0:c r="D60" s="1" t="n">
-        <ns0:v>6.214729993794608e+54</ns0:v>
+        <ns0:v>1.44534756981716e+54</ns0:v>
       </ns0:c>
       <ns0:c r="E60" s="1" t="n">
-        <ns0:v>6.214729993794608e+54</ns0:v>
+        <ns0:v>1.44534756981716e+54</ns0:v>
       </ns0:c>
       <ns0:c r="F60" s="1" t="n">
         <ns0:v>2.540456590803256e+27</ns0:v>
@@ -2863,10 +2863,10 @@
         </ns0:is>
       </ns0:c>
       <ns0:c r="D61" s="1" t="n">
-        <ns0:v>2.672220142913874e+55</ns0:v>
+        <ns0:v>2.997072720772863e+54</ns0:v>
       </ns0:c>
       <ns0:c r="E61" s="1" t="n">
-        <ns0:v>2.672220142913874e+55</ns0:v>
+        <ns0:v>2.997072720772863e+54</ns0:v>
       </ns0:c>
       <ns0:c r="F61" s="1" t="n">
         <ns0:v>5.267890786689631e+27</ns0:v>

</xml_diff>

<commit_message>
V27 income1.5x from21 and firstdock unlock30,3hbuild unchanged,35 growth128 provisional
</commit_message>
<xml_diff>
--- a/space-battleship/config_excel/level.xlsx
+++ b/space-battleship/config_excel/level.xlsx
@@ -1833,7 +1833,7 @@
         <ns0:v>4763067294395140</ns0:v>
       </ns0:c>
       <ns0:c r="F24" s="1" t="n">
-        <ns0:v>13912338633.23386</ns0:v>
+        <ns0:v>20868507949.85079</ns0:v>
       </ns0:c>
       <ns0:c r="G24" s="1" t="n">
         <ns0:v>5</ns0:v>
@@ -1861,7 +1861,7 @@
         <ns0:v>2.048031753406153e+16</ns0:v>
       </ns0:c>
       <ns0:c r="F25" s="1" t="n">
-        <ns0:v>59820509608.44215</ns0:v>
+        <ns0:v>89730764412.66322</ns0:v>
       </ns0:c>
       <ns0:c r="G25" s="1" t="n">
         <ns0:v>5.2</ns0:v>
@@ -1889,7 +1889,7 @@
         <ns0:v>8.80616166791431e+16</ns0:v>
       </ns0:c>
       <ns0:c r="F26" s="1" t="n">
-        <ns0:v>257217241770.2224</ns0:v>
+        <ns0:v>385825862655.3336</ns0:v>
       </ns0:c>
       <ns0:c r="G26" s="1" t="n">
         <ns0:v>5.4</ns0:v>
@@ -1917,7 +1917,7 @@
         <ns0:v>3.786488329219983e+17</ns0:v>
       </ns0:c>
       <ns0:c r="F27" s="1" t="n">
-        <ns0:v>1105987058568.022</ns0:v>
+        <ns0:v>1658980587852.034</ns0:v>
       </ns0:c>
       <ns0:c r="G27" s="1" t="n">
         <ns0:v>5.6</ns0:v>
@@ -1945,7 +1945,7 @@
         <ns0:v>1.628120673682214e+18</ns0:v>
       </ns0:c>
       <ns0:c r="F28" s="1" t="n">
-        <ns0:v>4755541911971.295</ns0:v>
+        <ns0:v>7133312867956.942</ns0:v>
       </ns0:c>
       <ns0:c r="G28" s="1" t="n">
         <ns0:v>5.8</ns0:v>
@@ -1973,7 +1973,7 @@
         <ns0:v>7.000620885625409e+18</ns0:v>
       </ns0:c>
       <ns0:c r="F29" s="1" t="n">
-        <ns0:v>20447959767085</ns0:v>
+        <ns0:v>30671939650627.49</ns0:v>
       </ns0:c>
       <ns0:c r="G29" s="1" t="n">
         <ns0:v>6</ns0:v>
@@ -2001,7 +2001,7 @@
         <ns0:v>3.010138841454234e+19</ns0:v>
       </ns0:c>
       <ns0:c r="F30" s="1" t="n">
-        <ns0:v>87922484203909.69</ns0:v>
+        <ns0:v>131883726305864.5</ns0:v>
       </ns0:c>
       <ns0:c r="G30" s="1" t="n">
         <ns0:v>6.2</ns0:v>
@@ -2029,7 +2029,7 @@
         <ns0:v>1.294304604243966e+20</ns0:v>
       </ns0:c>
       <ns0:c r="F31" s="1" t="n">
-        <ns0:v>378050588745302.9</ns0:v>
+        <ns0:v>567075883117954.2</ns0:v>
       </ns0:c>
       <ns0:c r="G31" s="1" t="n">
         <ns0:v>6.4</ns0:v>
@@ -2057,7 +2057,7 @@
         <ns0:v>5.565272888734292e+20</ns0:v>
       </ns0:c>
       <ns0:c r="F32" s="1" t="n">
-        <ns0:v>1625548333225038</ns0:v>
+        <ns0:v>2438322499837556</ns0:v>
       </ns0:c>
       <ns0:c r="G32" s="1" t="n">
         <ns0:v>6.6</ns0:v>
@@ -2085,7 +2085,7 @@
         <ns0:v>2.39296547540079e+21</ns0:v>
       </ns0:c>
       <ns0:c r="F33" s="1" t="n">
-        <ns0:v>6989560292500748</ns0:v>
+        <ns0:v>1.048434043875112e+16</ns0:v>
       </ns0:c>
       <ns0:c r="G33" s="1" t="n">
         <ns0:v>6.8</ns0:v>
@@ -2113,7 +2113,7 @@
         <ns0:v>1.512294048887176e+25</ns0:v>
       </ns0:c>
       <ns0:c r="F34" s="1" t="n">
-        <ns0:v>6989560292500748</ns0:v>
+        <ns0:v>1.048434043875112e+16</ns0:v>
       </ns0:c>
       <ns0:c r="G34" s="1" t="n">
         <ns0:v>7</ns0:v>
@@ -2141,7 +2141,7 @@
         <ns0:v>9.363726143873491e+25</ns0:v>
       </ns0:c>
       <ns0:c r="F35" s="1" t="n">
-        <ns0:v>6989560292500748</ns0:v>
+        <ns0:v>1.048434043875112e+16</ns0:v>
       </ns0:c>
       <ns0:c r="G35" s="1" t="n">
         <ns0:v>7.2</ns0:v>
@@ -2169,7 +2169,7 @@
         <ns0:v>8.348792286873683e+26</ns0:v>
       </ns0:c>
       <ns0:c r="F36" s="1" t="n">
-        <ns0:v>1.449355222252955e+16</ns0:v>
+        <ns0:v>2.174032833379432e+16</ns0:v>
       </ns0:c>
       <ns0:c r="G36" s="1" t="n">
         <ns0:v>7.4</ns0:v>
@@ -2197,7 +2197,7 @@
         <ns0:v>1.376253845651405e+29</ns0:v>
       </ns0:c>
       <ns0:c r="F37" s="1" t="n">
-        <ns0:v>1.449355222252955e+16</ns0:v>
+        <ns0:v>2.174032833379432e+16</ns0:v>
       </ns0:c>
       <ns0:c r="G37" s="1" t="n">
         <ns0:v>7.6</ns0:v>
@@ -2219,13 +2219,13 @@
         </ns0:is>
       </ns0:c>
       <ns0:c r="D38" s="1" t="n">
-        <ns0:v>2.268681005093663e+31</ns0:v>
+        <ns0:v>3.266900647334875e+31</ns0:v>
       </ns0:c>
       <ns0:c r="E38" s="1" t="n">
-        <ns0:v>2.268681005093663e+31</ns0:v>
+        <ns0:v>3.266900647334875e+31</ns0:v>
       </ns0:c>
       <ns0:c r="F38" s="1" t="n">
-        <ns0:v>4.327751503963766e+16</ns0:v>
+        <ns0:v>6.491627255945649e+16</ns0:v>
       </ns0:c>
       <ns0:c r="G38" s="1" t="n">
         <ns0:v>7.8</ns0:v>
@@ -2247,13 +2247,13 @@
         </ns0:is>
       </ns0:c>
       <ns0:c r="D39" s="1" t="n">
-        <ns0:v>4.70433693216222e+31</ns0:v>
+        <ns0:v>6.774245182313596e+31</ns0:v>
       </ns0:c>
       <ns0:c r="E39" s="1" t="n">
-        <ns0:v>4.70433693216222e+31</ns0:v>
+        <ns0:v>6.774245182313596e+31</ns0:v>
       </ns0:c>
       <ns0:c r="F39" s="1" t="n">
-        <ns0:v>8.974025518619266e+16</ns0:v>
+        <ns0:v>1.34610382779289e+17</ns0:v>
       </ns0:c>
       <ns0:c r="G39" s="1" t="n">
         <ns0:v>8</ns0:v>
@@ -2275,13 +2275,13 @@
         </ns0:is>
       </ns0:c>
       <ns0:c r="D40" s="1" t="n">
-        <ns0:v>9.754913062531577e+31</ns0:v>
+        <ns0:v>1.404707481004547e+32</ns0:v>
       </ns0:c>
       <ns0:c r="E40" s="1" t="n">
-        <ns0:v>9.754913062531577e+31</ns0:v>
+        <ns0:v>1.404707481004547e+32</ns0:v>
       </ns0:c>
       <ns0:c r="F40" s="1" t="n">
-        <ns0:v>1.86085393154089e+17</ns0:v>
+        <ns0:v>2.791280897311335e+17</ns0:v>
       </ns0:c>
       <ns0:c r="G40" s="1" t="n">
         <ns0:v>8.199999999999999</ns0:v>
@@ -2303,13 +2303,13 @@
         </ns0:is>
       </ns0:c>
       <ns0:c r="D41" s="1" t="n">
-        <ns0:v>2.022778772646547e+32</ns0:v>
+        <ns0:v>2.912801432611028e+32</ns0:v>
       </ns0:c>
       <ns0:c r="E41" s="1" t="n">
-        <ns0:v>2.022778772646547e+32</ns0:v>
+        <ns0:v>2.912801432611028e+32</ns0:v>
       </ns0:c>
       <ns0:c r="F41" s="1" t="n">
-        <ns0:v>3.85866671244319e+17</ns0:v>
+        <ns0:v>5.788000068664785e+17</ns0:v>
       </ns0:c>
       <ns0:c r="G41" s="1" t="n">
         <ns0:v>8.4</ns0:v>
@@ -2331,13 +2331,13 @@
         </ns0:is>
       </ns0:c>
       <ns0:c r="D42" s="1" t="n">
-        <ns0:v>4.801597686832596e+34</ns0:v>
+        <ns0:v>6.914300669038937e+34</ns0:v>
       </ns0:c>
       <ns0:c r="E42" s="1" t="n">
-        <ns0:v>4.801597686832596e+34</ns0:v>
+        <ns0:v>6.914300669038937e+34</ns0:v>
       </ns0:c>
       <ns0:c r="F42" s="1" t="n">
-        <ns0:v>1.659156057315067e+18</ns0:v>
+        <ns0:v>2.4887340859726e+18</ns0:v>
       </ns0:c>
       <ns0:c r="G42" s="1" t="n">
         <ns0:v>8.6</ns0:v>
@@ -2359,13 +2359,13 @@
         </ns0:is>
       </ns0:c>
       <ns0:c r="D43" s="1" t="n">
-        <ns0:v>7.91517749479043e+36</ns0:v>
+        <ns0:v>1.139785559249822e+37</ns0:v>
       </ns0:c>
       <ns0:c r="E43" s="1" t="n">
-        <ns0:v>7.91517749479043e+36</ns0:v>
+        <ns0:v>1.139785559249822e+37</ns0:v>
       </ns0:c>
       <ns0:c r="F43" s="1" t="n">
-        <ns0:v>1.479320206635352e+19</ns0:v>
+        <ns0:v>2.218980309953027e+19</ns0:v>
       </ns0:c>
       <ns0:c r="G43" s="1" t="n">
         <ns0:v>8.800000000000001</ns0:v>
@@ -2387,13 +2387,13 @@
         </ns0:is>
       </ns0:c>
       <ns0:c r="D44" s="1" t="n">
-        <ns0:v>1.641291205319743e+37</ns0:v>
+        <ns0:v>2.36345933566043e+37</ns0:v>
       </ns0:c>
       <ns0:c r="E44" s="1" t="n">
-        <ns0:v>1.641291205319743e+37</ns0:v>
+        <ns0:v>2.36345933566043e+37</ns0:v>
       </ns0:c>
       <ns0:c r="F44" s="1" t="n">
-        <ns0:v>3.067518380479065e+19</ns0:v>
+        <ns0:v>4.601277570718597e+19</ns0:v>
       </ns0:c>
       <ns0:c r="G44" s="1" t="n">
         <ns0:v>9</ns0:v>
@@ -2415,13 +2415,13 @@
         </ns0:is>
       </ns0:c>
       <ns0:c r="D45" s="1" t="n">
-        <ns0:v>3.403381443351019e+37</ns0:v>
+        <ns0:v>4.900869278425467e+37</ns0:v>
       </ns0:c>
       <ns0:c r="E45" s="1" t="n">
-        <ns0:v>3.403381443351019e+37</ns0:v>
+        <ns0:v>4.900869278425467e+37</ns0:v>
       </ns0:c>
       <ns0:c r="F45" s="1" t="n">
-        <ns0:v>6.360806113761387e+19</ns0:v>
+        <ns0:v>9.541209170642081e+19</ns0:v>
       </ns0:c>
       <ns0:c r="G45" s="1" t="n">
         <ns0:v>9.199999999999999</ns0:v>
@@ -2443,13 +2443,13 @@
         </ns0:is>
       </ns0:c>
       <ns0:c r="D46" s="1" t="n">
-        <ns0:v>7.057251760932672e+37</ns0:v>
+        <ns0:v>1.016244253574305e+38</ns0:v>
       </ns0:c>
       <ns0:c r="E46" s="1" t="n">
-        <ns0:v>7.057251760932672e+37</ns0:v>
+        <ns0:v>1.016244253574305e+38</ns0:v>
       </ns0:c>
       <ns0:c r="F46" s="1" t="n">
-        <ns0:v>1.318976755749561e+20</ns0:v>
+        <ns0:v>1.978465133624342e+20</ns0:v>
       </ns0:c>
       <ns0:c r="G46" s="1" t="n">
         <ns0:v>9.4</ns0:v>
@@ -2471,13 +2471,13 @@
         </ns0:is>
       </ns0:c>
       <ns0:c r="D47" s="1" t="n">
-        <ns0:v>1.67522440856713e+40</ns0:v>
+        <ns0:v>2.412323148336667e+40</ns0:v>
       </ns0:c>
       <ns0:c r="E47" s="1" t="n">
-        <ns0:v>1.67522440856713e+40</ns0:v>
+        <ns0:v>2.412323148336667e+40</ns0:v>
       </ns0:c>
       <ns0:c r="F47" s="1" t="n">
-        <ns0:v>5.671358624217739e+20</ns0:v>
+        <ns0:v>8.507037936326608e+20</ns0:v>
       </ns0:c>
       <ns0:c r="G47" s="1" t="n">
         <ns0:v>9.6</ns0:v>
@@ -2499,13 +2499,13 @@
         </ns0:is>
       </ns0:c>
       <ns0:c r="D48" s="1" t="n">
-        <ns0:v>2.761518020090726e+42</ns0:v>
+        <ns0:v>3.976585948930644e+42</ns0:v>
       </ns0:c>
       <ns0:c r="E48" s="1" t="n">
-        <ns0:v>2.761518020090726e+42</ns0:v>
+        <ns0:v>3.976585948930644e+42</ns0:v>
       </ns0:c>
       <ns0:c r="F48" s="1" t="n">
-        <ns0:v>5.056640317160829e+21</ns0:v>
+        <ns0:v>7.584960475741243e+21</ns0:v>
       </ns0:c>
       <ns0:c r="G48" s="1" t="n">
         <ns0:v>9.800000000000001</ns0:v>
@@ -2527,13 +2527,13 @@
         </ns0:is>
       </ns0:c>
       <ns0:c r="D49" s="1" t="n">
-        <ns0:v>5.726283766460129e+42</ns0:v>
+        <ns0:v>8.245848623702583e+42</ns0:v>
       </ns0:c>
       <ns0:c r="E49" s="1" t="n">
-        <ns0:v>5.726283766460129e+42</ns0:v>
+        <ns0:v>8.245848623702583e+42</ns0:v>
       </ns0:c>
       <ns0:c r="F49" s="1" t="n">
-        <ns0:v>1.048544936166469e+22</ns0:v>
+        <ns0:v>1.572817404249704e+22</ns0:v>
       </ns0:c>
       <ns0:c r="G49" s="1" t="n">
         <ns0:v>10</ns0:v>
@@ -2555,13 +2555,13 @@
         </ns0:is>
       </ns0:c>
       <ns0:c r="D50" s="1" t="n">
-        <ns0:v>1.187402201813172e+43</ns0:v>
+        <ns0:v>1.709859170610967e+43</ns0:v>
       </ns0:c>
       <ns0:c r="E50" s="1" t="n">
-        <ns0:v>1.187402201813172e+43</ns0:v>
+        <ns0:v>1.709859170610967e+43</ns0:v>
       </ns0:c>
       <ns0:c r="F50" s="1" t="n">
-        <ns0:v>2.17426277963479e+22</ns0:v>
+        <ns0:v>3.261394169452185e+22</ns0:v>
       </ns0:c>
       <ns0:c r="G50" s="1" t="n">
         <ns0:v>10.2</ns0:v>
@@ -2583,13 +2583,13 @@
         </ns0:is>
       </ns0:c>
       <ns0:c r="D51" s="1" t="n">
-        <ns0:v>2.462197205679793e+43</ns0:v>
+        <ns0:v>3.545563976178901e+43</ns0:v>
       </ns0:c>
       <ns0:c r="E51" s="1" t="n">
-        <ns0:v>2.462197205679793e+43</ns0:v>
+        <ns0:v>3.545563976178901e+43</ns0:v>
       </ns0:c>
       <ns0:c r="F51" s="1" t="n">
-        <ns0:v>4.508551299850701e+22</ns0:v>
+        <ns0:v>6.762826949776052e+22</ns0:v>
       </ns0:c>
       <ns0:c r="G51" s="1" t="n">
         <ns0:v>10.4</ns0:v>
@@ -2611,13 +2611,13 @@
         </ns0:is>
       </ns0:c>
       <ns0:c r="D52" s="1" t="n">
-        <ns0:v>5.844672965323622e+45</ns0:v>
+        <ns0:v>8.416329070066014e+45</ns0:v>
       </ns0:c>
       <ns0:c r="E52" s="1" t="n">
-        <ns0:v>5.844672965323622e+45</ns0:v>
+        <ns0:v>8.416329070066014e+45</ns0:v>
       </ns0:c>
       <ns0:c r="F52" s="1" t="n">
-        <ns0:v>1.938594534412808e+23</ns0:v>
+        <ns0:v>2.907891801619212e+23</ns0:v>
       </ns0:c>
       <ns0:c r="G52" s="1" t="n">
         <ns0:v>10.6</ns0:v>
@@ -2639,13 +2639,13 @@
         </ns0:is>
       </ns0:c>
       <ns0:c r="D53" s="1" t="n">
-        <ns0:v>9.634631415789513e+47</ns0:v>
+        <ns0:v>1.38738692387369e+48</ns0:v>
       </ns0:c>
       <ns0:c r="E53" s="1" t="n">
-        <ns0:v>9.634631415789513e+47</ns0:v>
+        <ns0:v>1.38738692387369e+48</ns0:v>
       </ns0:c>
       <ns0:c r="F53" s="1" t="n">
-        <ns0:v>1.728470359726467e+24</ns0:v>
+        <ns0:v>2.5927055395897e+24</ns0:v>
       </ns0:c>
       <ns0:c r="G53" s="1" t="n">
         <ns0:v>10.8</ns0:v>
@@ -2667,13 +2667,13 @@
         </ns0:is>
       </ns0:c>
       <ns0:c r="D54" s="1" t="n">
-        <ns0:v>1.997837170378113e+48</ns0:v>
+        <ns0:v>2.876885525344483e+48</ns0:v>
       </ns0:c>
       <ns0:c r="E54" s="1" t="n">
-        <ns0:v>1.997837170378113e+48</ns0:v>
+        <ns0:v>2.876885525344483e+48</ns0:v>
       </ns0:c>
       <ns0:c r="F54" s="1" t="n">
-        <ns0:v>3.584156137928801e+24</ns0:v>
+        <ns0:v>5.376234206893201e+24</ns0:v>
       </ns0:c>
       <ns0:c r="G54" s="1" t="n">
         <ns0:v>11</ns0:v>
@@ -2695,13 +2695,13 @@
         </ns0:is>
       </ns0:c>
       <ns0:c r="D55" s="1" t="n">
-        <ns0:v>4.142715156496054e+48</ns0:v>
+        <ns0:v>5.965509825354318e+48</ns0:v>
       </ns0:c>
       <ns0:c r="E55" s="1" t="n">
-        <ns0:v>4.142715156496054e+48</ns0:v>
+        <ns0:v>5.965509825354318e+48</ns0:v>
       </ns0:c>
       <ns0:c r="F55" s="1" t="n">
-        <ns0:v>7.43210616760916e+24</ns0:v>
+        <ns0:v>1.114815925141374e+25</ns0:v>
       </ns0:c>
       <ns0:c r="G55" s="1" t="n">
         <ns0:v>11.2</ns0:v>
@@ -2723,13 +2723,13 @@
         </ns0:is>
       </ns0:c>
       <ns0:c r="D56" s="1" t="n">
-        <ns0:v>8.590334148510218e+48</ns0:v>
+        <ns0:v>1.237008117385471e+49</ns0:v>
       </ns0:c>
       <ns0:c r="E56" s="1" t="n">
-        <ns0:v>8.590334148510218e+48</ns0:v>
+        <ns0:v>1.237008117385471e+49</ns0:v>
       </ns0:c>
       <ns0:c r="F56" s="1" t="n">
-        <ns0:v>1.541121534915435e+25</ns0:v>
+        <ns0:v>2.311682302373153e+25</ns0:v>
       </ns0:c>
       <ns0:c r="G56" s="1" t="n">
         <ns0:v>11.4</ns0:v>
@@ -2751,13 +2751,13 @@
         </ns0:is>
       </ns0:c>
       <ns0:c r="D57" s="1" t="n">
-        <ns0:v>2.039141854481638e+51</ns0:v>
+        <ns0:v>2.936364270453558e+51</ns0:v>
       </ns0:c>
       <ns0:c r="E57" s="1" t="n">
-        <ns0:v>2.039141854481638e+51</ns0:v>
+        <ns0:v>2.936364270453558e+51</ns0:v>
       </ns0:c>
       <ns0:c r="F57" s="1" t="n">
-        <ns0:v>6.626540513250619e+25</ns0:v>
+        <ns0:v>9.939810769875926e+25</ns0:v>
       </ns0:c>
       <ns0:c r="G57" s="1" t="n">
         <ns0:v>11.6</ns0:v>
@@ -2779,13 +2779,13 @@
         </ns0:is>
       </ns0:c>
       <ns0:c r="D58" s="1" t="n">
-        <ns0:v>3.361416505081092e+53</ns0:v>
+        <ns0:v>4.840439767316772e+53</ns0:v>
       </ns0:c>
       <ns0:c r="E58" s="1" t="n">
-        <ns0:v>3.361416505081092e+53</ns0:v>
+        <ns0:v>4.840439767316772e+53</ns0:v>
       </ns0:c>
       <ns0:c r="F58" s="1" t="n">
-        <ns0:v>5.908290084058036e+26</ns0:v>
+        <ns0:v>8.862435126087053e+26</ns0:v>
       </ns0:c>
       <ns0:c r="G58" s="1" t="n">
         <ns0:v>11.8</ns0:v>
@@ -2807,13 +2807,13 @@
         </ns0:is>
       </ns0:c>
       <ns0:c r="D59" s="1" t="n">
-        <ns0:v>6.970233264936152e+53</ns0:v>
+        <ns0:v>1.003713590150806e+54</ns0:v>
       </ns0:c>
       <ns0:c r="E59" s="1" t="n">
-        <ns0:v>6.970233264936152e+53</ns0:v>
+        <ns0:v>1.003713590150806e+54</ns0:v>
       </ns0:c>
       <ns0:c r="F59" s="1" t="n">
-        <ns0:v>1.225143031830274e+27</ns0:v>
+        <ns0:v>1.837714547745411e+27</ns0:v>
       </ns0:c>
       <ns0:c r="G59" s="1" t="n">
         <ns0:v>12</ns0:v>
@@ -2835,13 +2835,13 @@
         </ns0:is>
       </ns0:c>
       <ns0:c r="D60" s="1" t="n">
-        <ns0:v>1.44534756981716e+54</ns0:v>
+        <ns0:v>2.08130050053671e+54</ns0:v>
       </ns0:c>
       <ns0:c r="E60" s="1" t="n">
-        <ns0:v>1.44534756981716e+54</ns0:v>
+        <ns0:v>2.08130050053671e+54</ns0:v>
       </ns0:c>
       <ns0:c r="F60" s="1" t="n">
-        <ns0:v>2.540456590803256e+27</ns0:v>
+        <ns0:v>3.810684886204884e+27</ns0:v>
       </ns0:c>
       <ns0:c r="G60" s="1" t="n">
         <ns0:v>12.2</ns0:v>
@@ -2863,13 +2863,13 @@
         </ns0:is>
       </ns0:c>
       <ns0:c r="D61" s="1" t="n">
-        <ns0:v>2.997072720772863e+54</ns0:v>
+        <ns0:v>4.315784717912922e+54</ns0:v>
       </ns0:c>
       <ns0:c r="E61" s="1" t="n">
-        <ns0:v>2.997072720772863e+54</ns0:v>
+        <ns0:v>4.315784717912922e+54</ns0:v>
       </ns0:c>
       <ns0:c r="F61" s="1" t="n">
-        <ns0:v>5.267890786689631e+27</ns0:v>
+        <ns0:v>7.901836180034445e+27</ns0:v>
       </ns0:c>
       <ns0:c r="G61" s="1" t="n">
         <ns0:v>12.4</ns0:v>
@@ -2891,13 +2891,13 @@
         </ns0:is>
       </ns0:c>
       <ns0:c r="D62" s="1" t="n">
-        <ns0:v>7.114340746469082e+56</ns0:v>
+        <ns0:v>1.024465067491548e+57</ns0:v>
       </ns0:c>
       <ns0:c r="E62" s="1" t="n">
-        <ns0:v>7.114340746469082e+56</ns0:v>
+        <ns0:v>1.024465067491548e+57</ns0:v>
       </ns0:c>
       <ns0:c r="F62" s="1" t="n">
-        <ns0:v>2.265096614803581e+28</ns0:v>
+        <ns0:v>3.397644922205371e+28</ns0:v>
       </ns0:c>
       <ns0:c r="G62" s="1" t="n">
         <ns0:v>12.6</ns0:v>
@@ -2919,13 +2919,13 @@
         </ns0:is>
       </ns0:c>
       <ns0:c r="D63" s="1" t="n">
-        <ns0:v>1.172761098272453e+59</ns0:v>
+        <ns0:v>1.688775981512331e+59</ns0:v>
       </ns0:c>
       <ns0:c r="E63" s="1" t="n">
-        <ns0:v>1.172761098272453e+59</ns0:v>
+        <ns0:v>1.688775981512331e+59</ns0:v>
       </ns0:c>
       <ns0:c r="F63" s="1" t="n">
-        <ns0:v>2.019582894259335e+29</ns0:v>
+        <ns0:v>3.029374341389002e+29</ns0:v>
       </ns0:c>
       <ns0:c r="G63" s="1" t="n">
         <ns0:v>12.8</ns0:v>
@@ -2948,15 +2948,15 @@
       </ns0:c>
       <ns0:c r="D64" s="1">
         <ns0:f>ROUND(D63*10,0)</ns0:f>
-        <ns0:v>1.1727610982724526e+60</ns0:v>
+        <ns0:v>1.6887759815123313e+60</ns0:v>
       </ns0:c>
       <ns0:c r="E64" s="1">
         <ns0:f>D64</ns0:f>
-        <ns0:v>1.1727610982724526e+60</ns0:v>
+        <ns0:v>1.6887759815123313e+60</ns0:v>
       </ns0:c>
       <ns0:c r="F64" s="1">
         <ns0:f>ROUND(F63*1.4,-5)</ns0:f>
-        <ns0:v>2.8274160519630688e+29</ns0:v>
+        <ns0:v>4.241124077944603e+29</ns0:v>
       </ns0:c>
       <ns0:c r="G64" s="1" t="n">
         <ns0:v>13</ns0:v>
@@ -2979,15 +2979,15 @@
       </ns0:c>
       <ns0:c r="D65" s="1">
         <ns0:f>ROUND(D64*10,0)</ns0:f>
-        <ns0:v>1.1727610982724527e+61</ns0:v>
+        <ns0:v>1.6887759815123314e+61</ns0:v>
       </ns0:c>
       <ns0:c r="E65" s="1">
         <ns0:f>D65</ns0:f>
-        <ns0:v>1.1727610982724527e+61</ns0:v>
+        <ns0:v>1.6887759815123314e+61</ns0:v>
       </ns0:c>
       <ns0:c r="F65" s="1">
         <ns0:f>ROUND(F64*1.4,-5)</ns0:f>
-        <ns0:v>3.958382472748296e+29</ns0:v>
+        <ns0:v>5.937573709122444e+29</ns0:v>
       </ns0:c>
       <ns0:c r="G65" s="1" t="n">
         <ns0:v>13.2</ns0:v>
@@ -3010,15 +3010,15 @@
       </ns0:c>
       <ns0:c r="D66" s="1">
         <ns0:f>ROUND(D65*10,0)</ns0:f>
-        <ns0:v>1.1727610982724528e+62</ns0:v>
+        <ns0:v>1.6887759815123314e+62</ns0:v>
       </ns0:c>
       <ns0:c r="E66" s="1">
         <ns0:f>D66</ns0:f>
-        <ns0:v>1.1727610982724528e+62</ns0:v>
+        <ns0:v>1.6887759815123314e+62</ns0:v>
       </ns0:c>
       <ns0:c r="F66" s="1">
         <ns0:f>ROUND(F65*1.4,-5)</ns0:f>
-        <ns0:v>5.541735461847614e+29</ns0:v>
+        <ns0:v>8.312603192771421e+29</ns0:v>
       </ns0:c>
       <ns0:c r="G66" s="1" t="n">
         <ns0:v>13.4</ns0:v>
@@ -3041,15 +3041,15 @@
       </ns0:c>
       <ns0:c r="D67" s="1">
         <ns0:f>ROUND(D66*10,0)</ns0:f>
-        <ns0:v>1.1727610982724528e+63</ns0:v>
+        <ns0:v>1.6887759815123315e+63</ns0:v>
       </ns0:c>
       <ns0:c r="E67" s="1">
         <ns0:f>D67</ns0:f>
-        <ns0:v>1.1727610982724528e+63</ns0:v>
+        <ns0:v>1.6887759815123315e+63</ns0:v>
       </ns0:c>
       <ns0:c r="F67" s="1">
         <ns0:f>ROUND(F66*1.4,-5)</ns0:f>
-        <ns0:v>7.758429646586659e+29</ns0:v>
+        <ns0:v>1.1637644469879989e+30</ns0:v>
       </ns0:c>
       <ns0:c r="G67" s="1" t="n">
         <ns0:v>13.6</ns0:v>
@@ -3072,15 +3072,15 @@
       </ns0:c>
       <ns0:c r="D68" s="1">
         <ns0:f>ROUND(D67*10,0)</ns0:f>
-        <ns0:v>1.1727610982724528e+64</ns0:v>
+        <ns0:v>1.6887759815123314e+64</ns0:v>
       </ns0:c>
       <ns0:c r="E68" s="1">
         <ns0:f>D68</ns0:f>
-        <ns0:v>1.1727610982724528e+64</ns0:v>
+        <ns0:v>1.6887759815123314e+64</ns0:v>
       </ns0:c>
       <ns0:c r="F68" s="1">
         <ns0:f>ROUND(F67*1.4,-5)</ns0:f>
-        <ns0:v>1.0861801505221322e+30</ns0:v>
+        <ns0:v>1.6292702257831982e+30</ns0:v>
       </ns0:c>
       <ns0:c r="G68" s="1" t="n">
         <ns0:v>13.8</ns0:v>
@@ -3103,15 +3103,15 @@
       </ns0:c>
       <ns0:c r="D69" s="1">
         <ns0:f>ROUND(D68*10,0)</ns0:f>
-        <ns0:v>1.172761098272453e+65</ns0:v>
+        <ns0:v>1.6887759815123313e+65</ns0:v>
       </ns0:c>
       <ns0:c r="E69" s="1">
         <ns0:f>D69</ns0:f>
-        <ns0:v>1.172761098272453e+65</ns0:v>
+        <ns0:v>1.6887759815123313e+65</ns0:v>
       </ns0:c>
       <ns0:c r="F69" s="1">
         <ns0:f>ROUND(F68*1.4,-5)</ns0:f>
-        <ns0:v>1.520652210730985e+30</ns0:v>
+        <ns0:v>2.2809783160964777e+30</ns0:v>
       </ns0:c>
       <ns0:c r="G69" s="1" t="n">
         <ns0:v>14</ns0:v>
@@ -3134,15 +3134,15 @@
       </ns0:c>
       <ns0:c r="D70" s="1">
         <ns0:f>ROUND(D69*10,0)</ns0:f>
-        <ns0:v>1.1727610982724529e+66</ns0:v>
+        <ns0:v>1.688775981512331e+66</ns0:v>
       </ns0:c>
       <ns0:c r="E70" s="1">
         <ns0:f>D70</ns0:f>
-        <ns0:v>1.1727610982724529e+66</ns0:v>
+        <ns0:v>1.688775981512331e+66</ns0:v>
       </ns0:c>
       <ns0:c r="F70" s="1">
         <ns0:f>ROUND(F69*1.4,-5)</ns0:f>
-        <ns0:v>2.1289130950233787e+30</ns0:v>
+        <ns0:v>3.1933696425350686e+30</ns0:v>
       </ns0:c>
       <ns0:c r="G70" s="1" t="n">
         <ns0:v>14.2</ns0:v>
@@ -3165,15 +3165,15 @@
       </ns0:c>
       <ns0:c r="D71" s="1">
         <ns0:f>ROUND(D70*10,0)</ns0:f>
-        <ns0:v>1.1727610982724529e+67</ns0:v>
+        <ns0:v>1.688775981512331e+67</ns0:v>
       </ns0:c>
       <ns0:c r="E71" s="1">
         <ns0:f>D71</ns0:f>
-        <ns0:v>1.1727610982724529e+67</ns0:v>
+        <ns0:v>1.688775981512331e+67</ns0:v>
       </ns0:c>
       <ns0:c r="F71" s="1">
         <ns0:f>ROUND(F70*1.4,-5)</ns0:f>
-        <ns0:v>2.98047833303273e+30</ns0:v>
+        <ns0:v>4.4707174995490955e+30</ns0:v>
       </ns0:c>
       <ns0:c r="G71" s="1" t="n">
         <ns0:v>14.4</ns0:v>
@@ -3196,15 +3196,15 @@
       </ns0:c>
       <ns0:c r="D72" s="1">
         <ns0:f>ROUND(D71*10,0)</ns0:f>
-        <ns0:v>1.172761098272453e+68</ns0:v>
+        <ns0:v>1.688775981512331e+68</ns0:v>
       </ns0:c>
       <ns0:c r="E72" s="1">
         <ns0:f>D72</ns0:f>
-        <ns0:v>1.172761098272453e+68</ns0:v>
+        <ns0:v>1.688775981512331e+68</ns0:v>
       </ns0:c>
       <ns0:c r="F72" s="1">
         <ns0:f>ROUND(F71*1.4,-5)</ns0:f>
-        <ns0:v>4.172669666245821e+30</ns0:v>
+        <ns0:v>6.259004499368733e+30</ns0:v>
       </ns0:c>
       <ns0:c r="G72" s="1" t="n">
         <ns0:v>14.6</ns0:v>
@@ -3227,15 +3227,15 @@
       </ns0:c>
       <ns0:c r="D73" s="1">
         <ns0:f>ROUND(D72*10,0)</ns0:f>
-        <ns0:v>1.172761098272453e+69</ns0:v>
+        <ns0:v>1.688775981512331e+69</ns0:v>
       </ns0:c>
       <ns0:c r="E73" s="1">
         <ns0:f>D73</ns0:f>
-        <ns0:v>1.172761098272453e+69</ns0:v>
+        <ns0:v>1.688775981512331e+69</ns0:v>
       </ns0:c>
       <ns0:c r="F73" s="1">
         <ns0:f>ROUND(F72*1.4,-5)</ns0:f>
-        <ns0:v>5.841737532744149e+30</ns0:v>
+        <ns0:v>8.762606299116227e+30</ns0:v>
       </ns0:c>
       <ns0:c r="G73" s="1" t="n">
         <ns0:v>14.8</ns0:v>
@@ -3258,15 +3258,15 @@
       </ns0:c>
       <ns0:c r="D74" s="1">
         <ns0:f>ROUND(D73*10,0)</ns0:f>
-        <ns0:v>1.172761098272453e+70</ns0:v>
+        <ns0:v>1.688775981512331e+70</ns0:v>
       </ns0:c>
       <ns0:c r="E74" s="1">
         <ns0:f>D74</ns0:f>
-        <ns0:v>1.172761098272453e+70</ns0:v>
+        <ns0:v>1.688775981512331e+70</ns0:v>
       </ns0:c>
       <ns0:c r="F74" s="1">
         <ns0:f>ROUND(F73*1.4,-5)</ns0:f>
-        <ns0:v>8.178432545841808e+30</ns0:v>
+        <ns0:v>1.2267648818762717e+31</ns0:v>
       </ns0:c>
       <ns0:c r="G74" s="1" t="n">
         <ns0:v>15</ns0:v>
@@ -3290,15 +3290,15 @@
       </ns0:c>
       <ns0:c r="D75" s="1">
         <ns0:f>ROUND(D74*10,0)</ns0:f>
-        <ns0:v>1.172761098272453e+71</ns0:v>
+        <ns0:v>1.6887759815123311e+71</ns0:v>
       </ns0:c>
       <ns0:c r="E75" s="1">
         <ns0:f>D75</ns0:f>
-        <ns0:v>1.172761098272453e+71</ns0:v>
+        <ns0:v>1.6887759815123311e+71</ns0:v>
       </ns0:c>
       <ns0:c r="F75" s="1">
         <ns0:f>ROUND(F74*1.4,-5)</ns0:f>
-        <ns0:v>1.144980556417853e+31</ns0:v>
+        <ns0:v>1.71747083462678e+31</ns0:v>
       </ns0:c>
       <ns0:c r="G75" s="1" t="n">
         <ns0:v>15.2</ns0:v>
@@ -3322,15 +3322,15 @@
       </ns0:c>
       <ns0:c r="D76" s="1">
         <ns0:f>ROUND(D75*10,0)</ns0:f>
-        <ns0:v>1.172761098272453e+72</ns0:v>
+        <ns0:v>1.6887759815123311e+72</ns0:v>
       </ns0:c>
       <ns0:c r="E76" s="1">
         <ns0:f>D76</ns0:f>
-        <ns0:v>1.172761098272453e+72</ns0:v>
+        <ns0:v>1.6887759815123311e+72</ns0:v>
       </ns0:c>
       <ns0:c r="F76" s="1">
         <ns0:f>ROUND(F75*1.4,-5)</ns0:f>
-        <ns0:v>1.6029727789849941e+31</ns0:v>
+        <ns0:v>2.404459168477492e+31</ns0:v>
       </ns0:c>
       <ns0:c r="G76" s="1" t="n">
         <ns0:v>15.4</ns0:v>
@@ -3354,15 +3354,15 @@
       </ns0:c>
       <ns0:c r="D77" s="1">
         <ns0:f>ROUND(D76*10,0)</ns0:f>
-        <ns0:v>1.1727610982724531e+73</ns0:v>
+        <ns0:v>1.688775981512331e+73</ns0:v>
       </ns0:c>
       <ns0:c r="E77" s="1">
         <ns0:f>D77</ns0:f>
-        <ns0:v>1.1727610982724531e+73</ns0:v>
+        <ns0:v>1.688775981512331e+73</ns0:v>
       </ns0:c>
       <ns0:c r="F77" s="1">
         <ns0:f>ROUND(F76*1.4,-5)</ns0:f>
-        <ns0:v>2.2441618905789915e+31</ns0:v>
+        <ns0:v>3.366242835868489e+31</ns0:v>
       </ns0:c>
       <ns0:c r="G77" s="1" t="n">
         <ns0:v>15.6</ns0:v>
@@ -3386,15 +3386,15 @@
       </ns0:c>
       <ns0:c r="D78" s="1">
         <ns0:f>ROUND(D77*10,0)</ns0:f>
-        <ns0:v>1.172761098272453e+74</ns0:v>
+        <ns0:v>1.688775981512331e+74</ns0:v>
       </ns0:c>
       <ns0:c r="E78" s="1">
         <ns0:f>D78</ns0:f>
-        <ns0:v>1.172761098272453e+74</ns0:v>
+        <ns0:v>1.688775981512331e+74</ns0:v>
       </ns0:c>
       <ns0:c r="F78" s="1">
         <ns0:f>ROUND(F77*1.4,-5)</ns0:f>
-        <ns0:v>3.141826646810588e+31</ns0:v>
+        <ns0:v>4.712739970215884e+31</ns0:v>
       </ns0:c>
       <ns0:c r="G78" s="1" t="n">
         <ns0:v>15.8</ns0:v>
@@ -3418,15 +3418,15 @@
       </ns0:c>
       <ns0:c r="D79" s="1">
         <ns0:f>ROUND(D78*10,0)</ns0:f>
-        <ns0:v>1.1727610982724531e+75</ns0:v>
+        <ns0:v>1.688775981512331e+75</ns0:v>
       </ns0:c>
       <ns0:c r="E79" s="1">
         <ns0:f>D79</ns0:f>
-        <ns0:v>1.1727610982724531e+75</ns0:v>
+        <ns0:v>1.688775981512331e+75</ns0:v>
       </ns0:c>
       <ns0:c r="F79" s="1">
         <ns0:f>ROUND(F78*1.4,-5)</ns0:f>
-        <ns0:v>4.398557305534823e+31</ns0:v>
+        <ns0:v>6.597835958302237e+31</ns0:v>
       </ns0:c>
       <ns0:c r="G79" s="1" t="n">
         <ns0:v>16</ns0:v>
@@ -3450,15 +3450,15 @@
       </ns0:c>
       <ns0:c r="D80" s="1">
         <ns0:f>ROUND(D79*10,0)</ns0:f>
-        <ns0:v>1.1727610982724532e+76</ns0:v>
+        <ns0:v>1.6887759815123312e+76</ns0:v>
       </ns0:c>
       <ns0:c r="E80" s="1">
         <ns0:f>D80</ns0:f>
-        <ns0:v>1.1727610982724532e+76</ns0:v>
+        <ns0:v>1.6887759815123312e+76</ns0:v>
       </ns0:c>
       <ns0:c r="F80" s="1">
         <ns0:f>ROUND(F79*1.4,-5)</ns0:f>
-        <ns0:v>6.157980227748752e+31</ns0:v>
+        <ns0:v>9.236970341623131e+31</ns0:v>
       </ns0:c>
       <ns0:c r="G80" s="1" t="n">
         <ns0:v>16.2</ns0:v>
@@ -3482,15 +3482,15 @@
       </ns0:c>
       <ns0:c r="D81" s="1">
         <ns0:f>ROUND(D80*10,0)</ns0:f>
-        <ns0:v>1.1727610982724532e+77</ns0:v>
+        <ns0:v>1.6887759815123313e+77</ns0:v>
       </ns0:c>
       <ns0:c r="E81" s="1">
         <ns0:f>D81</ns0:f>
-        <ns0:v>1.1727610982724532e+77</ns0:v>
+        <ns0:v>1.6887759815123313e+77</ns0:v>
       </ns0:c>
       <ns0:c r="F81" s="1">
         <ns0:f>ROUND(F80*1.4,-5)</ns0:f>
-        <ns0:v>8.621172318848253e+31</ns0:v>
+        <ns0:v>1.2931758478272382e+32</ns0:v>
       </ns0:c>
       <ns0:c r="G81" s="1" t="n">
         <ns0:v>16.4</ns0:v>
@@ -3514,15 +3514,15 @@
       </ns0:c>
       <ns0:c r="D82" s="1">
         <ns0:f>ROUND(D81*10,0)</ns0:f>
-        <ns0:v>1.1727610982724532e+78</ns0:v>
+        <ns0:v>1.6887759815123314e+78</ns0:v>
       </ns0:c>
       <ns0:c r="E82" s="1">
         <ns0:f>D82</ns0:f>
-        <ns0:v>1.1727610982724532e+78</ns0:v>
+        <ns0:v>1.6887759815123314e+78</ns0:v>
       </ns0:c>
       <ns0:c r="F82" s="1">
         <ns0:f>ROUND(F81*1.4,-5)</ns0:f>
-        <ns0:v>1.2069641246387554e+32</ns0:v>
+        <ns0:v>1.8104461869581333e+32</ns0:v>
       </ns0:c>
       <ns0:c r="G82" s="1" t="n">
         <ns0:v>16.6</ns0:v>
@@ -3546,15 +3546,15 @@
       </ns0:c>
       <ns0:c r="D83" s="1">
         <ns0:f>ROUND(D82*10,0)</ns0:f>
-        <ns0:v>1.1727610982724531e+79</ns0:v>
+        <ns0:v>1.6887759815123314e+79</ns0:v>
       </ns0:c>
       <ns0:c r="E83" s="1">
         <ns0:f>D83</ns0:f>
-        <ns0:v>1.1727610982724531e+79</ns0:v>
+        <ns0:v>1.6887759815123314e+79</ns0:v>
       </ns0:c>
       <ns0:c r="F83" s="1">
         <ns0:f>ROUND(F82*1.4,-5)</ns0:f>
-        <ns0:v>1.6897497744942575e+32</ns0:v>
+        <ns0:v>2.5346246617413865e+32</ns0:v>
       </ns0:c>
       <ns0:c r="G83" s="1" t="n">
         <ns0:v>16.8</ns0:v>
@@ -3578,15 +3578,15 @@
       </ns0:c>
       <ns0:c r="D84" s="1">
         <ns0:f>ROUND(D83*20,2-INT(LOG10(ABS(D83*20))))</ns0:f>
-        <ns0:v>2.35e+80</ns0:v>
+        <ns0:v>3.38e+80</ns0:v>
       </ns0:c>
       <ns0:c r="E84" s="1">
         <ns0:f>D84</ns0:f>
-        <ns0:v>2.35e+80</ns0:v>
+        <ns0:v>3.38e+80</ns0:v>
       </ns0:c>
       <ns0:c r="F84" s="1">
         <ns0:f>ROUND(F83*1.4,-5)</ns0:f>
-        <ns0:v>2.3656496842919603e+32</ns0:v>
+        <ns0:v>3.5484745264379406e+32</ns0:v>
       </ns0:c>
       <ns0:c r="G84" s="1" t="n">
         <ns0:v>17</ns0:v>
@@ -3610,15 +3610,15 @@
       </ns0:c>
       <ns0:c r="D85" s="1">
         <ns0:f>ROUND(D84*20,2-INT(LOG10(ABS(D84*20))))</ns0:f>
-        <ns0:v>4.7e+81</ns0:v>
+        <ns0:v>6.76e+81</ns0:v>
       </ns0:c>
       <ns0:c r="E85" s="1">
         <ns0:f>D85</ns0:f>
-        <ns0:v>4.7e+81</ns0:v>
+        <ns0:v>6.76e+81</ns0:v>
       </ns0:c>
       <ns0:c r="F85" s="1">
         <ns0:f>ROUND(F84*1.4,-5)</ns0:f>
-        <ns0:v>3.3119095580087444e+32</ns0:v>
+        <ns0:v>4.967864337013117e+32</ns0:v>
       </ns0:c>
       <ns0:c r="G85" s="1" t="n">
         <ns0:v>17.2</ns0:v>
@@ -3642,15 +3642,15 @@
       </ns0:c>
       <ns0:c r="D86" s="1">
         <ns0:f>ROUND(D85*20,2-INT(LOG10(ABS(D85*20))))</ns0:f>
-        <ns0:v>9.4e+82</ns0:v>
+        <ns0:v>1.35e+83</ns0:v>
       </ns0:c>
       <ns0:c r="E86" s="1">
         <ns0:f>D86</ns0:f>
-        <ns0:v>9.4e+82</ns0:v>
+        <ns0:v>1.35e+83</ns0:v>
       </ns0:c>
       <ns0:c r="F86" s="1">
         <ns0:f>ROUND(F85*1.4,-5)</ns0:f>
-        <ns0:v>4.636673381212242e+32</ns0:v>
+        <ns0:v>6.955010071818362e+32</ns0:v>
       </ns0:c>
       <ns0:c r="G86" s="1" t="n">
         <ns0:v>17.4</ns0:v>
@@ -3674,15 +3674,15 @@
       </ns0:c>
       <ns0:c r="D87" s="1">
         <ns0:f>ROUND(D86*20,2-INT(LOG10(ABS(D86*20))))</ns0:f>
-        <ns0:v>1.8800000000000002e+84</ns0:v>
+        <ns0:v>2.7e+84</ns0:v>
       </ns0:c>
       <ns0:c r="E87" s="1">
         <ns0:f>D87</ns0:f>
-        <ns0:v>1.8800000000000002e+84</ns0:v>
+        <ns0:v>2.7e+84</ns0:v>
       </ns0:c>
       <ns0:c r="F87" s="1">
         <ns0:f>ROUND(F86*1.4,-5)</ns0:f>
-        <ns0:v>6.491342733697137e+32</ns0:v>
+        <ns0:v>9.737014100545707e+32</ns0:v>
       </ns0:c>
       <ns0:c r="G87" s="1" t="n">
         <ns0:v>17.6</ns0:v>
@@ -3706,15 +3706,15 @@
       </ns0:c>
       <ns0:c r="D88" s="1">
         <ns0:f>ROUND(D87*20,2-INT(LOG10(ABS(D87*20))))</ns0:f>
-        <ns0:v>3.76e+85</ns0:v>
+        <ns0:v>5.4e+85</ns0:v>
       </ns0:c>
       <ns0:c r="E88" s="1">
         <ns0:f>D88</ns0:f>
-        <ns0:v>3.76e+85</ns0:v>
+        <ns0:v>5.4e+85</ns0:v>
       </ns0:c>
       <ns0:c r="F88" s="1">
         <ns0:f>ROUND(F87*1.4,-5)</ns0:f>
-        <ns0:v>9.087879827175992e+32</ns0:v>
+        <ns0:v>1.363181974076399e+33</ns0:v>
       </ns0:c>
       <ns0:c r="G88" s="1" t="n">
         <ns0:v>17.8</ns0:v>
@@ -3738,15 +3738,15 @@
       </ns0:c>
       <ns0:c r="D89" s="1">
         <ns0:f>ROUND(D88*20,2-INT(LOG10(ABS(D88*20))))</ns0:f>
-        <ns0:v>7.519999999999999e+86</ns0:v>
+        <ns0:v>1.08e+87</ns0:v>
       </ns0:c>
       <ns0:c r="E89" s="1">
         <ns0:f>D89</ns0:f>
-        <ns0:v>7.519999999999999e+86</ns0:v>
+        <ns0:v>1.08e+87</ns0:v>
       </ns0:c>
       <ns0:c r="F89" s="1">
         <ns0:f>ROUND(F88*1.4,-5)</ns0:f>
-        <ns0:v>1.2723031758046388e+33</ns0:v>
+        <ns0:v>1.9084547637069585e+33</ns0:v>
       </ns0:c>
       <ns0:c r="G89" s="1" t="n">
         <ns0:v>18</ns0:v>
@@ -3770,15 +3770,15 @@
       </ns0:c>
       <ns0:c r="D90" s="1">
         <ns0:f>ROUND(D89*20,2-INT(LOG10(ABS(D89*20))))</ns0:f>
-        <ns0:v>1.4999999999999999e+88</ns0:v>
+        <ns0:v>2.1599999999999997e+88</ns0:v>
       </ns0:c>
       <ns0:c r="E90" s="1">
         <ns0:f>D90</ns0:f>
-        <ns0:v>1.4999999999999999e+88</ns0:v>
+        <ns0:v>2.1599999999999997e+88</ns0:v>
       </ns0:c>
       <ns0:c r="F90" s="1">
         <ns0:f>ROUND(F89*1.4,-5)</ns0:f>
-        <ns0:v>1.7812244461264942e+33</ns0:v>
+        <ns0:v>2.6718366691897416e+33</ns0:v>
       </ns0:c>
       <ns0:c r="G90" s="1" t="n">
         <ns0:v>18.2</ns0:v>
@@ -3802,15 +3802,15 @@
       </ns0:c>
       <ns0:c r="D91" s="1">
         <ns0:f>ROUND(D90*20,2-INT(LOG10(ABS(D90*20))))</ns0:f>
-        <ns0:v>3e+89</ns0:v>
+        <ns0:v>4.3199999999999997e+89</ns0:v>
       </ns0:c>
       <ns0:c r="E91" s="1">
         <ns0:f>D91</ns0:f>
-        <ns0:v>3e+89</ns0:v>
+        <ns0:v>4.3199999999999997e+89</ns0:v>
       </ns0:c>
       <ns0:c r="F91" s="1">
         <ns0:f>ROUND(F90*1.4,-5)</ns0:f>
-        <ns0:v>2.4937142245770916e+33</ns0:v>
+        <ns0:v>3.740571336865638e+33</ns0:v>
       </ns0:c>
       <ns0:c r="G91" s="1" t="n">
         <ns0:v>18.4</ns0:v>
@@ -3834,15 +3834,15 @@
       </ns0:c>
       <ns0:c r="D92" s="1">
         <ns0:f>ROUND(D91*20,2-INT(LOG10(ABS(D91*20))))</ns0:f>
-        <ns0:v>6.0000000000000005e+90</ns0:v>
+        <ns0:v>8.64e+90</ns0:v>
       </ns0:c>
       <ns0:c r="E92" s="1">
         <ns0:f>D92</ns0:f>
-        <ns0:v>6.0000000000000005e+90</ns0:v>
+        <ns0:v>8.64e+90</ns0:v>
       </ns0:c>
       <ns0:c r="F92" s="1">
         <ns0:f>ROUND(F91*1.4,-5)</ns0:f>
-        <ns0:v>3.491199914407928e+33</ns0:v>
+        <ns0:v>5.236799871611893e+33</ns0:v>
       </ns0:c>
       <ns0:c r="G92" s="1" t="n">
         <ns0:v>18.6</ns0:v>
@@ -3866,15 +3866,15 @@
       </ns0:c>
       <ns0:c r="D93" s="1">
         <ns0:f>ROUND(D92*20,2-INT(LOG10(ABS(D92*20))))</ns0:f>
-        <ns0:v>1.2e+92</ns0:v>
+        <ns0:v>1.73e+92</ns0:v>
       </ns0:c>
       <ns0:c r="E93" s="1">
         <ns0:f>D93</ns0:f>
-        <ns0:v>1.2e+92</ns0:v>
+        <ns0:v>1.73e+92</ns0:v>
       </ns0:c>
       <ns0:c r="F93" s="1">
         <ns0:f>ROUND(F92*1.4,-5)</ns0:f>
-        <ns0:v>4.8876798801710985e+33</ns0:v>
+        <ns0:v>7.33151982025665e+33</ns0:v>
       </ns0:c>
       <ns0:c r="G93" s="1" t="n">
         <ns0:v>18.8</ns0:v>
@@ -3898,15 +3898,15 @@
       </ns0:c>
       <ns0:c r="D94" s="1">
         <ns0:f>ROUND(D93*20,2-INT(LOG10(ABS(D93*20))))</ns0:f>
-        <ns0:v>2.4e+93</ns0:v>
+        <ns0:v>3.4599999999999997e+93</ns0:v>
       </ns0:c>
       <ns0:c r="E94" s="1">
         <ns0:f>D94</ns0:f>
-        <ns0:v>2.4e+93</ns0:v>
+        <ns0:v>3.4599999999999997e+93</ns0:v>
       </ns0:c>
       <ns0:c r="F94" s="1">
         <ns0:f>ROUND(F93*1.4,-5)</ns0:f>
-        <ns0:v>6.842751832239537e+33</ns0:v>
+        <ns0:v>1.026412774835931e+34</ns0:v>
       </ns0:c>
       <ns0:c r="G94" s="1" t="n">
         <ns0:v>19</ns0:v>
@@ -3930,15 +3930,15 @@
       </ns0:c>
       <ns0:c r="D95" s="1">
         <ns0:f>ROUND(D94*20,2-INT(LOG10(ABS(D94*20))))</ns0:f>
-        <ns0:v>4.8000000000000004e+94</ns0:v>
+        <ns0:v>6.92e+94</ns0:v>
       </ns0:c>
       <ns0:c r="E95" s="1">
         <ns0:f>D95</ns0:f>
-        <ns0:v>4.8000000000000004e+94</ns0:v>
+        <ns0:v>6.92e+94</ns0:v>
       </ns0:c>
       <ns0:c r="F95" s="1">
         <ns0:f>ROUND(F94*1.4,-5)</ns0:f>
-        <ns0:v>9.579852565135353e+33</ns0:v>
+        <ns0:v>1.4369778847703034e+34</ns0:v>
       </ns0:c>
       <ns0:c r="G95" s="1" t="n">
         <ns0:v>19.2</ns0:v>
@@ -3962,15 +3962,15 @@
       </ns0:c>
       <ns0:c r="D96" s="1">
         <ns0:f>ROUND(D95*20,2-INT(LOG10(ABS(D95*20))))</ns0:f>
-        <ns0:v>9.600000000000001e+95</ns0:v>
+        <ns0:v>1.38e+96</ns0:v>
       </ns0:c>
       <ns0:c r="E96" s="1">
         <ns0:f>D96</ns0:f>
-        <ns0:v>9.600000000000001e+95</ns0:v>
+        <ns0:v>1.38e+96</ns0:v>
       </ns0:c>
       <ns0:c r="F96" s="1">
         <ns0:f>ROUND(F95*1.4,-5)</ns0:f>
-        <ns0:v>1.3411793591189494e+34</ns0:v>
+        <ns0:v>2.0117690386784246e+34</ns0:v>
       </ns0:c>
       <ns0:c r="G96" s="1" t="n">
         <ns0:v>19.4</ns0:v>
@@ -3994,15 +3994,15 @@
       </ns0:c>
       <ns0:c r="D97" s="1">
         <ns0:f>ROUND(D96*20,2-INT(LOG10(ABS(D96*20))))</ns0:f>
-        <ns0:v>1.92e+97</ns0:v>
+        <ns0:v>2.76e+97</ns0:v>
       </ns0:c>
       <ns0:c r="E97" s="1">
         <ns0:f>D97</ns0:f>
-        <ns0:v>1.92e+97</ns0:v>
+        <ns0:v>2.76e+97</ns0:v>
       </ns0:c>
       <ns0:c r="F97" s="1">
         <ns0:f>ROUND(F96*1.4,-5)</ns0:f>
-        <ns0:v>1.877651102766529e+34</ns0:v>
+        <ns0:v>2.816476654149794e+34</ns0:v>
       </ns0:c>
       <ns0:c r="G97" s="1" t="n">
         <ns0:v>19.6</ns0:v>
@@ -4026,15 +4026,15 @@
       </ns0:c>
       <ns0:c r="D98" s="1">
         <ns0:f>ROUND(D97*20,2-INT(LOG10(ABS(D97*20))))</ns0:f>
-        <ns0:v>3.8400000000000006e+98</ns0:v>
+        <ns0:v>5.520000000000001e+98</ns0:v>
       </ns0:c>
       <ns0:c r="E98" s="1">
         <ns0:f>D98</ns0:f>
-        <ns0:v>3.8400000000000006e+98</ns0:v>
+        <ns0:v>5.520000000000001e+98</ns0:v>
       </ns0:c>
       <ns0:c r="F98" s="1">
         <ns0:f>ROUND(F97*1.4,-5)</ns0:f>
-        <ns0:v>2.6287115438731407e+34</ns0:v>
+        <ns0:v>3.943067315809711e+34</ns0:v>
       </ns0:c>
       <ns0:c r="G98" s="1" t="n">
         <ns0:v>19.8</ns0:v>
@@ -4058,15 +4058,15 @@
       </ns0:c>
       <ns0:c r="D99" s="1">
         <ns0:f>ROUND(D98*20,2-INT(LOG10(ABS(D98*20))))</ns0:f>
-        <ns0:v>7.68e+99</ns0:v>
+        <ns0:v>1.1e+100</ns0:v>
       </ns0:c>
       <ns0:c r="E99" s="1">
         <ns0:f>D99</ns0:f>
-        <ns0:v>7.68e+99</ns0:v>
+        <ns0:v>1.1e+100</ns0:v>
       </ns0:c>
       <ns0:c r="F99" s="1">
         <ns0:f>ROUND(F98*1.4,-5)</ns0:f>
-        <ns0:v>3.6801961614223965e+34</ns0:v>
+        <ns0:v>5.520294242133595e+34</ns0:v>
       </ns0:c>
       <ns0:c r="G99" s="1" t="n">
         <ns0:v>20</ns0:v>
@@ -4090,15 +4090,15 @@
       </ns0:c>
       <ns0:c r="D100" s="1">
         <ns0:f>ROUND(D99*20,2-INT(LOG10(ABS(D99*20))))</ns0:f>
-        <ns0:v>1.54e+101</ns0:v>
+        <ns0:v>2.2e+101</ns0:v>
       </ns0:c>
       <ns0:c r="E100" s="1">
         <ns0:f>D100</ns0:f>
-        <ns0:v>1.54e+101</ns0:v>
+        <ns0:v>2.2e+101</ns0:v>
       </ns0:c>
       <ns0:c r="F100" s="1">
         <ns0:f>ROUND(F99*1.4,-5)</ns0:f>
-        <ns0:v>5.152274625991355e+34</ns0:v>
+        <ns0:v>7.728411938987032e+34</ns0:v>
       </ns0:c>
       <ns0:c r="G100" s="1" t="n">
         <ns0:v>20.2</ns0:v>
@@ -4122,15 +4122,15 @@
       </ns0:c>
       <ns0:c r="D101" s="1">
         <ns0:f>ROUND(D100*20,2-INT(LOG10(ABS(D100*20))))</ns0:f>
-        <ns0:v>3.08e+102</ns0:v>
+        <ns0:v>4.4e+102</ns0:v>
       </ns0:c>
       <ns0:c r="E101" s="1">
         <ns0:f>D101</ns0:f>
-        <ns0:v>3.08e+102</ns0:v>
+        <ns0:v>4.4e+102</ns0:v>
       </ns0:c>
       <ns0:c r="F101" s="1">
         <ns0:f>ROUND(F100*1.4,-5)</ns0:f>
-        <ns0:v>7.213184476387896e+34</ns0:v>
+        <ns0:v>1.0819776714581845e+35</ns0:v>
       </ns0:c>
       <ns0:c r="G101" s="1" t="n">
         <ns0:v>20.4</ns0:v>
@@ -4154,15 +4154,15 @@
       </ns0:c>
       <ns0:c r="D102" s="1">
         <ns0:f>ROUND(D101*20,2-INT(LOG10(ABS(D101*20))))</ns0:f>
-        <ns0:v>6.159999999999999e+103</ns0:v>
+        <ns0:v>8.8e+103</ns0:v>
       </ns0:c>
       <ns0:c r="E102" s="1">
         <ns0:f>D102</ns0:f>
-        <ns0:v>6.159999999999999e+103</ns0:v>
+        <ns0:v>8.8e+103</ns0:v>
       </ns0:c>
       <ns0:c r="F102" s="1">
         <ns0:f>ROUND(F101*1.4,-5)</ns0:f>
-        <ns0:v>1.0098458266943055e+35</ns0:v>
+        <ns0:v>1.5147687400414581e+35</ns0:v>
       </ns0:c>
       <ns0:c r="G102" s="1" t="n">
         <ns0:v>20.6</ns0:v>
@@ -4186,15 +4186,15 @@
       </ns0:c>
       <ns0:c r="D103" s="1">
         <ns0:f>ROUND(D102*20,2-INT(LOG10(ABS(D102*20))))</ns0:f>
-        <ns0:v>1.23e+105</ns0:v>
+        <ns0:v>1.76e+105</ns0:v>
       </ns0:c>
       <ns0:c r="E103" s="1">
         <ns0:f>D103</ns0:f>
-        <ns0:v>1.23e+105</ns0:v>
+        <ns0:v>1.76e+105</ns0:v>
       </ns0:c>
       <ns0:c r="F103" s="1">
         <ns0:f>ROUND(F102*1.4,-5)</ns0:f>
-        <ns0:v>1.4137841573720276e+35</ns0:v>
+        <ns0:v>2.1206762360580413e+35</ns0:v>
       </ns0:c>
       <ns0:c r="G103" s="1" t="n">
         <ns0:v>20.8</ns0:v>
@@ -4218,15 +4218,15 @@
       </ns0:c>
       <ns0:c r="D104" s="1">
         <ns0:f>ROUND(D103*20,2-INT(LOG10(ABS(D103*20))))</ns0:f>
-        <ns0:v>2.46e+106</ns0:v>
+        <ns0:v>3.52e+106</ns0:v>
       </ns0:c>
       <ns0:c r="E104" s="1">
         <ns0:f>D104</ns0:f>
-        <ns0:v>2.46e+106</ns0:v>
+        <ns0:v>3.52e+106</ns0:v>
       </ns0:c>
       <ns0:c r="F104" s="1">
         <ns0:f>ROUND(F103*1.4,-5)</ns0:f>
-        <ns0:v>1.9792978203208386e+35</ns0:v>
+        <ns0:v>2.9689467304812575e+35</ns0:v>
       </ns0:c>
       <ns0:c r="G104" s="1" t="n">
         <ns0:v>21</ns0:v>
@@ -4250,15 +4250,15 @@
       </ns0:c>
       <ns0:c r="D105" s="1">
         <ns0:f>ROUND(D104*20,2-INT(LOG10(ABS(D104*20))))</ns0:f>
-        <ns0:v>4.92e+107</ns0:v>
+        <ns0:v>7.04e+107</ns0:v>
       </ns0:c>
       <ns0:c r="E105" s="1">
         <ns0:f>D105</ns0:f>
-        <ns0:v>4.92e+107</ns0:v>
+        <ns0:v>7.04e+107</ns0:v>
       </ns0:c>
       <ns0:c r="F105" s="1">
         <ns0:f>ROUND(F104*1.4,-5)</ns0:f>
-        <ns0:v>2.7710169484491734e+35</ns0:v>
+        <ns0:v>4.1565254226737606e+35</ns0:v>
       </ns0:c>
       <ns0:c r="G105" s="1" t="n">
         <ns0:v>21.2</ns0:v>
@@ -4282,15 +4282,15 @@
       </ns0:c>
       <ns0:c r="D106" s="1">
         <ns0:f>ROUND(D105*20,2-INT(LOG10(ABS(D105*20))))</ns0:f>
-        <ns0:v>9.84e+108</ns0:v>
+        <ns0:v>1.41e+109</ns0:v>
       </ns0:c>
       <ns0:c r="E106" s="1">
         <ns0:f>D106</ns0:f>
-        <ns0:v>9.84e+108</ns0:v>
+        <ns0:v>1.41e+109</ns0:v>
       </ns0:c>
       <ns0:c r="F106" s="1">
         <ns0:f>ROUND(F105*1.4,-5)</ns0:f>
-        <ns0:v>3.879423727828843e+35</ns0:v>
+        <ns0:v>5.8191355917432645e+35</ns0:v>
       </ns0:c>
       <ns0:c r="G106" s="1" t="n">
         <ns0:v>21.4</ns0:v>
@@ -4314,15 +4314,15 @@
       </ns0:c>
       <ns0:c r="D107" s="1">
         <ns0:f>ROUND(D106*20,2-INT(LOG10(ABS(D106*20))))</ns0:f>
-        <ns0:v>1.9699999999999998e+110</ns0:v>
+        <ns0:v>2.8199999999999998e+110</ns0:v>
       </ns0:c>
       <ns0:c r="E107" s="1">
         <ns0:f>D107</ns0:f>
-        <ns0:v>1.9699999999999998e+110</ns0:v>
+        <ns0:v>2.8199999999999998e+110</ns0:v>
       </ns0:c>
       <ns0:c r="F107" s="1">
         <ns0:f>ROUND(F106*1.4,-5)</ns0:f>
-        <ns0:v>5.431193218960379e+35</ns0:v>
+        <ns0:v>8.14678982844057e+35</ns0:v>
       </ns0:c>
       <ns0:c r="G107" s="1" t="n">
         <ns0:v>21.6</ns0:v>
@@ -4346,15 +4346,15 @@
       </ns0:c>
       <ns0:c r="D108" s="1">
         <ns0:f>ROUND(D107*20,2-INT(LOG10(ABS(D107*20))))</ns0:f>
-        <ns0:v>3.94e+111</ns0:v>
+        <ns0:v>5.64e+111</ns0:v>
       </ns0:c>
       <ns0:c r="E108" s="1">
         <ns0:f>D108</ns0:f>
-        <ns0:v>3.94e+111</ns0:v>
+        <ns0:v>5.64e+111</ns0:v>
       </ns0:c>
       <ns0:c r="F108" s="1">
         <ns0:f>ROUND(F107*1.4,-5)</ns0:f>
-        <ns0:v>7.60367050654453e+35</ns0:v>
+        <ns0:v>1.1405505759816794e+36</ns0:v>
       </ns0:c>
       <ns0:c r="G108" s="1" t="n">
         <ns0:v>21.8</ns0:v>
@@ -4378,15 +4378,15 @@
       </ns0:c>
       <ns0:c r="D109" s="1">
         <ns0:f>ROUND(D108*20,2-INT(LOG10(ABS(D108*20))))</ns0:f>
-        <ns0:v>7.88e+112</ns0:v>
+        <ns0:v>1.13e+113</ns0:v>
       </ns0:c>
       <ns0:c r="E109" s="1">
         <ns0:f>D109</ns0:f>
-        <ns0:v>7.88e+112</ns0:v>
+        <ns0:v>1.13e+113</ns0:v>
       </ns0:c>
       <ns0:c r="F109" s="1">
         <ns0:f>ROUND(F108*1.4,-5)</ns0:f>
-        <ns0:v>1.0645138709162343e+36</ns0:v>
+        <ns0:v>1.596770806374351e+36</ns0:v>
       </ns0:c>
       <ns0:c r="G109" s="1" t="n">
         <ns0:v>22</ns0:v>
@@ -4410,15 +4410,15 @@
       </ns0:c>
       <ns0:c r="D110" s="1">
         <ns0:f>ROUND(D109*20,2-INT(LOG10(ABS(D109*20))))</ns0:f>
-        <ns0:v>1.5800000000000002e+114</ns0:v>
+        <ns0:v>2.26e+114</ns0:v>
       </ns0:c>
       <ns0:c r="E110" s="1">
         <ns0:f>D110</ns0:f>
-        <ns0:v>1.5800000000000002e+114</ns0:v>
+        <ns0:v>2.26e+114</ns0:v>
       </ns0:c>
       <ns0:c r="F110" s="1">
         <ns0:f>ROUND(F109*1.4,-5)</ns0:f>
-        <ns0:v>1.4903194192827278e+36</ns0:v>
+        <ns0:v>2.2354791289240912e+36</ns0:v>
       </ns0:c>
       <ns0:c r="G110" s="1" t="n">
         <ns0:v>22.2</ns0:v>
@@ -4442,15 +4442,15 @@
       </ns0:c>
       <ns0:c r="D111" s="1">
         <ns0:f>ROUND(D110*20,2-INT(LOG10(ABS(D110*20))))</ns0:f>
-        <ns0:v>3.16e+115</ns0:v>
+        <ns0:v>4.52e+115</ns0:v>
       </ns0:c>
       <ns0:c r="E111" s="1">
         <ns0:f>D111</ns0:f>
-        <ns0:v>3.16e+115</ns0:v>
+        <ns0:v>4.52e+115</ns0:v>
       </ns0:c>
       <ns0:c r="F111" s="1">
         <ns0:f>ROUND(F110*1.4,-5)</ns0:f>
-        <ns0:v>2.0864471869958192e+36</ns0:v>
+        <ns0:v>3.1296707804937275e+36</ns0:v>
       </ns0:c>
       <ns0:c r="G111" s="1" t="n">
         <ns0:v>22.4</ns0:v>
@@ -4474,15 +4474,15 @@
       </ns0:c>
       <ns0:c r="D112" s="1">
         <ns0:f>ROUND(D111*20,2-INT(LOG10(ABS(D111*20))))</ns0:f>
-        <ns0:v>6.32e+116</ns0:v>
+        <ns0:v>9.039999999999999e+116</ns0:v>
       </ns0:c>
       <ns0:c r="E112" s="1">
         <ns0:f>D112</ns0:f>
-        <ns0:v>6.32e+116</ns0:v>
+        <ns0:v>9.039999999999999e+116</ns0:v>
       </ns0:c>
       <ns0:c r="F112" s="1">
         <ns0:f>ROUND(F111*1.4,-5)</ns0:f>
-        <ns0:v>2.9210260617941466e+36</ns0:v>
+        <ns0:v>4.3815390926912187e+36</ns0:v>
       </ns0:c>
       <ns0:c r="G112" s="1" t="n">
         <ns0:v>22.6</ns0:v>
@@ -4506,15 +4506,15 @@
       </ns0:c>
       <ns0:c r="D113" s="1">
         <ns0:f>ROUND(D112*20,2-INT(LOG10(ABS(D112*20))))</ns0:f>
-        <ns0:v>1.26e+118</ns0:v>
+        <ns0:v>1.81e+118</ns0:v>
       </ns0:c>
       <ns0:c r="E113" s="1">
         <ns0:f>D113</ns0:f>
-        <ns0:v>1.26e+118</ns0:v>
+        <ns0:v>1.81e+118</ns0:v>
       </ns0:c>
       <ns0:c r="F113" s="1">
         <ns0:f>ROUND(F112*1.4,-5)</ns0:f>
-        <ns0:v>4.0894364865118056e+36</ns0:v>
+        <ns0:v>6.134154729767706e+36</ns0:v>
       </ns0:c>
       <ns0:c r="G113" s="1" t="n">
         <ns0:v>22.8</ns0:v>
@@ -4538,15 +4538,15 @@
       </ns0:c>
       <ns0:c r="D114" s="1">
         <ns0:f>ROUND(D113*20,2-INT(LOG10(ABS(D113*20))))</ns0:f>
-        <ns0:v>2.52e+119</ns0:v>
+        <ns0:v>3.62e+119</ns0:v>
       </ns0:c>
       <ns0:c r="E114" s="1">
         <ns0:f>D114</ns0:f>
-        <ns0:v>2.52e+119</ns0:v>
+        <ns0:v>3.62e+119</ns0:v>
       </ns0:c>
       <ns0:c r="F114" s="1">
         <ns0:f>ROUND(F113*1.4,-5)</ns0:f>
-        <ns0:v>5.725211081116527e+36</ns0:v>
+        <ns0:v>8.587816621674789e+36</ns0:v>
       </ns0:c>
       <ns0:c r="G114" s="1" t="n">
         <ns0:v>23</ns0:v>
@@ -4570,15 +4570,15 @@
       </ns0:c>
       <ns0:c r="D115" s="1">
         <ns0:f>ROUND(D114*20,2-INT(LOG10(ABS(D114*20))))</ns0:f>
-        <ns0:v>5.04e+120</ns0:v>
+        <ns0:v>7.240000000000001e+120</ns0:v>
       </ns0:c>
       <ns0:c r="E115" s="1">
         <ns0:f>D115</ns0:f>
-        <ns0:v>5.04e+120</ns0:v>
+        <ns0:v>7.240000000000001e+120</ns0:v>
       </ns0:c>
       <ns0:c r="F115" s="1">
         <ns0:f>ROUND(F114*1.4,-5)</ns0:f>
-        <ns0:v>8.015295513563137e+36</ns0:v>
+        <ns0:v>1.2022943270344703e+37</ns0:v>
       </ns0:c>
       <ns0:c r="G115" s="1" t="n">
         <ns0:v>23.2</ns0:v>
@@ -4602,15 +4602,15 @@
       </ns0:c>
       <ns0:c r="D116" s="1">
         <ns0:f>ROUND(D115*20,2-INT(LOG10(ABS(D115*20))))</ns0:f>
-        <ns0:v>1.01e+122</ns0:v>
+        <ns0:v>1.45e+122</ns0:v>
       </ns0:c>
       <ns0:c r="E116" s="1">
         <ns0:f>D116</ns0:f>
-        <ns0:v>1.01e+122</ns0:v>
+        <ns0:v>1.45e+122</ns0:v>
       </ns0:c>
       <ns0:c r="F116" s="1">
         <ns0:f>ROUND(F115*1.4,-5)</ns0:f>
-        <ns0:v>1.122141371898839e+37</ns0:v>
+        <ns0:v>1.6832120578482584e+37</ns0:v>
       </ns0:c>
       <ns0:c r="G116" s="1" t="n">
         <ns0:v>23.4</ns0:v>
@@ -4634,15 +4634,15 @@
       </ns0:c>
       <ns0:c r="D117" s="1">
         <ns0:f>ROUND(D116*20,2-INT(LOG10(ABS(D116*20))))</ns0:f>
-        <ns0:v>2.02e+123</ns0:v>
+        <ns0:v>2.9e+123</ns0:v>
       </ns0:c>
       <ns0:c r="E117" s="1">
         <ns0:f>D117</ns0:f>
-        <ns0:v>2.02e+123</ns0:v>
+        <ns0:v>2.9e+123</ns0:v>
       </ns0:c>
       <ns0:c r="F117" s="1">
         <ns0:f>ROUND(F116*1.4,-5)</ns0:f>
-        <ns0:v>1.5709979206583747e+37</ns0:v>
+        <ns0:v>2.3564968809875614e+37</ns0:v>
       </ns0:c>
       <ns0:c r="G117" s="1" t="n">
         <ns0:v>23.6</ns0:v>
@@ -4666,15 +4666,15 @@
       </ns0:c>
       <ns0:c r="D118" s="1">
         <ns0:f>ROUND(D117*20,2-INT(LOG10(ABS(D117*20))))</ns0:f>
-        <ns0:v>4.04e+124</ns0:v>
+        <ns0:v>5.7999999999999995e+124</ns0:v>
       </ns0:c>
       <ns0:c r="E118" s="1">
         <ns0:f>D118</ns0:f>
-        <ns0:v>4.04e+124</ns0:v>
+        <ns0:v>5.7999999999999995e+124</ns0:v>
       </ns0:c>
       <ns0:c r="F118" s="1">
         <ns0:f>ROUND(F117*1.4,-5)</ns0:f>
-        <ns0:v>2.1993970889217245e+37</ns0:v>
+        <ns0:v>3.2990956333825863e+37</ns0:v>
       </ns0:c>
       <ns0:c r="G118" s="1" t="n">
         <ns0:v>23.8</ns0:v>
@@ -4698,15 +4698,15 @@
       </ns0:c>
       <ns0:c r="D119" s="1">
         <ns0:f>ROUND(D118*20,2-INT(LOG10(ABS(D118*20))))</ns0:f>
-        <ns0:v>8.08e+125</ns0:v>
+        <ns0:v>1.1600000000000001e+126</ns0:v>
       </ns0:c>
       <ns0:c r="E119" s="1">
         <ns0:f>D119</ns0:f>
-        <ns0:v>8.08e+125</ns0:v>
+        <ns0:v>1.1600000000000001e+126</ns0:v>
       </ns0:c>
       <ns0:c r="F119" s="1">
         <ns0:f>ROUND(F118*1.4,-5)</ns0:f>
-        <ns0:v>3.079155924490414e+37</ns0:v>
+        <ns0:v>4.61873388673562e+37</ns0:v>
       </ns0:c>
       <ns0:c r="G119" s="1" t="n">
         <ns0:v>24</ns0:v>
@@ -4730,15 +4730,15 @@
       </ns0:c>
       <ns0:c r="D120" s="1">
         <ns0:f>ROUND(D119*20,2-INT(LOG10(ABS(D119*20))))</ns0:f>
-        <ns0:v>1.62e+127</ns0:v>
+        <ns0:v>2.32e+127</ns0:v>
       </ns0:c>
       <ns0:c r="E120" s="1">
         <ns0:f>D120</ns0:f>
-        <ns0:v>1.62e+127</ns0:v>
+        <ns0:v>2.32e+127</ns0:v>
       </ns0:c>
       <ns0:c r="F120" s="1">
         <ns0:f>ROUND(F119*1.4,-5)</ns0:f>
-        <ns0:v>4.310818294286579e+37</ns0:v>
+        <ns0:v>6.466227441429868e+37</ns0:v>
       </ns0:c>
       <ns0:c r="G120" s="1" t="n">
         <ns0:v>24.2000000000001</ns0:v>
@@ -4762,15 +4762,15 @@
       </ns0:c>
       <ns0:c r="D121" s="1">
         <ns0:f>ROUND(D120*20,2-INT(LOG10(ABS(D120*20))))</ns0:f>
-        <ns0:v>3.2400000000000002e+128</ns0:v>
+        <ns0:v>4.64e+128</ns0:v>
       </ns0:c>
       <ns0:c r="E121" s="1">
         <ns0:f>D121</ns0:f>
-        <ns0:v>3.2400000000000002e+128</ns0:v>
+        <ns0:v>4.64e+128</ns0:v>
       </ns0:c>
       <ns0:c r="F121" s="1">
         <ns0:f>ROUND(F120*1.4,-5)</ns0:f>
-        <ns0:v>6.03514561200121e+37</ns0:v>
+        <ns0:v>9.052718418001815e+37</ns0:v>
       </ns0:c>
       <ns0:c r="G121" s="1" t="n">
         <ns0:v>24.4000000000001</ns0:v>
@@ -4794,15 +4794,15 @@
       </ns0:c>
       <ns0:c r="D122" s="1">
         <ns0:f>ROUND(D121*20,2-INT(LOG10(ABS(D121*20))))</ns0:f>
-        <ns0:v>6.48e+129</ns0:v>
+        <ns0:v>9.28e+129</ns0:v>
       </ns0:c>
       <ns0:c r="E122" s="1">
         <ns0:f>D122</ns0:f>
-        <ns0:v>6.48e+129</ns0:v>
+        <ns0:v>9.28e+129</ns0:v>
       </ns0:c>
       <ns0:c r="F122" s="1">
         <ns0:f>ROUND(F121*1.4,-5)</ns0:f>
-        <ns0:v>8.449203856801694e+37</ns0:v>
+        <ns0:v>1.2673805785202541e+38</ns0:v>
       </ns0:c>
       <ns0:c r="G122" s="1" t="n">
         <ns0:v>24.6000000000001</ns0:v>
@@ -4826,15 +4826,15 @@
       </ns0:c>
       <ns0:c r="D123" s="1">
         <ns0:f>ROUND(D122*20,2-INT(LOG10(ABS(D122*20))))</ns0:f>
-        <ns0:v>1.3e+131</ns0:v>
+        <ns0:v>1.86e+131</ns0:v>
       </ns0:c>
       <ns0:c r="E123" s="1">
         <ns0:f>D123</ns0:f>
-        <ns0:v>1.3e+131</ns0:v>
+        <ns0:v>1.86e+131</ns0:v>
       </ns0:c>
       <ns0:c r="F123" s="1">
         <ns0:f>ROUND(F122*1.4,-5)</ns0:f>
-        <ns0:v>1.182888539952237e+38</ns0:v>
+        <ns0:v>1.774332809928356e+38</ns0:v>
       </ns0:c>
       <ns0:c r="G123" s="1" t="n">
         <ns0:v>24.8000000000001</ns0:v>
@@ -4858,15 +4858,15 @@
       </ns0:c>
       <ns0:c r="D124" s="1">
         <ns0:f>ROUND(D123*20,2-INT(LOG10(ABS(D123*20))))</ns0:f>
-        <ns0:v>2.5999999999999997e+132</ns0:v>
+        <ns0:v>3.72e+132</ns0:v>
       </ns0:c>
       <ns0:c r="E124" s="1">
         <ns0:f>D124</ns0:f>
-        <ns0:v>2.5999999999999997e+132</ns0:v>
+        <ns0:v>3.72e+132</ns0:v>
       </ns0:c>
       <ns0:c r="F124" s="1">
         <ns0:f>ROUND(F123*1.4,-5)</ns0:f>
-        <ns0:v>1.6560439559331319e+38</ns0:v>
+        <ns0:v>2.484065933899698e+38</ns0:v>
       </ns0:c>
       <ns0:c r="G124" s="1" t="n">
         <ns0:v>25.0000000000001</ns0:v>
@@ -4890,15 +4890,15 @@
       </ns0:c>
       <ns0:c r="D125" s="1">
         <ns0:f>ROUND(D124*20,2-INT(LOG10(ABS(D124*20))))</ns0:f>
-        <ns0:v>5.200000000000001e+133</ns0:v>
+        <ns0:v>7.44e+133</ns0:v>
       </ns0:c>
       <ns0:c r="E125" s="1">
         <ns0:f>D125</ns0:f>
-        <ns0:v>5.200000000000001e+133</ns0:v>
+        <ns0:v>7.44e+133</ns0:v>
       </ns0:c>
       <ns0:c r="F125" s="1">
         <ns0:f>ROUND(F124*1.4,-5)</ns0:f>
-        <ns0:v>2.3184615383063845e+38</ns0:v>
+        <ns0:v>3.477692307459577e+38</ns0:v>
       </ns0:c>
       <ns0:c r="G125" s="1" t="n">
         <ns0:v>25.2000000000001</ns0:v>
@@ -4922,15 +4922,15 @@
       </ns0:c>
       <ns0:c r="D126" s="1">
         <ns0:f>ROUND(D125*20,2-INT(LOG10(ABS(D125*20))))</ns0:f>
-        <ns0:v>1.0399999999999999e+135</ns0:v>
+        <ns0:v>1.49e+135</ns0:v>
       </ns0:c>
       <ns0:c r="E126" s="1">
         <ns0:f>D126</ns0:f>
-        <ns0:v>1.0399999999999999e+135</ns0:v>
+        <ns0:v>1.49e+135</ns0:v>
       </ns0:c>
       <ns0:c r="F126" s="1">
         <ns0:f>ROUND(F125*1.4,-5)</ns0:f>
-        <ns0:v>3.245846153628938e+38</ns0:v>
+        <ns0:v>4.868769230443407e+38</ns0:v>
       </ns0:c>
       <ns0:c r="G126" s="1" t="n">
         <ns0:v>25.4000000000001</ns0:v>
@@ -4954,15 +4954,15 @@
       </ns0:c>
       <ns0:c r="D127" s="1">
         <ns0:f>ROUND(D126*20,2-INT(LOG10(ABS(D126*20))))</ns0:f>
-        <ns0:v>2.08e+136</ns0:v>
+        <ns0:v>2.98e+136</ns0:v>
       </ns0:c>
       <ns0:c r="E127" s="1">
         <ns0:f>D127</ns0:f>
-        <ns0:v>2.08e+136</ns0:v>
+        <ns0:v>2.98e+136</ns0:v>
       </ns0:c>
       <ns0:c r="F127" s="1">
         <ns0:f>ROUND(F126*1.4,-5)</ns0:f>
-        <ns0:v>4.544184615080513e+38</ns0:v>
+        <ns0:v>6.81627692262077e+38</ns0:v>
       </ns0:c>
       <ns0:c r="G127" s="1" t="n">
         <ns0:v>25.6000000000001</ns0:v>
@@ -4986,15 +4986,15 @@
       </ns0:c>
       <ns0:c r="D128" s="1">
         <ns0:f>ROUND(D127*20,2-INT(LOG10(ABS(D127*20))))</ns0:f>
-        <ns0:v>4.16e+137</ns0:v>
+        <ns0:v>5.96e+137</ns0:v>
       </ns0:c>
       <ns0:c r="E128" s="1">
         <ns0:f>D128</ns0:f>
-        <ns0:v>4.16e+137</ns0:v>
+        <ns0:v>5.96e+137</ns0:v>
       </ns0:c>
       <ns0:c r="F128" s="1">
         <ns0:f>ROUND(F127*1.4,-5)</ns0:f>
-        <ns0:v>6.361858461112718e+38</ns0:v>
+        <ns0:v>9.542787691669077e+38</ns0:v>
       </ns0:c>
       <ns0:c r="G128" s="1" t="n">
         <ns0:v>25.8000000000001</ns0:v>
@@ -5018,15 +5018,15 @@
       </ns0:c>
       <ns0:c r="D129" s="1">
         <ns0:f>ROUND(D128*20,2-INT(LOG10(ABS(D128*20))))</ns0:f>
-        <ns0:v>8.32e+138</ns0:v>
+        <ns0:v>1.19e+139</ns0:v>
       </ns0:c>
       <ns0:c r="E129" s="1">
         <ns0:f>D129</ns0:f>
-        <ns0:v>8.32e+138</ns0:v>
+        <ns0:v>1.19e+139</ns0:v>
       </ns0:c>
       <ns0:c r="F129" s="1">
         <ns0:f>ROUND(F128*1.4,-5)</ns0:f>
-        <ns0:v>8.906601845557804e+38</ns0:v>
+        <ns0:v>1.3359902768336709e+39</ns0:v>
       </ns0:c>
       <ns0:c r="G129" s="1" t="n">
         <ns0:v>26.0000000000001</ns0:v>
@@ -5050,15 +5050,15 @@
       </ns0:c>
       <ns0:c r="D130" s="1">
         <ns0:f>ROUND(D129*20,2-INT(LOG10(ABS(D129*20))))</ns0:f>
-        <ns0:v>1.6599999999999999e+140</ns0:v>
+        <ns0:v>2.38e+140</ns0:v>
       </ns0:c>
       <ns0:c r="E130" s="1">
         <ns0:f>D130</ns0:f>
-        <ns0:v>1.6599999999999999e+140</ns0:v>
+        <ns0:v>2.38e+140</ns0:v>
       </ns0:c>
       <ns0:c r="F130" s="1">
         <ns0:f>ROUND(F129*1.4,-5)</ns0:f>
-        <ns0:v>1.2469242583780926e+39</ns0:v>
+        <ns0:v>1.870386387567139e+39</ns0:v>
       </ns0:c>
       <ns0:c r="G130" s="1" t="n">
         <ns0:v>26.2000000000001</ns0:v>
@@ -5082,15 +5082,15 @@
       </ns0:c>
       <ns0:c r="D131" s="1">
         <ns0:f>ROUND(D130*20,2-INT(LOG10(ABS(D130*20))))</ns0:f>
-        <ns0:v>3.32e+141</ns0:v>
+        <ns0:v>4.76e+141</ns0:v>
       </ns0:c>
       <ns0:c r="E131" s="1">
         <ns0:f>D131</ns0:f>
-        <ns0:v>3.32e+141</ns0:v>
+        <ns0:v>4.76e+141</ns0:v>
       </ns0:c>
       <ns0:c r="F131" s="1">
         <ns0:f>ROUND(F130*1.4,-5)</ns0:f>
-        <ns0:v>1.7456939617293296e+39</ns0:v>
+        <ns0:v>2.618540942593995e+39</ns0:v>
       </ns0:c>
       <ns0:c r="G131" s="1" t="n">
         <ns0:v>26.4000000000001</ns0:v>
@@ -5114,15 +5114,15 @@
       </ns0:c>
       <ns0:c r="D132" s="1">
         <ns0:f>ROUND(D131*20,2-INT(LOG10(ABS(D131*20))))</ns0:f>
-        <ns0:v>6.64e+142</ns0:v>
+        <ns0:v>9.520000000000001e+142</ns0:v>
       </ns0:c>
       <ns0:c r="E132" s="1">
         <ns0:f>D132</ns0:f>
-        <ns0:v>6.64e+142</ns0:v>
+        <ns0:v>9.520000000000001e+142</ns0:v>
       </ns0:c>
       <ns0:c r="F132" s="1">
         <ns0:f>ROUND(F131*1.4,-5)</ns0:f>
-        <ns0:v>2.443971546421061e+39</ns0:v>
+        <ns0:v>3.665957319631593e+39</ns0:v>
       </ns0:c>
       <ns0:c r="G132" s="1" t="n">
         <ns0:v>26.6000000000001</ns0:v>
@@ -5146,15 +5146,15 @@
       </ns0:c>
       <ns0:c r="D133" s="1">
         <ns0:f>ROUND(D132*20,2-INT(LOG10(ABS(D132*20))))</ns0:f>
-        <ns0:v>1.33e+144</ns0:v>
+        <ns0:v>1.8999999999999998e+144</ns0:v>
       </ns0:c>
       <ns0:c r="E133" s="1">
         <ns0:f>D133</ns0:f>
-        <ns0:v>1.33e+144</ns0:v>
+        <ns0:v>1.8999999999999998e+144</ns0:v>
       </ns0:c>
       <ns0:c r="F133" s="1">
         <ns0:f>ROUND(F132*1.4,-5)</ns0:f>
-        <ns0:v>3.421560164989485e+39</ns0:v>
+        <ns0:v>5.13234024748423e+39</ns0:v>
       </ns0:c>
       <ns0:c r="G133" s="1" t="n">
         <ns0:v>26.8000000000001</ns0:v>
@@ -5178,15 +5178,15 @@
       </ns0:c>
       <ns0:c r="D134" s="1">
         <ns0:f>ROUND(D133*20,2-INT(LOG10(ABS(D133*20))))</ns0:f>
-        <ns0:v>2.66e+145</ns0:v>
+        <ns0:v>3.8e+145</ns0:v>
       </ns0:c>
       <ns0:c r="E134" s="1">
         <ns0:f>D134</ns0:f>
-        <ns0:v>2.66e+145</ns0:v>
+        <ns0:v>3.8e+145</ns0:v>
       </ns0:c>
       <ns0:c r="F134" s="1">
         <ns0:f>ROUND(F133*1.4,-5)</ns0:f>
-        <ns0:v>4.7901842309852785e+39</ns0:v>
+        <ns0:v>7.185276346477922e+39</ns0:v>
       </ns0:c>
       <ns0:c r="G134" s="1" t="n">
         <ns0:v>27.0000000000001</ns0:v>
@@ -5210,15 +5210,15 @@
       </ns0:c>
       <ns0:c r="D135" s="1">
         <ns0:f>ROUND(D134*20,2-INT(LOG10(ABS(D134*20))))</ns0:f>
-        <ns0:v>5.3200000000000005e+146</ns0:v>
+        <ns0:v>7.6000000000000005e+146</ns0:v>
       </ns0:c>
       <ns0:c r="E135" s="1">
         <ns0:f>D135</ns0:f>
-        <ns0:v>5.3200000000000005e+146</ns0:v>
+        <ns0:v>7.6000000000000005e+146</ns0:v>
       </ns0:c>
       <ns0:c r="F135" s="1">
         <ns0:f>ROUND(F134*1.4,-5)</ns0:f>
-        <ns0:v>6.70625792337939e+39</ns0:v>
+        <ns0:v>1.005938688506909e+40</ns0:v>
       </ns0:c>
       <ns0:c r="G135" s="1" t="n">
         <ns0:v>27.2000000000001</ns0:v>
@@ -5242,15 +5242,15 @@
       </ns0:c>
       <ns0:c r="D136" s="1">
         <ns0:f>ROUND(D135*20,2-INT(LOG10(ABS(D135*20))))</ns0:f>
-        <ns0:v>1.06e+148</ns0:v>
+        <ns0:v>1.52e+148</ns0:v>
       </ns0:c>
       <ns0:c r="E136" s="1">
         <ns0:f>D136</ns0:f>
-        <ns0:v>1.06e+148</ns0:v>
+        <ns0:v>1.52e+148</ns0:v>
       </ns0:c>
       <ns0:c r="F136" s="1">
         <ns0:f>ROUND(F135*1.4,-5)</ns0:f>
-        <ns0:v>9.388761092731144e+39</ns0:v>
+        <ns0:v>1.4083141639096726e+40</ns0:v>
       </ns0:c>
       <ns0:c r="G136" s="1" t="n">
         <ns0:v>27.4000000000001</ns0:v>
@@ -5274,15 +5274,15 @@
       </ns0:c>
       <ns0:c r="D137" s="1">
         <ns0:f>ROUND(D136*20,2-INT(LOG10(ABS(D136*20))))</ns0:f>
-        <ns0:v>2.12e+149</ns0:v>
+        <ns0:v>3.04e+149</ns0:v>
       </ns0:c>
       <ns0:c r="E137" s="1">
         <ns0:f>D137</ns0:f>
-        <ns0:v>2.12e+149</ns0:v>
+        <ns0:v>3.04e+149</ns0:v>
       </ns0:c>
       <ns0:c r="F137" s="1">
         <ns0:f>ROUND(F136*1.4,-5)</ns0:f>
-        <ns0:v>1.31442655298236e+40</ns0:v>
+        <ns0:v>1.9716398294735414e+40</ns0:v>
       </ns0:c>
       <ns0:c r="G137" s="1" t="n">
         <ns0:v>27.6000000000001</ns0:v>
@@ -5306,15 +5306,15 @@
       </ns0:c>
       <ns0:c r="D138" s="1">
         <ns0:f>ROUND(D137*20,2-INT(LOG10(ABS(D137*20))))</ns0:f>
-        <ns0:v>4.24e+150</ns0:v>
+        <ns0:v>6.08e+150</ns0:v>
       </ns0:c>
       <ns0:c r="E138" s="1">
         <ns0:f>D138</ns0:f>
-        <ns0:v>4.24e+150</ns0:v>
+        <ns0:v>6.08e+150</ns0:v>
       </ns0:c>
       <ns0:c r="F138" s="1">
         <ns0:f>ROUND(F137*1.4,-5)</ns0:f>
-        <ns0:v>1.8401971741753039e+40</ns0:v>
+        <ns0:v>2.7602957612629577e+40</ns0:v>
       </ns0:c>
       <ns0:c r="G138" s="1" t="n">
         <ns0:v>27.8000000000001</ns0:v>
@@ -5338,15 +5338,15 @@
       </ns0:c>
       <ns0:c r="D139" s="1">
         <ns0:f>ROUND(D138*20,2-INT(LOG10(ABS(D138*20))))</ns0:f>
-        <ns0:v>8.48e+151</ns0:v>
+        <ns0:v>1.22e+152</ns0:v>
       </ns0:c>
       <ns0:c r="E139" s="1">
         <ns0:f>D139</ns0:f>
-        <ns0:v>8.48e+151</ns0:v>
+        <ns0:v>1.22e+152</ns0:v>
       </ns0:c>
       <ns0:c r="F139" s="1">
         <ns0:f>ROUND(F138*1.4,-5)</ns0:f>
-        <ns0:v>2.576276043845425e+40</ns0:v>
+        <ns0:v>3.86441406576814e+40</ns0:v>
       </ns0:c>
       <ns0:c r="G139" s="1" t="n">
         <ns0:v>28.0000000000001</ns0:v>
@@ -5370,15 +5370,15 @@
       </ns0:c>
       <ns0:c r="D140" s="1">
         <ns0:f>ROUND(D139*20,2-INT(LOG10(ABS(D139*20))))</ns0:f>
-        <ns0:v>1.7000000000000002e+153</ns0:v>
+        <ns0:v>2.44e+153</ns0:v>
       </ns0:c>
       <ns0:c r="E140" s="1">
         <ns0:f>D140</ns0:f>
-        <ns0:v>1.7000000000000002e+153</ns0:v>
+        <ns0:v>2.44e+153</ns0:v>
       </ns0:c>
       <ns0:c r="F140" s="1">
         <ns0:f>ROUND(F139*1.4,-5)</ns0:f>
-        <ns0:v>3.606786461383595e+40</ns0:v>
+        <ns0:v>5.410179692075396e+40</ns0:v>
       </ns0:c>
       <ns0:c r="G140" s="1" t="n">
         <ns0:v>28.2000000000001</ns0:v>
@@ -5402,15 +5402,15 @@
       </ns0:c>
       <ns0:c r="D141" s="1">
         <ns0:f>ROUND(D140*20,2-INT(LOG10(ABS(D140*20))))</ns0:f>
-        <ns0:v>3.4e+154</ns0:v>
+        <ns0:v>4.88e+154</ns0:v>
       </ns0:c>
       <ns0:c r="E141" s="1">
         <ns0:f>D141</ns0:f>
-        <ns0:v>3.4e+154</ns0:v>
+        <ns0:v>4.88e+154</ns0:v>
       </ns0:c>
       <ns0:c r="F141" s="1">
         <ns0:f>ROUND(F140*1.4,-5)</ns0:f>
-        <ns0:v>5.049501045937033e+40</ns0:v>
+        <ns0:v>7.574251568905554e+40</ns0:v>
       </ns0:c>
       <ns0:c r="G141" s="1" t="n">
         <ns0:v>28.4000000000001</ns0:v>
@@ -5434,15 +5434,15 @@
       </ns0:c>
       <ns0:c r="D142" s="1">
         <ns0:f>ROUND(D141*20,2-INT(LOG10(ABS(D141*20))))</ns0:f>
-        <ns0:v>6.8e+155</ns0:v>
+        <ns0:v>9.76e+155</ns0:v>
       </ns0:c>
       <ns0:c r="E142" s="1">
         <ns0:f>D142</ns0:f>
-        <ns0:v>6.8e+155</ns0:v>
+        <ns0:v>9.76e+155</ns0:v>
       </ns0:c>
       <ns0:c r="F142" s="1">
         <ns0:f>ROUND(F141*1.4,-5)</ns0:f>
-        <ns0:v>7.069301464311845e+40</ns0:v>
+        <ns0:v>1.0603952196467774e+41</ns0:v>
       </ns0:c>
       <ns0:c r="G142" s="1" t="n">
         <ns0:v>28.6000000000001</ns0:v>
@@ -5466,15 +5466,15 @@
       </ns0:c>
       <ns0:c r="D143" s="1">
         <ns0:f>ROUND(D142*20,2-INT(LOG10(ABS(D142*20))))</ns0:f>
-        <ns0:v>1.36e+157</ns0:v>
+        <ns0:v>1.95e+157</ns0:v>
       </ns0:c>
       <ns0:c r="E143" s="1">
         <ns0:f>D143</ns0:f>
-        <ns0:v>1.36e+157</ns0:v>
+        <ns0:v>1.95e+157</ns0:v>
       </ns0:c>
       <ns0:c r="F143" s="1">
         <ns0:f>ROUND(F142*1.4,-5)</ns0:f>
-        <ns0:v>9.897022050036582e+40</ns0:v>
+        <ns0:v>1.4845533075054884e+41</ns0:v>
       </ns0:c>
       <ns0:c r="G143" s="1" t="n">
         <ns0:v>28.8000000000001</ns0:v>
@@ -5498,15 +5498,15 @@
       </ns0:c>
       <ns0:c r="D144" s="1">
         <ns0:f>ROUND(D143*20,2-INT(LOG10(ABS(D143*20))))</ns0:f>
-        <ns0:v>2.72e+158</ns0:v>
+        <ns0:v>3.9e+158</ns0:v>
       </ns0:c>
       <ns0:c r="E144" s="1">
         <ns0:f>D144</ns0:f>
-        <ns0:v>2.72e+158</ns0:v>
+        <ns0:v>3.9e+158</ns0:v>
       </ns0:c>
       <ns0:c r="F144" s="1">
         <ns0:f>ROUND(F143*1.4,-5)</ns0:f>
-        <ns0:v>1.3855830870051214e+41</ns0:v>
+        <ns0:v>2.0783746305076836e+41</ns0:v>
       </ns0:c>
       <ns0:c r="G144" s="1" t="n">
         <ns0:v>29.0000000000001</ns0:v>
@@ -5530,15 +5530,15 @@
       </ns0:c>
       <ns0:c r="D145" s="1">
         <ns0:f>ROUND(D144*20,2-INT(LOG10(ABS(D144*20))))</ns0:f>
-        <ns0:v>5.440000000000001e+159</ns0:v>
+        <ns0:v>7.8e+159</ns0:v>
       </ns0:c>
       <ns0:c r="E145" s="1">
         <ns0:f>D145</ns0:f>
-        <ns0:v>5.440000000000001e+159</ns0:v>
+        <ns0:v>7.8e+159</ns0:v>
       </ns0:c>
       <ns0:c r="F145" s="1">
         <ns0:f>ROUND(F144*1.4,-5)</ns0:f>
-        <ns0:v>1.9398163218071697e+41</ns0:v>
+        <ns0:v>2.9097244827107567e+41</ns0:v>
       </ns0:c>
       <ns0:c r="G145" s="1" t="n">
         <ns0:v>29.2000000000001</ns0:v>
@@ -5562,15 +5562,15 @@
       </ns0:c>
       <ns0:c r="D146" s="1">
         <ns0:f>ROUND(D145*20,2-INT(LOG10(ABS(D145*20))))</ns0:f>
-        <ns0:v>1.09e+161</ns0:v>
+        <ns0:v>1.56e+161</ns0:v>
       </ns0:c>
       <ns0:c r="E146" s="1">
         <ns0:f>D146</ns0:f>
-        <ns0:v>1.09e+161</ns0:v>
+        <ns0:v>1.56e+161</ns0:v>
       </ns0:c>
       <ns0:c r="F146" s="1">
         <ns0:f>ROUND(F145*1.4,-5)</ns0:f>
-        <ns0:v>2.7157428505300373e+41</ns0:v>
+        <ns0:v>4.073614275795059e+41</ns0:v>
       </ns0:c>
       <ns0:c r="G146" s="1" t="n">
         <ns0:v>29.4000000000001</ns0:v>
@@ -5594,15 +5594,15 @@
       </ns0:c>
       <ns0:c r="D147" s="1">
         <ns0:f>ROUND(D146*20,2-INT(LOG10(ABS(D146*20))))</ns0:f>
-        <ns0:v>2.18e+162</ns0:v>
+        <ns0:v>3.12e+162</ns0:v>
       </ns0:c>
       <ns0:c r="E147" s="1">
         <ns0:f>D147</ns0:f>
-        <ns0:v>2.18e+162</ns0:v>
+        <ns0:v>3.12e+162</ns0:v>
       </ns0:c>
       <ns0:c r="F147" s="1">
         <ns0:f>ROUND(F146*1.4,-5)</ns0:f>
-        <ns0:v>3.802039990742052e+41</ns0:v>
+        <ns0:v>5.703059986113083e+41</ns0:v>
       </ns0:c>
       <ns0:c r="G147" s="1" t="n">
         <ns0:v>29.6000000000001</ns0:v>
@@ -5626,15 +5626,15 @@
       </ns0:c>
       <ns0:c r="D148" s="1">
         <ns0:f>ROUND(D147*20,2-INT(LOG10(ABS(D147*20))))</ns0:f>
-        <ns0:v>4.3599999999999997e+163</ns0:v>
+        <ns0:v>6.239999999999999e+163</ns0:v>
       </ns0:c>
       <ns0:c r="E148" s="1">
         <ns0:f>D148</ns0:f>
-        <ns0:v>4.3599999999999997e+163</ns0:v>
+        <ns0:v>6.239999999999999e+163</ns0:v>
       </ns0:c>
       <ns0:c r="F148" s="1">
         <ns0:f>ROUND(F147*1.4,-5)</ns0:f>
-        <ns0:v>5.322855987038872e+41</ns0:v>
+        <ns0:v>7.984283980558315e+41</ns0:v>
       </ns0:c>
       <ns0:c r="G148" s="1" t="n">
         <ns0:v>29.8000000000001</ns0:v>
@@ -5658,15 +5658,15 @@
       </ns0:c>
       <ns0:c r="D149" s="1">
         <ns0:f>ROUND(D148*20,2-INT(LOG10(ABS(D148*20))))</ns0:f>
-        <ns0:v>8.72e+164</ns0:v>
+        <ns0:v>1.2500000000000001e+165</ns0:v>
       </ns0:c>
       <ns0:c r="E149" s="1">
         <ns0:f>D149</ns0:f>
-        <ns0:v>8.72e+164</ns0:v>
+        <ns0:v>1.2500000000000001e+165</ns0:v>
       </ns0:c>
       <ns0:c r="F149" s="1">
         <ns0:f>ROUND(F148*1.4,-5)</ns0:f>
-        <ns0:v>7.45199838185442e+41</ns0:v>
+        <ns0:v>1.117799757278164e+42</ns0:v>
       </ns0:c>
       <ns0:c r="G149" s="1" t="n">
         <ns0:v>30.0000000000001</ns0:v>
@@ -5690,15 +5690,15 @@
       </ns0:c>
       <ns0:c r="D150" s="1">
         <ns0:f>ROUND(D149*20,2-INT(LOG10(ABS(D149*20))))</ns0:f>
-        <ns0:v>1.74e+166</ns0:v>
+        <ns0:v>2.5e+166</ns0:v>
       </ns0:c>
       <ns0:c r="E150" s="1">
         <ns0:f>D150</ns0:f>
-        <ns0:v>1.74e+166</ns0:v>
+        <ns0:v>2.5e+166</ns0:v>
       </ns0:c>
       <ns0:c r="F150" s="1">
         <ns0:f>ROUND(F149*1.4,-5)</ns0:f>
-        <ns0:v>1.0432797734596187e+42</ns0:v>
+        <ns0:v>1.5649196601894296e+42</ns0:v>
       </ns0:c>
       <ns0:c r="G150" s="1" t="n">
         <ns0:v>30.2000000000001</ns0:v>
@@ -5722,15 +5722,15 @@
       </ns0:c>
       <ns0:c r="D151" s="1">
         <ns0:f>ROUND(D150*20,2-INT(LOG10(ABS(D150*20))))</ns0:f>
-        <ns0:v>3.48e+167</ns0:v>
+        <ns0:v>5e+167</ns0:v>
       </ns0:c>
       <ns0:c r="E151" s="1">
         <ns0:f>D151</ns0:f>
-        <ns0:v>3.48e+167</ns0:v>
+        <ns0:v>5e+167</ns0:v>
       </ns0:c>
       <ns0:c r="F151" s="1">
         <ns0:f>ROUND(F150*1.4,-5)</ns0:f>
-        <ns0:v>1.4605916828434662e+42</ns0:v>
+        <ns0:v>2.1908875242652015e+42</ns0:v>
       </ns0:c>
       <ns0:c r="G151" s="1" t="n">
         <ns0:v>30.4000000000001</ns0:v>
@@ -5754,15 +5754,15 @@
       </ns0:c>
       <ns0:c r="D152" s="1">
         <ns0:f>ROUND(D151*20,2-INT(LOG10(ABS(D151*20))))</ns0:f>
-        <ns0:v>6.96e+168</ns0:v>
+        <ns0:v>1e+169</ns0:v>
       </ns0:c>
       <ns0:c r="E152" s="1">
         <ns0:f>D152</ns0:f>
-        <ns0:v>6.96e+168</ns0:v>
+        <ns0:v>1e+169</ns0:v>
       </ns0:c>
       <ns0:c r="F152" s="1">
         <ns0:f>ROUND(F151*1.4,-5)</ns0:f>
-        <ns0:v>2.0448283559808525e+42</ns0:v>
+        <ns0:v>3.067242533971282e+42</ns0:v>
       </ns0:c>
       <ns0:c r="G152" s="1" t="n">
         <ns0:v>30.6000000000001</ns0:v>
@@ -5786,15 +5786,15 @@
       </ns0:c>
       <ns0:c r="D153" s="1">
         <ns0:f>ROUND(D152*20,2-INT(LOG10(ABS(D152*20))))</ns0:f>
-        <ns0:v>1.3899999999999998e+170</ns0:v>
+        <ns0:v>1.9999999999999998e+170</ns0:v>
       </ns0:c>
       <ns0:c r="E153" s="1">
         <ns0:f>D153</ns0:f>
-        <ns0:v>1.3899999999999998e+170</ns0:v>
+        <ns0:v>1.9999999999999998e+170</ns0:v>
       </ns0:c>
       <ns0:c r="F153" s="1">
         <ns0:f>ROUND(F152*1.4,-5)</ns0:f>
-        <ns0:v>2.8627596983731936e+42</ns0:v>
+        <ns0:v>4.294139547559795e+42</ns0:v>
       </ns0:c>
       <ns0:c r="G153" s="1" t="n">
         <ns0:v>30.8000000000001</ns0:v>
@@ -5818,15 +5818,15 @@
       </ns0:c>
       <ns0:c r="D154" s="1">
         <ns0:f>ROUND(D153*20,2-INT(LOG10(ABS(D153*20))))</ns0:f>
-        <ns0:v>2.7799999999999997e+171</ns0:v>
+        <ns0:v>4e+171</ns0:v>
       </ns0:c>
       <ns0:c r="E154" s="1">
         <ns0:f>D154</ns0:f>
-        <ns0:v>2.7799999999999997e+171</ns0:v>
+        <ns0:v>4e+171</ns0:v>
       </ns0:c>
       <ns0:c r="F154" s="1">
         <ns0:f>ROUND(F153*1.4,-5)</ns0:f>
-        <ns0:v>4.0078635777224706e+42</ns0:v>
+        <ns0:v>6.011795366583712e+42</ns0:v>
       </ns0:c>
       <ns0:c r="G154" s="1" t="n">
         <ns0:v>31.0000000000001</ns0:v>
@@ -5850,15 +5850,15 @@
       </ns0:c>
       <ns0:c r="D155" s="1">
         <ns0:f>ROUND(D154*20,2-INT(LOG10(ABS(D154*20))))</ns0:f>
-        <ns0:v>5.56e+172</ns0:v>
+        <ns0:v>8e+172</ns0:v>
       </ns0:c>
       <ns0:c r="E155" s="1">
         <ns0:f>D155</ns0:f>
-        <ns0:v>5.56e+172</ns0:v>
+        <ns0:v>8e+172</ns0:v>
       </ns0:c>
       <ns0:c r="F155" s="1">
         <ns0:f>ROUND(F154*1.4,-5)</ns0:f>
-        <ns0:v>5.611009008811459e+42</ns0:v>
+        <ns0:v>8.416513513217197e+42</ns0:v>
       </ns0:c>
       <ns0:c r="G155" s="1" t="n">
         <ns0:v>31.2000000000001</ns0:v>
@@ -5882,15 +5882,15 @@
       </ns0:c>
       <ns0:c r="D156" s="1">
         <ns0:f>ROUND(D155*20,2-INT(LOG10(ABS(D155*20))))</ns0:f>
-        <ns0:v>1.11e+174</ns0:v>
+        <ns0:v>1.6e+174</ns0:v>
       </ns0:c>
       <ns0:c r="E156" s="1">
         <ns0:f>D156</ns0:f>
-        <ns0:v>1.11e+174</ns0:v>
+        <ns0:v>1.6e+174</ns0:v>
       </ns0:c>
       <ns0:c r="F156" s="1">
         <ns0:f>ROUND(F155*1.4,-5)</ns0:f>
-        <ns0:v>7.855412612336042e+42</ns0:v>
+        <ns0:v>1.1783118918504076e+43</ns0:v>
       </ns0:c>
       <ns0:c r="G156" s="1" t="n">
         <ns0:v>31.4000000000001</ns0:v>
@@ -5914,15 +5914,15 @@
       </ns0:c>
       <ns0:c r="D157" s="1">
         <ns0:f>ROUND(D156*20,2-INT(LOG10(ABS(D156*20))))</ns0:f>
-        <ns0:v>2.22e+175</ns0:v>
+        <ns0:v>3.2e+175</ns0:v>
       </ns0:c>
       <ns0:c r="E157" s="1">
         <ns0:f>D157</ns0:f>
-        <ns0:v>2.22e+175</ns0:v>
+        <ns0:v>3.2e+175</ns0:v>
       </ns0:c>
       <ns0:c r="F157" s="1">
         <ns0:f>ROUND(F156*1.4,-5)</ns0:f>
-        <ns0:v>1.0997577657270457e+43</ns0:v>
+        <ns0:v>1.6496366485905706e+43</ns0:v>
       </ns0:c>
       <ns0:c r="G157" s="1" t="n">
         <ns0:v>31.6000000000001</ns0:v>
@@ -5946,15 +5946,15 @@
       </ns0:c>
       <ns0:c r="D158" s="1">
         <ns0:f>ROUND(D157*20,2-INT(LOG10(ABS(D157*20))))</ns0:f>
-        <ns0:v>4.44e+176</ns0:v>
+        <ns0:v>6.4e+176</ns0:v>
       </ns0:c>
       <ns0:c r="E158" s="1">
         <ns0:f>D158</ns0:f>
-        <ns0:v>4.44e+176</ns0:v>
+        <ns0:v>6.4e+176</ns0:v>
       </ns0:c>
       <ns0:c r="F158" s="1">
         <ns0:f>ROUND(F157*1.4,-5)</ns0:f>
-        <ns0:v>1.539660872017864e+43</ns0:v>
+        <ns0:v>2.3094913080267985e+43</ns0:v>
       </ns0:c>
       <ns0:c r="G158" s="1" t="n">
         <ns0:v>31.8000000000001</ns0:v>
@@ -5978,15 +5978,15 @@
       </ns0:c>
       <ns0:c r="D159" s="1">
         <ns0:f>ROUND(D158*20,2-INT(LOG10(ABS(D158*20))))</ns0:f>
-        <ns0:v>8.88e+177</ns0:v>
+        <ns0:v>1.28e+178</ns0:v>
       </ns0:c>
       <ns0:c r="E159" s="1">
         <ns0:f>D159</ns0:f>
-        <ns0:v>8.88e+177</ns0:v>
+        <ns0:v>1.28e+178</ns0:v>
       </ns0:c>
       <ns0:c r="F159" s="1">
         <ns0:f>ROUND(F158*1.4,-5)</ns0:f>
-        <ns0:v>2.1555252208250092e+43</ns0:v>
+        <ns0:v>3.2332878312375176e+43</ns0:v>
       </ns0:c>
       <ns0:c r="G159" s="1" t="n">
         <ns0:v>32.0000000000001</ns0:v>
@@ -6010,15 +6010,15 @@
       </ns0:c>
       <ns0:c r="D160" s="1">
         <ns0:f>ROUND(D159*20,2-INT(LOG10(ABS(D159*20))))</ns0:f>
-        <ns0:v>1.78e+179</ns0:v>
+        <ns0:v>2.56e+179</ns0:v>
       </ns0:c>
       <ns0:c r="E160" s="1">
         <ns0:f>D160</ns0:f>
-        <ns0:v>1.78e+179</ns0:v>
+        <ns0:v>2.56e+179</ns0:v>
       </ns0:c>
       <ns0:c r="F160" s="1">
         <ns0:f>ROUND(F159*1.4,-5)</ns0:f>
-        <ns0:v>3.0177353091550127e+43</ns0:v>
+        <ns0:v>4.526602963732524e+43</ns0:v>
       </ns0:c>
       <ns0:c r="G160" s="1" t="n">
         <ns0:v>32.2000000000001</ns0:v>
@@ -6042,15 +6042,15 @@
       </ns0:c>
       <ns0:c r="D161" s="1">
         <ns0:f>ROUND(D160*20,2-INT(LOG10(ABS(D160*20))))</ns0:f>
-        <ns0:v>3.56e+180</ns0:v>
+        <ns0:v>5.12e+180</ns0:v>
       </ns0:c>
       <ns0:c r="E161" s="1">
         <ns0:f>D161</ns0:f>
-        <ns0:v>3.56e+180</ns0:v>
+        <ns0:v>5.12e+180</ns0:v>
       </ns0:c>
       <ns0:c r="F161" s="1">
         <ns0:f>ROUND(F160*1.4,-5)</ns0:f>
-        <ns0:v>4.2248294328170174e+43</ns0:v>
+        <ns0:v>6.337244149225533e+43</ns0:v>
       </ns0:c>
       <ns0:c r="G161" s="1" t="n">
         <ns0:v>32.4000000000001</ns0:v>
@@ -6074,15 +6074,15 @@
       </ns0:c>
       <ns0:c r="D162" s="1">
         <ns0:f>ROUND(D161*20,2-INT(LOG10(ABS(D161*20))))</ns0:f>
-        <ns0:v>7.12e+181</ns0:v>
+        <ns0:v>1.02e+182</ns0:v>
       </ns0:c>
       <ns0:c r="E162" s="1">
         <ns0:f>D162</ns0:f>
-        <ns0:v>7.12e+181</ns0:v>
+        <ns0:v>1.02e+182</ns0:v>
       </ns0:c>
       <ns0:c r="F162" s="1">
         <ns0:f>ROUND(F161*1.4,-5)</ns0:f>
-        <ns0:v>5.914761205943824e+43</ns0:v>
+        <ns0:v>8.872141808915746e+43</ns0:v>
       </ns0:c>
       <ns0:c r="G162" s="1" t="n">
         <ns0:v>32.6000000000001</ns0:v>
@@ -6106,15 +6106,15 @@
       </ns0:c>
       <ns0:c r="D163" s="1">
         <ns0:f>ROUND(D162*20,2-INT(LOG10(ABS(D162*20))))</ns0:f>
-        <ns0:v>1.42e+183</ns0:v>
+        <ns0:v>2.0399999999999998e+183</ns0:v>
       </ns0:c>
       <ns0:c r="E163" s="1">
         <ns0:f>D163</ns0:f>
-        <ns0:v>1.42e+183</ns0:v>
+        <ns0:v>2.0399999999999998e+183</ns0:v>
       </ns0:c>
       <ns0:c r="F163" s="1">
         <ns0:f>ROUND(F162*1.4,-5)</ns0:f>
-        <ns0:v>8.280665688321353e+43</ns0:v>
+        <ns0:v>1.2420998532482043e+44</ns0:v>
       </ns0:c>
       <ns0:c r="G163" s="1" t="n">
         <ns0:v>32.8000000000001</ns0:v>
@@ -6138,15 +6138,15 @@
       </ns0:c>
       <ns0:c r="D164" s="1">
         <ns0:f>ROUND(D163*20,2-INT(LOG10(ABS(D163*20))))</ns0:f>
-        <ns0:v>2.84e+184</ns0:v>
+        <ns0:v>4.0799999999999996e+184</ns0:v>
       </ns0:c>
       <ns0:c r="E164" s="1">
         <ns0:f>D164</ns0:f>
-        <ns0:v>2.84e+184</ns0:v>
+        <ns0:v>4.0799999999999996e+184</ns0:v>
       </ns0:c>
       <ns0:c r="F164" s="1">
         <ns0:f>ROUND(F163*1.4,-5)</ns0:f>
-        <ns0:v>1.1592931963649895e+44</ns0:v>
+        <ns0:v>1.7389397945474857e+44</ns0:v>
       </ns0:c>
       <ns0:c r="G164" s="1" t="n">
         <ns0:v>33.0000000000001</ns0:v>
@@ -6170,15 +6170,15 @@
       </ns0:c>
       <ns0:c r="D165" s="1">
         <ns0:f>ROUND(D164*20,2-INT(LOG10(ABS(D164*20))))</ns0:f>
-        <ns0:v>5.68e+185</ns0:v>
+        <ns0:v>8.16e+185</ns0:v>
       </ns0:c>
       <ns0:c r="E165" s="1">
         <ns0:f>D165</ns0:f>
-        <ns0:v>5.68e+185</ns0:v>
+        <ns0:v>8.16e+185</ns0:v>
       </ns0:c>
       <ns0:c r="F165" s="1">
         <ns0:f>ROUND(F164*1.4,-5)</ns0:f>
-        <ns0:v>1.6230104749109852e+44</ns0:v>
+        <ns0:v>2.43451571236648e+44</ns0:v>
       </ns0:c>
       <ns0:c r="G165" s="1" t="n">
         <ns0:v>33.2000000000001</ns0:v>
@@ -6202,15 +6202,15 @@
       </ns0:c>
       <ns0:c r="D166" s="1">
         <ns0:f>ROUND(D165*20,2-INT(LOG10(ABS(D165*20))))</ns0:f>
-        <ns0:v>1.14e+187</ns0:v>
+        <ns0:v>1.6300000000000001e+187</ns0:v>
       </ns0:c>
       <ns0:c r="E166" s="1">
         <ns0:f>D166</ns0:f>
-        <ns0:v>1.14e+187</ns0:v>
+        <ns0:v>1.6300000000000001e+187</ns0:v>
       </ns0:c>
       <ns0:c r="F166" s="1">
         <ns0:f>ROUND(F165*1.4,-5)</ns0:f>
-        <ns0:v>2.2722146648753793e+44</ns0:v>
+        <ns0:v>3.4083219973130723e+44</ns0:v>
       </ns0:c>
       <ns0:c r="G166" s="1" t="n">
         <ns0:v>33.4000000000001</ns0:v>
@@ -6234,15 +6234,15 @@
       </ns0:c>
       <ns0:c r="D167" s="1">
         <ns0:f>ROUND(D166*20,2-INT(LOG10(ABS(D166*20))))</ns0:f>
-        <ns0:v>2.28e+188</ns0:v>
+        <ns0:v>3.2600000000000005e+188</ns0:v>
       </ns0:c>
       <ns0:c r="E167" s="1">
         <ns0:f>D167</ns0:f>
-        <ns0:v>2.28e+188</ns0:v>
+        <ns0:v>3.2600000000000005e+188</ns0:v>
       </ns0:c>
       <ns0:c r="F167" s="1">
         <ns0:f>ROUND(F166*1.4,-5)</ns0:f>
-        <ns0:v>3.181100530825531e+44</ns0:v>
+        <ns0:v>4.771650796238301e+44</ns0:v>
       </ns0:c>
       <ns0:c r="G167" s="1" t="n">
         <ns0:v>33.6000000000001</ns0:v>
@@ -6266,15 +6266,15 @@
       </ns0:c>
       <ns0:c r="D168" s="1">
         <ns0:f>ROUND(D167*20,2-INT(LOG10(ABS(D167*20))))</ns0:f>
-        <ns0:v>4.56e+189</ns0:v>
+        <ns0:v>6.52e+189</ns0:v>
       </ns0:c>
       <ns0:c r="E168" s="1">
         <ns0:f>D168</ns0:f>
-        <ns0:v>4.56e+189</ns0:v>
+        <ns0:v>6.52e+189</ns0:v>
       </ns0:c>
       <ns0:c r="F168" s="1">
         <ns0:f>ROUND(F167*1.4,-5)</ns0:f>
-        <ns0:v>4.4535407431557436e+44</ns0:v>
+        <ns0:v>6.680311114733622e+44</ns0:v>
       </ns0:c>
       <ns0:c r="G168" s="1" t="n">
         <ns0:v>33.8000000000001</ns0:v>
@@ -6298,15 +6298,15 @@
       </ns0:c>
       <ns0:c r="D169" s="1">
         <ns0:f>ROUND(D168*20,2-INT(LOG10(ABS(D168*20))))</ns0:f>
-        <ns0:v>9.12e+190</ns0:v>
+        <ns0:v>1.2999999999999999e+191</ns0:v>
       </ns0:c>
       <ns0:c r="E169" s="1">
         <ns0:f>D169</ns0:f>
-        <ns0:v>9.12e+190</ns0:v>
+        <ns0:v>1.2999999999999999e+191</ns0:v>
       </ns0:c>
       <ns0:c r="F169" s="1">
         <ns0:f>ROUND(F168*1.4,-5)</ns0:f>
-        <ns0:v>6.234957040418041e+44</ns0:v>
+        <ns0:v>9.35243556062707e+44</ns0:v>
       </ns0:c>
       <ns0:c r="G169" s="1" t="n">
         <ns0:v>34.0000000000001</ns0:v>
@@ -6330,15 +6330,15 @@
       </ns0:c>
       <ns0:c r="D170" s="1">
         <ns0:f>ROUND(D169*20,2-INT(LOG10(ABS(D169*20))))</ns0:f>
-        <ns0:v>1.82e+192</ns0:v>
+        <ns0:v>2.6e+192</ns0:v>
       </ns0:c>
       <ns0:c r="E170" s="1">
         <ns0:f>D170</ns0:f>
-        <ns0:v>1.82e+192</ns0:v>
+        <ns0:v>2.6e+192</ns0:v>
       </ns0:c>
       <ns0:c r="F170" s="1">
         <ns0:f>ROUND(F169*1.4,-5)</ns0:f>
-        <ns0:v>8.728939856585256e+44</ns0:v>
+        <ns0:v>1.3093409784877897e+45</ns0:v>
       </ns0:c>
       <ns0:c r="G170" s="1" t="n">
         <ns0:v>34.2000000000001</ns0:v>
@@ -6362,15 +6362,15 @@
       </ns0:c>
       <ns0:c r="D171" s="1">
         <ns0:f>ROUND(D170*20,2-INT(LOG10(ABS(D170*20))))</ns0:f>
-        <ns0:v>3.64e+193</ns0:v>
+        <ns0:v>5.2e+193</ns0:v>
       </ns0:c>
       <ns0:c r="E171" s="1">
         <ns0:f>D171</ns0:f>
-        <ns0:v>3.64e+193</ns0:v>
+        <ns0:v>5.2e+193</ns0:v>
       </ns0:c>
       <ns0:c r="F171" s="1">
         <ns0:f>ROUND(F170*1.4,-5)</ns0:f>
-        <ns0:v>1.2220515799219357e+45</ns0:v>
+        <ns0:v>1.8330773698829054e+45</ns0:v>
       </ns0:c>
       <ns0:c r="G171" s="1" t="n">
         <ns0:v>34.4000000000001</ns0:v>
@@ -6394,15 +6394,15 @@
       </ns0:c>
       <ns0:c r="D172" s="1">
         <ns0:f>ROUND(D171*20,2-INT(LOG10(ABS(D171*20))))</ns0:f>
-        <ns0:v>7.279999999999999e+194</ns0:v>
+        <ns0:v>1.04e+195</ns0:v>
       </ns0:c>
       <ns0:c r="E172" s="1">
         <ns0:f>D172</ns0:f>
-        <ns0:v>7.279999999999999e+194</ns0:v>
+        <ns0:v>1.04e+195</ns0:v>
       </ns0:c>
       <ns0:c r="F172" s="1">
         <ns0:f>ROUND(F171*1.4,-5)</ns0:f>
-        <ns0:v>1.71087221189071e+45</ns0:v>
+        <ns0:v>2.5663083178360675e+45</ns0:v>
       </ns0:c>
       <ns0:c r="G172" s="1" t="n">
         <ns0:v>34.6000000000001</ns0:v>
@@ -6426,15 +6426,15 @@
       </ns0:c>
       <ns0:c r="D173" s="1">
         <ns0:f>ROUND(D172*20,2-INT(LOG10(ABS(D172*20))))</ns0:f>
-        <ns0:v>1.4599999999999999e+196</ns0:v>
+        <ns0:v>2.08e+196</ns0:v>
       </ns0:c>
       <ns0:c r="E173" s="1">
         <ns0:f>D173</ns0:f>
-        <ns0:v>1.4599999999999999e+196</ns0:v>
+        <ns0:v>2.08e+196</ns0:v>
       </ns0:c>
       <ns0:c r="F173" s="1">
         <ns0:f>ROUND(F172*1.4,-5)</ns0:f>
-        <ns0:v>2.395221096646994e+45</ns0:v>
+        <ns0:v>3.592831644970494e+45</ns0:v>
       </ns0:c>
       <ns0:c r="G173" s="1" t="n">
         <ns0:v>34.8000000000001</ns0:v>
@@ -6458,15 +6458,15 @@
       </ns0:c>
       <ns0:c r="D174" s="1">
         <ns0:f>ROUND(D173*20,2-INT(LOG10(ABS(D173*20))))</ns0:f>
-        <ns0:v>2.9199999999999997e+197</ns0:v>
+        <ns0:v>4.1599999999999995e+197</ns0:v>
       </ns0:c>
       <ns0:c r="E174" s="1">
         <ns0:f>D174</ns0:f>
-        <ns0:v>2.9199999999999997e+197</ns0:v>
+        <ns0:v>4.1599999999999995e+197</ns0:v>
       </ns0:c>
       <ns0:c r="F174" s="1">
         <ns0:f>ROUND(F173*1.4,-5)</ns0:f>
-        <ns0:v>3.3533095353057913e+45</ns0:v>
+        <ns0:v>5.0299643029586914e+45</ns0:v>
       </ns0:c>
       <ns0:c r="G174" s="1" t="n">
         <ns0:v>35.0000000000001</ns0:v>
@@ -6490,15 +6490,15 @@
       </ns0:c>
       <ns0:c r="D175" s="1">
         <ns0:f>ROUND(D174*20,2-INT(LOG10(ABS(D174*20))))</ns0:f>
-        <ns0:v>5.84e+198</ns0:v>
+        <ns0:v>8.32e+198</ns0:v>
       </ns0:c>
       <ns0:c r="E175" s="1">
         <ns0:f>D175</ns0:f>
-        <ns0:v>5.84e+198</ns0:v>
+        <ns0:v>8.32e+198</ns0:v>
       </ns0:c>
       <ns0:c r="F175" s="1">
         <ns0:f>ROUND(F174*1.4,-5)</ns0:f>
-        <ns0:v>4.6946333494281075e+45</ns0:v>
+        <ns0:v>7.041950024142167e+45</ns0:v>
       </ns0:c>
       <ns0:c r="G175" s="1" t="n">
         <ns0:v>35.2000000000001</ns0:v>
@@ -6522,15 +6522,15 @@
       </ns0:c>
       <ns0:c r="D176" s="1">
         <ns0:f>ROUND(D175*20,2-INT(LOG10(ABS(D175*20))))</ns0:f>
-        <ns0:v>1.17e+200</ns0:v>
+        <ns0:v>1.66e+200</ns0:v>
       </ns0:c>
       <ns0:c r="E176" s="1">
         <ns0:f>D176</ns0:f>
-        <ns0:v>1.17e+200</ns0:v>
+        <ns0:v>1.66e+200</ns0:v>
       </ns0:c>
       <ns0:c r="F176" s="1">
         <ns0:f>ROUND(F175*1.4,-5)</ns0:f>
-        <ns0:v>6.57248668919935e+45</ns0:v>
+        <ns0:v>9.858730033799032e+45</ns0:v>
       </ns0:c>
       <ns0:c r="G176" s="1" t="n">
         <ns0:v>35.4000000000001</ns0:v>
@@ -6554,15 +6554,15 @@
       </ns0:c>
       <ns0:c r="D177" s="1">
         <ns0:f>ROUND(D176*20,2-INT(LOG10(ABS(D176*20))))</ns0:f>
-        <ns0:v>2.34e+201</ns0:v>
+        <ns0:v>3.32e+201</ns0:v>
       </ns0:c>
       <ns0:c r="E177" s="1">
         <ns0:f>D177</ns0:f>
-        <ns0:v>2.34e+201</ns0:v>
+        <ns0:v>3.32e+201</ns0:v>
       </ns0:c>
       <ns0:c r="F177" s="1">
         <ns0:f>ROUND(F176*1.4,-5)</ns0:f>
-        <ns0:v>9.20148136487909e+45</ns0:v>
+        <ns0:v>1.3802222047318644e+46</ns0:v>
       </ns0:c>
       <ns0:c r="G177" s="1" t="n">
         <ns0:v>35.6000000000001</ns0:v>
@@ -6586,15 +6586,15 @@
       </ns0:c>
       <ns0:c r="D178" s="1">
         <ns0:f>ROUND(D177*20,2-INT(LOG10(ABS(D177*20))))</ns0:f>
-        <ns0:v>4.6800000000000005e+202</ns0:v>
+        <ns0:v>6.64e+202</ns0:v>
       </ns0:c>
       <ns0:c r="E178" s="1">
         <ns0:f>D178</ns0:f>
-        <ns0:v>4.6800000000000005e+202</ns0:v>
+        <ns0:v>6.64e+202</ns0:v>
       </ns0:c>
       <ns0:c r="F178" s="1">
         <ns0:f>ROUND(F177*1.4,-5)</ns0:f>
-        <ns0:v>1.2882073910830726e+46</ns0:v>
+        <ns0:v>1.9323110866246103e+46</ns0:v>
       </ns0:c>
       <ns0:c r="G178" s="1" t="n">
         <ns0:v>35.8000000000001</ns0:v>
@@ -6618,15 +6618,15 @@
       </ns0:c>
       <ns0:c r="D179" s="1">
         <ns0:f>ROUND(D178*20,2-INT(LOG10(ABS(D178*20))))</ns0:f>
-        <ns0:v>9.36e+203</ns0:v>
+        <ns0:v>1.33e+204</ns0:v>
       </ns0:c>
       <ns0:c r="E179" s="1">
         <ns0:f>D179</ns0:f>
-        <ns0:v>9.36e+203</ns0:v>
+        <ns0:v>1.33e+204</ns0:v>
       </ns0:c>
       <ns0:c r="F179" s="1">
         <ns0:f>ROUND(F178*1.4,-5)</ns0:f>
-        <ns0:v>1.8034903475163013e+46</ns0:v>
+        <ns0:v>2.705235521274454e+46</ns0:v>
       </ns0:c>
       <ns0:c r="G179" s="1" t="n">
         <ns0:v>36.0000000000001</ns0:v>
@@ -6650,15 +6650,15 @@
       </ns0:c>
       <ns0:c r="D180" s="1">
         <ns0:f>ROUND(D179*20,2-INT(LOG10(ABS(D179*20))))</ns0:f>
-        <ns0:v>1.8699999999999999e+205</ns0:v>
+        <ns0:v>2.6599999999999998e+205</ns0:v>
       </ns0:c>
       <ns0:c r="E180" s="1">
         <ns0:f>D180</ns0:f>
-        <ns0:v>1.8699999999999999e+205</ns0:v>
+        <ns0:v>2.6599999999999998e+205</ns0:v>
       </ns0:c>
       <ns0:c r="F180" s="1">
         <ns0:f>ROUND(F179*1.4,-5)</ns0:f>
-        <ns0:v>2.524886486522822e+46</ns0:v>
+        <ns0:v>3.787329729784235e+46</ns0:v>
       </ns0:c>
       <ns0:c r="G180" s="1" t="n">
         <ns0:v>36.2000000000001</ns0:v>
@@ -6682,15 +6682,15 @@
       </ns0:c>
       <ns0:c r="D181" s="1">
         <ns0:f>ROUND(D180*20,2-INT(LOG10(ABS(D180*20))))</ns0:f>
-        <ns0:v>3.74e+206</ns0:v>
+        <ns0:v>5.32e+206</ns0:v>
       </ns0:c>
       <ns0:c r="E181" s="1">
         <ns0:f>D181</ns0:f>
-        <ns0:v>3.74e+206</ns0:v>
+        <ns0:v>5.32e+206</ns0:v>
       </ns0:c>
       <ns0:c r="F181" s="1">
         <ns0:f>ROUND(F180*1.4,-5)</ns0:f>
-        <ns0:v>3.5348410811319504e+46</ns0:v>
+        <ns0:v>5.302261621697928e+46</ns0:v>
       </ns0:c>
       <ns0:c r="G181" s="1" t="n">
         <ns0:v>36.4000000000001</ns0:v>
@@ -6714,15 +6714,15 @@
       </ns0:c>
       <ns0:c r="D182" s="1">
         <ns0:f>ROUND(D181*20,2-INT(LOG10(ABS(D181*20))))</ns0:f>
-        <ns0:v>7.48e+207</ns0:v>
+        <ns0:v>1.06e+208</ns0:v>
       </ns0:c>
       <ns0:c r="E182" s="1">
         <ns0:f>D182</ns0:f>
-        <ns0:v>7.48e+207</ns0:v>
+        <ns0:v>1.06e+208</ns0:v>
       </ns0:c>
       <ns0:c r="F182" s="1">
         <ns0:f>ROUND(F181*1.4,-5)</ns0:f>
-        <ns0:v>4.94877751358473e+46</ns0:v>
+        <ns0:v>7.423166270377099e+46</ns0:v>
       </ns0:c>
       <ns0:c r="G182" s="1" t="n">
         <ns0:v>36.6000000000001</ns0:v>
@@ -6746,15 +6746,15 @@
       </ns0:c>
       <ns0:c r="D183" s="1">
         <ns0:f>ROUND(D182*20,2-INT(LOG10(ABS(D182*20))))</ns0:f>
-        <ns0:v>1.5000000000000001e+209</ns0:v>
+        <ns0:v>2.12e+209</ns0:v>
       </ns0:c>
       <ns0:c r="E183" s="1">
         <ns0:f>D183</ns0:f>
-        <ns0:v>1.5000000000000001e+209</ns0:v>
+        <ns0:v>2.12e+209</ns0:v>
       </ns0:c>
       <ns0:c r="F183" s="1">
         <ns0:f>ROUND(F182*1.4,-5)</ns0:f>
-        <ns0:v>6.928288519018622e+46</ns0:v>
+        <ns0:v>1.0392432778527938e+47</ns0:v>
       </ns0:c>
       <ns0:c r="G183" s="1" t="n">
         <ns0:v>36.8000000000001</ns0:v>
@@ -6778,15 +6778,15 @@
       </ns0:c>
       <ns0:c r="D184" s="1">
         <ns0:f>ROUND(D183*20,2-INT(LOG10(ABS(D183*20))))</ns0:f>
-        <ns0:v>2.9999999999999996e+210</ns0:v>
+        <ns0:v>4.2399999999999994e+210</ns0:v>
       </ns0:c>
       <ns0:c r="E184" s="1">
         <ns0:f>D184</ns0:f>
-        <ns0:v>2.9999999999999996e+210</ns0:v>
+        <ns0:v>4.2399999999999994e+210</ns0:v>
       </ns0:c>
       <ns0:c r="F184" s="1">
         <ns0:f>ROUND(F183*1.4,-5)</ns0:f>
-        <ns0:v>9.699603926626071e+46</ns0:v>
+        <ns0:v>1.4549405889939113e+47</ns0:v>
       </ns0:c>
       <ns0:c r="G184" s="1" t="n">
         <ns0:v>37.0000000000001</ns0:v>
@@ -6810,15 +6810,15 @@
       </ns0:c>
       <ns0:c r="D185" s="1">
         <ns0:f>ROUND(D184*20,2-INT(LOG10(ABS(D184*20))))</ns0:f>
-        <ns0:v>5.999999999999999e+211</ns0:v>
+        <ns0:v>8.48e+211</ns0:v>
       </ns0:c>
       <ns0:c r="E185" s="1">
         <ns0:f>D185</ns0:f>
-        <ns0:v>5.999999999999999e+211</ns0:v>
+        <ns0:v>8.48e+211</ns0:v>
       </ns0:c>
       <ns0:c r="F185" s="1">
         <ns0:f>ROUND(F184*1.4,-5)</ns0:f>
-        <ns0:v>1.3579445497276498e+47</ns0:v>
+        <ns0:v>2.0369168245914757e+47</ns0:v>
       </ns0:c>
       <ns0:c r="G185" s="1" t="n">
         <ns0:v>37.2000000000001</ns0:v>
@@ -6842,15 +6842,15 @@
       </ns0:c>
       <ns0:c r="D186" s="1">
         <ns0:f>ROUND(D185*20,2-INT(LOG10(ABS(D185*20))))</ns0:f>
-        <ns0:v>1.1999999999999999e+213</ns0:v>
+        <ns0:v>1.7e+213</ns0:v>
       </ns0:c>
       <ns0:c r="E186" s="1">
         <ns0:f>D186</ns0:f>
-        <ns0:v>1.1999999999999999e+213</ns0:v>
+        <ns0:v>1.7e+213</ns0:v>
       </ns0:c>
       <ns0:c r="F186" s="1">
         <ns0:f>ROUND(F185*1.4,-5)</ns0:f>
-        <ns0:v>1.9011223696187096e+47</ns0:v>
+        <ns0:v>2.851683554428066e+47</ns0:v>
       </ns0:c>
       <ns0:c r="G186" s="1" t="n">
         <ns0:v>37.4000000000001</ns0:v>
@@ -6874,15 +6874,15 @@
       </ns0:c>
       <ns0:c r="D187" s="1">
         <ns0:f>ROUND(D186*20,2-INT(LOG10(ABS(D186*20))))</ns0:f>
-        <ns0:v>2.4e+214</ns0:v>
+        <ns0:v>3.4000000000000003e+214</ns0:v>
       </ns0:c>
       <ns0:c r="E187" s="1">
         <ns0:f>D187</ns0:f>
-        <ns0:v>2.4e+214</ns0:v>
+        <ns0:v>3.4000000000000003e+214</ns0:v>
       </ns0:c>
       <ns0:c r="F187" s="1">
         <ns0:f>ROUND(F186*1.4,-5)</ns0:f>
-        <ns0:v>2.661571317466193e+47</ns0:v>
+        <ns0:v>3.992356976199292e+47</ns0:v>
       </ns0:c>
       <ns0:c r="G187" s="1" t="n">
         <ns0:v>37.6000000000001</ns0:v>
@@ -6906,15 +6906,15 @@
       </ns0:c>
       <ns0:c r="D188" s="1">
         <ns0:f>ROUND(D187*20,2-INT(LOG10(ABS(D187*20))))</ns0:f>
-        <ns0:v>4.8e+215</ns0:v>
+        <ns0:v>6.8e+215</ns0:v>
       </ns0:c>
       <ns0:c r="E188" s="1">
         <ns0:f>D188</ns0:f>
-        <ns0:v>4.8e+215</ns0:v>
+        <ns0:v>6.8e+215</ns0:v>
       </ns0:c>
       <ns0:c r="F188" s="1">
         <ns0:f>ROUND(F187*1.4,-5)</ns0:f>
-        <ns0:v>3.72619984445267e+47</ns0:v>
+        <ns0:v>5.589299766679009e+47</ns0:v>
       </ns0:c>
       <ns0:c r="G188" s="1" t="n">
         <ns0:v>37.8000000000001</ns0:v>
@@ -6938,15 +6938,15 @@
       </ns0:c>
       <ns0:c r="D189" s="1">
         <ns0:f>ROUND(D188*20,2-INT(LOG10(ABS(D188*20))))</ns0:f>
-        <ns0:v>9.600000000000001e+216</ns0:v>
+        <ns0:v>1.3599999999999999e+217</ns0:v>
       </ns0:c>
       <ns0:c r="E189" s="1">
         <ns0:f>D189</ns0:f>
-        <ns0:v>9.600000000000001e+216</ns0:v>
+        <ns0:v>1.3599999999999999e+217</ns0:v>
       </ns0:c>
       <ns0:c r="F189" s="1">
         <ns0:f>ROUND(F188*1.4,-5)</ns0:f>
-        <ns0:v>5.216679782233738e+47</ns0:v>
+        <ns0:v>7.825019673350611e+47</ns0:v>
       </ns0:c>
       <ns0:c r="G189" s="1" t="n">
         <ns0:v>38.0000000000001</ns0:v>
@@ -6970,15 +6970,15 @@
       </ns0:c>
       <ns0:c r="D190" s="1">
         <ns0:f>ROUND(D189*20,2-INT(LOG10(ABS(D189*20))))</ns0:f>
-        <ns0:v>1.92e+218</ns0:v>
+        <ns0:v>2.72e+218</ns0:v>
       </ns0:c>
       <ns0:c r="E190" s="1">
         <ns0:f>D190</ns0:f>
-        <ns0:v>1.92e+218</ns0:v>
+        <ns0:v>2.72e+218</ns0:v>
       </ns0:c>
       <ns0:c r="F190" s="1">
         <ns0:f>ROUND(F189*1.4,-5)</ns0:f>
-        <ns0:v>7.3033516951272325e+47</ns0:v>
+        <ns0:v>1.0955027542690854e+48</ns0:v>
       </ns0:c>
       <ns0:c r="G190" s="1" t="n">
         <ns0:v>38.2000000000001</ns0:v>
@@ -7002,15 +7002,15 @@
       </ns0:c>
       <ns0:c r="D191" s="1">
         <ns0:f>ROUND(D190*20,2-INT(LOG10(ABS(D190*20))))</ns0:f>
-        <ns0:v>3.84e+219</ns0:v>
+        <ns0:v>5.4399999999999995e+219</ns0:v>
       </ns0:c>
       <ns0:c r="E191" s="1">
         <ns0:f>D191</ns0:f>
-        <ns0:v>3.84e+219</ns0:v>
+        <ns0:v>5.4399999999999995e+219</ns0:v>
       </ns0:c>
       <ns0:c r="F191" s="1">
         <ns0:f>ROUND(F190*1.4,-5)</ns0:f>
-        <ns0:v>1.0224692373178125e+48</ns0:v>
+        <ns0:v>1.5337038559767195e+48</ns0:v>
       </ns0:c>
       <ns0:c r="G191" s="1" t="n">
         <ns0:v>38.4000000000001</ns0:v>
@@ -7034,15 +7034,15 @@
       </ns0:c>
       <ns0:c r="D192" s="1">
         <ns0:f>ROUND(D191*20,2-INT(LOG10(ABS(D191*20))))</ns0:f>
-        <ns0:v>7.68e+220</ns0:v>
+        <ns0:v>1.09e+221</ns0:v>
       </ns0:c>
       <ns0:c r="E192" s="1">
         <ns0:f>D192</ns0:f>
-        <ns0:v>7.68e+220</ns0:v>
+        <ns0:v>1.09e+221</ns0:v>
       </ns0:c>
       <ns0:c r="F192" s="1">
         <ns0:f>ROUND(F191*1.4,-5)</ns0:f>
-        <ns0:v>1.4314569322449375e+48</ns0:v>
+        <ns0:v>2.147185398367407e+48</ns0:v>
       </ns0:c>
       <ns0:c r="G192" s="1" t="n">
         <ns0:v>38.6000000000001</ns0:v>
@@ -7066,15 +7066,15 @@
       </ns0:c>
       <ns0:c r="D193" s="1">
         <ns0:f>ROUND(D192*20,2-INT(LOG10(ABS(D192*20))))</ns0:f>
-        <ns0:v>1.54e+222</ns0:v>
+        <ns0:v>2.18e+222</ns0:v>
       </ns0:c>
       <ns0:c r="E193" s="1">
         <ns0:f>D193</ns0:f>
-        <ns0:v>1.54e+222</ns0:v>
+        <ns0:v>2.18e+222</ns0:v>
       </ns0:c>
       <ns0:c r="F193" s="1">
         <ns0:f>ROUND(F192*1.4,-5)</ns0:f>
-        <ns0:v>2.0040397051429124e+48</ns0:v>
+        <ns0:v>3.00605955771437e+48</ns0:v>
       </ns0:c>
       <ns0:c r="G193" s="1" t="n">
         <ns0:v>38.8000000000001</ns0:v>
@@ -7098,15 +7098,15 @@
       </ns0:c>
       <ns0:c r="D194" s="1">
         <ns0:f>ROUND(D193*20,2-INT(LOG10(ABS(D193*20))))</ns0:f>
-        <ns0:v>3.08e+223</ns0:v>
+        <ns0:v>4.36e+223</ns0:v>
       </ns0:c>
       <ns0:c r="E194" s="1">
         <ns0:f>D194</ns0:f>
-        <ns0:v>3.08e+223</ns0:v>
+        <ns0:v>4.36e+223</ns0:v>
       </ns0:c>
       <ns0:c r="F194" s="1">
         <ns0:f>ROUND(F193*1.4,-5)</ns0:f>
-        <ns0:v>2.8056555872000773e+48</ns0:v>
+        <ns0:v>4.208483380800117e+48</ns0:v>
       </ns0:c>
       <ns0:c r="G194" s="1" t="n">
         <ns0:v>39.0000000000001</ns0:v>
@@ -7130,15 +7130,15 @@
       </ns0:c>
       <ns0:c r="D195" s="1">
         <ns0:f>ROUND(D194*20,2-INT(LOG10(ABS(D194*20))))</ns0:f>
-        <ns0:v>6.16e+224</ns0:v>
+        <ns0:v>8.72e+224</ns0:v>
       </ns0:c>
       <ns0:c r="E195" s="1">
         <ns0:f>D195</ns0:f>
-        <ns0:v>6.16e+224</ns0:v>
+        <ns0:v>8.72e+224</ns0:v>
       </ns0:c>
       <ns0:c r="F195" s="1">
         <ns0:f>ROUND(F194*1.4,-5)</ns0:f>
-        <ns0:v>3.927917822080108e+48</ns0:v>
+        <ns0:v>5.891876733120163e+48</ns0:v>
       </ns0:c>
       <ns0:c r="G195" s="1" t="n">
         <ns0:v>39.2000000000001</ns0:v>
@@ -7162,15 +7162,15 @@
       </ns0:c>
       <ns0:c r="D196" s="1">
         <ns0:f>ROUND(D195*20,2-INT(LOG10(ABS(D195*20))))</ns0:f>
-        <ns0:v>1.23e+226</ns0:v>
+        <ns0:v>1.74e+226</ns0:v>
       </ns0:c>
       <ns0:c r="E196" s="1">
         <ns0:f>D196</ns0:f>
-        <ns0:v>1.23e+226</ns0:v>
+        <ns0:v>1.74e+226</ns0:v>
       </ns0:c>
       <ns0:c r="F196" s="1">
         <ns0:f>ROUND(F195*1.4,-5)</ns0:f>
-        <ns0:v>5.49908495091215e+48</ns0:v>
+        <ns0:v>8.248627426368228e+48</ns0:v>
       </ns0:c>
       <ns0:c r="G196" s="1" t="n">
         <ns0:v>39.4000000000001</ns0:v>
@@ -7194,15 +7194,15 @@
       </ns0:c>
       <ns0:c r="D197" s="1">
         <ns0:f>ROUND(D196*20,2-INT(LOG10(ABS(D196*20))))</ns0:f>
-        <ns0:v>2.4600000000000002e+227</ns0:v>
+        <ns0:v>3.4800000000000003e+227</ns0:v>
       </ns0:c>
       <ns0:c r="E197" s="1">
         <ns0:f>D197</ns0:f>
-        <ns0:v>2.4600000000000002e+227</ns0:v>
+        <ns0:v>3.4800000000000003e+227</ns0:v>
       </ns0:c>
       <ns0:c r="F197" s="1">
         <ns0:f>ROUND(F196*1.4,-5)</ns0:f>
-        <ns0:v>7.698718931277009e+48</ns0:v>
+        <ns0:v>1.1548078396915519e+49</ns0:v>
       </ns0:c>
       <ns0:c r="G197" s="1" t="n">
         <ns0:v>39.6000000000001</ns0:v>
@@ -7226,15 +7226,15 @@
       </ns0:c>
       <ns0:c r="D198" s="1">
         <ns0:f>ROUND(D197*20,2-INT(LOG10(ABS(D197*20))))</ns0:f>
-        <ns0:v>4.92e+228</ns0:v>
+        <ns0:v>6.96e+228</ns0:v>
       </ns0:c>
       <ns0:c r="E198" s="1">
         <ns0:f>D198</ns0:f>
-        <ns0:v>4.92e+228</ns0:v>
+        <ns0:v>6.96e+228</ns0:v>
       </ns0:c>
       <ns0:c r="F198" s="1">
         <ns0:f>ROUND(F197*1.4,-5)</ns0:f>
-        <ns0:v>1.0778206503787812e+49</ns0:v>
+        <ns0:v>1.6167309755681725e+49</ns0:v>
       </ns0:c>
       <ns0:c r="G198" s="1" t="n">
         <ns0:v>39.8000000000001</ns0:v>
@@ -7258,15 +7258,15 @@
       </ns0:c>
       <ns0:c r="D199" s="1">
         <ns0:f>ROUND(D198*20,2-INT(LOG10(ABS(D198*20))))</ns0:f>
-        <ns0:v>9.84e+229</ns0:v>
+        <ns0:v>1.3899999999999999e+230</ns0:v>
       </ns0:c>
       <ns0:c r="E199" s="1">
         <ns0:f>D199</ns0:f>
-        <ns0:v>9.84e+229</ns0:v>
+        <ns0:v>1.3899999999999999e+230</ns0:v>
       </ns0:c>
       <ns0:c r="F199" s="1">
         <ns0:f>ROUND(F198*1.4,-5)</ns0:f>
-        <ns0:v>1.5089489105302936e+49</ns0:v>
+        <ns0:v>2.2634233657954413e+49</ns0:v>
       </ns0:c>
       <ns0:c r="G199" s="1" t="n">
         <ns0:v>40.0000000000001</ns0:v>
@@ -7290,15 +7290,15 @@
       </ns0:c>
       <ns0:c r="D200" s="1">
         <ns0:f>ROUND(D199*20,2-INT(LOG10(ABS(D199*20))))</ns0:f>
-        <ns0:v>1.97e+231</ns0:v>
+        <ns0:v>2.7799999999999997e+231</ns0:v>
       </ns0:c>
       <ns0:c r="E200" s="1">
         <ns0:f>D200</ns0:f>
-        <ns0:v>1.97e+231</ns0:v>
+        <ns0:v>2.7799999999999997e+231</ns0:v>
       </ns0:c>
       <ns0:c r="F200" s="1">
         <ns0:f>ROUND(F199*1.4,-5)</ns0:f>
-        <ns0:v>2.112528474742411e+49</ns0:v>
+        <ns0:v>3.1687927121136177e+49</ns0:v>
       </ns0:c>
       <ns0:c r="G200" s="1" t="n">
         <ns0:v>40.2000000000001</ns0:v>
@@ -7322,15 +7322,15 @@
       </ns0:c>
       <ns0:c r="D201" s="1">
         <ns0:f>ROUND(D200*20,2-INT(LOG10(ABS(D200*20))))</ns0:f>
-        <ns0:v>3.94e+232</ns0:v>
+        <ns0:v>5.56e+232</ns0:v>
       </ns0:c>
       <ns0:c r="E201" s="1">
         <ns0:f>D201</ns0:f>
-        <ns0:v>3.94e+232</ns0:v>
+        <ns0:v>5.56e+232</ns0:v>
       </ns0:c>
       <ns0:c r="F201" s="1">
         <ns0:f>ROUND(F200*1.4,-5)</ns0:f>
-        <ns0:v>2.957539864639375e+49</ns0:v>
+        <ns0:v>4.4363097969590647e+49</ns0:v>
       </ns0:c>
       <ns0:c r="G201" s="1" t="n">
         <ns0:v>40.4000000000001</ns0:v>
@@ -7354,15 +7354,15 @@
       </ns0:c>
       <ns0:c r="D202" s="1">
         <ns0:f>ROUND(D201*20,2-INT(LOG10(ABS(D201*20))))</ns0:f>
-        <ns0:v>7.8800000000000005e+233</ns0:v>
+        <ns0:v>1.11e+234</ns0:v>
       </ns0:c>
       <ns0:c r="E202" s="1">
         <ns0:f>D202</ns0:f>
-        <ns0:v>7.8800000000000005e+233</ns0:v>
+        <ns0:v>1.11e+234</ns0:v>
       </ns0:c>
       <ns0:c r="F202" s="1">
         <ns0:f>ROUND(F201*1.4,-5)</ns0:f>
-        <ns0:v>4.1405558104951243e+49</ns0:v>
+        <ns0:v>6.21083371574269e+49</ns0:v>
       </ns0:c>
       <ns0:c r="G202" s="1" t="n">
         <ns0:v>40.6000000000001</ns0:v>
@@ -7386,15 +7386,15 @@
       </ns0:c>
       <ns0:c r="D203" s="1">
         <ns0:f>ROUND(D202*20,2-INT(LOG10(ABS(D202*20))))</ns0:f>
-        <ns0:v>1.58e+235</ns0:v>
+        <ns0:v>2.2200000000000002e+235</ns0:v>
       </ns0:c>
       <ns0:c r="E203" s="1">
         <ns0:f>D203</ns0:f>
-        <ns0:v>1.58e+235</ns0:v>
+        <ns0:v>2.2200000000000002e+235</ns0:v>
       </ns0:c>
       <ns0:c r="F203" s="1">
         <ns0:f>ROUND(F202*1.4,-5)</ns0:f>
-        <ns0:v>5.796778134693173e+49</ns0:v>
+        <ns0:v>8.695167202039765e+49</ns0:v>
       </ns0:c>
       <ns0:c r="G203" s="1" t="n">
         <ns0:v>40.8000000000001</ns0:v>
@@ -7418,15 +7418,15 @@
       </ns0:c>
       <ns0:c r="D204" s="1">
         <ns0:f>ROUND(D203*20,2-INT(LOG10(ABS(D203*20))))</ns0:f>
-        <ns0:v>3.16e+236</ns0:v>
+        <ns0:v>4.44e+236</ns0:v>
       </ns0:c>
       <ns0:c r="E204" s="1">
         <ns0:f>D204</ns0:f>
-        <ns0:v>3.16e+236</ns0:v>
+        <ns0:v>4.44e+236</ns0:v>
       </ns0:c>
       <ns0:c r="F204" s="1">
         <ns0:f>ROUND(F203*1.4,-5)</ns0:f>
-        <ns0:v>8.115489388570442e+49</ns0:v>
+        <ns0:v>1.217323408285567e+50</ns0:v>
       </ns0:c>
       <ns0:c r="G204" s="1" t="n">
         <ns0:v>41.0000000000001</ns0:v>
@@ -7450,15 +7450,15 @@
       </ns0:c>
       <ns0:c r="D205" s="1">
         <ns0:f>ROUND(D204*20,2-INT(LOG10(ABS(D204*20))))</ns0:f>
-        <ns0:v>6.3200000000000006e+237</ns0:v>
+        <ns0:v>8.88e+237</ns0:v>
       </ns0:c>
       <ns0:c r="E205" s="1">
         <ns0:f>D205</ns0:f>
-        <ns0:v>6.3200000000000006e+237</ns0:v>
+        <ns0:v>8.88e+237</ns0:v>
       </ns0:c>
       <ns0:c r="F205" s="1">
         <ns0:f>ROUND(F204*1.4,-5)</ns0:f>
-        <ns0:v>1.136168514399862e+50</ns0:v>
+        <ns0:v>1.7042527715997939e+50</ns0:v>
       </ns0:c>
       <ns0:c r="G205" s="1" t="n">
         <ns0:v>41.2000000000001</ns0:v>
@@ -7482,15 +7482,15 @@
       </ns0:c>
       <ns0:c r="D206" s="1">
         <ns0:f>ROUND(D205*20,2-INT(LOG10(ABS(D205*20))))</ns0:f>
-        <ns0:v>1.26e+239</ns0:v>
+        <ns0:v>1.78e+239</ns0:v>
       </ns0:c>
       <ns0:c r="E206" s="1">
         <ns0:f>D206</ns0:f>
-        <ns0:v>1.26e+239</ns0:v>
+        <ns0:v>1.78e+239</ns0:v>
       </ns0:c>
       <ns0:c r="F206" s="1">
         <ns0:f>ROUND(F205*1.4,-5)</ns0:f>
-        <ns0:v>1.5906359201598066e+50</ns0:v>
+        <ns0:v>2.3859538802397113e+50</ns0:v>
       </ns0:c>
       <ns0:c r="G206" s="1" t="n">
         <ns0:v>41.4000000000001</ns0:v>
@@ -7514,15 +7514,15 @@
       </ns0:c>
       <ns0:c r="D207" s="1">
         <ns0:f>ROUND(D206*20,2-INT(LOG10(ABS(D206*20))))</ns0:f>
-        <ns0:v>2.52e+240</ns0:v>
+        <ns0:v>3.56e+240</ns0:v>
       </ns0:c>
       <ns0:c r="E207" s="1">
         <ns0:f>D207</ns0:f>
-        <ns0:v>2.52e+240</ns0:v>
+        <ns0:v>3.56e+240</ns0:v>
       </ns0:c>
       <ns0:c r="F207" s="1">
         <ns0:f>ROUND(F206*1.4,-5)</ns0:f>
-        <ns0:v>2.226890288223729e+50</ns0:v>
+        <ns0:v>3.3403354323355957e+50</ns0:v>
       </ns0:c>
       <ns0:c r="G207" s="1" t="n">
         <ns0:v>41.6000000000001</ns0:v>
@@ -7546,15 +7546,15 @@
       </ns0:c>
       <ns0:c r="D208" s="1">
         <ns0:f>ROUND(D207*20,2-INT(LOG10(ABS(D207*20))))</ns0:f>
-        <ns0:v>5.04e+241</ns0:v>
+        <ns0:v>7.12e+241</ns0:v>
       </ns0:c>
       <ns0:c r="E208" s="1">
         <ns0:f>D208</ns0:f>
-        <ns0:v>5.04e+241</ns0:v>
+        <ns0:v>7.12e+241</ns0:v>
       </ns0:c>
       <ns0:c r="F208" s="1">
         <ns0:f>ROUND(F207*1.4,-5)</ns0:f>
-        <ns0:v>3.117646403513221e+50</ns0:v>
+        <ns0:v>4.676469605269834e+50</ns0:v>
       </ns0:c>
       <ns0:c r="G208" s="1" t="n">
         <ns0:v>41.8000000000001</ns0:v>
@@ -7578,15 +7578,15 @@
       </ns0:c>
       <ns0:c r="D209" s="1">
         <ns0:f>ROUND(D208*20,2-INT(LOG10(ABS(D208*20))))</ns0:f>
-        <ns0:v>1.01e+243</ns0:v>
+        <ns0:v>1.42e+243</ns0:v>
       </ns0:c>
       <ns0:c r="E209" s="1">
         <ns0:f>D209</ns0:f>
-        <ns0:v>1.01e+243</ns0:v>
+        <ns0:v>1.42e+243</ns0:v>
       </ns0:c>
       <ns0:c r="F209" s="1">
         <ns0:f>ROUND(F208*1.4,-5)</ns0:f>
-        <ns0:v>4.3647049649185085e+50</ns0:v>
+        <ns0:v>6.547057447377766e+50</ns0:v>
       </ns0:c>
       <ns0:c r="G209" s="1" t="n">
         <ns0:v>42.0000000000001</ns0:v>
@@ -7610,15 +7610,15 @@
       </ns0:c>
       <ns0:c r="D210" s="1">
         <ns0:f>ROUND(D209*20,2-INT(LOG10(ABS(D209*20))))</ns0:f>
-        <ns0:v>2.02e+244</ns0:v>
+        <ns0:v>2.84e+244</ns0:v>
       </ns0:c>
       <ns0:c r="E210" s="1">
         <ns0:f>D210</ns0:f>
-        <ns0:v>2.02e+244</ns0:v>
+        <ns0:v>2.84e+244</ns0:v>
       </ns0:c>
       <ns0:c r="F210" s="1">
         <ns0:f>ROUND(F209*1.4,-5)</ns0:f>
-        <ns0:v>6.110586950885911e+50</ns0:v>
+        <ns0:v>9.165880426328873e+50</ns0:v>
       </ns0:c>
       <ns0:c r="G210" s="1" t="n">
         <ns0:v>42.2000000000001</ns0:v>
@@ -7642,15 +7642,15 @@
       </ns0:c>
       <ns0:c r="D211" s="1">
         <ns0:f>ROUND(D210*20,2-INT(LOG10(ABS(D210*20))))</ns0:f>
-        <ns0:v>4.04e+245</ns0:v>
+        <ns0:v>5.68e+245</ns0:v>
       </ns0:c>
       <ns0:c r="E211" s="1">
         <ns0:f>D211</ns0:f>
-        <ns0:v>4.04e+245</ns0:v>
+        <ns0:v>5.68e+245</ns0:v>
       </ns0:c>
       <ns0:c r="F211" s="1">
         <ns0:f>ROUND(F210*1.4,-5)</ns0:f>
-        <ns0:v>8.554821731240276e+50</ns0:v>
+        <ns0:v>1.2832232596860421e+51</ns0:v>
       </ns0:c>
       <ns0:c r="G211" s="1" t="n">
         <ns0:v>42.4000000000001</ns0:v>
@@ -7674,15 +7674,15 @@
       </ns0:c>
       <ns0:c r="D212" s="1">
         <ns0:f>ROUND(D211*20,2-INT(LOG10(ABS(D211*20))))</ns0:f>
-        <ns0:v>8.08e+246</ns0:v>
+        <ns0:v>1.14e+247</ns0:v>
       </ns0:c>
       <ns0:c r="E212" s="1">
         <ns0:f>D212</ns0:f>
-        <ns0:v>8.08e+246</ns0:v>
+        <ns0:v>1.14e+247</ns0:v>
       </ns0:c>
       <ns0:c r="F212" s="1">
         <ns0:f>ROUND(F211*1.4,-5)</ns0:f>
-        <ns0:v>1.1976750423736385e+51</ns0:v>
+        <ns0:v>1.796512563560459e+51</ns0:v>
       </ns0:c>
       <ns0:c r="G212" s="1" t="n">
         <ns0:v>42.6000000000002</ns0:v>
@@ -7706,15 +7706,15 @@
       </ns0:c>
       <ns0:c r="D213" s="1">
         <ns0:f>ROUND(D212*20,2-INT(LOG10(ABS(D212*20))))</ns0:f>
-        <ns0:v>1.6200000000000001e+248</ns0:v>
+        <ns0:v>2.2800000000000003e+248</ns0:v>
       </ns0:c>
       <ns0:c r="E213" s="1">
         <ns0:f>D213</ns0:f>
-        <ns0:v>1.6200000000000001e+248</ns0:v>
+        <ns0:v>2.2800000000000003e+248</ns0:v>
       </ns0:c>
       <ns0:c r="F213" s="1">
         <ns0:f>ROUND(F212*1.4,-5)</ns0:f>
-        <ns0:v>1.6767450593230938e+51</ns0:v>
+        <ns0:v>2.5151175889846427e+51</ns0:v>
       </ns0:c>
       <ns0:c r="G213" s="1" t="n">
         <ns0:v>42.8000000000002</ns0:v>
@@ -7738,15 +7738,15 @@
       </ns0:c>
       <ns0:c r="D214" s="1">
         <ns0:f>ROUND(D213*20,2-INT(LOG10(ABS(D213*20))))</ns0:f>
-        <ns0:v>3.24e+249</ns0:v>
+        <ns0:v>4.56e+249</ns0:v>
       </ns0:c>
       <ns0:c r="E214" s="1">
         <ns0:f>D214</ns0:f>
-        <ns0:v>3.24e+249</ns0:v>
+        <ns0:v>4.56e+249</ns0:v>
       </ns0:c>
       <ns0:c r="F214" s="1">
         <ns0:f>ROUND(F213*1.4,-5)</ns0:f>
-        <ns0:v>2.347443083052331e+51</ns0:v>
+        <ns0:v>3.5211646245784995e+51</ns0:v>
       </ns0:c>
       <ns0:c r="G214" s="1" t="n">
         <ns0:v>43.0000000000001</ns0:v>
@@ -7770,15 +7770,15 @@
       </ns0:c>
       <ns0:c r="D215" s="1">
         <ns0:f>ROUND(D214*20,2-INT(LOG10(ABS(D214*20))))</ns0:f>
-        <ns0:v>6.480000000000001e+250</ns0:v>
+        <ns0:v>9.12e+250</ns0:v>
       </ns0:c>
       <ns0:c r="E215" s="1">
         <ns0:f>D215</ns0:f>
-        <ns0:v>6.480000000000001e+250</ns0:v>
+        <ns0:v>9.12e+250</ns0:v>
       </ns0:c>
       <ns0:c r="F215" s="1">
         <ns0:f>ROUND(F214*1.4,-5)</ns0:f>
-        <ns0:v>3.286420316273263e+51</ns0:v>
+        <ns0:v>4.929630474409899e+51</ns0:v>
       </ns0:c>
       <ns0:c r="G215" s="1" t="n">
         <ns0:v>43.2000000000002</ns0:v>
@@ -7802,15 +7802,15 @@
       </ns0:c>
       <ns0:c r="D216" s="1">
         <ns0:f>ROUND(D215*20,2-INT(LOG10(ABS(D215*20))))</ns0:f>
-        <ns0:v>1.2999999999999999e+252</ns0:v>
+        <ns0:v>1.82e+252</ns0:v>
       </ns0:c>
       <ns0:c r="E216" s="1">
         <ns0:f>D216</ns0:f>
-        <ns0:v>1.2999999999999999e+252</ns0:v>
+        <ns0:v>1.82e+252</ns0:v>
       </ns0:c>
       <ns0:c r="F216" s="1">
         <ns0:f>ROUND(F215*1.4,-5)</ns0:f>
-        <ns0:v>4.600988442782569e+51</ns0:v>
+        <ns0:v>6.901482664173858e+51</ns0:v>
       </ns0:c>
       <ns0:c r="G216" s="1" t="n">
         <ns0:v>43.4000000000002</ns0:v>
@@ -7834,15 +7834,15 @@
       </ns0:c>
       <ns0:c r="D217" s="1">
         <ns0:f>ROUND(D216*20,2-INT(LOG10(ABS(D216*20))))</ns0:f>
-        <ns0:v>2.6e+253</ns0:v>
+        <ns0:v>3.64e+253</ns0:v>
       </ns0:c>
       <ns0:c r="E217" s="1">
         <ns0:f>D217</ns0:f>
-        <ns0:v>2.6e+253</ns0:v>
+        <ns0:v>3.64e+253</ns0:v>
       </ns0:c>
       <ns0:c r="F217" s="1">
         <ns0:f>ROUND(F216*1.4,-5)</ns0:f>
-        <ns0:v>6.441383819895597e+51</ns0:v>
+        <ns0:v>9.6620757298434e+51</ns0:v>
       </ns0:c>
       <ns0:c r="G217" s="1" t="n">
         <ns0:v>43.6000000000002</ns0:v>
@@ -7866,15 +7866,15 @@
       </ns0:c>
       <ns0:c r="D218" s="1">
         <ns0:f>ROUND(D217*20,2-INT(LOG10(ABS(D217*20))))</ns0:f>
-        <ns0:v>5.2e+254</ns0:v>
+        <ns0:v>7.28e+254</ns0:v>
       </ns0:c>
       <ns0:c r="E218" s="1">
         <ns0:f>D218</ns0:f>
-        <ns0:v>5.2e+254</ns0:v>
+        <ns0:v>7.28e+254</ns0:v>
       </ns0:c>
       <ns0:c r="F218" s="1">
         <ns0:f>ROUND(F217*1.4,-5)</ns0:f>
-        <ns0:v>9.017937347853835e+51</ns0:v>
+        <ns0:v>1.352690602178076e+52</ns0:v>
       </ns0:c>
       <ns0:c r="G218" s="1" t="n">
         <ns0:v>43.8000000000002</ns0:v>
@@ -7898,15 +7898,15 @@
       </ns0:c>
       <ns0:c r="D219" s="1">
         <ns0:f>ROUND(D218*20,2-INT(LOG10(ABS(D218*20))))</ns0:f>
-        <ns0:v>1.04e+256</ns0:v>
+        <ns0:v>1.4600000000000002e+256</ns0:v>
       </ns0:c>
       <ns0:c r="E219" s="1">
         <ns0:f>D219</ns0:f>
-        <ns0:v>1.04e+256</ns0:v>
+        <ns0:v>1.4600000000000002e+256</ns0:v>
       </ns0:c>
       <ns0:c r="F219" s="1">
         <ns0:f>ROUND(F218*1.4,-5)</ns0:f>
-        <ns0:v>1.2625112286995368e+52</ns0:v>
+        <ns0:v>1.8937668430493063e+52</ns0:v>
       </ns0:c>
       <ns0:c r="G219" s="1" t="n">
         <ns0:v>44.0000000000002</ns0:v>
@@ -7930,15 +7930,15 @@
       </ns0:c>
       <ns0:c r="D220" s="1">
         <ns0:f>ROUND(D219*20,2-INT(LOG10(ABS(D219*20))))</ns0:f>
-        <ns0:v>2.08e+257</ns0:v>
+        <ns0:v>2.92e+257</ns0:v>
       </ns0:c>
       <ns0:c r="E220" s="1">
         <ns0:f>D220</ns0:f>
-        <ns0:v>2.08e+257</ns0:v>
+        <ns0:v>2.92e+257</ns0:v>
       </ns0:c>
       <ns0:c r="F220" s="1">
         <ns0:f>ROUND(F219*1.4,-5)</ns0:f>
-        <ns0:v>1.7675157201793514e+52</ns0:v>
+        <ns0:v>2.6512735802690286e+52</ns0:v>
       </ns0:c>
       <ns0:c r="G220" s="1" t="n">
         <ns0:v>44.2000000000002</ns0:v>
@@ -7962,15 +7962,15 @@
       </ns0:c>
       <ns0:c r="D221" s="1">
         <ns0:f>ROUND(D220*20,2-INT(LOG10(ABS(D220*20))))</ns0:f>
-        <ns0:v>4.16e+258</ns0:v>
+        <ns0:v>5.84e+258</ns0:v>
       </ns0:c>
       <ns0:c r="E221" s="1">
         <ns0:f>D221</ns0:f>
-        <ns0:v>4.16e+258</ns0:v>
+        <ns0:v>5.84e+258</ns0:v>
       </ns0:c>
       <ns0:c r="F221" s="1">
         <ns0:f>ROUND(F220*1.4,-5)</ns0:f>
-        <ns0:v>2.474522008251092e+52</ns0:v>
+        <ns0:v>3.71178301237664e+52</ns0:v>
       </ns0:c>
       <ns0:c r="G221" s="1" t="n">
         <ns0:v>44.4000000000002</ns0:v>
@@ -7994,15 +7994,15 @@
       </ns0:c>
       <ns0:c r="D222" s="1">
         <ns0:f>ROUND(D221*20,2-INT(LOG10(ABS(D221*20))))</ns0:f>
-        <ns0:v>8.32e+259</ns0:v>
+        <ns0:v>1.17e+260</ns0:v>
       </ns0:c>
       <ns0:c r="E222" s="1">
         <ns0:f>D222</ns0:f>
-        <ns0:v>8.32e+259</ns0:v>
+        <ns0:v>1.17e+260</ns0:v>
       </ns0:c>
       <ns0:c r="F222" s="1">
         <ns0:f>ROUND(F221*1.4,-5)</ns0:f>
-        <ns0:v>3.4643308115515286e+52</ns0:v>
+        <ns0:v>5.196496217327296e+52</ns0:v>
       </ns0:c>
       <ns0:c r="G222" s="1" t="n">
         <ns0:v>44.6000000000002</ns0:v>
@@ -8026,15 +8026,15 @@
       </ns0:c>
       <ns0:c r="D223" s="1">
         <ns0:f>ROUND(D222*20,2-INT(LOG10(ABS(D222*20))))</ns0:f>
-        <ns0:v>1.6599999999999999e+261</ns0:v>
+        <ns0:v>2.34e+261</ns0:v>
       </ns0:c>
       <ns0:c r="E223" s="1">
         <ns0:f>D223</ns0:f>
-        <ns0:v>1.6599999999999999e+261</ns0:v>
+        <ns0:v>2.34e+261</ns0:v>
       </ns0:c>
       <ns0:c r="F223" s="1">
         <ns0:f>ROUND(F222*1.4,-5)</ns0:f>
-        <ns0:v>4.85006313617214e+52</ns0:v>
+        <ns0:v>7.275094704258214e+52</ns0:v>
       </ns0:c>
       <ns0:c r="G223" s="1" t="n">
         <ns0:v>44.8000000000002</ns0:v>

</xml_diff>

<commit_message>
Tune only stage-one life and stage-two-to-ten drops through official workbook import
</commit_message>
<xml_diff>
--- a/space-battleship/config_excel/level.xlsx
+++ b/space-battleship/config_excel/level.xlsx
@@ -1270,7 +1270,7 @@
         <ns0:v>1</ns0:v>
       </ns0:c>
       <ns0:c r="E4" s="1" t="n">
-        <ns0:v>1</ns0:v>
+        <ns0:v>0.65</ns0:v>
       </ns0:c>
       <ns0:c r="F4" s="1" t="n">
         <ns0:v>1</ns0:v>
@@ -1301,7 +1301,7 @@
         <ns0:v>1.5</ns0:v>
       </ns0:c>
       <ns0:c r="F5" s="1" t="n">
-        <ns0:v>1.4</ns0:v>
+        <ns0:v>0.7</ns0:v>
       </ns0:c>
       <ns0:c r="G5" s="1" t="n">
         <ns0:v>1.2</ns0:v>
@@ -1329,7 +1329,7 @@
         <ns0:v>2</ns0:v>
       </ns0:c>
       <ns0:c r="F6" s="1" t="n">
-        <ns0:v>1.96</ns0:v>
+        <ns0:v>0.98</ns0:v>
       </ns0:c>
       <ns0:c r="G6" s="1" t="n">
         <ns0:v>1.4</ns0:v>
@@ -1357,7 +1357,7 @@
         <ns0:v>3</ns0:v>
       </ns0:c>
       <ns0:c r="F7" s="1" t="n">
-        <ns0:v>2.743999999999999</ns0:v>
+        <ns0:v>1.3719999999999994</ns0:v>
       </ns0:c>
       <ns0:c r="G7" s="1" t="n">
         <ns0:v>1.6</ns0:v>
@@ -1385,7 +1385,7 @@
         <ns0:v>4.5</ns0:v>
       </ns0:c>
       <ns0:c r="F8" s="1" t="n">
-        <ns0:v>5.762399999999999</ns0:v>
+        <ns0:v>2.8811999999999993</ns0:v>
       </ns0:c>
       <ns0:c r="G8" s="1" t="n">
         <ns0:v>1.8</ns0:v>
@@ -1413,7 +1413,7 @@
         <ns0:v>15.40702157458636</ns0:v>
       </ns0:c>
       <ns0:c r="F9" s="1" t="n">
-        <ns0:v>12</ns0:v>
+        <ns0:v>6.0</ns0:v>
       </ns0:c>
       <ns0:c r="G9" s="1" t="n">
         <ns0:v>2</ns0:v>
@@ -1441,7 +1441,7 @@
         <ns0:v>237.3763137997695</ns0:v>
       </ns0:c>
       <ns0:c r="F10" s="1" t="n">
-        <ns0:v>74.30083706879996</ns0:v>
+        <ns0:v>37.15041853439998</ns0:v>
       </ns0:c>
       <ns0:c r="G10" s="1" t="n">
         <ns0:v>2.2</ns0:v>
@@ -1469,7 +1469,7 @@
         <ns0:v>1469.771567969084</ns0:v>
       </ns0:c>
       <ns0:c r="F11" s="1" t="n">
-        <ns0:v>460.0511990936967</ns0:v>
+        <ns0:v>230.02559954684835</ns0:v>
       </ns0:c>
       <ns0:c r="G11" s="1" t="n">
         <ns0:v>2.4</ns0:v>
@@ -1497,7 +1497,7 @@
         <ns0:v>9100.438150002134</ns0:v>
       </ns0:c>
       <ns0:c r="F12" s="1" t="n">
-        <ns0:v>2848.515765597234</ns0:v>
+        <ns0:v>1424.257882798617</ns0:v>
       </ns0:c>
       <ns0:c r="G12" s="1" t="n">
         <ns0:v>2.6</ns0:v>
@@ -1525,7 +1525,7 @@
         <ns0:v>56347.51435316666</ns0:v>
       </ns0:c>
       <ns0:c r="F13" s="1" t="n">
-        <ns0:v>17637.25881562901</ns0:v>
+        <ns0:v>8818.629407814506</ns0:v>
       </ns0:c>
       <ns0:c r="G13" s="1" t="n">
         <ns0:v>2.8</ns0:v>

</xml_diff>

<commit_message>
balance: apply authorized candidate B early life and late resource ratios
</commit_message>
<xml_diff>
--- a/space-battleship/config_excel/level.xlsx
+++ b/space-battleship/config_excel/level.xlsx
@@ -1270,7 +1270,7 @@
         <ns0:v>1</ns0:v>
       </ns0:c>
       <ns0:c r="E4" s="1" t="n">
-        <ns0:v>0.65</ns0:v>
+        <ns0:v>.40</ns0:v>
       </ns0:c>
       <ns0:c r="F4" s="1" t="n">
         <ns0:v>1</ns0:v>
@@ -1298,7 +1298,7 @@
         <ns0:v>1.5</ns0:v>
       </ns0:c>
       <ns0:c r="E5" s="1" t="n">
-        <ns0:v>1.5</ns0:v>
+        <ns0:v>2.50</ns0:v>
       </ns0:c>
       <ns0:c r="F5" s="1" t="n">
         <ns0:v>0.7</ns0:v>
@@ -1326,7 +1326,7 @@
         <ns0:v>2</ns0:v>
       </ns0:c>
       <ns0:c r="E6" s="1" t="n">
-        <ns0:v>2</ns0:v>
+        <ns0:v>4.00</ns0:v>
       </ns0:c>
       <ns0:c r="F6" s="1" t="n">
         <ns0:v>0.98</ns0:v>
@@ -1354,7 +1354,7 @@
         <ns0:v>3</ns0:v>
       </ns0:c>
       <ns0:c r="E7" s="1" t="n">
-        <ns0:v>3</ns0:v>
+        <ns0:v>2.50</ns0:v>
       </ns0:c>
       <ns0:c r="F7" s="1" t="n">
         <ns0:v>1.3719999999999994</ns0:v>
@@ -1382,7 +1382,7 @@
         <ns0:v>4.5</ns0:v>
       </ns0:c>
       <ns0:c r="E8" s="1" t="n">
-        <ns0:v>4.5</ns0:v>
+        <ns0:v>6.50</ns0:v>
       </ns0:c>
       <ns0:c r="F8" s="1" t="n">
         <ns0:v>2.8811999999999993</ns0:v>
@@ -1469,7 +1469,7 @@
         <ns0:v>1469.771567969084</ns0:v>
       </ns0:c>
       <ns0:c r="F11" s="1" t="n">
-        <ns0:v>230.02559954684835</ns0:v>
+        <ns0:v>39.1043519229642195</ns0:v>
       </ns0:c>
       <ns0:c r="G11" s="1" t="n">
         <ns0:v>2.4</ns0:v>
@@ -1497,7 +1497,7 @@
         <ns0:v>9100.438150002134</ns0:v>
       </ns0:c>
       <ns0:c r="F12" s="1" t="n">
-        <ns0:v>1424.257882798617</ns0:v>
+        <ns0:v>242.12384007576489</ns0:v>
       </ns0:c>
       <ns0:c r="G12" s="1" t="n">
         <ns0:v>2.6</ns0:v>
@@ -1525,7 +1525,7 @@
         <ns0:v>56347.51435316666</ns0:v>
       </ns0:c>
       <ns0:c r="F13" s="1" t="n">
-        <ns0:v>8818.629407814506</ns0:v>
+        <ns0:v>1499.16699932846602</ns0:v>
       </ns0:c>
       <ns0:c r="G13" s="1" t="n">
         <ns0:v>2.8</ns0:v>

</xml_diff>

<commit_message>
balance: freeze candidate C with visible majority plans and safe farming from stage four
</commit_message>
<xml_diff>
--- a/space-battleship/config_excel/level.xlsx
+++ b/space-battleship/config_excel/level.xlsx
@@ -1298,7 +1298,7 @@
         <ns0:v>1.5</ns0:v>
       </ns0:c>
       <ns0:c r="E5" s="1" t="n">
-        <ns0:v>2.50</ns0:v>
+        <ns0:v>3.2</ns0:v>
       </ns0:c>
       <ns0:c r="F5" s="1" t="n">
         <ns0:v>0.7</ns0:v>
@@ -1382,7 +1382,7 @@
         <ns0:v>4.5</ns0:v>
       </ns0:c>
       <ns0:c r="E8" s="1" t="n">
-        <ns0:v>6.50</ns0:v>
+        <ns0:v>5.0</ns0:v>
       </ns0:c>
       <ns0:c r="F8" s="1" t="n">
         <ns0:v>2.8811999999999993</ns0:v>
@@ -1413,7 +1413,7 @@
         <ns0:v>15.40702157458636</ns0:v>
       </ns0:c>
       <ns0:c r="F9" s="1" t="n">
-        <ns0:v>6.0</ns0:v>
+        <ns0:v>3.600</ns0:v>
       </ns0:c>
       <ns0:c r="G9" s="1" t="n">
         <ns0:v>2</ns0:v>
@@ -1441,7 +1441,7 @@
         <ns0:v>237.3763137997695</ns0:v>
       </ns0:c>
       <ns0:c r="F10" s="1" t="n">
-        <ns0:v>37.15041853439998</ns0:v>
+        <ns0:v>22.2902511206399880</ns0:v>
       </ns0:c>
       <ns0:c r="G10" s="1" t="n">
         <ns0:v>2.2</ns0:v>
@@ -1469,7 +1469,7 @@
         <ns0:v>1469.771567969084</ns0:v>
       </ns0:c>
       <ns0:c r="F11" s="1" t="n">
-        <ns0:v>39.1043519229642195</ns0:v>
+        <ns0:v>23.462611153778531700</ns0:v>
       </ns0:c>
       <ns0:c r="G11" s="1" t="n">
         <ns0:v>2.4</ns0:v>
@@ -1497,7 +1497,7 @@
         <ns0:v>9100.438150002134</ns0:v>
       </ns0:c>
       <ns0:c r="F12" s="1" t="n">
-        <ns0:v>242.12384007576489</ns0:v>
+        <ns0:v>145.2743040454589340</ns0:v>
       </ns0:c>
       <ns0:c r="G12" s="1" t="n">
         <ns0:v>2.6</ns0:v>
@@ -1525,7 +1525,7 @@
         <ns0:v>56347.51435316666</ns0:v>
       </ns0:c>
       <ns0:c r="F13" s="1" t="n">
-        <ns0:v>1499.16699932846602</ns0:v>
+        <ns0:v>899.5001995970796120</ns0:v>
       </ns0:c>
       <ns0:c r="G13" s="1" t="n">
         <ns0:v>2.8</ns0:v>

</xml_diff>

<commit_message>
balance: taper midgame income and remove the extra sixfold stage21 reward jump
</commit_message>
<xml_diff>
--- a/space-battleship/config_excel/level.xlsx
+++ b/space-battleship/config_excel/level.xlsx
@@ -1553,7 +1553,7 @@
         <ns0:v>602880.1175788565</ns0:v>
       </ns0:c>
       <ns0:c r="F14" s="1" t="n">
-        <ns0:v>18870.66854784442</ns0:v>
+        <ns0:v>18120.833112711232</ns0:v>
       </ns0:c>
       <ns0:c r="G14" s="1" t="n">
         <ns0:v>3</ns0:v>
@@ -1581,7 +1581,7 @@
         <ns0:v>6450407.623907364</ns0:v>
       </ns0:c>
       <ns0:c r="F15" s="1" t="n">
-        <ns0:v>61725.60934115101</ns0:v>
+        <ns0:v>56917.67271450579</ns0:v>
       </ns0:c>
       <ns0:c r="G15" s="1" t="n">
         <ns0:v>3.2</ns0:v>
@@ -1609,7 +1609,7 @@
         <ns0:v>69014978.76834521</ns0:v>
       </ns0:c>
       <ns0:c r="F16" s="1" t="n">
-        <ns0:v>201903.3315579912</ns0:v>
+        <ns0:v>178778.836882676</ns0:v>
       </ns0:c>
       <ns0:c r="G16" s="1" t="n">
         <ns0:v>3.4</ns0:v>
@@ -1637,7 +1637,7 @@
         <ns0:v>738413379.7593849</ns0:v>
       </ns0:c>
       <ns0:c r="F17" s="1" t="n">
-        <ns0:v>660422.0797386132</ns0:v>
+        <ns0:v>561545.6675019113</ns0:v>
       </ns0:c>
       <ns0:c r="G17" s="1" t="n">
         <ns0:v>3.6</ns0:v>
@@ -1665,7 +1665,7 @@
         <ns0:v>7900521439.525051</ns0:v>
       </ns0:c>
       <ns0:c r="F18" s="1" t="n">
-        <ns0:v>2160228.462010301</ns0:v>
+        <ns0:v>1763819.1532541711</ns0:v>
       </ns0:c>
       <ns0:c r="G18" s="1" t="n">
         <ns0:v>3.8</ns0:v>
@@ -1693,7 +1693,7 @@
         <ns0:v>84530211298.0865</ns0:v>
       </ns0:c>
       <ns0:c r="F19" s="1" t="n">
-        <ns0:v>7066067.521434727</ns0:v>
+        <ns0:v>5540169.189134865</ns0:v>
       </ns0:c>
       <ns0:c r="G19" s="1" t="n">
         <ns0:v>4</ns0:v>
@@ -1721,7 +1721,7 @@
         <ns0:v>904415825815.2517</ns0:v>
       </ns0:c>
       <ns0:c r="F20" s="1" t="n">
-        <ns0:v>23112976.75015849</ns0:v>
+        <ns0:v>17401712.974718027</ns0:v>
       </ns0:c>
       <ns0:c r="G20" s="1" t="n">
         <ns0:v>4.2</ns0:v>
@@ -1749,7 +1749,7 @@
         <ns0:v>9676634819953.418</ns0:v>
       </ns0:c>
       <ns0:c r="F21" s="1" t="n">
-        <ns0:v>75602121.35432556</ns0:v>
+        <ns0:v>54658910.967619196</ns0:v>
       </ns0:c>
       <ns0:c r="G21" s="1" t="n">
         <ns0:v>4.4</ns0:v>
@@ -1777,7 +1777,7 @@
         <ns0:v>103533417666955.5</ns0:v>
       </ns0:c>
       <ns0:c r="F22" s="1" t="n">
-        <ns0:v>247293146.8351422</ns0:v>
+        <ns0:v>171684049.29483864</ns0:v>
       </ns0:c>
       <ns0:c r="G22" s="1" t="n">
         <ns0:v>4.6</ns0:v>
@@ -1805,7 +1805,7 @@
         <ns0:v>1107737222003781</ns0:v>
       </ns0:c>
       <ns0:c r="F23" s="1" t="n">
-        <ns0:v>808891329.7156876</ns0:v>
+        <ns0:v>539260886.477125</ns0:v>
       </ns0:c>
       <ns0:c r="G23" s="1" t="n">
         <ns0:v>4.8</ns0:v>
@@ -1833,7 +1833,7 @@
         <ns0:v>4763067294395140</ns0:v>
       </ns0:c>
       <ns0:c r="F24" s="1" t="n">
-        <ns0:v>20868507949.85079</ns0:v>
+        <ns0:v>2414671274.0354667</ns0:v>
       </ns0:c>
       <ns0:c r="G24" s="1" t="n">
         <ns0:v>5</ns0:v>
@@ -1861,7 +1861,7 @@
         <ns0:v>2.048031753406153e+16</ns0:v>
       </ns0:c>
       <ns0:c r="F25" s="1" t="n">
-        <ns0:v>89730764412.66322</ns0:v>
+        <ns0:v>10812275668.169369</ns0:v>
       </ns0:c>
       <ns0:c r="G25" s="1" t="n">
         <ns0:v>5.2</ns0:v>
@@ -1889,7 +1889,7 @@
         <ns0:v>8.80616166791431e+16</ns0:v>
       </ns0:c>
       <ns0:c r="F26" s="1" t="n">
-        <ns0:v>385825862655.3336</ns0:v>
+        <ns0:v>48414583956.644295</ns0:v>
       </ns0:c>
       <ns0:c r="G26" s="1" t="n">
         <ns0:v>5.4</ns0:v>
@@ -1917,7 +1917,7 @@
         <ns0:v>3.786488329219983e+17</ns0:v>
       </ns0:c>
       <ns0:c r="F27" s="1" t="n">
-        <ns0:v>1658980587852.034</ns0:v>
+        <ns0:v>216788029794.26984</ns0:v>
       </ns0:c>
       <ns0:c r="G27" s="1" t="n">
         <ns0:v>5.6</ns0:v>
@@ -1945,7 +1945,7 @@
         <ns0:v>1.628120673682214e+18</ns0:v>
       </ns0:c>
       <ns0:c r="F28" s="1" t="n">
-        <ns0:v>7133312867956.942</ns0:v>
+        <ns0:v>970720927895.766</ns0:v>
       </ns0:c>
       <ns0:c r="G28" s="1" t="n">
         <ns0:v>5.8</ns0:v>
@@ -1973,7 +1973,7 @@
         <ns0:v>7.000620885625409e+18</ns0:v>
       </ns0:c>
       <ns0:c r="F29" s="1" t="n">
-        <ns0:v>30671939650627.49</ns0:v>
+        <ns0:v>4346638145791.773</ns0:v>
       </ns0:c>
       <ns0:c r="G29" s="1" t="n">
         <ns0:v>6</ns0:v>
@@ -2001,7 +2001,7 @@
         <ns0:v>3.010138841454234e+19</ns0:v>
       </ns0:c>
       <ns0:c r="F30" s="1" t="n">
-        <ns0:v>131883726305864.5</ns0:v>
+        <ns0:v>19463125423088.504</ns0:v>
       </ns0:c>
       <ns0:c r="G30" s="1" t="n">
         <ns0:v>6.2</ns0:v>
@@ -2029,7 +2029,7 @@
         <ns0:v>1.294304604243966e+20</ns0:v>
       </ns0:c>
       <ns0:c r="F31" s="1" t="n">
-        <ns0:v>567075883117954.2</ns0:v>
+        <ns0:v>87150859705592.19</ns0:v>
       </ns0:c>
       <ns0:c r="G31" s="1" t="n">
         <ns0:v>6.4</ns0:v>
@@ -2057,7 +2057,7 @@
         <ns0:v>5.565272888734292e+20</ns0:v>
       </ns0:c>
       <ns0:c r="F32" s="1" t="n">
-        <ns0:v>2438322499837556</ns0:v>
+        <ns0:v>390239089679490.7</ns0:v>
       </ns0:c>
       <ns0:c r="G32" s="1" t="n">
         <ns0:v>6.6</ns0:v>
@@ -2085,7 +2085,7 @@
         <ns0:v>2.39296547540079e+21</ns0:v>
       </ns0:c>
       <ns0:c r="F33" s="1" t="n">
-        <ns0:v>1.048434043875112e+16</ns0:v>
+        <ns0:v>1747390073125186.8</ns0:v>
       </ns0:c>
       <ns0:c r="G33" s="1" t="n">
         <ns0:v>6.8</ns0:v>

</xml_diff>

<commit_message>
Candidate stage20 triple baseline and spread growth through30 from formal workbook
</commit_message>
<xml_diff>
--- a/space-battleship/config_excel/level.xlsx
+++ b/space-battleship/config_excel/level.xlsx
@@ -1799,10 +1799,10 @@
         </ns0:is>
       </ns0:c>
       <ns0:c r="D23" s="1" t="n">
-        <ns0:v>1107737222003781</ns0:v>
+        <ns0:v>3323211666011343</ns0:v>
       </ns0:c>
       <ns0:c r="E23" s="1" t="n">
-        <ns0:v>1107737222003781</ns0:v>
+        <ns0:v>3323211666011343</ns0:v>
       </ns0:c>
       <ns0:c r="F23" s="1" t="n">
         <ns0:v>539260886.477125</ns0:v>
@@ -1827,10 +1827,10 @@
         </ns0:is>
       </ns0:c>
       <ns0:c r="D24" s="1" t="n">
-        <ns0:v>4763067294395140</ns0:v>
+        <ns0:v>2.160087582907373e+16</ns0:v>
       </ns0:c>
       <ns0:c r="E24" s="1" t="n">
-        <ns0:v>4763067294395140</ns0:v>
+        <ns0:v>2.160087582907373e+16</ns0:v>
       </ns0:c>
       <ns0:c r="F24" s="1" t="n">
         <ns0:v>2414671274.0354667</ns0:v>
@@ -1855,10 +1855,10 @@
         </ns0:is>
       </ns0:c>
       <ns0:c r="D25" s="1" t="n">
-        <ns0:v>2.048031753406153e+16</ns0:v>
+        <ns0:v>1.404056928889792e+17</ns0:v>
       </ns0:c>
       <ns0:c r="E25" s="1" t="n">
-        <ns0:v>2.048031753406153e+16</ns0:v>
+        <ns0:v>1.404056928889792e+17</ns0:v>
       </ns0:c>
       <ns0:c r="F25" s="1" t="n">
         <ns0:v>10812275668.169369</ns0:v>
@@ -1883,10 +1883,10 @@
         </ns0:is>
       </ns0:c>
       <ns0:c r="D26" s="1" t="n">
-        <ns0:v>8.80616166791431e+16</ns0:v>
+        <ns0:v>9.126370037783651e+17</ns0:v>
       </ns0:c>
       <ns0:c r="E26" s="1" t="n">
-        <ns0:v>8.80616166791431e+16</ns0:v>
+        <ns0:v>9.126370037783651e+17</ns0:v>
       </ns0:c>
       <ns0:c r="F26" s="1" t="n">
         <ns0:v>48414583956.644295</ns0:v>
@@ -1911,10 +1911,10 @@
         </ns0:is>
       </ns0:c>
       <ns0:c r="D27" s="1" t="n">
-        <ns0:v>3.786488329219983e+17</ns0:v>
+        <ns0:v>5.932140524559373e+18</ns0:v>
       </ns0:c>
       <ns0:c r="E27" s="1" t="n">
-        <ns0:v>3.786488329219983e+17</ns0:v>
+        <ns0:v>5.932140524559373e+18</ns0:v>
       </ns0:c>
       <ns0:c r="F27" s="1" t="n">
         <ns0:v>216788029794.26984</ns0:v>
@@ -1939,10 +1939,10 @@
         </ns0:is>
       </ns0:c>
       <ns0:c r="D28" s="1" t="n">
-        <ns0:v>1.628120673682214e+18</ns0:v>
+        <ns0:v>3.855891340963593e+19</ns0:v>
       </ns0:c>
       <ns0:c r="E28" s="1" t="n">
-        <ns0:v>1.628120673682214e+18</ns0:v>
+        <ns0:v>3.855891340963593e+19</ns0:v>
       </ns0:c>
       <ns0:c r="F28" s="1" t="n">
         <ns0:v>970720927895.766</ns0:v>
@@ -1967,10 +1967,10 @@
         </ns0:is>
       </ns0:c>
       <ns0:c r="D29" s="1" t="n">
-        <ns0:v>7.000620885625409e+18</ns0:v>
+        <ns0:v>2.506329371626335e+20</ns0:v>
       </ns0:c>
       <ns0:c r="E29" s="1" t="n">
-        <ns0:v>7.000620885625409e+18</ns0:v>
+        <ns0:v>2.506329371626335e+20</ns0:v>
       </ns0:c>
       <ns0:c r="F29" s="1" t="n">
         <ns0:v>4346638145791.773</ns0:v>
@@ -1995,10 +1995,10 @@
         </ns0:is>
       </ns0:c>
       <ns0:c r="D30" s="1" t="n">
-        <ns0:v>3.010138841454234e+19</ns0:v>
+        <ns0:v>1.629114091557118e+21</ns0:v>
       </ns0:c>
       <ns0:c r="E30" s="1" t="n">
-        <ns0:v>3.010138841454234e+19</ns0:v>
+        <ns0:v>1.629114091557118e+21</ns0:v>
       </ns0:c>
       <ns0:c r="F30" s="1" t="n">
         <ns0:v>19463125423088.504</ns0:v>
@@ -2023,10 +2023,10 @@
         </ns0:is>
       </ns0:c>
       <ns0:c r="D31" s="1" t="n">
-        <ns0:v>1.294304604243966e+20</ns0:v>
+        <ns0:v>1.058924159512127e+22</ns0:v>
       </ns0:c>
       <ns0:c r="E31" s="1" t="n">
-        <ns0:v>1.294304604243966e+20</ns0:v>
+        <ns0:v>1.058924159512127e+22</ns0:v>
       </ns0:c>
       <ns0:c r="F31" s="1" t="n">
         <ns0:v>87150859705592.19</ns0:v>
@@ -2051,10 +2051,10 @@
         </ns0:is>
       </ns0:c>
       <ns0:c r="D32" s="1" t="n">
-        <ns0:v>5.565272888734292e+20</ns0:v>
+        <ns0:v>6.883007036828823e+22</ns0:v>
       </ns0:c>
       <ns0:c r="E32" s="1" t="n">
-        <ns0:v>5.565272888734292e+20</ns0:v>
+        <ns0:v>6.883007036828823e+22</ns0:v>
       </ns0:c>
       <ns0:c r="F32" s="1" t="n">
         <ns0:v>390239089679490.7</ns0:v>
@@ -2079,10 +2079,10 @@
         </ns0:is>
       </ns0:c>
       <ns0:c r="D33" s="1" t="n">
-        <ns0:v>2.39296547540079e+21</ns0:v>
+        <ns0:v>4.473954573938735e+23</ns0:v>
       </ns0:c>
       <ns0:c r="E33" s="1" t="n">
-        <ns0:v>2.39296547540079e+21</ns0:v>
+        <ns0:v>4.473954573938735e+23</ns0:v>
       </ns0:c>
       <ns0:c r="F33" s="1" t="n">
         <ns0:v>1747390073125186.8</ns0:v>

</xml_diff>

<commit_message>
qa: freeze reforge checkpoint37 with formal stage34x4 stage35x2 candidate
</commit_message>
<xml_diff>
--- a/space-battleship/config_excel/level.xlsx
+++ b/space-battleship/config_excel/level.xlsx
@@ -2191,10 +2191,10 @@
         </ns0:is>
       </ns0:c>
       <ns0:c r="D37" s="1" t="n">
-        <ns0:v>2.853799974342753e+29</ns0:v>
+        <ns0:v>1.1415199897371012e+30</ns0:v>
       </ns0:c>
       <ns0:c r="E37" s="1" t="n">
-        <ns0:v>1.376253845651405e+29</ns0:v>
+        <ns0:v>5.5050153826056202e+29</ns0:v>
       </ns0:c>
       <ns0:c r="F37" s="1" t="n">
         <ns0:v>2.174032833379432e+16</ns0:v>
@@ -2219,10 +2219,10 @@
         </ns0:is>
       </ns0:c>
       <ns0:c r="D38" s="1" t="n">
-        <ns0:v>3.266900647334875e+31</ns0:v>
+        <ns0:v>6.5338012946697504e+31</ns0:v>
       </ns0:c>
       <ns0:c r="E38" s="1" t="n">
-        <ns0:v>3.266900647334875e+31</ns0:v>
+        <ns0:v>6.5338012946697504e+31</ns0:v>
       </ns0:c>
       <ns0:c r="F38" s="1" t="n">
         <ns0:v>6.491627255945649e+16</ns0:v>

</xml_diff>

<commit_message>
balance: test stage35 terminal sixfold with unchanged stage34 and combined QA
</commit_message>
<xml_diff>
--- a/space-battleship/config_excel/level.xlsx
+++ b/space-battleship/config_excel/level.xlsx
@@ -2219,10 +2219,10 @@
         </ns0:is>
       </ns0:c>
       <ns0:c r="D38" s="1" t="n">
-        <ns0:v>6.5338012946697504e+31</ns0:v>
+        <ns0:v>1.960140388400925e+32</ns0:v>
       </ns0:c>
       <ns0:c r="E38" s="1" t="n">
-        <ns0:v>6.5338012946697504e+31</ns0:v>
+        <ns0:v>1.960140388400925e+32</ns0:v>
       </ns0:c>
       <ns0:c r="F38" s="1" t="n">
         <ns0:v>6.491627255945649e+16</ns0:v>

</xml_diff>

<commit_message>
Add optional level entry attack and life ratios; restore36 baseline ramp
</commit_message>
<xml_diff>
--- a/space-battleship/config_excel/level.xlsx
+++ b/space-battleship/config_excel/level.xlsx
@@ -1123,7 +1123,7 @@
     <ns0:outlinePr summaryBelow="1" summaryRight="1"/>
     <ns0:pageSetUpPr/>
   </ns0:sheetPr>
-  <ns0:dimension ref="A1:H223"/>
+  <ns0:dimension ref="A1:J223"/>
   <ns0:sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="14.4"/>
   <ns0:cols>
     <ns0:col width="78.2222222222222" customWidth="1" style="2" min="3" max="3"/>
@@ -1174,6 +1174,16 @@
           <ns0:t>planetExpRatio</ns0:t>
         </ns0:is>
       </ns0:c>
+      <ns0:c r="I1" t="inlineStr">
+        <ns0:is>
+          <ns0:t>entryAtkRatio</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="J1" t="inlineStr">
+        <ns0:is>
+          <ns0:t>entryLifeRatio</ns0:t>
+        </ns0:is>
+      </ns0:c>
     </ns0:row>
     <ns0:row r="2">
       <ns0:c r="A2" s="1" t="inlineStr">
@@ -1216,6 +1226,16 @@
           <ns0:t>星球探索经验系数</ns0:t>
         </ns0:is>
       </ns0:c>
+      <ns0:c r="I2" t="inlineStr">
+        <ns0:is>
+          <ns0:t>首战点攻击倍率（可选）</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="J2" t="inlineStr">
+        <ns0:is>
+          <ns0:t>首战点生命倍率（可选）</ns0:t>
+        </ns0:is>
+      </ns0:c>
     </ns0:row>
     <ns0:row r="3">
       <ns0:c r="A3" s="1" t="inlineStr">
@@ -1251,6 +1271,16 @@
       <ns0:c r="H3" s="1" t="inlineStr">
         <ns0:is>
           <ns0:t>30关为1，之前为0，之后每关增长20%并保留两位小数</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="I3" t="inlineStr">
+        <ns0:is>
+          <ns0:t>正有限数；空值继承上一关终点</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="J3" t="inlineStr">
+        <ns0:is>
+          <ns0:t>正有限数；空值继承上一关终点</ns0:t>
         </ns0:is>
       </ns0:c>
     </ns0:row>
@@ -2260,6 +2290,12 @@
       </ns0:c>
       <ns0:c r="H39" s="1" t="n">
         <ns0:v>1.244564747203978</ns0:v>
+      </ns0:c>
+      <ns0:c r="I39" t="n">
+        <ns0:v>3.266900647334875e31</ns0:v>
+      </ns0:c>
+      <ns0:c r="J39" t="n">
+        <ns0:v>3.266900647334875e31</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="40">

</xml_diff>

<commit_message>
Experiment: double level 21–25 resource ratios from official workbook
</commit_message>
<xml_diff>
--- a/space-battleship/config_excel/level.xlsx
+++ b/space-battleship/config_excel/level.xlsx
@@ -1833,7 +1833,7 @@
         <ns0:v>2.160087582907373e+16</ns0:v>
       </ns0:c>
       <ns0:c r="F24" s="1" t="n">
-        <ns0:v>2414671274.0354667</ns0:v>
+        <ns0:v>4829342548.070933</ns0:v>
       </ns0:c>
       <ns0:c r="G24" s="1" t="n">
         <ns0:v>5</ns0:v>
@@ -1861,7 +1861,7 @@
         <ns0:v>1.404056928889792e+17</ns0:v>
       </ns0:c>
       <ns0:c r="F25" s="1" t="n">
-        <ns0:v>10812275668.169369</ns0:v>
+        <ns0:v>21624551336.338737</ns0:v>
       </ns0:c>
       <ns0:c r="G25" s="1" t="n">
         <ns0:v>5.2</ns0:v>
@@ -1889,7 +1889,7 @@
         <ns0:v>9.126370037783651e+17</ns0:v>
       </ns0:c>
       <ns0:c r="F26" s="1" t="n">
-        <ns0:v>48414583956.644295</ns0:v>
+        <ns0:v>96829167913.28859</ns0:v>
       </ns0:c>
       <ns0:c r="G26" s="1" t="n">
         <ns0:v>5.4</ns0:v>
@@ -1917,7 +1917,7 @@
         <ns0:v>5.932140524559373e+18</ns0:v>
       </ns0:c>
       <ns0:c r="F27" s="1" t="n">
-        <ns0:v>216788029794.26984</ns0:v>
+        <ns0:v>433576059588.5397</ns0:v>
       </ns0:c>
       <ns0:c r="G27" s="1" t="n">
         <ns0:v>5.6</ns0:v>
@@ -1945,7 +1945,7 @@
         <ns0:v>3.855891340963593e+19</ns0:v>
       </ns0:c>
       <ns0:c r="F28" s="1" t="n">
-        <ns0:v>970720927895.766</ns0:v>
+        <ns0:v>1941441855791.532</ns0:v>
       </ns0:c>
       <ns0:c r="G28" s="1" t="n">
         <ns0:v>5.8</ns0:v>

</xml_diff>

<commit_message>
Apply adopted planet XP curve to all authored stages
</commit_message>
<xml_diff>
--- a/space-battleship/config_excel/level.xlsx
+++ b/space-battleship/config_excel/level.xlsx
@@ -1308,7 +1308,7 @@
       <ns0:c r="G4" s="1" t="n">
         <ns0:v>1</ns0:v>
       </ns0:c>
-      <ns0:c r="H4" s="1" t="n">
+      <ns0:c r="H4" s="1">
         <ns0:v>0</ns0:v>
       </ns0:c>
     </ns0:row>
@@ -1336,7 +1336,7 @@
       <ns0:c r="G5" s="1" t="n">
         <ns0:v>1.2</ns0:v>
       </ns0:c>
-      <ns0:c r="H5" s="1" t="n">
+      <ns0:c r="H5" s="1">
         <ns0:v>0</ns0:v>
       </ns0:c>
     </ns0:row>
@@ -1364,7 +1364,7 @@
       <ns0:c r="G6" s="1" t="n">
         <ns0:v>1.4</ns0:v>
       </ns0:c>
-      <ns0:c r="H6" s="1" t="n">
+      <ns0:c r="H6" s="1">
         <ns0:v>0</ns0:v>
       </ns0:c>
     </ns0:row>
@@ -1392,7 +1392,7 @@
       <ns0:c r="G7" s="1" t="n">
         <ns0:v>1.6</ns0:v>
       </ns0:c>
-      <ns0:c r="H7" s="1" t="n">
+      <ns0:c r="H7" s="1">
         <ns0:v>0</ns0:v>
       </ns0:c>
     </ns0:row>
@@ -1420,7 +1420,7 @@
       <ns0:c r="G8" s="1" t="n">
         <ns0:v>1.8</ns0:v>
       </ns0:c>
-      <ns0:c r="H8" s="1" t="n">
+      <ns0:c r="H8" s="1">
         <ns0:v>0</ns0:v>
       </ns0:c>
     </ns0:row>
@@ -1448,7 +1448,7 @@
       <ns0:c r="G9" s="1" t="n">
         <ns0:v>2</ns0:v>
       </ns0:c>
-      <ns0:c r="H9" s="1" t="n">
+      <ns0:c r="H9" s="1">
         <ns0:v>0</ns0:v>
       </ns0:c>
     </ns0:row>
@@ -1476,7 +1476,7 @@
       <ns0:c r="G10" s="1" t="n">
         <ns0:v>2.2</ns0:v>
       </ns0:c>
-      <ns0:c r="H10" s="1" t="n">
+      <ns0:c r="H10" s="1">
         <ns0:v>0</ns0:v>
       </ns0:c>
     </ns0:row>
@@ -1504,7 +1504,7 @@
       <ns0:c r="G11" s="1" t="n">
         <ns0:v>2.4</ns0:v>
       </ns0:c>
-      <ns0:c r="H11" s="1" t="n">
+      <ns0:c r="H11" s="1">
         <ns0:v>0</ns0:v>
       </ns0:c>
     </ns0:row>
@@ -1532,7 +1532,7 @@
       <ns0:c r="G12" s="1" t="n">
         <ns0:v>2.6</ns0:v>
       </ns0:c>
-      <ns0:c r="H12" s="1" t="n">
+      <ns0:c r="H12" s="1">
         <ns0:v>0</ns0:v>
       </ns0:c>
     </ns0:row>
@@ -1560,7 +1560,7 @@
       <ns0:c r="G13" s="1" t="n">
         <ns0:v>2.8</ns0:v>
       </ns0:c>
-      <ns0:c r="H13" s="1" t="n">
+      <ns0:c r="H13" s="1">
         <ns0:v>0</ns0:v>
       </ns0:c>
     </ns0:row>
@@ -1588,7 +1588,7 @@
       <ns0:c r="G14" s="1" t="n">
         <ns0:v>3</ns0:v>
       </ns0:c>
-      <ns0:c r="H14" s="1" t="n">
+      <ns0:c r="H14" s="1">
         <ns0:v>0</ns0:v>
       </ns0:c>
     </ns0:row>
@@ -1616,7 +1616,7 @@
       <ns0:c r="G15" s="1" t="n">
         <ns0:v>3.2</ns0:v>
       </ns0:c>
-      <ns0:c r="H15" s="1" t="n">
+      <ns0:c r="H15" s="1">
         <ns0:v>0</ns0:v>
       </ns0:c>
     </ns0:row>
@@ -1644,7 +1644,7 @@
       <ns0:c r="G16" s="1" t="n">
         <ns0:v>3.4</ns0:v>
       </ns0:c>
-      <ns0:c r="H16" s="1" t="n">
+      <ns0:c r="H16" s="1">
         <ns0:v>0</ns0:v>
       </ns0:c>
     </ns0:row>
@@ -1672,7 +1672,7 @@
       <ns0:c r="G17" s="1" t="n">
         <ns0:v>3.6</ns0:v>
       </ns0:c>
-      <ns0:c r="H17" s="1" t="n">
+      <ns0:c r="H17" s="1">
         <ns0:v>0</ns0:v>
       </ns0:c>
     </ns0:row>
@@ -1700,7 +1700,7 @@
       <ns0:c r="G18" s="1" t="n">
         <ns0:v>3.8</ns0:v>
       </ns0:c>
-      <ns0:c r="H18" s="1" t="n">
+      <ns0:c r="H18" s="1">
         <ns0:v>0</ns0:v>
       </ns0:c>
     </ns0:row>
@@ -1728,7 +1728,7 @@
       <ns0:c r="G19" s="1" t="n">
         <ns0:v>4</ns0:v>
       </ns0:c>
-      <ns0:c r="H19" s="1" t="n">
+      <ns0:c r="H19" s="1">
         <ns0:v>0</ns0:v>
       </ns0:c>
     </ns0:row>
@@ -1756,7 +1756,7 @@
       <ns0:c r="G20" s="1" t="n">
         <ns0:v>4.2</ns0:v>
       </ns0:c>
-      <ns0:c r="H20" s="1" t="n">
+      <ns0:c r="H20" s="1">
         <ns0:v>0</ns0:v>
       </ns0:c>
     </ns0:row>
@@ -1784,7 +1784,7 @@
       <ns0:c r="G21" s="1" t="n">
         <ns0:v>4.4</ns0:v>
       </ns0:c>
-      <ns0:c r="H21" s="1" t="n">
+      <ns0:c r="H21" s="1">
         <ns0:v>0</ns0:v>
       </ns0:c>
     </ns0:row>
@@ -1812,7 +1812,7 @@
       <ns0:c r="G22" s="1" t="n">
         <ns0:v>4.6</ns0:v>
       </ns0:c>
-      <ns0:c r="H22" s="1" t="n">
+      <ns0:c r="H22" s="1">
         <ns0:v>0</ns0:v>
       </ns0:c>
     </ns0:row>
@@ -1840,7 +1840,7 @@
       <ns0:c r="G23" s="1" t="n">
         <ns0:v>4.8</ns0:v>
       </ns0:c>
-      <ns0:c r="H23" s="1" t="n">
+      <ns0:c r="H23" s="1">
         <ns0:v>0</ns0:v>
       </ns0:c>
     </ns0:row>
@@ -1868,7 +1868,7 @@
       <ns0:c r="G24" s="1" t="n">
         <ns0:v>5</ns0:v>
       </ns0:c>
-      <ns0:c r="H24" s="1" t="n">
+      <ns0:c r="H24" s="1">
         <ns0:v>0</ns0:v>
       </ns0:c>
     </ns0:row>
@@ -1896,7 +1896,7 @@
       <ns0:c r="G25" s="1" t="n">
         <ns0:v>5.2</ns0:v>
       </ns0:c>
-      <ns0:c r="H25" s="1" t="n">
+      <ns0:c r="H25" s="1">
         <ns0:v>0</ns0:v>
       </ns0:c>
     </ns0:row>
@@ -1924,7 +1924,7 @@
       <ns0:c r="G26" s="1" t="n">
         <ns0:v>5.4</ns0:v>
       </ns0:c>
-      <ns0:c r="H26" s="1" t="n">
+      <ns0:c r="H26" s="1">
         <ns0:v>0</ns0:v>
       </ns0:c>
     </ns0:row>
@@ -1952,7 +1952,7 @@
       <ns0:c r="G27" s="1" t="n">
         <ns0:v>5.6</ns0:v>
       </ns0:c>
-      <ns0:c r="H27" s="1" t="n">
+      <ns0:c r="H27" s="1">
         <ns0:v>0</ns0:v>
       </ns0:c>
     </ns0:row>
@@ -1980,7 +1980,7 @@
       <ns0:c r="G28" s="1" t="n">
         <ns0:v>5.8</ns0:v>
       </ns0:c>
-      <ns0:c r="H28" s="1" t="n">
+      <ns0:c r="H28" s="1">
         <ns0:v>0</ns0:v>
       </ns0:c>
     </ns0:row>
@@ -2008,7 +2008,7 @@
       <ns0:c r="G29" s="1" t="n">
         <ns0:v>6</ns0:v>
       </ns0:c>
-      <ns0:c r="H29" s="1" t="n">
+      <ns0:c r="H29" s="1">
         <ns0:v>0</ns0:v>
       </ns0:c>
     </ns0:row>
@@ -2036,7 +2036,7 @@
       <ns0:c r="G30" s="1" t="n">
         <ns0:v>6.2</ns0:v>
       </ns0:c>
-      <ns0:c r="H30" s="1" t="n">
+      <ns0:c r="H30" s="1">
         <ns0:v>0</ns0:v>
       </ns0:c>
     </ns0:row>
@@ -2064,7 +2064,7 @@
       <ns0:c r="G31" s="1" t="n">
         <ns0:v>6.4</ns0:v>
       </ns0:c>
-      <ns0:c r="H31" s="1" t="n">
+      <ns0:c r="H31" s="1">
         <ns0:v>0</ns0:v>
       </ns0:c>
     </ns0:row>
@@ -2092,7 +2092,7 @@
       <ns0:c r="G32" s="1" t="n">
         <ns0:v>6.6</ns0:v>
       </ns0:c>
-      <ns0:c r="H32" s="1" t="n">
+      <ns0:c r="H32" s="1">
         <ns0:v>0</ns0:v>
       </ns0:c>
     </ns0:row>
@@ -2120,8 +2120,8 @@
       <ns0:c r="G33" s="1" t="n">
         <ns0:v>6.8</ns0:v>
       </ns0:c>
-      <ns0:c r="H33" s="1" t="n">
-        <ns0:v>1</ns0:v>
+      <ns0:c r="H33" s="1">
+        <ns0:v>1.0</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="34">
@@ -2148,8 +2148,8 @@
       <ns0:c r="G34" s="1" t="n">
         <ns0:v>7</ns0:v>
       </ns0:c>
-      <ns0:c r="H34" s="1" t="n">
-        <ns0:v>1.037137289336648</ns0:v>
+      <ns0:c r="H34" s="1">
+        <ns0:v>1.0371372893366482</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="35">
@@ -2176,8 +2176,8 @@
       <ns0:c r="G35" s="1" t="n">
         <ns0:v>7.2</ns0:v>
       </ns0:c>
-      <ns0:c r="H35" s="1" t="n">
-        <ns0:v>1.07565375693257</ns0:v>
+      <ns0:c r="H35" s="1">
+        <ns0:v>1.0756537569325701</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="36">
@@ -2204,8 +2204,8 @@
       <ns0:c r="G36" s="1" t="n">
         <ns0:v>7.4</ns0:v>
       </ns0:c>
-      <ns0:c r="H36" s="1" t="n">
-        <ns0:v>1.115600621729828</ns0:v>
+      <ns0:c r="H36" s="1">
+        <ns0:v>1.1156006217298275</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="37">
@@ -2232,8 +2232,8 @@
       <ns0:c r="G37" s="1" t="n">
         <ns0:v>7.6</ns0:v>
       </ns0:c>
-      <ns0:c r="H37" s="1" t="n">
-        <ns0:v>1.157031004803153</ns0:v>
+      <ns0:c r="H37" s="1">
+        <ns0:v>1.1570310048031527</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="38">
@@ -2260,7 +2260,7 @@
       <ns0:c r="G38" s="1" t="n">
         <ns0:v>7.8</ns0:v>
       </ns0:c>
-      <ns0:c r="H38" s="1" t="n">
+      <ns0:c r="H38" s="1">
         <ns0:v>1.2</ns0:v>
       </ns0:c>
     </ns0:row>
@@ -2288,8 +2288,8 @@
       <ns0:c r="G39" s="1" t="n">
         <ns0:v>8</ns0:v>
       </ns0:c>
-      <ns0:c r="H39" s="1" t="n">
-        <ns0:v>1.244564747203978</ns0:v>
+      <ns0:c r="H39" s="1">
+        <ns0:v>1.2445647472039776</ns0:v>
       </ns0:c>
       <ns0:c r="I39" t="n">
         <ns0:v>3.266900647334875e31</ns0:v>
@@ -2322,7 +2322,7 @@
       <ns0:c r="G40" s="1" t="n">
         <ns0:v>8.199999999999999</ns0:v>
       </ns0:c>
-      <ns0:c r="H40" s="1" t="n">
+      <ns0:c r="H40" s="1">
         <ns0:v>1.290784508319084</ns0:v>
       </ns0:c>
     </ns0:row>
@@ -2350,7 +2350,7 @@
       <ns0:c r="G41" s="1" t="n">
         <ns0:v>8.4</ns0:v>
       </ns0:c>
-      <ns0:c r="H41" s="1" t="n">
+      <ns0:c r="H41" s="1">
         <ns0:v>1.338720746075793</ns0:v>
       </ns0:c>
     </ns0:row>
@@ -2378,7 +2378,7 @@
       <ns0:c r="G42" s="1" t="n">
         <ns0:v>8.6</ns0:v>
       </ns0:c>
-      <ns0:c r="H42" s="1" t="n">
+      <ns0:c r="H42" s="1">
         <ns0:v>1.388437205763783</ns0:v>
       </ns0:c>
     </ns0:row>
@@ -2406,7 +2406,7 @@
       <ns0:c r="G43" s="1" t="n">
         <ns0:v>8.800000000000001</ns0:v>
       </ns0:c>
-      <ns0:c r="H43" s="1" t="n">
+      <ns0:c r="H43" s="1">
         <ns0:v>1.44</ns0:v>
       </ns0:c>
     </ns0:row>
@@ -2434,8 +2434,8 @@
       <ns0:c r="G44" s="1" t="n">
         <ns0:v>9</ns0:v>
       </ns0:c>
-      <ns0:c r="H44" s="1" t="n">
-        <ns0:v>1.493477696644773</ns0:v>
+      <ns0:c r="H44" s="1">
+        <ns0:v>1.4934776966447731</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="45">
@@ -2462,8 +2462,8 @@
       <ns0:c r="G45" s="1" t="n">
         <ns0:v>9.199999999999999</ns0:v>
       </ns0:c>
-      <ns0:c r="H45" s="1" t="n">
-        <ns0:v>1.548941409982901</ns0:v>
+      <ns0:c r="H45" s="1">
+        <ns0:v>1.5489414099829009</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="46">
@@ -2490,8 +2490,8 @@
       <ns0:c r="G46" s="1" t="n">
         <ns0:v>9.4</ns0:v>
       </ns0:c>
-      <ns0:c r="H46" s="1" t="n">
-        <ns0:v>1.606464895290951</ns0:v>
+      <ns0:c r="H46" s="1">
+        <ns0:v>1.6064648952909515</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="47">
@@ -2518,8 +2518,8 @@
       <ns0:c r="G47" s="1" t="n">
         <ns0:v>9.6</ns0:v>
       </ns0:c>
-      <ns0:c r="H47" s="1" t="n">
-        <ns0:v>1.66612464691654</ns0:v>
+      <ns0:c r="H47" s="1">
+        <ns0:v>1.6661246469165396</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="48">
@@ -2546,8 +2546,8 @@
       <ns0:c r="G48" s="1" t="n">
         <ns0:v>9.800000000000001</ns0:v>
       </ns0:c>
-      <ns0:c r="H48" s="1" t="n">
-        <ns0:v>1.728</ns0:v>
+      <ns0:c r="H48" s="1">
+        <ns0:v>1.7279999999999998</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="49">
@@ -2574,8 +2574,8 @@
       <ns0:c r="G49" s="1" t="n">
         <ns0:v>10</ns0:v>
       </ns0:c>
-      <ns0:c r="H49" s="1" t="n">
-        <ns0:v>1.792173235973728</ns0:v>
+      <ns0:c r="H49" s="1">
+        <ns0:v>1.7921732359737277</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="50">
@@ -2602,7 +2602,7 @@
       <ns0:c r="G50" s="1" t="n">
         <ns0:v>10.2</ns0:v>
       </ns0:c>
-      <ns0:c r="H50" s="1" t="n">
+      <ns0:c r="H50" s="1">
         <ns0:v>1.858729691979481</ns0:v>
       </ns0:c>
     </ns0:row>
@@ -2630,8 +2630,8 @@
       <ns0:c r="G51" s="1" t="n">
         <ns0:v>10.4</ns0:v>
       </ns0:c>
-      <ns0:c r="H51" s="1" t="n">
-        <ns0:v>1.927757874349142</ns0:v>
+      <ns0:c r="H51" s="1">
+        <ns0:v>1.9277578743491417</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="52">
@@ -2658,8 +2658,8 @@
       <ns0:c r="G52" s="1" t="n">
         <ns0:v>10.6</ns0:v>
       </ns0:c>
-      <ns0:c r="H52" s="1" t="n">
-        <ns0:v>1.999349576299847</ns0:v>
+      <ns0:c r="H52" s="1">
+        <ns0:v>1.9993495762998474</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="53">
@@ -2686,7 +2686,7 @@
       <ns0:c r="G53" s="1" t="n">
         <ns0:v>10.8</ns0:v>
       </ns0:c>
-      <ns0:c r="H53" s="1" t="n">
+      <ns0:c r="H53" s="1">
         <ns0:v>2.0736</ns0:v>
       </ns0:c>
     </ns0:row>
@@ -2714,8 +2714,8 @@
       <ns0:c r="G54" s="1" t="n">
         <ns0:v>11</ns0:v>
       </ns0:c>
-      <ns0:c r="H54" s="1" t="n">
-        <ns0:v>2.150607883168473</ns0:v>
+      <ns0:c r="H54" s="1">
+        <ns0:v>2.1506078831684734</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="55">
@@ -2742,7 +2742,7 @@
       <ns0:c r="G55" s="1" t="n">
         <ns0:v>11.2</ns0:v>
       </ns0:c>
-      <ns0:c r="H55" s="1" t="n">
+      <ns0:c r="H55" s="1">
         <ns0:v>2.230475630375377</ns0:v>
       </ns0:c>
     </ns0:row>
@@ -2770,7 +2770,7 @@
       <ns0:c r="G56" s="1" t="n">
         <ns0:v>11.4</ns0:v>
       </ns0:c>
-      <ns0:c r="H56" s="1" t="n">
+      <ns0:c r="H56" s="1">
         <ns0:v>2.31330944921897</ns0:v>
       </ns0:c>
     </ns0:row>
@@ -2798,7 +2798,7 @@
       <ns0:c r="G57" s="1" t="n">
         <ns0:v>11.6</ns0:v>
       </ns0:c>
-      <ns0:c r="H57" s="1" t="n">
+      <ns0:c r="H57" s="1">
         <ns0:v>2.399219491559817</ns0:v>
       </ns0:c>
     </ns0:row>
@@ -2826,8 +2826,8 @@
       <ns0:c r="G58" s="1" t="n">
         <ns0:v>11.8</ns0:v>
       </ns0:c>
-      <ns0:c r="H58" s="1" t="n">
-        <ns0:v>2.488319999999999</ns0:v>
+      <ns0:c r="H58" s="1">
+        <ns0:v>2.4883199999999994</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="59">
@@ -2854,8 +2854,8 @@
       <ns0:c r="G59" s="1" t="n">
         <ns0:v>12</ns0:v>
       </ns0:c>
-      <ns0:c r="H59" s="1" t="n">
-        <ns0:v>2.580729459802168</ns0:v>
+      <ns0:c r="H59" s="1">
+        <ns0:v>2.5807294598021677</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="60">
@@ -2882,8 +2882,8 @@
       <ns0:c r="G60" s="1" t="n">
         <ns0:v>12.2</ns0:v>
       </ns0:c>
-      <ns0:c r="H60" s="1" t="n">
-        <ns0:v>2.676570756450452</ns0:v>
+      <ns0:c r="H60" s="1">
+        <ns0:v>2.6765707564504524</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="61">
@@ -2910,7 +2910,7 @@
       <ns0:c r="G61" s="1" t="n">
         <ns0:v>12.4</ns0:v>
       </ns0:c>
-      <ns0:c r="H61" s="1" t="n">
+      <ns0:c r="H61" s="1">
         <ns0:v>2.775971339062764</ns0:v>
       </ns0:c>
     </ns0:row>
@@ -2938,7 +2938,7 @@
       <ns0:c r="G62" s="1" t="n">
         <ns0:v>12.6</ns0:v>
       </ns0:c>
-      <ns0:c r="H62" s="1" t="n">
+      <ns0:c r="H62" s="1">
         <ns0:v>2.87906338987178</ns0:v>
       </ns0:c>
     </ns0:row>
@@ -2966,8 +2966,8 @@
       <ns0:c r="G63" s="1" t="n">
         <ns0:v>12.8</ns0:v>
       </ns0:c>
-      <ns0:c r="H63" s="1" t="n">
-        <ns0:v>2.985983999999999</ns0:v>
+      <ns0:c r="H63" s="1">
+        <ns0:v>2.9859839999999993</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="64">
@@ -2997,8 +2997,8 @@
       <ns0:c r="G64" s="1" t="n">
         <ns0:v>13</ns0:v>
       </ns0:c>
-      <ns0:c r="H64" s="1" t="n">
-        <ns0:v>285.78</ns0:v>
+      <ns0:c r="H64" s="1">
+        <ns0:v>3.096875351762601</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="65">
@@ -3028,8 +3028,8 @@
       <ns0:c r="G65" s="1" t="n">
         <ns0:v>13.2</ns0:v>
       </ns0:c>
-      <ns0:c r="H65" s="1" t="n">
-        <ns0:v>342.94</ns0:v>
+      <ns0:c r="H65" s="1">
+        <ns0:v>3.2118849077405427</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="66">
@@ -3059,8 +3059,8 @@
       <ns0:c r="G66" s="1" t="n">
         <ns0:v>13.4</ns0:v>
       </ns0:c>
-      <ns0:c r="H66" s="1" t="n">
-        <ns0:v>411.53</ns0:v>
+      <ns0:c r="H66" s="1">
+        <ns0:v>3.331165606875316</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="67">
@@ -3090,8 +3090,8 @@
       <ns0:c r="G67" s="1" t="n">
         <ns0:v>13.6</ns0:v>
       </ns0:c>
-      <ns0:c r="H67" s="1" t="n">
-        <ns0:v>493.84</ns0:v>
+      <ns0:c r="H67" s="1">
+        <ns0:v>3.454876067846136</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="68">
@@ -3121,8 +3121,8 @@
       <ns0:c r="G68" s="1" t="n">
         <ns0:v>13.8</ns0:v>
       </ns0:c>
-      <ns0:c r="H68" s="1" t="n">
-        <ns0:v>592.61</ns0:v>
+      <ns0:c r="H68" s="1">
+        <ns0:v>3.583180799999999</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="69">
@@ -3152,8 +3152,8 @@
       <ns0:c r="G69" s="1" t="n">
         <ns0:v>14</ns0:v>
       </ns0:c>
-      <ns0:c r="H69" s="1" t="n">
-        <ns0:v>711.13</ns0:v>
+      <ns0:c r="H69" s="1">
+        <ns0:v>3.716250422115121</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="70">
@@ -3183,8 +3183,8 @@
       <ns0:c r="G70" s="1" t="n">
         <ns0:v>14.2</ns0:v>
       </ns0:c>
-      <ns0:c r="H70" s="1" t="n">
-        <ns0:v>853.36</ns0:v>
+      <ns0:c r="H70" s="1">
+        <ns0:v>3.8542618892886513</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="71">
@@ -3214,8 +3214,8 @@
       <ns0:c r="G71" s="1" t="n">
         <ns0:v>14.4</ns0:v>
       </ns0:c>
-      <ns0:c r="H71" s="1" t="n">
-        <ns0:v>1024.03</ns0:v>
+      <ns0:c r="H71" s="1">
+        <ns0:v>3.9973987282503796</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="72">
@@ -3245,8 +3245,8 @@
       <ns0:c r="G72" s="1" t="n">
         <ns0:v>14.6</ns0:v>
       </ns0:c>
-      <ns0:c r="H72" s="1" t="n">
-        <ns0:v>1228.84</ns0:v>
+      <ns0:c r="H72" s="1">
+        <ns0:v>4.145851281415363</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="73">
@@ -3276,8 +3276,8 @@
       <ns0:c r="G73" s="1" t="n">
         <ns0:v>14.8</ns0:v>
       </ns0:c>
-      <ns0:c r="H73" s="1" t="n">
-        <ns0:v>1474.61</ns0:v>
+      <ns0:c r="H73" s="1">
+        <ns0:v>4.2998169599999985</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="74">
@@ -3308,8 +3308,7 @@
         <ns0:v>15</ns0:v>
       </ns0:c>
       <ns0:c r="H74" s="1">
-        <ns0:f>ROUND(H73*1.2,2)</ns0:f>
-        <ns0:v>1769.53</ns0:v>
+        <ns0:v>4.459500506538145</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="75">
@@ -3340,8 +3339,7 @@
         <ns0:v>15.2</ns0:v>
       </ns0:c>
       <ns0:c r="H75" s="1">
-        <ns0:f>ROUND(H74*1.2,2)</ns0:f>
-        <ns0:v>2123.44</ns0:v>
+        <ns0:v>4.625114267146381</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="76">
@@ -3372,8 +3370,7 @@
         <ns0:v>15.4</ns0:v>
       </ns0:c>
       <ns0:c r="H76" s="1">
-        <ns0:f>ROUND(H75*1.2,2)</ns0:f>
-        <ns0:v>2548.13</ns0:v>
+        <ns0:v>4.796878473900455</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="77">
@@ -3404,8 +3401,7 @@
         <ns0:v>15.6</ns0:v>
       </ns0:c>
       <ns0:c r="H77" s="1">
-        <ns0:f>ROUND(H76*1.2,2)</ns0:f>
-        <ns0:v>3057.76</ns0:v>
+        <ns0:v>4.975021537698436</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="78">
@@ -3436,8 +3432,7 @@
         <ns0:v>15.8</ns0:v>
       </ns0:c>
       <ns0:c r="H78" s="1">
-        <ns0:f>ROUND(H77*1.2,2)</ns0:f>
-        <ns0:v>3669.31</ns0:v>
+        <ns0:v>5.1597803519999985</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="79">
@@ -3468,8 +3463,7 @@
         <ns0:v>16</ns0:v>
       </ns0:c>
       <ns0:c r="H79" s="1">
-        <ns0:f>ROUND(H78*1.2,2)</ns0:f>
-        <ns0:v>4403.17</ns0:v>
+        <ns0:v>5.351400607845774</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="80">
@@ -3500,8 +3494,7 @@
         <ns0:v>16.2</ns0:v>
       </ns0:c>
       <ns0:c r="H80" s="1">
-        <ns0:f>ROUND(H79*1.2,2)</ns0:f>
-        <ns0:v>5283.8</ns0:v>
+        <ns0:v>5.550137120575657</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="81">
@@ -3532,8 +3525,7 @@
         <ns0:v>16.4</ns0:v>
       </ns0:c>
       <ns0:c r="H81" s="1">
-        <ns0:f>ROUND(H80*1.2,2)</ns0:f>
-        <ns0:v>6340.56</ns0:v>
+        <ns0:v>5.756254168680546</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="82">
@@ -3564,8 +3556,7 @@
         <ns0:v>16.6</ns0:v>
       </ns0:c>
       <ns0:c r="H82" s="1">
-        <ns0:f>ROUND(H81*1.2,2)</ns0:f>
-        <ns0:v>7608.67</ns0:v>
+        <ns0:v>5.970025845238124</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="83">
@@ -3596,8 +3587,7 @@
         <ns0:v>16.8</ns0:v>
       </ns0:c>
       <ns0:c r="H83" s="1">
-        <ns0:f>ROUND(H82*1.2,2)</ns0:f>
-        <ns0:v>9130.4</ns0:v>
+        <ns0:v>6.191736422399997</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="84">
@@ -3628,8 +3618,7 @@
         <ns0:v>17</ns0:v>
       </ns0:c>
       <ns0:c r="H84" s="1">
-        <ns0:f>ROUND(H83*1.2,2)</ns0:f>
-        <ns0:v>10956.48</ns0:v>
+        <ns0:v>6.421680729414928</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="85">
@@ -3660,8 +3649,7 @@
         <ns0:v>17.2</ns0:v>
       </ns0:c>
       <ns0:c r="H85" s="1">
-        <ns0:f>ROUND(H84*1.2,2)</ns0:f>
-        <ns0:v>13147.78</ns0:v>
+        <ns0:v>6.6601645446907884</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="86">
@@ -3692,8 +3680,7 @@
         <ns0:v>17.4</ns0:v>
       </ns0:c>
       <ns0:c r="H86" s="1">
-        <ns0:f>ROUND(H85*1.2,2)</ns0:f>
-        <ns0:v>15777.34</ns0:v>
+        <ns0:v>6.907505002416655</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="87">
@@ -3724,8 +3711,7 @@
         <ns0:v>17.6</ns0:v>
       </ns0:c>
       <ns0:c r="H87" s="1">
-        <ns0:f>ROUND(H86*1.2,2)</ns0:f>
-        <ns0:v>18932.81</ns0:v>
+        <ns0:v>7.164031014285747</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="88">
@@ -3756,8 +3742,7 @@
         <ns0:v>17.8</ns0:v>
       </ns0:c>
       <ns0:c r="H88" s="1">
-        <ns0:f>ROUND(H87*1.2,2)</ns0:f>
-        <ns0:v>22719.37</ns0:v>
+        <ns0:v>7.430083706879997</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="89">
@@ -3788,8 +3773,7 @@
         <ns0:v>18</ns0:v>
       </ns0:c>
       <ns0:c r="H89" s="1">
-        <ns0:f>ROUND(H88*1.2,2)</ns0:f>
-        <ns0:v>27263.24</ns0:v>
+        <ns0:v>7.706016875297913</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="90">
@@ -3820,8 +3804,7 @@
         <ns0:v>18.2</ns0:v>
       </ns0:c>
       <ns0:c r="H90" s="1">
-        <ns0:f>ROUND(H89*1.2,2)</ns0:f>
-        <ns0:v>32715.89</ns0:v>
+        <ns0:v>7.992197453628946</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="91">
@@ -3852,8 +3835,7 @@
         <ns0:v>18.4</ns0:v>
       </ns0:c>
       <ns0:c r="H91" s="1">
-        <ns0:f>ROUND(H90*1.2,2)</ns0:f>
-        <ns0:v>39259.07</ns0:v>
+        <ns0:v>8.289006002899985</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="92">
@@ -3884,8 +3866,7 @@
         <ns0:v>18.6</ns0:v>
       </ns0:c>
       <ns0:c r="H92" s="1">
-        <ns0:f>ROUND(H91*1.2,2)</ns0:f>
-        <ns0:v>47110.88</ns0:v>
+        <ns0:v>8.596837217142896</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="93">
@@ -3916,8 +3897,7 @@
         <ns0:v>18.8</ns0:v>
       </ns0:c>
       <ns0:c r="H93" s="1">
-        <ns0:f>ROUND(H92*1.2,2)</ns0:f>
-        <ns0:v>56533.06</ns0:v>
+        <ns0:v>8.916100448255996</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="94">
@@ -3948,8 +3928,7 @@
         <ns0:v>19</ns0:v>
       </ns0:c>
       <ns0:c r="H94" s="1">
-        <ns0:f>ROUND(H93*1.2,2)</ns0:f>
-        <ns0:v>67839.67</ns0:v>
+        <ns0:v>9.247220250357495</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="95">
@@ -3980,8 +3959,7 @@
         <ns0:v>19.2</ns0:v>
       </ns0:c>
       <ns0:c r="H95" s="1">
-        <ns0:f>ROUND(H94*1.2,2)</ns0:f>
-        <ns0:v>81407.6</ns0:v>
+        <ns0:v>9.590636944354735</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="96">
@@ -4012,8 +3990,7 @@
         <ns0:v>19.4</ns0:v>
       </ns0:c>
       <ns0:c r="H96" s="1">
-        <ns0:f>ROUND(H95*1.2,2)</ns0:f>
-        <ns0:v>97689.12</ns0:v>
+        <ns0:v>9.946807203479983</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="97">
@@ -4044,8 +4021,7 @@
         <ns0:v>19.6</ns0:v>
       </ns0:c>
       <ns0:c r="H97" s="1">
-        <ns0:f>ROUND(H96*1.2,2)</ns0:f>
-        <ns0:v>117226.94</ns0:v>
+        <ns0:v>10.316204660571476</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="98">
@@ -4076,8 +4052,7 @@
         <ns0:v>19.8</ns0:v>
       </ns0:c>
       <ns0:c r="H98" s="1">
-        <ns0:f>ROUND(H97*1.2,2)</ns0:f>
-        <ns0:v>140672.33</ns0:v>
+        <ns0:v>10.699320537907195</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="99">
@@ -4108,8 +4083,7 @@
         <ns0:v>20</ns0:v>
       </ns0:c>
       <ns0:c r="H99" s="1">
-        <ns0:f>ROUND(H98*1.2,2)</ns0:f>
-        <ns0:v>168806.8</ns0:v>
+        <ns0:v>11.096664300428994</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="100">
@@ -4140,8 +4114,7 @@
         <ns0:v>20.2</ns0:v>
       </ns0:c>
       <ns0:c r="H100" s="1">
-        <ns0:f>ROUND(H99*1.2,2)</ns0:f>
-        <ns0:v>202568.16</ns0:v>
+        <ns0:v>11.508764333225681</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="101">
@@ -4172,8 +4145,7 @@
         <ns0:v>20.4</ns0:v>
       </ns0:c>
       <ns0:c r="H101" s="1">
-        <ns0:f>ROUND(H100*1.2,2)</ns0:f>
-        <ns0:v>243081.79</ns0:v>
+        <ns0:v>11.936168644175979</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="102">
@@ -4204,8 +4176,7 @@
         <ns0:v>20.6</ns0:v>
       </ns0:c>
       <ns0:c r="H102" s="1">
-        <ns0:f>ROUND(H101*1.2,2)</ns0:f>
-        <ns0:v>291698.15</ns0:v>
+        <ns0:v>12.379445592685771</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="103">
@@ -4236,8 +4207,7 @@
         <ns0:v>20.8</ns0:v>
       </ns0:c>
       <ns0:c r="H103" s="1">
-        <ns0:f>ROUND(H102*1.2,2)</ns0:f>
-        <ns0:v>350037.78</ns0:v>
+        <ns0:v>12.839184645488633</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="104">
@@ -4268,8 +4238,7 @@
         <ns0:v>21</ns0:v>
       </ns0:c>
       <ns0:c r="H104" s="1">
-        <ns0:f>ROUND(H103*1.2,2)</ns0:f>
-        <ns0:v>420045.34</ns0:v>
+        <ns0:v>13.315997160514792</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="105">
@@ -4300,8 +4269,7 @@
         <ns0:v>21.2</ns0:v>
       </ns0:c>
       <ns0:c r="H105" s="1">
-        <ns0:f>ROUND(H104*1.2,2)</ns0:f>
-        <ns0:v>504054.41</ns0:v>
+        <ns0:v>13.810517199870818</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="106">
@@ -4332,8 +4300,7 @@
         <ns0:v>21.4</ns0:v>
       </ns0:c>
       <ns0:c r="H106" s="1">
-        <ns0:f>ROUND(H105*1.2,2)</ns0:f>
-        <ns0:v>604865.29</ns0:v>
+        <ns0:v>14.323402373011174</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="107">
@@ -4364,8 +4331,7 @@
         <ns0:v>21.6</ns0:v>
       </ns0:c>
       <ns0:c r="H107" s="1">
-        <ns0:f>ROUND(H106*1.2,2)</ns0:f>
-        <ns0:v>725838.35</ns0:v>
+        <ns0:v>14.855334711222923</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="108">
@@ -4396,8 +4362,7 @@
         <ns0:v>21.8</ns0:v>
       </ns0:c>
       <ns0:c r="H108" s="1">
-        <ns0:f>ROUND(H107*1.2,2)</ns0:f>
-        <ns0:v>871006.02</ns0:v>
+        <ns0:v>15.40702157458636</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="109">
@@ -4428,8 +4393,7 @@
         <ns0:v>22</ns0:v>
       </ns0:c>
       <ns0:c r="H109" s="1">
-        <ns0:f>ROUND(H108*1.2,2)</ns0:f>
-        <ns0:v>1045207.22</ns0:v>
+        <ns0:v>15.97919659261775</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="110">
@@ -4460,8 +4424,7 @@
         <ns0:v>22.2</ns0:v>
       </ns0:c>
       <ns0:c r="H110" s="1">
-        <ns0:f>ROUND(H109*1.2,2)</ns0:f>
-        <ns0:v>1254248.66</ns0:v>
+        <ns0:v>16.57262063984498</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="111">
@@ -4492,8 +4455,7 @@
         <ns0:v>22.4</ns0:v>
       </ns0:c>
       <ns0:c r="H111" s="1">
-        <ns0:f>ROUND(H110*1.2,2)</ns0:f>
-        <ns0:v>1505098.39</ns0:v>
+        <ns0:v>17.18808284761341</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="112">
@@ -4524,8 +4486,7 @@
         <ns0:v>22.6</ns0:v>
       </ns0:c>
       <ns0:c r="H112" s="1">
-        <ns0:f>ROUND(H111*1.2,2)</ns0:f>
-        <ns0:v>1806118.07</ns0:v>
+        <ns0:v>17.826401653467506</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="113">
@@ -4556,8 +4517,7 @@
         <ns0:v>22.8</ns0:v>
       </ns0:c>
       <ns0:c r="H113" s="1">
-        <ns0:f>ROUND(H112*1.2,2)</ns0:f>
-        <ns0:v>2167341.68</ns0:v>
+        <ns0:v>18.48842588950363</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="114">
@@ -4588,8 +4548,7 @@
         <ns0:v>23</ns0:v>
       </ns0:c>
       <ns0:c r="H114" s="1">
-        <ns0:f>ROUND(H113*1.2,2)</ns0:f>
-        <ns0:v>2600810.02</ns0:v>
+        <ns0:v>19.1750359111413</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="115">
@@ -4620,8 +4579,7 @@
         <ns0:v>23.2</ns0:v>
       </ns0:c>
       <ns0:c r="H115" s="1">
-        <ns0:f>ROUND(H114*1.2,2)</ns0:f>
-        <ns0:v>3120972.02</ns0:v>
+        <ns0:v>19.887144767813968</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="116">
@@ -4652,8 +4610,7 @@
         <ns0:v>23.4</ns0:v>
       </ns0:c>
       <ns0:c r="H116" s="1">
-        <ns0:f>ROUND(H115*1.2,2)</ns0:f>
-        <ns0:v>3745166.42</ns0:v>
+        <ns0:v>20.625699417136094</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="117">
@@ -4684,8 +4641,7 @@
         <ns0:v>23.6</ns0:v>
       </ns0:c>
       <ns0:c r="H117" s="1">
-        <ns0:f>ROUND(H116*1.2,2)</ns0:f>
-        <ns0:v>4494199.7</ns0:v>
+        <ns0:v>21.39168198416101</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="118">
@@ -4716,8 +4672,7 @@
         <ns0:v>23.8</ns0:v>
       </ns0:c>
       <ns0:c r="H118" s="1">
-        <ns0:f>ROUND(H117*1.2,2)</ns0:f>
-        <ns0:v>5393039.64</ns0:v>
+        <ns0:v>22.186111067404354</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="119">
@@ -4748,8 +4703,7 @@
         <ns0:v>24</ns0:v>
       </ns0:c>
       <ns0:c r="H119" s="1">
-        <ns0:f>ROUND(H118*1.2,2)</ns0:f>
-        <ns0:v>6471647.57</ns0:v>
+        <ns0:v>23.01004309336956</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="120">
@@ -4780,8 +4734,7 @@
         <ns0:v>24.2000000000001</ns0:v>
       </ns0:c>
       <ns0:c r="H120" s="1">
-        <ns0:f>ROUND(H119*1.2,2)</ns0:f>
-        <ns0:v>7765977.08</ns0:v>
+        <ns0:v>23.86457372137676</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="121">
@@ -4812,8 +4765,7 @@
         <ns0:v>24.4000000000001</ns0:v>
       </ns0:c>
       <ns0:c r="H121" s="1">
-        <ns0:f>ROUND(H120*1.2,2)</ns0:f>
-        <ns0:v>9319172.5</ns0:v>
+        <ns0:v>24.750839300563314</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="122">
@@ -4844,8 +4796,7 @@
         <ns0:v>24.6000000000001</ns0:v>
       </ns0:c>
       <ns0:c r="H122" s="1">
-        <ns0:f>ROUND(H121*1.2,2)</ns0:f>
-        <ns0:v>11183007</ns0:v>
+        <ns0:v>25.67001838099321</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="123">
@@ -4876,8 +4827,7 @@
         <ns0:v>24.8000000000001</ns0:v>
       </ns0:c>
       <ns0:c r="H123" s="1">
-        <ns0:f>ROUND(H122*1.2,2)</ns0:f>
-        <ns0:v>13419608.4</ns0:v>
+        <ns0:v>26.623333280885227</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="124">
@@ -4908,8 +4858,7 @@
         <ns0:v>25.0000000000001</ns0:v>
       </ns0:c>
       <ns0:c r="H124" s="1">
-        <ns0:f>ROUND(H123*1.2,2)</ns0:f>
-        <ns0:v>16103530.08</ns0:v>
+        <ns0:v>27.61205171204347</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="125">
@@ -4940,8 +4889,7 @@
         <ns0:v>25.2000000000001</ns0:v>
       </ns0:c>
       <ns0:c r="H125" s="1">
-        <ns0:f>ROUND(H124*1.2,2)</ns0:f>
-        <ns0:v>19324236.1</ns0:v>
+        <ns0:v>28.637488465652115</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="126">
@@ -4972,8 +4920,7 @@
         <ns0:v>25.4000000000001</ns0:v>
       </ns0:c>
       <ns0:c r="H126" s="1">
-        <ns0:f>ROUND(H125*1.2,2)</ns0:f>
-        <ns0:v>23189083.32</ns0:v>
+        <ns0:v>29.701007160675974</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="127">
@@ -5004,8 +4951,7 @@
         <ns0:v>25.6000000000001</ns0:v>
       </ns0:c>
       <ns0:c r="H127" s="1">
-        <ns0:f>ROUND(H126*1.2,2)</ns0:f>
-        <ns0:v>27826899.98</ns0:v>
+        <ns0:v>30.80402205719185</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="128">
@@ -5036,8 +4982,7 @@
         <ns0:v>25.8000000000001</ns0:v>
       </ns0:c>
       <ns0:c r="H128" s="1">
-        <ns0:f>ROUND(H127*1.2,2)</ns0:f>
-        <ns0:v>33392279.98</ns0:v>
+        <ns0:v>31.94799993706227</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="129">
@@ -5068,8 +5013,7 @@
         <ns0:v>26.0000000000001</ns0:v>
       </ns0:c>
       <ns0:c r="H129" s="1">
-        <ns0:f>ROUND(H128*1.2,2)</ns0:f>
-        <ns0:v>40070735.98</ns0:v>
+        <ns0:v>33.134462054452165</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="130">
@@ -5100,8 +5044,7 @@
         <ns0:v>26.2000000000001</ns0:v>
       </ns0:c>
       <ns0:c r="H130" s="1">
-        <ns0:f>ROUND(H129*1.2,2)</ns0:f>
-        <ns0:v>48084883.18</ns0:v>
+        <ns0:v>34.364986158782536</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="131">
@@ -5132,8 +5075,7 @@
         <ns0:v>26.4000000000001</ns0:v>
       </ns0:c>
       <ns0:c r="H131" s="1">
-        <ns0:f>ROUND(H130*1.2,2)</ns0:f>
-        <ns0:v>57701859.82</ns0:v>
+        <ns0:v>35.64120859281117</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="132">
@@ -5164,8 +5106,7 @@
         <ns0:v>26.6000000000001</ns0:v>
       </ns0:c>
       <ns0:c r="H132" s="1">
-        <ns0:f>ROUND(H131*1.2,2)</ns0:f>
-        <ns0:v>69242231.78</ns0:v>
+        <ns0:v>36.96482646863022</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="133">
@@ -5196,8 +5137,7 @@
         <ns0:v>26.8000000000001</ns0:v>
       </ns0:c>
       <ns0:c r="H133" s="1">
-        <ns0:f>ROUND(H132*1.2,2)</ns0:f>
-        <ns0:v>83090678.14</ns0:v>
+        <ns0:v>38.33759992447472</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="134">
@@ -5228,8 +5168,7 @@
         <ns0:v>27.0000000000001</ns0:v>
       </ns0:c>
       <ns0:c r="H134" s="1">
-        <ns0:f>ROUND(H133*1.2,2)</ns0:f>
-        <ns0:v>99708813.77</ns0:v>
+        <ns0:v>39.76135446534259</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="135">
@@ -5260,8 +5199,7 @@
         <ns0:v>27.2000000000001</ns0:v>
       </ns0:c>
       <ns0:c r="H135" s="1">
-        <ns0:f>ROUND(H134*1.2,2)</ns0:f>
-        <ns0:v>119650576.52</ns0:v>
+        <ns0:v>41.23798339053904</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="136">
@@ -5292,8 +5230,7 @@
         <ns0:v>27.4000000000001</ns0:v>
       </ns0:c>
       <ns0:c r="H136" s="1">
-        <ns0:f>ROUND(H135*1.2,2)</ns0:f>
-        <ns0:v>143580691.82</ns0:v>
+        <ns0:v>42.7694503113734</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="137">
@@ -5324,8 +5261,7 @@
         <ns0:v>27.6000000000001</ns0:v>
       </ns0:c>
       <ns0:c r="H137" s="1">
-        <ns0:f>ROUND(H136*1.2,2)</ns0:f>
-        <ns0:v>172296830.18</ns0:v>
+        <ns0:v>44.357791762356264</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="138">
@@ -5356,8 +5292,7 @@
         <ns0:v>27.8000000000001</ns0:v>
       </ns0:c>
       <ns0:c r="H138" s="1">
-        <ns0:f>ROUND(H137*1.2,2)</ns0:f>
-        <ns0:v>206756196.22</ns0:v>
+        <ns0:v>46.00511990936967</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="139">
@@ -5388,8 +5323,7 @@
         <ns0:v>28.0000000000001</ns0:v>
       </ns0:c>
       <ns0:c r="H139" s="1">
-        <ns0:f>ROUND(H138*1.2,2)</ns0:f>
-        <ns0:v>248107435.46</ns0:v>
+        <ns0:v>47.71362535841111</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="140">
@@ -5420,8 +5354,7 @@
         <ns0:v>28.2000000000001</ns0:v>
       </ns0:c>
       <ns0:c r="H140" s="1">
-        <ns0:f>ROUND(H139*1.2,2)</ns0:f>
-        <ns0:v>297728922.55</ns0:v>
+        <ns0:v>49.48558006864685</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="141">
@@ -5452,8 +5385,7 @@
         <ns0:v>28.4000000000001</ns0:v>
       </ns0:c>
       <ns0:c r="H141" s="1">
-        <ns0:f>ROUND(H140*1.2,2)</ns0:f>
-        <ns0:v>357274707.06</ns0:v>
+        <ns0:v>51.32334037364808</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="142">
@@ -5484,8 +5416,7 @@
         <ns0:v>28.6000000000001</ns0:v>
       </ns0:c>
       <ns0:c r="H142" s="1">
-        <ns0:f>ROUND(H141*1.2,2)</ns0:f>
-        <ns0:v>428729648.47</ns0:v>
+        <ns0:v>53.22935011482751</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="143">
@@ -5516,8 +5447,7 @@
         <ns0:v>28.8000000000001</ns0:v>
       </ns0:c>
       <ns0:c r="H143" s="1">
-        <ns0:f>ROUND(H142*1.2,2)</ns0:f>
-        <ns0:v>514475578.16</ns0:v>
+        <ns0:v>55.2061438912436</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="144">
@@ -5548,8 +5478,7 @@
         <ns0:v>29.0000000000001</ns0:v>
       </ns0:c>
       <ns0:c r="H144" s="1">
-        <ns0:f>ROUND(H143*1.2,2)</ns0:f>
-        <ns0:v>617370693.79</ns0:v>
+        <ns0:v>57.25635043009333</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="145">
@@ -5580,8 +5509,7 @@
         <ns0:v>29.2000000000001</ns0:v>
       </ns0:c>
       <ns0:c r="H145" s="1">
-        <ns0:f>ROUND(H144*1.2,2)</ns0:f>
-        <ns0:v>740844832.55</ns0:v>
+        <ns0:v>59.382696082376214</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="146">
@@ -5612,8 +5540,7 @@
         <ns0:v>29.4000000000001</ns0:v>
       </ns0:c>
       <ns0:c r="H146" s="1">
-        <ns0:f>ROUND(H145*1.2,2)</ns0:f>
-        <ns0:v>889013799.06</ns0:v>
+        <ns0:v>61.58800844837769</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="147">
@@ -5644,8 +5571,7 @@
         <ns0:v>29.6000000000001</ns0:v>
       </ns0:c>
       <ns0:c r="H147" s="1">
-        <ns0:f>ROUND(H146*1.2,2)</ns0:f>
-        <ns0:v>1066816558.87</ns0:v>
+        <ns0:v>63.875220137793015</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="148">
@@ -5676,8 +5602,7 @@
         <ns0:v>29.8000000000001</ns0:v>
       </ns0:c>
       <ns0:c r="H148" s="1">
-        <ns0:f>ROUND(H147*1.2,2)</ns0:f>
-        <ns0:v>1280179870.64</ns0:v>
+        <ns0:v>66.24737266949231</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="149">
@@ -5708,8 +5633,7 @@
         <ns0:v>30.0000000000001</ns0:v>
       </ns0:c>
       <ns0:c r="H149" s="1">
-        <ns0:f>ROUND(H148*1.2,2)</ns0:f>
-        <ns0:v>1536215844.77</ns0:v>
+        <ns0:v>68.70762051611199</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="150">
@@ -5740,8 +5664,7 @@
         <ns0:v>30.2000000000001</ns0:v>
       </ns0:c>
       <ns0:c r="H150" s="1">
-        <ns0:f>ROUND(H149*1.2,2)</ns0:f>
-        <ns0:v>1843459013.72</ns0:v>
+        <ns0:v>71.25923529885145</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="151">
@@ -5772,8 +5695,7 @@
         <ns0:v>30.4000000000001</ns0:v>
       </ns0:c>
       <ns0:c r="H151" s="1">
-        <ns0:f>ROUND(H150*1.2,2)</ns0:f>
-        <ns0:v>2212150816.46</ns0:v>
+        <ns0:v>73.90561013805322</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="152">
@@ -5804,8 +5726,7 @@
         <ns0:v>30.6000000000001</ns0:v>
       </ns0:c>
       <ns0:c r="H152" s="1">
-        <ns0:f>ROUND(H151*1.2,2)</ns0:f>
-        <ns0:v>2654580979.75</ns0:v>
+        <ns0:v>76.65026416535162</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="153">
@@ -5836,8 +5757,7 @@
         <ns0:v>30.8000000000001</ns0:v>
       </ns0:c>
       <ns0:c r="H153" s="1">
-        <ns0:f>ROUND(H152*1.2,2)</ns0:f>
-        <ns0:v>3185497175.7</ns0:v>
+        <ns0:v>79.49684720339077</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="154">
@@ -5868,8 +5788,7 @@
         <ns0:v>31.0000000000001</ns0:v>
       </ns0:c>
       <ns0:c r="H154" s="1">
-        <ns0:f>ROUND(H153*1.2,2)</ns0:f>
-        <ns0:v>3822596610.84</ns0:v>
+        <ns0:v>82.44914461933439</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="155">
@@ -5900,8 +5819,7 @@
         <ns0:v>31.2000000000001</ns0:v>
       </ns0:c>
       <ns0:c r="H155" s="1">
-        <ns0:f>ROUND(H154*1.2,2)</ns0:f>
-        <ns0:v>4587115933.01</ns0:v>
+        <ns0:v>85.51108235862175</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="156">
@@ -5932,8 +5850,7 @@
         <ns0:v>31.4000000000001</ns0:v>
       </ns0:c>
       <ns0:c r="H156" s="1">
-        <ns0:f>ROUND(H155*1.2,2)</ns0:f>
-        <ns0:v>5504539119.61</ns0:v>
+        <ns0:v>88.68673216566387</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="157">
@@ -5964,8 +5881,7 @@
         <ns0:v>31.6000000000001</ns0:v>
       </ns0:c>
       <ns0:c r="H157" s="1">
-        <ns0:f>ROUND(H156*1.2,2)</ns0:f>
-        <ns0:v>6605446943.53</ns0:v>
+        <ns0:v>91.98031699842193</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="158">
@@ -5996,8 +5912,7 @@
         <ns0:v>31.8000000000001</ns0:v>
       </ns0:c>
       <ns0:c r="H158" s="1">
-        <ns0:f>ROUND(H157*1.2,2)</ns0:f>
-        <ns0:v>7926536332.24</ns0:v>
+        <ns0:v>95.39621664406893</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="159">
@@ -6028,8 +5943,7 @@
         <ns0:v>32.0000000000001</ns0:v>
       </ns0:c>
       <ns0:c r="H159" s="1">
-        <ns0:f>ROUND(H158*1.2,2)</ns0:f>
-        <ns0:v>9511843598.69</ns0:v>
+        <ns0:v>98.93897354320126</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="160">
@@ -6060,8 +5974,7 @@
         <ns0:v>32.2000000000001</ns0:v>
       </ns0:c>
       <ns0:c r="H160" s="1">
-        <ns0:f>ROUND(H159*1.2,2)</ns0:f>
-        <ns0:v>11414212318.43</ns0:v>
+        <ns0:v>102.61329883034608</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="161">
@@ -6092,8 +6005,7 @@
         <ns0:v>32.4000000000001</ns0:v>
       </ns0:c>
       <ns0:c r="H161" s="1">
-        <ns0:f>ROUND(H160*1.2,2)</ns0:f>
-        <ns0:v>13697054782.12</ns0:v>
+        <ns0:v>106.42407859879664</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="162">
@@ -6124,8 +6036,7 @@
         <ns0:v>32.6000000000001</ns0:v>
       </ns0:c>
       <ns0:c r="H162" s="1">
-        <ns0:f>ROUND(H161*1.2,2)</ns0:f>
-        <ns0:v>16436465738.54</ns0:v>
+        <ns0:v>110.3763803981063</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="163">
@@ -6156,8 +6067,7 @@
         <ns0:v>32.8000000000001</ns0:v>
       </ns0:c>
       <ns0:c r="H163" s="1">
-        <ns0:f>ROUND(H162*1.2,2)</ns0:f>
-        <ns0:v>19723758886.25</ns0:v>
+        <ns0:v>114.4754599728827</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="164">
@@ -6188,8 +6098,7 @@
         <ns0:v>33.0000000000001</ns0:v>
       </ns0:c>
       <ns0:c r="H164" s="1">
-        <ns0:f>ROUND(H163*1.2,2)</ns0:f>
-        <ns0:v>23668510663.5</ns0:v>
+        <ns0:v>118.7267682518415</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="165">
@@ -6220,8 +6129,7 @@
         <ns0:v>33.2000000000001</ns0:v>
       </ns0:c>
       <ns0:c r="H165" s="1">
-        <ns0:f>ROUND(H164*1.2,2)</ns0:f>
-        <ns0:v>28402212796.2</ns0:v>
+        <ns0:v>123.1359585964153</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="166">
@@ -6252,8 +6160,7 @@
         <ns0:v>33.4000000000001</ns0:v>
       </ns0:c>
       <ns0:c r="H166" s="1">
-        <ns0:f>ROUND(H165*1.2,2)</ns0:f>
-        <ns0:v>34082655355.44</ns0:v>
+        <ns0:v>127.70889431855596</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="167">
@@ -6284,8 +6191,7 @@
         <ns0:v>33.6000000000001</ns0:v>
       </ns0:c>
       <ns0:c r="H167" s="1">
-        <ns0:f>ROUND(H166*1.2,2)</ns0:f>
-        <ns0:v>40899186426.53</ns0:v>
+        <ns0:v>132.45165647772757</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="168">
@@ -6316,8 +6222,7 @@
         <ns0:v>33.8000000000001</ns0:v>
       </ns0:c>
       <ns0:c r="H168" s="1">
-        <ns0:f>ROUND(H167*1.2,2)</ns0:f>
-        <ns0:v>49079023711.84</ns0:v>
+        <ns0:v>137.37055196745925</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="169">
@@ -6348,8 +6253,7 @@
         <ns0:v>34.0000000000001</ns0:v>
       </ns0:c>
       <ns0:c r="H169" s="1">
-        <ns0:f>ROUND(H168*1.2,2)</ns0:f>
-        <ns0:v>58894828454.21</ns0:v>
+        <ns0:v>142.4721219022098</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="170">
@@ -6380,8 +6284,7 @@
         <ns0:v>34.2000000000001</ns0:v>
       </ns0:c>
       <ns0:c r="H170" s="1">
-        <ns0:f>ROUND(H169*1.2,2)</ns0:f>
-        <ns0:v>70673794145.05</ns0:v>
+        <ns0:v>147.76315031569837</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="171">
@@ -6412,8 +6315,7 @@
         <ns0:v>34.4000000000001</ns0:v>
       </ns0:c>
       <ns0:c r="H171" s="1">
-        <ns0:f>ROUND(H170*1.2,2)</ns0:f>
-        <ns0:v>84808552974.06</ns0:v>
+        <ns0:v>153.25067318226715</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="172">
@@ -6444,8 +6346,7 @@
         <ns0:v>34.6000000000001</ns0:v>
       </ns0:c>
       <ns0:c r="H172" s="1">
-        <ns0:f>ROUND(H171*1.2,2)</ns0:f>
-        <ns0:v>101770263568.87</ns0:v>
+        <ns0:v>158.94198777327307</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="173">
@@ -6476,8 +6377,7 @@
         <ns0:v>34.8000000000001</ns0:v>
       </ns0:c>
       <ns0:c r="H173" s="1">
-        <ns0:f>ROUND(H172*1.2,2)</ns0:f>
-        <ns0:v>122124316282.64</ns0:v>
+        <ns0:v>164.84466236095108</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="174">
@@ -6508,8 +6408,7 @@
         <ns0:v>35.0000000000001</ns0:v>
       </ns0:c>
       <ns0:c r="H174" s="1">
-        <ns0:f>ROUND(H173*1.2,2)</ns0:f>
-        <ns0:v>146549179539.17</ns0:v>
+        <ns0:v>170.96654628265176</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="175">
@@ -6540,8 +6439,7 @@
         <ns0:v>35.2000000000001</ns0:v>
       </ns0:c>
       <ns0:c r="H175" s="1">
-        <ns0:f>ROUND(H174*1.2,2)</ns0:f>
-        <ns0:v>175859015447</ns0:v>
+        <ns0:v>177.315780378838</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="176">
@@ -6572,8 +6470,7 @@
         <ns0:v>35.4000000000001</ns0:v>
       </ns0:c>
       <ns0:c r="H176" s="1">
-        <ns0:f>ROUND(H175*1.2,2)</ns0:f>
-        <ns0:v>211030818536.4</ns0:v>
+        <ns0:v>183.90080781872058</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="177">
@@ -6604,8 +6501,7 @@
         <ns0:v>35.6000000000001</ns0:v>
       </ns0:c>
       <ns0:c r="H177" s="1">
-        <ns0:f>ROUND(H176*1.2,2)</ns0:f>
-        <ns0:v>253236982243.68</ns0:v>
+        <ns0:v>190.73038532792768</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="178">
@@ -6636,8 +6532,7 @@
         <ns0:v>35.8000000000001</ns0:v>
       </ns0:c>
       <ns0:c r="H178" s="1">
-        <ns0:f>ROUND(H177*1.2,2)</ns0:f>
-        <ns0:v>303884378692.42</ns0:v>
+        <ns0:v>197.81359483314128</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="179">
@@ -6668,8 +6563,7 @@
         <ns0:v>36.0000000000001</ns0:v>
       </ns0:c>
       <ns0:c r="H179" s="1">
-        <ns0:f>ROUND(H178*1.2,2)</ns0:f>
-        <ns0:v>364661254430.9</ns0:v>
+        <ns0:v>205.1598555391821</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="180">
@@ -6700,8 +6594,7 @@
         <ns0:v>36.2000000000001</ns0:v>
       </ns0:c>
       <ns0:c r="H180" s="1">
-        <ns0:f>ROUND(H179*1.2,2)</ns0:f>
-        <ns0:v>437593505317.08</ns0:v>
+        <ns0:v>212.77893645460563</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="181">
@@ -6732,8 +6625,7 @@
         <ns0:v>36.4000000000001</ns0:v>
       </ns0:c>
       <ns0:c r="H181" s="1">
-        <ns0:f>ROUND(H180*1.2,2)</ns0:f>
-        <ns0:v>525112206380.5</ns0:v>
+        <ns0:v>220.68096938246467</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="182">
@@ -6764,8 +6656,7 @@
         <ns0:v>36.6000000000001</ns0:v>
       </ns0:c>
       <ns0:c r="H182" s="1">
-        <ns0:f>ROUND(H181*1.2,2)</ns0:f>
-        <ns0:v>630134647656.6</ns0:v>
+        <ns0:v>228.8764623935132</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="183">
@@ -6796,8 +6687,7 @@
         <ns0:v>36.8000000000001</ns0:v>
       </ns0:c>
       <ns0:c r="H183" s="1">
-        <ns0:f>ROUND(H182*1.2,2)</ns0:f>
-        <ns0:v>756161577187.92</ns0:v>
+        <ns0:v>237.37631379976955</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="184">
@@ -6828,8 +6718,7 @@
         <ns0:v>37.0000000000001</ns0:v>
       </ns0:c>
       <ns0:c r="H184" s="1">
-        <ns0:f>ROUND(H183*1.2,2)</ns0:f>
-        <ns0:v>907393892625.5</ns0:v>
+        <ns0:v>246.19182664701853</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="185">
@@ -6860,8 +6749,7 @@
         <ns0:v>37.2000000000001</ns0:v>
       </ns0:c>
       <ns0:c r="H185" s="1">
-        <ns0:f>ROUND(H184*1.2,2)</ns0:f>
-        <ns0:v>1088872671150.6</ns0:v>
+        <ns0:v>255.33472374552673</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="186">
@@ -6892,8 +6780,7 @@
         <ns0:v>37.4000000000001</ns0:v>
       </ns0:c>
       <ns0:c r="H186" s="1">
-        <ns0:f>ROUND(H185*1.2,2)</ns0:f>
-        <ns0:v>1306647205380.72</ns0:v>
+        <ns0:v>264.8171632589576</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="187">
@@ -6924,8 +6811,7 @@
         <ns0:v>37.6000000000001</ns0:v>
       </ns0:c>
       <ns0:c r="H187" s="1">
-        <ns0:f>ROUND(H186*1.2,2)</ns0:f>
-        <ns0:v>1567976646456.86</ns0:v>
+        <ns0:v>274.65175487221586</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="188">
@@ -6956,8 +6842,7 @@
         <ns0:v>37.8000000000001</ns0:v>
       </ns0:c>
       <ns0:c r="H188" s="1">
-        <ns0:f>ROUND(H187*1.2,2)</ns0:f>
-        <ns0:v>1881571975748.23</ns0:v>
+        <ns0:v>284.85157655972347</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="189">
@@ -6988,8 +6873,7 @@
         <ns0:v>38.0000000000001</ns0:v>
       </ns0:c>
       <ns0:c r="H189" s="1">
-        <ns0:f>ROUND(H188*1.2,2)</ns0:f>
-        <ns0:v>2257886370897.88</ns0:v>
+        <ns0:v>295.43019197642224</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="190">
@@ -7020,8 +6904,7 @@
         <ns0:v>38.2000000000001</ns0:v>
       </ns0:c>
       <ns0:c r="H190" s="1">
-        <ns0:f>ROUND(H189*1.2,2)</ns0:f>
-        <ns0:v>2709463645077.46</ns0:v>
+        <ns0:v>306.4016684946321</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="191">
@@ -7052,8 +6935,7 @@
         <ns0:v>38.4000000000001</ns0:v>
       </ns0:c>
       <ns0:c r="H191" s="1">
-        <ns0:f>ROUND(H190*1.2,2)</ns0:f>
-        <ns0:v>3251356374092.95</ns0:v>
+        <ns0:v>317.7805959107491</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="192">
@@ -7084,8 +6966,7 @@
         <ns0:v>38.6000000000001</ns0:v>
       </ns0:c>
       <ns0:c r="H192" s="1">
-        <ns0:f>ROUND(H191*1.2,2)</ns0:f>
-        <ns0:v>3901627648911.54</ns0:v>
+        <ns0:v>329.58210584665903</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="193">
@@ -7116,8 +6997,7 @@
         <ns0:v>38.8000000000001</ns0:v>
       </ns0:c>
       <ns0:c r="H193" s="1">
-        <ns0:f>ROUND(H192*1.2,2)</ns0:f>
-        <ns0:v>4681953178693.85</ns0:v>
+        <ns0:v>341.82189187166813</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="194">
@@ -7148,8 +7028,7 @@
         <ns0:v>39.0000000000001</ns0:v>
       </ns0:c>
       <ns0:c r="H194" s="1">
-        <ns0:f>ROUND(H193*1.2,2)</ns0:f>
-        <ns0:v>5618343814432.62</ns0:v>
+        <ns0:v>354.51623037170685</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="195">
@@ -7180,8 +7059,7 @@
         <ns0:v>39.2000000000001</ns0:v>
       </ns0:c>
       <ns0:c r="H195" s="1">
-        <ns0:f>ROUND(H194*1.2,2)</ns0:f>
-        <ns0:v>6742012577319.14</ns0:v>
+        <ns0:v>367.68200219355845</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="196">
@@ -7212,8 +7090,7 @@
         <ns0:v>39.4000000000001</ns0:v>
       </ns0:c>
       <ns0:c r="H196" s="1">
-        <ns0:f>ROUND(H195*1.2,2)</ns0:f>
-        <ns0:v>8090415092782.97</ns0:v>
+        <ns0:v>381.33671509289894</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="197">
@@ -7244,8 +7121,7 @@
         <ns0:v>39.6000000000001</ns0:v>
       </ns0:c>
       <ns0:c r="H197" s="1">
-        <ns0:f>ROUND(H196*1.2,2)</ns0:f>
-        <ns0:v>9708498111339.56</ns0:v>
+        <ns0:v>395.49852701599053</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="198">
@@ -7276,8 +7152,7 @@
         <ns0:v>39.8000000000001</ns0:v>
       </ns0:c>
       <ns0:c r="H198" s="1">
-        <ns0:f>ROUND(H197*1.2,2)</ns0:f>
-        <ns0:v>11650197733607.5</ns0:v>
+        <ns0:v>410.1862702460017</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="199">
@@ -7308,8 +7183,7 @@
         <ns0:v>40.0000000000001</ns0:v>
       </ns0:c>
       <ns0:c r="H199" s="1">
-        <ns0:f>ROUND(H198*1.2,2)</ns0:f>
-        <ns0:v>13980237280329</ns0:v>
+        <ns0:v>425.41947644604824</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="200">
@@ -7340,8 +7214,7 @@
         <ns0:v>40.2000000000001</ns0:v>
       </ns0:c>
       <ns0:c r="H200" s="1">
-        <ns0:f>ROUND(H199*1.2,2)</ns0:f>
-        <ns0:v>16776284736394.8</ns0:v>
+        <ns0:v>441.2184026322701</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="201">
@@ -7372,8 +7245,7 @@
         <ns0:v>40.4000000000001</ns0:v>
       </ns0:c>
       <ns0:c r="H201" s="1">
-        <ns0:f>ROUND(H200*1.2,2)</ns0:f>
-        <ns0:v>20131541683673.8</ns0:v>
+        <ns0:v>457.6040581114787</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="202">
@@ -7404,8 +7276,7 @@
         <ns0:v>40.6000000000001</ns0:v>
       </ns0:c>
       <ns0:c r="H202" s="1">
-        <ns0:f>ROUND(H201*1.2,2)</ns0:f>
-        <ns0:v>24157850020408.6</ns0:v>
+        <ns0:v>474.5982324191886</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="203">
@@ -7436,8 +7307,7 @@
         <ns0:v>40.8000000000001</ns0:v>
       </ns0:c>
       <ns0:c r="H203" s="1">
-        <ns0:f>ROUND(H202*1.2,2)</ns0:f>
-        <ns0:v>28989420024490.3</ns0:v>
+        <ns0:v>492.223524295202</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="204">
@@ -7468,8 +7338,7 @@
         <ns0:v>41.0000000000001</ns0:v>
       </ns0:c>
       <ns0:c r="H204" s="1">
-        <ns0:f>ROUND(H203*1.2,2)</ns0:f>
-        <ns0:v>34787304029388.4</ns0:v>
+        <ns0:v>510.5033717352579</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="205">
@@ -7500,8 +7369,7 @@
         <ns0:v>41.2000000000001</ns0:v>
       </ns0:c>
       <ns0:c r="H205" s="1">
-        <ns0:f>ROUND(H204*1.2,2)</ns0:f>
-        <ns0:v>41744764835266.1</ns0:v>
+        <ns0:v>529.4620831587241</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="206">
@@ -7532,8 +7400,7 @@
         <ns0:v>41.4000000000001</ns0:v>
       </ns0:c>
       <ns0:c r="H206" s="1">
-        <ns0:f>ROUND(H205*1.2,2)</ns0:f>
-        <ns0:v>50093717802319.3</ns0:v>
+        <ns0:v>549.1248697337744</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="207">
@@ -7564,8 +7431,7 @@
         <ns0:v>41.6000000000001</ns0:v>
       </ns0:c>
       <ns0:c r="H207" s="1">
-        <ns0:f>ROUND(H206*1.2,2)</ns0:f>
-        <ns0:v>60112461362783.2</ns0:v>
+        <ns0:v>569.5178789030264</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="208">
@@ -7596,8 +7462,7 @@
         <ns0:v>41.8000000000001</ns0:v>
       </ns0:c>
       <ns0:c r="H208" s="1">
-        <ns0:f>ROUND(H207*1.2,2)</ns0:f>
-        <ns0:v>72134953635339.9</ns0:v>
+        <ns0:v>590.6682291542425</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="209">
@@ -7628,8 +7493,7 @@
         <ns0:v>42.0000000000001</ns0:v>
       </ns0:c>
       <ns0:c r="H209" s="1">
-        <ns0:f>ROUND(H208*1.2,2)</ns0:f>
-        <ns0:v>86561944362407.9</ns0:v>
+        <ns0:v>612.6040460823094</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="210">
@@ -7660,8 +7524,7 @@
         <ns0:v>42.2000000000001</ns0:v>
       </ns0:c>
       <ns0:c r="H210" s="1">
-        <ns0:f>ROUND(H209*1.2,2)</ns0:f>
-        <ns0:v>103874333234889</ns0:v>
+        <ns0:v>635.3544997904689</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="211">
@@ -7692,8 +7555,7 @@
         <ns0:v>42.4000000000001</ns0:v>
       </ns0:c>
       <ns0:c r="H211" s="1">
-        <ns0:f>ROUND(H210*1.2,2)</ns0:f>
-        <ns0:v>124649199881867</ns0:v>
+        <ns0:v>658.9498436805293</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="212">
@@ -7724,8 +7586,7 @@
         <ns0:v>42.6000000000002</ns0:v>
       </ns0:c>
       <ns0:c r="H212" s="1">
-        <ns0:f>ROUND(H211*1.2,2)</ns0:f>
-        <ns0:v>149579039858240</ns0:v>
+        <ns0:v>683.4214546836316</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="213">
@@ -7756,8 +7617,7 @@
         <ns0:v>42.8000000000002</ns0:v>
       </ns0:c>
       <ns0:c r="H213" s="1">
-        <ns0:f>ROUND(H212*1.2,2)</ns0:f>
-        <ns0:v>179494847829888</ns0:v>
+        <ns0:v>708.8018749850909</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="214">
@@ -7788,8 +7648,7 @@
         <ns0:v>43.0000000000001</ns0:v>
       </ns0:c>
       <ns0:c r="H214" s="1">
-        <ns0:f>ROUND(H213*1.2,2)</ns0:f>
-        <ns0:v>215393817395866</ns0:v>
+        <ns0:v>735.1248552987713</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="215">
@@ -7820,8 +7679,7 @@
         <ns0:v>43.2000000000002</ns0:v>
       </ns0:c>
       <ns0:c r="H215" s="1">
-        <ns0:f>ROUND(H214*1.2,2)</ns0:f>
-        <ns0:v>258472580875039</ns0:v>
+        <ns0:v>762.4253997485628</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="216">
@@ -7852,8 +7710,7 @@
         <ns0:v>43.4000000000002</ns0:v>
       </ns0:c>
       <ns0:c r="H216" s="1">
-        <ns0:f>ROUND(H215*1.2,2)</ns0:f>
-        <ns0:v>310167097050047</ns0:v>
+        <ns0:v>790.7398124166351</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="217">
@@ -7884,8 +7741,7 @@
         <ns0:v>43.6000000000002</ns0:v>
       </ns0:c>
       <ns0:c r="H217" s="1">
-        <ns0:f>ROUND(H216*1.2,2)</ns0:f>
-        <ns0:v>372200516460056</ns0:v>
+        <ns0:v>820.1057456203579</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="218">
@@ -7916,8 +7772,7 @@
         <ns0:v>43.8000000000002</ns0:v>
       </ns0:c>
       <ns0:c r="H218" s="1">
-        <ns0:f>ROUND(H217*1.2,2)</ns0:f>
-        <ns0:v>446640619752067</ns0:v>
+        <ns0:v>850.562249982109</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="219">
@@ -7948,8 +7803,7 @@
         <ns0:v>44.0000000000002</ns0:v>
       </ns0:c>
       <ns0:c r="H219" s="1">
-        <ns0:f>ROUND(H218*1.2,2)</ns0:f>
-        <ns0:v>535968743702480</ns0:v>
+        <ns0:v>882.1498263585255</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="220">
@@ -7980,8 +7834,7 @@
         <ns0:v>44.2000000000002</ns0:v>
       </ns0:c>
       <ns0:c r="H220" s="1">
-        <ns0:f>ROUND(H219*1.2,2)</ns0:f>
-        <ns0:v>643162492442976</ns0:v>
+        <ns0:v>914.9104796982753</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="221">
@@ -8012,8 +7865,7 @@
         <ns0:v>44.4000000000002</ns0:v>
       </ns0:c>
       <ns0:c r="H221" s="1">
-        <ns0:f>ROUND(H220*1.2,2)</ns0:f>
-        <ns0:v>771794990931571</ns0:v>
+        <ns0:v>948.8877748999621</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="222">
@@ -8044,8 +7896,7 @@
         <ns0:v>44.6000000000002</ns0:v>
       </ns0:c>
       <ns0:c r="H222" s="1">
-        <ns0:f>ROUND(H221*1.2,2)</ns0:f>
-        <ns0:v>926153989117885</ns0:v>
+        <ns0:v>984.1268947444294</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="223">
@@ -8076,8 +7927,7 @@
         <ns0:v>44.8000000000002</ns0:v>
       </ns0:c>
       <ns0:c r="H223" s="1">
-        <ns0:f>ROUND(H222*1.2,2)</ns0:f>
-        <ns0:v>1111384786941460</ns0:v>
+        <ns0:v>1020.6746999785308</ns0:v>
       </ns0:c>
     </ns0:row>
   </ns0:sheetData>

</xml_diff>

<commit_message>
Propose conservative levels 8-20 difficulty with the level 21 entry preserved
</commit_message>
<xml_diff>
--- a/space-battleship/config_excel/level.xlsx
+++ b/space-battleship/config_excel/level.xlsx
@@ -1493,7 +1493,7 @@
         </ns0:is>
       </ns0:c>
       <ns0:c r="D11" s="1" t="n">
-        <ns0:v>1469.771567969084</ns0:v>
+        <ns0:v>1543.26014636753820</ns0:v>
       </ns0:c>
       <ns0:c r="E11" s="1" t="n">
         <ns0:v>1469.771567969084</ns0:v>
@@ -1521,7 +1521,7 @@
         </ns0:is>
       </ns0:c>
       <ns0:c r="D12" s="1" t="n">
-        <ns0:v>9100.438150002134</ns0:v>
+        <ns0:v>9555.46005750224070</ns0:v>
       </ns0:c>
       <ns0:c r="E12" s="1" t="n">
         <ns0:v>9100.438150002134</ns0:v>
@@ -1549,7 +1549,7 @@
         </ns0:is>
       </ns0:c>
       <ns0:c r="D13" s="1" t="n">
-        <ns0:v>56347.51435316666</ns0:v>
+        <ns0:v>59164.8900708249930</ns0:v>
       </ns0:c>
       <ns0:c r="E13" s="1" t="n">
         <ns0:v>56347.51435316666</ns0:v>
@@ -1577,10 +1577,10 @@
         </ns0:is>
       </ns0:c>
       <ns0:c r="D14" s="1" t="n">
-        <ns0:v>602880.1175788565</ns0:v>
+        <ns0:v>663168.129336742150</ns0:v>
       </ns0:c>
       <ns0:c r="E14" s="1" t="n">
-        <ns0:v>602880.1175788565</ns0:v>
+        <ns0:v>633024.123457799325</ns0:v>
       </ns0:c>
       <ns0:c r="F14" s="1" t="n">
         <ns0:v>18120.833112711232</ns0:v>
@@ -1605,10 +1605,10 @@
         </ns0:is>
       </ns0:c>
       <ns0:c r="D15" s="1" t="n">
-        <ns0:v>6450407.623907364</ns0:v>
+        <ns0:v>7095448.38629810040</ns0:v>
       </ns0:c>
       <ns0:c r="E15" s="1" t="n">
-        <ns0:v>6450407.623907364</ns0:v>
+        <ns0:v>6772928.00510273220</ns0:v>
       </ns0:c>
       <ns0:c r="F15" s="1" t="n">
         <ns0:v>56917.67271450579</ns0:v>
@@ -1633,10 +1633,10 @@
         </ns0:is>
       </ns0:c>
       <ns0:c r="D16" s="1" t="n">
-        <ns0:v>69014978.76834521</ns0:v>
+        <ns0:v>75916476.645179720</ns0:v>
       </ns0:c>
       <ns0:c r="E16" s="1" t="n">
-        <ns0:v>69014978.76834521</ns0:v>
+        <ns0:v>72465727.706762460</ns0:v>
       </ns0:c>
       <ns0:c r="F16" s="1" t="n">
         <ns0:v>178778.836882676</ns0:v>
@@ -1661,10 +1661,10 @@
         </ns0:is>
       </ns0:c>
       <ns0:c r="D17" s="1" t="n">
-        <ns0:v>738413379.7593849</ns0:v>
+        <ns0:v>812254717.735323390</ns0:v>
       </ns0:c>
       <ns0:c r="E17" s="1" t="n">
-        <ns0:v>738413379.7593849</ns0:v>
+        <ns0:v>775334048.747354145</ns0:v>
       </ns0:c>
       <ns0:c r="F17" s="1" t="n">
         <ns0:v>561545.6675019113</ns0:v>
@@ -1689,10 +1689,10 @@
         </ns0:is>
       </ns0:c>
       <ns0:c r="D18" s="1" t="n">
-        <ns0:v>7900521439.525051</ns0:v>
+        <ns0:v>8690573583.47755610</ns0:v>
       </ns0:c>
       <ns0:c r="E18" s="1" t="n">
-        <ns0:v>7900521439.525051</ns0:v>
+        <ns0:v>8295547511.50130355</ns0:v>
       </ns0:c>
       <ns0:c r="F18" s="1" t="n">
         <ns0:v>1763819.1532541711</ns0:v>
@@ -1717,10 +1717,10 @@
         </ns0:is>
       </ns0:c>
       <ns0:c r="D19" s="1" t="n">
-        <ns0:v>84530211298.0865</ns0:v>
+        <ns0:v>92983232427.895150</ns0:v>
       </ns0:c>
       <ns0:c r="E19" s="1" t="n">
-        <ns0:v>84530211298.0865</ns0:v>
+        <ns0:v>88756721862.990825</ns0:v>
       </ns0:c>
       <ns0:c r="F19" s="1" t="n">
         <ns0:v>5540169.189134865</ns0:v>
@@ -1745,10 +1745,10 @@
         </ns0:is>
       </ns0:c>
       <ns0:c r="D20" s="1" t="n">
-        <ns0:v>904415825815.2517</ns0:v>
+        <ns0:v>994857408396.776870</ns0:v>
       </ns0:c>
       <ns0:c r="E20" s="1" t="n">
-        <ns0:v>904415825815.2517</ns0:v>
+        <ns0:v>949636617106.014285</ns0:v>
       </ns0:c>
       <ns0:c r="F20" s="1" t="n">
         <ns0:v>17401712.974718027</ns0:v>
@@ -1773,10 +1773,10 @@
         </ns0:is>
       </ns0:c>
       <ns0:c r="D21" s="1" t="n">
-        <ns0:v>9676634819953.418</ns0:v>
+        <ns0:v>10644298301948.75980</ns0:v>
       </ns0:c>
       <ns0:c r="E21" s="1" t="n">
-        <ns0:v>9676634819953.418</ns0:v>
+        <ns0:v>10160466560951.08890</ns0:v>
       </ns0:c>
       <ns0:c r="F21" s="1" t="n">
         <ns0:v>54658910.967619196</ns0:v>
@@ -1801,10 +1801,10 @@
         </ns0:is>
       </ns0:c>
       <ns0:c r="D22" s="1" t="n">
-        <ns0:v>103533417666955.5</ns0:v>
+        <ns0:v>113886759433651.050</ns0:v>
       </ns0:c>
       <ns0:c r="E22" s="1" t="n">
-        <ns0:v>103533417666955.5</ns0:v>
+        <ns0:v>108710088550303.275</ns0:v>
       </ns0:c>
       <ns0:c r="F22" s="1" t="n">
         <ns0:v>171684049.29483864</ns0:v>
@@ -1829,10 +1829,10 @@
         </ns0:is>
       </ns0:c>
       <ns0:c r="D23" s="1" t="n">
-        <ns0:v>3323211666011343</ns0:v>
+        <ns0:v>3655532832612477.30</ns0:v>
       </ns0:c>
       <ns0:c r="E23" s="1" t="n">
-        <ns0:v>3323211666011343</ns0:v>
+        <ns0:v>3489372249311910.15</ns0:v>
       </ns0:c>
       <ns0:c r="F23" s="1" t="n">
         <ns0:v>539260886.477125</ns0:v>
@@ -1870,6 +1870,12 @@
       </ns0:c>
       <ns0:c r="H24" s="1">
         <ns0:v>0</ns0:v>
+      </ns0:c>
+      <ns0:c r="I24" s="1" t="n">
+        <ns0:v>3323211666011343</ns0:v>
+      </ns0:c>
+      <ns0:c r="J24" s="1" t="n">
+        <ns0:v>3323211666011343</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="25">

</xml_diff>

<commit_message>
Freeze third early-game candidate: drone foundation, optional reactor automation, advanced DPS and conservative stage tuning
</commit_message>
<xml_diff>
--- a/space-battleship/config_excel/level.xlsx
+++ b/space-battleship/config_excel/level.xlsx
@@ -1493,7 +1493,7 @@
         </ns0:is>
       </ns0:c>
       <ns0:c r="D11" s="1" t="n">
-        <ns0:v>1469.771567969084</ns0:v>
+        <ns0:v>1543.26014636753820</ns0:v>
       </ns0:c>
       <ns0:c r="E11" s="1" t="n">
         <ns0:v>1469.771567969084</ns0:v>
@@ -1521,7 +1521,7 @@
         </ns0:is>
       </ns0:c>
       <ns0:c r="D12" s="1" t="n">
-        <ns0:v>9100.438150002134</ns0:v>
+        <ns0:v>9555.46005750224070</ns0:v>
       </ns0:c>
       <ns0:c r="E12" s="1" t="n">
         <ns0:v>9100.438150002134</ns0:v>
@@ -1549,7 +1549,7 @@
         </ns0:is>
       </ns0:c>
       <ns0:c r="D13" s="1" t="n">
-        <ns0:v>56347.51435316666</ns0:v>
+        <ns0:v>59164.8900708249930</ns0:v>
       </ns0:c>
       <ns0:c r="E13" s="1" t="n">
         <ns0:v>56347.51435316666</ns0:v>
@@ -1577,10 +1577,10 @@
         </ns0:is>
       </ns0:c>
       <ns0:c r="D14" s="1" t="n">
-        <ns0:v>602880.1175788565</ns0:v>
+        <ns0:v>663168.129336742150</ns0:v>
       </ns0:c>
       <ns0:c r="E14" s="1" t="n">
-        <ns0:v>602880.1175788565</ns0:v>
+        <ns0:v>633024.123457799325</ns0:v>
       </ns0:c>
       <ns0:c r="F14" s="1" t="n">
         <ns0:v>18120.833112711232</ns0:v>
@@ -1605,10 +1605,10 @@
         </ns0:is>
       </ns0:c>
       <ns0:c r="D15" s="1" t="n">
-        <ns0:v>6450407.623907364</ns0:v>
+        <ns0:v>7095448.38629810040</ns0:v>
       </ns0:c>
       <ns0:c r="E15" s="1" t="n">
-        <ns0:v>6450407.623907364</ns0:v>
+        <ns0:v>6772928.00510273220</ns0:v>
       </ns0:c>
       <ns0:c r="F15" s="1" t="n">
         <ns0:v>56917.67271450579</ns0:v>
@@ -1633,10 +1633,10 @@
         </ns0:is>
       </ns0:c>
       <ns0:c r="D16" s="1" t="n">
-        <ns0:v>69014978.76834521</ns0:v>
+        <ns0:v>75916476.645179720</ns0:v>
       </ns0:c>
       <ns0:c r="E16" s="1" t="n">
-        <ns0:v>69014978.76834521</ns0:v>
+        <ns0:v>72465727.706762460</ns0:v>
       </ns0:c>
       <ns0:c r="F16" s="1" t="n">
         <ns0:v>178778.836882676</ns0:v>
@@ -1661,10 +1661,10 @@
         </ns0:is>
       </ns0:c>
       <ns0:c r="D17" s="1" t="n">
-        <ns0:v>738413379.7593849</ns0:v>
+        <ns0:v>812254717.735323390</ns0:v>
       </ns0:c>
       <ns0:c r="E17" s="1" t="n">
-        <ns0:v>738413379.7593849</ns0:v>
+        <ns0:v>775334048.747354145</ns0:v>
       </ns0:c>
       <ns0:c r="F17" s="1" t="n">
         <ns0:v>561545.6675019113</ns0:v>
@@ -1689,10 +1689,10 @@
         </ns0:is>
       </ns0:c>
       <ns0:c r="D18" s="1" t="n">
-        <ns0:v>7900521439.525051</ns0:v>
+        <ns0:v>8690573583.47755610</ns0:v>
       </ns0:c>
       <ns0:c r="E18" s="1" t="n">
-        <ns0:v>7900521439.525051</ns0:v>
+        <ns0:v>8295547511.50130355</ns0:v>
       </ns0:c>
       <ns0:c r="F18" s="1" t="n">
         <ns0:v>1763819.1532541711</ns0:v>
@@ -1717,10 +1717,10 @@
         </ns0:is>
       </ns0:c>
       <ns0:c r="D19" s="1" t="n">
-        <ns0:v>84530211298.0865</ns0:v>
+        <ns0:v>92983232427.895150</ns0:v>
       </ns0:c>
       <ns0:c r="E19" s="1" t="n">
-        <ns0:v>84530211298.0865</ns0:v>
+        <ns0:v>88756721862.990825</ns0:v>
       </ns0:c>
       <ns0:c r="F19" s="1" t="n">
         <ns0:v>5540169.189134865</ns0:v>
@@ -1745,10 +1745,10 @@
         </ns0:is>
       </ns0:c>
       <ns0:c r="D20" s="1" t="n">
-        <ns0:v>904415825815.2517</ns0:v>
+        <ns0:v>994857408396.776870</ns0:v>
       </ns0:c>
       <ns0:c r="E20" s="1" t="n">
-        <ns0:v>904415825815.2517</ns0:v>
+        <ns0:v>949636617106.014285</ns0:v>
       </ns0:c>
       <ns0:c r="F20" s="1" t="n">
         <ns0:v>17401712.974718027</ns0:v>
@@ -1773,10 +1773,10 @@
         </ns0:is>
       </ns0:c>
       <ns0:c r="D21" s="1" t="n">
-        <ns0:v>9676634819953.418</ns0:v>
+        <ns0:v>10644298301948.75980</ns0:v>
       </ns0:c>
       <ns0:c r="E21" s="1" t="n">
-        <ns0:v>9676634819953.418</ns0:v>
+        <ns0:v>10160466560951.08890</ns0:v>
       </ns0:c>
       <ns0:c r="F21" s="1" t="n">
         <ns0:v>54658910.967619196</ns0:v>
@@ -1801,10 +1801,10 @@
         </ns0:is>
       </ns0:c>
       <ns0:c r="D22" s="1" t="n">
-        <ns0:v>103533417666955.5</ns0:v>
+        <ns0:v>113886759433651.050</ns0:v>
       </ns0:c>
       <ns0:c r="E22" s="1" t="n">
-        <ns0:v>103533417666955.5</ns0:v>
+        <ns0:v>108710088550303.275</ns0:v>
       </ns0:c>
       <ns0:c r="F22" s="1" t="n">
         <ns0:v>171684049.29483864</ns0:v>
@@ -1829,10 +1829,10 @@
         </ns0:is>
       </ns0:c>
       <ns0:c r="D23" s="1" t="n">
-        <ns0:v>3323211666011343</ns0:v>
+        <ns0:v>3655532832612477.30</ns0:v>
       </ns0:c>
       <ns0:c r="E23" s="1" t="n">
-        <ns0:v>3323211666011343</ns0:v>
+        <ns0:v>3489372249311910.15</ns0:v>
       </ns0:c>
       <ns0:c r="F23" s="1" t="n">
         <ns0:v>539260886.477125</ns0:v>
@@ -1870,6 +1870,12 @@
       </ns0:c>
       <ns0:c r="H24" s="1">
         <ns0:v>0</ns0:v>
+      </ns0:c>
+      <ns0:c r="I24" s="1" t="n">
+        <ns0:v>3323211666011343</ns0:v>
+      </ns0:c>
+      <ns0:c r="J24" s="1" t="n">
+        <ns0:v>3323211666011343</ns0:v>
       </ns0:c>
     </ns0:row>
     <ns0:row r="25">

</xml_diff>

<commit_message>
Calibrate early combat endpoints and taper stage 19 to preserve stage 20
</commit_message>
<xml_diff>
--- a/space-battleship/config_excel/level.xlsx
+++ b/space-battleship/config_excel/level.xlsx
@@ -1437,10 +1437,10 @@
         </ns0:is>
       </ns0:c>
       <ns0:c r="D9" s="1" t="n">
-        <ns0:v>15.40702157458636</ns0:v>
+        <ns0:v>10.784915102210451</ns0:v>
       </ns0:c>
       <ns0:c r="E9" s="1" t="n">
-        <ns0:v>15.40702157458636</ns0:v>
+        <ns0:v>10.784915102210451</ns0:v>
       </ns0:c>
       <ns0:c r="F9" s="1" t="n">
         <ns0:v>3.600</ns0:v>
@@ -1465,10 +1465,10 @@
         </ns0:is>
       </ns0:c>
       <ns0:c r="D10" s="1" t="n">
-        <ns0:v>237.3763137997695</ns0:v>
+        <ns0:v>154.29460396985016</ns0:v>
       </ns0:c>
       <ns0:c r="E10" s="1" t="n">
-        <ns0:v>237.3763137997695</ns0:v>
+        <ns0:v>154.29460396985016</ns0:v>
       </ns0:c>
       <ns0:c r="F10" s="1" t="n">
         <ns0:v>22.2902511206399880</ns0:v>
@@ -1493,10 +1493,10 @@
         </ns0:is>
       </ns0:c>
       <ns0:c r="D11" s="1" t="n">
-        <ns0:v>1543.26014636753820</ns0:v>
+        <ns0:v>925.956087820523</ns0:v>
       </ns0:c>
       <ns0:c r="E11" s="1" t="n">
-        <ns0:v>1469.771567969084</ns0:v>
+        <ns0:v>881.8629407814503</ns0:v>
       </ns0:c>
       <ns0:c r="F11" s="1" t="n">
         <ns0:v>23.462611153778531700</ns0:v>
@@ -1521,10 +1521,10 @@
         </ns0:is>
       </ns0:c>
       <ns0:c r="D12" s="1" t="n">
-        <ns0:v>9555.46005750224070</ns0:v>
+        <ns0:v>5255.503031626232</ns0:v>
       </ns0:c>
       <ns0:c r="E12" s="1" t="n">
-        <ns0:v>9100.438150002134</ns0:v>
+        <ns0:v>5005.240982501173</ns0:v>
       </ns0:c>
       <ns0:c r="F12" s="1" t="n">
         <ns0:v>145.2743040454589340</ns0:v>
@@ -1549,10 +1549,10 @@
         </ns0:is>
       </ns0:c>
       <ns0:c r="D13" s="1" t="n">
-        <ns0:v>59164.8900708249930</ns0:v>
+        <ns0:v>29582.445035412493</ns0:v>
       </ns0:c>
       <ns0:c r="E13" s="1" t="n">
-        <ns0:v>56347.51435316666</ns0:v>
+        <ns0:v>28173.757176583327</ns0:v>
       </ns0:c>
       <ns0:c r="F13" s="1" t="n">
         <ns0:v>899.5001995970796120</ns0:v>
@@ -1577,10 +1577,10 @@
         </ns0:is>
       </ns0:c>
       <ns0:c r="D14" s="1" t="n">
-        <ns0:v>663168.129336742150</ns0:v>
+        <ns0:v>557061.2286428633</ns0:v>
       </ns0:c>
       <ns0:c r="E14" s="1" t="n">
-        <ns0:v>633024.123457799325</ns0:v>
+        <ns0:v>553896.1080255744</ns0:v>
       </ns0:c>
       <ns0:c r="F14" s="1" t="n">
         <ns0:v>18120.833112711232</ns0:v>
@@ -1605,10 +1605,10 @@
         </ns0:is>
       </ns0:c>
       <ns0:c r="D15" s="1" t="n">
-        <ns0:v>7095448.38629810040</ns0:v>
+        <ns0:v>7152211.973388486</ns0:v>
       </ns0:c>
       <ns0:c r="E15" s="1" t="n">
-        <ns0:v>6772928.00510273220</ns0:v>
+        <ns0:v>7407890.0055811135</ns0:v>
       </ns0:c>
       <ns0:c r="F15" s="1" t="n">
         <ns0:v>56917.67271450579</ns0:v>
@@ -1633,10 +1633,10 @@
         </ns0:is>
       </ns0:c>
       <ns0:c r="D16" s="1" t="n">
-        <ns0:v>75916476.645179720</ns0:v>
+        <ns0:v>91828570.15000938</ns0:v>
       </ns0:c>
       <ns0:c r="E16" s="1" t="n">
-        <ns0:v>72465727.706762460</ns0:v>
+        <ns0:v>99074237.09908931</ns0:v>
       </ns0:c>
       <ns0:c r="F16" s="1" t="n">
         <ns0:v>178778.836882676</ns0:v>
@@ -1661,10 +1661,10 @@
         </ns0:is>
       </ns0:c>
       <ns0:c r="D17" s="1" t="n">
-        <ns0:v>812254717.735323390</ns0:v>
+        <ns0:v>1179003967.8871765</ns0:v>
       </ns0:c>
       <ns0:c r="E17" s="1" t="n">
-        <ns0:v>775334048.747354145</ns0:v>
+        <ns0:v>1325033774.7147167</ns0:v>
       </ns0:c>
       <ns0:c r="F17" s="1" t="n">
         <ns0:v>561545.6675019113</ns0:v>
@@ -1689,10 +1689,10 @@
         </ns0:is>
       </ns0:c>
       <ns0:c r="D18" s="1" t="n">
-        <ns0:v>8690573583.47755610</ns0:v>
+        <ns0:v>15137449641.467207</ns0:v>
       </ns0:c>
       <ns0:c r="E18" s="1" t="n">
-        <ns0:v>8295547511.50130355</ns0:v>
+        <ns0:v>17721201349.032326</ns0:v>
       </ns0:c>
       <ns0:c r="F18" s="1" t="n">
         <ns0:v>1763819.1532541711</ns0:v>
@@ -1717,10 +1717,10 @@
         </ns0:is>
       </ns0:c>
       <ns0:c r="D19" s="1" t="n">
-        <ns0:v>92983232427.895150</ns0:v>
+        <ns0:v>194352511008.58322</ns0:v>
       </ns0:c>
       <ns0:c r="E19" s="1" t="n">
-        <ns0:v>88756721862.990825</ns0:v>
+        <ns0:v>237006016937.61285</ns0:v>
       </ns0:c>
       <ns0:c r="F19" s="1" t="n">
         <ns0:v>5540169.189134865</ns0:v>
@@ -1745,10 +1745,10 @@
         </ns0:is>
       </ns0:c>
       <ns0:c r="D20" s="1" t="n">
-        <ns0:v>994857408396.776870</ns0:v>
+        <ns0:v>2495327775153.562</ns0:v>
       </ns0:c>
       <ns0:c r="E20" s="1" t="n">
-        <ns0:v>949636617106.014285</ns0:v>
+        <ns0:v>3169754180785.227</ns0:v>
       </ns0:c>
       <ns0:c r="F20" s="1" t="n">
         <ns0:v>17401712.974718027</ns0:v>
@@ -1773,10 +1773,10 @@
         </ns0:is>
       </ns0:c>
       <ns0:c r="D21" s="1" t="n">
-        <ns0:v>10644298301948.75980</ns0:v>
+        <ns0:v>32037974056212.92</ns0:v>
       </ns0:c>
       <ns0:c r="E21" s="1" t="n">
-        <ns0:v>10160466560951.08890</ns0:v>
+        <ns0:v>42392770008240.72</ns0:v>
       </ns0:c>
       <ns0:c r="F21" s="1" t="n">
         <ns0:v>54658910.967619196</ns0:v>

</xml_diff>

<commit_message>
Raise midgame investment thresholds with a bounded stage 11-20 ramp
</commit_message>
<xml_diff>
--- a/space-battleship/config_excel/level.xlsx
+++ b/space-battleship/config_excel/level.xlsx
@@ -1577,10 +1577,10 @@
         </ns0:is>
       </ns0:c>
       <ns0:c r="D14" s="1" t="n">
-        <ns0:v>557061.2286428633</ns0:v>
+        <ns0:v>603482.9976964353</ns0:v>
       </ns0:c>
       <ns0:c r="E14" s="1" t="n">
-        <ns0:v>553896.1080255744</ns0:v>
+        <ns0:v>797610.3955568272</ns0:v>
       </ns0:c>
       <ns0:c r="F14" s="1" t="n">
         <ns0:v>18120.833112711232</ns0:v>
@@ -1605,10 +1605,10 @@
         </ns0:is>
       </ns0:c>
       <ns0:c r="D15" s="1" t="n">
-        <ns0:v>7152211.973388486</ns0:v>
+        <ns0:v>8393915.440990653</ns0:v>
       </ns0:c>
       <ns0:c r="E15" s="1" t="n">
-        <ns0:v>7407890.0055811135</ns0:v>
+        <ns0:v>15361000.715572996</ns0:v>
       </ns0:c>
       <ns0:c r="F15" s="1" t="n">
         <ns0:v>56917.67271450579</ns0:v>
@@ -1633,10 +1633,10 @@
         </ns0:is>
       </ns0:c>
       <ns0:c r="D16" s="1" t="n">
-        <ns0:v>91828570.15000938</ns0:v>
+        <ns0:v>116751949.4326219</ns0:v>
       </ns0:c>
       <ns0:c r="E16" s="1" t="n">
-        <ns0:v>99074237.09908931</ns0:v>
+        <ns0:v>295834086.7900871</ns0:v>
       </ns0:c>
       <ns0:c r="F16" s="1" t="n">
         <ns0:v>178778.836882676</ns0:v>
@@ -1661,10 +1661,10 @@
         </ns0:is>
       </ns0:c>
       <ns0:c r="D17" s="1" t="n">
-        <ns0:v>1179003967.8871765</ns0:v>
+        <ns0:v>1623916489.5267003</ns0:v>
       </ns0:c>
       <ns0:c r="E17" s="1" t="n">
-        <ns0:v>1325033774.7147167</ns0:v>
+        <ns0:v>5697402697.091157</ns0:v>
       </ns0:c>
       <ns0:c r="F17" s="1" t="n">
         <ns0:v>561545.6675019113</ns0:v>
@@ -1689,10 +1689,10 @@
         </ns0:is>
       </ns0:c>
       <ns0:c r="D18" s="1" t="n">
-        <ns0:v>15137449641.467207</ns0:v>
+        <ns0:v>19981023505.47505</ns0:v>
       </ns0:c>
       <ns0:c r="E18" s="1" t="n">
-        <ns0:v>17721201349.032326</ns0:v>
+        <ns0:v>76197922112.14407</ns0:v>
       </ns0:c>
       <ns0:c r="F18" s="1" t="n">
         <ns0:v>1763819.1532541711</ns0:v>
@@ -1717,10 +1717,10 @@
         </ns0:is>
       </ns0:c>
       <ns0:c r="D19" s="1" t="n">
-        <ns0:v>194352511008.58322</ns0:v>
+        <ns0:v>245850881434.616</ns0:v>
       </ns0:c>
       <ns0:c r="E19" s="1" t="n">
-        <ns0:v>237006016937.61285</ns0:v>
+        <ns0:v>1019082491250.3948</ns0:v>
       </ns0:c>
       <ns0:c r="F19" s="1" t="n">
         <ns0:v>5540169.189134865</ns0:v>
@@ -1745,10 +1745,10 @@
         </ns0:is>
       </ns0:c>
       <ns0:c r="D20" s="1" t="n">
-        <ns0:v>2495327775153.562</ns0:v>
+        <ns0:v>3025002992745.369</ns0:v>
       </ns0:c>
       <ns0:c r="E20" s="1" t="n">
-        <ns0:v>3169754180785.227</ns0:v>
+        <ns0:v>13629362785571.225</ns0:v>
       </ns0:c>
       <ns0:c r="F20" s="1" t="n">
         <ns0:v>17401712.974718027</ns0:v>
@@ -1773,10 +1773,10 @@
         </ns0:is>
       </ns0:c>
       <ns0:c r="D21" s="1" t="n">
-        <ns0:v>32037974056212.92</ns0:v>
+        <ns0:v>37220298144637.94</ns0:v>
       </ns0:c>
       <ns0:c r="E21" s="1" t="n">
-        <ns0:v>42392770008240.72</ns0:v>
+        <ns0:v>182281151462812.78</ns0:v>
       </ns0:c>
       <ns0:c r="F21" s="1" t="n">
         <ns0:v>54658910.967619196</ns0:v>
@@ -1801,10 +1801,10 @@
         </ns0:is>
       </ns0:c>
       <ns0:c r="D22" s="1" t="n">
-        <ns0:v>113886759433651.050</ns0:v>
+        <ns0:v>457966685420846.8</ns0:v>
       </ns0:c>
       <ns0:c r="E22" s="1" t="n">
-        <ns0:v>108710088550303.275</ns0:v>
+        <ns0:v>2437855584399305.5</ns0:v>
       </ns0:c>
       <ns0:c r="F22" s="1" t="n">
         <ns0:v>171684049.29483864</ns0:v>
@@ -1829,10 +1829,10 @@
         </ns0:is>
       </ns0:c>
       <ns0:c r="D23" s="1" t="n">
-        <ns0:v>3655532832612477.30</ns0:v>
+        <ns0:v>1.6904766652351906e+16</ns0:v>
       </ns0:c>
       <ns0:c r="E23" s="1" t="n">
-        <ns0:v>3489372249311910.15</ns0:v>
+        <ns0:v>9.781274370980717e+16</ns0:v>
       </ns0:c>
       <ns0:c r="F23" s="1" t="n">
         <ns0:v>539260886.477125</ns0:v>

</xml_diff>

<commit_message>
balance: replace stage14 firing wall with reward-bound mixed fleets and shorter boss
</commit_message>
<xml_diff>
--- a/space-battleship/config_excel/level.xlsx
+++ b/space-battleship/config_excel/level.xlsx
@@ -1123,7 +1123,7 @@
     <ns0:outlinePr summaryBelow="1" summaryRight="1"/>
     <ns0:pageSetUpPr/>
   </ns0:sheetPr>
-  <ns0:dimension ref="A1:J223"/>
+  <ns0:dimension ref="A1:K223"/>
   <ns0:sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="14.4"/>
   <ns0:cols>
     <ns0:col width="78.2222222222222" customWidth="1" style="2" min="3" max="3"/>
@@ -1184,6 +1184,11 @@
           <ns0:t>entryLifeRatio</ns0:t>
         </ns0:is>
       </ns0:c>
+      <ns0:c r="K1" t="inlineStr">
+        <ns0:is>
+          <ns0:t>rewardReferenceGroups</ns0:t>
+        </ns0:is>
+      </ns0:c>
     </ns0:row>
     <ns0:row r="2">
       <ns0:c r="A2" s="1" t="inlineStr">
@@ -1236,6 +1241,11 @@
           <ns0:t>首战点生命倍率（可选）</ns0:t>
         </ns0:is>
       </ns0:c>
+      <ns0:c r="K2" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Optional existing candidate reward references</ns0:t>
+        </ns0:is>
+      </ns0:c>
     </ns0:row>
     <ns0:row r="3">
       <ns0:c r="A3" s="1" t="inlineStr">
@@ -1281,6 +1291,11 @@
       <ns0:c r="J3" t="inlineStr">
         <ns0:is>
           <ns0:t>正有限数；空值继承上一关终点</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="K3" t="inlineStr">
+        <ns0:is>
+          <ns0:t>json</ns0:t>
         </ns0:is>
       </ns0:c>
     </ns0:row>
@@ -1674,6 +1689,11 @@
       </ns0:c>
       <ns0:c r="H17" s="1">
         <ns0:v>0</ns0:v>
+      </ns0:c>
+      <ns0:c r="K17" t="inlineStr">
+        <ns0:is>
+          <ns0:t>[{"id":34146,"position":0.6},{"id":34147,"position":0.7},{"id":34148,"position":0.8},{"id":34149,"position":0.9}]</ns0:t>
+        </ns0:is>
       </ns0:c>
     </ns0:row>
     <ns0:row r="18">

</xml_diff>

<commit_message>
Balance weapon roles and shield recovery with scale evidence
</commit_message>
<xml_diff>
--- a/space-battleship/config_excel/level.xlsx
+++ b/space-battleship/config_excel/level.xlsx
@@ -1293,14 +1293,14 @@
       </ns0:c>
       <ns0:c r="C4" s="1" t="inlineStr">
         <ns0:is>
-          <ns0:t>{33001|0.140000,33002|0.325000,33003|0.510000,33004|0.695000,33005|0.880000}</ns0:t>
+          <ns0:t>{30011|0.180000,30012|0.360000,30013|0.540000,30014|0.720000,30015|0.900000}</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="D4" s="1" t="n">
         <ns0:v>1</ns0:v>
       </ns0:c>
       <ns0:c r="E4" s="1" t="n">
-        <ns0:v>1.0</ns0:v>
+        <ns0:v>.40</ns0:v>
       </ns0:c>
       <ns0:c r="F4" s="1" t="n">
         <ns0:v>1.0</ns0:v>
@@ -1321,17 +1321,17 @@
       </ns0:c>
       <ns0:c r="C5" s="1" t="inlineStr">
         <ns0:is>
-          <ns0:t>{33006|0.140000,33007|0.288000,33008|0.436000,33009|0.584000,33010|0.732000,33011|0.880000}</ns0:t>
+          <ns0:t>{30021|0.180000,30022|0.360000,30023|0.540000,30024|0.720000,30025|0.900000}</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="D5" s="1" t="n">
         <ns0:v>1.5</ns0:v>
       </ns0:c>
       <ns0:c r="E5" s="1" t="n">
-        <ns0:v>1.6</ns0:v>
+        <ns0:v>3.2</ns0:v>
       </ns0:c>
       <ns0:c r="F5" s="1" t="n">
-        <ns0:v>1.15</ns0:v>
+        <ns0:v>0.7</ns0:v>
       </ns0:c>
       <ns0:c r="G5" s="1" t="n">
         <ns0:v>1.2</ns0:v>
@@ -1349,17 +1349,17 @@
       </ns0:c>
       <ns0:c r="C6" s="1" t="inlineStr">
         <ns0:is>
-          <ns0:t>{33012|0.140000,33013|0.263333,33014|0.386667,33015|0.510000,33016|0.633333,33017|0.756667,33018|0.880000}</ns0:t>
+          <ns0:t>{30031|0.180000,30032|0.360000,30033|0.540000,30034|0.720000,30035|0.900000}</ns0:t>
         </ns0:is>
       </ns0:c>
       <ns0:c r="D6" s="1" t="n">
         <ns0:v>2</ns0:v>
       </ns0:c>
       <ns0:c r="E6" s="1" t="n">
-        <ns0:v>2.2</ns0:v>
+        <ns0:v>4.00</ns0:v>
       </ns0:c>
       <ns0:c r="F6" s="1" t="n">
-        <ns0:v>1.6</ns0:v>
+        <ns0:v>0.98</ns0:v>
       </ns0:c>
       <ns0:c r="G6" s="1" t="n">
         <ns0:v>1.4</ns0:v>

</xml_diff>

<commit_message>
Design stage 1-7 encounter themes and pacing candidate
</commit_message>
<xml_diff>
--- a/space-battleship/config_excel/level.xlsx
+++ b/space-battleship/config_excel/level.xlsx
@@ -1469,7 +1469,7 @@
         <ns0:v>6</ns0:v>
       </ns0:c>
       <ns0:c r="B9" s="1" t="n">
-        <ns0:v>1000</ns0:v>
+        <ns0:v>2200</ns0:v>
       </ns0:c>
       <ns0:c r="C9" s="1" t="inlineStr">
         <ns0:is>
@@ -1502,7 +1502,7 @@
         <ns0:v>7</ns0:v>
       </ns0:c>
       <ns0:c r="B10" s="1" t="n">
-        <ns0:v>1000</ns0:v>
+        <ns0:v>2200</ns0:v>
       </ns0:c>
       <ns0:c r="C10" s="1" t="inlineStr">
         <ns0:is>

</xml_diff>